<commit_message>
Powtorna kontrola: napraw zbyt agresywne scalanie wariantow, odzyskaj 70 pytan
Reguła scalania wariantow grupowala pytania po poczatku tresci, przez co
laczyla ROZNE pytania majace ten sam stem (Digoksyna:, Kwas acetylosalicylowy:,
Wskaz prawdziwe polaczenie lek-wskazanie:) i kasowala je.

- warianty scalane teraz tylko gdy maja tyle samo opcji i kazda para
  odpowiada sobie tekstowo (jedna jest prefiksem drugiej)
- odzyskane 70 pytan: 802 -> 872
- poprawiony 1 artefakt: numer strony wklejony w tresc opcji

Kontrole: integralnosc 5 plikow bez zastrzezen; weryfikacja wzrokowa 2 nowych
stron PDF 13/13 zgodnych; 0 utraconych opcji przy wyborze wariantu; audyt
zanieczyszczen 0 trafien; importer 1085/1240.

Udokumentowane 5 przypadkow, gdzie zrodlo samo sobie przeczy miedzy latami.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sDWkA2eXfHxFn4vQGjL1J
</commit_message>
<xml_diff>
--- a/farmakologia_ARCYBAZA_OnlyPharms.xlsx
+++ b/farmakologia_ARCYBAZA_OnlyPharms.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Pytania" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pytania'!$A$1:$Q$803</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pytania'!$A$1:$Q$873</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,5 +424,5 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"><sheetPr><outlinePr summaryBelow="1" summaryRight="1" /><pageSetUpPr /></sheetPr><dimension ref="A1:Q803" /><sheetFormatPr baseColWidth="8" defaultRowHeight="15" /><cols><col width="30" customWidth="1" min="1" max="1" /><col width="21" customWidth="1" min="2" max="2" /><col width="9" customWidth="1" min="3" max="3" /><col width="9" customWidth="1" min="4" max="4" /><col width="60" customWidth="1" min="5" max="5" /><col width="32" customWidth="1" min="6" max="6" /><col width="32" customWidth="1" min="7" max="7" /><col width="32" customWidth="1" min="8" max="8" /><col width="32" customWidth="1" min="9" max="9" /><col width="32" customWidth="1" min="10" max="10" /><col width="32" customWidth="1" min="11" max="11" /><col width="32" customWidth="1" min="12" max="12" /><col width="32" customWidth="1" min="13" max="13" /><col width="32" customWidth="1" min="14" max="14" /><col width="32" customWidth="1" min="15" max="15" /><col width="26" customWidth="1" min="16" max="16" /><col width="10" customWidth="1" min="17" max="17" /></cols><sheetData><row r="1"><c r="A1" s="1" t="inlineStr"><is><t>Section</t></is></c><c r="B1" s="1" t="inlineStr"><is><t>Category</t></is></c><c r="C1" s="1" t="inlineStr"><is><t>Poziom</t></is></c><c r="D1" s="1" t="inlineStr"><is><t>Type</t></is></c><c r="E1" s="1" t="inlineStr"><is><t>Question</t></is></c><c r="F1" s="1" t="inlineStr"><is><t>True 1</t></is></c><c r="G1" s="1" t="inlineStr"><is><t>True 2</t></is></c><c r="H1" s="1" t="inlineStr"><is><t>True 3</t></is></c><c r="I1" s="1" t="inlineStr"><is><t>True 4</t></is></c><c r="J1" s="1" t="inlineStr"><is><t>True 5</t></is></c><c r="K1" s="1" t="inlineStr"><is><t>False 1</t></is></c><c r="L1" s="1" t="inlineStr"><is><t>False 2</t></is></c><c r="M1" s="1" t="inlineStr"><is><t>False 3</t></is></c><c r="N1" s="1" t="inlineStr"><is><t>False 4</t></is></c><c r="O1" s="1" t="inlineStr"><is><t>False 5</t></is></c><c r="P1" s="1" t="inlineStr"><is><t>Zrodlo</t></is></c><c r="Q1" s="1" t="inlineStr"><is><t>Pewnosc</t></is></c></row><row r="2"><c r="A2" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B2" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C2" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D2" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E2" s="2" t="inlineStr"><is><t>Czarne zabarwienie stolca powoduje podanie preparatów:</t></is></c><c r="F2" s="2" t="inlineStr"><is><t>Bizmutu</t></is></c><c r="G2" s="2" t="inlineStr"><is><t>Żelaza</t></is></c><c r="H2" s="2" t="inlineStr" /><c r="I2" s="2" t="inlineStr" /><c r="J2" s="2" t="inlineStr" /><c r="K2" s="2" t="inlineStr"><is><t>Wapnia</t></is></c><c r="L2" s="2" t="inlineStr"><is><t>Glinu</t></is></c><c r="M2" s="2" t="inlineStr" /><c r="N2" s="2" t="inlineStr" /><c r="O2" s="2" t="inlineStr" /><c r="P2" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q2" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="3"><c r="A3" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B3" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C3" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D3" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E3" s="2" t="inlineStr"><is><t>Uzasadnionym wskazaniem do przewlekłego stosowania inhibitorów pompy protonowej jest:</t></is></c><c r="F3" s="2" t="inlineStr"><is><t>Choroba refluksowa żołądka</t></is></c><c r="G3" s="2" t="inlineStr"><is><t>Profilaktyka gastropatii u osób leczonych niesteroidowymi lekami przeciwzapalnymi powyżej 65 r.ż</t></is></c><c r="H3" s="2" t="inlineStr"><is><t>Eradykacja Helicobacter Pylori</t></is></c><c r="I3" s="2" t="inlineStr" /><c r="J3" s="2" t="inlineStr" /><c r="K3" s="2" t="inlineStr"><is><t>Profilaktyka wrzodów stresowych</t></is></c><c r="L3" s="2" t="inlineStr" /><c r="M3" s="2" t="inlineStr" /><c r="N3" s="2" t="inlineStr" /><c r="O3" s="2" t="inlineStr" /><c r="P3" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q3" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="4"><c r="A4" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B4" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C4" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D4" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E4" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek – wskazanie</t></is></c><c r="F4" s="2" t="inlineStr"><is><t>Mesalazyna – choroba Leśniowskiego crohna</t></is></c><c r="G4" s="2" t="inlineStr"><is><t>Rifaksymina – biegunka podróżnych</t></is></c><c r="H4" s="2" t="inlineStr"><is><t>Metylonaltrekson – zaparcia w trakcie terapii opioidami</t></is></c><c r="I4" s="2" t="inlineStr" /><c r="J4" s="2" t="inlineStr" /><c r="K4" s="2" t="inlineStr"><is><t>Racekadotryl – śpiączka wątrobowa</t></is></c><c r="L4" s="2" t="inlineStr" /><c r="M4" s="2" t="inlineStr" /><c r="N4" s="2" t="inlineStr" /><c r="O4" s="2" t="inlineStr" /><c r="P4" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q4" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="5"><c r="A5" s="2" t="inlineStr"><is><t>ZNIECZULENIA OGÓLNE</t></is></c><c r="B5" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C5" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D5" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E5" s="2" t="inlineStr"><is><t>Do leków które wykazują miejscowe działanie przeciwbólowe po podaniu na skórę należy:</t></is></c><c r="F5" s="2" t="inlineStr"><is><t>Kapsaicyna</t></is></c><c r="G5" s="2" t="inlineStr"><is><t>Ketoprofen</t></is></c><c r="H5" s="2" t="inlineStr" /><c r="I5" s="2" t="inlineStr" /><c r="J5" s="2" t="inlineStr" /><c r="K5" s="2" t="inlineStr"><is><t>Propofol</t></is></c><c r="L5" s="2" t="inlineStr"><is><t>Tiopental</t></is></c><c r="M5" s="2" t="inlineStr" /><c r="N5" s="2" t="inlineStr" /><c r="O5" s="2" t="inlineStr" /><c r="P5" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q5" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="6"><c r="A6" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B6" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C6" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D6" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E6" s="2" t="inlineStr"><is><t>Ryzyko uszkodzenia wątroby przez paracetamol rośnie w przypadku:</t></is></c><c r="F6" s="2" t="inlineStr"><is><t>Zespołu zależności alkoholowej (ZAA)</t></is></c><c r="G6" s="2" t="inlineStr"><is><t>Wygłodzenia (kacheksji)</t></is></c><c r="H6" s="2" t="inlineStr"><is><t>Indukcji enzymów mikrosomalnych wątroby</t></is></c><c r="I6" s="2" t="inlineStr"><is><t>Przedawkowania</t></is></c><c r="J6" s="2" t="inlineStr" /><c r="K6" s="2" t="inlineStr" /><c r="L6" s="2" t="inlineStr" /><c r="M6" s="2" t="inlineStr" /><c r="N6" s="2" t="inlineStr" /><c r="O6" s="2" t="inlineStr" /><c r="P6" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q6" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="7"><c r="A7" s="2" t="inlineStr"><is><t>BÓLE GŁOWY</t></is></c><c r="B7" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C7" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D7" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E7" s="2" t="inlineStr"><is><t>W przerywaniu bólów migrenowych stosuje się:</t></is></c><c r="F7" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="G7" s="2" t="inlineStr"><is><t>Dihydroergotaminę</t></is></c><c r="H7" s="2" t="inlineStr"><is><t>Zolmitryptan</t></is></c><c r="I7" s="2" t="inlineStr" /><c r="J7" s="2" t="inlineStr" /><c r="K7" s="2" t="inlineStr"><is><t>Morfinę</t></is></c><c r="L7" s="2" t="inlineStr" /><c r="M7" s="2" t="inlineStr" /><c r="N7" s="2" t="inlineStr" /><c r="O7" s="2" t="inlineStr" /><c r="P7" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q7" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="8"><c r="A8" s="2" t="inlineStr"><is><t>JASKRA</t></is></c><c r="B8" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C8" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D8" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E8" s="2" t="inlineStr"><is><t>Analogi prostaglandyny E1 mogą powodować</t></is></c><c r="F8" s="2" t="inlineStr"><is><t>Hamowanie wydzielania soku żołądkowego</t></is></c><c r="G8" s="2" t="inlineStr" /><c r="H8" s="2" t="inlineStr" /><c r="I8" s="2" t="inlineStr" /><c r="J8" s="2" t="inlineStr" /><c r="K8" s="2" t="inlineStr"><is><t>Poprawę odpływu cieczy wodnistej z oka</t></is></c><c r="L8" s="2" t="inlineStr"><is><t>Rozszerzanie naczyń krwionośnych tętniczych</t></is></c><c r="M8" s="2" t="inlineStr"><is><t>Hamowanie agregacji płytek krwi</t></is></c><c r="N8" s="2" t="inlineStr" /><c r="O8" s="2" t="inlineStr" /><c r="P8" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q8" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="9"><c r="A9" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B9" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C9" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D9" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E9" s="2" t="inlineStr"><is><t>Substytucja enzymów trzustkowych jest wskazana:</t></is></c><c r="F9" s="2" t="inlineStr"><is><t>W mukowiscydozie</t></is></c><c r="G9" s="2" t="inlineStr"><is><t>Po resekcji trzustki</t></is></c><c r="H9" s="2" t="inlineStr" /><c r="I9" s="2" t="inlineStr" /><c r="J9" s="2" t="inlineStr" /><c r="K9" s="2" t="inlineStr"><is><t>W cukrzycy typu 1</t></is></c><c r="L9" s="2" t="inlineStr"><is><t>W anoreksji</t></is></c><c r="M9" s="2" t="inlineStr" /><c r="N9" s="2" t="inlineStr" /><c r="O9" s="2" t="inlineStr" /><c r="P9" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q9" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="10"><c r="A10" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B10" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C10" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D10" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E10" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek – wskazanie do podania:</t></is></c><c r="F10" s="2" t="inlineStr"><is><t>Haloperydol – agresja u pacjentów z ograniczonym uszkodzeniem mózgu</t></is></c><c r="G10" s="2" t="inlineStr"><is><t>Betahistyna – zawroty głowy w przebiegu choroby Meniere’a</t></is></c><c r="H10" s="2" t="inlineStr"><is><t>Topiramat – profilaktyka migreny</t></is></c><c r="I10" s="2" t="inlineStr"><is><t>Lamotrygina – profilaktyka choroby afektywnej dwubiegunowej</t></is></c><c r="J10" s="2" t="inlineStr" /><c r="K10" s="2" t="inlineStr" /><c r="L10" s="2" t="inlineStr" /><c r="M10" s="2" t="inlineStr" /><c r="N10" s="2" t="inlineStr" /><c r="O10" s="2" t="inlineStr" /><c r="P10" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q10" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="11"><c r="A11" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B11" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C11" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D11" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E11" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy:</t></is></c><c r="F11" s="2" t="inlineStr"><is><t>może być przyczyną wystąpienia szczególnej postaci astmy</t></is></c><c r="G11" s="2" t="inlineStr"><is><t>nieodwracalnie hamuje COX</t></is></c><c r="H11" s="2" t="inlineStr" /><c r="I11" s="2" t="inlineStr" /><c r="J11" s="2" t="inlineStr" /><c r="K11" s="2" t="inlineStr"><is><t>zwiększa ryzyko sercowo-naczyniowe</t></is></c><c r="L11" s="2" t="inlineStr"><is><t>podawany łącznie z ibuprofenem wykazuje silniejszy efekt przeciwzapalny</t></is></c><c r="M11" s="2" t="inlineStr" /><c r="N11" s="2" t="inlineStr" /><c r="O11" s="2" t="inlineStr" /><c r="P11" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q11" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="12"><c r="A12" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B12" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C12" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D12" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E12" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące leczenia heparyną niefrakcjonowaną:</t></is></c><c r="F12" s="2" t="inlineStr"><is><t>Może być podawana podskórnie ale jej biodostępność jest wtedy mała i zmienna osobniczo</t></is></c><c r="G12" s="2" t="inlineStr"><is><t>Białka osoczowe mogą zmniejszać jej działanie przeciwkrzepliwe i być przyczyną oporności na leczenie</t></is></c><c r="H12" s="2" t="inlineStr"><is><t>Przedłużenie aPTT 1,5-2 razy w stosunku do wartości wyjściowej jest pożądanym efektem terapeutycznym</t></is></c><c r="I12" s="2" t="inlineStr"><is><t>Jej antidotum jest siarczan protaminy</t></is></c><c r="J12" s="2" t="inlineStr" /><c r="K12" s="2" t="inlineStr" /><c r="L12" s="2" t="inlineStr" /><c r="M12" s="2" t="inlineStr" /><c r="N12" s="2" t="inlineStr" /><c r="O12" s="2" t="inlineStr" /><c r="P12" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q12" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="13"><c r="A13" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B13" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C13" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D13" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E13" s="2" t="inlineStr"><is><t>Przeciwwskazaniem do podania cholinolityków jest:</t></is></c><c r="F13" s="2" t="inlineStr"><is><t>Rozrost gruczołu krokowego</t></is></c><c r="G13" s="2" t="inlineStr"><is><t>Jaskra</t></is></c><c r="H13" s="2" t="inlineStr" /><c r="I13" s="2" t="inlineStr" /><c r="J13" s="2" t="inlineStr" /><c r="K13" s="2" t="inlineStr"><is><t>Choroba wrzodowa żołądka i dwunastnicy</t></is></c><c r="L13" s="2" t="inlineStr"><is><t>Choroba lokomocyjna</t></is></c><c r="M13" s="2" t="inlineStr" /><c r="N13" s="2" t="inlineStr" /><c r="O13" s="2" t="inlineStr" /><c r="P13" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q13" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="14"><c r="A14" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B14" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C14" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D14" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E14" s="2" t="inlineStr"><is><t>Warfaryna:</t></is></c><c r="F14" s="2" t="inlineStr"><is><t>Jest sotosowana w profilaktyce i leczeniu żylnej choroby zakrzepowo-zatorowej</t></is></c><c r="G14" s="2" t="inlineStr"><is><t>Może być przyczyną zespołu purpurowego palucha</t></is></c><c r="H14" s="2" t="inlineStr" /><c r="I14" s="2" t="inlineStr" /><c r="J14" s="2" t="inlineStr" /><c r="K14" s="2" t="inlineStr"><is><t>Wymaga utrzymania INR&gt;4</t></is></c><c r="L14" s="2" t="inlineStr"><is><t>Jest eliminowana niezmieniona przez nerki</t></is></c><c r="M14" s="2" t="inlineStr" /><c r="N14" s="2" t="inlineStr" /><c r="O14" s="2" t="inlineStr" /><c r="P14" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q14" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="15"><c r="A15" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B15" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C15" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D15" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E15" s="2" t="inlineStr"><is><t>Fondaparynuks:</t></is></c><c r="F15" s="2" t="inlineStr"><is><t>Jest stosowana u osób z zawałem serca z przetrwałym uniesieniem odcinka ST (STEMI) oraz bez jego uniesienia (NSTEMI)</t></is></c><c r="G15" s="2" t="inlineStr" /><c r="H15" s="2" t="inlineStr" /><c r="I15" s="2" t="inlineStr" /><c r="J15" s="2" t="inlineStr" /><c r="K15" s="2" t="inlineStr"><is><t>Wybiórczo hamuje czynnik IIa</t></is></c><c r="L15" s="2" t="inlineStr"><is><t>W zalecanych dawkach hamuje istotnie wydłuża aPTT</t></is></c><c r="M15" s="2" t="inlineStr"><is><t>Nie jest wydalany przez nerki i może być stosowany u pacjentów z klirensem kreatyniny poniżej 30ml/min</t></is></c><c r="N15" s="2" t="inlineStr" /><c r="O15" s="2" t="inlineStr" /><c r="P15" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q15" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="16"><c r="A16" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B16" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C16" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D16" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E16" s="2" t="inlineStr"><is><t>Bezpośrednim inhibitorem trombiny podawanym dożylnie jest:</t></is></c><c r="F16" s="2" t="inlineStr"><is><t>Argatroban</t></is></c><c r="G16" s="2" t="inlineStr"><is><t>Biwalirudyna</t></is></c><c r="H16" s="2" t="inlineStr" /><c r="I16" s="2" t="inlineStr" /><c r="J16" s="2" t="inlineStr" /><c r="K16" s="2" t="inlineStr"><is><t>Dabigatran</t></is></c><c r="L16" s="2" t="inlineStr"><is><t>Dalteparyna</t></is></c><c r="M16" s="2" t="inlineStr" /><c r="N16" s="2" t="inlineStr" /><c r="O16" s="2" t="inlineStr" /><c r="P16" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q16" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="17"><c r="A17" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B17" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C17" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D17" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E17" s="2" t="inlineStr"><is><t>Odwracalne inhibitory acetylocholinesterazy są stosowane w leczeniu:</t></is></c><c r="F17" s="2" t="inlineStr"><is><t>Nużliwości mięśni</t></is></c><c r="G17" s="2" t="inlineStr"><is><t>Pooperacyjnej niedrożności jelit</t></is></c><c r="H17" s="2" t="inlineStr"><is><t>Choroby Alzheimera</t></is></c><c r="I17" s="2" t="inlineStr" /><c r="J17" s="2" t="inlineStr" /><c r="K17" s="2" t="inlineStr"><is><t>Zatruć związakmi fosfoorganicznymi</t></is></c><c r="L17" s="2" t="inlineStr" /><c r="M17" s="2" t="inlineStr" /><c r="N17" s="2" t="inlineStr" /><c r="O17" s="2" t="inlineStr" /><c r="P17" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q17" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="18"><c r="A18" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B18" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C18" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D18" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E18" s="2" t="inlineStr"><is><t>Zaznacza prawidłowe pary dotyczące leczenia uzależnień i wybranego leku:</t></is></c><c r="F18" s="2" t="inlineStr"><is><t>Uzależnienie od alkoholu – nalmefen</t></is></c><c r="G18" s="2" t="inlineStr"><is><t>Uzależnienie od heroiny – metadon</t></is></c><c r="H18" s="2" t="inlineStr" /><c r="I18" s="2" t="inlineStr" /><c r="J18" s="2" t="inlineStr" /><c r="K18" s="2" t="inlineStr"><is><t>Uzależnienie od nikotyny – klonidyna</t></is></c><c r="L18" s="2" t="inlineStr"><is><t>Uzależnienie od amfetaminy – wereniklina</t></is></c><c r="M18" s="2" t="inlineStr" /><c r="N18" s="2" t="inlineStr" /><c r="O18" s="2" t="inlineStr" /><c r="P18" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q18" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="19"><c r="A19" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B19" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C19" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D19" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E19" s="2" t="inlineStr"><is><t>Wskaż prawidłowe pary płyn infuzyjny – możliwe działania niepożądane:</t></is></c><c r="F19" s="2" t="inlineStr"><is><t>5% roztwór glukozy – hiponatremia</t></is></c><c r="G19" s="2" t="inlineStr"><is><t>HES (hydroksyetylowana skrobia) – ostre uszkodzenie nerek</t></is></c><c r="H19" s="2" t="inlineStr"><is><t>5% roztwór albuminy – anafilaksja</t></is></c><c r="I19" s="2" t="inlineStr"><is><t>Dekstran 70000 – działanie przeciwkrzepliwe</t></is></c><c r="J19" s="2" t="inlineStr" /><c r="K19" s="2" t="inlineStr" /><c r="L19" s="2" t="inlineStr" /><c r="M19" s="2" t="inlineStr" /><c r="N19" s="2" t="inlineStr" /><c r="O19" s="2" t="inlineStr" /><c r="P19" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q19" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="20"><c r="A20" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B20" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C20" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D20" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E20" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące leczenia hipotensyjnego:</t></is></c><c r="F20" s="2" t="inlineStr"><is><t>Tiazydy mogą bezpośrednio oddziaływać na ścianę naczyń i zmniejszać systemowy opór naczyniowy</t></is></c><c r="G20" s="2" t="inlineStr"><is><t>Pełny efekt hipotensyjny występuje po kilkunastu dniach leczenia</t></is></c><c r="H20" s="2" t="inlineStr"><is><t>Blokada kotransportera Na-Cl w kanaliku dystalnym prowadzi do zwiększeniu natriurezy</t></is></c><c r="I20" s="2" t="inlineStr" /><c r="J20" s="2" t="inlineStr" /><c r="K20" s="2" t="inlineStr"><is><t>Ich skuteczność w leczeniu przewlekłym wynika przede wszystkim ze zmniejszenia objętości osocza i rzutu serca</t></is></c><c r="L20" s="2" t="inlineStr" /><c r="M20" s="2" t="inlineStr" /><c r="N20" s="2" t="inlineStr" /><c r="O20" s="2" t="inlineStr" /><c r="P20" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q20" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="21"><c r="A21" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B21" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C21" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D21" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E21" s="2" t="inlineStr"><is><t>Suksametonium może być przyczyną:</t></is></c><c r="F21" s="2" t="inlineStr"><is><t>Drżenia włókienkowego mięśni szkieletowych</t></is></c><c r="G21" s="2" t="inlineStr"><is><t>Zaburzeń oddychania</t></is></c><c r="H21" s="2" t="inlineStr"><is><t>Zespołu hipertermii złośliwej</t></is></c><c r="I21" s="2" t="inlineStr"><is><t>Długotrwałego efektu zwiotczającego u osób z dysfunkcją acetylocholinesterazy</t></is></c><c r="J21" s="2" t="inlineStr" /><c r="K21" s="2" t="inlineStr" /><c r="L21" s="2" t="inlineStr" /><c r="M21" s="2" t="inlineStr" /><c r="N21" s="2" t="inlineStr" /><c r="O21" s="2" t="inlineStr" /><c r="P21" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q21" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="22"><c r="A22" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B22" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C22" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D22" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E22" s="2" t="inlineStr"><is><t>W celu łagodzenia suchego kaszlu można wybrać:</t></is></c><c r="F22" s="2" t="inlineStr"><is><t>Dekstrometorfan</t></is></c><c r="G22" s="2" t="inlineStr"><is><t>Kodeinę</t></is></c><c r="H22" s="2" t="inlineStr"><is><t>Butamirat</t></is></c><c r="I22" s="2" t="inlineStr" /><c r="J22" s="2" t="inlineStr" /><c r="K22" s="2" t="inlineStr"><is><t>Bromheksynę</t></is></c><c r="L22" s="2" t="inlineStr" /><c r="M22" s="2" t="inlineStr" /><c r="N22" s="2" t="inlineStr" /><c r="O22" s="2" t="inlineStr" /><c r="P22" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q22" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="23"><c r="A23" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B23" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C23" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D23" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E23" s="2" t="inlineStr"><is><t>Albendazol stosowany jest w jelitowej infestacji:</t></is></c><c r="F23" s="2" t="inlineStr"><is><t>Glistą ludzką</t></is></c><c r="G23" s="2" t="inlineStr"><is><t>Tasiemcem uzbrojonym</t></is></c><c r="H23" s="2" t="inlineStr"><is><t>Owsikami</t></is></c><c r="I23" s="2" t="inlineStr" /><c r="J23" s="2" t="inlineStr" /><c r="K23" s="2" t="inlineStr"><is><t>Lambliami</t></is></c><c r="L23" s="2" t="inlineStr" /><c r="M23" s="2" t="inlineStr" /><c r="N23" s="2" t="inlineStr" /><c r="O23" s="2" t="inlineStr" /><c r="P23" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q23" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="24"><c r="A24" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B24" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C24" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D24" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E24" s="2" t="inlineStr"><is><t>Napad paniki należy leczyć stosując doraźnie:</t></is></c><c r="F24" s="2" t="inlineStr"><is><t>Techniki relaksacyjne</t></is></c><c r="G24" s="2" t="inlineStr"><is><t>Alprazolam</t></is></c><c r="H24" s="2" t="inlineStr" /><c r="I24" s="2" t="inlineStr" /><c r="J24" s="2" t="inlineStr" /><c r="K24" s="2" t="inlineStr"><is><t>Pregabalinę</t></is></c><c r="L24" s="2" t="inlineStr"><is><t>Fluoksetynę</t></is></c><c r="M24" s="2" t="inlineStr" /><c r="N24" s="2" t="inlineStr" /><c r="O24" s="2" t="inlineStr" /><c r="P24" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q24" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="25"><c r="A25" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B25" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C25" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D25" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E25" s="2" t="inlineStr"><is><t>Fenoterol może być przyczyną:</t></is></c><c r="F25" s="2" t="inlineStr"><is><t>Tachykardii</t></is></c><c r="G25" s="2" t="inlineStr"><is><t>Drżenia mięśni</t></is></c><c r="H25" s="2" t="inlineStr"><is><t>Hiperglikemii</t></is></c><c r="I25" s="2" t="inlineStr"><is><t>Hamowania skurczów ciężarnej macicy</t></is></c><c r="J25" s="2" t="inlineStr" /><c r="K25" s="2" t="inlineStr" /><c r="L25" s="2" t="inlineStr" /><c r="M25" s="2" t="inlineStr" /><c r="N25" s="2" t="inlineStr" /><c r="O25" s="2" t="inlineStr" /><c r="P25" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q25" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="26"><c r="A26" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B26" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C26" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D26" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E26" s="2" t="inlineStr"><is><t>Długo działające beta2-mimetyki (LABA):</t></is></c><c r="F26" s="2" t="inlineStr"><is><t>Podawane przewlekle powodują down-regulację receptorów beta2-adrenergicznych w oskrzelach</t></is></c><c r="G26" s="2" t="inlineStr" /><c r="H26" s="2" t="inlineStr" /><c r="I26" s="2" t="inlineStr" /><c r="J26" s="2" t="inlineStr" /><c r="K26" s="2" t="inlineStr"><is><t>Nie powinny być podawane razem z glikokortykosteroidami które blokują wytwarzanie białek receptorów beta2-adrenergicznych</t></is></c><c r="L26" s="2" t="inlineStr"><is><t>Mogą być przyczyną istotnej klinicznie hieprkaliemi</t></is></c><c r="M26" s="2" t="inlineStr"><is><t>Wykazują działanie przeciwzapalne</t></is></c><c r="N26" s="2" t="inlineStr" /><c r="O26" s="2" t="inlineStr" /><c r="P26" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q26" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="27"><c r="A27" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B27" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C27" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D27" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E27" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące NLPZ:</t></is></c><c r="F27" s="2" t="inlineStr"><is><t>Ketoprofen powoduje większe ryzyko krwawienia z górnego odcinka przewodu pokarmowego niż ibuprofen</t></is></c><c r="G27" s="2" t="inlineStr" /><c r="H27" s="2" t="inlineStr" /><c r="I27" s="2" t="inlineStr" /><c r="J27" s="2" t="inlineStr" /><c r="K27" s="2" t="inlineStr"><is><t>Meloksykam jest preferencyjnym inhibitorem COX-1</t></is></c><c r="L27" s="2" t="inlineStr"><is><t>Zastąpienie drogi doustnej podania diklofenaku drogą doodbytniczą zmniejsza ryzyko wystąpienia działań niepożądanych</t></is></c><c r="M27" s="2" t="inlineStr"><is><t>Nimesulid należy do najmniej hepatotoksycznych NLPZ</t></is></c><c r="N27" s="2" t="inlineStr" /><c r="O27" s="2" t="inlineStr" /><c r="P27" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q27" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="28"><c r="A28" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B28" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C28" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D28" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E28" s="2" t="inlineStr"><is><t>Lekiem prkeursorowym jest:</t></is></c><c r="F28" s="2" t="inlineStr"><is><t>Enalapryl</t></is></c><c r="G28" s="2" t="inlineStr"><is><t>Cyklezonid</t></is></c><c r="H28" s="2" t="inlineStr"><is><t>Lewodopa</t></is></c><c r="I28" s="2" t="inlineStr" /><c r="J28" s="2" t="inlineStr" /><c r="K28" s="2" t="inlineStr"><is><t>Furosemid</t></is></c><c r="L28" s="2" t="inlineStr" /><c r="M28" s="2" t="inlineStr" /><c r="N28" s="2" t="inlineStr" /><c r="O28" s="2" t="inlineStr" /><c r="P28" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q28" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="29"><c r="A29" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B29" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C29" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D29" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E29" s="2" t="inlineStr"><is><t>Cyklosporyna</t></is></c><c r="F29" s="2" t="inlineStr"><is><t>Jest eliminowana przez wątrobę</t></is></c><c r="G29" s="2" t="inlineStr"><is><t>Jest stosowana w celu zapobiegania odrzucania przeszczepów</t></is></c><c r="H29" s="2" t="inlineStr" /><c r="I29" s="2" t="inlineStr" /><c r="J29" s="2" t="inlineStr" /><c r="K29" s="2" t="inlineStr"><is><t>Jest aktywatorem kalcyneuryny</t></is></c><c r="L29" s="2" t="inlineStr"><is><t>Może powodować atrofię dziąseł</t></is></c><c r="M29" s="2" t="inlineStr" /><c r="N29" s="2" t="inlineStr" /><c r="O29" s="2" t="inlineStr" /><c r="P29" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q29" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="30"><c r="A30" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B30" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C30" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D30" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E30" s="2" t="inlineStr"><is><t>Do leków o udowodnionym korzystnym działaniu w profilaktyce wtórnej niedokrwiennego udaru mózgu należy:</t></is></c><c r="F30" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="G30" s="2" t="inlineStr"><is><t>Atorwastatyna</t></is></c><c r="H30" s="2" t="inlineStr"><is><t>Klopidogrel</t></is></c><c r="I30" s="2" t="inlineStr" /><c r="J30" s="2" t="inlineStr" /><c r="K30" s="2" t="inlineStr"><is><t>Kwas traneksamowy</t></is></c><c r="L30" s="2" t="inlineStr" /><c r="M30" s="2" t="inlineStr" /><c r="N30" s="2" t="inlineStr" /><c r="O30" s="2" t="inlineStr" /><c r="P30" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q30" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="31"><c r="A31" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B31" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C31" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D31" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E31" s="2" t="inlineStr"><is><t>Lewodopa:</t></is></c><c r="F31" s="2" t="inlineStr"><is><t>Jest jednym z najskuteczniejszych leków stosowanych w terapii choroby Parkinsona</t></is></c><c r="G31" s="2" t="inlineStr"><is><t>Ma krótki okres półtrwania i dlatego wymaga wielokrotnego podawania w ciągu doby</t></is></c><c r="H31" s="2" t="inlineStr"><is><t>Podczas długotrwałego leczenia może wywołać fluktuacje ruchowe i dyskinezy</t></is></c><c r="I31" s="2" t="inlineStr"><is><t>Może wywoływać działania niepożądane ze strony przewodu pokarmowego</t></is></c><c r="J31" s="2" t="inlineStr" /><c r="K31" s="2" t="inlineStr" /><c r="L31" s="2" t="inlineStr" /><c r="M31" s="2" t="inlineStr" /><c r="N31" s="2" t="inlineStr" /><c r="O31" s="2" t="inlineStr" /><c r="P31" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q31" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="32"><c r="A32" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B32" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C32" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D32" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E32" s="2" t="inlineStr"><is><t>Kokaina:</t></is></c><c r="F32" s="2" t="inlineStr"><is><t>Hamuje wychwyt zwrotny dopaminy w szczelinie synaptycznej</t></is></c><c r="G32" s="2" t="inlineStr"><is><t>Może powodować wystąpienie zawału mięśnia sercowego</t></is></c><c r="H32" s="2" t="inlineStr"><is><t>Może powodować krwawienia wewnątrzczaszkowe</t></is></c><c r="I32" s="2" t="inlineStr" /><c r="J32" s="2" t="inlineStr" /><c r="K32" s="2" t="inlineStr"><is><t>Hamuje aktywność receptora dla kwasu glutaminowego</t></is></c><c r="L32" s="2" t="inlineStr" /><c r="M32" s="2" t="inlineStr" /><c r="N32" s="2" t="inlineStr" /><c r="O32" s="2" t="inlineStr" /><c r="P32" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q32" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="33"><c r="A33" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B33" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C33" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D33" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E33" s="2" t="inlineStr"><is><t>W alergicznym zapaleniu spojówek może stosować dospojówkowo:</t></is></c><c r="F33" s="2" t="inlineStr"><is><t>Antazolinę</t></is></c><c r="G33" s="2" t="inlineStr"><is><t>Azelastynę</t></is></c><c r="H33" s="2" t="inlineStr"><is><t>Kromoglikan sodowy</t></is></c><c r="I33" s="2" t="inlineStr"><is><t>Olopatadynę</t></is></c><c r="J33" s="2" t="inlineStr" /><c r="K33" s="2" t="inlineStr" /><c r="L33" s="2" t="inlineStr" /><c r="M33" s="2" t="inlineStr" /><c r="N33" s="2" t="inlineStr" /><c r="O33" s="2" t="inlineStr" /><c r="P33" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q33" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="34"><c r="A34" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B34" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C34" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D34" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E34" s="2" t="inlineStr"><is><t>Stosowanie preparatu złożonego bupropionu z naltreksonem w leczeniu otyłości:</t></is></c><c r="F34" s="2" t="inlineStr"><is><t>Ma wpływ na ośrodkowy układ nagrody</t></is></c><c r="G34" s="2" t="inlineStr"><is><t>Zwiększa i wydłuża uczucie sytości</t></is></c><c r="H34" s="2" t="inlineStr"><is><t>Ma zwiększoną skuteczność kliniczną ze względu na efekt synergistyczny bupropionu i naltreksonu</t></is></c><c r="I34" s="2" t="inlineStr" /><c r="J34" s="2" t="inlineStr" /><c r="K34" s="2" t="inlineStr"><is><t>Jest wskazane dla wszystkich osób z wyjściową wartością BMI wynoszącą ≥27</t></is></c><c r="L34" s="2" t="inlineStr" /><c r="M34" s="2" t="inlineStr" /><c r="N34" s="2" t="inlineStr" /><c r="O34" s="2" t="inlineStr" /><c r="P34" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q34" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="35"><c r="A35" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B35" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C35" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D35" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E35" s="2" t="inlineStr"><is><t>Dodatek adrenaliny do lidokainy w lekach do znieczulania miejscowego może powodować:</t></is></c><c r="F35" s="2" t="inlineStr"><is><t>Zwiększone ryzyko martwicy tkanek po podaniach obwodowych</t></is></c><c r="G35" s="2" t="inlineStr"><is><t>Wydłużenie czasu działania lidokainy</t></is></c><c r="H35" s="2" t="inlineStr" /><c r="I35" s="2" t="inlineStr" /><c r="J35" s="2" t="inlineStr" /><c r="K35" s="2" t="inlineStr"><is><t>Zwiększone niebezpieczeństwo zatrzymania oddechu</t></is></c><c r="L35" s="2" t="inlineStr"><is><t>Zahamowanie metabolizmu lidokainy</t></is></c><c r="M35" s="2" t="inlineStr" /><c r="N35" s="2" t="inlineStr" /><c r="O35" s="2" t="inlineStr" /><c r="P35" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q35" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="36"><c r="A36" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B36" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C36" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D36" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E36" s="2" t="inlineStr"><is><t>Digoksyna:</t></is></c><c r="F36" s="2" t="inlineStr"><is><t>aktywuje układ przywspółczulny</t></is></c><c r="G36" s="2" t="inlineStr"><is><t>wywiera arytmie i zaburzenia przewodzenia</t></is></c><c r="H36" s="2" t="inlineStr"><is><t>jest stosowana w celu kontroli częstotliwości rytmu komór u chorych z migotaniem przedsionków</t></is></c><c r="I36" s="2" t="inlineStr"><is><t>w zatruciu można zastosować fragmenty Fab przeciwciał wiążących</t></is></c><c r="J36" s="2" t="inlineStr" /><c r="K36" s="2" t="inlineStr" /><c r="L36" s="2" t="inlineStr" /><c r="M36" s="2" t="inlineStr" /><c r="N36" s="2" t="inlineStr" /><c r="O36" s="2" t="inlineStr" /><c r="P36" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q36" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="37"><c r="A37" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B37" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C37" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D37" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E37" s="2" t="inlineStr"><is><t>Teoretyczną przesłanką stosowania beta-adrenolityków w przewlekłej skurczowej niewydolności serca jest:</t></is></c><c r="F37" s="2" t="inlineStr"><is><t>Odwracanie beta-down regulacji</t></is></c><c r="G37" s="2" t="inlineStr"><is><t>Zapobieganie proarytmicznemu działaniu katecholamin</t></is></c><c r="H37" s="2" t="inlineStr" /><c r="I37" s="2" t="inlineStr" /><c r="J37" s="2" t="inlineStr" /><c r="K37" s="2" t="inlineStr"><is><t>Korzystny bezpośredni wpływ hemodynamiczny</t></is></c><c r="L37" s="2" t="inlineStr"><is><t>Zwiększenie naprężenia ściany lewej komory</t></is></c><c r="M37" s="2" t="inlineStr" /><c r="N37" s="2" t="inlineStr" /><c r="O37" s="2" t="inlineStr" /><c r="P37" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q37" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="38"><c r="A38" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B38" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C38" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D38" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E38" s="2" t="inlineStr"><is><t>Rupatadyna:</t></is></c><c r="F38" s="2" t="inlineStr"><is><t>jest selektywnym niesedatywnym antagonistą receptorów H1</t></is></c><c r="G38" s="2" t="inlineStr"><is><t>hamuje degranulację komórek tucznych in vitro</t></is></c><c r="H38" s="2" t="inlineStr"><is><t>ma aktywny metabolit – desloratadynę zaliczaną do 3 generacji leków przeciwhistaminowych</t></is></c><c r="I38" s="2" t="inlineStr"><is><t>w dawkach zalecanych nie wydłuża odstępu QTc</t></is></c><c r="J38" s="2" t="inlineStr" /><c r="K38" s="2" t="inlineStr" /><c r="L38" s="2" t="inlineStr" /><c r="M38" s="2" t="inlineStr" /><c r="N38" s="2" t="inlineStr" /><c r="O38" s="2" t="inlineStr" /><c r="P38" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q38" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="39"><c r="A39" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B39" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C39" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D39" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E39" s="2" t="inlineStr"><is><t>U pacjentów z eGFR&lt;30ml/min należy rezygnować ze stosowania:</t></is></c><c r="F39" s="2" t="inlineStr"><is><t>Metyforminy</t></is></c><c r="G39" s="2" t="inlineStr"><is><t>Hydrochlorotiazydu</t></is></c><c r="H39" s="2" t="inlineStr" /><c r="I39" s="2" t="inlineStr" /><c r="J39" s="2" t="inlineStr" /><c r="K39" s="2" t="inlineStr"><is><t>Metoprololu</t></is></c><c r="L39" s="2" t="inlineStr"><is><t>Amlodypiny</t></is></c><c r="M39" s="2" t="inlineStr" /><c r="N39" s="2" t="inlineStr" /><c r="O39" s="2" t="inlineStr" /><c r="P39" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q39" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="40"><c r="A40" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B40" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C40" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D40" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E40" s="2" t="inlineStr"><is><t>Wenlafaksyna:</t></is></c><c r="F40" s="2" t="inlineStr"><is><t>Może być podawana w uogólnionych zaburzeniach lękowych</t></is></c><c r="G40" s="2" t="inlineStr"><is><t>Stosowana razem z tryptanami może powodować wystąpienie zespołu serotoninowego</t></is></c><c r="H40" s="2" t="inlineStr" /><c r="I40" s="2" t="inlineStr" /><c r="J40" s="2" t="inlineStr" /><c r="K40" s="2" t="inlineStr"><is><t>Ma istotne działanie cholinolityczne</t></is></c><c r="L40" s="2" t="inlineStr"><is><t>Można ją bezpiecznie stosować w terapii skojarzonej z inhibitorami MAO</t></is></c><c r="M40" s="2" t="inlineStr" /><c r="N40" s="2" t="inlineStr" /><c r="O40" s="2" t="inlineStr" /><c r="P40" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q40" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="41"><c r="A41" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B41" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C41" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D41" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E41" s="2" t="inlineStr"><is><t>Czy słuszna jest przedstawiona interpretacja działania leku na podstawie nazwy międzynarodowej:</t></is></c><c r="F41" s="2" t="inlineStr"><is><t>Paliwizumab – humanizowane przeciwciało monoklonalne o działaniu p￾wirusowym</t></is></c><c r="G41" s="2" t="inlineStr"><is><t>Ekulizumab – humanizowane przeciwciało monoklonalne o wpływie na układ odpornościowy</t></is></c><c r="H41" s="2" t="inlineStr" /><c r="I41" s="2" t="inlineStr" /><c r="J41" s="2" t="inlineStr" /><c r="K41" s="2" t="inlineStr"><is><t>Ofatumumab – mysie przeciwciało monoklonalne o wpływie p-nowotworowym</t></is></c><c r="L41" s="2" t="inlineStr"><is><t>Pomalidomid – mysie przeciwciało monoklonalne o wpływie na układ odpornościowy</t></is></c><c r="M41" s="2" t="inlineStr" /><c r="N41" s="2" t="inlineStr" /><c r="O41" s="2" t="inlineStr" /><c r="P41" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q41" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="42"><c r="A42" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B42" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C42" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D42" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E42" s="2" t="inlineStr"><is><t>Do przeciwciał monoklonalnych anty-TNF należy:</t></is></c><c r="F42" s="2" t="inlineStr"><is><t>Adalimumab</t></is></c><c r="G42" s="2" t="inlineStr" /><c r="H42" s="2" t="inlineStr" /><c r="I42" s="2" t="inlineStr" /><c r="J42" s="2" t="inlineStr" /><c r="K42" s="2" t="inlineStr"><is><t>Omalizumab</t></is></c><c r="L42" s="2" t="inlineStr"><is><t>Trastuzumab</t></is></c><c r="M42" s="2" t="inlineStr"><is><t>Rytuksymab</t></is></c><c r="N42" s="2" t="inlineStr" /><c r="O42" s="2" t="inlineStr" /><c r="P42" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q42" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="43"><c r="A43" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B43" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C43" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D43" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E43" s="2" t="inlineStr"><is><t>Werapamil można stosować w:</t></is></c><c r="F43" s="2" t="inlineStr"><is><t>Postaci naczynioskurczowej choroby niedokrwiennej serca</t></is></c><c r="G43" s="2" t="inlineStr"><is><t>Napadowym częstoskurczu z łącza przedsionkowo-komorowego</t></is></c><c r="H43" s="2" t="inlineStr" /><c r="I43" s="2" t="inlineStr" /><c r="J43" s="2" t="inlineStr" /><c r="K43" s="2" t="inlineStr"><is><t>Bradykardii</t></is></c><c r="L43" s="2" t="inlineStr"><is><t>Migotaniu przedsionków u osób z zespołem preekscytacji</t></is></c><c r="M43" s="2" t="inlineStr" /><c r="N43" s="2" t="inlineStr" /><c r="O43" s="2" t="inlineStr" /><c r="P43" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q43" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="44"><c r="A44" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B44" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C44" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D44" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E44" s="2" t="inlineStr"><is><t>Inhibitory neprylizyny:</t></is></c><c r="F44" s="2" t="inlineStr"><is><t>Zmniejszają przebudowę mięśnia sercowego</t></is></c><c r="G44" s="2" t="inlineStr"><is><t>Zwiększają stężenie angiotensyny II</t></is></c><c r="H44" s="2" t="inlineStr"><is><t>Są stosowane w przewlekłej niewydolności serca z upośledzoną frakcją wyrzutową</t></is></c><c r="I44" s="2" t="inlineStr" /><c r="J44" s="2" t="inlineStr" /><c r="K44" s="2" t="inlineStr"><is><t>Rozkładają peptydy natriuretyczne</t></is></c><c r="L44" s="2" t="inlineStr" /><c r="M44" s="2" t="inlineStr" /><c r="N44" s="2" t="inlineStr" /><c r="O44" s="2" t="inlineStr" /><c r="P44" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q44" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="45"><c r="A45" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B45" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C45" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D45" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E45" s="2" t="inlineStr"><is><t>Biodostępność leku A po jednorazowym podaniu doustnym wynosi 50%. Tmax wynosi 30min, Cmax 2µg/dl. Oznacza to, że:</t></is></c><c r="F45" s="2" t="inlineStr"><is><t>Lek A może podlegać nawet w 50% efektowi pierwszego przejścia</t></is></c><c r="G45" s="2" t="inlineStr" /><c r="H45" s="2" t="inlineStr" /><c r="I45" s="2" t="inlineStr" /><c r="J45" s="2" t="inlineStr" /><c r="K45" s="2" t="inlineStr"><is><t>Dawka wynosiła 4µg</t></is></c><c r="L45" s="2" t="inlineStr"><is><t>Lek A słabo się wiąże z białkami krwi</t></is></c><c r="M45" s="2" t="inlineStr"><is><t>Okres półtrwania leku A wynosi również około 30min</t></is></c><c r="N45" s="2" t="inlineStr" /><c r="O45" s="2" t="inlineStr" /><c r="P45" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q45" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="46"><c r="A46" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B46" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C46" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D46" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E46" s="2" t="inlineStr"><is><t>Podanie doodbytnicze leku:</t></is></c><c r="F46" s="2" t="inlineStr"><is><t>Może łatwo doprowadzić do miejscowego uszkodzenia błony śluzowej odbytnicy</t></is></c><c r="G46" s="2" t="inlineStr" /><c r="H46" s="2" t="inlineStr" /><c r="I46" s="2" t="inlineStr" /><c r="J46" s="2" t="inlineStr" /><c r="K46" s="2" t="inlineStr"><is><t>Zwiększa efekt pierwszego przejścia</t></is></c><c r="L46" s="2" t="inlineStr"><is><t>Jest metodą z wyboru u dzieci</t></is></c><c r="M46" s="2" t="inlineStr"><is><t>Wymaga podania większej dawki leku w porównaniu do podania doustnego</t></is></c><c r="N46" s="2" t="inlineStr" /><c r="O46" s="2" t="inlineStr" /><c r="P46" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q46" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="47"><c r="A47" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B47" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C47" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D47" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E47" s="2" t="inlineStr"><is><t>Zaburzenia erekcji mogą być spowodowane stosowaniem:</t></is></c><c r="F47" s="2" t="inlineStr"><is><t>Inhibitorów 5-alfa reduktazy</t></is></c><c r="G47" s="2" t="inlineStr"><is><t>Tiazydów moczopędnych</t></is></c><c r="H47" s="2" t="inlineStr"><is><t>Beta-adrenolityków niekardioselektywnych</t></is></c><c r="I47" s="2" t="inlineStr"><is><t>Inhibitorów wychwytu zwrotnego serotoniny</t></is></c><c r="J47" s="2" t="inlineStr" /><c r="K47" s="2" t="inlineStr" /><c r="L47" s="2" t="inlineStr" /><c r="M47" s="2" t="inlineStr" /><c r="N47" s="2" t="inlineStr" /><c r="O47" s="2" t="inlineStr" /><c r="P47" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q47" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="48"><c r="A48" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B48" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C48" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D48" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E48" s="2" t="inlineStr"><is><t>Doneuronalny wychwyt monoamin jest hamowany przez:</t></is></c><c r="F48" s="2" t="inlineStr"><is><t>Citalopram</t></is></c><c r="G48" s="2" t="inlineStr"><is><t>Reboksetynę</t></is></c><c r="H48" s="2" t="inlineStr" /><c r="I48" s="2" t="inlineStr" /><c r="J48" s="2" t="inlineStr" /><c r="K48" s="2" t="inlineStr"><is><t>Tianeptynę</t></is></c><c r="L48" s="2" t="inlineStr"><is><t>Mirtazapinę</t></is></c><c r="M48" s="2" t="inlineStr" /><c r="N48" s="2" t="inlineStr" /><c r="O48" s="2" t="inlineStr" /><c r="P48" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q48" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="49"><c r="A49" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B49" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C49" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D49" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E49" s="2" t="inlineStr"><is><t>W leczeniu gruźlicy płucnej lekowrażliwej:</t></is></c><c r="F49" s="2" t="inlineStr"><is><t>Leczenie wyjaławiające powinno trwać co najmniej 4 miesiące</t></is></c><c r="G49" s="2" t="inlineStr"><is><t>U kobiet ciężarnych podaje się leki według zwykłego schematu z wyłączeniem streptomycyny</t></is></c><c r="H49" s="2" t="inlineStr" /><c r="I49" s="2" t="inlineStr" /><c r="J49" s="2" t="inlineStr" /><c r="K49" s="2" t="inlineStr"><is><t>W intensywnej fazie leczenia przez 2 miesiące podaje się 2 leki – rifampicynę i izoniazyd</t></is></c><c r="L49" s="2" t="inlineStr"><is><t>W fazie kontynuacji każdy pacjent powinien otrzymać etambutol</t></is></c><c r="M49" s="2" t="inlineStr" /><c r="N49" s="2" t="inlineStr" /><c r="O49" s="2" t="inlineStr" /><c r="P49" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q49" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="50"><c r="A50" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B50" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C50" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D50" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E50" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-wskazanie:</t></is></c><c r="F50" s="2" t="inlineStr"><is><t>Sulpiryd – schizofrenia</t></is></c><c r="G50" s="2" t="inlineStr"><is><t>Metylofenidat – ADHD</t></is></c><c r="H50" s="2" t="inlineStr" /><c r="I50" s="2" t="inlineStr" /><c r="J50" s="2" t="inlineStr" /><c r="K50" s="2" t="inlineStr"><is><t>Moklobemid – bezsenność</t></is></c><c r="L50" s="2" t="inlineStr"><is><t>Sertindol – depresja</t></is></c><c r="M50" s="2" t="inlineStr" /><c r="N50" s="2" t="inlineStr" /><c r="O50" s="2" t="inlineStr" /><c r="P50" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q50" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="51"><c r="A51" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B51" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C51" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D51" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E51" s="2" t="inlineStr"><is><t>Hiperprolaktynemia może wiązać się z leczeniem:</t></is></c><c r="F51" s="2" t="inlineStr"><is><t>Promazyną</t></is></c><c r="G51" s="2" t="inlineStr"><is><t>Rysperydonem</t></is></c><c r="H51" s="2" t="inlineStr"><is><t>Metoklopramidem</t></is></c><c r="I51" s="2" t="inlineStr" /><c r="J51" s="2" t="inlineStr" /><c r="K51" s="2" t="inlineStr"><is><t>Bromokryptyną</t></is></c><c r="L51" s="2" t="inlineStr" /><c r="M51" s="2" t="inlineStr" /><c r="N51" s="2" t="inlineStr" /><c r="O51" s="2" t="inlineStr" /><c r="P51" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q51" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="52"><c r="A52" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B52" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C52" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D52" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E52" s="2" t="inlineStr"><is><t>Ośrodkowy zespół cholinolityczny może wystąpić w wyniku ostrego przedawkowania:</t></is></c><c r="F52" s="2" t="inlineStr"><is><t>Doksepiny</t></is></c><c r="G52" s="2" t="inlineStr"><is><t>Olanzapiny</t></is></c><c r="H52" s="2" t="inlineStr"><is><t>Perfenazyny</t></is></c><c r="I52" s="2" t="inlineStr"><is><t>Klemastyny</t></is></c><c r="J52" s="2" t="inlineStr" /><c r="K52" s="2" t="inlineStr" /><c r="L52" s="2" t="inlineStr" /><c r="M52" s="2" t="inlineStr" /><c r="N52" s="2" t="inlineStr" /><c r="O52" s="2" t="inlineStr" /><c r="P52" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q52" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="53"><c r="A53" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B53" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C53" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D53" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E53" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące metamizolu:</t></is></c><c r="F53" s="2" t="inlineStr"><is><t>Podczas szybkiego wstrzykiwania dożylnego leku może dojść do gwałtownych spadków ciśnienia krwi</t></is></c><c r="G53" s="2" t="inlineStr"><is><t>Może powodować ciężkie uszkodzenia szpiku w mechanizmie nadwrażliwości</t></is></c><c r="H53" s="2" t="inlineStr"><is><t>Zwiększa częstość występowania guzów Wilmsa (nephroblastoma, nerczak zarodkowy)</t></is></c><c r="I53" s="2" t="inlineStr" /><c r="J53" s="2" t="inlineStr" /><c r="K53" s="2" t="inlineStr"><is><t>Ma silne działanie przeciwzapalne</t></is></c><c r="L53" s="2" t="inlineStr" /><c r="M53" s="2" t="inlineStr" /><c r="N53" s="2" t="inlineStr" /><c r="O53" s="2" t="inlineStr" /><c r="P53" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q53" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="54"><c r="A54" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B54" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C54" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D54" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E54" s="2" t="inlineStr"><is><t>Które połączenie lekowe jest bezwzględnie konieczne w wymienionej sytuacji klinicznej:</t></is></c><c r="F54" s="2" t="inlineStr"><is><t>Sartan + sakubitryl w skurczowej niewydolności serca</t></is></c><c r="G54" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy + antagonista receptorów P2Y12 po angioplastyce wieńcowej z implantacją stentu</t></is></c><c r="H54" s="2" t="inlineStr" /><c r="I54" s="2" t="inlineStr" /><c r="J54" s="2" t="inlineStr" /><c r="K54" s="2" t="inlineStr"><is><t>Heparyna drobnocząsteczkowa + ksaban w początkowym okresie leczenia żylnej choroby zakrzepowo zatorowej</t></is></c><c r="L54" s="2" t="inlineStr"><is><t>Adrenalina + atropina w resuscytacji krążeniowo-oddechowej w przebiegu NZK z asystolią</t></is></c><c r="M54" s="2" t="inlineStr" /><c r="N54" s="2" t="inlineStr" /><c r="O54" s="2" t="inlineStr" /><c r="P54" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q54" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="55"><c r="A55" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B55" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C55" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D55" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E55" s="2" t="inlineStr"><is><t>Efekt prokinetyczny można uzyskać:</t></is></c><c r="F55" s="2" t="inlineStr"><is><t>Pobudzając receptory 5-HT4</t></is></c><c r="G55" s="2" t="inlineStr"><is><t>Blokując receptory dopaminowe D2</t></is></c><c r="H55" s="2" t="inlineStr"><is><t>Hamując aktywność acetylocholinoesterazy</t></is></c><c r="I55" s="2" t="inlineStr"><is><t>Pobudzając receptory motylinowe</t></is></c><c r="J55" s="2" t="inlineStr" /><c r="K55" s="2" t="inlineStr" /><c r="L55" s="2" t="inlineStr" /><c r="M55" s="2" t="inlineStr" /><c r="N55" s="2" t="inlineStr" /><c r="O55" s="2" t="inlineStr" /><c r="P55" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q55" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="56"><c r="A56" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B56" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C56" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D56" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E56" s="2" t="inlineStr"><is><t>Glukagon:</t></is></c><c r="F56" s="2" t="inlineStr"><is><t>Stosowany jest w leczeniu ciężkiej hipoglikemii gdy nie można podać dożylnie glukozy</t></is></c><c r="G56" s="2" t="inlineStr"><is><t>Jest podawany parenteralnie</t></is></c><c r="H56" s="2" t="inlineStr"><is><t>Ma zastosowanie w zatruciach lekami beta-adrenolitycznymi</t></is></c><c r="I56" s="2" t="inlineStr"><is><t>Jest nieskuteczny w przypadku glikemii</t></is></c><c r="J56" s="2" t="inlineStr" /><c r="K56" s="2" t="inlineStr" /><c r="L56" s="2" t="inlineStr" /><c r="M56" s="2" t="inlineStr" /><c r="N56" s="2" t="inlineStr" /><c r="O56" s="2" t="inlineStr" /><c r="P56" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q56" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="57"><c r="A57" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B57" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C57" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D57" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E57" s="2" t="inlineStr"><is><t>Ryzyko encefalopatii w przebiegu marskości wątroby zmniejsza stosowanie:</t></is></c><c r="F57" s="2" t="inlineStr"><is><t>Ryfaksyminy</t></is></c><c r="G57" s="2" t="inlineStr"><is><t>Asparaginianu ornityny</t></is></c><c r="H57" s="2" t="inlineStr"><is><t>Laktulozy</t></is></c><c r="I57" s="2" t="inlineStr" /><c r="J57" s="2" t="inlineStr" /><c r="K57" s="2" t="inlineStr"><is><t>Benzodiazepin</t></is></c><c r="L57" s="2" t="inlineStr" /><c r="M57" s="2" t="inlineStr" /><c r="N57" s="2" t="inlineStr" /><c r="O57" s="2" t="inlineStr" /><c r="P57" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q57" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="58"><c r="A58" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B58" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C58" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D58" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E58" s="2" t="inlineStr"><is><t>W celu przerwania ataku duszności uzasadnione jest podanie wziewne:</t></is></c><c r="F58" s="2" t="inlineStr"><is><t>Bromku ipratriopium</t></is></c><c r="G58" s="2" t="inlineStr"><is><t>Salbutamolu</t></is></c><c r="H58" s="2" t="inlineStr" /><c r="I58" s="2" t="inlineStr" /><c r="J58" s="2" t="inlineStr" /><c r="K58" s="2" t="inlineStr"><is><t>Roflumilastu</t></is></c><c r="L58" s="2" t="inlineStr"><is><t>flutykazonu</t></is></c><c r="M58" s="2" t="inlineStr" /><c r="N58" s="2" t="inlineStr" /><c r="O58" s="2" t="inlineStr" /><c r="P58" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q58" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="59"><c r="A59" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B59" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C59" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D59" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E59" s="2" t="inlineStr"><is><t>W leczeniu małopłytkowości stosuje się:</t></is></c><c r="F59" s="2" t="inlineStr"><is><t>Preparaty immunoglobulin poliwalentnych</t></is></c><c r="G59" s="2" t="inlineStr"><is><t>Eltrombopag</t></is></c><c r="H59" s="2" t="inlineStr"><is><t>Romiplostym</t></is></c><c r="I59" s="2" t="inlineStr"><is><t>Prednizon</t></is></c><c r="J59" s="2" t="inlineStr" /><c r="K59" s="2" t="inlineStr" /><c r="L59" s="2" t="inlineStr" /><c r="M59" s="2" t="inlineStr" /><c r="N59" s="2" t="inlineStr" /><c r="O59" s="2" t="inlineStr" /><c r="P59" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q59" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="60"><c r="A60" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B60" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C60" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D60" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E60" s="2" t="inlineStr"><is><t>Ewerolimus jest stosowany w:</t></is></c><c r="F60" s="2" t="inlineStr"><is><t>Kardiologii (stenty wieńcowe)</t></is></c><c r="G60" s="2" t="inlineStr"><is><t>Onkologii (wybrane zaawansowane nowotwory piersi i nerki)</t></is></c><c r="H60" s="2" t="inlineStr" /><c r="I60" s="2" t="inlineStr" /><c r="J60" s="2" t="inlineStr" /><c r="K60" s="2" t="inlineStr"><is><t>Neurologii (stwardnienie rozsiane)</t></is></c><c r="L60" s="2" t="inlineStr"><is><t>Dermatologii (łuszczyca)</t></is></c><c r="M60" s="2" t="inlineStr" /><c r="N60" s="2" t="inlineStr" /><c r="O60" s="2" t="inlineStr" /><c r="P60" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q60" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="61"><c r="A61" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B61" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C61" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D61" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E61" s="2" t="inlineStr"><is><t>Wskaż prawdziwe zdanie:</t></is></c><c r="F61" s="2" t="inlineStr"><is><t>W chromaniu przestankowym znaczenie kliniczne ma leczenie przeciwpłytkowe i hipolipemizujące</t></is></c><c r="G61" s="2" t="inlineStr"><is><t>Zaleca się podawanie inhibitora P2Y12 przed przezskórną interwencją wieńcową u osoby z ostrym zespołem wieńcowym, a następnie kontynuację tego leczenia przez co najmniej 12 miesięcy</t></is></c><c r="H61" s="2" t="inlineStr"><is><t>Po rozpoczęciu leczenia inhibitorami konwertazy angiotensyny należy się spodziewać niewielkiego wzrostu stężenia kreatyniny we krwi</t></is></c><c r="I61" s="2" t="inlineStr" /><c r="J61" s="2" t="inlineStr" /><c r="K61" s="2" t="inlineStr"><is><t>Niedihydropirydynowi antagoniści wapnia są wskazani w leczeniu pacjentów z niewydolnością serca z obniżoną frakcją wyrzutową</t></is></c><c r="L61" s="2" t="inlineStr" /><c r="M61" s="2" t="inlineStr" /><c r="N61" s="2" t="inlineStr" /><c r="O61" s="2" t="inlineStr" /><c r="P61" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q61" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="62"><c r="A62" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B62" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C62" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D62" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E62" s="2" t="inlineStr"><is><t>U osób z pierwotnym wydłużenie QTc bezpieczne jest zastosowanie:</t></is></c><c r="F62" s="2" t="inlineStr"><is><t>Propranololu</t></is></c><c r="G62" s="2" t="inlineStr" /><c r="H62" s="2" t="inlineStr" /><c r="I62" s="2" t="inlineStr" /><c r="J62" s="2" t="inlineStr" /><c r="K62" s="2" t="inlineStr"><is><t>Digoksyny</t></is></c><c r="L62" s="2" t="inlineStr"><is><t>Sotalolu</t></is></c><c r="M62" s="2" t="inlineStr"><is><t>Amiodaronu</t></is></c><c r="N62" s="2" t="inlineStr" /><c r="O62" s="2" t="inlineStr" /><c r="P62" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q62" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="63"><c r="A63" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B63" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C63" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D63" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E63" s="2" t="inlineStr"><is><t>Beta-adrenolityki można zastosować w:</t></is></c><c r="F63" s="2" t="inlineStr"><is><t>Tachykardii zatokowej</t></is></c><c r="G63" s="2" t="inlineStr"><is><t>Niewydolności mięśnia serca z upośledzoną frakcją wyrzutową</t></is></c><c r="H63" s="2" t="inlineStr"><is><t>W kontroli rytmu komór w migotaniu przedsionków</t></is></c><c r="I63" s="2" t="inlineStr" /><c r="J63" s="2" t="inlineStr" /><c r="K63" s="2" t="inlineStr"><is><t>Naczynioskurczowym wariancie choroby niedokrwiennej serca</t></is></c><c r="L63" s="2" t="inlineStr" /><c r="M63" s="2" t="inlineStr" /><c r="N63" s="2" t="inlineStr" /><c r="O63" s="2" t="inlineStr" /><c r="P63" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q63" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="64"><c r="A64" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B64" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C64" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D64" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E64" s="2" t="inlineStr"><is><t>Lidokaina:</t></is></c><c r="F64" s="2" t="inlineStr"><is><t>Jest skuteczna w znieczulaniu nasiękowym</t></is></c><c r="G64" s="2" t="inlineStr"><is><t>Jest metabolizowana w wątrobie</t></is></c><c r="H64" s="2" t="inlineStr"><is><t>Może powodować drgawki</t></is></c><c r="I64" s="2" t="inlineStr" /><c r="J64" s="2" t="inlineStr" /><c r="K64" s="2" t="inlineStr"><is><t>Silnie blokuje kanały potasowe</t></is></c><c r="L64" s="2" t="inlineStr" /><c r="M64" s="2" t="inlineStr" /><c r="N64" s="2" t="inlineStr" /><c r="O64" s="2" t="inlineStr" /><c r="P64" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q64" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="65"><c r="A65" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B65" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C65" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D65" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E65" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-działanie niepożądane:</t></is></c><c r="F65" s="2" t="inlineStr"><is><t>Ramipryl-obrzęk naczynioruchowy</t></is></c><c r="G65" s="2" t="inlineStr"><is><t>Metoprolol-zasłabnięcie lub omdlenie</t></is></c><c r="H65" s="2" t="inlineStr" /><c r="I65" s="2" t="inlineStr" /><c r="J65" s="2" t="inlineStr" /><c r="K65" s="2" t="inlineStr"><is><t>Losartan-zwiększenie stężenia kwasu moczowego</t></is></c><c r="L65" s="2" t="inlineStr"><is><t>Simwastatyna-poprawa tolerancji glukozy</t></is></c><c r="M65" s="2" t="inlineStr" /><c r="N65" s="2" t="inlineStr" /><c r="O65" s="2" t="inlineStr" /><c r="P65" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q65" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="66"><c r="A66" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B66" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C66" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D66" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E66" s="2" t="inlineStr"><is><t>Która ordynacja jest błędna i wymaga korekty?</t></is></c><c r="F66" s="2" t="inlineStr"><is><t>Furosemid p.o. 1xd w obrzękach pochodzenia sercowego</t></is></c><c r="G66" s="2" t="inlineStr"><is><t>Hydrochlorotiazyd p.o. 1xd w obrzękach kończyn dolnych w przebiegu zespołu pozakrzepowego podudzi</t></is></c><c r="H66" s="2" t="inlineStr" /><c r="I66" s="2" t="inlineStr" /><c r="J66" s="2" t="inlineStr" /><c r="K66" s="2" t="inlineStr"><is><t>Torasemid p.o. 1xd w obrzękach pochodzenia nerkowego</t></is></c><c r="L66" s="2" t="inlineStr"><is><t>Spironolakton p.o. 1xd w wodobrzuszu w przebiegu niewydolności wątroby</t></is></c><c r="M66" s="2" t="inlineStr" /><c r="N66" s="2" t="inlineStr" /><c r="O66" s="2" t="inlineStr" /><c r="P66" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q66" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="67"><c r="A67" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B67" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C67" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D67" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E67" s="2" t="inlineStr"><is><t>Koangiokardianem, czyli lekiem działającym bezpośrednio na serce i naczynia jest:</t></is></c><c r="F67" s="2" t="inlineStr"><is><t>Lewosymendan</t></is></c><c r="G67" s="2" t="inlineStr" /><c r="H67" s="2" t="inlineStr" /><c r="I67" s="2" t="inlineStr" /><c r="J67" s="2" t="inlineStr" /><c r="K67" s="2" t="inlineStr"><is><t>Midodryna</t></is></c><c r="L67" s="2" t="inlineStr"><is><t>Epoprostenol</t></is></c><c r="M67" s="2" t="inlineStr"><is><t>Riocyguat</t></is></c><c r="N67" s="2" t="inlineStr" /><c r="O67" s="2" t="inlineStr" /><c r="P67" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q67" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="68"><c r="A68" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B68" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C68" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D68" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E68" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące bisfosfonianów:</t></is></c><c r="F68" s="2" t="inlineStr"><is><t>Są lekami pierwszego rzutu w profilaktyce i leczeniu osteoporozy pomenopauzalnej u kobiet</t></is></c><c r="G68" s="2" t="inlineStr"><is><t>Mogą być stosowane w zapobieganiu i leczeniu osteoporozy posteroidowej</t></is></c><c r="H68" s="2" t="inlineStr"><is><t>U osób z przerzutami nowotworowymi do układu kostnego łagodzą bóle kostne</t></is></c><c r="I68" s="2" t="inlineStr"><is><t>Przeciwwskazaniem do ich podawania jest ciężka niewydolność nerek (GFR&lt;30)</t></is></c><c r="J68" s="2" t="inlineStr" /><c r="K68" s="2" t="inlineStr" /><c r="L68" s="2" t="inlineStr" /><c r="M68" s="2" t="inlineStr" /><c r="N68" s="2" t="inlineStr" /><c r="O68" s="2" t="inlineStr" /><c r="P68" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q68" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="69"><c r="A69" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B69" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C69" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D69" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E69" s="2" t="inlineStr"><is><t>Zmniejszenie hipertriglicerydemii można osiągnąć stosując:</t></is></c><c r="F69" s="2" t="inlineStr"><is><t>Atorwastatynę</t></is></c><c r="G69" s="2" t="inlineStr"><is><t>Fenofibrat</t></is></c><c r="H69" s="2" t="inlineStr"><is><t>PUFA-wielonienasycone kwasy tłuszczowe</t></is></c><c r="I69" s="2" t="inlineStr" /><c r="J69" s="2" t="inlineStr" /><c r="K69" s="2" t="inlineStr"><is><t>Koleswelam</t></is></c><c r="L69" s="2" t="inlineStr" /><c r="M69" s="2" t="inlineStr" /><c r="N69" s="2" t="inlineStr" /><c r="O69" s="2" t="inlineStr" /><c r="P69" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q69" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="70"><c r="A70" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B70" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C70" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D70" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E70" s="2" t="inlineStr"><is><t>Lekiem wydłużającym dystans chromania przestankowego jest:</t></is></c><c r="F70" s="2" t="inlineStr"><is><t>Natydrofuryl</t></is></c><c r="G70" s="2" t="inlineStr"><is><t>Cilostazol</t></is></c><c r="H70" s="2" t="inlineStr" /><c r="I70" s="2" t="inlineStr" /><c r="J70" s="2" t="inlineStr" /><c r="K70" s="2" t="inlineStr"><is><t>Pentoksyfilina</t></is></c><c r="L70" s="2" t="inlineStr"><is><t>Diosmina mikronizowana</t></is></c><c r="M70" s="2" t="inlineStr" /><c r="N70" s="2" t="inlineStr" /><c r="O70" s="2" t="inlineStr" /><c r="P70" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q70" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="71"><c r="A71" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B71" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C71" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D71" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E71" s="2" t="inlineStr"><is><t>W prawidłowo przeprowadzonym leczeniu statynami należy:</t></is></c><c r="F71" s="2" t="inlineStr"><is><t>Oznaczyć aktywność ALAT i CK w surowicy przed rozpoczęciem leczenia</t></is></c><c r="G71" s="2" t="inlineStr"><is><t>Odstawić statynę jeśli aktywność ALAT przekroczy w surowicy 3-krotnie górną granicę wartości prawidłowych</t></is></c><c r="H71" s="2" t="inlineStr" /><c r="I71" s="2" t="inlineStr" /><c r="J71" s="2" t="inlineStr" /><c r="K71" s="2" t="inlineStr"><is><t>Ocenić skuteczność leczenia hipolipemizującego po 2 tygodniach od jego rozpoczęcia</t></is></c><c r="L71" s="2" t="inlineStr"><is><t>Mintorować aktywność CK u każdego pacjenta</t></is></c><c r="M71" s="2" t="inlineStr" /><c r="N71" s="2" t="inlineStr" /><c r="O71" s="2" t="inlineStr" /><c r="P71" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q71" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="72"><c r="A72" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B72" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C72" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D72" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E72" s="2" t="inlineStr"><is><t>Na kanały sodowe ma wpływ:</t></is></c><c r="F72" s="2" t="inlineStr"><is><t>propafenon</t></is></c><c r="G72" s="2" t="inlineStr"><is><t>ranolazyna</t></is></c><c r="H72" s="2" t="inlineStr"><is><t>bupiwakaina</t></is></c><c r="I72" s="2" t="inlineStr" /><c r="J72" s="2" t="inlineStr" /><c r="K72" s="2" t="inlineStr"><is><t>adenozyna</t></is></c><c r="L72" s="2" t="inlineStr" /><c r="M72" s="2" t="inlineStr" /><c r="N72" s="2" t="inlineStr" /><c r="O72" s="2" t="inlineStr" /><c r="P72" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q72" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="73"><c r="A73" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B73" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C73" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D73" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E73" s="2" t="inlineStr"><is><t>Interakcją farmakokinetyczną jest:</t></is></c><c r="F73" s="2" t="inlineStr"><is><t>Hamowanie wchłaniania z przewodu pokarmowego leków podawanych jednocześnie</t></is></c><c r="G73" s="2" t="inlineStr"><is><t>Zwiększanie metabolizmu leków podawanych jednocześnie</t></is></c><c r="H73" s="2" t="inlineStr" /><c r="I73" s="2" t="inlineStr" /><c r="J73" s="2" t="inlineStr" /><c r="K73" s="2" t="inlineStr"><is><t>Wytrącanie się osadu po zmieszaniu dwóch leków w jednym roztworze do wstrzyknięcia</t></is></c><c r="L73" s="2" t="inlineStr"><is><t>Nasilenie sedacji po skojarzeniu opioidów z etanolem</t></is></c><c r="M73" s="2" t="inlineStr" /><c r="N73" s="2" t="inlineStr" /><c r="O73" s="2" t="inlineStr" /><c r="P73" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q73" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="74"><c r="A74" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B74" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C74" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D74" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E74" s="2" t="inlineStr"><is><t>Właściwości farmakodynamiczne i parametry farmakokinetyczne leków mają wpływ na podejmowanie decyzji klinicznych. Czy słuszne jest wobec tego:</t></is></c><c r="F74" s="2" t="inlineStr"><is><t>Wielokrotne powtórzenie dawki naloksonu(t1/2=63min+/-12min) po przedawkowaniu metadonu</t></is></c><c r="G74" s="2" t="inlineStr" /><c r="H74" s="2" t="inlineStr" /><c r="I74" s="2" t="inlineStr" /><c r="J74" s="2" t="inlineStr" /><c r="K74" s="2" t="inlineStr"><is><t>Przetoczenie koncentratu płytek krwi 13h po podaniu tikagrelolu (tikagrelol ze swoim czynnym metabolitem mają łączny czas półtrwania eliminacji 12h)</t></is></c><c r="L74" s="2" t="inlineStr"><is><t>Odstawienie suplementacji potasu w hiperaldosteronizmie pierwotnym po 16-17h po włączeniu spironolaktonu (Cmax karnenonu=16,5h po podaniu spironolaktonu)</t></is></c><c r="M74" s="2" t="inlineStr"><is><t>Przeprowadzenie operacji neurochirurgicznej po 36h po odstawieniu klopidogrelu(t1/2=6h, jego aktywne mają pomijalnie krótki t1/2)</t></is></c><c r="N74" s="2" t="inlineStr" /><c r="O74" s="2" t="inlineStr" /><c r="P74" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q74" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="75"><c r="A75" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B75" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C75" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D75" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E75" s="2" t="inlineStr"><is><t>Kolistyna</t></is></c><c r="F75" s="2" t="inlineStr"><is><t>Działa nefrotoksycznie</t></is></c><c r="G75" s="2" t="inlineStr" /><c r="H75" s="2" t="inlineStr" /><c r="I75" s="2" t="inlineStr" /><c r="J75" s="2" t="inlineStr" /><c r="K75" s="2" t="inlineStr"><is><t>Działa głównie na bakterie Gram+</t></is></c><c r="L75" s="2" t="inlineStr"><is><t>Dobrze wchłania się po podaniu PO</t></is></c><c r="M75" s="2" t="inlineStr"><is><t>Jest wydalana głównie z kałem</t></is></c><c r="N75" s="2" t="inlineStr" /><c r="O75" s="2" t="inlineStr" /><c r="P75" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q75" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="76"><c r="A76" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B76" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C76" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D76" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E76" s="2" t="inlineStr"><is><t>Doksycyklina</t></is></c><c r="F76" s="2" t="inlineStr"><is><t>Działa na bakterie atypowe</t></is></c><c r="G76" s="2" t="inlineStr" /><c r="H76" s="2" t="inlineStr" /><c r="I76" s="2" t="inlineStr" /><c r="J76" s="2" t="inlineStr" /><c r="K76" s="2" t="inlineStr"><is><t>Może być bezpiecznie stosowana u dzieci powyżej 2r.ż</t></is></c><c r="L76" s="2" t="inlineStr"><is><t>Jest anatgonistą receptorów GABA-A wywołujących efekt sedatywny</t></is></c><c r="M76" s="2" t="inlineStr"><is><t>Jest bezpieczna w terapii kobiet w ciąży</t></is></c><c r="N76" s="2" t="inlineStr" /><c r="O76" s="2" t="inlineStr" /><c r="P76" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q76" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="77"><c r="A77" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B77" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C77" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D77" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E77" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – mechanizm działania:</t></is></c><c r="F77" s="2" t="inlineStr"><is><t>linezolid- hamowanie biosyntezy białka w komórkach bakterii poprzez wiązanie się z podjednostką 50 S rybosomu</t></is></c><c r="G77" s="2" t="inlineStr" /><c r="H77" s="2" t="inlineStr" /><c r="I77" s="2" t="inlineStr" /><c r="J77" s="2" t="inlineStr" /><c r="K77" s="2" t="inlineStr"><is><t>cefuroksym – hamowanie topoizomerazy II</t></is></c><c r="L77" s="2" t="inlineStr"><is><t>moksyfloksacyna - blokowanie syntezy ściany komórkowej bakterii</t></is></c><c r="M77" s="2" t="inlineStr"><is><t>wankomycyna - uszkodzenie DNA</t></is></c><c r="N77" s="2" t="inlineStr" /><c r="O77" s="2" t="inlineStr" /><c r="P77" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q77" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="78"><c r="A78" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B78" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C78" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D78" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E78" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – działania niepożądane:</t></is></c><c r="F78" s="2" t="inlineStr"><is><t>lewofloksacyna - drgawki</t></is></c><c r="G78" s="2" t="inlineStr"><is><t>ceftriakson – zagęszczenie żółci</t></is></c><c r="H78" s="2" t="inlineStr"><is><t>wankomycyna – zespół czerwonego karku</t></is></c><c r="I78" s="2" t="inlineStr"><is><t>linezolid – trombocytopenia</t></is></c><c r="J78" s="2" t="inlineStr" /><c r="K78" s="2" t="inlineStr" /><c r="L78" s="2" t="inlineStr" /><c r="M78" s="2" t="inlineStr" /><c r="N78" s="2" t="inlineStr" /><c r="O78" s="2" t="inlineStr" /><c r="P78" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q78" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="79"><c r="A79" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B79" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C79" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D79" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E79" s="2" t="inlineStr"><is><t>Właściwy wybór leku przeciwwirusowego w zakażeniu to:</t></is></c><c r="F79" s="2" t="inlineStr"><is><t>Wirus HBV-lamiwudyna</t></is></c><c r="G79" s="2" t="inlineStr"><is><t>Cytomegalowirus-walgancyklowir</t></is></c><c r="H79" s="2" t="inlineStr" /><c r="I79" s="2" t="inlineStr" /><c r="J79" s="2" t="inlineStr" /><c r="K79" s="2" t="inlineStr"><is><t>Norowirus-sakwinawir</t></is></c><c r="L79" s="2" t="inlineStr"><is><t>Wirus opryszczki-rybawiryna</t></is></c><c r="M79" s="2" t="inlineStr" /><c r="N79" s="2" t="inlineStr" /><c r="O79" s="2" t="inlineStr" /><c r="P79" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q79" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="80"><c r="A80" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B80" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C80" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D80" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E80" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – wrażliwy drobnoustrój:</t></is></c><c r="F80" s="2" t="inlineStr"><is><t>kaspofungina _ Candida spp</t></is></c><c r="G80" s="2" t="inlineStr"><is><t>amfoterycyna B – Cryptococcus neoformans</t></is></c><c r="H80" s="2" t="inlineStr"><is><t>worykonazol - Candida crusei</t></is></c><c r="I80" s="2" t="inlineStr" /><c r="J80" s="2" t="inlineStr" /><c r="K80" s="2" t="inlineStr"><is><t>flukonazol – Aspergillus fumigatus</t></is></c><c r="L80" s="2" t="inlineStr" /><c r="M80" s="2" t="inlineStr" /><c r="N80" s="2" t="inlineStr" /><c r="O80" s="2" t="inlineStr" /><c r="P80" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q80" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="81"><c r="A81" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B81" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C81" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D81" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E81" s="2" t="inlineStr"><is><t>Flukonazol:</t></is></c><c r="F81" s="2" t="inlineStr"><is><t>W leczeniu kandydozy jamy ustnej nie jest skuteczny po podaniu dawki jednorazowej</t></is></c><c r="G81" s="2" t="inlineStr" /><c r="H81" s="2" t="inlineStr" /><c r="I81" s="2" t="inlineStr" /><c r="J81" s="2" t="inlineStr" /><c r="K81" s="2" t="inlineStr"><is><t>Ma małą biodostępność po podaniu doustnym</t></is></c><c r="L81" s="2" t="inlineStr"><is><t>Powinien być podawany profilaktycznie pacjentom leczonym szerokospektralnymi lekami przeciwbakteryjnymi z powodu zakażenia układu oddechowego</t></is></c><c r="M81" s="2" t="inlineStr"><is><t>Istotnie hamuje syntezę hormonów steroidowych</t></is></c><c r="N81" s="2" t="inlineStr" /><c r="O81" s="2" t="inlineStr" /><c r="P81" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q81" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="82"><c r="A82" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B82" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C82" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D82" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E82" s="2" t="inlineStr"><is><t>Wyłącznie na ustroje gram dodatnie działa:</t></is></c><c r="F82" s="2" t="inlineStr"><is><t>Mupriocyna</t></is></c><c r="G82" s="2" t="inlineStr" /><c r="H82" s="2" t="inlineStr" /><c r="I82" s="2" t="inlineStr" /><c r="J82" s="2" t="inlineStr" /><c r="K82" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="L82" s="2" t="inlineStr"><is><t>Fosfomycyna</t></is></c><c r="M82" s="2" t="inlineStr"><is><t>Gentamycyna</t></is></c><c r="N82" s="2" t="inlineStr" /><c r="O82" s="2" t="inlineStr" /><c r="P82" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q82" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="83"><c r="A83" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B83" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C83" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D83" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E83" s="2" t="inlineStr"><is><t>W leczeniu rzęsistkowicy (Trichomonas Vaginalis) wykorzystuje się:</t></is></c><c r="F83" s="2" t="inlineStr"><is><t>Tynidazol</t></is></c><c r="G83" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="H83" s="2" t="inlineStr" /><c r="I83" s="2" t="inlineStr" /><c r="J83" s="2" t="inlineStr" /><c r="K83" s="2" t="inlineStr"><is><t>Sulfametoksazol+trymetoprym</t></is></c><c r="L83" s="2" t="inlineStr"><is><t>Spiramycynę</t></is></c><c r="M83" s="2" t="inlineStr" /><c r="N83" s="2" t="inlineStr" /><c r="O83" s="2" t="inlineStr" /><c r="P83" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q83" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="84"><c r="A84" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B84" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C84" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D84" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E84" s="2" t="inlineStr"><is><t>Do charakterystycznych działań niepożądanych inhibitorów proteazy HIV należy/należą:</t></is></c><c r="F84" s="2" t="inlineStr"><is><t>Liczne interakcje lekowe</t></is></c><c r="G84" s="2" t="inlineStr"><is><t>Cukrzyca</t></is></c><c r="H84" s="2" t="inlineStr"><is><t>Uszkodzenie wątroby</t></is></c><c r="I84" s="2" t="inlineStr"><is><t>Hipertriglicerydemia</t></is></c><c r="J84" s="2" t="inlineStr" /><c r="K84" s="2" t="inlineStr" /><c r="L84" s="2" t="inlineStr" /><c r="M84" s="2" t="inlineStr" /><c r="N84" s="2" t="inlineStr" /><c r="O84" s="2" t="inlineStr" /><c r="P84" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q84" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="85"><c r="A85" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B85" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C85" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D85" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E85" s="2" t="inlineStr"><is><t>W zakażeniu o etiologii Candida albicans można zastosować miejscowo:</t></is></c><c r="F85" s="2" t="inlineStr"><is><t>Natamycynę</t></is></c><c r="G85" s="2" t="inlineStr"><is><t>Mykonazol</t></is></c><c r="H85" s="2" t="inlineStr" /><c r="I85" s="2" t="inlineStr" /><c r="J85" s="2" t="inlineStr" /><c r="K85" s="2" t="inlineStr"><is><t>Mykafunginę</t></is></c><c r="L85" s="2" t="inlineStr"><is><t>Izawukonazol</t></is></c><c r="M85" s="2" t="inlineStr" /><c r="N85" s="2" t="inlineStr" /><c r="O85" s="2" t="inlineStr" /><c r="P85" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q85" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="86"><c r="A86" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B86" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C86" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D86" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E86" s="2" t="inlineStr"><is><t>Jeśli celem farmakodynamicznym dla stosowanego antybiotyku jest wysoka wartość T&gt;MIC to powinno się:</t></is></c><c r="F86" s="2" t="inlineStr"><is><t>Monitorować stężenie leku we krwi w celu modyfikacji dawkowania</t></is></c><c r="G86" s="2" t="inlineStr"><is><t>Podawać lek w przedłużonym wlewie dożylnym</t></is></c><c r="H86" s="2" t="inlineStr"><is><t>Zwiększać częstość podawania leku w ciągu doby</t></is></c><c r="I86" s="2" t="inlineStr" /><c r="J86" s="2" t="inlineStr" /><c r="K86" s="2" t="inlineStr"><is><t>Podać lek w pojedynczej skumulowanej dawce dobowej</t></is></c><c r="L86" s="2" t="inlineStr" /><c r="M86" s="2" t="inlineStr" /><c r="N86" s="2" t="inlineStr" /><c r="O86" s="2" t="inlineStr" /><c r="P86" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q86" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="87"><c r="A87" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B87" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C87" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D87" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E87" s="2" t="inlineStr"><is><t>Do przestarzałych środków odkażających, które z powodu braku skuteczności lub istotnych działań niepożądanych nie powinny być obecnie stosowane należy:</t></is></c><c r="F87" s="2" t="inlineStr"><is><t>Nadmanganian potasu</t></is></c><c r="G87" s="2" t="inlineStr"><is><t>Tetraboran sodowy</t></is></c><c r="H87" s="2" t="inlineStr" /><c r="I87" s="2" t="inlineStr" /><c r="J87" s="2" t="inlineStr" /><c r="K87" s="2" t="inlineStr"><is><t>Oktenidyna</t></is></c><c r="L87" s="2" t="inlineStr"><is><t>Jodopowidon</t></is></c><c r="M87" s="2" t="inlineStr" /><c r="N87" s="2" t="inlineStr" /><c r="O87" s="2" t="inlineStr" /><c r="P87" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q87" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="88"><c r="A88" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B88" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C88" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D88" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E88" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenia dotyczące profilaktyki i leczenia malarii:</t></is></c><c r="F88" s="2" t="inlineStr"><is><t>Lumefantryna w połączeniu z artemeterem może być skuteczna w zakażeniu Plasmodium falciparum</t></is></c><c r="G88" s="2" t="inlineStr"><is><t>W przypadkach wymagających profilaktyki długoterminowej można zastosować chlorochinę</t></is></c><c r="H88" s="2" t="inlineStr" /><c r="I88" s="2" t="inlineStr" /><c r="J88" s="2" t="inlineStr" /><c r="K88" s="2" t="inlineStr"><is><t>Pochodne artemizyniny zalecane są tylko do profilaktyki malarii</t></is></c><c r="L88" s="2" t="inlineStr"><is><t>Atowakwon z proguanilem może być stosowany u osób z upośledzoną czynnością nerek (GFR&lt;30)</t></is></c><c r="M88" s="2" t="inlineStr" /><c r="N88" s="2" t="inlineStr" /><c r="O88" s="2" t="inlineStr" /><c r="P88" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q88" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="89"><c r="A89" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B89" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C89" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D89" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E89" s="2" t="inlineStr"><is><t>Do przyczyn jatrogennej nefropatii można zaliczyć stosowanie:</t></is></c><c r="F89" s="2" t="inlineStr"><is><t>Jodowych środków kontrastowych podczas koronarografii</t></is></c><c r="G89" s="2" t="inlineStr"><is><t>Ibuprofenu przewlekle w reumatoidalnym zapaleniu stawów</t></is></c><c r="H89" s="2" t="inlineStr"><is><t>Ramiprylu w niewydolności serca</t></is></c><c r="I89" s="2" t="inlineStr" /><c r="J89" s="2" t="inlineStr" /><c r="K89" s="2" t="inlineStr"><is><t>Loratadyny przewlekle w alergicznym zapaleniu błony śluzowej nosa</t></is></c><c r="L89" s="2" t="inlineStr" /><c r="M89" s="2" t="inlineStr" /><c r="N89" s="2" t="inlineStr" /><c r="O89" s="2" t="inlineStr" /><c r="P89" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q89" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="90"><c r="A90" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B90" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C90" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D90" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E90" s="2" t="inlineStr"><is><t>Wskaż prawdziwe zdania dotyczące leczenia morfiną:</t></is></c><c r="F90" s="2" t="inlineStr"><is><t>Metabolity morfiny wydalane są przez nerki</t></is></c><c r="G90" s="2" t="inlineStr"><is><t>Przy przewlekłym stosowaniu morfiny powstaje morfino-6-glukuronian – metabolit, którego siła działania analgetycznego przewyższa siłę działania związku macierzystego</t></is></c><c r="H90" s="2" t="inlineStr"><is><t>Morfina może być podawana zewnątrzoponowo</t></is></c><c r="I90" s="2" t="inlineStr" /><c r="J90" s="2" t="inlineStr" /><c r="K90" s="2" t="inlineStr"><is><t>Morfina ma dużą biodostępność po podaniu doustnym</t></is></c><c r="L90" s="2" t="inlineStr" /><c r="M90" s="2" t="inlineStr" /><c r="N90" s="2" t="inlineStr" /><c r="O90" s="2" t="inlineStr" /><c r="P90" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q90" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="91"><c r="A91" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B91" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C91" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D91" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E91" s="2" t="inlineStr"><is><t>Wskazanie do insulinoterapii jest:</t></is></c><c r="F91" s="2" t="inlineStr"><is><t>Cukrzyca typu LADA</t></is></c><c r="G91" s="2" t="inlineStr"><is><t>Ostry zespół wieńcowy u osoby z cukrzycą typu II</t></is></c><c r="H91" s="2" t="inlineStr"><is><t>Znaczna hiperglikemia (&gt;300) w przebiegu cukrzycy typu II</t></is></c><c r="I91" s="2" t="inlineStr"><is><t>Cukrzyca ciężarnych</t></is></c><c r="J91" s="2" t="inlineStr" /><c r="K91" s="2" t="inlineStr" /><c r="L91" s="2" t="inlineStr" /><c r="M91" s="2" t="inlineStr" /><c r="N91" s="2" t="inlineStr" /><c r="O91" s="2" t="inlineStr" /><c r="P91" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q91" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="92"><c r="A92" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B92" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C92" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D92" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E92" s="2" t="inlineStr"><is><t>Długodziałające analogii insuliny w porównaniu do insuliny protaminowo-cynkowej (NPH) charakteryzują się:</t></is></c><c r="F92" s="2" t="inlineStr"><is><t>Mniejszym ryzykiem hipoglikemii</t></is></c><c r="G92" s="2" t="inlineStr" /><c r="H92" s="2" t="inlineStr" /><c r="I92" s="2" t="inlineStr" /><c r="J92" s="2" t="inlineStr" /><c r="K92" s="2" t="inlineStr"><is><t>Mniejszym ryzykiem onkologicznym</t></is></c><c r="L92" s="2" t="inlineStr"><is><t>Większym ryzykiem zjawiska brzasku</t></is></c><c r="M92" s="2" t="inlineStr"><is><t>Działaniem anorektycznym</t></is></c><c r="N92" s="2" t="inlineStr" /><c r="O92" s="2" t="inlineStr" /><c r="P92" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q92" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="93"><c r="A93" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B93" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C93" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D93" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E93" s="2" t="inlineStr"><is><t>Zmniejszenie obwodowej konwersji tyroksyny do trójjodotyroniny jest efektem stosowania:</t></is></c><c r="F93" s="2" t="inlineStr"><is><t>Hydrokortyzonu</t></is></c><c r="G93" s="2" t="inlineStr"><is><t>Propylotiouracylu</t></is></c><c r="H93" s="2" t="inlineStr"><is><t>Propanololu</t></is></c><c r="I93" s="2" t="inlineStr" /><c r="J93" s="2" t="inlineStr" /><c r="K93" s="2" t="inlineStr"><is><t>Płynu Lugola</t></is></c><c r="L93" s="2" t="inlineStr" /><c r="M93" s="2" t="inlineStr" /><c r="N93" s="2" t="inlineStr" /><c r="O93" s="2" t="inlineStr" /><c r="P93" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q93" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="94"><c r="A94" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B94" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C94" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D94" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E94" s="2" t="inlineStr"><is><t>Wskazaniem do stosowania hormonalnej terapii zastępczej u kobiet po menopauzie jest:</t></is></c><c r="F94" s="2" t="inlineStr"><is><t>Obecność objawów wypadowych</t></is></c><c r="G94" s="2" t="inlineStr" /><c r="H94" s="2" t="inlineStr" /><c r="I94" s="2" t="inlineStr" /><c r="J94" s="2" t="inlineStr" /><c r="K94" s="2" t="inlineStr"><is><t>Wtórna profilaktyka chorób układu krążenia</t></is></c><c r="L94" s="2" t="inlineStr"><is><t>Profilaktyka osteoporozy</t></is></c><c r="M94" s="2" t="inlineStr"><is><t>Zapobieganie chorobie Alzheimera</t></is></c><c r="N94" s="2" t="inlineStr" /><c r="O94" s="2" t="inlineStr" /><c r="P94" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q94" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="95"><c r="A95" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B95" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C95" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D95" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E95" s="2" t="inlineStr"><is><t>Przeciwbólowy efekt pułapowy wykazuje:</t></is></c><c r="F95" s="2" t="inlineStr"><is><t>Naproksen</t></is></c><c r="G95" s="2" t="inlineStr"><is><t>Buprenorfina</t></is></c><c r="H95" s="2" t="inlineStr"><is><t>Ibuprofen</t></is></c><c r="I95" s="2" t="inlineStr" /><c r="J95" s="2" t="inlineStr" /><c r="K95" s="2" t="inlineStr"><is><t>Oksykodon</t></is></c><c r="L95" s="2" t="inlineStr" /><c r="M95" s="2" t="inlineStr" /><c r="N95" s="2" t="inlineStr" /><c r="O95" s="2" t="inlineStr" /><c r="P95" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q95" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="96"><c r="A96" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B96" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C96" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D96" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E96" s="2" t="inlineStr"><is><t>Teofilina:</t></is></c><c r="F96" s="2" t="inlineStr"><is><t>Jest anatgonistą receptora adenozynowego</t></is></c><c r="G96" s="2" t="inlineStr"><is><t>Hamuje aktywność fosfodiesteraz</t></is></c><c r="H96" s="2" t="inlineStr"><is><t>Zwiększa przepływ nerkowy</t></is></c><c r="I96" s="2" t="inlineStr"><is><t>Pobudza ośrodek oddechowy w rdzeniu przedłużonym</t></is></c><c r="J96" s="2" t="inlineStr" /><c r="K96" s="2" t="inlineStr" /><c r="L96" s="2" t="inlineStr" /><c r="M96" s="2" t="inlineStr" /><c r="N96" s="2" t="inlineStr" /><c r="O96" s="2" t="inlineStr" /><c r="P96" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q96" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="97"><c r="A97" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B97" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C97" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D97" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E97" s="2" t="inlineStr"><is><t>Idealny glikokortykosteroid wziewny:</t></is></c><c r="F97" s="2" t="inlineStr"><is><t>Połknięty charakteryzuje się niewielką biodostępnością</t></is></c><c r="G97" s="2" t="inlineStr" /><c r="H97" s="2" t="inlineStr" /><c r="I97" s="2" t="inlineStr" /><c r="J97" s="2" t="inlineStr" /><c r="K97" s="2" t="inlineStr"><is><t>Dobrze wchłania się z pęcherzyków płucnych</t></is></c><c r="L97" s="2" t="inlineStr"><is><t>Nie podlega efektowi pierwszego przejścia przez wątrobę</t></is></c><c r="M97" s="2" t="inlineStr"><is><t>Ma krótki okres półtrwania kompleksu glikokortkosteroidu z receptorem t1/2=2-3h</t></is></c><c r="N97" s="2" t="inlineStr" /><c r="O97" s="2" t="inlineStr" /><c r="P97" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q97" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="98"><c r="A98" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B98" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C98" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D98" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E98" s="2" t="inlineStr"><is><t>Działanie keratolityczne wykazuje:</t></is></c><c r="F98" s="2" t="inlineStr"><is><t>Mocznik</t></is></c><c r="G98" s="2" t="inlineStr"><is><t>Kwas salicylowy</t></is></c><c r="H98" s="2" t="inlineStr"><is><t>Nadtlenek benzoilu</t></is></c><c r="I98" s="2" t="inlineStr" /><c r="J98" s="2" t="inlineStr" /><c r="K98" s="2" t="inlineStr"><is><t>Metoksalen</t></is></c><c r="L98" s="2" t="inlineStr" /><c r="M98" s="2" t="inlineStr" /><c r="N98" s="2" t="inlineStr" /><c r="O98" s="2" t="inlineStr" /><c r="P98" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q98" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="99"><c r="A99" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B99" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C99" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D99" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E99" s="2" t="inlineStr"><is><t>W zatruciu solami litu:</t></is></c><c r="F99" s="2" t="inlineStr"><is><t>Należy natychmiast zakończyć podawanie litu</t></is></c><c r="G99" s="2" t="inlineStr"><is><t>W leczeniu ostrego zatrucia istotne znaczenie ma intensywne wyrównanie zaburzeń gospodarki wodno-elektrolitowej, zwłaszcza uzupełnianie niedoboru sodu poprzez przetaczanie roztworu 0,9% NaCl dożylnie</t></is></c><c r="H99" s="2" t="inlineStr"><is><t>Podstawową metodą eliminacji leku jest hemodializa</t></is></c><c r="I99" s="2" t="inlineStr" /><c r="J99" s="2" t="inlineStr" /><c r="K99" s="2" t="inlineStr"><is><t>Korzystne działanie ma stosowanie węgla aktywowanego</t></is></c><c r="L99" s="2" t="inlineStr" /><c r="M99" s="2" t="inlineStr" /><c r="N99" s="2" t="inlineStr" /><c r="O99" s="2" t="inlineStr" /><c r="P99" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q99" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="100"><c r="A100" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B100" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C100" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D100" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E100" s="2" t="inlineStr"><is><t>Fluorochinolony:</t></is></c><c r="F100" s="2" t="inlineStr"><is><t>mogą powodować zapalenie więzadeł</t></is></c><c r="G100" s="2" t="inlineStr" /><c r="H100" s="2" t="inlineStr" /><c r="I100" s="2" t="inlineStr" /><c r="J100" s="2" t="inlineStr" /><c r="K100" s="2" t="inlineStr"><is><t>słabo wchłaniają się z przewodu pokarmowego</t></is></c><c r="L100" s="2" t="inlineStr"><is><t>są grupą, na którą rzadko stwierdza się oporność bakteryjną</t></is></c><c r="M100" s="2" t="inlineStr"><is><t>niezależnie od generacji wykazują aktywność wyłącznie wobec bakterii tlenowych</t></is></c><c r="N100" s="2" t="inlineStr" /><c r="O100" s="2" t="inlineStr" /><c r="P100" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q100" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="101"><c r="A101" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B101" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C101" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D101" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E101" s="2" t="inlineStr"><is><t>Błędny schemat terapeutyczny to zastosowanie:</t></is></c><c r="F101" s="2" t="inlineStr"><is><t>loperamidu w zapalnej biegunce poantybiotykowej przez 10 dni</t></is></c><c r="G101" s="2" t="inlineStr" /><c r="H101" s="2" t="inlineStr" /><c r="I101" s="2" t="inlineStr" /><c r="J101" s="2" t="inlineStr" /><c r="K101" s="2" t="inlineStr"><is><t>azytromycyny w krztuścu przez 5 dni</t></is></c><c r="L101" s="2" t="inlineStr"><is><t>kotrymoksazolu w niepowikłanym zakażeniu układu moczowego przez 3 dni</t></is></c><c r="M101" s="2" t="inlineStr"><is><t>fenoksymetylpenicyliny w anginie paciorkowcowej przez 10 dni</t></is></c><c r="N101" s="2" t="inlineStr" /><c r="O101" s="2" t="inlineStr" /><c r="P101" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q101" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="102"><c r="A102" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B102" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C102" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D102" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E102" s="2" t="inlineStr"><is><t>W leczeniu 60-letniego pacjenta z pozaszpitalnym zapaleniem płuc (skala CURB-0pkt) uwzględniającym typową etiologię zakażenia u dorosłych należy:</t></is></c><c r="F102" s="2" t="inlineStr"><is><t>stosować stałe optymalne przedziały dawkowania w ciągu całej doby</t></is></c><c r="G102" s="2" t="inlineStr"><is><t>w razie nadwrażliwości na leczenie początkowe w wywiadach zastosować lewofloksacynę lub moksyfloksacynę</t></is></c><c r="H102" s="2" t="inlineStr" /><c r="I102" s="2" t="inlineStr" /><c r="J102" s="2" t="inlineStr" /><c r="K102" s="2" t="inlineStr"><is><t>leczyć 2 lekami przeciwbakteryjnymi o różnych mechanizmach działania</t></is></c><c r="L102" s="2" t="inlineStr"><is><t>prowadzić terapię co najmniej 21 dni</t></is></c><c r="M102" s="2" t="inlineStr" /><c r="N102" s="2" t="inlineStr" /><c r="O102" s="2" t="inlineStr" /><c r="P102" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q102" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="103"><c r="A103" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B103" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C103" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D103" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E103" s="2" t="inlineStr"><is><t>W leczeniu zapalenia opon mózgowo-rdzeniowych uzasadnione jest zastosowanie:</t></is></c><c r="F103" s="2" t="inlineStr"><is><t>ceftriaksonu</t></is></c><c r="G103" s="2" t="inlineStr"><is><t>acyklowiru</t></is></c><c r="H103" s="2" t="inlineStr"><is><t>meropenemu</t></is></c><c r="I103" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="J103" s="2" t="inlineStr" /><c r="K103" s="2" t="inlineStr" /><c r="L103" s="2" t="inlineStr" /><c r="M103" s="2" t="inlineStr" /><c r="N103" s="2" t="inlineStr" /><c r="O103" s="2" t="inlineStr" /><c r="P103" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q103" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="104"><c r="A104" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B104" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C104" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D104" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E104" s="2" t="inlineStr"><is><t>Wyłącznie na drobnoustroje Gram ujemne działa:</t></is></c><c r="F104" s="2" t="inlineStr"><is><t>aztreonam</t></is></c><c r="G104" s="2" t="inlineStr" /><c r="H104" s="2" t="inlineStr" /><c r="I104" s="2" t="inlineStr" /><c r="J104" s="2" t="inlineStr" /><c r="K104" s="2" t="inlineStr"><is><t>mupirocyna</t></is></c><c r="L104" s="2" t="inlineStr"><is><t>kwas fusydowy</t></is></c><c r="M104" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="N104" s="2" t="inlineStr" /><c r="O104" s="2" t="inlineStr" /><c r="P104" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q104" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="105"><c r="A105" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B105" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C105" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D105" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E105" s="2" t="inlineStr"><is><t>W leczeniu toksoplazmozy wykorzystuje się:</t></is></c><c r="F105" s="2" t="inlineStr"><is><t>pirymetaminę z sulfadiazyną</t></is></c><c r="G105" s="2" t="inlineStr"><is><t>spiramycynę</t></is></c><c r="H105" s="2" t="inlineStr" /><c r="I105" s="2" t="inlineStr" /><c r="J105" s="2" t="inlineStr" /><c r="K105" s="2" t="inlineStr"><is><t>dalfoprystynę/chinuprystynę</t></is></c><c r="L105" s="2" t="inlineStr"><is><t>oksytetracyklinę</t></is></c><c r="M105" s="2" t="inlineStr" /><c r="N105" s="2" t="inlineStr" /><c r="O105" s="2" t="inlineStr" /><c r="P105" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q105" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="106"><c r="A106" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B106" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C106" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D106" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E106" s="2" t="inlineStr"><is><t>Do odległych działań niepożądanych terapii HAART (Highly Active Antiretroviral Therapy) należy:</t></is></c><c r="F106" s="2" t="inlineStr"><is><t>uszkodzenie wątroby</t></is></c><c r="G106" s="2" t="inlineStr"><is><t>lipodystrofia</t></is></c><c r="H106" s="2" t="inlineStr"><is><t>kwasica mleczanowa</t></is></c><c r="I106" s="2" t="inlineStr"><is><t>insulinooporność</t></is></c><c r="J106" s="2" t="inlineStr" /><c r="K106" s="2" t="inlineStr" /><c r="L106" s="2" t="inlineStr" /><c r="M106" s="2" t="inlineStr" /><c r="N106" s="2" t="inlineStr" /><c r="O106" s="2" t="inlineStr" /><c r="P106" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q106" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="107"><c r="A107" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B107" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C107" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D107" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E107" s="2" t="inlineStr"><is><t>W grzybiczym zakażeniu paznokci można zastosować</t></is></c><c r="F107" s="2" t="inlineStr"><is><t>amorolfinę</t></is></c><c r="G107" s="2" t="inlineStr" /><c r="H107" s="2" t="inlineStr" /><c r="I107" s="2" t="inlineStr" /><c r="J107" s="2" t="inlineStr" /><c r="K107" s="2" t="inlineStr"><is><t>natamycynę</t></is></c><c r="L107" s="2" t="inlineStr"><is><t>klotrymazol</t></is></c><c r="M107" s="2" t="inlineStr"><is><t>kaspofunginę</t></is></c><c r="N107" s="2" t="inlineStr" /><c r="O107" s="2" t="inlineStr" /><c r="P107" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q107" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="108"><c r="A108" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B108" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C108" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D108" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E108" s="2" t="inlineStr"><is><t>Efekt bakteriobójczy zależny od skumulowanej ekspozycji (AUC24/MIC) wykazuje:</t></is></c><c r="F108" s="2" t="inlineStr"><is><t>lewofloksacyna</t></is></c><c r="G108" s="2" t="inlineStr"><is><t>azytromycyna</t></is></c><c r="H108" s="2" t="inlineStr" /><c r="I108" s="2" t="inlineStr" /><c r="J108" s="2" t="inlineStr" /><c r="K108" s="2" t="inlineStr"><is><t>amoksycylina z kwasem klawulanowym</t></is></c><c r="L108" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="M108" s="2" t="inlineStr" /><c r="N108" s="2" t="inlineStr" /><c r="O108" s="2" t="inlineStr" /><c r="P108" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q108" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="109"><c r="A109" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B109" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C109" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D109" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E109" s="2" t="inlineStr"><is><t>Do odkażania rany w obrębie skóry można zastosować:</t></is></c><c r="F109" s="2" t="inlineStr"><is><t>oktenidynę</t></is></c><c r="G109" s="2" t="inlineStr"><is><t>jodopowidon</t></is></c><c r="H109" s="2" t="inlineStr" /><c r="I109" s="2" t="inlineStr" /><c r="J109" s="2" t="inlineStr" /><c r="K109" s="2" t="inlineStr"><is><t>wodę do wstrzyknięć</t></is></c><c r="L109" s="2" t="inlineStr"><is><t>kwas borowy</t></is></c><c r="M109" s="2" t="inlineStr" /><c r="N109" s="2" t="inlineStr" /><c r="O109" s="2" t="inlineStr" /><c r="P109" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q109" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="110"><c r="A110" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B110" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C110" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D110" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E110" s="2" t="inlineStr"><is><t>Koszt dodatkowego roku życia skorygowanego o jakość (ang. QALY – quality adjusted life year):</t></is></c><c r="F110" s="2" t="inlineStr"><is><t>stanowi formalne kryterium refundacyjne zgodnie z obowiązującymi regulacjami prawnymi</t></is></c><c r="G110" s="2" t="inlineStr"><is><t>jest wynikiem analizy kosztów użyteczności</t></is></c><c r="H110" s="2" t="inlineStr"><is><t>jego wartość progowa, czyli maksymalna dla procedur uznanych za kosztowo efektywne, stanowi 3-krotność produktu krajowego brutto per capita zgodnie z obowiązującymi regulacjami prawnymi</t></is></c><c r="I110" s="2" t="inlineStr" /><c r="J110" s="2" t="inlineStr" /><c r="K110" s="2" t="inlineStr"><is><t>możliwy jest do oszacowania tylko w przypadku procedur zmniejszających umieralność całkowitą</t></is></c><c r="L110" s="2" t="inlineStr" /><c r="M110" s="2" t="inlineStr" /><c r="N110" s="2" t="inlineStr" /><c r="O110" s="2" t="inlineStr" /><c r="P110" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q110" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="111"><c r="A111" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B111" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C111" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D111" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E111" s="2" t="inlineStr"><is><t>U pacjenta z niewydolnością nerek należy dokonać modyfikacji dawek:</t></is></c><c r="F111" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="G111" s="2" t="inlineStr"><is><t>cyprofloksacyny</t></is></c><c r="H111" s="2" t="inlineStr"><is><t>gentamycyny</t></is></c><c r="I111" s="2" t="inlineStr" /><c r="J111" s="2" t="inlineStr" /><c r="K111" s="2" t="inlineStr"><is><t>erytromycyny</t></is></c><c r="L111" s="2" t="inlineStr" /><c r="M111" s="2" t="inlineStr" /><c r="N111" s="2" t="inlineStr" /><c r="O111" s="2" t="inlineStr" /><c r="P111" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q111" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="112"><c r="A112" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B112" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C112" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D112" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E112" s="2" t="inlineStr"><is><t>Rotacja opioidów jest uzasadniona w przypadku:</t></is></c><c r="F112" s="2" t="inlineStr"><is><t>nudności</t></is></c><c r="G112" s="2" t="inlineStr"><is><t>zaburzeń świadomości</t></is></c><c r="H112" s="2" t="inlineStr"><is><t>długotrwałej (bezterminowej) terapii w celu ułatwienia jej prowadzenia</t></is></c><c r="I112" s="2" t="inlineStr" /><c r="J112" s="2" t="inlineStr" /><c r="K112" s="2" t="inlineStr"><is><t>zaparć</t></is></c><c r="L112" s="2" t="inlineStr" /><c r="M112" s="2" t="inlineStr" /><c r="N112" s="2" t="inlineStr" /><c r="O112" s="2" t="inlineStr" /><c r="P112" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q112" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="113"><c r="A113" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B113" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C113" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D113" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E113" s="2" t="inlineStr"><is><t>Dapagliflozyna:</t></is></c><c r="F113" s="2" t="inlineStr"><is><t>zwiększa ryzyko zakażeń układu moczowo-płciowego</t></is></c><c r="G113" s="2" t="inlineStr"><is><t>może spowodować kwasicę ketonową</t></is></c><c r="H113" s="2" t="inlineStr" /><c r="I113" s="2" t="inlineStr" /><c r="J113" s="2" t="inlineStr" /><c r="K113" s="2" t="inlineStr"><is><t>zmniejsza glukozurię</t></is></c><c r="L113" s="2" t="inlineStr"><is><t>nie może być stosowana łącznie z insuliną</t></is></c><c r="M113" s="2" t="inlineStr" /><c r="N113" s="2" t="inlineStr" /><c r="O113" s="2" t="inlineStr" /><c r="P113" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q113" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="114"><c r="A114" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B114" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C114" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D114" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E114" s="2" t="inlineStr"><is><t>Wskaż zdanie prawdziwe:</t></is></c><c r="F114" s="2" t="inlineStr"><is><t>zwiększenie stężenia glukozy w godzinach porannych poprzedzone hipoglikemią nocną może być wskazaniem do zmniejszenia dawki insuliny bazowej</t></is></c><c r="G114" s="2" t="inlineStr"><is><t>efekt brzasku może zmniejszyć zastosowanie długodziałających bezszczytowych analogów insuliny</t></is></c><c r="H114" s="2" t="inlineStr"><is><t>kardioprotekcyjne działanie empagliflozyny może mieć związek z usprawnieniem procesów energetycznych w komórkach mięśnia sercowego</t></is></c><c r="I114" s="2" t="inlineStr" /><c r="J114" s="2" t="inlineStr" /><c r="K114" s="2" t="inlineStr"><is><t>insulina izofanowa (NPH) jest przeznaczona do stosowana przed głównymi posiłkami</t></is></c><c r="L114" s="2" t="inlineStr" /><c r="M114" s="2" t="inlineStr" /><c r="N114" s="2" t="inlineStr" /><c r="O114" s="2" t="inlineStr" /><c r="P114" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q114" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="115"><c r="A115" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B115" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C115" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D115" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E115" s="2" t="inlineStr"><is><t>W leczeniu nadczynności tarczycy można zastosować:</t></is></c><c r="F115" s="2" t="inlineStr"><is><t>jod promieniotwórczy 131 I</t></is></c><c r="G115" s="2" t="inlineStr"><is><t>płyn Lugola</t></is></c><c r="H115" s="2" t="inlineStr"><is><t>tiamazol</t></is></c><c r="I115" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="J115" s="2" t="inlineStr" /><c r="K115" s="2" t="inlineStr" /><c r="L115" s="2" t="inlineStr" /><c r="M115" s="2" t="inlineStr" /><c r="N115" s="2" t="inlineStr" /><c r="O115" s="2" t="inlineStr" /><c r="P115" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q115" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="116"><c r="A116" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B116" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C116" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D116" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E116" s="2" t="inlineStr"><is><t>Do progestagenów należy:</t></is></c><c r="F116" s="2" t="inlineStr"><is><t>megestrol</t></is></c><c r="G116" s="2" t="inlineStr"><is><t>noretysteron</t></is></c><c r="H116" s="2" t="inlineStr" /><c r="I116" s="2" t="inlineStr" /><c r="J116" s="2" t="inlineStr" /><c r="K116" s="2" t="inlineStr"><is><t>dutasteryd</t></is></c><c r="L116" s="2" t="inlineStr"><is><t>anastrozol</t></is></c><c r="M116" s="2" t="inlineStr" /><c r="N116" s="2" t="inlineStr" /><c r="O116" s="2" t="inlineStr" /><c r="P116" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q116" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="117"><c r="A117" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B117" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C117" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D117" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E117" s="2" t="inlineStr"><is><t>Do leków antyagregacyjnych stosowanych w profilaktyce wtórnej udaru niedokrwiennego mózgu na podłożu miażdżycy naczyń do- i mózgowych należą:</t></is></c><c r="F117" s="2" t="inlineStr"><is><t>klopidogrel</t></is></c><c r="G117" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="H117" s="2" t="inlineStr" /><c r="I117" s="2" t="inlineStr" /><c r="J117" s="2" t="inlineStr" /><c r="K117" s="2" t="inlineStr"><is><t>tikagrelor</t></is></c><c r="L117" s="2" t="inlineStr"><is><t>prasugrel</t></is></c><c r="M117" s="2" t="inlineStr" /><c r="N117" s="2" t="inlineStr" /><c r="O117" s="2" t="inlineStr" /><c r="P117" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q117" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="118"><c r="A118" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B118" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C118" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D118" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E118" s="2" t="inlineStr"><is><t>W ciężkiej hiperkalcemii (&gt;15mg/dl) można zastosować dożylnie:</t></is></c><c r="F118" s="2" t="inlineStr"><is><t>kalcytoninę</t></is></c><c r="G118" s="2" t="inlineStr"><is><t>pamidronian</t></is></c><c r="H118" s="2" t="inlineStr"><is><t>hydrokortyzon</t></is></c><c r="I118" s="2" t="inlineStr"><is><t>furosemid</t></is></c><c r="J118" s="2" t="inlineStr" /><c r="K118" s="2" t="inlineStr" /><c r="L118" s="2" t="inlineStr" /><c r="M118" s="2" t="inlineStr" /><c r="N118" s="2" t="inlineStr" /><c r="O118" s="2" t="inlineStr" /><c r="P118" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q118" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="119"><c r="A119" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B119" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C119" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D119" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E119" s="2" t="inlineStr"><is><t>Immunosupresyjne działanie glikokortykosteroidów jest spowodowane:</t></is></c><c r="F119" s="2" t="inlineStr"><is><t>redukcją liczby limfocytów T</t></is></c><c r="G119" s="2" t="inlineStr"><is><t>zahamowaniem funkcji makrofagów tkankowych</t></is></c><c r="H119" s="2" t="inlineStr" /><c r="I119" s="2" t="inlineStr" /><c r="J119" s="2" t="inlineStr" /><c r="K119" s="2" t="inlineStr"><is><t>zwiększeniem syntezy IL-2</t></is></c><c r="L119" s="2" t="inlineStr"><is><t>aktywacją fosfolipazy A2 i zmniejszeniem syntezy prostaglandyn</t></is></c><c r="M119" s="2" t="inlineStr" /><c r="N119" s="2" t="inlineStr" /><c r="O119" s="2" t="inlineStr" /><c r="P119" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q119" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="120"><c r="A120" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B120" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C120" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D120" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E120" s="2" t="inlineStr"><is><t>91-letni mężczyzna jest leczony od co najmniej 6 miesięcy tamsulozyną, finasterydem, diosminą, piracetamem, zolpidemem, witaminą D3 w dużej dawce i węglanem wapnia. Na tej podstawie można powiedzieć, że:</t></is></c><c r="F120" s="2" t="inlineStr"><is><t>choruje na rozrost gruczołu krokowego</t></is></c><c r="G120" s="2" t="inlineStr"><is><t>jest uzależniony od zolpidemu</t></is></c><c r="H120" s="2" t="inlineStr"><is><t>można bez konsekwencji odstawić piracetam</t></is></c><c r="I120" s="2" t="inlineStr"><is><t>terapia zmniejsza ryzyko osteoporotycznych złamań kości</t></is></c><c r="J120" s="2" t="inlineStr" /><c r="K120" s="2" t="inlineStr" /><c r="L120" s="2" t="inlineStr" /><c r="M120" s="2" t="inlineStr" /><c r="N120" s="2" t="inlineStr" /><c r="O120" s="2" t="inlineStr" /><c r="P120" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q120" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="121"><c r="A121" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B121" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C121" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D121" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E121" s="2" t="inlineStr"><is><t>Witamina K1 (fitomenadion):</t></is></c><c r="F121" s="2" t="inlineStr"><is><t>może być wskazana u osób ze spontanicznym zwiększeniem INR&gt;GGN (górnej granicy normy) spowodowanym antybiotykami niszczącymi fizjologiczną florę jelit</t></is></c><c r="G121" s="2" t="inlineStr"><is><t>nie antagonizuje działania heparyny</t></is></c><c r="H121" s="2" t="inlineStr"><is><t>może spowodować reakcję rzekomoanafilaktyczną</t></is></c><c r="I121" s="2" t="inlineStr"><is><t>jest antidotum w przedawkowaniu pochodnych hydroksykumaryny</t></is></c><c r="J121" s="2" t="inlineStr" /><c r="K121" s="2" t="inlineStr" /><c r="L121" s="2" t="inlineStr" /><c r="M121" s="2" t="inlineStr" /><c r="N121" s="2" t="inlineStr" /><c r="O121" s="2" t="inlineStr" /><c r="P121" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q121" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="122"><c r="A122" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B122" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C122" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D122" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E122" s="2" t="inlineStr"><is><t>Działanie zapierające wykazuje:</t></is></c><c r="F122" s="2" t="inlineStr"><is><t>oksykodon</t></is></c><c r="G122" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="H122" s="2" t="inlineStr"><is><t>oktreotyd</t></is></c><c r="I122" s="2" t="inlineStr" /><c r="J122" s="2" t="inlineStr" /><c r="K122" s="2" t="inlineStr"><is><t>fosforan sodu</t></is></c><c r="L122" s="2" t="inlineStr" /><c r="M122" s="2" t="inlineStr" /><c r="N122" s="2" t="inlineStr" /><c r="O122" s="2" t="inlineStr" /><c r="P122" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q122" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="123"><c r="A123" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B123" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C123" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D123" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E123" s="2" t="inlineStr"><is><t>W leczeniu ostrej biegunki u dzieci uzasadnione jest zastosowanie:</t></is></c><c r="F123" s="2" t="inlineStr"><is><t>probiotyku S. boulardi</t></is></c><c r="G123" s="2" t="inlineStr"><is><t>racekadotrylu</t></is></c><c r="H123" s="2" t="inlineStr"><is><t>doustnego płynu nawadniającego</t></is></c><c r="I123" s="2" t="inlineStr" /><c r="J123" s="2" t="inlineStr" /><c r="K123" s="2" t="inlineStr"><is><t>loperamidu</t></is></c><c r="L123" s="2" t="inlineStr" /><c r="M123" s="2" t="inlineStr" /><c r="N123" s="2" t="inlineStr" /><c r="O123" s="2" t="inlineStr" /><c r="P123" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q123" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="124"><c r="A124" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B124" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C124" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D124" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E124" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek - mechanizm działania:</t></is></c><c r="F124" s="2" t="inlineStr"><is><t>itopryd - antagonista receptora D2</t></is></c><c r="G124" s="2" t="inlineStr"><is><t>alwimopan - antagonista receptora μ</t></is></c><c r="H124" s="2" t="inlineStr" /><c r="I124" s="2" t="inlineStr" /><c r="J124" s="2" t="inlineStr" /><c r="K124" s="2" t="inlineStr"><is><t>alweryna - agonista receptora motylinowego</t></is></c><c r="L124" s="2" t="inlineStr"><is><t>simetykon - agonista receptora 5-HT4</t></is></c><c r="M124" s="2" t="inlineStr" /><c r="N124" s="2" t="inlineStr" /><c r="O124" s="2" t="inlineStr" /><c r="P124" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q124" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="125"><c r="A125" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B125" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C125" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D125" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E125" s="2" t="inlineStr"><is><t>W kolce wątrobowej uzasadnione jest podanie:</t></is></c><c r="F125" s="2" t="inlineStr"><is><t>ketoprofenu i.v</t></is></c><c r="G125" s="2" t="inlineStr"><is><t>papaweryny i.m</t></is></c><c r="H125" s="2" t="inlineStr"><is><t>butylobromku skopolaminy p.r</t></is></c><c r="I125" s="2" t="inlineStr"><is><t>buprenorfiny i.m</t></is></c><c r="J125" s="2" t="inlineStr" /><c r="K125" s="2" t="inlineStr" /><c r="L125" s="2" t="inlineStr" /><c r="M125" s="2" t="inlineStr" /><c r="N125" s="2" t="inlineStr" /><c r="O125" s="2" t="inlineStr" /><c r="P125" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q125" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="126"><c r="A126" s="2" t="inlineStr"><is><t>BÓLE GŁOWY</t></is></c><c r="B126" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C126" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D126" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E126" s="2" t="inlineStr"><is><t>Sumatryptan:</t></is></c><c r="F126" s="2" t="inlineStr"><is><t>pobudzając receptory 5-HT1D wywołuje wybiórczy skurcz naczyń i przerywa napad migreny</t></is></c><c r="G126" s="2" t="inlineStr"><is><t>jest niezalecany u pacjentów z chorobą niedokrwienną serca</t></is></c><c r="H126" s="2" t="inlineStr" /><c r="I126" s="2" t="inlineStr" /><c r="J126" s="2" t="inlineStr" /><c r="K126" s="2" t="inlineStr"><is><t>może być stosowany jedynie podskórnie</t></is></c><c r="L126" s="2" t="inlineStr"><is><t>może być podawany w czasie ciąży</t></is></c><c r="M126" s="2" t="inlineStr" /><c r="N126" s="2" t="inlineStr" /><c r="O126" s="2" t="inlineStr" /><c r="P126" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q126" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="127"><c r="A127" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B127" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C127" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D127" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E127" s="2" t="inlineStr"><is><t>W profilaktyce bólów migrenowych znalazł zastosowanie:</t></is></c><c r="F127" s="2" t="inlineStr"><is><t>topiramat</t></is></c><c r="G127" s="2" t="inlineStr"><is><t>erenumab</t></is></c><c r="H127" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="I127" s="2" t="inlineStr"><is><t>toksyna botulinowa</t></is></c><c r="J127" s="2" t="inlineStr" /><c r="K127" s="2" t="inlineStr" /><c r="L127" s="2" t="inlineStr" /><c r="M127" s="2" t="inlineStr" /><c r="N127" s="2" t="inlineStr" /><c r="O127" s="2" t="inlineStr" /><c r="P127" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q127" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="128"><c r="A128" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B128" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C128" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D128" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E128" s="2" t="inlineStr"><is><t>Erytropoetyna może zwiększyć:</t></is></c><c r="F128" s="2" t="inlineStr"><is><t>wartości ciśnienia tętniczego</t></is></c><c r="G128" s="2" t="inlineStr"><is><t>krzepliwość krwi</t></is></c><c r="H128" s="2" t="inlineStr"><is><t>maksymalną wydolność wysiłkową</t></is></c><c r="I128" s="2" t="inlineStr" /><c r="J128" s="2" t="inlineStr" /><c r="K128" s="2" t="inlineStr"><is><t>aktywność amylazy w surowicy</t></is></c><c r="L128" s="2" t="inlineStr" /><c r="M128" s="2" t="inlineStr" /><c r="N128" s="2" t="inlineStr" /><c r="O128" s="2" t="inlineStr" /><c r="P128" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q128" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="129"><c r="A129" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B129" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C129" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D129" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E129" s="2" t="inlineStr"><is><t>W profilaktyce wymiotów w przebiegu kinetoz stosuje się:</t></is></c><c r="F129" s="2" t="inlineStr"><is><t>skopolaminę</t></is></c><c r="G129" s="2" t="inlineStr"><is><t>dimenhydrinat</t></is></c><c r="H129" s="2" t="inlineStr" /><c r="I129" s="2" t="inlineStr" /><c r="J129" s="2" t="inlineStr" /><c r="K129" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="L129" s="2" t="inlineStr"><is><t>betahistynę</t></is></c><c r="M129" s="2" t="inlineStr" /><c r="N129" s="2" t="inlineStr" /><c r="O129" s="2" t="inlineStr" /><c r="P129" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q129" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="130"><c r="A130" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B130" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C130" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D130" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E130" s="2" t="inlineStr"><is><t>Oksymetazolina:</t></is></c><c r="F130" s="2" t="inlineStr"><is><t>może doprowadzić do wystąpienia tzw. efektu „ z odbicia”</t></is></c><c r="G130" s="2" t="inlineStr" /><c r="H130" s="2" t="inlineStr" /><c r="I130" s="2" t="inlineStr" /><c r="J130" s="2" t="inlineStr" /><c r="K130" s="2" t="inlineStr"><is><t>jest antagonistą receptorów adrenergicznych alfa</t></is></c><c r="L130" s="2" t="inlineStr"><is><t>wykazuje skuteczność kliniczną po 5. dniach terapii</t></is></c><c r="M130" s="2" t="inlineStr"><is><t>jest podawana doustnie</t></is></c><c r="N130" s="2" t="inlineStr" /><c r="O130" s="2" t="inlineStr" /><c r="P130" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q130" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="131"><c r="A131" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B131" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C131" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D131" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E131" s="2" t="inlineStr"><is><t>Petydyna:</t></is></c><c r="F131" s="2" t="inlineStr"><is><t>ma działanie zapierające</t></is></c><c r="G131" s="2" t="inlineStr"><is><t>nietypowo dla swojej grupy farmakologicznej rozszerza źrenice</t></is></c><c r="H131" s="2" t="inlineStr"><is><t>hamuje ośrodek oddechowy</t></is></c><c r="I131" s="2" t="inlineStr"><is><t>stosowana długotrwale działa neurotoksycznie przez kumulujący się metabolit</t></is></c><c r="J131" s="2" t="inlineStr" /><c r="K131" s="2" t="inlineStr" /><c r="L131" s="2" t="inlineStr" /><c r="M131" s="2" t="inlineStr" /><c r="N131" s="2" t="inlineStr" /><c r="O131" s="2" t="inlineStr" /><c r="P131" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q131" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="132"><c r="A132" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B132" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C132" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D132" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E132" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące małopłytkowości typu II wywołanej heparyną:</t></is></c><c r="F132" s="2" t="inlineStr"><is><t>stwierdzenie małopłytkowości immunologicznej w przebiegu leczenia heparyną jest wskazaniem do jej natychmiastowego odstawienia</t></is></c><c r="G132" s="2" t="inlineStr"><is><t>HIT II wiąże się z 20–40-krotnym zwiększeniem ryzyka zakrzepicy żylnej</t></is></c><c r="H132" s="2" t="inlineStr" /><c r="I132" s="2" t="inlineStr" /><c r="J132" s="2" t="inlineStr" /><c r="K132" s="2" t="inlineStr"><is><t>HIT II występuje najczęściej po 3 tygodniach od rozpoczęcia terapii heparyną</t></is></c><c r="L132" s="2" t="inlineStr"><is><t>heparyny drobnocząsteczkowe nie stwarzają ryzyka wystąpienia trombocytopenii immunologicznej</t></is></c><c r="M132" s="2" t="inlineStr" /><c r="N132" s="2" t="inlineStr" /><c r="O132" s="2" t="inlineStr" /><c r="P132" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q132" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="133"><c r="A133" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B133" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C133" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D133" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E133" s="2" t="inlineStr"><is><t>U kobiet w trzecim trymestrze ciąży przeciwwskazany/-a jest:</t></is></c><c r="F133" s="2" t="inlineStr"><is><t>ketoprofen</t></is></c><c r="G133" s="2" t="inlineStr"><is><t>walsartan</t></is></c><c r="H133" s="2" t="inlineStr"><is><t>acenokumarol</t></is></c><c r="I133" s="2" t="inlineStr" /><c r="J133" s="2" t="inlineStr" /><c r="K133" s="2" t="inlineStr"><is><t>enoksaparyna</t></is></c><c r="L133" s="2" t="inlineStr" /><c r="M133" s="2" t="inlineStr" /><c r="N133" s="2" t="inlineStr" /><c r="O133" s="2" t="inlineStr" /><c r="P133" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q133" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="134"><c r="A134" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B134" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C134" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D134" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E134" s="2" t="inlineStr"><is><t>U pacjenta leczonego przeciwzakrzepowo dabigatranem ze stwierdzonym umiarkowanym aktywnym krwawieniem należy:</t></is></c><c r="F134" s="2" t="inlineStr"><is><t>odroczyć podanie kolejnej dawki leku</t></is></c><c r="G134" s="2" t="inlineStr"><is><t>zapewnić podaż płynów</t></is></c><c r="H134" s="2" t="inlineStr"><is><t>rozważyć podanie węgla aktywowanego jeśli dabigatran był podany niedawno</t></is></c><c r="I134" s="2" t="inlineStr" /><c r="J134" s="2" t="inlineStr" /><c r="K134" s="2" t="inlineStr"><is><t>zastosować siarczan protaminy</t></is></c><c r="L134" s="2" t="inlineStr" /><c r="M134" s="2" t="inlineStr" /><c r="N134" s="2" t="inlineStr" /><c r="O134" s="2" t="inlineStr" /><c r="P134" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q134" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="135"><c r="A135" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B135" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C135" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D135" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E135" s="2" t="inlineStr"><is><t>Nadroparyna:</t></is></c><c r="F135" s="2" t="inlineStr"><is><t>może być podawana dożylnie</t></is></c><c r="G135" s="2" t="inlineStr"><is><t>jest skuteczna w leczeniu zakrzepicy żył głębokich</t></is></c><c r="H135" s="2" t="inlineStr" /><c r="I135" s="2" t="inlineStr" /><c r="J135" s="2" t="inlineStr" /><c r="K135" s="2" t="inlineStr"><is><t>jest antagonistą receptora PAR-1</t></is></c><c r="L135" s="2" t="inlineStr"><is><t>w profilaktyce zakrzepicy żylnej powinna być podana nie później niż 36 godzin przed zabiegiem chirurgicznym</t></is></c><c r="M135" s="2" t="inlineStr" /><c r="N135" s="2" t="inlineStr" /><c r="O135" s="2" t="inlineStr" /><c r="P135" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q135" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="136"><c r="A136" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B136" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C136" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D136" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E136" s="2" t="inlineStr"><is><t>Wskazaniem do podania tkankowego aktywatora plazminogenu (t-PA) może być:</t></is></c><c r="F136" s="2" t="inlineStr"><is><t>zatorowość płucna wysokiego ryzyka (czyli z niestabilnością hemodynamiczną)</t></is></c><c r="G136" s="2" t="inlineStr"><is><t>ostry zator tętnicy kończyny dolnej</t></is></c><c r="H136" s="2" t="inlineStr"><is><t>ostry udar niedokrwienny mózgu</t></is></c><c r="I136" s="2" t="inlineStr" /><c r="J136" s="2" t="inlineStr" /><c r="K136" s="2" t="inlineStr"><is><t>ostry zespół wieńcowy bez uniesienia odcinka ST</t></is></c><c r="L136" s="2" t="inlineStr" /><c r="M136" s="2" t="inlineStr" /><c r="N136" s="2" t="inlineStr" /><c r="O136" s="2" t="inlineStr" /><c r="P136" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q136" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="137"><c r="A137" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B137" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C137" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D137" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E137" s="2" t="inlineStr"><is><t>W udarze niedokrwiennym mózgu należy:</t></is></c><c r="F137" s="2" t="inlineStr"><is><t>obniżać ciśnienie tętnicze jeśli przekracza wartości 220/120 mmHg</t></is></c><c r="G137" s="2" t="inlineStr"><is><t>podać doustnie kwas acetylosalicylowy jeżeli nie można zastosować leczenia trombolitycznego</t></is></c><c r="H137" s="2" t="inlineStr" /><c r="I137" s="2" t="inlineStr" /><c r="J137" s="2" t="inlineStr" /><c r="K137" s="2" t="inlineStr"><is><t>stosować duże dawki heparyny niefrakcjonowanej</t></is></c><c r="L137" s="2" t="inlineStr"><is><t>profilaktycznie podawać antybiotyki β-laktamowe ze względu na bardzo częste występowanie infekcji dróg oddechowych</t></is></c><c r="M137" s="2" t="inlineStr" /><c r="N137" s="2" t="inlineStr" /><c r="O137" s="2" t="inlineStr" /><c r="P137" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q137" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="138"><c r="A138" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B138" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C138" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D138" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E138" s="2" t="inlineStr"><is><t>Inhibitory reduktazy HMG-CoA zwiększają produkcję:</t></is></c><c r="F138" s="2" t="inlineStr"><is><t>tkankowego aktywatora plazminogenu</t></is></c><c r="G138" s="2" t="inlineStr"><is><t>tlenku azotu</t></is></c><c r="H138" s="2" t="inlineStr" /><c r="I138" s="2" t="inlineStr" /><c r="J138" s="2" t="inlineStr" /><c r="K138" s="2" t="inlineStr"><is><t>metaloproteinaz</t></is></c><c r="L138" s="2" t="inlineStr"><is><t>tromboksanu A2</t></is></c><c r="M138" s="2" t="inlineStr" /><c r="N138" s="2" t="inlineStr" /><c r="O138" s="2" t="inlineStr" /><c r="P138" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q138" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="139"><c r="A139" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B139" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C139" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D139" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E139" s="2" t="inlineStr"><is><t>20% roztwór albumin:</t></is></c><c r="F139" s="2" t="inlineStr"><is><t>powoduje ponad 100% przyrost objętości osocza</t></is></c><c r="G139" s="2" t="inlineStr"><is><t>działa objętościowo do 6 h</t></is></c><c r="H139" s="2" t="inlineStr" /><c r="I139" s="2" t="inlineStr" /><c r="J139" s="2" t="inlineStr" /><c r="K139" s="2" t="inlineStr"><is><t>może spowodować uszkodzenie nerek</t></is></c><c r="L139" s="2" t="inlineStr"><is><t>ma istotny wpływ na krzepnięcie krwi</t></is></c><c r="M139" s="2" t="inlineStr" /><c r="N139" s="2" t="inlineStr" /><c r="O139" s="2" t="inlineStr" /><c r="P139" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q139" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="140"><c r="A140" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B140" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C140" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D140" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E140" s="2" t="inlineStr"><is><t>Zastosowanie atrakurium może być przyczyną:</t></is></c><c r="F140" s="2" t="inlineStr"><is><t>długotrwałego efektu zwiotczającego</t></is></c><c r="G140" s="2" t="inlineStr" /><c r="H140" s="2" t="inlineStr" /><c r="I140" s="2" t="inlineStr" /><c r="J140" s="2" t="inlineStr" /><c r="K140" s="2" t="inlineStr"><is><t>drżenia włókienkowego mięśni szkieletowych</t></is></c><c r="L140" s="2" t="inlineStr"><is><t>anestezji</t></is></c><c r="M140" s="2" t="inlineStr"><is><t>hipertermii złośliwej</t></is></c><c r="N140" s="2" t="inlineStr" /><c r="O140" s="2" t="inlineStr" /><c r="P140" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q140" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="141"><c r="A141" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B141" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C141" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D141" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E141" s="2" t="inlineStr"><is><t>Torasemid:</t></is></c><c r="F141" s="2" t="inlineStr"><is><t>hamuje symporter sodowo-potasowo-chlorkowy części grubościennej ramienia wstępującego pętli Henlego</t></is></c><c r="G141" s="2" t="inlineStr"><is><t>zwiększa aktywność reninową osocza</t></is></c><c r="H141" s="2" t="inlineStr" /><c r="I141" s="2" t="inlineStr" /><c r="J141" s="2" t="inlineStr" /><c r="K141" s="2" t="inlineStr"><is><t>zmniejsza wydalanie wapnia z moczem</t></is></c><c r="L141" s="2" t="inlineStr"><is><t>jest nieskuteczny, jeśli eGFRr &lt; 30 ml/min</t></is></c><c r="M141" s="2" t="inlineStr" /><c r="N141" s="2" t="inlineStr" /><c r="O141" s="2" t="inlineStr" /><c r="P141" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q141" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="142"><c r="A142" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B142" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C142" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D142" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E142" s="2" t="inlineStr"><is><t>Formularz świadomej zgody uczestnika na udział w badaniu klinicznym powinien zostać podpisany:</t></is></c><c r="F142" s="2" t="inlineStr"><is><t>przez uczestnika badania</t></is></c><c r="G142" s="2" t="inlineStr"><is><t>przez badacza</t></is></c><c r="H142" s="2" t="inlineStr"><is><t>w dwóch egzemplarzach</t></is></c><c r="I142" s="2" t="inlineStr" /><c r="J142" s="2" t="inlineStr" /><c r="K142" s="2" t="inlineStr"><is><t>bezpośrednio po badaniach oceniających czy pacjent spełnia kryteria włączenia do badania</t></is></c><c r="L142" s="2" t="inlineStr" /><c r="M142" s="2" t="inlineStr" /><c r="N142" s="2" t="inlineStr" /><c r="O142" s="2" t="inlineStr" /><c r="P142" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q142" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="143"><c r="A143" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B143" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C143" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D143" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E143" s="2" t="inlineStr"><is><t>W leczeniu zarażenia owsikiem skuteczny jest:</t></is></c><c r="F143" s="2" t="inlineStr"><is><t>mebendazol</t></is></c><c r="G143" s="2" t="inlineStr"><is><t>albendazol</t></is></c><c r="H143" s="2" t="inlineStr"><is><t>pyrantel</t></is></c><c r="I143" s="2" t="inlineStr" /><c r="J143" s="2" t="inlineStr" /><c r="K143" s="2" t="inlineStr"><is><t>tynidazol</t></is></c><c r="L143" s="2" t="inlineStr" /><c r="M143" s="2" t="inlineStr" /><c r="N143" s="2" t="inlineStr" /><c r="O143" s="2" t="inlineStr" /><c r="P143" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q143" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="144"><c r="A144" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B144" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C144" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D144" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E144" s="2" t="inlineStr"><is><t>Cytomegalię u osób z niedoborami odporności należy leczyć stosując:</t></is></c><c r="F144" s="2" t="inlineStr"><is><t>gancyklowir</t></is></c><c r="G144" s="2" t="inlineStr" /><c r="H144" s="2" t="inlineStr" /><c r="I144" s="2" t="inlineStr" /><c r="J144" s="2" t="inlineStr" /><c r="K144" s="2" t="inlineStr"><is><t>zanamiwir</t></is></c><c r="L144" s="2" t="inlineStr"><is><t>acyklowir</t></is></c><c r="M144" s="2" t="inlineStr"><is><t>oseltamiwir</t></is></c><c r="N144" s="2" t="inlineStr" /><c r="O144" s="2" t="inlineStr" /><c r="P144" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q144" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="145"><c r="A145" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B145" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C145" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D145" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E145" s="2" t="inlineStr"><is><t>W terapii POChP u osób o wysokim ryzyku zaostrzeń i dużym nasileniu objawów (grupa</t></is></c><c r="F145" s="2" t="inlineStr"><is><t>bromek tiotropium z formoterolem i cyklezonidem</t></is></c><c r="G145" s="2" t="inlineStr"><is><t>budezonid z formoterolem</t></is></c><c r="H145" s="2" t="inlineStr"><is><t>bromek aklidynium z salmeterolem i flutikazonem</t></is></c><c r="I145" s="2" t="inlineStr"><is><t>bromek glikopironium z roflumilastem</t></is></c><c r="J145" s="2" t="inlineStr" /><c r="K145" s="2" t="inlineStr"><is><t>można zastosować:</t></is></c><c r="L145" s="2" t="inlineStr" /><c r="M145" s="2" t="inlineStr" /><c r="N145" s="2" t="inlineStr" /><c r="O145" s="2" t="inlineStr" /><c r="P145" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q145" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="146"><c r="A146" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B146" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C146" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D146" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E146" s="2" t="inlineStr"><is><t>Wskaż prawidłowe twierdzenie dotyczące farmakoterapii astmy oskrzelowej :</t></is></c><c r="F146" s="2" t="inlineStr"><is><t>wziewne glikokortykosteroidy zmniejszają częstość/liczbę hospitalizacji i umieralność z powodu astmy</t></is></c><c r="G146" s="2" t="inlineStr"><is><t>długodziałające wziewne betaadrenomimetyki w monoterapii mogą zwiększać ryzyko zgonu z powodu astmy</t></is></c><c r="H146" s="2" t="inlineStr"><is><t>kromony mogą być skuteczne u chorych ze skurczem oskrzeli wywoływanym przez wysiłek fizyczny</t></is></c><c r="I146" s="2" t="inlineStr" /><c r="J146" s="2" t="inlineStr" /><c r="K146" s="2" t="inlineStr"><is><t>leki przeciwleukotrienowe w monoterapii są bardziej skuteczne od wziewnych glikokortykosteroidów w małych dawkach</t></is></c><c r="L146" s="2" t="inlineStr" /><c r="M146" s="2" t="inlineStr" /><c r="N146" s="2" t="inlineStr" /><c r="O146" s="2" t="inlineStr" /><c r="P146" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q146" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="147"><c r="A147" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B147" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C147" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D147" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E147" s="2" t="inlineStr"><is><t>W leczeniu wodobrzusza w przebiegu marskości wątroby wskazane jest stosowanie:</t></is></c><c r="F147" s="2" t="inlineStr"><is><t>furosemidu</t></is></c><c r="G147" s="2" t="inlineStr"><is><t>spironolaktonu</t></is></c><c r="H147" s="2" t="inlineStr"><is><t>karwedilolu</t></is></c><c r="I147" s="2" t="inlineStr" /><c r="J147" s="2" t="inlineStr" /><c r="K147" s="2" t="inlineStr"><is><t>ramiprylu</t></is></c><c r="L147" s="2" t="inlineStr" /><c r="M147" s="2" t="inlineStr" /><c r="N147" s="2" t="inlineStr" /><c r="O147" s="2" t="inlineStr" /><c r="P147" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q147" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="148"><c r="A148" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B148" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C148" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D148" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E148" s="2" t="inlineStr"><is><t>W leczeniu dny moczanowej należy:</t></is></c><c r="F148" s="2" t="inlineStr"><is><t>stosować dietę z ograniczeniem podaży mięs, podrobów i fruktozy</t></is></c><c r="G148" s="2" t="inlineStr"><is><t>objawowo stosować leki z grupy NLPZ</t></is></c><c r="H148" s="2" t="inlineStr" /><c r="I148" s="2" t="inlineStr" /><c r="J148" s="2" t="inlineStr" /><c r="K148" s="2" t="inlineStr"><is><t>podać jak najszybciej allopurynol przy podejrzeniu ostrego napadu</t></is></c><c r="L148" s="2" t="inlineStr"><is><t>w każdym przypadku bezobjawowej hiperurykemii stosować kolchicynę</t></is></c><c r="M148" s="2" t="inlineStr" /><c r="N148" s="2" t="inlineStr" /><c r="O148" s="2" t="inlineStr" /><c r="P148" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q148" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="149"><c r="A149" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B149" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C149" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D149" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E149" s="2" t="inlineStr"><is><t>Zotarolimus:</t></is></c><c r="F149" s="2" t="inlineStr"><is><t>jest stosowany w stentach wieńcowych uwalniających lek</t></is></c><c r="G149" s="2" t="inlineStr" /><c r="H149" s="2" t="inlineStr" /><c r="I149" s="2" t="inlineStr" /><c r="J149" s="2" t="inlineStr" /><c r="K149" s="2" t="inlineStr"><is><t>jest rekombinowanym w pełni ludzkim przeciwciałem monoklonalnym</t></is></c><c r="L149" s="2" t="inlineStr"><is><t>nie może być stosowany łącznie z kwasem acetylosalicylowym</t></is></c><c r="M149" s="2" t="inlineStr"><is><t>neutralizuje biologiczną aktywność TNF</t></is></c><c r="N149" s="2" t="inlineStr" /><c r="O149" s="2" t="inlineStr" /><c r="P149" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q149" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="150"><c r="A150" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B150" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C150" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D150" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E150" s="2" t="inlineStr"><is><t>W leczeniu choroby Alzheimera:</t></is></c><c r="F150" s="2" t="inlineStr"><is><t>w zaawansowanych przypadkach wskazane jest włączenie do leczenia antagonisty receptorów NMDA</t></is></c><c r="G150" s="2" t="inlineStr"><is><t>donepezil korzystnie wpływa na globalne zdolności intelektualne w łagodnych stadiach choroby</t></is></c><c r="H150" s="2" t="inlineStr" /><c r="I150" s="2" t="inlineStr" /><c r="J150" s="2" t="inlineStr" /><c r="K150" s="2" t="inlineStr"><is><t>stosuje się leki cholinolityczne</t></is></c><c r="L150" s="2" t="inlineStr"><is><t>istotną rolę odgrywa zastosowanie piracetamu</t></is></c><c r="M150" s="2" t="inlineStr" /><c r="N150" s="2" t="inlineStr" /><c r="O150" s="2" t="inlineStr" /><c r="P150" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q150" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="151"><c r="A151" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B151" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C151" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D151" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E151" s="2" t="inlineStr"><is><t>Przewlekłe stosowanie lorazepamu może spowodować:</t></is></c><c r="F151" s="2" t="inlineStr"><is><t>otępienie</t></is></c><c r="G151" s="2" t="inlineStr"><is><t>tolerancję na jego działanie</t></is></c><c r="H151" s="2" t="inlineStr"><is><t>uzależnienie psychiczne i fizyczne</t></is></c><c r="I151" s="2" t="inlineStr" /><c r="J151" s="2" t="inlineStr" /><c r="K151" s="2" t="inlineStr"><is><t>stan padaczkowy</t></is></c><c r="L151" s="2" t="inlineStr" /><c r="M151" s="2" t="inlineStr" /><c r="N151" s="2" t="inlineStr" /><c r="O151" s="2" t="inlineStr" /><c r="P151" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q151" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="152"><c r="A152" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B152" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C152" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D152" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E152" s="2" t="inlineStr"><is><t>Do leczenia ostrego zamknięcia kąta przesączania (potocznie ataku jaskry) można zastosować:</t></is></c><c r="F152" s="2" t="inlineStr"><is><t>tymolol</t></is></c><c r="G152" s="2" t="inlineStr"><is><t>acetazolamid</t></is></c><c r="H152" s="2" t="inlineStr"><is><t>mannitol</t></is></c><c r="I152" s="2" t="inlineStr" /><c r="J152" s="2" t="inlineStr" /><c r="K152" s="2" t="inlineStr"><is><t>zydowudynę</t></is></c><c r="L152" s="2" t="inlineStr" /><c r="M152" s="2" t="inlineStr" /><c r="N152" s="2" t="inlineStr" /><c r="O152" s="2" t="inlineStr" /><c r="P152" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q152" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="153"><c r="A153" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B153" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C153" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D153" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E153" s="2" t="inlineStr"><is><t>W leczeniu stanu padaczkowego:</t></is></c><c r="F153" s="2" t="inlineStr"><is><t>lekiem pierwszego rzutu jest diazepam i.v</t></is></c><c r="G153" s="2" t="inlineStr"><is><t>w przypadku postaci opornej na leczenie można zastosować wlew dożylny midazolamu</t></is></c><c r="H153" s="2" t="inlineStr" /><c r="I153" s="2" t="inlineStr" /><c r="J153" s="2" t="inlineStr" /><c r="K153" s="2" t="inlineStr"><is><t>nie powinno się stosować fenytoiny we wlewie dożylnym</t></is></c><c r="L153" s="2" t="inlineStr"><is><t>należy stosować duże dawki steroidów i.v</t></is></c><c r="M153" s="2" t="inlineStr" /><c r="N153" s="2" t="inlineStr" /><c r="O153" s="2" t="inlineStr" /><c r="P153" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q153" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="154"><c r="A154" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B154" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C154" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D154" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E154" s="2" t="inlineStr"><is><t>Charakterystyka Produktu Leczniczego (ChPL) zawiera informacje o:</t></is></c><c r="F154" s="2" t="inlineStr"><is><t>specjalnych środkach ostrożności podczas przechowywania produktu leczniczego</t></is></c><c r="G154" s="2" t="inlineStr"><is><t>właściwościach farmakokinetycznych leku</t></is></c><c r="H154" s="2" t="inlineStr"><is><t>dacie wydania pierwszego pozwolenia na dopuszczenie do obrotu</t></is></c><c r="I154" s="2" t="inlineStr" /><c r="J154" s="2" t="inlineStr" /><c r="K154" s="2" t="inlineStr"><is><t>cenie produktu leczniczego</t></is></c><c r="L154" s="2" t="inlineStr" /><c r="M154" s="2" t="inlineStr" /><c r="N154" s="2" t="inlineStr" /><c r="O154" s="2" t="inlineStr" /><c r="P154" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q154" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="155"><c r="A155" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B155" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C155" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D155" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E155" s="2" t="inlineStr"><is><t>Agencja Oceny Technologii Medycznych i Taryfikacji:</t></is></c><c r="F155" s="2" t="inlineStr"><is><t>wycenia procedury medyczne</t></is></c><c r="G155" s="2" t="inlineStr"><is><t>zajmuje stanowisko w sprawie skuteczności i bezpieczeństwa leków</t></is></c><c r="H155" s="2" t="inlineStr"><is><t>rekomenduje leki do refundacji</t></is></c><c r="I155" s="2" t="inlineStr" /><c r="J155" s="2" t="inlineStr" /><c r="K155" s="2" t="inlineStr"><is><t>rejestruje leki</t></is></c><c r="L155" s="2" t="inlineStr" /><c r="M155" s="2" t="inlineStr" /><c r="N155" s="2" t="inlineStr" /><c r="O155" s="2" t="inlineStr" /><c r="P155" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q155" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="156"><c r="A156" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B156" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C156" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D156" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E156" s="2" t="inlineStr"><is><t>W hierarchii badań naukowych:</t></is></c><c r="F156" s="2" t="inlineStr"><is><t>badania kohortowe mają wyższą pozycję niż serie przypadków</t></is></c><c r="G156" s="2" t="inlineStr" /><c r="H156" s="2" t="inlineStr" /><c r="I156" s="2" t="inlineStr" /><c r="J156" s="2" t="inlineStr" /><c r="K156" s="2" t="inlineStr"><is><t>metaanalizy są na tym samym poziomie co randomizowane badania kontrolowane</t></is></c><c r="L156" s="2" t="inlineStr"><is><t>najwyższą pozycję mają randomizowane badania kontrolowane</t></is></c><c r="M156" s="2" t="inlineStr"><is><t>badania kohortowe są na tym samym poziomie co randomizowane badania kliniczne</t></is></c><c r="N156" s="2" t="inlineStr" /><c r="O156" s="2" t="inlineStr" /><c r="P156" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q156" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="157"><c r="A157" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B157" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C157" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D157" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E157" s="2" t="inlineStr"><is><t>Desloratadyna:</t></is></c><c r="F157" s="2" t="inlineStr"><is><t>selektywnie blokuje receptory H1</t></is></c><c r="G157" s="2" t="inlineStr"><is><t>ma zastosowanie w leczeniu przewlekłego alergicznego nieżytu nosa</t></is></c><c r="H157" s="2" t="inlineStr" /><c r="I157" s="2" t="inlineStr" /><c r="J157" s="2" t="inlineStr" /><c r="K157" s="2" t="inlineStr"><is><t>dobrze przenika przez barierę krew- mózg</t></is></c><c r="L157" s="2" t="inlineStr"><is><t>ma znaczące działanie proarytmiczne</t></is></c><c r="M157" s="2" t="inlineStr" /><c r="N157" s="2" t="inlineStr" /><c r="O157" s="2" t="inlineStr" /><c r="P157" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q157" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="158"><c r="A158" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B158" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C158" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D158" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E158" s="2" t="inlineStr"><is><t>Mannitol podany iv. zmniejsza:</t></is></c><c r="F158" s="2" t="inlineStr"><is><t>ciśnienie wewnątrzczaszkowe</t></is></c><c r="G158" s="2" t="inlineStr" /><c r="H158" s="2" t="inlineStr" /><c r="I158" s="2" t="inlineStr" /><c r="J158" s="2" t="inlineStr" /><c r="K158" s="2" t="inlineStr"><is><t>ciśnienie osmotyczne płynu zewnątrzkomórkowego</t></is></c><c r="L158" s="2" t="inlineStr"><is><t>wydalanie sodu i chlorków</t></is></c><c r="M158" s="2" t="inlineStr"><is><t>filtrację nerkową</t></is></c><c r="N158" s="2" t="inlineStr" /><c r="O158" s="2" t="inlineStr" /><c r="P158" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q158" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="159"><c r="A159" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B159" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C159" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D159" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E159" s="2" t="inlineStr"><is><t>Podanie inhibitorów wychwytu zwrotnego serotoniny (SSRI) jest uzasadnione u pacjentów z:</t></is></c><c r="F159" s="2" t="inlineStr"><is><t>lękiem uogólnionym</t></is></c><c r="G159" s="2" t="inlineStr"><is><t>chorobą afektywną dwubiegunową</t></is></c><c r="H159" s="2" t="inlineStr"><is><t>nerwicą natręctw</t></is></c><c r="I159" s="2" t="inlineStr"><is><t>chorobą afektywną jednobiegunową</t></is></c><c r="J159" s="2" t="inlineStr" /><c r="K159" s="2" t="inlineStr" /><c r="L159" s="2" t="inlineStr" /><c r="M159" s="2" t="inlineStr" /><c r="N159" s="2" t="inlineStr" /><c r="O159" s="2" t="inlineStr" /><c r="P159" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q159" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="160"><c r="A160" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B160" s="2" t="inlineStr"><is><t>Struktura chemiczna</t></is></c><c r="C160" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D160" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E160" s="2" t="inlineStr"><is><t>Do wspólnych cech wenlafaksyny i amitryptyliny należy:</t></is></c><c r="F160" s="2" t="inlineStr"><is><t>hamowanie wychwytu zwrotnego serotoniny i noradrenaliny</t></is></c><c r="G160" s="2" t="inlineStr" /><c r="H160" s="2" t="inlineStr" /><c r="I160" s="2" t="inlineStr" /><c r="J160" s="2" t="inlineStr" /><c r="K160" s="2" t="inlineStr"><is><t>trójpierścieniowa budowa chemiczna</t></is></c><c r="L160" s="2" t="inlineStr"><is><t>konieczność znacznych ograniczeń dietetycznych podczas ich stosowania ze względu na ryzyko wystąpienia tzw. zespołu serowego (cheese effect)</t></is></c><c r="M160" s="2" t="inlineStr"><is><t>antagonizm wobec receptorów muskarynowych M1</t></is></c><c r="N160" s="2" t="inlineStr" /><c r="O160" s="2" t="inlineStr" /><c r="P160" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q160" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="161"><c r="A161" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B161" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C161" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D161" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E161" s="2" t="inlineStr"><is><t>Leki, które hamują kompleks kalcyneuryny to:</t></is></c><c r="F161" s="2" t="inlineStr"><is><t>cyklosporyna</t></is></c><c r="G161" s="2" t="inlineStr"><is><t>takrolimus</t></is></c><c r="H161" s="2" t="inlineStr" /><c r="I161" s="2" t="inlineStr" /><c r="J161" s="2" t="inlineStr" /><c r="K161" s="2" t="inlineStr"><is><t>talidomid</t></is></c><c r="L161" s="2" t="inlineStr"><is><t>mykofenolan mofetylu</t></is></c><c r="M161" s="2" t="inlineStr" /><c r="N161" s="2" t="inlineStr" /><c r="O161" s="2" t="inlineStr" /><c r="P161" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q161" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="162"><c r="A162" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B162" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C162" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D162" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E162" s="2" t="inlineStr"><is><t>Lacydypina:</t></is></c><c r="F162" s="2" t="inlineStr"><is><t>zmniejsza obciążenie następcze serca</t></is></c><c r="G162" s="2" t="inlineStr" /><c r="H162" s="2" t="inlineStr" /><c r="I162" s="2" t="inlineStr" /><c r="J162" s="2" t="inlineStr" /><c r="K162" s="2" t="inlineStr"><is><t>ma silne działanie inotropowe ujemne</t></is></c><c r="L162" s="2" t="inlineStr"><is><t>ma działanie dromotropowe ujemne</t></is></c><c r="M162" s="2" t="inlineStr"><is><t>ma działanie chronotropowe dodatnie</t></is></c><c r="N162" s="2" t="inlineStr" /><c r="O162" s="2" t="inlineStr" /><c r="P162" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q162" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="163"><c r="A163" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B163" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C163" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D163" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E163" s="2" t="inlineStr"><is><t>Do donorów tlenku azotu należy:</t></is></c><c r="F163" s="2" t="inlineStr"><is><t>nikorandil</t></is></c><c r="G163" s="2" t="inlineStr"><is><t>molsidomina</t></is></c><c r="H163" s="2" t="inlineStr"><is><t>diazotan izosorbitolu</t></is></c><c r="I163" s="2" t="inlineStr" /><c r="J163" s="2" t="inlineStr" /><c r="K163" s="2" t="inlineStr"><is><t>trimetazydyna</t></is></c><c r="L163" s="2" t="inlineStr" /><c r="M163" s="2" t="inlineStr" /><c r="N163" s="2" t="inlineStr" /><c r="O163" s="2" t="inlineStr" /><c r="P163" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q163" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="164"><c r="A164" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B164" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C164" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D164" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E164" s="2" t="inlineStr"><is><t>Względna dostępność biologiczna leku (biorównoważność) może być określona przez porównanie AUC:</t></is></c><c r="F164" s="2" t="inlineStr"><is><t>leku wzorcowego podanego drogą pozanaczyniową i dożylnie</t></is></c><c r="G164" s="2" t="inlineStr"><is><t>leku wzorcowego i badanego podanych tą samą drogą</t></is></c><c r="H164" s="2" t="inlineStr" /><c r="I164" s="2" t="inlineStr" /><c r="J164" s="2" t="inlineStr" /><c r="K164" s="2" t="inlineStr"><is><t>tylko leków podawanych drogą dożylną</t></is></c><c r="L164" s="2" t="inlineStr"><is><t>leku badanego podanego drogą pozanaczyniową i wzorcowego podanego dożylnie</t></is></c><c r="M164" s="2" t="inlineStr" /><c r="N164" s="2" t="inlineStr" /><c r="O164" s="2" t="inlineStr" /><c r="P164" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q164" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="165"><c r="A165" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B165" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C165" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D165" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E165" s="2" t="inlineStr"><is><t>Benzodiazepiną, która nie podlega metabolizmowi wątrobowemu jest:</t></is></c><c r="F165" s="2" t="inlineStr"><is><t>lorazepam</t></is></c><c r="G165" s="2" t="inlineStr"><is><t>oksazepam</t></is></c><c r="H165" s="2" t="inlineStr" /><c r="I165" s="2" t="inlineStr" /><c r="J165" s="2" t="inlineStr" /><c r="K165" s="2" t="inlineStr"><is><t>nitrazepam</t></is></c><c r="L165" s="2" t="inlineStr"><is><t>diazepam</t></is></c><c r="M165" s="2" t="inlineStr" /><c r="N165" s="2" t="inlineStr" /><c r="O165" s="2" t="inlineStr" /><c r="P165" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q165" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="166"><c r="A166" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B166" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C166" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D166" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E166" s="2" t="inlineStr"><is><t>Objętość dystrybucji ma znaczenie w określeniu wielkości dawki:</t></is></c><c r="F166" s="2" t="inlineStr"><is><t>nasycającej</t></is></c><c r="G166" s="2" t="inlineStr"><is><t>podtrzymującej</t></is></c><c r="H166" s="2" t="inlineStr" /><c r="I166" s="2" t="inlineStr" /><c r="J166" s="2" t="inlineStr" /><c r="K166" s="2" t="inlineStr"><is><t>śmiertelnej</t></is></c><c r="L166" s="2" t="inlineStr"><is><t>toksycznej</t></is></c><c r="M166" s="2" t="inlineStr" /><c r="N166" s="2" t="inlineStr" /><c r="O166" s="2" t="inlineStr" /><c r="P166" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q166" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="167"><c r="A167" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B167" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C167" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D167" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E167" s="2" t="inlineStr"><is><t>Do obniżenia gorączki u 2-letniego dziecka można zastosować:</t></is></c><c r="F167" s="2" t="inlineStr"><is><t>czopek doodbytniczy zawierający paracetamol</t></is></c><c r="G167" s="2" t="inlineStr"><is><t>zawiesinę doustną zawierającą ibuprofen</t></is></c><c r="H167" s="2" t="inlineStr" /><c r="I167" s="2" t="inlineStr" /><c r="J167" s="2" t="inlineStr" /><c r="K167" s="2" t="inlineStr"><is><t>tabletki o natychmiastowym uwalnianiu w jamie ustnej zawierające kwas acetylosalicylowy</t></is></c><c r="L167" s="2" t="inlineStr"><is><t>wstrzyknięcie domięśniowe metamizolu</t></is></c><c r="M167" s="2" t="inlineStr" /><c r="N167" s="2" t="inlineStr" /><c r="O167" s="2" t="inlineStr" /><c r="P167" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q167" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="168"><c r="A168" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B168" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C168" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D168" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E168" s="2" t="inlineStr"><is><t>Typowe leki podlegające monitorowaniu stężeń to:</t></is></c><c r="F168" s="2" t="inlineStr"><is><t>cyklosporyna</t></is></c><c r="G168" s="2" t="inlineStr"><is><t>fenytoina</t></is></c><c r="H168" s="2" t="inlineStr"><is><t>gentamycyna</t></is></c><c r="I168" s="2" t="inlineStr"><is><t>Digoksyna</t></is></c><c r="J168" s="2" t="inlineStr" /><c r="K168" s="2" t="inlineStr" /><c r="L168" s="2" t="inlineStr" /><c r="M168" s="2" t="inlineStr" /><c r="N168" s="2" t="inlineStr" /><c r="O168" s="2" t="inlineStr" /><c r="P168" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q168" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="169"><c r="A169" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B169" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C169" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D169" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E169" s="2" t="inlineStr"><is><t>Izoniazyd:</t></is></c><c r="F169" s="2" t="inlineStr"><is><t>działa bakteriobójczo na prątki szybko namnażające się</t></is></c><c r="G169" s="2" t="inlineStr" /><c r="H169" s="2" t="inlineStr" /><c r="I169" s="2" t="inlineStr" /><c r="J169" s="2" t="inlineStr" /><c r="K169" s="2" t="inlineStr"><is><t>nie powinien być stosowany przez kobiety w ciąży</t></is></c><c r="L169" s="2" t="inlineStr"><is><t>nie jest stosowany w leczeniu gruźlicy pozapłucnej</t></is></c><c r="M169" s="2" t="inlineStr"><is><t>może spowodować neuropatię obwodową</t></is></c><c r="N169" s="2" t="inlineStr" /><c r="O169" s="2" t="inlineStr" /><c r="P169" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q169" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="170"><c r="A170" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B170" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C170" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D170" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E170" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-działanie niepożądne:</t></is></c><c r="F170" s="2" t="inlineStr"><is><t>zolpidem – niepamięć następcza</t></is></c><c r="G170" s="2" t="inlineStr"><is><t>rotygotyna – nudności i wymioty</t></is></c><c r="H170" s="2" t="inlineStr"><is><t>alprazolam - senność</t></is></c><c r="I170" s="2" t="inlineStr"><is><t>fluoksetyna – zaburzenia libido i funkcji seksualnych</t></is></c><c r="J170" s="2" t="inlineStr" /><c r="K170" s="2" t="inlineStr" /><c r="L170" s="2" t="inlineStr" /><c r="M170" s="2" t="inlineStr" /><c r="N170" s="2" t="inlineStr" /><c r="O170" s="2" t="inlineStr" /><c r="P170" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q170" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="171"><c r="A171" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B171" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C171" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D171" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E171" s="2" t="inlineStr"><is><t>Do leczenia zaburzeń psychotycznych z nasilonymi objawami negatywnymi należy wybrać:</t></is></c><c r="F171" s="2" t="inlineStr"><is><t>amisulpiryd</t></is></c><c r="G171" s="2" t="inlineStr"><is><t>olanzapinę</t></is></c><c r="H171" s="2" t="inlineStr" /><c r="I171" s="2" t="inlineStr" /><c r="J171" s="2" t="inlineStr" /><c r="K171" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="L171" s="2" t="inlineStr"><is><t>chlorpromazynę</t></is></c><c r="M171" s="2" t="inlineStr" /><c r="N171" s="2" t="inlineStr" /><c r="O171" s="2" t="inlineStr" /><c r="P171" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q171" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="172"><c r="A172" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B172" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C172" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D172" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E172" s="2" t="inlineStr"><is><t>Działanie przeciwwymiotne metoklopramidu wynika z blokady receptorów:</t></is></c><c r="F172" s="2" t="inlineStr"><is><t>dopaminowych (D2)</t></is></c><c r="G172" s="2" t="inlineStr"><is><t>serotoninowych (5-HT3)</t></is></c><c r="H172" s="2" t="inlineStr" /><c r="I172" s="2" t="inlineStr" /><c r="J172" s="2" t="inlineStr" /><c r="K172" s="2" t="inlineStr"><is><t>neurokininowych (NK1)</t></is></c><c r="L172" s="2" t="inlineStr"><is><t>kannabinoidowych (CB1)</t></is></c><c r="M172" s="2" t="inlineStr" /><c r="N172" s="2" t="inlineStr" /><c r="O172" s="2" t="inlineStr" /><c r="P172" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q172" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="173"><c r="A173" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B173" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C173" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D173" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E173" s="2" t="inlineStr"><is><t>Rozszerzenie źrenic, suchość w ustach, osłabienie lub porażenie perystaltyki jelit obserwowane jest w przebiegu zatrucia:</t></is></c><c r="F173" s="2" t="inlineStr"><is><t>amitryptyliną</t></is></c><c r="G173" s="2" t="inlineStr" /><c r="H173" s="2" t="inlineStr" /><c r="I173" s="2" t="inlineStr" /><c r="J173" s="2" t="inlineStr" /><c r="K173" s="2" t="inlineStr"><is><t>escitalopramem</t></is></c><c r="L173" s="2" t="inlineStr"><is><t>pestycydami fosforoorganicznymi</t></is></c><c r="M173" s="2" t="inlineStr"><is><t>glikozydami naparstnicy</t></is></c><c r="N173" s="2" t="inlineStr" /><c r="O173" s="2" t="inlineStr" /><c r="P173" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q173" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="174"><c r="A174" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B174" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C174" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D174" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E174" s="2" t="inlineStr"><is><t>U 70-letniego mężczyzny z przewlekłą niewydolnością żylną wspomagająco do kompresjoterapii należy zastosować:</t></is></c><c r="F174" s="2" t="inlineStr"><is><t>mikronizowaną diosminę + hesperydynę</t></is></c><c r="G174" s="2" t="inlineStr" /><c r="H174" s="2" t="inlineStr" /><c r="I174" s="2" t="inlineStr" /><c r="J174" s="2" t="inlineStr" /><c r="K174" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy w dawce antyagregacyjnej</t></is></c><c r="L174" s="2" t="inlineStr"><is><t>enoksaparynę w dawce profilaktycznej</t></is></c><c r="M174" s="2" t="inlineStr"><is><t>furosemid w dawce leczniczej</t></is></c><c r="N174" s="2" t="inlineStr" /><c r="O174" s="2" t="inlineStr" /><c r="P174" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q174" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="175"><c r="A175" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B175" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C175" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D175" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E175" s="2" t="inlineStr"><is><t>Nie powinno się zwalniać pasażu jelitowego w przebiegu:</t></is></c><c r="F175" s="2" t="inlineStr"><is><t>zatrucia z objawami ogólnymi</t></is></c><c r="G175" s="2" t="inlineStr"><is><t>biegunki z krwią w stolcu i gorączką</t></is></c><c r="H175" s="2" t="inlineStr"><is><t>ostrej biegunki o niewielkim nasileniu</t></is></c><c r="I175" s="2" t="inlineStr" /><c r="J175" s="2" t="inlineStr" /><c r="K175" s="2" t="inlineStr"><is><t>przewlekłej biegunki związanej z chorobą zapalną jelit</t></is></c><c r="L175" s="2" t="inlineStr" /><c r="M175" s="2" t="inlineStr" /><c r="N175" s="2" t="inlineStr" /><c r="O175" s="2" t="inlineStr" /><c r="P175" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q175" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="176"><c r="A176" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B176" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C176" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D176" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E176" s="2" t="inlineStr"><is><t>Związki bizmutu:</t></is></c><c r="F176" s="2" t="inlineStr"><is><t>tworzą nierozpuszczalne kompleksy z białkami wysiękowymi na powierzchni owrzodzenia, działając osłaniająco wobec kwasu solnego i pepsyny na uszkodzoną błonę śluzową żołądka i dwunastnicy</t></is></c><c r="G176" s="2" t="inlineStr"><is><t>wchłaniają się z przewodu pokarmowego</t></is></c><c r="H176" s="2" t="inlineStr"><is><t>bezpośrednio niszczą komórki Helicobacter pylori</t></is></c><c r="I176" s="2" t="inlineStr"><is><t>mogą spowodować czarne zabarwienie języka i kału</t></is></c><c r="J176" s="2" t="inlineStr" /><c r="K176" s="2" t="inlineStr" /><c r="L176" s="2" t="inlineStr" /><c r="M176" s="2" t="inlineStr" /><c r="N176" s="2" t="inlineStr" /><c r="O176" s="2" t="inlineStr" /><c r="P176" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q176" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="177"><c r="A177" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B177" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C177" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D177" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E177" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek – wskazanie - dawka:</t></is></c><c r="F177" s="2" t="inlineStr"><is><t>dobutamina – diagnostyka niedokrwienia mięśnia serca –wlew 2-20 mcg/kg m.c./min</t></is></c><c r="G177" s="2" t="inlineStr"><is><t>adrenalina – resuscytacja krążeniowo-oddechowa– w dawkach frakcjonowanych i.v. po 1 mg w rozcieńczeniu w 10 ml 0,9% NaCl</t></is></c><c r="H177" s="2" t="inlineStr" /><c r="I177" s="2" t="inlineStr" /><c r="J177" s="2" t="inlineStr" /><c r="K177" s="2" t="inlineStr"><is><t>noradrenalina – ciężka hipotonia – wlew 2-10 mcg/kg m.c./min</t></is></c><c r="L177" s="2" t="inlineStr"><is><t>dopamina – ostra niewydolność mięśnia sercowego – wlew 1-3 mcg/kg m.c./min</t></is></c><c r="M177" s="2" t="inlineStr" /><c r="N177" s="2" t="inlineStr" /><c r="O177" s="2" t="inlineStr" /><c r="P177" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q177" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="178"><c r="A178" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B178" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C178" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D178" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E178" s="2" t="inlineStr"><is><t>Skala HAS-BLED określa ryzyko krwawienia u osób z migotaniem przedsionków stosujących leczenie przeciwkrzepliwe na podstawie oceny:</t></is></c><c r="F178" s="2" t="inlineStr"><is><t>wartości skurczowego ciśnienia tętniczego</t></is></c><c r="G178" s="2" t="inlineStr"><is><t>czynności wątroby</t></is></c><c r="H178" s="2" t="inlineStr"><is><t>stężenia kreatyniny</t></is></c><c r="I178" s="2" t="inlineStr" /><c r="J178" s="2" t="inlineStr" /><c r="K178" s="2" t="inlineStr"><is><t>glikemii</t></is></c><c r="L178" s="2" t="inlineStr" /><c r="M178" s="2" t="inlineStr" /><c r="N178" s="2" t="inlineStr" /><c r="O178" s="2" t="inlineStr" /><c r="P178" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q178" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="179"><c r="A179" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B179" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C179" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D179" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E179" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie substancja uzależniająca - lek stosowany w terapii uzależnienia:</t></is></c><c r="F179" s="2" t="inlineStr"><is><t>heroina - metadon</t></is></c><c r="G179" s="2" t="inlineStr"><is><t>nikotyna – wareniklina</t></is></c><c r="H179" s="2" t="inlineStr"><is><t>alkohol - nalmefen</t></is></c><c r="I179" s="2" t="inlineStr" /><c r="J179" s="2" t="inlineStr" /><c r="K179" s="2" t="inlineStr"><is><t>amfetamina - deferoksamina</t></is></c><c r="L179" s="2" t="inlineStr" /><c r="M179" s="2" t="inlineStr" /><c r="N179" s="2" t="inlineStr" /><c r="O179" s="2" t="inlineStr" /><c r="P179" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q179" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="180"><c r="A180" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B180" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C180" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D180" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E180" s="2" t="inlineStr"><is><t>Peptydy natriuretyczne zwiększają:</t></is></c><c r="F180" s="2" t="inlineStr"><is><t>filtrację kłębuszkową</t></is></c><c r="G180" s="2" t="inlineStr" /><c r="H180" s="2" t="inlineStr" /><c r="I180" s="2" t="inlineStr" /><c r="J180" s="2" t="inlineStr" /><c r="K180" s="2" t="inlineStr"><is><t>wydzielanie aldosteronu</t></is></c><c r="L180" s="2" t="inlineStr"><is><t>glikemię</t></is></c><c r="M180" s="2" t="inlineStr"><is><t>aktywność układu współczulnego</t></is></c><c r="N180" s="2" t="inlineStr" /><c r="O180" s="2" t="inlineStr" /><c r="P180" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q180" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="181"><c r="A181" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B181" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C181" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D181" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E181" s="2" t="inlineStr"><is><t>Pacjent z objawową bradykardią = 35 uderzeń/min jest leczony poniższym zestawem leków. Który z nich należy niezwłocznie odstawić?</t></is></c><c r="F181" s="2" t="inlineStr"><is><t>digoksynę</t></is></c><c r="G181" s="2" t="inlineStr"><is><t>amiodaron</t></is></c><c r="H181" s="2" t="inlineStr"><is><t>betaksolol</t></is></c><c r="I181" s="2" t="inlineStr" /><c r="J181" s="2" t="inlineStr" /><c r="K181" s="2" t="inlineStr"><is><t>losartan</t></is></c><c r="L181" s="2" t="inlineStr" /><c r="M181" s="2" t="inlineStr" /><c r="N181" s="2" t="inlineStr" /><c r="O181" s="2" t="inlineStr" /><c r="P181" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q181" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="182"><c r="A182" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B182" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C182" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D182" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E182" s="2" t="inlineStr"><is><t>Irbesartan zwiększa w osoczu stężenie:</t></is></c><c r="F182" s="2" t="inlineStr"><is><t>reniny</t></is></c><c r="G182" s="2" t="inlineStr"><is><t>potasu</t></is></c><c r="H182" s="2" t="inlineStr" /><c r="I182" s="2" t="inlineStr" /><c r="J182" s="2" t="inlineStr" /><c r="K182" s="2" t="inlineStr"><is><t>bradykininy</t></is></c><c r="L182" s="2" t="inlineStr"><is><t>aldosteronu</t></is></c><c r="M182" s="2" t="inlineStr" /><c r="N182" s="2" t="inlineStr" /><c r="O182" s="2" t="inlineStr" /><c r="P182" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q182" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="183"><c r="A183" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B183" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C183" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D183" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E183" s="2" t="inlineStr"><is><t>70-letnia kobieta od miesiąca po wypisie ze szpitala otrzymuje kwas acetylosalicylowy + klopidogrel. Na tej podstawie można sądzić, że przebyła:</t></is></c><c r="F183" s="2" t="inlineStr"><is><t>angioplastykę wieńcową z wszczepieniem stentu</t></is></c><c r="G183" s="2" t="inlineStr"><is><t>zawał serca</t></is></c><c r="H183" s="2" t="inlineStr" /><c r="I183" s="2" t="inlineStr" /><c r="J183" s="2" t="inlineStr" /><c r="K183" s="2" t="inlineStr"><is><t>udar niedokrwienny mózgu</t></is></c><c r="L183" s="2" t="inlineStr"><is><t>zatorowość płucną niewysokiego ryzyka</t></is></c><c r="M183" s="2" t="inlineStr" /><c r="N183" s="2" t="inlineStr" /><c r="O183" s="2" t="inlineStr" /><c r="P183" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q183" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="184"><c r="A184" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B184" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C184" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D184" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E184" s="2" t="inlineStr"><is><t>59-letni mężczyzna z pozawałową niewydolnością serca (EF ok. 30%), z implantowanym ICD (kardiowerterem defibrylatorem) w prewencji pierwotnej NZK, z eGFR = 95%, z bólami pleców na skutek wielopoziomowej dyskopatii jest leczony: ramiprylem, karwedilolem, eplerenonem, indapamidem, preparatami chlorku potasu, magnezu z witaminą B6 i węglanu wapnia oraz paracetamolem i ketoprofenem. Które stwierdzenie jest prawdziwe?</t></is></c><c r="F184" s="2" t="inlineStr"><is><t>opisana terapia stwarza zagrożenie hiperkaliemią, co trzeba monitorować</t></is></c><c r="G184" s="2" t="inlineStr"><is><t>należy odstawić ketoprofen, bo może on osłabiać działanie leków w niewydolności serca</t></is></c><c r="H184" s="2" t="inlineStr" /><c r="I184" s="2" t="inlineStr" /><c r="J184" s="2" t="inlineStr" /><c r="K184" s="2" t="inlineStr"><is><t>ze względu na lepszą kontrolę choroby zamiast ramiprylu należy podać walsartan</t></is></c><c r="L184" s="2" t="inlineStr"><is><t>indapamid jako lek potencjalnie nieskuteczny powinien zostać zastąpiony torasemidem</t></is></c><c r="M184" s="2" t="inlineStr" /><c r="N184" s="2" t="inlineStr" /><c r="O184" s="2" t="inlineStr" /><c r="P184" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q184" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="185"><c r="A185" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B185" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C185" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D185" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E185" s="2" t="inlineStr"><is><t>Wartości ciśnienia tętniczego może zwiększyć stosowanie:</t></is></c><c r="F185" s="2" t="inlineStr"><is><t>piroksykamu</t></is></c><c r="G185" s="2" t="inlineStr"><is><t>prednizonu</t></is></c><c r="H185" s="2" t="inlineStr" /><c r="I185" s="2" t="inlineStr" /><c r="J185" s="2" t="inlineStr" /><c r="K185" s="2" t="inlineStr"><is><t>eplerenonu</t></is></c><c r="L185" s="2" t="inlineStr"><is><t>morfiny</t></is></c><c r="M185" s="2" t="inlineStr" /><c r="N185" s="2" t="inlineStr" /><c r="O185" s="2" t="inlineStr" /><c r="P185" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q185" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="186"><c r="A186" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B186" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C186" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D186" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E186" s="2" t="inlineStr"><is><t>Kwas ibandronowy:</t></is></c><c r="F186" s="2" t="inlineStr"><is><t>z dużym powinowactwem wiąże się ze zmineralizowaną kością</t></is></c><c r="G186" s="2" t="inlineStr"><is><t>zmniejsza ryzyko złamania kręgów kręgosłupa u kobiet po menopauzie</t></is></c><c r="H186" s="2" t="inlineStr"><is><t>hamuje aktywację osteoklastów</t></is></c><c r="I186" s="2" t="inlineStr"><is><t>może spowodować martwicę szczęki</t></is></c><c r="J186" s="2" t="inlineStr" /><c r="K186" s="2" t="inlineStr" /><c r="L186" s="2" t="inlineStr" /><c r="M186" s="2" t="inlineStr" /><c r="N186" s="2" t="inlineStr" /><c r="O186" s="2" t="inlineStr" /><c r="P186" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q186" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="187"><c r="A187" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B187" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C187" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D187" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E187" s="2" t="inlineStr"><is><t>Dodatkowe zmniejszenie stężenia cholesterolu LDL w surowicy można osiągnąć przez dodanie do statyn:</t></is></c><c r="F187" s="2" t="inlineStr"><is><t>kolesewelamu</t></is></c><c r="G187" s="2" t="inlineStr"><is><t>ewolokumabu</t></is></c><c r="H187" s="2" t="inlineStr"><is><t>ezetymibu</t></is></c><c r="I187" s="2" t="inlineStr" /><c r="J187" s="2" t="inlineStr" /><c r="K187" s="2" t="inlineStr"><is><t>PUFA – wielonienasyconych kwasów tłuszczowych</t></is></c><c r="L187" s="2" t="inlineStr" /><c r="M187" s="2" t="inlineStr" /><c r="N187" s="2" t="inlineStr" /><c r="O187" s="2" t="inlineStr" /><c r="P187" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q187" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="188"><c r="A188" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B188" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C188" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D188" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E188" s="2" t="inlineStr"><is><t>Które stwierdzenie jest prawdziwe?</t></is></c><c r="F188" s="2" t="inlineStr"><is><t>takrolimus i ewerolimus tworzą kompleks z immunofiliną FKBP</t></is></c><c r="G188" s="2" t="inlineStr"><is><t>takrolimus i ewerolimus należą do leków o wąskim indeksie (wskaźniku) terapeutycznym</t></is></c><c r="H188" s="2" t="inlineStr" /><c r="I188" s="2" t="inlineStr" /><c r="J188" s="2" t="inlineStr" /><c r="K188" s="2" t="inlineStr"><is><t>takrolimus i ewerolimus mają ten sam mechanizm działania</t></is></c><c r="L188" s="2" t="inlineStr"><is><t>takrolimus i ewerolimus działają przeciwnowotorowo</t></is></c><c r="M188" s="2" t="inlineStr" /><c r="N188" s="2" t="inlineStr" /><c r="O188" s="2" t="inlineStr" /><c r="P188" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q188" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="189"><c r="A189" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B189" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C189" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D189" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E189" s="2" t="inlineStr"><is><t>Fibraty (pochodne kwasu fibrynowego):</t></is></c><c r="F189" s="2" t="inlineStr"><is><t>hamują uwalnianie frakcji lipidowej VLDL z wątroby</t></is></c><c r="G189" s="2" t="inlineStr"><is><t>nasilają aktywność lipazy lipoproteinowej</t></is></c><c r="H189" s="2" t="inlineStr" /><c r="I189" s="2" t="inlineStr" /><c r="J189" s="2" t="inlineStr" /><c r="K189" s="2" t="inlineStr"><is><t>hamują wchłanianie tłuszczów złożonych z przewodu pokarmowego</t></is></c><c r="L189" s="2" t="inlineStr"><is><t>zmniejszają stężenie frakcji HDL poprzez spadek syntezy Apo-A1 i Apo-AII</t></is></c><c r="M189" s="2" t="inlineStr" /><c r="N189" s="2" t="inlineStr" /><c r="O189" s="2" t="inlineStr" /><c r="P189" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q189" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="190"><c r="A190" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B190" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C190" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D190" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E190" s="2" t="inlineStr"><is><t>U chorych ze zdekompensowaną obukomorową niewydolnością serca:</t></is></c><c r="F190" s="2" t="inlineStr"><is><t>znacznie opóźnione jest wchłanianie leków z przewodu pokarmowego</t></is></c><c r="G190" s="2" t="inlineStr"><is><t>leki hydrofilne dystrybuują się do płynu obrzękowego, co dodatkowo negatywnie wpływa na ich dystrybucję do narządów docelowych</t></is></c><c r="H190" s="2" t="inlineStr"><is><t>zmniejsza się klirens wątrobowy wszystkich leków metabolizowanych w wątrobie niezależnie od stopnia ich ekstrakcji wątrobowej</t></is></c><c r="I190" s="2" t="inlineStr" /><c r="J190" s="2" t="inlineStr" /><c r="K190" s="2" t="inlineStr"><is><t>stosunkowo mało zmniejsza się klirens nerkowy leków</t></is></c><c r="L190" s="2" t="inlineStr" /><c r="M190" s="2" t="inlineStr" /><c r="N190" s="2" t="inlineStr" /><c r="O190" s="2" t="inlineStr" /><c r="P190" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q190" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="191"><c r="A191" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B191" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C191" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D191" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E191" s="2" t="inlineStr"><is><t>Interakcją farmakodynamiczną jest:</t></is></c><c r="F191" s="2" t="inlineStr"><is><t>nasilenie depresji OUN po skojarzeniu opioidów z etanolem</t></is></c><c r="G191" s="2" t="inlineStr" /><c r="H191" s="2" t="inlineStr" /><c r="I191" s="2" t="inlineStr" /><c r="J191" s="2" t="inlineStr" /><c r="K191" s="2" t="inlineStr"><is><t>hamowanie wchłaniania z przewodu pokarmowego leków podawanych jednocześnie</t></is></c><c r="L191" s="2" t="inlineStr"><is><t>wytrącenie się osadu po zmieszaniu dwóch leków w jednym roztworze do wstrzyknięcia</t></is></c><c r="M191" s="2" t="inlineStr"><is><t>zwiększenie metabolizmu leków podawanych jednocześnie</t></is></c><c r="N191" s="2" t="inlineStr" /><c r="O191" s="2" t="inlineStr" /><c r="P191" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q191" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="192"><c r="A192" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B192" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C192" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D192" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E192" s="2" t="inlineStr"><is><t>Kwasicę metaboliczną mogą powodować:</t></is></c><c r="F192" s="2" t="inlineStr"><is><t>metformina</t></is></c><c r="G192" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="H192" s="2" t="inlineStr" /><c r="I192" s="2" t="inlineStr" /><c r="J192" s="2" t="inlineStr" /><c r="K192" s="2" t="inlineStr"><is><t>diuretyki pętlowe</t></is></c><c r="L192" s="2" t="inlineStr"><is><t>etanol</t></is></c><c r="M192" s="2" t="inlineStr" /><c r="N192" s="2" t="inlineStr" /><c r="O192" s="2" t="inlineStr" /><c r="P192" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q192" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="193"><c r="A193" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B193" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C193" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D193" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E193" s="2" t="inlineStr"><is><t>Klindamycyna:</t></is></c><c r="F193" s="2" t="inlineStr"><is><t>jest aktywna wobec beztlenowców</t></is></c><c r="G193" s="2" t="inlineStr" /><c r="H193" s="2" t="inlineStr" /><c r="I193" s="2" t="inlineStr" /><c r="J193" s="2" t="inlineStr" /><c r="K193" s="2" t="inlineStr"><is><t>dobrze przenika do płynu mózgowo-rdzeniowego</t></is></c><c r="L193" s="2" t="inlineStr"><is><t>słabo selekcjonuje szczepy Clostridium difficile w jelicie</t></is></c><c r="M193" s="2" t="inlineStr"><is><t>stosowana jest jako lek z wyboru w nierzeżączkowym zapaleniu cewki moczowej</t></is></c><c r="N193" s="2" t="inlineStr" /><c r="O193" s="2" t="inlineStr" /><c r="P193" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q193" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="194"><c r="A194" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B194" s="2" t="inlineStr"><is><t>Struktura chemiczna</t></is></c><c r="C194" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D194" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E194" s="2" t="inlineStr"><is><t>Pierścień beta-laktamowy znajduje się w cząsteczce:</t></is></c><c r="F194" s="2" t="inlineStr"><is><t>kloksacyliny</t></is></c><c r="G194" s="2" t="inlineStr"><is><t>ceftazydymu</t></is></c><c r="H194" s="2" t="inlineStr"><is><t>meropenemu</t></is></c><c r="I194" s="2" t="inlineStr" /><c r="J194" s="2" t="inlineStr" /><c r="K194" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="L194" s="2" t="inlineStr" /><c r="M194" s="2" t="inlineStr" /><c r="N194" s="2" t="inlineStr" /><c r="O194" s="2" t="inlineStr" /><c r="P194" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q194" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="195"><c r="A195" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B195" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C195" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D195" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E195" s="2" t="inlineStr"><is><t>W celu zwiększenia bezpieczeństwa leczenia amikacyną mężczyzny z powikłanym zakażeniem układu moczowego należy:</t></is></c><c r="F195" s="2" t="inlineStr"><is><t>podawać dawkę dobową w pojedynczym wlewie dożylnym</t></is></c><c r="G195" s="2" t="inlineStr"><is><t>monitorować okresowo stężenie antybiotyku we krwi przed podaniem kolejnej dawki leku</t></is></c><c r="H195" s="2" t="inlineStr"><is><t>monitorować stężenie kreatyniny w surowicy</t></is></c><c r="I195" s="2" t="inlineStr" /><c r="J195" s="2" t="inlineStr" /><c r="K195" s="2" t="inlineStr"><is><t>kontrolować co kilka dni stężenie TSH w surowicy</t></is></c><c r="L195" s="2" t="inlineStr" /><c r="M195" s="2" t="inlineStr" /><c r="N195" s="2" t="inlineStr" /><c r="O195" s="2" t="inlineStr" /><c r="P195" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q195" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="196"><c r="A196" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B196" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C196" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D196" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E196" s="2" t="inlineStr"><is><t>W leczeniu pacjentki z niepowikłanym zapaleniem pęcherza moczowego można zastosować:</t></is></c><c r="F196" s="2" t="inlineStr"><is><t>amoksycylinę z inhibitorem beta-laktamazy</t></is></c><c r="G196" s="2" t="inlineStr"><is><t>fosfomycynę</t></is></c><c r="H196" s="2" t="inlineStr"><is><t>cyprofloksacynę</t></is></c><c r="I196" s="2" t="inlineStr"><is><t>furazydynę</t></is></c><c r="J196" s="2" t="inlineStr" /><c r="K196" s="2" t="inlineStr" /><c r="L196" s="2" t="inlineStr" /><c r="M196" s="2" t="inlineStr" /><c r="N196" s="2" t="inlineStr" /><c r="O196" s="2" t="inlineStr" /><c r="P196" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q196" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="197"><c r="A197" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B197" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C197" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D197" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E197" s="2" t="inlineStr"><is><t>Lekiem przeciwbakteryjnym o wąskim zakresie działania przeciwbakteryjnego jest:</t></is></c><c r="F197" s="2" t="inlineStr"><is><t>fenoksymetylopenicylina</t></is></c><c r="G197" s="2" t="inlineStr"><is><t>nystatyna</t></is></c><c r="H197" s="2" t="inlineStr" /><c r="I197" s="2" t="inlineStr" /><c r="J197" s="2" t="inlineStr" /><c r="K197" s="2" t="inlineStr"><is><t>aksetyl cefuroksymu</t></is></c><c r="L197" s="2" t="inlineStr"><is><t>chloramfenikol</t></is></c><c r="M197" s="2" t="inlineStr" /><c r="N197" s="2" t="inlineStr" /><c r="O197" s="2" t="inlineStr" /><c r="P197" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q197" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="198"><c r="A198" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B198" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C198" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D198" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E198" s="2" t="inlineStr"><is><t>Aktywność przeciwbakteryjną względem opornych na metycylinę szczepów Staphylococcus aureus (MRSA) ma:</t></is></c><c r="F198" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="G198" s="2" t="inlineStr"><is><t>mupirocyna</t></is></c><c r="H198" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="I198" s="2" t="inlineStr"><is><t>dalfoprystyna/chinuprystyna</t></is></c><c r="J198" s="2" t="inlineStr" /><c r="K198" s="2" t="inlineStr" /><c r="L198" s="2" t="inlineStr" /><c r="M198" s="2" t="inlineStr" /><c r="N198" s="2" t="inlineStr" /><c r="O198" s="2" t="inlineStr" /><c r="P198" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q198" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="199"><c r="A199" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B199" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C199" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D199" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E199" s="2" t="inlineStr"><is><t>Profilaktyka infekcyjnego zapalenia wsierdzia (IZW) jest wskazana u osób z grup wysokiego ryzyka IZW w przypadku procedur:</t></is></c><c r="F199" s="2" t="inlineStr"><is><t>dentystycznych z manipulacją w obrębie dziąseł lub okolicy około-wierzchołkowej zębów</t></is></c><c r="G199" s="2" t="inlineStr"><is><t>inwazyjnych w obrębie górnych dróg oddechowych, tj. usunięcie migdałka</t></is></c><c r="H199" s="2" t="inlineStr" /><c r="I199" s="2" t="inlineStr" /><c r="J199" s="2" t="inlineStr" /><c r="K199" s="2" t="inlineStr"><is><t>inwazyjnych w obrębie układu moczowo-płciowego</t></is></c><c r="L199" s="2" t="inlineStr"><is><t>inwazyjnych w obrębie przewodu pokarmowego</t></is></c><c r="M199" s="2" t="inlineStr" /><c r="N199" s="2" t="inlineStr" /><c r="O199" s="2" t="inlineStr" /><c r="P199" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q199" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="200"><c r="A200" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B200" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C200" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D200" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E200" s="2" t="inlineStr"><is><t>Gancyklowir:</t></is></c><c r="F200" s="2" t="inlineStr"><is><t>może powodować uszkodzenie szpiku</t></is></c><c r="G200" s="2" t="inlineStr" /><c r="H200" s="2" t="inlineStr" /><c r="I200" s="2" t="inlineStr" /><c r="J200" s="2" t="inlineStr" /><c r="K200" s="2" t="inlineStr"><is><t>jest inhibitorem proteazy wirusowej</t></is></c><c r="L200" s="2" t="inlineStr"><is><t>bezpośrednio hamuje uwalnianie wirusów z zakażonych komórek</t></is></c><c r="M200" s="2" t="inlineStr"><is><t>nie przenika do ośrodkowego układu nerwowego</t></is></c><c r="N200" s="2" t="inlineStr" /><c r="O200" s="2" t="inlineStr" /><c r="P200" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q200" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="201"><c r="A201" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B201" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C201" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D201" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E201" s="2" t="inlineStr"><is><t>W standardowej profilaktyce okołooperacyjnej wskazane jest stosowanie:</t></is></c><c r="F201" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="G201" s="2" t="inlineStr"><is><t>metronidazolu</t></is></c><c r="H201" s="2" t="inlineStr"><is><t>cyprofloksacyny</t></is></c><c r="I201" s="2" t="inlineStr"><is><t>cefazoliny</t></is></c><c r="J201" s="2" t="inlineStr" /><c r="K201" s="2" t="inlineStr" /><c r="L201" s="2" t="inlineStr" /><c r="M201" s="2" t="inlineStr" /><c r="N201" s="2" t="inlineStr" /><c r="O201" s="2" t="inlineStr" /><c r="P201" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q201" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="202"><c r="A202" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B202" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C202" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D202" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E202" s="2" t="inlineStr"><is><t>W grzybiczym zakażeniu skóry gładkiej można zastosować miejscowo:</t></is></c><c r="F202" s="2" t="inlineStr"><is><t>cyklopiroksolaminę</t></is></c><c r="G202" s="2" t="inlineStr"><is><t>natamycynę</t></is></c><c r="H202" s="2" t="inlineStr"><is><t>klotrimazol</t></is></c><c r="I202" s="2" t="inlineStr" /><c r="J202" s="2" t="inlineStr" /><c r="K202" s="2" t="inlineStr"><is><t>kaspofunginę</t></is></c><c r="L202" s="2" t="inlineStr" /><c r="M202" s="2" t="inlineStr" /><c r="N202" s="2" t="inlineStr" /><c r="O202" s="2" t="inlineStr" /><c r="P202" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q202" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="203"><c r="A203" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B203" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C203" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D203" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E203" s="2" t="inlineStr"><is><t>Wskaż poprawną strategię postępowania w zakresie leczenia zakażeń:</t></is></c><c r="F203" s="2" t="inlineStr"><is><t>leczenie empiryczne powinno uwzględniać miejsce powstania zakażenia: domowe lub związane z kontaktem ze służbą zdrowia</t></is></c><c r="G203" s="2" t="inlineStr"><is><t>na podstawie antybiogramu należy dokonać deeskalacji leczenia</t></is></c><c r="H203" s="2" t="inlineStr"><is><t>zasadą jest doustne leczenie przeciwinfekcyjne poza uzasadnionymi wyjątkami poza dekolonizacją MRSA przed operacjami</t></is></c><c r="I203" s="2" t="inlineStr" /><c r="J203" s="2" t="inlineStr" /><c r="K203" s="2" t="inlineStr" /><c r="L203" s="2" t="inlineStr" /><c r="M203" s="2" t="inlineStr" /><c r="N203" s="2" t="inlineStr" /><c r="O203" s="2" t="inlineStr" /><c r="P203" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q203" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="204"><c r="A204" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B204" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C204" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D204" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E204" s="2" t="inlineStr"><is><t>W Polsce granica opłacalności procedur medycznych jest:</t></is></c><c r="F204" s="2" t="inlineStr"><is><t>wykorzystywanym i usankcjonowanym prawnie kryterium refundacyjnym</t></is></c><c r="G204" s="2" t="inlineStr"><is><t>ustalona w oparciu o roczny koszt dializoterapii – przewlekłej, powszechnej i jednej z najdroższych procedur medycznych</t></is></c><c r="H204" s="2" t="inlineStr"><is><t>ustalona w oparciu o 3 krotność produktu krajowego brutto per capita</t></is></c><c r="I204" s="2" t="inlineStr"><is><t>odmienna dla leków stosowanych w chorobach onkologicznych</t></is></c><c r="J204" s="2" t="inlineStr" /><c r="K204" s="2" t="inlineStr" /><c r="L204" s="2" t="inlineStr" /><c r="M204" s="2" t="inlineStr" /><c r="N204" s="2" t="inlineStr" /><c r="O204" s="2" t="inlineStr" /><c r="P204" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q204" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="205"><c r="A205" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B205" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C205" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D205" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E205" s="2" t="inlineStr"><is><t>W leczeniu trądziku młodzieńczego racjonalne jest zastosowanie:</t></is></c><c r="F205" s="2" t="inlineStr"><is><t>klindamycyny</t></is></c><c r="G205" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="H205" s="2" t="inlineStr"><is><t>izotretinoiny</t></is></c><c r="I205" s="2" t="inlineStr" /><c r="J205" s="2" t="inlineStr" /><c r="K205" s="2" t="inlineStr"><is><t>norfloksacyny</t></is></c><c r="L205" s="2" t="inlineStr" /><c r="M205" s="2" t="inlineStr" /><c r="N205" s="2" t="inlineStr" /><c r="O205" s="2" t="inlineStr" /><c r="P205" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q205" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="206"><c r="A206" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B206" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C206" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D206" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E206" s="2" t="inlineStr"><is><t>Istotne genetycznie uwarunkowane różnice działania stwierdzono dla:</t></is></c><c r="F206" s="2" t="inlineStr"><is><t>abakawiru</t></is></c><c r="G206" s="2" t="inlineStr"><is><t>karbamazepiny</t></is></c><c r="H206" s="2" t="inlineStr"><is><t>warfaryny</t></is></c><c r="I206" s="2" t="inlineStr" /><c r="J206" s="2" t="inlineStr" /><c r="K206" s="2" t="inlineStr"><is><t>diltiazemu</t></is></c><c r="L206" s="2" t="inlineStr" /><c r="M206" s="2" t="inlineStr" /><c r="N206" s="2" t="inlineStr" /><c r="O206" s="2" t="inlineStr" /><c r="P206" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q206" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="207"><c r="A207" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B207" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C207" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D207" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E207" s="2" t="inlineStr"><is><t>Inhibitory dipeptydylopeptydazy IV (DPP IV):</t></is></c><c r="F207" s="2" t="inlineStr"><is><t>mogą być stosowane łącznie z insuliną</t></is></c><c r="G207" s="2" t="inlineStr"><is><t>zwiększają ryzyko wystąpienia dolegliwości ze strony przewodu pokarmowego</t></is></c><c r="H207" s="2" t="inlineStr" /><c r="I207" s="2" t="inlineStr" /><c r="J207" s="2" t="inlineStr" /><c r="K207" s="2" t="inlineStr"><is><t>powodują przyrost masy ciała</t></is></c><c r="L207" s="2" t="inlineStr"><is><t>są podawane podskórnie</t></is></c><c r="M207" s="2" t="inlineStr" /><c r="N207" s="2" t="inlineStr" /><c r="O207" s="2" t="inlineStr" /><c r="P207" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q207" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="208"><c r="A208" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B208" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C208" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D208" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E208" s="2" t="inlineStr"><is><t>Wskaż zdanie/zdania prawdziwe:</t></is></c><c r="F208" s="2" t="inlineStr"><is><t>empagliflozyna – zmniejsza ryzyko śmierci z przyczyn sercowo￾naczyniowych u chorych z cukrzycą typu 2</t></is></c><c r="G208" s="2" t="inlineStr"><is><t>metformina – zmniejsza ryzyko powikłań makroangiopatycznych</t></is></c><c r="H208" s="2" t="inlineStr" /><c r="I208" s="2" t="inlineStr" /><c r="J208" s="2" t="inlineStr" /><c r="K208" s="2" t="inlineStr"><is><t>sitagliptyna - pomimo euglikemii może spowodować kwasicę ketonową</t></is></c><c r="L208" s="2" t="inlineStr"><is><t>gliklazyd – powoduje redukcję masy ciała</t></is></c><c r="M208" s="2" t="inlineStr" /><c r="N208" s="2" t="inlineStr" /><c r="O208" s="2" t="inlineStr" /><c r="P208" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q208" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="209"><c r="A209" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B209" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C209" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D209" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E209" s="2" t="inlineStr"><is><t>Stosowanie tiamazolu może być przyczyną:</t></is></c><c r="F209" s="2" t="inlineStr"><is><t>żółtaczki cholestatycznej</t></is></c><c r="G209" s="2" t="inlineStr"><is><t>agranulocytozy</t></is></c><c r="H209" s="2" t="inlineStr"><is><t>wysypki skórnej</t></is></c><c r="I209" s="2" t="inlineStr"><is><t>niedoczynności tarczycy</t></is></c><c r="J209" s="2" t="inlineStr" /><c r="K209" s="2" t="inlineStr" /><c r="L209" s="2" t="inlineStr" /><c r="M209" s="2" t="inlineStr" /><c r="N209" s="2" t="inlineStr" /><c r="O209" s="2" t="inlineStr" /><c r="P209" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q209" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="210"><c r="A210" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B210" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C210" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D210" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E210" s="2" t="inlineStr"><is><t>Leczenie triamcynolonem może pogorszyć przebieg:</t></is></c><c r="F210" s="2" t="inlineStr"><is><t>jaskry</t></is></c><c r="G210" s="2" t="inlineStr"><is><t>zaburzeń nastroju</t></is></c><c r="H210" s="2" t="inlineStr"><is><t>zaćmy</t></is></c><c r="I210" s="2" t="inlineStr"><is><t>osteoporozy</t></is></c><c r="J210" s="2" t="inlineStr" /><c r="K210" s="2" t="inlineStr" /><c r="L210" s="2" t="inlineStr" /><c r="M210" s="2" t="inlineStr" /><c r="N210" s="2" t="inlineStr" /><c r="O210" s="2" t="inlineStr" /><c r="P210" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q210" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="211"><c r="A211" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B211" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C211" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D211" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E211" s="2" t="inlineStr"><is><t>Pacjent nieprzytomny, z hipoglikemią po spożyciu alkoholu, powinien otrzymać:</t></is></c><c r="F211" s="2" t="inlineStr"><is><t>20% roztwór glukozy i.v</t></is></c><c r="G211" s="2" t="inlineStr" /><c r="H211" s="2" t="inlineStr" /><c r="I211" s="2" t="inlineStr" /><c r="J211" s="2" t="inlineStr" /><c r="K211" s="2" t="inlineStr"><is><t>glukagon i.m</t></is></c><c r="L211" s="2" t="inlineStr"><is><t>glukozę p.o</t></is></c><c r="M211" s="2" t="inlineStr"><is><t>glukagon s.c</t></is></c><c r="N211" s="2" t="inlineStr" /><c r="O211" s="2" t="inlineStr" /><c r="P211" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q211" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="212"><c r="A212" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B212" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C212" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D212" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E212" s="2" t="inlineStr"><is><t>Potwierdzone klinicznie zmniejszenie ryzyka złamania kości udowej w przebiegu osteoporozy występuje w wyniku leczenia:</t></is></c><c r="F212" s="2" t="inlineStr"><is><t>ranelinianem strontu</t></is></c><c r="G212" s="2" t="inlineStr"><is><t>kwasem ibandronowy</t></is></c><c r="H212" s="2" t="inlineStr" /><c r="I212" s="2" t="inlineStr" /><c r="J212" s="2" t="inlineStr" /><c r="K212" s="2" t="inlineStr"><is><t>raloksyfenem</t></is></c><c r="L212" s="2" t="inlineStr"><is><t>kalcytoniną</t></is></c><c r="M212" s="2" t="inlineStr" /><c r="N212" s="2" t="inlineStr" /><c r="O212" s="2" t="inlineStr" /><c r="P212" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q212" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="213"><c r="A213" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B213" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C213" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D213" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E213" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie - wskazanie do stosowania glikokortykosteroidów - uzasadnienie zastosowania:</t></is></c><c r="F213" s="2" t="inlineStr"><is><t>poród przedwczesny – stymulowanie dojrzewania płuc płodu</t></is></c><c r="G213" s="2" t="inlineStr"><is><t>astma – ograniczenie procesu zapalnego</t></is></c><c r="H213" s="2" t="inlineStr"><is><t>przełom nadnerczowy – leczenie substytucyjne</t></is></c><c r="I213" s="2" t="inlineStr" /><c r="J213" s="2" t="inlineStr" /><c r="K213" s="2" t="inlineStr"><is><t>mononukleoza zakaźna – efekt immunosupresyjny</t></is></c><c r="L213" s="2" t="inlineStr" /><c r="M213" s="2" t="inlineStr" /><c r="N213" s="2" t="inlineStr" /><c r="O213" s="2" t="inlineStr" /><c r="P213" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q213" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="214"><c r="A214" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B214" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C214" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D214" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E214" s="2" t="inlineStr"><is><t>Do działań niepożądanych środków antykoncepcyjnych zalicza się:</t></is></c><c r="F214" s="2" t="inlineStr"><is><t>trądzik</t></is></c><c r="G214" s="2" t="inlineStr"><is><t>depresję</t></is></c><c r="H214" s="2" t="inlineStr"><is><t>zwiększenie ryzyka udaru mózgu</t></is></c><c r="I214" s="2" t="inlineStr" /><c r="J214" s="2" t="inlineStr" /><c r="K214" s="2" t="inlineStr"><is><t>zwiększenie ryzyka raka jajnika</t></is></c><c r="L214" s="2" t="inlineStr" /><c r="M214" s="2" t="inlineStr" /><c r="N214" s="2" t="inlineStr" /><c r="O214" s="2" t="inlineStr" /><c r="P214" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q214" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="215"><c r="A215" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B215" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C215" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D215" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E215" s="2" t="inlineStr"><is><t>Witamina D3 (cholekalcyferol):</t></is></c><c r="F215" s="2" t="inlineStr"><is><t>może być stosowana w niedoczynności przytarczyc</t></is></c><c r="G215" s="2" t="inlineStr"><is><t>w nadmiarze hamuje wzrost kości</t></is></c><c r="H215" s="2" t="inlineStr" /><c r="I215" s="2" t="inlineStr" /><c r="J215" s="2" t="inlineStr" /><c r="K215" s="2" t="inlineStr"><is><t>mimo stosowania w dużych dawkach nie chroni przed osteoporotycznymi złamaniami kości</t></is></c><c r="L215" s="2" t="inlineStr"><is><t>jest nieaktywna u chorych z niewydolnością nerek</t></is></c><c r="M215" s="2" t="inlineStr" /><c r="N215" s="2" t="inlineStr" /><c r="O215" s="2" t="inlineStr" /><c r="P215" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q215" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="216"><c r="A216" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B216" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C216" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D216" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E216" s="2" t="inlineStr"><is><t>Działanie przeczyszczające wykazuje:</t></is></c><c r="F216" s="2" t="inlineStr"><is><t>siarczan magnezu</t></is></c><c r="G216" s="2" t="inlineStr"><is><t>dokusan sodowy</t></is></c><c r="H216" s="2" t="inlineStr" /><c r="I216" s="2" t="inlineStr" /><c r="J216" s="2" t="inlineStr" /><c r="K216" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="L216" s="2" t="inlineStr"><is><t>racekadotryl</t></is></c><c r="M216" s="2" t="inlineStr" /><c r="N216" s="2" t="inlineStr" /><c r="O216" s="2" t="inlineStr" /><c r="P216" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q216" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="217"><c r="A217" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B217" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C217" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D217" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E217" s="2" t="inlineStr"><is><t>Mesna :</t></is></c><c r="F217" s="2" t="inlineStr"><is><t>powoduje upłynnienie wydzieliny w drzewie oskrzelowym</t></is></c><c r="G217" s="2" t="inlineStr"><is><t>jest antidotum przeciw metabolitowi cyklofosfamidu drażniącemu błonę śluzową dróg moczowych</t></is></c><c r="H217" s="2" t="inlineStr"><is><t>jest stosowana miejscowo w postaci inhalacji</t></is></c><c r="I217" s="2" t="inlineStr"><is><t>może wywołać skurcz oskrzeli</t></is></c><c r="J217" s="2" t="inlineStr" /><c r="K217" s="2" t="inlineStr" /><c r="L217" s="2" t="inlineStr" /><c r="M217" s="2" t="inlineStr" /><c r="N217" s="2" t="inlineStr" /><c r="O217" s="2" t="inlineStr" /><c r="P217" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q217" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="218"><c r="A218" s="2" t="inlineStr"><is><t>ZNIECZULENIA MIEJSCOWE</t></is></c><c r="B218" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C218" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D218" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E218" s="2" t="inlineStr"><is><t>Do leków znieczulających miejscowo stosowanych na błony śluzowe należy:</t></is></c><c r="F218" s="2" t="inlineStr"><is><t>prylokaina</t></is></c><c r="G218" s="2" t="inlineStr"><is><t>lidokaina</t></is></c><c r="H218" s="2" t="inlineStr" /><c r="I218" s="2" t="inlineStr" /><c r="J218" s="2" t="inlineStr" /><c r="K218" s="2" t="inlineStr"><is><t>chlorek etylu</t></is></c><c r="L218" s="2" t="inlineStr"><is><t>kapsaicyna</t></is></c><c r="M218" s="2" t="inlineStr" /><c r="N218" s="2" t="inlineStr" /><c r="O218" s="2" t="inlineStr" /><c r="P218" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q218" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="219"><c r="A219" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B219" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C219" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D219" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E219" s="2" t="inlineStr"><is><t>Inhibitorem kinaz białkowych jest:</t></is></c><c r="F219" s="2" t="inlineStr"><is><t>rapamycyna</t></is></c><c r="G219" s="2" t="inlineStr"><is><t>imatynib</t></is></c><c r="H219" s="2" t="inlineStr" /><c r="I219" s="2" t="inlineStr" /><c r="J219" s="2" t="inlineStr" /><c r="K219" s="2" t="inlineStr"><is><t>bortezomib</t></is></c><c r="L219" s="2" t="inlineStr"><is><t>lenalidomid</t></is></c><c r="M219" s="2" t="inlineStr" /><c r="N219" s="2" t="inlineStr" /><c r="O219" s="2" t="inlineStr" /><c r="P219" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q219" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="220"><c r="A220" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B220" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C220" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D220" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E220" s="2" t="inlineStr"><is><t>Betahistyna:</t></is></c><c r="F220" s="2" t="inlineStr"><is><t>zwiększa przepływ krwi w uchu wewnętrznym</t></is></c><c r="G220" s="2" t="inlineStr"><is><t>jest stosowana w leczeniu choroby Méniére'a</t></is></c><c r="H220" s="2" t="inlineStr" /><c r="I220" s="2" t="inlineStr" /><c r="J220" s="2" t="inlineStr" /><c r="K220" s="2" t="inlineStr"><is><t>jest agonistą receptorów H3</t></is></c><c r="L220" s="2" t="inlineStr"><is><t>jest lekiem z wyboru w przedsionkowych zawrotach głowy</t></is></c><c r="M220" s="2" t="inlineStr" /><c r="N220" s="2" t="inlineStr" /><c r="O220" s="2" t="inlineStr" /><c r="P220" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q220" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="221"><c r="A221" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B221" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C221" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D221" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E221" s="2" t="inlineStr"><is><t>Lekiem stosowanym w neuropatii popółpaścowej jest:</t></is></c><c r="F221" s="2" t="inlineStr"><is><t>amitryptylina</t></is></c><c r="G221" s="2" t="inlineStr"><is><t>pregabalina</t></is></c><c r="H221" s="2" t="inlineStr"><is><t>lidokaina</t></is></c><c r="I221" s="2" t="inlineStr"><is><t>gabapentyna</t></is></c><c r="J221" s="2" t="inlineStr" /><c r="K221" s="2" t="inlineStr" /><c r="L221" s="2" t="inlineStr" /><c r="M221" s="2" t="inlineStr" /><c r="N221" s="2" t="inlineStr" /><c r="O221" s="2" t="inlineStr" /><c r="P221" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q221" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="222"><c r="A222" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B222" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C222" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D222" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E222" s="2" t="inlineStr"><is><t>Na drugim stopniu drabiny analgetycznej wg WHO znajduje się:</t></is></c><c r="F222" s="2" t="inlineStr"><is><t>morfina w dawce ≤ 30 mg/dobę</t></is></c><c r="G222" s="2" t="inlineStr"><is><t>kodeina w dawce ≤360 mg/dobę</t></is></c><c r="H222" s="2" t="inlineStr"><is><t>oksykodon w dawce ≤20 mg/dobę</t></is></c><c r="I222" s="2" t="inlineStr" /><c r="J222" s="2" t="inlineStr" /><c r="K222" s="2" t="inlineStr"><is><t>fentanyl w dawce ≤ 10 mg/dobę</t></is></c><c r="L222" s="2" t="inlineStr" /><c r="M222" s="2" t="inlineStr" /><c r="N222" s="2" t="inlineStr" /><c r="O222" s="2" t="inlineStr" /><c r="P222" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q222" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="223"><c r="A223" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B223" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C223" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D223" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E223" s="2" t="inlineStr"><is><t>Wskaż prawidłowe zdanie:</t></is></c><c r="F223" s="2" t="inlineStr"><is><t>czas odstawienia rywaroksabanu przed planowanym zabiegiem chirurgicznym zależy od ryzyka krwawienia</t></is></c><c r="G223" s="2" t="inlineStr"><is><t>jeśli uzyskano stabilną hemostazę antagonisty witaminy K włącza się w 1. dobie po zabiegu chirurgicznym</t></is></c><c r="H223" s="2" t="inlineStr" /><c r="I223" s="2" t="inlineStr" /><c r="J223" s="2" t="inlineStr" /><c r="K223" s="2" t="inlineStr"><is><t>warfaryny nie należy odstawiać wcześniej niż na 2 dni przed planowanym zabiegiem chirurgicznym</t></is></c><c r="L223" s="2" t="inlineStr"><is><t>czas odstawienia edoksabanu przed zabiegiem chirurgicznym nie zależy od wartości klirensu kreatyniny</t></is></c><c r="M223" s="2" t="inlineStr" /><c r="N223" s="2" t="inlineStr" /><c r="O223" s="2" t="inlineStr" /><c r="P223" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q223" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="224"><c r="A224" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B224" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C224" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D224" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E224" s="2" t="inlineStr"><is><t>Wskaż prawidłowy lek przeciwzakrzepowego u osoby z:</t></is></c><c r="F224" s="2" t="inlineStr"><is><t>zapaleniem żył głębokich - rywaroksaban</t></is></c><c r="G224" s="2" t="inlineStr"><is><t>ciążą - enoksaparyna</t></is></c><c r="H224" s="2" t="inlineStr"><is><t>mechaniczną zastawką serca – warfaryna</t></is></c><c r="I224" s="2" t="inlineStr" /><c r="J224" s="2" t="inlineStr" /><c r="K224" s="2" t="inlineStr"><is><t>niewydolnością nerek (CCr &lt;30ml/min) – dabigatran</t></is></c><c r="L224" s="2" t="inlineStr" /><c r="M224" s="2" t="inlineStr" /><c r="N224" s="2" t="inlineStr" /><c r="O224" s="2" t="inlineStr" /><c r="P224" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q224" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="225"><c r="A225" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B225" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C225" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D225" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E225" s="2" t="inlineStr"><is><t>Podczas leczenia przeciwzakrzepowego z zastosowaniem nadroparyny należy:</t></is></c><c r="F225" s="2" t="inlineStr"><is><t>kontrolować liczbę płytek</t></is></c><c r="G225" s="2" t="inlineStr"><is><t>rozważyć korektę dawek u osób otyłych</t></is></c><c r="H225" s="2" t="inlineStr" /><c r="I225" s="2" t="inlineStr" /><c r="J225" s="2" t="inlineStr" /><c r="K225" s="2" t="inlineStr"><is><t>monitorować dawki za pomocą oznaczenia APTT</t></is></c><c r="L225" s="2" t="inlineStr"><is><t>zmniejszyć dawkę w każdym przypadku, jeśli eGFR osiąga wartość mniejszą niż 90 ml/min</t></is></c><c r="M225" s="2" t="inlineStr" /><c r="N225" s="2" t="inlineStr" /><c r="O225" s="2" t="inlineStr" /><c r="P225" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q225" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="226"><c r="A226" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B226" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C226" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D226" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E226" s="2" t="inlineStr"><is><t>Kangrelor:</t></is></c><c r="F226" s="2" t="inlineStr"><is><t>jest wskazany podczas przezskórnych interwencji wieńcowych łącznie z kwasem acetylosalicylowym</t></is></c><c r="G226" s="2" t="inlineStr" /><c r="H226" s="2" t="inlineStr" /><c r="I226" s="2" t="inlineStr" /><c r="J226" s="2" t="inlineStr" /><c r="K226" s="2" t="inlineStr"><is><t>jest agonistą receptora P2Y12</t></is></c><c r="L226" s="2" t="inlineStr"><is><t>wymaga aktywacji w przewodzie pokarmowym</t></is></c><c r="M226" s="2" t="inlineStr"><is><t>działa przez 1-2 doby</t></is></c><c r="N226" s="2" t="inlineStr" /><c r="O226" s="2" t="inlineStr" /><c r="P226" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q226" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="227"><c r="A227" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B227" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C227" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D227" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E227" s="2" t="inlineStr"><is><t>Na istotnie zmniejszoną skuteczność doustnych antagonistów witaminy K może mieć wpływ spożywanie:</t></is></c><c r="F227" s="2" t="inlineStr"><is><t>szpinaku</t></is></c><c r="G227" s="2" t="inlineStr" /><c r="H227" s="2" t="inlineStr" /><c r="I227" s="2" t="inlineStr" /><c r="J227" s="2" t="inlineStr" /><c r="K227" s="2" t="inlineStr"><is><t>oleju rybnego zawierającego nienasycone kwasy tłuszczowe omega -3</t></is></c><c r="L227" s="2" t="inlineStr"><is><t>witaminy E</t></is></c><c r="M227" s="2" t="inlineStr"><is><t>czosnku</t></is></c><c r="N227" s="2" t="inlineStr" /><c r="O227" s="2" t="inlineStr" /><c r="P227" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q227" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="228"><c r="A228" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B228" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C228" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D228" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E228" s="2" t="inlineStr"><is><t>Pacjentom, którzy przebyli udar niedokrwienny mózgu należy zalecić profilaktykę wtórną. Do leków o udokumentowanym działaniu zmniejszających ryzyko następnego udaru należy:</t></is></c><c r="F228" s="2" t="inlineStr"><is><t>simwastatyna</t></is></c><c r="G228" s="2" t="inlineStr"><is><t>klopidogrel</t></is></c><c r="H228" s="2" t="inlineStr"><is><t>lizynopryl</t></is></c><c r="I228" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="J228" s="2" t="inlineStr" /><c r="K228" s="2" t="inlineStr" /><c r="L228" s="2" t="inlineStr" /><c r="M228" s="2" t="inlineStr" /><c r="N228" s="2" t="inlineStr" /><c r="O228" s="2" t="inlineStr" /><c r="P228" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q228" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="229"><c r="A229" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B229" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C229" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D229" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E229" s="2" t="inlineStr"><is><t>Fenofibrat:</t></is></c><c r="F229" s="2" t="inlineStr"><is><t>zmniejsza stężenie trójglicerydów i zwiększa stężenie cholesterolu HDL</t></is></c><c r="G229" s="2" t="inlineStr"><is><t>zwiększa ryzyko kamicy pęcherzyka żółciowego</t></is></c><c r="H229" s="2" t="inlineStr" /><c r="I229" s="2" t="inlineStr" /><c r="J229" s="2" t="inlineStr" /><c r="K229" s="2" t="inlineStr"><is><t>hamuje reduktazę 3-hydroksy-3-metyloglutarylo-CoA (HMG-CoA)</t></is></c><c r="L229" s="2" t="inlineStr"><is><t>nie może być stosowany w połączeniu ze statyną</t></is></c><c r="M229" s="2" t="inlineStr" /><c r="N229" s="2" t="inlineStr" /><c r="O229" s="2" t="inlineStr" /><c r="P229" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q229" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="230"><c r="A230" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B230" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C230" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D230" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E230" s="2" t="inlineStr"><is><t>Hiperurykemię może spowodować:</t></is></c><c r="F230" s="2" t="inlineStr"><is><t>torasemid</t></is></c><c r="G230" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="H230" s="2" t="inlineStr" /><c r="I230" s="2" t="inlineStr" /><c r="J230" s="2" t="inlineStr" /><c r="K230" s="2" t="inlineStr"><is><t>losartan</t></is></c><c r="L230" s="2" t="inlineStr"><is><t>allopurynol</t></is></c><c r="M230" s="2" t="inlineStr" /><c r="N230" s="2" t="inlineStr" /><c r="O230" s="2" t="inlineStr" /><c r="P230" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q230" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="231"><c r="A231" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B231" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C231" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D231" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E231" s="2" t="inlineStr"><is><t>Odstęp QT mogą wydłużać:</t></is></c><c r="F231" s="2" t="inlineStr"><is><t>amiodaron</t></is></c><c r="G231" s="2" t="inlineStr"><is><t>sotalol</t></is></c><c r="H231" s="2" t="inlineStr" /><c r="I231" s="2" t="inlineStr" /><c r="J231" s="2" t="inlineStr" /><c r="K231" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="L231" s="2" t="inlineStr"><is><t>diltiazem</t></is></c><c r="M231" s="2" t="inlineStr" /><c r="N231" s="2" t="inlineStr" /><c r="O231" s="2" t="inlineStr" /><c r="P231" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q231" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="232"><c r="A232" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B232" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C232" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D232" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E232" s="2" t="inlineStr"><is><t>Indapamid:</t></is></c><c r="F232" s="2" t="inlineStr"><is><t>ma działanie naczyniorozszerzające</t></is></c><c r="G232" s="2" t="inlineStr"><is><t>może spowodować hiponatremię</t></is></c><c r="H232" s="2" t="inlineStr"><is><t>zmniejsza wydalanie wapnia z moczem</t></is></c><c r="I232" s="2" t="inlineStr"><is><t>jest chętnie stosowany w przewlekłej terapii nadciśnienia tętniczego u osób po 80 roku życia</t></is></c><c r="J232" s="2" t="inlineStr" /><c r="K232" s="2" t="inlineStr" /><c r="L232" s="2" t="inlineStr" /><c r="M232" s="2" t="inlineStr" /><c r="N232" s="2" t="inlineStr" /><c r="O232" s="2" t="inlineStr" /><c r="P232" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q232" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="233"><c r="A233" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B233" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C233" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D233" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E233" s="2" t="inlineStr"><is><t>Produkty biopodobne:</t></is></c><c r="F233" s="2" t="inlineStr"><is><t>są automatycznie zamienne (substytucja)</t></is></c><c r="G233" s="2" t="inlineStr"><is><t>muszą mieć potwierdzoną podobną immunogenność</t></is></c><c r="H233" s="2" t="inlineStr" /><c r="I233" s="2" t="inlineStr" /><c r="J233" s="2" t="inlineStr" /><c r="K233" s="2" t="inlineStr"><is><t>są rejestrowane w procedurze zdecentralizowanej</t></is></c><c r="L233" s="2" t="inlineStr"><is><t>po dopuszczeniu do obrotu mogą być stosowane we wszystkich wskazaniach zamiennie</t></is></c><c r="M233" s="2" t="inlineStr" /><c r="N233" s="2" t="inlineStr" /><c r="O233" s="2" t="inlineStr" /><c r="P233" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q233" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="234"><c r="A234" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B234" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C234" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D234" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E234" s="2" t="inlineStr"><is><t>W leczeniu zarażenia glistą ludzką stosujemy:</t></is></c><c r="F234" s="2" t="inlineStr"><is><t>pyrantel</t></is></c><c r="G234" s="2" t="inlineStr"><is><t>albendazol</t></is></c><c r="H234" s="2" t="inlineStr" /><c r="I234" s="2" t="inlineStr" /><c r="J234" s="2" t="inlineStr" /><c r="K234" s="2" t="inlineStr"><is><t>tynidazol</t></is></c><c r="L234" s="2" t="inlineStr"><is><t>krotamiton</t></is></c><c r="M234" s="2" t="inlineStr" /><c r="N234" s="2" t="inlineStr" /><c r="O234" s="2" t="inlineStr" /><c r="P234" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q234" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="235"><c r="A235" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B235" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C235" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D235" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E235" s="2" t="inlineStr"><is><t>W leczeniu grypy zaleca się:</t></is></c><c r="F235" s="2" t="inlineStr"><is><t>zanamiwir</t></is></c><c r="G235" s="2" t="inlineStr"><is><t>oseltamiwir</t></is></c><c r="H235" s="2" t="inlineStr" /><c r="I235" s="2" t="inlineStr" /><c r="J235" s="2" t="inlineStr" /><c r="K235" s="2" t="inlineStr"><is><t>acyklowir</t></is></c><c r="L235" s="2" t="inlineStr"><is><t>foskarnet</t></is></c><c r="M235" s="2" t="inlineStr" /><c r="N235" s="2" t="inlineStr" /><c r="O235" s="2" t="inlineStr" /><c r="P235" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q235" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="236"><c r="A236" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B236" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C236" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D236" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E236" s="2" t="inlineStr"><is><t>W przypadku dotychczas nieleczonych chorych, u których objawy astmy oskrzelowej w ciągu dnia występują sporadycznie (&lt;2 razy w miesiącu), objawy nocne nie występują, nie ma czynników ryzyka zaostrzeń (także w wywiadzie), a czynność płuc jest prawidłowa należy zastosować:</t></is></c><c r="F236" s="2" t="inlineStr"><is><t>fenoterol doraźnie</t></is></c><c r="G236" s="2" t="inlineStr" /><c r="H236" s="2" t="inlineStr" /><c r="I236" s="2" t="inlineStr" /><c r="J236" s="2" t="inlineStr" /><c r="K236" s="2" t="inlineStr"><is><t>montelukast przewlekle</t></is></c><c r="L236" s="2" t="inlineStr"><is><t>regularnie małe dawki cyklezonidu</t></is></c><c r="M236" s="2" t="inlineStr"><is><t>teofilinę krótkodziałającą</t></is></c><c r="N236" s="2" t="inlineStr" /><c r="O236" s="2" t="inlineStr" /><c r="P236" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q236" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="237"><c r="A237" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B237" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C237" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D237" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E237" s="2" t="inlineStr"><is><t>Bromek glikopironium :</t></is></c><c r="F237" s="2" t="inlineStr"><is><t>wykazuje synergizm działania bronchodylatacyjnego z indakaterolem</t></is></c><c r="G237" s="2" t="inlineStr"><is><t>jest stosowany w leczeniu podtrzymującym w POChP</t></is></c><c r="H237" s="2" t="inlineStr" /><c r="I237" s="2" t="inlineStr" /><c r="J237" s="2" t="inlineStr" /><c r="K237" s="2" t="inlineStr"><is><t>jest wziewnym agonistą receptorów muskarynowych</t></is></c><c r="L237" s="2" t="inlineStr"><is><t>rozszczepia wiązania disiarczkowe w glikoproteinach śluzu</t></is></c><c r="M237" s="2" t="inlineStr" /><c r="N237" s="2" t="inlineStr" /><c r="O237" s="2" t="inlineStr" /><c r="P237" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q237" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="238"><c r="A238" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B238" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C238" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D238" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E238" s="2" t="inlineStr"><is><t>W leczeniu przewlekłego zapalenia trzustki celowe może być zastosowanie:</t></is></c><c r="F238" s="2" t="inlineStr"><is><t>suplementacji enzymów trzustkowych</t></is></c><c r="G238" s="2" t="inlineStr"><is><t>tramadolu</t></is></c><c r="H238" s="2" t="inlineStr"><is><t>pantoprazolu</t></is></c><c r="I238" s="2" t="inlineStr"><is><t>fluoksetyny</t></is></c><c r="J238" s="2" t="inlineStr" /><c r="K238" s="2" t="inlineStr" /><c r="L238" s="2" t="inlineStr" /><c r="M238" s="2" t="inlineStr" /><c r="N238" s="2" t="inlineStr" /><c r="O238" s="2" t="inlineStr" /><c r="P238" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q238" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="239"><c r="A239" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B239" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C239" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D239" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E239" s="2" t="inlineStr"><is><t>Profilaktyka przeciwmalaryczna w warunkach wysokiego ryzyka zakażenia Plasmodium falciparum obejmuje stosowanie:</t></is></c><c r="F239" s="2" t="inlineStr"><is><t>repelentów</t></is></c><c r="G239" s="2" t="inlineStr"><is><t>atowakwonu/proguanilu</t></is></c><c r="H239" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="I239" s="2" t="inlineStr" /><c r="J239" s="2" t="inlineStr" /><c r="K239" s="2" t="inlineStr"><is><t>artemetru/lumefantryny</t></is></c><c r="L239" s="2" t="inlineStr" /><c r="M239" s="2" t="inlineStr" /><c r="N239" s="2" t="inlineStr" /><c r="O239" s="2" t="inlineStr" /><c r="P239" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q239" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="240"><c r="A240" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B240" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C240" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D240" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E240" s="2" t="inlineStr"><is><t>Adalimumab:</t></is></c><c r="F240" s="2" t="inlineStr"><is><t>jest rekombinowanym w pełni ludzkim przeciwciałem monoklonalnym</t></is></c><c r="G240" s="2" t="inlineStr"><is><t>neutralizuje biologiczną czynność TNF</t></is></c><c r="H240" s="2" t="inlineStr"><is><t>jest przeciwwskazany w ciężkich zakażeniach</t></is></c><c r="I240" s="2" t="inlineStr" /><c r="J240" s="2" t="inlineStr" /><c r="K240" s="2" t="inlineStr"><is><t>jest wytwarzany z użyciem komórek zwierzęcych, co wiadomo na podstawie ujednoliconych zasad nadawania nazw przeciwciałom monoklonalnym</t></is></c><c r="L240" s="2" t="inlineStr" /><c r="M240" s="2" t="inlineStr" /><c r="N240" s="2" t="inlineStr" /><c r="O240" s="2" t="inlineStr" /><c r="P240" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q240" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="241"><c r="A241" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B241" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C241" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D241" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E241" s="2" t="inlineStr"><is><t>Dla insuliny aspart u pacjentów z umiarkowaną i ciężką niewydolnością wątroby stwierdzono: t max = ok. 85 min (tmax = ok. 40 minut u pacjentów z prawidłową czynnością wątroby); AUC, Cmax i CL/F były podobne do pacjentów z prawidłową czynnością wątroby. Na tej podstawie u osób z niewydolnością wątroby uzasadnione jest:</t></is></c><c r="F241" s="2" t="inlineStr"><is><t>wcześniejsze podanie leku przed posiłkiem</t></is></c><c r="G241" s="2" t="inlineStr"><is><t>stosowanie leku u osób z 7-15 pkt wg skali Childa-Pugha</t></is></c><c r="H241" s="2" t="inlineStr" /><c r="I241" s="2" t="inlineStr" /><c r="J241" s="2" t="inlineStr" /><c r="K241" s="2" t="inlineStr"><is><t>wyłącznie dożylne podawanie leku</t></is></c><c r="L241" s="2" t="inlineStr"><is><t>redukcja dawki początkowej o ½ oszacowanej na podstawie m.c. i wyjściowej glikemii</t></is></c><c r="M241" s="2" t="inlineStr" /><c r="N241" s="2" t="inlineStr" /><c r="O241" s="2" t="inlineStr" /><c r="P241" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q241" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="242"><c r="A242" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B242" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C242" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D242" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E242" s="2" t="inlineStr"><is><t>Wartości ciśnienia tętniczego mogą się zwiększyć po włączeniu:</t></is></c><c r="F242" s="2" t="inlineStr"><is><t>metyloprednizolonu</t></is></c><c r="G242" s="2" t="inlineStr"><is><t>diklofenaku</t></is></c><c r="H242" s="2" t="inlineStr" /><c r="I242" s="2" t="inlineStr" /><c r="J242" s="2" t="inlineStr" /><c r="K242" s="2" t="inlineStr"><is><t>eplerenonu</t></is></c><c r="L242" s="2" t="inlineStr"><is><t>urapidylu</t></is></c><c r="M242" s="2" t="inlineStr" /><c r="N242" s="2" t="inlineStr" /><c r="O242" s="2" t="inlineStr" /><c r="P242" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q242" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="243"><c r="A243" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B243" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C243" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D243" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E243" s="2" t="inlineStr"><is><t>Farmakoterapię otyłości należy rozważyć, gdy:</t></is></c><c r="F243" s="2" t="inlineStr"><is><t>BMI&gt; 27 kg/m2 i glikemia na czczo &gt;100mg/dl</t></is></c><c r="G243" s="2" t="inlineStr"><is><t>BMI≥ 30 kg/m2 i stwierdzono ponowny wzrost masy ciała pomimo wdrożonych procedur niefarmakologicznych</t></is></c><c r="H243" s="2" t="inlineStr"><is><t>BMI&gt; 27 kg/m2 i SBP ≥160 mmHg</t></is></c><c r="I243" s="2" t="inlineStr" /><c r="J243" s="2" t="inlineStr" /><c r="K243" s="2" t="inlineStr"><is><t>BMI≥ 30 kg/m2, a wcześniejsze procedury niefarmakologiczne spowodowały redukcję masy ciała w przedziale 7-10 kg</t></is></c><c r="L243" s="2" t="inlineStr" /><c r="M243" s="2" t="inlineStr" /><c r="N243" s="2" t="inlineStr" /><c r="O243" s="2" t="inlineStr" /><c r="P243" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q243" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="244"><c r="A244" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B244" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C244" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D244" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E244" s="2" t="inlineStr"><is><t>Wzrost masy ciała mogą spowodować:</t></is></c><c r="F244" s="2" t="inlineStr"><is><t>chlorpromazyna</t></is></c><c r="G244" s="2" t="inlineStr"><is><t>insulina</t></is></c><c r="H244" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="I244" s="2" t="inlineStr" /><c r="J244" s="2" t="inlineStr" /><c r="K244" s="2" t="inlineStr"><is><t>liraglutyd</t></is></c><c r="L244" s="2" t="inlineStr" /><c r="M244" s="2" t="inlineStr" /><c r="N244" s="2" t="inlineStr" /><c r="O244" s="2" t="inlineStr" /><c r="P244" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q244" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="245"><c r="A245" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B245" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C245" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D245" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E245" s="2" t="inlineStr"><is><t>Który z leków istotnie zwiększa ryzyko napadów drgawkowych:</t></is></c><c r="F245" s="2" t="inlineStr"><is><t>tramadol</t></is></c><c r="G245" s="2" t="inlineStr"><is><t>amitryptylina</t></is></c><c r="H245" s="2" t="inlineStr"><is><t>prometazyna</t></is></c><c r="I245" s="2" t="inlineStr" /><c r="J245" s="2" t="inlineStr" /><c r="K245" s="2" t="inlineStr"><is><t>klorazepan</t></is></c><c r="L245" s="2" t="inlineStr" /><c r="M245" s="2" t="inlineStr" /><c r="N245" s="2" t="inlineStr" /><c r="O245" s="2" t="inlineStr" /><c r="P245" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q245" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="246"><c r="A246" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B246" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C246" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D246" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E246" s="2" t="inlineStr"><is><t>Zgoda komisji bioetycznej jest niezbędna, gdy planowane jest przeprowadzenie:</t></is></c><c r="F246" s="2" t="inlineStr"><is><t>badania klinicznego fazy III</t></is></c><c r="G246" s="2" t="inlineStr"><is><t>eksperymentu leczniczego</t></is></c><c r="H246" s="2" t="inlineStr"><is><t>badania klinicznego niekomercyjnego</t></is></c><c r="I246" s="2" t="inlineStr" /><c r="J246" s="2" t="inlineStr" /><c r="K246" s="2" t="inlineStr"><is><t>zastosowania leku off-label, ale zgodnie z aktualną wiedzą medyczną</t></is></c><c r="L246" s="2" t="inlineStr" /><c r="M246" s="2" t="inlineStr" /><c r="N246" s="2" t="inlineStr" /><c r="O246" s="2" t="inlineStr" /><c r="P246" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q246" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="247"><c r="A247" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B247" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C247" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D247" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E247" s="2" t="inlineStr"><is><t>W procedurze centralnej rejestruje się leki stosowane w:</t></is></c><c r="F247" s="2" t="inlineStr"><is><t>chorobach rzadkich</t></is></c><c r="G247" s="2" t="inlineStr"><is><t>terapii HIV</t></is></c><c r="H247" s="2" t="inlineStr"><is><t>terapii genowej</t></is></c><c r="I247" s="2" t="inlineStr" /><c r="J247" s="2" t="inlineStr" /><c r="K247" s="2" t="inlineStr"><is><t>populacji geriatrycznej</t></is></c><c r="L247" s="2" t="inlineStr" /><c r="M247" s="2" t="inlineStr" /><c r="N247" s="2" t="inlineStr" /><c r="O247" s="2" t="inlineStr" /><c r="P247" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q247" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="248"><c r="A248" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B248" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C248" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D248" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E248" s="2" t="inlineStr"><is><t>Pierwotnym źródłem wiedzy o lekach są:</t></is></c><c r="F248" s="2" t="inlineStr"><is><t>publikacje wyników badań klinicznych</t></is></c><c r="G248" s="2" t="inlineStr" /><c r="H248" s="2" t="inlineStr" /><c r="I248" s="2" t="inlineStr" /><c r="J248" s="2" t="inlineStr" /><c r="K248" s="2" t="inlineStr"><is><t>wytyczne praktyki klinicznej</t></is></c><c r="L248" s="2" t="inlineStr"><is><t>charakterystyki produktów leczniczych</t></is></c><c r="M248" s="2" t="inlineStr"><is><t>podręczniki farmakologii i indeksy leków</t></is></c><c r="N248" s="2" t="inlineStr" /><c r="O248" s="2" t="inlineStr" /><c r="P248" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q248" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="249"><c r="A249" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B249" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C249" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D249" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E249" s="2" t="inlineStr"><is><t>Wskazaniem do stosowania retinolu jest:</t></is></c><c r="F249" s="2" t="inlineStr"><is><t>łuszczyca</t></is></c><c r="G249" s="2" t="inlineStr"><is><t>niedowidzenie o zmierzchu</t></is></c><c r="H249" s="2" t="inlineStr" /><c r="I249" s="2" t="inlineStr" /><c r="J249" s="2" t="inlineStr" /><c r="K249" s="2" t="inlineStr"><is><t>polineuropatia obwodowa</t></is></c><c r="L249" s="2" t="inlineStr"><is><t>osteomalacja</t></is></c><c r="M249" s="2" t="inlineStr" /><c r="N249" s="2" t="inlineStr" /><c r="O249" s="2" t="inlineStr" /><c r="P249" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q249" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="250"><c r="A250" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B250" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C250" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D250" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E250" s="2" t="inlineStr"><is><t>Feksofenadyna:</t></is></c><c r="F250" s="2" t="inlineStr"><is><t>jest podawana doustnie</t></is></c><c r="G250" s="2" t="inlineStr" /><c r="H250" s="2" t="inlineStr" /><c r="I250" s="2" t="inlineStr" /><c r="J250" s="2" t="inlineStr" /><c r="K250" s="2" t="inlineStr"><is><t>działa nieselektywnie na rec. H1</t></is></c><c r="L250" s="2" t="inlineStr"><is><t>przenika w znacznym stopniu przez barierę krew- mózg</t></is></c><c r="M250" s="2" t="inlineStr"><is><t>działa kardiotoksycznie i jest przeciwwskazana w chorobie niedokrwiennej serca</t></is></c><c r="N250" s="2" t="inlineStr" /><c r="O250" s="2" t="inlineStr" /><c r="P250" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q250" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="251"><c r="A251" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B251" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C251" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D251" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E251" s="2" t="inlineStr"><is><t>Wskaż wady dekstranów:</t></is></c><c r="F251" s="2" t="inlineStr"><is><t>utrudniają wiarygodne oznaczenie grupy krwi i próby krzyżowej</t></is></c><c r="G251" s="2" t="inlineStr"><is><t>są immunogenne</t></is></c><c r="H251" s="2" t="inlineStr" /><c r="I251" s="2" t="inlineStr" /><c r="J251" s="2" t="inlineStr" /><c r="K251" s="2" t="inlineStr"><is><t>powodują przyrost objętości wewnątrznaczyniowej przekraczający ich objętość</t></is></c><c r="L251" s="2" t="inlineStr"><is><t>działają prozakrzepowo</t></is></c><c r="M251" s="2" t="inlineStr" /><c r="N251" s="2" t="inlineStr" /><c r="O251" s="2" t="inlineStr" /><c r="P251" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q251" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="252"><c r="A252" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B252" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C252" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D252" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E252" s="2" t="inlineStr"><is><t>Podanie rywastygminy jest uzasadnione u pacjentów z:</t></is></c><c r="F252" s="2" t="inlineStr"><is><t>otępieniem w przebiegu choroby Parkinsona</t></is></c><c r="G252" s="2" t="inlineStr"><is><t>chorobą Alzheimera</t></is></c><c r="H252" s="2" t="inlineStr" /><c r="I252" s="2" t="inlineStr" /><c r="J252" s="2" t="inlineStr" /><c r="K252" s="2" t="inlineStr"><is><t>otępieniem naczyniopochodnym</t></is></c><c r="L252" s="2" t="inlineStr"><is><t>otępieniem czołowo-skroniowym</t></is></c><c r="M252" s="2" t="inlineStr" /><c r="N252" s="2" t="inlineStr" /><c r="O252" s="2" t="inlineStr" /><c r="P252" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q252" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="253"><c r="A253" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B253" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C253" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D253" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E253" s="2" t="inlineStr"><is><t>W alkoholowym zespole odstawiennym celowe może być zastosowanie:</t></is></c><c r="F253" s="2" t="inlineStr"><is><t>tiaminy</t></is></c><c r="G253" s="2" t="inlineStr"><is><t>diazepamu</t></is></c><c r="H253" s="2" t="inlineStr"><is><t>płynoterapia z suplementacją elektrolitów</t></is></c><c r="I253" s="2" t="inlineStr" /><c r="J253" s="2" t="inlineStr" /><c r="K253" s="2" t="inlineStr"><is><t>akamprozatu</t></is></c><c r="L253" s="2" t="inlineStr" /><c r="M253" s="2" t="inlineStr" /><c r="N253" s="2" t="inlineStr" /><c r="O253" s="2" t="inlineStr" /><c r="P253" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q253" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="254"><c r="A254" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B254" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C254" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D254" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E254" s="2" t="inlineStr"><is><t>Mykofenolan mofetylu:</t></is></c><c r="F254" s="2" t="inlineStr"><is><t>jest wskazany w profilaktyce ostrego odrzucania przeszczepu serca</t></is></c><c r="G254" s="2" t="inlineStr"><is><t>zwiększa ryzyko wystąpienia nowotworów</t></is></c><c r="H254" s="2" t="inlineStr" /><c r="I254" s="2" t="inlineStr" /><c r="J254" s="2" t="inlineStr" /><c r="K254" s="2" t="inlineStr"><is><t>należy do inhibitorów mTOR</t></is></c><c r="L254" s="2" t="inlineStr"><is><t>stosowany w czasie ciąży jest bezpieczny dla płodu</t></is></c><c r="M254" s="2" t="inlineStr" /><c r="N254" s="2" t="inlineStr" /><c r="O254" s="2" t="inlineStr" /><c r="P254" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q254" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="255"><c r="A255" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B255" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C255" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D255" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E255" s="2" t="inlineStr"><is><t>Iwabradyna:</t></is></c><c r="F255" s="2" t="inlineStr"><is><t>może powodować zaburzenia widzenia</t></is></c><c r="G255" s="2" t="inlineStr"><is><t>wybiórczo i swoiście wpływa na na prąd If rozrusznika serca</t></is></c><c r="H255" s="2" t="inlineStr" /><c r="I255" s="2" t="inlineStr" /><c r="J255" s="2" t="inlineStr" /><c r="K255" s="2" t="inlineStr"><is><t>obniża kurczliwość mięśnia sercowego</t></is></c><c r="L255" s="2" t="inlineStr"><is><t>wydłuża czas repolaryzacji komór</t></is></c><c r="M255" s="2" t="inlineStr" /><c r="N255" s="2" t="inlineStr" /><c r="O255" s="2" t="inlineStr" /><c r="P255" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q255" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="256"><c r="A256" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B256" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C256" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D256" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E256" s="2" t="inlineStr"><is><t>Monoazotan izosorbidu:</t></is></c><c r="F256" s="2" t="inlineStr"><is><t>jest skuteczny po podaniu doustnym</t></is></c><c r="G256" s="2" t="inlineStr"><is><t>poprawia ukrwienie obszarów podwsierdziowych serca</t></is></c><c r="H256" s="2" t="inlineStr" /><c r="I256" s="2" t="inlineStr" /><c r="J256" s="2" t="inlineStr" /><c r="K256" s="2" t="inlineStr"><is><t>podlega istotnemu efektowi pierwszego przejścia przez wątrobę</t></is></c><c r="L256" s="2" t="inlineStr"><is><t>jest przeciwwskazany w naczynioskurczowej postaci choroby wieńcowej</t></is></c><c r="M256" s="2" t="inlineStr" /><c r="N256" s="2" t="inlineStr" /><c r="O256" s="2" t="inlineStr" /><c r="P256" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q256" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="257"><c r="A257" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B257" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C257" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D257" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E257" s="2" t="inlineStr"><is><t>W leczeniu owrzodzeń żylnych, jako leczenie uzupełniające, skuteczne są:</t></is></c><c r="F257" s="2" t="inlineStr"><is><t>mikronizowana diosmina</t></is></c><c r="G257" s="2" t="inlineStr"><is><t>opatrunki ze srebrem</t></is></c><c r="H257" s="2" t="inlineStr"><is><t>pentoksyfilina</t></is></c><c r="I257" s="2" t="inlineStr"><is><t>filgrastym</t></is></c><c r="J257" s="2" t="inlineStr" /><c r="K257" s="2" t="inlineStr" /><c r="L257" s="2" t="inlineStr" /><c r="M257" s="2" t="inlineStr" /><c r="N257" s="2" t="inlineStr" /><c r="O257" s="2" t="inlineStr" /><c r="P257" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q257" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="258"><c r="A258" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B258" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C258" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D258" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E258" s="2" t="inlineStr"><is><t>Funkcje kognitywne u osób bez zaburzeń poznawczych poprawiają:</t></is></c><c r="F258" s="2" t="inlineStr"><is><t>piracetam</t></is></c><c r="G258" s="2" t="inlineStr"><is><t>winpocetyna</t></is></c><c r="H258" s="2" t="inlineStr"><is><t>nicergolina</t></is></c><c r="I258" s="2" t="inlineStr"><is><t>metylfenidat</t></is></c><c r="J258" s="2" t="inlineStr" /><c r="K258" s="2" t="inlineStr" /><c r="L258" s="2" t="inlineStr" /><c r="M258" s="2" t="inlineStr" /><c r="N258" s="2" t="inlineStr" /><c r="O258" s="2" t="inlineStr" /><c r="P258" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q258" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="259"><c r="A259" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B259" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C259" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D259" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E259" s="2" t="inlineStr"><is><t>Klozapina:</t></is></c><c r="F259" s="2" t="inlineStr"><is><t>może być skuteczna w lekoopornej schizofrenii</t></is></c><c r="G259" s="2" t="inlineStr"><is><t>wymaga monitorowania morfologii krwi</t></is></c><c r="H259" s="2" t="inlineStr"><is><t>nasila objawy zespołu metabolicznego</t></is></c><c r="I259" s="2" t="inlineStr" /><c r="J259" s="2" t="inlineStr" /><c r="K259" s="2" t="inlineStr"><is><t>w małych dawkach zalecana jest do leczenia bezsenności</t></is></c><c r="L259" s="2" t="inlineStr" /><c r="M259" s="2" t="inlineStr" /><c r="N259" s="2" t="inlineStr" /><c r="O259" s="2" t="inlineStr" /><c r="P259" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q259" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="260"><c r="A260" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B260" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C260" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D260" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E260" s="2" t="inlineStr"><is><t>W terapii substytucyjnej uzależnienia od opioidów celowe może być zastosowanie:</t></is></c><c r="F260" s="2" t="inlineStr"><is><t>buprenorfiny</t></is></c><c r="G260" s="2" t="inlineStr"><is><t>metadonu</t></is></c><c r="H260" s="2" t="inlineStr" /><c r="I260" s="2" t="inlineStr" /><c r="J260" s="2" t="inlineStr" /><c r="K260" s="2" t="inlineStr"><is><t>nalokson</t></is></c><c r="L260" s="2" t="inlineStr"><is><t>warenikliny</t></is></c><c r="M260" s="2" t="inlineStr" /><c r="N260" s="2" t="inlineStr" /><c r="O260" s="2" t="inlineStr" /><c r="P260" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q260" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="261"><c r="A261" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B261" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C261" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D261" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E261" s="2" t="inlineStr"><is><t>Silnie hepatotoksycznie działa:</t></is></c><c r="F261" s="2" t="inlineStr"><is><t>izoniazyd</t></is></c><c r="G261" s="2" t="inlineStr"><is><t>pirazynamid</t></is></c><c r="H261" s="2" t="inlineStr"><is><t>ryfampicyna</t></is></c><c r="I261" s="2" t="inlineStr" /><c r="J261" s="2" t="inlineStr" /><c r="K261" s="2" t="inlineStr"><is><t>streptomycyna</t></is></c><c r="L261" s="2" t="inlineStr" /><c r="M261" s="2" t="inlineStr" /><c r="N261" s="2" t="inlineStr" /><c r="O261" s="2" t="inlineStr" /><c r="P261" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q261" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="262"><c r="A262" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B262" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C262" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D262" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E262" s="2" t="inlineStr"><is><t>Etambutol:</t></is></c><c r="F262" s="2" t="inlineStr"><is><t>zapobiega powstawaniu lekooporności na inne leki przeciwprątkowe</t></is></c><c r="G262" s="2" t="inlineStr"><is><t>może spowodować zaburzenia widzenia barwnego</t></is></c><c r="H262" s="2" t="inlineStr" /><c r="I262" s="2" t="inlineStr" /><c r="J262" s="2" t="inlineStr" /><c r="K262" s="2" t="inlineStr"><is><t>nie powinien być stosowany przez kobiety w ciąży</t></is></c><c r="L262" s="2" t="inlineStr"><is><t>nie jest stosowany w leczeniu gruźlicy pozapłucnej</t></is></c><c r="M262" s="2" t="inlineStr" /><c r="N262" s="2" t="inlineStr" /><c r="O262" s="2" t="inlineStr" /><c r="P262" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q262" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="263"><c r="A263" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B263" s="2" t="inlineStr"><is><t>Struktura chemiczna</t></is></c><c r="C263" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D263" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E263" s="2" t="inlineStr"><is><t>Jeśli leczymy depresję, to:</t></is></c><c r="F263" s="2" t="inlineStr"><is><t>u pacjentów z niewydolnością nerek lekiem pierwszego wyboru może być sertralina</t></is></c><c r="G263" s="2" t="inlineStr"><is><t>istnieje zwiększone ryzyko zachowań samobójczych u pacjentów w wieku poniżej 25 lat w okresie rozpoczynania leczenia przeciwdepresyjnego</t></is></c><c r="H263" s="2" t="inlineStr" /><c r="I263" s="2" t="inlineStr" /><c r="J263" s="2" t="inlineStr" /><c r="K263" s="2" t="inlineStr"><is><t>u osób starszych preferujemy trójpierścieniowe laki przeciwdepresyjne</t></is></c><c r="L263" s="2" t="inlineStr"><is><t>brak poprawy po 4 tygodniach leczenia sugeruje rozpoznanie depresji lekoopornej</t></is></c><c r="M263" s="2" t="inlineStr" /><c r="N263" s="2" t="inlineStr" /><c r="O263" s="2" t="inlineStr" /><c r="P263" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q263" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="264"><c r="A264" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B264" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C264" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D264" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E264" s="2" t="inlineStr"><is><t>Działanie przeciwkaszlowe wykazuje:</t></is></c><c r="F264" s="2" t="inlineStr"><is><t>dekstrometorfan</t></is></c><c r="G264" s="2" t="inlineStr"><is><t>kodeina</t></is></c><c r="H264" s="2" t="inlineStr" /><c r="I264" s="2" t="inlineStr" /><c r="J264" s="2" t="inlineStr" /><c r="K264" s="2" t="inlineStr"><is><t>loperamid</t></is></c><c r="L264" s="2" t="inlineStr"><is><t>prometazyna</t></is></c><c r="M264" s="2" t="inlineStr" /><c r="N264" s="2" t="inlineStr" /><c r="O264" s="2" t="inlineStr" /><c r="P264" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q264" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="265"><c r="A265" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B265" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C265" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D265" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E265" s="2" t="inlineStr"><is><t>Atropina jest stosowana w przypadku zatrucia:</t></is></c><c r="F265" s="2" t="inlineStr"><is><t>grzybami strzępiakami i lejkówkami</t></is></c><c r="G265" s="2" t="inlineStr"><is><t>glikozydami naparstnicy</t></is></c><c r="H265" s="2" t="inlineStr"><is><t>związkami fosforoorganicznymi</t></is></c><c r="I265" s="2" t="inlineStr" /><c r="J265" s="2" t="inlineStr" /><c r="K265" s="2" t="inlineStr"><is><t>pokrzykiem wilczą jagodą</t></is></c><c r="L265" s="2" t="inlineStr" /><c r="M265" s="2" t="inlineStr" /><c r="N265" s="2" t="inlineStr" /><c r="O265" s="2" t="inlineStr" /><c r="P265" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q265" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="266"><c r="A266" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B266" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C266" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D266" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E266" s="2" t="inlineStr"><is><t>W porównaniu do osób dorosłych w populacji pediatrycznej:</t></is></c><c r="F266" s="2" t="inlineStr"><is><t>zmieniona reakcja na leki jest uwarunkowana przede wszystkim zmianami w farmakokinetyce leków</t></is></c><c r="G266" s="2" t="inlineStr"><is><t>do osiągnięcia stężenia terapeutycznego leku mogą wystarczyć w pierwszym kwartale życia (w przeliczeniu na masę ciała) mniejsze dawki leku</t></is></c><c r="H266" s="2" t="inlineStr"><is><t>w pierwszym półroczu życia leki wydalane przez nerki są eliminowane wolniej, a ich biologiczny okres półtrwania jest dłuższy</t></is></c><c r="I266" s="2" t="inlineStr"><is><t>w pierwszym roku życia frakcja wolna leku może być większa</t></is></c><c r="J266" s="2" t="inlineStr" /><c r="K266" s="2" t="inlineStr" /><c r="L266" s="2" t="inlineStr" /><c r="M266" s="2" t="inlineStr" /><c r="N266" s="2" t="inlineStr" /><c r="O266" s="2" t="inlineStr" /><c r="P266" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q266" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="267"><c r="A267" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B267" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C267" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D267" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E267" s="2" t="inlineStr"><is><t>Inhibitory fosfodiesterazy typu 5:</t></is></c><c r="F267" s="2" t="inlineStr"><is><t>są skuteczne w leczeniu zaburzeń erekcji</t></is></c><c r="G267" s="2" t="inlineStr"><is><t>nie mogą być przyjmowane jednocześnie z azotanami z uwagi na duże ryzyko wystąpienia ciężkiej, niekorygowalnej hipotonii</t></is></c><c r="H267" s="2" t="inlineStr" /><c r="I267" s="2" t="inlineStr" /><c r="J267" s="2" t="inlineStr" /><c r="K267" s="2" t="inlineStr"><is><t>wydłużają dystans marszu bez bólu u pacjentów z chromaniem przestankowym</t></is></c><c r="L267" s="2" t="inlineStr"><is><t>mają działanie inotropowe dodatnie</t></is></c><c r="M267" s="2" t="inlineStr" /><c r="N267" s="2" t="inlineStr" /><c r="O267" s="2" t="inlineStr" /><c r="P267" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q267" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="268"><c r="A268" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B268" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C268" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D268" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E268" s="2" t="inlineStr"><is><t>Wpływ rozkurczający na mięśniówkę przewodu pokarmowego ma:</t></is></c><c r="F268" s="2" t="inlineStr"><is><t>drotaweryna</t></is></c><c r="G268" s="2" t="inlineStr" /><c r="H268" s="2" t="inlineStr" /><c r="I268" s="2" t="inlineStr" /><c r="J268" s="2" t="inlineStr" /><c r="K268" s="2" t="inlineStr"><is><t>itopryd</t></is></c><c r="L268" s="2" t="inlineStr"><is><t>mesalazyna</t></is></c><c r="M268" s="2" t="inlineStr"><is><t>ryfaksymina</t></is></c><c r="N268" s="2" t="inlineStr" /><c r="O268" s="2" t="inlineStr" /><c r="P268" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q268" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="269"><c r="A269" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B269" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C269" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D269" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E269" s="2" t="inlineStr"><is><t>Lanzoprazol stosowany przewlekle powoduje:</t></is></c><c r="F269" s="2" t="inlineStr"><is><t>wzrost ryzyka zakażenia Clostridum difficile</t></is></c><c r="G269" s="2" t="inlineStr"><is><t>wzrost ryzyka infekcji dróg oddechowych</t></is></c><c r="H269" s="2" t="inlineStr"><is><t>zmniejszenie wchłaniania wapnia z przewodu pokarmowego</t></is></c><c r="I269" s="2" t="inlineStr"><is><t>zmniejszenie przekształcania klopidogrelu do aktywnych pochodnych</t></is></c><c r="J269" s="2" t="inlineStr" /><c r="K269" s="2" t="inlineStr" /><c r="L269" s="2" t="inlineStr" /><c r="M269" s="2" t="inlineStr" /><c r="N269" s="2" t="inlineStr" /><c r="O269" s="2" t="inlineStr" /><c r="P269" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q269" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="270"><c r="A270" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B270" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C270" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D270" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E270" s="2" t="inlineStr"><is><t>Sposób eradykacji Helicobacter pylori zalecany w Polsce to:</t></is></c><c r="F270" s="2" t="inlineStr"><is><t>podwójna dawka IPP, metronidazol, tetracyklina, cytrynian bizmutu przez 14 dni</t></is></c><c r="G270" s="2" t="inlineStr" /><c r="H270" s="2" t="inlineStr" /><c r="I270" s="2" t="inlineStr" /><c r="J270" s="2" t="inlineStr" /><c r="K270" s="2" t="inlineStr"><is><t>terapia sekwencyjna przez 10 dni - podwójna dawka IPP (inhibitora pompy protonowej) z amoksycyliną (dni 1-5), a następnie z klarytromycyną i metronidazolem (dni 6-10)</t></is></c><c r="L270" s="2" t="inlineStr"><is><t>podwójna dawka IPP, amoksycylina, klarytromycyna przez 10 dni</t></is></c><c r="M270" s="2" t="inlineStr"><is><t>podwójna dawka IPP, amoksycylina, klarytromycyna, metronidazol przez 14 dni</t></is></c><c r="N270" s="2" t="inlineStr" /><c r="O270" s="2" t="inlineStr" /><c r="P270" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q270" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="271"><c r="A271" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B271" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C271" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D271" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E271" s="2" t="inlineStr"><is><t>Udokumentowane działanie teratogenne wykazuje:</t></is></c><c r="F271" s="2" t="inlineStr"><is><t>trimetoprim-sulfametoksazol</t></is></c><c r="G271" s="2" t="inlineStr"><is><t>warfaryna</t></is></c><c r="H271" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="I271" s="2" t="inlineStr"><is><t>gentamycyna</t></is></c><c r="J271" s="2" t="inlineStr" /><c r="K271" s="2" t="inlineStr" /><c r="L271" s="2" t="inlineStr" /><c r="M271" s="2" t="inlineStr" /><c r="N271" s="2" t="inlineStr" /><c r="O271" s="2" t="inlineStr" /><c r="P271" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q271" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="272"><c r="A272" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B272" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C272" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D272" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E272" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – odtrutka:</t></is></c><c r="F272" s="2" t="inlineStr"><is><t>oksazepam - flumazenil</t></is></c><c r="G272" s="2" t="inlineStr"><is><t>trójpierścieniowe leki przeciwdepresyjne – wodorowęglan sodu</t></is></c><c r="H272" s="2" t="inlineStr"><is><t>żelazo - deferoksamina</t></is></c><c r="I272" s="2" t="inlineStr"><is><t>warfaryna - fitomenadion</t></is></c><c r="J272" s="2" t="inlineStr" /><c r="K272" s="2" t="inlineStr" /><c r="L272" s="2" t="inlineStr" /><c r="M272" s="2" t="inlineStr" /><c r="N272" s="2" t="inlineStr" /><c r="O272" s="2" t="inlineStr" /><c r="P272" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q272" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="273"><c r="A273" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B273" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C273" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D273" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E273" s="2" t="inlineStr"><is><t>Wazodylatacyjny mechanizm działania azotanów zależy od:</t></is></c><c r="F273" s="2" t="inlineStr"><is><t>wzrostu stężenia cGMP</t></is></c><c r="G273" s="2" t="inlineStr"><is><t>defosforylacji łańcuchów lekkich miozyny</t></is></c><c r="H273" s="2" t="inlineStr" /><c r="I273" s="2" t="inlineStr" /><c r="J273" s="2" t="inlineStr" /><c r="K273" s="2" t="inlineStr"><is><t>hamowania aktywności cyklazy guanylowej</t></is></c><c r="L273" s="2" t="inlineStr"><is><t>pobudzania kanałów potasowych</t></is></c><c r="M273" s="2" t="inlineStr" /><c r="N273" s="2" t="inlineStr" /><c r="O273" s="2" t="inlineStr" /><c r="P273" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q273" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="274"><c r="A274" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B274" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C274" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D274" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E274" s="2" t="inlineStr"><is><t>Bradykardia może wystąpić po zastosowaniu:</t></is></c><c r="F274" s="2" t="inlineStr"><is><t>werapamilu</t></is></c><c r="G274" s="2" t="inlineStr" /><c r="H274" s="2" t="inlineStr" /><c r="I274" s="2" t="inlineStr" /><c r="J274" s="2" t="inlineStr" /><c r="K274" s="2" t="inlineStr"><is><t>nifedypiny</t></is></c><c r="L274" s="2" t="inlineStr"><is><t>trimetazydyny</t></is></c><c r="M274" s="2" t="inlineStr"><is><t>spironolaktonu</t></is></c><c r="N274" s="2" t="inlineStr" /><c r="O274" s="2" t="inlineStr" /><c r="P274" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q274" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="275"><c r="A275" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B275" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C275" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D275" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E275" s="2" t="inlineStr"><is><t>Teoretyczną przesłanką stosowania beta-adrenolityków w chorobie wieńcowej serca jest:</t></is></c><c r="F275" s="2" t="inlineStr"><is><t>usprawnienie metabolizmu kardiomiocytów</t></is></c><c r="G275" s="2" t="inlineStr"><is><t>zapobieganie proarytmicznemu działaniu katecholamin</t></is></c><c r="H275" s="2" t="inlineStr"><is><t>poprawa perfuzji warstwy podwsierdziowej</t></is></c><c r="I275" s="2" t="inlineStr"><is><t>korzystny wpływ hemodynamiczny zmniejszający zapotrzebowanie mięśnia sercowego na tlen</t></is></c><c r="J275" s="2" t="inlineStr" /><c r="K275" s="2" t="inlineStr" /><c r="L275" s="2" t="inlineStr" /><c r="M275" s="2" t="inlineStr" /><c r="N275" s="2" t="inlineStr" /><c r="O275" s="2" t="inlineStr" /><c r="P275" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q275" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="276"><c r="A276" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B276" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C276" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D276" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E276" s="2" t="inlineStr"><is><t>Do leków stosowanych w leczeniu nadciśnienia tętniczego ze wskazań naglących (RR&gt;180/120 mmHg z powikłaniami narządowymi) należą:</t></is></c><c r="F276" s="2" t="inlineStr"><is><t>esmolol</t></is></c><c r="G276" s="2" t="inlineStr"><is><t>urapidyl</t></is></c><c r="H276" s="2" t="inlineStr" /><c r="I276" s="2" t="inlineStr" /><c r="J276" s="2" t="inlineStr" /><c r="K276" s="2" t="inlineStr"><is><t>doksazosyna</t></is></c><c r="L276" s="2" t="inlineStr"><is><t>kaptopryl</t></is></c><c r="M276" s="2" t="inlineStr" /><c r="N276" s="2" t="inlineStr" /><c r="O276" s="2" t="inlineStr" /><c r="P276" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q276" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="277"><c r="A277" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B277" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C277" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D277" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E277" s="2" t="inlineStr"><is><t>Do leków zmniejszających ryzyko zgonu sercowo-naczyniowego w przebiegu skurczowej niewydolności serca należy:</t></is></c><c r="F277" s="2" t="inlineStr"><is><t>bisoprolol</t></is></c><c r="G277" s="2" t="inlineStr"><is><t>eplerenon</t></is></c><c r="H277" s="2" t="inlineStr"><is><t>sakubitril w skojarzeniu z walsartanem</t></is></c><c r="I277" s="2" t="inlineStr" /><c r="J277" s="2" t="inlineStr" /><c r="K277" s="2" t="inlineStr"><is><t>digoksyna</t></is></c><c r="L277" s="2" t="inlineStr" /><c r="M277" s="2" t="inlineStr" /><c r="N277" s="2" t="inlineStr" /><c r="O277" s="2" t="inlineStr" /><c r="P277" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q277" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="278"><c r="A278" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B278" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C278" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D278" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E278" s="2" t="inlineStr"><is><t>U 67-letniej kobiety z dyskomfortem zamostkowym występującym przy wchodzeniu na 3 piętro i ustępującym w spoczynku, z blokiem przedsionkowo-komorowym II stopnia typu Mobitza w badaniu met. Holtera należy zastosować:</t></is></c><c r="F278" s="2" t="inlineStr"><is><t>rosuwastatynę</t></is></c><c r="G278" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="H278" s="2" t="inlineStr"><is><t>triazotan glicerolu w aerozolu</t></is></c><c r="I278" s="2" t="inlineStr" /><c r="J278" s="2" t="inlineStr" /><c r="K278" s="2" t="inlineStr"><is><t>nebiwolol</t></is></c><c r="L278" s="2" t="inlineStr" /><c r="M278" s="2" t="inlineStr" /><c r="N278" s="2" t="inlineStr" /><c r="O278" s="2" t="inlineStr" /><c r="P278" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q278" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="279"><c r="A279" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B279" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C279" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D279" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E279" s="2" t="inlineStr"><is><t>Wskaż prawidłowe zasady prowadzenia terapii monitorowanej stężeniami leku:</t></is></c><c r="F279" s="2" t="inlineStr"><is><t>oznaczenia należy wykonywać po osiągnięciu przez lek stanu stacjonarnego</t></is></c><c r="G279" s="2" t="inlineStr"><is><t>pomiary należy wykonywać w momencie Cmin, czyli tuż przed podaniem kolejnej, zwykle porannej dawki leku</t></is></c><c r="H279" s="2" t="inlineStr"><is><t>w większości przypadków wystarczy oznaczenie całkowitego stężenia leku</t></is></c><c r="I279" s="2" t="inlineStr"><is><t>w przypadku leków o kinetyce liniowej można wyliczyć modyfikację dawki na podstawie pomiarów aktualnych i znajomości docelowych stężeń leku we krwi</t></is></c><c r="J279" s="2" t="inlineStr" /><c r="K279" s="2" t="inlineStr" /><c r="L279" s="2" t="inlineStr" /><c r="M279" s="2" t="inlineStr" /><c r="N279" s="2" t="inlineStr" /><c r="O279" s="2" t="inlineStr" /><c r="P279" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q279" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="280"><c r="A280" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B280" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C280" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D280" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E280" s="2" t="inlineStr"><is><t>W celu oceny działań niepożądanych w trakcie leczenia atorwastatyną należy sprawdzić:</t></is></c><c r="F280" s="2" t="inlineStr"><is><t>aktywność kinazy fosfokreatynowej (CPK)</t></is></c><c r="G280" s="2" t="inlineStr"><is><t>aktywność enzymów wątrobowych (AST/ALT)</t></is></c><c r="H280" s="2" t="inlineStr" /><c r="I280" s="2" t="inlineStr" /><c r="J280" s="2" t="inlineStr" /><c r="K280" s="2" t="inlineStr"><is><t>stężenie glukozy</t></is></c><c r="L280" s="2" t="inlineStr"><is><t>stężenie peptydu natriuretycznego typu B (BNP)</t></is></c><c r="M280" s="2" t="inlineStr" /><c r="N280" s="2" t="inlineStr" /><c r="O280" s="2" t="inlineStr" /><c r="P280" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q280" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="281"><c r="A281" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B281" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C281" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D281" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E281" s="2" t="inlineStr"><is><t>W leczeniu zagrażającej życiu hiperkaliemii można zastosować:</t></is></c><c r="F281" s="2" t="inlineStr"><is><t>10 ml 10% chlorku lub glukonianu wapnia i.v. w 10 min bolusie</t></is></c><c r="G281" s="2" t="inlineStr"><is><t>500 ml 20% glukozy z 20 j.m. insuliny krótkodziałającej i.v. przez 1-2 godziny</t></is></c><c r="H281" s="2" t="inlineStr"><is><t>hemodializę</t></is></c><c r="I281" s="2" t="inlineStr" /><c r="J281" s="2" t="inlineStr" /><c r="K281" s="2" t="inlineStr"><is><t>diuretyki pętlowe i.v</t></is></c><c r="L281" s="2" t="inlineStr" /><c r="M281" s="2" t="inlineStr" /><c r="N281" s="2" t="inlineStr" /><c r="O281" s="2" t="inlineStr" /><c r="P281" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q281" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="282"><c r="A282" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B282" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C282" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D282" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E282" s="2" t="inlineStr"><is><t>Powinowactwo do receptorów alfa-1-adrenergicznych wykazuje:</t></is></c><c r="F282" s="2" t="inlineStr"><is><t>doksazosyna</t></is></c><c r="G282" s="2" t="inlineStr"><is><t>labetalol</t></is></c><c r="H282" s="2" t="inlineStr"><is><t>adrenalina</t></is></c><c r="I282" s="2" t="inlineStr"><is><t>karwedilol</t></is></c><c r="J282" s="2" t="inlineStr" /><c r="K282" s="2" t="inlineStr" /><c r="L282" s="2" t="inlineStr" /><c r="M282" s="2" t="inlineStr" /><c r="N282" s="2" t="inlineStr" /><c r="O282" s="2" t="inlineStr" /><c r="P282" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q282" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="283"><c r="A283" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B283" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C283" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D283" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E283" s="2" t="inlineStr"><is><t>Apiksaban jest substratem dla P-gp. Co to oznacza?</t></is></c><c r="F283" s="2" t="inlineStr"><is><t>silne induktory P-gp o działaniu ogólnoustrojowym zmniejszają skuteczność apiksabanu</t></is></c><c r="G283" s="2" t="inlineStr" /><c r="H283" s="2" t="inlineStr" /><c r="I283" s="2" t="inlineStr" /><c r="J283" s="2" t="inlineStr" /><c r="K283" s="2" t="inlineStr"><is><t>lek jest wchłaniany z p. pokarmowego z wykorzystaniem transportu ułatwionego</t></is></c><c r="L283" s="2" t="inlineStr"><is><t>jest metabolizowany w wątrobie i nie powinien być stosowany u osób z 10- 15 pkt wg skali Childa-Pugha</t></is></c><c r="M283" s="2" t="inlineStr"><is><t>jest prawdopodobne, że hemodializa byłaby skutecznym środkiem zaradczym podczas przedawkowania apiksabanu</t></is></c><c r="N283" s="2" t="inlineStr" /><c r="O283" s="2" t="inlineStr" /><c r="P283" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q283" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="284"><c r="A284" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B284" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C284" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D284" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E284" s="2" t="inlineStr"><is><t>Opis rzedowości procesu:</t></is></c><c r="F284" s="2" t="inlineStr"><is><t>Dotyczy wszystkich etapów farmakokinetycznych</t></is></c><c r="G284" s="2" t="inlineStr"><is><t>Definiuje dynamiki zmian w układzie stężenie-czas w zależności od budowy chemicznej leku</t></is></c><c r="H284" s="2" t="inlineStr"><is><t>Może się zmienić dla leku w trakcie pojedynczej ekspozycji</t></is></c><c r="I284" s="2" t="inlineStr"><is><t>Powstaje ostatecznie w badaniach w medelu zwierzęcym</t></is></c><c r="J284" s="2" t="inlineStr" /><c r="K284" s="2" t="inlineStr" /><c r="L284" s="2" t="inlineStr" /><c r="M284" s="2" t="inlineStr" /><c r="N284" s="2" t="inlineStr" /><c r="O284" s="2" t="inlineStr" /><c r="P284" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q284" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="285"><c r="A285" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B285" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C285" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D285" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E285" s="2" t="inlineStr"><is><t>Jeśli proces eliminacji leku przez nerki jest opisany kinetyką zerowego rzędu to:</t></is></c><c r="F285" s="2" t="inlineStr"><is><t>Procesy wchłaniania i dystrybucji również opisane są kinetyką zerowego rzędu</t></is></c><c r="G285" s="2" t="inlineStr"><is><t>Szybkość procesu eliminacji nerkowej jest stała</t></is></c><c r="H285" s="2" t="inlineStr" /><c r="I285" s="2" t="inlineStr" /><c r="J285" s="2" t="inlineStr" /><c r="K285" s="2" t="inlineStr"><is><t>Stężenie leku w moczu jest odwrotnie proporocjonalne do stężenia leku we krwi</t></is></c><c r="L285" s="2" t="inlineStr"><is><t>Klirens nerkowy leku jest wprost proporcjonalny do stężeniu leku</t></is></c><c r="M285" s="2" t="inlineStr" /><c r="N285" s="2" t="inlineStr" /><c r="O285" s="2" t="inlineStr" /><c r="P285" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q285" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="286"><c r="A286" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B286" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C286" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D286" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E286" s="2" t="inlineStr"><is><t>Wskaż właściwie zdefiniowane parametry farmakokinetyczne</t></is></c><c r="F286" s="2" t="inlineStr"><is><t>AUC – pole pod krzywą zmian stężenia leku we krwi w czasie</t></is></c><c r="G286" s="2" t="inlineStr" /><c r="H286" s="2" t="inlineStr" /><c r="I286" s="2" t="inlineStr" /><c r="J286" s="2" t="inlineStr" /><c r="K286" s="2" t="inlineStr"><is><t>T1/2 – czas po którym stężenie leku we krwi jest równe stężeniu leku gdyby biodostępność wynosiła 50%</t></is></c><c r="L286" s="2" t="inlineStr"><is><t>Tmax – maksymalny czas w którym stężeniu leku we krwi jest wykrywalne</t></is></c><c r="M286" s="2" t="inlineStr"><is><t>Cmax – stężenie leku we krwi osiągane po podaniu dożylnym</t></is></c><c r="N286" s="2" t="inlineStr" /><c r="O286" s="2" t="inlineStr" /><c r="P286" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q286" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="287"><c r="A287" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B287" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C287" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D287" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E287" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie antybiotyk – mechanizm działania</t></is></c><c r="F287" s="2" t="inlineStr"><is><t>Trimetoprim – zaburzenia kwasu foliowego</t></is></c><c r="G287" s="2" t="inlineStr"><is><t>Amikacyna – hamowanie syntezy białek</t></is></c><c r="H287" s="2" t="inlineStr"><is><t>Cyprofloksacyna – hamowanie replikacji DNA</t></is></c><c r="I287" s="2" t="inlineStr" /><c r="J287" s="2" t="inlineStr" /><c r="K287" s="2" t="inlineStr"><is><t>Klindamycyna – hamowanie transkrypcji genów translacji</t></is></c><c r="L287" s="2" t="inlineStr" /><c r="M287" s="2" t="inlineStr" /><c r="N287" s="2" t="inlineStr" /><c r="O287" s="2" t="inlineStr" /><c r="P287" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q287" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="288"><c r="A288" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B288" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C288" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D288" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E288" s="2" t="inlineStr"><is><t>Azytromycyna</t></is></c><c r="F288" s="2" t="inlineStr"><is><t>Kumuluje się w makrofagach</t></is></c><c r="G288" s="2" t="inlineStr"><is><t>Ma długi okres półtrwania</t></is></c><c r="H288" s="2" t="inlineStr" /><c r="I288" s="2" t="inlineStr" /><c r="J288" s="2" t="inlineStr" /><c r="K288" s="2" t="inlineStr"><is><t>Słabo wchłania się z PP</t></is></c><c r="L288" s="2" t="inlineStr"><is><t>Hamuje enzymy cytochromu P-450</t></is></c><c r="M288" s="2" t="inlineStr" /><c r="N288" s="2" t="inlineStr" /><c r="O288" s="2" t="inlineStr" /><c r="P288" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q288" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="289"><c r="A289" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B289" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C289" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D289" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E289" s="2" t="inlineStr"><is><t>Działanie ototoksyczne wskazują</t></is></c><c r="F289" s="2" t="inlineStr"><is><t>Salicylany</t></is></c><c r="G289" s="2" t="inlineStr"><is><t>Aminoglikozydy</t></is></c><c r="H289" s="2" t="inlineStr" /><c r="I289" s="2" t="inlineStr" /><c r="J289" s="2" t="inlineStr" /><c r="K289" s="2" t="inlineStr"><is><t>Glitazony</t></is></c><c r="L289" s="2" t="inlineStr"><is><t>Penicyliny</t></is></c><c r="M289" s="2" t="inlineStr" /><c r="N289" s="2" t="inlineStr" /><c r="O289" s="2" t="inlineStr" /><c r="P289" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q289" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="290"><c r="A290" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B290" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C290" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D290" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E290" s="2" t="inlineStr"><is><t>W leczeniu boreliozy można użyć</t></is></c><c r="F290" s="2" t="inlineStr"><is><t>Amoksycyliny</t></is></c><c r="G290" s="2" t="inlineStr"><is><t>Cefuroksymu aksetylu</t></is></c><c r="H290" s="2" t="inlineStr"><is><t>Azytromycyny</t></is></c><c r="I290" s="2" t="inlineStr"><is><t>Doksycykliny</t></is></c><c r="J290" s="2" t="inlineStr" /><c r="K290" s="2" t="inlineStr" /><c r="L290" s="2" t="inlineStr" /><c r="M290" s="2" t="inlineStr" /><c r="N290" s="2" t="inlineStr" /><c r="O290" s="2" t="inlineStr" /><c r="P290" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q290" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="291"><c r="A291" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B291" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C291" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D291" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E291" s="2" t="inlineStr"><is><t>Syntezę ściany komórkowej hamuje:</t></is></c><c r="F291" s="2" t="inlineStr"><is><t>Kaspofungina</t></is></c><c r="G291" s="2" t="inlineStr"><is><t>Imipenem</t></is></c><c r="H291" s="2" t="inlineStr" /><c r="I291" s="2" t="inlineStr" /><c r="J291" s="2" t="inlineStr" /><c r="K291" s="2" t="inlineStr"><is><t>Nystatyna</t></is></c><c r="L291" s="2" t="inlineStr"><is><t>Tygecyklina</t></is></c><c r="M291" s="2" t="inlineStr" /><c r="N291" s="2" t="inlineStr" /><c r="O291" s="2" t="inlineStr" /><c r="P291" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q291" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="292"><c r="A292" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B292" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C292" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D292" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E292" s="2" t="inlineStr"><is><t>Reakcje disulfiramową może spowodować spożycie alkoholu podczas terapii</t></is></c><c r="F292" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="G292" s="2" t="inlineStr" /><c r="H292" s="2" t="inlineStr" /><c r="I292" s="2" t="inlineStr" /><c r="J292" s="2" t="inlineStr" /><c r="K292" s="2" t="inlineStr"><is><t>Klindamycyną</t></is></c><c r="L292" s="2" t="inlineStr"><is><t>Piperalicyna</t></is></c><c r="M292" s="2" t="inlineStr"><is><t>Cyprofloksacyna</t></is></c><c r="N292" s="2" t="inlineStr" /><c r="O292" s="2" t="inlineStr" /><c r="P292" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q292" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="293"><c r="A293" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B293" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C293" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D293" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E293" s="2" t="inlineStr"><is><t>W zakażeniach Mycoplasama pneumoniae można zastosować</t></is></c><c r="F293" s="2" t="inlineStr"><is><t>Doksycykline</t></is></c><c r="G293" s="2" t="inlineStr"><is><t>Klarytromycyne</t></is></c><c r="H293" s="2" t="inlineStr" /><c r="I293" s="2" t="inlineStr" /><c r="J293" s="2" t="inlineStr" /><c r="K293" s="2" t="inlineStr"><is><t>Amoksycyline</t></is></c><c r="L293" s="2" t="inlineStr"><is><t>Ceftriakson</t></is></c><c r="M293" s="2" t="inlineStr" /><c r="N293" s="2" t="inlineStr" /><c r="O293" s="2" t="inlineStr" /><c r="P293" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q293" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="294"><c r="A294" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B294" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C294" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D294" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E294" s="2" t="inlineStr"><is><t>Makrolidy mogą być skuteczne w zakażeniach</t></is></c><c r="F294" s="2" t="inlineStr"><is><t>H. influenza</t></is></c><c r="G294" s="2" t="inlineStr"><is><t>L. pneumophila</t></is></c><c r="H294" s="2" t="inlineStr"><is><t>H. pylori</t></is></c><c r="I294" s="2" t="inlineStr"><is><t>T. gondi</t></is></c><c r="J294" s="2" t="inlineStr" /><c r="K294" s="2" t="inlineStr" /><c r="L294" s="2" t="inlineStr" /><c r="M294" s="2" t="inlineStr" /><c r="N294" s="2" t="inlineStr" /><c r="O294" s="2" t="inlineStr" /><c r="P294" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q294" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="295"><c r="A295" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B295" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C295" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D295" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E295" s="2" t="inlineStr"><is><t>W zakazeniu Clostridium diff. skuteczne sa:</t></is></c><c r="F295" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="G295" s="2" t="inlineStr"><is><t>Wankomycyna</t></is></c><c r="H295" s="2" t="inlineStr" /><c r="I295" s="2" t="inlineStr" /><c r="J295" s="2" t="inlineStr" /><c r="K295" s="2" t="inlineStr"><is><t>Amoksycylina</t></is></c><c r="L295" s="2" t="inlineStr"><is><t>Klindamycyna</t></is></c><c r="M295" s="2" t="inlineStr" /><c r="N295" s="2" t="inlineStr" /><c r="O295" s="2" t="inlineStr" /><c r="P295" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q295" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="296"><c r="A296" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B296" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C296" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D296" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E296" s="2" t="inlineStr"><is><t>Na MRSA działa</t></is></c><c r="F296" s="2" t="inlineStr"><is><t>Wankomycyna</t></is></c><c r="G296" s="2" t="inlineStr"><is><t>Linezolid</t></is></c><c r="H296" s="2" t="inlineStr" /><c r="I296" s="2" t="inlineStr" /><c r="J296" s="2" t="inlineStr" /><c r="K296" s="2" t="inlineStr"><is><t>Cefazolina</t></is></c><c r="L296" s="2" t="inlineStr"><is><t>Meropenem</t></is></c><c r="M296" s="2" t="inlineStr" /><c r="N296" s="2" t="inlineStr" /><c r="O296" s="2" t="inlineStr" /><c r="P296" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q296" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="297"><c r="A297" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B297" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C297" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D297" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E297" s="2" t="inlineStr"><is><t>Zagrożenia dla płodu jest mało prawdopodobne po</t></is></c><c r="F297" s="2" t="inlineStr"><is><t>Amoksycyliny z kwasem klawulanowym</t></is></c><c r="G297" s="2" t="inlineStr"><is><t>Erytromycyny</t></is></c><c r="H297" s="2" t="inlineStr"><is><t>Cefuroksymu</t></is></c><c r="I297" s="2" t="inlineStr" /><c r="J297" s="2" t="inlineStr" /><c r="K297" s="2" t="inlineStr"><is><t>Amikacyny</t></is></c><c r="L297" s="2" t="inlineStr" /><c r="M297" s="2" t="inlineStr" /><c r="N297" s="2" t="inlineStr" /><c r="O297" s="2" t="inlineStr" /><c r="P297" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q297" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="298"><c r="A298" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B298" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C298" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D298" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E298" s="2" t="inlineStr"><is><t>Ketokonazol</t></is></c><c r="F298" s="2" t="inlineStr"><is><t>Jest dostępny w postaci szamponu</t></is></c><c r="G298" s="2" t="inlineStr"><is><t>Ma zostosowanie w zespole Cushinga</t></is></c><c r="H298" s="2" t="inlineStr"><is><t>Wykazuje działanie hepatotoksyczne</t></is></c><c r="I298" s="2" t="inlineStr" /><c r="J298" s="2" t="inlineStr" /><c r="K298" s="2" t="inlineStr"><is><t>Nie wchłania się po podaniu doustnym</t></is></c><c r="L298" s="2" t="inlineStr" /><c r="M298" s="2" t="inlineStr" /><c r="N298" s="2" t="inlineStr" /><c r="O298" s="2" t="inlineStr" /><c r="P298" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q298" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="299"><c r="A299" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B299" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C299" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D299" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E299" s="2" t="inlineStr"><is><t>Do leków i rzutu w gruźlicy należy</t></is></c><c r="F299" s="2" t="inlineStr"><is><t>Ryfampicyna</t></is></c><c r="G299" s="2" t="inlineStr"><is><t>Izoniazyd</t></is></c><c r="H299" s="2" t="inlineStr"><is><t>Pyryzynamid</t></is></c><c r="I299" s="2" t="inlineStr" /><c r="J299" s="2" t="inlineStr" /><c r="K299" s="2" t="inlineStr"><is><t>Kanamycna</t></is></c><c r="L299" s="2" t="inlineStr" /><c r="M299" s="2" t="inlineStr" /><c r="N299" s="2" t="inlineStr" /><c r="O299" s="2" t="inlineStr" /><c r="P299" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q299" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="300"><c r="A300" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B300" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C300" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D300" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E300" s="2" t="inlineStr"><is><t>W farmakoterapii silnego bólu przebijającego stosujemy</t></is></c><c r="F300" s="2" t="inlineStr"><is><t>Morfinę doustnie w dawkach ratunkowych</t></is></c><c r="G300" s="2" t="inlineStr"><is><t>Fentanyl w postaci dopoliczkowej</t></is></c><c r="H300" s="2" t="inlineStr"><is><t>Buprenorfinę podjęzykowo</t></is></c><c r="I300" s="2" t="inlineStr"><is><t>Fentanyl w postaci donosowej</t></is></c><c r="J300" s="2" t="inlineStr" /><c r="K300" s="2" t="inlineStr" /><c r="L300" s="2" t="inlineStr" /><c r="M300" s="2" t="inlineStr" /><c r="N300" s="2" t="inlineStr" /><c r="O300" s="2" t="inlineStr" /><c r="P300" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q300" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="301"><c r="A301" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B301" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C301" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D301" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E301" s="2" t="inlineStr"><is><t>Ośrodkowe działania opioidów obejmują</t></is></c><c r="F301" s="2" t="inlineStr"><is><t>Działanie przeciwkaszlowe</t></is></c><c r="G301" s="2" t="inlineStr"><is><t>Wymioty</t></is></c><c r="H301" s="2" t="inlineStr" /><c r="I301" s="2" t="inlineStr" /><c r="J301" s="2" t="inlineStr" /><c r="K301" s="2" t="inlineStr"><is><t>Zwiększenie ciśnienia w drogach żółciowych</t></is></c><c r="L301" s="2" t="inlineStr"><is><t>Zaparcia</t></is></c><c r="M301" s="2" t="inlineStr" /><c r="N301" s="2" t="inlineStr" /><c r="O301" s="2" t="inlineStr" /><c r="P301" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q301" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="302"><c r="A302" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B302" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C302" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D302" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E302" s="2" t="inlineStr"><is><t>Efekt pułapowy wykazuje</t></is></c><c r="F302" s="2" t="inlineStr"><is><t>Buprenorfina</t></is></c><c r="G302" s="2" t="inlineStr" /><c r="H302" s="2" t="inlineStr" /><c r="I302" s="2" t="inlineStr" /><c r="J302" s="2" t="inlineStr" /><c r="K302" s="2" t="inlineStr"><is><t>Morfina</t></is></c><c r="L302" s="2" t="inlineStr"><is><t>Kodeina</t></is></c><c r="M302" s="2" t="inlineStr"><is><t>Metadon</t></is></c><c r="N302" s="2" t="inlineStr" /><c r="O302" s="2" t="inlineStr" /><c r="P302" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q302" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="303"><c r="A303" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B303" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C303" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D303" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E303" s="2" t="inlineStr"><is><t>Metformina</t></is></c><c r="F303" s="2" t="inlineStr"><is><t>Zaburza wchłanianie witaminy B12</t></is></c><c r="G303" s="2" t="inlineStr"><is><t>Może powodować kwasicę metaboliczną</t></is></c><c r="H303" s="2" t="inlineStr" /><c r="I303" s="2" t="inlineStr" /><c r="J303" s="2" t="inlineStr" /><c r="K303" s="2" t="inlineStr"><is><t>Stymuluje wydzielanie insuliny</t></is></c><c r="L303" s="2" t="inlineStr"><is><t>Powoduje przyrost masy ciała</t></is></c><c r="M303" s="2" t="inlineStr" /><c r="N303" s="2" t="inlineStr" /><c r="O303" s="2" t="inlineStr" /><c r="P303" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q303" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="304"><c r="A304" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B304" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C304" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D304" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E304" s="2" t="inlineStr"><is><t>Szybkie analogi insuliny</t></is></c><c r="F304" s="2" t="inlineStr"><is><t>Lispro</t></is></c><c r="G304" s="2" t="inlineStr"><is><t>Aspart</t></is></c><c r="H304" s="2" t="inlineStr" /><c r="I304" s="2" t="inlineStr" /><c r="J304" s="2" t="inlineStr" /><c r="K304" s="2" t="inlineStr"><is><t>Glargina</t></is></c><c r="L304" s="2" t="inlineStr"><is><t>Detemir</t></is></c><c r="M304" s="2" t="inlineStr" /><c r="N304" s="2" t="inlineStr" /><c r="O304" s="2" t="inlineStr" /><c r="P304" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q304" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="305"><c r="A305" s="2" t="inlineStr"><is><t>ANTYKONCEPCJA</t></is></c><c r="B305" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C305" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D305" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E305" s="2" t="inlineStr"><is><t>Działania niepożądane hormonalnych środków antykoncepcyjnych z powodu obecności gestagenu</t></is></c><c r="F305" s="2" t="inlineStr"><is><t>Przyrost masy ciała</t></is></c><c r="G305" s="2" t="inlineStr"><is><t>Obniżenie libido</t></is></c><c r="H305" s="2" t="inlineStr"><is><t>Depresja</t></is></c><c r="I305" s="2" t="inlineStr"><is><t>Hirsutyzm</t></is></c><c r="J305" s="2" t="inlineStr" /><c r="K305" s="2" t="inlineStr" /><c r="L305" s="2" t="inlineStr" /><c r="M305" s="2" t="inlineStr" /><c r="N305" s="2" t="inlineStr" /><c r="O305" s="2" t="inlineStr" /><c r="P305" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q305" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="306"><c r="A306" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B306" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C306" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D306" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E306" s="2" t="inlineStr"><is><t>Hiperprolaktynemia</t></is></c><c r="F306" s="2" t="inlineStr"><is><t>Karbegolina</t></is></c><c r="G306" s="2" t="inlineStr"><is><t>Bromokryptyna</t></is></c><c r="H306" s="2" t="inlineStr" /><c r="I306" s="2" t="inlineStr" /><c r="J306" s="2" t="inlineStr" /><c r="K306" s="2" t="inlineStr"><is><t>Gorserelina</t></is></c><c r="L306" s="2" t="inlineStr"><is><t>Finasteryd</t></is></c><c r="M306" s="2" t="inlineStr" /><c r="N306" s="2" t="inlineStr" /><c r="O306" s="2" t="inlineStr" /><c r="P306" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q306" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="307"><c r="A307" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B307" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C307" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D307" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E307" s="2" t="inlineStr"><is><t>Terapia cukrzycy typu 2 podskórnie</t></is></c><c r="F307" s="2" t="inlineStr"><is><t>Detemir</t></is></c><c r="G307" s="2" t="inlineStr" /><c r="H307" s="2" t="inlineStr" /><c r="I307" s="2" t="inlineStr" /><c r="J307" s="2" t="inlineStr" /><c r="K307" s="2" t="inlineStr"><is><t>Glipizyd</t></is></c><c r="L307" s="2" t="inlineStr"><is><t>Liraglutyd</t></is></c><c r="M307" s="2" t="inlineStr"><is><t>Linagliptyna</t></is></c><c r="N307" s="2" t="inlineStr" /><c r="O307" s="2" t="inlineStr" /><c r="P307" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q307" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="308"><c r="A308" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B308" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C308" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D308" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E308" s="2" t="inlineStr"><is><t>Terapia nadczynności tarczycy</t></is></c><c r="F308" s="2" t="inlineStr"><is><t>Jod radioaktywny</t></is></c><c r="G308" s="2" t="inlineStr"><is><t>Bisoprolol</t></is></c><c r="H308" s="2" t="inlineStr"><is><t>Tiamazol</t></is></c><c r="I308" s="2" t="inlineStr"><is><t>Propylotiouracyl</t></is></c><c r="J308" s="2" t="inlineStr" /><c r="K308" s="2" t="inlineStr" /><c r="L308" s="2" t="inlineStr" /><c r="M308" s="2" t="inlineStr" /><c r="N308" s="2" t="inlineStr" /><c r="O308" s="2" t="inlineStr" /><c r="P308" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q308" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="309"><c r="A309" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B309" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C309" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D309" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E309" s="2" t="inlineStr"><is><t>Podczas terapii GKS może dojsć do pogorszenia przebiegu</t></is></c><c r="F309" s="2" t="inlineStr"><is><t>Cukrzycy</t></is></c><c r="G309" s="2" t="inlineStr"><is><t>Gruźlicy</t></is></c><c r="H309" s="2" t="inlineStr"><is><t>Osteoporozy</t></is></c><c r="I309" s="2" t="inlineStr" /><c r="J309" s="2" t="inlineStr" /><c r="K309" s="2" t="inlineStr"><is><t>Małopłytkowości idiopatycznej</t></is></c><c r="L309" s="2" t="inlineStr" /><c r="M309" s="2" t="inlineStr" /><c r="N309" s="2" t="inlineStr" /><c r="O309" s="2" t="inlineStr" /><c r="P309" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q309" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="310"><c r="A310" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B310" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C310" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D310" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E310" s="2" t="inlineStr"><is><t>Wzrostu ryzyka sercowo-naczyniowego NIE powoduje</t></is></c><c r="F310" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="G310" s="2" t="inlineStr" /><c r="H310" s="2" t="inlineStr" /><c r="I310" s="2" t="inlineStr" /><c r="J310" s="2" t="inlineStr" /><c r="K310" s="2" t="inlineStr"><is><t>Celekoksyb</t></is></c><c r="L310" s="2" t="inlineStr"><is><t>Indometacyna</t></is></c><c r="M310" s="2" t="inlineStr"><is><t>Ketoprofen</t></is></c><c r="N310" s="2" t="inlineStr" /><c r="O310" s="2" t="inlineStr" /><c r="P310" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q310" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="311"><c r="A311" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B311" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C311" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D311" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E311" s="2" t="inlineStr"><is><t>Zmniejszenie ryzyka gastrotoksyczności NLPZ – co możemy</t></is></c><c r="F311" s="2" t="inlineStr"><is><t>Analogi PGE1</t></is></c><c r="G311" s="2" t="inlineStr"><is><t>IPP</t></is></c><c r="H311" s="2" t="inlineStr" /><c r="I311" s="2" t="inlineStr" /><c r="J311" s="2" t="inlineStr" /><c r="K311" s="2" t="inlineStr"><is><t>GKS</t></is></c><c r="L311" s="2" t="inlineStr"><is><t>Preparaty o wybiórczym powinowactwie do COX1</t></is></c><c r="M311" s="2" t="inlineStr" /><c r="N311" s="2" t="inlineStr" /><c r="O311" s="2" t="inlineStr" /><c r="P311" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q311" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="312"><c r="A312" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B312" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C312" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D312" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E312" s="2" t="inlineStr"><is><t>Paracetamol</t></is></c><c r="F312" s="2" t="inlineStr"><is><t>Jest metabolizowany przez enzymy cytochromu P-450</t></is></c><c r="G312" s="2" t="inlineStr" /><c r="H312" s="2" t="inlineStr" /><c r="I312" s="2" t="inlineStr" /><c r="J312" s="2" t="inlineStr" /><c r="K312" s="2" t="inlineStr"><is><t>Działa silnie przeciwzapalnie</t></is></c><c r="L312" s="2" t="inlineStr"><is><t>Hamuje COX2 w OUN</t></is></c><c r="M312" s="2" t="inlineStr"><is><t>Wykazuje działanie gastrotoksyczne</t></is></c><c r="N312" s="2" t="inlineStr" /><c r="O312" s="2" t="inlineStr" /><c r="P312" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q312" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="313"><c r="A313" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B313" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C313" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D313" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E313" s="2" t="inlineStr"><is><t>Leki immunosupresyjne</t></is></c><c r="F313" s="2" t="inlineStr"><is><t>Powodują upośledzenie odporności komórkowej</t></is></c><c r="G313" s="2" t="inlineStr"><is><t>Są lekami o wąskim wskaźniku terapeutycznym</t></is></c><c r="H313" s="2" t="inlineStr" /><c r="I313" s="2" t="inlineStr" /><c r="J313" s="2" t="inlineStr" /><c r="K313" s="2" t="inlineStr"><is><t>Zapobiegają rozwojowi nowotworów</t></is></c><c r="L313" s="2" t="inlineStr"><is><t>Znajdują zastosowanie w terapii chorób neurodegeneracyjnych</t></is></c><c r="M313" s="2" t="inlineStr" /><c r="N313" s="2" t="inlineStr" /><c r="O313" s="2" t="inlineStr" /><c r="P313" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q313" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="314"><c r="A314" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B314" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C314" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D314" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E314" s="2" t="inlineStr"><is><t>Wskaż prawidłowe pary lek – wskazanie</t></is></c><c r="F314" s="2" t="inlineStr"><is><t>Bromoheksyna – astma oskrzelowa</t></is></c><c r="G314" s="2" t="inlineStr" /><c r="H314" s="2" t="inlineStr" /><c r="I314" s="2" t="inlineStr" /><c r="J314" s="2" t="inlineStr" /><c r="K314" s="2" t="inlineStr"><is><t>Acetylocysteina – ostre zapalenie zatok obocznych nosa</t></is></c><c r="L314" s="2" t="inlineStr"><is><t>Dornaza alfa – sarkoidoza</t></is></c><c r="M314" s="2" t="inlineStr"><is><t>Ambroksol – infekcyjne zaostrzenie POChP</t></is></c><c r="N314" s="2" t="inlineStr" /><c r="O314" s="2" t="inlineStr" /><c r="P314" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q314" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="315"><c r="A315" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B315" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C315" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D315" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E315" s="2" t="inlineStr"><is><t>W celu przerwania ataku duszności Zależy jakiej dusznosći. Duszności przygodnej będą same SABA, jak mamy zaostrzenie astmy to GKS też</t></is></c><c r="F315" s="2" t="inlineStr"><is><t>Fenoterol</t></is></c><c r="G315" s="2" t="inlineStr"><is><t>Salbutamol</t></is></c><c r="H315" s="2" t="inlineStr" /><c r="I315" s="2" t="inlineStr" /><c r="J315" s="2" t="inlineStr" /><c r="K315" s="2" t="inlineStr"><is><t>Salmeterol</t></is></c><c r="L315" s="2" t="inlineStr"><is><t>Flutikazon</t></is></c><c r="M315" s="2" t="inlineStr" /><c r="N315" s="2" t="inlineStr" /><c r="O315" s="2" t="inlineStr" /><c r="P315" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q315" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="316"><c r="A316" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B316" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C316" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D316" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E316" s="2" t="inlineStr"><is><t>Omalizumab</t></is></c><c r="F316" s="2" t="inlineStr"><is><t>Blokuje łączenie IgE z komórkami tucznymi</t></is></c><c r="G316" s="2" t="inlineStr"><is><t>Zmniejsza liczbę zaostrzeń astmy</t></is></c><c r="H316" s="2" t="inlineStr" /><c r="I316" s="2" t="inlineStr" /><c r="J316" s="2" t="inlineStr" /><c r="K316" s="2" t="inlineStr"><is><t>Stosowany jest w astmie o umiarkowanej ciężkości</t></is></c><c r="L316" s="2" t="inlineStr"><is><t>Zwiększa zapotrzebowanie na GKS</t></is></c><c r="M316" s="2" t="inlineStr" /><c r="N316" s="2" t="inlineStr" /><c r="O316" s="2" t="inlineStr" /><c r="P316" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q316" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="317"><c r="A317" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B317" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C317" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D317" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E317" s="2" t="inlineStr"><is><t>Farmakoterapia POChP kategoria A i B</t></is></c><c r="F317" s="2" t="inlineStr"><is><t>Krótko i długo działające cholinolityki</t></is></c><c r="G317" s="2" t="inlineStr"><is><t>Krótko i długo działające beta2 adrenomimetyki</t></is></c><c r="H317" s="2" t="inlineStr" /><c r="I317" s="2" t="inlineStr" /><c r="J317" s="2" t="inlineStr" /><c r="K317" s="2" t="inlineStr"><is><t>GKS</t></is></c><c r="L317" s="2" t="inlineStr"><is><t>Inhibitory fosfodiesterazy 4</t></is></c><c r="M317" s="2" t="inlineStr" /><c r="N317" s="2" t="inlineStr" /><c r="O317" s="2" t="inlineStr" /><c r="P317" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q317" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="318"><c r="A318" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B318" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C318" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D318" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E318" s="2" t="inlineStr"><is><t>Omeprazol</t></is></c><c r="F318" s="2" t="inlineStr"><is><t>Powoduje nieodwracalne zablokowanie pompy protonowej</t></is></c><c r="G318" s="2" t="inlineStr"><is><t>Jest inhibitorem enzymów cytochromu P-450</t></is></c><c r="H318" s="2" t="inlineStr" /><c r="I318" s="2" t="inlineStr" /><c r="J318" s="2" t="inlineStr" /><c r="K318" s="2" t="inlineStr"><is><t>Hamuje wydzielanie kwasu solnego przez 6-12h</t></is></c><c r="L318" s="2" t="inlineStr"><is><t>Jest aktywowany przez pepsynę</t></is></c><c r="M318" s="2" t="inlineStr" /><c r="N318" s="2" t="inlineStr" /><c r="O318" s="2" t="inlineStr" /><c r="P318" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q318" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="319"><c r="A319" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B319" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C319" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D319" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E319" s="2" t="inlineStr"><is><t>Metoklopramid:</t></is></c><c r="F319" s="2" t="inlineStr"><is><t>to lek przeciwwymiotny</t></is></c><c r="G319" s="2" t="inlineStr"><is><t>może spowodować hiperprolaktynemię</t></is></c><c r="H319" s="2" t="inlineStr"><is><t>to lek prokinetyczny</t></is></c><c r="I319" s="2" t="inlineStr"><is><t>może spowodować objawy pozapiramidowe</t></is></c><c r="J319" s="2" t="inlineStr" /><c r="K319" s="2" t="inlineStr" /><c r="L319" s="2" t="inlineStr" /><c r="M319" s="2" t="inlineStr" /><c r="N319" s="2" t="inlineStr" /><c r="O319" s="2" t="inlineStr" /><c r="P319" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q319" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="320"><c r="A320" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B320" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C320" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D320" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E320" s="2" t="inlineStr"><is><t>Przewlekłe zapalenie trzustki z alkoholu</t></is></c><c r="F320" s="2" t="inlineStr"><is><t>Preparaty enzymów trzustkowych</t></is></c><c r="G320" s="2" t="inlineStr"><is><t>Leki przeciwbólowe</t></is></c><c r="H320" s="2" t="inlineStr" /><c r="I320" s="2" t="inlineStr" /><c r="J320" s="2" t="inlineStr" /><c r="K320" s="2" t="inlineStr"><is><t>GKS</t></is></c><c r="L320" s="2" t="inlineStr"><is><t>Leki przeciwbakteryjne</t></is></c><c r="M320" s="2" t="inlineStr" /><c r="N320" s="2" t="inlineStr" /><c r="O320" s="2" t="inlineStr" /><c r="P320" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q320" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="321"><c r="A321" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B321" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C321" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D321" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E321" s="2" t="inlineStr"><is><t>Chory z encefalopatią wątrobową, możemy</t></is></c><c r="F321" s="2" t="inlineStr"><is><t>Asparaginian ornityny</t></is></c><c r="G321" s="2" t="inlineStr"><is><t>Laktuloza</t></is></c><c r="H321" s="2" t="inlineStr"><is><t>Ryfaksymina</t></is></c><c r="I321" s="2" t="inlineStr" /><c r="J321" s="2" t="inlineStr" /><c r="K321" s="2" t="inlineStr"><is><t>Piracetam</t></is></c><c r="L321" s="2" t="inlineStr" /><c r="M321" s="2" t="inlineStr" /><c r="N321" s="2" t="inlineStr" /><c r="O321" s="2" t="inlineStr" /><c r="P321" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q321" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="322"><c r="A322" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B322" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C322" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D322" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E322" s="2" t="inlineStr"><is><t>Schematy eradykacji H. Pylori (rekomendowane)</t></is></c><c r="F322" s="2" t="inlineStr"><is><t>Pantoprazol/cytrynian bizmutu/tetracyklina/metronidazol</t></is></c><c r="G322" s="2" t="inlineStr" /><c r="H322" s="2" t="inlineStr" /><c r="I322" s="2" t="inlineStr" /><c r="J322" s="2" t="inlineStr" /><c r="K322" s="2" t="inlineStr"><is><t>Cytrynian bizmutu/metronidazol</t></is></c><c r="L322" s="2" t="inlineStr"><is><t>Mizoprostol/metronidazol/klarytromycyna</t></is></c><c r="M322" s="2" t="inlineStr"><is><t>Ranitydyna/amoksycylina/metronidazol</t></is></c><c r="N322" s="2" t="inlineStr" /><c r="O322" s="2" t="inlineStr" /><c r="P322" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q322" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="323"><c r="A323" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B323" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C323" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D323" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E323" s="2" t="inlineStr"><is><t>Lek przeciwzakrzepowy – czas odstawienia (planowa, duże ryzyko krwawienia, nerki prawidłowe)</t></is></c><c r="F323" s="2" t="inlineStr"><is><t>Dabigatran – 1 dzień</t></is></c><c r="G323" s="2" t="inlineStr" /><c r="H323" s="2" t="inlineStr" /><c r="I323" s="2" t="inlineStr" /><c r="J323" s="2" t="inlineStr" /><c r="K323" s="2" t="inlineStr"><is><t>Warfaryna – 2 dni</t></is></c><c r="L323" s="2" t="inlineStr"><is><t>Acenokumarol – 10 dni</t></is></c><c r="M323" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy – 5 dni</t></is></c><c r="N323" s="2" t="inlineStr" /><c r="O323" s="2" t="inlineStr" /><c r="P323" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q323" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="324"><c r="A324" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B324" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C324" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D324" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E324" s="2" t="inlineStr"><is><t>Lek – monitorowanie</t></is></c><c r="F324" s="2" t="inlineStr"><is><t>Heparyna niefrakcjonowana – APTT</t></is></c><c r="G324" s="2" t="inlineStr" /><c r="H324" s="2" t="inlineStr" /><c r="I324" s="2" t="inlineStr" /><c r="J324" s="2" t="inlineStr" /><c r="K324" s="2" t="inlineStr"><is><t>Dabigatran – INR</t></is></c><c r="L324" s="2" t="inlineStr"><is><t>Acenokumarol – czas ekarynowy</t></is></c><c r="M324" s="2" t="inlineStr"><is><t>Rywaroksaban – czas trombinowy</t></is></c><c r="N324" s="2" t="inlineStr" /><c r="O324" s="2" t="inlineStr" /><c r="P324" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q324" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="325"><c r="A325" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B325" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C325" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D325" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E325" s="2" t="inlineStr"><is><t>Działanie antyagregacyjne</t></is></c><c r="F325" s="2" t="inlineStr"><is><t>Antagoniści receptorów P2Y12</t></is></c><c r="G325" s="2" t="inlineStr" /><c r="H325" s="2" t="inlineStr" /><c r="I325" s="2" t="inlineStr" /><c r="J325" s="2" t="inlineStr" /><c r="K325" s="2" t="inlineStr"><is><t>Agoniści receptorów GP IIb/IIIa</t></is></c><c r="L325" s="2" t="inlineStr"><is><t>Inhibitory COX2</t></is></c><c r="M325" s="2" t="inlineStr"><is><t>Agoniści receptorów TXA2</t></is></c><c r="N325" s="2" t="inlineStr" /><c r="O325" s="2" t="inlineStr" /><c r="P325" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q325" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="326"><c r="A326" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B326" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C326" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D326" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E326" s="2" t="inlineStr"><is><t>Zahamowanie agregacji płytek zależne od ADP po</t></is></c><c r="F326" s="2" t="inlineStr"><is><t>Klopidogrelu</t></is></c><c r="G326" s="2" t="inlineStr"><is><t>Tikagreloru</t></is></c><c r="H326" s="2" t="inlineStr" /><c r="I326" s="2" t="inlineStr" /><c r="J326" s="2" t="inlineStr" /><c r="K326" s="2" t="inlineStr"><is><t>Enoksaparyny</t></is></c><c r="L326" s="2" t="inlineStr"><is><t>Dipyridamolu</t></is></c><c r="M326" s="2" t="inlineStr" /><c r="N326" s="2" t="inlineStr" /><c r="O326" s="2" t="inlineStr" /><c r="P326" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q326" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="327"><c r="A327" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B327" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C327" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D327" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E327" s="2" t="inlineStr"><is><t>Statyny</t></is></c><c r="F327" s="2" t="inlineStr"><is><t>Zmniejszają stężenie cholesterolu LDL</t></is></c><c r="G327" s="2" t="inlineStr"><is><t>Zmniejszą stężenie triglicerydów</t></is></c><c r="H327" s="2" t="inlineStr" /><c r="I327" s="2" t="inlineStr" /><c r="J327" s="2" t="inlineStr" /><c r="K327" s="2" t="inlineStr"><is><t>Nie wpływają na stężenie cholesterolu wewnątrzkomórkowego</t></is></c><c r="L327" s="2" t="inlineStr"><is><t>Zmniejszają stężęnie cholesterolu HDL</t></is></c><c r="M327" s="2" t="inlineStr" /><c r="N327" s="2" t="inlineStr" /><c r="O327" s="2" t="inlineStr" /><c r="P327" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q327" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="328"><c r="A328" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B328" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C328" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D328" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E328" s="2" t="inlineStr"><is><t>Wielokierunkowe działanie statyn</t></is></c><c r="F328" s="2" t="inlineStr"><is><t>Poprawę funkcji śródbłonka</t></is></c><c r="G328" s="2" t="inlineStr"><is><t>Efekt przeciwzapalny</t></is></c><c r="H328" s="2" t="inlineStr"><is><t>Wpływ na fibrynolizę</t></is></c><c r="I328" s="2" t="inlineStr"><is><t>Stabilizację blaszki miażdżycowej</t></is></c><c r="J328" s="2" t="inlineStr" /><c r="K328" s="2" t="inlineStr" /><c r="L328" s="2" t="inlineStr" /><c r="M328" s="2" t="inlineStr" /><c r="N328" s="2" t="inlineStr" /><c r="O328" s="2" t="inlineStr" /><c r="P328" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q328" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="329"><c r="A329" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B329" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C329" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D329" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E329" s="2" t="inlineStr"><is><t>Farmakoterapia otyłości</t></is></c><c r="F329" s="2" t="inlineStr"><is><t>Liraglutyd</t></is></c><c r="G329" s="2" t="inlineStr"><is><t>Orlistat</t></is></c><c r="H329" s="2" t="inlineStr" /><c r="I329" s="2" t="inlineStr" /><c r="J329" s="2" t="inlineStr" /><c r="K329" s="2" t="inlineStr"><is><t>Paroksetyna</t></is></c><c r="L329" s="2" t="inlineStr"><is><t>Naltrekson</t></is></c><c r="M329" s="2" t="inlineStr" /><c r="N329" s="2" t="inlineStr" /><c r="O329" s="2" t="inlineStr" /><c r="P329" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q329" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="330"><c r="A330" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B330" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C330" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D330" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E330" s="2" t="inlineStr"><is><t>Do beta adrenolityków zmniejszających śmiertelność w skurczowej niewydolności serca</t></is></c><c r="F330" s="2" t="inlineStr"><is><t>Nebiwolol</t></is></c><c r="G330" s="2" t="inlineStr" /><c r="H330" s="2" t="inlineStr" /><c r="I330" s="2" t="inlineStr" /><c r="J330" s="2" t="inlineStr" /><c r="K330" s="2" t="inlineStr"><is><t>Atenolol</t></is></c><c r="L330" s="2" t="inlineStr"><is><t>Esmolol</t></is></c><c r="M330" s="2" t="inlineStr"><is><t>Acebutolol</t></is></c><c r="N330" s="2" t="inlineStr" /><c r="O330" s="2" t="inlineStr" /><c r="P330" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q330" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="331"><c r="A331" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B331" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C331" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D331" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E331" s="2" t="inlineStr"><is><t>Donory NO</t></is></c><c r="F331" s="2" t="inlineStr"><is><t>Nikorandil</t></is></c><c r="G331" s="2" t="inlineStr"><is><t>Molsidomina</t></is></c><c r="H331" s="2" t="inlineStr"><is><t>Diazontanizosorbitol</t></is></c><c r="I331" s="2" t="inlineStr" /><c r="J331" s="2" t="inlineStr" /><c r="K331" s="2" t="inlineStr"><is><t>Trimetazydyna</t></is></c><c r="L331" s="2" t="inlineStr" /><c r="M331" s="2" t="inlineStr" /><c r="N331" s="2" t="inlineStr" /><c r="O331" s="2" t="inlineStr" /><c r="P331" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q331" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="332"><c r="A332" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B332" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C332" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D332" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E332" s="2" t="inlineStr"><is><t>Leki I wyborou w monoterapii NT</t></is></c><c r="F332" s="2" t="inlineStr"><is><t>Antagoniści receptora angiotensynowego</t></is></c><c r="G332" s="2" t="inlineStr"><is><t>Antagoniści kanałów wapniowych</t></is></c><c r="H332" s="2" t="inlineStr" /><c r="I332" s="2" t="inlineStr" /><c r="J332" s="2" t="inlineStr" /><c r="K332" s="2" t="inlineStr"><is><t>Alfa1 adrenolityki</t></is></c><c r="L332" s="2" t="inlineStr"><is><t>Inhibitory reniny</t></is></c><c r="M332" s="2" t="inlineStr" /><c r="N332" s="2" t="inlineStr" /><c r="O332" s="2" t="inlineStr" /><c r="P332" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q332" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="333"><c r="A333" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B333" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C333" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D333" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E333" s="2" t="inlineStr"><is><t>Zmniejszenie śmiertnelności w skurczowej niewydolności serca</t></is></c><c r="F333" s="2" t="inlineStr"><is><t>Inhibitory konwertazy angiotensyny</t></is></c><c r="G333" s="2" t="inlineStr"><is><t>Antagoniści aldosteronu</t></is></c><c r="H333" s="2" t="inlineStr" /><c r="I333" s="2" t="inlineStr" /><c r="J333" s="2" t="inlineStr" /><c r="K333" s="2" t="inlineStr"><is><t>Waptany</t></is></c><c r="L333" s="2" t="inlineStr"><is><t>Diuretyki pętlowe</t></is></c><c r="M333" s="2" t="inlineStr" /><c r="N333" s="2" t="inlineStr" /><c r="O333" s="2" t="inlineStr" /><c r="P333" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q333" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="334"><c r="A334" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B334" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C334" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D334" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E334" s="2" t="inlineStr"><is><t>Przeciwskane jest jednoczesne stosowanie beta adrenolityków i</t></is></c><c r="F334" s="2" t="inlineStr"><is><t>Werapamilu</t></is></c><c r="G334" s="2" t="inlineStr" /><c r="H334" s="2" t="inlineStr" /><c r="I334" s="2" t="inlineStr" /><c r="J334" s="2" t="inlineStr" /><c r="K334" s="2" t="inlineStr"><is><t>Kaptoprylu</t></is></c><c r="L334" s="2" t="inlineStr"><is><t>Torasemidu</t></is></c><c r="M334" s="2" t="inlineStr"><is><t>Irbesartanu</t></is></c><c r="N334" s="2" t="inlineStr" /><c r="O334" s="2" t="inlineStr" /><c r="P334" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q334" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="335"><c r="A335" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B335" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C335" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D335" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E335" s="2" t="inlineStr"><is><t>Stan kliniczny – lek nadciśnieniowy</t></is></c><c r="F335" s="2" t="inlineStr"><is><t>Mikroalbuminuria – peryndopryl</t></is></c><c r="G335" s="2" t="inlineStr"><is><t>Tętniak aorty – bisoprolol</t></is></c><c r="H335" s="2" t="inlineStr"><is><t>Ciąża – metyldopa</t></is></c><c r="I335" s="2" t="inlineStr"><is><t>Chory po 80 rż. – indapamid</t></is></c><c r="J335" s="2" t="inlineStr" /><c r="K335" s="2" t="inlineStr" /><c r="L335" s="2" t="inlineStr" /><c r="M335" s="2" t="inlineStr" /><c r="N335" s="2" t="inlineStr" /><c r="O335" s="2" t="inlineStr" /><c r="P335" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q335" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="336"><c r="A336" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B336" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C336" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D336" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E336" s="2" t="inlineStr"><is><t>Inotropowe dodatnie</t></is></c><c r="F336" s="2" t="inlineStr"><is><t>Lewosymendan</t></is></c><c r="G336" s="2" t="inlineStr"><is><t>Milrinon</t></is></c><c r="H336" s="2" t="inlineStr" /><c r="I336" s="2" t="inlineStr" /><c r="J336" s="2" t="inlineStr" /><c r="K336" s="2" t="inlineStr"><is><t>Nesirytyd</t></is></c><c r="L336" s="2" t="inlineStr"><is><t>Sakubitryl</t></is></c><c r="M336" s="2" t="inlineStr" /><c r="N336" s="2" t="inlineStr" /><c r="O336" s="2" t="inlineStr" /><c r="P336" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q336" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="337"><c r="A337" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B337" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C337" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D337" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E337" s="2" t="inlineStr"><is><t>Skojarzenia leków w nadciśnieniu</t></is></c><c r="F337" s="2" t="inlineStr"><is><t>Inhibitor konwertazy angiotensyny + diuretyk tiazydowy</t></is></c><c r="G337" s="2" t="inlineStr"><is><t>Inhibitor konwertazy angiotensyny + antagonista wapnia</t></is></c><c r="H337" s="2" t="inlineStr"><is><t>Diuretyk tiazydowy + antagonista wapnia</t></is></c><c r="I337" s="2" t="inlineStr" /><c r="J337" s="2" t="inlineStr" /><c r="K337" s="2" t="inlineStr"><is><t>Sartan + inhibitor konwertazy angiotensyny</t></is></c><c r="L337" s="2" t="inlineStr" /><c r="M337" s="2" t="inlineStr" /><c r="N337" s="2" t="inlineStr" /><c r="O337" s="2" t="inlineStr" /><c r="P337" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q337" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="338"><c r="A338" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B338" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C338" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D338" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E338" s="2" t="inlineStr"><is><t>Amlodypina – działanie</t></is></c><c r="F338" s="2" t="inlineStr"><is><t>Zmniejszające opór obwodowy</t></is></c><c r="G338" s="2" t="inlineStr" /><c r="H338" s="2" t="inlineStr" /><c r="I338" s="2" t="inlineStr" /><c r="J338" s="2" t="inlineStr" /><c r="K338" s="2" t="inlineStr"><is><t>Chronotropowe dodatnie</t></is></c><c r="L338" s="2" t="inlineStr"><is><t>Inotropowe ujemne</t></is></c><c r="M338" s="2" t="inlineStr"><is><t>Dromotropowe ujemne</t></is></c><c r="N338" s="2" t="inlineStr" /><c r="O338" s="2" t="inlineStr" /><c r="P338" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q338" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="339"><c r="A339" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B339" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C339" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D339" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E339" s="2" t="inlineStr"><is><t>Dławica naczynioskurczowa (Prinzmetala)</t></is></c><c r="F339" s="2" t="inlineStr"><is><t>Diltiazem</t></is></c><c r="G339" s="2" t="inlineStr"><is><t>Werapamil</t></is></c><c r="H339" s="2" t="inlineStr" /><c r="I339" s="2" t="inlineStr" /><c r="J339" s="2" t="inlineStr" /><c r="K339" s="2" t="inlineStr"><is><t>Atenolol</t></is></c><c r="L339" s="2" t="inlineStr"><is><t>Prazosyna</t></is></c><c r="M339" s="2" t="inlineStr" /><c r="N339" s="2" t="inlineStr" /><c r="O339" s="2" t="inlineStr" /><c r="P339" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q339" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="340"><c r="A340" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B340" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C340" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D340" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E340" s="2" t="inlineStr"><is><t>Hiperkaliemia przy stosowaniu</t></is></c><c r="F340" s="2" t="inlineStr"><is><t>Kaptoprylu</t></is></c><c r="G340" s="2" t="inlineStr"><is><t>Amilorlydu</t></is></c><c r="H340" s="2" t="inlineStr" /><c r="I340" s="2" t="inlineStr" /><c r="J340" s="2" t="inlineStr" /><c r="K340" s="2" t="inlineStr"><is><t>Torasemidu</t></is></c><c r="L340" s="2" t="inlineStr"><is><t>Hydrochlortiazydu</t></is></c><c r="M340" s="2" t="inlineStr" /><c r="N340" s="2" t="inlineStr" /><c r="O340" s="2" t="inlineStr" /><c r="P340" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q340" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="341"><c r="A341" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B341" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C341" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D341" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E341" s="2" t="inlineStr"><is><t>OZW – postepowanie</t></is></c><c r="F341" s="2" t="inlineStr"><is><t>Furasemidu i.m</t></is></c><c r="G341" s="2" t="inlineStr"><is><t>Tikaglerolu p.o Klopidogrel bardziej, ale powiedzmy ze tak</t></is></c><c r="H341" s="2" t="inlineStr"><is><t>Morfiny s.c</t></is></c><c r="I341" s="2" t="inlineStr"><is><t>Kwasu acetylosalicylowego p.o</t></is></c><c r="J341" s="2" t="inlineStr" /><c r="K341" s="2" t="inlineStr" /><c r="L341" s="2" t="inlineStr" /><c r="M341" s="2" t="inlineStr" /><c r="N341" s="2" t="inlineStr" /><c r="O341" s="2" t="inlineStr" /><c r="P341" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q341" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="342"><c r="A342" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B342" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C342" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D342" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E342" s="2" t="inlineStr"><is><t>Eplerenon</t></is></c><c r="F342" s="2" t="inlineStr"><is><t>Selektywnie wiąże się z receptorem dla mineralokortykoidów</t></is></c><c r="G342" s="2" t="inlineStr" /><c r="H342" s="2" t="inlineStr" /><c r="I342" s="2" t="inlineStr" /><c r="J342" s="2" t="inlineStr" /><c r="K342" s="2" t="inlineStr"><is><t>Nie powoduje hiperkaliemii</t></is></c><c r="L342" s="2" t="inlineStr"><is><t>Jest agonistą receptorów dla androgenów</t></is></c><c r="M342" s="2" t="inlineStr"><is><t>Powoduje hipernatremię</t></is></c><c r="N342" s="2" t="inlineStr" /><c r="O342" s="2" t="inlineStr" /><c r="P342" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q342" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="343"><c r="A343" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B343" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C343" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D343" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E343" s="2" t="inlineStr"><is><t>TLPD – działania niepożądane</t></is></c><c r="F343" s="2" t="inlineStr"><is><t>Zwiększenie masy ciała</t></is></c><c r="G343" s="2" t="inlineStr"><is><t>Obniżenie progu drgawkowego</t></is></c><c r="H343" s="2" t="inlineStr"><is><t>Suchowść w ustach</t></is></c><c r="I343" s="2" t="inlineStr"><is><t>Nad lub niedociśnienie tętnicze</t></is></c><c r="J343" s="2" t="inlineStr" /><c r="K343" s="2" t="inlineStr" /><c r="L343" s="2" t="inlineStr" /><c r="M343" s="2" t="inlineStr" /><c r="N343" s="2" t="inlineStr" /><c r="O343" s="2" t="inlineStr" /><c r="P343" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q343" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="344"><c r="A344" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B344" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C344" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D344" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E344" s="2" t="inlineStr"><is><t>Lek przeciwpadaczkowy – mechanizm</t></is></c><c r="F344" s="2" t="inlineStr"><is><t>Gabapentyna – nasilenie transmisji GABA</t></is></c><c r="G344" s="2" t="inlineStr"><is><t>Karbamazepina – blokokowanie kanałów sodowych</t></is></c><c r="H344" s="2" t="inlineStr"><is><t>Etosuksymid – blokowanie kanałów wapniowych</t></is></c><c r="I344" s="2" t="inlineStr" /><c r="J344" s="2" t="inlineStr" /><c r="K344" s="2" t="inlineStr"><is><t>Lamotrygina – pobudzenie synaptycznego uwalniania aminokwasów</t></is></c><c r="L344" s="2" t="inlineStr" /><c r="M344" s="2" t="inlineStr" /><c r="N344" s="2" t="inlineStr" /><c r="O344" s="2" t="inlineStr" /><c r="P344" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q344" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="345"><c r="A345" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B345" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C345" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D345" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E345" s="2" t="inlineStr"><is><t>Klozapina wymaga monitorowania Wszystkie wymagają LPP</t></is></c><c r="F345" s="2" t="inlineStr"><is><t>Morfologii</t></is></c><c r="G345" s="2" t="inlineStr"><is><t>Masy ciała</t></is></c><c r="H345" s="2" t="inlineStr"><is><t>Lipidogramu</t></is></c><c r="I345" s="2" t="inlineStr"><is><t>Glikemii</t></is></c><c r="J345" s="2" t="inlineStr" /><c r="K345" s="2" t="inlineStr" /><c r="L345" s="2" t="inlineStr" /><c r="M345" s="2" t="inlineStr" /><c r="N345" s="2" t="inlineStr" /><c r="O345" s="2" t="inlineStr" /><c r="P345" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q345" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="346"><c r="A346" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B346" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C346" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D346" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E346" s="2" t="inlineStr"><is><t>Fluoksetyna</t></is></c><c r="F346" s="2" t="inlineStr"><is><t>Hamuje wychwyt zwrotny serotoniny</t></is></c><c r="G346" s="2" t="inlineStr" /><c r="H346" s="2" t="inlineStr" /><c r="I346" s="2" t="inlineStr" /><c r="J346" s="2" t="inlineStr" /><c r="K346" s="2" t="inlineStr"><is><t>Ma istotny wpływ na układ krążenia</t></is></c><c r="L346" s="2" t="inlineStr"><is><t>Często powoduje zaparcia</t></is></c><c r="M346" s="2" t="inlineStr"><is><t>Nie działa na enzymy cytochromu P-450</t></is></c><c r="N346" s="2" t="inlineStr" /><c r="O346" s="2" t="inlineStr" /><c r="P346" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q346" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="347"><c r="A347" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B347" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C347" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D347" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E347" s="2" t="inlineStr"><is><t>Zespoł serotoninowy – fluoksetyna i… MAO A i = 5-HT, NA, A, DA, tyramina.... MAO B i = DA i 5-HT</t></is></c><c r="F347" s="2" t="inlineStr"><is><t>Klomipramina</t></is></c><c r="G347" s="2" t="inlineStr"><is><t>Linezolid</t></is></c><c r="H347" s="2" t="inlineStr"><is><t>Wenlafaksyna</t></is></c><c r="I347" s="2" t="inlineStr"><is><t>Moklobemid</t></is></c><c r="J347" s="2" t="inlineStr" /><c r="K347" s="2" t="inlineStr" /><c r="L347" s="2" t="inlineStr" /><c r="M347" s="2" t="inlineStr" /><c r="N347" s="2" t="inlineStr" /><c r="O347" s="2" t="inlineStr" /><c r="P347" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q347" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="348"><c r="A348" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B348" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C348" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D348" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E348" s="2" t="inlineStr"><is><t>Choroba Wilsona</t></is></c><c r="F348" s="2" t="inlineStr"><is><t>Siarczan cynku</t></is></c><c r="G348" s="2" t="inlineStr"><is><t>D-penicylamina</t></is></c><c r="H348" s="2" t="inlineStr" /><c r="I348" s="2" t="inlineStr" /><c r="J348" s="2" t="inlineStr" /><c r="K348" s="2" t="inlineStr"><is><t>Ropinirol</t></is></c><c r="L348" s="2" t="inlineStr"><is><t>Siarczan magnezu</t></is></c><c r="M348" s="2" t="inlineStr" /><c r="N348" s="2" t="inlineStr" /><c r="O348" s="2" t="inlineStr" /><c r="P348" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q348" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="349"><c r="A349" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B349" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C349" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D349" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E349" s="2" t="inlineStr"><is><t>Farmakoterapia bólu neuropatycznego jakiego? :D Tako to wszystkie LPD i przeciwpadaczkowe</t></is></c><c r="F349" s="2" t="inlineStr"><is><t>Gabapentyna</t></is></c><c r="G349" s="2" t="inlineStr"><is><t>Amitryptylina</t></is></c><c r="H349" s="2" t="inlineStr"><is><t>Duloksetyna</t></is></c><c r="I349" s="2" t="inlineStr" /><c r="J349" s="2" t="inlineStr" /><c r="K349" s="2" t="inlineStr"><is><t>Ibuprofen</t></is></c><c r="L349" s="2" t="inlineStr" /><c r="M349" s="2" t="inlineStr" /><c r="N349" s="2" t="inlineStr" /><c r="O349" s="2" t="inlineStr" /><c r="P349" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q349" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="350"><c r="A350" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B350" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C350" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D350" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E350" s="2" t="inlineStr"><is><t>Profilaktyka migreny</t></is></c><c r="F350" s="2" t="inlineStr"><is><t>Metoprolol</t></is></c><c r="G350" s="2" t="inlineStr"><is><t>Flunaryzyna</t></is></c><c r="H350" s="2" t="inlineStr" /><c r="I350" s="2" t="inlineStr" /><c r="J350" s="2" t="inlineStr" /><c r="K350" s="2" t="inlineStr"><is><t>Indometacyna to w hemikranii</t></is></c><c r="L350" s="2" t="inlineStr"><is><t>Toksyna botulinowa</t></is></c><c r="M350" s="2" t="inlineStr" /><c r="N350" s="2" t="inlineStr" /><c r="O350" s="2" t="inlineStr" /><c r="P350" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q350" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="351"><c r="A351" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B351" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C351" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D351" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E351" s="2" t="inlineStr"><is><t>Alteplaza</t></is></c><c r="F351" s="2" t="inlineStr"><is><t>W udarze niedokrwiennym mózgu</t></is></c><c r="G351" s="2" t="inlineStr" /><c r="H351" s="2" t="inlineStr" /><c r="I351" s="2" t="inlineStr" /><c r="J351" s="2" t="inlineStr" /><c r="K351" s="2" t="inlineStr"><is><t>Przed planowaną kardiowersją</t></is></c><c r="L351" s="2" t="inlineStr"><is><t>W zatorowości płucnej niewysokiego ryzyka</t></is></c><c r="M351" s="2" t="inlineStr"><is><t>W TIA</t></is></c><c r="N351" s="2" t="inlineStr" /><c r="O351" s="2" t="inlineStr" /><c r="P351" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q351" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="352"><c r="A352" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B352" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C352" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D352" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E352" s="2" t="inlineStr"><is><t>Profilaktyka wtórna udaru mózgu</t></is></c><c r="F352" s="2" t="inlineStr"><is><t>Dipirydamol</t></is></c><c r="G352" s="2" t="inlineStr"><is><t>Atorwastatyna</t></is></c><c r="H352" s="2" t="inlineStr"><is><t>Enoksapyrana</t></is></c><c r="I352" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="J352" s="2" t="inlineStr" /><c r="K352" s="2" t="inlineStr" /><c r="L352" s="2" t="inlineStr" /><c r="M352" s="2" t="inlineStr" /><c r="N352" s="2" t="inlineStr" /><c r="O352" s="2" t="inlineStr" /><c r="P352" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q352" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="353"><c r="A353" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B353" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C353" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D353" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E353" s="2" t="inlineStr"><is><t>Do działań niepożądanych doksycykliny zaliczamy:</t></is></c><c r="F353" s="2" t="inlineStr"><is><t>fotodermatozy</t></is></c><c r="G353" s="2" t="inlineStr"><is><t>zaburzenia czynności cewek nerkowych wywołane przez jej produkty rozpadu</t></is></c><c r="H353" s="2" t="inlineStr"><is><t>zapalenie wątroby</t></is></c><c r="I353" s="2" t="inlineStr"><is><t>zaburzenia rozwoju zębów i kości</t></is></c><c r="J353" s="2" t="inlineStr" /><c r="K353" s="2" t="inlineStr" /><c r="L353" s="2" t="inlineStr" /><c r="M353" s="2" t="inlineStr" /><c r="N353" s="2" t="inlineStr" /><c r="O353" s="2" t="inlineStr" /><c r="P353" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q353" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="354"><c r="A354" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B354" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C354" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D354" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E354" s="2" t="inlineStr"><is><t>Ceftriakson:</t></is></c><c r="F354" s="2" t="inlineStr"><is><t>należy do cefalosporyn III generacji</t></is></c><c r="G354" s="2" t="inlineStr"><is><t>może być podawany dożylnie</t></is></c><c r="H354" s="2" t="inlineStr" /><c r="I354" s="2" t="inlineStr" /><c r="J354" s="2" t="inlineStr" /><c r="K354" s="2" t="inlineStr"><is><t>wykazuje aktywność wobec MRSA</t></is></c><c r="L354" s="2" t="inlineStr"><is><t>nie wykazuje aktywności wobec Borrelia burgdorferi</t></is></c><c r="M354" s="2" t="inlineStr" /><c r="N354" s="2" t="inlineStr" /><c r="O354" s="2" t="inlineStr" /><c r="P354" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q354" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="355"><c r="A355" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B355" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C355" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D355" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E355" s="2" t="inlineStr"><is><t>Pseudomonas aeruginosa jest wrażliwy na działanie:</t></is></c><c r="F355" s="2" t="inlineStr"><is><t>kolistyny</t></is></c><c r="G355" s="2" t="inlineStr"><is><t>tobramycyn</t></is></c><c r="H355" s="2" t="inlineStr" /><c r="I355" s="2" t="inlineStr" /><c r="J355" s="2" t="inlineStr" /><c r="K355" s="2" t="inlineStr"><is><t>telawancyny</t></is></c><c r="L355" s="2" t="inlineStr"><is><t>cefazoliny</t></is></c><c r="M355" s="2" t="inlineStr" /><c r="N355" s="2" t="inlineStr" /><c r="O355" s="2" t="inlineStr" /><c r="P355" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q355" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="356"><c r="A356" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B356" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C356" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D356" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E356" s="2" t="inlineStr"><is><t>W terapii empirycznej bakteryjnego zapalenia opon mózgowo-rdzeniowych u osób dorosłych zalecane są:</t></is></c><c r="F356" s="2" t="inlineStr"><is><t>cefotaksym z wankomycyną</t></is></c><c r="G356" s="2" t="inlineStr"><is><t>ceftriakson z wankomycyną</t></is></c><c r="H356" s="2" t="inlineStr" /><c r="I356" s="2" t="inlineStr" /><c r="J356" s="2" t="inlineStr" /><c r="K356" s="2" t="inlineStr"><is><t>ampicylina z gentamycyną</t></is></c><c r="L356" s="2" t="inlineStr"><is><t>ampicylina z deksametazonem</t></is></c><c r="M356" s="2" t="inlineStr" /><c r="N356" s="2" t="inlineStr" /><c r="O356" s="2" t="inlineStr" /><c r="P356" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q356" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="357"><c r="A357" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B357" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C357" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D357" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E357" s="2" t="inlineStr"><is><t>Efekt bakteriobójczy zależny od czasu, w którym stężenie leku jest większe od MIC wykazują:</t></is></c><c r="F357" s="2" t="inlineStr"><is><t>amoksycylina z kwasem klawulanowym</t></is></c><c r="G357" s="2" t="inlineStr"><is><t>ceftriakson</t></is></c><c r="H357" s="2" t="inlineStr" /><c r="I357" s="2" t="inlineStr" /><c r="J357" s="2" t="inlineStr" /><c r="K357" s="2" t="inlineStr"><is><t>lewofloksacyna</t></is></c><c r="L357" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="M357" s="2" t="inlineStr" /><c r="N357" s="2" t="inlineStr" /><c r="O357" s="2" t="inlineStr" /><c r="P357" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q357" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="358"><c r="A358" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B358" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C358" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D358" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E358" s="2" t="inlineStr"><is><t>Leki przeciwdrobnoustrojowe, których mechanizm działania polega na hamowaniu biosyntezy ściany komórkowej bakterii to:</t></is></c><c r="F358" s="2" t="inlineStr"><is><t>cefadroksyl</t></is></c><c r="G358" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="H358" s="2" t="inlineStr"><is><t>bacytracyna</t></is></c><c r="I358" s="2" t="inlineStr" /><c r="J358" s="2" t="inlineStr" /><c r="K358" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="L358" s="2" t="inlineStr" /><c r="M358" s="2" t="inlineStr" /><c r="N358" s="2" t="inlineStr" /><c r="O358" s="2" t="inlineStr" /><c r="P358" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q358" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="359"><c r="A359" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B359" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C359" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D359" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E359" s="2" t="inlineStr"><is><t>Aktywność przeciwbakteryjną względem Legionella spp. ma:</t></is></c><c r="F359" s="2" t="inlineStr"><is><t>moksyfloksacyna</t></is></c><c r="G359" s="2" t="inlineStr"><is><t>azytromycyna</t></is></c><c r="H359" s="2" t="inlineStr"><is><t>tygecyklina</t></is></c><c r="I359" s="2" t="inlineStr" /><c r="J359" s="2" t="inlineStr" /><c r="K359" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="L359" s="2" t="inlineStr" /><c r="M359" s="2" t="inlineStr" /><c r="N359" s="2" t="inlineStr" /><c r="O359" s="2" t="inlineStr" /><c r="P359" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q359" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="360"><c r="A360" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B360" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C360" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D360" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E360" s="2" t="inlineStr"><is><t>Jodopowidon znalazł zastosowanie w:</t></is></c><c r="F360" s="2" t="inlineStr"><is><t>dezynfekcji skóry przed nakłuciem</t></is></c><c r="G360" s="2" t="inlineStr"><is><t>leczeniu zakażeń pochwy florą mieszaną</t></is></c><c r="H360" s="2" t="inlineStr"><is><t>profilaktyce zakażeń ran</t></is></c><c r="I360" s="2" t="inlineStr"><is><t>leczeniu zakażeń błony śluzowej jamy ustnej</t></is></c><c r="J360" s="2" t="inlineStr" /><c r="K360" s="2" t="inlineStr" /><c r="L360" s="2" t="inlineStr" /><c r="M360" s="2" t="inlineStr" /><c r="N360" s="2" t="inlineStr" /><c r="O360" s="2" t="inlineStr" /><c r="P360" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q360" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="361"><c r="A361" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B361" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C361" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D361" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E361" s="2" t="inlineStr"><is><t>Inhibitory neuraminidazy:</t></is></c><c r="F361" s="2" t="inlineStr"><is><t>hamują uwalnianie wirusów z zakażonych komórek</t></is></c><c r="G361" s="2" t="inlineStr"><is><t>można je stosować w leczeniu grypy typu A i B</t></is></c><c r="H361" s="2" t="inlineStr" /><c r="I361" s="2" t="inlineStr" /><c r="J361" s="2" t="inlineStr" /><c r="K361" s="2" t="inlineStr"><is><t>nie różnią się między sobą pod względem skuteczności i działań niepożądanych</t></is></c><c r="L361" s="2" t="inlineStr"><is><t>nie są skuteczne w profilaktyce grypy</t></is></c><c r="M361" s="2" t="inlineStr" /><c r="N361" s="2" t="inlineStr" /><c r="O361" s="2" t="inlineStr" /><c r="P361" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q361" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="362"><c r="A362" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B362" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C362" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D362" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E362" s="2" t="inlineStr"><is><t>Cyprofloksacyna:</t></is></c><c r="F362" s="2" t="inlineStr"><is><t>ma efekt działania zależny od skumulowanej ekspozycji</t></is></c><c r="G362" s="2" t="inlineStr"><is><t>jest stosowana w leczeniu empirycznym niepowikłanego ostrego odmiedniczkowego zapalenia nerek</t></is></c><c r="H362" s="2" t="inlineStr"><is><t>może być podawana dożylnie</t></is></c><c r="I362" s="2" t="inlineStr" /><c r="J362" s="2" t="inlineStr" /><c r="K362" s="2" t="inlineStr"><is><t>nie wydłuża odstępu QT</t></is></c><c r="L362" s="2" t="inlineStr" /><c r="M362" s="2" t="inlineStr" /><c r="N362" s="2" t="inlineStr" /><c r="O362" s="2" t="inlineStr" /><c r="P362" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q362" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="363"><c r="A363" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B363" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C363" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D363" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E363" s="2" t="inlineStr"><is><t>Leczenie przeciwbakteryjne powinno być zlecone, jeśli w badaniu mikrobiologicznym zostanie stwierdzone:</t></is></c><c r="F363" s="2" t="inlineStr"><is><t>obecność Escherichia coli w dwóch posiewach krwi obwodowej</t></is></c><c r="G363" s="2" t="inlineStr"><is><t>brak wzrostu bakterii we krwi u osoby z klinicznymi i radiologicznymi cechami zapalenia płuc</t></is></c><c r="H363" s="2" t="inlineStr" /><c r="I363" s="2" t="inlineStr" /><c r="J363" s="2" t="inlineStr" /><c r="K363" s="2" t="inlineStr"><is><t>nosicielstwo szczepu alarmowego w przewodzie pokarmowym</t></is></c><c r="L363" s="2" t="inlineStr"><is><t>trzy gatunki bakterii w posiewie moczu</t></is></c><c r="M363" s="2" t="inlineStr" /><c r="N363" s="2" t="inlineStr" /><c r="O363" s="2" t="inlineStr" /><c r="P363" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q363" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="364"><c r="A364" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B364" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C364" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D364" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E364" s="2" t="inlineStr"><is><t>Przeciwinfekcyjna farmakoprofilaktyka medyczna jest zalecana:</t></is></c><c r="F364" s="2" t="inlineStr"><is><t>w ciężkiej neutropenii trwającej &gt; 7 dni u osób z ostrymi białaczkami</t></is></c><c r="G364" s="2" t="inlineStr"><is><t>nieszczepionym osobom z grup ryzyka ciężkiego przebiegu choroby po kontakcie z chorym na grypę</t></is></c><c r="H364" s="2" t="inlineStr" /><c r="I364" s="2" t="inlineStr" /><c r="J364" s="2" t="inlineStr" /><c r="K364" s="2" t="inlineStr"><is><t>po implantacji stentów wieńcowych przez 12 miesięcy</t></is></c><c r="L364" s="2" t="inlineStr"><is><t>podczas przewlekłego cewnikowania pęcherza moczowego</t></is></c><c r="M364" s="2" t="inlineStr" /><c r="N364" s="2" t="inlineStr" /><c r="O364" s="2" t="inlineStr" /><c r="P364" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q364" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="365"><c r="A365" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B365" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C365" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D365" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E365" s="2" t="inlineStr"><is><t>W grzybiczym zakażeniu paznokci zastosowanie ma:</t></is></c><c r="F365" s="2" t="inlineStr"><is><t>itrakonazol</t></is></c><c r="G365" s="2" t="inlineStr"><is><t>terbinafina</t></is></c><c r="H365" s="2" t="inlineStr" /><c r="I365" s="2" t="inlineStr" /><c r="J365" s="2" t="inlineStr" /><c r="K365" s="2" t="inlineStr"><is><t>natamycyna</t></is></c><c r="L365" s="2" t="inlineStr"><is><t>kaspofungina</t></is></c><c r="M365" s="2" t="inlineStr" /><c r="N365" s="2" t="inlineStr" /><c r="O365" s="2" t="inlineStr" /><c r="P365" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q365" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="366"><c r="A366" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B366" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C366" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D366" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E366" s="2" t="inlineStr"><is><t>Po ugryzieniu przez kleszcza, gdy obserwujemy rumień wędrujący, racjonalne jest zastosowanie:</t></is></c><c r="F366" s="2" t="inlineStr"><is><t>amoksycyliny</t></is></c><c r="G366" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="H366" s="2" t="inlineStr"><is><t>cefuroksymu</t></is></c><c r="I366" s="2" t="inlineStr"><is><t>azytromycyny</t></is></c><c r="J366" s="2" t="inlineStr" /><c r="K366" s="2" t="inlineStr" /><c r="L366" s="2" t="inlineStr" /><c r="M366" s="2" t="inlineStr" /><c r="N366" s="2" t="inlineStr" /><c r="O366" s="2" t="inlineStr" /><c r="P366" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q366" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="367"><c r="A367" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B367" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C367" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D367" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E367" s="2" t="inlineStr"><is><t>W leczeniu zakażenia wirusem opryszczki (Herpes) stosuje się:</t></is></c><c r="F367" s="2" t="inlineStr"><is><t>foskarnet</t></is></c><c r="G367" s="2" t="inlineStr"><is><t>acyklowir</t></is></c><c r="H367" s="2" t="inlineStr" /><c r="I367" s="2" t="inlineStr" /><c r="J367" s="2" t="inlineStr" /><c r="K367" s="2" t="inlineStr"><is><t>rymantadynę</t></is></c><c r="L367" s="2" t="inlineStr"><is><t>lamiwudynę</t></is></c><c r="M367" s="2" t="inlineStr" /><c r="N367" s="2" t="inlineStr" /><c r="O367" s="2" t="inlineStr" /><c r="P367" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q367" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="368"><c r="A368" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B368" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C368" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D368" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E368" s="2" t="inlineStr"><is><t>W leczeniu hipoglikemii stosuje się:</t></is></c><c r="F368" s="2" t="inlineStr"><is><t>węglowodany proste doustnie</t></is></c><c r="G368" s="2" t="inlineStr"><is><t>glukozę dożylnie</t></is></c><c r="H368" s="2" t="inlineStr"><is><t>węglowodany złożone doustnie</t></is></c><c r="I368" s="2" t="inlineStr" /><c r="J368" s="2" t="inlineStr" /><c r="K368" s="2" t="inlineStr"><is><t>glukagon doustnie</t></is></c><c r="L368" s="2" t="inlineStr" /><c r="M368" s="2" t="inlineStr" /><c r="N368" s="2" t="inlineStr" /><c r="O368" s="2" t="inlineStr" /><c r="P368" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q368" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="369"><c r="A369" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B369" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C369" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D369" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E369" s="2" t="inlineStr"><is><t>Liotyronina:</t></is></c><c r="F369" s="2" t="inlineStr"><is><t>odpowiada ona naturalnemu hormonowi T3</t></is></c><c r="G369" s="2" t="inlineStr"><is><t>ma krótszy okres półtrwania niż lewotyroksyna</t></is></c><c r="H369" s="2" t="inlineStr" /><c r="I369" s="2" t="inlineStr" /><c r="J369" s="2" t="inlineStr" /><c r="K369" s="2" t="inlineStr"><is><t>jest lekiem z wyboru w niedoczynności tarczycy</t></is></c><c r="L369" s="2" t="inlineStr"><is><t>jest przeciwwskazana w leczeniu śpiączki hipometabolicznej</t></is></c><c r="M369" s="2" t="inlineStr" /><c r="N369" s="2" t="inlineStr" /><c r="O369" s="2" t="inlineStr" /><c r="P369" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q369" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="370"><c r="A370" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B370" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C370" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D370" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E370" s="2" t="inlineStr"><is><t>Wskazaniem do zastosowania jodku potasu może być:</t></is></c><c r="F370" s="2" t="inlineStr"><is><t>ochrona tarczycy przed jodem radioaktywnym</t></is></c><c r="G370" s="2" t="inlineStr"><is><t>przygotowanie do usunięcia tarczycy</t></is></c><c r="H370" s="2" t="inlineStr"><is><t>przełom tyreotoksyczny</t></is></c><c r="I370" s="2" t="inlineStr"><is><t>zapobieganie powstawaniu wola z niedoboru jodu</t></is></c><c r="J370" s="2" t="inlineStr" /><c r="K370" s="2" t="inlineStr" /><c r="L370" s="2" t="inlineStr" /><c r="M370" s="2" t="inlineStr" /><c r="N370" s="2" t="inlineStr" /><c r="O370" s="2" t="inlineStr" /><c r="P370" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q370" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="371"><c r="A371" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B371" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C371" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D371" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E371" s="2" t="inlineStr"><is><t>W leczeniu hiperprolaktynemii stosuje się:</t></is></c><c r="F371" s="2" t="inlineStr"><is><t>bromokryptynę</t></is></c><c r="G371" s="2" t="inlineStr"><is><t>karbegolinę</t></is></c><c r="H371" s="2" t="inlineStr" /><c r="I371" s="2" t="inlineStr" /><c r="J371" s="2" t="inlineStr" /><c r="K371" s="2" t="inlineStr"><is><t>somatostatynę</t></is></c><c r="L371" s="2" t="inlineStr"><is><t>terlipresynę</t></is></c><c r="M371" s="2" t="inlineStr" /><c r="N371" s="2" t="inlineStr" /><c r="O371" s="2" t="inlineStr" /><c r="P371" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q371" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="372"><c r="A372" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B372" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C372" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D372" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E372" s="2" t="inlineStr"><is><t>Działanie antyandrogenne wykazuje:</t></is></c><c r="F372" s="2" t="inlineStr"><is><t>octan cyproteronu</t></is></c><c r="G372" s="2" t="inlineStr"><is><t>ketokonazol</t></is></c><c r="H372" s="2" t="inlineStr"><is><t>finasteryd</t></is></c><c r="I372" s="2" t="inlineStr"><is><t>bikalutamid</t></is></c><c r="J372" s="2" t="inlineStr" /><c r="K372" s="2" t="inlineStr" /><c r="L372" s="2" t="inlineStr" /><c r="M372" s="2" t="inlineStr" /><c r="N372" s="2" t="inlineStr" /><c r="O372" s="2" t="inlineStr" /><c r="P372" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q372" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="373"><c r="A373" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B373" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C373" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D373" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E373" s="2" t="inlineStr"><is><t>Glikokortykosteroidy zwiększają:</t></is></c><c r="F373" s="2" t="inlineStr"><is><t>produkcję surfaktantu</t></is></c><c r="G373" s="2" t="inlineStr" /><c r="H373" s="2" t="inlineStr" /><c r="I373" s="2" t="inlineStr" /><c r="J373" s="2" t="inlineStr" /><c r="K373" s="2" t="inlineStr"><is><t>ekspresję genu osteokalcyny</t></is></c><c r="L373" s="2" t="inlineStr"><is><t>stężenie wapnia w surowicy krwi</t></is></c><c r="M373" s="2" t="inlineStr"><is><t>syntezę testosteronu</t></is></c><c r="N373" s="2" t="inlineStr" /><c r="O373" s="2" t="inlineStr" /><c r="P373" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q373" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="374"><c r="A374" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B374" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C374" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D374" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E374" s="2" t="inlineStr"><is><t>Efektem nadmiaru gestagenów może być:</t></is></c><c r="F374" s="2" t="inlineStr"><is><t>depresja</t></is></c><c r="G374" s="2" t="inlineStr"><is><t>łojotok skóry</t></is></c><c r="H374" s="2" t="inlineStr"><is><t>przyrost masy ciała</t></is></c><c r="I374" s="2" t="inlineStr"><is><t>hirsutyzm</t></is></c><c r="J374" s="2" t="inlineStr" /><c r="K374" s="2" t="inlineStr" /><c r="L374" s="2" t="inlineStr" /><c r="M374" s="2" t="inlineStr" /><c r="N374" s="2" t="inlineStr" /><c r="O374" s="2" t="inlineStr" /><c r="P374" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q374" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="375"><c r="A375" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B375" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C375" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D375" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E375" s="2" t="inlineStr"><is><t>W leczeniu wągrzycy (cysticerkozy) stosujemy:</t></is></c><c r="F375" s="2" t="inlineStr"><is><t>prazykwantel</t></is></c><c r="G375" s="2" t="inlineStr"><is><t>albendazol</t></is></c><c r="H375" s="2" t="inlineStr" /><c r="I375" s="2" t="inlineStr" /><c r="J375" s="2" t="inlineStr" /><c r="K375" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="L375" s="2" t="inlineStr"><is><t>iwermektynę bo</t></is></c><c r="M375" s="2" t="inlineStr" /><c r="N375" s="2" t="inlineStr" /><c r="O375" s="2" t="inlineStr" /><c r="P375" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q375" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="376"><c r="A376" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B376" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C376" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D376" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E376" s="2" t="inlineStr"><is><t>Stosowanie kwasu acetylosalicylowego może być przyczyną:</t></is></c><c r="F376" s="2" t="inlineStr"><is><t>zaostrzenia astmy</t></is></c><c r="G376" s="2" t="inlineStr"><is><t>retencji sodu i wody</t></is></c><c r="H376" s="2" t="inlineStr"><is><t>niedokrwistości</t></is></c><c r="I376" s="2" t="inlineStr" /><c r="J376" s="2" t="inlineStr" /><c r="K376" s="2" t="inlineStr"><is><t>zakrzepicy żył głębokich</t></is></c><c r="L376" s="2" t="inlineStr" /><c r="M376" s="2" t="inlineStr" /><c r="N376" s="2" t="inlineStr" /><c r="O376" s="2" t="inlineStr" /><c r="P376" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q376" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="377"><c r="A377" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B377" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C377" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D377" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E377" s="2" t="inlineStr"><is><t>Efekty gastrotoksyczne związane ze stosowaniem niesteroidowych leków przeciwzapalnych może nasilać:</t></is></c><c r="F377" s="2" t="inlineStr"><is><t>zolendronian</t></is></c><c r="G377" s="2" t="inlineStr"><is><t>fluoksetyna tak, SSRI też</t></is></c><c r="H377" s="2" t="inlineStr"><is><t>acenokumarol</t></is></c><c r="I377" s="2" t="inlineStr"><is><t>prednizon</t></is></c><c r="J377" s="2" t="inlineStr" /><c r="K377" s="2" t="inlineStr" /><c r="L377" s="2" t="inlineStr" /><c r="M377" s="2" t="inlineStr" /><c r="N377" s="2" t="inlineStr" /><c r="O377" s="2" t="inlineStr" /><c r="P377" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q377" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="378"><c r="A378" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B378" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C378" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D378" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E378" s="2" t="inlineStr"><is><t>Zastosowanie ibuprofenu w 3 trymestrze ciąży może spowodować:</t></is></c><c r="F378" s="2" t="inlineStr"><is><t>przedwczesne zamknięcie przewodu Botalla</t></is></c><c r="G378" s="2" t="inlineStr"><is><t>zwiększone ryzyko krwawienia u matki</t></is></c><c r="H378" s="2" t="inlineStr"><is><t>zwiększone ryzyko obrzęków u matki</t></is></c><c r="I378" s="2" t="inlineStr" /><c r="J378" s="2" t="inlineStr" /><c r="K378" s="2" t="inlineStr"><is><t>zwiększenie czynności skurczowej macicy</t></is></c><c r="L378" s="2" t="inlineStr" /><c r="M378" s="2" t="inlineStr" /><c r="N378" s="2" t="inlineStr" /><c r="O378" s="2" t="inlineStr" /><c r="P378" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q378" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="379"><c r="A379" s="2" t="inlineStr"><is><t>BÓLE GŁOWY</t></is></c><c r="B379" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C379" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D379" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E379" s="2" t="inlineStr"><is><t>Napad migreny przerywa:</t></is></c><c r="F379" s="2" t="inlineStr"><is><t>winian ergotaminy</t></is></c><c r="G379" s="2" t="inlineStr"><is><t>sumatryptan</t></is></c><c r="H379" s="2" t="inlineStr"><is><t>ibuprofen</t></is></c><c r="I379" s="2" t="inlineStr" /><c r="J379" s="2" t="inlineStr" /><c r="K379" s="2" t="inlineStr"><is><t>metoklopramid</t></is></c><c r="L379" s="2" t="inlineStr" /><c r="M379" s="2" t="inlineStr" /><c r="N379" s="2" t="inlineStr" /><c r="O379" s="2" t="inlineStr" /><c r="P379" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q379" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="380"><c r="A380" s="2" t="inlineStr"><is><t>ZNIECZULENIA MIEJSCOWE</t></is></c><c r="B380" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C380" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D380" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E380" s="2" t="inlineStr"><is><t>W leczeniu neuralgii popółpaśćcowej można zastosować:</t></is></c><c r="F380" s="2" t="inlineStr"><is><t>8% kapsaicynę w kremie</t></is></c><c r="G380" s="2" t="inlineStr"><is><t>5% lidokainę w plastrach</t></is></c><c r="H380" s="2" t="inlineStr"><is><t>amitryptylinę</t></is></c><c r="I380" s="2" t="inlineStr" /><c r="J380" s="2" t="inlineStr" /><c r="K380" s="2" t="inlineStr"><is><t>metamizol</t></is></c><c r="L380" s="2" t="inlineStr" /><c r="M380" s="2" t="inlineStr" /><c r="N380" s="2" t="inlineStr" /><c r="O380" s="2" t="inlineStr" /><c r="P380" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q380" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="381"><c r="A381" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B381" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C381" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D381" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E381" s="2" t="inlineStr"><is><t>Loperamid:</t></is></c><c r="F381" s="2" t="inlineStr"><is><t>w dawkach terapeutycznych nie działa ośrodkowo</t></is></c><c r="G381" s="2" t="inlineStr"><is><t>jest przeciwwskazany we wrzodziejącym zapaleniu jelita grubego</t></is></c><c r="H381" s="2" t="inlineStr" /><c r="I381" s="2" t="inlineStr" /><c r="J381" s="2" t="inlineStr" /><c r="K381" s="2" t="inlineStr"><is><t>jest agonistą receptorów serotoninowych w jelicie</t></is></c><c r="L381" s="2" t="inlineStr"><is><t>wykazuje działanie przeciwbólowe</t></is></c><c r="M381" s="2" t="inlineStr" /><c r="N381" s="2" t="inlineStr" /><c r="O381" s="2" t="inlineStr" /><c r="P381" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q381" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="382"><c r="A382" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B382" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C382" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D382" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E382" s="2" t="inlineStr"><is><t>Fentanyl:</t></is></c><c r="F382" s="2" t="inlineStr"><is><t>hamuje ośrodek oddechowy</t></is></c><c r="G382" s="2" t="inlineStr" /><c r="H382" s="2" t="inlineStr" /><c r="I382" s="2" t="inlineStr" /><c r="J382" s="2" t="inlineStr" /><c r="K382" s="2" t="inlineStr"><is><t>działa neurotoksycznie</t></is></c><c r="L382" s="2" t="inlineStr"><is><t>ma aktywne metabolity</t></is></c><c r="M382" s="2" t="inlineStr"><is><t>uwalnia histaminę</t></is></c><c r="N382" s="2" t="inlineStr" /><c r="O382" s="2" t="inlineStr" /><c r="P382" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q382" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="383"><c r="A383" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B383" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C383" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D383" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E383" s="2" t="inlineStr"><is><t>Nefopam</t></is></c><c r="F383" s="2" t="inlineStr"><is><t>jest inhibitorem wychwytu zwrotnego serotoniny i noradrenaliny</t></is></c><c r="G383" s="2" t="inlineStr"><is><t>u osób starszych może wywoływać omamy</t></is></c><c r="H383" s="2" t="inlineStr" /><c r="I383" s="2" t="inlineStr" /><c r="J383" s="2" t="inlineStr" /><c r="K383" s="2" t="inlineStr"><is><t>hamuje wybiórczo cyklooksygenazę typu 2</t></is></c><c r="L383" s="2" t="inlineStr"><is><t>u dzieci może być stosowany w profilaktyce drgawek gorączkowych</t></is></c><c r="M383" s="2" t="inlineStr" /><c r="N383" s="2" t="inlineStr" /><c r="O383" s="2" t="inlineStr" /><c r="P383" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q383" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="384"><c r="A384" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B384" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C384" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D384" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E384" s="2" t="inlineStr"><is><t>W zespole abstynencyjnym w uzależnieniu od opioidów występują:</t></is></c><c r="F384" s="2" t="inlineStr"><is><t>rozszerzenie źrenic</t></is></c><c r="G384" s="2" t="inlineStr"><is><t>wymioty i biegunka</t></is></c><c r="H384" s="2" t="inlineStr"><is><t>bezsenność</t></is></c><c r="I384" s="2" t="inlineStr"><is><t>łzawienie i wyciek z nosa</t></is></c><c r="J384" s="2" t="inlineStr" /><c r="K384" s="2" t="inlineStr" /><c r="L384" s="2" t="inlineStr" /><c r="M384" s="2" t="inlineStr" /><c r="N384" s="2" t="inlineStr" /><c r="O384" s="2" t="inlineStr" /><c r="P384" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q384" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="385"><c r="A385" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B385" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C385" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D385" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E385" s="2" t="inlineStr"><is><t>Redukcję masy ciała może powodować stosowanie:</t></is></c><c r="F385" s="2" t="inlineStr"><is><t>fluoksetyny</t></is></c><c r="G385" s="2" t="inlineStr"><is><t>metforminy</t></is></c><c r="H385" s="2" t="inlineStr"><is><t>liraglutydu</t></is></c><c r="I385" s="2" t="inlineStr" /><c r="J385" s="2" t="inlineStr" /><c r="K385" s="2" t="inlineStr"><is><t>insuliny</t></is></c><c r="L385" s="2" t="inlineStr" /><c r="M385" s="2" t="inlineStr" /><c r="N385" s="2" t="inlineStr" /><c r="O385" s="2" t="inlineStr" /><c r="P385" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q385" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="386"><c r="A386" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B386" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C386" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D386" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E386" s="2" t="inlineStr"><is><t>W udarze niedokrwiennym mózgu możesz zastosować tkankowy aktywator plazminogenu jeśli stwierdzisz, że pacjent:</t></is></c><c r="F386" s="2" t="inlineStr"><is><t>doustne leczenie przeciwkrzepliwe (INR=1.5)</t></is></c><c r="G386" s="2" t="inlineStr"><is><t>ma wartości ciśnienia tętniczego: SBP ≤ 185 mm Hg lub DBP ≤ 110 mm Hg</t></is></c><c r="H386" s="2" t="inlineStr"><is><t>ma czas od wystąpienia objawów udaru mózgu nie przekraczający 4.5h</t></is></c><c r="I386" s="2" t="inlineStr" /><c r="J386" s="2" t="inlineStr" /><c r="K386" s="2" t="inlineStr"><is><t>jest w podeszłym wieku (&gt; 80 lat)</t></is></c><c r="L386" s="2" t="inlineStr" /><c r="M386" s="2" t="inlineStr" /><c r="N386" s="2" t="inlineStr" /><c r="O386" s="2" t="inlineStr" /><c r="P386" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q386" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="387"><c r="A387" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B387" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C387" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D387" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E387" s="2" t="inlineStr"><is><t>U 76 letniej kobiety z napadowym migotaniem przedsionków, cukrzycą i nadciśnieniem tętniczym (Cha2DS2VASc = 5 pkt) i niskim ryzykiem krwawienia (HAS-BLED = 2 pkt) wskazane w przewlekłej profilaktyce są:</t></is></c><c r="F387" s="2" t="inlineStr"><is><t>warfaryna</t></is></c><c r="G387" s="2" t="inlineStr"><is><t>eteksylan dabigatranu</t></is></c><c r="H387" s="2" t="inlineStr" /><c r="I387" s="2" t="inlineStr" /><c r="J387" s="2" t="inlineStr" /><c r="K387" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="L387" s="2" t="inlineStr"><is><t>fondaparynuks</t></is></c><c r="M387" s="2" t="inlineStr" /><c r="N387" s="2" t="inlineStr" /><c r="O387" s="2" t="inlineStr" /><c r="P387" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q387" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="388"><c r="A388" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B388" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C388" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D388" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E388" s="2" t="inlineStr"><is><t>Rywaroksaban:</t></is></c><c r="F388" s="2" t="inlineStr"><is><t>wymaga redukcji dawki w niewydolności nerek</t></is></c><c r="G388" s="2" t="inlineStr" /><c r="H388" s="2" t="inlineStr" /><c r="I388" s="2" t="inlineStr" /><c r="J388" s="2" t="inlineStr" /><c r="K388" s="2" t="inlineStr"><is><t>odwracalnie blokuje receptor GP IIb/IIIa</t></is></c><c r="L388" s="2" t="inlineStr"><is><t>występuje w postaci proleku</t></is></c><c r="M388" s="2" t="inlineStr"><is><t>jest stosowany w profilaktyce choroby zakrzepowo-zatorowej w czasie ciąży</t></is></c><c r="N388" s="2" t="inlineStr" /><c r="O388" s="2" t="inlineStr" /><c r="P388" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q388" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="389"><c r="A389" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B389" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C389" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D389" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E389" s="2" t="inlineStr"><is><t>Do leków działających na receptor P2Y12 zaliczamy:</t></is></c><c r="F389" s="2" t="inlineStr"><is><t>prasugrel</t></is></c><c r="G389" s="2" t="inlineStr" /><c r="H389" s="2" t="inlineStr" /><c r="I389" s="2" t="inlineStr" /><c r="J389" s="2" t="inlineStr" /><c r="K389" s="2" t="inlineStr"><is><t>apiksaban</t></is></c><c r="L389" s="2" t="inlineStr"><is><t>worapaksar</t></is></c><c r="M389" s="2" t="inlineStr"><is><t>dypirydamol</t></is></c><c r="N389" s="2" t="inlineStr" /><c r="O389" s="2" t="inlineStr" /><c r="P389" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q389" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="390"><c r="A390" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B390" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C390" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D390" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E390" s="2" t="inlineStr"><is><t>Do częstych działań niepożądanych atorwastatyny należy:</t></is></c><c r="F390" s="2" t="inlineStr"><is><t>uszkodzenie wątroby</t></is></c><c r="G390" s="2" t="inlineStr" /><c r="H390" s="2" t="inlineStr" /><c r="I390" s="2" t="inlineStr" /><c r="J390" s="2" t="inlineStr" /><c r="K390" s="2" t="inlineStr"><is><t>rogowacenie ciemne</t></is></c><c r="L390" s="2" t="inlineStr"><is><t>miopatia</t></is></c><c r="M390" s="2" t="inlineStr"><is><t>uderzenia gorąca</t></is></c><c r="N390" s="2" t="inlineStr" /><c r="O390" s="2" t="inlineStr" /><c r="P390" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q390" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="391"><c r="A391" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B391" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C391" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D391" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E391" s="2" t="inlineStr"><is><t>Orlistat:</t></is></c><c r="F391" s="2" t="inlineStr"><is><t>może być przyczyną wystąpienia tłuszczowych stolców</t></is></c><c r="G391" s="2" t="inlineStr"><is><t>może być stosowany u osób z chorobami układu krążenia</t></is></c><c r="H391" s="2" t="inlineStr" /><c r="I391" s="2" t="inlineStr" /><c r="J391" s="2" t="inlineStr" /><c r="K391" s="2" t="inlineStr"><is><t>ma wysoką biodostępność po podaniu doustnym</t></is></c><c r="L391" s="2" t="inlineStr"><is><t>zwiększa wchłanianie witaminy D</t></is></c><c r="M391" s="2" t="inlineStr" /><c r="N391" s="2" t="inlineStr" /><c r="O391" s="2" t="inlineStr" /><c r="P391" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q391" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="392"><c r="A392" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B392" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C392" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D392" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E392" s="2" t="inlineStr"><is><t>Wybierz właściwe zestawienia lek prekursorowy – jego aktywny metabolit:</t></is></c><c r="F392" s="2" t="inlineStr"><is><t>cileksetyl kandesartanu → kandesartan</t></is></c><c r="G392" s="2" t="inlineStr" /><c r="H392" s="2" t="inlineStr" /><c r="I392" s="2" t="inlineStr" /><c r="J392" s="2" t="inlineStr" /><c r="K392" s="2" t="inlineStr"><is><t>eplerenon → kanrenon</t></is></c><c r="L392" s="2" t="inlineStr"><is><t>lizynopryl → lizynoprylat</t></is></c><c r="M392" s="2" t="inlineStr"><is><t>nebiwolol → tlenek azotu</t></is></c><c r="N392" s="2" t="inlineStr" /><c r="O392" s="2" t="inlineStr" /><c r="P392" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q392" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="393"><c r="A393" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B393" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C393" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D393" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E393" s="2" t="inlineStr"><is><t>Torasemid w przeciwieństwie do furosemidu nie powoduje:</t></is></c><c r="F393" s="2" t="inlineStr"><is><t>retencji sodu po efekcie natiuretycznym przy podaniu 1 x 24 h</t></is></c><c r="G393" s="2" t="inlineStr" /><c r="H393" s="2" t="inlineStr" /><c r="I393" s="2" t="inlineStr" /><c r="J393" s="2" t="inlineStr" /><c r="K393" s="2" t="inlineStr"><is><t>efektu natiuretycznego po podaniu doustnym</t></is></c><c r="L393" s="2" t="inlineStr"><is><t>reakcji alergicznych w nadwrażliwości na związki sulfonamidowe</t></is></c><c r="M393" s="2" t="inlineStr"><is><t>hiperkalcemii</t></is></c><c r="N393" s="2" t="inlineStr" /><c r="O393" s="2" t="inlineStr" /><c r="P393" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q393" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="394"><c r="A394" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B394" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C394" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D394" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E394" s="2" t="inlineStr"><is><t>Hiponatremię z dużym stężeniem Na+ w moczu (&gt; 20 mmol/l) może spowodować:</t></is></c><c r="F394" s="2" t="inlineStr"><is><t>karbamazepina</t></is></c><c r="G394" s="2" t="inlineStr"><is><t>fluoksetyna</t></is></c><c r="H394" s="2" t="inlineStr"><is><t>indapamid</t></is></c><c r="I394" s="2" t="inlineStr" /><c r="J394" s="2" t="inlineStr" /><c r="K394" s="2" t="inlineStr"><is><t>prednizon</t></is></c><c r="L394" s="2" t="inlineStr" /><c r="M394" s="2" t="inlineStr" /><c r="N394" s="2" t="inlineStr" /><c r="O394" s="2" t="inlineStr" /><c r="P394" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q394" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="395"><c r="A395" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B395" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C395" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D395" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E395" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek-wskazanie:</t></is></c><c r="F395" s="2" t="inlineStr"><is><t>omalizumab – astma</t></is></c><c r="G395" s="2" t="inlineStr"><is><t>denosumab – osteoporoza</t></is></c><c r="H395" s="2" t="inlineStr" /><c r="I395" s="2" t="inlineStr" /><c r="J395" s="2" t="inlineStr" /><c r="K395" s="2" t="inlineStr"><is><t>natalizumab – reumatoidalne zapalenie stawów</t></is></c><c r="L395" s="2" t="inlineStr"><is><t>infliksymab – stwardnienie rozsiane</t></is></c><c r="M395" s="2" t="inlineStr" /><c r="N395" s="2" t="inlineStr" /><c r="O395" s="2" t="inlineStr" /><c r="P395" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q395" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="396"><c r="A396" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B396" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C396" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D396" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E396" s="2" t="inlineStr"><is><t>Jeśli wartość AUC leku oceniona w badaniach przedklinicznych jest większa po podaniu dożylnym niż po podaniu doustnym, to oznacza, że:</t></is></c><c r="F396" s="2" t="inlineStr"><is><t>brak jest wystarczających danych do określenia przyczyny mniejszej wartości AUC leku po podaniu p.o</t></is></c><c r="G396" s="2" t="inlineStr"><is><t>biodostępność leku po podaniu i.v. jest większa niż po podaniu p.o</t></is></c><c r="H396" s="2" t="inlineStr" /><c r="I396" s="2" t="inlineStr" /><c r="J396" s="2" t="inlineStr" /><c r="K396" s="2" t="inlineStr"><is><t>AUC leku ocenione w badaniach klinicznych będzie podobne</t></is></c><c r="L396" s="2" t="inlineStr"><is><t>lek powinien być stosowany na czczo</t></is></c><c r="M396" s="2" t="inlineStr" /><c r="N396" s="2" t="inlineStr" /><c r="O396" s="2" t="inlineStr" /><c r="P396" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q396" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="397"><c r="A397" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B397" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C397" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D397" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E397" s="2" t="inlineStr"><is><t>Daptomycyna ma dwukompartmentowy model rozmieszczenia w organizmie (t 1/2 α= 7 min i t 1/2β = 5 h). Na tej podstawie uzasadniony jest następujący wniosek:</t></is></c><c r="F397" s="2" t="inlineStr"><is><t>po szybkiej fazie dystrybucji następuje wolniejsza faza eliminacji</t></is></c><c r="G397" s="2" t="inlineStr"><is><t>występuje utrudnienie w redystrybucji leku z tkanek do krążenia ogólnego</t></is></c><c r="H397" s="2" t="inlineStr" /><c r="I397" s="2" t="inlineStr" /><c r="J397" s="2" t="inlineStr" /><c r="K397" s="2" t="inlineStr"><is><t>lek wchłania się na dużej długości przewodu pokarmowego</t></is></c><c r="L397" s="2" t="inlineStr"><is><t>lek rozmieszcza się głównie w obszarach hydrofilnych</t></is></c><c r="M397" s="2" t="inlineStr" /><c r="N397" s="2" t="inlineStr" /><c r="O397" s="2" t="inlineStr" /><c r="P397" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q397" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="398"><c r="A398" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B398" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C398" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D398" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E398" s="2" t="inlineStr"><is><t>W terapii POChP u osób o niewielkim ryzyku i nasilonych objawach (kategoria B) stosuje się:</t></is></c><c r="F398" s="2" t="inlineStr"><is><t>salmeterol</t></is></c><c r="G398" s="2" t="inlineStr"><is><t>bromek aklidynium</t></is></c><c r="H398" s="2" t="inlineStr" /><c r="I398" s="2" t="inlineStr" /><c r="J398" s="2" t="inlineStr" /><c r="K398" s="2" t="inlineStr"><is><t>wziewne glikokortykosteroidy</t></is></c><c r="L398" s="2" t="inlineStr"><is><t>roflumilast</t></is></c><c r="M398" s="2" t="inlineStr" /><c r="N398" s="2" t="inlineStr" /><c r="O398" s="2" t="inlineStr" /><c r="P398" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q398" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="399"><c r="A399" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B399" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C399" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D399" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E399" s="2" t="inlineStr"><is><t>Działanie wykrztuśne ma:</t></is></c><c r="F399" s="2" t="inlineStr"><is><t>wyciąg z prawoślazu lekarskiego</t></is></c><c r="G399" s="2" t="inlineStr"><is><t>gwajafenazyna</t></is></c><c r="H399" s="2" t="inlineStr" /><c r="I399" s="2" t="inlineStr" /><c r="J399" s="2" t="inlineStr" /><c r="K399" s="2" t="inlineStr"><is><t>oksykodon</t></is></c><c r="L399" s="2" t="inlineStr"><is><t>mesna</t></is></c><c r="M399" s="2" t="inlineStr" /><c r="N399" s="2" t="inlineStr" /><c r="O399" s="2" t="inlineStr" /><c r="P399" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q399" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="400"><c r="A400" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B400" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C400" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D400" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E400" s="2" t="inlineStr"><is><t>Indakaterol:</t></is></c><c r="F400" s="2" t="inlineStr"><is><t>zwiększa aktywność ruchową rzęsek</t></is></c><c r="G400" s="2" t="inlineStr"><is><t>wykazuje synergizm działania z glikokortykosteroidami</t></is></c><c r="H400" s="2" t="inlineStr" /><c r="I400" s="2" t="inlineStr" /><c r="J400" s="2" t="inlineStr" /><c r="K400" s="2" t="inlineStr"><is><t>jest beta-adrenomimetykiem wziewnym o krótkim czasie działania (SABA)</t></is></c><c r="L400" s="2" t="inlineStr"><is><t>rozszczepia wiązania disiarczkowe w glikoproteinach śluzu</t></is></c><c r="M400" s="2" t="inlineStr" /><c r="N400" s="2" t="inlineStr" /><c r="O400" s="2" t="inlineStr" /><c r="P400" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q400" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="401"><c r="A401" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B401" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C401" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D401" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E401" s="2" t="inlineStr"><is><t>Meta-analiza badań klinicznych:</t></is></c><c r="F401" s="2" t="inlineStr"><is><t>jest uzupełnieniem przeglądu systematycznego</t></is></c><c r="G401" s="2" t="inlineStr"><is><t>może przynieść zupełnie nowe - odmienne wyniki niż badania, na których jest oparta</t></is></c><c r="H401" s="2" t="inlineStr"><is><t>pozwala zwiększyć precyzję oszacowania efektu klinicznego</t></is></c><c r="I401" s="2" t="inlineStr"><is><t>charakteryzuje się heterogenicznością statystyczną, która istotnie wpływa na interpretację wyników</t></is></c><c r="J401" s="2" t="inlineStr" /><c r="K401" s="2" t="inlineStr" /><c r="L401" s="2" t="inlineStr" /><c r="M401" s="2" t="inlineStr" /><c r="N401" s="2" t="inlineStr" /><c r="O401" s="2" t="inlineStr" /><c r="P401" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q401" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="402"><c r="A402" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B402" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C402" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D402" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E402" s="2" t="inlineStr"><is><t>Mieloidalne czynniki wzrostu (G-CSF oraz GM-CSF) znalazły zastosowanie u pacjentów:</t></is></c><c r="F402" s="2" t="inlineStr"><is><t>z ciężką przewlekłą neutropenią</t></is></c><c r="G402" s="2" t="inlineStr"><is><t>po przeszczepieniu komórek macierzystych szpiku kostnego</t></is></c><c r="H402" s="2" t="inlineStr" /><c r="I402" s="2" t="inlineStr" /><c r="J402" s="2" t="inlineStr" /><c r="K402" s="2" t="inlineStr"><is><t>zakażonych wirusem HIV</t></is></c><c r="L402" s="2" t="inlineStr"><is><t>z idiopatyczną plamicą małopłytkową</t></is></c><c r="M402" s="2" t="inlineStr" /><c r="N402" s="2" t="inlineStr" /><c r="O402" s="2" t="inlineStr" /><c r="P402" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q402" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="403"><c r="A403" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B403" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C403" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D403" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E403" s="2" t="inlineStr"><is><t>Które stwierdzenie dotyczące profilaktyki malarii jest prawdziwe?</t></is></c><c r="F403" s="2" t="inlineStr"><is><t>dla większości leków standardowy czas rozpoczynania stosowania leku w profilaktyce wynosi tydzień przed planowaną podróżą</t></is></c><c r="G403" s="2" t="inlineStr"><is><t>nie dysponujemy uniwersalnym lekiem stosowanym w profilaktyce</t></is></c><c r="H403" s="2" t="inlineStr"><is><t>profilaktyka farmakologiczna stanowi uzupełnienie profilaktyki barierowej (odpowiednie ubrania, moskitiery i siatki nasączone DEET)</t></is></c><c r="I403" s="2" t="inlineStr" /><c r="J403" s="2" t="inlineStr" /><c r="K403" s="2" t="inlineStr"><is><t>leki stosuje się profilaktycznie tylko przez tydzień w czasie pobytu na terenie endemicznym</t></is></c><c r="L403" s="2" t="inlineStr" /><c r="M403" s="2" t="inlineStr" /><c r="N403" s="2" t="inlineStr" /><c r="O403" s="2" t="inlineStr" /><c r="P403" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q403" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="404"><c r="A404" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B404" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C404" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D404" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E404" s="2" t="inlineStr"><is><t>Przeprowadzenie eksperymentu leczniczego:</t></is></c><c r="F404" s="2" t="inlineStr"><is><t>jest możliwe, jeśli dostępne metody leczenia okazały się nieskuteczne</t></is></c><c r="G404" s="2" t="inlineStr"><is><t>wymaga świadomej zgody pacjenta</t></is></c><c r="H404" s="2" t="inlineStr" /><c r="I404" s="2" t="inlineStr" /><c r="J404" s="2" t="inlineStr" /><c r="K404" s="2" t="inlineStr"><is><t>ma na celu głównie poszerzenie wiedzy medycznej</t></is></c><c r="L404" s="2" t="inlineStr"><is><t>nie wymaga pozytywnej opinii Komisji Bioetycznej</t></is></c><c r="M404" s="2" t="inlineStr" /><c r="N404" s="2" t="inlineStr" /><c r="O404" s="2" t="inlineStr" /><c r="P404" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q404" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="405"><c r="A405" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B405" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C405" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D405" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E405" s="2" t="inlineStr"><is><t>W leczeniu niedokrwistości megaloblastycznej zastosowanie ma:</t></is></c><c r="F405" s="2" t="inlineStr"><is><t>cyjanokobalamina</t></is></c><c r="G405" s="2" t="inlineStr"><is><t>kwas foliowy</t></is></c><c r="H405" s="2" t="inlineStr" /><c r="I405" s="2" t="inlineStr" /><c r="J405" s="2" t="inlineStr" /><c r="K405" s="2" t="inlineStr"><is><t>siarczan żelaza</t></is></c><c r="L405" s="2" t="inlineStr"><is><t>erytropoetyna</t></is></c><c r="M405" s="2" t="inlineStr" /><c r="N405" s="2" t="inlineStr" /><c r="O405" s="2" t="inlineStr" /><c r="P405" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q405" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="406"><c r="A406" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B406" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C406" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D406" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E406" s="2" t="inlineStr"><is><t>Preparat złożony naltreksonu z bupropionem:</t></is></c><c r="F406" s="2" t="inlineStr"><is><t>istotnie obniża masę ciała w porównaniu z placebo</t></is></c><c r="G406" s="2" t="inlineStr"><is><t>jest zarejestrowany w Europie do leczenia otyłości</t></is></c><c r="H406" s="2" t="inlineStr"><is><t>sprzyja pojawianiu się myśli samobójczych</t></is></c><c r="I406" s="2" t="inlineStr"><is><t>działa antagonistycznie na receptory 5HT2c</t></is></c><c r="J406" s="2" t="inlineStr" /><c r="K406" s="2" t="inlineStr" /><c r="L406" s="2" t="inlineStr" /><c r="M406" s="2" t="inlineStr" /><c r="N406" s="2" t="inlineStr" /><c r="O406" s="2" t="inlineStr" /><c r="P406" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q406" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="407"><c r="A407" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B407" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C407" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D407" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E407" s="2" t="inlineStr"><is><t>W leczeniu uzależnienia od nikotyny wykazano skuteczność:</t></is></c><c r="F407" s="2" t="inlineStr"><is><t>warenikliny</t></is></c><c r="G407" s="2" t="inlineStr"><is><t>cytyzyny</t></is></c><c r="H407" s="2" t="inlineStr"><is><t>nikotynowej terapii zastępczej</t></is></c><c r="I407" s="2" t="inlineStr" /><c r="J407" s="2" t="inlineStr" /><c r="K407" s="2" t="inlineStr"><is><t>benzodiazepin</t></is></c><c r="L407" s="2" t="inlineStr" /><c r="M407" s="2" t="inlineStr" /><c r="N407" s="2" t="inlineStr" /><c r="O407" s="2" t="inlineStr" /><c r="P407" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q407" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="408"><c r="A408" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B408" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C408" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D408" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E408" s="2" t="inlineStr"><is><t>Elementami nadzoru nad bezpieczeństwem farmakoterapii jest:</t></is></c><c r="F408" s="2" t="inlineStr"><is><t>plan Zarządzania Ryzykiem</t></is></c><c r="G408" s="2" t="inlineStr"><is><t>strona internetowa Urzędu Rejestracji Produktów Leczniczych, Wyrobów Medycznych i Produktów Biobójczych</t></is></c><c r="H408" s="2" t="inlineStr"><is><t>raport PSUR</t></is></c><c r="I408" s="2" t="inlineStr"><is><t>baza zarejestrowanych produktów leczniczych prowadzona przez Europejską Agencję Leków</t></is></c><c r="J408" s="2" t="inlineStr" /><c r="K408" s="2" t="inlineStr" /><c r="L408" s="2" t="inlineStr" /><c r="M408" s="2" t="inlineStr" /><c r="N408" s="2" t="inlineStr" /><c r="O408" s="2" t="inlineStr" /><c r="P408" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q408" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="409"><c r="A409" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B409" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C409" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D409" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E409" s="2" t="inlineStr"><is><t>URPL - Urząd Rejestracji Produktów Leczniczych, Wyrobów Medycznych i Produktów Biobójczych ocenia działania niepożądane zarejestrowanych:</t></is></c><c r="F409" s="2" t="inlineStr"><is><t>leków homeopatycznych</t></is></c><c r="G409" s="2" t="inlineStr"><is><t>leków dostępnych bez recepty</t></is></c><c r="H409" s="2" t="inlineStr"><is><t>leków pochodzenia roślinnego</t></is></c><c r="I409" s="2" t="inlineStr" /><c r="J409" s="2" t="inlineStr" /><c r="K409" s="2" t="inlineStr"><is><t>suplementów diety</t></is></c><c r="L409" s="2" t="inlineStr" /><c r="M409" s="2" t="inlineStr" /><c r="N409" s="2" t="inlineStr" /><c r="O409" s="2" t="inlineStr" /><c r="P409" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q409" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="410"><c r="A410" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B410" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C410" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D410" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E410" s="2" t="inlineStr"><is><t>Teratogenem człowieka o udokumentowanym działaniu jest:</t></is></c><c r="F410" s="2" t="inlineStr"><is><t>metotreksat</t></is></c><c r="G410" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="H410" s="2" t="inlineStr"><is><t>lit</t></is></c><c r="I410" s="2" t="inlineStr" /><c r="J410" s="2" t="inlineStr" /><c r="K410" s="2" t="inlineStr"><is><t>tiamazol tiamazol ma kategorię D</t></is></c><c r="L410" s="2" t="inlineStr" /><c r="M410" s="2" t="inlineStr" /><c r="N410" s="2" t="inlineStr" /><c r="O410" s="2" t="inlineStr" /><c r="P410" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q410" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="411"><c r="A411" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B411" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C411" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D411" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E411" s="2" t="inlineStr"><is><t>Alfakalcydol:</t></is></c><c r="F411" s="2" t="inlineStr"><is><t>koryguje zaburzenia wapniowe w przewlekłej chorobie nerek</t></is></c><c r="G411" s="2" t="inlineStr"><is><t>koryguje zaburzenia wapniowe w niedoczynności przytarczyc</t></is></c><c r="H411" s="2" t="inlineStr"><is><t>zmniejsza ryzyko osteoporotycznych złamań kości</t></is></c><c r="I411" s="2" t="inlineStr" /><c r="J411" s="2" t="inlineStr" /><c r="K411" s="2" t="inlineStr"><is><t>chroni przed chorobami wirusowymi</t></is></c><c r="L411" s="2" t="inlineStr" /><c r="M411" s="2" t="inlineStr" /><c r="N411" s="2" t="inlineStr" /><c r="O411" s="2" t="inlineStr" /><c r="P411" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q411" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="412"><c r="A412" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B412" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C412" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D412" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E412" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie:</t></is></c><c r="F412" s="2" t="inlineStr"><is><t>gliklazyd może powodować przyrost masy ciała</t></is></c><c r="G412" s="2" t="inlineStr"><is><t>metformina może być przyczyną kwasicy mleczanowej</t></is></c><c r="H412" s="2" t="inlineStr"><is><t>empagliflozyna zwiększa ryzyko zakażeń w obrębie miednicy mniejszej</t></is></c><c r="I412" s="2" t="inlineStr" /><c r="J412" s="2" t="inlineStr" /><c r="K412" s="2" t="inlineStr"><is><t>liraglutyd wykazuje niekorzystny efekt sercowo-naczyniowy</t></is></c><c r="L412" s="2" t="inlineStr" /><c r="M412" s="2" t="inlineStr" /><c r="N412" s="2" t="inlineStr" /><c r="O412" s="2" t="inlineStr" /><c r="P412" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q412" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="413"><c r="A413" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B413" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C413" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D413" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E413" s="2" t="inlineStr"><is><t>Klemastyna:</t></is></c><c r="F413" s="2" t="inlineStr"><is><t>dobrze przenika przez barierę krew- mózg 22</t></is></c><c r="G413" s="2" t="inlineStr"><is><t>może być stosowana od 2 r. ż</t></is></c><c r="H413" s="2" t="inlineStr" /><c r="I413" s="2" t="inlineStr" /><c r="J413" s="2" t="inlineStr" /><c r="K413" s="2" t="inlineStr"><is><t>selektywnie działa na rec. H1</t></is></c><c r="L413" s="2" t="inlineStr"><is><t>jest lekiem z wyboru w leczeniu przewlekłego alergicznego nieżytu nosa</t></is></c><c r="M413" s="2" t="inlineStr" /><c r="N413" s="2" t="inlineStr" /><c r="O413" s="2" t="inlineStr" /><c r="P413" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q413" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="414"><c r="A414" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B414" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C414" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D414" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E414" s="2" t="inlineStr"><is><t>W stanie padaczkowym zalecane jest zastosowanie:</t></is></c><c r="F414" s="2" t="inlineStr"><is><t>lorazepamu dożylnie</t></is></c><c r="G414" s="2" t="inlineStr"><is><t>fenytoiny we wlewie dożylnym</t></is></c><c r="H414" s="2" t="inlineStr" /><c r="I414" s="2" t="inlineStr" /><c r="J414" s="2" t="inlineStr" /><c r="K414" s="2" t="inlineStr"><is><t>diazepamu domięśniowo</t></is></c><c r="L414" s="2" t="inlineStr"><is><t>fenobarbitalu podskórnie</t></is></c><c r="M414" s="2" t="inlineStr" /><c r="N414" s="2" t="inlineStr" /><c r="O414" s="2" t="inlineStr" /><c r="P414" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q414" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="415"><c r="A415" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B415" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C415" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D415" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E415" s="2" t="inlineStr"><is><t>Inhibitorem kinazy tyrozynowej o działaniu przeciwnowotworowym jest:</t></is></c><c r="F415" s="2" t="inlineStr"><is><t>imatynib</t></is></c><c r="G415" s="2" t="inlineStr"><is><t>sunitynib</t></is></c><c r="H415" s="2" t="inlineStr" /><c r="I415" s="2" t="inlineStr" /><c r="J415" s="2" t="inlineStr" /><c r="K415" s="2" t="inlineStr"><is><t>ewerolimus</t></is></c><c r="L415" s="2" t="inlineStr"><is><t>bortezomib</t></is></c><c r="M415" s="2" t="inlineStr" /><c r="N415" s="2" t="inlineStr" /><c r="O415" s="2" t="inlineStr" /><c r="P415" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q415" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="416"><c r="A416" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B416" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C416" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D416" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E416" s="2" t="inlineStr"><is><t>Skuteczne leczenie w owrzodzeniach żylnych obejmuje:</t></is></c><c r="F416" s="2" t="inlineStr"><is><t>opatrunki hydrokoloidowe</t></is></c><c r="G416" s="2" t="inlineStr" /><c r="H416" s="2" t="inlineStr" /><c r="I416" s="2" t="inlineStr" /><c r="J416" s="2" t="inlineStr" /><c r="K416" s="2" t="inlineStr"><is><t>wyciągi zawierające glikozydy kasztanowca</t></is></c><c r="L416" s="2" t="inlineStr"><is><t>heparynoidy do stosowania miejscowego</t></is></c><c r="M416" s="2" t="inlineStr"><is><t>dobesylan wapnia</t></is></c><c r="N416" s="2" t="inlineStr" /><c r="O416" s="2" t="inlineStr" /><c r="P416" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q416" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="417"><c r="A417" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B417" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C417" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D417" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E417" s="2" t="inlineStr"><is><t>W leczeniu zaburzeń lękowych z napadami paniki można zastosować:</t></is></c><c r="F417" s="2" t="inlineStr"><is><t>doksepinę</t></is></c><c r="G417" s="2" t="inlineStr"><is><t>alprazolam</t></is></c><c r="H417" s="2" t="inlineStr" /><c r="I417" s="2" t="inlineStr" /><c r="J417" s="2" t="inlineStr" /><c r="K417" s="2" t="inlineStr"><is><t>rysperydon</t></is></c><c r="L417" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="M417" s="2" t="inlineStr" /><c r="N417" s="2" t="inlineStr" /><c r="O417" s="2" t="inlineStr" /><c r="P417" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q417" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="418"><c r="A418" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B418" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C418" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D418" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E418" s="2" t="inlineStr"><is><t>Działanie przeciwwymiotne ma:</t></is></c><c r="F418" s="2" t="inlineStr"><is><t>skopolamina</t></is></c><c r="G418" s="2" t="inlineStr"><is><t>dimenhydrinat</t></is></c><c r="H418" s="2" t="inlineStr" /><c r="I418" s="2" t="inlineStr" /><c r="J418" s="2" t="inlineStr" /><c r="K418" s="2" t="inlineStr"><is><t>lewetyracetam</t></is></c><c r="L418" s="2" t="inlineStr"><is><t>wortioksetyna</t></is></c><c r="M418" s="2" t="inlineStr" /><c r="N418" s="2" t="inlineStr" /><c r="O418" s="2" t="inlineStr" /><c r="P418" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q418" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="419"><c r="A419" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B419" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C419" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D419" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E419" s="2" t="inlineStr"><is><t>Amfetamina:</t></is></c><c r="F419" s="2" t="inlineStr"><is><t>może działać neurotoksycznie</t></is></c><c r="G419" s="2" t="inlineStr" /><c r="H419" s="2" t="inlineStr" /><c r="I419" s="2" t="inlineStr" /><c r="J419" s="2" t="inlineStr" /><c r="K419" s="2" t="inlineStr"><is><t>bezpośrednio pobudza receptory dopaminergiczne</t></is></c><c r="L419" s="2" t="inlineStr"><is><t>wzmaga apetyt</t></is></c><c r="M419" s="2" t="inlineStr"><is><t>obniża ciśnienie tętnicze krwi</t></is></c><c r="N419" s="2" t="inlineStr" /><c r="O419" s="2" t="inlineStr" /><c r="P419" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q419" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="420"><c r="A420" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B420" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C420" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D420" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E420" s="2" t="inlineStr"><is><t>Kwetiapina:</t></is></c><c r="F420" s="2" t="inlineStr"><is><t>zwiększa ryzyko wystąpienia zespołu metabolicznego</t></is></c><c r="G420" s="2" t="inlineStr"><is><t>może być stosowana jako lek normotymiczny</t></is></c><c r="H420" s="2" t="inlineStr" /><c r="I420" s="2" t="inlineStr" /><c r="J420" s="2" t="inlineStr" /><c r="K420" s="2" t="inlineStr"><is><t>nie powoduje złośliwego zespołu neuroleptycznego</t></is></c><c r="L420" s="2" t="inlineStr"><is><t>nie wykazuje aktywności cholinolitycznej</t></is></c><c r="M420" s="2" t="inlineStr" /><c r="N420" s="2" t="inlineStr" /><c r="O420" s="2" t="inlineStr" /><c r="P420" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q420" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="421"><c r="A421" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B421" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C421" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D421" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E421" s="2" t="inlineStr"><is><t>W chorobie Parkinsona lewodopę można podawać jednocześnie z:</t></is></c><c r="F421" s="2" t="inlineStr"><is><t>benserazydem</t></is></c><c r="G421" s="2" t="inlineStr"><is><t>bromokryptyną</t></is></c><c r="H421" s="2" t="inlineStr"><is><t>rotygotyną</t></is></c><c r="I421" s="2" t="inlineStr"><is><t>entekaponem</t></is></c><c r="J421" s="2" t="inlineStr" /><c r="K421" s="2" t="inlineStr" /><c r="L421" s="2" t="inlineStr" /><c r="M421" s="2" t="inlineStr" /><c r="N421" s="2" t="inlineStr" /><c r="O421" s="2" t="inlineStr" /><c r="P421" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q421" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="422"><c r="A422" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B422" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C422" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D422" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E422" s="2" t="inlineStr"><is><t>Wystąpienie objawów pozapiramidowych w przebiegu leczenia lekami przeciwpsychotycznymi:</t></is></c><c r="F422" s="2" t="inlineStr"><is><t>jest wskazaniem do modyfikacji dawki leku</t></is></c><c r="G422" s="2" t="inlineStr"><is><t>zależy od procentu zablokowania receptorów D2 w układzie nigrostriatalnym</t></is></c><c r="H422" s="2" t="inlineStr" /><c r="I422" s="2" t="inlineStr" /><c r="J422" s="2" t="inlineStr" /><c r="K422" s="2" t="inlineStr"><is><t>jest wskazaniem do natychmiastowej zmiany leku</t></is></c><c r="L422" s="2" t="inlineStr"><is><t>jest nieodłącznym elementem leczenia przeciwpsychotycznego, obserwowanym u wszystkich leczonych pacjentów</t></is></c><c r="M422" s="2" t="inlineStr" /><c r="N422" s="2" t="inlineStr" /><c r="O422" s="2" t="inlineStr" /><c r="P422" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q422" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="423"><c r="A423" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B423" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C423" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D423" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E423" s="2" t="inlineStr"><is><t>W leczeniu epizodu depresyjnego można zastosować w monoterapii:</t></is></c><c r="F423" s="2" t="inlineStr"><is><t>sertralinę</t></is></c><c r="G423" s="2" t="inlineStr"><is><t>mirtazapinę</t></is></c><c r="H423" s="2" t="inlineStr" /><c r="I423" s="2" t="inlineStr" /><c r="J423" s="2" t="inlineStr" /><c r="K423" s="2" t="inlineStr"><is><t>sulpiryd</t></is></c><c r="L423" s="2" t="inlineStr"><is><t>sertindol</t></is></c><c r="M423" s="2" t="inlineStr" /><c r="N423" s="2" t="inlineStr" /><c r="O423" s="2" t="inlineStr" /><c r="P423" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q423" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="424"><c r="A424" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B424" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C424" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D424" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E424" s="2" t="inlineStr"><is><t>U chorego leczonego escitalopramem ryzyko wystąpienia zespołu serotoninergicznego rośnie gdy dołączymy do terapii:</t></is></c><c r="F424" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="G424" s="2" t="inlineStr"><is><t>tramadol</t></is></c><c r="H424" s="2" t="inlineStr"><is><t>ziele dziurawca</t></is></c><c r="I424" s="2" t="inlineStr"><is><t>korzeń żeń-szenia</t></is></c><c r="J424" s="2" t="inlineStr" /><c r="K424" s="2" t="inlineStr" /><c r="L424" s="2" t="inlineStr" /><c r="M424" s="2" t="inlineStr" /><c r="N424" s="2" t="inlineStr" /><c r="O424" s="2" t="inlineStr" /><c r="P424" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q424" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="425"><c r="A425" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B425" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C425" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D425" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E425" s="2" t="inlineStr"><is><t>Podanie węgla aktywowanego nie przyniesie efektu w przypadku zatrucia:</t></is></c><c r="F425" s="2" t="inlineStr"><is><t>etanolem</t></is></c><c r="G425" s="2" t="inlineStr"><is><t>ołowiem</t></is></c><c r="H425" s="2" t="inlineStr"><is><t>benzyną</t></is></c><c r="I425" s="2" t="inlineStr" /><c r="J425" s="2" t="inlineStr" /><c r="K425" s="2" t="inlineStr"><is><t>benzodiazepinami</t></is></c><c r="L425" s="2" t="inlineStr" /><c r="M425" s="2" t="inlineStr" /><c r="N425" s="2" t="inlineStr" /><c r="O425" s="2" t="inlineStr" /><c r="P425" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q425" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="426"><c r="A426" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B426" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C426" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D426" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E426" s="2" t="inlineStr"><is><t>U osób w starszym wieku na zmiany farmakokinetyki leków mogą wpływać:</t></is></c><c r="F426" s="2" t="inlineStr"><is><t>hipoproteinemia</t></is></c><c r="G426" s="2" t="inlineStr"><is><t>spadek masy wątroby</t></is></c><c r="H426" s="2" t="inlineStr" /><c r="I426" s="2" t="inlineStr" /><c r="J426" s="2" t="inlineStr" /><c r="K426" s="2" t="inlineStr"><is><t>zanik kosmków jelitowych</t></is></c><c r="L426" s="2" t="inlineStr"><is><t>obniżenie stężenia kwaśnej alfa-1 glikoproteiny</t></is></c><c r="M426" s="2" t="inlineStr" /><c r="N426" s="2" t="inlineStr" /><c r="O426" s="2" t="inlineStr" /><c r="P426" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q426" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="427"><c r="A427" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B427" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C427" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D427" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E427" s="2" t="inlineStr"><is><t>Inhibitorem fosfodiesterazy typu 5 jest:</t></is></c><c r="F427" s="2" t="inlineStr"><is><t>tadalafil</t></is></c><c r="G427" s="2" t="inlineStr" /><c r="H427" s="2" t="inlineStr" /><c r="I427" s="2" t="inlineStr" /><c r="J427" s="2" t="inlineStr" /><c r="K427" s="2" t="inlineStr"><is><t>trospium</t></is></c><c r="L427" s="2" t="inlineStr"><is><t>alprostadyl</t></is></c><c r="M427" s="2" t="inlineStr"><is><t>solifenacyna</t></is></c><c r="N427" s="2" t="inlineStr" /><c r="O427" s="2" t="inlineStr" /><c r="P427" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q427" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="428"><c r="A428" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B428" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C428" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D428" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E428" s="2" t="inlineStr"><is><t>W zespole jelita drażliwego może być skuteczne zastosowanie:</t></is></c><c r="F428" s="2" t="inlineStr"><is><t>mebeweryny</t></is></c><c r="G428" s="2" t="inlineStr"><is><t>atropiny z difenoksylatem</t></is></c><c r="H428" s="2" t="inlineStr"><is><t>trimebutyny</t></is></c><c r="I428" s="2" t="inlineStr"><is><t>Bifidobacterium</t></is></c><c r="J428" s="2" t="inlineStr" /><c r="K428" s="2" t="inlineStr" /><c r="L428" s="2" t="inlineStr" /><c r="M428" s="2" t="inlineStr" /><c r="N428" s="2" t="inlineStr" /><c r="O428" s="2" t="inlineStr" /><c r="P428" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q428" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="429"><c r="A429" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B429" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C429" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D429" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E429" s="2" t="inlineStr"><is><t>Przewlekłe stosowanie pantoprazolu:</t></is></c><c r="F429" s="2" t="inlineStr"><is><t>zwiększa ryzyko zakażeń dróg oddechowych</t></is></c><c r="G429" s="2" t="inlineStr"><is><t>zaburza wchłanianie wapnia z przewodu pokarmowego</t></is></c><c r="H429" s="2" t="inlineStr"><is><t>zmniejsza działanie klopidogrelu</t></is></c><c r="I429" s="2" t="inlineStr" /><c r="J429" s="2" t="inlineStr" /><c r="K429" s="2" t="inlineStr"><is><t>zmniejsza ryzyko złamania szyjki kości udowej</t></is></c><c r="L429" s="2" t="inlineStr" /><c r="M429" s="2" t="inlineStr" /><c r="N429" s="2" t="inlineStr" /><c r="O429" s="2" t="inlineStr" /><c r="P429" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q429" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="430"><c r="A430" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B430" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C430" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D430" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E430" s="2" t="inlineStr"><is><t>Wskazaniem do eradykacji Helicobacter pylori może być:</t></is></c><c r="F430" s="2" t="inlineStr"><is><t>planowane leczenie niesteroidowymi lekami przeciwzapalnymi</t></is></c><c r="G430" s="2" t="inlineStr"><is><t>niedokrwistość syderopeniczna</t></is></c><c r="H430" s="2" t="inlineStr"><is><t>chłoniak żołądka typu MALT</t></is></c><c r="I430" s="2" t="inlineStr"><is><t>aktywna choroba wrzodowa żołądka/dwunastnicy</t></is></c><c r="J430" s="2" t="inlineStr" /><c r="K430" s="2" t="inlineStr" /><c r="L430" s="2" t="inlineStr" /><c r="M430" s="2" t="inlineStr" /><c r="N430" s="2" t="inlineStr" /><c r="O430" s="2" t="inlineStr" /><c r="P430" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q430" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="431"><c r="A431" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B431" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C431" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D431" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E431" s="2" t="inlineStr"><is><t>W profilaktyce krwawienia z żylaków przełyku w przebiegu nadciśnienia wrotnego stosuje się:</t></is></c><c r="F431" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="G431" s="2" t="inlineStr"><is><t>karwedilol</t></is></c><c r="H431" s="2" t="inlineStr" /><c r="I431" s="2" t="inlineStr" /><c r="J431" s="2" t="inlineStr" /><c r="K431" s="2" t="inlineStr"><is><t>doksazosynę</t></is></c><c r="L431" s="2" t="inlineStr"><is><t>klonidynę</t></is></c><c r="M431" s="2" t="inlineStr" /><c r="N431" s="2" t="inlineStr" /><c r="O431" s="2" t="inlineStr" /><c r="P431" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q431" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="432"><c r="A432" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B432" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C432" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D432" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E432" s="2" t="inlineStr"><is><t>Noradrenalinę (NA) podaje się w dawce 0,2-1 μg/kg/min rozpoczynając od najmniejszej dawki. Wskaż właściwą szybkość wlewu w początkowym leczeniu 50 kg kobiety z ciśnieniem skurczowym ok. 60 mmHg w przebiegu ostrej niewydolności serca:</t></is></c><c r="F432" s="2" t="inlineStr"><is><t>roztwór 4 mg NA/40 ml 0,9% NaCl – 6 ml/h</t></is></c><c r="G432" s="2" t="inlineStr"><is><t>roztwór 1 mg NA/50 ml 0,9% NaCl – 30 ml/h</t></is></c><c r="H432" s="2" t="inlineStr"><is><t>roztwór 5 mg NA/25 ml 0,9% NaCl - 3 ml/h</t></is></c><c r="I432" s="2" t="inlineStr"><is><t>roztwór 3 mg NA/30 ml 0,9 % NaCl – 6 ml/h</t></is></c><c r="J432" s="2" t="inlineStr" /><c r="K432" s="2" t="inlineStr" /><c r="L432" s="2" t="inlineStr" /><c r="M432" s="2" t="inlineStr" /><c r="N432" s="2" t="inlineStr" /><c r="O432" s="2" t="inlineStr" /><c r="P432" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q432" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="433"><c r="A433" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B433" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C433" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D433" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E433" s="2" t="inlineStr"><is><t>Działanie naczyniorozszerzające ma:</t></is></c><c r="F433" s="2" t="inlineStr"><is><t>terazosyna</t></is></c><c r="G433" s="2" t="inlineStr"><is><t>nebiwolol</t></is></c><c r="H433" s="2" t="inlineStr"><is><t>zofenopryl</t></is></c><c r="I433" s="2" t="inlineStr"><is><t>lerkanidypina</t></is></c><c r="J433" s="2" t="inlineStr" /><c r="K433" s="2" t="inlineStr" /><c r="L433" s="2" t="inlineStr" /><c r="M433" s="2" t="inlineStr" /><c r="N433" s="2" t="inlineStr" /><c r="O433" s="2" t="inlineStr" /><c r="P433" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q433" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="434"><c r="A434" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B434" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C434" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D434" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E434" s="2" t="inlineStr"><is><t>Podobny mechanizm działania na poziomie molekularnym mają:</t></is></c><c r="F434" s="2" t="inlineStr"><is><t>monoazotan izosorbidu</t></is></c><c r="G434" s="2" t="inlineStr"><is><t>nesirytyd</t></is></c><c r="H434" s="2" t="inlineStr"><is><t>riociguat</t></is></c><c r="I434" s="2" t="inlineStr"><is><t>wardenafil</t></is></c><c r="J434" s="2" t="inlineStr" /><c r="K434" s="2" t="inlineStr" /><c r="L434" s="2" t="inlineStr" /><c r="M434" s="2" t="inlineStr" /><c r="N434" s="2" t="inlineStr" /><c r="O434" s="2" t="inlineStr" /><c r="P434" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q434" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="435"><c r="A435" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B435" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C435" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D435" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E435" s="2" t="inlineStr"><is><t>Beta-adrenolityki w chorobie niedokrwiennej serca:</t></is></c><c r="F435" s="2" t="inlineStr"><is><t>zmniejszają agregację płytek krwi</t></is></c><c r="G435" s="2" t="inlineStr"><is><t>zwiększają przepływ wieńcowy</t></is></c><c r="H435" s="2" t="inlineStr"><is><t>zapobiegają proarytmicznemu działaniu katecholamin</t></is></c><c r="I435" s="2" t="inlineStr"><is><t>zmniejszają kurczliwość mięśnia sercowego</t></is></c><c r="J435" s="2" t="inlineStr" /><c r="K435" s="2" t="inlineStr" /><c r="L435" s="2" t="inlineStr" /><c r="M435" s="2" t="inlineStr" /><c r="N435" s="2" t="inlineStr" /><c r="O435" s="2" t="inlineStr" /><c r="P435" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q435" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="436"><c r="A436" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B436" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C436" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D436" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E436" s="2" t="inlineStr"><is><t>Ranolazyna ma działanie:</t></is></c><c r="F436" s="2" t="inlineStr"><is><t>antyarytmiczne</t></is></c><c r="G436" s="2" t="inlineStr"><is><t>korzystne metaboliczne w kardiomiocytach</t></is></c><c r="H436" s="2" t="inlineStr"><is><t>zmniejszające naprężenie ściany lewej komory</t></is></c><c r="I436" s="2" t="inlineStr" /><c r="J436" s="2" t="inlineStr" /><c r="K436" s="2" t="inlineStr"><is><t>inotropowe dodatnie</t></is></c><c r="L436" s="2" t="inlineStr" /><c r="M436" s="2" t="inlineStr" /><c r="N436" s="2" t="inlineStr" /><c r="O436" s="2" t="inlineStr" /><c r="P436" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q436" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="437"><c r="A437" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B437" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C437" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D437" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E437" s="2" t="inlineStr"><is><t>Jakie leki zlecisz 48-letniemu bezobjawowemu mężczyźnie z BMI = 24,1 kg/m2, palącemu 20 papierosów dziennie od ok. 30 lat, z ciśnieniem tętniczym 150-155 mmHg w powtarzanych pomiarach i ze stężeniem cholesterolu LDL w surowicy = 200 mg/dl:</t></is></c><c r="F437" s="2" t="inlineStr"><is><t>ramipryl</t></is></c><c r="G437" s="2" t="inlineStr"><is><t>nikotynę w inhalacjach pod warunkiem zaprzestania palenia papierosów</t></is></c><c r="H437" s="2" t="inlineStr"><is><t>rosuwastatynę</t></is></c><c r="I437" s="2" t="inlineStr" /><c r="J437" s="2" t="inlineStr" /><c r="K437" s="2" t="inlineStr"><is><t>klopidogrel</t></is></c><c r="L437" s="2" t="inlineStr" /><c r="M437" s="2" t="inlineStr" /><c r="N437" s="2" t="inlineStr" /><c r="O437" s="2" t="inlineStr" /><c r="P437" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q437" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="438"><c r="A438" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B438" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C438" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D438" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E438" s="2" t="inlineStr"><is><t>W niewydolności serca przeżycie chorych poprawia:</t></is></c><c r="F438" s="2" t="inlineStr"><is><t>eplerenon</t></is></c><c r="G438" s="2" t="inlineStr" /><c r="H438" s="2" t="inlineStr" /><c r="I438" s="2" t="inlineStr" /><c r="J438" s="2" t="inlineStr" /><c r="K438" s="2" t="inlineStr"><is><t>atenolol</t></is></c><c r="L438" s="2" t="inlineStr"><is><t>tolwaptan</t></is></c><c r="M438" s="2" t="inlineStr"><is><t>digoksyna</t></is></c><c r="N438" s="2" t="inlineStr" /><c r="O438" s="2" t="inlineStr" /><c r="P438" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q438" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="439"><c r="A439" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B439" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C439" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D439" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E439" s="2" t="inlineStr"><is><t>55-letni mężczyzna ma trwający od ok. 60-min ucisk za mostkiem, który wystąpił podczas ubierania się po wstaniu z łóżka, w EKG rozlane obniżenia ST w odprowadzeniach znad ściany przedniej. Jako lekarz pierwszego kontaktu medycznego zastosujesz:</t></is></c><c r="F439" s="2" t="inlineStr"><is><t>tikagrelor w dawce 180 mg p.o</t></is></c><c r="G439" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy w dawce 300 mg p.o</t></is></c><c r="H439" s="2" t="inlineStr" /><c r="I439" s="2" t="inlineStr" /><c r="J439" s="2" t="inlineStr" /><c r="K439" s="2" t="inlineStr"><is><t>morfinę w dawkach frakcjonowanych i.v</t></is></c><c r="L439" s="2" t="inlineStr"><is><t>enoksaparynę w dawce leczniczej s.c</t></is></c><c r="M439" s="2" t="inlineStr" /><c r="N439" s="2" t="inlineStr" /><c r="O439" s="2" t="inlineStr" /><c r="P439" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q439" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="440"><c r="A440" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B440" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C440" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D440" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E440" s="2" t="inlineStr"><is><t>Które stwierdzenie dotyczące redukcji ryzyka sercowo-naczyniowego jest prawdziwe:</t></is></c><c r="F440" s="2" t="inlineStr"><is><t>nikotynowa terapia zastępcza jest bezpieczna i powinna być rutynowo oferowana</t></is></c><c r="G440" s="2" t="inlineStr" /><c r="H440" s="2" t="inlineStr" /><c r="I440" s="2" t="inlineStr" /><c r="J440" s="2" t="inlineStr" /><c r="K440" s="2" t="inlineStr"><is><t>niezależnie od wieku należy dążyć do redukcji ciśnienia tętniczego do &lt; 140/90 mmHg</t></is></c><c r="L440" s="2" t="inlineStr"><is><t>obniżenie poziomu hemoglobiny glikowanej HgbA1c do ≤ 6% u osób z cukrzycą poprawia przeżycie w porównaniu z wyższymi wartościami HbA1c</t></is></c><c r="M440" s="2" t="inlineStr"><is><t>wysokie prawidłowe ciśnienie krwi powinno być leczone farmakologicznie</t></is></c><c r="N440" s="2" t="inlineStr" /><c r="O440" s="2" t="inlineStr" /><c r="P440" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q440" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="441"><c r="A441" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B441" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C441" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D441" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E441" s="2" t="inlineStr"><is><t>W leczeniu nadciśnienia tętniczego przeciwwskazane jest połączenie:</t></is></c><c r="F441" s="2" t="inlineStr"><is><t>ramipryl + telmisartan</t></is></c><c r="G441" s="2" t="inlineStr" /><c r="H441" s="2" t="inlineStr" /><c r="I441" s="2" t="inlineStr" /><c r="J441" s="2" t="inlineStr" /><c r="K441" s="2" t="inlineStr"><is><t>amlodypina + chlortalidon</t></is></c><c r="L441" s="2" t="inlineStr"><is><t>amlodypina + peryndopryl</t></is></c><c r="M441" s="2" t="inlineStr"><is><t>peryndopryl + indapamid</t></is></c><c r="N441" s="2" t="inlineStr" /><c r="O441" s="2" t="inlineStr" /><c r="P441" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q441" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="442"><c r="A442" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B442" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C442" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D442" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E442" s="2" t="inlineStr"><is><t>U pacjenta z dławicą piersiową i niskim ciśnieniem tętniczym krwi można zastosować:</t></is></c><c r="F442" s="2" t="inlineStr"><is><t>ranolazynę</t></is></c><c r="G442" s="2" t="inlineStr"><is><t>iwabradynę</t></is></c><c r="H442" s="2" t="inlineStr"><is><t>trimetazydynę</t></is></c><c r="I442" s="2" t="inlineStr" /><c r="J442" s="2" t="inlineStr" /><c r="K442" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="L442" s="2" t="inlineStr" /><c r="M442" s="2" t="inlineStr" /><c r="N442" s="2" t="inlineStr" /><c r="O442" s="2" t="inlineStr" /><c r="P442" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q442" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="443"><c r="A443" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B443" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C443" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D443" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E443" s="2" t="inlineStr"><is><t>Propafenon:</t></is></c><c r="F443" s="2" t="inlineStr"><is><t>jest antagonistą kanału sodowego</t></is></c><c r="G443" s="2" t="inlineStr"><is><t>ma działanie betaadrenolityczne</t></is></c><c r="H443" s="2" t="inlineStr" /><c r="I443" s="2" t="inlineStr" /><c r="J443" s="2" t="inlineStr" /><c r="K443" s="2" t="inlineStr"><is><t>rozszerza nasierdziowe tętnice wieńcowe</t></is></c><c r="L443" s="2" t="inlineStr"><is><t>jest przeciwwskazany w zespole preekscytacji (WPW)</t></is></c><c r="M443" s="2" t="inlineStr" /><c r="N443" s="2" t="inlineStr" /><c r="O443" s="2" t="inlineStr" /><c r="P443" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q443" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="444"><c r="A444" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B444" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C444" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D444" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E444" s="2" t="inlineStr"><is><t>Teoretyczną przesłanką stosowania inhibitorów konwertazy angiotensyny w przewlekłej skurczowej niewydolności serca jest:</t></is></c><c r="F444" s="2" t="inlineStr"><is><t>odwracanie włóknienia miokardium</t></is></c><c r="G444" s="2" t="inlineStr"><is><t>odwracanie przerostu kardiomiocytów</t></is></c><c r="H444" s="2" t="inlineStr"><is><t>korzystne bezpośrednie działanie hemodynamiczne</t></is></c><c r="I444" s="2" t="inlineStr" /><c r="J444" s="2" t="inlineStr" /><c r="K444" s="2" t="inlineStr"><is><t>zwiększenie naprężenia ściany lewej komory</t></is></c><c r="L444" s="2" t="inlineStr" /><c r="M444" s="2" t="inlineStr" /><c r="N444" s="2" t="inlineStr" /><c r="O444" s="2" t="inlineStr" /><c r="P444" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q444" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="445"><c r="A445" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B445" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C445" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D445" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E445" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie:</t></is></c><c r="F445" s="2" t="inlineStr"><is><t>Diklofenak działa hepatotoksycznie</t></is></c><c r="G445" s="2" t="inlineStr" /><c r="H445" s="2" t="inlineStr" /><c r="I445" s="2" t="inlineStr" /><c r="J445" s="2" t="inlineStr" /><c r="K445" s="2" t="inlineStr"><is><t>Paracetamol działa antyagregacyjnie</t></is></c><c r="L445" s="2" t="inlineStr"><is><t>Naproksen działa hipotensyjnie</t></is></c><c r="M445" s="2" t="inlineStr"><is><t>Metamizol działa prozakrzepowo</t></is></c><c r="N445" s="2" t="inlineStr" /><c r="O445" s="2" t="inlineStr" /><c r="P445" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q445" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="446"><c r="A446" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B446" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C446" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D446" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E446" s="2" t="inlineStr"><is><t>Tramadol jest:</t></is></c><c r="F446" s="2" t="inlineStr"><is><t>Inhibitorem wychwytu zwrotnego serotoniny</t></is></c><c r="G446" s="2" t="inlineStr"><is><t>Agonistą receptorów opioidowych typu μ</t></is></c><c r="H446" s="2" t="inlineStr" /><c r="I446" s="2" t="inlineStr" /><c r="J446" s="2" t="inlineStr" /><c r="K446" s="2" t="inlineStr"><is><t>Inhibitorem wychwytu zwrotnego dopaminy</t></is></c><c r="L446" s="2" t="inlineStr"><is><t>Agonistą receptorów NMDA</t></is></c><c r="M446" s="2" t="inlineStr" /><c r="N446" s="2" t="inlineStr" /><c r="O446" s="2" t="inlineStr" /><c r="P446" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q446" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="447"><c r="A447" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B447" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C447" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D447" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E447" s="2" t="inlineStr"><is><t>Hamowanie enzymu stanowi zasadniczy mechanizm działania:</t></is></c><c r="F447" s="2" t="inlineStr"><is><t>cyklosporyny</t></is></c><c r="G447" s="2" t="inlineStr" /><c r="H447" s="2" t="inlineStr" /><c r="I447" s="2" t="inlineStr" /><c r="J447" s="2" t="inlineStr" /><c r="K447" s="2" t="inlineStr"><is><t>Liraglutydu</t></is></c><c r="L447" s="2" t="inlineStr"><is><t>Lorazepamu</t></is></c><c r="M447" s="2" t="inlineStr"><is><t>Buprenorfiny</t></is></c><c r="N447" s="2" t="inlineStr" /><c r="O447" s="2" t="inlineStr" /><c r="P447" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q447" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="448"><c r="A448" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B448" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C448" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D448" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E448" s="2" t="inlineStr"><is><t>Ryzyko wzrostu masy ciała jest związane z terapią:</t></is></c><c r="F448" s="2" t="inlineStr"><is><t>Olanzapiną</t></is></c><c r="G448" s="2" t="inlineStr"><is><t>Insuliną</t></is></c><c r="H448" s="2" t="inlineStr"><is><t>prednizonem</t></is></c><c r="I448" s="2" t="inlineStr" /><c r="J448" s="2" t="inlineStr" /><c r="K448" s="2" t="inlineStr"><is><t>Liraglutydem</t></is></c><c r="L448" s="2" t="inlineStr" /><c r="M448" s="2" t="inlineStr" /><c r="N448" s="2" t="inlineStr" /><c r="O448" s="2" t="inlineStr" /><c r="P448" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q448" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="449"><c r="A449" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B449" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C449" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D449" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E449" s="2" t="inlineStr"><is><t>Lek A jest stosowany doustnie. Ma właściwości przeciwbólowe, ale nie ma właściwości przeciwzapalnych. Nie powoduje istotnego wzrostu ryzyka powikłań sercowo – naczyniowych. Lekiem A może być:</t></is></c><c r="F449" s="2" t="inlineStr"><is><t>Tramadol</t></is></c><c r="G449" s="2" t="inlineStr"><is><t>Paracetamol</t></is></c><c r="H449" s="2" t="inlineStr" /><c r="I449" s="2" t="inlineStr" /><c r="J449" s="2" t="inlineStr" /><c r="K449" s="2" t="inlineStr"><is><t>Naproksen</t></is></c><c r="L449" s="2" t="inlineStr"><is><t>Celekoksyb</t></is></c><c r="M449" s="2" t="inlineStr" /><c r="N449" s="2" t="inlineStr" /><c r="O449" s="2" t="inlineStr" /><c r="P449" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q449" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="450"><c r="A450" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B450" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C450" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D450" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E450" s="2" t="inlineStr"><is><t>Bisfosfoniany są stosowane:</t></is></c><c r="F450" s="2" t="inlineStr"><is><t>w leczeniu osteoporozy posteroidowej</t></is></c><c r="G450" s="2" t="inlineStr"><is><t>w leczeniu ciężkiej hiperkalcemii</t></is></c><c r="H450" s="2" t="inlineStr" /><c r="I450" s="2" t="inlineStr" /><c r="J450" s="2" t="inlineStr" /><c r="K450" s="2" t="inlineStr"><is><t>w celu przyspieszania zrostu kości po złamaniach</t></is></c><c r="L450" s="2" t="inlineStr"><is><t>przeciwbólowo w chorobie zwyrodnieniowej stawów</t></is></c><c r="M450" s="2" t="inlineStr" /><c r="N450" s="2" t="inlineStr" /><c r="O450" s="2" t="inlineStr" /><c r="P450" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q450" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="451"><c r="A451" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B451" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C451" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D451" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E451" s="2" t="inlineStr"><is><t>20% roztwór albumin to:</t></is></c><c r="F451" s="2" t="inlineStr"><is><t>lek krwiopochodny</t></is></c><c r="G451" s="2" t="inlineStr"><is><t>koloid zatrzymujący płyny w przestrzeni wewnątrznaczyniowej</t></is></c><c r="H451" s="2" t="inlineStr" /><c r="I451" s="2" t="inlineStr" /><c r="J451" s="2" t="inlineStr" /><c r="K451" s="2" t="inlineStr"><is><t>substancja do żywienia pozajelitowego</t></is></c><c r="L451" s="2" t="inlineStr"><is><t>łatwo dostępny i tani płyn do nawadniania</t></is></c><c r="M451" s="2" t="inlineStr" /><c r="N451" s="2" t="inlineStr" /><c r="O451" s="2" t="inlineStr" /><c r="P451" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q451" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="452"><c r="A452" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B452" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C452" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D452" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E452" s="2" t="inlineStr"><is><t>W leczeniu wymiotów indukowanych chemioterapią znajduje zastosowanie:</t></is></c><c r="F452" s="2" t="inlineStr"><is><t>Deksametazon</t></is></c><c r="G452" s="2" t="inlineStr"><is><t>Palonosetron</t></is></c><c r="H452" s="2" t="inlineStr"><is><t>metoklopramid</t></is></c><c r="I452" s="2" t="inlineStr" /><c r="J452" s="2" t="inlineStr" /><c r="K452" s="2" t="inlineStr"><is><t>Dimenhydrynat</t></is></c><c r="L452" s="2" t="inlineStr" /><c r="M452" s="2" t="inlineStr" /><c r="N452" s="2" t="inlineStr" /><c r="O452" s="2" t="inlineStr" /><c r="P452" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q452" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="453"><c r="A453" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B453" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C453" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D453" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E453" s="2" t="inlineStr"><is><t>Klozapina może być przyczyną:</t></is></c><c r="F453" s="2" t="inlineStr"><is><t>obniżenia progu drgawkowego</t></is></c><c r="G453" s="2" t="inlineStr"><is><t>przyrostu masy ciała</t></is></c><c r="H453" s="2" t="inlineStr"><is><t>agranulocytozy</t></is></c><c r="I453" s="2" t="inlineStr" /><c r="J453" s="2" t="inlineStr" /><c r="K453" s="2" t="inlineStr"><is><t>Hiperprolaktynemii</t></is></c><c r="L453" s="2" t="inlineStr" /><c r="M453" s="2" t="inlineStr" /><c r="N453" s="2" t="inlineStr" /><c r="O453" s="2" t="inlineStr" /><c r="P453" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q453" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="454"><c r="A454" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B454" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C454" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D454" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E454" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – mechanizm działania:</t></is></c><c r="F454" s="2" t="inlineStr"><is><t>buspiron – agonista rec. 5HT1A</t></is></c><c r="G454" s="2" t="inlineStr"><is><t>diazepam – agonista rec. GABA-A</t></is></c><c r="H454" s="2" t="inlineStr" /><c r="I454" s="2" t="inlineStr" /><c r="J454" s="2" t="inlineStr" /><c r="K454" s="2" t="inlineStr"><is><t>zolpidem – agonista rec. H2</t></is></c><c r="L454" s="2" t="inlineStr"><is><t>mirtazapina – agonista rec. alfa2</t></is></c><c r="M454" s="2" t="inlineStr" /><c r="N454" s="2" t="inlineStr" /><c r="O454" s="2" t="inlineStr" /><c r="P454" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q454" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="455"><c r="A455" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B455" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C455" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D455" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E455" s="2" t="inlineStr"><is><t>Benzodiazepiny są stosowane w:</t></is></c><c r="F455" s="2" t="inlineStr"><is><t>premedykacji</t></is></c><c r="G455" s="2" t="inlineStr"><is><t>terapii padaczki</t></is></c><c r="H455" s="2" t="inlineStr" /><c r="I455" s="2" t="inlineStr" /><c r="J455" s="2" t="inlineStr" /><c r="K455" s="2" t="inlineStr"><is><t>długotrwałej terapii bezsenności</t></is></c><c r="L455" s="2" t="inlineStr"><is><t>zespole abstynencyjnym u chorych uzależnionych od morfiny</t></is></c><c r="M455" s="2" t="inlineStr" /><c r="N455" s="2" t="inlineStr" /><c r="O455" s="2" t="inlineStr" /><c r="P455" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q455" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="456"><c r="A456" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B456" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C456" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D456" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E456" s="2" t="inlineStr"><is><t>Zespół serotoninowy może być wynikiem interakcji cytalopramu z:</t></is></c><c r="F456" s="2" t="inlineStr"><is><t>Tramadolem</t></is></c><c r="G456" s="2" t="inlineStr"><is><t>klomipraminą</t></is></c><c r="H456" s="2" t="inlineStr" /><c r="I456" s="2" t="inlineStr" /><c r="J456" s="2" t="inlineStr" /><c r="K456" s="2" t="inlineStr"><is><t>Oksazepamem</t></is></c><c r="L456" s="2" t="inlineStr"><is><t>Buprenorfiną</t></is></c><c r="M456" s="2" t="inlineStr" /><c r="N456" s="2" t="inlineStr" /><c r="O456" s="2" t="inlineStr" /><c r="P456" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q456" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="457"><c r="A457" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B457" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C457" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D457" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E457" s="2" t="inlineStr"><is><t>Charakterystyka Produktu Leczniczego zawiera informacje o:</t></is></c><c r="F457" s="2" t="inlineStr"><is><t>mechanizmie działania</t></is></c><c r="G457" s="2" t="inlineStr"><is><t>interakcjach</t></is></c><c r="H457" s="2" t="inlineStr"><is><t>substancjach pomocniczych</t></is></c><c r="I457" s="2" t="inlineStr"><is><t>działaniach niepożądanych</t></is></c><c r="J457" s="2" t="inlineStr" /><c r="K457" s="2" t="inlineStr" /><c r="L457" s="2" t="inlineStr" /><c r="M457" s="2" t="inlineStr" /><c r="N457" s="2" t="inlineStr" /><c r="O457" s="2" t="inlineStr" /><c r="P457" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q457" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="458"><c r="A458" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B458" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C458" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D458" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E458" s="2" t="inlineStr"><is><t>Przyczyną nieliniowego przebiegu procesów farmakokinetycznych może być:</t></is></c><c r="F458" s="2" t="inlineStr"><is><t>autoindukcja metabolizmu</t></is></c><c r="G458" s="2" t="inlineStr"><is><t>niedobór kosubstratów w procesie sprzęgania</t></is></c><c r="H458" s="2" t="inlineStr"><is><t>wysycenie transporterów</t></is></c><c r="I458" s="2" t="inlineStr" /><c r="J458" s="2" t="inlineStr" /><c r="K458" s="2" t="inlineStr"><is><t>wąski wskaźnik terapeutyczny leku</t></is></c><c r="L458" s="2" t="inlineStr" /><c r="M458" s="2" t="inlineStr" /><c r="N458" s="2" t="inlineStr" /><c r="O458" s="2" t="inlineStr" /><c r="P458" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q458" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="459"><c r="A459" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B459" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C459" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D459" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E459" s="2" t="inlineStr"><is><t>Insulina aspart:</t></is></c><c r="F459" s="2" t="inlineStr"><is><t>działa za pośrednictwem receptora błonowego</t></is></c><c r="G459" s="2" t="inlineStr"><is><t>może być podawana we wstrzyknięciu podskórnym</t></is></c><c r="H459" s="2" t="inlineStr" /><c r="I459" s="2" t="inlineStr" /><c r="J459" s="2" t="inlineStr" /><c r="K459" s="2" t="inlineStr"><is><t>jest stosowana wyłącznie w cukrzycy typu 1</t></is></c><c r="L459" s="2" t="inlineStr"><is><t>jest analogiem długodziałającym</t></is></c><c r="M459" s="2" t="inlineStr" /><c r="N459" s="2" t="inlineStr" /><c r="O459" s="2" t="inlineStr" /><c r="P459" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q459" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="460"><c r="A460" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B460" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C460" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D460" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E460" s="2" t="inlineStr"><is><t>Na proces dystrybucji leku może mieć wpływ:</t></is></c><c r="F460" s="2" t="inlineStr"><is><t>niewydolność krążenia</t></is></c><c r="G460" s="2" t="inlineStr"><is><t>Hipoalbuminemia</t></is></c><c r="H460" s="2" t="inlineStr" /><c r="I460" s="2" t="inlineStr" /><c r="J460" s="2" t="inlineStr" /><c r="K460" s="2" t="inlineStr"><is><t>obecność pokarmu w przypadku podania doustnego</t></is></c><c r="L460" s="2" t="inlineStr"><is><t>możliwość sprzęgania z kwasem glukuronowym</t></is></c><c r="M460" s="2" t="inlineStr" /><c r="N460" s="2" t="inlineStr" /><c r="O460" s="2" t="inlineStr" /><c r="P460" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q460" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="461"><c r="A461" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B461" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C461" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D461" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E461" s="2" t="inlineStr"><is><t>Agonistą receptorów jest:</t></is></c><c r="F461" s="2" t="inlineStr"><is><t>tapentadol</t></is></c><c r="G461" s="2" t="inlineStr" /><c r="H461" s="2" t="inlineStr" /><c r="I461" s="2" t="inlineStr" /><c r="J461" s="2" t="inlineStr" /><c r="K461" s="2" t="inlineStr"><is><t>Sertralina</t></is></c><c r="L461" s="2" t="inlineStr"><is><t>Eplerenon</t></is></c><c r="M461" s="2" t="inlineStr"><is><t>Fenytoina</t></is></c><c r="N461" s="2" t="inlineStr" /><c r="O461" s="2" t="inlineStr" /><c r="P461" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q461" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="462"><c r="A462" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B462" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C462" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D462" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E462" s="2" t="inlineStr"><is><t>W trakcie długotrwałej terapii glikokortykosteroidami, wskazane jest monitorowanie:</t></is></c><c r="F462" s="2" t="inlineStr"><is><t>stężenia potasu we krwi</t></is></c><c r="G462" s="2" t="inlineStr"><is><t>ciśnienia tętniczego krwi</t></is></c><c r="H462" s="2" t="inlineStr"><is><t>ciśnienia wewnątrzgałkowego</t></is></c><c r="I462" s="2" t="inlineStr"><is><t>glikemii</t></is></c><c r="J462" s="2" t="inlineStr" /><c r="K462" s="2" t="inlineStr" /><c r="L462" s="2" t="inlineStr" /><c r="M462" s="2" t="inlineStr" /><c r="N462" s="2" t="inlineStr" /><c r="O462" s="2" t="inlineStr" /><c r="P462" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q462" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="463"><c r="A463" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B463" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C463" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D463" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E463" s="2" t="inlineStr"><is><t>Inhibitory kotransportera sodowo-glukozowego 2 (SGLT-2, flozyny):</t></is></c><c r="F463" s="2" t="inlineStr"><is><t>Mogą być stosowane łącznie z metforminą</t></is></c><c r="G463" s="2" t="inlineStr"><is><t>Mogą zwiększać diurezę</t></is></c><c r="H463" s="2" t="inlineStr"><is><t>Mają udowodnione korzystne działanie w zakresie ryzyka sercowo-naczyniowego</t></is></c><c r="I463" s="2" t="inlineStr" /><c r="J463" s="2" t="inlineStr" /><c r="K463" s="2" t="inlineStr"><is><t>Charakteryzują się wysokim ryzykiem wystąpienia hipoglikemii</t></is></c><c r="L463" s="2" t="inlineStr" /><c r="M463" s="2" t="inlineStr" /><c r="N463" s="2" t="inlineStr" /><c r="O463" s="2" t="inlineStr" /><c r="P463" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q463" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="464"><c r="A464" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B464" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C464" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D464" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E464" s="2" t="inlineStr"><is><t>Przeciwciała monoklonalne znajdują zastosowanie w terapii:</t></is></c><c r="F464" s="2" t="inlineStr"><is><t>choroby Leśniowskiego i Crohna</t></is></c><c r="G464" s="2" t="inlineStr"><is><t>stwardnienia rozsianego</t></is></c><c r="H464" s="2" t="inlineStr"><is><t>reumatoidalnego zapalenia stawów</t></is></c><c r="I464" s="2" t="inlineStr" /><c r="J464" s="2" t="inlineStr" /><c r="K464" s="2" t="inlineStr"><is><t>mononukleozy</t></is></c><c r="L464" s="2" t="inlineStr" /><c r="M464" s="2" t="inlineStr" /><c r="N464" s="2" t="inlineStr" /><c r="O464" s="2" t="inlineStr" /><c r="P464" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q464" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="465"><c r="A465" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B465" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C465" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D465" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E465" s="2" t="inlineStr"><is><t>Zaburzenia rytmu serca mogą wystąpić w trakcie podawania:</t></is></c><c r="F465" s="2" t="inlineStr"><is><t>Amisulpirydu</t></is></c><c r="G465" s="2" t="inlineStr"><is><t>Ondansetronu</t></is></c><c r="H465" s="2" t="inlineStr"><is><t>Chlorpromazyny</t></is></c><c r="I465" s="2" t="inlineStr"><is><t>metadonu</t></is></c><c r="J465" s="2" t="inlineStr" /><c r="K465" s="2" t="inlineStr" /><c r="L465" s="2" t="inlineStr" /><c r="M465" s="2" t="inlineStr" /><c r="N465" s="2" t="inlineStr" /><c r="O465" s="2" t="inlineStr" /><c r="P465" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q465" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="466"><c r="A466" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B466" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C466" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D466" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E466" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące terapii niedokrwistości z niedoboru żelaza:</t></is></c><c r="F466" s="2" t="inlineStr"><is><t>preferowana jest doustna suplementacja żelaza</t></is></c><c r="G466" s="2" t="inlineStr" /><c r="H466" s="2" t="inlineStr" /><c r="I466" s="2" t="inlineStr" /><c r="J466" s="2" t="inlineStr" /><c r="K466" s="2" t="inlineStr"><is><t>terapia trwa 2 tygodnie</t></is></c><c r="L466" s="2" t="inlineStr"><is><t>preparaty dożylne żelaza są przeciwwskazane u chorych z przewlekłą niewydolnością nerek</t></is></c><c r="M466" s="2" t="inlineStr"><is><t>tabletki z żelazem należy popijać herbatą</t></is></c><c r="N466" s="2" t="inlineStr" /><c r="O466" s="2" t="inlineStr" /><c r="P466" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q466" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="467"><c r="A467" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B467" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C467" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D467" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E467" s="2" t="inlineStr"><is><t>Działanie normotymizujące wykazują:</t></is></c><c r="F467" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="G467" s="2" t="inlineStr"><is><t>Lamotrygina</t></is></c><c r="H467" s="2" t="inlineStr"><is><t>Olanzapina</t></is></c><c r="I467" s="2" t="inlineStr"><is><t>sole litu</t></is></c><c r="J467" s="2" t="inlineStr" /><c r="K467" s="2" t="inlineStr" /><c r="L467" s="2" t="inlineStr" /><c r="M467" s="2" t="inlineStr" /><c r="N467" s="2" t="inlineStr" /><c r="O467" s="2" t="inlineStr" /><c r="P467" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q467" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="468"><c r="A468" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B468" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C468" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D468" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E468" s="2" t="inlineStr"><is><t>Udowodnione działanie immunostymulujące wykazuje:</t></is></c><c r="F468" s="2" t="inlineStr"><is><t>filgrastym</t></is></c><c r="G468" s="2" t="inlineStr" /><c r="H468" s="2" t="inlineStr" /><c r="I468" s="2" t="inlineStr" /><c r="J468" s="2" t="inlineStr" /><c r="K468" s="2" t="inlineStr"><is><t>wyciąg z korzenia jeżówki purpurowej</t></is></c><c r="L468" s="2" t="inlineStr"><is><t>pranobeks inozyny</t></is></c><c r="M468" s="2" t="inlineStr"><is><t>alkoholowy wyciąg z dziurawca</t></is></c><c r="N468" s="2" t="inlineStr" /><c r="O468" s="2" t="inlineStr" /><c r="P468" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q468" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="469"><c r="A469" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B469" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C469" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D469" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E469" s="2" t="inlineStr"><is><t>Ryzyka rozwoju zależności można się spodziewać przy stosowaniu:</t></is></c><c r="F469" s="2" t="inlineStr"><is><t>Dihydrokodeiny</t></is></c><c r="G469" s="2" t="inlineStr"><is><t>Diazepamu</t></is></c><c r="H469" s="2" t="inlineStr" /><c r="I469" s="2" t="inlineStr" /><c r="J469" s="2" t="inlineStr" /><c r="K469" s="2" t="inlineStr"><is><t>Diklofenaku</t></is></c><c r="L469" s="2" t="inlineStr"><is><t>duloksetyny</t></is></c><c r="M469" s="2" t="inlineStr" /><c r="N469" s="2" t="inlineStr" /><c r="O469" s="2" t="inlineStr" /><c r="P469" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q469" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="470"><c r="A470" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B470" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C470" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D470" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E470" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek przeciwdepresyjny – mechanizm działania:</t></is></c><c r="F470" s="2" t="inlineStr"><is><t>reboksetyna – selektywny inhibitor wychwytu zwrotnego noradrenaliny</t></is></c><c r="G470" s="2" t="inlineStr"><is><t>bupropion – inhibitor wychwytu zwrotnego noradrenaliny i dopaminy</t></is></c><c r="H470" s="2" t="inlineStr"><is><t>fluoksetyna – selektywny inhibitor wychwytu zwrotnego serotoniny</t></is></c><c r="I470" s="2" t="inlineStr"><is><t>wenlafaksyna – inhibitor wychwytu zwrotnego serotoniny i noradrenaliny</t></is></c><c r="J470" s="2" t="inlineStr" /><c r="K470" s="2" t="inlineStr" /><c r="L470" s="2" t="inlineStr" /><c r="M470" s="2" t="inlineStr" /><c r="N470" s="2" t="inlineStr" /><c r="O470" s="2" t="inlineStr" /><c r="P470" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q470" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="471"><c r="A471" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B471" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C471" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D471" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E471" s="2" t="inlineStr"><is><t>Ryzyko gastrotoksycznego działania ketoprofenu może istotnie wzrosnąć przy jednoczesnym podawaniu:</t></is></c><c r="F471" s="2" t="inlineStr"><is><t>Spironolaktonu</t></is></c><c r="G471" s="2" t="inlineStr"><is><t>prednizonu</t></is></c><c r="H471" s="2" t="inlineStr" /><c r="I471" s="2" t="inlineStr" /><c r="J471" s="2" t="inlineStr" /><c r="K471" s="2" t="inlineStr"><is><t>Mizoprostolu</t></is></c><c r="L471" s="2" t="inlineStr"><is><t>Omeprazolu</t></is></c><c r="M471" s="2" t="inlineStr" /><c r="N471" s="2" t="inlineStr" /><c r="O471" s="2" t="inlineStr" /><c r="P471" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q471" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="472"><c r="A472" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B472" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C472" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D472" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E472" s="2" t="inlineStr"><is><t>Morfina może być przyczyną:</t></is></c><c r="F472" s="2" t="inlineStr"><is><t>obniżenia progu drgawkowego</t></is></c><c r="G472" s="2" t="inlineStr"><is><t>skurczu oskrzeli</t></is></c><c r="H472" s="2" t="inlineStr" /><c r="I472" s="2" t="inlineStr" /><c r="J472" s="2" t="inlineStr" /><c r="K472" s="2" t="inlineStr"><is><t>rozszerzenia źrenic</t></is></c><c r="L472" s="2" t="inlineStr"><is><t>działania moczopędnego</t></is></c><c r="M472" s="2" t="inlineStr" /><c r="N472" s="2" t="inlineStr" /><c r="O472" s="2" t="inlineStr" /><c r="P472" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q472" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="473"><c r="A473" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B473" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C473" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D473" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E473" s="2" t="inlineStr"><is><t>Wskaż fałszywe stwierdzenie:</t></is></c><c r="F473" s="2" t="inlineStr"><is><t>suplement diety to lek stosowany wspomagająco</t></is></c><c r="G473" s="2" t="inlineStr" /><c r="H473" s="2" t="inlineStr" /><c r="I473" s="2" t="inlineStr" /><c r="J473" s="2" t="inlineStr" /><c r="K473" s="2" t="inlineStr"><is><t>produkt leczniczy to substancja, której przypisuje się, między innymi, właściwości zapobiegania chorobom występującym u ludzi</t></is></c><c r="L473" s="2" t="inlineStr"><is><t>wyrób medyczny to przyrząd lub inny artykuł stosowany w celu diagnozowania, zapobiegania, monitorowania, leczenia lub łagodzenia przebiegu chorób</t></is></c><c r="M473" s="2" t="inlineStr"><is><t>roztwór albumin należy do kategorii produktów krwiopochodnych</t></is></c><c r="N473" s="2" t="inlineStr" /><c r="O473" s="2" t="inlineStr" /><c r="P473" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q473" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="474"><c r="A474" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B474" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C474" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D474" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E474" s="2" t="inlineStr"><is><t>Nalokson:</t></is></c><c r="F474" s="2" t="inlineStr"><is><t>słabo wchłania się z przewodu pokarmowego</t></is></c><c r="G474" s="2" t="inlineStr"><is><t>nie wywołuje uzależnienia</t></is></c><c r="H474" s="2" t="inlineStr" /><c r="I474" s="2" t="inlineStr" /><c r="J474" s="2" t="inlineStr" /><c r="K474" s="2" t="inlineStr"><is><t>jest agonistą receptorów opioidowych</t></is></c><c r="L474" s="2" t="inlineStr"><is><t>powoduje depresję ośrodka oddechowego</t></is></c><c r="M474" s="2" t="inlineStr" /><c r="N474" s="2" t="inlineStr" /><c r="O474" s="2" t="inlineStr" /><c r="P474" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q474" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="475"><c r="A475" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B475" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C475" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D475" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E475" s="2" t="inlineStr"><is><t>Antagonizm wobec receptora stanowi zasadniczy mechanizm działania:</t></is></c><c r="F475" s="2" t="inlineStr"><is><t>flumazenilu</t></is></c><c r="G475" s="2" t="inlineStr" /><c r="H475" s="2" t="inlineStr" /><c r="I475" s="2" t="inlineStr" /><c r="J475" s="2" t="inlineStr" /><c r="K475" s="2" t="inlineStr"><is><t>Cyklosporyny</t></is></c><c r="L475" s="2" t="inlineStr"><is><t>Lorazepamu</t></is></c><c r="M475" s="2" t="inlineStr"><is><t>Tapentadolu</t></is></c><c r="N475" s="2" t="inlineStr" /><c r="O475" s="2" t="inlineStr" /><c r="P475" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q475" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="476"><c r="A476" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B476" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C476" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D476" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E476" s="2" t="inlineStr"><is><t>Zmniejszenie masy ciała może wiązać się z terapią:</t></is></c><c r="F476" s="2" t="inlineStr"><is><t>Lewotyroksyną</t></is></c><c r="G476" s="2" t="inlineStr"><is><t>metforminą</t></is></c><c r="H476" s="2" t="inlineStr" /><c r="I476" s="2" t="inlineStr" /><c r="J476" s="2" t="inlineStr" /><c r="K476" s="2" t="inlineStr"><is><t>Olanzapiną</t></is></c><c r="L476" s="2" t="inlineStr"><is><t>Prednizonem</t></is></c><c r="M476" s="2" t="inlineStr" /><c r="N476" s="2" t="inlineStr" /><c r="O476" s="2" t="inlineStr" /><c r="P476" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q476" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="477"><c r="A477" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B477" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C477" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D477" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E477" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – działanie niepożądane:</t></is></c><c r="F477" s="2" t="inlineStr"><is><t>tietylperazyna - akatyzja</t></is></c><c r="G477" s="2" t="inlineStr"><is><t>metoklopramid – późne dyskinezy</t></is></c><c r="H477" s="2" t="inlineStr"><is><t>ondansetron – wydłużenie odstępu QT</t></is></c><c r="I477" s="2" t="inlineStr" /><c r="J477" s="2" t="inlineStr" /><c r="K477" s="2" t="inlineStr"><is><t>dimenhydrynat - wymioty</t></is></c><c r="L477" s="2" t="inlineStr" /><c r="M477" s="2" t="inlineStr" /><c r="N477" s="2" t="inlineStr" /><c r="O477" s="2" t="inlineStr" /><c r="P477" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q477" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="478"><c r="A478" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B478" s="2" t="inlineStr"><is><t>Struktura chemiczna</t></is></c><c r="C478" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D478" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E478" s="2" t="inlineStr"><is><t>Trójpierścieniowe leki przeciwdepresyjne:</t></is></c><c r="F478" s="2" t="inlineStr"><is><t>blokują receptory histaminowe</t></is></c><c r="G478" s="2" t="inlineStr"><is><t>hamują wychwyt zwrotny dopaminy</t></is></c><c r="H478" s="2" t="inlineStr" /><c r="I478" s="2" t="inlineStr" /><c r="J478" s="2" t="inlineStr" /><c r="K478" s="2" t="inlineStr"><is><t>pobudzają receptory muskarynowe</t></is></c><c r="L478" s="2" t="inlineStr"><is><t>nie wpływają na przekaźnictwo serotoninergiczne</t></is></c><c r="M478" s="2" t="inlineStr" /><c r="N478" s="2" t="inlineStr" /><c r="O478" s="2" t="inlineStr" /><c r="P478" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q478" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="479"><c r="A479" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B479" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C479" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D479" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E479" s="2" t="inlineStr"><is><t>Na dostępność biologiczną leku może mieć wpływ:</t></is></c><c r="F479" s="2" t="inlineStr"><is><t>stopień uwalniania substancji czynnej</t></is></c><c r="G479" s="2" t="inlineStr"><is><t>efekt I przejścia</t></is></c><c r="H479" s="2" t="inlineStr"><is><t>szybkość transportu substancji czynnej przez błony biologiczne</t></is></c><c r="I479" s="2" t="inlineStr" /><c r="J479" s="2" t="inlineStr" /><c r="K479" s="2" t="inlineStr"><is><t>stopień wiązania z białkami krwi</t></is></c><c r="L479" s="2" t="inlineStr" /><c r="M479" s="2" t="inlineStr" /><c r="N479" s="2" t="inlineStr" /><c r="O479" s="2" t="inlineStr" /><c r="P479" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q479" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="480"><c r="A480" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B480" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C480" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D480" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E480" s="2" t="inlineStr"><is><t>Stan stacjonarny leku ustala się:</t></is></c><c r="F480" s="2" t="inlineStr"><is><t>po okresie równym około 4–5 T1/2</t></is></c><c r="G480" s="2" t="inlineStr" /><c r="H480" s="2" t="inlineStr" /><c r="I480" s="2" t="inlineStr" /><c r="J480" s="2" t="inlineStr" /><c r="K480" s="2" t="inlineStr"><is><t>w momencie, który zależy od dawki leku</t></is></c><c r="L480" s="2" t="inlineStr"><is><t>jedynie w wyniku wielokrotnego podania doustnego</t></is></c><c r="M480" s="2" t="inlineStr"><is><t>w czasie wprost proporcjonalnym do klirensu leku</t></is></c><c r="N480" s="2" t="inlineStr" /><c r="O480" s="2" t="inlineStr" /><c r="P480" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q480" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="481"><c r="A481" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B481" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C481" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D481" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E481" s="2" t="inlineStr"><is><t>Biologiczny okres półtrwania (T1/2):</t></is></c><c r="F481" s="2" t="inlineStr"><is><t>zależy od objętości dystrybucji</t></is></c><c r="G481" s="2" t="inlineStr"><is><t>jest odwrotnie proporcjonalny do klirensu całkowitego</t></is></c><c r="H481" s="2" t="inlineStr"><is><t>ma wpływ na moment osiągnięcia stanu stacjonarnego</t></is></c><c r="I481" s="2" t="inlineStr" /><c r="J481" s="2" t="inlineStr" /><c r="K481" s="2" t="inlineStr"><is><t>zależy od szybkości wchłaniania</t></is></c><c r="L481" s="2" t="inlineStr" /><c r="M481" s="2" t="inlineStr" /><c r="N481" s="2" t="inlineStr" /><c r="O481" s="2" t="inlineStr" /><c r="P481" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q481" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="482"><c r="A482" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B482" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C482" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D482" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E482" s="2" t="inlineStr"><is><t>Do typowych objawów zatrucia opioidami należą:</t></is></c><c r="F482" s="2" t="inlineStr"><is><t>Śpiączka</t></is></c><c r="G482" s="2" t="inlineStr"><is><t>Depresja oddechowa</t></is></c><c r="H482" s="2" t="inlineStr" /><c r="I482" s="2" t="inlineStr" /><c r="J482" s="2" t="inlineStr" /><c r="K482" s="2" t="inlineStr"><is><t>Wzrost ciśnienia tętniczego</t></is></c><c r="L482" s="2" t="inlineStr"><is><t>wzrost temperatury ciała</t></is></c><c r="M482" s="2" t="inlineStr" /><c r="N482" s="2" t="inlineStr" /><c r="O482" s="2" t="inlineStr" /><c r="P482" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q482" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="483"><c r="A483" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B483" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C483" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D483" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E483" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące glikokortykosteroidów:</t></is></c><c r="F483" s="2" t="inlineStr"><is><t>Działają za pośrednictwem receptorów wewnątrzkomórkowych</t></is></c><c r="G483" s="2" t="inlineStr"><is><t>mechanizm niegenomowy odpowiedzialny jest za ich działanie rozkurczające mięśniówkę dróg oddechowych</t></is></c><c r="H483" s="2" t="inlineStr"><is><t>Nagłe ich odstawienie po co najmniej tygodniowym zastosowaniu dawek farmakologicznych może być przyczyną ostrej niewydolności kory nadnerczy</t></is></c><c r="I483" s="2" t="inlineStr" /><c r="J483" s="2" t="inlineStr" /><c r="K483" s="2" t="inlineStr"><is><t>Powodują zmniejszenie zapotrzebowania na insulinę u chorych na cukrzycę</t></is></c><c r="L483" s="2" t="inlineStr" /><c r="M483" s="2" t="inlineStr" /><c r="N483" s="2" t="inlineStr" /><c r="O483" s="2" t="inlineStr" /><c r="P483" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q483" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="484"><c r="A484" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B484" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C484" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D484" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E484" s="2" t="inlineStr"><is><t>Insulina ludzka neutralna:</t></is></c><c r="F484" s="2" t="inlineStr"><is><t>działa za pośrednictwem receptora błonowego</t></is></c><c r="G484" s="2" t="inlineStr"><is><t>jest otrzymywana metodą rekombinacji DNA</t></is></c><c r="H484" s="2" t="inlineStr" /><c r="I484" s="2" t="inlineStr" /><c r="J484" s="2" t="inlineStr" /><c r="K484" s="2" t="inlineStr"><is><t>może być podawana doustnie</t></is></c><c r="L484" s="2" t="inlineStr"><is><t>jest analogiem długodziałającym</t></is></c><c r="M484" s="2" t="inlineStr" /><c r="N484" s="2" t="inlineStr" /><c r="O484" s="2" t="inlineStr" /><c r="P484" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q484" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="485"><c r="A485" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B485" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C485" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D485" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E485" s="2" t="inlineStr"><is><t>Stosowanie estrogenów może być przyczyną:</t></is></c><c r="F485" s="2" t="inlineStr"><is><t>wzrostu ciśnienia tętniczego krwi</t></is></c><c r="G485" s="2" t="inlineStr"><is><t>kamicy żółciowej</t></is></c><c r="H485" s="2" t="inlineStr"><is><t>wzrostu ryzyka wystąpienia raka piersi</t></is></c><c r="I485" s="2" t="inlineStr"><is><t>zatorowości płucnej</t></is></c><c r="J485" s="2" t="inlineStr" /><c r="K485" s="2" t="inlineStr" /><c r="L485" s="2" t="inlineStr" /><c r="M485" s="2" t="inlineStr" /><c r="N485" s="2" t="inlineStr" /><c r="O485" s="2" t="inlineStr" /><c r="P485" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q485" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="486"><c r="A486" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B486" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C486" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D486" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E486" s="2" t="inlineStr"><is><t>Metamizol:</t></is></c><c r="F486" s="2" t="inlineStr"><is><t>działa przeciwbólowo i przeciwgorączkowo</t></is></c><c r="G486" s="2" t="inlineStr"><is><t>działa spazmolitycznie</t></is></c><c r="H486" s="2" t="inlineStr"><is><t>może być przyczyną agranulocytozy</t></is></c><c r="I486" s="2" t="inlineStr" /><c r="J486" s="2" t="inlineStr" /><c r="K486" s="2" t="inlineStr"><is><t>może być bezpiecznie stosowany w ciąży</t></is></c><c r="L486" s="2" t="inlineStr" /><c r="M486" s="2" t="inlineStr" /><c r="N486" s="2" t="inlineStr" /><c r="O486" s="2" t="inlineStr" /><c r="P486" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q486" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="487"><c r="A487" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B487" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C487" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D487" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E487" s="2" t="inlineStr"><is><t>Do leków biotechnologicznych należą:</t></is></c><c r="F487" s="2" t="inlineStr"><is><t>szczepionki</t></is></c><c r="G487" s="2" t="inlineStr"><is><t>przeciwciała monoklonalne</t></is></c><c r="H487" s="2" t="inlineStr"><is><t>Hormony</t></is></c><c r="I487" s="2" t="inlineStr"><is><t>czynniki krzepnięcia</t></is></c><c r="J487" s="2" t="inlineStr" /><c r="K487" s="2" t="inlineStr" /><c r="L487" s="2" t="inlineStr" /><c r="M487" s="2" t="inlineStr" /><c r="N487" s="2" t="inlineStr" /><c r="O487" s="2" t="inlineStr" /><c r="P487" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q487" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="488"><c r="A488" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B488" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C488" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D488" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E488" s="2" t="inlineStr"><is><t>Doustne preparaty żelaza:</t></is></c><c r="F488" s="2" t="inlineStr"><is><t>najlepiej przyswajalne zawierają żelazo dwuwartościowe</t></is></c><c r="G488" s="2" t="inlineStr"><is><t>należy przyjmować przez okres 3 miesięcy po uzyskaniu normalizacji morfologii</t></is></c><c r="H488" s="2" t="inlineStr" /><c r="I488" s="2" t="inlineStr" /><c r="J488" s="2" t="inlineStr" /><c r="K488" s="2" t="inlineStr"><is><t>należy przyjmować z posiłkiem wysokotłuszczowym</t></is></c><c r="L488" s="2" t="inlineStr"><is><t>mogą być przyczyną jasno-żółtego zabarwienia stolca</t></is></c><c r="M488" s="2" t="inlineStr" /><c r="N488" s="2" t="inlineStr" /><c r="O488" s="2" t="inlineStr" /><c r="P488" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q488" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="489"><c r="A489" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B489" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C489" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D489" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E489" s="2" t="inlineStr"><is><t>Diazepam:</t></is></c><c r="F489" s="2" t="inlineStr"><is><t>działa sedatywnie</t></is></c><c r="G489" s="2" t="inlineStr"><is><t>działa powyżej 24 godzin</t></is></c><c r="H489" s="2" t="inlineStr" /><c r="I489" s="2" t="inlineStr" /><c r="J489" s="2" t="inlineStr" /><c r="K489" s="2" t="inlineStr"><is><t>obniża próg drgawkowy</t></is></c><c r="L489" s="2" t="inlineStr"><is><t>nie podlega metabolizmowi</t></is></c><c r="M489" s="2" t="inlineStr" /><c r="N489" s="2" t="inlineStr" /><c r="O489" s="2" t="inlineStr" /><c r="P489" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q489" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="490"><c r="A490" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B490" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C490" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D490" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E490" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek przeciwpadaczkowy – mechanizm działania: B</t></is></c><c r="F490" s="2" t="inlineStr"><is><t>fenytoina – hamowanie kanałów sodowych</t></is></c><c r="G490" s="2" t="inlineStr"><is><t>karbamazepina - hamowanie kanałów sodowych i kanałów wapniowych</t></is></c><c r="H490" s="2" t="inlineStr" /><c r="I490" s="2" t="inlineStr" /><c r="J490" s="2" t="inlineStr" /><c r="K490" s="2" t="inlineStr"><is><t>fenobarbital – hamowanie transmisji GABA-ergicznej</t></is></c><c r="L490" s="2" t="inlineStr"><is><t>kwas walproinowy – hamowanie kanałów sodowych i transmisji GABA-ergicznej</t></is></c><c r="M490" s="2" t="inlineStr" /><c r="N490" s="2" t="inlineStr" /><c r="O490" s="2" t="inlineStr" /><c r="P490" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q490" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="491"><c r="A491" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B491" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C491" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D491" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E491" s="2" t="inlineStr"><is><t>Selektywne inhibitory wychwytu zwrotnego serotoniny (SSRI) charakteryzuje:</t></is></c><c r="F491" s="2" t="inlineStr"><is><t>niewielki wpływ na układ krążenia</t></is></c><c r="G491" s="2" t="inlineStr"><is><t>małe ryzyko teratogenności</t></is></c><c r="H491" s="2" t="inlineStr" /><c r="I491" s="2" t="inlineStr" /><c r="J491" s="2" t="inlineStr" /><c r="K491" s="2" t="inlineStr"><is><t>obniżanie progu drgawkowego</t></is></c><c r="L491" s="2" t="inlineStr"><is><t>brak ryzyka wystąpienia istotnych interakcji z inhibitorami MAO</t></is></c><c r="M491" s="2" t="inlineStr" /><c r="N491" s="2" t="inlineStr" /><c r="O491" s="2" t="inlineStr" /><c r="P491" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q491" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="492"><c r="A492" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B492" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C492" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D492" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E492" s="2" t="inlineStr"><is><t>Potencjał uzależniający wykazują:</t></is></c><c r="F492" s="2" t="inlineStr"><is><t>Kanabinoidy</t></is></c><c r="G492" s="2" t="inlineStr"><is><t>dysocjacyjne środki znieczulające</t></is></c><c r="H492" s="2" t="inlineStr"><is><t>Benzodiazepiny</t></is></c><c r="I492" s="2" t="inlineStr"><is><t>opioidy</t></is></c><c r="J492" s="2" t="inlineStr" /><c r="K492" s="2" t="inlineStr" /><c r="L492" s="2" t="inlineStr" /><c r="M492" s="2" t="inlineStr" /><c r="N492" s="2" t="inlineStr" /><c r="O492" s="2" t="inlineStr" /><c r="P492" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q492" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="493"><c r="A493" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B493" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C493" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D493" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E493" s="2" t="inlineStr"><is><t>Działanie immunosupresyjne wykazują:</t></is></c><c r="F493" s="2" t="inlineStr"><is><t>inhibitory kalcyneuryny</t></is></c><c r="G493" s="2" t="inlineStr"><is><t>alkilujące inhibitory proliferacji</t></is></c><c r="H493" s="2" t="inlineStr" /><c r="I493" s="2" t="inlineStr" /><c r="J493" s="2" t="inlineStr" /><c r="K493" s="2" t="inlineStr"><is><t>czynniki stymulujące tworzenie kolonii granulocytów</t></is></c><c r="L493" s="2" t="inlineStr"><is><t>interferon beta</t></is></c><c r="M493" s="2" t="inlineStr" /><c r="N493" s="2" t="inlineStr" /><c r="O493" s="2" t="inlineStr" /><c r="P493" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q493" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="494"><c r="A494" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B494" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C494" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D494" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E494" s="2" t="inlineStr"><is><t>Hamowanie transmisji dopaminergicznej może być przyczyną wystąpienia:</t></is></c><c r="F494" s="2" t="inlineStr"><is><t>Dyskinez</t></is></c><c r="G494" s="2" t="inlineStr"><is><t>zwiększenia masy ciała</t></is></c><c r="H494" s="2" t="inlineStr"><is><t>działania przeciwwymiotnego</t></is></c><c r="I494" s="2" t="inlineStr" /><c r="J494" s="2" t="inlineStr" /><c r="K494" s="2" t="inlineStr"><is><t>hipoprolaktynemii</t></is></c><c r="L494" s="2" t="inlineStr" /><c r="M494" s="2" t="inlineStr" /><c r="N494" s="2" t="inlineStr" /><c r="O494" s="2" t="inlineStr" /><c r="P494" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q494" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="495"><c r="A495" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B495" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C495" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D495" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E495" s="2" t="inlineStr"><is><t>W przypadku rozpoznania anginy paciorkowcowej można zastosować:</t></is></c><c r="F495" s="2" t="inlineStr"><is><t>Klindamycynę</t></is></c><c r="G495" s="2" t="inlineStr"><is><t>Fenoksymetylopenicylinę</t></is></c><c r="H495" s="2" t="inlineStr" /><c r="I495" s="2" t="inlineStr" /><c r="J495" s="2" t="inlineStr" /><c r="K495" s="2" t="inlineStr"><is><t>Cyprofloksacynę</t></is></c><c r="L495" s="2" t="inlineStr"><is><t>Amikacynę</t></is></c><c r="M495" s="2" t="inlineStr" /><c r="N495" s="2" t="inlineStr" /><c r="O495" s="2" t="inlineStr" /><c r="P495" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q495" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="496"><c r="A496" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B496" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C496" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D496" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E496" s="2" t="inlineStr"><is><t>Chlorochina:</t></is></c><c r="F496" s="2" t="inlineStr"><is><t>Może być przyczyną wypadania włosów</t></is></c><c r="G496" s="2" t="inlineStr"><is><t>Niszczy formy wewnątrzkrwinkowe pierwotniaka</t></is></c><c r="H496" s="2" t="inlineStr" /><c r="I496" s="2" t="inlineStr" /><c r="J496" s="2" t="inlineStr" /><c r="K496" s="2" t="inlineStr"><is><t>Jest stosowana w każdym schemacie profilaktyki malarii</t></is></c><c r="L496" s="2" t="inlineStr"><is><t>Jest szczególnie skuteczna w leczeniu zakażenia Plasmodium falciparium</t></is></c><c r="M496" s="2" t="inlineStr" /><c r="N496" s="2" t="inlineStr" /><c r="O496" s="2" t="inlineStr" /><c r="P496" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q496" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="497"><c r="A497" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B497" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C497" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D497" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E497" s="2" t="inlineStr"><is><t>Lek bakteriobójczy, którego aktywność przeciwbakteryjną najlepiej charakteryzuje AUC24/MIC, działający na bakterie G(+). Lek nie ma aktywnych metabolitów i działa nefrotoksycznie. Opis może dotyczyć:</t></is></c><c r="F497" s="2" t="inlineStr"><is><t>Wankomycyny</t></is></c><c r="G497" s="2" t="inlineStr" /><c r="H497" s="2" t="inlineStr" /><c r="I497" s="2" t="inlineStr" /><c r="J497" s="2" t="inlineStr" /><c r="K497" s="2" t="inlineStr"><is><t>Kolistyny</t></is></c><c r="L497" s="2" t="inlineStr"><is><t>Klindamycyny</t></is></c><c r="M497" s="2" t="inlineStr"><is><t>Gentamycyny</t></is></c><c r="N497" s="2" t="inlineStr" /><c r="O497" s="2" t="inlineStr" /><c r="P497" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q497" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="498"><c r="A498" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B498" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C498" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D498" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E498" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Pseudomonas aeruginosa uzasadnione może być podanie:</t></is></c><c r="F498" s="2" t="inlineStr"><is><t>Piperacykliny z tazobaktamem</t></is></c><c r="G498" s="2" t="inlineStr"><is><t>Gentamycyny</t></is></c><c r="H498" s="2" t="inlineStr"><is><t>Cyprofloksacyny</t></is></c><c r="I498" s="2" t="inlineStr"><is><t>Ceftazydymu</t></is></c><c r="J498" s="2" t="inlineStr" /><c r="K498" s="2" t="inlineStr" /><c r="L498" s="2" t="inlineStr" /><c r="M498" s="2" t="inlineStr" /><c r="N498" s="2" t="inlineStr" /><c r="O498" s="2" t="inlineStr" /><c r="P498" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q498" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="499"><c r="A499" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B499" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C499" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D499" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E499" s="2" t="inlineStr"><is><t>Po podaniu doustnym działa miejscowo:</t></is></c><c r="F499" s="2" t="inlineStr"><is><t>Ryfaksymina</t></is></c><c r="G499" s="2" t="inlineStr"><is><t>Fidaksomycyna</t></is></c><c r="H499" s="2" t="inlineStr" /><c r="I499" s="2" t="inlineStr" /><c r="J499" s="2" t="inlineStr" /><c r="K499" s="2" t="inlineStr"><is><t>Kwas fusydowy</t></is></c><c r="L499" s="2" t="inlineStr"><is><t>Norfloksacyna</t></is></c><c r="M499" s="2" t="inlineStr" /><c r="N499" s="2" t="inlineStr" /><c r="O499" s="2" t="inlineStr" /><c r="P499" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q499" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="500"><c r="A500" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B500" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C500" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D500" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E500" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – punkt uchwytu:</t></is></c><c r="F500" s="2" t="inlineStr"><is><t>Acyklowir – polimeraza DNA</t></is></c><c r="G500" s="2" t="inlineStr"><is><t>Oseltamiwir – neuraminidaza</t></is></c><c r="H500" s="2" t="inlineStr"><is><t>Lamiwudyna – odwrotna transkryptaza</t></is></c><c r="I500" s="2" t="inlineStr"><is><t>Raltegrawir – integraza</t></is></c><c r="J500" s="2" t="inlineStr" /><c r="K500" s="2" t="inlineStr" /><c r="L500" s="2" t="inlineStr" /><c r="M500" s="2" t="inlineStr" /><c r="N500" s="2" t="inlineStr" /><c r="O500" s="2" t="inlineStr" /><c r="P500" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q500" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="501"><c r="A501" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B501" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C501" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D501" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E501" s="2" t="inlineStr"><is><t>Wybierz właściwe skojarzenie wskazanie – lek, który można zastosować jako alternatywę dla antybiotków beta-laktamowych u pacjenta z nadwrażliwością na tę grupę leków przeciwbakteryjnych</t></is></c><c r="F501" s="2" t="inlineStr"><is><t>Borelioza – azytromycyna</t></is></c><c r="G501" s="2" t="inlineStr"><is><t>Zapalenie płuc o etiologii pneumokokowej – lewofloksacyna</t></is></c><c r="H501" s="2" t="inlineStr"><is><t>Profilaktyka okołozabiegowa - wankomycyna</t></is></c><c r="I501" s="2" t="inlineStr" /><c r="J501" s="2" t="inlineStr" /><c r="K501" s="2" t="inlineStr"><is><t>Urosepsa o etiologii Escherichia coli – linezolid</t></is></c><c r="L501" s="2" t="inlineStr" /><c r="M501" s="2" t="inlineStr" /><c r="N501" s="2" t="inlineStr" /><c r="O501" s="2" t="inlineStr" /><c r="P501" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q501" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="502"><c r="A502" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B502" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C502" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D502" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E502" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – wskazanie:</t></is></c><c r="F502" s="2" t="inlineStr"><is><t>Metronidazol – lamblioza</t></is></c><c r="G502" s="2" t="inlineStr"><is><t>Spiramycyna – toksoplazmoza</t></is></c><c r="H502" s="2" t="inlineStr" /><c r="I502" s="2" t="inlineStr" /><c r="J502" s="2" t="inlineStr" /><c r="K502" s="2" t="inlineStr"><is><t>Nifuroksazyd – biegunka poantybiotykowa</t></is></c><c r="L502" s="2" t="inlineStr"><is><t>Amikacyna – borelioza</t></is></c><c r="M502" s="2" t="inlineStr" /><c r="N502" s="2" t="inlineStr" /><c r="O502" s="2" t="inlineStr" /><c r="P502" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q502" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="503"><c r="A503" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B503" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C503" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D503" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E503" s="2" t="inlineStr"><is><t>Wskazaniem do doustnej terapii przeciwgrzybiczej jest:</t></is></c><c r="F503" s="2" t="inlineStr"><is><t>Nieskuteczność leczenia miejscowego</t></is></c><c r="G503" s="2" t="inlineStr"><is><t>Grzybica inwazyjna</t></is></c><c r="H503" s="2" t="inlineStr"><is><t>Stwierdzenie rozległych zmian skórnych</t></is></c><c r="I503" s="2" t="inlineStr" /><c r="J503" s="2" t="inlineStr" /><c r="K503" s="2" t="inlineStr"><is><t>Grzybica paznokci dotycząca pojedynczych płytek paznokciowych</t></is></c><c r="L503" s="2" t="inlineStr" /><c r="M503" s="2" t="inlineStr" /><c r="N503" s="2" t="inlineStr" /><c r="O503" s="2" t="inlineStr" /><c r="P503" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q503" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="504"><c r="A504" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B504" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C504" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D504" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E504" s="2" t="inlineStr"><is><t>Działanie neurotoksyczne wykazuje:</t></is></c><c r="F504" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="G504" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="H504" s="2" t="inlineStr"><is><t>kolistyna</t></is></c><c r="I504" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="J504" s="2" t="inlineStr" /><c r="K504" s="2" t="inlineStr" /><c r="L504" s="2" t="inlineStr" /><c r="M504" s="2" t="inlineStr" /><c r="N504" s="2" t="inlineStr" /><c r="O504" s="2" t="inlineStr" /><c r="P504" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q504" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="505"><c r="A505" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B505" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C505" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D505" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E505" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – mechanizm działania (należy uwzględnić główny mechanizm działania):</t></is></c><c r="F505" s="2" t="inlineStr"><is><t>Azytromycyna – hamowanie syntezy białek</t></is></c><c r="G505" s="2" t="inlineStr"><is><t>Daptomycyna – uszkodzenie błony komórkowej</t></is></c><c r="H505" s="2" t="inlineStr" /><c r="I505" s="2" t="inlineStr" /><c r="J505" s="2" t="inlineStr" /><c r="K505" s="2" t="inlineStr"><is><t>Cyprofloksacyna – hamowanie biosyntezy ściany komórkowej</t></is></c><c r="L505" s="2" t="inlineStr"><is><t>Amoksycyina – hamowanie syntezy DNA</t></is></c><c r="M505" s="2" t="inlineStr" /><c r="N505" s="2" t="inlineStr" /><c r="O505" s="2" t="inlineStr" /><c r="P505" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q505" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="506"><c r="A506" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B506" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C506" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D506" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E506" s="2" t="inlineStr"><is><t>W schematach eradykacji Helicobacter pylori znajdują zastosowanie:</t></is></c><c r="F506" s="2" t="inlineStr"><is><t>Amoksycylina</t></is></c><c r="G506" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="H506" s="2" t="inlineStr" /><c r="I506" s="2" t="inlineStr" /><c r="J506" s="2" t="inlineStr" /><c r="K506" s="2" t="inlineStr"><is><t>Lewofloksacyna</t></is></c><c r="L506" s="2" t="inlineStr"><is><t>Tetracyklina</t></is></c><c r="M506" s="2" t="inlineStr" /><c r="N506" s="2" t="inlineStr" /><c r="O506" s="2" t="inlineStr" /><c r="P506" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q506" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="507"><c r="A507" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B507" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C507" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D507" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E507" s="2" t="inlineStr"><is><t>Linezolid może być skuteczny w zakażeniach szczepami:</t></is></c><c r="F507" s="2" t="inlineStr"><is><t>MRSA (methicyllin-resistant Staphylococcus aureus)</t></is></c><c r="G507" s="2" t="inlineStr"><is><t>MSSA (methicyllin-sensitive Staphylococcus aureus)</t></is></c><c r="H507" s="2" t="inlineStr"><is><t>VRE (Vancomycin-resistant Enterococcus)</t></is></c><c r="I507" s="2" t="inlineStr" /><c r="J507" s="2" t="inlineStr" /><c r="K507" s="2" t="inlineStr"><is><t>CPE (Carbapenemase-producing Enterobacteriaceae)</t></is></c><c r="L507" s="2" t="inlineStr" /><c r="M507" s="2" t="inlineStr" /><c r="N507" s="2" t="inlineStr" /><c r="O507" s="2" t="inlineStr" /><c r="P507" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q507" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="508"><c r="A508" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B508" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C508" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D508" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E508" s="2" t="inlineStr"><is><t>Profilaktyczne zastosowanie leków przeciwinfekcyjnych jest uzasadnione:</t></is></c><c r="F508" s="2" t="inlineStr"><is><t>W planowej operacji cięcia cesarskiego (pole czyste-skażone)</t></is></c><c r="G508" s="2" t="inlineStr"><is><t>W planowej implantacji endoprotezy stawu kolanowego (pole czyste)</t></is></c><c r="H508" s="2" t="inlineStr" /><c r="I508" s="2" t="inlineStr" /><c r="J508" s="2" t="inlineStr" /><c r="K508" s="2" t="inlineStr"><is><t>W planowanym usunięciu zmiany skórnej w obrębie dłoni (pole czyste)</t></is></c><c r="L508" s="2" t="inlineStr"><is><t>W planowym usunięciu tarczycy w wolu guzkowym nadczynnym (pole czyste)</t></is></c><c r="M508" s="2" t="inlineStr" /><c r="N508" s="2" t="inlineStr" /><c r="O508" s="2" t="inlineStr" /><c r="P508" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q508" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="509"><c r="A509" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B509" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C509" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D509" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E509" s="2" t="inlineStr"><is><t>Do bezpiecznych i skutecznych środków do dezynfekcji należą:</t></is></c><c r="F509" s="2" t="inlineStr"><is><t>Oktenidyna</t></is></c><c r="G509" s="2" t="inlineStr" /><c r="H509" s="2" t="inlineStr" /><c r="I509" s="2" t="inlineStr" /><c r="J509" s="2" t="inlineStr" /><c r="K509" s="2" t="inlineStr"><is><t>Spirytus salicylowy</t></is></c><c r="L509" s="2" t="inlineStr"><is><t>Woda utleniona</t></is></c><c r="M509" s="2" t="inlineStr"><is><t>Mleczan etakrydyny</t></is></c><c r="N509" s="2" t="inlineStr" /><c r="O509" s="2" t="inlineStr" /><c r="P509" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q509" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="510"><c r="A510" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B510" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C510" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D510" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E510" s="2" t="inlineStr"><is><t>U kobiety w ciąży można bezpiecznie zastosować:</t></is></c><c r="F510" s="2" t="inlineStr"><is><t>Cefuroksym</t></is></c><c r="G510" s="2" t="inlineStr"><is><t>Fenoksymetylopenicylinę</t></is></c><c r="H510" s="2" t="inlineStr" /><c r="I510" s="2" t="inlineStr" /><c r="J510" s="2" t="inlineStr" /><c r="K510" s="2" t="inlineStr"><is><t>Amikacynę</t></is></c><c r="L510" s="2" t="inlineStr"><is><t>Moksyfloksacynę</t></is></c><c r="M510" s="2" t="inlineStr" /><c r="N510" s="2" t="inlineStr" /><c r="O510" s="2" t="inlineStr" /><c r="P510" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q510" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="511"><c r="A511" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B511" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C511" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D511" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E511" s="2" t="inlineStr"><is><t>Wskaż właściwe skojarzenie lek – potencjalne działanie nipożądane:</t></is></c><c r="F511" s="2" t="inlineStr"><is><t>Doksycyklina – fotodermatoza</t></is></c><c r="G511" s="2" t="inlineStr"><is><t>Linezolid - zespół serotoninowy</t></is></c><c r="H511" s="2" t="inlineStr" /><c r="I511" s="2" t="inlineStr" /><c r="J511" s="2" t="inlineStr" /><c r="K511" s="2" t="inlineStr"><is><t>Mupirocyna - zespół czerwonego dziecka</t></is></c><c r="L511" s="2" t="inlineStr"><is><t>Gentamycyna - żółtaczka cholestatyczna</t></is></c><c r="M511" s="2" t="inlineStr" /><c r="N511" s="2" t="inlineStr" /><c r="O511" s="2" t="inlineStr" /><c r="P511" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q511" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="512"><c r="A512" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B512" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C512" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D512" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E512" s="2" t="inlineStr"><is><t>Działanie nefrotoksyczne wykazuje:</t></is></c><c r="F512" s="2" t="inlineStr"><is><t>Gentamycyna</t></is></c><c r="G512" s="2" t="inlineStr"><is><t>Kolistyna</t></is></c><c r="H512" s="2" t="inlineStr"><is><t>Wankomycyna</t></is></c><c r="I512" s="2" t="inlineStr" /><c r="J512" s="2" t="inlineStr" /><c r="K512" s="2" t="inlineStr"><is><t>Klindamycyna</t></is></c><c r="L512" s="2" t="inlineStr" /><c r="M512" s="2" t="inlineStr" /><c r="N512" s="2" t="inlineStr" /><c r="O512" s="2" t="inlineStr" /><c r="P512" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q512" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="513"><c r="A513" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B513" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C513" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D513" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E513" s="2" t="inlineStr"><is><t>W biegunce o etiologii Clostridioides difficile uzasadnione może być podanie doustne:</t></is></c><c r="F513" s="2" t="inlineStr"><is><t>Fidaksomycyny</t></is></c><c r="G513" s="2" t="inlineStr"><is><t>Metronidazolu</t></is></c><c r="H513" s="2" t="inlineStr" /><c r="I513" s="2" t="inlineStr" /><c r="J513" s="2" t="inlineStr" /><c r="K513" s="2" t="inlineStr"><is><t>Neomycyny</t></is></c><c r="L513" s="2" t="inlineStr"><is><t>Nifuroksazydu</t></is></c><c r="M513" s="2" t="inlineStr" /><c r="N513" s="2" t="inlineStr" /><c r="O513" s="2" t="inlineStr" /><c r="P513" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q513" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="514"><c r="A514" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B514" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C514" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D514" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E514" s="2" t="inlineStr"><is><t>Wskaż stwierdzenie/a prawdziwe:</t></is></c><c r="F514" s="2" t="inlineStr"><is><t>Ketokonazol stosuje się wyłącznie miejscowo w leczeniu grzybic</t></is></c><c r="G514" s="2" t="inlineStr" /><c r="H514" s="2" t="inlineStr" /><c r="I514" s="2" t="inlineStr" /><c r="J514" s="2" t="inlineStr" /><c r="K514" s="2" t="inlineStr"><is><t>Terbinafina hamuje enzym związany z ukłądem CYP450</t></is></c><c r="L514" s="2" t="inlineStr"><is><t>Zastosowanie technologii liposomów pozwoliło na otrzymanie preparatów amfoterycyny B o istotnie zmniejszonej hepatotoksyczności</t></is></c><c r="M514" s="2" t="inlineStr"><is><t>Kaspofungina osiąga bardzo wysokie stężenia w OUN</t></is></c><c r="N514" s="2" t="inlineStr" /><c r="O514" s="2" t="inlineStr" /><c r="P514" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q514" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="515"><c r="A515" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B515" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C515" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D515" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E515" s="2" t="inlineStr"><is><t>Metronidazol:</t></is></c><c r="F515" s="2" t="inlineStr"><is><t>Dobrze penetruje do OUN</t></is></c><c r="G515" s="2" t="inlineStr"><is><t>Działa na Entamoeba histolytica</t></is></c><c r="H515" s="2" t="inlineStr" /><c r="I515" s="2" t="inlineStr" /><c r="J515" s="2" t="inlineStr" /><c r="K515" s="2" t="inlineStr"><is><t>Bardzo często jest przyczyną zapalenia ścięgna Achillesa</t></is></c><c r="L515" s="2" t="inlineStr"><is><t>Jest stosowany w wewnątrzbrzusznych zakażeniach szczepami wielolekoopornymi</t></is></c><c r="M515" s="2" t="inlineStr" /><c r="N515" s="2" t="inlineStr" /><c r="O515" s="2" t="inlineStr" /><c r="P515" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q515" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="516"><c r="A516" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B516" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C516" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D516" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E516" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie drobnoustrój - lek, który może być skuteczny w zakażeniu o takiej etiologii:</t></is></c><c r="F516" s="2" t="inlineStr"><is><t>Staphylococcus aureus (MSSA) - kloksacylina</t></is></c><c r="G516" s="2" t="inlineStr"><is><t>Clostridioides difficile – wankomycyna</t></is></c><c r="H516" s="2" t="inlineStr" /><c r="I516" s="2" t="inlineStr" /><c r="J516" s="2" t="inlineStr" /><c r="K516" s="2" t="inlineStr"><is><t>Staphylococcus aureus (MRSA) - meropenem</t></is></c><c r="L516" s="2" t="inlineStr"><is><t>Trichomonas vaginalis - ketokonazol</t></is></c><c r="M516" s="2" t="inlineStr" /><c r="N516" s="2" t="inlineStr" /><c r="O516" s="2" t="inlineStr" /><c r="P516" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q516" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="517"><c r="A517" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B517" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C517" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D517" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E517" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – wskazanie do leczenia:</t></is></c><c r="F517" s="2" t="inlineStr"><is><t>Acyklowir - półpasiec</t></is></c><c r="G517" s="2" t="inlineStr"><is><t>Gancyklowir – cytomegalowirusowe zapalenie siatkówki</t></is></c><c r="H517" s="2" t="inlineStr"><is><t>Osetamiwir – grypa</t></is></c><c r="I517" s="2" t="inlineStr" /><c r="J517" s="2" t="inlineStr" /><c r="K517" s="2" t="inlineStr"><is><t>Amantadyna – mononukleoza</t></is></c><c r="L517" s="2" t="inlineStr" /><c r="M517" s="2" t="inlineStr" /><c r="N517" s="2" t="inlineStr" /><c r="O517" s="2" t="inlineStr" /><c r="P517" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q517" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="518"><c r="A518" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B518" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C518" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D518" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E518" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie drobnoustrój - lek, który może być skuteczny w zakażeniu o tej etiologii:</t></is></c><c r="F518" s="2" t="inlineStr"><is><t>Helicobacter pylori – tetracyklina</t></is></c><c r="G518" s="2" t="inlineStr"><is><t>Staphylococcus aureus (MSSA) - cefazolina</t></is></c><c r="H518" s="2" t="inlineStr" /><c r="I518" s="2" t="inlineStr" /><c r="J518" s="2" t="inlineStr" /><c r="K518" s="2" t="inlineStr"><is><t>Escherichia coli – klindamycyna</t></is></c><c r="L518" s="2" t="inlineStr"><is><t>Mycoplasma pneumoniae - teikoplanina</t></is></c><c r="M518" s="2" t="inlineStr" /><c r="N518" s="2" t="inlineStr" /><c r="O518" s="2" t="inlineStr" /><c r="P518" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q518" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="519"><c r="A519" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B519" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C519" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D519" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E519" s="2" t="inlineStr"><is><t>Wytyczne PRISMA:</t></is></c><c r="F519" s="2" t="inlineStr"><is><t>dotyczą prowadzenia przeglądów systematycznych i metaanaliz</t></is></c><c r="G519" s="2" t="inlineStr" /><c r="H519" s="2" t="inlineStr" /><c r="I519" s="2" t="inlineStr" /><c r="J519" s="2" t="inlineStr" /><c r="K519" s="2" t="inlineStr"><is><t>dotyczą prowadzenia randomizowanych badań klinicznych</t></is></c><c r="L519" s="2" t="inlineStr"><is><t>dotyczą formułowania wytycznych klinicznych</t></is></c><c r="M519" s="2" t="inlineStr"><is><t>dotyczą prowadzenia badań obserwacyjnych</t></is></c><c r="N519" s="2" t="inlineStr" /><c r="O519" s="2" t="inlineStr" /><c r="P519" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q519" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="520"><c r="A520" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B520" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C520" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D520" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E520" s="2" t="inlineStr"><is><t>Lek ma Vd=6 l/kg m.c. i CL=10 ml/min/kg m.c. Na tej podstawie spodziewasz się, że lek będzie:</t></is></c><c r="F520" s="2" t="inlineStr"><is><t>wymagał dużej dawki nasycającej</t></is></c><c r="G520" s="2" t="inlineStr" /><c r="H520" s="2" t="inlineStr" /><c r="I520" s="2" t="inlineStr" /><c r="J520" s="2" t="inlineStr" /><c r="K520" s="2" t="inlineStr"><is><t>kumulował się w tkance tłuszczowej</t></is></c><c r="L520" s="2" t="inlineStr"><is><t>miał długi okres półtrwania</t></is></c><c r="M520" s="2" t="inlineStr"><is><t>wymagał korekty dawkowania w niewydolności nerek</t></is></c><c r="N520" s="2" t="inlineStr" /><c r="O520" s="2" t="inlineStr" /><c r="P520" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q520" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="521"><c r="A521" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B521" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C521" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D521" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E521" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenia dotyczące wiązania leków z białkami osocza:</t></is></c><c r="F521" s="2" t="inlineStr"><is><t>może być przyczyną istotnych klinicznie interakcji lekowych</t></is></c><c r="G521" s="2" t="inlineStr" /><c r="H521" s="2" t="inlineStr" /><c r="I521" s="2" t="inlineStr" /><c r="J521" s="2" t="inlineStr" /><c r="K521" s="2" t="inlineStr"><is><t>z powodu zmniejszenia stężenia albumin we krwi leki o dużym stopniu wiązaniu z albuminami mogą wykazywać niedostateczny efekt terapeutyczny</t></is></c><c r="L521" s="2" t="inlineStr"><is><t>jest istotne klinicznie wtedy, gdy frakcja wolna wynosi 80%</t></is></c><c r="M521" s="2" t="inlineStr"><is><t>przebiega w wątrobie, gdzie zachodzi sprzęganie leku z albuminami</t></is></c><c r="N521" s="2" t="inlineStr" /><c r="O521" s="2" t="inlineStr" /><c r="P521" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q521" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="522"><c r="A522" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B522" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C522" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D522" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E522" s="2" t="inlineStr"><is><t>Lek o kinetyce pierwszego rzędu po podaniu doustnym ma biodostępność ok. 100% i okres półtrwania =12 godzin. Pacjent A przyjmuje doustnie ten lek w dawce D co 12 godzin (o godz. 8:00 i 20:00). Pacjent B przyjmuje doustnie ten lek w dawce 2D co 24 godziny (o godz. 8:00). Pacjent C przyjmuje ten lek w ciągłym wlewie dożylnym w dawce odpowiadającej 2D/24h. Wszyscy pacjenci mają prawidłową czynność narządów uczestniczących w eliminacji. Wskaż prawdziwe stwierdzenie:</t></is></c><c r="F522" s="2" t="inlineStr"><is><t>czas eliminacji leku po zakończeniu podawania jest taki sam u wszystkich pacjentów</t></is></c><c r="G522" s="2" t="inlineStr" /><c r="H522" s="2" t="inlineStr" /><c r="I522" s="2" t="inlineStr" /><c r="J522" s="2" t="inlineStr" /><c r="K522" s="2" t="inlineStr"><is><t>w stanie stacjonarnym po pobraniu próbki krwi o godzinie 7:30 rano stężenie tego leku we krwi ma taką samą wartość u wszystkich pacjentów</t></is></c><c r="L522" s="2" t="inlineStr"><is><t>stan stacjonarny ustala się szybciej u pacjenta A niż u pacjenta B</t></is></c><c r="M522" s="2" t="inlineStr"><is><t>wiązanie leku z białkami jest największe u pacjenta C, a najmniejsze u pacjenta A</t></is></c><c r="N522" s="2" t="inlineStr" /><c r="O522" s="2" t="inlineStr" /><c r="P522" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q522" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="523"><c r="A523" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B523" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C523" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D523" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E523" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące warfaryny:</t></is></c><c r="F523" s="2" t="inlineStr"><is><t>blokuje aktywność reduktazy epoksydowej fitomenadionu</t></is></c><c r="G523" s="2" t="inlineStr"><is><t>aktywność warfaryny zależy od polimorfizmu genetycznego izoenzymu CYP2C9</t></is></c><c r="H523" s="2" t="inlineStr" /><c r="I523" s="2" t="inlineStr" /><c r="J523" s="2" t="inlineStr" /><c r="K523" s="2" t="inlineStr"><is><t>zwiększa aktywność białka C i jego kofaktora - białka S o działaniu przeciwzakrzepowym</t></is></c><c r="L523" s="2" t="inlineStr"><is><t>zmniejsza aktywność biologiczną czynników krzepnięcia zespołu protrombiny skutecznie zapobiegając zakrzepicy od 2. doby po włączeniuleczenia</t></is></c><c r="M523" s="2" t="inlineStr" /><c r="N523" s="2" t="inlineStr" /><c r="O523" s="2" t="inlineStr" /><c r="P523" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q523" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="524"><c r="A524" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B524" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C524" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D524" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E524" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące małopłytkowości indukowanej heparyną (HIT) typu II:</t></is></c><c r="F524" s="2" t="inlineStr"><is><t>Występuje typowo między 5. a 10. dniem ekspozycji na heparyny ze znacznym nadmiarem liczby płytek (30 000-50 000/mikrolitr)</t></is></c><c r="G524" s="2" t="inlineStr"><is><t>Stwarza istotne ryzyko powikła zakrzepowo-zatorowych</t></is></c><c r="H524" s="2" t="inlineStr"><is><t>Jest potwierdzana identyfikacją przeciwciał przeciw kompleksom heparyna-PF4 w surowicy</t></is></c><c r="I524" s="2" t="inlineStr"><is><t>Jest bezterminowym przeciwwskazaniem do reekspozycji chorego na heparyny</t></is></c><c r="J524" s="2" t="inlineStr" /><c r="K524" s="2" t="inlineStr" /><c r="L524" s="2" t="inlineStr" /><c r="M524" s="2" t="inlineStr" /><c r="N524" s="2" t="inlineStr" /><c r="O524" s="2" t="inlineStr" /><c r="P524" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q524" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="525"><c r="A525" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B525" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C525" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D525" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E525" s="2" t="inlineStr"><is><t>Kwas traneksamowy:</t></is></c><c r="F525" s="2" t="inlineStr"><is><t>hamuje aktywatory plazminogenu</t></is></c><c r="G525" s="2" t="inlineStr"><is><t>powoduje zagrożenie powikłaniami zakrzepowo-zatorowymi</t></is></c><c r="H525" s="2" t="inlineStr"><is><t>jest antidotum w krwawieniach związanych ze stosowaniem leków fibrynolitycznych</t></is></c><c r="I525" s="2" t="inlineStr" /><c r="J525" s="2" t="inlineStr" /><c r="K525" s="2" t="inlineStr"><is><t>zwiększa śmiertelność w krwotokach operacyjnych i pourazowych</t></is></c><c r="L525" s="2" t="inlineStr" /><c r="M525" s="2" t="inlineStr" /><c r="N525" s="2" t="inlineStr" /><c r="O525" s="2" t="inlineStr" /><c r="P525" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q525" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="526"><c r="A526" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B526" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C526" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D526" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E526" s="2" t="inlineStr"><is><t>Efekt działania w czasie do 10 minut od podania występuje po podaniu:</t></is></c><c r="F526" s="2" t="inlineStr"><is><t>fentanylu donosowo</t></is></c><c r="G526" s="2" t="inlineStr"><is><t>naloksonu dożylnie</t></is></c><c r="H526" s="2" t="inlineStr"><is><t>glukagonu domięśniowo</t></is></c><c r="I526" s="2" t="inlineStr" /><c r="J526" s="2" t="inlineStr" /><c r="K526" s="2" t="inlineStr"><is><t>węgla medycznego (aktywowanego) w dawce 1 g przez zgłębnik nosowo￾żoładkowy</t></is></c><c r="L526" s="2" t="inlineStr" /><c r="M526" s="2" t="inlineStr" /><c r="N526" s="2" t="inlineStr" /><c r="O526" s="2" t="inlineStr" /><c r="P526" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q526" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="527"><c r="A527" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B527" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C527" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D527" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E527" s="2" t="inlineStr"><is><t>Wskaż zestaw, gdzie prawidłowo uszeregowano insuliny od najkrócej do najdłużej działającej:</t></is></c><c r="F527" s="2" t="inlineStr"><is><t>lispro–insulina ludzka–glargina</t></is></c><c r="G527" s="2" t="inlineStr"><is><t>glulizyna–insulina ludzka izofanowa–degludec</t></is></c><c r="H527" s="2" t="inlineStr" /><c r="I527" s="2" t="inlineStr" /><c r="J527" s="2" t="inlineStr" /><c r="K527" s="2" t="inlineStr"><is><t>aspart – degludec – detemir</t></is></c><c r="L527" s="2" t="inlineStr"><is><t>detemir–glulizyna–insulina protaminowo-cynkowa</t></is></c><c r="M527" s="2" t="inlineStr" /><c r="N527" s="2" t="inlineStr" /><c r="O527" s="2" t="inlineStr" /><c r="P527" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q527" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="528"><c r="A528" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B528" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C528" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D528" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E528" s="2" t="inlineStr"><is><t>Ostre zapalenie trzustki może być powikłaniem stosowania:</t></is></c><c r="F528" s="2" t="inlineStr"><is><t>inhibitorów dipeptydylopeptydazy 4 (DPP-4)</t></is></c><c r="G528" s="2" t="inlineStr"><is><t>inhibitory reduktazy HMG-Ca</t></is></c><c r="H528" s="2" t="inlineStr"><is><t>związków kwasu 5-aminosalicylowego</t></is></c><c r="I528" s="2" t="inlineStr"><is><t>doustnych środków antykoncepcyjnych</t></is></c><c r="J528" s="2" t="inlineStr" /><c r="K528" s="2" t="inlineStr" /><c r="L528" s="2" t="inlineStr" /><c r="M528" s="2" t="inlineStr" /><c r="N528" s="2" t="inlineStr" /><c r="O528" s="2" t="inlineStr" /><c r="P528" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q528" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="529"><c r="A529" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B529" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C529" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D529" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E529" s="2" t="inlineStr"><is><t>Pacjentka z obustronnym ostrym pozagałkowym zapaleniem nerwu wzrokowego, co zagraża ślepotą, wymaga leczenia metyloprednizolonem (brak alternatywy leczniczej). Zostałeś poproszona/-y o konsultację w celu oceny przeciwwskazań do steroidoterapii. Która z chorób współistniejących jest w tej sytuacji przeciwwskazaniem do zastosowania leku:</t></is></c><c r="F529" s="2" t="inlineStr"><is><t>ciężka sepsa o niejasnej etiologii</t></is></c><c r="G529" s="2" t="inlineStr" /><c r="H529" s="2" t="inlineStr" /><c r="I529" s="2" t="inlineStr" /><c r="J529" s="2" t="inlineStr" /><c r="K529" s="2" t="inlineStr"><is><t>cukrzyca typu 1</t></is></c><c r="L529" s="2" t="inlineStr"><is><t>nadciśnienie tętnicze</t></is></c><c r="M529" s="2" t="inlineStr"><is><t>zaburzenia psychotyczne pod postacią omamów i agresji</t></is></c><c r="N529" s="2" t="inlineStr" /><c r="O529" s="2" t="inlineStr" /><c r="P529" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q529" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="530"><c r="A530" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B530" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C530" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D530" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E530" s="2" t="inlineStr"><is><t>Które połączenie rozważysz w przypadku nie osiągnięcia zakładanej redukcji stężenia cholesterolu frakcji LDL podczas stosowania diety i atorwastatyny?</t></is></c><c r="F530" s="2" t="inlineStr"><is><t>atorwastatyna + anacetrapib</t></is></c><c r="G530" s="2" t="inlineStr"><is><t>atorwastatyna + ezetymib</t></is></c><c r="H530" s="2" t="inlineStr"><is><t>atorwastatyna + kwas eikozapentaenowy</t></is></c><c r="I530" s="2" t="inlineStr"><is><t>atorwastatyna + ewolokumab</t></is></c><c r="J530" s="2" t="inlineStr" /><c r="K530" s="2" t="inlineStr" /><c r="L530" s="2" t="inlineStr" /><c r="M530" s="2" t="inlineStr" /><c r="N530" s="2" t="inlineStr" /><c r="O530" s="2" t="inlineStr" /><c r="P530" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q530" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="531"><c r="A531" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B531" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C531" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D531" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E531" s="2" t="inlineStr"><is><t>Taki sam mechanizm działania mają:</t></is></c><c r="F531" s="2" t="inlineStr"><is><t>bazyliksymab i daklizumab</t></is></c><c r="G531" s="2" t="inlineStr"><is><t>rytuksymab i okrelizumab</t></is></c><c r="H531" s="2" t="inlineStr" /><c r="I531" s="2" t="inlineStr" /><c r="J531" s="2" t="inlineStr" /><c r="K531" s="2" t="inlineStr"><is><t>natalizumab i fingolimod</t></is></c><c r="L531" s="2" t="inlineStr"><is><t>filgrastym i romiplostym</t></is></c><c r="M531" s="2" t="inlineStr" /><c r="N531" s="2" t="inlineStr" /><c r="O531" s="2" t="inlineStr" /><c r="P531" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q531" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="532"><c r="A532" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B532" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C532" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D532" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E532" s="2" t="inlineStr"><is><t>Powikłaniem stosowania inhibitora H+ K+ –ATPazy komórek okładzinowych może być:</t></is></c><c r="F532" s="2" t="inlineStr"><is><t>niedokrwistość makrocytarna z powodu niedoboru witaminy B12</t></is></c><c r="G532" s="2" t="inlineStr"><is><t>osteoporoza z powodu zaburzeń wchłaniania wapnia</t></is></c><c r="H532" s="2" t="inlineStr"><is><t>bakteryjne zakażenia przewodu pokarmowego</t></is></c><c r="I532" s="2" t="inlineStr"><is><t>zmiany wchłaniania wielu leków z przewodu pokarmowego</t></is></c><c r="J532" s="2" t="inlineStr" /><c r="K532" s="2" t="inlineStr" /><c r="L532" s="2" t="inlineStr" /><c r="M532" s="2" t="inlineStr" /><c r="N532" s="2" t="inlineStr" /><c r="O532" s="2" t="inlineStr" /><c r="P532" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q532" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="533"><c r="A533" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B533" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C533" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D533" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E533" s="2" t="inlineStr"><is><t>Lekiem stosowanym w objawach ze strony przewodu pokarmowego o wpływie na układ opioidowy jest:</t></is></c><c r="F533" s="2" t="inlineStr"><is><t>trimebutyna</t></is></c><c r="G533" s="2" t="inlineStr"><is><t>racekadotryl</t></is></c><c r="H533" s="2" t="inlineStr"><is><t>metylnaltrekson</t></is></c><c r="I533" s="2" t="inlineStr" /><c r="J533" s="2" t="inlineStr" /><c r="K533" s="2" t="inlineStr"><is><t>dekstrometorfan</t></is></c><c r="L533" s="2" t="inlineStr" /><c r="M533" s="2" t="inlineStr" /><c r="N533" s="2" t="inlineStr" /><c r="O533" s="2" t="inlineStr" /><c r="P533" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q533" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="534"><c r="A534" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B534" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C534" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D534" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E534" s="2" t="inlineStr"><is><t>W niewydolności nerek należy zmodyfikować dawkowanie:</t></is></c><c r="F534" s="2" t="inlineStr"><is><t>eteksylanu dabigatranu</t></is></c><c r="G534" s="2" t="inlineStr" /><c r="H534" s="2" t="inlineStr" /><c r="I534" s="2" t="inlineStr" /><c r="J534" s="2" t="inlineStr" /><c r="K534" s="2" t="inlineStr"><is><t>atorwastatyny</t></is></c><c r="L534" s="2" t="inlineStr"><is><t>kwasu acetylosalicylowego</t></is></c><c r="M534" s="2" t="inlineStr"><is><t>lewotyroksyny</t></is></c><c r="N534" s="2" t="inlineStr" /><c r="O534" s="2" t="inlineStr" /><c r="P534" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q534" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="535"><c r="A535" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B535" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C535" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D535" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E535" s="2" t="inlineStr"><is><t>Tramadol:</t></is></c><c r="F535" s="2" t="inlineStr"><is><t>ma mechanizm działania podobny do tapentadolu</t></is></c><c r="G535" s="2" t="inlineStr"><is><t>może powodować drgawki</t></is></c><c r="H535" s="2" t="inlineStr" /><c r="I535" s="2" t="inlineStr" /><c r="J535" s="2" t="inlineStr" /><c r="K535" s="2" t="inlineStr"><is><t>może zwiększać ryzyko hiperglikemii i pogarszać kontrolę cukrzycy</t></is></c><c r="L535" s="2" t="inlineStr"><is><t>działa przeciwbólowo skuteczniej w połączeniu z lekami przeciwdepresyjnymi z powodu synergizmu działania</t></is></c><c r="M535" s="2" t="inlineStr" /><c r="N535" s="2" t="inlineStr" /><c r="O535" s="2" t="inlineStr" /><c r="P535" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q535" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="536"><c r="A536" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B536" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C536" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D536" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E536" s="2" t="inlineStr"><is><t>Rotacja opioidów:</t></is></c><c r="F536" s="2" t="inlineStr"><is><t>wymaga ustalenia ekwianelgetycznych dawek zamienianych opioidów, np. morfina : oksykodon p.o. odpowiednio 10 mg : 6,67 mg</t></is></c><c r="G536" s="2" t="inlineStr" /><c r="H536" s="2" t="inlineStr" /><c r="I536" s="2" t="inlineStr" /><c r="J536" s="2" t="inlineStr" /><c r="K536" s="2" t="inlineStr"><is><t>wymaga nie łączenia opioidów z innymi lekami przeciwbólowymi</t></is></c><c r="L536" s="2" t="inlineStr"><is><t>pomaga zapobiec immunosupresyjnemu działaniu opioidów</t></is></c><c r="M536" s="2" t="inlineStr"><is><t>powinna być oparta o tą samą drogę podania, to znaczy rotowane opioidy powinny mieć tę samą postać farmaceutyczną</t></is></c><c r="N536" s="2" t="inlineStr" /><c r="O536" s="2" t="inlineStr" /><c r="P536" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q536" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="537"><c r="A537" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B537" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C537" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D537" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E537" s="2" t="inlineStr"><is><t>Pasażerowie podróżujący wagonem metra, w którym odnaleziono porzucony bagaż, zostali przyjęci na oddział ratunkowy z powodu bolesnych skurczów jelit, wymiotów, duszności i osłabienia siły mięśniowej. W badaniu fizykalnym stwierdzono zwiększoną częstość oddechów, świsty oskrzelowe, bradykardię i zwężenie źrenic. Lek/leki z wyboru w powyższej sytuacji to:</t></is></c><c r="F537" s="2" t="inlineStr"><is><t>acetylocysteina</t></is></c><c r="G537" s="2" t="inlineStr"><is><t>pralidoksym</t></is></c><c r="H537" s="2" t="inlineStr"><is><t>pirydostygmina</t></is></c><c r="I537" s="2" t="inlineStr"><is><t>atropina</t></is></c><c r="J537" s="2" t="inlineStr" /><c r="K537" s="2" t="inlineStr" /><c r="L537" s="2" t="inlineStr" /><c r="M537" s="2" t="inlineStr" /><c r="N537" s="2" t="inlineStr" /><c r="O537" s="2" t="inlineStr" /><c r="P537" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q537" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="538"><c r="A538" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B538" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C538" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D538" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E538" s="2" t="inlineStr"><is><t>Inhibitory immunologicznych punktów kontrolnych:</t></is></c><c r="F538" s="2" t="inlineStr"><is><t>są przeciwciałami monoklonalnymi przeciw CLTA-4, PD-1 i PDL-1</t></is></c><c r="G538" s="2" t="inlineStr"><is><t>nawiązują koncepcyjnie do immunostymulującego działania szczepionki BCG w raku pęcherza moczowego</t></is></c><c r="H538" s="2" t="inlineStr"><is><t>są skuteczne w leczeniu różnych typów nowotworów</t></is></c><c r="I538" s="2" t="inlineStr"><is><t>indukują zjawiska autoimmunologiczne</t></is></c><c r="J538" s="2" t="inlineStr" /><c r="K538" s="2" t="inlineStr" /><c r="L538" s="2" t="inlineStr" /><c r="M538" s="2" t="inlineStr" /><c r="N538" s="2" t="inlineStr" /><c r="O538" s="2" t="inlineStr" /><c r="P538" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q538" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="539"><c r="A539" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B539" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C539" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D539" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E539" s="2" t="inlineStr"><is><t>Projektant mody Alexander McQeen (1969-2010) był uzależniony od wielu substancji psychoaktywnych. Które cechy opisu jego zachowania z filmu biograficznego „Wizjoner. Buntownik. Geniusz” wskazują na ekspozycję na kokainę?</t></is></c><c r="F539" s="2" t="inlineStr"><is><t>gadatliwy, w świetnym nastroju, pełen energii i bardzo ruchliwy mimo 16 h pracy przed pokazem, ale spocony i z nawracającymi krwawieniami z nosa</t></is></c><c r="G539" s="2" t="inlineStr" /><c r="H539" s="2" t="inlineStr" /><c r="I539" s="2" t="inlineStr" /><c r="J539" s="2" t="inlineStr" /><c r="K539" s="2" t="inlineStr"><is><t>brawurowy i agresywny, z zaburzeniami mowy i równowagi ruchowej</t></is></c><c r="L539" s="2" t="inlineStr"><is><t>błyskotliwy, dowcipny, szybko przyswajający duże ilości nowych informacji, ale ciągle głodny i z okresowymi napadami paniki</t></is></c><c r="M539" s="2" t="inlineStr"><is><t>w euforii, komplementujący współpracowników, okresowo z barwnymi wizjami, okresowo podsypiający, z przekrwionymi twardówkami</t></is></c><c r="N539" s="2" t="inlineStr" /><c r="O539" s="2" t="inlineStr" /><c r="P539" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q539" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="540"><c r="A540" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B540" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C540" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D540" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E540" s="2" t="inlineStr"><is><t>Działanie farmakologiczne inne niż suplementacja w stanach niedoboru ma:</t></is></c><c r="F540" s="2" t="inlineStr"><is><t>fitomenadion w niewydolności wątroby i przedawkowaniu warfaryny</t></is></c><c r="G540" s="2" t="inlineStr"><is><t>cholekalcyferol w profilaktyce i leczeniu osteoporozy</t></is></c><c r="H540" s="2" t="inlineStr" /><c r="I540" s="2" t="inlineStr" /><c r="J540" s="2" t="inlineStr" /><c r="K540" s="2" t="inlineStr"><is><t>nikotynamid w hiperurykemii i atakach dny moczanowej</t></is></c><c r="L540" s="2" t="inlineStr"><is><t>tokoferol w profilatyce raka płuc</t></is></c><c r="M540" s="2" t="inlineStr" /><c r="N540" s="2" t="inlineStr" /><c r="O540" s="2" t="inlineStr" /><c r="P540" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q540" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="541"><c r="A541" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B541" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C541" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D541" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E541" s="2" t="inlineStr"><is><t>Obniżenie stężenia potasu w surowicy może być spowodowane zastosowaniem:</t></is></c><c r="F541" s="2" t="inlineStr"><is><t>bisakodylu</t></is></c><c r="G541" s="2" t="inlineStr"><is><t>prednizonu</t></is></c><c r="H541" s="2" t="inlineStr"><is><t>glukozy z insuliną</t></is></c><c r="I541" s="2" t="inlineStr" /><c r="J541" s="2" t="inlineStr" /><c r="K541" s="2" t="inlineStr"><is><t>glukonianu wapnia</t></is></c><c r="L541" s="2" t="inlineStr" /><c r="M541" s="2" t="inlineStr" /><c r="N541" s="2" t="inlineStr" /><c r="O541" s="2" t="inlineStr" /><c r="P541" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q541" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="542"><c r="A542" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B542" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C542" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D542" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E542" s="2" t="inlineStr"><is><t>Zasadzką płynoterapii jest:</t></is></c><c r="F542" s="2" t="inlineStr"><is><t>obrzęk płuc po nawadnianiu płynem wieloelektrolitowym</t></is></c><c r="G542" s="2" t="inlineStr"><is><t>brak możliwości wiarygodnego oznaczenia grupy krwi i wykonania próby krzyżowej po padaniu dekstranu 70 000</t></is></c><c r="H542" s="2" t="inlineStr"><is><t>hiperonkotyczna niewydolność nerek po podaniu hydroksyetylowanej skrobi 130/0,4</t></is></c><c r="I542" s="2" t="inlineStr" /><c r="J542" s="2" t="inlineStr" /><c r="K542" s="2" t="inlineStr"><is><t>zakrzepica podczas stosowania 20% roztworu albumin</t></is></c><c r="L542" s="2" t="inlineStr" /><c r="M542" s="2" t="inlineStr" /><c r="N542" s="2" t="inlineStr" /><c r="O542" s="2" t="inlineStr" /><c r="P542" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q542" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="543"><c r="A543" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B543" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C543" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D543" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E543" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenia:</t></is></c><c r="F543" s="2" t="inlineStr"><is><t>w USA obowiązuje nazewnictwo leków w pewnym zakresie autonomiczne od tworzonej przez WHO listy nazw międzynarodowych, przykłady paracetamol i acetaminofen czy petydyna i meperydyna</t></is></c><c r="G543" s="2" t="inlineStr" /><c r="H543" s="2" t="inlineStr" /><c r="I543" s="2" t="inlineStr" /><c r="J543" s="2" t="inlineStr" /><c r="K543" s="2" t="inlineStr"><is><t>po wygaśnięciu ochrony patentowej enoksaparyny wprowadzono jej odtwórcze odpowiedniki tylko na podstawie wykazania ich biorównoważności</t></is></c><c r="L543" s="2" t="inlineStr"><is><t>antysensowne oligonukleotydy mają w nazwie końcówkę -stim</t></is></c><c r="M543" s="2" t="inlineStr"><is><t>przy konwersji między lekami biopodobnymi obowiązuje zasada zamiany automatycznej (substytucji)</t></is></c><c r="N543" s="2" t="inlineStr" /><c r="O543" s="2" t="inlineStr" /><c r="P543" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q543" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="544"><c r="A544" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B544" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C544" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D544" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E544" s="2" t="inlineStr"><is><t>Wskaż prawidłowe zestawienia lek-spektrum działania:</t></is></c><c r="F544" s="2" t="inlineStr"><is><t>cyprofloksacyna – Pseudomonas aeruginosa, Mycoplasma pneumoniae</t></is></c><c r="G544" s="2" t="inlineStr"><is><t>penicylina G – Fusobacterium spp., Streptococcus pyogenes</t></is></c><c r="H544" s="2" t="inlineStr"><is><t>rifaksymina – Escherichia coli, Campylobacter jejuni</t></is></c><c r="I544" s="2" t="inlineStr" /><c r="J544" s="2" t="inlineStr" /><c r="K544" s="2" t="inlineStr"><is><t>gentamycyna – Clostridium spp., Helicobacter pylori</t></is></c><c r="L544" s="2" t="inlineStr" /><c r="M544" s="2" t="inlineStr" /><c r="N544" s="2" t="inlineStr" /><c r="O544" s="2" t="inlineStr" /><c r="P544" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q544" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="545"><c r="A545" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B545" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C545" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D545" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E545" s="2" t="inlineStr"><is><t>Wskaż zdania prawdziwe:</t></is></c><c r="F545" s="2" t="inlineStr"><is><t>zastosowanie technologii liposomów pozwoliło na otrzymanie preparatów amfoterycyny B o zmniejszonej nefrotoksyczności</t></is></c><c r="G545" s="2" t="inlineStr" /><c r="H545" s="2" t="inlineStr" /><c r="I545" s="2" t="inlineStr" /><c r="J545" s="2" t="inlineStr" /><c r="K545" s="2" t="inlineStr"><is><t>w przeciwieństwie do terbinafiny, azole hamują enzym szlaku biosyntezy ergosterolu niezwiązany z układem CYP450</t></is></c><c r="L545" s="2" t="inlineStr"><is><t>kaspofungina może być skuteczna w leczeniu i profilaktyce zapalenia opon mózgowo-rdzeniowych o etiologii Cryptococcus neoformans</t></is></c><c r="M545" s="2" t="inlineStr"><is><t>dla uzyskania możliwie najlepszych efektów leczenia amfoterycyną B najistotniejsze z punktu widzenia PK/PD jest, aby stężenie leku pomiędzy kolejnymi podaniami utrzymywało się na poziomie 4 x MIC optymalnie przez 100% czasu</t></is></c><c r="N545" s="2" t="inlineStr" /><c r="O545" s="2" t="inlineStr" /><c r="P545" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q545" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="546"><c r="A546" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B546" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C546" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D546" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E546" s="2" t="inlineStr"><is><t>Modyfikacja dawki nie jest wymagana u pacjenta z eGFR wg wzoru Cockcrofta- Gaulta = 24 ml/min podczas stosowania:</t></is></c><c r="F546" s="2" t="inlineStr"><is><t>ceftriaksonu</t></is></c><c r="G546" s="2" t="inlineStr"><is><t>cefoperazonu</t></is></c><c r="H546" s="2" t="inlineStr" /><c r="I546" s="2" t="inlineStr" /><c r="J546" s="2" t="inlineStr" /><c r="K546" s="2" t="inlineStr"><is><t>ceftazydymu</t></is></c><c r="L546" s="2" t="inlineStr"><is><t>cefepimu</t></is></c><c r="M546" s="2" t="inlineStr" /><c r="N546" s="2" t="inlineStr" /><c r="O546" s="2" t="inlineStr" /><c r="P546" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q546" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="547"><c r="A547" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B547" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C547" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D547" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E547" s="2" t="inlineStr"><is><t>Jaki lek można opisać w następujący sposób: ma działanie bójcze, jego celem farmakodynamicznym jest jak największy stosunek AUC24:MIC i łatwa jest jego sekwencja do stosowania doustnego:</t></is></c><c r="F547" s="2" t="inlineStr"><is><t>Lewofloksacyna</t></is></c><c r="G547" s="2" t="inlineStr" /><c r="H547" s="2" t="inlineStr" /><c r="I547" s="2" t="inlineStr" /><c r="J547" s="2" t="inlineStr" /><c r="K547" s="2" t="inlineStr"><is><t>Neomycyna</t></is></c><c r="L547" s="2" t="inlineStr"><is><t>Wankomycyna</t></is></c><c r="M547" s="2" t="inlineStr"><is><t>Klarytromycyna</t></is></c><c r="N547" s="2" t="inlineStr" /><c r="O547" s="2" t="inlineStr" /><c r="P547" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q547" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="548"><c r="A548" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B548" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C548" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D548" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E548" s="2" t="inlineStr"><is><t>Które stwierdzenie jest prawdziwe w leczeniu zakażeń?</t></is></c><c r="F548" s="2" t="inlineStr"><is><t>leki przeciwinfekcyjne są jedynie uzupełnieniem leczenia zabiegowego w postaci aspiracji lub drenażu w przypadku ropni i ropniaków</t></is></c><c r="G548" s="2" t="inlineStr"><is><t>leczenie zakażenia w obrębie tylnej komory oka (szklistki) wymaga podania leków przeciwinfekcyjnych doszklistkowo</t></is></c><c r="H548" s="2" t="inlineStr"><is><t>nie jest możliwe wyleczenia „zakażenia” sztucznych materiałów: protez, cewników, sztucznych zastawek</t></is></c><c r="I548" s="2" t="inlineStr"><is><t>w przewlekłym zapaleniu zatok konieczne jest chirurgiczna korekta nieprawidłowości anatomicznych, tj. polip czy, skrzywienie przegrody nosa</t></is></c><c r="J548" s="2" t="inlineStr" /><c r="K548" s="2" t="inlineStr" /><c r="L548" s="2" t="inlineStr" /><c r="M548" s="2" t="inlineStr" /><c r="N548" s="2" t="inlineStr" /><c r="O548" s="2" t="inlineStr" /><c r="P548" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q548" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="549"><c r="A549" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B549" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C549" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D549" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E549" s="2" t="inlineStr"><is><t>U pacjenta z podejrzeniem atypowego zakażenia układu oddechowego, stosującego na co dzień leki z grupy inhibitorów reduktazy HMG-CoA (pacjent nie pamięta nazwy leku), planujesz włączyć antybiotyk makrolidowy. Za bezpieczną opcję terapeutyczną w tej sytuacji uznasz:</t></is></c><c r="F549" s="2" t="inlineStr"><is><t>azytromycynę</t></is></c><c r="G549" s="2" t="inlineStr" /><c r="H549" s="2" t="inlineStr" /><c r="I549" s="2" t="inlineStr" /><c r="J549" s="2" t="inlineStr" /><c r="K549" s="2" t="inlineStr"><is><t>klarytromycynę</t></is></c><c r="L549" s="2" t="inlineStr"><is><t>telitromycynę</t></is></c><c r="M549" s="2" t="inlineStr"><is><t>erytromycynę</t></is></c><c r="N549" s="2" t="inlineStr" /><c r="O549" s="2" t="inlineStr" /><c r="P549" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q549" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="550"><c r="A550" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B550" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C550" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D550" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E550" s="2" t="inlineStr"><is><t>Wskaż prawidłowe zestawienia lek-działanie niepożądane:</t></is></c><c r="F550" s="2" t="inlineStr"><is><t>izoniazyd – toczeń polekowy</t></is></c><c r="G550" s="2" t="inlineStr"><is><t>pirazynamid– hiperurikemia</t></is></c><c r="H550" s="2" t="inlineStr"><is><t>ryfampicyna – małopłytkowość</t></is></c><c r="I550" s="2" t="inlineStr"><is><t>etambutol – pozagałkowe zapalenie nerwu wzrokowego</t></is></c><c r="J550" s="2" t="inlineStr" /><c r="K550" s="2" t="inlineStr" /><c r="L550" s="2" t="inlineStr" /><c r="M550" s="2" t="inlineStr" /><c r="N550" s="2" t="inlineStr" /><c r="O550" s="2" t="inlineStr" /><c r="P550" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q550" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="551"><c r="A551" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B551" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C551" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D551" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E551" s="2" t="inlineStr"><is><t>Leki przeciwbakteryjne o wysokim potencjale do selekcji szczepów Clostridium difficile to:</t></is></c><c r="F551" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="G551" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="H551" s="2" t="inlineStr" /><c r="I551" s="2" t="inlineStr" /><c r="J551" s="2" t="inlineStr" /><c r="K551" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="L551" s="2" t="inlineStr"><is><t>fidaksomycyna</t></is></c><c r="M551" s="2" t="inlineStr" /><c r="N551" s="2" t="inlineStr" /><c r="O551" s="2" t="inlineStr" /><c r="P551" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q551" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="552"><c r="A552" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B552" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C552" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D552" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E552" s="2" t="inlineStr"><is><t>Pacjent leczony jest dożylnie lekiem, którego farmakokinetyka opisana jest następująco: słabo wchłania się z przewodu pokarmowego, podlega ograniczonej dystrybucji do tkanek, nie jest metabolizowany (bądź jest metabolizowany w minimalnym stopniu), wydalany jest głównie przez nerki. Lekiem tym może być:</t></is></c><c r="F552" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="G552" s="2" t="inlineStr"><is><t>kolistymetat sodu</t></is></c><c r="H552" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="I552" s="2" t="inlineStr" /><c r="J552" s="2" t="inlineStr" /><c r="K552" s="2" t="inlineStr"><is><t>erytromycyna</t></is></c><c r="L552" s="2" t="inlineStr" /><c r="M552" s="2" t="inlineStr" /><c r="N552" s="2" t="inlineStr" /><c r="O552" s="2" t="inlineStr" /><c r="P552" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q552" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="553"><c r="A553" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B553" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C553" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D553" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E553" s="2" t="inlineStr"><is><t>W leczeniu inwazyjnej aspergilozy znalazły zastosowanie:</t></is></c><c r="F553" s="2" t="inlineStr"><is><t>amfoterycyna B podawana dożylnie</t></is></c><c r="G553" s="2" t="inlineStr"><is><t>worykonazol podawany dożylnie</t></is></c><c r="H553" s="2" t="inlineStr" /><c r="I553" s="2" t="inlineStr" /><c r="J553" s="2" t="inlineStr" /><c r="K553" s="2" t="inlineStr"><is><t>kaspofungina podawana doustnie</t></is></c><c r="L553" s="2" t="inlineStr"><is><t>terbinafina podawana doustnie</t></is></c><c r="M553" s="2" t="inlineStr" /><c r="N553" s="2" t="inlineStr" /><c r="O553" s="2" t="inlineStr" /><c r="P553" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q553" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="554"><c r="A554" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B554" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C554" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D554" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E554" s="2" t="inlineStr"><is><t>Dobrą dystrybucją do ośrodkowego układu nerwowego charakteryzuje się:</t></is></c><c r="F554" s="2" t="inlineStr"><is><t>ceftriakson</t></is></c><c r="G554" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="H554" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="I554" s="2" t="inlineStr" /><c r="J554" s="2" t="inlineStr" /><c r="K554" s="2" t="inlineStr"><is><t>kaspofungina</t></is></c><c r="L554" s="2" t="inlineStr" /><c r="M554" s="2" t="inlineStr" /><c r="N554" s="2" t="inlineStr" /><c r="O554" s="2" t="inlineStr" /><c r="P554" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q554" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="555"><c r="A555" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B555" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C555" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D555" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E555" s="2" t="inlineStr"><is><t>W schematach eradykacji Helicobacter pylori są stosowane:</t></is></c><c r="F555" s="2" t="inlineStr"><is><t>klarytromycyna</t></is></c><c r="G555" s="2" t="inlineStr"><is><t>Amoksycylina</t></is></c><c r="H555" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="I555" s="2" t="inlineStr"><is><t>tetracyklina</t></is></c><c r="J555" s="2" t="inlineStr" /><c r="K555" s="2" t="inlineStr" /><c r="L555" s="2" t="inlineStr" /><c r="M555" s="2" t="inlineStr" /><c r="N555" s="2" t="inlineStr" /><c r="O555" s="2" t="inlineStr" /><c r="P555" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q555" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="556"><c r="A556" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B556" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C556" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D556" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E556" s="2" t="inlineStr"><is><t>U kobiety w ciąży z rumieniem wędrującym można zastosować:</t></is></c><c r="F556" s="2" t="inlineStr"><is><t>azytromycynę</t></is></c><c r="G556" s="2" t="inlineStr"><is><t>amoksycylinę</t></is></c><c r="H556" s="2" t="inlineStr" /><c r="I556" s="2" t="inlineStr" /><c r="J556" s="2" t="inlineStr" /><c r="K556" s="2" t="inlineStr"><is><t>doksycyklinę</t></is></c><c r="L556" s="2" t="inlineStr"><is><t>klindamycynę</t></is></c><c r="M556" s="2" t="inlineStr" /><c r="N556" s="2" t="inlineStr" /><c r="O556" s="2" t="inlineStr" /><c r="P556" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q556" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="557"><c r="A557" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B557" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C557" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D557" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E557" s="2" t="inlineStr"><is><t>W zakażeniu o etiologii MRSA(methicyllin-resistant Staphylococcus aureus) zasadne jest zastosowanie:</t></is></c><c r="F557" s="2" t="inlineStr"><is><t>ceftaroliny</t></is></c><c r="G557" s="2" t="inlineStr"><is><t>linezolidu</t></is></c><c r="H557" s="2" t="inlineStr" /><c r="I557" s="2" t="inlineStr" /><c r="J557" s="2" t="inlineStr" /><c r="K557" s="2" t="inlineStr"><is><t>kloksacyliny</t></is></c><c r="L557" s="2" t="inlineStr"><is><t>meropenemu</t></is></c><c r="M557" s="2" t="inlineStr" /><c r="N557" s="2" t="inlineStr" /><c r="O557" s="2" t="inlineStr" /><c r="P557" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q557" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="558"><c r="A558" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B558" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C558" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D558" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E558" s="2" t="inlineStr"><is><t>W biegunce o etiologii Clostridium difficile uzasadnione może być podanie doustne:</t></is></c><c r="F558" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="G558" s="2" t="inlineStr"><is><t>metronidazolu</t></is></c><c r="H558" s="2" t="inlineStr"><is><t>fidaksomycyny</t></is></c><c r="I558" s="2" t="inlineStr" /><c r="J558" s="2" t="inlineStr" /><c r="K558" s="2" t="inlineStr"><is><t>nifuroksazydu</t></is></c><c r="L558" s="2" t="inlineStr" /><c r="M558" s="2" t="inlineStr" /><c r="N558" s="2" t="inlineStr" /><c r="O558" s="2" t="inlineStr" /><c r="P558" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q558" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="559"><c r="A559" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B559" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C559" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D559" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E559" s="2" t="inlineStr"><is><t>Wskaż właściwe skojarzenie lek – potencjalne działanie niepożądane:</t></is></c><c r="F559" s="2" t="inlineStr"><is><t>chloramfenikol – zespół szarego dziecka</t></is></c><c r="G559" s="2" t="inlineStr"><is><t>doksycyklina - fotodermatoza</t></is></c><c r="H559" s="2" t="inlineStr" /><c r="I559" s="2" t="inlineStr" /><c r="J559" s="2" t="inlineStr" /><c r="K559" s="2" t="inlineStr"><is><t>gentamycyna - żółtaczka cholestatyczna</t></is></c><c r="L559" s="2" t="inlineStr"><is><t>klindamycyna – zespół serotoninowy</t></is></c><c r="M559" s="2" t="inlineStr" /><c r="N559" s="2" t="inlineStr" /><c r="O559" s="2" t="inlineStr" /><c r="P559" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q559" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="560"><c r="A560" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B560" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C560" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D560" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E560" s="2" t="inlineStr"><is><t>Zaburzenia rytmu serca mogą wystąpić w trakcie stosowania:</t></is></c><c r="F560" s="2" t="inlineStr"><is><t>moksyfloksacyny</t></is></c><c r="G560" s="2" t="inlineStr"><is><t>klarytromycyny</t></is></c><c r="H560" s="2" t="inlineStr" /><c r="I560" s="2" t="inlineStr" /><c r="J560" s="2" t="inlineStr" /><c r="K560" s="2" t="inlineStr"><is><t>fidaksomycyny</t></is></c><c r="L560" s="2" t="inlineStr"><is><t>Mupirocyny</t></is></c><c r="M560" s="2" t="inlineStr" /><c r="N560" s="2" t="inlineStr" /><c r="O560" s="2" t="inlineStr" /><c r="P560" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q560" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="561"><c r="A561" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B561" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C561" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D561" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E561" s="2" t="inlineStr"><is><t>Kolistymetat sodu:</t></is></c><c r="F561" s="2" t="inlineStr"><is><t>jest prolekiem</t></is></c><c r="G561" s="2" t="inlineStr"><is><t>jest zarezerwowany do leczenia zakażeń szczepami wielolekoopornymi G(-)</t></is></c><c r="H561" s="2" t="inlineStr" /><c r="I561" s="2" t="inlineStr" /><c r="J561" s="2" t="inlineStr" /><c r="K561" s="2" t="inlineStr"><is><t>działa na VRE (Vancomycin-Resistant Enterococcus)</t></is></c><c r="L561" s="2" t="inlineStr"><is><t>dobrze wchłania się z przewodu pokarmowego</t></is></c><c r="M561" s="2" t="inlineStr" /><c r="N561" s="2" t="inlineStr" /><c r="O561" s="2" t="inlineStr" /><c r="P561" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q561" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="562"><c r="A562" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B562" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C562" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D562" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E562" s="2" t="inlineStr"><is><t>Tygecyklina:</t></is></c><c r="F562" s="2" t="inlineStr"><is><t>jest stosowana w wewnątrzbrzusznych zakażeniach szczepami wielolekoopornymi</t></is></c><c r="G562" s="2" t="inlineStr" /><c r="H562" s="2" t="inlineStr" /><c r="I562" s="2" t="inlineStr" /><c r="J562" s="2" t="inlineStr" /><c r="K562" s="2" t="inlineStr"><is><t>dobrze wchłania się z przewodu pokarmowego</t></is></c><c r="L562" s="2" t="inlineStr"><is><t>bardzo często jest przyczyną zapalenia ścięgna Achillesa</t></is></c><c r="M562" s="2" t="inlineStr"><is><t>działa na Pseudomonas aeruginosa</t></is></c><c r="N562" s="2" t="inlineStr" /><c r="O562" s="2" t="inlineStr" /><c r="P562" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q562" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="563"><c r="A563" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B563" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C563" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D563" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E563" s="2" t="inlineStr"><is><t>Daptomycyna może być skuteczna w zakażeniach szczepami:</t></is></c><c r="F563" s="2" t="inlineStr"><is><t>MRSA (methicyllin-resistant Staphylococcus aureus)</t></is></c><c r="G563" s="2" t="inlineStr"><is><t>MSSA (methicillin-sensitive Staphylococcus aureus)</t></is></c><c r="H563" s="2" t="inlineStr"><is><t>VRE (Vancomycin-Resistant Enterococcus)</t></is></c><c r="I563" s="2" t="inlineStr" /><c r="J563" s="2" t="inlineStr" /><c r="K563" s="2" t="inlineStr"><is><t>CPE (Carbapenemase-producing Enterobacteriaceae)</t></is></c><c r="L563" s="2" t="inlineStr" /><c r="M563" s="2" t="inlineStr" /><c r="N563" s="2" t="inlineStr" /><c r="O563" s="2" t="inlineStr" /><c r="P563" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q563" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="564"><c r="A564" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B564" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C564" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D564" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E564" s="2" t="inlineStr"><is><t>Lewofloksacyna:</t></is></c><c r="F564" s="2" t="inlineStr"><is><t>wykazuje aktywność wobec Streptococcus pneumoniae</t></is></c><c r="G564" s="2" t="inlineStr"><is><t>wykazuje aktywność wobec Legionella pneumophila</t></is></c><c r="H564" s="2" t="inlineStr" /><c r="I564" s="2" t="inlineStr" /><c r="J564" s="2" t="inlineStr" /><c r="K564" s="2" t="inlineStr"><is><t>ma taki sam zakres działania jak moksyfloksacyna</t></is></c><c r="L564" s="2" t="inlineStr"><is><t>nie działa na Pseudomonas aeruginosa</t></is></c><c r="M564" s="2" t="inlineStr" /><c r="N564" s="2" t="inlineStr" /><c r="O564" s="2" t="inlineStr" /><c r="P564" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q564" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="565"><c r="A565" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B565" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C565" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D565" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E565" s="2" t="inlineStr"><is><t>W przypadku rozpoznania anginy paciorkowcowej u osoby uczulonej na antybiotyki beta￾laktamowe, można zastosować:</t></is></c><c r="F565" s="2" t="inlineStr"><is><t>klindamycynę</t></is></c><c r="G565" s="2" t="inlineStr"><is><t>azytromycynę</t></is></c><c r="H565" s="2" t="inlineStr" /><c r="I565" s="2" t="inlineStr" /><c r="J565" s="2" t="inlineStr" /><c r="K565" s="2" t="inlineStr"><is><t>norfloksacynę</t></is></c><c r="L565" s="2" t="inlineStr"><is><t>kloksacylinę</t></is></c><c r="M565" s="2" t="inlineStr" /><c r="N565" s="2" t="inlineStr" /><c r="O565" s="2" t="inlineStr" /><c r="P565" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q565" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="566"><c r="A566" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B566" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C566" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D566" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E566" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie:</t></is></c><c r="F566" s="2" t="inlineStr"><is><t>owsica – pyrantel, WZW C (wirusowe zapalenie wątroby typu C) – daklataswir</t></is></c><c r="G566" s="2" t="inlineStr"><is><t>wszawica – permetryna, CMV – walgancyklowir</t></is></c><c r="H566" s="2" t="inlineStr" /><c r="I566" s="2" t="inlineStr" /><c r="J566" s="2" t="inlineStr" /><c r="K566" s="2" t="inlineStr"><is><t>CMV (cytomegalovirus) – acyklowir, owsica – pyrantel</t></is></c><c r="L566" s="2" t="inlineStr"><is><t>acyklowir – HSV-2 (herpes simplex 2), amantadyna – profilaktyka grypy typu B</t></is></c><c r="M566" s="2" t="inlineStr" /><c r="N566" s="2" t="inlineStr" /><c r="O566" s="2" t="inlineStr" /><c r="P566" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q566" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="567"><c r="A567" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B567" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C567" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D567" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E567" s="2" t="inlineStr"><is><t>Które pary leków mających ten sam zasadniczy mechanizm działania różnią się istotnie profilem działań klinicznych?</t></is></c><c r="F567" s="2" t="inlineStr"><is><t>werapamil i nitrendypina</t></is></c><c r="G567" s="2" t="inlineStr"><is><t>doksazosyna i tamsulozyna</t></is></c><c r="H567" s="2" t="inlineStr" /><c r="I567" s="2" t="inlineStr" /><c r="J567" s="2" t="inlineStr" /><c r="K567" s="2" t="inlineStr"><is><t>moksonidyna i rylmenidyna</t></is></c><c r="L567" s="2" t="inlineStr"><is><t>spironolakton i kanrenon</t></is></c><c r="M567" s="2" t="inlineStr" /><c r="N567" s="2" t="inlineStr" /><c r="O567" s="2" t="inlineStr" /><c r="P567" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q567" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="568"><c r="A568" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B568" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C568" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D568" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E568" s="2" t="inlineStr"><is><t>Do leków aktywujących pośrednio lub bezpośrednio cyklazę guanylową komórek mięśniówki gładkiej naczyń należy:</t></is></c><c r="F568" s="2" t="inlineStr"><is><t>nitroprusydek sodu</t></is></c><c r="G568" s="2" t="inlineStr"><is><t>riocyguat</t></is></c><c r="H568" s="2" t="inlineStr"><is><t>sakubitryl</t></is></c><c r="I568" s="2" t="inlineStr" /><c r="J568" s="2" t="inlineStr" /><c r="K568" s="2" t="inlineStr"><is><t>wardenafil</t></is></c><c r="L568" s="2" t="inlineStr" /><c r="M568" s="2" t="inlineStr" /><c r="N568" s="2" t="inlineStr" /><c r="O568" s="2" t="inlineStr" /><c r="P568" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q568" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="569"><c r="A569" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B569" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C569" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D569" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E569" s="2" t="inlineStr"><is><t>Czy zaproponowany wlew poszczególnych amin katecholowych jest adekwatny na początku leczenia (wybierz najmniejszą dawkę zalecaną) u pacjenta z przedstawionym rozpoznaniem?</t></is></c><c r="F569" s="2" t="inlineStr"><is><t>pacjent = 50 kg z ostrą niewydolnością serca i ciśnieniem skurczowym 85 mmHg – dopamina 200 mg/40 ml 0,9% NaCl → wlew = 3 ml/h</t></is></c><c r="G569" s="2" t="inlineStr"><is><t>pacjent = 100 kg we wstrząsie septycznym z ciśnieniem skurczowym 60 mmHg – noradrenalina 4 mg/40 ml 0,9% NaCl → wlew = 12 ml/h</t></is></c><c r="H569" s="2" t="inlineStr"><is><t>pacjent = 50 kg z zaostrzeniem przewlekłej niewydolności serca skurczowym 105 mmHg – dobutamina 250 mg/50 ml 0,9% NaCl → wlew =1,2 ml/h</t></is></c><c r="I569" s="2" t="inlineStr" /><c r="J569" s="2" t="inlineStr" /><c r="K569" s="2" t="inlineStr"><is><t>pacjent = 100 kg z ostrą niewydolnością serca i ciśnieniem skurczowym 80 mmHg – dobutamina 250 mg/50 ml 0,9% NaCl → wlew = 2,4 ml/h</t></is></c><c r="L569" s="2" t="inlineStr" /><c r="M569" s="2" t="inlineStr" /><c r="N569" s="2" t="inlineStr" /><c r="O569" s="2" t="inlineStr" /><c r="P569" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q569" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="570"><c r="A570" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B570" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C570" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D570" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E570" s="2" t="inlineStr"><is><t>Wskaż lek o bardzo krótkim okresie półtrwania (&lt;5 min), który z tego powodu wymaga stosowania we wlewie dożylnym lub jest wykorzystywany w celu osiągnięcia błyskawicznego krótkotrwałego efektu terapeutycznego:</t></is></c><c r="F570" s="2" t="inlineStr"><is><t>esmolol</t></is></c><c r="G570" s="2" t="inlineStr"><is><t>sukcynylocholina</t></is></c><c r="H570" s="2" t="inlineStr"><is><t>adenozyna</t></is></c><c r="I570" s="2" t="inlineStr" /><c r="J570" s="2" t="inlineStr" /><c r="K570" s="2" t="inlineStr"><is><t>diazepam</t></is></c><c r="L570" s="2" t="inlineStr" /><c r="M570" s="2" t="inlineStr" /><c r="N570" s="2" t="inlineStr" /><c r="O570" s="2" t="inlineStr" /><c r="P570" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q570" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="571"><c r="A571" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B571" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C571" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D571" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E571" s="2" t="inlineStr"><is><t>Wskaż poprawną kombinację terapeutyczną w leczeniu zapalnego kaszlu w infekcji oskrzeli:</t></is></c><c r="F571" s="2" t="inlineStr"><is><t>ambroksol w nebulizacji + acetylocysteina doustnie</t></is></c><c r="G571" s="2" t="inlineStr" /><c r="H571" s="2" t="inlineStr" /><c r="I571" s="2" t="inlineStr" /><c r="J571" s="2" t="inlineStr" /><c r="K571" s="2" t="inlineStr"><is><t>wazycyna doustnie + 10% NaCl w nebulizacji</t></is></c><c r="L571" s="2" t="inlineStr"><is><t>sulfagwajakol + kodeina w doustnym preparacie złożonym</t></is></c><c r="M571" s="2" t="inlineStr"><is><t>dornaza alfa w inhalacjach + erdosteina doustnie</t></is></c><c r="N571" s="2" t="inlineStr" /><c r="O571" s="2" t="inlineStr" /><c r="P571" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q571" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="572"><c r="A572" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B572" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C572" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D572" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E572" s="2" t="inlineStr"><is><t>W napadzie duszności u osoby z cechami skurczu oskrzeli (cichy szmer pęcherzykowy, głośne świsty, wydłużona faza wydechu) w celu przerwania napadu zasadne jest zastosowanie:</t></is></c><c r="F572" s="2" t="inlineStr"><is><t>salbutamolu wziewnie w nebulizacji</t></is></c><c r="G572" s="2" t="inlineStr"><is><t>bromku ipratropium wziewnie w nebulizacji</t></is></c><c r="H572" s="2" t="inlineStr" /><c r="I572" s="2" t="inlineStr" /><c r="J572" s="2" t="inlineStr" /><c r="K572" s="2" t="inlineStr"><is><t>triazotanu glicerolu w aerozolu na błonę śluzową jamy ustnej</t></is></c><c r="L572" s="2" t="inlineStr"><is><t>cyklezonidu wziewnie z inhalatora aerozolowego</t></is></c><c r="M572" s="2" t="inlineStr" /><c r="N572" s="2" t="inlineStr" /><c r="O572" s="2" t="inlineStr" /><c r="P572" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q572" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="573"><c r="A573" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B573" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C573" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D573" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E573" s="2" t="inlineStr"><is><t>Który lek ma w swojej grupie farmakologicznej nietypową, wyróżniającą go farmakokinetykę:</t></is></c><c r="F573" s="2" t="inlineStr"><is><t>cyklezonid</t></is></c><c r="G573" s="2" t="inlineStr"><is><t>amlodypina</t></is></c><c r="H573" s="2" t="inlineStr" /><c r="I573" s="2" t="inlineStr" /><c r="J573" s="2" t="inlineStr" /><c r="K573" s="2" t="inlineStr"><is><t>metoprolol</t></is></c><c r="L573" s="2" t="inlineStr"><is><t>iwabradyna</t></is></c><c r="M573" s="2" t="inlineStr" /><c r="N573" s="2" t="inlineStr" /><c r="O573" s="2" t="inlineStr" /><c r="P573" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q573" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="574"><c r="A574" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B574" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C574" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D574" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E574" s="2" t="inlineStr"><is><t>Lekiem stosowanym „ratunkowo” w poważnych powikłaniach polekowych jest:</t></is></c><c r="F574" s="2" t="inlineStr"><is><t>adrenalina</t></is></c><c r="G574" s="2" t="inlineStr"><is><t>półbursztynian hydrokortyzonu</t></is></c><c r="H574" s="2" t="inlineStr"><is><t>dantrolen</t></is></c><c r="I574" s="2" t="inlineStr"><is><t>acetylocysteina</t></is></c><c r="J574" s="2" t="inlineStr" /><c r="K574" s="2" t="inlineStr" /><c r="L574" s="2" t="inlineStr" /><c r="M574" s="2" t="inlineStr" /><c r="N574" s="2" t="inlineStr" /><c r="O574" s="2" t="inlineStr" /><c r="P574" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q574" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="575"><c r="A575" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B575" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C575" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D575" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E575" s="2" t="inlineStr"><is><t>Do leków zmniejszających obciążenie wstępne należy:</t></is></c><c r="F575" s="2" t="inlineStr"><is><t>diazotan izosorbidu</t></is></c><c r="G575" s="2" t="inlineStr"><is><t>furosemid</t></is></c><c r="H575" s="2" t="inlineStr" /><c r="I575" s="2" t="inlineStr" /><c r="J575" s="2" t="inlineStr" /><c r="K575" s="2" t="inlineStr"><is><t>diosmina</t></is></c><c r="L575" s="2" t="inlineStr"><is><t>pentoksyfilina</t></is></c><c r="M575" s="2" t="inlineStr" /><c r="N575" s="2" t="inlineStr" /><c r="O575" s="2" t="inlineStr" /><c r="P575" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q575" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="576"><c r="A576" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B576" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C576" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D576" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E576" s="2" t="inlineStr"><is><t>Pacjentka z zespołem depresyjnym stosująca tryptany ma zwiększone ryzyko zespołu serotoninowego po włączeniu:</t></is></c><c r="F576" s="2" t="inlineStr"><is><t>fluoksetyny</t></is></c><c r="G576" s="2" t="inlineStr"><is><t>wenlafaksyny</t></is></c><c r="H576" s="2" t="inlineStr"><is><t>klomipraminy</t></is></c><c r="I576" s="2" t="inlineStr"><is><t>duloksetyny</t></is></c><c r="J576" s="2" t="inlineStr" /><c r="K576" s="2" t="inlineStr" /><c r="L576" s="2" t="inlineStr" /><c r="M576" s="2" t="inlineStr" /><c r="N576" s="2" t="inlineStr" /><c r="O576" s="2" t="inlineStr" /><c r="P576" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q576" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="577"><c r="A577" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B577" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C577" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D577" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E577" s="2" t="inlineStr"><is><t>Jeśli splątany i agresywny pacjent odmawia przyjmowania leków doustnie to po zastosowaniu krótkotrwałego unieruchomienia kończyn można mu podać dożylnie lek uspokajający, którym jest:</t></is></c><c r="F577" s="2" t="inlineStr"><is><t>midazolam</t></is></c><c r="G577" s="2" t="inlineStr" /><c r="H577" s="2" t="inlineStr" /><c r="I577" s="2" t="inlineStr" /><c r="J577" s="2" t="inlineStr" /><c r="K577" s="2" t="inlineStr"><is><t>piracetam</t></is></c><c r="L577" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="M577" s="2" t="inlineStr"><is><t>rysperydon</t></is></c><c r="N577" s="2" t="inlineStr" /><c r="O577" s="2" t="inlineStr" /><c r="P577" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q577" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="578"><c r="A578" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B578" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C578" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D578" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E578" s="2" t="inlineStr"><is><t>Jako lek normotymiczny w chorobie afektywnej dwubiegunowej można zastosować:</t></is></c><c r="F578" s="2" t="inlineStr"><is><t>lamotryginę</t></is></c><c r="G578" s="2" t="inlineStr"><is><t>olanzapinę</t></is></c><c r="H578" s="2" t="inlineStr" /><c r="I578" s="2" t="inlineStr" /><c r="J578" s="2" t="inlineStr" /><c r="K578" s="2" t="inlineStr"><is><t>fluoksetynę</t></is></c><c r="L578" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="M578" s="2" t="inlineStr" /><c r="N578" s="2" t="inlineStr" /><c r="O578" s="2" t="inlineStr" /><c r="P578" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q578" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="579"><c r="A579" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B579" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C579" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D579" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E579" s="2" t="inlineStr"><is><t>Który lek jest stosowany jedynie we wskazaniu wymienionym przy tym leku?</t></is></c><c r="F579" s="2" t="inlineStr"><is><t>netupitant – terapia wspomagająca stosowanie wysoce emetogennej chemioterapii przeciwnowotworowej</t></is></c><c r="G579" s="2" t="inlineStr"><is><t>memantyna – choroba Alzheimera</t></is></c><c r="H579" s="2" t="inlineStr" /><c r="I579" s="2" t="inlineStr" /><c r="J579" s="2" t="inlineStr" /><c r="K579" s="2" t="inlineStr"><is><t>karbamazepina – padaczka</t></is></c><c r="L579" s="2" t="inlineStr"><is><t>pregabalina – polineuropatia cukrzycowa</t></is></c><c r="M579" s="2" t="inlineStr" /><c r="N579" s="2" t="inlineStr" /><c r="O579" s="2" t="inlineStr" /><c r="P579" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q579" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="580"><c r="A580" s="2" t="inlineStr"><is><t>ZNIECZULENIA OGÓLNE</t></is></c><c r="B580" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C580" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D580" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E580" s="2" t="inlineStr"><is><t>Idealny lek znieczulenia ogólnego:</t></is></c><c r="F580" s="2" t="inlineStr"><is><t>jest skuteczny we wszystkich grupach pacjentów</t></is></c><c r="G580" s="2" t="inlineStr"><is><t>działa przeciwbólowo</t></is></c><c r="H580" s="2" t="inlineStr"><is><t>jest bezpieczny dla wszystkich grup pacjentów</t></is></c><c r="I580" s="2" t="inlineStr"><is><t>jest tani</t></is></c><c r="J580" s="2" t="inlineStr" /><c r="K580" s="2" t="inlineStr" /><c r="L580" s="2" t="inlineStr" /><c r="M580" s="2" t="inlineStr" /><c r="N580" s="2" t="inlineStr" /><c r="O580" s="2" t="inlineStr" /><c r="P580" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q580" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="581"><c r="A581" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B581" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C581" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D581" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E581" s="2" t="inlineStr"><is><t>Cholinolityki:</t></is></c><c r="F581" s="2" t="inlineStr"><is><t>są lekami z wyboru w polekowym zespole parkinsonowskim</t></is></c><c r="G581" s="2" t="inlineStr"><is><t>zmniejszają drżenie w chorobie Parkinsona</t></is></c><c r="H581" s="2" t="inlineStr"><is><t>nie różnią się skutecznością w chorobie Parkinsona</t></is></c><c r="I581" s="2" t="inlineStr"><is><t>można podawać w połączeniu z lewodopą</t></is></c><c r="J581" s="2" t="inlineStr" /><c r="K581" s="2" t="inlineStr" /><c r="L581" s="2" t="inlineStr" /><c r="M581" s="2" t="inlineStr" /><c r="N581" s="2" t="inlineStr" /><c r="O581" s="2" t="inlineStr" /><c r="P581" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q581" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="582"><c r="A582" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B582" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C582" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D582" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E582" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie mykotoksyny z zagrożeniem poekspozycyjnym:</t></is></c><c r="F582" s="2" t="inlineStr"><is><t>zearaleon – działanie estrogenne i anaboliczne</t></is></c><c r="G582" s="2" t="inlineStr"><is><t>aflatoksyna – ryzyko nowotworów wątroby</t></is></c><c r="H582" s="2" t="inlineStr" /><c r="I582" s="2" t="inlineStr" /><c r="J582" s="2" t="inlineStr" /><c r="K582" s="2" t="inlineStr"><is><t>patulina – ryzyko nowotworów dróg moczowych</t></is></c><c r="L582" s="2" t="inlineStr"><is><t>ochratoksyna – silne działanie alergizujące</t></is></c><c r="M582" s="2" t="inlineStr" /><c r="N582" s="2" t="inlineStr" /><c r="O582" s="2" t="inlineStr" /><c r="P582" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q582" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="583"><c r="A583" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B583" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C583" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D583" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E583" s="2" t="inlineStr"><is><t>Leki przeciwhistaminowe drugiej generacji blokujące receptor H1 w odróżnieniu od leków pierwszej generacji:</t></is></c><c r="F583" s="2" t="inlineStr"><is><t>są w znaczącym stopniu pozbawione działania sedatywnego</t></is></c><c r="G583" s="2" t="inlineStr" /><c r="H583" s="2" t="inlineStr" /><c r="I583" s="2" t="inlineStr" /><c r="J583" s="2" t="inlineStr" /><c r="K583" s="2" t="inlineStr"><is><t>mają istotne działanie cholinolityczne</t></is></c><c r="L583" s="2" t="inlineStr"><is><t>mogą być stosowane w postaci wstrzyknięć</t></is></c><c r="M583" s="2" t="inlineStr"><is><t>są skuteczne w profilaktyce choroby lokomocyjnej</t></is></c><c r="N583" s="2" t="inlineStr" /><c r="O583" s="2" t="inlineStr" /><c r="P583" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q583" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="584"><c r="A584" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B584" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C584" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D584" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E584" s="2" t="inlineStr"><is><t>W leczeniu ostrego napadu dny moczanowej stosuje się:</t></is></c><c r="F584" s="2" t="inlineStr"><is><t>kolchicynę</t></is></c><c r="G584" s="2" t="inlineStr"><is><t>glikokortykosteroidy</t></is></c><c r="H584" s="2" t="inlineStr"><is><t>niesteroidowe leki przeciwzapalne</t></is></c><c r="I584" s="2" t="inlineStr" /><c r="J584" s="2" t="inlineStr" /><c r="K584" s="2" t="inlineStr"><is><t>allopurynol</t></is></c><c r="L584" s="2" t="inlineStr" /><c r="M584" s="2" t="inlineStr" /><c r="N584" s="2" t="inlineStr" /><c r="O584" s="2" t="inlineStr" /><c r="P584" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q584" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="585"><c r="A585" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B585" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C585" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D585" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E585" s="2" t="inlineStr"><is><t>Diuretyki pętlowe:</t></is></c><c r="F585" s="2" t="inlineStr"><is><t>zwiększają filtrację kłębuszkową też przez korzystny wpływ na syntezę prostaglandyn w nerkach</t></is></c><c r="G585" s="2" t="inlineStr"><is><t>ulegają wydzielaniu cewkowemu w kanalikach proksymalnych</t></is></c><c r="H585" s="2" t="inlineStr"><is><t>tworzą wysoki ładunek sodowy w kanaliku dalszym aktywując układ reninowo￾angiotensynowy</t></is></c><c r="I585" s="2" t="inlineStr"><is><t>zwiększają pojemność łożyska żylnego jeszcze przed wystąpieniem efektu diuretycznego</t></is></c><c r="J585" s="2" t="inlineStr" /><c r="K585" s="2" t="inlineStr" /><c r="L585" s="2" t="inlineStr" /><c r="M585" s="2" t="inlineStr" /><c r="N585" s="2" t="inlineStr" /><c r="O585" s="2" t="inlineStr" /><c r="P585" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q585" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="586"><c r="A586" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B586" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C586" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D586" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E586" s="2" t="inlineStr"><is><t>Który lek może być zastosowany u chorego z nadwrażliwością na sulfonamidy?</t></is></c><c r="F586" s="2" t="inlineStr"><is><t>torasemid</t></is></c><c r="G586" s="2" t="inlineStr"><is><t>eplerenon</t></is></c><c r="H586" s="2" t="inlineStr" /><c r="I586" s="2" t="inlineStr" /><c r="J586" s="2" t="inlineStr" /><c r="K586" s="2" t="inlineStr"><is><t>furosemid</t></is></c><c r="L586" s="2" t="inlineStr"><is><t>hydrochlorotiazyd</t></is></c><c r="M586" s="2" t="inlineStr" /><c r="N586" s="2" t="inlineStr" /><c r="O586" s="2" t="inlineStr" /><c r="P586" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q586" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="587"><c r="A587" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B587" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C587" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D587" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E587" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące metoprololu:</t></is></c><c r="F587" s="2" t="inlineStr"><is><t>ma działanie hipotensyjne związane ze zmniejszeniem aktywności reninowej osocza</t></is></c><c r="G587" s="2" t="inlineStr"><is><t>zmienia działanie układu współczulnego na poziomie ośrodkowego układu nerwowego</t></is></c><c r="H587" s="2" t="inlineStr"><is><t>jest niebezpieczny w naczynioskurczowych chorobach tętnic</t></is></c><c r="I587" s="2" t="inlineStr" /><c r="J587" s="2" t="inlineStr" /><c r="K587" s="2" t="inlineStr"><is><t>w terapii przewlekłej powoduje down-regulację receptorów beta-adrenergicznych</t></is></c><c r="L587" s="2" t="inlineStr" /><c r="M587" s="2" t="inlineStr" /><c r="N587" s="2" t="inlineStr" /><c r="O587" s="2" t="inlineStr" /><c r="P587" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q587" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="588"><c r="A588" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B588" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C588" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D588" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E588" s="2" t="inlineStr"><is><t>W filmie „Piękny umysł” Alicia, żona chorego na schizofrenię Johna Nasha, pyta go: „Czy to przez lek?”, a on odpowiada: „Tak”. O którym działaniu niepożądanym chloropromazyny mogli rozmawiać?</t></is></c><c r="F588" s="2" t="inlineStr"><is><t>zmniejszeniu libido</t></is></c><c r="G588" s="2" t="inlineStr" /><c r="H588" s="2" t="inlineStr" /><c r="I588" s="2" t="inlineStr" /><c r="J588" s="2" t="inlineStr" /><c r="K588" s="2" t="inlineStr"><is><t>nadciśnieniu tętniczym</t></is></c><c r="L588" s="2" t="inlineStr"><is><t>ślinotoku</t></is></c><c r="M588" s="2" t="inlineStr"><is><t>przymusie robienia notatek na ścianach</t></is></c><c r="N588" s="2" t="inlineStr" /><c r="O588" s="2" t="inlineStr" /><c r="P588" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q588" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="589"><c r="A589" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B589" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C589" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D589" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E589" s="2" t="inlineStr"><is><t>W arcydziele „Sto lat samotności” Gabriela Garcii Marqueza wioskę Macondo nawiedza zaraza bezsenności i zapomnienia. Wskaż uzasadnioną opcję terapeutyczną do zaproponowania w leczeniu krótkotrwałej bezsenności, gdyby wydarzenia opisane przez Marqueza działy się współcześnie:</t></is></c><c r="F589" s="2" t="inlineStr"><is><t>trazodon</t></is></c><c r="G589" s="2" t="inlineStr" /><c r="H589" s="2" t="inlineStr" /><c r="I589" s="2" t="inlineStr" /><c r="J589" s="2" t="inlineStr" /><c r="K589" s="2" t="inlineStr"><is><t>triazolam</t></is></c><c r="L589" s="2" t="inlineStr"><is><t>dezimipramina</t></is></c><c r="M589" s="2" t="inlineStr"><is><t>hydroksyzyna</t></is></c><c r="N589" s="2" t="inlineStr" /><c r="O589" s="2" t="inlineStr" /><c r="P589" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q589" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="590"><c r="A590" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B590" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C590" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D590" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E590" s="2" t="inlineStr"><is><t>Amitryptylina w przeciwieństwie do wenlafaksyny:</t></is></c><c r="F590" s="2" t="inlineStr"><is><t>działa antagonistycznie wobec receptora muskarynowego (M1)</t></is></c><c r="G590" s="2" t="inlineStr" /><c r="H590" s="2" t="inlineStr" /><c r="I590" s="2" t="inlineStr" /><c r="J590" s="2" t="inlineStr" /><c r="K590" s="2" t="inlineStr"><is><t>jest skuteczna w bólach neuropatycznych</t></is></c><c r="L590" s="2" t="inlineStr"><is><t>zmniejsza wychwyt zwrotny noradrenaliny i serotoniny</t></is></c><c r="M590" s="2" t="inlineStr"><is><t>jest agonistą receptora dopaminowego (D2)</t></is></c><c r="N590" s="2" t="inlineStr" /><c r="O590" s="2" t="inlineStr" /><c r="P590" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q590" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="591"><c r="A591" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B591" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C591" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D591" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E591" s="2" t="inlineStr"><is><t>Za reakcję paradoksalną uznasz:</t></is></c><c r="F591" s="2" t="inlineStr"><is><t>agresję po lorazepamie</t></is></c><c r="G591" s="2" t="inlineStr" /><c r="H591" s="2" t="inlineStr" /><c r="I591" s="2" t="inlineStr" /><c r="J591" s="2" t="inlineStr" /><c r="K591" s="2" t="inlineStr"><is><t>drgawki po amitryptylinie</t></is></c><c r="L591" s="2" t="inlineStr"><is><t>niepamięć następczą po zopiklonie</t></is></c><c r="M591" s="2" t="inlineStr"><is><t>jadłowstręt po fluoksetynie</t></is></c><c r="N591" s="2" t="inlineStr" /><c r="O591" s="2" t="inlineStr" /><c r="P591" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q591" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="592"><c r="A592" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B592" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C592" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D592" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E592" s="2" t="inlineStr"><is><t>Który lek ma zastosowanie w wymiotach związanych z chemioterapią przeciwnowotworową?</t></is></c><c r="F592" s="2" t="inlineStr"><is><t>deksametazon</t></is></c><c r="G592" s="2" t="inlineStr"><is><t>palonosetron</t></is></c><c r="H592" s="2" t="inlineStr"><is><t>aprepitant</t></is></c><c r="I592" s="2" t="inlineStr"><is><t>metoklopramid</t></is></c><c r="J592" s="2" t="inlineStr" /><c r="K592" s="2" t="inlineStr" /><c r="L592" s="2" t="inlineStr" /><c r="M592" s="2" t="inlineStr" /><c r="N592" s="2" t="inlineStr" /><c r="O592" s="2" t="inlineStr" /><c r="P592" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q592" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="593"><c r="A593" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B593" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C593" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D593" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E593" s="2" t="inlineStr"><is><t>Pacjentka od wielu lat otrzymuje perazynę, mianserynę i lorazepam. Na tej podstawie można rozpoznać (możliwe jest więcej niż jedno rozpoznanie):</t></is></c><c r="F593" s="2" t="inlineStr"><is><t>zaburzenia depresyjno-urojeniowe</t></is></c><c r="G593" s="2" t="inlineStr"><is><t>uzależnienie lekowe</t></is></c><c r="H593" s="2" t="inlineStr" /><c r="I593" s="2" t="inlineStr" /><c r="J593" s="2" t="inlineStr" /><c r="K593" s="2" t="inlineStr"><is><t>dwubiegunową chorobę afektywną</t></is></c><c r="L593" s="2" t="inlineStr"><is><t>fobię społeczną</t></is></c><c r="M593" s="2" t="inlineStr" /><c r="N593" s="2" t="inlineStr" /><c r="O593" s="2" t="inlineStr" /><c r="P593" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q593" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="594"><c r="A594" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B594" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C594" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D594" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E594" s="2" t="inlineStr"><is><t>Podczas stosowania kwetiapiny, bardzo popularnej w psychotycznych zaburzeniach zachowania u pacjentów oddziałów somatycznych, trzeba pamiętać, że zwiększa się ryzyko:</t></is></c><c r="F594" s="2" t="inlineStr"><is><t>hipertriglicerydemii</t></is></c><c r="G594" s="2" t="inlineStr"><is><t>zespołu pozapiramidowego</t></is></c><c r="H594" s="2" t="inlineStr"><is><t>hiperglikemii</t></is></c><c r="I594" s="2" t="inlineStr"><is><t>zakrzepowego zapalenia żył</t></is></c><c r="J594" s="2" t="inlineStr" /><c r="K594" s="2" t="inlineStr" /><c r="L594" s="2" t="inlineStr" /><c r="M594" s="2" t="inlineStr" /><c r="N594" s="2" t="inlineStr" /><c r="O594" s="2" t="inlineStr" /><c r="P594" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q594" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="595"><c r="A595" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B595" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C595" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D595" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E595" s="2" t="inlineStr"><is><t>Która z poniższych informacji znajduje się w charakterystyce produktu leczniczego:</t></is></c><c r="F595" s="2" t="inlineStr"><is><t>informacja o warunkach przechowywania produktu leczniczego</t></is></c><c r="G595" s="2" t="inlineStr"><is><t>data wydania pierwszego pozwolenia na dopuszczenie do obrotu produktu leczniczego</t></is></c><c r="H595" s="2" t="inlineStr" /><c r="I595" s="2" t="inlineStr" /><c r="J595" s="2" t="inlineStr" /><c r="K595" s="2" t="inlineStr"><is><t>cena produktu leczniczego</t></is></c><c r="L595" s="2" t="inlineStr"><is><t>informacja o okresowym wstrzymaniu produktu leczniczego w obrocie</t></is></c><c r="M595" s="2" t="inlineStr" /><c r="N595" s="2" t="inlineStr" /><c r="O595" s="2" t="inlineStr" /><c r="P595" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q595" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="596"><c r="A596" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B596" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C596" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D596" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E596" s="2" t="inlineStr"><is><t>Do określenia biodostępności leku po podaniu doustnym konieczna jest znajomość:</t></is></c><c r="F596" s="2" t="inlineStr"><is><t>AUC0→t po podaniu dożylnym</t></is></c><c r="G596" s="2" t="inlineStr"><is><t>AUC0→t po podaniu doustnym</t></is></c><c r="H596" s="2" t="inlineStr" /><c r="I596" s="2" t="inlineStr" /><c r="J596" s="2" t="inlineStr" /><c r="K596" s="2" t="inlineStr"><is><t>stopnia wchłaniania ksylozy z przewodu pokarmowego</t></is></c><c r="L596" s="2" t="inlineStr"><is><t>Cmax leku po podaniu dożylnym</t></is></c><c r="M596" s="2" t="inlineStr" /><c r="N596" s="2" t="inlineStr" /><c r="O596" s="2" t="inlineStr" /><c r="P596" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q596" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="597"><c r="A597" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B597" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C597" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D597" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E597" s="2" t="inlineStr"><is><t>W stanie stacjonarnym objętość dystrybucji leku A = 6 l, a leku B = 206 l. Na podstawie tych danych można stwierdzić, że w stanie stacjonarnym lek A:</t></is></c><c r="F597" s="2" t="inlineStr"><is><t>osiąga większe stężenie we krwi niż lek B po podaniu takiej samej dawki obu leków i.v</t></is></c><c r="G597" s="2" t="inlineStr"><is><t>jest rozmieszczony nierównomiernie w przestrzeniach płynowych organizmu</t></is></c><c r="H597" s="2" t="inlineStr" /><c r="I597" s="2" t="inlineStr" /><c r="J597" s="2" t="inlineStr" /><c r="K597" s="2" t="inlineStr"><is><t>działa w kompartmencie obwodowym</t></is></c><c r="L597" s="2" t="inlineStr"><is><t>jest eliminowany zgodnie z kinetyką 0 rzędu</t></is></c><c r="M597" s="2" t="inlineStr" /><c r="N597" s="2" t="inlineStr" /><c r="O597" s="2" t="inlineStr" /><c r="P597" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q597" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="598"><c r="A598" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B598" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C598" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D598" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E598" s="2" t="inlineStr"><is><t>Która z poniższych par lek-zagrażające życiu działanie niepożądane jest prawdziwa?</t></is></c><c r="F598" s="2" t="inlineStr"><is><t>glargina – hipoglikemia</t></is></c><c r="G598" s="2" t="inlineStr" /><c r="H598" s="2" t="inlineStr" /><c r="I598" s="2" t="inlineStr" /><c r="J598" s="2" t="inlineStr" /><c r="K598" s="2" t="inlineStr"><is><t>metformina - zapalenie trzustki</t></is></c><c r="L598" s="2" t="inlineStr"><is><t>liraglutyd – kwasica ketonowa</t></is></c><c r="M598" s="2" t="inlineStr"><is><t>empagliflozyna – niewydolność serca</t></is></c><c r="N598" s="2" t="inlineStr" /><c r="O598" s="2" t="inlineStr" /><c r="P598" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q598" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="599"><c r="A599" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B599" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C599" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D599" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E599" s="2" t="inlineStr"><is><t>W celu obniżenia glikemii przed posiłkiem można podać:</t></is></c><c r="F599" s="2" t="inlineStr"><is><t>glulizynę</t></is></c><c r="G599" s="2" t="inlineStr" /><c r="H599" s="2" t="inlineStr" /><c r="I599" s="2" t="inlineStr" /><c r="J599" s="2" t="inlineStr" /><c r="K599" s="2" t="inlineStr"><is><t>degludec</t></is></c><c r="L599" s="2" t="inlineStr"><is><t>detemir</t></is></c><c r="M599" s="2" t="inlineStr"><is><t>glarginę</t></is></c><c r="N599" s="2" t="inlineStr" /><c r="O599" s="2" t="inlineStr" /><c r="P599" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q599" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="600"><c r="A600" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B600" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C600" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D600" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E600" s="2" t="inlineStr"><is><t>W leczeniu hiperprolaktynemii (prolaktynoma to najczęstszy typ gruczolaka przysadki) uzasadnione jest zastosowanie:</t></is></c><c r="F600" s="2" t="inlineStr"><is><t>bromokryptyny</t></is></c><c r="G600" s="2" t="inlineStr" /><c r="H600" s="2" t="inlineStr" /><c r="I600" s="2" t="inlineStr" /><c r="J600" s="2" t="inlineStr" /><c r="K600" s="2" t="inlineStr"><is><t>ketokonazolu</t></is></c><c r="L600" s="2" t="inlineStr"><is><t>eplerenonu</t></is></c><c r="M600" s="2" t="inlineStr"><is><t>klomifenu</t></is></c><c r="N600" s="2" t="inlineStr" /><c r="O600" s="2" t="inlineStr" /><c r="P600" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q600" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="601"><c r="A601" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B601" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C601" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D601" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E601" s="2" t="inlineStr"><is><t>Odtwórczy (generyczny) produkt leczniczy to produkt leczniczy :</t></is></c><c r="F601" s="2" t="inlineStr"><is><t>zawierający tę samą substancję aktywną co produkt oryginalny (innowacyjny)</t></is></c><c r="G601" s="2" t="inlineStr"><is><t>biorównoważny z produktem oryginalnym (innowacyjnym)</t></is></c><c r="H601" s="2" t="inlineStr" /><c r="I601" s="2" t="inlineStr" /><c r="J601" s="2" t="inlineStr" /><c r="K601" s="2" t="inlineStr"><is><t>mający ten sam skład co produkt oryginalny (innowacyjny)</t></is></c><c r="L601" s="2" t="inlineStr"><is><t>zarejestrowany także w innych wskazaniach niż produkt oryginalny (innowacyjny)</t></is></c><c r="M601" s="2" t="inlineStr" /><c r="N601" s="2" t="inlineStr" /><c r="O601" s="2" t="inlineStr" /><c r="P601" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q601" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="602"><c r="A602" s="2" t="inlineStr"><is><t>ANTYKONCEPCJA</t></is></c><c r="B602" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C602" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D602" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E602" s="2" t="inlineStr"><is><t>„Lekiem” o nieudokumentowanej skuteczności (de facto bezwartościowym) jest:</t></is></c><c r="F602" s="2" t="inlineStr"><is><t>beta-glukan</t></is></c><c r="G602" s="2" t="inlineStr" /><c r="H602" s="2" t="inlineStr" /><c r="I602" s="2" t="inlineStr" /><c r="J602" s="2" t="inlineStr" /><c r="K602" s="2" t="inlineStr"><is><t>drospirenon</t></is></c><c r="L602" s="2" t="inlineStr"><is><t>metamizol</t></is></c><c r="M602" s="2" t="inlineStr"><is><t>aprotynina</t></is></c><c r="N602" s="2" t="inlineStr" /><c r="O602" s="2" t="inlineStr" /><c r="P602" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q602" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="603"><c r="A603" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B603" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C603" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D603" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E603" s="2" t="inlineStr"><is><t>U chorych obciążonych dodatnią historią krwawienia z wrzodów żołądka w przypadku planowanego przewlekłego leczenia NLPZ należy:</t></is></c><c r="F603" s="2" t="inlineStr"><is><t>przepisać dodatkowo pantoprazol</t></is></c><c r="G603" s="2" t="inlineStr"><is><t>wykonać test na nosicielstwo Helicobacter pylori w celu ewentualnej eradykacji</t></is></c><c r="H603" s="2" t="inlineStr"><is><t>przy braku innych przeciwwskazań wybrać lek z grupy koksybów</t></is></c><c r="I603" s="2" t="inlineStr" /><c r="J603" s="2" t="inlineStr" /><c r="K603" s="2" t="inlineStr"><is><t>bezwzględnie odstąpić od terapii klasycznymi (nieselektywnymi) NLPZ</t></is></c><c r="L603" s="2" t="inlineStr" /><c r="M603" s="2" t="inlineStr" /><c r="N603" s="2" t="inlineStr" /><c r="O603" s="2" t="inlineStr" /><c r="P603" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q603" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="604"><c r="A604" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B604" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C604" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D604" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E604" s="2" t="inlineStr"><is><t>Do leków zwiększających niekorzystny wpływ NLPZ na przewód pokarmowy zaliczysz:</t></is></c><c r="F604" s="2" t="inlineStr"><is><t>warfarynę</t></is></c><c r="G604" s="2" t="inlineStr"><is><t>prednizon</t></is></c><c r="H604" s="2" t="inlineStr" /><c r="I604" s="2" t="inlineStr" /><c r="J604" s="2" t="inlineStr" /><c r="K604" s="2" t="inlineStr"><is><t>etamsylat</t></is></c><c r="L604" s="2" t="inlineStr"><is><t>sukralfat</t></is></c><c r="M604" s="2" t="inlineStr" /><c r="N604" s="2" t="inlineStr" /><c r="O604" s="2" t="inlineStr" /><c r="P604" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q604" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="605"><c r="A605" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B605" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C605" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D605" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E605" s="2" t="inlineStr"><is><t>Czynniki stymulujące erytropoezę:</t></is></c><c r="F605" s="2" t="inlineStr"><is><t>powodują przemijające objawy grypopodobne</t></is></c><c r="G605" s="2" t="inlineStr"><is><t>zwiększają ciśnienie tętnicze krwi</t></is></c><c r="H605" s="2" t="inlineStr"><is><t>rzadko powodują wybiórczą aplazję czerwonokrwinkową</t></is></c><c r="I605" s="2" t="inlineStr"><is><t>predysponują do powikłań zakrzepowych</t></is></c><c r="J605" s="2" t="inlineStr" /><c r="K605" s="2" t="inlineStr" /><c r="L605" s="2" t="inlineStr" /><c r="M605" s="2" t="inlineStr" /><c r="N605" s="2" t="inlineStr" /><c r="O605" s="2" t="inlineStr" /><c r="P605" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q605" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="606"><c r="A606" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B606" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C606" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D606" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E606" s="2" t="inlineStr"><is><t>Którego/których leków może dotyczyć poniższy opis: pośrednio hamuje aktywność czynnika krzepnięcia Xa:</t></is></c><c r="F606" s="2" t="inlineStr"><is><t>enoksaparyna</t></is></c><c r="G606" s="2" t="inlineStr"><is><t>fondaparyna</t></is></c><c r="H606" s="2" t="inlineStr" /><c r="I606" s="2" t="inlineStr" /><c r="J606" s="2" t="inlineStr" /><c r="K606" s="2" t="inlineStr"><is><t>edoksaban</t></is></c><c r="L606" s="2" t="inlineStr"><is><t>biwalirudyna</t></is></c><c r="M606" s="2" t="inlineStr" /><c r="N606" s="2" t="inlineStr" /><c r="O606" s="2" t="inlineStr" /><c r="P606" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q606" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="607"><c r="A607" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B607" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C607" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D607" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E607" s="2" t="inlineStr"><is><t>Którego/których leków może dotyczyć poniższy opis: prolek, nieodwracalnie blokujący receptory P2Y12:</t></is></c><c r="F607" s="2" t="inlineStr"><is><t>prasugrel</t></is></c><c r="G607" s="2" t="inlineStr" /><c r="H607" s="2" t="inlineStr" /><c r="I607" s="2" t="inlineStr" /><c r="J607" s="2" t="inlineStr" /><c r="K607" s="2" t="inlineStr"><is><t>dipyrydamol</t></is></c><c r="L607" s="2" t="inlineStr"><is><t>tikagrelor</t></is></c><c r="M607" s="2" t="inlineStr"><is><t>cilostazol</t></is></c><c r="N607" s="2" t="inlineStr" /><c r="O607" s="2" t="inlineStr" /><c r="P607" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q607" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="608"><c r="A608" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B608" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C608" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D608" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E608" s="2" t="inlineStr"><is><t>Wadą heparyny niefrakcjonowanej w porównaniu z drobnocząsteczkowymi jest:</t></is></c><c r="F608" s="2" t="inlineStr"><is><t>wymaga monitorowania APTT</t></is></c><c r="G608" s="2" t="inlineStr"><is><t>silniej indukuje powstawanie przeciwciał p-kompleksowi PF4 z heparyną</t></is></c><c r="H608" s="2" t="inlineStr" /><c r="I608" s="2" t="inlineStr" /><c r="J608" s="2" t="inlineStr" /><c r="K608" s="2" t="inlineStr"><is><t>jest mniej bezpieczna w niewydolności nerek</t></is></c><c r="L608" s="2" t="inlineStr"><is><t>trudniej jest zneutralizować jej działanie siarczanem protaminy</t></is></c><c r="M608" s="2" t="inlineStr" /><c r="N608" s="2" t="inlineStr" /><c r="O608" s="2" t="inlineStr" /><c r="P608" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q608" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="609"><c r="A609" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B609" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C609" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D609" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E609" s="2" t="inlineStr"><is><t>Rosuwastatyna zmniejsza:</t></is></c><c r="F609" s="2" t="inlineStr"><is><t>syntezę cholesterolu w wątrobie poprzez konkurencyjne hamowanie aktywności reduktazy HMG-CoA</t></is></c><c r="G609" s="2" t="inlineStr"><is><t>stężenie cholesterolu LDL</t></is></c><c r="H609" s="2" t="inlineStr"><is><t>stężenie lipoprotein zawierających apoB, w tym cząsteczek o dużej zawartości triglicerydów</t></is></c><c r="I609" s="2" t="inlineStr" /><c r="J609" s="2" t="inlineStr" /><c r="K609" s="2" t="inlineStr"><is><t>ekspresję receptorów dla LDL na powierzchni hepatocytów</t></is></c><c r="L609" s="2" t="inlineStr" /><c r="M609" s="2" t="inlineStr" /><c r="N609" s="2" t="inlineStr" /><c r="O609" s="2" t="inlineStr" /><c r="P609" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q609" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="610"><c r="A610" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B610" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C610" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D610" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E610" s="2" t="inlineStr"><is><t>W prawidłowo prowadzonej profilaktyce sercowo-naczyniowej (czyli profilaktyce miażdżycy) należy osiągnąć następujące cele terapeutyczne:</t></is></c><c r="F610" s="2" t="inlineStr"><is><t>w grupie osób dużego ryzyka zmniejszenie stężenia cholesterolu LDL w surowicy poniżej 70 mg/dl</t></is></c><c r="G610" s="2" t="inlineStr" /><c r="H610" s="2" t="inlineStr" /><c r="I610" s="2" t="inlineStr" /><c r="J610" s="2" t="inlineStr" /><c r="K610" s="2" t="inlineStr"><is><t>obniżenie stężenia trójglicerydów w surowicy poniżej 115 mg/dl</t></is></c><c r="L610" s="2" t="inlineStr"><is><t>zmniejszenie masy ciała do wartości BMI poniżej 27 kg/m2</t></is></c><c r="M610" s="2" t="inlineStr"><is><t>podwyższenie stężenia cholesterolu HDL w surowicy u mężczyzn powyżej 30 mg/dl</t></is></c><c r="N610" s="2" t="inlineStr" /><c r="O610" s="2" t="inlineStr" /><c r="P610" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q610" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="611"><c r="A611" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B611" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C611" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D611" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E611" s="2" t="inlineStr"><is><t>W leczeniu immunosupresyjnym jest/są stosowana/-e:</t></is></c><c r="F611" s="2" t="inlineStr"><is><t>przeciwciała przeciwtymocytarne królicze</t></is></c><c r="G611" s="2" t="inlineStr" /><c r="H611" s="2" t="inlineStr" /><c r="I611" s="2" t="inlineStr" /><c r="J611" s="2" t="inlineStr" /><c r="K611" s="2" t="inlineStr"><is><t>cyklofilina</t></is></c><c r="L611" s="2" t="inlineStr"><is><t>inozyna</t></is></c><c r="M611" s="2" t="inlineStr"><is><t>kolchicyna</t></is></c><c r="N611" s="2" t="inlineStr" /><c r="O611" s="2" t="inlineStr" /><c r="P611" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q611" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="612"><c r="A612" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B612" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C612" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D612" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E612" s="2" t="inlineStr"><is><t>Lekiem terapii genowej jest:</t></is></c><c r="F612" s="2" t="inlineStr"><is><t>fomiwirsen</t></is></c><c r="G612" s="2" t="inlineStr"><is><t>mipomersen</t></is></c><c r="H612" s="2" t="inlineStr"><is><t>typarwowek alipogenu</t></is></c><c r="I612" s="2" t="inlineStr" /><c r="J612" s="2" t="inlineStr" /><c r="K612" s="2" t="inlineStr"><is><t>OKT3</t></is></c><c r="L612" s="2" t="inlineStr" /><c r="M612" s="2" t="inlineStr" /><c r="N612" s="2" t="inlineStr" /><c r="O612" s="2" t="inlineStr" /><c r="P612" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q612" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="613"><c r="A613" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B613" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C613" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D613" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E613" s="2" t="inlineStr"><is><t>Długotrwałe stosowanie pantoprazolu może być przyczyną:</t></is></c><c r="F613" s="2" t="inlineStr"><is><t>zakażeń dolnego odcinka układu oddechowego</t></is></c><c r="G613" s="2" t="inlineStr"><is><t>zwyrodnienia tylnosznurowego z powodu zmniejszonego wchłaniania witaminy B12</t></is></c><c r="H613" s="2" t="inlineStr"><is><t>osteoporozy</t></is></c><c r="I613" s="2" t="inlineStr"><is><t>zakażeń przewodu pokarmowego</t></is></c><c r="J613" s="2" t="inlineStr" /><c r="K613" s="2" t="inlineStr" /><c r="L613" s="2" t="inlineStr" /><c r="M613" s="2" t="inlineStr" /><c r="N613" s="2" t="inlineStr" /><c r="O613" s="2" t="inlineStr" /><c r="P613" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q613" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="614"><c r="A614" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B614" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C614" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D614" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E614" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące inhibitorów pompy protonowej (IPP):</t></is></c><c r="F614" s="2" t="inlineStr"><is><t>są lekami prekursorowymi</t></is></c><c r="G614" s="2" t="inlineStr"><is><t>aktywność osiągają w komórkach okładzinowych w fazie czynnej=wydzielniczej</t></is></c><c r="H614" s="2" t="inlineStr"><is><t>powodują nieodwracalne zablokowanie pompy protonowej</t></is></c><c r="I614" s="2" t="inlineStr"><is><t>w różnym stopniu hamują izoenzymy CYP (CYP2C19 i CYP3A4)</t></is></c><c r="J614" s="2" t="inlineStr" /><c r="K614" s="2" t="inlineStr" /><c r="L614" s="2" t="inlineStr" /><c r="M614" s="2" t="inlineStr" /><c r="N614" s="2" t="inlineStr" /><c r="O614" s="2" t="inlineStr" /><c r="P614" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q614" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="615"><c r="A615" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B615" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C615" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D615" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E615" s="2" t="inlineStr"><is><t>W leczeniu zaparć będących działaniem niepożądanym agonistów receptorów opioidowych zastosowanie ma:</t></is></c><c r="F615" s="2" t="inlineStr"><is><t>alwimopan</t></is></c><c r="G615" s="2" t="inlineStr"><is><t>metylnaltrekson</t></is></c><c r="H615" s="2" t="inlineStr" /><c r="I615" s="2" t="inlineStr" /><c r="J615" s="2" t="inlineStr" /><c r="K615" s="2" t="inlineStr"><is><t>papaweryna</t></is></c><c r="L615" s="2" t="inlineStr"><is><t>metadon</t></is></c><c r="M615" s="2" t="inlineStr" /><c r="N615" s="2" t="inlineStr" /><c r="O615" s="2" t="inlineStr" /><c r="P615" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q615" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="616"><c r="A616" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B616" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C616" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D616" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E616" s="2" t="inlineStr"><is><t>Wybierz stwierdzenie opisujące 20% roztwór albumin:</t></is></c><c r="F616" s="2" t="inlineStr"><is><t>powoduje ponad 100% przyrost objętości osocza</t></is></c><c r="G616" s="2" t="inlineStr"><is><t>działa objętościowo do 6 h</t></is></c><c r="H616" s="2" t="inlineStr" /><c r="I616" s="2" t="inlineStr" /><c r="J616" s="2" t="inlineStr" /><c r="K616" s="2" t="inlineStr"><is><t>może spowodować uszkodzenie nerek</t></is></c><c r="L616" s="2" t="inlineStr"><is><t>ma istotny wpływ na krzepnięcie krwi</t></is></c><c r="M616" s="2" t="inlineStr" /><c r="N616" s="2" t="inlineStr" /><c r="O616" s="2" t="inlineStr" /><c r="P616" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q616" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="617"><c r="A617" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B617" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C617" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D617" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E617" s="2" t="inlineStr"><is><t>Lekiem genotoksycznym jest:</t></is></c><c r="F617" s="2" t="inlineStr"><is><t>busulfan</t></is></c><c r="G617" s="2" t="inlineStr"><is><t>mitomycyna</t></is></c><c r="H617" s="2" t="inlineStr"><is><t>daktynomycyna</t></is></c><c r="I617" s="2" t="inlineStr"><is><t>etopozyd</t></is></c><c r="J617" s="2" t="inlineStr" /><c r="K617" s="2" t="inlineStr" /><c r="L617" s="2" t="inlineStr" /><c r="M617" s="2" t="inlineStr" /><c r="N617" s="2" t="inlineStr" /><c r="O617" s="2" t="inlineStr" /><c r="P617" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q617" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="618"><c r="A618" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B618" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C618" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D618" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E618" s="2" t="inlineStr"><is><t>Psychoaktywne substancje uzależniające aktywują:</t></is></c><c r="F618" s="2" t="inlineStr"><is><t>obszar brzuszny nakrywki</t></is></c><c r="G618" s="2" t="inlineStr"><is><t>jądro półleżące</t></is></c><c r="H618" s="2" t="inlineStr"><is><t>korę przedczołową</t></is></c><c r="I618" s="2" t="inlineStr"><is><t>mezolimbiczny układ dopaminowy</t></is></c><c r="J618" s="2" t="inlineStr" /><c r="K618" s="2" t="inlineStr" /><c r="L618" s="2" t="inlineStr" /><c r="M618" s="2" t="inlineStr" /><c r="N618" s="2" t="inlineStr" /><c r="O618" s="2" t="inlineStr" /><c r="P618" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q618" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="619"><c r="A619" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B619" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C619" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D619" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E619" s="2" t="inlineStr"><is><t>Patulina:</t></is></c><c r="F619" s="2" t="inlineStr"><is><t>ma działanie mutagenne</t></is></c><c r="G619" s="2" t="inlineStr"><is><t>w warunkach naturalnych znana jest jako substancja skażająca jabłka i powodująca brązową zgniliznę innych owoców</t></is></c><c r="H619" s="2" t="inlineStr" /><c r="I619" s="2" t="inlineStr" /><c r="J619" s="2" t="inlineStr" /><c r="K619" s="2" t="inlineStr"><is><t>powoduje endemiczną epidemię bałkańską</t></is></c><c r="L619" s="2" t="inlineStr"><is><t>jest związkiem, który zwiększa ryzyko nowotworu wątroby</t></is></c><c r="M619" s="2" t="inlineStr" /><c r="N619" s="2" t="inlineStr" /><c r="O619" s="2" t="inlineStr" /><c r="P619" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q619" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="620"><c r="A620" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B620" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C620" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D620" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E620" s="2" t="inlineStr"><is><t>Blaszki miażdżycowe w naczyniach wieńcowych stabilizuje:</t></is></c><c r="F620" s="2" t="inlineStr"><is><t>atorwastatyna</t></is></c><c r="G620" s="2" t="inlineStr" /><c r="H620" s="2" t="inlineStr" /><c r="I620" s="2" t="inlineStr" /><c r="J620" s="2" t="inlineStr" /><c r="K620" s="2" t="inlineStr"><is><t>fondaparyna</t></is></c><c r="L620" s="2" t="inlineStr"><is><t>gliklazyd</t></is></c><c r="M620" s="2" t="inlineStr"><is><t>kwasy omega 6</t></is></c><c r="N620" s="2" t="inlineStr" /><c r="O620" s="2" t="inlineStr" /><c r="P620" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q620" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="621"><c r="A621" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B621" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C621" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D621" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E621" s="2" t="inlineStr"><is><t>Wyrób medyczny to narzędzie, przyrząd, aparat, sprzęt, materiał lub inny artykuł, który może służyć do:</t></is></c><c r="F621" s="2" t="inlineStr"><is><t>regulacji poczęć</t></is></c><c r="G621" s="2" t="inlineStr"><is><t>diagnozowania chorób</t></is></c><c r="H621" s="2" t="inlineStr"><is><t>modyfikowania procesów fizjologicznych</t></is></c><c r="I621" s="2" t="inlineStr" /><c r="J621" s="2" t="inlineStr" /><c r="K621" s="2" t="inlineStr"><is><t>leczenia farmakologicznego</t></is></c><c r="L621" s="2" t="inlineStr" /><c r="M621" s="2" t="inlineStr" /><c r="N621" s="2" t="inlineStr" /><c r="O621" s="2" t="inlineStr" /><c r="P621" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q621" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="622"><c r="A622" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B622" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C622" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D622" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E622" s="2" t="inlineStr"><is><t>W stosowanej do korekty dawkowania leków skali Childa-Turcotte’a-Pugh należy uwzględnić m.in. następujący parametr:</t></is></c><c r="F622" s="2" t="inlineStr"><is><t>stężenie albumin w surowicy</t></is></c><c r="G622" s="2" t="inlineStr"><is><t>stężenie bilirubiny w surowicy</t></is></c><c r="H622" s="2" t="inlineStr"><is><t>ocenę neurologiczną (zmiany osobowości, zaburzenia nastroju, spowolnienie myślenia, zaburzenia koncentracji uwagi, drżenia grubofaliste kończyn, zaburzenia mowy)</t></is></c><c r="I622" s="2" t="inlineStr" /><c r="J622" s="2" t="inlineStr" /><c r="K622" s="2" t="inlineStr"><is><t>stężenie kreatyniny w surowicy</t></is></c><c r="L622" s="2" t="inlineStr" /><c r="M622" s="2" t="inlineStr" /><c r="N622" s="2" t="inlineStr" /><c r="O622" s="2" t="inlineStr" /><c r="P622" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q622" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="623"><c r="A623" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B623" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C623" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D623" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E623" s="2" t="inlineStr"><is><t>Lek L jest metabolizowany w wątrobie przy udziale enzymów CYP do nieaktywnych i nietoksycznych metabolitów, które następnie wydalane są przez nerki. Można się zatem spodziewać, że wystąpienie działań toksycznych tego leku jest:</t></is></c><c r="F623" s="2" t="inlineStr"><is><t>bardziej prawdopodobne u osób pijących regularnie soki owocowe, zwłaszcza grejfrutowy</t></is></c><c r="G623" s="2" t="inlineStr" /><c r="H623" s="2" t="inlineStr" /><c r="I623" s="2" t="inlineStr" /><c r="J623" s="2" t="inlineStr" /><c r="K623" s="2" t="inlineStr"><is><t>zależne głównie od stopnia wydolności nerek</t></is></c><c r="L623" s="2" t="inlineStr"><is><t>częstsze podczas stosowania induktorów enzymów CYP</t></is></c><c r="M623" s="2" t="inlineStr"><is><t>związane ze stosowaniem leków wiążących kwasy żółciowe w przewodzie pokarmowym</t></is></c><c r="N623" s="2" t="inlineStr" /><c r="O623" s="2" t="inlineStr" /><c r="P623" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q623" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="624"><c r="A624" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B624" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C624" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D624" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E624" s="2" t="inlineStr"><is><t>Glikokortykosteroidy są stosowane w:</t></is></c><c r="F624" s="2" t="inlineStr"><is><t>diagnostyce zespołu Cushinga</t></is></c><c r="G624" s="2" t="inlineStr"><is><t>leczeniu chorób alergicznych</t></is></c><c r="H624" s="2" t="inlineStr"><is><t>leczeniu ostrej niewydolności kory nadnerczy</t></is></c><c r="I624" s="2" t="inlineStr" /><c r="J624" s="2" t="inlineStr" /><c r="K624" s="2" t="inlineStr"><is><t>w kardiogennym obrzęku płuc</t></is></c><c r="L624" s="2" t="inlineStr" /><c r="M624" s="2" t="inlineStr" /><c r="N624" s="2" t="inlineStr" /><c r="O624" s="2" t="inlineStr" /><c r="P624" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q624" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="625"><c r="A625" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B625" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C625" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D625" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E625" s="2" t="inlineStr"><is><t>Przyrost masy ciała powoduje:</t></is></c><c r="F625" s="2" t="inlineStr"><is><t>gliklazyd</t></is></c><c r="G625" s="2" t="inlineStr"><is><t>insulina izofanowa</t></is></c><c r="H625" s="2" t="inlineStr" /><c r="I625" s="2" t="inlineStr" /><c r="J625" s="2" t="inlineStr" /><c r="K625" s="2" t="inlineStr"><is><t>liraglutyd</t></is></c><c r="L625" s="2" t="inlineStr"><is><t>metformina</t></is></c><c r="M625" s="2" t="inlineStr" /><c r="N625" s="2" t="inlineStr" /><c r="O625" s="2" t="inlineStr" /><c r="P625" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q625" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="626"><c r="A626" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B626" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C626" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D626" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E626" s="2" t="inlineStr"><is><t>Glikokortykosteroidy dzieli się na słabo i silnie działające na podstawie:</t></is></c><c r="F626" s="2" t="inlineStr"><is><t>testu wazokonstrykcji naczyń (zblednięcia skóry)</t></is></c><c r="G626" s="2" t="inlineStr"><is><t>działania przeciwzapalnego</t></is></c><c r="H626" s="2" t="inlineStr" /><c r="I626" s="2" t="inlineStr" /><c r="J626" s="2" t="inlineStr" /><c r="K626" s="2" t="inlineStr"><is><t>działania mineralokortykoidowego</t></is></c><c r="L626" s="2" t="inlineStr"><is><t>działania immunosupresyjnego</t></is></c><c r="M626" s="2" t="inlineStr" /><c r="N626" s="2" t="inlineStr" /><c r="O626" s="2" t="inlineStr" /><c r="P626" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q626" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="627"><c r="A627" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B627" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C627" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D627" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E627" s="2" t="inlineStr"><is><t>Za typowe polekowe działanie niepożądane podczas stosowania niesteroidowych leków przeciwzapalnych uznasz:</t></is></c><c r="F627" s="2" t="inlineStr"><is><t>krwawienie z wrzodu dwunastnicy</t></is></c><c r="G627" s="2" t="inlineStr"><is><t>skurcz oskrzeli u chorego z polipami nosa i przewlekłym zapaleniem zatok</t></is></c><c r="H627" s="2" t="inlineStr"><is><t>hipernatremię (zwiększenie stężenia sodu w surowicy)</t></is></c><c r="I627" s="2" t="inlineStr" /><c r="J627" s="2" t="inlineStr" /><c r="K627" s="2" t="inlineStr"><is><t>hipokaliemię (obniżenie stężenia potasu w surowicy)</t></is></c><c r="L627" s="2" t="inlineStr" /><c r="M627" s="2" t="inlineStr" /><c r="N627" s="2" t="inlineStr" /><c r="O627" s="2" t="inlineStr" /><c r="P627" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q627" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="628"><c r="A628" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B628" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C628" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D628" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E628" s="2" t="inlineStr"><is><t>Wskaż poprawną definicję:</t></is></c><c r="F628" s="2" t="inlineStr"><is><t>wpółczynnik (indeks) terapeutyczny leku – zakres między najmniejszą dawką skuteczną a maksymalną nie powodującą efektów toksycznych, im większy tym korzystniej</t></is></c><c r="G628" s="2" t="inlineStr"><is><t>placebo - interwencja pozbawiona bezpośredniego działania biologicznego, mająca stworzyć u pacjenta wrażenie, że otrzymuje on leczenie</t></is></c><c r="H628" s="2" t="inlineStr" /><c r="I628" s="2" t="inlineStr" /><c r="J628" s="2" t="inlineStr" /><c r="K628" s="2" t="inlineStr"><is><t>polekowe działanie niepożądane – każde niepożądane i niezamierzone zdarzenie podczas stosowania leku, bez konieczności ustalenia związku przyczynowo-skutkowego</t></is></c><c r="L628" s="2" t="inlineStr"><is><t>metaanaliza - badanie wieloośrodkowe, w którym grupa eksperymentalna porównywana jest do grupy kontrolne</t></is></c><c r="M628" s="2" t="inlineStr" /><c r="N628" s="2" t="inlineStr" /><c r="O628" s="2" t="inlineStr" /><c r="P628" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q628" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="629"><c r="A629" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B629" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C629" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D629" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E629" s="2" t="inlineStr"><is><t>Objawy przedawkowania oksykodonu to:</t></is></c><c r="F629" s="2" t="inlineStr"><is><t>zmniejszenie częstości oddechów</t></is></c><c r="G629" s="2" t="inlineStr" /><c r="H629" s="2" t="inlineStr" /><c r="I629" s="2" t="inlineStr" /><c r="J629" s="2" t="inlineStr" /><c r="K629" s="2" t="inlineStr"><is><t>rozszerzone źrenice</t></is></c><c r="L629" s="2" t="inlineStr"><is><t>pobudzenie psychoruchowe</t></is></c><c r="M629" s="2" t="inlineStr"><is><t>gorączka obwodowa</t></is></c><c r="N629" s="2" t="inlineStr" /><c r="O629" s="2" t="inlineStr" /><c r="P629" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q629" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="630"><c r="A630" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B630" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C630" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D630" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E630" s="2" t="inlineStr"><is><t>Szybki efekt przeciwbólowy można osiągnąć, stosując:</t></is></c><c r="F630" s="2" t="inlineStr"><is><t>fentanyl w postaci donosowej</t></is></c><c r="G630" s="2" t="inlineStr"><is><t>buprenorfinę w tabletkach podjęzykowych</t></is></c><c r="H630" s="2" t="inlineStr" /><c r="I630" s="2" t="inlineStr" /><c r="J630" s="2" t="inlineStr" /><c r="K630" s="2" t="inlineStr"><is><t>tramadol w systemie transdermalnym</t></is></c><c r="L630" s="2" t="inlineStr"><is><t>nalokson we wlewie dożylnym</t></is></c><c r="M630" s="2" t="inlineStr" /><c r="N630" s="2" t="inlineStr" /><c r="O630" s="2" t="inlineStr" /><c r="P630" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q630" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="631"><c r="A631" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B631" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C631" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D631" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E631" s="2" t="inlineStr"><is><t>Działanie przeciwgorączkowe ma:</t></is></c><c r="F631" s="2" t="inlineStr"><is><t>metamizol</t></is></c><c r="G631" s="2" t="inlineStr"><is><t>paracetamol</t></is></c><c r="H631" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="I631" s="2" t="inlineStr"><is><t>ibuprofen</t></is></c><c r="J631" s="2" t="inlineStr" /><c r="K631" s="2" t="inlineStr" /><c r="L631" s="2" t="inlineStr" /><c r="M631" s="2" t="inlineStr" /><c r="N631" s="2" t="inlineStr" /><c r="O631" s="2" t="inlineStr" /><c r="P631" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q631" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="632"><c r="A632" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B632" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C632" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D632" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E632" s="2" t="inlineStr"><is><t>Popularna aspiryna, czyli poprawnie kwas acetylosalicylowy:</t></is></c><c r="F632" s="2" t="inlineStr"><is><t>jest przeciwwskazana u dzieci do 12 r.ż</t></is></c><c r="G632" s="2" t="inlineStr"><is><t>konkuruje o miejsce wiązania z ibuprofenem</t></is></c><c r="H632" s="2" t="inlineStr" /><c r="I632" s="2" t="inlineStr" /><c r="J632" s="2" t="inlineStr" /><c r="K632" s="2" t="inlineStr"><is><t>działa odwracalnie antyagregacyjnie</t></is></c><c r="L632" s="2" t="inlineStr"><is><t>w małych dawkach preferencyjnie hamuje cyklooksygenazę 2</t></is></c><c r="M632" s="2" t="inlineStr" /><c r="N632" s="2" t="inlineStr" /><c r="O632" s="2" t="inlineStr" /><c r="P632" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q632" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="633"><c r="A633" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B633" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C633" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D633" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E633" s="2" t="inlineStr"><is><t>Wskaż prawidłowy zestaw lek – antidotum:</t></is></c><c r="F633" s="2" t="inlineStr"><is><t>heparyna – siarczan protaminy</t></is></c><c r="G633" s="2" t="inlineStr"><is><t>warfaryna - fitomenadion</t></is></c><c r="H633" s="2" t="inlineStr"><is><t>dabigatraban – idarucizumab</t></is></c><c r="I633" s="2" t="inlineStr"><is><t>acenokumarol – koncentrat zespołu czynników protrombiny</t></is></c><c r="J633" s="2" t="inlineStr" /><c r="K633" s="2" t="inlineStr" /><c r="L633" s="2" t="inlineStr" /><c r="M633" s="2" t="inlineStr" /><c r="N633" s="2" t="inlineStr" /><c r="O633" s="2" t="inlineStr" /><c r="P633" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q633" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="634"><c r="A634" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B634" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C634" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D634" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E634" s="2" t="inlineStr"><is><t>U pacjentów z mechaniczną zastawką serca potwierdzono skuteczność przeciwzakrzepową:</t></is></c><c r="F634" s="2" t="inlineStr"><is><t>warfaryny</t></is></c><c r="G634" s="2" t="inlineStr" /><c r="H634" s="2" t="inlineStr" /><c r="I634" s="2" t="inlineStr" /><c r="J634" s="2" t="inlineStr" /><c r="K634" s="2" t="inlineStr"><is><t>fondaparyny</t></is></c><c r="L634" s="2" t="inlineStr"><is><t>kwasu acetylosalicylowego + klopidogrelu</t></is></c><c r="M634" s="2" t="inlineStr"><is><t>dabigatranu</t></is></c><c r="N634" s="2" t="inlineStr" /><c r="O634" s="2" t="inlineStr" /><c r="P634" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q634" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="635"><c r="A635" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B635" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C635" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D635" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E635" s="2" t="inlineStr"><is><t>Hematopoetycznymi czynnikami wzrostu, które znalazły zastosowanie kliniczne są:</t></is></c><c r="F635" s="2" t="inlineStr"><is><t>darbepoetyna</t></is></c><c r="G635" s="2" t="inlineStr"><is><t>filgrastym</t></is></c><c r="H635" s="2" t="inlineStr"><is><t>lenograstym</t></is></c><c r="I635" s="2" t="inlineStr"><is><t>interleukina-11</t></is></c><c r="J635" s="2" t="inlineStr" /><c r="K635" s="2" t="inlineStr" /><c r="L635" s="2" t="inlineStr" /><c r="M635" s="2" t="inlineStr" /><c r="N635" s="2" t="inlineStr" /><c r="O635" s="2" t="inlineStr" /><c r="P635" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q635" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="636"><c r="A636" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B636" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C636" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D636" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E636" s="2" t="inlineStr"><is><t>Przeciwwskazaniem do stosowania kwasu acetylosalicylowego w dawce antyagregacyjnej jest:</t></is></c><c r="F636" s="2" t="inlineStr"><is><t>nadwrażliwość na NLPZ (niesteroidowe leki przeciwzapalne)</t></is></c><c r="G636" s="2" t="inlineStr" /><c r="H636" s="2" t="inlineStr" /><c r="I636" s="2" t="inlineStr" /><c r="J636" s="2" t="inlineStr" /><c r="K636" s="2" t="inlineStr"><is><t>choroba wrzodowa górnego odcinka przewodu pokarmowego w wywiadach</t></is></c><c r="L636" s="2" t="inlineStr"><is><t>zespół zależności alkoholowej</t></is></c><c r="M636" s="2" t="inlineStr"><is><t>niewydolność nerek</t></is></c><c r="N636" s="2" t="inlineStr" /><c r="O636" s="2" t="inlineStr" /><c r="P636" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q636" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="637"><c r="A637" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B637" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C637" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D637" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E637" s="2" t="inlineStr"><is><t>Istotnemu metabolizmowi wątrobowemu za pośrednictwem izoenzymów CYP podlega:</t></is></c><c r="F637" s="2" t="inlineStr"><is><t>atorwastatyna</t></is></c><c r="G637" s="2" t="inlineStr"><is><t>symwastatyna</t></is></c><c r="H637" s="2" t="inlineStr" /><c r="I637" s="2" t="inlineStr" /><c r="J637" s="2" t="inlineStr" /><c r="K637" s="2" t="inlineStr"><is><t>rosuwastatyna</t></is></c><c r="L637" s="2" t="inlineStr"><is><t>prawastayna</t></is></c><c r="M637" s="2" t="inlineStr" /><c r="N637" s="2" t="inlineStr" /><c r="O637" s="2" t="inlineStr" /><c r="P637" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q637" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="638"><c r="A638" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B638" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C638" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D638" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E638" s="2" t="inlineStr"><is><t>Inhibitory reduktazy HMG-CoA:</t></is></c><c r="F638" s="2" t="inlineStr"><is><t>w większym stopniu zmniejszają stężenie cholesterolu LDL w surowicy w porównaniu z fibratami</t></is></c><c r="G638" s="2" t="inlineStr" /><c r="H638" s="2" t="inlineStr" /><c r="I638" s="2" t="inlineStr" /><c r="J638" s="2" t="inlineStr" /><c r="K638" s="2" t="inlineStr"><is><t>w większym stopniu zmniejszają stężenie triglicerydów w surowicy w porównaniu z fibratami</t></is></c><c r="L638" s="2" t="inlineStr"><is><t>mają istotny wpływ na stężenie Lp(a) = lipoproteiny a</t></is></c><c r="M638" s="2" t="inlineStr"><is><t>nie powinny być łączone z inhibitorami PCSK9</t></is></c><c r="N638" s="2" t="inlineStr" /><c r="O638" s="2" t="inlineStr" /><c r="P638" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q638" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="639"><c r="A639" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B639" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C639" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D639" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E639" s="2" t="inlineStr"><is><t>Wskaż prawidłowy zestaw lek – akceptowany sposób monitorowania działania:</t></is></c><c r="F639" s="2" t="inlineStr"><is><t>rywaroksaban – aktywność czynnika anty - Xa</t></is></c><c r="G639" s="2" t="inlineStr"><is><t>dabigatran - APTT</t></is></c><c r="H639" s="2" t="inlineStr"><is><t>acenokumarol – INR</t></is></c><c r="I639" s="2" t="inlineStr" /><c r="J639" s="2" t="inlineStr" /><c r="K639" s="2" t="inlineStr"><is><t>heparyna niefrakcjonowana – czas protrombinowy</t></is></c><c r="L639" s="2" t="inlineStr" /><c r="M639" s="2" t="inlineStr" /><c r="N639" s="2" t="inlineStr" /><c r="O639" s="2" t="inlineStr" /><c r="P639" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q639" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="640"><c r="A640" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B640" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C640" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D640" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E640" s="2" t="inlineStr"><is><t>Wskaż zestaw zawierający inhibitory kalcyneuryny:</t></is></c><c r="F640" s="2" t="inlineStr"><is><t>pimekrolimus, takrolimus, cyklosporyna</t></is></c><c r="G640" s="2" t="inlineStr" /><c r="H640" s="2" t="inlineStr" /><c r="I640" s="2" t="inlineStr" /><c r="J640" s="2" t="inlineStr" /><c r="K640" s="2" t="inlineStr"><is><t>cyklosporyna, pimekrolimus, sirolimus</t></is></c><c r="L640" s="2" t="inlineStr"><is><t>ewerolimus, takrolimus, cyklosporyna</t></is></c><c r="M640" s="2" t="inlineStr"><is><t>takrolimus, azatiopryna, pimekrolimus</t></is></c><c r="N640" s="2" t="inlineStr" /><c r="O640" s="2" t="inlineStr" /><c r="P640" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q640" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="641"><c r="A641" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B641" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C641" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D641" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E641" s="2" t="inlineStr"><is><t>W Europie dopuszczono do obrotu biopodobne produkty zawierające infliksymab. Oznacza to, że:</t></is></c><c r="F641" s="2" t="inlineStr"><is><t>wykazano ich podobieństwo farmaceutyczne z produktem oryginalnym</t></is></c><c r="G641" s="2" t="inlineStr"><is><t>wykazano ich podobieństwo z produktem oryginalnym w modelach przedklinicznych</t></is></c><c r="H641" s="2" t="inlineStr"><is><t>wykazano jego podobieństwo z produktem oryginalnym w badaniach klinicznych</t></is></c><c r="I641" s="2" t="inlineStr"><is><t>wykazano ich podobną immunogenność z produktem oryginalnym w badaniach klinicznych</t></is></c><c r="J641" s="2" t="inlineStr" /><c r="K641" s="2" t="inlineStr" /><c r="L641" s="2" t="inlineStr" /><c r="M641" s="2" t="inlineStr" /><c r="N641" s="2" t="inlineStr" /><c r="O641" s="2" t="inlineStr" /><c r="P641" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q641" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="642"><c r="A642" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B642" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C642" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D642" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E642" s="2" t="inlineStr"><is><t>Rozkurczający wpływ na mięśniówkę przewodu pokarmowego wywiera:</t></is></c><c r="F642" s="2" t="inlineStr"><is><t>mebeweryna</t></is></c><c r="G642" s="2" t="inlineStr" /><c r="H642" s="2" t="inlineStr" /><c r="I642" s="2" t="inlineStr" /><c r="J642" s="2" t="inlineStr" /><c r="K642" s="2" t="inlineStr"><is><t>racekadotryl</t></is></c><c r="L642" s="2" t="inlineStr"><is><t>mesalazyna</t></is></c><c r="M642" s="2" t="inlineStr"><is><t>ryfaksymina</t></is></c><c r="N642" s="2" t="inlineStr" /><c r="O642" s="2" t="inlineStr" /><c r="P642" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q642" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="643"><c r="A643" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B643" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C643" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D643" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E643" s="2" t="inlineStr"><is><t>W skojarzonej terapii eradykacyjnej H. pylori zastosujesz zgodnie z aktualną wiedzą medyczną:</t></is></c><c r="F643" s="2" t="inlineStr"><is><t>omeprazol</t></is></c><c r="G643" s="2" t="inlineStr"><is><t>pantoprazol</t></is></c><c r="H643" s="2" t="inlineStr"><is><t>cytrynian bizmutu</t></is></c><c r="I643" s="2" t="inlineStr" /><c r="J643" s="2" t="inlineStr" /><c r="K643" s="2" t="inlineStr"><is><t>ranitydynę</t></is></c><c r="L643" s="2" t="inlineStr" /><c r="M643" s="2" t="inlineStr" /><c r="N643" s="2" t="inlineStr" /><c r="O643" s="2" t="inlineStr" /><c r="P643" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q643" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="644"><c r="A644" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B644" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C644" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D644" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E644" s="2" t="inlineStr"><is><t>Izotonicznym krystaloidem do uzupełnienie płynów jest:</t></is></c><c r="F644" s="2" t="inlineStr"><is><t>0,9% NaCl</t></is></c><c r="G644" s="2" t="inlineStr"><is><t>płyn wieloelektrolitowy</t></is></c><c r="H644" s="2" t="inlineStr"><is><t>płyn 2 : 1 (5% glukoza + 0,9% NaCl)</t></is></c><c r="I644" s="2" t="inlineStr" /><c r="J644" s="2" t="inlineStr" /><c r="K644" s="2" t="inlineStr"><is><t>4% roztw. żelatyny</t></is></c><c r="L644" s="2" t="inlineStr" /><c r="M644" s="2" t="inlineStr" /><c r="N644" s="2" t="inlineStr" /><c r="O644" s="2" t="inlineStr" /><c r="P644" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q644" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="645"><c r="A645" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B645" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C645" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D645" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E645" s="2" t="inlineStr"><is><t>Dysforia, nudności, wymioty, biegunka, bóle mięśni, łzawienie, wyciek z nosa, pocenie, rozszerzenie źrenic, piloerekcja, ziewanie i gorączka to cechy zespołu odstawiennego u uzależnionych od:</t></is></c><c r="F645" s="2" t="inlineStr"><is><t>heroiny</t></is></c><c r="G645" s="2" t="inlineStr" /><c r="H645" s="2" t="inlineStr" /><c r="I645" s="2" t="inlineStr" /><c r="J645" s="2" t="inlineStr" /><c r="K645" s="2" t="inlineStr"><is><t>etanolu</t></is></c><c r="L645" s="2" t="inlineStr"><is><t>nikotyny</t></is></c><c r="M645" s="2" t="inlineStr"><is><t>kokainy</t></is></c><c r="N645" s="2" t="inlineStr" /><c r="O645" s="2" t="inlineStr" /><c r="P645" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q645" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="646"><c r="A646" s="2" t="inlineStr"><is><t>LEKI TOKSYCZNE W CIĄŻY</t></is></c><c r="B646" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C646" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D646" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E646" s="2" t="inlineStr"><is><t>Mykotoksyny:</t></is></c><c r="F646" s="2" t="inlineStr"><is><t>to produkty wtórnego metabolizmu różnych rodzajów grzybów pleśniowych</t></is></c><c r="G646" s="2" t="inlineStr"><is><t>są wytwarzane jako produkt uboczny w procesach metabolicznych lub są produktem wytwarzanym w celach obronnych</t></is></c><c r="H646" s="2" t="inlineStr"><is><t>mogą mieć silne właściwości mutagenne lub teratogenne</t></is></c><c r="I646" s="2" t="inlineStr"><is><t>są potencjalnie toksyczne dla ludzi i zwierząt</t></is></c><c r="J646" s="2" t="inlineStr" /><c r="K646" s="2" t="inlineStr" /><c r="L646" s="2" t="inlineStr" /><c r="M646" s="2" t="inlineStr" /><c r="N646" s="2" t="inlineStr" /><c r="O646" s="2" t="inlineStr" /><c r="P646" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q646" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="647"><c r="A647" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B647" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C647" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D647" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E647" s="2" t="inlineStr"><is><t>Wskaż korzystne cechy leku:</t></is></c><c r="F647" s="2" t="inlineStr"><is><t>biodostępność po podaniu p.o. dorównująca biodostępności po podaniu i.v</t></is></c><c r="G647" s="2" t="inlineStr"><is><t>dostępne swoiste antidotum</t></is></c><c r="H647" s="2" t="inlineStr" /><c r="I647" s="2" t="inlineStr" /><c r="J647" s="2" t="inlineStr" /><c r="K647" s="2" t="inlineStr"><is><t>procesy kinetyczne zgodne z kinetyką 0 rzędu</t></is></c><c r="L647" s="2" t="inlineStr"><is><t>duża kumulacja w tkankach – wiązanie z biomolekułami</t></is></c><c r="M647" s="2" t="inlineStr" /><c r="N647" s="2" t="inlineStr" /><c r="O647" s="2" t="inlineStr" /><c r="P647" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q647" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="648"><c r="A648" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B648" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C648" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D648" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E648" s="2" t="inlineStr"><is><t>Jaki lek przeciwbakteryjny może odpowiadać poniższej charakterystyce? Ma dobrą biodostępność po podaniu doustnym i jest skuteczny w zakażeniach Streptococcus pneumoniae przy obecnym profilu oporności tego gatunku pod warunkiem właściwego schematu ekspozycji na lek:</t></is></c><c r="F648" s="2" t="inlineStr"><is><t>lewofloksacyna</t></is></c><c r="G648" s="2" t="inlineStr"><is><t>amoksycylina</t></is></c><c r="H648" s="2" t="inlineStr" /><c r="I648" s="2" t="inlineStr" /><c r="J648" s="2" t="inlineStr" /><c r="K648" s="2" t="inlineStr"><is><t>doksycyklina</t></is></c><c r="L648" s="2" t="inlineStr"><is><t>ceftriakson</t></is></c><c r="M648" s="2" t="inlineStr" /><c r="N648" s="2" t="inlineStr" /><c r="O648" s="2" t="inlineStr" /><c r="P648" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q648" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="649"><c r="A649" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B649" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C649" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D649" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E649" s="2" t="inlineStr"><is><t>Co jest zasadniczym warunkiem skuteczności cefadroksylu w leczeniu niepowikłanych zakażeń układu moczowego?</t></is></c><c r="F649" s="2" t="inlineStr"><is><t>przestrzeganie stałego interwału dawkowania zgodnie z parametrami farmakokinetycznymi leku</t></is></c><c r="G649" s="2" t="inlineStr"><is><t>fT%&gt;MIC ≥ 60%</t></is></c><c r="H649" s="2" t="inlineStr" /><c r="I649" s="2" t="inlineStr" /><c r="J649" s="2" t="inlineStr" /><c r="K649" s="2" t="inlineStr"><is><t>stały 10-dniowy cykl leczenia</t></is></c><c r="L649" s="2" t="inlineStr"><is><t>podanie jak największej bezpiecznej dawki jednorazowej, czyli uzyskanie maksymalnego bezpiecznego stężenia leku w surowicy</t></is></c><c r="M649" s="2" t="inlineStr" /><c r="N649" s="2" t="inlineStr" /><c r="O649" s="2" t="inlineStr" /><c r="P649" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q649" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="650"><c r="A650" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B650" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C650" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D650" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E650" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenia dotyczące kwasu klawulanowego:</t></is></c><c r="F650" s="2" t="inlineStr"><is><t>kwas klawulanowy powoduje niezależnie działania niepożądane, np. Polekowe zapalenie wątroby</t></is></c><c r="G650" s="2" t="inlineStr"><is><t>zmniejszona wrażliwość Streptococcus pneumoniae na beta-laktamy ma mechanizm nieenzymatyczny, zatem stosowanie połączeń z kwasem klawulanowym w zakażeniach o tej etiologii nie ma uzasadnienia</t></is></c><c r="H650" s="2" t="inlineStr"><is><t>amoksycylina + kwas klawulanowy powodują znaczną dysbakteriozę i skłonność do nadkażeń florą szpitalną</t></is></c><c r="I650" s="2" t="inlineStr" /><c r="J650" s="2" t="inlineStr" /><c r="K650" s="2" t="inlineStr"><is><t>kwas klawulanowy jest przeciwwskazany w ciąży</t></is></c><c r="L650" s="2" t="inlineStr" /><c r="M650" s="2" t="inlineStr" /><c r="N650" s="2" t="inlineStr" /><c r="O650" s="2" t="inlineStr" /><c r="P650" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q650" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="651"><c r="A651" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B651" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C651" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D651" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E651" s="2" t="inlineStr"><is><t>Podaj prawidłową interpretację sytuacji klinicznej:</t></is></c><c r="F651" s="2" t="inlineStr"><is><t>w 1 h po zakończeniu dożylnego podania piperacyliny + tazobaktamu (pip + taz) wystąpiła pokrzywka i duszność, ciśnienie skurczowe = 80 mmHg → nadwrażliwość typu natychmiastowego na penicyliny → zakaz leczenia wszystkimi penicylinami</t></is></c><c r="G651" s="2" t="inlineStr"><is><t>po 1 tygodniu leczenia ceftriaksonem + azytromycyną domowego zapalenia płuc w szpitalu wystąpiła małopłytkowość PLT = 60 G/l → nadwrażliwość typu cytotoksycznego najprawdopodobniej po ceftriaksonie → zakaz leczenia wszystkimi cefalosporynami</t></is></c><c r="H651" s="2" t="inlineStr"><is><t>po 5 dniach leczenia ceftriaksonem z metronidazolem w ramach leczenia powikłanego zapalenia wyrostka robaczkowego po operacji apendektomii wystąpił atak kolki żółciowej, w USG złogi w pęcherzyku żółciowym → prawdopodobnie wzrost gęstości żółci z powodu wydzielania ceftriaksonu → zakaz kontynuacji ceftriaksonu</t></is></c><c r="I651" s="2" t="inlineStr" /><c r="J651" s="2" t="inlineStr" /><c r="K651" s="2" t="inlineStr"><is><t>po 1 tygodniu leczenia pip + taz z powodu powikłanego zakażenia jamy brzusznej wystąpiły uogólnione obrzęki, w bad. laboratoryjnych hipernatremia = 153 mmol/l → bez związku z antybiotykoterapią, należy szukać innej przyczyny → kontynuacja leczenia pip + taz</t></is></c><c r="L651" s="2" t="inlineStr" /><c r="M651" s="2" t="inlineStr" /><c r="N651" s="2" t="inlineStr" /><c r="O651" s="2" t="inlineStr" /><c r="P651" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q651" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="652"><c r="A652" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B652" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C652" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D652" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E652" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii metycylinooporne Staphylococcus spp. uzasadnione może być zastosowanie:</t></is></c><c r="F652" s="2" t="inlineStr"><is><t>tigecyklina</t></is></c><c r="G652" s="2" t="inlineStr" /><c r="H652" s="2" t="inlineStr" /><c r="I652" s="2" t="inlineStr" /><c r="J652" s="2" t="inlineStr" /><c r="K652" s="2" t="inlineStr"><is><t>ceftolozanu + tazobaktamu</t></is></c><c r="L652" s="2" t="inlineStr"><is><t>meropenemu</t></is></c><c r="M652" s="2" t="inlineStr"><is><t>ceftazydymu + awibaktamu</t></is></c><c r="N652" s="2" t="inlineStr" /><c r="O652" s="2" t="inlineStr" /><c r="P652" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q652" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="653"><c r="A653" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B653" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C653" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D653" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E653" s="2" t="inlineStr"><is><t>Łatwo jest prowadzić leczenie sekwencyjne w przypadku:</t></is></c><c r="F653" s="2" t="inlineStr"><is><t>kloksacyliny</t></is></c><c r="G653" s="2" t="inlineStr"><is><t>amoksycyliny + kwasu klawulanowego</t></is></c><c r="H653" s="2" t="inlineStr"><is><t>cefuroksymu</t></is></c><c r="I653" s="2" t="inlineStr" /><c r="J653" s="2" t="inlineStr" /><c r="K653" s="2" t="inlineStr"><is><t>ceftazydymu</t></is></c><c r="L653" s="2" t="inlineStr" /><c r="M653" s="2" t="inlineStr" /><c r="N653" s="2" t="inlineStr" /><c r="O653" s="2" t="inlineStr" /><c r="P653" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q653" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="654"><c r="A654" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B654" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C654" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D654" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E654" s="2" t="inlineStr"><is><t>Prawdziwe jest stwierdzenie:</t></is></c><c r="F654" s="2" t="inlineStr"><is><t>cefazolina i cefuroksym i.v. są lekami z wyboru w p-infekcyjnej profilaktyce okołozabiegowej</t></is></c><c r="G654" s="2" t="inlineStr"><is><t>amoksycylina + kwas klawulanowy p.o. jest lekiem z wyboru w leczeniu z wyprzedzeniem po pogryzieniu przez psa</t></is></c><c r="H654" s="2" t="inlineStr" /><c r="I654" s="2" t="inlineStr" /><c r="J654" s="2" t="inlineStr" /><c r="K654" s="2" t="inlineStr"><is><t>ampicylina i.v. jest lekiem z wyboru w p-infekcyjnej profilaktyce rany skórnej spowodowanej ostrym przedmiotem</t></is></c><c r="L654" s="2" t="inlineStr"><is><t>aksetyl cefuroksymu jest lekiem z wyboru w leczeniu z wyprzedzeniem asymptomatycznej bakteriurii u 75-letniej kobiety z nietrzymaniem moczu</t></is></c><c r="M654" s="2" t="inlineStr" /><c r="N654" s="2" t="inlineStr" /><c r="O654" s="2" t="inlineStr" /><c r="P654" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q654" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="655"><c r="A655" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B655" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C655" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D655" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E655" s="2" t="inlineStr"><is><t>W którym przypadku decyzja dotycząca racjonalnego leczenia początkowego domowego zakażenia jest prawidłowa u pacjenta bez nadwrażliwości na leki w wywiadach?</t></is></c><c r="F655" s="2" t="inlineStr"><is><t>grypa u nieszczepionego 80-letniego mężczyzny z POChP – oseltamiwir</t></is></c><c r="G655" s="2" t="inlineStr"><is><t>zapalenie płuc u osoby bez chorób współtowarzyszących – amoksycylina w dawce 3-4 g/24 h</t></is></c><c r="H655" s="2" t="inlineStr" /><c r="I655" s="2" t="inlineStr" /><c r="J655" s="2" t="inlineStr" /><c r="K655" s="2" t="inlineStr"><is><t>angina paciorkowcowa – azytromycyna</t></is></c><c r="L655" s="2" t="inlineStr"><is><t>niezapalna ostra biegunka – cyprofloksacyna</t></is></c><c r="M655" s="2" t="inlineStr" /><c r="N655" s="2" t="inlineStr" /><c r="O655" s="2" t="inlineStr" /><c r="P655" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q655" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="656"><c r="A656" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B656" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C656" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D656" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E656" s="2" t="inlineStr"><is><t>Linezolid jest wskazany w terapii zakażeń o etiologii:</t></is></c><c r="F656" s="2" t="inlineStr"><is><t>wankomycynooporny Enterococcus faecium (WRE)</t></is></c><c r="G656" s="2" t="inlineStr"><is><t>Streptococcus pneumoniae opornej na penicylinę</t></is></c><c r="H656" s="2" t="inlineStr"><is><t>metycylinooporny gronkowiec złocisty (MRSA)</t></is></c><c r="I656" s="2" t="inlineStr" /><c r="J656" s="2" t="inlineStr" /><c r="K656" s="2" t="inlineStr"><is><t>Klebsiella pneumonae oporna na karbapenemy</t></is></c><c r="L656" s="2" t="inlineStr" /><c r="M656" s="2" t="inlineStr" /><c r="N656" s="2" t="inlineStr" /><c r="O656" s="2" t="inlineStr" /><c r="P656" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q656" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="657"><c r="A657" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B657" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C657" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D657" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E657" s="2" t="inlineStr"><is><t>Który zestaw przedstawia leki od najwęższego do najszerszego spektrum działania przeciwbakteryjnego:</t></is></c><c r="F657" s="2" t="inlineStr"><is><t>ampicylina – piperacylina – piperacylina + tazobaktam</t></is></c><c r="G657" s="2" t="inlineStr"><is><t>ertapenem – imipenem – meropenem + waborbaktam</t></is></c><c r="H657" s="2" t="inlineStr" /><c r="I657" s="2" t="inlineStr" /><c r="J657" s="2" t="inlineStr" /><c r="K657" s="2" t="inlineStr"><is><t>ceftazydym – cefotaksym – cefepim</t></is></c><c r="L657" s="2" t="inlineStr"><is><t>ampicylina – fenoksymetylopenicylina – kloksacylina</t></is></c><c r="M657" s="2" t="inlineStr" /><c r="N657" s="2" t="inlineStr" /><c r="O657" s="2" t="inlineStr" /><c r="P657" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q657" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="658"><c r="A658" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B658" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C658" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D658" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E658" s="2" t="inlineStr"><is><t>W leczeniu zakażenia bakteriami atypowymi u chorego z pierwotnym wydłużeniem QTc racjonalne jest zastosowanie:</t></is></c><c r="F658" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="G658" s="2" t="inlineStr" /><c r="H658" s="2" t="inlineStr" /><c r="I658" s="2" t="inlineStr" /><c r="J658" s="2" t="inlineStr" /><c r="K658" s="2" t="inlineStr"><is><t>moksyfloksacyny</t></is></c><c r="L658" s="2" t="inlineStr"><is><t>klarytromycyny</t></is></c><c r="M658" s="2" t="inlineStr"><is><t>klindamycyny</t></is></c><c r="N658" s="2" t="inlineStr" /><c r="O658" s="2" t="inlineStr" /><c r="P658" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q658" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="659"><c r="A659" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B659" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C659" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D659" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E659" s="2" t="inlineStr"><is><t>Wskazaniem do zastosowania metronidazolu jest:</t></is></c><c r="F659" s="2" t="inlineStr"><is><t>biegunka o etiologii Clostridium difficile o nieciężkim przebiegu</t></is></c><c r="G659" s="2" t="inlineStr"><is><t>lamblioza</t></is></c><c r="H659" s="2" t="inlineStr" /><c r="I659" s="2" t="inlineStr" /><c r="J659" s="2" t="inlineStr" /><c r="K659" s="2" t="inlineStr"><is><t>eradykacja nosicielstwa Bacteroides fragilis z przewodu pokarmowego przed wszystkimi operacjami w polu czystym-skażonym</t></is></c><c r="L659" s="2" t="inlineStr"><is><t>toksoplazmoza</t></is></c><c r="M659" s="2" t="inlineStr" /><c r="N659" s="2" t="inlineStr" /><c r="O659" s="2" t="inlineStr" /><c r="P659" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q659" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="660"><c r="A660" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B660" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C660" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D660" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E660" s="2" t="inlineStr"><is><t>Ze względu na podobieństwo w farmakologicznym mechanizmie działania nie należy łączyć:</t></is></c><c r="F660" s="2" t="inlineStr"><is><t>kotrymoksazolu i trimetoprimu</t></is></c><c r="G660" s="2" t="inlineStr"><is><t>erytromycyny i klindamycyny</t></is></c><c r="H660" s="2" t="inlineStr" /><c r="I660" s="2" t="inlineStr" /><c r="J660" s="2" t="inlineStr" /><c r="K660" s="2" t="inlineStr"><is><t>ampicyliny i gentamycyny</t></is></c><c r="L660" s="2" t="inlineStr"><is><t>wankomycyny i aztreonamu</t></is></c><c r="M660" s="2" t="inlineStr" /><c r="N660" s="2" t="inlineStr" /><c r="O660" s="2" t="inlineStr" /><c r="P660" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q660" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="661"><c r="A661" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B661" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C661" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D661" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E661" s="2" t="inlineStr"><is><t>Nadwrażliwość na promieniowanie ultrafioletowe (UV) może być związana ze stosowaniem:</t></is></c><c r="F661" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="G661" s="2" t="inlineStr"><is><t>lewofloksacyny</t></is></c><c r="H661" s="2" t="inlineStr"><is><t>kotrymoksazolu</t></is></c><c r="I661" s="2" t="inlineStr" /><c r="J661" s="2" t="inlineStr" /><c r="K661" s="2" t="inlineStr"><is><t>amoksycyliny</t></is></c><c r="L661" s="2" t="inlineStr" /><c r="M661" s="2" t="inlineStr" /><c r="N661" s="2" t="inlineStr" /><c r="O661" s="2" t="inlineStr" /><c r="P661" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q661" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="662"><c r="A662" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B662" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C662" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D662" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E662" s="2" t="inlineStr"><is><t>Za uzasadnione uznasz dodanie metronidazolu do:</t></is></c><c r="F662" s="2" t="inlineStr"><is><t>cyprofloksacyny w leczeniu zakażenia mieszanego dróg żółciowych z udziałem beztlenowców</t></is></c><c r="G662" s="2" t="inlineStr" /><c r="H662" s="2" t="inlineStr" /><c r="I662" s="2" t="inlineStr" /><c r="J662" s="2" t="inlineStr" /><c r="K662" s="2" t="inlineStr"><is><t>amoksycyliny + kwasu klawulanowego w leczeniu zakażenia mieszanego zatok szczękowych z udziałem beztlenowców</t></is></c><c r="L662" s="2" t="inlineStr"><is><t>piperacyliny + tazobaktamu w leczeniu zachłystowego zapalenia płuc (zakażenie florą przewodu pokarmowego)</t></is></c><c r="M662" s="2" t="inlineStr"><is><t>imipenemu + cilastatyny w leczeniu kałowego zapalenia otrzewnej po perforacji jelita grubego (zakażenie florą przewodu pokarmowego)</t></is></c><c r="N662" s="2" t="inlineStr" /><c r="O662" s="2" t="inlineStr" /><c r="P662" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q662" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="663"><c r="A663" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B663" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C663" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D663" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E663" s="2" t="inlineStr"><is><t>Właściwy wybór leku w infestacji pasożytniczej to:</t></is></c><c r="F663" s="2" t="inlineStr"><is><t>wszawica - permetryna</t></is></c><c r="G663" s="2" t="inlineStr"><is><t>rzęsistkowica - metronidazol</t></is></c><c r="H663" s="2" t="inlineStr"><is><t>toksoplazmoza – kotrymoksazol</t></is></c><c r="I663" s="2" t="inlineStr"><is><t>infestacja owsikiem - pyrantel</t></is></c><c r="J663" s="2" t="inlineStr" /><c r="K663" s="2" t="inlineStr" /><c r="L663" s="2" t="inlineStr" /><c r="M663" s="2" t="inlineStr" /><c r="N663" s="2" t="inlineStr" /><c r="O663" s="2" t="inlineStr" /><c r="P663" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q663" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="664"><c r="A664" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B664" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C664" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D664" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E664" s="2" t="inlineStr"><is><t>Właściwy wybór leku przeciwwirusowego w zakażeniu wirusowym to:</t></is></c><c r="F664" s="2" t="inlineStr"><is><t>wirus półpaśca – acyklowir</t></is></c><c r="G664" s="2" t="inlineStr"><is><t>przewlekłe wirusowe zapalenie wątroby typu C - bezpośrednio działające ledipaswir + sofosbuwir</t></is></c><c r="H664" s="2" t="inlineStr" /><c r="I664" s="2" t="inlineStr" /><c r="J664" s="2" t="inlineStr" /><c r="K664" s="2" t="inlineStr"><is><t>rotawirus – loperamid</t></is></c><c r="L664" s="2" t="inlineStr"><is><t>kłykciny kończyste – pranobeks inozyny</t></is></c><c r="M664" s="2" t="inlineStr" /><c r="N664" s="2" t="inlineStr" /><c r="O664" s="2" t="inlineStr" /><c r="P664" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q664" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="665"><c r="A665" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B665" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C665" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D665" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E665" s="2" t="inlineStr"><is><t>W dermatofitozach skuteczne jest miejscowe użycie:</t></is></c><c r="F665" s="2" t="inlineStr"><is><t>naftyfiny</t></is></c><c r="G665" s="2" t="inlineStr"><is><t>klotrimazolu</t></is></c><c r="H665" s="2" t="inlineStr" /><c r="I665" s="2" t="inlineStr" /><c r="J665" s="2" t="inlineStr" /><c r="K665" s="2" t="inlineStr"><is><t>natamycyny</t></is></c><c r="L665" s="2" t="inlineStr"><is><t>imikwimodu</t></is></c><c r="M665" s="2" t="inlineStr" /><c r="N665" s="2" t="inlineStr" /><c r="O665" s="2" t="inlineStr" /><c r="P665" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q665" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="666"><c r="A666" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B666" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C666" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D666" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E666" s="2" t="inlineStr"><is><t>W przypadku biegunki o etiologii Clostridium difficile uzasadnione może być stosowanie:</t></is></c><c r="F666" s="2" t="inlineStr"><is><t>fidaksomycyny doustnie</t></is></c><c r="G666" s="2" t="inlineStr"><is><t>wankomycyny doustnie</t></is></c><c r="H666" s="2" t="inlineStr" /><c r="I666" s="2" t="inlineStr" /><c r="J666" s="2" t="inlineStr" /><c r="K666" s="2" t="inlineStr"><is><t>nifuroksazydu doustnie</t></is></c><c r="L666" s="2" t="inlineStr"><is><t>kotrymoksazolu doustnie</t></is></c><c r="M666" s="2" t="inlineStr" /><c r="N666" s="2" t="inlineStr" /><c r="O666" s="2" t="inlineStr" /><c r="P666" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q666" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="667"><c r="A667" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B667" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C667" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D667" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E667" s="2" t="inlineStr"><is><t>W leczeniu gruźlicy wielolekoopornej (MDR-TB) do leków podstawowych (grupa A, B i C wg wytycznych WHO) należy:</t></is></c><c r="F667" s="2" t="inlineStr"><is><t>moksyfloksacyna</t></is></c><c r="G667" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="H667" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="I667" s="2" t="inlineStr"><is><t>kapreomycyna</t></is></c><c r="J667" s="2" t="inlineStr" /><c r="K667" s="2" t="inlineStr" /><c r="L667" s="2" t="inlineStr" /><c r="M667" s="2" t="inlineStr" /><c r="N667" s="2" t="inlineStr" /><c r="O667" s="2" t="inlineStr" /><c r="P667" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q667" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="668"><c r="A668" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B668" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C668" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D668" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E668" s="2" t="inlineStr"><is><t>Opis farmakokinetyki leku A: lek A dobrze wchłania się z przewodu pokarmowego, dobrze przenika przez barierę krew – mózg, podlega metabolizmowi wątrobowemu. Lekiem A może być:</t></is></c><c r="F668" s="2" t="inlineStr"><is><t>worykonazol</t></is></c><c r="G668" s="2" t="inlineStr" /><c r="H668" s="2" t="inlineStr" /><c r="I668" s="2" t="inlineStr" /><c r="J668" s="2" t="inlineStr" /><c r="K668" s="2" t="inlineStr"><is><t>amoksycylina</t></is></c><c r="L668" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="M668" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="N668" s="2" t="inlineStr" /><c r="O668" s="2" t="inlineStr" /><c r="P668" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q668" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="669"><c r="A669" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B669" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C669" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D669" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E669" s="2" t="inlineStr"><is><t>Zmiany na płytkach paznokciowych polegające na ich zgrubieniu, przebarwieniu, łamliwości, nadmiernym rogowaceniu i pobruzdowaniu można leczyć:</t></is></c><c r="F669" s="2" t="inlineStr"><is><t>amorolfiną miejscowo</t></is></c><c r="G669" s="2" t="inlineStr"><is><t>terbinafiną doustnie</t></is></c><c r="H669" s="2" t="inlineStr"><is><t>itrakonazolem doustnie</t></is></c><c r="I669" s="2" t="inlineStr"><is><t>cyklopiroksolaminą miejscowo</t></is></c><c r="J669" s="2" t="inlineStr" /><c r="K669" s="2" t="inlineStr" /><c r="L669" s="2" t="inlineStr" /><c r="M669" s="2" t="inlineStr" /><c r="N669" s="2" t="inlineStr" /><c r="O669" s="2" t="inlineStr" /><c r="P669" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q669" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="670"><c r="A670" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B670" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C670" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D670" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E670" s="2" t="inlineStr"><is><t>Aktualnie wg komunikatu WHO krytyczny problem wielolekooporności na większość leków p-bakteryjnych dotyczy:</t></is></c><c r="F670" s="2" t="inlineStr"><is><t>Acinetobacter baumani z opornością na karbapenemy</t></is></c><c r="G670" s="2" t="inlineStr"><is><t>Pseudomonas aeruginosa z opornością na karbapenemy</t></is></c><c r="H670" s="2" t="inlineStr"><is><t>Enterobacteriacae z opornością na karbapenemy</t></is></c><c r="I670" s="2" t="inlineStr" /><c r="J670" s="2" t="inlineStr" /><c r="K670" s="2" t="inlineStr"><is><t>Stenotrophomonas maltophilia z opornością na karbapenemy</t></is></c><c r="L670" s="2" t="inlineStr" /><c r="M670" s="2" t="inlineStr" /><c r="N670" s="2" t="inlineStr" /><c r="O670" s="2" t="inlineStr" /><c r="P670" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q670" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="671"><c r="A671" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B671" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C671" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D671" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E671" s="2" t="inlineStr"><is><t>Dla leków p-infekcyjnych dla których celem farmakodynamicznym jest wysoka wartość fAUC : MIC, np. fluorochinolonów zasadne jest:</t></is></c><c r="F671" s="2" t="inlineStr"><is><t>zwiększenie w bezpiecznych granicach skumulowanej dobowej dawki leku</t></is></c><c r="G671" s="2" t="inlineStr" /><c r="H671" s="2" t="inlineStr" /><c r="I671" s="2" t="inlineStr" /><c r="J671" s="2" t="inlineStr" /><c r="K671" s="2" t="inlineStr"><is><t>precyzyjne ustalenie jak najczęstszego dawkowania leku</t></is></c><c r="L671" s="2" t="inlineStr"><is><t>monitorowanie stężenia maksymalnego (peak) w celu modyfikacji dawki</t></is></c><c r="M671" s="2" t="inlineStr"><is><t>osiągnięcie zdefiniowanej wartości fCmin : MIC</t></is></c><c r="N671" s="2" t="inlineStr" /><c r="O671" s="2" t="inlineStr" /><c r="P671" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q671" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="672"><c r="A672" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B672" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C672" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D672" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E672" s="2" t="inlineStr"><is><t>U pacjenta z eGFR &lt; 30 ml/min (wyliczony z wzoru Cockcrofta-Gaulta) należy zmodyfikować dawkowanie:</t></is></c><c r="F672" s="2" t="inlineStr"><is><t>gentamycyny</t></is></c><c r="G672" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="H672" s="2" t="inlineStr"><is><t>imipenemu</t></is></c><c r="I672" s="2" t="inlineStr" /><c r="J672" s="2" t="inlineStr" /><c r="K672" s="2" t="inlineStr"><is><t>klindamycyny</t></is></c><c r="L672" s="2" t="inlineStr" /><c r="M672" s="2" t="inlineStr" /><c r="N672" s="2" t="inlineStr" /><c r="O672" s="2" t="inlineStr" /><c r="P672" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q672" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="673"><c r="A673" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B673" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C673" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D673" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E673" s="2" t="inlineStr"><is><t>Do długoterminowych działań niepożądanych terapii HAART należy:</t></is></c><c r="F673" s="2" t="inlineStr"><is><t>uszkodzenie wątroby</t></is></c><c r="G673" s="2" t="inlineStr"><is><t>zespół lipodystrofii</t></is></c><c r="H673" s="2" t="inlineStr"><is><t>kwasica mleczanowa</t></is></c><c r="I673" s="2" t="inlineStr"><is><t>insulinooporność</t></is></c><c r="J673" s="2" t="inlineStr" /><c r="K673" s="2" t="inlineStr" /><c r="L673" s="2" t="inlineStr" /><c r="M673" s="2" t="inlineStr" /><c r="N673" s="2" t="inlineStr" /><c r="O673" s="2" t="inlineStr" /><c r="P673" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q673" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="674"><c r="A674" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B674" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C674" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D674" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E674" s="2" t="inlineStr"><is><t>Do jakiego związku może się odnosić następujący opis: ma słabe działanie antyseptyczne, po wchłonięciu może powodować ciężkie powikłania tj. Uszkodzenia wątroby i nerek, niewydolność serca, splątanie, a nawet zgon:</t></is></c><c r="F674" s="2" t="inlineStr"><is><t>boran sodu</t></is></c><c r="G674" s="2" t="inlineStr" /><c r="H674" s="2" t="inlineStr" /><c r="I674" s="2" t="inlineStr" /><c r="J674" s="2" t="inlineStr" /><c r="K674" s="2" t="inlineStr"><is><t>oktenidyna</t></is></c><c r="L674" s="2" t="inlineStr"><is><t>woda utleniona</t></is></c><c r="M674" s="2" t="inlineStr"><is><t>jodopowidon</t></is></c><c r="N674" s="2" t="inlineStr" /><c r="O674" s="2" t="inlineStr" /><c r="P674" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q674" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="675"><c r="A675" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B675" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C675" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D675" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E675" s="2" t="inlineStr"><is><t>U pacjenta leczonego antagonistą witaminy K (warfaryną, acenokumarolem) zmianę efektu przeciwzakrzepowego bez adekwatnej modyfikacji dawki tego leku może spowodować:</t></is></c><c r="F675" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="G675" s="2" t="inlineStr"><is><t>klarytromycyna</t></is></c><c r="H675" s="2" t="inlineStr"><is><t>ryfampicyna</t></is></c><c r="I675" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="J675" s="2" t="inlineStr" /><c r="K675" s="2" t="inlineStr" /><c r="L675" s="2" t="inlineStr" /><c r="M675" s="2" t="inlineStr" /><c r="N675" s="2" t="inlineStr" /><c r="O675" s="2" t="inlineStr" /><c r="P675" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q675" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="676"><c r="A676" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B676" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C676" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D676" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E676" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Streptococcus pneumoniae skuteczny/a może być:</t></is></c><c r="F676" s="2" t="inlineStr"><is><t>ceftriakson</t></is></c><c r="G676" s="2" t="inlineStr"><is><t>klarytromycyna</t></is></c><c r="H676" s="2" t="inlineStr"><is><t>amoksycylina</t></is></c><c r="I676" s="2" t="inlineStr"><is><t>lewofloksacyna</t></is></c><c r="J676" s="2" t="inlineStr" /><c r="K676" s="2" t="inlineStr" /><c r="L676" s="2" t="inlineStr" /><c r="M676" s="2" t="inlineStr" /><c r="N676" s="2" t="inlineStr" /><c r="O676" s="2" t="inlineStr" /><c r="P676" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q676" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="677"><c r="A677" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B677" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C677" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D677" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E677" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Escherichia coli skuteczny/a może być:</t></is></c><c r="F677" s="2" t="inlineStr"><is><t>cefuroksym</t></is></c><c r="G677" s="2" t="inlineStr"><is><t>kotrymoksazol</t></is></c><c r="H677" s="2" t="inlineStr"><is><t>fosfomycyna</t></is></c><c r="I677" s="2" t="inlineStr" /><c r="J677" s="2" t="inlineStr" /><c r="K677" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="L677" s="2" t="inlineStr" /><c r="M677" s="2" t="inlineStr" /><c r="N677" s="2" t="inlineStr" /><c r="O677" s="2" t="inlineStr" /><c r="P677" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q677" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="678"><c r="A678" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B678" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C678" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D678" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E678" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Staphylococcus aureus metycylinowrażliwy (MSSA) skuteczny/a może być:</t></is></c><c r="F678" s="2" t="inlineStr"><is><t>cefadroksyl</t></is></c><c r="G678" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="H678" s="2" t="inlineStr"><is><t>kloksacylina</t></is></c><c r="I678" s="2" t="inlineStr" /><c r="J678" s="2" t="inlineStr" /><c r="K678" s="2" t="inlineStr"><is><t>fenoksymetylopenicylina</t></is></c><c r="L678" s="2" t="inlineStr" /><c r="M678" s="2" t="inlineStr" /><c r="N678" s="2" t="inlineStr" /><c r="O678" s="2" t="inlineStr" /><c r="P678" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q678" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="679"><c r="A679" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B679" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C679" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D679" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E679" s="2" t="inlineStr"><is><t>W zakażeniu o etiologii Streptococcus pyogenes skuteczny/a może być:</t></is></c><c r="F679" s="2" t="inlineStr"><is><t>penicylina benzylowa</t></is></c><c r="G679" s="2" t="inlineStr"><is><t>erytromycyna</t></is></c><c r="H679" s="2" t="inlineStr"><is><t>fenoksymetylopenicylina</t></is></c><c r="I679" s="2" t="inlineStr" /><c r="J679" s="2" t="inlineStr" /><c r="K679" s="2" t="inlineStr"><is><t>aztreonam</t></is></c><c r="L679" s="2" t="inlineStr" /><c r="M679" s="2" t="inlineStr" /><c r="N679" s="2" t="inlineStr" /><c r="O679" s="2" t="inlineStr" /><c r="P679" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q679" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="680"><c r="A680" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B680" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C680" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D680" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E680" s="2" t="inlineStr"><is><t>W zakażeniu o etiologii Pseudomonas aeruginosa skuteczny/a może być:</t></is></c><c r="F680" s="2" t="inlineStr"><is><t>gentamycyna</t></is></c><c r="G680" s="2" t="inlineStr"><is><t>cefepim</t></is></c><c r="H680" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="I680" s="2" t="inlineStr"><is><t>piperacylina</t></is></c><c r="J680" s="2" t="inlineStr" /><c r="K680" s="2" t="inlineStr" /><c r="L680" s="2" t="inlineStr" /><c r="M680" s="2" t="inlineStr" /><c r="N680" s="2" t="inlineStr" /><c r="O680" s="2" t="inlineStr" /><c r="P680" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q680" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="681"><c r="A681" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B681" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C681" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D681" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E681" s="2" t="inlineStr"><is><t>W zakażeniach wywołanych przez beztlenowce (w tym Bacteroides fragilis) skuteczny/a może być:</t></is></c><c r="F681" s="2" t="inlineStr"><is><t>amoksycylina + kwas klawulanowy</t></is></c><c r="G681" s="2" t="inlineStr"><is><t>imipenem + cilastatyna</t></is></c><c r="H681" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="I681" s="2" t="inlineStr" /><c r="J681" s="2" t="inlineStr" /><c r="K681" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="L681" s="2" t="inlineStr" /><c r="M681" s="2" t="inlineStr" /><c r="N681" s="2" t="inlineStr" /><c r="O681" s="2" t="inlineStr" /><c r="P681" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q681" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="682"><c r="A682" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B682" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C682" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D682" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E682" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Mycoplasma pneumoniae skuteczny/a może być:</t></is></c><c r="F682" s="2" t="inlineStr"><is><t>azytromycyna</t></is></c><c r="G682" s="2" t="inlineStr"><is><t>doksycyklina</t></is></c><c r="H682" s="2" t="inlineStr"><is><t>moksyfloksacyna</t></is></c><c r="I682" s="2" t="inlineStr" /><c r="J682" s="2" t="inlineStr" /><c r="K682" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="L682" s="2" t="inlineStr" /><c r="M682" s="2" t="inlineStr" /><c r="N682" s="2" t="inlineStr" /><c r="O682" s="2" t="inlineStr" /><c r="P682" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q682" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="683"><c r="A683" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B683" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C683" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D683" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E683" s="2" t="inlineStr"><is><t>W eradykacji Helicobacter pylori można zastosować:</t></is></c><c r="F683" s="2" t="inlineStr"><is><t>tetracyklina</t></is></c><c r="G683" s="2" t="inlineStr"><is><t>amoksycylina</t></is></c><c r="H683" s="2" t="inlineStr"><is><t>cytrynian bizmutu</t></is></c><c r="I683" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="J683" s="2" t="inlineStr" /><c r="K683" s="2" t="inlineStr" /><c r="L683" s="2" t="inlineStr" /><c r="M683" s="2" t="inlineStr" /><c r="N683" s="2" t="inlineStr" /><c r="O683" s="2" t="inlineStr" /><c r="P683" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q683" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="684"><c r="A684" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B684" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C684" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D684" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E684" s="2" t="inlineStr"><is><t>Ciężarna kobieta leczona była z konieczności gentamycyną z powodu powikłanego zapalenia nerek. Na jakie ryzyka narażone zostało jej dziecko w czasie takiej terapii?</t></is></c><c r="F684" s="2" t="inlineStr"><is><t>głuchotę</t></is></c><c r="G684" s="2" t="inlineStr" /><c r="H684" s="2" t="inlineStr" /><c r="I684" s="2" t="inlineStr" /><c r="J684" s="2" t="inlineStr" /><c r="K684" s="2" t="inlineStr"><is><t>powstanie deformacji kostnych</t></is></c><c r="L684" s="2" t="inlineStr"><is><t>utratę wzroku</t></is></c><c r="M684" s="2" t="inlineStr"><is><t>zahamowanie rozwoju chrząstek</t></is></c><c r="N684" s="2" t="inlineStr" /><c r="O684" s="2" t="inlineStr" /><c r="P684" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q684" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="685"><c r="A685" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B685" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C685" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D685" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E685" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek przeciwbakteryjny – mechanizm działania</t></is></c><c r="F685" s="2" t="inlineStr"><is><t>kolistyna – uszkadza błonę komórkową</t></is></c><c r="G685" s="2" t="inlineStr" /><c r="H685" s="2" t="inlineStr" /><c r="I685" s="2" t="inlineStr" /><c r="J685" s="2" t="inlineStr" /><c r="K685" s="2" t="inlineStr"><is><t>cyprofloksacyna – działa cytotoksycznie uszkadzając DNA</t></is></c><c r="L685" s="2" t="inlineStr"><is><t>azytromycyna – hamuje syntezę ściany bakteryjnej</t></is></c><c r="M685" s="2" t="inlineStr"><is><t>metronidazol – hamuje syntezę DNA</t></is></c><c r="N685" s="2" t="inlineStr" /><c r="O685" s="2" t="inlineStr" /><c r="P685" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q685" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="686"><c r="A686" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B686" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C686" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D686" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E686" s="2" t="inlineStr"><is><t>Aby uzyskać działanie ogólnoustrojowe, doustnie można podać:</t></is></c><c r="F686" s="2" t="inlineStr"><is><t>lewofloksacynę</t></is></c><c r="G686" s="2" t="inlineStr" /><c r="H686" s="2" t="inlineStr" /><c r="I686" s="2" t="inlineStr" /><c r="J686" s="2" t="inlineStr" /><c r="K686" s="2" t="inlineStr"><is><t>wankomycynę</t></is></c><c r="L686" s="2" t="inlineStr"><is><t>fidaksomycynę</t></is></c><c r="M686" s="2" t="inlineStr"><is><t>ryfaksyminę</t></is></c><c r="N686" s="2" t="inlineStr" /><c r="O686" s="2" t="inlineStr" /><c r="P686" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q686" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="687"><c r="A687" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B687" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C687" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D687" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E687" s="2" t="inlineStr"><is><t>Do antybiotyków o szerokim zakresie działania przeciwbakteryjnego na bakterie Gram (+) i Gram (-) należy:</t></is></c><c r="F687" s="2" t="inlineStr"><is><t>tygecyklina</t></is></c><c r="G687" s="2" t="inlineStr"><is><t>piperacylina + tazobaktam</t></is></c><c r="H687" s="2" t="inlineStr" /><c r="I687" s="2" t="inlineStr" /><c r="J687" s="2" t="inlineStr" /><c r="K687" s="2" t="inlineStr"><is><t>kolistyna</t></is></c><c r="L687" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="M687" s="2" t="inlineStr" /><c r="N687" s="2" t="inlineStr" /><c r="O687" s="2" t="inlineStr" /><c r="P687" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q687" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="688"><c r="A688" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B688" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C688" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D688" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E688" s="2" t="inlineStr"><is><t>Do leków do stosowania wyłącznie miejscowego należy:</t></is></c><c r="F688" s="2" t="inlineStr"><is><t>bacytracyna</t></is></c><c r="G688" s="2" t="inlineStr"><is><t>mupirocyna</t></is></c><c r="H688" s="2" t="inlineStr"><is><t>nystatyna</t></is></c><c r="I688" s="2" t="inlineStr" /><c r="J688" s="2" t="inlineStr" /><c r="K688" s="2" t="inlineStr"><is><t>fosfomycyna</t></is></c><c r="L688" s="2" t="inlineStr" /><c r="M688" s="2" t="inlineStr" /><c r="N688" s="2" t="inlineStr" /><c r="O688" s="2" t="inlineStr" /><c r="P688" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q688" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="689"><c r="A689" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B689" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C689" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D689" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E689" s="2" t="inlineStr"><is><t>Leki przeciwbakteryjne o wysokim potencjale selekcji szczepów Clostridium difficile to:</t></is></c><c r="F689" s="2" t="inlineStr"><is><t>amoksycylina + kwas klawulanowy</t></is></c><c r="G689" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="H689" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="I689" s="2" t="inlineStr" /><c r="J689" s="2" t="inlineStr" /><c r="K689" s="2" t="inlineStr"><is><t>teikoplanina</t></is></c><c r="L689" s="2" t="inlineStr" /><c r="M689" s="2" t="inlineStr" /><c r="N689" s="2" t="inlineStr" /><c r="O689" s="2" t="inlineStr" /><c r="P689" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q689" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="690"><c r="A690" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B690" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C690" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D690" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E690" s="2" t="inlineStr"><is><t>Wskaż właściwe połączenia: mechanizm oporności na lek przeciwbakteryjny – lek unieczynniany w tym mechanizmie:</t></is></c><c r="F690" s="2" t="inlineStr"><is><t>wytwarzanie β-laktamaz – amoksycylina</t></is></c><c r="G690" s="2" t="inlineStr" /><c r="H690" s="2" t="inlineStr" /><c r="I690" s="2" t="inlineStr" /><c r="J690" s="2" t="inlineStr" /><c r="K690" s="2" t="inlineStr"><is><t>wytwarzanie karbapenemaz – tazobaktam</t></is></c><c r="L690" s="2" t="inlineStr"><is><t>metylacja podjednostki 50S rybosomu - fosfomycyna</t></is></c><c r="M690" s="2" t="inlineStr"><is><t>modyfikacja/ochrona topoizomerazy II – metronidazol</t></is></c><c r="N690" s="2" t="inlineStr" /><c r="O690" s="2" t="inlineStr" /><c r="P690" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q690" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="691"><c r="A691" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B691" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C691" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D691" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E691" s="2" t="inlineStr"><is><t>Cel farmakodynamiczny, jakim jest zależność efektu od czasu w jakim stężenie leku przekracza MIC (fT&gt;MIC) należy osiągnąć w trakcie stosowania:</t></is></c><c r="F691" s="2" t="inlineStr"><is><t>linezolidu</t></is></c><c r="G691" s="2" t="inlineStr"><is><t>ceftriaksonu</t></is></c><c r="H691" s="2" t="inlineStr" /><c r="I691" s="2" t="inlineStr" /><c r="J691" s="2" t="inlineStr" /><c r="K691" s="2" t="inlineStr"><is><t>metronidazolu</t></is></c><c r="L691" s="2" t="inlineStr"><is><t>cyprofloksacyny</t></is></c><c r="M691" s="2" t="inlineStr" /><c r="N691" s="2" t="inlineStr" /><c r="O691" s="2" t="inlineStr" /><c r="P691" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q691" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="692"><c r="A692" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B692" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C692" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D692" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E692" s="2" t="inlineStr"><is><t>Który z poniższych leków hamuje podjędnostkę 30S rybosomów?</t></is></c><c r="F692" s="2" t="inlineStr"><is><t>tygecyklina</t></is></c><c r="G692" s="2" t="inlineStr"><is><t>streptomycyna</t></is></c><c r="H692" s="2" t="inlineStr" /><c r="I692" s="2" t="inlineStr" /><c r="J692" s="2" t="inlineStr" /><c r="K692" s="2" t="inlineStr"><is><t>chinuprystyna-dalfoprystyna</t></is></c><c r="L692" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="M692" s="2" t="inlineStr" /><c r="N692" s="2" t="inlineStr" /><c r="O692" s="2" t="inlineStr" /><c r="P692" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q692" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="693"><c r="A693" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B693" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C693" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D693" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E693" s="2" t="inlineStr"><is><t>Antybiotyki beta-laktamowe:</t></is></c><c r="F693" s="2" t="inlineStr"><is><t>cechują się bardzo dobrym profilem bezpieczeństwa</t></is></c><c r="G693" s="2" t="inlineStr"><is><t>są praktycznie pozbawione istotnych interakcji lekowych</t></is></c><c r="H693" s="2" t="inlineStr" /><c r="I693" s="2" t="inlineStr" /><c r="J693" s="2" t="inlineStr" /><c r="K693" s="2" t="inlineStr"><is><t>bardzo dobrze dystrybuują do płynu mózgowo rdzeniowego</t></is></c><c r="L693" s="2" t="inlineStr"><is><t>są przeciwwskazane w umiarkowanej i ciężkiej niewydolności wątroby</t></is></c><c r="M693" s="2" t="inlineStr" /><c r="N693" s="2" t="inlineStr" /><c r="O693" s="2" t="inlineStr" /><c r="P693" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q693" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="694"><c r="A694" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B694" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C694" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D694" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E694" s="2" t="inlineStr"><is><t>Tetracykliny:</t></is></c><c r="F694" s="2" t="inlineStr"><is><t>są przeciwwskazane u dzieci</t></is></c><c r="G694" s="2" t="inlineStr"><is><t>działają także na bakterie atypowe</t></is></c><c r="H694" s="2" t="inlineStr"><is><t>mogą być przyczyną fotosensytyzacji</t></is></c><c r="I694" s="2" t="inlineStr" /><c r="J694" s="2" t="inlineStr" /><c r="K694" s="2" t="inlineStr"><is><t>mają nadal szeroki zakres działania przeciwbakteryjnego wobec bakterii tlenowych i mogą być stosowane w empirycznym leczeniu wielu zespołów klinicznych</t></is></c><c r="L694" s="2" t="inlineStr" /><c r="M694" s="2" t="inlineStr" /><c r="N694" s="2" t="inlineStr" /><c r="O694" s="2" t="inlineStr" /><c r="P694" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q694" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="695"><c r="A695" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B695" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C695" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D695" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E695" s="2" t="inlineStr"><is><t>Oseltamiwir należy stosować u nieszczepionych osób z grup ryzyka ciężkiego przebiegu grypy, do których należą:</t></is></c><c r="F695" s="2" t="inlineStr"><is><t>kobiety w ciąży i w 2 tyg. po porodzie</t></is></c><c r="G695" s="2" t="inlineStr"><is><t>dzieci do 2 roku życia</t></is></c><c r="H695" s="2" t="inlineStr"><is><t>osoby z wieku podeszłym &gt;= 65 lat</t></is></c><c r="I695" s="2" t="inlineStr" /><c r="J695" s="2" t="inlineStr" /><c r="K695" s="2" t="inlineStr"><is><t>kobiety karmiące piersią</t></is></c><c r="L695" s="2" t="inlineStr" /><c r="M695" s="2" t="inlineStr" /><c r="N695" s="2" t="inlineStr" /><c r="O695" s="2" t="inlineStr" /><c r="P695" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q695" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="696"><c r="A696" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B696" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C696" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D696" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E696" s="2" t="inlineStr"><is><t>Acyklowir służy do leczenia:</t></is></c><c r="F696" s="2" t="inlineStr"><is><t>opryszczki pospolitej (HSV)</t></is></c><c r="G696" s="2" t="inlineStr"><is><t>ospy wietrznej i półpaśca (VZV)</t></is></c><c r="H696" s="2" t="inlineStr" /><c r="I696" s="2" t="inlineStr" /><c r="J696" s="2" t="inlineStr" /><c r="K696" s="2" t="inlineStr"><is><t>mononukleozy zakaźnej (EBV)</t></is></c><c r="L696" s="2" t="inlineStr"><is><t>cytomegalii (CMV)</t></is></c><c r="M696" s="2" t="inlineStr" /><c r="N696" s="2" t="inlineStr" /><c r="O696" s="2" t="inlineStr" /><c r="P696" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q696" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="697"><c r="A697" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B697" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C697" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D697" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E697" s="2" t="inlineStr"><is><t>W bezinterferonowej terapii przewlekłego wirusowego zapalenia wątroby typu C zastosowanie mają leki przeciwwirusowe działające bezpośrednio (DAA) na wirusa typu C, do których należy:</t></is></c><c r="F697" s="2" t="inlineStr"><is><t>symeprewir</t></is></c><c r="G697" s="2" t="inlineStr"><is><t>ledipaswir</t></is></c><c r="H697" s="2" t="inlineStr" /><c r="I697" s="2" t="inlineStr" /><c r="J697" s="2" t="inlineStr" /><c r="K697" s="2" t="inlineStr"><is><t>zydowudyna</t></is></c><c r="L697" s="2" t="inlineStr"><is><t>lamiwudyna</t></is></c><c r="M697" s="2" t="inlineStr" /><c r="N697" s="2" t="inlineStr" /><c r="O697" s="2" t="inlineStr" /><c r="P697" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q697" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="698"><c r="A698" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B698" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C698" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D698" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E698" s="2" t="inlineStr"><is><t>Metronidazol służy do leczenia:</t></is></c><c r="F698" s="2" t="inlineStr"><is><t>rzęsistkowicy (Trichomonas vaginalis)</t></is></c><c r="G698" s="2" t="inlineStr"><is><t>lambliozy (Giargia lamblia)</t></is></c><c r="H698" s="2" t="inlineStr" /><c r="I698" s="2" t="inlineStr" /><c r="J698" s="2" t="inlineStr" /><c r="K698" s="2" t="inlineStr"><is><t>toksoplazmozy (Toxoplasma godi)</t></is></c><c r="L698" s="2" t="inlineStr"><is><t>pneumocystozy (Pneumocystis jirovecii)</t></is></c><c r="M698" s="2" t="inlineStr" /><c r="N698" s="2" t="inlineStr" /><c r="O698" s="2" t="inlineStr" /><c r="P698" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q698" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="699"><c r="A699" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B699" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C699" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D699" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E699" s="2" t="inlineStr"><is><t>Do leków 2 fazy (kontynuacji) w leczeniu gruźlicy należą:</t></is></c><c r="F699" s="2" t="inlineStr"><is><t>izoniazyd</t></is></c><c r="G699" s="2" t="inlineStr"><is><t>ryfampicyna</t></is></c><c r="H699" s="2" t="inlineStr" /><c r="I699" s="2" t="inlineStr" /><c r="J699" s="2" t="inlineStr" /><c r="K699" s="2" t="inlineStr"><is><t>etambutol</t></is></c><c r="L699" s="2" t="inlineStr"><is><t>pirazynamid</t></is></c><c r="M699" s="2" t="inlineStr" /><c r="N699" s="2" t="inlineStr" /><c r="O699" s="2" t="inlineStr" /><c r="P699" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q699" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="700"><c r="A700" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B700" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C700" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D700" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E700" s="2" t="inlineStr"><is><t>Aktywność wobec dermatofitów ma:</t></is></c><c r="F700" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="G700" s="2" t="inlineStr"><is><t>amorolfina</t></is></c><c r="H700" s="2" t="inlineStr"><is><t>klotrymazol</t></is></c><c r="I700" s="2" t="inlineStr"><is><t>terbinafina</t></is></c><c r="J700" s="2" t="inlineStr" /><c r="K700" s="2" t="inlineStr" /><c r="L700" s="2" t="inlineStr" /><c r="M700" s="2" t="inlineStr" /><c r="N700" s="2" t="inlineStr" /><c r="O700" s="2" t="inlineStr" /><c r="P700" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q700" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="701"><c r="A701" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B701" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C701" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D701" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E701" s="2" t="inlineStr"><is><t>Cechą charakterystyczną dla azoli jest:</t></is></c><c r="F701" s="2" t="inlineStr"><is><t>hamowanie syntezy ergosterolu</t></is></c><c r="G701" s="2" t="inlineStr"><is><t>hamowanie izoenzymów CYP</t></is></c><c r="H701" s="2" t="inlineStr" /><c r="I701" s="2" t="inlineStr" /><c r="J701" s="2" t="inlineStr" /><c r="K701" s="2" t="inlineStr"><is><t>duże podobieństwo parametrów farmakokinetycznych leków tej grupy</t></is></c><c r="L701" s="2" t="inlineStr"><is><t>zależność ekspozycja-efekt typu fT&gt;MIC</t></is></c><c r="M701" s="2" t="inlineStr" /><c r="N701" s="2" t="inlineStr" /><c r="O701" s="2" t="inlineStr" /><c r="P701" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q701" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="702"><c r="A702" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B702" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C702" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D702" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E702" s="2" t="inlineStr"><is><t>Dobrą biodostępność po podaniu doustnym ma:</t></is></c><c r="F702" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="G702" s="2" t="inlineStr"><is><t>worykonazol</t></is></c><c r="H702" s="2" t="inlineStr" /><c r="I702" s="2" t="inlineStr" /><c r="J702" s="2" t="inlineStr" /><c r="K702" s="2" t="inlineStr"><is><t>amfoterycyna B</t></is></c><c r="L702" s="2" t="inlineStr"><is><t>pozakonazol</t></is></c><c r="M702" s="2" t="inlineStr" /><c r="N702" s="2" t="inlineStr" /><c r="O702" s="2" t="inlineStr" /><c r="P702" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q702" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="703"><c r="A703" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B703" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C703" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D703" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E703" s="2" t="inlineStr"><is><t>W kandydozie jamy ustnej (pleśniawkach) zastosować można:</t></is></c><c r="F703" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="G703" s="2" t="inlineStr"><is><t>nystatynę</t></is></c><c r="H703" s="2" t="inlineStr" /><c r="I703" s="2" t="inlineStr" /><c r="J703" s="2" t="inlineStr" /><c r="K703" s="2" t="inlineStr"><is><t>kwas borowy z gliceryną</t></is></c><c r="L703" s="2" t="inlineStr"><is><t>kaspofunginę</t></is></c><c r="M703" s="2" t="inlineStr" /><c r="N703" s="2" t="inlineStr" /><c r="O703" s="2" t="inlineStr" /><c r="P703" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q703" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="704"><c r="A704" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B704" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C704" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D704" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E704" s="2" t="inlineStr"><is><t>Spośród wymienionych glikokortykosteroidów stosowanych wziewnie w leczeniu chorób układu oddechowego w formie proleku dostępny jest:</t></is></c><c r="F704" s="2" t="inlineStr"><is><t>dipropionian beklometazonu</t></is></c><c r="G704" s="2" t="inlineStr"><is><t>cyklezonid</t></is></c><c r="H704" s="2" t="inlineStr" /><c r="I704" s="2" t="inlineStr" /><c r="J704" s="2" t="inlineStr" /><c r="K704" s="2" t="inlineStr"><is><t>budezonid</t></is></c><c r="L704" s="2" t="inlineStr"><is><t>propionian flutykazonu</t></is></c><c r="M704" s="2" t="inlineStr" /><c r="N704" s="2" t="inlineStr" /><c r="O704" s="2" t="inlineStr" /><c r="P704" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q704" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="705"><c r="A705" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B705" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C705" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D705" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E705" s="2" t="inlineStr"><is><t>Długodziałającym lekiem o wpływie na receptory komórkowe jest:</t></is></c><c r="F705" s="2" t="inlineStr"><is><t>bromek umeklidynium</t></is></c><c r="G705" s="2" t="inlineStr" /><c r="H705" s="2" t="inlineStr" /><c r="I705" s="2" t="inlineStr" /><c r="J705" s="2" t="inlineStr" /><c r="K705" s="2" t="inlineStr"><is><t>dornaza alfa</t></is></c><c r="L705" s="2" t="inlineStr"><is><t>nedokromil</t></is></c><c r="M705" s="2" t="inlineStr"><is><t>roflumilast</t></is></c><c r="N705" s="2" t="inlineStr" /><c r="O705" s="2" t="inlineStr" /><c r="P705" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q705" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="706"><c r="A706" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B706" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C706" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D706" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E706" s="2" t="inlineStr"><is><t>Unikalny profil działania klinicznego w swojej grupie farmakologicznej ma:</t></is></c><c r="F706" s="2" t="inlineStr"><is><t>formoterol</t></is></c><c r="G706" s="2" t="inlineStr"><is><t>celiprolol</t></is></c><c r="H706" s="2" t="inlineStr"><is><t>dekstrometorfan</t></is></c><c r="I706" s="2" t="inlineStr" /><c r="J706" s="2" t="inlineStr" /><c r="K706" s="2" t="inlineStr"><is><t>poraktant alfa</t></is></c><c r="L706" s="2" t="inlineStr" /><c r="M706" s="2" t="inlineStr" /><c r="N706" s="2" t="inlineStr" /><c r="O706" s="2" t="inlineStr" /><c r="P706" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q706" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="707"><c r="A707" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B707" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C707" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D707" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E707" s="2" t="inlineStr"><is><t>Do groźnych powikłań po podaniu ramiprylu może dojść w przypadku zastosowania leku u:</t></is></c><c r="F707" s="2" t="inlineStr"><is><t>20-letniej kobiety w ciąży</t></is></c><c r="G707" s="2" t="inlineStr"><is><t>35-letniej kobiety z obustronnym istotnym zwężeniem tętnic nerkowych w przebiegu dysplazji włóknistej</t></is></c><c r="H707" s="2" t="inlineStr" /><c r="I707" s="2" t="inlineStr" /><c r="J707" s="2" t="inlineStr" /><c r="K707" s="2" t="inlineStr"><is><t>70-letniego mężczyzny z POChP</t></is></c><c r="L707" s="2" t="inlineStr"><is><t>50-letniego mężczyzny ze źle kontrolowanym zespołem metabolicznym (otyłość, cukrzyca, nadciśnienie tętnicze, dyslipidemia), aktywnego palacza nikotyny b</t></is></c><c r="M707" s="2" t="inlineStr" /><c r="N707" s="2" t="inlineStr" /><c r="O707" s="2" t="inlineStr" /><c r="P707" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q707" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="708"><c r="A708" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B708" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C708" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D708" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E708" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące współczynnika T/P (trough-to-peak ratio):</t></is></c><c r="F708" s="2" t="inlineStr"><is><t>im większa dawka leku, tym lepszy T/P</t></is></c><c r="G708" s="2" t="inlineStr"><is><t>im dłuższy czas leczenia, tym lepszy T/P</t></is></c><c r="H708" s="2" t="inlineStr"><is><t>pożądany T/P jest większy od 0,75, a optymalny =1,0</t></is></c><c r="I708" s="2" t="inlineStr" /><c r="J708" s="2" t="inlineStr" /><c r="K708" s="2" t="inlineStr"><is><t>jest taki sam dla rozkurczowego i skurczowego ciśnienia tętniczego krwi</t></is></c><c r="L708" s="2" t="inlineStr" /><c r="M708" s="2" t="inlineStr" /><c r="N708" s="2" t="inlineStr" /><c r="O708" s="2" t="inlineStr" /><c r="P708" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q708" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="709"><c r="A709" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B709" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C709" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D709" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E709" s="2" t="inlineStr"><is><t>β – adrenolityki:</t></is></c><c r="F709" s="2" t="inlineStr"><is><t>zwalniają częstość rytmu serca, a przez to zapotrzebowanie serca na tlen</t></is></c><c r="G709" s="2" t="inlineStr" /><c r="H709" s="2" t="inlineStr" /><c r="I709" s="2" t="inlineStr" /><c r="J709" s="2" t="inlineStr" /><c r="K709" s="2" t="inlineStr"><is><t>zmniejszają ciśnienie tętnicze i w efekcie powodują spadek przepływu wieńcowego</t></is></c><c r="L709" s="2" t="inlineStr"><is><t>powodują wzrost stężenia glukozy we krwi i dlatego maskują objawy hipoglikemii</t></is></c><c r="M709" s="2" t="inlineStr"><is><t>powodują skurcz oskrzeli i dlatego są bezwzględnie przeciwwskazane w POChP</t></is></c><c r="N709" s="2" t="inlineStr" /><c r="O709" s="2" t="inlineStr" /><c r="P709" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q709" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="710"><c r="A710" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B710" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C710" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D710" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E710" s="2" t="inlineStr"><is><t>Zaburzenia widzenia powoduje:</t></is></c><c r="F710" s="2" t="inlineStr"><is><t>digoksyna</t></is></c><c r="G710" s="2" t="inlineStr"><is><t>sildenafil</t></is></c><c r="H710" s="2" t="inlineStr"><is><t>iwabradyna</t></is></c><c r="I710" s="2" t="inlineStr" /><c r="J710" s="2" t="inlineStr" /><c r="K710" s="2" t="inlineStr"><is><t>piracetam</t></is></c><c r="L710" s="2" t="inlineStr" /><c r="M710" s="2" t="inlineStr" /><c r="N710" s="2" t="inlineStr" /><c r="O710" s="2" t="inlineStr" /><c r="P710" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q710" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="711"><c r="A711" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B711" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C711" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D711" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E711" s="2" t="inlineStr"><is><t>Do kardiowersji farmakologicznej w migotaniu przedsionków stosuje się:</t></is></c><c r="F711" s="2" t="inlineStr"><is><t>amiodaron</t></is></c><c r="G711" s="2" t="inlineStr"><is><t>propafenon</t></is></c><c r="H711" s="2" t="inlineStr" /><c r="I711" s="2" t="inlineStr" /><c r="J711" s="2" t="inlineStr" /><c r="K711" s="2" t="inlineStr"><is><t>adenozynę</t></is></c><c r="L711" s="2" t="inlineStr"><is><t>lidokainę</t></is></c><c r="M711" s="2" t="inlineStr" /><c r="N711" s="2" t="inlineStr" /><c r="O711" s="2" t="inlineStr" /><c r="P711" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q711" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="712"><c r="A712" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B712" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C712" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D712" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E712" s="2" t="inlineStr"><is><t>Poprzez aktywację białkowej kinazy G via cGMP działa:</t></is></c><c r="F712" s="2" t="inlineStr"><is><t>nitroprusydek sodu</t></is></c><c r="G712" s="2" t="inlineStr"><is><t>sakubitryl</t></is></c><c r="H712" s="2" t="inlineStr"><is><t>riocyguat</t></is></c><c r="I712" s="2" t="inlineStr"><is><t>nesirytyd</t></is></c><c r="J712" s="2" t="inlineStr" /><c r="K712" s="2" t="inlineStr" /><c r="L712" s="2" t="inlineStr" /><c r="M712" s="2" t="inlineStr" /><c r="N712" s="2" t="inlineStr" /><c r="O712" s="2" t="inlineStr" /><c r="P712" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q712" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="713"><c r="A713" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B713" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C713" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D713" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E713" s="2" t="inlineStr"><is><t>Wybierz prawidłowy zestaw lek – wskazanie do stosowania:</t></is></c><c r="F713" s="2" t="inlineStr"><is><t>bupropion – uzależnienie od nikotyny</t></is></c><c r="G713" s="2" t="inlineStr"><is><t>atomoksetyna – ADHD (zespół nadpobudliwości z deficytem uwagi)</t></is></c><c r="H713" s="2" t="inlineStr"><is><t>lamotrygina - profilaktyka zaburzeń afektywnych dwubiegunowych</t></is></c><c r="I713" s="2" t="inlineStr" /><c r="J713" s="2" t="inlineStr" /><c r="K713" s="2" t="inlineStr"><is><t>agomelatyna – bezsenność krótkotrwała</t></is></c><c r="L713" s="2" t="inlineStr" /><c r="M713" s="2" t="inlineStr" /><c r="N713" s="2" t="inlineStr" /><c r="O713" s="2" t="inlineStr" /><c r="P713" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q713" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="714"><c r="A714" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B714" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C714" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D714" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E714" s="2" t="inlineStr"><is><t>Meghan skarżącej się na bezsenność, która związana jest ze stresem wywołanym planowanym wydarzeniem z jej udziałem emitowanym we wszystkich telewizjach świata za 2 tygodnie, przepiszesz:</t></is></c><c r="F714" s="2" t="inlineStr"><is><t>zaleplon</t></is></c><c r="G714" s="2" t="inlineStr" /><c r="H714" s="2" t="inlineStr" /><c r="I714" s="2" t="inlineStr" /><c r="J714" s="2" t="inlineStr" /><c r="K714" s="2" t="inlineStr"><is><t>diazepam</t></is></c><c r="L714" s="2" t="inlineStr"><is><t>mirtazapinę</t></is></c><c r="M714" s="2" t="inlineStr"><is><t>hydroksyzynę</t></is></c><c r="N714" s="2" t="inlineStr" /><c r="O714" s="2" t="inlineStr" /><c r="P714" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q714" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="715"><c r="A715" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B715" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C715" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D715" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E715" s="2" t="inlineStr"><is><t>Pozapsychiatryczne zastosowania leków przeciwdepresyjnych obejmują:</t></is></c><c r="F715" s="2" t="inlineStr"><is><t>ból neuropatyczny</t></is></c><c r="G715" s="2" t="inlineStr"><is><t>bezsenność przewlekłą po niepowodzeniu wprowadzenia zasad higieny snu</t></is></c><c r="H715" s="2" t="inlineStr" /><c r="I715" s="2" t="inlineStr" /><c r="J715" s="2" t="inlineStr" /><c r="K715" s="2" t="inlineStr"><is><t>otępienie naczyniopochodne</t></is></c><c r="L715" s="2" t="inlineStr"><is><t>przerywanie napadów migren</t></is></c><c r="M715" s="2" t="inlineStr" /><c r="N715" s="2" t="inlineStr" /><c r="O715" s="2" t="inlineStr" /><c r="P715" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q715" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="716"><c r="A716" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B716" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C716" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D716" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E716" s="2" t="inlineStr"><is><t>W leczeniu lęku uogólnionego zastosowanie ma:</t></is></c><c r="F716" s="2" t="inlineStr"><is><t>sertralina</t></is></c><c r="G716" s="2" t="inlineStr"><is><t>pregabalina</t></is></c><c r="H716" s="2" t="inlineStr"><is><t>buspiron</t></is></c><c r="I716" s="2" t="inlineStr" /><c r="J716" s="2" t="inlineStr" /><c r="K716" s="2" t="inlineStr"><is><t>klorazepat</t></is></c><c r="L716" s="2" t="inlineStr" /><c r="M716" s="2" t="inlineStr" /><c r="N716" s="2" t="inlineStr" /><c r="O716" s="2" t="inlineStr" /><c r="P716" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q716" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="717"><c r="A717" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B717" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C717" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D717" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E717" s="2" t="inlineStr"><is><t>W początkowym okresie leczenia depresji selektywnymi inhibitorami wychwytu zwrotnego serotoniny:</t></is></c><c r="F717" s="2" t="inlineStr"><is><t>mogą nasilać lęk, choć są uważane za leki przeciwlękowe podczas długotrwałej terapii</t></is></c><c r="G717" s="2" t="inlineStr"><is><t>częściej niż w późniejszym okresie terapii dochodzi do myśli lub prób samobójczych</t></is></c><c r="H717" s="2" t="inlineStr" /><c r="I717" s="2" t="inlineStr" /><c r="J717" s="2" t="inlineStr" /><c r="K717" s="2" t="inlineStr"><is><t>występują fluktuacje nastroju polegające na szybkiej poprawie, ale z okresami gwałtownych pogorszeń</t></is></c><c r="L717" s="2" t="inlineStr"><is><t>stosuje się równocześnie karbamazepinę aby zapobiec przejściu depresji w manię</t></is></c><c r="M717" s="2" t="inlineStr" /><c r="N717" s="2" t="inlineStr" /><c r="O717" s="2" t="inlineStr" /><c r="P717" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q717" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="718"><c r="A718" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B718" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C718" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D718" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E718" s="2" t="inlineStr"><is><t>Pacjentka od wielu lat otrzymuje perazynę, mianseryną i lorazepam. Na tej podstawie można rozpoznać:</t></is></c><c r="F718" s="2" t="inlineStr"><is><t>zaburzenia depresyjno-urojeniowe</t></is></c><c r="G718" s="2" t="inlineStr"><is><t>uzależnienie lekowe</t></is></c><c r="H718" s="2" t="inlineStr" /><c r="I718" s="2" t="inlineStr" /><c r="J718" s="2" t="inlineStr" /><c r="K718" s="2" t="inlineStr"><is><t>dwubiegunową chorobę afektywną</t></is></c><c r="L718" s="2" t="inlineStr"><is><t>fobię społeczną</t></is></c><c r="M718" s="2" t="inlineStr" /><c r="N718" s="2" t="inlineStr" /><c r="O718" s="2" t="inlineStr" /><c r="P718" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q718" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="719"><c r="A719" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B719" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C719" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D719" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E719" s="2" t="inlineStr"><is><t>Układ dopaminowy OUN aktywuje bezpośrednio:</t></is></c><c r="F719" s="2" t="inlineStr"><is><t>ropinirol</t></is></c><c r="G719" s="2" t="inlineStr"><is><t>metylfenidat</t></is></c><c r="H719" s="2" t="inlineStr" /><c r="I719" s="2" t="inlineStr" /><c r="J719" s="2" t="inlineStr" /><c r="K719" s="2" t="inlineStr"><is><t>piracetam</t></is></c><c r="L719" s="2" t="inlineStr"><is><t>kofeina</t></is></c><c r="M719" s="2" t="inlineStr" /><c r="N719" s="2" t="inlineStr" /><c r="O719" s="2" t="inlineStr" /><c r="P719" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q719" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="720"><c r="A720" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B720" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C720" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D720" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E720" s="2" t="inlineStr"><is><t>Przy stosowaniu neuroleptyków największe ryzyko przyrostu masy ciała dotyczy:</t></is></c><c r="F720" s="2" t="inlineStr"><is><t>chlorpromazyny</t></is></c><c r="G720" s="2" t="inlineStr"><is><t>olanzapiny</t></is></c><c r="H720" s="2" t="inlineStr" /><c r="I720" s="2" t="inlineStr" /><c r="J720" s="2" t="inlineStr" /><c r="K720" s="2" t="inlineStr"><is><t>arypiprazolu</t></is></c><c r="L720" s="2" t="inlineStr"><is><t>haloperidolu</t></is></c><c r="M720" s="2" t="inlineStr" /><c r="N720" s="2" t="inlineStr" /><c r="O720" s="2" t="inlineStr" /><c r="P720" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q720" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="721"><c r="A721" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B721" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C721" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D721" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E721" s="2" t="inlineStr"><is><t>Na acetylocholinestarazę ma wpływ:</t></is></c><c r="F721" s="2" t="inlineStr"><is><t>neostygmina</t></is></c><c r="G721" s="2" t="inlineStr"><is><t>donepezil</t></is></c><c r="H721" s="2" t="inlineStr" /><c r="I721" s="2" t="inlineStr" /><c r="J721" s="2" t="inlineStr" /><c r="K721" s="2" t="inlineStr"><is><t>suksametonium</t></is></c><c r="L721" s="2" t="inlineStr"><is><t>tropikamid</t></is></c><c r="M721" s="2" t="inlineStr" /><c r="N721" s="2" t="inlineStr" /><c r="O721" s="2" t="inlineStr" /><c r="P721" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q721" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="722"><c r="A722" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B722" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C722" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D722" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E722" s="2" t="inlineStr"><is><t>Hiponatremia polekowa może być rozpoznana podczas stosowania:</t></is></c><c r="F722" s="2" t="inlineStr"><is><t>torasemidu</t></is></c><c r="G722" s="2" t="inlineStr"><is><t>indapamidu</t></is></c><c r="H722" s="2" t="inlineStr"><is><t>karbamazepiny</t></is></c><c r="I722" s="2" t="inlineStr" /><c r="J722" s="2" t="inlineStr" /><c r="K722" s="2" t="inlineStr"><is><t>tolwaptanu</t></is></c><c r="L722" s="2" t="inlineStr" /><c r="M722" s="2" t="inlineStr" /><c r="N722" s="2" t="inlineStr" /><c r="O722" s="2" t="inlineStr" /><c r="P722" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q722" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="723"><c r="A723" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B723" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C723" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D723" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E723" s="2" t="inlineStr"><is><t>Czy na podstawie informacji o stosowaniu leku można jednoznacznie postawić wymienione rozpoznanie?</t></is></c><c r="F723" s="2" t="inlineStr"><is><t>fingolimod – stwardnienie rozsiane</t></is></c><c r="G723" s="2" t="inlineStr"><is><t>memantyna – choroba Alzheimera</t></is></c><c r="H723" s="2" t="inlineStr" /><c r="I723" s="2" t="inlineStr" /><c r="J723" s="2" t="inlineStr" /><c r="K723" s="2" t="inlineStr"><is><t>kwas walproinowy – padaczka</t></is></c><c r="L723" s="2" t="inlineStr"><is><t>pregabalina – polineuropatia cukrzycowa</t></is></c><c r="M723" s="2" t="inlineStr" /><c r="N723" s="2" t="inlineStr" /><c r="O723" s="2" t="inlineStr" /><c r="P723" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q723" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="724"><c r="A724" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B724" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C724" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D724" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E724" s="2" t="inlineStr"><is><t>Które z powyższych stwierdzeń jest prawdziwe?</t></is></c><c r="F724" s="2" t="inlineStr"><is><t>podczas leczenia takalcytolem należy monitorować stężenie wapnia w moczu</t></is></c><c r="G724" s="2" t="inlineStr"><is><t>metoksalen powinno się podawać 1-2 h przed planowaną ekspozycją na promieniowanie UVA</t></is></c><c r="H724" s="2" t="inlineStr"><is><t>nadtlenek benzoilu ma zastosowanie w leczeniu trądziku</t></is></c><c r="I724" s="2" t="inlineStr" /><c r="J724" s="2" t="inlineStr" /><c r="K724" s="2" t="inlineStr"><is><t>podczas stosowania acytretyny skuteczną antykoncepcję należy stosować przez miesiąc po zakończeniu terapii</t></is></c><c r="L724" s="2" t="inlineStr" /><c r="M724" s="2" t="inlineStr" /><c r="N724" s="2" t="inlineStr" /><c r="O724" s="2" t="inlineStr" /><c r="P724" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q724" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="725"><c r="A725" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B725" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C725" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D725" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E725" s="2" t="inlineStr"><is><t>Doping genetyczny może dotyczyć genu kodującego:</t></is></c><c r="F725" s="2" t="inlineStr"><is><t>enzym konwertujący angiotensynę</t></is></c><c r="G725" s="2" t="inlineStr"><is><t>erytropoetynę</t></is></c><c r="H725" s="2" t="inlineStr"><is><t>kolagen</t></is></c><c r="I725" s="2" t="inlineStr"><is><t>hormon wzrostu</t></is></c><c r="J725" s="2" t="inlineStr" /><c r="K725" s="2" t="inlineStr" /><c r="L725" s="2" t="inlineStr" /><c r="M725" s="2" t="inlineStr" /><c r="N725" s="2" t="inlineStr" /><c r="O725" s="2" t="inlineStr" /><c r="P725" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q725" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="726"><c r="A726" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B726" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C726" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D726" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E726" s="2" t="inlineStr"><is><t>Terapia genowa w okulistyce ma zastosowanie w leczeniu:</t></is></c><c r="F726" s="2" t="inlineStr"><is><t>zwyrodnienia barwnikowego siatkówki (retinitis pigmentosa)</t></is></c><c r="G726" s="2" t="inlineStr" /><c r="H726" s="2" t="inlineStr" /><c r="I726" s="2" t="inlineStr" /><c r="J726" s="2" t="inlineStr" /><c r="K726" s="2" t="inlineStr"><is><t>jaskry</t></is></c><c r="L726" s="2" t="inlineStr"><is><t>zapalenia współczulnego oka</t></is></c><c r="M726" s="2" t="inlineStr"><is><t>choroby Besta</t></is></c><c r="N726" s="2" t="inlineStr" /><c r="O726" s="2" t="inlineStr" /><c r="P726" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q726" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="727"><c r="A727" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B727" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C727" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D727" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E727" s="2" t="inlineStr"><is><t>W leczeniu astmy używane są wziewne postaci:</t></is></c><c r="F727" s="2" t="inlineStr"><is><t>propionianu flutykazonu</t></is></c><c r="G727" s="2" t="inlineStr"><is><t>indakaterolu</t></is></c><c r="H727" s="2" t="inlineStr" /><c r="I727" s="2" t="inlineStr" /><c r="J727" s="2" t="inlineStr" /><c r="K727" s="2" t="inlineStr"><is><t>montelukastu</t></is></c><c r="L727" s="2" t="inlineStr"><is><t>acetylocysteiny</t></is></c><c r="M727" s="2" t="inlineStr" /><c r="N727" s="2" t="inlineStr" /><c r="O727" s="2" t="inlineStr" /><c r="P727" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q727" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="728"><c r="A728" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B728" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C728" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D728" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E728" s="2" t="inlineStr"><is><t>U małego dziecka wygodną formą podania leku wziewnego jest:</t></is></c><c r="F728" s="2" t="inlineStr"><is><t>pomocnicze użycie komory inhalacyjnej, tzw. spacera</t></is></c><c r="G728" s="2" t="inlineStr"><is><t>nebulizacja</t></is></c><c r="H728" s="2" t="inlineStr" /><c r="I728" s="2" t="inlineStr" /><c r="J728" s="2" t="inlineStr" /><c r="K728" s="2" t="inlineStr"><is><t>inhalacja z inhalatora suchego proszku</t></is></c><c r="L728" s="2" t="inlineStr"><is><t>inhalacja z dozownika ciśnieniowego</t></is></c><c r="M728" s="2" t="inlineStr" /><c r="N728" s="2" t="inlineStr" /><c r="O728" s="2" t="inlineStr" /><c r="P728" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q728" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="729"><c r="A729" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B729" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C729" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D729" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E729" s="2" t="inlineStr"><is><t>Chorzy na pierwotne nadciśnienie tętnicze z towarzyszącą cukrzycą największe korzyści osiągają z zastosowania:</t></is></c><c r="F729" s="2" t="inlineStr"><is><t>ramiprylu</t></is></c><c r="G729" s="2" t="inlineStr"><is><t>telmisartanu</t></is></c><c r="H729" s="2" t="inlineStr" /><c r="I729" s="2" t="inlineStr" /><c r="J729" s="2" t="inlineStr" /><c r="K729" s="2" t="inlineStr"><is><t>metoprololu</t></is></c><c r="L729" s="2" t="inlineStr"><is><t>hydrochlorotiazydu</t></is></c><c r="M729" s="2" t="inlineStr" /><c r="N729" s="2" t="inlineStr" /><c r="O729" s="2" t="inlineStr" /><c r="P729" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q729" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="730"><c r="A730" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B730" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C730" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D730" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E730" s="2" t="inlineStr"><is><t>Istotnym działaniem niepożądanym inhibitorów konwertazy angiotensyny jest:</t></is></c><c r="F730" s="2" t="inlineStr"><is><t>kaszel</t></is></c><c r="G730" s="2" t="inlineStr"><is><t>obrzęk naczynioruchowy</t></is></c><c r="H730" s="2" t="inlineStr" /><c r="I730" s="2" t="inlineStr" /><c r="J730" s="2" t="inlineStr" /><c r="K730" s="2" t="inlineStr"><is><t>hipokaliemia</t></is></c><c r="L730" s="2" t="inlineStr"><is><t>nasilenie białkomoczu</t></is></c><c r="M730" s="2" t="inlineStr" /><c r="N730" s="2" t="inlineStr" /><c r="O730" s="2" t="inlineStr" /><c r="P730" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q730" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="731"><c r="A731" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B731" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C731" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D731" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E731" s="2" t="inlineStr"><is><t>Wybierz prawidłowe pary lek – efekt działania:</t></is></c><c r="F731" s="2" t="inlineStr"><is><t>torasemid - hiperurykemia</t></is></c><c r="G731" s="2" t="inlineStr"><is><t>indapamid - hiponatremia</t></is></c><c r="H731" s="2" t="inlineStr" /><c r="I731" s="2" t="inlineStr" /><c r="J731" s="2" t="inlineStr" /><c r="K731" s="2" t="inlineStr"><is><t>mannitol – hiperglikemia</t></is></c><c r="L731" s="2" t="inlineStr"><is><t>eplerenon - hipokaliemia</t></is></c><c r="M731" s="2" t="inlineStr" /><c r="N731" s="2" t="inlineStr" /><c r="O731" s="2" t="inlineStr" /><c r="P731" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q731" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="732"><c r="A732" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B732" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C732" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D732" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E732" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące digoksyny:</t></is></c><c r="F732" s="2" t="inlineStr"><is><t>jest wskazana u pacjentów z niewydolnością serca i migotaniem przedsionków</t></is></c><c r="G732" s="2" t="inlineStr"><is><t>zmniejsza chorobowość pacjentów z niewydolnością serca</t></is></c><c r="H732" s="2" t="inlineStr" /><c r="I732" s="2" t="inlineStr" /><c r="J732" s="2" t="inlineStr" /><c r="K732" s="2" t="inlineStr"><is><t>poprawia przeżycie chorych z niewydolnością serca</t></is></c><c r="L732" s="2" t="inlineStr"><is><t>jest pozbawiona działania proarytmicznego</t></is></c><c r="M732" s="2" t="inlineStr" /><c r="N732" s="2" t="inlineStr" /><c r="O732" s="2" t="inlineStr" /><c r="P732" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q732" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="733"><c r="A733" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B733" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C733" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D733" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E733" s="2" t="inlineStr"><is><t>Wskaż prawdziwe zdanie dotyczące leczenia niewydolności serca:</t></is></c><c r="F733" s="2" t="inlineStr"><is><t>enalapryl przez zniesienie niekorzystnej adaptacji zmniejsza umieralność chorych ze skurczową niewydolnością serca</t></is></c><c r="G733" s="2" t="inlineStr"><is><t>karwedilol przez zniesienie niekorzystnej adaptacji zmniejsza umieralność chorych ze skurczową niewydolnością serca</t></is></c><c r="H733" s="2" t="inlineStr"><is><t>leki moczopędne są zalecane w celu zmniejszenia objawów i poprawy wydolności wysiłkowej u pacjentów z objawami zastoju</t></is></c><c r="I733" s="2" t="inlineStr" /><c r="J733" s="2" t="inlineStr" /><c r="K733" s="2" t="inlineStr"><is><t>statyny powinny być stosowane rutynowo u wszystkich chorych z niewydolnością mięśnia sercowego</t></is></c><c r="L733" s="2" t="inlineStr" /><c r="M733" s="2" t="inlineStr" /><c r="N733" s="2" t="inlineStr" /><c r="O733" s="2" t="inlineStr" /><c r="P733" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q733" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="734"><c r="A734" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B734" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C734" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D734" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E734" s="2" t="inlineStr"><is><t>Do leków przeciwskazanych u pacjentów z niewydolnością serca należy:</t></is></c><c r="F734" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="G734" s="2" t="inlineStr"><is><t>ketoprofen</t></is></c><c r="H734" s="2" t="inlineStr" /><c r="I734" s="2" t="inlineStr" /><c r="J734" s="2" t="inlineStr" /><c r="K734" s="2" t="inlineStr"><is><t>nebiwolol</t></is></c><c r="L734" s="2" t="inlineStr"><is><t>iwabradyna</t></is></c><c r="M734" s="2" t="inlineStr" /><c r="N734" s="2" t="inlineStr" /><c r="O734" s="2" t="inlineStr" /><c r="P734" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q734" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="735"><c r="A735" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B735" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C735" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D735" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E735" s="2" t="inlineStr"><is><t>W postaci naczynioskurczowej choroby niedokrwiennej serca przeciwwskazane jest stosowanie:</t></is></c><c r="F735" s="2" t="inlineStr"><is><t>metoprololu</t></is></c><c r="G735" s="2" t="inlineStr" /><c r="H735" s="2" t="inlineStr" /><c r="I735" s="2" t="inlineStr" /><c r="J735" s="2" t="inlineStr" /><c r="K735" s="2" t="inlineStr"><is><t>diltiazemu</t></is></c><c r="L735" s="2" t="inlineStr"><is><t>diazotanu izosorbidu</t></is></c><c r="M735" s="2" t="inlineStr"><is><t>werapamilu</t></is></c><c r="N735" s="2" t="inlineStr" /><c r="O735" s="2" t="inlineStr" /><c r="P735" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q735" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="736"><c r="A736" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B736" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C736" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D736" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E736" s="2" t="inlineStr"><is><t>Do działań niepożądanych amiodaronu należy:</t></is></c><c r="F736" s="2" t="inlineStr"><is><t>hipotonia</t></is></c><c r="G736" s="2" t="inlineStr"><is><t>fotosensytyzacja</t></is></c><c r="H736" s="2" t="inlineStr"><is><t>śródmiąższowe zapalenie płuc</t></is></c><c r="I736" s="2" t="inlineStr" /><c r="J736" s="2" t="inlineStr" /><c r="K736" s="2" t="inlineStr"><is><t>tachykardia</t></is></c><c r="L736" s="2" t="inlineStr" /><c r="M736" s="2" t="inlineStr" /><c r="N736" s="2" t="inlineStr" /><c r="O736" s="2" t="inlineStr" /><c r="P736" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q736" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="737"><c r="A737" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B737" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C737" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D737" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E737" s="2" t="inlineStr"><is><t>Lekiem rozkurczającym tętnice pozawieńcowe jest:</t></is></c><c r="F737" s="2" t="inlineStr"><is><t>nicergolina</t></is></c><c r="G737" s="2" t="inlineStr"><is><t>alprostadyl</t></is></c><c r="H737" s="2" t="inlineStr"><is><t>fentolamina</t></is></c><c r="I737" s="2" t="inlineStr"><is><t>cilostazol</t></is></c><c r="J737" s="2" t="inlineStr" /><c r="K737" s="2" t="inlineStr" /><c r="L737" s="2" t="inlineStr" /><c r="M737" s="2" t="inlineStr" /><c r="N737" s="2" t="inlineStr" /><c r="O737" s="2" t="inlineStr" /><c r="P737" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q737" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="738"><c r="A738" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B738" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C738" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D738" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E738" s="2" t="inlineStr"><is><t>Midazolam może być stosowany zgodnie z aktualną wiedzą:</t></is></c><c r="F738" s="2" t="inlineStr"><is><t>doustnie do sedacji w premedykacji przed zabiegami chirurgicznymi</t></is></c><c r="G738" s="2" t="inlineStr"><is><t>dożylnie w sedacji do nieprzyjemnych zabiegów diagnostycznych</t></is></c><c r="H738" s="2" t="inlineStr"><is><t>dożylnie w długotrwałej sedacji na oddziale intensywnej opieki medycznej</t></is></c><c r="I738" s="2" t="inlineStr" /><c r="J738" s="2" t="inlineStr" /><c r="K738" s="2" t="inlineStr"><is><t>doustnie w przewlekłym leczeniu bezsenności</t></is></c><c r="L738" s="2" t="inlineStr" /><c r="M738" s="2" t="inlineStr" /><c r="N738" s="2" t="inlineStr" /><c r="O738" s="2" t="inlineStr" /><c r="P738" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q738" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="739"><c r="A739" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B739" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C739" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D739" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E739" s="2" t="inlineStr"><is><t>W zaburzeniach lękowych można racjonalnie zastosować:</t></is></c><c r="F739" s="2" t="inlineStr"><is><t>escitalopram</t></is></c><c r="G739" s="2" t="inlineStr"><is><t>alprazolam</t></is></c><c r="H739" s="2" t="inlineStr" /><c r="I739" s="2" t="inlineStr" /><c r="J739" s="2" t="inlineStr" /><c r="K739" s="2" t="inlineStr"><is><t>baklofen</t></is></c><c r="L739" s="2" t="inlineStr"><is><t>moklobemid</t></is></c><c r="M739" s="2" t="inlineStr" /><c r="N739" s="2" t="inlineStr" /><c r="O739" s="2" t="inlineStr" /><c r="P739" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q739" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="740"><c r="A740" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B740" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C740" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D740" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E740" s="2" t="inlineStr"><is><t>Flumazenil to:</t></is></c><c r="F740" s="2" t="inlineStr"><is><t>antagonista receptora benzodiazepinowego</t></is></c><c r="G740" s="2" t="inlineStr"><is><t>antidotum w przedawkowaniu benzodiazepin</t></is></c><c r="H740" s="2" t="inlineStr" /><c r="I740" s="2" t="inlineStr" /><c r="J740" s="2" t="inlineStr" /><c r="K740" s="2" t="inlineStr"><is><t>odwrotny agonista receptora GABA-A</t></is></c><c r="L740" s="2" t="inlineStr"><is><t>antidotum w przedawkowaniu trójpierścieniowych leków przeciwdepresyjnych</t></is></c><c r="M740" s="2" t="inlineStr" /><c r="N740" s="2" t="inlineStr" /><c r="O740" s="2" t="inlineStr" /><c r="P740" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q740" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="741"><c r="A741" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B741" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C741" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D741" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E741" s="2" t="inlineStr"><is><t>Do krótkodziałających benzodiazepin należy:</t></is></c><c r="F741" s="2" t="inlineStr"><is><t>midazolam</t></is></c><c r="G741" s="2" t="inlineStr"><is><t>triazolam</t></is></c><c r="H741" s="2" t="inlineStr" /><c r="I741" s="2" t="inlineStr" /><c r="J741" s="2" t="inlineStr" /><c r="K741" s="2" t="inlineStr"><is><t>diazepam</t></is></c><c r="L741" s="2" t="inlineStr"><is><t>flunitrazepam</t></is></c><c r="M741" s="2" t="inlineStr" /><c r="N741" s="2" t="inlineStr" /><c r="O741" s="2" t="inlineStr" /><c r="P741" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q741" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="742"><c r="A742" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B742" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C742" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D742" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E742" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek – mechanizm działania:</t></is></c><c r="F742" s="2" t="inlineStr"><is><t>Iwabradyna – zahamowanie prądu potasowego w węźle przedsionkowo￾komorowym</t></is></c><c r="G742" s="2" t="inlineStr"><is><t>Sakubitril – zahamowanie aktywności neprylizyny</t></is></c><c r="H742" s="2" t="inlineStr"><is><t>Riociguat – aktywacja cyklazy adenylowej</t></is></c><c r="I742" s="2" t="inlineStr"><is><t>Digoksyna – aktywacja wymiennika sodowo-wapniowego</t></is></c><c r="J742" s="2" t="inlineStr" /><c r="K742" s="2" t="inlineStr" /><c r="L742" s="2" t="inlineStr" /><c r="M742" s="2" t="inlineStr" /><c r="N742" s="2" t="inlineStr" /><c r="O742" s="2" t="inlineStr" /><c r="P742" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q742" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="743"><c r="A743" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B743" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C743" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D743" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E743" s="2" t="inlineStr"><is><t>Do działań niepożądanych neuroleptyków zalicza się:</t></is></c><c r="F743" s="2" t="inlineStr"><is><t>dyskinezy</t></is></c><c r="G743" s="2" t="inlineStr"><is><t>dysfunkcje seksualne</t></is></c><c r="H743" s="2" t="inlineStr" /><c r="I743" s="2" t="inlineStr" /><c r="J743" s="2" t="inlineStr" /><c r="K743" s="2" t="inlineStr"><is><t>skłonność do hazardu</t></is></c><c r="L743" s="2" t="inlineStr"><is><t>somnambulizm (sennowłóctwo)</t></is></c><c r="M743" s="2" t="inlineStr" /><c r="N743" s="2" t="inlineStr" /><c r="O743" s="2" t="inlineStr" /><c r="P743" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q743" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="744"><c r="A744" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B744" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C744" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D744" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E744" s="2" t="inlineStr"><is><t>Stężenie cholesterolu LDL w surowicy zwiększa:</t></is></c><c r="F744" s="2" t="inlineStr"><is><t>olanzapina</t></is></c><c r="G744" s="2" t="inlineStr"><is><t>rysperydon</t></is></c><c r="H744" s="2" t="inlineStr"><is><t>kwetiapina</t></is></c><c r="I744" s="2" t="inlineStr" /><c r="J744" s="2" t="inlineStr" /><c r="K744" s="2" t="inlineStr"><is><t>zyprazydon</t></is></c><c r="L744" s="2" t="inlineStr" /><c r="M744" s="2" t="inlineStr" /><c r="N744" s="2" t="inlineStr" /><c r="O744" s="2" t="inlineStr" /><c r="P744" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q744" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="745"><c r="A745" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B745" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C745" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D745" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E745" s="2" t="inlineStr"><is><t>Przez wpływ na prąd sodowy działa:</t></is></c><c r="F745" s="2" t="inlineStr"><is><t>okskarbazepina</t></is></c><c r="G745" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="H745" s="2" t="inlineStr"><is><t>lamotrygina</t></is></c><c r="I745" s="2" t="inlineStr" /><c r="J745" s="2" t="inlineStr" /><c r="K745" s="2" t="inlineStr"><is><t>pregabalina</t></is></c><c r="L745" s="2" t="inlineStr" /><c r="M745" s="2" t="inlineStr" /><c r="N745" s="2" t="inlineStr" /><c r="O745" s="2" t="inlineStr" /><c r="P745" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q745" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="746"><c r="A746" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B746" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C746" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D746" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E746" s="2" t="inlineStr"><is><t>W profilaktyce migreny wykazano skuteczność:</t></is></c><c r="F746" s="2" t="inlineStr"><is><t>kwasu walproinowego</t></is></c><c r="G746" s="2" t="inlineStr"><is><t>toksyny botulinowej (w migrenie występującej co najmniej 14 dni w miesiącu)</t></is></c><c r="H746" s="2" t="inlineStr"><is><t>topiramatu</t></is></c><c r="I746" s="2" t="inlineStr"><is><t>propranololu</t></is></c><c r="J746" s="2" t="inlineStr" /><c r="K746" s="2" t="inlineStr" /><c r="L746" s="2" t="inlineStr" /><c r="M746" s="2" t="inlineStr" /><c r="N746" s="2" t="inlineStr" /><c r="O746" s="2" t="inlineStr" /><c r="P746" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q746" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="747"><c r="A747" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B747" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C747" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D747" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E747" s="2" t="inlineStr"><is><t>W leczeniu bólu neuropatycznego stosuje się:</t></is></c><c r="F747" s="2" t="inlineStr"><is><t>wenlafaksynę</t></is></c><c r="G747" s="2" t="inlineStr"><is><t>duloksetynę</t></is></c><c r="H747" s="2" t="inlineStr"><is><t>amitryptylinę</t></is></c><c r="I747" s="2" t="inlineStr" /><c r="J747" s="2" t="inlineStr" /><c r="K747" s="2" t="inlineStr"><is><t>tianeptynę</t></is></c><c r="L747" s="2" t="inlineStr" /><c r="M747" s="2" t="inlineStr" /><c r="N747" s="2" t="inlineStr" /><c r="O747" s="2" t="inlineStr" /><c r="P747" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q747" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="748"><c r="A748" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B748" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C748" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D748" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E748" s="2" t="inlineStr"><is><t>W leczeniu łuszczycy stosuje się:</t></is></c><c r="F748" s="2" t="inlineStr"><is><t>preparaty dziegciowe</t></is></c><c r="G748" s="2" t="inlineStr"><is><t>adapalen</t></is></c><c r="H748" s="2" t="inlineStr"><is><t>adalimumab</t></is></c><c r="I748" s="2" t="inlineStr" /><c r="J748" s="2" t="inlineStr" /><c r="K748" s="2" t="inlineStr"><is><t>kwas azelainowy</t></is></c><c r="L748" s="2" t="inlineStr" /><c r="M748" s="2" t="inlineStr" /><c r="N748" s="2" t="inlineStr" /><c r="O748" s="2" t="inlineStr" /><c r="P748" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q748" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="749"><c r="A749" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B749" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C749" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D749" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E749" s="2" t="inlineStr"><is><t>Działanie niepożądane sterydów anabolicznych to:</t></is></c><c r="F749" s="2" t="inlineStr"><is><t>uszkodzenie ścięgien</t></is></c><c r="G749" s="2" t="inlineStr"><is><t>wzrost hematokrytu</t></is></c><c r="H749" s="2" t="inlineStr"><is><t>łysienie</t></is></c><c r="I749" s="2" t="inlineStr"><is><t>ginekomastia</t></is></c><c r="J749" s="2" t="inlineStr" /><c r="K749" s="2" t="inlineStr" /><c r="L749" s="2" t="inlineStr" /><c r="M749" s="2" t="inlineStr" /><c r="N749" s="2" t="inlineStr" /><c r="O749" s="2" t="inlineStr" /><c r="P749" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q749" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="750"><c r="A750" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B750" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C750" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D750" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E750" s="2" t="inlineStr"><is><t>Kwas walproinowy:</t></is></c><c r="F750" s="2" t="inlineStr"><is><t>może powodować zwiększenie masy ciała</t></is></c><c r="G750" s="2" t="inlineStr"><is><t>nie powinien być stosowany u ciężarnych</t></is></c><c r="H750" s="2" t="inlineStr"><is><t>może być zastosowany w profilaktyce dwubiegunowej choroby afektywnej</t></is></c><c r="I750" s="2" t="inlineStr" /><c r="J750" s="2" t="inlineStr" /><c r="K750" s="2" t="inlineStr"><is><t>jest induktorem izoenzymów CYP</t></is></c><c r="L750" s="2" t="inlineStr" /><c r="M750" s="2" t="inlineStr" /><c r="N750" s="2" t="inlineStr" /><c r="O750" s="2" t="inlineStr" /><c r="P750" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q750" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="751"><c r="A751" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B751" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C751" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D751" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E751" s="2" t="inlineStr"><is><t>W terapii jaskry pierwotnej otwartego kąta można zastosować:</t></is></c><c r="F751" s="2" t="inlineStr"><is><t>timolol</t></is></c><c r="G751" s="2" t="inlineStr"><is><t>dorzolamid</t></is></c><c r="H751" s="2" t="inlineStr"><is><t>betaksolol</t></is></c><c r="I751" s="2" t="inlineStr"><is><t>latanoprost</t></is></c><c r="J751" s="2" t="inlineStr" /><c r="K751" s="2" t="inlineStr" /><c r="L751" s="2" t="inlineStr" /><c r="M751" s="2" t="inlineStr" /><c r="N751" s="2" t="inlineStr" /><c r="O751" s="2" t="inlineStr" /><c r="P751" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q751" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="752"><c r="A752" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B752" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C752" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D752" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E752" s="2" t="inlineStr"><is><t>Wskazaniem do stosowania bisfosfonianów jest:</t></is></c><c r="F752" s="2" t="inlineStr"><is><t>osteoporoza posteroidowa</t></is></c><c r="G752" s="2" t="inlineStr"><is><t>ból z powodu osteolitycznych przerzutów nowotworowych do kości</t></is></c><c r="H752" s="2" t="inlineStr" /><c r="I752" s="2" t="inlineStr" /><c r="J752" s="2" t="inlineStr" /><c r="K752" s="2" t="inlineStr"><is><t>ciężka hiperkaliemia</t></is></c><c r="L752" s="2" t="inlineStr"><is><t>ciężka hipokalcemia</t></is></c><c r="M752" s="2" t="inlineStr" /><c r="N752" s="2" t="inlineStr" /><c r="O752" s="2" t="inlineStr" /><c r="P752" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q752" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="753"><c r="A753" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B753" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C753" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D753" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E753" s="2" t="inlineStr"><is><t>Korzystne cechy leku przeciwhistaminowego stosowanego do leczenia przewlekłego alergicznego nieżytu nosa to:</t></is></c><c r="F753" s="2" t="inlineStr"><is><t>utrudnione przechodzenie do ośrodkowego układu nerwowego</t></is></c><c r="G753" s="2" t="inlineStr" /><c r="H753" s="2" t="inlineStr" /><c r="I753" s="2" t="inlineStr" /><c r="J753" s="2" t="inlineStr" /><c r="K753" s="2" t="inlineStr"><is><t>krótki czas działania 3-6 godzin</t></is></c><c r="L753" s="2" t="inlineStr"><is><t>działanie cholinolityczne</t></is></c><c r="M753" s="2" t="inlineStr"><is><t>zdolność do kumulacji w tkankach obwodowych</t></is></c><c r="N753" s="2" t="inlineStr" /><c r="O753" s="2" t="inlineStr" /><c r="P753" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q753" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="754"><c r="A754" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B754" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C754" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D754" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E754" s="2" t="inlineStr"><is><t>Wskaż prawidłowe ordynacje lekarskie:</t></is></c><c r="F754" s="2" t="inlineStr"><is><t>biegunka o etiologii Clostridium difficile o nieciężkim przebiegu – metronidazol przez 10 dni</t></is></c><c r="G754" s="2" t="inlineStr" /><c r="H754" s="2" t="inlineStr" /><c r="I754" s="2" t="inlineStr" /><c r="J754" s="2" t="inlineStr" /><c r="K754" s="2" t="inlineStr"><is><t>nosicielstwo Klebsiella pneumoniae ESBL (+) w przewodzie pokarmowym – meropenem przez 5 dni</t></is></c><c r="L754" s="2" t="inlineStr"><is><t>posiew krwi Streptococcus epidermidis oporny na metycylinę (MR) w butelce tlenowej i beztlenowej u pacjenta niegorączkującego, leukocyty = 8,9 G/l (N 4-10 G/L), CRP – 100 mg/l (N do 10 mg/l), prokalcytonina = 0,01 ng/ml (N do 0,5ng/ml) – wankomycyna przez 3 tygodnie</t></is></c><c r="M754" s="2" t="inlineStr"><is><t>posiew moczu Escherichia coli &gt; 10 5 jtk/ml (cfu/ml) u pacjentki z objawami dysurycznymi – imipenem + cilastatyna z powodu najniższej wartości MIC wg antybiogramu przez 3 dni</t></is></c><c r="N754" s="2" t="inlineStr" /><c r="O754" s="2" t="inlineStr" /><c r="P754" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q754" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="755"><c r="A755" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B755" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C755" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D755" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E755" s="2" t="inlineStr"><is><t>Kobieta z zakażeniem Enteroccocus faecium opornym na glikopeptydy (VRE) jest leczona lekiem przeciwbakteryjnym wiążącym się z jednostką 50S rybosomu bakteryjnego. Zaznacz prawdziwe informacje dotyczące tego leku:</t></is></c><c r="F755" s="2" t="inlineStr"><is><t>podczas jego stosowania &gt;10 dni może dojść do rozwoju trombocytopenii</t></is></c><c r="G755" s="2" t="inlineStr"><is><t>może być bezpiecznie stosowany u pacjentów leczonych lekami blokującymi CYP3A4, ponieważ nie wchodzi z nimi w interakcje</t></is></c><c r="H755" s="2" t="inlineStr" /><c r="I755" s="2" t="inlineStr" /><c r="J755" s="2" t="inlineStr" /><c r="K755" s="2" t="inlineStr"><is><t>jego działanie przeciwbakteryjne zależy od stężenia maksymalnego</t></is></c><c r="L755" s="2" t="inlineStr"><is><t>może być bezpiecznie zastosowany w trakcie leczenia inhibitorami wychwytu zwrotnego serotoniny, ponieważ nie wchodzi z nimi w interakcje</t></is></c><c r="M755" s="2" t="inlineStr" /><c r="N755" s="2" t="inlineStr" /><c r="O755" s="2" t="inlineStr" /><c r="P755" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q755" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="756"><c r="A756" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B756" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C756" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D756" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E756" s="2" t="inlineStr"><is><t>60-letnia kobieta z domowym zapaleniem płuc, w skali CURB-65 = 0 pkt jest leczona zgodnie ze standardem postępowania uwzględniającym dominującą etiologię tego zakażenia u osób dorosłych. Zaznacz prawdziwe informacje dotyczące tego leczenia:</t></is></c><c r="F756" s="2" t="inlineStr"><is><t>wymaga stałych optymalnych przedziałów dawkowania w ciągu całej doby</t></is></c><c r="G756" s="2" t="inlineStr"><is><t>w razie nadwrażliwości na leczenie początkowe w wywiadach wskazane jest zastosowanie lewofloksacyny lub moksyfloksacyny</t></is></c><c r="H756" s="2" t="inlineStr" /><c r="I756" s="2" t="inlineStr" /><c r="J756" s="2" t="inlineStr" /><c r="K756" s="2" t="inlineStr"><is><t>konieczne jest leczenie skojarzone 2 lekami przeciwbakteryjnymi o różnych mechanizmach działania</t></is></c><c r="L756" s="2" t="inlineStr"><is><t>powinno trwać co najmniej 21 dni</t></is></c><c r="M756" s="2" t="inlineStr" /><c r="N756" s="2" t="inlineStr" /><c r="O756" s="2" t="inlineStr" /><c r="P756" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q756" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="757"><c r="A757" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B757" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C757" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D757" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E757" s="2" t="inlineStr"><is><t>Amoksycylina z kwasem klawulanowym jest powszechnie stosowanym połączeniem antybiotykowym, które ma jednak ograniczenia. Wskaż istotne wady tego połączenia:</t></is></c><c r="F757" s="2" t="inlineStr"><is><t>aktywność wobec fizjologicznego mikrobiomu przewodu pokarmowego człowieka</t></is></c><c r="G757" s="2" t="inlineStr"><is><t>zależne od kwasu klawulanowego biegunka i uszkodzenie wątroby</t></is></c><c r="H757" s="2" t="inlineStr"><is><t>konieczność korekty dawki proporcjonalnie do eGFR (wskaźnika filtracji kłębuszkowej)</t></is></c><c r="I757" s="2" t="inlineStr" /><c r="J757" s="2" t="inlineStr" /><c r="K757" s="2" t="inlineStr"><is><t>ograniczona biodostępność po podaniu doustnym</t></is></c><c r="L757" s="2" t="inlineStr" /><c r="M757" s="2" t="inlineStr" /><c r="N757" s="2" t="inlineStr" /><c r="O757" s="2" t="inlineStr" /><c r="P757" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q757" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="758"><c r="A758" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B758" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C758" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D758" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E758" s="2" t="inlineStr"><is><t>W zakażeniach dermatofitami stosuje się:</t></is></c><c r="F758" s="2" t="inlineStr"><is><t>klotrimazol</t></is></c><c r="G758" s="2" t="inlineStr"><is><t>terbinafinę</t></is></c><c r="H758" s="2" t="inlineStr"><is><t>itrakonazol</t></is></c><c r="I758" s="2" t="inlineStr" /><c r="J758" s="2" t="inlineStr" /><c r="K758" s="2" t="inlineStr"><is><t>natamycynę</t></is></c><c r="L758" s="2" t="inlineStr" /><c r="M758" s="2" t="inlineStr" /><c r="N758" s="2" t="inlineStr" /><c r="O758" s="2" t="inlineStr" /><c r="P758" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q758" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="759"><c r="A759" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B759" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C759" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D759" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E759" s="2" t="inlineStr"><is><t>Anidulafungina w odróżnieniu od amfoterycyny B:</t></is></c><c r="F759" s="2" t="inlineStr"><is><t>ma wąskie spektrum działania przeciwgrzybiczego</t></is></c><c r="G759" s="2" t="inlineStr"><is><t>działa poprzez zahamowanie syntezy ściany komórkowej grzyba</t></is></c><c r="H759" s="2" t="inlineStr"><is><t>nie powoduje uszkodzenia nerek</t></is></c><c r="I759" s="2" t="inlineStr" /><c r="J759" s="2" t="inlineStr" /><c r="K759" s="2" t="inlineStr"><is><t>w leczeniu inwazyjnej kandydozy podawana jest drogą dożylną</t></is></c><c r="L759" s="2" t="inlineStr" /><c r="M759" s="2" t="inlineStr" /><c r="N759" s="2" t="inlineStr" /><c r="O759" s="2" t="inlineStr" /><c r="P759" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q759" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="760"><c r="A760" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B760" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C760" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D760" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E760" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenia dotyczące inhibitorów neuraminidazy:</t></is></c><c r="F760" s="2" t="inlineStr"><is><t>są skuteczne wobec wirusa grypy A i B</t></is></c><c r="G760" s="2" t="inlineStr"><is><t>leczenie lekami tej grupy powinno być wdrożone do 48 h od początku objawów u nieszczepionych osób z grup ryzyka ciężkiego przebiegu grypy</t></is></c><c r="H760" s="2" t="inlineStr" /><c r="I760" s="2" t="inlineStr" /><c r="J760" s="2" t="inlineStr" /><c r="K760" s="2" t="inlineStr"><is><t>oseltamiwir ma działanie tylko w drogach oddechowych, a zanamiwir ogólnoustrojowe, co wiąże się ze sposobem podania tych leków</t></is></c><c r="L760" s="2" t="inlineStr"><is><t>są nieskuteczne wobec wirusa świńskiej grypy H1N1</t></is></c><c r="M760" s="2" t="inlineStr" /><c r="N760" s="2" t="inlineStr" /><c r="O760" s="2" t="inlineStr" /><c r="P760" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q760" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="761"><c r="A761" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B761" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C761" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D761" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E761" s="2" t="inlineStr"><is><t>Flukonazol zgodnie z aktualną widzą medyczną można zastosować w profilaktyce medycznej u:</t></is></c><c r="F761" s="2" t="inlineStr"><is><t>pacjentów z agranulocytozą przez czas jej trwania</t></is></c><c r="G761" s="2" t="inlineStr"><is><t>biorców przeszczepów wątroby w okresie okołoprzeszczepiennym</t></is></c><c r="H761" s="2" t="inlineStr" /><c r="I761" s="2" t="inlineStr" /><c r="J761" s="2" t="inlineStr" /><c r="K761" s="2" t="inlineStr"><is><t>pacjentów leczonych szerokospektralnymi lekami przeciwbakteryjnymi przez czas takiej antybiotykoterapii</t></is></c><c r="L761" s="2" t="inlineStr"><is><t>wszystkich pacjentów oddziałów intensywnej terapii</t></is></c><c r="M761" s="2" t="inlineStr" /><c r="N761" s="2" t="inlineStr" /><c r="O761" s="2" t="inlineStr" /><c r="P761" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q761" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="762"><c r="A762" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B762" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C762" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D762" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E762" s="2" t="inlineStr"><is><t>Intrygujące konsekwencje stosowania leków to:</t></is></c><c r="F762" s="2" t="inlineStr"><is><t>pomarańczowe łzy i pot podczas stosowania ryfampicyny</t></is></c><c r="G762" s="2" t="inlineStr"><is><t>widzenie przedmiotów w żółtych obwódkach, tzw. „halo”, podczas stosowania digoksyny</t></is></c><c r="H762" s="2" t="inlineStr"><is><t>lepsze wyniki sportowe podczas stosowania meldonium u zawodowych sportowców</t></is></c><c r="I762" s="2" t="inlineStr" /><c r="J762" s="2" t="inlineStr" /><c r="K762" s="2" t="inlineStr"><is><t>poprawa IQ podczas stosowania piracetamu u licealistów i studentów</t></is></c><c r="L762" s="2" t="inlineStr" /><c r="M762" s="2" t="inlineStr" /><c r="N762" s="2" t="inlineStr" /><c r="O762" s="2" t="inlineStr" /><c r="P762" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q762" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="763"><c r="A763" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B763" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C763" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D763" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E763" s="2" t="inlineStr"><is><t>Do antyseptyki na ranę zastosujesz:</t></is></c><c r="F763" s="2" t="inlineStr"><is><t>jodopowidon</t></is></c><c r="G763" s="2" t="inlineStr"><is><t>oktenidynę</t></is></c><c r="H763" s="2" t="inlineStr" /><c r="I763" s="2" t="inlineStr" /><c r="J763" s="2" t="inlineStr" /><c r="K763" s="2" t="inlineStr"><is><t>wodę utlenioną</t></is></c><c r="L763" s="2" t="inlineStr"><is><t>0,9% roztwór NaCl</t></is></c><c r="M763" s="2" t="inlineStr" /><c r="N763" s="2" t="inlineStr" /><c r="O763" s="2" t="inlineStr" /><c r="P763" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q763" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="764"><c r="A764" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B764" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C764" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D764" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E764" s="2" t="inlineStr"><is><t>W leczeniu astmy są stosowane leki z grupy:</t></is></c><c r="F764" s="2" t="inlineStr"><is><t>agonistów receptora glikokortykosteroidowego</t></is></c><c r="G764" s="2" t="inlineStr"><is><t>antagonistów receptora M 3</t></is></c><c r="H764" s="2" t="inlineStr" /><c r="I764" s="2" t="inlineStr" /><c r="J764" s="2" t="inlineStr" /><c r="K764" s="2" t="inlineStr"><is><t>przeciwciał monoklonalnych przeciwko receptorowi dla interleukiny 1 (IL-1)</t></is></c><c r="L764" s="2" t="inlineStr"><is><t>agonistów recepta leukotrienowego CysLT 1 (B)</t></is></c><c r="M764" s="2" t="inlineStr" /><c r="N764" s="2" t="inlineStr" /><c r="O764" s="2" t="inlineStr" /><c r="P764" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q764" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="765"><c r="A765" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B765" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C765" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D765" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E765" s="2" t="inlineStr"><is><t>Wskaż zestaw leków o identycznym molekularnym mechanizmie działania:</t></is></c><c r="F765" s="2" t="inlineStr"><is><t>acetylocysteina, mesna, erdosteina</t></is></c><c r="G765" s="2" t="inlineStr"><is><t>indekaterol, wilanterol, salbutamol</t></is></c><c r="H765" s="2" t="inlineStr"><is><t>tiotropium, glikopironium, umeklidynium</t></is></c><c r="I765" s="2" t="inlineStr" /><c r="J765" s="2" t="inlineStr" /><c r="K765" s="2" t="inlineStr"><is><t>zileuton, zafirlukast, cyklezonid</t></is></c><c r="L765" s="2" t="inlineStr" /><c r="M765" s="2" t="inlineStr" /><c r="N765" s="2" t="inlineStr" /><c r="O765" s="2" t="inlineStr" /><c r="P765" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q765" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="766"><c r="A766" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B766" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C766" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D766" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E766" s="2" t="inlineStr"><is><t>Obciążenie wstępne serca zmniejsza:</t></is></c><c r="F766" s="2" t="inlineStr"><is><t>triazotan izosorbidu</t></is></c><c r="G766" s="2" t="inlineStr"><is><t>torasemid</t></is></c><c r="H766" s="2" t="inlineStr" /><c r="I766" s="2" t="inlineStr" /><c r="J766" s="2" t="inlineStr" /><c r="K766" s="2" t="inlineStr"><is><t>amlodypina</t></is></c><c r="L766" s="2" t="inlineStr"><is><t>bisoprolol</t></is></c><c r="M766" s="2" t="inlineStr" /><c r="N766" s="2" t="inlineStr" /><c r="O766" s="2" t="inlineStr" /><c r="P766" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q766" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="767"><c r="A767" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B767" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C767" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D767" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E767" s="2" t="inlineStr"><is><t>Wskaż prawidłowe pary lek - działanie niepożądane:</t></is></c><c r="F767" s="2" t="inlineStr"><is><t>propafenon - epizody nieutrwalonego częstoskurczu komorowego</t></is></c><c r="G767" s="2" t="inlineStr"><is><t>adenozyna - ból w klatce piersiowej</t></is></c><c r="H767" s="2" t="inlineStr" /><c r="I767" s="2" t="inlineStr" /><c r="J767" s="2" t="inlineStr" /><c r="K767" s="2" t="inlineStr"><is><t>wernakalant - migotanie przedsionków</t></is></c><c r="L767" s="2" t="inlineStr"><is><t>sotalol – zwiększenie progu defibrylacji</t></is></c><c r="M767" s="2" t="inlineStr" /><c r="N767" s="2" t="inlineStr" /><c r="O767" s="2" t="inlineStr" /><c r="P767" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q767" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="768"><c r="A768" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B768" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C768" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D768" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E768" s="2" t="inlineStr"><is><t>Działanie inotropowe dodatnie i rozkurczające naczynia ma:</t></is></c><c r="F768" s="2" t="inlineStr"><is><t>lewosimendan</t></is></c><c r="G768" s="2" t="inlineStr"><is><t>dobutamina</t></is></c><c r="H768" s="2" t="inlineStr" /><c r="I768" s="2" t="inlineStr" /><c r="J768" s="2" t="inlineStr" /><c r="K768" s="2" t="inlineStr"><is><t>nebiwolol</t></is></c><c r="L768" s="2" t="inlineStr"><is><t>efedryna</t></is></c><c r="M768" s="2" t="inlineStr" /><c r="N768" s="2" t="inlineStr" /><c r="O768" s="2" t="inlineStr" /><c r="P768" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q768" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="769"><c r="A769" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B769" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C769" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D769" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E769" s="2" t="inlineStr"><is><t>Wskaż minusy leczenia lipofilnym beta-adrenolitykiem:</t></is></c><c r="F769" s="2" t="inlineStr"><is><t>zaburzenia potencji</t></is></c><c r="G769" s="2" t="inlineStr"><is><t>ograniczenie wydolności fizycznej</t></is></c><c r="H769" s="2" t="inlineStr"><is><t>zaburzenia lipidowe</t></is></c><c r="I769" s="2" t="inlineStr" /><c r="J769" s="2" t="inlineStr" /><c r="K769" s="2" t="inlineStr"><is><t>działanie proarytmiczne, w tym obniżenie progu migotania komór</t></is></c><c r="L769" s="2" t="inlineStr" /><c r="M769" s="2" t="inlineStr" /><c r="N769" s="2" t="inlineStr" /><c r="O769" s="2" t="inlineStr" /><c r="P769" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q769" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="770"><c r="A770" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B770" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C770" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D770" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E770" s="2" t="inlineStr"><is><t>U 70-letniego mężczyzny z przewlekłą niewydolnością żylną wspomagająco do kompresjoterapii zastosujesz:</t></is></c><c r="F770" s="2" t="inlineStr"><is><t>mikronizowaną diosminę + hesperydynę</t></is></c><c r="G770" s="2" t="inlineStr" /><c r="H770" s="2" t="inlineStr" /><c r="I770" s="2" t="inlineStr" /><c r="J770" s="2" t="inlineStr" /><c r="K770" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy w dawce antyagregacyjnej</t></is></c><c r="L770" s="2" t="inlineStr"><is><t>enoksaparynę w dawce profilaktycznej</t></is></c><c r="M770" s="2" t="inlineStr"><is><t>furosemid w dawce leczniczej</t></is></c><c r="N770" s="2" t="inlineStr" /><c r="O770" s="2" t="inlineStr" /><c r="P770" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q770" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="771"><c r="A771" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B771" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C771" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D771" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E771" s="2" t="inlineStr"><is><t>80-letniemu mężczyźnie przesypiającemu w nocy 5 h, uskarżającemu na trudności z zasypianiem należy zalecić:</t></is></c><c r="F771" s="2" t="inlineStr"><is><t>zasady higieny snu</t></is></c><c r="G771" s="2" t="inlineStr" /><c r="H771" s="2" t="inlineStr" /><c r="I771" s="2" t="inlineStr" /><c r="J771" s="2" t="inlineStr" /><c r="K771" s="2" t="inlineStr"><is><t>alprazolam</t></is></c><c r="L771" s="2" t="inlineStr"><is><t>zolpidem</t></is></c><c r="M771" s="2" t="inlineStr"><is><t>hydroksyzynę</t></is></c><c r="N771" s="2" t="inlineStr" /><c r="O771" s="2" t="inlineStr" /><c r="P771" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q771" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="772"><c r="A772" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B772" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C772" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D772" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E772" s="2" t="inlineStr"><is><t>Zyprazydonu, leku istotnie wydłużającego odstęp QT nie należy stosować:</t></is></c><c r="F772" s="2" t="inlineStr"><is><t>w hipokaliemii</t></is></c><c r="G772" s="2" t="inlineStr"><is><t>łącznie z moksyfloksacyną</t></is></c><c r="H772" s="2" t="inlineStr"><is><t>w objawowej bradykardii</t></is></c><c r="I772" s="2" t="inlineStr"><is><t>łącznie z amiodaronem</t></is></c><c r="J772" s="2" t="inlineStr" /><c r="K772" s="2" t="inlineStr" /><c r="L772" s="2" t="inlineStr" /><c r="M772" s="2" t="inlineStr" /><c r="N772" s="2" t="inlineStr" /><c r="O772" s="2" t="inlineStr" /><c r="P772" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q772" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="773"><c r="A773" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B773" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C773" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D773" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E773" s="2" t="inlineStr"><is><t>Zaburzenia pozapiramidowe mogą wystąpić w przebiegu stosowania:</t></is></c><c r="F773" s="2" t="inlineStr"><is><t>flunaryzyny</t></is></c><c r="G773" s="2" t="inlineStr"><is><t>metoklopramidu</t></is></c><c r="H773" s="2" t="inlineStr" /><c r="I773" s="2" t="inlineStr" /><c r="J773" s="2" t="inlineStr" /><c r="K773" s="2" t="inlineStr"><is><t>betahistyny</t></is></c><c r="L773" s="2" t="inlineStr"><is><t>rywastygminy</t></is></c><c r="M773" s="2" t="inlineStr" /><c r="N773" s="2" t="inlineStr" /><c r="O773" s="2" t="inlineStr" /><c r="P773" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q773" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="774"><c r="A774" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B774" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C774" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D774" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E774" s="2" t="inlineStr"><is><t>Parkinsonizm polekowy w przebiegu leczenia lekami przeciwpsychotycznymi wynika z:</t></is></c><c r="F774" s="2" t="inlineStr"><is><t>zmniejszania działania dopaminy w układzie nigrostriatalnym</t></is></c><c r="G774" s="2" t="inlineStr" /><c r="H774" s="2" t="inlineStr" /><c r="I774" s="2" t="inlineStr" /><c r="J774" s="2" t="inlineStr" /><c r="K774" s="2" t="inlineStr"><is><t>patogenezy schizofrenii</t></is></c><c r="L774" s="2" t="inlineStr"><is><t>zmniejszania działania dopaminy w obszarze mezokortykalnym</t></is></c><c r="M774" s="2" t="inlineStr"><is><t>blokowania receptorów muskarynowych</t></is></c><c r="N774" s="2" t="inlineStr" /><c r="O774" s="2" t="inlineStr" /><c r="P774" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q774" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="775"><c r="A775" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B775" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C775" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D775" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E775" s="2" t="inlineStr"><is><t>Napływ sodu do komórki hamuje:</t></is></c><c r="F775" s="2" t="inlineStr"><is><t>ranolzyna</t></is></c><c r="G775" s="2" t="inlineStr"><is><t>iwabradyna</t></is></c><c r="H775" s="2" t="inlineStr"><is><t>okskarbamazepina</t></is></c><c r="I775" s="2" t="inlineStr" /><c r="J775" s="2" t="inlineStr" /><c r="K775" s="2" t="inlineStr"><is><t>gabapentyna</t></is></c><c r="L775" s="2" t="inlineStr" /><c r="M775" s="2" t="inlineStr" /><c r="N775" s="2" t="inlineStr" /><c r="O775" s="2" t="inlineStr" /><c r="P775" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q775" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="776"><c r="A776" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B776" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C776" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D776" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E776" s="2" t="inlineStr"><is><t>W ramach badania geriatrycznego u 80-letniej kobiety ze średnim wykształceniem wynik MMSE = 25 pkt. Za niezgodne z aktualną wiedzą medyczną uznasz zastosowanie u niej:</t></is></c><c r="F776" s="2" t="inlineStr"><is><t>piracetamu</t></is></c><c r="G776" s="2" t="inlineStr"><is><t>winpocetyny</t></is></c><c r="H776" s="2" t="inlineStr"><is><t>suplementacji cynku</t></is></c><c r="I776" s="2" t="inlineStr" /><c r="J776" s="2" t="inlineStr" /><c r="K776" s="2" t="inlineStr"><is><t>treningu mózgu (np. zgadnij co to za zawód: arlzek)</t></is></c><c r="L776" s="2" t="inlineStr" /><c r="M776" s="2" t="inlineStr" /><c r="N776" s="2" t="inlineStr" /><c r="O776" s="2" t="inlineStr" /><c r="P776" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q776" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="777"><c r="A777" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B777" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C777" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D777" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E777" s="2" t="inlineStr"><is><t>W zapobieganiu wymiotom w przebiegu chemioterapii należy zastosować:</t></is></c><c r="F777" s="2" t="inlineStr"><is><t>aprepitant</t></is></c><c r="G777" s="2" t="inlineStr"><is><t>ondansetron</t></is></c><c r="H777" s="2" t="inlineStr" /><c r="I777" s="2" t="inlineStr" /><c r="J777" s="2" t="inlineStr" /><c r="K777" s="2" t="inlineStr"><is><t>skopolaminę</t></is></c><c r="L777" s="2" t="inlineStr"><is><t>dimenhydrinat</t></is></c><c r="M777" s="2" t="inlineStr" /><c r="N777" s="2" t="inlineStr" /><c r="O777" s="2" t="inlineStr" /><c r="P777" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q777" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="778"><c r="A778" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B778" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C778" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D778" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E778" s="2" t="inlineStr"><is><t>Wg Światowej Agencji Antydopingowej (WADA) za doping uważa się:</t></is></c><c r="F778" s="2" t="inlineStr"><is><t>użycie przez sportowców czynników stymulujących erytropoezę</t></is></c><c r="G778" s="2" t="inlineStr"><is><t>podanie sportowcowi autopreparatu krwinek czerwonych</t></is></c><c r="H778" s="2" t="inlineStr"><is><t>obecność we krwi sportowca egzogennych substancji o działaniu agonistycznym w stosunku do receptorów androgenowych i dla IGF-1</t></is></c><c r="I778" s="2" t="inlineStr"><is><t>podanie sportowcowi polimerów kwasów nukleinowych lub analogów kwasu nukleinowego</t></is></c><c r="J778" s="2" t="inlineStr" /><c r="K778" s="2" t="inlineStr" /><c r="L778" s="2" t="inlineStr" /><c r="M778" s="2" t="inlineStr" /><c r="N778" s="2" t="inlineStr" /><c r="O778" s="2" t="inlineStr" /><c r="P778" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q778" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="779"><c r="A779" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B779" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C779" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D779" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E779" s="2" t="inlineStr"><is><t>U chorego z zaburzeniami świadomości, sennością, zaburzeniami równowagi, mowy, widzenia, omamy, pobudzeniem psychoruchowym, drgawkami, hipotonia z nieutrwalonymi częstoskurczami komorowymi będziesz podejrzewał zatrucie i podasz:</t></is></c><c r="F779" s="2" t="inlineStr"><is><t>imipraminą - fizostygminę</t></is></c><c r="G779" s="2" t="inlineStr" /><c r="H779" s="2" t="inlineStr" /><c r="I779" s="2" t="inlineStr" /><c r="J779" s="2" t="inlineStr" /><c r="K779" s="2" t="inlineStr"><is><t>paracetamolem- N-acetylocysteinę</t></is></c><c r="L779" s="2" t="inlineStr"><is><t>kodeiną - naltrekson</t></is></c><c r="M779" s="2" t="inlineStr"><is><t>litem - fizostygminę</t></is></c><c r="N779" s="2" t="inlineStr" /><c r="O779" s="2" t="inlineStr" /><c r="P779" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q779" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="780"><c r="A780" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B780" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C780" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D780" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E780" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące przedawkowania leków znieczulenia miejscowego:</t></is></c><c r="F780" s="2" t="inlineStr"><is><t>Powodują drgawki, bradykardię i hipotonię</t></is></c><c r="G780" s="2" t="inlineStr"><is><t>Parestezje (drętwienie) języka i ust są wczesnym charakterystycznym objawem zwiastunowym</t></is></c><c r="H780" s="2" t="inlineStr"><is><t>W resuscytacji krążeniowo oddechowej, oprócz typowego algorytmu, stosuje się wlew emulsji tłuszczowej</t></is></c><c r="I780" s="2" t="inlineStr"><is><t>Na wystąpienie objawów nie ma wpływu miejscu wstrzyknięcia leku, a jedynie jego dawka</t></is></c><c r="J780" s="2" t="inlineStr" /><c r="K780" s="2" t="inlineStr" /><c r="L780" s="2" t="inlineStr" /><c r="M780" s="2" t="inlineStr" /><c r="N780" s="2" t="inlineStr" /><c r="O780" s="2" t="inlineStr" /><c r="P780" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q780" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="781"><c r="A781" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B781" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C781" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D781" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E781" s="2" t="inlineStr"><is><t>Do leków przeciwhistaminowych stosowanych wyłącznie miejscowo na błony śluzowe należą:</t></is></c><c r="F781" s="2" t="inlineStr"><is><t>Emedastyna</t></is></c><c r="G781" s="2" t="inlineStr"><is><t>Azelastyna</t></is></c><c r="H781" s="2" t="inlineStr" /><c r="I781" s="2" t="inlineStr" /><c r="J781" s="2" t="inlineStr" /><c r="K781" s="2" t="inlineStr"><is><t>Desforatadyna</t></is></c><c r="L781" s="2" t="inlineStr"><is><t>Bilastyna</t></is></c><c r="M781" s="2" t="inlineStr" /><c r="N781" s="2" t="inlineStr" /><c r="O781" s="2" t="inlineStr" /><c r="P781" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q781" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="782"><c r="A782" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B782" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C782" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D782" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E782" s="2" t="inlineStr"><is><t>Dorosły pacjent trafił do szpitala 3 godziny po samobójczym przedawkowaniu fenobarbitalu (pochodna kwasu barbiturowego). Należy zastosować:</t></is></c><c r="F782" s="2" t="inlineStr"><is><t>Rozcienczenie trucizny przez podanie do wypicia dużej ilości wody pitnej</t></is></c><c r="G782" s="2" t="inlineStr"><is><t>Alkalizację moczu do pH co najmniej 7,5 przez dodanie wodorowęglanu sodu do dożylnych płynów infuzyjnych</t></is></c><c r="H782" s="2" t="inlineStr" /><c r="I782" s="2" t="inlineStr" /><c r="J782" s="2" t="inlineStr" /><c r="K782" s="2" t="inlineStr"><is><t>Płukanie żołądka z zastosowaniem wody pitnej przez sondę ustno-żołądkową w małych porcjach jedna po drugiej</t></is></c><c r="L782" s="2" t="inlineStr"><is><t>Irygację całego jelita przez doustne podanie płynów elektrolitowych z polietylenoglikolem (tzw. makrogolami)</t></is></c><c r="M782" s="2" t="inlineStr" /><c r="N782" s="2" t="inlineStr" /><c r="O782" s="2" t="inlineStr" /><c r="P782" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q782" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="783"><c r="A783" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B783" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C783" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D783" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E783" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie trucizna – antidotum – mechanizm działania antidotum:</t></is></c><c r="F783" s="2" t="inlineStr"><is><t>Paracetamol – acetylocysteina – neutralizacja metaboliczna</t></is></c><c r="G783" s="2" t="inlineStr"><is><t>Amitryptylina - fizostygmina - antagonizm fizjologiczny</t></is></c><c r="H783" s="2" t="inlineStr"><is><t>Dabigatran – idarucyzumab - neutralizujące przeciwciało</t></is></c><c r="I783" s="2" t="inlineStr"><is><t>Diazepam – flomazenil – antagonizm receptorowy</t></is></c><c r="J783" s="2" t="inlineStr" /><c r="K783" s="2" t="inlineStr" /><c r="L783" s="2" t="inlineStr" /><c r="M783" s="2" t="inlineStr" /><c r="N783" s="2" t="inlineStr" /><c r="O783" s="2" t="inlineStr" /><c r="P783" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q783" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="784"><c r="A784" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B784" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C784" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D784" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E784" s="2" t="inlineStr"><is><t>Który z leków działa przeciwdrgawkowo głównie poprzez nasilenie transmisji GABA￾ergicznej:</t></is></c><c r="F784" s="2" t="inlineStr"><is><t>Tiagabina</t></is></c><c r="G784" s="2" t="inlineStr" /><c r="H784" s="2" t="inlineStr" /><c r="I784" s="2" t="inlineStr" /><c r="J784" s="2" t="inlineStr" /><c r="K784" s="2" t="inlineStr"><is><t>Lamotrygina</t></is></c><c r="L784" s="2" t="inlineStr"><is><t>Lewetriacetam</t></is></c><c r="M784" s="2" t="inlineStr"><is><t>Zonisamid</t></is></c><c r="N784" s="2" t="inlineStr" /><c r="O784" s="2" t="inlineStr" /><c r="P784" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q784" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="785"><c r="A785" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B785" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C785" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D785" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E785" s="2" t="inlineStr"><is><t>Które leki mogą zaostrzyć objawy otępienia u osoby z chorobą Alzheimera?</t></is></c><c r="F785" s="2" t="inlineStr"><is><t>Olanzapina</t></is></c><c r="G785" s="2" t="inlineStr"><is><t>Memantyna</t></is></c><c r="H785" s="2" t="inlineStr"><is><t>Biperiden</t></is></c><c r="I785" s="2" t="inlineStr" /><c r="J785" s="2" t="inlineStr" /><c r="K785" s="2" t="inlineStr"><is><t>Piracetam</t></is></c><c r="L785" s="2" t="inlineStr" /><c r="M785" s="2" t="inlineStr" /><c r="N785" s="2" t="inlineStr" /><c r="O785" s="2" t="inlineStr" /><c r="P785" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q785" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="786"><c r="A786" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B786" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C786" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D786" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E786" s="2" t="inlineStr"><is><t>Skłonność do hazardu, kompulsywne objadanie i obsesje seksualne to działania niepożądane obserwowane w terapii:</t></is></c><c r="F786" s="2" t="inlineStr"><is><t>L-dopą</t></is></c><c r="G786" s="2" t="inlineStr"><is><t>Pramipeksolem</t></is></c><c r="H786" s="2" t="inlineStr" /><c r="I786" s="2" t="inlineStr" /><c r="J786" s="2" t="inlineStr" /><c r="K786" s="2" t="inlineStr"><is><t>Metylofenidatem</t></is></c><c r="L786" s="2" t="inlineStr"><is><t>Zolpidemem</t></is></c><c r="M786" s="2" t="inlineStr" /><c r="N786" s="2" t="inlineStr" /><c r="O786" s="2" t="inlineStr" /><c r="P786" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q786" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="787"><c r="A787" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B787" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C787" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D787" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E787" s="2" t="inlineStr"><is><t>Zolendronian:</t></is></c><c r="F787" s="2" t="inlineStr"><is><t>Z dużym powinowactwem wiąże się ze zmineralizowaną kością</t></is></c><c r="G787" s="2" t="inlineStr"><is><t>Hamuje resorbcję kości</t></is></c><c r="H787" s="2" t="inlineStr" /><c r="I787" s="2" t="inlineStr" /><c r="J787" s="2" t="inlineStr" /><c r="K787" s="2" t="inlineStr"><is><t>Koryguje hiperkalcemię w chorobach nowotworowych zwiększając jednoczeście kalcurię</t></is></c><c r="L787" s="2" t="inlineStr"><is><t>Może spowodować martwicę szczęki szczególnie w przypadku złego stanu uzębienia</t></is></c><c r="M787" s="2" t="inlineStr" /><c r="N787" s="2" t="inlineStr" /><c r="O787" s="2" t="inlineStr" /><c r="P787" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q787" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="788"><c r="A788" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B788" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C788" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D788" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E788" s="2" t="inlineStr"><is><t>Leki stosowane przewlekle w stwardnieniu rozsianym w celu modyfikacji przebiegu choroby to:</t></is></c><c r="F788" s="2" t="inlineStr"><is><t>PEG-interferon-beta</t></is></c><c r="G788" s="2" t="inlineStr"><is><t>Natalizumab</t></is></c><c r="H788" s="2" t="inlineStr"><is><t>Adalimumab</t></is></c><c r="I788" s="2" t="inlineStr" /><c r="J788" s="2" t="inlineStr" /><c r="K788" s="2" t="inlineStr"><is><t>Interferon-gamma</t></is></c><c r="L788" s="2" t="inlineStr" /><c r="M788" s="2" t="inlineStr" /><c r="N788" s="2" t="inlineStr" /><c r="O788" s="2" t="inlineStr" /><c r="P788" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q788" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="789"><c r="A789" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B789" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C789" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D789" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E789" s="2" t="inlineStr"><is><t>Który mechanizm opisuje działanie aprepitantu:</t></is></c><c r="F789" s="2" t="inlineStr"><is><t>Stymulowanie receptora neurokininy (NK1) w strefie chemoreceptorowej mózgu</t></is></c><c r="G789" s="2" t="inlineStr" /><c r="H789" s="2" t="inlineStr" /><c r="I789" s="2" t="inlineStr" /><c r="J789" s="2" t="inlineStr" /><c r="K789" s="2" t="inlineStr"><is><t>Stymulowanie receptora O2 w strefie chemoreceptorowej mózgu</t></is></c><c r="L789" s="2" t="inlineStr"><is><t>Stymulowanie receptora 5-HT3 na włóknach aferentnych nerwu błędnego</t></is></c><c r="M789" s="2" t="inlineStr"><is><t>Blokowanie receptora muskarynowego w ośrodku wymiotnym w rdzeniu przedłużonym</t></is></c><c r="N789" s="2" t="inlineStr" /><c r="O789" s="2" t="inlineStr" /><c r="P789" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q789" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="790"><c r="A790" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B790" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C790" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D790" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E790" s="2" t="inlineStr"><is><t>Amitryptylina ma zastosowanie w leczeniu:</t></is></c><c r="F790" s="2" t="inlineStr"><is><t>Bólu neuropatycznego</t></is></c><c r="G790" s="2" t="inlineStr"><is><t>Choroby afektywnej jednobiegunowej</t></is></c><c r="H790" s="2" t="inlineStr" /><c r="I790" s="2" t="inlineStr" /><c r="J790" s="2" t="inlineStr" /><c r="K790" s="2" t="inlineStr"><is><t>Bezsenności</t></is></c><c r="L790" s="2" t="inlineStr"><is><t>Padaczki</t></is></c><c r="M790" s="2" t="inlineStr" /><c r="N790" s="2" t="inlineStr" /><c r="O790" s="2" t="inlineStr" /><c r="P790" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q790" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="791"><c r="A791" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B791" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C791" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D791" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E791" s="2" t="inlineStr"><is><t>Zespół serotoninowy może być wynikiem podawania:</t></is></c><c r="F791" s="2" t="inlineStr"><is><t>Tramadolu</t></is></c><c r="G791" s="2" t="inlineStr"><is><t>Escitalopramu</t></is></c><c r="H791" s="2" t="inlineStr" /><c r="I791" s="2" t="inlineStr" /><c r="J791" s="2" t="inlineStr" /><c r="K791" s="2" t="inlineStr"><is><t>Litu</t></is></c><c r="L791" s="2" t="inlineStr"><is><t>Buspironu</t></is></c><c r="M791" s="2" t="inlineStr" /><c r="N791" s="2" t="inlineStr" /><c r="O791" s="2" t="inlineStr" /><c r="P791" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q791" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="792"><c r="A792" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B792" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C792" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D792" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E792" s="2" t="inlineStr"><is><t>Benzodiazepiną nie mającą wątrobowego metabolizmu jest:</t></is></c><c r="F792" s="2" t="inlineStr"><is><t>Lorazepam</t></is></c><c r="G792" s="2" t="inlineStr"><is><t>Oksazepam</t></is></c><c r="H792" s="2" t="inlineStr" /><c r="I792" s="2" t="inlineStr" /><c r="J792" s="2" t="inlineStr" /><c r="K792" s="2" t="inlineStr"><is><t>Nitrazepam</t></is></c><c r="L792" s="2" t="inlineStr"><is><t>Diazepam</t></is></c><c r="M792" s="2" t="inlineStr" /><c r="N792" s="2" t="inlineStr" /><c r="O792" s="2" t="inlineStr" /><c r="P792" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q792" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="793"><c r="A793" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B793" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C793" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D793" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E793" s="2" t="inlineStr"><is><t>Acetylocysteina:</t></is></c><c r="F793" s="2" t="inlineStr"><is><t>Jest odtrutką w zatruciu paracetamolem ze względu na udział w detoksykacji toksycznego metabolitu N-acetylo-4-benzochinoiminy (NAPO)</t></is></c><c r="G793" s="2" t="inlineStr" /><c r="H793" s="2" t="inlineStr" /><c r="I793" s="2" t="inlineStr" /><c r="J793" s="2" t="inlineStr" /><c r="K793" s="2" t="inlineStr"><is><t>Może być stosowana doustnie, dożylnie i wziewnie</t></is></c><c r="L793" s="2" t="inlineStr"><is><t>W dużej dawce pobudza ruchomość rzęsek nabłonka oddechowego</t></is></c><c r="M793" s="2" t="inlineStr"><is><t>Rozrzedza śluz poprzez zmniejszenie oddziaływania ładunków elektrycznych występujących w sieci mucyn (działanie niedestrukcyjne)</t></is></c><c r="N793" s="2" t="inlineStr" /><c r="O793" s="2" t="inlineStr" /><c r="P793" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q793" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="794"><c r="A794" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B794" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C794" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D794" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E794" s="2" t="inlineStr"><is><t>Przewlekłe stosowanie pantoprazolu może prowadzić do:</t></is></c><c r="F794" s="2" t="inlineStr"><is><t>Zmniejszonego wchłaniania witaminy B12, Mg2+, Ca2+</t></is></c><c r="G794" s="2" t="inlineStr"><is><t>Zwiększonego ryzyka zakażenia przewodu pokarmowego, np. biegunka Clostridium difficile</t></is></c><c r="H794" s="2" t="inlineStr"><is><t>Zwiększonego ryzyka złamania kościu udowej</t></is></c><c r="I794" s="2" t="inlineStr" /><c r="J794" s="2" t="inlineStr" /><c r="K794" s="2" t="inlineStr"><is><t>Zwiększonego ryzyka zakażenia układu oddechowego</t></is></c><c r="L794" s="2" t="inlineStr" /><c r="M794" s="2" t="inlineStr" /><c r="N794" s="2" t="inlineStr" /><c r="O794" s="2" t="inlineStr" /><c r="P794" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q794" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="795"><c r="A795" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B795" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C795" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D795" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E795" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie - lek prokinetyczny / mechanizm działania:</t></is></c><c r="F795" s="2" t="inlineStr"><is><t>Erytromycyna - agonista rec. Motylinowego</t></is></c><c r="G795" s="2" t="inlineStr"><is><t>Cizapryd – agonista rec. 5-HT4</t></is></c><c r="H795" s="2" t="inlineStr" /><c r="I795" s="2" t="inlineStr" /><c r="J795" s="2" t="inlineStr" /><c r="K795" s="2" t="inlineStr"><is><t>Metoklopramid – agonista rec. 5-HT3 i rec. D2</t></is></c><c r="L795" s="2" t="inlineStr"><is><t>Itopryd – agonista rec. 5-HT4 i rec. D2</t></is></c><c r="M795" s="2" t="inlineStr" /><c r="N795" s="2" t="inlineStr" /><c r="O795" s="2" t="inlineStr" /><c r="P795" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q795" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="796"><c r="A796" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B796" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C796" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D796" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E796" s="2" t="inlineStr"><is><t>Kwerolimus jest stosowany w:</t></is></c><c r="F796" s="2" t="inlineStr"><is><t>Kardiologii (stenty wiecowe)</t></is></c><c r="G796" s="2" t="inlineStr"><is><t>Onkologii (wybrane zaawansowane nowotwory piersi i nerki)</t></is></c><c r="H796" s="2" t="inlineStr" /><c r="I796" s="2" t="inlineStr" /><c r="J796" s="2" t="inlineStr" /><c r="K796" s="2" t="inlineStr"><is><t>Neurologii (stwardnieni rozsiane)</t></is></c><c r="L796" s="2" t="inlineStr"><is><t>Dermatologii (łuszczyca)</t></is></c><c r="M796" s="2" t="inlineStr" /><c r="N796" s="2" t="inlineStr" /><c r="O796" s="2" t="inlineStr" /><c r="P796" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q796" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="797"><c r="A797" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B797" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C797" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D797" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E797" s="2" t="inlineStr"><is><t>Mykofenolan mofetylu (MMF):</t></is></c><c r="F797" s="2" t="inlineStr"><is><t>Jest odwracalnym inhibitorem dehydrogenazy inozynomonofosforanu hamującym syntezę de novo nukleotydów guaninowych</t></is></c><c r="G797" s="2" t="inlineStr"><is><t>Działa silniej na limfocyty niż na inne komórki</t></is></c><c r="H797" s="2" t="inlineStr" /><c r="I797" s="2" t="inlineStr" /><c r="J797" s="2" t="inlineStr" /><c r="K797" s="2" t="inlineStr"><is><t>Bezpośrednio hamuje wytwarzanie interleukiny 2 (IL-2)</t></is></c><c r="L797" s="2" t="inlineStr"><is><t>Jest inhibitorem sygnału po pobudzeniu receptorów dla IL-2</t></is></c><c r="M797" s="2" t="inlineStr" /><c r="N797" s="2" t="inlineStr" /><c r="O797" s="2" t="inlineStr" /><c r="P797" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q797" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="798"><c r="A798" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B798" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C798" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D798" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E798" s="2" t="inlineStr"><is><t>Adenozyna</t></is></c><c r="F798" s="2" t="inlineStr"><is><t>To nukleotyd purynowy występujący we wszystkich komórkach organizmu</t></is></c><c r="G798" s="2" t="inlineStr" /><c r="H798" s="2" t="inlineStr" /><c r="I798" s="2" t="inlineStr" /><c r="J798" s="2" t="inlineStr" /><c r="K798" s="2" t="inlineStr"><is><t>Aktywuje kanały potasowe i powoduje depolaryzację komórek</t></is></c><c r="L798" s="2" t="inlineStr"><is><t>Działa dromotropowo ujemnie w węźle przedsionkowo-komorowym</t></is></c><c r="M798" s="2" t="inlineStr"><is><t>Jest skuteczna kardiowersji farmakologicznej częstoskurczów komorowych</t></is></c><c r="N798" s="2" t="inlineStr" /><c r="O798" s="2" t="inlineStr" /><c r="P798" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q798" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="799"><c r="A799" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B799" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C799" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D799" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E799" s="2" t="inlineStr"><is><t>Ewolokumab:</t></is></c><c r="F799" s="2" t="inlineStr"><is><t>Jest ludzkim przeciwciałem poliklonalnym</t></is></c><c r="G799" s="2" t="inlineStr"><is><t>Hamuje aktywność konwertazy białkowej subtylizyna/keksyna typu 9 (PCSK9) - enzymu biorącego udział w degradacji receptorów dla LDL</t></is></c><c r="H799" s="2" t="inlineStr" /><c r="I799" s="2" t="inlineStr" /><c r="J799" s="2" t="inlineStr" /><c r="K799" s="2" t="inlineStr"><is><t>Jest stosowany dożylnie</t></is></c><c r="L799" s="2" t="inlineStr"><is><t>Zwiększa stęężenie cholesterolu HDL o ponad 100%</t></is></c><c r="M799" s="2" t="inlineStr" /><c r="N799" s="2" t="inlineStr" /><c r="O799" s="2" t="inlineStr" /><c r="P799" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q799" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="800"><c r="A800" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B800" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C800" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D800" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E800" s="2" t="inlineStr"><is><t>Przyczyną wzrostu masy ciała może być:</t></is></c><c r="F800" s="2" t="inlineStr"><is><t>Klemastyny</t></is></c><c r="G800" s="2" t="inlineStr"><is><t>Kwetiapiny</t></is></c><c r="H800" s="2" t="inlineStr"><is><t>Citalopramu</t></is></c><c r="I800" s="2" t="inlineStr" /><c r="J800" s="2" t="inlineStr" /><c r="K800" s="2" t="inlineStr"><is><t>Liraglutydu</t></is></c><c r="L800" s="2" t="inlineStr" /><c r="M800" s="2" t="inlineStr" /><c r="N800" s="2" t="inlineStr" /><c r="O800" s="2" t="inlineStr" /><c r="P800" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q800" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="801"><c r="A801" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B801" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C801" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D801" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E801" s="2" t="inlineStr"><is><t>Reguła Robertsa mówi o:</t></is></c><c r="F801" s="2" t="inlineStr"><is><t>Podwajaniu dawki statyny</t></is></c><c r="G801" s="2" t="inlineStr"><is><t>Obniżeniu stężenia cholesterolu LDL o dodatkowe 7% po odpowiednim zwiększeniu dawki statyny</t></is></c><c r="H801" s="2" t="inlineStr" /><c r="I801" s="2" t="inlineStr" /><c r="J801" s="2" t="inlineStr" /><c r="K801" s="2" t="inlineStr"><is><t>Obniżeniu stężenia cholesterolu LDL o dodatkowe 5% po odpowiednim zwiększeniu dawki statyny</t></is></c><c r="L801" s="2" t="inlineStr"><is><t>Potrajaniu dawki statyny</t></is></c><c r="M801" s="2" t="inlineStr" /><c r="N801" s="2" t="inlineStr" /><c r="O801" s="2" t="inlineStr" /><c r="P801" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q801" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="802"><c r="A802" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B802" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C802" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D802" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E802" s="2" t="inlineStr"><is><t>Do leków hamujących układ RAA należy:</t></is></c><c r="F802" s="2" t="inlineStr"><is><t>Zofenopryl</t></is></c><c r="G802" s="2" t="inlineStr"><is><t>Eplerenon</t></is></c><c r="H802" s="2" t="inlineStr" /><c r="I802" s="2" t="inlineStr" /><c r="J802" s="2" t="inlineStr" /><c r="K802" s="2" t="inlineStr"><is><t>Aliskiren</t></is></c><c r="L802" s="2" t="inlineStr"><is><t>Nebiwolol</t></is></c><c r="M802" s="2" t="inlineStr" /><c r="N802" s="2" t="inlineStr" /><c r="O802" s="2" t="inlineStr" /><c r="P802" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q802" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="803"><c r="A803" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B803" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C803" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D803" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E803" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące torasemidu:</t></is></c><c r="F803" s="2" t="inlineStr"><is><t>Hamuje symporter sodowo-potasowo-chlorkowy części grubościennej ramienia wstępującego pętli Henlego</t></is></c><c r="G803" s="2" t="inlineStr"><is><t>Zwiększa aktywność reninową osocza</t></is></c><c r="H803" s="2" t="inlineStr" /><c r="I803" s="2" t="inlineStr" /><c r="J803" s="2" t="inlineStr" /><c r="K803" s="2" t="inlineStr"><is><t>Powoduje słabszy efekt natiuretyczny niż furosemid</t></is></c><c r="L803" s="2" t="inlineStr"><is><t>Jest nieskuteczny jeśli eGFR (wskaźnik filtracji kłębuszkowej) &lt; 30 ml/min</t></is></c><c r="M803" s="2" t="inlineStr" /><c r="N803" s="2" t="inlineStr" /><c r="O803" s="2" t="inlineStr" /><c r="P803" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q803" s="2" t="inlineStr"><is><t>srednia</t></is></c></row></sheetData><autoFilter ref="A1:Q803" /><pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5" /></worksheet>
+<file path=xl/worksheets/sheet1.xml><worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"><sheetPr><outlinePr summaryBelow="1" summaryRight="1" /><pageSetUpPr /></sheetPr><dimension ref="A1:Q873" /><sheetFormatPr baseColWidth="8" defaultRowHeight="15" /><cols><col width="30" customWidth="1" min="1" max="1" /><col width="21" customWidth="1" min="2" max="2" /><col width="9" customWidth="1" min="3" max="3" /><col width="9" customWidth="1" min="4" max="4" /><col width="60" customWidth="1" min="5" max="5" /><col width="32" customWidth="1" min="6" max="6" /><col width="32" customWidth="1" min="7" max="7" /><col width="32" customWidth="1" min="8" max="8" /><col width="32" customWidth="1" min="9" max="9" /><col width="32" customWidth="1" min="10" max="10" /><col width="32" customWidth="1" min="11" max="11" /><col width="32" customWidth="1" min="12" max="12" /><col width="32" customWidth="1" min="13" max="13" /><col width="32" customWidth="1" min="14" max="14" /><col width="32" customWidth="1" min="15" max="15" /><col width="26" customWidth="1" min="16" max="16" /><col width="10" customWidth="1" min="17" max="17" /></cols><sheetData><row r="1"><c r="A1" s="1" t="inlineStr"><is><t>Section</t></is></c><c r="B1" s="1" t="inlineStr"><is><t>Category</t></is></c><c r="C1" s="1" t="inlineStr"><is><t>Poziom</t></is></c><c r="D1" s="1" t="inlineStr"><is><t>Type</t></is></c><c r="E1" s="1" t="inlineStr"><is><t>Question</t></is></c><c r="F1" s="1" t="inlineStr"><is><t>True 1</t></is></c><c r="G1" s="1" t="inlineStr"><is><t>True 2</t></is></c><c r="H1" s="1" t="inlineStr"><is><t>True 3</t></is></c><c r="I1" s="1" t="inlineStr"><is><t>True 4</t></is></c><c r="J1" s="1" t="inlineStr"><is><t>True 5</t></is></c><c r="K1" s="1" t="inlineStr"><is><t>False 1</t></is></c><c r="L1" s="1" t="inlineStr"><is><t>False 2</t></is></c><c r="M1" s="1" t="inlineStr"><is><t>False 3</t></is></c><c r="N1" s="1" t="inlineStr"><is><t>False 4</t></is></c><c r="O1" s="1" t="inlineStr"><is><t>False 5</t></is></c><c r="P1" s="1" t="inlineStr"><is><t>Zrodlo</t></is></c><c r="Q1" s="1" t="inlineStr"><is><t>Pewnosc</t></is></c></row><row r="2"><c r="A2" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B2" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C2" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D2" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E2" s="2" t="inlineStr"><is><t>Czarne zabarwienie stolca powoduje podanie preparatów:</t></is></c><c r="F2" s="2" t="inlineStr"><is><t>Bizmutu</t></is></c><c r="G2" s="2" t="inlineStr"><is><t>Żelaza</t></is></c><c r="H2" s="2" t="inlineStr" /><c r="I2" s="2" t="inlineStr" /><c r="J2" s="2" t="inlineStr" /><c r="K2" s="2" t="inlineStr"><is><t>Wapnia</t></is></c><c r="L2" s="2" t="inlineStr"><is><t>Glinu</t></is></c><c r="M2" s="2" t="inlineStr" /><c r="N2" s="2" t="inlineStr" /><c r="O2" s="2" t="inlineStr" /><c r="P2" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q2" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="3"><c r="A3" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B3" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C3" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D3" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E3" s="2" t="inlineStr"><is><t>Uzasadnionym wskazaniem do przewlekłego stosowania inhibitorów pompy protonowej jest:</t></is></c><c r="F3" s="2" t="inlineStr"><is><t>Choroba refluksowa żołądka</t></is></c><c r="G3" s="2" t="inlineStr"><is><t>Profilaktyka gastropatii u osób leczonych niesteroidowymi lekami przeciwzapalnymi powyżej 65 r.ż</t></is></c><c r="H3" s="2" t="inlineStr"><is><t>Eradykacja Helicobacter Pylori</t></is></c><c r="I3" s="2" t="inlineStr" /><c r="J3" s="2" t="inlineStr" /><c r="K3" s="2" t="inlineStr"><is><t>Profilaktyka wrzodów stresowych</t></is></c><c r="L3" s="2" t="inlineStr" /><c r="M3" s="2" t="inlineStr" /><c r="N3" s="2" t="inlineStr" /><c r="O3" s="2" t="inlineStr" /><c r="P3" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q3" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="4"><c r="A4" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B4" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C4" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D4" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E4" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek – wskazanie</t></is></c><c r="F4" s="2" t="inlineStr"><is><t>Mesalazyna – choroba Leśniowskiego crohna</t></is></c><c r="G4" s="2" t="inlineStr"><is><t>Rifaksymina – biegunka podróżnych</t></is></c><c r="H4" s="2" t="inlineStr"><is><t>Metylonaltrekson – zaparcia w trakcie terapii opioidami</t></is></c><c r="I4" s="2" t="inlineStr" /><c r="J4" s="2" t="inlineStr" /><c r="K4" s="2" t="inlineStr"><is><t>Racekadotryl – śpiączka wątrobowa</t></is></c><c r="L4" s="2" t="inlineStr" /><c r="M4" s="2" t="inlineStr" /><c r="N4" s="2" t="inlineStr" /><c r="O4" s="2" t="inlineStr" /><c r="P4" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q4" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="5"><c r="A5" s="2" t="inlineStr"><is><t>ZNIECZULENIA OGÓLNE</t></is></c><c r="B5" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C5" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D5" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E5" s="2" t="inlineStr"><is><t>Do leków które wykazują miejscowe działanie przeciwbólowe po podaniu na skórę należy:</t></is></c><c r="F5" s="2" t="inlineStr"><is><t>Kapsaicyna</t></is></c><c r="G5" s="2" t="inlineStr"><is><t>Ketoprofen</t></is></c><c r="H5" s="2" t="inlineStr" /><c r="I5" s="2" t="inlineStr" /><c r="J5" s="2" t="inlineStr" /><c r="K5" s="2" t="inlineStr"><is><t>Propofol</t></is></c><c r="L5" s="2" t="inlineStr"><is><t>Tiopental</t></is></c><c r="M5" s="2" t="inlineStr" /><c r="N5" s="2" t="inlineStr" /><c r="O5" s="2" t="inlineStr" /><c r="P5" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q5" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="6"><c r="A6" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B6" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C6" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D6" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E6" s="2" t="inlineStr"><is><t>Ryzyko uszkodzenia wątroby przez paracetamol rośnie w przypadku:</t></is></c><c r="F6" s="2" t="inlineStr"><is><t>Zespołu zależności alkoholowej (ZAA)</t></is></c><c r="G6" s="2" t="inlineStr"><is><t>Wygłodzenia (kacheksji)</t></is></c><c r="H6" s="2" t="inlineStr"><is><t>Indukcji enzymów mikrosomalnych wątroby</t></is></c><c r="I6" s="2" t="inlineStr"><is><t>Przedawkowania</t></is></c><c r="J6" s="2" t="inlineStr" /><c r="K6" s="2" t="inlineStr" /><c r="L6" s="2" t="inlineStr" /><c r="M6" s="2" t="inlineStr" /><c r="N6" s="2" t="inlineStr" /><c r="O6" s="2" t="inlineStr" /><c r="P6" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q6" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="7"><c r="A7" s="2" t="inlineStr"><is><t>BÓLE GŁOWY</t></is></c><c r="B7" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C7" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D7" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E7" s="2" t="inlineStr"><is><t>W przerywaniu bólów migrenowych stosuje się:</t></is></c><c r="F7" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="G7" s="2" t="inlineStr"><is><t>Dihydroergotaminę</t></is></c><c r="H7" s="2" t="inlineStr"><is><t>Zolmitryptan</t></is></c><c r="I7" s="2" t="inlineStr" /><c r="J7" s="2" t="inlineStr" /><c r="K7" s="2" t="inlineStr"><is><t>Morfinę</t></is></c><c r="L7" s="2" t="inlineStr" /><c r="M7" s="2" t="inlineStr" /><c r="N7" s="2" t="inlineStr" /><c r="O7" s="2" t="inlineStr" /><c r="P7" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q7" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="8"><c r="A8" s="2" t="inlineStr"><is><t>JASKRA</t></is></c><c r="B8" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C8" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D8" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E8" s="2" t="inlineStr"><is><t>Analogi prostaglandyny E1 mogą powodować</t></is></c><c r="F8" s="2" t="inlineStr"><is><t>Hamowanie wydzielania soku żołądkowego</t></is></c><c r="G8" s="2" t="inlineStr" /><c r="H8" s="2" t="inlineStr" /><c r="I8" s="2" t="inlineStr" /><c r="J8" s="2" t="inlineStr" /><c r="K8" s="2" t="inlineStr"><is><t>Poprawę odpływu cieczy wodnistej z oka</t></is></c><c r="L8" s="2" t="inlineStr"><is><t>Rozszerzanie naczyń krwionośnych tętniczych</t></is></c><c r="M8" s="2" t="inlineStr"><is><t>Hamowanie agregacji płytek krwi</t></is></c><c r="N8" s="2" t="inlineStr" /><c r="O8" s="2" t="inlineStr" /><c r="P8" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q8" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="9"><c r="A9" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B9" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C9" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D9" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E9" s="2" t="inlineStr"><is><t>Substytucja enzymów trzustkowych jest wskazana:</t></is></c><c r="F9" s="2" t="inlineStr"><is><t>W mukowiscydozie</t></is></c><c r="G9" s="2" t="inlineStr"><is><t>Po resekcji trzustki</t></is></c><c r="H9" s="2" t="inlineStr" /><c r="I9" s="2" t="inlineStr" /><c r="J9" s="2" t="inlineStr" /><c r="K9" s="2" t="inlineStr"><is><t>W cukrzycy typu 1</t></is></c><c r="L9" s="2" t="inlineStr"><is><t>W anoreksji</t></is></c><c r="M9" s="2" t="inlineStr" /><c r="N9" s="2" t="inlineStr" /><c r="O9" s="2" t="inlineStr" /><c r="P9" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q9" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="10"><c r="A10" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B10" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C10" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D10" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E10" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek – wskazanie do podania:</t></is></c><c r="F10" s="2" t="inlineStr"><is><t>Haloperydol – agresja u pacjentów z ograniczonym uszkodzeniem mózgu</t></is></c><c r="G10" s="2" t="inlineStr"><is><t>Betahistyna – zawroty głowy w przebiegu choroby Meniere’a</t></is></c><c r="H10" s="2" t="inlineStr"><is><t>Topiramat – profilaktyka migreny</t></is></c><c r="I10" s="2" t="inlineStr"><is><t>Lamotrygina – profilaktyka choroby afektywnej dwubiegunowej</t></is></c><c r="J10" s="2" t="inlineStr" /><c r="K10" s="2" t="inlineStr" /><c r="L10" s="2" t="inlineStr" /><c r="M10" s="2" t="inlineStr" /><c r="N10" s="2" t="inlineStr" /><c r="O10" s="2" t="inlineStr" /><c r="P10" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q10" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="11"><c r="A11" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B11" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C11" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D11" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E11" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy:</t></is></c><c r="F11" s="2" t="inlineStr"><is><t>Ma eliminację metabolitów zgodnie z kinetyką I rzędu po podaniu małych dawek kardiologicznych</t></is></c><c r="G11" s="2" t="inlineStr"><is><t>Może być przyczyną zapalenia jelita cienkiego</t></is></c><c r="H11" s="2" t="inlineStr"><is><t>Po przedawkowaniu szybciej wydala się przez nerki po dożylnym podaniu wodorowęglanu sodu</t></is></c><c r="I11" s="2" t="inlineStr" /><c r="J11" s="2" t="inlineStr" /><c r="K11" s="2" t="inlineStr"><is><t>Słabiej zapobiega powstawaniu zakrzepu na blaszce miażdżycowej</t></is></c><c r="L11" s="2" t="inlineStr" /><c r="M11" s="2" t="inlineStr" /><c r="N11" s="2" t="inlineStr" /><c r="O11" s="2" t="inlineStr" /><c r="P11" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q11" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="12"><c r="A12" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B12" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C12" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D12" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E12" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy:</t></is></c><c r="F12" s="2" t="inlineStr"><is><t>może być przyczyną wystąpienia szczególnej postaci astmy</t></is></c><c r="G12" s="2" t="inlineStr"><is><t>nieodwracalnie hamuje COX</t></is></c><c r="H12" s="2" t="inlineStr" /><c r="I12" s="2" t="inlineStr" /><c r="J12" s="2" t="inlineStr" /><c r="K12" s="2" t="inlineStr"><is><t>zwiększa ryzyko sercowo-naczyniowe</t></is></c><c r="L12" s="2" t="inlineStr"><is><t>podawany łącznie z ibuprofenem wykazuje silniejszy efekt przeciwzapalny</t></is></c><c r="M12" s="2" t="inlineStr" /><c r="N12" s="2" t="inlineStr" /><c r="O12" s="2" t="inlineStr" /><c r="P12" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q12" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="13"><c r="A13" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B13" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C13" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D13" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E13" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące leczenia heparyną niefrakcjonowaną:</t></is></c><c r="F13" s="2" t="inlineStr"><is><t>Może być podawana podskórnie ale jej biodostępność jest wtedy mała i zmienna osobniczo</t></is></c><c r="G13" s="2" t="inlineStr"><is><t>Białka osoczowe mogą zmniejszać jej działanie przeciwkrzepliwe i być przyczyną oporności na leczenie</t></is></c><c r="H13" s="2" t="inlineStr"><is><t>Przedłużenie aPTT 1,5-2 razy w stosunku do wartości wyjściowej jest pożądanym efektem terapeutycznym</t></is></c><c r="I13" s="2" t="inlineStr"><is><t>Jej antidotum jest siarczan protaminy</t></is></c><c r="J13" s="2" t="inlineStr" /><c r="K13" s="2" t="inlineStr" /><c r="L13" s="2" t="inlineStr" /><c r="M13" s="2" t="inlineStr" /><c r="N13" s="2" t="inlineStr" /><c r="O13" s="2" t="inlineStr" /><c r="P13" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q13" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="14"><c r="A14" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B14" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C14" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D14" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E14" s="2" t="inlineStr"><is><t>Przeciwwskazaniem do podania cholinolityków jest:</t></is></c><c r="F14" s="2" t="inlineStr"><is><t>Rozrost gruczołu krokowego</t></is></c><c r="G14" s="2" t="inlineStr"><is><t>Jaskra</t></is></c><c r="H14" s="2" t="inlineStr" /><c r="I14" s="2" t="inlineStr" /><c r="J14" s="2" t="inlineStr" /><c r="K14" s="2" t="inlineStr"><is><t>Choroba wrzodowa żołądka i dwunastnicy</t></is></c><c r="L14" s="2" t="inlineStr"><is><t>Choroba lokomocyjna</t></is></c><c r="M14" s="2" t="inlineStr" /><c r="N14" s="2" t="inlineStr" /><c r="O14" s="2" t="inlineStr" /><c r="P14" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q14" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="15"><c r="A15" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B15" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C15" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D15" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E15" s="2" t="inlineStr"><is><t>Warfaryna:</t></is></c><c r="F15" s="2" t="inlineStr"><is><t>Jest sotosowana w profilaktyce i leczeniu żylnej choroby zakrzepowo-zatorowej</t></is></c><c r="G15" s="2" t="inlineStr"><is><t>Może być przyczyną zespołu purpurowego palucha</t></is></c><c r="H15" s="2" t="inlineStr" /><c r="I15" s="2" t="inlineStr" /><c r="J15" s="2" t="inlineStr" /><c r="K15" s="2" t="inlineStr"><is><t>Wymaga utrzymania INR&gt;4</t></is></c><c r="L15" s="2" t="inlineStr"><is><t>Jest eliminowana niezmieniona przez nerki</t></is></c><c r="M15" s="2" t="inlineStr" /><c r="N15" s="2" t="inlineStr" /><c r="O15" s="2" t="inlineStr" /><c r="P15" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q15" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="16"><c r="A16" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B16" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C16" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D16" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E16" s="2" t="inlineStr"><is><t>Fondaparynuks:</t></is></c><c r="F16" s="2" t="inlineStr"><is><t>Jest stosowana u osób z zawałem serca z przetrwałym uniesieniem odcinka ST (STEMI) oraz bez jego uniesienia (NSTEMI)</t></is></c><c r="G16" s="2" t="inlineStr" /><c r="H16" s="2" t="inlineStr" /><c r="I16" s="2" t="inlineStr" /><c r="J16" s="2" t="inlineStr" /><c r="K16" s="2" t="inlineStr"><is><t>Wybiórczo hamuje czynnik IIa</t></is></c><c r="L16" s="2" t="inlineStr"><is><t>W zalecanych dawkach hamuje istotnie wydłuża aPTT</t></is></c><c r="M16" s="2" t="inlineStr"><is><t>Nie jest wydalany przez nerki i może być stosowany u pacjentów z klirensem kreatyniny poniżej 30ml/min</t></is></c><c r="N16" s="2" t="inlineStr" /><c r="O16" s="2" t="inlineStr" /><c r="P16" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q16" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="17"><c r="A17" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B17" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C17" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D17" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E17" s="2" t="inlineStr"><is><t>Bezpośrednim inhibitorem trombiny podawanym dożylnie jest:</t></is></c><c r="F17" s="2" t="inlineStr"><is><t>Argatroban</t></is></c><c r="G17" s="2" t="inlineStr"><is><t>Biwalirudyna</t></is></c><c r="H17" s="2" t="inlineStr" /><c r="I17" s="2" t="inlineStr" /><c r="J17" s="2" t="inlineStr" /><c r="K17" s="2" t="inlineStr"><is><t>Dabigatran</t></is></c><c r="L17" s="2" t="inlineStr"><is><t>Dalteparyna</t></is></c><c r="M17" s="2" t="inlineStr" /><c r="N17" s="2" t="inlineStr" /><c r="O17" s="2" t="inlineStr" /><c r="P17" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q17" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="18"><c r="A18" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B18" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C18" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D18" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E18" s="2" t="inlineStr"><is><t>Odwracalne inhibitory acetylocholinesterazy są stosowane w leczeniu:</t></is></c><c r="F18" s="2" t="inlineStr"><is><t>Nużliwości mięśni</t></is></c><c r="G18" s="2" t="inlineStr"><is><t>Pooperacyjnej niedrożności jelit</t></is></c><c r="H18" s="2" t="inlineStr"><is><t>Choroby Alzheimera</t></is></c><c r="I18" s="2" t="inlineStr" /><c r="J18" s="2" t="inlineStr" /><c r="K18" s="2" t="inlineStr"><is><t>Zatruć związakmi fosfoorganicznymi</t></is></c><c r="L18" s="2" t="inlineStr" /><c r="M18" s="2" t="inlineStr" /><c r="N18" s="2" t="inlineStr" /><c r="O18" s="2" t="inlineStr" /><c r="P18" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q18" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="19"><c r="A19" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B19" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C19" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D19" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E19" s="2" t="inlineStr"><is><t>Zaznacza prawidłowe pary dotyczące leczenia uzależnień i wybranego leku:</t></is></c><c r="F19" s="2" t="inlineStr"><is><t>Uzależnienie od alkoholu – nalmefen</t></is></c><c r="G19" s="2" t="inlineStr"><is><t>Uzależnienie od heroiny – metadon</t></is></c><c r="H19" s="2" t="inlineStr" /><c r="I19" s="2" t="inlineStr" /><c r="J19" s="2" t="inlineStr" /><c r="K19" s="2" t="inlineStr"><is><t>Uzależnienie od nikotyny – klonidyna</t></is></c><c r="L19" s="2" t="inlineStr"><is><t>Uzależnienie od amfetaminy – wereniklina</t></is></c><c r="M19" s="2" t="inlineStr" /><c r="N19" s="2" t="inlineStr" /><c r="O19" s="2" t="inlineStr" /><c r="P19" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q19" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="20"><c r="A20" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B20" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C20" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D20" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E20" s="2" t="inlineStr"><is><t>Wskaż prawidłowe pary płyn infuzyjny – możliwe działania niepożądane:</t></is></c><c r="F20" s="2" t="inlineStr"><is><t>5% roztwór glukozy – hiponatremia</t></is></c><c r="G20" s="2" t="inlineStr"><is><t>HES (hydroksyetylowana skrobia) – ostre uszkodzenie nerek</t></is></c><c r="H20" s="2" t="inlineStr"><is><t>5% roztwór albuminy – anafilaksja</t></is></c><c r="I20" s="2" t="inlineStr"><is><t>Dekstran 70000 – działanie przeciwkrzepliwe</t></is></c><c r="J20" s="2" t="inlineStr" /><c r="K20" s="2" t="inlineStr" /><c r="L20" s="2" t="inlineStr" /><c r="M20" s="2" t="inlineStr" /><c r="N20" s="2" t="inlineStr" /><c r="O20" s="2" t="inlineStr" /><c r="P20" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q20" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="21"><c r="A21" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B21" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C21" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D21" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E21" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące leczenia hipotensyjnego:</t></is></c><c r="F21" s="2" t="inlineStr"><is><t>Tiazydy mogą bezpośrednio oddziaływać na ścianę naczyń i zmniejszać systemowy opór naczyniowy</t></is></c><c r="G21" s="2" t="inlineStr"><is><t>Pełny efekt hipotensyjny występuje po kilkunastu dniach leczenia</t></is></c><c r="H21" s="2" t="inlineStr"><is><t>Blokada kotransportera Na-Cl w kanaliku dystalnym prowadzi do zwiększeniu natriurezy</t></is></c><c r="I21" s="2" t="inlineStr" /><c r="J21" s="2" t="inlineStr" /><c r="K21" s="2" t="inlineStr"><is><t>Ich skuteczność w leczeniu przewlekłym wynika przede wszystkim ze zmniejszenia objętości osocza i rzutu serca</t></is></c><c r="L21" s="2" t="inlineStr" /><c r="M21" s="2" t="inlineStr" /><c r="N21" s="2" t="inlineStr" /><c r="O21" s="2" t="inlineStr" /><c r="P21" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q21" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="22"><c r="A22" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B22" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C22" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D22" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E22" s="2" t="inlineStr"><is><t>Suksametonium może być przyczyną:</t></is></c><c r="F22" s="2" t="inlineStr"><is><t>Drżenia włókienkowego mięśni szkieletowych</t></is></c><c r="G22" s="2" t="inlineStr"><is><t>Zaburzeń oddychania</t></is></c><c r="H22" s="2" t="inlineStr"><is><t>Zespołu hipertermii złośliwej</t></is></c><c r="I22" s="2" t="inlineStr"><is><t>Długotrwałego efektu zwiotczającego u osób z dysfunkcją acetylocholinesterazy</t></is></c><c r="J22" s="2" t="inlineStr" /><c r="K22" s="2" t="inlineStr" /><c r="L22" s="2" t="inlineStr" /><c r="M22" s="2" t="inlineStr" /><c r="N22" s="2" t="inlineStr" /><c r="O22" s="2" t="inlineStr" /><c r="P22" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q22" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="23"><c r="A23" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B23" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C23" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D23" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E23" s="2" t="inlineStr"><is><t>W celu łagodzenia suchego kaszlu można wybrać:</t></is></c><c r="F23" s="2" t="inlineStr"><is><t>Dekstrometorfan</t></is></c><c r="G23" s="2" t="inlineStr"><is><t>Kodeinę</t></is></c><c r="H23" s="2" t="inlineStr"><is><t>Butamirat</t></is></c><c r="I23" s="2" t="inlineStr" /><c r="J23" s="2" t="inlineStr" /><c r="K23" s="2" t="inlineStr"><is><t>Bromheksynę</t></is></c><c r="L23" s="2" t="inlineStr" /><c r="M23" s="2" t="inlineStr" /><c r="N23" s="2" t="inlineStr" /><c r="O23" s="2" t="inlineStr" /><c r="P23" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q23" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="24"><c r="A24" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B24" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C24" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D24" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E24" s="2" t="inlineStr"><is><t>Albendazol stosowany jest w jelitowej infestacji:</t></is></c><c r="F24" s="2" t="inlineStr"><is><t>Glistą ludzką</t></is></c><c r="G24" s="2" t="inlineStr"><is><t>Tasiemcem uzbrojonym</t></is></c><c r="H24" s="2" t="inlineStr"><is><t>Owsikami</t></is></c><c r="I24" s="2" t="inlineStr" /><c r="J24" s="2" t="inlineStr" /><c r="K24" s="2" t="inlineStr"><is><t>Lambliami</t></is></c><c r="L24" s="2" t="inlineStr" /><c r="M24" s="2" t="inlineStr" /><c r="N24" s="2" t="inlineStr" /><c r="O24" s="2" t="inlineStr" /><c r="P24" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q24" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="25"><c r="A25" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B25" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C25" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D25" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E25" s="2" t="inlineStr"><is><t>Napad paniki należy leczyć stosując doraźnie:</t></is></c><c r="F25" s="2" t="inlineStr"><is><t>Techniki relaksacyjne</t></is></c><c r="G25" s="2" t="inlineStr"><is><t>Alprazolam</t></is></c><c r="H25" s="2" t="inlineStr" /><c r="I25" s="2" t="inlineStr" /><c r="J25" s="2" t="inlineStr" /><c r="K25" s="2" t="inlineStr"><is><t>Pregabalinę</t></is></c><c r="L25" s="2" t="inlineStr"><is><t>Fluoksetynę</t></is></c><c r="M25" s="2" t="inlineStr" /><c r="N25" s="2" t="inlineStr" /><c r="O25" s="2" t="inlineStr" /><c r="P25" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q25" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="26"><c r="A26" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B26" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C26" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D26" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E26" s="2" t="inlineStr"><is><t>Fenoterol może być przyczyną:</t></is></c><c r="F26" s="2" t="inlineStr"><is><t>Tachykardii</t></is></c><c r="G26" s="2" t="inlineStr"><is><t>Drżenia mięśni</t></is></c><c r="H26" s="2" t="inlineStr"><is><t>Hiperglikemii</t></is></c><c r="I26" s="2" t="inlineStr"><is><t>Hamowania skurczów ciężarnej macicy</t></is></c><c r="J26" s="2" t="inlineStr" /><c r="K26" s="2" t="inlineStr" /><c r="L26" s="2" t="inlineStr" /><c r="M26" s="2" t="inlineStr" /><c r="N26" s="2" t="inlineStr" /><c r="O26" s="2" t="inlineStr" /><c r="P26" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q26" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="27"><c r="A27" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B27" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C27" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D27" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E27" s="2" t="inlineStr"><is><t>Długo działające beta2-mimetyki (LABA):</t></is></c><c r="F27" s="2" t="inlineStr"><is><t>Podawane przewlekle powodują down-regulację receptorów beta2-adrenergicznych w oskrzelach</t></is></c><c r="G27" s="2" t="inlineStr" /><c r="H27" s="2" t="inlineStr" /><c r="I27" s="2" t="inlineStr" /><c r="J27" s="2" t="inlineStr" /><c r="K27" s="2" t="inlineStr"><is><t>Nie powinny być podawane razem z glikokortykosteroidami które blokują wytwarzanie białek receptorów beta2-adrenergicznych</t></is></c><c r="L27" s="2" t="inlineStr"><is><t>Mogą być przyczyną istotnej klinicznie hieprkaliemi</t></is></c><c r="M27" s="2" t="inlineStr"><is><t>Wykazują działanie przeciwzapalne</t></is></c><c r="N27" s="2" t="inlineStr" /><c r="O27" s="2" t="inlineStr" /><c r="P27" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q27" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="28"><c r="A28" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B28" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C28" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D28" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E28" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące NLPZ:</t></is></c><c r="F28" s="2" t="inlineStr"><is><t>Ketoprofen powoduje większe ryzyko krwawienia z górnego odcinka przewodu pokarmowego niż ibuprofen</t></is></c><c r="G28" s="2" t="inlineStr" /><c r="H28" s="2" t="inlineStr" /><c r="I28" s="2" t="inlineStr" /><c r="J28" s="2" t="inlineStr" /><c r="K28" s="2" t="inlineStr"><is><t>Meloksykam jest preferencyjnym inhibitorem COX-1</t></is></c><c r="L28" s="2" t="inlineStr"><is><t>Zastąpienie drogi doustnej podania diklofenaku drogą doodbytniczą zmniejsza ryzyko wystąpienia działań niepożądanych</t></is></c><c r="M28" s="2" t="inlineStr"><is><t>Nimesulid należy do najmniej hepatotoksycznych NLPZ</t></is></c><c r="N28" s="2" t="inlineStr" /><c r="O28" s="2" t="inlineStr" /><c r="P28" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q28" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="29"><c r="A29" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B29" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C29" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D29" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E29" s="2" t="inlineStr"><is><t>Lekiem prkeursorowym jest:</t></is></c><c r="F29" s="2" t="inlineStr"><is><t>Enalapryl</t></is></c><c r="G29" s="2" t="inlineStr"><is><t>Cyklezonid</t></is></c><c r="H29" s="2" t="inlineStr"><is><t>Lewodopa</t></is></c><c r="I29" s="2" t="inlineStr" /><c r="J29" s="2" t="inlineStr" /><c r="K29" s="2" t="inlineStr"><is><t>Furosemid</t></is></c><c r="L29" s="2" t="inlineStr" /><c r="M29" s="2" t="inlineStr" /><c r="N29" s="2" t="inlineStr" /><c r="O29" s="2" t="inlineStr" /><c r="P29" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q29" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="30"><c r="A30" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B30" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C30" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D30" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E30" s="2" t="inlineStr"><is><t>Cyklosporyna:</t></is></c><c r="F30" s="2" t="inlineStr"><is><t>Jest stosowana w zapobieganiu odrzucania przeszczepu allogenicznego narządów unaczynionych</t></is></c><c r="G30" s="2" t="inlineStr"><is><t>Zwiększa ryzyko chorób rozrostowych układu chłonnego</t></is></c><c r="H30" s="2" t="inlineStr" /><c r="I30" s="2" t="inlineStr" /><c r="J30" s="2" t="inlineStr" /><c r="K30" s="2" t="inlineStr"><is><t>Jest rekombinowanym w pełni ludzkim przeciwciałem monoklonalnym</t></is></c><c r="L30" s="2" t="inlineStr"><is><t>Neutralizuje biologiczną aktywność TNF</t></is></c><c r="M30" s="2" t="inlineStr" /><c r="N30" s="2" t="inlineStr" /><c r="O30" s="2" t="inlineStr" /><c r="P30" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q30" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="31"><c r="A31" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B31" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C31" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D31" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E31" s="2" t="inlineStr"><is><t>Cyklosporyna</t></is></c><c r="F31" s="2" t="inlineStr"><is><t>Jest eliminowana przez wątrobę</t></is></c><c r="G31" s="2" t="inlineStr"><is><t>Jest stosowana w celu zapobiegania odrzucania przeszczepów</t></is></c><c r="H31" s="2" t="inlineStr" /><c r="I31" s="2" t="inlineStr" /><c r="J31" s="2" t="inlineStr" /><c r="K31" s="2" t="inlineStr"><is><t>Jest aktywatorem kalcyneuryny</t></is></c><c r="L31" s="2" t="inlineStr"><is><t>Może powodować atrofię dziąseł</t></is></c><c r="M31" s="2" t="inlineStr" /><c r="N31" s="2" t="inlineStr" /><c r="O31" s="2" t="inlineStr" /><c r="P31" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q31" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="32"><c r="A32" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B32" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C32" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D32" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E32" s="2" t="inlineStr"><is><t>Do leków o udowodnionym korzystnym działaniu w profilaktyce wtórnej niedokrwiennego udaru mózgu należy:</t></is></c><c r="F32" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="G32" s="2" t="inlineStr"><is><t>Atorwastatyna</t></is></c><c r="H32" s="2" t="inlineStr"><is><t>Klopidogrel</t></is></c><c r="I32" s="2" t="inlineStr" /><c r="J32" s="2" t="inlineStr" /><c r="K32" s="2" t="inlineStr"><is><t>Kwas traneksamowy</t></is></c><c r="L32" s="2" t="inlineStr" /><c r="M32" s="2" t="inlineStr" /><c r="N32" s="2" t="inlineStr" /><c r="O32" s="2" t="inlineStr" /><c r="P32" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q32" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="33"><c r="A33" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B33" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C33" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D33" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E33" s="2" t="inlineStr"><is><t>Lewodopa:</t></is></c><c r="F33" s="2" t="inlineStr"><is><t>Jest jednym z najskuteczniejszych leków stosowanych w terapii choroby Parkinsona</t></is></c><c r="G33" s="2" t="inlineStr"><is><t>Ma krótki okres półtrwania i dlatego wymaga wielokrotnego podawania w ciągu doby</t></is></c><c r="H33" s="2" t="inlineStr"><is><t>Podczas długotrwałego leczenia może wywołać fluktuacje ruchowe i dyskinezy</t></is></c><c r="I33" s="2" t="inlineStr"><is><t>Może wywoływać działania niepożądane ze strony przewodu pokarmowego</t></is></c><c r="J33" s="2" t="inlineStr" /><c r="K33" s="2" t="inlineStr" /><c r="L33" s="2" t="inlineStr" /><c r="M33" s="2" t="inlineStr" /><c r="N33" s="2" t="inlineStr" /><c r="O33" s="2" t="inlineStr" /><c r="P33" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q33" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="34"><c r="A34" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B34" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C34" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D34" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E34" s="2" t="inlineStr"><is><t>Kokaina:</t></is></c><c r="F34" s="2" t="inlineStr"><is><t>Hamuje wychwyt zwrotny dopaminy w szczelinie synaptycznej</t></is></c><c r="G34" s="2" t="inlineStr"><is><t>Może powodować wystąpienie zawału mięśnia sercowego</t></is></c><c r="H34" s="2" t="inlineStr"><is><t>Może powodować krwawienia wewnątrzczaszkowe</t></is></c><c r="I34" s="2" t="inlineStr" /><c r="J34" s="2" t="inlineStr" /><c r="K34" s="2" t="inlineStr"><is><t>Hamuje aktywność receptora dla kwasu glutaminowego</t></is></c><c r="L34" s="2" t="inlineStr" /><c r="M34" s="2" t="inlineStr" /><c r="N34" s="2" t="inlineStr" /><c r="O34" s="2" t="inlineStr" /><c r="P34" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q34" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="35"><c r="A35" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B35" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C35" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D35" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E35" s="2" t="inlineStr"><is><t>W alergicznym zapaleniu spojówek może stosować dospojówkowo:</t></is></c><c r="F35" s="2" t="inlineStr"><is><t>Antazolinę</t></is></c><c r="G35" s="2" t="inlineStr"><is><t>Azelastynę</t></is></c><c r="H35" s="2" t="inlineStr"><is><t>Kromoglikan sodowy</t></is></c><c r="I35" s="2" t="inlineStr"><is><t>Olopatadynę</t></is></c><c r="J35" s="2" t="inlineStr" /><c r="K35" s="2" t="inlineStr" /><c r="L35" s="2" t="inlineStr" /><c r="M35" s="2" t="inlineStr" /><c r="N35" s="2" t="inlineStr" /><c r="O35" s="2" t="inlineStr" /><c r="P35" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q35" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="36"><c r="A36" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B36" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C36" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D36" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E36" s="2" t="inlineStr"><is><t>Stosowanie preparatu złożonego bupropionu z naltreksonem w leczeniu otyłości:</t></is></c><c r="F36" s="2" t="inlineStr"><is><t>Ma wpływ na ośrodkowy układ nagrody</t></is></c><c r="G36" s="2" t="inlineStr"><is><t>Zwiększa i wydłuża uczucie sytości</t></is></c><c r="H36" s="2" t="inlineStr"><is><t>Ma zwiększoną skuteczność kliniczną ze względu na efekt synergistyczny bupropionu i naltreksonu</t></is></c><c r="I36" s="2" t="inlineStr" /><c r="J36" s="2" t="inlineStr" /><c r="K36" s="2" t="inlineStr"><is><t>Jest wskazane dla wszystkich osób z wyjściową wartością BMI wynoszącą ≥27</t></is></c><c r="L36" s="2" t="inlineStr" /><c r="M36" s="2" t="inlineStr" /><c r="N36" s="2" t="inlineStr" /><c r="O36" s="2" t="inlineStr" /><c r="P36" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q36" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="37"><c r="A37" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B37" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C37" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D37" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E37" s="2" t="inlineStr"><is><t>Dodatek adrenaliny do lidokainy w lekach do znieczulania miejscowego może powodować:</t></is></c><c r="F37" s="2" t="inlineStr"><is><t>Zwiększone ryzyko martwicy tkanek po podaniach obwodowych</t></is></c><c r="G37" s="2" t="inlineStr"><is><t>Wydłużenie czasu działania lidokainy</t></is></c><c r="H37" s="2" t="inlineStr" /><c r="I37" s="2" t="inlineStr" /><c r="J37" s="2" t="inlineStr" /><c r="K37" s="2" t="inlineStr"><is><t>Zwiększone niebezpieczeństwo zatrzymania oddechu</t></is></c><c r="L37" s="2" t="inlineStr"><is><t>Zahamowanie metabolizmu lidokainy</t></is></c><c r="M37" s="2" t="inlineStr" /><c r="N37" s="2" t="inlineStr" /><c r="O37" s="2" t="inlineStr" /><c r="P37" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q37" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="38"><c r="A38" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B38" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C38" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D38" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E38" s="2" t="inlineStr"><is><t>Digoksyna</t></is></c><c r="F38" s="2" t="inlineStr"><is><t>Podtrzymuje aktywację baroreceptorów zatoki szyjnej przy obniżeniu ciśnienia krwi u osób z niewydolnością serca</t></is></c><c r="G38" s="2" t="inlineStr"><is><t>Podana doustnie może być nieskuteczna z powodu dezaktywacji przez bakterie jelitowe</t></is></c><c r="H38" s="2" t="inlineStr" /><c r="I38" s="2" t="inlineStr" /><c r="J38" s="2" t="inlineStr" /><c r="K38" s="2" t="inlineStr"><is><t>Powoduje kardiowersję migotania przedsionków do rytmu zatokowego</t></is></c><c r="L38" s="2" t="inlineStr"><is><t>Jest lekiem o korzystnym działaniu rokowniczym w skurczowej niewydolności serca</t></is></c><c r="M38" s="2" t="inlineStr" /><c r="N38" s="2" t="inlineStr" /><c r="O38" s="2" t="inlineStr" /><c r="P38" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q38" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="39"><c r="A39" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B39" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C39" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D39" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E39" s="2" t="inlineStr"><is><t>Digoksyna:</t></is></c><c r="F39" s="2" t="inlineStr"><is><t>aktywuje układ przywspółczulny</t></is></c><c r="G39" s="2" t="inlineStr"><is><t>wywiera arytmie i zaburzenia przewodzenia</t></is></c><c r="H39" s="2" t="inlineStr"><is><t>jest stosowana w celu kontroli częstotliwości rytmu komór u chorych z migotaniem przedsionków</t></is></c><c r="I39" s="2" t="inlineStr"><is><t>w zatruciu można zastosować fragmenty Fab przeciwciał wiążących</t></is></c><c r="J39" s="2" t="inlineStr" /><c r="K39" s="2" t="inlineStr" /><c r="L39" s="2" t="inlineStr" /><c r="M39" s="2" t="inlineStr" /><c r="N39" s="2" t="inlineStr" /><c r="O39" s="2" t="inlineStr" /><c r="P39" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q39" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="40"><c r="A40" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B40" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C40" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D40" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E40" s="2" t="inlineStr"><is><t>Digoksyna:</t></is></c><c r="F40" s="2" t="inlineStr"><is><t>zmniejsza aktywację układu współczulnego u osób z niewydolnością serca</t></is></c><c r="G40" s="2" t="inlineStr"><is><t>może sprzyjać wystąpieniu depresji</t></is></c><c r="H40" s="2" t="inlineStr"><is><t>jest stosowana w celu kontroli rytmu serca w utrwalonym migotaniu przedsionków</t></is></c><c r="I40" s="2" t="inlineStr"><is><t>może być nieskuteczna z powodu dezaktywacji przez bakterie jelitowe</t></is></c><c r="J40" s="2" t="inlineStr" /><c r="K40" s="2" t="inlineStr" /><c r="L40" s="2" t="inlineStr" /><c r="M40" s="2" t="inlineStr" /><c r="N40" s="2" t="inlineStr" /><c r="O40" s="2" t="inlineStr" /><c r="P40" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q40" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="41"><c r="A41" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B41" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C41" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D41" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E41" s="2" t="inlineStr"><is><t>Teoretyczną przesłanką stosowania beta-adrenolityków w przewlekłej skurczowej niewydolności serca jest:</t></is></c><c r="F41" s="2" t="inlineStr"><is><t>Odwracanie beta-down regulacji</t></is></c><c r="G41" s="2" t="inlineStr"><is><t>Zapobieganie proarytmicznemu działaniu katecholamin</t></is></c><c r="H41" s="2" t="inlineStr" /><c r="I41" s="2" t="inlineStr" /><c r="J41" s="2" t="inlineStr" /><c r="K41" s="2" t="inlineStr"><is><t>Korzystny bezpośredni wpływ hemodynamiczny</t></is></c><c r="L41" s="2" t="inlineStr"><is><t>Zwiększenie naprężenia ściany lewej komory</t></is></c><c r="M41" s="2" t="inlineStr" /><c r="N41" s="2" t="inlineStr" /><c r="O41" s="2" t="inlineStr" /><c r="P41" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q41" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="42"><c r="A42" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B42" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C42" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D42" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E42" s="2" t="inlineStr"><is><t>Rupatadyna:</t></is></c><c r="F42" s="2" t="inlineStr"><is><t>Ma minimalny potencjał sedatywny</t></is></c><c r="G42" s="2" t="inlineStr"><is><t>Oprócz antagonizmu wobec receptora H1 wykazuje przeciwzapalną aktywność pozareceptorową</t></is></c><c r="H42" s="2" t="inlineStr"><is><t>W znacznym stopniu ulega efektowi pierwszego przejścia z powstaniem aktywnych metabolitów</t></is></c><c r="I42" s="2" t="inlineStr"><is><t>W dawkach zalecanych nie wydłuża skorygowanego odstępu cQT</t></is></c><c r="J42" s="2" t="inlineStr" /><c r="K42" s="2" t="inlineStr" /><c r="L42" s="2" t="inlineStr" /><c r="M42" s="2" t="inlineStr" /><c r="N42" s="2" t="inlineStr" /><c r="O42" s="2" t="inlineStr" /><c r="P42" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q42" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="43"><c r="A43" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B43" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C43" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D43" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E43" s="2" t="inlineStr"><is><t>Rupatadyna:</t></is></c><c r="F43" s="2" t="inlineStr"><is><t>jest selektywnym niesedatywnym antagonistą receptorów H1</t></is></c><c r="G43" s="2" t="inlineStr"><is><t>hamuje degranulację komórek tucznych in vitro</t></is></c><c r="H43" s="2" t="inlineStr"><is><t>ma aktywny metabolit – desloratadynę zaliczaną do 3 generacji leków przeciwhistaminowych</t></is></c><c r="I43" s="2" t="inlineStr"><is><t>w dawkach zalecanych nie wydłuża odstępu QTc</t></is></c><c r="J43" s="2" t="inlineStr" /><c r="K43" s="2" t="inlineStr" /><c r="L43" s="2" t="inlineStr" /><c r="M43" s="2" t="inlineStr" /><c r="N43" s="2" t="inlineStr" /><c r="O43" s="2" t="inlineStr" /><c r="P43" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q43" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="44"><c r="A44" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B44" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C44" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D44" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E44" s="2" t="inlineStr"><is><t>U pacjentów z eGFR&lt;30ml/min należy rezygnować ze stosowania:</t></is></c><c r="F44" s="2" t="inlineStr"><is><t>Metyforminy</t></is></c><c r="G44" s="2" t="inlineStr"><is><t>Hydrochlorotiazydu</t></is></c><c r="H44" s="2" t="inlineStr" /><c r="I44" s="2" t="inlineStr" /><c r="J44" s="2" t="inlineStr" /><c r="K44" s="2" t="inlineStr"><is><t>Metoprololu</t></is></c><c r="L44" s="2" t="inlineStr"><is><t>Amlodypiny</t></is></c><c r="M44" s="2" t="inlineStr" /><c r="N44" s="2" t="inlineStr" /><c r="O44" s="2" t="inlineStr" /><c r="P44" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q44" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="45"><c r="A45" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B45" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C45" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D45" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E45" s="2" t="inlineStr"><is><t>Wenlafaksyna:</t></is></c><c r="F45" s="2" t="inlineStr"><is><t>Może być podawana w uogólnionych zaburzeniach lękowych</t></is></c><c r="G45" s="2" t="inlineStr"><is><t>Stosowana razem z tryptanami może powodować wystąpienie zespołu serotoninowego</t></is></c><c r="H45" s="2" t="inlineStr" /><c r="I45" s="2" t="inlineStr" /><c r="J45" s="2" t="inlineStr" /><c r="K45" s="2" t="inlineStr"><is><t>Ma istotne działanie cholinolityczne</t></is></c><c r="L45" s="2" t="inlineStr"><is><t>Można ją bezpiecznie stosować w terapii skojarzonej z inhibitorami MAO</t></is></c><c r="M45" s="2" t="inlineStr" /><c r="N45" s="2" t="inlineStr" /><c r="O45" s="2" t="inlineStr" /><c r="P45" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q45" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="46"><c r="A46" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B46" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C46" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D46" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E46" s="2" t="inlineStr"><is><t>Czy słuszna jest przedstawiona interpretacja działania leku na podstawie nazwy międzynarodowej:</t></is></c><c r="F46" s="2" t="inlineStr"><is><t>Paliwizumab – humanizowane przeciwciało monoklonalne o działaniu p￾wirusowym</t></is></c><c r="G46" s="2" t="inlineStr"><is><t>Ekulizumab – humanizowane przeciwciało monoklonalne o wpływie na układ odpornościowy</t></is></c><c r="H46" s="2" t="inlineStr" /><c r="I46" s="2" t="inlineStr" /><c r="J46" s="2" t="inlineStr" /><c r="K46" s="2" t="inlineStr"><is><t>Ofatumumab – mysie przeciwciało monoklonalne o wpływie p-nowotworowym</t></is></c><c r="L46" s="2" t="inlineStr"><is><t>Pomalidomid – mysie przeciwciało monoklonalne o wpływie na układ odpornościowy</t></is></c><c r="M46" s="2" t="inlineStr" /><c r="N46" s="2" t="inlineStr" /><c r="O46" s="2" t="inlineStr" /><c r="P46" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q46" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="47"><c r="A47" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B47" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C47" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D47" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E47" s="2" t="inlineStr"><is><t>Do przeciwciał monoklonalnych anty-TNF należy:</t></is></c><c r="F47" s="2" t="inlineStr"><is><t>Adalimumab</t></is></c><c r="G47" s="2" t="inlineStr" /><c r="H47" s="2" t="inlineStr" /><c r="I47" s="2" t="inlineStr" /><c r="J47" s="2" t="inlineStr" /><c r="K47" s="2" t="inlineStr"><is><t>Omalizumab</t></is></c><c r="L47" s="2" t="inlineStr"><is><t>Trastuzumab</t></is></c><c r="M47" s="2" t="inlineStr"><is><t>Rytuksymab</t></is></c><c r="N47" s="2" t="inlineStr" /><c r="O47" s="2" t="inlineStr" /><c r="P47" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q47" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="48"><c r="A48" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B48" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C48" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D48" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E48" s="2" t="inlineStr"><is><t>Werapamil można stosować w:</t></is></c><c r="F48" s="2" t="inlineStr"><is><t>Postaci naczynioskurczowej choroby niedokrwiennej serca</t></is></c><c r="G48" s="2" t="inlineStr"><is><t>Napadowym częstoskurczu z łącza przedsionkowo-komorowego</t></is></c><c r="H48" s="2" t="inlineStr" /><c r="I48" s="2" t="inlineStr" /><c r="J48" s="2" t="inlineStr" /><c r="K48" s="2" t="inlineStr"><is><t>Bradykardii</t></is></c><c r="L48" s="2" t="inlineStr"><is><t>Migotaniu przedsionków u osób z zespołem preekscytacji</t></is></c><c r="M48" s="2" t="inlineStr" /><c r="N48" s="2" t="inlineStr" /><c r="O48" s="2" t="inlineStr" /><c r="P48" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q48" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="49"><c r="A49" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B49" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C49" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D49" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E49" s="2" t="inlineStr"><is><t>Inhibitory neprylizyny:</t></is></c><c r="F49" s="2" t="inlineStr"><is><t>Zmniejszają przebudowę mięśnia sercowego</t></is></c><c r="G49" s="2" t="inlineStr"><is><t>Zwiększają stężenie angiotensyny II</t></is></c><c r="H49" s="2" t="inlineStr"><is><t>Są stosowane w przewlekłej niewydolności serca z upośledzoną frakcją wyrzutową</t></is></c><c r="I49" s="2" t="inlineStr" /><c r="J49" s="2" t="inlineStr" /><c r="K49" s="2" t="inlineStr"><is><t>Rozkładają peptydy natriuretyczne</t></is></c><c r="L49" s="2" t="inlineStr" /><c r="M49" s="2" t="inlineStr" /><c r="N49" s="2" t="inlineStr" /><c r="O49" s="2" t="inlineStr" /><c r="P49" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q49" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="50"><c r="A50" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B50" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C50" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D50" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E50" s="2" t="inlineStr"><is><t>Biodostępność leku A po jednorazowym podaniu doustnym wynosi 50%. Tmax wynosi 30min, Cmax 2µg/dl. Oznacza to, że:</t></is></c><c r="F50" s="2" t="inlineStr"><is><t>Lek A może podlegać nawet w 50% efektowi pierwszego przejścia</t></is></c><c r="G50" s="2" t="inlineStr" /><c r="H50" s="2" t="inlineStr" /><c r="I50" s="2" t="inlineStr" /><c r="J50" s="2" t="inlineStr" /><c r="K50" s="2" t="inlineStr"><is><t>Dawka wynosiła 4µg</t></is></c><c r="L50" s="2" t="inlineStr"><is><t>Lek A słabo się wiąże z białkami krwi</t></is></c><c r="M50" s="2" t="inlineStr"><is><t>Okres półtrwania leku A wynosi również około 30min</t></is></c><c r="N50" s="2" t="inlineStr" /><c r="O50" s="2" t="inlineStr" /><c r="P50" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q50" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="51"><c r="A51" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B51" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C51" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D51" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E51" s="2" t="inlineStr"><is><t>Podanie doodbytnicze leku:</t></is></c><c r="F51" s="2" t="inlineStr"><is><t>Może łatwo doprowadzić do miejscowego uszkodzenia błony śluzowej odbytnicy</t></is></c><c r="G51" s="2" t="inlineStr" /><c r="H51" s="2" t="inlineStr" /><c r="I51" s="2" t="inlineStr" /><c r="J51" s="2" t="inlineStr" /><c r="K51" s="2" t="inlineStr"><is><t>Zwiększa efekt pierwszego przejścia</t></is></c><c r="L51" s="2" t="inlineStr"><is><t>Jest metodą z wyboru u dzieci</t></is></c><c r="M51" s="2" t="inlineStr"><is><t>Wymaga podania większej dawki leku w porównaniu do podania doustnego</t></is></c><c r="N51" s="2" t="inlineStr" /><c r="O51" s="2" t="inlineStr" /><c r="P51" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q51" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="52"><c r="A52" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B52" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C52" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D52" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E52" s="2" t="inlineStr"><is><t>Zaburzenia erekcji mogą być spowodowane stosowaniem:</t></is></c><c r="F52" s="2" t="inlineStr"><is><t>Inhibitorów 5-alfa reduktazy</t></is></c><c r="G52" s="2" t="inlineStr"><is><t>Tiazydów moczopędnych</t></is></c><c r="H52" s="2" t="inlineStr"><is><t>Beta-adrenolityków niekardioselektywnych</t></is></c><c r="I52" s="2" t="inlineStr"><is><t>Inhibitorów wychwytu zwrotnego serotoniny</t></is></c><c r="J52" s="2" t="inlineStr" /><c r="K52" s="2" t="inlineStr" /><c r="L52" s="2" t="inlineStr" /><c r="M52" s="2" t="inlineStr" /><c r="N52" s="2" t="inlineStr" /><c r="O52" s="2" t="inlineStr" /><c r="P52" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q52" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="53"><c r="A53" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B53" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C53" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D53" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E53" s="2" t="inlineStr"><is><t>Doneuronalny wychwyt monoamin jest hamowany przez:</t></is></c><c r="F53" s="2" t="inlineStr"><is><t>Citalopram</t></is></c><c r="G53" s="2" t="inlineStr"><is><t>Reboksetynę</t></is></c><c r="H53" s="2" t="inlineStr" /><c r="I53" s="2" t="inlineStr" /><c r="J53" s="2" t="inlineStr" /><c r="K53" s="2" t="inlineStr"><is><t>Tianeptynę</t></is></c><c r="L53" s="2" t="inlineStr"><is><t>Mirtazapinę</t></is></c><c r="M53" s="2" t="inlineStr" /><c r="N53" s="2" t="inlineStr" /><c r="O53" s="2" t="inlineStr" /><c r="P53" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q53" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="54"><c r="A54" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B54" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C54" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D54" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E54" s="2" t="inlineStr"><is><t>W leczeniu gruźlicy płucnej lekowrażliwej:</t></is></c><c r="F54" s="2" t="inlineStr"><is><t>Leczenie wyjaławiające powinno trwać co najmniej 4 miesiące</t></is></c><c r="G54" s="2" t="inlineStr"><is><t>U kobiet ciężarnych podaje się leki według zwykłego schematu z wyłączeniem streptomycyny</t></is></c><c r="H54" s="2" t="inlineStr" /><c r="I54" s="2" t="inlineStr" /><c r="J54" s="2" t="inlineStr" /><c r="K54" s="2" t="inlineStr"><is><t>W intensywnej fazie leczenia przez 2 miesiące podaje się 2 leki – rifampicynę i izoniazyd</t></is></c><c r="L54" s="2" t="inlineStr"><is><t>W fazie kontynuacji każdy pacjent powinien otrzymać etambutol</t></is></c><c r="M54" s="2" t="inlineStr" /><c r="N54" s="2" t="inlineStr" /><c r="O54" s="2" t="inlineStr" /><c r="P54" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q54" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="55"><c r="A55" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B55" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C55" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D55" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E55" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-wskazanie:</t></is></c><c r="F55" s="2" t="inlineStr"><is><t>Sulpiryd – schizofrenia</t></is></c><c r="G55" s="2" t="inlineStr"><is><t>Metylofenidat – ADHD</t></is></c><c r="H55" s="2" t="inlineStr" /><c r="I55" s="2" t="inlineStr" /><c r="J55" s="2" t="inlineStr" /><c r="K55" s="2" t="inlineStr"><is><t>Moklobemid – bezsenność</t></is></c><c r="L55" s="2" t="inlineStr"><is><t>Sertindol – depresja</t></is></c><c r="M55" s="2" t="inlineStr" /><c r="N55" s="2" t="inlineStr" /><c r="O55" s="2" t="inlineStr" /><c r="P55" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q55" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="56"><c r="A56" s="2" t="inlineStr"><is><t>LEKI NASENNE</t></is></c><c r="B56" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C56" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D56" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E56" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – wskazanie:</t></is></c><c r="F56" s="2" t="inlineStr"><is><t>zolpidem - bezsenność</t></is></c><c r="G56" s="2" t="inlineStr"><is><t>rotygotyna – zespół niespokojnych nóg</t></is></c><c r="H56" s="2" t="inlineStr"><is><t>alprazolam - napady paniki</t></is></c><c r="I56" s="2" t="inlineStr"><is><t>fluoksetyna – zaburzenia kompulsywne</t></is></c><c r="J56" s="2" t="inlineStr" /><c r="K56" s="2" t="inlineStr" /><c r="L56" s="2" t="inlineStr" /><c r="M56" s="2" t="inlineStr" /><c r="N56" s="2" t="inlineStr" /><c r="O56" s="2" t="inlineStr" /><c r="P56" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q56" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="57"><c r="A57" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B57" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C57" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D57" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E57" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – wskazanie:</t></is></c><c r="F57" s="2" t="inlineStr"><is><t>ranolazyna - stabilna choroba niedokrwienna serca</t></is></c><c r="G57" s="2" t="inlineStr" /><c r="H57" s="2" t="inlineStr" /><c r="I57" s="2" t="inlineStr" /><c r="J57" s="2" t="inlineStr" /><c r="K57" s="2" t="inlineStr"><is><t>cilostazol - ostra niewydolność mięśnia sercowego</t></is></c><c r="L57" s="2" t="inlineStr"><is><t>milrynon - migotanie przedsionków</t></is></c><c r="M57" s="2" t="inlineStr"><is><t>riocyguat - nadciśnienie tętnicze</t></is></c><c r="N57" s="2" t="inlineStr" /><c r="O57" s="2" t="inlineStr" /><c r="P57" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q57" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="58"><c r="A58" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B58" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C58" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D58" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E58" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – wskazanie:</t></is></c><c r="F58" s="2" t="inlineStr"><is><t>zolpidem-bezsenność</t></is></c><c r="G58" s="2" t="inlineStr"><is><t>ondansetron – wymioty w przebiegu chemioterapii przeciwnowotworowej</t></is></c><c r="H58" s="2" t="inlineStr"><is><t>alprazolam-napady paniki</t></is></c><c r="I58" s="2" t="inlineStr"><is><t>fluoksetyna–epizody dużej depresji</t></is></c><c r="J58" s="2" t="inlineStr" /><c r="K58" s="2" t="inlineStr" /><c r="L58" s="2" t="inlineStr" /><c r="M58" s="2" t="inlineStr" /><c r="N58" s="2" t="inlineStr" /><c r="O58" s="2" t="inlineStr" /><c r="P58" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q58" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="59"><c r="A59" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B59" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C59" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D59" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E59" s="2" t="inlineStr"><is><t>Hiperprolaktynemia może wiązać się z leczeniem:</t></is></c><c r="F59" s="2" t="inlineStr"><is><t>Promazyną</t></is></c><c r="G59" s="2" t="inlineStr"><is><t>Rysperydonem</t></is></c><c r="H59" s="2" t="inlineStr"><is><t>Metoklopramidem</t></is></c><c r="I59" s="2" t="inlineStr" /><c r="J59" s="2" t="inlineStr" /><c r="K59" s="2" t="inlineStr"><is><t>Bromokryptyną</t></is></c><c r="L59" s="2" t="inlineStr" /><c r="M59" s="2" t="inlineStr" /><c r="N59" s="2" t="inlineStr" /><c r="O59" s="2" t="inlineStr" /><c r="P59" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q59" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="60"><c r="A60" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B60" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C60" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D60" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E60" s="2" t="inlineStr"><is><t>Ośrodkowy zespół cholinolityczny może wystąpić w wyniku ostrego przedawkowania:</t></is></c><c r="F60" s="2" t="inlineStr"><is><t>Doksepiny</t></is></c><c r="G60" s="2" t="inlineStr"><is><t>Olanzapiny</t></is></c><c r="H60" s="2" t="inlineStr"><is><t>Perfenazyny</t></is></c><c r="I60" s="2" t="inlineStr"><is><t>Klemastyny</t></is></c><c r="J60" s="2" t="inlineStr" /><c r="K60" s="2" t="inlineStr" /><c r="L60" s="2" t="inlineStr" /><c r="M60" s="2" t="inlineStr" /><c r="N60" s="2" t="inlineStr" /><c r="O60" s="2" t="inlineStr" /><c r="P60" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q60" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="61"><c r="A61" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B61" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C61" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D61" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E61" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące metamizolu:</t></is></c><c r="F61" s="2" t="inlineStr"><is><t>Podczas szybkiego wstrzykiwania dożylnego leku może dojść do gwałtownych spadków ciśnienia krwi</t></is></c><c r="G61" s="2" t="inlineStr"><is><t>Może powodować ciężkie uszkodzenia szpiku w mechanizmie nadwrażliwości</t></is></c><c r="H61" s="2" t="inlineStr"><is><t>Zwiększa częstość występowania guzów Wilmsa (nephroblastoma, nerczak zarodkowy)</t></is></c><c r="I61" s="2" t="inlineStr" /><c r="J61" s="2" t="inlineStr" /><c r="K61" s="2" t="inlineStr"><is><t>Ma silne działanie przeciwzapalne</t></is></c><c r="L61" s="2" t="inlineStr" /><c r="M61" s="2" t="inlineStr" /><c r="N61" s="2" t="inlineStr" /><c r="O61" s="2" t="inlineStr" /><c r="P61" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q61" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="62"><c r="A62" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B62" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C62" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D62" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E62" s="2" t="inlineStr"><is><t>Które połączenie lekowe jest bezwzględnie konieczne w wymienionej sytuacji klinicznej:</t></is></c><c r="F62" s="2" t="inlineStr"><is><t>Sartan + sakubitryl w skurczowej niewydolności serca</t></is></c><c r="G62" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy + antagonista receptorów P2Y12 po angioplastyce wieńcowej z implantacją stentu</t></is></c><c r="H62" s="2" t="inlineStr" /><c r="I62" s="2" t="inlineStr" /><c r="J62" s="2" t="inlineStr" /><c r="K62" s="2" t="inlineStr"><is><t>Heparyna drobnocząsteczkowa + ksaban w początkowym okresie leczenia żylnej choroby zakrzepowo zatorowej</t></is></c><c r="L62" s="2" t="inlineStr"><is><t>Adrenalina + atropina w resuscytacji krążeniowo-oddechowej w przebiegu NZK z asystolią</t></is></c><c r="M62" s="2" t="inlineStr" /><c r="N62" s="2" t="inlineStr" /><c r="O62" s="2" t="inlineStr" /><c r="P62" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q62" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="63"><c r="A63" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B63" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C63" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D63" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E63" s="2" t="inlineStr"><is><t>Efekt prokinetyczny można uzyskać:</t></is></c><c r="F63" s="2" t="inlineStr"><is><t>Pobudzając receptory 5-HT4</t></is></c><c r="G63" s="2" t="inlineStr"><is><t>Blokując receptory dopaminowe D2</t></is></c><c r="H63" s="2" t="inlineStr"><is><t>Hamując aktywność acetylocholinoesterazy</t></is></c><c r="I63" s="2" t="inlineStr"><is><t>Pobudzając receptory motylinowe</t></is></c><c r="J63" s="2" t="inlineStr" /><c r="K63" s="2" t="inlineStr" /><c r="L63" s="2" t="inlineStr" /><c r="M63" s="2" t="inlineStr" /><c r="N63" s="2" t="inlineStr" /><c r="O63" s="2" t="inlineStr" /><c r="P63" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q63" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="64"><c r="A64" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B64" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C64" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D64" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E64" s="2" t="inlineStr"><is><t>Glukagon:</t></is></c><c r="F64" s="2" t="inlineStr"><is><t>Stosowany jest w leczeniu ciężkiej hipoglikemii gdy nie można podać dożylnie glukozy</t></is></c><c r="G64" s="2" t="inlineStr"><is><t>Jest podawany parenteralnie</t></is></c><c r="H64" s="2" t="inlineStr"><is><t>Ma zastosowanie w zatruciach lekami beta-adrenolitycznymi</t></is></c><c r="I64" s="2" t="inlineStr"><is><t>Jest nieskuteczny w przypadku glikemii</t></is></c><c r="J64" s="2" t="inlineStr" /><c r="K64" s="2" t="inlineStr" /><c r="L64" s="2" t="inlineStr" /><c r="M64" s="2" t="inlineStr" /><c r="N64" s="2" t="inlineStr" /><c r="O64" s="2" t="inlineStr" /><c r="P64" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q64" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="65"><c r="A65" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B65" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C65" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D65" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E65" s="2" t="inlineStr"><is><t>Ryzyko encefalopatii w przebiegu marskości wątroby zmniejsza stosowanie:</t></is></c><c r="F65" s="2" t="inlineStr"><is><t>Ryfaksyminy</t></is></c><c r="G65" s="2" t="inlineStr"><is><t>Asparaginianu ornityny</t></is></c><c r="H65" s="2" t="inlineStr"><is><t>Laktulozy</t></is></c><c r="I65" s="2" t="inlineStr" /><c r="J65" s="2" t="inlineStr" /><c r="K65" s="2" t="inlineStr"><is><t>Benzodiazepin</t></is></c><c r="L65" s="2" t="inlineStr" /><c r="M65" s="2" t="inlineStr" /><c r="N65" s="2" t="inlineStr" /><c r="O65" s="2" t="inlineStr" /><c r="P65" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q65" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="66"><c r="A66" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B66" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C66" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D66" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E66" s="2" t="inlineStr"><is><t>W celu przerwania ataku duszności uzasadnione jest podanie wziewne:</t></is></c><c r="F66" s="2" t="inlineStr"><is><t>Bromku ipratriopium</t></is></c><c r="G66" s="2" t="inlineStr"><is><t>Salbutamolu</t></is></c><c r="H66" s="2" t="inlineStr" /><c r="I66" s="2" t="inlineStr" /><c r="J66" s="2" t="inlineStr" /><c r="K66" s="2" t="inlineStr"><is><t>Roflumilastu</t></is></c><c r="L66" s="2" t="inlineStr"><is><t>flutykazonu</t></is></c><c r="M66" s="2" t="inlineStr" /><c r="N66" s="2" t="inlineStr" /><c r="O66" s="2" t="inlineStr" /><c r="P66" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q66" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="67"><c r="A67" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B67" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C67" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D67" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E67" s="2" t="inlineStr"><is><t>W leczeniu małopłytkowości stosuje się:</t></is></c><c r="F67" s="2" t="inlineStr"><is><t>Preparaty immunoglobulin poliwalentnych</t></is></c><c r="G67" s="2" t="inlineStr"><is><t>Eltrombopag</t></is></c><c r="H67" s="2" t="inlineStr"><is><t>Romiplostym</t></is></c><c r="I67" s="2" t="inlineStr"><is><t>Prednizon</t></is></c><c r="J67" s="2" t="inlineStr" /><c r="K67" s="2" t="inlineStr" /><c r="L67" s="2" t="inlineStr" /><c r="M67" s="2" t="inlineStr" /><c r="N67" s="2" t="inlineStr" /><c r="O67" s="2" t="inlineStr" /><c r="P67" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q67" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="68"><c r="A68" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B68" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C68" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D68" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E68" s="2" t="inlineStr"><is><t>Ewerolimus jest stosowany w:</t></is></c><c r="F68" s="2" t="inlineStr"><is><t>Kardiologii (stenty wieńcowe)</t></is></c><c r="G68" s="2" t="inlineStr"><is><t>Onkologii (wybrane zaawansowane nowotwory piersi i nerki)</t></is></c><c r="H68" s="2" t="inlineStr" /><c r="I68" s="2" t="inlineStr" /><c r="J68" s="2" t="inlineStr" /><c r="K68" s="2" t="inlineStr"><is><t>Neurologii (stwardnienie rozsiane)</t></is></c><c r="L68" s="2" t="inlineStr"><is><t>Dermatologii (łuszczyca)</t></is></c><c r="M68" s="2" t="inlineStr" /><c r="N68" s="2" t="inlineStr" /><c r="O68" s="2" t="inlineStr" /><c r="P68" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q68" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="69"><c r="A69" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B69" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C69" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D69" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E69" s="2" t="inlineStr"><is><t>Wskaż prawdziwe zdanie:</t></is></c><c r="F69" s="2" t="inlineStr"><is><t>W chromaniu przestankowym znaczenie kliniczne ma leczenie przeciwpłytkowe i hipolipemizujące</t></is></c><c r="G69" s="2" t="inlineStr"><is><t>Zaleca się podawanie inhibitora P2Y12 przed przezskórną interwencją wieńcową u osoby z ostrym zespołem wieńcowym, a następnie kontynuację tego leczenia przez co najmniej 12 miesięcy</t></is></c><c r="H69" s="2" t="inlineStr"><is><t>Po rozpoczęciu leczenia inhibitorami konwertazy angiotensyny należy się spodziewać niewielkiego wzrostu stężenia kreatyniny we krwi</t></is></c><c r="I69" s="2" t="inlineStr" /><c r="J69" s="2" t="inlineStr" /><c r="K69" s="2" t="inlineStr"><is><t>Niedihydropirydynowi antagoniści wapnia są wskazani w leczeniu pacjentów z niewydolnością serca z obniżoną frakcją wyrzutową</t></is></c><c r="L69" s="2" t="inlineStr" /><c r="M69" s="2" t="inlineStr" /><c r="N69" s="2" t="inlineStr" /><c r="O69" s="2" t="inlineStr" /><c r="P69" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q69" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="70"><c r="A70" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B70" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C70" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D70" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E70" s="2" t="inlineStr"><is><t>U osób z pierwotnym wydłużenie QTc bezpieczne jest zastosowanie:</t></is></c><c r="F70" s="2" t="inlineStr"><is><t>Propranololu</t></is></c><c r="G70" s="2" t="inlineStr" /><c r="H70" s="2" t="inlineStr" /><c r="I70" s="2" t="inlineStr" /><c r="J70" s="2" t="inlineStr" /><c r="K70" s="2" t="inlineStr"><is><t>Digoksyny</t></is></c><c r="L70" s="2" t="inlineStr"><is><t>Sotalolu</t></is></c><c r="M70" s="2" t="inlineStr"><is><t>Amiodaronu</t></is></c><c r="N70" s="2" t="inlineStr" /><c r="O70" s="2" t="inlineStr" /><c r="P70" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q70" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="71"><c r="A71" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B71" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C71" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D71" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E71" s="2" t="inlineStr"><is><t>Beta-adrenolityki można zastosować w:</t></is></c><c r="F71" s="2" t="inlineStr"><is><t>Tachykardii zatokowej</t></is></c><c r="G71" s="2" t="inlineStr"><is><t>Niewydolności mięśnia serca z upośledzoną frakcją wyrzutową</t></is></c><c r="H71" s="2" t="inlineStr"><is><t>W kontroli rytmu komór w migotaniu przedsionków</t></is></c><c r="I71" s="2" t="inlineStr" /><c r="J71" s="2" t="inlineStr" /><c r="K71" s="2" t="inlineStr"><is><t>Naczynioskurczowym wariancie choroby niedokrwiennej serca</t></is></c><c r="L71" s="2" t="inlineStr" /><c r="M71" s="2" t="inlineStr" /><c r="N71" s="2" t="inlineStr" /><c r="O71" s="2" t="inlineStr" /><c r="P71" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q71" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="72"><c r="A72" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B72" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C72" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D72" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E72" s="2" t="inlineStr"><is><t>Lidokaina:</t></is></c><c r="F72" s="2" t="inlineStr"><is><t>Jest skuteczna w znieczulaniu nasiękowym</t></is></c><c r="G72" s="2" t="inlineStr"><is><t>Jest metabolizowana w wątrobie</t></is></c><c r="H72" s="2" t="inlineStr"><is><t>Może powodować drgawki</t></is></c><c r="I72" s="2" t="inlineStr" /><c r="J72" s="2" t="inlineStr" /><c r="K72" s="2" t="inlineStr"><is><t>Silnie blokuje kanały potasowe</t></is></c><c r="L72" s="2" t="inlineStr" /><c r="M72" s="2" t="inlineStr" /><c r="N72" s="2" t="inlineStr" /><c r="O72" s="2" t="inlineStr" /><c r="P72" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q72" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="73"><c r="A73" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B73" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C73" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D73" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E73" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-działanie niepożądane:</t></is></c><c r="F73" s="2" t="inlineStr"><is><t>Ramipryl-obrzęk naczynioruchowy</t></is></c><c r="G73" s="2" t="inlineStr"><is><t>Metoprolol-zasłabnięcie lub omdlenie</t></is></c><c r="H73" s="2" t="inlineStr" /><c r="I73" s="2" t="inlineStr" /><c r="J73" s="2" t="inlineStr" /><c r="K73" s="2" t="inlineStr"><is><t>Losartan-zwiększenie stężenia kwasu moczowego</t></is></c><c r="L73" s="2" t="inlineStr"><is><t>Simwastatyna-poprawa tolerancji glukozy</t></is></c><c r="M73" s="2" t="inlineStr" /><c r="N73" s="2" t="inlineStr" /><c r="O73" s="2" t="inlineStr" /><c r="P73" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q73" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="74"><c r="A74" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B74" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C74" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D74" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E74" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – działanie niepożądane:</t></is></c><c r="F74" s="2" t="inlineStr"><is><t>metoprolol – blok przedsionkowo-komorowy I stopnia</t></is></c><c r="G74" s="2" t="inlineStr"><is><t>sotalol - wydłużenie odstępu QT</t></is></c><c r="H74" s="2" t="inlineStr"><is><t>propafenon - zaburzenia hematopoezy</t></is></c><c r="I74" s="2" t="inlineStr"><is><t>adenozyna - ból w klatce piersiowej</t></is></c><c r="J74" s="2" t="inlineStr" /><c r="K74" s="2" t="inlineStr" /><c r="L74" s="2" t="inlineStr" /><c r="M74" s="2" t="inlineStr" /><c r="N74" s="2" t="inlineStr" /><c r="O74" s="2" t="inlineStr" /><c r="P74" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q74" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="75"><c r="A75" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B75" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C75" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D75" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E75" s="2" t="inlineStr"><is><t>Która ordynacja jest błędna i wymaga korekty?</t></is></c><c r="F75" s="2" t="inlineStr"><is><t>Furosemid p.o. 1xd w obrzękach pochodzenia sercowego</t></is></c><c r="G75" s="2" t="inlineStr"><is><t>Hydrochlorotiazyd p.o. 1xd w obrzękach kończyn dolnych w przebiegu zespołu pozakrzepowego podudzi</t></is></c><c r="H75" s="2" t="inlineStr" /><c r="I75" s="2" t="inlineStr" /><c r="J75" s="2" t="inlineStr" /><c r="K75" s="2" t="inlineStr"><is><t>Torasemid p.o. 1xd w obrzękach pochodzenia nerkowego</t></is></c><c r="L75" s="2" t="inlineStr"><is><t>Spironolakton p.o. 1xd w wodobrzuszu w przebiegu niewydolności wątroby</t></is></c><c r="M75" s="2" t="inlineStr" /><c r="N75" s="2" t="inlineStr" /><c r="O75" s="2" t="inlineStr" /><c r="P75" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q75" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="76"><c r="A76" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B76" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C76" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D76" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E76" s="2" t="inlineStr"><is><t>Koangiokardianem, czyli lekiem działającym bezpośrednio na serce i naczynia jest:</t></is></c><c r="F76" s="2" t="inlineStr"><is><t>Lewosymendan</t></is></c><c r="G76" s="2" t="inlineStr" /><c r="H76" s="2" t="inlineStr" /><c r="I76" s="2" t="inlineStr" /><c r="J76" s="2" t="inlineStr" /><c r="K76" s="2" t="inlineStr"><is><t>Midodryna</t></is></c><c r="L76" s="2" t="inlineStr"><is><t>Epoprostenol</t></is></c><c r="M76" s="2" t="inlineStr"><is><t>Riocyguat</t></is></c><c r="N76" s="2" t="inlineStr" /><c r="O76" s="2" t="inlineStr" /><c r="P76" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q76" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="77"><c r="A77" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B77" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C77" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D77" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E77" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące bisfosfonianów:</t></is></c><c r="F77" s="2" t="inlineStr"><is><t>Są lekami pierwszego rzutu w profilaktyce i leczeniu osteoporozy pomenopauzalnej u kobiet</t></is></c><c r="G77" s="2" t="inlineStr"><is><t>Mogą być stosowane w zapobieganiu i leczeniu osteoporozy posteroidowej</t></is></c><c r="H77" s="2" t="inlineStr"><is><t>U osób z przerzutami nowotworowymi do układu kostnego łagodzą bóle kostne</t></is></c><c r="I77" s="2" t="inlineStr"><is><t>Przeciwwskazaniem do ich podawania jest ciężka niewydolność nerek (GFR&lt;30)</t></is></c><c r="J77" s="2" t="inlineStr" /><c r="K77" s="2" t="inlineStr" /><c r="L77" s="2" t="inlineStr" /><c r="M77" s="2" t="inlineStr" /><c r="N77" s="2" t="inlineStr" /><c r="O77" s="2" t="inlineStr" /><c r="P77" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q77" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="78"><c r="A78" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B78" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C78" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D78" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E78" s="2" t="inlineStr"><is><t>Zmniejszenie hipertriglicerydemii można osiągnąć stosując:</t></is></c><c r="F78" s="2" t="inlineStr"><is><t>Atorwastatynę</t></is></c><c r="G78" s="2" t="inlineStr"><is><t>Fenofibrat</t></is></c><c r="H78" s="2" t="inlineStr"><is><t>PUFA-wielonienasycone kwasy tłuszczowe</t></is></c><c r="I78" s="2" t="inlineStr" /><c r="J78" s="2" t="inlineStr" /><c r="K78" s="2" t="inlineStr"><is><t>Koleswelam</t></is></c><c r="L78" s="2" t="inlineStr" /><c r="M78" s="2" t="inlineStr" /><c r="N78" s="2" t="inlineStr" /><c r="O78" s="2" t="inlineStr" /><c r="P78" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q78" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="79"><c r="A79" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B79" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C79" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D79" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E79" s="2" t="inlineStr"><is><t>Lekiem wydłużającym dystans chromania przestankowego jest:</t></is></c><c r="F79" s="2" t="inlineStr"><is><t>Natydrofuryl</t></is></c><c r="G79" s="2" t="inlineStr"><is><t>Cilostazol</t></is></c><c r="H79" s="2" t="inlineStr" /><c r="I79" s="2" t="inlineStr" /><c r="J79" s="2" t="inlineStr" /><c r="K79" s="2" t="inlineStr"><is><t>Pentoksyfilina</t></is></c><c r="L79" s="2" t="inlineStr"><is><t>Diosmina mikronizowana</t></is></c><c r="M79" s="2" t="inlineStr" /><c r="N79" s="2" t="inlineStr" /><c r="O79" s="2" t="inlineStr" /><c r="P79" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q79" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="80"><c r="A80" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B80" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C80" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D80" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E80" s="2" t="inlineStr"><is><t>W prawidłowo przeprowadzonym leczeniu statynami należy:</t></is></c><c r="F80" s="2" t="inlineStr"><is><t>Oznaczyć aktywność ALAT i CK w surowicy przed rozpoczęciem leczenia</t></is></c><c r="G80" s="2" t="inlineStr"><is><t>Odstawić statynę jeśli aktywność ALAT przekroczy w surowicy 3-krotnie górną granicę wartości prawidłowych</t></is></c><c r="H80" s="2" t="inlineStr" /><c r="I80" s="2" t="inlineStr" /><c r="J80" s="2" t="inlineStr" /><c r="K80" s="2" t="inlineStr"><is><t>Ocenić skuteczność leczenia hipolipemizującego po 2 tygodniach od jego rozpoczęcia</t></is></c><c r="L80" s="2" t="inlineStr"><is><t>Mintorować aktywność CK u każdego pacjenta</t></is></c><c r="M80" s="2" t="inlineStr" /><c r="N80" s="2" t="inlineStr" /><c r="O80" s="2" t="inlineStr" /><c r="P80" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q80" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="81"><c r="A81" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B81" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C81" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D81" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E81" s="2" t="inlineStr"><is><t>Na kanały sodowe ma wpływ:</t></is></c><c r="F81" s="2" t="inlineStr"><is><t>Ranolazyna</t></is></c><c r="G81" s="2" t="inlineStr"><is><t>Iwabradyna</t></is></c><c r="H81" s="2" t="inlineStr" /><c r="I81" s="2" t="inlineStr" /><c r="J81" s="2" t="inlineStr" /><c r="K81" s="2" t="inlineStr"><is><t>Adenozyna</t></is></c><c r="L81" s="2" t="inlineStr"><is><t>Nitrendypina</t></is></c><c r="M81" s="2" t="inlineStr" /><c r="N81" s="2" t="inlineStr" /><c r="O81" s="2" t="inlineStr" /><c r="P81" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q81" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="82"><c r="A82" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B82" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C82" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D82" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E82" s="2" t="inlineStr"><is><t>Na kanały sodowe ma wpływ:</t></is></c><c r="F82" s="2" t="inlineStr"><is><t>propafenon</t></is></c><c r="G82" s="2" t="inlineStr"><is><t>ranolazyna</t></is></c><c r="H82" s="2" t="inlineStr"><is><t>bupiwakaina</t></is></c><c r="I82" s="2" t="inlineStr" /><c r="J82" s="2" t="inlineStr" /><c r="K82" s="2" t="inlineStr"><is><t>adenozyna</t></is></c><c r="L82" s="2" t="inlineStr" /><c r="M82" s="2" t="inlineStr" /><c r="N82" s="2" t="inlineStr" /><c r="O82" s="2" t="inlineStr" /><c r="P82" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q82" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="83"><c r="A83" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B83" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C83" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D83" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E83" s="2" t="inlineStr"><is><t>Interakcją farmakokinetyczną jest:</t></is></c><c r="F83" s="2" t="inlineStr"><is><t>Hamowanie wchłaniania z przewodu pokarmowego leków podawanych jednocześnie</t></is></c><c r="G83" s="2" t="inlineStr"><is><t>Zwiększanie metabolizmu leków podawanych jednocześnie</t></is></c><c r="H83" s="2" t="inlineStr" /><c r="I83" s="2" t="inlineStr" /><c r="J83" s="2" t="inlineStr" /><c r="K83" s="2" t="inlineStr"><is><t>Wytrącanie się osadu po zmieszaniu dwóch leków w jednym roztworze do wstrzyknięcia</t></is></c><c r="L83" s="2" t="inlineStr"><is><t>Nasilenie sedacji po skojarzeniu opioidów z etanolem</t></is></c><c r="M83" s="2" t="inlineStr" /><c r="N83" s="2" t="inlineStr" /><c r="O83" s="2" t="inlineStr" /><c r="P83" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q83" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="84"><c r="A84" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B84" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C84" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D84" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E84" s="2" t="inlineStr"><is><t>Właściwości farmakodynamiczne i parametry farmakokinetyczne leków mają wpływ na podejmowanie decyzji klinicznych. Czy słuszne jest wobec tego:</t></is></c><c r="F84" s="2" t="inlineStr"><is><t>Wielokrotne powtórzenie dawki naloksonu(t1/2=63min+/-12min) po przedawkowaniu metadonu</t></is></c><c r="G84" s="2" t="inlineStr" /><c r="H84" s="2" t="inlineStr" /><c r="I84" s="2" t="inlineStr" /><c r="J84" s="2" t="inlineStr" /><c r="K84" s="2" t="inlineStr"><is><t>Przetoczenie koncentratu płytek krwi 13h po podaniu tikagrelolu (tikagrelol ze swoim czynnym metabolitem mają łączny czas półtrwania eliminacji 12h)</t></is></c><c r="L84" s="2" t="inlineStr"><is><t>Odstawienie suplementacji potasu w hiperaldosteronizmie pierwotnym po 16-17h po włączeniu spironolaktonu (Cmax karnenonu=16,5h po podaniu spironolaktonu)</t></is></c><c r="M84" s="2" t="inlineStr"><is><t>Przeprowadzenie operacji neurochirurgicznej po 36h po odstawieniu klopidogrelu(t1/2=6h, jego aktywne mają pomijalnie krótki t1/2)</t></is></c><c r="N84" s="2" t="inlineStr" /><c r="O84" s="2" t="inlineStr" /><c r="P84" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q84" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="85"><c r="A85" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B85" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C85" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D85" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E85" s="2" t="inlineStr"><is><t>Kolistyna:</t></is></c><c r="F85" s="2" t="inlineStr"><is><t>Może być podawana wziewnie u osób z mukowiscydozą</t></is></c><c r="G85" s="2" t="inlineStr"><is><t>Może być stosowana w leczeniu ciężkich zakażeń uogólnionych wywołanych prze Klebsiella pneumoniae wytwarzającą karbapenemazy</t></is></c><c r="H85" s="2" t="inlineStr"><is><t>Wykazuje aktywność wobec Pseudomonas aeruginosa</t></is></c><c r="I85" s="2" t="inlineStr" /><c r="J85" s="2" t="inlineStr" /><c r="K85" s="2" t="inlineStr"><is><t>Jest skuteczna w neuroinfekcjach</t></is></c><c r="L85" s="2" t="inlineStr" /><c r="M85" s="2" t="inlineStr" /><c r="N85" s="2" t="inlineStr" /><c r="O85" s="2" t="inlineStr" /><c r="P85" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q85" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="86"><c r="A86" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B86" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C86" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D86" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E86" s="2" t="inlineStr"><is><t>Kolistyna</t></is></c><c r="F86" s="2" t="inlineStr"><is><t>Działa nefrotoksycznie</t></is></c><c r="G86" s="2" t="inlineStr" /><c r="H86" s="2" t="inlineStr" /><c r="I86" s="2" t="inlineStr" /><c r="J86" s="2" t="inlineStr" /><c r="K86" s="2" t="inlineStr"><is><t>Działa głównie na bakterie Gram+</t></is></c><c r="L86" s="2" t="inlineStr"><is><t>Dobrze wchłania się po podaniu PO</t></is></c><c r="M86" s="2" t="inlineStr"><is><t>Jest wydalana głównie z kałem</t></is></c><c r="N86" s="2" t="inlineStr" /><c r="O86" s="2" t="inlineStr" /><c r="P86" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q86" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="87"><c r="A87" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B87" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C87" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D87" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E87" s="2" t="inlineStr"><is><t>Doksycyklina</t></is></c><c r="F87" s="2" t="inlineStr"><is><t>Działa na bakterie atypowe</t></is></c><c r="G87" s="2" t="inlineStr" /><c r="H87" s="2" t="inlineStr" /><c r="I87" s="2" t="inlineStr" /><c r="J87" s="2" t="inlineStr" /><c r="K87" s="2" t="inlineStr"><is><t>Może być bezpiecznie stosowana u dzieci powyżej 2r.ż</t></is></c><c r="L87" s="2" t="inlineStr"><is><t>Jest anatgonistą receptorów GABA-A wywołujących efekt sedatywny</t></is></c><c r="M87" s="2" t="inlineStr"><is><t>Jest bezpieczna w terapii kobiet w ciąży</t></is></c><c r="N87" s="2" t="inlineStr" /><c r="O87" s="2" t="inlineStr" /><c r="P87" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q87" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="88"><c r="A88" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B88" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C88" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D88" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E88" s="2" t="inlineStr"><is><t>Doksycyklina:</t></is></c><c r="F88" s="2" t="inlineStr"><is><t>w niewielkim stopniu penetruje do ośrodkowego układu nerwowego</t></is></c><c r="G88" s="2" t="inlineStr"><is><t>tworzy chelaty z solami żelaza</t></is></c><c r="H88" s="2" t="inlineStr"><is><t>jest stosowana w leczeniu zakażeń układu moczowego o etiologii Chlamydia trachomatis</t></is></c><c r="I88" s="2" t="inlineStr"><is><t>nie wykazuje aktywności wobec Pseudomonas aeruginosa</t></is></c><c r="J88" s="2" t="inlineStr" /><c r="K88" s="2" t="inlineStr" /><c r="L88" s="2" t="inlineStr" /><c r="M88" s="2" t="inlineStr" /><c r="N88" s="2" t="inlineStr" /><c r="O88" s="2" t="inlineStr" /><c r="P88" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q88" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="89"><c r="A89" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B89" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C89" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D89" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E89" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-mechanizm działania:</t></is></c><c r="F89" s="2" t="inlineStr"><is><t>Fosfomycyna-blokowanie syntezy ściany komórkowej bakterii</t></is></c><c r="G89" s="2" t="inlineStr" /><c r="H89" s="2" t="inlineStr" /><c r="I89" s="2" t="inlineStr" /><c r="J89" s="2" t="inlineStr" /><c r="K89" s="2" t="inlineStr"><is><t>Cefepim-hamowanie topoizomerazy II</t></is></c><c r="L89" s="2" t="inlineStr"><is><t>Pefloksacyna-hamowanie biosyntezy białka w komórkach bakterii poprzez wiązanie się z podjednostką 50S rybosomu</t></is></c><c r="M89" s="2" t="inlineStr"><is><t>Trimetoprim-bezpośrednie uszkodzenie DNA</t></is></c><c r="N89" s="2" t="inlineStr" /><c r="O89" s="2" t="inlineStr" /><c r="P89" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q89" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="90"><c r="A90" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B90" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C90" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D90" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E90" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – mechanizm działania:</t></is></c><c r="F90" s="2" t="inlineStr"><is><t>linezolid- hamowanie biosyntezy białka w komórkach bakterii poprzez wiązanie się z podjednostką 50 S rybosomu</t></is></c><c r="G90" s="2" t="inlineStr" /><c r="H90" s="2" t="inlineStr" /><c r="I90" s="2" t="inlineStr" /><c r="J90" s="2" t="inlineStr" /><c r="K90" s="2" t="inlineStr"><is><t>cefuroksym – hamowanie topoizomerazy II</t></is></c><c r="L90" s="2" t="inlineStr"><is><t>moksyfloksacyna - blokowanie syntezy ściany komórkowej bakterii</t></is></c><c r="M90" s="2" t="inlineStr"><is><t>wankomycyna - uszkodzenie DNA</t></is></c><c r="N90" s="2" t="inlineStr" /><c r="O90" s="2" t="inlineStr" /><c r="P90" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q90" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="91"><c r="A91" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B91" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C91" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D91" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E91" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – mechanizm działania:</t></is></c><c r="F91" s="2" t="inlineStr"><is><t>tygecyklina - hamowanie biosyntezy białka w komórkach bakterii poprzez wiązanie się z podjednostką 30 S rybosomu</t></is></c><c r="G91" s="2" t="inlineStr"><is><t>trimetoprim - inhibicja reduktazy kwasu dihydrofoliowego (DHFR)</t></is></c><c r="H91" s="2" t="inlineStr" /><c r="I91" s="2" t="inlineStr" /><c r="J91" s="2" t="inlineStr" /><c r="K91" s="2" t="inlineStr"><is><t>metronidazol - blokowanie syntezy ściany komórkowej bakterii</t></is></c><c r="L91" s="2" t="inlineStr"><is><t>teikoplanina - uszkodzenie DNA</t></is></c><c r="M91" s="2" t="inlineStr" /><c r="N91" s="2" t="inlineStr" /><c r="O91" s="2" t="inlineStr" /><c r="P91" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q91" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="92"><c r="A92" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B92" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C92" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D92" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E92" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – mechanizm działania:</t></is></c><c r="F92" s="2" t="inlineStr"><is><t>linagliptyna – pośrednio aktywacja wydzielania insuliny przez pobudzenie receptora dla GLP-1 (peptydu glukagonopodobnego typu 1)</t></is></c><c r="G92" s="2" t="inlineStr"><is><t>empagliflozyna – indukcja stałej łagodnej hiperketonemii ze zwiększeniem stężenia kwasu beta-hydroksymasłowego w surowicy</t></is></c><c r="H92" s="2" t="inlineStr"><is><t>ezetymib – redukcja jelitowego wchłaniania cholesterolu i steroli roślinnych</t></is></c><c r="I92" s="2" t="inlineStr" /><c r="J92" s="2" t="inlineStr" /><c r="K92" s="2" t="inlineStr"><is><t>orlistat – aktywacja lipazy trzustkowej w świetle przewodu pokarmowego</t></is></c><c r="L92" s="2" t="inlineStr" /><c r="M92" s="2" t="inlineStr" /><c r="N92" s="2" t="inlineStr" /><c r="O92" s="2" t="inlineStr" /><c r="P92" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q92" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="93"><c r="A93" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B93" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C93" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D93" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E93" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-działania niepożądane:</t></is></c><c r="F93" s="2" t="inlineStr"><is><t>Amoksycylina-leukopenia w mechanizmie nadwrażliwości immunologicznej</t></is></c><c r="G93" s="2" t="inlineStr"><is><t>Tynidazol-neuropatia obwodowa</t></is></c><c r="H93" s="2" t="inlineStr"><is><t>Amikacyna-zaburzenia słuchu i równowagi</t></is></c><c r="I93" s="2" t="inlineStr" /><c r="J93" s="2" t="inlineStr" /><c r="K93" s="2" t="inlineStr"><is><t>Roksytromycyna-uszkodzenie nerek</t></is></c><c r="L93" s="2" t="inlineStr" /><c r="M93" s="2" t="inlineStr" /><c r="N93" s="2" t="inlineStr" /><c r="O93" s="2" t="inlineStr" /><c r="P93" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q93" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="94"><c r="A94" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B94" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C94" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D94" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E94" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – działania niepożądane:</t></is></c><c r="F94" s="2" t="inlineStr"><is><t>tygecyklina - nadwrażliwość na światło</t></is></c><c r="G94" s="2" t="inlineStr"><is><t>metronidazol - neuropatia obwodowa</t></is></c><c r="H94" s="2" t="inlineStr"><is><t>wankomycyna – uwalnianie histaminy</t></is></c><c r="I94" s="2" t="inlineStr" /><c r="J94" s="2" t="inlineStr" /><c r="K94" s="2" t="inlineStr"><is><t>azytromycyna – blokowanie wątrobowych enzymów mikrosomalnych (CYP)</t></is></c><c r="L94" s="2" t="inlineStr" /><c r="M94" s="2" t="inlineStr" /><c r="N94" s="2" t="inlineStr" /><c r="O94" s="2" t="inlineStr" /><c r="P94" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q94" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="95"><c r="A95" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B95" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C95" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D95" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E95" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – działania niepożądane:</t></is></c><c r="F95" s="2" t="inlineStr"><is><t>lewofloksacyna - drgawki</t></is></c><c r="G95" s="2" t="inlineStr"><is><t>ceftriakson – zagęszczenie żółci</t></is></c><c r="H95" s="2" t="inlineStr"><is><t>wankomycyna – zespół czerwonego karku</t></is></c><c r="I95" s="2" t="inlineStr"><is><t>linezolid – trombocytopenia</t></is></c><c r="J95" s="2" t="inlineStr" /><c r="K95" s="2" t="inlineStr" /><c r="L95" s="2" t="inlineStr" /><c r="M95" s="2" t="inlineStr" /><c r="N95" s="2" t="inlineStr" /><c r="O95" s="2" t="inlineStr" /><c r="P95" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q95" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="96"><c r="A96" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B96" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C96" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D96" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E96" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – działania niepożądane:</t></is></c><c r="F96" s="2" t="inlineStr"><is><t>bromek glikopironium - tachykardia</t></is></c><c r="G96" s="2" t="inlineStr"><is><t>budezonid – kandydoza jamy ustnej</t></is></c><c r="H96" s="2" t="inlineStr"><is><t>teofilina – zaburzenia rytmu serca</t></is></c><c r="I96" s="2" t="inlineStr"><is><t>omalizumab – reakcje w miejscu podskórnego podania leku, takie jak ból, zaczerwienienie, świąd, obrzęk</t></is></c><c r="J96" s="2" t="inlineStr" /><c r="K96" s="2" t="inlineStr" /><c r="L96" s="2" t="inlineStr" /><c r="M96" s="2" t="inlineStr" /><c r="N96" s="2" t="inlineStr" /><c r="O96" s="2" t="inlineStr" /><c r="P96" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q96" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="97"><c r="A97" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B97" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C97" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D97" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E97" s="2" t="inlineStr"><is><t>Właściwy wybór leku przeciwwirusowego w zakażeniu to:</t></is></c><c r="F97" s="2" t="inlineStr"><is><t>Wirus HBV-lamiwudyna</t></is></c><c r="G97" s="2" t="inlineStr"><is><t>Cytomegalowirus-walgancyklowir</t></is></c><c r="H97" s="2" t="inlineStr" /><c r="I97" s="2" t="inlineStr" /><c r="J97" s="2" t="inlineStr" /><c r="K97" s="2" t="inlineStr"><is><t>Norowirus-sakwinawir</t></is></c><c r="L97" s="2" t="inlineStr"><is><t>Wirus opryszczki-rybawiryna</t></is></c><c r="M97" s="2" t="inlineStr" /><c r="N97" s="2" t="inlineStr" /><c r="O97" s="2" t="inlineStr" /><c r="P97" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q97" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="98"><c r="A98" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B98" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C98" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D98" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E98" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-wrażliwy drobnoustrój:</t></is></c><c r="F98" s="2" t="inlineStr"><is><t>Lewofloksacyna-Streptococcus pneumoniae</t></is></c><c r="G98" s="2" t="inlineStr"><is><t>Aksetyl cefuroksymu-Hemophilus influenzae</t></is></c><c r="H98" s="2" t="inlineStr" /><c r="I98" s="2" t="inlineStr" /><c r="J98" s="2" t="inlineStr" /><c r="K98" s="2" t="inlineStr"><is><t>Fenoksymetylopenicylina-Staphylococcus aureus MSSA</t></is></c><c r="L98" s="2" t="inlineStr"><is><t>Fidaksomycyna-Bacteroides fragilis</t></is></c><c r="M98" s="2" t="inlineStr" /><c r="N98" s="2" t="inlineStr" /><c r="O98" s="2" t="inlineStr" /><c r="P98" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q98" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="99"><c r="A99" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B99" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C99" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D99" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E99" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – wrażliwy drobnoustrój:</t></is></c><c r="F99" s="2" t="inlineStr"><is><t>kaspofungina _ Candida spp</t></is></c><c r="G99" s="2" t="inlineStr"><is><t>amfoterycyna B – Cryptococcus neoformans</t></is></c><c r="H99" s="2" t="inlineStr"><is><t>worykonazol - Candida crusei</t></is></c><c r="I99" s="2" t="inlineStr" /><c r="J99" s="2" t="inlineStr" /><c r="K99" s="2" t="inlineStr"><is><t>flukonazol – Aspergillus fumigatus</t></is></c><c r="L99" s="2" t="inlineStr" /><c r="M99" s="2" t="inlineStr" /><c r="N99" s="2" t="inlineStr" /><c r="O99" s="2" t="inlineStr" /><c r="P99" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q99" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="100"><c r="A100" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B100" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C100" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D100" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E100" s="2" t="inlineStr"><is><t>Flukonazol:</t></is></c><c r="F100" s="2" t="inlineStr"><is><t>W leczeniu kandydozy jamy ustnej nie jest skuteczny po podaniu dawki jednorazowej</t></is></c><c r="G100" s="2" t="inlineStr" /><c r="H100" s="2" t="inlineStr" /><c r="I100" s="2" t="inlineStr" /><c r="J100" s="2" t="inlineStr" /><c r="K100" s="2" t="inlineStr"><is><t>Ma małą biodostępność po podaniu doustnym</t></is></c><c r="L100" s="2" t="inlineStr"><is><t>Powinien być podawany profilaktycznie pacjentom leczonym szerokospektralnymi lekami przeciwbakteryjnymi z powodu zakażenia układu oddechowego</t></is></c><c r="M100" s="2" t="inlineStr"><is><t>Istotnie hamuje syntezę hormonów steroidowych</t></is></c><c r="N100" s="2" t="inlineStr" /><c r="O100" s="2" t="inlineStr" /><c r="P100" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q100" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="101"><c r="A101" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B101" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C101" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D101" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E101" s="2" t="inlineStr"><is><t>Wyłącznie na ustroje gram dodatnie działa:</t></is></c><c r="F101" s="2" t="inlineStr"><is><t>Mupriocyna</t></is></c><c r="G101" s="2" t="inlineStr" /><c r="H101" s="2" t="inlineStr" /><c r="I101" s="2" t="inlineStr" /><c r="J101" s="2" t="inlineStr" /><c r="K101" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="L101" s="2" t="inlineStr"><is><t>Fosfomycyna</t></is></c><c r="M101" s="2" t="inlineStr"><is><t>Gentamycyna</t></is></c><c r="N101" s="2" t="inlineStr" /><c r="O101" s="2" t="inlineStr" /><c r="P101" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q101" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="102"><c r="A102" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B102" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C102" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D102" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E102" s="2" t="inlineStr"><is><t>W leczeniu rzęsistkowicy (Trichomonas Vaginalis) wykorzystuje się:</t></is></c><c r="F102" s="2" t="inlineStr"><is><t>Tynidazol</t></is></c><c r="G102" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="H102" s="2" t="inlineStr" /><c r="I102" s="2" t="inlineStr" /><c r="J102" s="2" t="inlineStr" /><c r="K102" s="2" t="inlineStr"><is><t>Sulfametoksazol+trymetoprym</t></is></c><c r="L102" s="2" t="inlineStr"><is><t>Spiramycynę</t></is></c><c r="M102" s="2" t="inlineStr" /><c r="N102" s="2" t="inlineStr" /><c r="O102" s="2" t="inlineStr" /><c r="P102" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q102" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="103"><c r="A103" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B103" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C103" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D103" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E103" s="2" t="inlineStr"><is><t>Do charakterystycznych działań niepożądanych inhibitorów proteazy HIV należy/należą:</t></is></c><c r="F103" s="2" t="inlineStr"><is><t>Liczne interakcje lekowe</t></is></c><c r="G103" s="2" t="inlineStr"><is><t>Cukrzyca</t></is></c><c r="H103" s="2" t="inlineStr"><is><t>Uszkodzenie wątroby</t></is></c><c r="I103" s="2" t="inlineStr"><is><t>Hipertriglicerydemia</t></is></c><c r="J103" s="2" t="inlineStr" /><c r="K103" s="2" t="inlineStr" /><c r="L103" s="2" t="inlineStr" /><c r="M103" s="2" t="inlineStr" /><c r="N103" s="2" t="inlineStr" /><c r="O103" s="2" t="inlineStr" /><c r="P103" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q103" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="104"><c r="A104" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B104" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C104" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D104" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E104" s="2" t="inlineStr"><is><t>W zakażeniu o etiologii Candida albicans można zastosować miejscowo:</t></is></c><c r="F104" s="2" t="inlineStr"><is><t>Natamycynę</t></is></c><c r="G104" s="2" t="inlineStr"><is><t>Mykonazol</t></is></c><c r="H104" s="2" t="inlineStr" /><c r="I104" s="2" t="inlineStr" /><c r="J104" s="2" t="inlineStr" /><c r="K104" s="2" t="inlineStr"><is><t>Mykafunginę</t></is></c><c r="L104" s="2" t="inlineStr"><is><t>Izawukonazol</t></is></c><c r="M104" s="2" t="inlineStr" /><c r="N104" s="2" t="inlineStr" /><c r="O104" s="2" t="inlineStr" /><c r="P104" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q104" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="105"><c r="A105" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B105" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C105" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D105" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E105" s="2" t="inlineStr"><is><t>Jeśli celem farmakodynamicznym dla stosowanego antybiotyku jest wysoka wartość T&gt;MIC to powinno się:</t></is></c><c r="F105" s="2" t="inlineStr"><is><t>Monitorować stężenie leku we krwi w celu modyfikacji dawkowania</t></is></c><c r="G105" s="2" t="inlineStr"><is><t>Podawać lek w przedłużonym wlewie dożylnym</t></is></c><c r="H105" s="2" t="inlineStr"><is><t>Zwiększać częstość podawania leku w ciągu doby</t></is></c><c r="I105" s="2" t="inlineStr" /><c r="J105" s="2" t="inlineStr" /><c r="K105" s="2" t="inlineStr"><is><t>Podać lek w pojedynczej skumulowanej dawce dobowej</t></is></c><c r="L105" s="2" t="inlineStr" /><c r="M105" s="2" t="inlineStr" /><c r="N105" s="2" t="inlineStr" /><c r="O105" s="2" t="inlineStr" /><c r="P105" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q105" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="106"><c r="A106" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B106" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C106" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D106" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E106" s="2" t="inlineStr"><is><t>Do przestarzałych środków odkażających, które z powodu braku skuteczności lub istotnych działań niepożądanych nie powinny być obecnie stosowane należy:</t></is></c><c r="F106" s="2" t="inlineStr"><is><t>Nadmanganian potasu</t></is></c><c r="G106" s="2" t="inlineStr"><is><t>Tetraboran sodowy</t></is></c><c r="H106" s="2" t="inlineStr" /><c r="I106" s="2" t="inlineStr" /><c r="J106" s="2" t="inlineStr" /><c r="K106" s="2" t="inlineStr"><is><t>Oktenidyna</t></is></c><c r="L106" s="2" t="inlineStr"><is><t>Jodopowidon</t></is></c><c r="M106" s="2" t="inlineStr" /><c r="N106" s="2" t="inlineStr" /><c r="O106" s="2" t="inlineStr" /><c r="P106" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q106" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="107"><c r="A107" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B107" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C107" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D107" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E107" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenia dotyczące profilaktyki i leczenia malarii:</t></is></c><c r="F107" s="2" t="inlineStr"><is><t>Lumefantryna w połączeniu z artemeterem może być skuteczna w zakażeniu Plasmodium falciparum</t></is></c><c r="G107" s="2" t="inlineStr"><is><t>W przypadkach wymagających profilaktyki długoterminowej można zastosować chlorochinę</t></is></c><c r="H107" s="2" t="inlineStr" /><c r="I107" s="2" t="inlineStr" /><c r="J107" s="2" t="inlineStr" /><c r="K107" s="2" t="inlineStr"><is><t>Pochodne artemizyniny zalecane są tylko do profilaktyki malarii</t></is></c><c r="L107" s="2" t="inlineStr"><is><t>Atowakwon z proguanilem może być stosowany u osób z upośledzoną czynnością nerek (GFR&lt;30)</t></is></c><c r="M107" s="2" t="inlineStr" /><c r="N107" s="2" t="inlineStr" /><c r="O107" s="2" t="inlineStr" /><c r="P107" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q107" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="108"><c r="A108" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B108" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C108" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D108" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E108" s="2" t="inlineStr"><is><t>Do przyczyn jatrogennej nefropatii można zaliczyć stosowanie:</t></is></c><c r="F108" s="2" t="inlineStr"><is><t>Jodowych środków kontrastowych podczas koronarografii</t></is></c><c r="G108" s="2" t="inlineStr"><is><t>Ibuprofenu przewlekle w reumatoidalnym zapaleniu stawów</t></is></c><c r="H108" s="2" t="inlineStr"><is><t>Ramiprylu w niewydolności serca</t></is></c><c r="I108" s="2" t="inlineStr" /><c r="J108" s="2" t="inlineStr" /><c r="K108" s="2" t="inlineStr"><is><t>Loratadyny przewlekle w alergicznym zapaleniu błony śluzowej nosa</t></is></c><c r="L108" s="2" t="inlineStr" /><c r="M108" s="2" t="inlineStr" /><c r="N108" s="2" t="inlineStr" /><c r="O108" s="2" t="inlineStr" /><c r="P108" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q108" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="109"><c r="A109" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B109" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C109" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D109" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E109" s="2" t="inlineStr"><is><t>Wskaż prawdziwe zdania dotyczące leczenia morfiną:</t></is></c><c r="F109" s="2" t="inlineStr"><is><t>Metabolity morfiny wydalane są przez nerki</t></is></c><c r="G109" s="2" t="inlineStr"><is><t>Przy przewlekłym stosowaniu morfiny powstaje morfino-6-glukuronian – metabolit, którego siła działania analgetycznego przewyższa siłę działania związku macierzystego</t></is></c><c r="H109" s="2" t="inlineStr"><is><t>Morfina może być podawana zewnątrzoponowo</t></is></c><c r="I109" s="2" t="inlineStr" /><c r="J109" s="2" t="inlineStr" /><c r="K109" s="2" t="inlineStr"><is><t>Morfina ma dużą biodostępność po podaniu doustnym</t></is></c><c r="L109" s="2" t="inlineStr" /><c r="M109" s="2" t="inlineStr" /><c r="N109" s="2" t="inlineStr" /><c r="O109" s="2" t="inlineStr" /><c r="P109" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q109" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="110"><c r="A110" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B110" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C110" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D110" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E110" s="2" t="inlineStr"><is><t>Wskazanie do insulinoterapii jest:</t></is></c><c r="F110" s="2" t="inlineStr"><is><t>Cukrzyca typu LADA</t></is></c><c r="G110" s="2" t="inlineStr"><is><t>Ostry zespół wieńcowy u osoby z cukrzycą typu II</t></is></c><c r="H110" s="2" t="inlineStr"><is><t>Znaczna hiperglikemia (&gt;300) w przebiegu cukrzycy typu II</t></is></c><c r="I110" s="2" t="inlineStr"><is><t>Cukrzyca ciężarnych</t></is></c><c r="J110" s="2" t="inlineStr" /><c r="K110" s="2" t="inlineStr" /><c r="L110" s="2" t="inlineStr" /><c r="M110" s="2" t="inlineStr" /><c r="N110" s="2" t="inlineStr" /><c r="O110" s="2" t="inlineStr" /><c r="P110" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q110" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="111"><c r="A111" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B111" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C111" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D111" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E111" s="2" t="inlineStr"><is><t>Długodziałające analogii insuliny w porównaniu do insuliny protaminowo-cynkowej (NPH) charakteryzują się:</t></is></c><c r="F111" s="2" t="inlineStr"><is><t>Mniejszym ryzykiem hipoglikemii</t></is></c><c r="G111" s="2" t="inlineStr" /><c r="H111" s="2" t="inlineStr" /><c r="I111" s="2" t="inlineStr" /><c r="J111" s="2" t="inlineStr" /><c r="K111" s="2" t="inlineStr"><is><t>Mniejszym ryzykiem onkologicznym</t></is></c><c r="L111" s="2" t="inlineStr"><is><t>Większym ryzykiem zjawiska brzasku</t></is></c><c r="M111" s="2" t="inlineStr"><is><t>Działaniem anorektycznym</t></is></c><c r="N111" s="2" t="inlineStr" /><c r="O111" s="2" t="inlineStr" /><c r="P111" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q111" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="112"><c r="A112" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B112" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C112" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D112" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E112" s="2" t="inlineStr"><is><t>Zmniejszenie obwodowej konwersji tyroksyny do trójjodotyroniny jest efektem stosowania:</t></is></c><c r="F112" s="2" t="inlineStr"><is><t>Hydrokortyzonu</t></is></c><c r="G112" s="2" t="inlineStr"><is><t>Propylotiouracylu</t></is></c><c r="H112" s="2" t="inlineStr"><is><t>Propanololu</t></is></c><c r="I112" s="2" t="inlineStr" /><c r="J112" s="2" t="inlineStr" /><c r="K112" s="2" t="inlineStr"><is><t>Płynu Lugola</t></is></c><c r="L112" s="2" t="inlineStr" /><c r="M112" s="2" t="inlineStr" /><c r="N112" s="2" t="inlineStr" /><c r="O112" s="2" t="inlineStr" /><c r="P112" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q112" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="113"><c r="A113" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B113" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C113" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D113" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E113" s="2" t="inlineStr"><is><t>Wskazaniem do stosowania hormonalnej terapii zastępczej u kobiet po menopauzie jest:</t></is></c><c r="F113" s="2" t="inlineStr"><is><t>Obecność objawów wypadowych</t></is></c><c r="G113" s="2" t="inlineStr" /><c r="H113" s="2" t="inlineStr" /><c r="I113" s="2" t="inlineStr" /><c r="J113" s="2" t="inlineStr" /><c r="K113" s="2" t="inlineStr"><is><t>Wtórna profilaktyka chorób układu krążenia</t></is></c><c r="L113" s="2" t="inlineStr"><is><t>Profilaktyka osteoporozy</t></is></c><c r="M113" s="2" t="inlineStr"><is><t>Zapobieganie chorobie Alzheimera</t></is></c><c r="N113" s="2" t="inlineStr" /><c r="O113" s="2" t="inlineStr" /><c r="P113" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q113" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="114"><c r="A114" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B114" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C114" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D114" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E114" s="2" t="inlineStr"><is><t>Przeciwbólowy efekt pułapowy wykazuje:</t></is></c><c r="F114" s="2" t="inlineStr"><is><t>Naproksen</t></is></c><c r="G114" s="2" t="inlineStr"><is><t>Buprenorfina</t></is></c><c r="H114" s="2" t="inlineStr"><is><t>Ibuprofen</t></is></c><c r="I114" s="2" t="inlineStr" /><c r="J114" s="2" t="inlineStr" /><c r="K114" s="2" t="inlineStr"><is><t>Oksykodon</t></is></c><c r="L114" s="2" t="inlineStr" /><c r="M114" s="2" t="inlineStr" /><c r="N114" s="2" t="inlineStr" /><c r="O114" s="2" t="inlineStr" /><c r="P114" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q114" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="115"><c r="A115" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B115" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C115" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D115" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E115" s="2" t="inlineStr"><is><t>Teofilina:</t></is></c><c r="F115" s="2" t="inlineStr"><is><t>Jest anatgonistą receptora adenozynowego</t></is></c><c r="G115" s="2" t="inlineStr"><is><t>Hamuje aktywność fosfodiesteraz</t></is></c><c r="H115" s="2" t="inlineStr"><is><t>Zwiększa przepływ nerkowy</t></is></c><c r="I115" s="2" t="inlineStr"><is><t>Pobudza ośrodek oddechowy w rdzeniu przedłużonym</t></is></c><c r="J115" s="2" t="inlineStr" /><c r="K115" s="2" t="inlineStr" /><c r="L115" s="2" t="inlineStr" /><c r="M115" s="2" t="inlineStr" /><c r="N115" s="2" t="inlineStr" /><c r="O115" s="2" t="inlineStr" /><c r="P115" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q115" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="116"><c r="A116" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B116" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C116" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D116" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E116" s="2" t="inlineStr"><is><t>Idealny glikokortykosteroid wziewny:</t></is></c><c r="F116" s="2" t="inlineStr"><is><t>Połknięty charakteryzuje się niewielką biodostępnością</t></is></c><c r="G116" s="2" t="inlineStr" /><c r="H116" s="2" t="inlineStr" /><c r="I116" s="2" t="inlineStr" /><c r="J116" s="2" t="inlineStr" /><c r="K116" s="2" t="inlineStr"><is><t>Dobrze wchłania się z pęcherzyków płucnych</t></is></c><c r="L116" s="2" t="inlineStr"><is><t>Nie podlega efektowi pierwszego przejścia przez wątrobę</t></is></c><c r="M116" s="2" t="inlineStr"><is><t>Ma krótki okres półtrwania kompleksu glikokortkosteroidu z receptorem t1/2=2-3h</t></is></c><c r="N116" s="2" t="inlineStr" /><c r="O116" s="2" t="inlineStr" /><c r="P116" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q116" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="117"><c r="A117" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B117" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C117" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D117" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E117" s="2" t="inlineStr"><is><t>Działanie keratolityczne wykazuje:</t></is></c><c r="F117" s="2" t="inlineStr"><is><t>Mocznik</t></is></c><c r="G117" s="2" t="inlineStr"><is><t>Kwas salicylowy</t></is></c><c r="H117" s="2" t="inlineStr"><is><t>Nadtlenek benzoilu</t></is></c><c r="I117" s="2" t="inlineStr" /><c r="J117" s="2" t="inlineStr" /><c r="K117" s="2" t="inlineStr"><is><t>Metoksalen</t></is></c><c r="L117" s="2" t="inlineStr" /><c r="M117" s="2" t="inlineStr" /><c r="N117" s="2" t="inlineStr" /><c r="O117" s="2" t="inlineStr" /><c r="P117" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q117" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="118"><c r="A118" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B118" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C118" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D118" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E118" s="2" t="inlineStr"><is><t>W zatruciu solami litu:</t></is></c><c r="F118" s="2" t="inlineStr"><is><t>Należy natychmiast zakończyć podawanie litu</t></is></c><c r="G118" s="2" t="inlineStr"><is><t>W leczeniu ostrego zatrucia istotne znaczenie ma intensywne wyrównanie zaburzeń gospodarki wodno-elektrolitowej, zwłaszcza uzupełnianie niedoboru sodu poprzez przetaczanie roztworu 0,9% NaCl dożylnie</t></is></c><c r="H118" s="2" t="inlineStr"><is><t>Podstawową metodą eliminacji leku jest hemodializa</t></is></c><c r="I118" s="2" t="inlineStr" /><c r="J118" s="2" t="inlineStr" /><c r="K118" s="2" t="inlineStr"><is><t>Korzystne działanie ma stosowanie węgla aktywowanego</t></is></c><c r="L118" s="2" t="inlineStr" /><c r="M118" s="2" t="inlineStr" /><c r="N118" s="2" t="inlineStr" /><c r="O118" s="2" t="inlineStr" /><c r="P118" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q118" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="119"><c r="A119" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B119" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C119" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D119" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E119" s="2" t="inlineStr"><is><t>Fluorochinolony:</t></is></c><c r="F119" s="2" t="inlineStr"><is><t>mogą spowodować zapalenie ścięgien</t></is></c><c r="G119" s="2" t="inlineStr"><is><t>mogą być przyczyną zaburzeń rytmu serca</t></is></c><c r="H119" s="2" t="inlineStr" /><c r="I119" s="2" t="inlineStr" /><c r="J119" s="2" t="inlineStr" /><c r="K119" s="2" t="inlineStr"><is><t>wszystkie generacje mają zbliżoną skuteczność przeciwko Gram ujemnym pałeczkom niefermentującym</t></is></c><c r="L119" s="2" t="inlineStr"><is><t>są agonistami receptorów GABA-A wywołując efekt sedatywny</t></is></c><c r="M119" s="2" t="inlineStr" /><c r="N119" s="2" t="inlineStr" /><c r="O119" s="2" t="inlineStr" /><c r="P119" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q119" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="120"><c r="A120" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B120" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C120" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D120" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E120" s="2" t="inlineStr"><is><t>Fluorochinolony:</t></is></c><c r="F120" s="2" t="inlineStr"><is><t>mogą powodować zapalenie więzadeł</t></is></c><c r="G120" s="2" t="inlineStr" /><c r="H120" s="2" t="inlineStr" /><c r="I120" s="2" t="inlineStr" /><c r="J120" s="2" t="inlineStr" /><c r="K120" s="2" t="inlineStr"><is><t>słabo wchłaniają się z przewodu pokarmowego</t></is></c><c r="L120" s="2" t="inlineStr"><is><t>są grupą, na którą rzadko stwierdza się oporność bakteryjną</t></is></c><c r="M120" s="2" t="inlineStr"><is><t>niezależnie od generacji wykazują aktywność wyłącznie wobec bakterii tlenowych</t></is></c><c r="N120" s="2" t="inlineStr" /><c r="O120" s="2" t="inlineStr" /><c r="P120" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q120" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="121"><c r="A121" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B121" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C121" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D121" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E121" s="2" t="inlineStr"><is><t>Błędny schemat terapeutyczny to zastosowanie:</t></is></c><c r="F121" s="2" t="inlineStr"><is><t>loperamidu w zapalnej biegunce poantybiotykowej przez 10 dni</t></is></c><c r="G121" s="2" t="inlineStr" /><c r="H121" s="2" t="inlineStr" /><c r="I121" s="2" t="inlineStr" /><c r="J121" s="2" t="inlineStr" /><c r="K121" s="2" t="inlineStr"><is><t>azytromycyny w krztuścu przez 5 dni</t></is></c><c r="L121" s="2" t="inlineStr"><is><t>kotrymoksazolu w niepowikłanym zakażeniu układu moczowego przez 3 dni</t></is></c><c r="M121" s="2" t="inlineStr"><is><t>fenoksymetylpenicyliny w anginie paciorkowcowej przez 10 dni</t></is></c><c r="N121" s="2" t="inlineStr" /><c r="O121" s="2" t="inlineStr" /><c r="P121" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q121" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="122"><c r="A122" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B122" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C122" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D122" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E122" s="2" t="inlineStr"><is><t>W leczeniu 60-letniego pacjenta z pozaszpitalnym zapaleniem płuc (skala CURB-0pkt) uwzględniającym typową etiologię zakażenia u dorosłych należy:</t></is></c><c r="F122" s="2" t="inlineStr"><is><t>stosować stałe optymalne przedziały dawkowania w ciągu całej doby</t></is></c><c r="G122" s="2" t="inlineStr"><is><t>w razie nadwrażliwości na leczenie początkowe w wywiadach zastosować lewofloksacynę lub moksyfloksacynę</t></is></c><c r="H122" s="2" t="inlineStr" /><c r="I122" s="2" t="inlineStr" /><c r="J122" s="2" t="inlineStr" /><c r="K122" s="2" t="inlineStr"><is><t>leczyć 2 lekami przeciwbakteryjnymi o różnych mechanizmach działania</t></is></c><c r="L122" s="2" t="inlineStr"><is><t>prowadzić terapię co najmniej 21 dni</t></is></c><c r="M122" s="2" t="inlineStr" /><c r="N122" s="2" t="inlineStr" /><c r="O122" s="2" t="inlineStr" /><c r="P122" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q122" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="123"><c r="A123" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B123" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C123" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D123" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E123" s="2" t="inlineStr"><is><t>W leczeniu zapalenia opon mózgowo-rdzeniowych uzasadnione jest zastosowanie:</t></is></c><c r="F123" s="2" t="inlineStr"><is><t>ceftriaksonu</t></is></c><c r="G123" s="2" t="inlineStr"><is><t>acyklowiru</t></is></c><c r="H123" s="2" t="inlineStr"><is><t>meropenemu</t></is></c><c r="I123" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="J123" s="2" t="inlineStr" /><c r="K123" s="2" t="inlineStr" /><c r="L123" s="2" t="inlineStr" /><c r="M123" s="2" t="inlineStr" /><c r="N123" s="2" t="inlineStr" /><c r="O123" s="2" t="inlineStr" /><c r="P123" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q123" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="124"><c r="A124" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B124" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C124" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D124" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E124" s="2" t="inlineStr"><is><t>Wyłącznie na drobnoustroje Gram ujemne działa:</t></is></c><c r="F124" s="2" t="inlineStr"><is><t>aztreonam</t></is></c><c r="G124" s="2" t="inlineStr" /><c r="H124" s="2" t="inlineStr" /><c r="I124" s="2" t="inlineStr" /><c r="J124" s="2" t="inlineStr" /><c r="K124" s="2" t="inlineStr"><is><t>mupirocyna</t></is></c><c r="L124" s="2" t="inlineStr"><is><t>kwas fusydowy</t></is></c><c r="M124" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="N124" s="2" t="inlineStr" /><c r="O124" s="2" t="inlineStr" /><c r="P124" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q124" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="125"><c r="A125" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B125" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C125" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D125" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E125" s="2" t="inlineStr"><is><t>W leczeniu toksoplazmozy wykorzystuje się:</t></is></c><c r="F125" s="2" t="inlineStr"><is><t>pirymetaminę z sulfadiazyną</t></is></c><c r="G125" s="2" t="inlineStr"><is><t>spiramycynę</t></is></c><c r="H125" s="2" t="inlineStr" /><c r="I125" s="2" t="inlineStr" /><c r="J125" s="2" t="inlineStr" /><c r="K125" s="2" t="inlineStr"><is><t>dalfoprystynę/chinuprystynę</t></is></c><c r="L125" s="2" t="inlineStr"><is><t>oksytetracyklinę</t></is></c><c r="M125" s="2" t="inlineStr" /><c r="N125" s="2" t="inlineStr" /><c r="O125" s="2" t="inlineStr" /><c r="P125" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q125" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="126"><c r="A126" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B126" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C126" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D126" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E126" s="2" t="inlineStr"><is><t>Do odległych działań niepożądanych terapii HAART (Highly Active Antiretroviral Therapy) należy:</t></is></c><c r="F126" s="2" t="inlineStr"><is><t>uszkodzenie wątroby</t></is></c><c r="G126" s="2" t="inlineStr"><is><t>lipodystrofia</t></is></c><c r="H126" s="2" t="inlineStr"><is><t>kwasica mleczanowa</t></is></c><c r="I126" s="2" t="inlineStr"><is><t>insulinooporność</t></is></c><c r="J126" s="2" t="inlineStr" /><c r="K126" s="2" t="inlineStr" /><c r="L126" s="2" t="inlineStr" /><c r="M126" s="2" t="inlineStr" /><c r="N126" s="2" t="inlineStr" /><c r="O126" s="2" t="inlineStr" /><c r="P126" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q126" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="127"><c r="A127" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B127" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C127" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D127" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E127" s="2" t="inlineStr"><is><t>W grzybiczym zakażeniu paznokci można zastosować</t></is></c><c r="F127" s="2" t="inlineStr"><is><t>amorolfinę</t></is></c><c r="G127" s="2" t="inlineStr" /><c r="H127" s="2" t="inlineStr" /><c r="I127" s="2" t="inlineStr" /><c r="J127" s="2" t="inlineStr" /><c r="K127" s="2" t="inlineStr"><is><t>natamycynę</t></is></c><c r="L127" s="2" t="inlineStr"><is><t>klotrymazol</t></is></c><c r="M127" s="2" t="inlineStr"><is><t>kaspofunginę</t></is></c><c r="N127" s="2" t="inlineStr" /><c r="O127" s="2" t="inlineStr" /><c r="P127" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q127" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="128"><c r="A128" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B128" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C128" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D128" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E128" s="2" t="inlineStr"><is><t>Efekt bakteriobójczy zależny od skumulowanej ekspozycji (AUC24/MIC) wykazuje:</t></is></c><c r="F128" s="2" t="inlineStr"><is><t>lewofloksacyna</t></is></c><c r="G128" s="2" t="inlineStr"><is><t>azytromycyna</t></is></c><c r="H128" s="2" t="inlineStr" /><c r="I128" s="2" t="inlineStr" /><c r="J128" s="2" t="inlineStr" /><c r="K128" s="2" t="inlineStr"><is><t>amoksycylina z kwasem klawulanowym</t></is></c><c r="L128" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="M128" s="2" t="inlineStr" /><c r="N128" s="2" t="inlineStr" /><c r="O128" s="2" t="inlineStr" /><c r="P128" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q128" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="129"><c r="A129" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B129" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C129" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D129" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E129" s="2" t="inlineStr"><is><t>Do odkażania rany w obrębie skóry można zastosować:</t></is></c><c r="F129" s="2" t="inlineStr"><is><t>oktenidynę</t></is></c><c r="G129" s="2" t="inlineStr"><is><t>jodopowidon</t></is></c><c r="H129" s="2" t="inlineStr" /><c r="I129" s="2" t="inlineStr" /><c r="J129" s="2" t="inlineStr" /><c r="K129" s="2" t="inlineStr"><is><t>wodę do wstrzyknięć</t></is></c><c r="L129" s="2" t="inlineStr"><is><t>kwas borowy</t></is></c><c r="M129" s="2" t="inlineStr" /><c r="N129" s="2" t="inlineStr" /><c r="O129" s="2" t="inlineStr" /><c r="P129" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q129" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="130"><c r="A130" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B130" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C130" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D130" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E130" s="2" t="inlineStr"><is><t>Koszt dodatkowego roku życia skorygowanego o jakość (ang. QALY – quality adjusted life year):</t></is></c><c r="F130" s="2" t="inlineStr"><is><t>stanowi formalne kryterium refundacyjne zgodnie z obowiązującymi regulacjami prawnymi</t></is></c><c r="G130" s="2" t="inlineStr"><is><t>jest wynikiem analizy kosztów użyteczności</t></is></c><c r="H130" s="2" t="inlineStr"><is><t>jego wartość progowa, czyli maksymalna dla procedur uznanych za kosztowo efektywne, stanowi 3-krotność produktu krajowego brutto per capita zgodnie z obowiązującymi regulacjami prawnymi</t></is></c><c r="I130" s="2" t="inlineStr" /><c r="J130" s="2" t="inlineStr" /><c r="K130" s="2" t="inlineStr"><is><t>możliwy jest do oszacowania tylko w przypadku procedur zmniejszających umieralność całkowitą</t></is></c><c r="L130" s="2" t="inlineStr" /><c r="M130" s="2" t="inlineStr" /><c r="N130" s="2" t="inlineStr" /><c r="O130" s="2" t="inlineStr" /><c r="P130" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q130" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="131"><c r="A131" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B131" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C131" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D131" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E131" s="2" t="inlineStr"><is><t>U pacjenta z niewydolnością nerek należy dokonać modyfikacji dawek:</t></is></c><c r="F131" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="G131" s="2" t="inlineStr"><is><t>cyprofloksacyny</t></is></c><c r="H131" s="2" t="inlineStr"><is><t>gentamycyny</t></is></c><c r="I131" s="2" t="inlineStr" /><c r="J131" s="2" t="inlineStr" /><c r="K131" s="2" t="inlineStr"><is><t>erytromycyny</t></is></c><c r="L131" s="2" t="inlineStr" /><c r="M131" s="2" t="inlineStr" /><c r="N131" s="2" t="inlineStr" /><c r="O131" s="2" t="inlineStr" /><c r="P131" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q131" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="132"><c r="A132" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B132" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C132" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D132" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E132" s="2" t="inlineStr"><is><t>Rotacja opioidów jest uzasadniona w przypadku:</t></is></c><c r="F132" s="2" t="inlineStr"><is><t>nudności</t></is></c><c r="G132" s="2" t="inlineStr"><is><t>zaburzeń świadomości</t></is></c><c r="H132" s="2" t="inlineStr"><is><t>długotrwałej (bezterminowej) terapii w celu ułatwienia jej prowadzenia</t></is></c><c r="I132" s="2" t="inlineStr" /><c r="J132" s="2" t="inlineStr" /><c r="K132" s="2" t="inlineStr"><is><t>zaparć</t></is></c><c r="L132" s="2" t="inlineStr" /><c r="M132" s="2" t="inlineStr" /><c r="N132" s="2" t="inlineStr" /><c r="O132" s="2" t="inlineStr" /><c r="P132" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q132" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="133"><c r="A133" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B133" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C133" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D133" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E133" s="2" t="inlineStr"><is><t>Dapagliflozyna:</t></is></c><c r="F133" s="2" t="inlineStr"><is><t>zwiększa ryzyko zakażeń układu moczowo-płciowego</t></is></c><c r="G133" s="2" t="inlineStr"><is><t>może spowodować kwasicę ketonową</t></is></c><c r="H133" s="2" t="inlineStr" /><c r="I133" s="2" t="inlineStr" /><c r="J133" s="2" t="inlineStr" /><c r="K133" s="2" t="inlineStr"><is><t>zmniejsza glukozurię</t></is></c><c r="L133" s="2" t="inlineStr"><is><t>nie może być stosowana łącznie z insuliną</t></is></c><c r="M133" s="2" t="inlineStr" /><c r="N133" s="2" t="inlineStr" /><c r="O133" s="2" t="inlineStr" /><c r="P133" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q133" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="134"><c r="A134" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B134" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C134" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D134" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E134" s="2" t="inlineStr"><is><t>Wskaż zdanie prawdziwe:</t></is></c><c r="F134" s="2" t="inlineStr"><is><t>zwiększenie stężenia glukozy w godzinach porannych poprzedzone hipoglikemią nocną może być wskazaniem do zmniejszenia dawki insuliny bazowej</t></is></c><c r="G134" s="2" t="inlineStr"><is><t>efekt brzasku może zmniejszyć zastosowanie długodziałających bezszczytowych analogów insuliny</t></is></c><c r="H134" s="2" t="inlineStr"><is><t>kardioprotekcyjne działanie empagliflozyny może mieć związek z usprawnieniem procesów energetycznych w komórkach mięśnia sercowego</t></is></c><c r="I134" s="2" t="inlineStr" /><c r="J134" s="2" t="inlineStr" /><c r="K134" s="2" t="inlineStr"><is><t>insulina izofanowa (NPH) jest przeznaczona do stosowana przed głównymi posiłkami</t></is></c><c r="L134" s="2" t="inlineStr" /><c r="M134" s="2" t="inlineStr" /><c r="N134" s="2" t="inlineStr" /><c r="O134" s="2" t="inlineStr" /><c r="P134" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q134" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="135"><c r="A135" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B135" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C135" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D135" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E135" s="2" t="inlineStr"><is><t>W leczeniu nadczynności tarczycy można zastosować:</t></is></c><c r="F135" s="2" t="inlineStr"><is><t>jod promieniotwórczy 131 I</t></is></c><c r="G135" s="2" t="inlineStr"><is><t>płyn Lugola</t></is></c><c r="H135" s="2" t="inlineStr"><is><t>tiamazol</t></is></c><c r="I135" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="J135" s="2" t="inlineStr" /><c r="K135" s="2" t="inlineStr" /><c r="L135" s="2" t="inlineStr" /><c r="M135" s="2" t="inlineStr" /><c r="N135" s="2" t="inlineStr" /><c r="O135" s="2" t="inlineStr" /><c r="P135" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q135" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="136"><c r="A136" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B136" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C136" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D136" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E136" s="2" t="inlineStr"><is><t>Do progestagenów należy:</t></is></c><c r="F136" s="2" t="inlineStr"><is><t>megestrol</t></is></c><c r="G136" s="2" t="inlineStr"><is><t>noretysteron</t></is></c><c r="H136" s="2" t="inlineStr" /><c r="I136" s="2" t="inlineStr" /><c r="J136" s="2" t="inlineStr" /><c r="K136" s="2" t="inlineStr"><is><t>dutasteryd</t></is></c><c r="L136" s="2" t="inlineStr"><is><t>anastrozol</t></is></c><c r="M136" s="2" t="inlineStr" /><c r="N136" s="2" t="inlineStr" /><c r="O136" s="2" t="inlineStr" /><c r="P136" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q136" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="137"><c r="A137" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B137" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C137" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D137" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E137" s="2" t="inlineStr"><is><t>Do leków antyagregacyjnych stosowanych w profilaktyce wtórnej udaru niedokrwiennego mózgu na podłożu miażdżycy naczyń do- i mózgowych należą:</t></is></c><c r="F137" s="2" t="inlineStr"><is><t>klopidogrel</t></is></c><c r="G137" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="H137" s="2" t="inlineStr" /><c r="I137" s="2" t="inlineStr" /><c r="J137" s="2" t="inlineStr" /><c r="K137" s="2" t="inlineStr"><is><t>tikagrelor</t></is></c><c r="L137" s="2" t="inlineStr"><is><t>prasugrel</t></is></c><c r="M137" s="2" t="inlineStr" /><c r="N137" s="2" t="inlineStr" /><c r="O137" s="2" t="inlineStr" /><c r="P137" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q137" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="138"><c r="A138" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B138" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C138" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D138" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E138" s="2" t="inlineStr"><is><t>W ciężkiej hiperkalcemii (&gt;15mg/dl) można zastosować dożylnie:</t></is></c><c r="F138" s="2" t="inlineStr"><is><t>kalcytoninę</t></is></c><c r="G138" s="2" t="inlineStr"><is><t>pamidronian</t></is></c><c r="H138" s="2" t="inlineStr"><is><t>hydrokortyzon</t></is></c><c r="I138" s="2" t="inlineStr"><is><t>furosemid</t></is></c><c r="J138" s="2" t="inlineStr" /><c r="K138" s="2" t="inlineStr" /><c r="L138" s="2" t="inlineStr" /><c r="M138" s="2" t="inlineStr" /><c r="N138" s="2" t="inlineStr" /><c r="O138" s="2" t="inlineStr" /><c r="P138" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q138" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="139"><c r="A139" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B139" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C139" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D139" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E139" s="2" t="inlineStr"><is><t>Immunosupresyjne działanie glikokortykosteroidów jest spowodowane:</t></is></c><c r="F139" s="2" t="inlineStr"><is><t>redukcją liczby limfocytów T</t></is></c><c r="G139" s="2" t="inlineStr"><is><t>zahamowaniem funkcji makrofagów tkankowych</t></is></c><c r="H139" s="2" t="inlineStr" /><c r="I139" s="2" t="inlineStr" /><c r="J139" s="2" t="inlineStr" /><c r="K139" s="2" t="inlineStr"><is><t>zwiększeniem syntezy IL-2</t></is></c><c r="L139" s="2" t="inlineStr"><is><t>aktywacją fosfolipazy A2 i zmniejszeniem syntezy prostaglandyn</t></is></c><c r="M139" s="2" t="inlineStr" /><c r="N139" s="2" t="inlineStr" /><c r="O139" s="2" t="inlineStr" /><c r="P139" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q139" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="140"><c r="A140" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B140" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C140" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D140" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E140" s="2" t="inlineStr"><is><t>91-letni mężczyzna jest leczony od co najmniej 6 miesięcy tamsulozyną, finasterydem, diosminą, piracetamem, zolpidemem, witaminą D3 w dużej dawce i węglanem wapnia. Na tej podstawie można powiedzieć, że:</t></is></c><c r="F140" s="2" t="inlineStr"><is><t>choruje na rozrost gruczołu krokowego</t></is></c><c r="G140" s="2" t="inlineStr"><is><t>jest uzależniony od zolpidemu</t></is></c><c r="H140" s="2" t="inlineStr"><is><t>można bez konsekwencji odstawić piracetam</t></is></c><c r="I140" s="2" t="inlineStr"><is><t>terapia zmniejsza ryzyko osteoporotycznych złamań kości</t></is></c><c r="J140" s="2" t="inlineStr" /><c r="K140" s="2" t="inlineStr" /><c r="L140" s="2" t="inlineStr" /><c r="M140" s="2" t="inlineStr" /><c r="N140" s="2" t="inlineStr" /><c r="O140" s="2" t="inlineStr" /><c r="P140" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q140" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="141"><c r="A141" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B141" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C141" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D141" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E141" s="2" t="inlineStr"><is><t>Witamina K1 (fitomenadion):</t></is></c><c r="F141" s="2" t="inlineStr"><is><t>może być wskazana u osób ze spontanicznym zwiększeniem INR&gt;GGN (górnej granicy normy) spowodowanym antybiotykami niszczącymi fizjologiczną florę jelit</t></is></c><c r="G141" s="2" t="inlineStr"><is><t>nie antagonizuje działania heparyny</t></is></c><c r="H141" s="2" t="inlineStr"><is><t>może spowodować reakcję rzekomoanafilaktyczną</t></is></c><c r="I141" s="2" t="inlineStr"><is><t>jest antidotum w przedawkowaniu pochodnych hydroksykumaryny</t></is></c><c r="J141" s="2" t="inlineStr" /><c r="K141" s="2" t="inlineStr" /><c r="L141" s="2" t="inlineStr" /><c r="M141" s="2" t="inlineStr" /><c r="N141" s="2" t="inlineStr" /><c r="O141" s="2" t="inlineStr" /><c r="P141" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q141" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="142"><c r="A142" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B142" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C142" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D142" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E142" s="2" t="inlineStr"><is><t>Działanie zapierające wykazuje:</t></is></c><c r="F142" s="2" t="inlineStr"><is><t>oksykodon</t></is></c><c r="G142" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="H142" s="2" t="inlineStr"><is><t>oktreotyd</t></is></c><c r="I142" s="2" t="inlineStr" /><c r="J142" s="2" t="inlineStr" /><c r="K142" s="2" t="inlineStr"><is><t>fosforan sodu</t></is></c><c r="L142" s="2" t="inlineStr" /><c r="M142" s="2" t="inlineStr" /><c r="N142" s="2" t="inlineStr" /><c r="O142" s="2" t="inlineStr" /><c r="P142" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q142" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="143"><c r="A143" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B143" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C143" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D143" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E143" s="2" t="inlineStr"><is><t>Działanie zapierające wykazuje:</t></is></c><c r="F143" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="G143" s="2" t="inlineStr"><is><t>węglan wapnia</t></is></c><c r="H143" s="2" t="inlineStr"><is><t>odwar z suchych owoców borówki czernicy</t></is></c><c r="I143" s="2" t="inlineStr" /><c r="J143" s="2" t="inlineStr" /><c r="K143" s="2" t="inlineStr"><is><t>erytromycyna</t></is></c><c r="L143" s="2" t="inlineStr" /><c r="M143" s="2" t="inlineStr" /><c r="N143" s="2" t="inlineStr" /><c r="O143" s="2" t="inlineStr" /><c r="P143" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q143" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="144"><c r="A144" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B144" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C144" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D144" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E144" s="2" t="inlineStr"><is><t>W leczeniu ostrej biegunki u dzieci uzasadnione jest zastosowanie:</t></is></c><c r="F144" s="2" t="inlineStr"><is><t>probiotyku S. boulardi</t></is></c><c r="G144" s="2" t="inlineStr"><is><t>racekadotrylu</t></is></c><c r="H144" s="2" t="inlineStr"><is><t>doustnego płynu nawadniającego</t></is></c><c r="I144" s="2" t="inlineStr" /><c r="J144" s="2" t="inlineStr" /><c r="K144" s="2" t="inlineStr"><is><t>loperamidu</t></is></c><c r="L144" s="2" t="inlineStr" /><c r="M144" s="2" t="inlineStr" /><c r="N144" s="2" t="inlineStr" /><c r="O144" s="2" t="inlineStr" /><c r="P144" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q144" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="145"><c r="A145" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B145" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C145" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D145" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E145" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek - mechanizm działania:</t></is></c><c r="F145" s="2" t="inlineStr"><is><t>itopryd - antagonista receptora D2</t></is></c><c r="G145" s="2" t="inlineStr"><is><t>alwimopan - antagonista receptora μ</t></is></c><c r="H145" s="2" t="inlineStr" /><c r="I145" s="2" t="inlineStr" /><c r="J145" s="2" t="inlineStr" /><c r="K145" s="2" t="inlineStr"><is><t>alweryna - agonista receptora motylinowego</t></is></c><c r="L145" s="2" t="inlineStr"><is><t>simetykon - agonista receptora 5-HT4</t></is></c><c r="M145" s="2" t="inlineStr" /><c r="N145" s="2" t="inlineStr" /><c r="O145" s="2" t="inlineStr" /><c r="P145" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q145" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="146"><c r="A146" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B146" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C146" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D146" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E146" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek - mechanizm działania:</t></is></c><c r="F146" s="2" t="inlineStr"><is><t>orlistat - blokowanie lipaz wytwarzanych w przewodzie pokarmowym</t></is></c><c r="G146" s="2" t="inlineStr"><is><t>tramadol – blokowanie zwrotnego wychwytu noradrenaliny i serotoniny w synapsach zstępującego układu analgetycznego</t></is></c><c r="H146" s="2" t="inlineStr"><is><t>ezetymib – hamowanie aktywności białka NPC1L1 w nabłonku błony śluzowej jelita</t></is></c><c r="I146" s="2" t="inlineStr"><is><t>celekoksyb -wybiórcze zablokowanie COX-2</t></is></c><c r="J146" s="2" t="inlineStr" /><c r="K146" s="2" t="inlineStr" /><c r="L146" s="2" t="inlineStr" /><c r="M146" s="2" t="inlineStr" /><c r="N146" s="2" t="inlineStr" /><c r="O146" s="2" t="inlineStr" /><c r="P146" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q146" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="147"><c r="A147" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B147" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C147" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D147" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E147" s="2" t="inlineStr"><is><t>W kolce wątrobowej uzasadnione jest podanie:</t></is></c><c r="F147" s="2" t="inlineStr"><is><t>ketoprofenu i.v</t></is></c><c r="G147" s="2" t="inlineStr"><is><t>papaweryny i.m</t></is></c><c r="H147" s="2" t="inlineStr"><is><t>butylobromku skopolaminy p.r</t></is></c><c r="I147" s="2" t="inlineStr"><is><t>buprenorfiny i.m</t></is></c><c r="J147" s="2" t="inlineStr" /><c r="K147" s="2" t="inlineStr" /><c r="L147" s="2" t="inlineStr" /><c r="M147" s="2" t="inlineStr" /><c r="N147" s="2" t="inlineStr" /><c r="O147" s="2" t="inlineStr" /><c r="P147" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q147" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="148"><c r="A148" s="2" t="inlineStr"><is><t>BÓLE GŁOWY</t></is></c><c r="B148" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C148" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D148" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E148" s="2" t="inlineStr"><is><t>Sumatryptan:</t></is></c><c r="F148" s="2" t="inlineStr"><is><t>pobudzając receptory 5-HT1D wywołuje wybiórczy skurcz naczyń i przerywa napad migreny</t></is></c><c r="G148" s="2" t="inlineStr"><is><t>jest niezalecany u pacjentów z chorobą niedokrwienną serca</t></is></c><c r="H148" s="2" t="inlineStr" /><c r="I148" s="2" t="inlineStr" /><c r="J148" s="2" t="inlineStr" /><c r="K148" s="2" t="inlineStr"><is><t>może być stosowany jedynie podskórnie</t></is></c><c r="L148" s="2" t="inlineStr"><is><t>może być podawany w czasie ciąży</t></is></c><c r="M148" s="2" t="inlineStr" /><c r="N148" s="2" t="inlineStr" /><c r="O148" s="2" t="inlineStr" /><c r="P148" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q148" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="149"><c r="A149" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B149" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C149" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D149" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E149" s="2" t="inlineStr"><is><t>W profilaktyce bólów migrenowych znalazł zastosowanie:</t></is></c><c r="F149" s="2" t="inlineStr"><is><t>topiramat</t></is></c><c r="G149" s="2" t="inlineStr"><is><t>erenumab</t></is></c><c r="H149" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="I149" s="2" t="inlineStr"><is><t>toksyna botulinowa</t></is></c><c r="J149" s="2" t="inlineStr" /><c r="K149" s="2" t="inlineStr" /><c r="L149" s="2" t="inlineStr" /><c r="M149" s="2" t="inlineStr" /><c r="N149" s="2" t="inlineStr" /><c r="O149" s="2" t="inlineStr" /><c r="P149" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q149" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="150"><c r="A150" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B150" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C150" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D150" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E150" s="2" t="inlineStr"><is><t>Erytropoetyna może zwiększyć:</t></is></c><c r="F150" s="2" t="inlineStr"><is><t>wartości ciśnienia tętniczego</t></is></c><c r="G150" s="2" t="inlineStr"><is><t>krzepliwość krwi</t></is></c><c r="H150" s="2" t="inlineStr"><is><t>maksymalną wydolność wysiłkową</t></is></c><c r="I150" s="2" t="inlineStr" /><c r="J150" s="2" t="inlineStr" /><c r="K150" s="2" t="inlineStr"><is><t>aktywność amylazy w surowicy</t></is></c><c r="L150" s="2" t="inlineStr" /><c r="M150" s="2" t="inlineStr" /><c r="N150" s="2" t="inlineStr" /><c r="O150" s="2" t="inlineStr" /><c r="P150" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q150" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="151"><c r="A151" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B151" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C151" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D151" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E151" s="2" t="inlineStr"><is><t>W profilaktyce wymiotów w przebiegu kinetoz stosuje się:</t></is></c><c r="F151" s="2" t="inlineStr"><is><t>skopolaminę</t></is></c><c r="G151" s="2" t="inlineStr"><is><t>dimenhydrinat</t></is></c><c r="H151" s="2" t="inlineStr" /><c r="I151" s="2" t="inlineStr" /><c r="J151" s="2" t="inlineStr" /><c r="K151" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="L151" s="2" t="inlineStr"><is><t>betahistynę</t></is></c><c r="M151" s="2" t="inlineStr" /><c r="N151" s="2" t="inlineStr" /><c r="O151" s="2" t="inlineStr" /><c r="P151" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q151" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="152"><c r="A152" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B152" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C152" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D152" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E152" s="2" t="inlineStr"><is><t>Oksymetazolina:</t></is></c><c r="F152" s="2" t="inlineStr"><is><t>może doprowadzić do wystąpienia tzw. efektu „ z odbicia”</t></is></c><c r="G152" s="2" t="inlineStr" /><c r="H152" s="2" t="inlineStr" /><c r="I152" s="2" t="inlineStr" /><c r="J152" s="2" t="inlineStr" /><c r="K152" s="2" t="inlineStr"><is><t>jest antagonistą receptorów adrenergicznych alfa</t></is></c><c r="L152" s="2" t="inlineStr"><is><t>wykazuje skuteczność kliniczną po 5. dniach terapii</t></is></c><c r="M152" s="2" t="inlineStr"><is><t>jest podawana doustnie</t></is></c><c r="N152" s="2" t="inlineStr" /><c r="O152" s="2" t="inlineStr" /><c r="P152" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q152" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="153"><c r="A153" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B153" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C153" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D153" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E153" s="2" t="inlineStr"><is><t>Petydyna:</t></is></c><c r="F153" s="2" t="inlineStr"><is><t>ma działanie zapierające</t></is></c><c r="G153" s="2" t="inlineStr"><is><t>nietypowo dla swojej grupy farmakologicznej rozszerza źrenice</t></is></c><c r="H153" s="2" t="inlineStr"><is><t>hamuje ośrodek oddechowy</t></is></c><c r="I153" s="2" t="inlineStr"><is><t>stosowana długotrwale działa neurotoksycznie przez kumulujący się metabolit</t></is></c><c r="J153" s="2" t="inlineStr" /><c r="K153" s="2" t="inlineStr" /><c r="L153" s="2" t="inlineStr" /><c r="M153" s="2" t="inlineStr" /><c r="N153" s="2" t="inlineStr" /><c r="O153" s="2" t="inlineStr" /><c r="P153" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q153" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="154"><c r="A154" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B154" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C154" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D154" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E154" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące małopłytkowości typu II wywołanej heparyną:</t></is></c><c r="F154" s="2" t="inlineStr"><is><t>stwierdzenie małopłytkowości immunologicznej w przebiegu leczenia heparyną jest wskazaniem do jej natychmiastowego odstawienia</t></is></c><c r="G154" s="2" t="inlineStr"><is><t>HIT II wiąże się z 20–40-krotnym zwiększeniem ryzyka zakrzepicy żylnej</t></is></c><c r="H154" s="2" t="inlineStr" /><c r="I154" s="2" t="inlineStr" /><c r="J154" s="2" t="inlineStr" /><c r="K154" s="2" t="inlineStr"><is><t>HIT II występuje najczęściej po 3 tygodniach od rozpoczęcia terapii heparyną</t></is></c><c r="L154" s="2" t="inlineStr"><is><t>heparyny drobnocząsteczkowe nie stwarzają ryzyka wystąpienia trombocytopenii immunologicznej</t></is></c><c r="M154" s="2" t="inlineStr" /><c r="N154" s="2" t="inlineStr" /><c r="O154" s="2" t="inlineStr" /><c r="P154" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q154" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="155"><c r="A155" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B155" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C155" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D155" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E155" s="2" t="inlineStr"><is><t>U kobiet w trzecim trymestrze ciąży przeciwwskazany/-a jest:</t></is></c><c r="F155" s="2" t="inlineStr"><is><t>ketoprofen</t></is></c><c r="G155" s="2" t="inlineStr"><is><t>walsartan</t></is></c><c r="H155" s="2" t="inlineStr"><is><t>acenokumarol</t></is></c><c r="I155" s="2" t="inlineStr" /><c r="J155" s="2" t="inlineStr" /><c r="K155" s="2" t="inlineStr"><is><t>enoksaparyna</t></is></c><c r="L155" s="2" t="inlineStr" /><c r="M155" s="2" t="inlineStr" /><c r="N155" s="2" t="inlineStr" /><c r="O155" s="2" t="inlineStr" /><c r="P155" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q155" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="156"><c r="A156" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B156" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C156" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D156" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E156" s="2" t="inlineStr"><is><t>U pacjenta leczonego przeciwzakrzepowo dabigatranem ze stwierdzonym umiarkowanym aktywnym krwawieniem należy:</t></is></c><c r="F156" s="2" t="inlineStr"><is><t>odroczyć podanie kolejnej dawki leku</t></is></c><c r="G156" s="2" t="inlineStr"><is><t>zapewnić podaż płynów</t></is></c><c r="H156" s="2" t="inlineStr"><is><t>rozważyć podanie węgla aktywowanego jeśli dabigatran był podany niedawno</t></is></c><c r="I156" s="2" t="inlineStr" /><c r="J156" s="2" t="inlineStr" /><c r="K156" s="2" t="inlineStr"><is><t>zastosować siarczan protaminy</t></is></c><c r="L156" s="2" t="inlineStr" /><c r="M156" s="2" t="inlineStr" /><c r="N156" s="2" t="inlineStr" /><c r="O156" s="2" t="inlineStr" /><c r="P156" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q156" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="157"><c r="A157" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B157" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C157" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D157" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E157" s="2" t="inlineStr"><is><t>Nadroparyna:</t></is></c><c r="F157" s="2" t="inlineStr"><is><t>może być podawana dożylnie</t></is></c><c r="G157" s="2" t="inlineStr"><is><t>jest skuteczna w leczeniu zakrzepicy żył głębokich</t></is></c><c r="H157" s="2" t="inlineStr" /><c r="I157" s="2" t="inlineStr" /><c r="J157" s="2" t="inlineStr" /><c r="K157" s="2" t="inlineStr"><is><t>jest antagonistą receptora PAR-1</t></is></c><c r="L157" s="2" t="inlineStr"><is><t>w profilaktyce zakrzepicy żylnej powinna być podana nie później niż 36 godzin przed zabiegiem chirurgicznym</t></is></c><c r="M157" s="2" t="inlineStr" /><c r="N157" s="2" t="inlineStr" /><c r="O157" s="2" t="inlineStr" /><c r="P157" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q157" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="158"><c r="A158" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B158" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C158" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D158" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E158" s="2" t="inlineStr"><is><t>Wskazaniem do podania tkankowego aktywatora plazminogenu (t-PA) może być:</t></is></c><c r="F158" s="2" t="inlineStr"><is><t>zatorowość płucna wysokiego ryzyka (czyli z niestabilnością hemodynamiczną)</t></is></c><c r="G158" s="2" t="inlineStr"><is><t>ostry zator tętnicy kończyny dolnej</t></is></c><c r="H158" s="2" t="inlineStr"><is><t>ostry udar niedokrwienny mózgu</t></is></c><c r="I158" s="2" t="inlineStr" /><c r="J158" s="2" t="inlineStr" /><c r="K158" s="2" t="inlineStr"><is><t>ostry zespół wieńcowy bez uniesienia odcinka ST</t></is></c><c r="L158" s="2" t="inlineStr" /><c r="M158" s="2" t="inlineStr" /><c r="N158" s="2" t="inlineStr" /><c r="O158" s="2" t="inlineStr" /><c r="P158" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q158" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="159"><c r="A159" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B159" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C159" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D159" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E159" s="2" t="inlineStr"><is><t>W udarze niedokrwiennym mózgu należy:</t></is></c><c r="F159" s="2" t="inlineStr"><is><t>obniżać ciśnienie tętnicze jeśli przekracza wartości 220/120 mmHg</t></is></c><c r="G159" s="2" t="inlineStr"><is><t>podać doustnie kwas acetylosalicylowy jeżeli nie można zastosować leczenia trombolitycznego</t></is></c><c r="H159" s="2" t="inlineStr" /><c r="I159" s="2" t="inlineStr" /><c r="J159" s="2" t="inlineStr" /><c r="K159" s="2" t="inlineStr"><is><t>stosować duże dawki heparyny niefrakcjonowanej</t></is></c><c r="L159" s="2" t="inlineStr"><is><t>profilaktycznie podawać antybiotyki β-laktamowe ze względu na bardzo częste występowanie infekcji dróg oddechowych</t></is></c><c r="M159" s="2" t="inlineStr" /><c r="N159" s="2" t="inlineStr" /><c r="O159" s="2" t="inlineStr" /><c r="P159" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q159" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="160"><c r="A160" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B160" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C160" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D160" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E160" s="2" t="inlineStr"><is><t>Inhibitory reduktazy HMG-CoA zwiększają produkcję:</t></is></c><c r="F160" s="2" t="inlineStr"><is><t>tkankowego aktywatora plazminogenu</t></is></c><c r="G160" s="2" t="inlineStr"><is><t>tlenku azotu</t></is></c><c r="H160" s="2" t="inlineStr" /><c r="I160" s="2" t="inlineStr" /><c r="J160" s="2" t="inlineStr" /><c r="K160" s="2" t="inlineStr"><is><t>metaloproteinaz</t></is></c><c r="L160" s="2" t="inlineStr"><is><t>tromboksanu A2</t></is></c><c r="M160" s="2" t="inlineStr" /><c r="N160" s="2" t="inlineStr" /><c r="O160" s="2" t="inlineStr" /><c r="P160" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q160" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="161"><c r="A161" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B161" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C161" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D161" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E161" s="2" t="inlineStr"><is><t>20% roztwór albumin:</t></is></c><c r="F161" s="2" t="inlineStr"><is><t>powoduje ponad 100% przyrost objętości osocza</t></is></c><c r="G161" s="2" t="inlineStr"><is><t>działa objętościowo do 6 h</t></is></c><c r="H161" s="2" t="inlineStr" /><c r="I161" s="2" t="inlineStr" /><c r="J161" s="2" t="inlineStr" /><c r="K161" s="2" t="inlineStr"><is><t>może spowodować uszkodzenie nerek</t></is></c><c r="L161" s="2" t="inlineStr"><is><t>ma istotny wpływ na krzepnięcie krwi</t></is></c><c r="M161" s="2" t="inlineStr" /><c r="N161" s="2" t="inlineStr" /><c r="O161" s="2" t="inlineStr" /><c r="P161" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q161" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="162"><c r="A162" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B162" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C162" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D162" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E162" s="2" t="inlineStr"><is><t>Zastosowanie atrakurium może być przyczyną:</t></is></c><c r="F162" s="2" t="inlineStr"><is><t>długotrwałego efektu zwiotczającego</t></is></c><c r="G162" s="2" t="inlineStr" /><c r="H162" s="2" t="inlineStr" /><c r="I162" s="2" t="inlineStr" /><c r="J162" s="2" t="inlineStr" /><c r="K162" s="2" t="inlineStr"><is><t>drżenia włókienkowego mięśni szkieletowych</t></is></c><c r="L162" s="2" t="inlineStr"><is><t>anestezji</t></is></c><c r="M162" s="2" t="inlineStr"><is><t>hipertermii złośliwej</t></is></c><c r="N162" s="2" t="inlineStr" /><c r="O162" s="2" t="inlineStr" /><c r="P162" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q162" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="163"><c r="A163" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B163" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C163" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D163" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E163" s="2" t="inlineStr"><is><t>Torasemid:</t></is></c><c r="F163" s="2" t="inlineStr"><is><t>hamuje symporter sodowo-potasowo-chlorkowy części grubościennej ramienia wstępującego pętli Henlego</t></is></c><c r="G163" s="2" t="inlineStr"><is><t>zwiększa aktywność reninową osocza</t></is></c><c r="H163" s="2" t="inlineStr" /><c r="I163" s="2" t="inlineStr" /><c r="J163" s="2" t="inlineStr" /><c r="K163" s="2" t="inlineStr"><is><t>zmniejsza wydalanie wapnia z moczem</t></is></c><c r="L163" s="2" t="inlineStr"><is><t>jest nieskuteczny, jeśli eGFRr &lt; 30 ml/min</t></is></c><c r="M163" s="2" t="inlineStr" /><c r="N163" s="2" t="inlineStr" /><c r="O163" s="2" t="inlineStr" /><c r="P163" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q163" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="164"><c r="A164" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B164" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C164" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D164" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E164" s="2" t="inlineStr"><is><t>Formularz świadomej zgody uczestnika na udział w badaniu klinicznym powinien zostać podpisany:</t></is></c><c r="F164" s="2" t="inlineStr"><is><t>przez uczestnika badania</t></is></c><c r="G164" s="2" t="inlineStr"><is><t>przez badacza</t></is></c><c r="H164" s="2" t="inlineStr"><is><t>w dwóch egzemplarzach</t></is></c><c r="I164" s="2" t="inlineStr" /><c r="J164" s="2" t="inlineStr" /><c r="K164" s="2" t="inlineStr"><is><t>bezpośrednio po badaniach oceniających czy pacjent spełnia kryteria włączenia do badania</t></is></c><c r="L164" s="2" t="inlineStr" /><c r="M164" s="2" t="inlineStr" /><c r="N164" s="2" t="inlineStr" /><c r="O164" s="2" t="inlineStr" /><c r="P164" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q164" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="165"><c r="A165" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B165" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C165" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D165" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E165" s="2" t="inlineStr"><is><t>W leczeniu zarażenia owsikiem skuteczny jest:</t></is></c><c r="F165" s="2" t="inlineStr"><is><t>mebendazol</t></is></c><c r="G165" s="2" t="inlineStr"><is><t>albendazol</t></is></c><c r="H165" s="2" t="inlineStr"><is><t>pyrantel</t></is></c><c r="I165" s="2" t="inlineStr" /><c r="J165" s="2" t="inlineStr" /><c r="K165" s="2" t="inlineStr"><is><t>tynidazol</t></is></c><c r="L165" s="2" t="inlineStr" /><c r="M165" s="2" t="inlineStr" /><c r="N165" s="2" t="inlineStr" /><c r="O165" s="2" t="inlineStr" /><c r="P165" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q165" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="166"><c r="A166" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B166" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C166" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D166" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E166" s="2" t="inlineStr"><is><t>Cytomegalię u osób z niedoborami odporności należy leczyć stosując:</t></is></c><c r="F166" s="2" t="inlineStr"><is><t>gancyklowir</t></is></c><c r="G166" s="2" t="inlineStr" /><c r="H166" s="2" t="inlineStr" /><c r="I166" s="2" t="inlineStr" /><c r="J166" s="2" t="inlineStr" /><c r="K166" s="2" t="inlineStr"><is><t>zanamiwir</t></is></c><c r="L166" s="2" t="inlineStr"><is><t>acyklowir</t></is></c><c r="M166" s="2" t="inlineStr"><is><t>oseltamiwir</t></is></c><c r="N166" s="2" t="inlineStr" /><c r="O166" s="2" t="inlineStr" /><c r="P166" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q166" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="167"><c r="A167" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B167" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C167" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D167" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E167" s="2" t="inlineStr"><is><t>W terapii POChP u osób o wysokim ryzyku zaostrzeń i dużym nasileniu objawów (grupa</t></is></c><c r="F167" s="2" t="inlineStr"><is><t>bromek tiotropium z formoterolem i cyklezonidem</t></is></c><c r="G167" s="2" t="inlineStr"><is><t>budezonid z formoterolem</t></is></c><c r="H167" s="2" t="inlineStr"><is><t>bromek aklidynium z salmeterolem i flutikazonem</t></is></c><c r="I167" s="2" t="inlineStr"><is><t>bromek glikopironium z roflumilastem</t></is></c><c r="J167" s="2" t="inlineStr" /><c r="K167" s="2" t="inlineStr"><is><t>można zastosować:</t></is></c><c r="L167" s="2" t="inlineStr" /><c r="M167" s="2" t="inlineStr" /><c r="N167" s="2" t="inlineStr" /><c r="O167" s="2" t="inlineStr" /><c r="P167" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q167" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="168"><c r="A168" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B168" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C168" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D168" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E168" s="2" t="inlineStr"><is><t>Wskaż prawidłowe twierdzenie dotyczące farmakoterapii astmy oskrzelowej :</t></is></c><c r="F168" s="2" t="inlineStr"><is><t>wziewne glikokortykosteroidy zmniejszają częstość/liczbę hospitalizacji i umieralność z powodu astmy</t></is></c><c r="G168" s="2" t="inlineStr"><is><t>długodziałające wziewne betaadrenomimetyki w monoterapii mogą zwiększać ryzyko zgonu z powodu astmy</t></is></c><c r="H168" s="2" t="inlineStr"><is><t>kromony mogą być skuteczne u chorych ze skurczem oskrzeli wywoływanym przez wysiłek fizyczny</t></is></c><c r="I168" s="2" t="inlineStr" /><c r="J168" s="2" t="inlineStr" /><c r="K168" s="2" t="inlineStr"><is><t>leki przeciwleukotrienowe w monoterapii są bardziej skuteczne od wziewnych glikokortykosteroidów w małych dawkach</t></is></c><c r="L168" s="2" t="inlineStr" /><c r="M168" s="2" t="inlineStr" /><c r="N168" s="2" t="inlineStr" /><c r="O168" s="2" t="inlineStr" /><c r="P168" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q168" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="169"><c r="A169" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B169" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C169" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D169" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E169" s="2" t="inlineStr"><is><t>W leczeniu wodobrzusza w przebiegu marskości wątroby wskazane jest stosowanie:</t></is></c><c r="F169" s="2" t="inlineStr"><is><t>furosemidu</t></is></c><c r="G169" s="2" t="inlineStr"><is><t>spironolaktonu</t></is></c><c r="H169" s="2" t="inlineStr"><is><t>karwedilolu</t></is></c><c r="I169" s="2" t="inlineStr" /><c r="J169" s="2" t="inlineStr" /><c r="K169" s="2" t="inlineStr"><is><t>ramiprylu</t></is></c><c r="L169" s="2" t="inlineStr" /><c r="M169" s="2" t="inlineStr" /><c r="N169" s="2" t="inlineStr" /><c r="O169" s="2" t="inlineStr" /><c r="P169" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q169" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="170"><c r="A170" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B170" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C170" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D170" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E170" s="2" t="inlineStr"><is><t>W leczeniu dny moczanowej należy:</t></is></c><c r="F170" s="2" t="inlineStr"><is><t>stosować dietę z ograniczeniem podaży mięs, podrobów i fruktozy</t></is></c><c r="G170" s="2" t="inlineStr"><is><t>objawowo stosować leki z grupy NLPZ</t></is></c><c r="H170" s="2" t="inlineStr" /><c r="I170" s="2" t="inlineStr" /><c r="J170" s="2" t="inlineStr" /><c r="K170" s="2" t="inlineStr"><is><t>podać jak najszybciej allopurynol przy podejrzeniu ostrego napadu</t></is></c><c r="L170" s="2" t="inlineStr"><is><t>w każdym przypadku bezobjawowej hiperurykemii stosować kolchicynę</t></is></c><c r="M170" s="2" t="inlineStr" /><c r="N170" s="2" t="inlineStr" /><c r="O170" s="2" t="inlineStr" /><c r="P170" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q170" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="171"><c r="A171" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B171" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C171" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D171" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E171" s="2" t="inlineStr"><is><t>Zotarolimus:</t></is></c><c r="F171" s="2" t="inlineStr"><is><t>jest stosowany w stentach wieńcowych uwalniających lek</t></is></c><c r="G171" s="2" t="inlineStr" /><c r="H171" s="2" t="inlineStr" /><c r="I171" s="2" t="inlineStr" /><c r="J171" s="2" t="inlineStr" /><c r="K171" s="2" t="inlineStr"><is><t>jest rekombinowanym w pełni ludzkim przeciwciałem monoklonalnym</t></is></c><c r="L171" s="2" t="inlineStr"><is><t>nie może być stosowany łącznie z kwasem acetylosalicylowym</t></is></c><c r="M171" s="2" t="inlineStr"><is><t>neutralizuje biologiczną aktywność TNF</t></is></c><c r="N171" s="2" t="inlineStr" /><c r="O171" s="2" t="inlineStr" /><c r="P171" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q171" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="172"><c r="A172" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B172" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C172" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D172" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E172" s="2" t="inlineStr"><is><t>W leczeniu choroby Alzheimera:</t></is></c><c r="F172" s="2" t="inlineStr"><is><t>w zaawansowanych przypadkach wskazane jest włączenie do leczenia antagonisty receptorów NMDA</t></is></c><c r="G172" s="2" t="inlineStr"><is><t>donepezil korzystnie wpływa na globalne zdolności intelektualne w łagodnych stadiach choroby</t></is></c><c r="H172" s="2" t="inlineStr" /><c r="I172" s="2" t="inlineStr" /><c r="J172" s="2" t="inlineStr" /><c r="K172" s="2" t="inlineStr"><is><t>stosuje się leki cholinolityczne</t></is></c><c r="L172" s="2" t="inlineStr"><is><t>istotną rolę odgrywa zastosowanie piracetamu</t></is></c><c r="M172" s="2" t="inlineStr" /><c r="N172" s="2" t="inlineStr" /><c r="O172" s="2" t="inlineStr" /><c r="P172" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q172" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="173"><c r="A173" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B173" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C173" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D173" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E173" s="2" t="inlineStr"><is><t>Przewlekłe stosowanie lorazepamu może spowodować:</t></is></c><c r="F173" s="2" t="inlineStr"><is><t>otępienie</t></is></c><c r="G173" s="2" t="inlineStr"><is><t>tolerancję na jego działanie</t></is></c><c r="H173" s="2" t="inlineStr"><is><t>uzależnienie psychiczne i fizyczne</t></is></c><c r="I173" s="2" t="inlineStr" /><c r="J173" s="2" t="inlineStr" /><c r="K173" s="2" t="inlineStr"><is><t>stan padaczkowy</t></is></c><c r="L173" s="2" t="inlineStr" /><c r="M173" s="2" t="inlineStr" /><c r="N173" s="2" t="inlineStr" /><c r="O173" s="2" t="inlineStr" /><c r="P173" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q173" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="174"><c r="A174" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B174" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C174" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D174" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E174" s="2" t="inlineStr"><is><t>Do leczenia ostrego zamknięcia kąta przesączania (potocznie ataku jaskry) można zastosować:</t></is></c><c r="F174" s="2" t="inlineStr"><is><t>tymolol</t></is></c><c r="G174" s="2" t="inlineStr"><is><t>acetazolamid</t></is></c><c r="H174" s="2" t="inlineStr"><is><t>mannitol</t></is></c><c r="I174" s="2" t="inlineStr" /><c r="J174" s="2" t="inlineStr" /><c r="K174" s="2" t="inlineStr"><is><t>zydowudynę</t></is></c><c r="L174" s="2" t="inlineStr" /><c r="M174" s="2" t="inlineStr" /><c r="N174" s="2" t="inlineStr" /><c r="O174" s="2" t="inlineStr" /><c r="P174" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q174" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="175"><c r="A175" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B175" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C175" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D175" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E175" s="2" t="inlineStr"><is><t>Do leczenia ostrego zamknięcia kąta przesączania (potocznie ataku jaskry) można zastosować:</t></is></c><c r="F175" s="2" t="inlineStr"><is><t>Timolol</t></is></c><c r="G175" s="2" t="inlineStr"><is><t>Acetazolamid</t></is></c><c r="H175" s="2" t="inlineStr"><is><t>Mannitol</t></is></c><c r="I175" s="2" t="inlineStr" /><c r="J175" s="2" t="inlineStr" /><c r="K175" s="2" t="inlineStr"><is><t>Zydowudynę</t></is></c><c r="L175" s="2" t="inlineStr" /><c r="M175" s="2" t="inlineStr" /><c r="N175" s="2" t="inlineStr" /><c r="O175" s="2" t="inlineStr" /><c r="P175" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q175" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="176"><c r="A176" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B176" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C176" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D176" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E176" s="2" t="inlineStr"><is><t>W leczeniu stanu padaczkowego:</t></is></c><c r="F176" s="2" t="inlineStr"><is><t>lekiem pierwszego rzutu jest diazepam i.v</t></is></c><c r="G176" s="2" t="inlineStr"><is><t>w przypadku postaci opornej na leczenie można zastosować wlew dożylny midazolamu</t></is></c><c r="H176" s="2" t="inlineStr" /><c r="I176" s="2" t="inlineStr" /><c r="J176" s="2" t="inlineStr" /><c r="K176" s="2" t="inlineStr"><is><t>nie powinno się stosować fenytoiny we wlewie dożylnym</t></is></c><c r="L176" s="2" t="inlineStr"><is><t>należy stosować duże dawki steroidów i.v</t></is></c><c r="M176" s="2" t="inlineStr" /><c r="N176" s="2" t="inlineStr" /><c r="O176" s="2" t="inlineStr" /><c r="P176" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q176" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="177"><c r="A177" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B177" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C177" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D177" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E177" s="2" t="inlineStr"><is><t>Charakterystyka Produktu Leczniczego (ChPL) zawiera informacje o:</t></is></c><c r="F177" s="2" t="inlineStr"><is><t>specjalnych środkach ostrożności podczas przechowywania produktu leczniczego</t></is></c><c r="G177" s="2" t="inlineStr"><is><t>właściwościach farmakokinetycznych leku</t></is></c><c r="H177" s="2" t="inlineStr"><is><t>dacie wydania pierwszego pozwolenia na dopuszczenie do obrotu</t></is></c><c r="I177" s="2" t="inlineStr" /><c r="J177" s="2" t="inlineStr" /><c r="K177" s="2" t="inlineStr"><is><t>cenie produktu leczniczego</t></is></c><c r="L177" s="2" t="inlineStr" /><c r="M177" s="2" t="inlineStr" /><c r="N177" s="2" t="inlineStr" /><c r="O177" s="2" t="inlineStr" /><c r="P177" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q177" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="178"><c r="A178" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B178" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C178" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D178" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E178" s="2" t="inlineStr"><is><t>Agencja Oceny Technologii Medycznych i Taryfikacji:</t></is></c><c r="F178" s="2" t="inlineStr"><is><t>wycenia procedury medyczne</t></is></c><c r="G178" s="2" t="inlineStr"><is><t>zajmuje stanowisko w sprawie skuteczności i bezpieczeństwa leków</t></is></c><c r="H178" s="2" t="inlineStr"><is><t>rekomenduje leki do refundacji</t></is></c><c r="I178" s="2" t="inlineStr" /><c r="J178" s="2" t="inlineStr" /><c r="K178" s="2" t="inlineStr"><is><t>rejestruje leki</t></is></c><c r="L178" s="2" t="inlineStr" /><c r="M178" s="2" t="inlineStr" /><c r="N178" s="2" t="inlineStr" /><c r="O178" s="2" t="inlineStr" /><c r="P178" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q178" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="179"><c r="A179" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B179" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C179" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D179" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E179" s="2" t="inlineStr"><is><t>W hierarchii badań naukowych:</t></is></c><c r="F179" s="2" t="inlineStr"><is><t>badania kohortowe mają wyższą pozycję niż serie przypadków</t></is></c><c r="G179" s="2" t="inlineStr" /><c r="H179" s="2" t="inlineStr" /><c r="I179" s="2" t="inlineStr" /><c r="J179" s="2" t="inlineStr" /><c r="K179" s="2" t="inlineStr"><is><t>metaanalizy są na tym samym poziomie co randomizowane badania kontrolowane</t></is></c><c r="L179" s="2" t="inlineStr"><is><t>najwyższą pozycję mają randomizowane badania kontrolowane</t></is></c><c r="M179" s="2" t="inlineStr"><is><t>badania kohortowe są na tym samym poziomie co randomizowane badania kliniczne</t></is></c><c r="N179" s="2" t="inlineStr" /><c r="O179" s="2" t="inlineStr" /><c r="P179" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q179" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="180"><c r="A180" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B180" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C180" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D180" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E180" s="2" t="inlineStr"><is><t>Desloratadyna:</t></is></c><c r="F180" s="2" t="inlineStr"><is><t>selektywnie blokuje receptory H1</t></is></c><c r="G180" s="2" t="inlineStr"><is><t>ma zastosowanie w leczeniu przewlekłego alergicznego nieżytu nosa</t></is></c><c r="H180" s="2" t="inlineStr" /><c r="I180" s="2" t="inlineStr" /><c r="J180" s="2" t="inlineStr" /><c r="K180" s="2" t="inlineStr"><is><t>dobrze przenika przez barierę krew- mózg</t></is></c><c r="L180" s="2" t="inlineStr"><is><t>ma znaczące działanie proarytmiczne</t></is></c><c r="M180" s="2" t="inlineStr" /><c r="N180" s="2" t="inlineStr" /><c r="O180" s="2" t="inlineStr" /><c r="P180" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q180" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="181"><c r="A181" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B181" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C181" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D181" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E181" s="2" t="inlineStr"><is><t>Mannitol podany iv. zmniejsza:</t></is></c><c r="F181" s="2" t="inlineStr"><is><t>ciśnienie wewnątrzczaszkowe</t></is></c><c r="G181" s="2" t="inlineStr" /><c r="H181" s="2" t="inlineStr" /><c r="I181" s="2" t="inlineStr" /><c r="J181" s="2" t="inlineStr" /><c r="K181" s="2" t="inlineStr"><is><t>ciśnienie osmotyczne płynu zewnątrzkomórkowego</t></is></c><c r="L181" s="2" t="inlineStr"><is><t>wydalanie sodu i chlorków</t></is></c><c r="M181" s="2" t="inlineStr"><is><t>filtrację nerkową</t></is></c><c r="N181" s="2" t="inlineStr" /><c r="O181" s="2" t="inlineStr" /><c r="P181" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q181" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="182"><c r="A182" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B182" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C182" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D182" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E182" s="2" t="inlineStr"><is><t>Podanie inhibitorów wychwytu zwrotnego serotoniny (SSRI) jest uzasadnione u pacjentów z:</t></is></c><c r="F182" s="2" t="inlineStr"><is><t>lękiem uogólnionym</t></is></c><c r="G182" s="2" t="inlineStr"><is><t>chorobą afektywną dwubiegunową</t></is></c><c r="H182" s="2" t="inlineStr"><is><t>nerwicą natręctw</t></is></c><c r="I182" s="2" t="inlineStr"><is><t>chorobą afektywną jednobiegunową</t></is></c><c r="J182" s="2" t="inlineStr" /><c r="K182" s="2" t="inlineStr" /><c r="L182" s="2" t="inlineStr" /><c r="M182" s="2" t="inlineStr" /><c r="N182" s="2" t="inlineStr" /><c r="O182" s="2" t="inlineStr" /><c r="P182" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q182" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="183"><c r="A183" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B183" s="2" t="inlineStr"><is><t>Struktura chemiczna</t></is></c><c r="C183" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D183" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E183" s="2" t="inlineStr"><is><t>Do wspólnych cech wenlafaksyny i amitryptyliny należy:</t></is></c><c r="F183" s="2" t="inlineStr"><is><t>hamowanie wychwytu zwrotnego serotoniny i noradrenaliny</t></is></c><c r="G183" s="2" t="inlineStr" /><c r="H183" s="2" t="inlineStr" /><c r="I183" s="2" t="inlineStr" /><c r="J183" s="2" t="inlineStr" /><c r="K183" s="2" t="inlineStr"><is><t>trójpierścieniowa budowa chemiczna</t></is></c><c r="L183" s="2" t="inlineStr"><is><t>konieczność znacznych ograniczeń dietetycznych podczas ich stosowania ze względu na ryzyko wystąpienia tzw. zespołu serowego (cheese effect)</t></is></c><c r="M183" s="2" t="inlineStr"><is><t>antagonizm wobec receptorów muskarynowych M1</t></is></c><c r="N183" s="2" t="inlineStr" /><c r="O183" s="2" t="inlineStr" /><c r="P183" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q183" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="184"><c r="A184" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B184" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C184" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D184" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E184" s="2" t="inlineStr"><is><t>Leki, które hamują kompleks kalcyneuryny to:</t></is></c><c r="F184" s="2" t="inlineStr"><is><t>cyklosporyna</t></is></c><c r="G184" s="2" t="inlineStr"><is><t>takrolimus</t></is></c><c r="H184" s="2" t="inlineStr" /><c r="I184" s="2" t="inlineStr" /><c r="J184" s="2" t="inlineStr" /><c r="K184" s="2" t="inlineStr"><is><t>talidomid</t></is></c><c r="L184" s="2" t="inlineStr"><is><t>mykofenolan mofetylu</t></is></c><c r="M184" s="2" t="inlineStr" /><c r="N184" s="2" t="inlineStr" /><c r="O184" s="2" t="inlineStr" /><c r="P184" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q184" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="185"><c r="A185" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B185" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C185" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D185" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E185" s="2" t="inlineStr"><is><t>Lacydypina:</t></is></c><c r="F185" s="2" t="inlineStr"><is><t>zmniejsza obciążenie następcze serca</t></is></c><c r="G185" s="2" t="inlineStr" /><c r="H185" s="2" t="inlineStr" /><c r="I185" s="2" t="inlineStr" /><c r="J185" s="2" t="inlineStr" /><c r="K185" s="2" t="inlineStr"><is><t>ma silne działanie inotropowe ujemne</t></is></c><c r="L185" s="2" t="inlineStr"><is><t>ma działanie dromotropowe ujemne</t></is></c><c r="M185" s="2" t="inlineStr"><is><t>ma działanie chronotropowe dodatnie</t></is></c><c r="N185" s="2" t="inlineStr" /><c r="O185" s="2" t="inlineStr" /><c r="P185" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q185" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="186"><c r="A186" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B186" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C186" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D186" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E186" s="2" t="inlineStr"><is><t>Do donorów tlenku azotu należy:</t></is></c><c r="F186" s="2" t="inlineStr"><is><t>nikorandil</t></is></c><c r="G186" s="2" t="inlineStr"><is><t>molsidomina</t></is></c><c r="H186" s="2" t="inlineStr"><is><t>diazotan izosorbitolu</t></is></c><c r="I186" s="2" t="inlineStr" /><c r="J186" s="2" t="inlineStr" /><c r="K186" s="2" t="inlineStr"><is><t>trimetazydyna</t></is></c><c r="L186" s="2" t="inlineStr" /><c r="M186" s="2" t="inlineStr" /><c r="N186" s="2" t="inlineStr" /><c r="O186" s="2" t="inlineStr" /><c r="P186" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q186" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="187"><c r="A187" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B187" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C187" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D187" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E187" s="2" t="inlineStr"><is><t>Względna dostępność biologiczna leku (biorównoważność) może być określona przez porównanie AUC:</t></is></c><c r="F187" s="2" t="inlineStr"><is><t>leku wzorcowego podanego drogą pozanaczyniową i dożylnie</t></is></c><c r="G187" s="2" t="inlineStr"><is><t>leku wzorcowego i badanego podanych tą samą drogą</t></is></c><c r="H187" s="2" t="inlineStr" /><c r="I187" s="2" t="inlineStr" /><c r="J187" s="2" t="inlineStr" /><c r="K187" s="2" t="inlineStr"><is><t>tylko leków podawanych drogą dożylną</t></is></c><c r="L187" s="2" t="inlineStr"><is><t>leku badanego podanego drogą pozanaczyniową i wzorcowego podanego dożylnie</t></is></c><c r="M187" s="2" t="inlineStr" /><c r="N187" s="2" t="inlineStr" /><c r="O187" s="2" t="inlineStr" /><c r="P187" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q187" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="188"><c r="A188" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B188" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C188" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D188" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E188" s="2" t="inlineStr"><is><t>Benzodiazepiną, która nie podlega metabolizmowi wątrobowemu jest:</t></is></c><c r="F188" s="2" t="inlineStr"><is><t>lorazepam</t></is></c><c r="G188" s="2" t="inlineStr"><is><t>oksazepam</t></is></c><c r="H188" s="2" t="inlineStr" /><c r="I188" s="2" t="inlineStr" /><c r="J188" s="2" t="inlineStr" /><c r="K188" s="2" t="inlineStr"><is><t>nitrazepam</t></is></c><c r="L188" s="2" t="inlineStr"><is><t>diazepam</t></is></c><c r="M188" s="2" t="inlineStr" /><c r="N188" s="2" t="inlineStr" /><c r="O188" s="2" t="inlineStr" /><c r="P188" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q188" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="189"><c r="A189" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B189" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C189" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D189" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E189" s="2" t="inlineStr"><is><t>Objętość dystrybucji ma znaczenie w określeniu wielkości dawki:</t></is></c><c r="F189" s="2" t="inlineStr"><is><t>nasycającej</t></is></c><c r="G189" s="2" t="inlineStr"><is><t>podtrzymującej</t></is></c><c r="H189" s="2" t="inlineStr" /><c r="I189" s="2" t="inlineStr" /><c r="J189" s="2" t="inlineStr" /><c r="K189" s="2" t="inlineStr"><is><t>śmiertelnej</t></is></c><c r="L189" s="2" t="inlineStr"><is><t>toksycznej</t></is></c><c r="M189" s="2" t="inlineStr" /><c r="N189" s="2" t="inlineStr" /><c r="O189" s="2" t="inlineStr" /><c r="P189" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q189" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="190"><c r="A190" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B190" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C190" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D190" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E190" s="2" t="inlineStr"><is><t>Do obniżenia gorączki u 2-letniego dziecka można zastosować:</t></is></c><c r="F190" s="2" t="inlineStr"><is><t>czopek doodbytniczy zawierający paracetamol</t></is></c><c r="G190" s="2" t="inlineStr"><is><t>zawiesinę doustną zawierającą ibuprofen</t></is></c><c r="H190" s="2" t="inlineStr" /><c r="I190" s="2" t="inlineStr" /><c r="J190" s="2" t="inlineStr" /><c r="K190" s="2" t="inlineStr"><is><t>tabletki o natychmiastowym uwalnianiu w jamie ustnej zawierające kwas acetylosalicylowy</t></is></c><c r="L190" s="2" t="inlineStr"><is><t>wstrzyknięcie domięśniowe metamizolu</t></is></c><c r="M190" s="2" t="inlineStr" /><c r="N190" s="2" t="inlineStr" /><c r="O190" s="2" t="inlineStr" /><c r="P190" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q190" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="191"><c r="A191" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B191" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C191" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D191" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E191" s="2" t="inlineStr"><is><t>Typowe leki podlegające monitorowaniu stężeń to:</t></is></c><c r="F191" s="2" t="inlineStr"><is><t>cyklosporyna</t></is></c><c r="G191" s="2" t="inlineStr"><is><t>fenytoina</t></is></c><c r="H191" s="2" t="inlineStr"><is><t>gentamycyna</t></is></c><c r="I191" s="2" t="inlineStr"><is><t>Digoksyna</t></is></c><c r="J191" s="2" t="inlineStr" /><c r="K191" s="2" t="inlineStr" /><c r="L191" s="2" t="inlineStr" /><c r="M191" s="2" t="inlineStr" /><c r="N191" s="2" t="inlineStr" /><c r="O191" s="2" t="inlineStr" /><c r="P191" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q191" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="192"><c r="A192" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B192" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C192" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D192" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E192" s="2" t="inlineStr"><is><t>Izoniazyd:</t></is></c><c r="F192" s="2" t="inlineStr"><is><t>działa bakteriobójczo na prątki szybko namnażające się</t></is></c><c r="G192" s="2" t="inlineStr" /><c r="H192" s="2" t="inlineStr" /><c r="I192" s="2" t="inlineStr" /><c r="J192" s="2" t="inlineStr" /><c r="K192" s="2" t="inlineStr"><is><t>nie powinien być stosowany przez kobiety w ciąży</t></is></c><c r="L192" s="2" t="inlineStr"><is><t>nie jest stosowany w leczeniu gruźlicy pozapłucnej</t></is></c><c r="M192" s="2" t="inlineStr"><is><t>może spowodować neuropatię obwodową</t></is></c><c r="N192" s="2" t="inlineStr" /><c r="O192" s="2" t="inlineStr" /><c r="P192" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q192" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="193"><c r="A193" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B193" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C193" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D193" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E193" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-działanie niepożądne:</t></is></c><c r="F193" s="2" t="inlineStr"><is><t>zolpidem – niepamięć następcza</t></is></c><c r="G193" s="2" t="inlineStr"><is><t>rotygotyna – nudności i wymioty</t></is></c><c r="H193" s="2" t="inlineStr"><is><t>alprazolam - senność</t></is></c><c r="I193" s="2" t="inlineStr"><is><t>fluoksetyna – zaburzenia libido i funkcji seksualnych</t></is></c><c r="J193" s="2" t="inlineStr" /><c r="K193" s="2" t="inlineStr" /><c r="L193" s="2" t="inlineStr" /><c r="M193" s="2" t="inlineStr" /><c r="N193" s="2" t="inlineStr" /><c r="O193" s="2" t="inlineStr" /><c r="P193" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q193" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="194"><c r="A194" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B194" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C194" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D194" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E194" s="2" t="inlineStr"><is><t>Do leczenia zaburzeń psychotycznych z nasilonymi objawami negatywnymi należy wybrać:</t></is></c><c r="F194" s="2" t="inlineStr"><is><t>amisulpiryd</t></is></c><c r="G194" s="2" t="inlineStr"><is><t>olanzapinę</t></is></c><c r="H194" s="2" t="inlineStr" /><c r="I194" s="2" t="inlineStr" /><c r="J194" s="2" t="inlineStr" /><c r="K194" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="L194" s="2" t="inlineStr"><is><t>chlorpromazynę</t></is></c><c r="M194" s="2" t="inlineStr" /><c r="N194" s="2" t="inlineStr" /><c r="O194" s="2" t="inlineStr" /><c r="P194" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q194" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="195"><c r="A195" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B195" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C195" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D195" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E195" s="2" t="inlineStr"><is><t>Działanie przeciwwymiotne metoklopramidu wynika z blokady receptorów:</t></is></c><c r="F195" s="2" t="inlineStr"><is><t>dopaminowych (D2)</t></is></c><c r="G195" s="2" t="inlineStr"><is><t>serotoninowych (5-HT3)</t></is></c><c r="H195" s="2" t="inlineStr" /><c r="I195" s="2" t="inlineStr" /><c r="J195" s="2" t="inlineStr" /><c r="K195" s="2" t="inlineStr"><is><t>neurokininowych (NK1)</t></is></c><c r="L195" s="2" t="inlineStr"><is><t>kannabinoidowych (CB1)</t></is></c><c r="M195" s="2" t="inlineStr" /><c r="N195" s="2" t="inlineStr" /><c r="O195" s="2" t="inlineStr" /><c r="P195" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q195" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="196"><c r="A196" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B196" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C196" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D196" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E196" s="2" t="inlineStr"><is><t>Rozszerzenie źrenic, suchość w ustach, osłabienie lub porażenie perystaltyki jelit obserwowane jest w przebiegu zatrucia:</t></is></c><c r="F196" s="2" t="inlineStr"><is><t>amitryptyliną</t></is></c><c r="G196" s="2" t="inlineStr" /><c r="H196" s="2" t="inlineStr" /><c r="I196" s="2" t="inlineStr" /><c r="J196" s="2" t="inlineStr" /><c r="K196" s="2" t="inlineStr"><is><t>escitalopramem</t></is></c><c r="L196" s="2" t="inlineStr"><is><t>pestycydami fosforoorganicznymi</t></is></c><c r="M196" s="2" t="inlineStr"><is><t>glikozydami naparstnicy</t></is></c><c r="N196" s="2" t="inlineStr" /><c r="O196" s="2" t="inlineStr" /><c r="P196" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q196" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="197"><c r="A197" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B197" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C197" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D197" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E197" s="2" t="inlineStr"><is><t>U 70-letniego mężczyzny z przewlekłą niewydolnością żylną wspomagająco do kompresjoterapii należy zastosować:</t></is></c><c r="F197" s="2" t="inlineStr"><is><t>mikronizowaną diosminę + hesperydynę</t></is></c><c r="G197" s="2" t="inlineStr" /><c r="H197" s="2" t="inlineStr" /><c r="I197" s="2" t="inlineStr" /><c r="J197" s="2" t="inlineStr" /><c r="K197" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy w dawce antyagregacyjnej</t></is></c><c r="L197" s="2" t="inlineStr"><is><t>enoksaparynę w dawce profilaktycznej</t></is></c><c r="M197" s="2" t="inlineStr"><is><t>furosemid w dawce leczniczej</t></is></c><c r="N197" s="2" t="inlineStr" /><c r="O197" s="2" t="inlineStr" /><c r="P197" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q197" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="198"><c r="A198" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B198" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C198" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D198" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E198" s="2" t="inlineStr"><is><t>Nie powinno się zwalniać pasażu jelitowego w przebiegu:</t></is></c><c r="F198" s="2" t="inlineStr"><is><t>zatrucia z objawami ogólnymi</t></is></c><c r="G198" s="2" t="inlineStr"><is><t>biegunki z krwią w stolcu i gorączką</t></is></c><c r="H198" s="2" t="inlineStr"><is><t>ostrej biegunki o niewielkim nasileniu</t></is></c><c r="I198" s="2" t="inlineStr" /><c r="J198" s="2" t="inlineStr" /><c r="K198" s="2" t="inlineStr"><is><t>przewlekłej biegunki związanej z chorobą zapalną jelit</t></is></c><c r="L198" s="2" t="inlineStr" /><c r="M198" s="2" t="inlineStr" /><c r="N198" s="2" t="inlineStr" /><c r="O198" s="2" t="inlineStr" /><c r="P198" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q198" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="199"><c r="A199" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B199" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C199" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D199" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E199" s="2" t="inlineStr"><is><t>Związki bizmutu:</t></is></c><c r="F199" s="2" t="inlineStr"><is><t>tworzą nierozpuszczalne kompleksy z białkami wysiękowymi na powierzchni owrzodzenia, działając osłaniająco wobec kwasu solnego i pepsyny na uszkodzoną błonę śluzową żołądka i dwunastnicy</t></is></c><c r="G199" s="2" t="inlineStr"><is><t>wchłaniają się z przewodu pokarmowego</t></is></c><c r="H199" s="2" t="inlineStr"><is><t>bezpośrednio niszczą komórki Helicobacter pylori</t></is></c><c r="I199" s="2" t="inlineStr"><is><t>mogą spowodować czarne zabarwienie języka i kału</t></is></c><c r="J199" s="2" t="inlineStr" /><c r="K199" s="2" t="inlineStr" /><c r="L199" s="2" t="inlineStr" /><c r="M199" s="2" t="inlineStr" /><c r="N199" s="2" t="inlineStr" /><c r="O199" s="2" t="inlineStr" /><c r="P199" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q199" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="200"><c r="A200" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B200" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C200" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D200" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E200" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek – wskazanie - dawka:</t></is></c><c r="F200" s="2" t="inlineStr"><is><t>dobutamina – diagnostyka niedokrwienia mięśnia serca –wlew 2-20 mcg/kg m.c./min</t></is></c><c r="G200" s="2" t="inlineStr"><is><t>adrenalina – resuscytacja krążeniowo-oddechowa– w dawkach frakcjonowanych i.v. po 1 mg w rozcieńczeniu w 10 ml 0,9% NaCl</t></is></c><c r="H200" s="2" t="inlineStr" /><c r="I200" s="2" t="inlineStr" /><c r="J200" s="2" t="inlineStr" /><c r="K200" s="2" t="inlineStr"><is><t>noradrenalina – ciężka hipotonia – wlew 2-10 mcg/kg m.c./min</t></is></c><c r="L200" s="2" t="inlineStr"><is><t>dopamina – ostra niewydolność mięśnia sercowego – wlew 1-3 mcg/kg m.c./min</t></is></c><c r="M200" s="2" t="inlineStr" /><c r="N200" s="2" t="inlineStr" /><c r="O200" s="2" t="inlineStr" /><c r="P200" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q200" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="201"><c r="A201" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B201" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C201" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D201" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E201" s="2" t="inlineStr"><is><t>Skala HAS-BLED określa ryzyko krwawienia u osób z migotaniem przedsionków stosujących leczenie przeciwkrzepliwe na podstawie oceny:</t></is></c><c r="F201" s="2" t="inlineStr"><is><t>wartości skurczowego ciśnienia tętniczego</t></is></c><c r="G201" s="2" t="inlineStr"><is><t>czynności wątroby</t></is></c><c r="H201" s="2" t="inlineStr"><is><t>stężenia kreatyniny</t></is></c><c r="I201" s="2" t="inlineStr" /><c r="J201" s="2" t="inlineStr" /><c r="K201" s="2" t="inlineStr"><is><t>glikemii</t></is></c><c r="L201" s="2" t="inlineStr" /><c r="M201" s="2" t="inlineStr" /><c r="N201" s="2" t="inlineStr" /><c r="O201" s="2" t="inlineStr" /><c r="P201" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q201" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="202"><c r="A202" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B202" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C202" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D202" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E202" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie substancja uzależniająca - lek stosowany w terapii uzależnienia:</t></is></c><c r="F202" s="2" t="inlineStr"><is><t>heroina - metadon</t></is></c><c r="G202" s="2" t="inlineStr"><is><t>nikotyna – wareniklina</t></is></c><c r="H202" s="2" t="inlineStr"><is><t>alkohol - nalmefen</t></is></c><c r="I202" s="2" t="inlineStr" /><c r="J202" s="2" t="inlineStr" /><c r="K202" s="2" t="inlineStr"><is><t>amfetamina - deferoksamina</t></is></c><c r="L202" s="2" t="inlineStr" /><c r="M202" s="2" t="inlineStr" /><c r="N202" s="2" t="inlineStr" /><c r="O202" s="2" t="inlineStr" /><c r="P202" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q202" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="203"><c r="A203" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B203" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C203" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D203" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E203" s="2" t="inlineStr"><is><t>Peptydy natriuretyczne zwiększają:</t></is></c><c r="F203" s="2" t="inlineStr"><is><t>filtrację kłębuszkową</t></is></c><c r="G203" s="2" t="inlineStr" /><c r="H203" s="2" t="inlineStr" /><c r="I203" s="2" t="inlineStr" /><c r="J203" s="2" t="inlineStr" /><c r="K203" s="2" t="inlineStr"><is><t>wydzielanie aldosteronu</t></is></c><c r="L203" s="2" t="inlineStr"><is><t>glikemię</t></is></c><c r="M203" s="2" t="inlineStr"><is><t>aktywność układu współczulnego</t></is></c><c r="N203" s="2" t="inlineStr" /><c r="O203" s="2" t="inlineStr" /><c r="P203" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q203" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="204"><c r="A204" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B204" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C204" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D204" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E204" s="2" t="inlineStr"><is><t>Pacjent z objawową bradykardią = 35 uderzeń/min jest leczony poniższym zestawem leków. Który z nich należy niezwłocznie odstawić?</t></is></c><c r="F204" s="2" t="inlineStr"><is><t>digoksynę</t></is></c><c r="G204" s="2" t="inlineStr"><is><t>amiodaron</t></is></c><c r="H204" s="2" t="inlineStr"><is><t>betaksolol</t></is></c><c r="I204" s="2" t="inlineStr" /><c r="J204" s="2" t="inlineStr" /><c r="K204" s="2" t="inlineStr"><is><t>losartan</t></is></c><c r="L204" s="2" t="inlineStr" /><c r="M204" s="2" t="inlineStr" /><c r="N204" s="2" t="inlineStr" /><c r="O204" s="2" t="inlineStr" /><c r="P204" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q204" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="205"><c r="A205" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B205" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C205" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D205" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E205" s="2" t="inlineStr"><is><t>Pacjent z objawową bradykardią = 35 uderzeń/min jest leczony poniższym zestawem leków. Który z nich należy niezwłocznie odstawić?</t></is></c><c r="F205" s="2" t="inlineStr"><is><t>digoksyna</t></is></c><c r="G205" s="2" t="inlineStr"><is><t>amiodaron</t></is></c><c r="H205" s="2" t="inlineStr"><is><t>betaksolol</t></is></c><c r="I205" s="2" t="inlineStr" /><c r="J205" s="2" t="inlineStr" /><c r="K205" s="2" t="inlineStr"><is><t>losartan</t></is></c><c r="L205" s="2" t="inlineStr" /><c r="M205" s="2" t="inlineStr" /><c r="N205" s="2" t="inlineStr" /><c r="O205" s="2" t="inlineStr" /><c r="P205" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q205" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="206"><c r="A206" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B206" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C206" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D206" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E206" s="2" t="inlineStr"><is><t>Irbesartan zwiększa w osoczu stężenie:</t></is></c><c r="F206" s="2" t="inlineStr"><is><t>reniny</t></is></c><c r="G206" s="2" t="inlineStr"><is><t>potasu</t></is></c><c r="H206" s="2" t="inlineStr" /><c r="I206" s="2" t="inlineStr" /><c r="J206" s="2" t="inlineStr" /><c r="K206" s="2" t="inlineStr"><is><t>bradykininy</t></is></c><c r="L206" s="2" t="inlineStr"><is><t>aldosteronu</t></is></c><c r="M206" s="2" t="inlineStr" /><c r="N206" s="2" t="inlineStr" /><c r="O206" s="2" t="inlineStr" /><c r="P206" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q206" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="207"><c r="A207" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B207" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C207" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D207" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E207" s="2" t="inlineStr"><is><t>70-letnia kobieta od miesiąca po wypisie ze szpitala otrzymuje kwas acetylosalicylowy + klopidogrel. Na tej podstawie można sądzić, że przebyła:</t></is></c><c r="F207" s="2" t="inlineStr"><is><t>angioplastykę wieńcową z wszczepieniem stentu</t></is></c><c r="G207" s="2" t="inlineStr"><is><t>zawał serca</t></is></c><c r="H207" s="2" t="inlineStr" /><c r="I207" s="2" t="inlineStr" /><c r="J207" s="2" t="inlineStr" /><c r="K207" s="2" t="inlineStr"><is><t>udar niedokrwienny mózgu</t></is></c><c r="L207" s="2" t="inlineStr"><is><t>zatorowość płucną niewysokiego ryzyka</t></is></c><c r="M207" s="2" t="inlineStr" /><c r="N207" s="2" t="inlineStr" /><c r="O207" s="2" t="inlineStr" /><c r="P207" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q207" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="208"><c r="A208" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B208" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C208" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D208" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E208" s="2" t="inlineStr"><is><t>59-letni mężczyzna z pozawałową niewydolnością serca (EF ok. 30%), z implantowanym ICD (kardiowerterem defibrylatorem) w prewencji pierwotnej NZK, z eGFR = 95%, z bólami pleców na skutek wielopoziomowej dyskopatii jest leczony: ramiprylem, karwedilolem, eplerenonem, indapamidem, preparatami chlorku potasu, magnezu z witaminą B6 i węglanu wapnia oraz paracetamolem i ketoprofenem. Które stwierdzenie jest prawdziwe?</t></is></c><c r="F208" s="2" t="inlineStr"><is><t>opisana terapia stwarza zagrożenie hiperkaliemią, co trzeba monitorować</t></is></c><c r="G208" s="2" t="inlineStr"><is><t>należy odstawić ketoprofen, bo może on osłabiać działanie leków w niewydolności serca</t></is></c><c r="H208" s="2" t="inlineStr" /><c r="I208" s="2" t="inlineStr" /><c r="J208" s="2" t="inlineStr" /><c r="K208" s="2" t="inlineStr"><is><t>ze względu na lepszą kontrolę choroby zamiast ramiprylu należy podać walsartan</t></is></c><c r="L208" s="2" t="inlineStr"><is><t>indapamid jako lek potencjalnie nieskuteczny powinien zostać zastąpiony torasemidem</t></is></c><c r="M208" s="2" t="inlineStr" /><c r="N208" s="2" t="inlineStr" /><c r="O208" s="2" t="inlineStr" /><c r="P208" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q208" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="209"><c r="A209" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B209" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C209" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D209" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E209" s="2" t="inlineStr"><is><t>Wartości ciśnienia tętniczego może zwiększyć stosowanie:</t></is></c><c r="F209" s="2" t="inlineStr"><is><t>piroksykamu</t></is></c><c r="G209" s="2" t="inlineStr"><is><t>prednizonu</t></is></c><c r="H209" s="2" t="inlineStr" /><c r="I209" s="2" t="inlineStr" /><c r="J209" s="2" t="inlineStr" /><c r="K209" s="2" t="inlineStr"><is><t>eplerenonu</t></is></c><c r="L209" s="2" t="inlineStr"><is><t>morfiny</t></is></c><c r="M209" s="2" t="inlineStr" /><c r="N209" s="2" t="inlineStr" /><c r="O209" s="2" t="inlineStr" /><c r="P209" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q209" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="210"><c r="A210" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B210" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C210" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D210" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E210" s="2" t="inlineStr"><is><t>Kwas ibandronowy:</t></is></c><c r="F210" s="2" t="inlineStr"><is><t>z dużym powinowactwem wiąże się ze zmineralizowaną kością</t></is></c><c r="G210" s="2" t="inlineStr"><is><t>zmniejsza ryzyko złamania kręgów kręgosłupa u kobiet po menopauzie</t></is></c><c r="H210" s="2" t="inlineStr"><is><t>hamuje aktywację osteoklastów</t></is></c><c r="I210" s="2" t="inlineStr"><is><t>może spowodować martwicę szczęki</t></is></c><c r="J210" s="2" t="inlineStr" /><c r="K210" s="2" t="inlineStr" /><c r="L210" s="2" t="inlineStr" /><c r="M210" s="2" t="inlineStr" /><c r="N210" s="2" t="inlineStr" /><c r="O210" s="2" t="inlineStr" /><c r="P210" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q210" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="211"><c r="A211" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B211" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C211" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D211" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E211" s="2" t="inlineStr"><is><t>Dodatkowe zmniejszenie stężenia cholesterolu LDL w surowicy można osiągnąć przez dodanie do statyn:</t></is></c><c r="F211" s="2" t="inlineStr"><is><t>kolesewelamu</t></is></c><c r="G211" s="2" t="inlineStr"><is><t>ewolokumabu</t></is></c><c r="H211" s="2" t="inlineStr"><is><t>ezetymibu</t></is></c><c r="I211" s="2" t="inlineStr" /><c r="J211" s="2" t="inlineStr" /><c r="K211" s="2" t="inlineStr"><is><t>PUFA – wielonienasyconych kwasów tłuszczowych</t></is></c><c r="L211" s="2" t="inlineStr" /><c r="M211" s="2" t="inlineStr" /><c r="N211" s="2" t="inlineStr" /><c r="O211" s="2" t="inlineStr" /><c r="P211" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q211" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="212"><c r="A212" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B212" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C212" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D212" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E212" s="2" t="inlineStr"><is><t>Które stwierdzenie jest prawdziwe:</t></is></c><c r="F212" s="2" t="inlineStr"><is><t>cilostazol wydłuża dystans marszu bez bólu u pacjentów z chromaniem przestankowym</t></is></c><c r="G212" s="2" t="inlineStr"><is><t>stosowanie serelaksyny może przynieść korzyści pacjentom z ostrą niewydolnością mięśnia sercowego</t></is></c><c r="H212" s="2" t="inlineStr"><is><t>do działań niepożądanych milrynonu należą zaburzenia rytmu serca</t></is></c><c r="I212" s="2" t="inlineStr" /><c r="J212" s="2" t="inlineStr" /><c r="K212" s="2" t="inlineStr"><is><t>inhibitory fosfodiesterazy 5 mogą być podane łącznie z azotanami</t></is></c><c r="L212" s="2" t="inlineStr" /><c r="M212" s="2" t="inlineStr" /><c r="N212" s="2" t="inlineStr" /><c r="O212" s="2" t="inlineStr" /><c r="P212" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q212" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="213"><c r="A213" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B213" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C213" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D213" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E213" s="2" t="inlineStr"><is><t>Które stwierdzenie jest prawdziwe:</t></is></c><c r="F213" s="2" t="inlineStr"><is><t>propafenon nie jest zalecany u pacjentów z chorobą wieńcową</t></is></c><c r="G213" s="2" t="inlineStr"><is><t>amiodaron można stosować w celu zwiększenia skuteczności kardiowersji elektrycznej</t></is></c><c r="H213" s="2" t="inlineStr" /><c r="I213" s="2" t="inlineStr" /><c r="J213" s="2" t="inlineStr" /><c r="K213" s="2" t="inlineStr"><is><t>dronedaron zmniejsza umieralność u pacjentów z niewydolnością serca w klasie III/IV NYHA</t></is></c><c r="L213" s="2" t="inlineStr"><is><t>beta-adrenolityki stosuje się w celu kardiowersji farmakologicznej</t></is></c><c r="M213" s="2" t="inlineStr" /><c r="N213" s="2" t="inlineStr" /><c r="O213" s="2" t="inlineStr" /><c r="P213" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q213" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="214"><c r="A214" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B214" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C214" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D214" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E214" s="2" t="inlineStr"><is><t>Które stwierdzenie jest prawdziwe?</t></is></c><c r="F214" s="2" t="inlineStr"><is><t>takrolimus i ewerolimus tworzą kompleks z immunofiliną FKBP</t></is></c><c r="G214" s="2" t="inlineStr"><is><t>takrolimus i ewerolimus należą do leków o wąskim indeksie (wskaźniku) terapeutycznym</t></is></c><c r="H214" s="2" t="inlineStr" /><c r="I214" s="2" t="inlineStr" /><c r="J214" s="2" t="inlineStr" /><c r="K214" s="2" t="inlineStr"><is><t>takrolimus i ewerolimus mają ten sam mechanizm działania</t></is></c><c r="L214" s="2" t="inlineStr"><is><t>takrolimus i ewerolimus działają przeciwnowotorowo</t></is></c><c r="M214" s="2" t="inlineStr" /><c r="N214" s="2" t="inlineStr" /><c r="O214" s="2" t="inlineStr" /><c r="P214" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q214" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="215"><c r="A215" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B215" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C215" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D215" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E215" s="2" t="inlineStr"><is><t>Które stwierdzenie jest prawdziwe:</t></is></c><c r="F215" s="2" t="inlineStr"><is><t>dyfuzja bierna to główny mechanizm transportu leków przez błony półprzepuszczalne</t></is></c><c r="G215" s="2" t="inlineStr"><is><t>P-glikoproteina (P-gp) usuwa leki z komórki do środowiska pozakomórkowego w sposób zależny od ATP</t></is></c><c r="H215" s="2" t="inlineStr"><is><t>CYP3A4 jest głównym izoenzymem uczestniczącym w metabolizmie 1 fazy leków</t></is></c><c r="I215" s="2" t="inlineStr" /><c r="J215" s="2" t="inlineStr" /><c r="K215" s="2" t="inlineStr"><is><t>istotne klinicznie jest wiązanie leku z białkami transportującymi we krwi ≥ 60%</t></is></c><c r="L215" s="2" t="inlineStr" /><c r="M215" s="2" t="inlineStr" /><c r="N215" s="2" t="inlineStr" /><c r="O215" s="2" t="inlineStr" /><c r="P215" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q215" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="216"><c r="A216" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B216" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C216" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D216" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E216" s="2" t="inlineStr"><is><t>Fibraty (pochodne kwasu fibrynowego):</t></is></c><c r="F216" s="2" t="inlineStr"><is><t>hamują uwalnianie frakcji lipidowej VLDL z wątroby</t></is></c><c r="G216" s="2" t="inlineStr"><is><t>nasilają aktywność lipazy lipoproteinowej</t></is></c><c r="H216" s="2" t="inlineStr" /><c r="I216" s="2" t="inlineStr" /><c r="J216" s="2" t="inlineStr" /><c r="K216" s="2" t="inlineStr"><is><t>hamują wchłanianie tłuszczów złożonych z przewodu pokarmowego</t></is></c><c r="L216" s="2" t="inlineStr"><is><t>zmniejszają stężenie frakcji HDL poprzez spadek syntezy Apo-A1 i Apo-AII</t></is></c><c r="M216" s="2" t="inlineStr" /><c r="N216" s="2" t="inlineStr" /><c r="O216" s="2" t="inlineStr" /><c r="P216" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q216" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="217"><c r="A217" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B217" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C217" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D217" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E217" s="2" t="inlineStr"><is><t>U chorych ze zdekompensowaną obukomorową niewydolnością serca:</t></is></c><c r="F217" s="2" t="inlineStr"><is><t>znacznie opóźnione jest wchłanianie leków z przewodu pokarmowego</t></is></c><c r="G217" s="2" t="inlineStr"><is><t>leki hydrofilne dystrybuują się do płynu obrzękowego, co dodatkowo negatywnie wpływa na ich dystrybucję do narządów docelowych</t></is></c><c r="H217" s="2" t="inlineStr"><is><t>zmniejsza się klirens wątrobowy wszystkich leków metabolizowanych w wątrobie niezależnie od stopnia ich ekstrakcji wątrobowej</t></is></c><c r="I217" s="2" t="inlineStr" /><c r="J217" s="2" t="inlineStr" /><c r="K217" s="2" t="inlineStr"><is><t>stosunkowo mało zmniejsza się klirens nerkowy leków</t></is></c><c r="L217" s="2" t="inlineStr" /><c r="M217" s="2" t="inlineStr" /><c r="N217" s="2" t="inlineStr" /><c r="O217" s="2" t="inlineStr" /><c r="P217" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q217" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="218"><c r="A218" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B218" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C218" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D218" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E218" s="2" t="inlineStr"><is><t>Interakcją farmakodynamiczną jest:</t></is></c><c r="F218" s="2" t="inlineStr"><is><t>nasilenie depresji OUN po skojarzeniu opioidów z etanolem</t></is></c><c r="G218" s="2" t="inlineStr" /><c r="H218" s="2" t="inlineStr" /><c r="I218" s="2" t="inlineStr" /><c r="J218" s="2" t="inlineStr" /><c r="K218" s="2" t="inlineStr"><is><t>hamowanie wchłaniania z przewodu pokarmowego leków podawanych jednocześnie</t></is></c><c r="L218" s="2" t="inlineStr"><is><t>wytrącenie się osadu po zmieszaniu dwóch leków w jednym roztworze do wstrzyknięcia</t></is></c><c r="M218" s="2" t="inlineStr"><is><t>zwiększenie metabolizmu leków podawanych jednocześnie</t></is></c><c r="N218" s="2" t="inlineStr" /><c r="O218" s="2" t="inlineStr" /><c r="P218" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q218" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="219"><c r="A219" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B219" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C219" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D219" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E219" s="2" t="inlineStr"><is><t>Kwasicę metaboliczną mogą powodować:</t></is></c><c r="F219" s="2" t="inlineStr"><is><t>metformina</t></is></c><c r="G219" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="H219" s="2" t="inlineStr" /><c r="I219" s="2" t="inlineStr" /><c r="J219" s="2" t="inlineStr" /><c r="K219" s="2" t="inlineStr"><is><t>diuretyki pętlowe</t></is></c><c r="L219" s="2" t="inlineStr"><is><t>etanol</t></is></c><c r="M219" s="2" t="inlineStr" /><c r="N219" s="2" t="inlineStr" /><c r="O219" s="2" t="inlineStr" /><c r="P219" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q219" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="220"><c r="A220" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B220" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C220" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D220" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E220" s="2" t="inlineStr"><is><t>Klindamycyna:</t></is></c><c r="F220" s="2" t="inlineStr"><is><t>jest aktywna wobec beztlenowców</t></is></c><c r="G220" s="2" t="inlineStr" /><c r="H220" s="2" t="inlineStr" /><c r="I220" s="2" t="inlineStr" /><c r="J220" s="2" t="inlineStr" /><c r="K220" s="2" t="inlineStr"><is><t>dobrze przenika do płynu mózgowo-rdzeniowego</t></is></c><c r="L220" s="2" t="inlineStr"><is><t>słabo selekcjonuje szczepy Clostridium difficile w jelicie</t></is></c><c r="M220" s="2" t="inlineStr"><is><t>stosowana jest jako lek z wyboru w nierzeżączkowym zapaleniu cewki moczowej</t></is></c><c r="N220" s="2" t="inlineStr" /><c r="O220" s="2" t="inlineStr" /><c r="P220" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q220" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="221"><c r="A221" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B221" s="2" t="inlineStr"><is><t>Struktura chemiczna</t></is></c><c r="C221" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D221" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E221" s="2" t="inlineStr"><is><t>Pierścień beta-laktamowy znajduje się w cząsteczce:</t></is></c><c r="F221" s="2" t="inlineStr"><is><t>kloksacyliny</t></is></c><c r="G221" s="2" t="inlineStr"><is><t>ceftazydymu</t></is></c><c r="H221" s="2" t="inlineStr"><is><t>meropenemu</t></is></c><c r="I221" s="2" t="inlineStr" /><c r="J221" s="2" t="inlineStr" /><c r="K221" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="L221" s="2" t="inlineStr" /><c r="M221" s="2" t="inlineStr" /><c r="N221" s="2" t="inlineStr" /><c r="O221" s="2" t="inlineStr" /><c r="P221" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q221" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="222"><c r="A222" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B222" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C222" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D222" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E222" s="2" t="inlineStr"><is><t>W celu zwiększenia bezpieczeństwa leczenia amikacyną mężczyzny z powikłanym zakażeniem układu moczowego należy:</t></is></c><c r="F222" s="2" t="inlineStr"><is><t>podawać dawkę dobową w pojedynczym wlewie dożylnym</t></is></c><c r="G222" s="2" t="inlineStr"><is><t>monitorować okresowo stężenie antybiotyku we krwi przed podaniem kolejnej dawki leku</t></is></c><c r="H222" s="2" t="inlineStr"><is><t>monitorować stężenie kreatyniny w surowicy</t></is></c><c r="I222" s="2" t="inlineStr" /><c r="J222" s="2" t="inlineStr" /><c r="K222" s="2" t="inlineStr"><is><t>kontrolować co kilka dni stężenie TSH w surowicy</t></is></c><c r="L222" s="2" t="inlineStr" /><c r="M222" s="2" t="inlineStr" /><c r="N222" s="2" t="inlineStr" /><c r="O222" s="2" t="inlineStr" /><c r="P222" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q222" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="223"><c r="A223" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B223" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C223" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D223" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E223" s="2" t="inlineStr"><is><t>W leczeniu pacjentki z niepowikłanym zapaleniem pęcherza moczowego można zastosować:</t></is></c><c r="F223" s="2" t="inlineStr"><is><t>amoksycylinę z inhibitorem beta-laktamazy</t></is></c><c r="G223" s="2" t="inlineStr"><is><t>fosfomycynę</t></is></c><c r="H223" s="2" t="inlineStr"><is><t>cyprofloksacynę</t></is></c><c r="I223" s="2" t="inlineStr"><is><t>furazydynę</t></is></c><c r="J223" s="2" t="inlineStr" /><c r="K223" s="2" t="inlineStr" /><c r="L223" s="2" t="inlineStr" /><c r="M223" s="2" t="inlineStr" /><c r="N223" s="2" t="inlineStr" /><c r="O223" s="2" t="inlineStr" /><c r="P223" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q223" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="224"><c r="A224" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B224" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C224" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D224" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E224" s="2" t="inlineStr"><is><t>Lekiem przeciwbakteryjnym o wąskim zakresie działania przeciwbakteryjnego jest:</t></is></c><c r="F224" s="2" t="inlineStr"><is><t>fenoksymetylopenicylina</t></is></c><c r="G224" s="2" t="inlineStr"><is><t>nystatyna</t></is></c><c r="H224" s="2" t="inlineStr" /><c r="I224" s="2" t="inlineStr" /><c r="J224" s="2" t="inlineStr" /><c r="K224" s="2" t="inlineStr"><is><t>aksetyl cefuroksymu</t></is></c><c r="L224" s="2" t="inlineStr"><is><t>chloramfenikol</t></is></c><c r="M224" s="2" t="inlineStr" /><c r="N224" s="2" t="inlineStr" /><c r="O224" s="2" t="inlineStr" /><c r="P224" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q224" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="225"><c r="A225" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B225" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C225" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D225" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E225" s="2" t="inlineStr"><is><t>Aktywność przeciwbakteryjną względem opornych na metycylinę szczepów Staphylococcus aureus (MRSA) ma:</t></is></c><c r="F225" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="G225" s="2" t="inlineStr"><is><t>mupirocyna</t></is></c><c r="H225" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="I225" s="2" t="inlineStr"><is><t>dalfoprystyna/chinuprystyna</t></is></c><c r="J225" s="2" t="inlineStr" /><c r="K225" s="2" t="inlineStr" /><c r="L225" s="2" t="inlineStr" /><c r="M225" s="2" t="inlineStr" /><c r="N225" s="2" t="inlineStr" /><c r="O225" s="2" t="inlineStr" /><c r="P225" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q225" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="226"><c r="A226" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B226" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C226" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D226" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E226" s="2" t="inlineStr"><is><t>Profilaktyka infekcyjnego zapalenia wsierdzia (IZW) jest wskazana u osób z grup wysokiego ryzyka IZW w przypadku procedur:</t></is></c><c r="F226" s="2" t="inlineStr"><is><t>dentystycznych z manipulacją w obrębie dziąseł lub okolicy około-wierzchołkowej zębów</t></is></c><c r="G226" s="2" t="inlineStr"><is><t>inwazyjnych w obrębie górnych dróg oddechowych, tj. usunięcie migdałka</t></is></c><c r="H226" s="2" t="inlineStr" /><c r="I226" s="2" t="inlineStr" /><c r="J226" s="2" t="inlineStr" /><c r="K226" s="2" t="inlineStr"><is><t>inwazyjnych w obrębie układu moczowo-płciowego</t></is></c><c r="L226" s="2" t="inlineStr"><is><t>inwazyjnych w obrębie przewodu pokarmowego</t></is></c><c r="M226" s="2" t="inlineStr" /><c r="N226" s="2" t="inlineStr" /><c r="O226" s="2" t="inlineStr" /><c r="P226" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q226" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="227"><c r="A227" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B227" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C227" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D227" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E227" s="2" t="inlineStr"><is><t>Gancyklowir:</t></is></c><c r="F227" s="2" t="inlineStr"><is><t>może powodować uszkodzenie szpiku</t></is></c><c r="G227" s="2" t="inlineStr" /><c r="H227" s="2" t="inlineStr" /><c r="I227" s="2" t="inlineStr" /><c r="J227" s="2" t="inlineStr" /><c r="K227" s="2" t="inlineStr"><is><t>jest inhibitorem proteazy wirusowej</t></is></c><c r="L227" s="2" t="inlineStr"><is><t>bezpośrednio hamuje uwalnianie wirusów z zakażonych komórek</t></is></c><c r="M227" s="2" t="inlineStr"><is><t>nie przenika do ośrodkowego układu nerwowego</t></is></c><c r="N227" s="2" t="inlineStr" /><c r="O227" s="2" t="inlineStr" /><c r="P227" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q227" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="228"><c r="A228" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B228" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C228" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D228" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E228" s="2" t="inlineStr"><is><t>W standardowej profilaktyce okołooperacyjnej wskazane jest stosowanie:</t></is></c><c r="F228" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="G228" s="2" t="inlineStr"><is><t>metronidazolu</t></is></c><c r="H228" s="2" t="inlineStr"><is><t>cyprofloksacyny</t></is></c><c r="I228" s="2" t="inlineStr"><is><t>cefazoliny</t></is></c><c r="J228" s="2" t="inlineStr" /><c r="K228" s="2" t="inlineStr" /><c r="L228" s="2" t="inlineStr" /><c r="M228" s="2" t="inlineStr" /><c r="N228" s="2" t="inlineStr" /><c r="O228" s="2" t="inlineStr" /><c r="P228" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q228" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="229"><c r="A229" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B229" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C229" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D229" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E229" s="2" t="inlineStr"><is><t>W grzybiczym zakażeniu skóry gładkiej można zastosować miejscowo:</t></is></c><c r="F229" s="2" t="inlineStr"><is><t>cyklopiroksolaminę</t></is></c><c r="G229" s="2" t="inlineStr"><is><t>natamycynę</t></is></c><c r="H229" s="2" t="inlineStr"><is><t>klotrimazol</t></is></c><c r="I229" s="2" t="inlineStr" /><c r="J229" s="2" t="inlineStr" /><c r="K229" s="2" t="inlineStr"><is><t>kaspofunginę</t></is></c><c r="L229" s="2" t="inlineStr" /><c r="M229" s="2" t="inlineStr" /><c r="N229" s="2" t="inlineStr" /><c r="O229" s="2" t="inlineStr" /><c r="P229" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q229" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="230"><c r="A230" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B230" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C230" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D230" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E230" s="2" t="inlineStr"><is><t>Wskaż poprawną strategię postępowania w zakresie leczenia zakażeń:</t></is></c><c r="F230" s="2" t="inlineStr"><is><t>leczenie empiryczne powinno uwzględniać miejsce powstania zakażenia: domowe lub związane z kontaktem ze służbą zdrowia</t></is></c><c r="G230" s="2" t="inlineStr"><is><t>na podstawie antybiogramu należy dokonać deeskalacji leczenia</t></is></c><c r="H230" s="2" t="inlineStr"><is><t>zasadą jest doustne leczenie przeciwinfekcyjne poza uzasadnionymi wyjątkami poza dekolonizacją MRSA przed operacjami</t></is></c><c r="I230" s="2" t="inlineStr" /><c r="J230" s="2" t="inlineStr" /><c r="K230" s="2" t="inlineStr" /><c r="L230" s="2" t="inlineStr" /><c r="M230" s="2" t="inlineStr" /><c r="N230" s="2" t="inlineStr" /><c r="O230" s="2" t="inlineStr" /><c r="P230" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q230" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="231"><c r="A231" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B231" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C231" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D231" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E231" s="2" t="inlineStr"><is><t>W Polsce granica opłacalności procedur medycznych jest:</t></is></c><c r="F231" s="2" t="inlineStr"><is><t>wykorzystywanym i usankcjonowanym prawnie kryterium refundacyjnym</t></is></c><c r="G231" s="2" t="inlineStr"><is><t>ustalona w oparciu o roczny koszt dializoterapii – przewlekłej, powszechnej i jednej z najdroższych procedur medycznych</t></is></c><c r="H231" s="2" t="inlineStr"><is><t>ustalona w oparciu o 3 krotność produktu krajowego brutto per capita</t></is></c><c r="I231" s="2" t="inlineStr"><is><t>odmienna dla leków stosowanych w chorobach onkologicznych</t></is></c><c r="J231" s="2" t="inlineStr" /><c r="K231" s="2" t="inlineStr" /><c r="L231" s="2" t="inlineStr" /><c r="M231" s="2" t="inlineStr" /><c r="N231" s="2" t="inlineStr" /><c r="O231" s="2" t="inlineStr" /><c r="P231" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q231" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="232"><c r="A232" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B232" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C232" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D232" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E232" s="2" t="inlineStr"><is><t>W leczeniu trądziku młodzieńczego racjonalne jest zastosowanie:</t></is></c><c r="F232" s="2" t="inlineStr"><is><t>klindamycyny</t></is></c><c r="G232" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="H232" s="2" t="inlineStr"><is><t>izotretinoiny</t></is></c><c r="I232" s="2" t="inlineStr" /><c r="J232" s="2" t="inlineStr" /><c r="K232" s="2" t="inlineStr"><is><t>norfloksacyny</t></is></c><c r="L232" s="2" t="inlineStr" /><c r="M232" s="2" t="inlineStr" /><c r="N232" s="2" t="inlineStr" /><c r="O232" s="2" t="inlineStr" /><c r="P232" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q232" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="233"><c r="A233" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B233" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C233" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D233" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E233" s="2" t="inlineStr"><is><t>Istotne genetycznie uwarunkowane różnice działania stwierdzono dla:</t></is></c><c r="F233" s="2" t="inlineStr"><is><t>abakawiru</t></is></c><c r="G233" s="2" t="inlineStr"><is><t>karbamazepiny</t></is></c><c r="H233" s="2" t="inlineStr"><is><t>warfaryny</t></is></c><c r="I233" s="2" t="inlineStr" /><c r="J233" s="2" t="inlineStr" /><c r="K233" s="2" t="inlineStr"><is><t>diltiazemu</t></is></c><c r="L233" s="2" t="inlineStr" /><c r="M233" s="2" t="inlineStr" /><c r="N233" s="2" t="inlineStr" /><c r="O233" s="2" t="inlineStr" /><c r="P233" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q233" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="234"><c r="A234" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B234" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C234" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D234" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E234" s="2" t="inlineStr"><is><t>Inhibitory dipeptydylopeptydazy IV (DPP IV):</t></is></c><c r="F234" s="2" t="inlineStr"><is><t>mogą być stosowane łącznie z insuliną</t></is></c><c r="G234" s="2" t="inlineStr"><is><t>zwiększają ryzyko wystąpienia dolegliwości ze strony przewodu pokarmowego</t></is></c><c r="H234" s="2" t="inlineStr" /><c r="I234" s="2" t="inlineStr" /><c r="J234" s="2" t="inlineStr" /><c r="K234" s="2" t="inlineStr"><is><t>powodują przyrost masy ciała</t></is></c><c r="L234" s="2" t="inlineStr"><is><t>są podawane podskórnie</t></is></c><c r="M234" s="2" t="inlineStr" /><c r="N234" s="2" t="inlineStr" /><c r="O234" s="2" t="inlineStr" /><c r="P234" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q234" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="235"><c r="A235" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B235" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C235" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D235" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E235" s="2" t="inlineStr"><is><t>Wskaż zdanie/zdania prawdziwe:</t></is></c><c r="F235" s="2" t="inlineStr"><is><t>empagliflozyna – zmniejsza ryzyko śmierci z przyczyn sercowo￾naczyniowych u chorych z cukrzycą typu 2</t></is></c><c r="G235" s="2" t="inlineStr"><is><t>metformina – zmniejsza ryzyko powikłań makroangiopatycznych</t></is></c><c r="H235" s="2" t="inlineStr" /><c r="I235" s="2" t="inlineStr" /><c r="J235" s="2" t="inlineStr" /><c r="K235" s="2" t="inlineStr"><is><t>sitagliptyna - pomimo euglikemii może spowodować kwasicę ketonową</t></is></c><c r="L235" s="2" t="inlineStr"><is><t>gliklazyd – powoduje redukcję masy ciała</t></is></c><c r="M235" s="2" t="inlineStr" /><c r="N235" s="2" t="inlineStr" /><c r="O235" s="2" t="inlineStr" /><c r="P235" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q235" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="236"><c r="A236" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B236" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C236" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D236" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E236" s="2" t="inlineStr"><is><t>Stosowanie tiamazolu może być przyczyną:</t></is></c><c r="F236" s="2" t="inlineStr"><is><t>żółtaczki cholestatycznej</t></is></c><c r="G236" s="2" t="inlineStr"><is><t>agranulocytozy</t></is></c><c r="H236" s="2" t="inlineStr"><is><t>wysypki skórnej</t></is></c><c r="I236" s="2" t="inlineStr"><is><t>niedoczynności tarczycy</t></is></c><c r="J236" s="2" t="inlineStr" /><c r="K236" s="2" t="inlineStr" /><c r="L236" s="2" t="inlineStr" /><c r="M236" s="2" t="inlineStr" /><c r="N236" s="2" t="inlineStr" /><c r="O236" s="2" t="inlineStr" /><c r="P236" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q236" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="237"><c r="A237" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B237" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C237" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D237" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E237" s="2" t="inlineStr"><is><t>Leczenie triamcynolonem może pogorszyć przebieg:</t></is></c><c r="F237" s="2" t="inlineStr"><is><t>jaskry</t></is></c><c r="G237" s="2" t="inlineStr"><is><t>zaburzeń nastroju</t></is></c><c r="H237" s="2" t="inlineStr"><is><t>zaćmy</t></is></c><c r="I237" s="2" t="inlineStr"><is><t>osteoporozy</t></is></c><c r="J237" s="2" t="inlineStr" /><c r="K237" s="2" t="inlineStr" /><c r="L237" s="2" t="inlineStr" /><c r="M237" s="2" t="inlineStr" /><c r="N237" s="2" t="inlineStr" /><c r="O237" s="2" t="inlineStr" /><c r="P237" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q237" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="238"><c r="A238" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B238" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C238" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D238" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E238" s="2" t="inlineStr"><is><t>Pacjent nieprzytomny, z hipoglikemią po spożyciu alkoholu, powinien otrzymać:</t></is></c><c r="F238" s="2" t="inlineStr"><is><t>20% roztwór glukozy i.v</t></is></c><c r="G238" s="2" t="inlineStr" /><c r="H238" s="2" t="inlineStr" /><c r="I238" s="2" t="inlineStr" /><c r="J238" s="2" t="inlineStr" /><c r="K238" s="2" t="inlineStr"><is><t>glukagon i.m</t></is></c><c r="L238" s="2" t="inlineStr"><is><t>glukozę p.o</t></is></c><c r="M238" s="2" t="inlineStr"><is><t>glukagon s.c</t></is></c><c r="N238" s="2" t="inlineStr" /><c r="O238" s="2" t="inlineStr" /><c r="P238" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q238" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="239"><c r="A239" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B239" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C239" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D239" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E239" s="2" t="inlineStr"><is><t>Potwierdzone klinicznie zmniejszenie ryzyka złamania kości udowej w przebiegu osteoporozy występuje w wyniku leczenia:</t></is></c><c r="F239" s="2" t="inlineStr"><is><t>ranelinianem strontu</t></is></c><c r="G239" s="2" t="inlineStr"><is><t>kwasem ibandronowy</t></is></c><c r="H239" s="2" t="inlineStr" /><c r="I239" s="2" t="inlineStr" /><c r="J239" s="2" t="inlineStr" /><c r="K239" s="2" t="inlineStr"><is><t>raloksyfenem</t></is></c><c r="L239" s="2" t="inlineStr"><is><t>kalcytoniną</t></is></c><c r="M239" s="2" t="inlineStr" /><c r="N239" s="2" t="inlineStr" /><c r="O239" s="2" t="inlineStr" /><c r="P239" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q239" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="240"><c r="A240" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B240" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C240" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D240" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E240" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie - wskazanie do stosowania glikokortykosteroidów - uzasadnienie zastosowania:</t></is></c><c r="F240" s="2" t="inlineStr"><is><t>poród przedwczesny – stymulowanie dojrzewania płuc płodu</t></is></c><c r="G240" s="2" t="inlineStr"><is><t>astma – ograniczenie procesu zapalnego</t></is></c><c r="H240" s="2" t="inlineStr"><is><t>przełom nadnerczowy – leczenie substytucyjne</t></is></c><c r="I240" s="2" t="inlineStr" /><c r="J240" s="2" t="inlineStr" /><c r="K240" s="2" t="inlineStr"><is><t>mononukleoza zakaźna – efekt immunosupresyjny</t></is></c><c r="L240" s="2" t="inlineStr" /><c r="M240" s="2" t="inlineStr" /><c r="N240" s="2" t="inlineStr" /><c r="O240" s="2" t="inlineStr" /><c r="P240" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q240" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="241"><c r="A241" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B241" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C241" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D241" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E241" s="2" t="inlineStr"><is><t>Do działań niepożądanych środków antykoncepcyjnych zalicza się:</t></is></c><c r="F241" s="2" t="inlineStr"><is><t>trądzik</t></is></c><c r="G241" s="2" t="inlineStr"><is><t>depresję</t></is></c><c r="H241" s="2" t="inlineStr"><is><t>zwiększenie ryzyka udaru mózgu</t></is></c><c r="I241" s="2" t="inlineStr" /><c r="J241" s="2" t="inlineStr" /><c r="K241" s="2" t="inlineStr"><is><t>zwiększenie ryzyka raka jajnika</t></is></c><c r="L241" s="2" t="inlineStr" /><c r="M241" s="2" t="inlineStr" /><c r="N241" s="2" t="inlineStr" /><c r="O241" s="2" t="inlineStr" /><c r="P241" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q241" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="242"><c r="A242" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B242" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C242" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D242" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E242" s="2" t="inlineStr"><is><t>Witamina D3 (cholekalcyferol):</t></is></c><c r="F242" s="2" t="inlineStr"><is><t>może być stosowana w niedoczynności przytarczyc</t></is></c><c r="G242" s="2" t="inlineStr"><is><t>w nadmiarze hamuje wzrost kości</t></is></c><c r="H242" s="2" t="inlineStr" /><c r="I242" s="2" t="inlineStr" /><c r="J242" s="2" t="inlineStr" /><c r="K242" s="2" t="inlineStr"><is><t>mimo stosowania w dużych dawkach nie chroni przed osteoporotycznymi złamaniami kości</t></is></c><c r="L242" s="2" t="inlineStr"><is><t>jest nieaktywna u chorych z niewydolnością nerek</t></is></c><c r="M242" s="2" t="inlineStr" /><c r="N242" s="2" t="inlineStr" /><c r="O242" s="2" t="inlineStr" /><c r="P242" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q242" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="243"><c r="A243" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B243" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C243" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D243" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E243" s="2" t="inlineStr"><is><t>Działanie przeczyszczające wykazuje:</t></is></c><c r="F243" s="2" t="inlineStr"><is><t>siarczan magnezu</t></is></c><c r="G243" s="2" t="inlineStr"><is><t>dokusan sodowy</t></is></c><c r="H243" s="2" t="inlineStr" /><c r="I243" s="2" t="inlineStr" /><c r="J243" s="2" t="inlineStr" /><c r="K243" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="L243" s="2" t="inlineStr"><is><t>racekadotryl</t></is></c><c r="M243" s="2" t="inlineStr" /><c r="N243" s="2" t="inlineStr" /><c r="O243" s="2" t="inlineStr" /><c r="P243" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q243" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="244"><c r="A244" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B244" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C244" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D244" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E244" s="2" t="inlineStr"><is><t>Mesna :</t></is></c><c r="F244" s="2" t="inlineStr"><is><t>powoduje upłynnienie wydzieliny w drzewie oskrzelowym</t></is></c><c r="G244" s="2" t="inlineStr"><is><t>jest antidotum przeciw metabolitowi cyklofosfamidu drażniącemu błonę śluzową dróg moczowych</t></is></c><c r="H244" s="2" t="inlineStr"><is><t>jest stosowana miejscowo w postaci inhalacji</t></is></c><c r="I244" s="2" t="inlineStr"><is><t>może wywołać skurcz oskrzeli</t></is></c><c r="J244" s="2" t="inlineStr" /><c r="K244" s="2" t="inlineStr" /><c r="L244" s="2" t="inlineStr" /><c r="M244" s="2" t="inlineStr" /><c r="N244" s="2" t="inlineStr" /><c r="O244" s="2" t="inlineStr" /><c r="P244" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q244" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="245"><c r="A245" s="2" t="inlineStr"><is><t>ZNIECZULENIA MIEJSCOWE</t></is></c><c r="B245" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C245" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D245" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E245" s="2" t="inlineStr"><is><t>Do leków znieczulających miejscowo stosowanych na błony śluzowe należy:</t></is></c><c r="F245" s="2" t="inlineStr"><is><t>prylokaina</t></is></c><c r="G245" s="2" t="inlineStr"><is><t>lidokaina</t></is></c><c r="H245" s="2" t="inlineStr" /><c r="I245" s="2" t="inlineStr" /><c r="J245" s="2" t="inlineStr" /><c r="K245" s="2" t="inlineStr"><is><t>chlorek etylu</t></is></c><c r="L245" s="2" t="inlineStr"><is><t>kapsaicyna</t></is></c><c r="M245" s="2" t="inlineStr" /><c r="N245" s="2" t="inlineStr" /><c r="O245" s="2" t="inlineStr" /><c r="P245" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q245" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="246"><c r="A246" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B246" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C246" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D246" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E246" s="2" t="inlineStr"><is><t>Inhibitorem kinaz białkowych jest:</t></is></c><c r="F246" s="2" t="inlineStr"><is><t>rapamycyna</t></is></c><c r="G246" s="2" t="inlineStr"><is><t>imatynib</t></is></c><c r="H246" s="2" t="inlineStr" /><c r="I246" s="2" t="inlineStr" /><c r="J246" s="2" t="inlineStr" /><c r="K246" s="2" t="inlineStr"><is><t>bortezomib</t></is></c><c r="L246" s="2" t="inlineStr"><is><t>lenalidomid</t></is></c><c r="M246" s="2" t="inlineStr" /><c r="N246" s="2" t="inlineStr" /><c r="O246" s="2" t="inlineStr" /><c r="P246" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q246" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="247"><c r="A247" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B247" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C247" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D247" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E247" s="2" t="inlineStr"><is><t>Betahistyna:</t></is></c><c r="F247" s="2" t="inlineStr"><is><t>zwiększa przepływ krwi w uchu wewnętrznym</t></is></c><c r="G247" s="2" t="inlineStr"><is><t>jest stosowana w leczeniu choroby Méniére'a</t></is></c><c r="H247" s="2" t="inlineStr" /><c r="I247" s="2" t="inlineStr" /><c r="J247" s="2" t="inlineStr" /><c r="K247" s="2" t="inlineStr"><is><t>jest agonistą receptorów H3</t></is></c><c r="L247" s="2" t="inlineStr"><is><t>jest lekiem z wyboru w przedsionkowych zawrotach głowy</t></is></c><c r="M247" s="2" t="inlineStr" /><c r="N247" s="2" t="inlineStr" /><c r="O247" s="2" t="inlineStr" /><c r="P247" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q247" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="248"><c r="A248" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B248" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C248" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D248" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E248" s="2" t="inlineStr"><is><t>Lekiem stosowanym w neuropatii popółpaścowej jest:</t></is></c><c r="F248" s="2" t="inlineStr"><is><t>amitryptylina</t></is></c><c r="G248" s="2" t="inlineStr"><is><t>pregabalina</t></is></c><c r="H248" s="2" t="inlineStr"><is><t>lidokaina</t></is></c><c r="I248" s="2" t="inlineStr"><is><t>gabapentyna</t></is></c><c r="J248" s="2" t="inlineStr" /><c r="K248" s="2" t="inlineStr" /><c r="L248" s="2" t="inlineStr" /><c r="M248" s="2" t="inlineStr" /><c r="N248" s="2" t="inlineStr" /><c r="O248" s="2" t="inlineStr" /><c r="P248" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q248" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="249"><c r="A249" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B249" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C249" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D249" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E249" s="2" t="inlineStr"><is><t>Na drugim stopniu drabiny analgetycznej wg WHO znajduje się:</t></is></c><c r="F249" s="2" t="inlineStr"><is><t>morfina w dawce ≤ 30 mg/dobę</t></is></c><c r="G249" s="2" t="inlineStr"><is><t>kodeina w dawce ≤360 mg/dobę</t></is></c><c r="H249" s="2" t="inlineStr"><is><t>oksykodon w dawce ≤20 mg/dobę</t></is></c><c r="I249" s="2" t="inlineStr" /><c r="J249" s="2" t="inlineStr" /><c r="K249" s="2" t="inlineStr"><is><t>fentanyl w dawce ≤ 10 mg/dobę</t></is></c><c r="L249" s="2" t="inlineStr" /><c r="M249" s="2" t="inlineStr" /><c r="N249" s="2" t="inlineStr" /><c r="O249" s="2" t="inlineStr" /><c r="P249" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q249" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="250"><c r="A250" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B250" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C250" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D250" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E250" s="2" t="inlineStr"><is><t>Wskaż prawidłowe zdanie:</t></is></c><c r="F250" s="2" t="inlineStr"><is><t>czas odstawienia rywaroksabanu przed planowanym zabiegiem chirurgicznym zależy od ryzyka krwawienia</t></is></c><c r="G250" s="2" t="inlineStr"><is><t>jeśli uzyskano stabilną hemostazę antagonisty witaminy K włącza się w 1. dobie po zabiegu chirurgicznym</t></is></c><c r="H250" s="2" t="inlineStr" /><c r="I250" s="2" t="inlineStr" /><c r="J250" s="2" t="inlineStr" /><c r="K250" s="2" t="inlineStr"><is><t>warfaryny nie należy odstawiać wcześniej niż na 2 dni przed planowanym zabiegiem chirurgicznym</t></is></c><c r="L250" s="2" t="inlineStr"><is><t>czas odstawienia edoksabanu przed zabiegiem chirurgicznym nie zależy od wartości klirensu kreatyniny</t></is></c><c r="M250" s="2" t="inlineStr" /><c r="N250" s="2" t="inlineStr" /><c r="O250" s="2" t="inlineStr" /><c r="P250" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q250" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="251"><c r="A251" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B251" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C251" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D251" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E251" s="2" t="inlineStr"><is><t>Wskaż prawidłowy lek przeciwzakrzepowego u osoby z:</t></is></c><c r="F251" s="2" t="inlineStr"><is><t>zapaleniem żył głębokich - rywaroksaban</t></is></c><c r="G251" s="2" t="inlineStr"><is><t>ciążą - enoksaparyna</t></is></c><c r="H251" s="2" t="inlineStr"><is><t>mechaniczną zastawką serca – warfaryna</t></is></c><c r="I251" s="2" t="inlineStr" /><c r="J251" s="2" t="inlineStr" /><c r="K251" s="2" t="inlineStr"><is><t>niewydolnością nerek (CCr &lt;30ml/min) – dabigatran</t></is></c><c r="L251" s="2" t="inlineStr" /><c r="M251" s="2" t="inlineStr" /><c r="N251" s="2" t="inlineStr" /><c r="O251" s="2" t="inlineStr" /><c r="P251" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q251" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="252"><c r="A252" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B252" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C252" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D252" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E252" s="2" t="inlineStr"><is><t>Podczas leczenia przeciwzakrzepowego z zastosowaniem nadroparyny należy:</t></is></c><c r="F252" s="2" t="inlineStr"><is><t>kontrolować liczbę płytek</t></is></c><c r="G252" s="2" t="inlineStr"><is><t>rozważyć korektę dawek u osób otyłych</t></is></c><c r="H252" s="2" t="inlineStr" /><c r="I252" s="2" t="inlineStr" /><c r="J252" s="2" t="inlineStr" /><c r="K252" s="2" t="inlineStr"><is><t>monitorować dawki za pomocą oznaczenia APTT</t></is></c><c r="L252" s="2" t="inlineStr"><is><t>zmniejszyć dawkę w każdym przypadku, jeśli eGFR osiąga wartość mniejszą niż 90 ml/min</t></is></c><c r="M252" s="2" t="inlineStr" /><c r="N252" s="2" t="inlineStr" /><c r="O252" s="2" t="inlineStr" /><c r="P252" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q252" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="253"><c r="A253" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B253" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C253" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D253" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E253" s="2" t="inlineStr"><is><t>Kangrelor:</t></is></c><c r="F253" s="2" t="inlineStr"><is><t>jest wskazany podczas przezskórnych interwencji wieńcowych łącznie z kwasem acetylosalicylowym</t></is></c><c r="G253" s="2" t="inlineStr" /><c r="H253" s="2" t="inlineStr" /><c r="I253" s="2" t="inlineStr" /><c r="J253" s="2" t="inlineStr" /><c r="K253" s="2" t="inlineStr"><is><t>jest agonistą receptora P2Y12</t></is></c><c r="L253" s="2" t="inlineStr"><is><t>wymaga aktywacji w przewodzie pokarmowym</t></is></c><c r="M253" s="2" t="inlineStr"><is><t>działa przez 1-2 doby</t></is></c><c r="N253" s="2" t="inlineStr" /><c r="O253" s="2" t="inlineStr" /><c r="P253" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q253" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="254"><c r="A254" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B254" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C254" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D254" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E254" s="2" t="inlineStr"><is><t>Na istotnie zmniejszoną skuteczność doustnych antagonistów witaminy K może mieć wpływ spożywanie:</t></is></c><c r="F254" s="2" t="inlineStr"><is><t>szpinaku</t></is></c><c r="G254" s="2" t="inlineStr" /><c r="H254" s="2" t="inlineStr" /><c r="I254" s="2" t="inlineStr" /><c r="J254" s="2" t="inlineStr" /><c r="K254" s="2" t="inlineStr"><is><t>oleju rybnego zawierającego nienasycone kwasy tłuszczowe omega -3</t></is></c><c r="L254" s="2" t="inlineStr"><is><t>witaminy E</t></is></c><c r="M254" s="2" t="inlineStr"><is><t>czosnku</t></is></c><c r="N254" s="2" t="inlineStr" /><c r="O254" s="2" t="inlineStr" /><c r="P254" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q254" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="255"><c r="A255" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B255" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C255" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D255" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E255" s="2" t="inlineStr"><is><t>Pacjentom, którzy przebyli udar niedokrwienny mózgu należy zalecić profilaktykę wtórną. Do leków o udokumentowanym działaniu zmniejszających ryzyko następnego udaru należy:</t></is></c><c r="F255" s="2" t="inlineStr"><is><t>simwastatyna</t></is></c><c r="G255" s="2" t="inlineStr"><is><t>klopidogrel</t></is></c><c r="H255" s="2" t="inlineStr"><is><t>lizynopryl</t></is></c><c r="I255" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="J255" s="2" t="inlineStr" /><c r="K255" s="2" t="inlineStr" /><c r="L255" s="2" t="inlineStr" /><c r="M255" s="2" t="inlineStr" /><c r="N255" s="2" t="inlineStr" /><c r="O255" s="2" t="inlineStr" /><c r="P255" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q255" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="256"><c r="A256" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B256" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C256" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D256" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E256" s="2" t="inlineStr"><is><t>Fenofibrat:</t></is></c><c r="F256" s="2" t="inlineStr"><is><t>zmniejsza stężenie trójglicerydów i zwiększa stężenie cholesterolu HDL</t></is></c><c r="G256" s="2" t="inlineStr"><is><t>zwiększa ryzyko kamicy pęcherzyka żółciowego</t></is></c><c r="H256" s="2" t="inlineStr" /><c r="I256" s="2" t="inlineStr" /><c r="J256" s="2" t="inlineStr" /><c r="K256" s="2" t="inlineStr"><is><t>hamuje reduktazę 3-hydroksy-3-metyloglutarylo-CoA (HMG-CoA)</t></is></c><c r="L256" s="2" t="inlineStr"><is><t>nie może być stosowany w połączeniu ze statyną</t></is></c><c r="M256" s="2" t="inlineStr" /><c r="N256" s="2" t="inlineStr" /><c r="O256" s="2" t="inlineStr" /><c r="P256" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q256" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="257"><c r="A257" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B257" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C257" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D257" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E257" s="2" t="inlineStr"><is><t>Hiperurykemię może spowodować:</t></is></c><c r="F257" s="2" t="inlineStr"><is><t>torasemid</t></is></c><c r="G257" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="H257" s="2" t="inlineStr" /><c r="I257" s="2" t="inlineStr" /><c r="J257" s="2" t="inlineStr" /><c r="K257" s="2" t="inlineStr"><is><t>losartan</t></is></c><c r="L257" s="2" t="inlineStr"><is><t>allopurynol</t></is></c><c r="M257" s="2" t="inlineStr" /><c r="N257" s="2" t="inlineStr" /><c r="O257" s="2" t="inlineStr" /><c r="P257" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q257" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="258"><c r="A258" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B258" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C258" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D258" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E258" s="2" t="inlineStr"><is><t>Odstęp QT mogą wydłużać:</t></is></c><c r="F258" s="2" t="inlineStr"><is><t>amiodaron</t></is></c><c r="G258" s="2" t="inlineStr"><is><t>sotalol</t></is></c><c r="H258" s="2" t="inlineStr" /><c r="I258" s="2" t="inlineStr" /><c r="J258" s="2" t="inlineStr" /><c r="K258" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="L258" s="2" t="inlineStr"><is><t>diltiazem</t></is></c><c r="M258" s="2" t="inlineStr" /><c r="N258" s="2" t="inlineStr" /><c r="O258" s="2" t="inlineStr" /><c r="P258" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q258" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="259"><c r="A259" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B259" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C259" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D259" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E259" s="2" t="inlineStr"><is><t>Indapamid:</t></is></c><c r="F259" s="2" t="inlineStr"><is><t>ma działanie naczyniorozszerzające</t></is></c><c r="G259" s="2" t="inlineStr"><is><t>może spowodować hiponatremię</t></is></c><c r="H259" s="2" t="inlineStr"><is><t>zmniejsza wydalanie wapnia z moczem</t></is></c><c r="I259" s="2" t="inlineStr"><is><t>jest chętnie stosowany w przewlekłej terapii nadciśnienia tętniczego u osób po 80 roku życia</t></is></c><c r="J259" s="2" t="inlineStr" /><c r="K259" s="2" t="inlineStr" /><c r="L259" s="2" t="inlineStr" /><c r="M259" s="2" t="inlineStr" /><c r="N259" s="2" t="inlineStr" /><c r="O259" s="2" t="inlineStr" /><c r="P259" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q259" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="260"><c r="A260" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B260" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C260" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D260" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E260" s="2" t="inlineStr"><is><t>Produkty biopodobne:</t></is></c><c r="F260" s="2" t="inlineStr"><is><t>są automatycznie zamienne (substytucja)</t></is></c><c r="G260" s="2" t="inlineStr"><is><t>muszą mieć potwierdzoną podobną immunogenność</t></is></c><c r="H260" s="2" t="inlineStr" /><c r="I260" s="2" t="inlineStr" /><c r="J260" s="2" t="inlineStr" /><c r="K260" s="2" t="inlineStr"><is><t>są rejestrowane w procedurze zdecentralizowanej</t></is></c><c r="L260" s="2" t="inlineStr"><is><t>po dopuszczeniu do obrotu mogą być stosowane we wszystkich wskazaniach zamiennie</t></is></c><c r="M260" s="2" t="inlineStr" /><c r="N260" s="2" t="inlineStr" /><c r="O260" s="2" t="inlineStr" /><c r="P260" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q260" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="261"><c r="A261" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B261" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C261" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D261" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E261" s="2" t="inlineStr"><is><t>W leczeniu zarażenia glistą ludzką stosujemy:</t></is></c><c r="F261" s="2" t="inlineStr"><is><t>pyrantel</t></is></c><c r="G261" s="2" t="inlineStr"><is><t>albendazol</t></is></c><c r="H261" s="2" t="inlineStr" /><c r="I261" s="2" t="inlineStr" /><c r="J261" s="2" t="inlineStr" /><c r="K261" s="2" t="inlineStr"><is><t>tynidazol</t></is></c><c r="L261" s="2" t="inlineStr"><is><t>krotamiton</t></is></c><c r="M261" s="2" t="inlineStr" /><c r="N261" s="2" t="inlineStr" /><c r="O261" s="2" t="inlineStr" /><c r="P261" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q261" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="262"><c r="A262" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B262" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C262" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D262" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E262" s="2" t="inlineStr"><is><t>W leczeniu grypy zaleca się:</t></is></c><c r="F262" s="2" t="inlineStr"><is><t>zanamiwir</t></is></c><c r="G262" s="2" t="inlineStr"><is><t>oseltamiwir</t></is></c><c r="H262" s="2" t="inlineStr" /><c r="I262" s="2" t="inlineStr" /><c r="J262" s="2" t="inlineStr" /><c r="K262" s="2" t="inlineStr"><is><t>acyklowir</t></is></c><c r="L262" s="2" t="inlineStr"><is><t>foskarnet</t></is></c><c r="M262" s="2" t="inlineStr" /><c r="N262" s="2" t="inlineStr" /><c r="O262" s="2" t="inlineStr" /><c r="P262" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q262" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="263"><c r="A263" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B263" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C263" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D263" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E263" s="2" t="inlineStr"><is><t>W przypadku dotychczas nieleczonych chorych, u których objawy astmy oskrzelowej w ciągu dnia występują sporadycznie (&lt;2 razy w miesiącu), objawy nocne nie występują, nie ma czynników ryzyka zaostrzeń (także w wywiadzie), a czynność płuc jest prawidłowa należy zastosować:</t></is></c><c r="F263" s="2" t="inlineStr"><is><t>fenoterol doraźnie</t></is></c><c r="G263" s="2" t="inlineStr" /><c r="H263" s="2" t="inlineStr" /><c r="I263" s="2" t="inlineStr" /><c r="J263" s="2" t="inlineStr" /><c r="K263" s="2" t="inlineStr"><is><t>montelukast przewlekle</t></is></c><c r="L263" s="2" t="inlineStr"><is><t>regularnie małe dawki cyklezonidu</t></is></c><c r="M263" s="2" t="inlineStr"><is><t>teofilinę krótkodziałającą</t></is></c><c r="N263" s="2" t="inlineStr" /><c r="O263" s="2" t="inlineStr" /><c r="P263" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q263" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="264"><c r="A264" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B264" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C264" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D264" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E264" s="2" t="inlineStr"><is><t>Bromek glikopironium :</t></is></c><c r="F264" s="2" t="inlineStr"><is><t>wykazuje synergizm działania bronchodylatacyjnego z indakaterolem</t></is></c><c r="G264" s="2" t="inlineStr"><is><t>jest stosowany w leczeniu podtrzymującym w POChP</t></is></c><c r="H264" s="2" t="inlineStr" /><c r="I264" s="2" t="inlineStr" /><c r="J264" s="2" t="inlineStr" /><c r="K264" s="2" t="inlineStr"><is><t>jest wziewnym agonistą receptorów muskarynowych</t></is></c><c r="L264" s="2" t="inlineStr"><is><t>rozszczepia wiązania disiarczkowe w glikoproteinach śluzu</t></is></c><c r="M264" s="2" t="inlineStr" /><c r="N264" s="2" t="inlineStr" /><c r="O264" s="2" t="inlineStr" /><c r="P264" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q264" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="265"><c r="A265" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B265" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C265" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D265" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E265" s="2" t="inlineStr"><is><t>W leczeniu przewlekłego zapalenia trzustki celowe może być zastosowanie:</t></is></c><c r="F265" s="2" t="inlineStr"><is><t>suplementacji enzymów trzustkowych</t></is></c><c r="G265" s="2" t="inlineStr"><is><t>tramadolu</t></is></c><c r="H265" s="2" t="inlineStr"><is><t>pantoprazolu</t></is></c><c r="I265" s="2" t="inlineStr"><is><t>fluoksetyny</t></is></c><c r="J265" s="2" t="inlineStr" /><c r="K265" s="2" t="inlineStr" /><c r="L265" s="2" t="inlineStr" /><c r="M265" s="2" t="inlineStr" /><c r="N265" s="2" t="inlineStr" /><c r="O265" s="2" t="inlineStr" /><c r="P265" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q265" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="266"><c r="A266" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B266" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C266" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D266" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E266" s="2" t="inlineStr"><is><t>Profilaktyka przeciwmalaryczna w warunkach wysokiego ryzyka zakażenia Plasmodium falciparum obejmuje stosowanie:</t></is></c><c r="F266" s="2" t="inlineStr"><is><t>repelentów</t></is></c><c r="G266" s="2" t="inlineStr"><is><t>atowakwonu/proguanilu</t></is></c><c r="H266" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="I266" s="2" t="inlineStr" /><c r="J266" s="2" t="inlineStr" /><c r="K266" s="2" t="inlineStr"><is><t>artemetru/lumefantryny</t></is></c><c r="L266" s="2" t="inlineStr" /><c r="M266" s="2" t="inlineStr" /><c r="N266" s="2" t="inlineStr" /><c r="O266" s="2" t="inlineStr" /><c r="P266" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q266" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="267"><c r="A267" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B267" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C267" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D267" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E267" s="2" t="inlineStr"><is><t>Adalimumab:</t></is></c><c r="F267" s="2" t="inlineStr"><is><t>jest rekombinowanym w pełni ludzkim przeciwciałem monoklonalnym</t></is></c><c r="G267" s="2" t="inlineStr"><is><t>neutralizuje biologiczną czynność TNF</t></is></c><c r="H267" s="2" t="inlineStr"><is><t>jest przeciwwskazany w ciężkich zakażeniach</t></is></c><c r="I267" s="2" t="inlineStr" /><c r="J267" s="2" t="inlineStr" /><c r="K267" s="2" t="inlineStr"><is><t>jest wytwarzany z użyciem komórek zwierzęcych, co wiadomo na podstawie ujednoliconych zasad nadawania nazw przeciwciałom monoklonalnym</t></is></c><c r="L267" s="2" t="inlineStr" /><c r="M267" s="2" t="inlineStr" /><c r="N267" s="2" t="inlineStr" /><c r="O267" s="2" t="inlineStr" /><c r="P267" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q267" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="268"><c r="A268" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B268" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C268" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D268" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E268" s="2" t="inlineStr"><is><t>Dla insuliny aspart u pacjentów z umiarkowaną i ciężką niewydolnością wątroby stwierdzono: t max = ok. 85 min (tmax = ok. 40 minut u pacjentów z prawidłową czynnością wątroby); AUC, Cmax i CL/F były podobne do pacjentów z prawidłową czynnością wątroby. Na tej podstawie u osób z niewydolnością wątroby uzasadnione jest:</t></is></c><c r="F268" s="2" t="inlineStr"><is><t>wcześniejsze podanie leku przed posiłkiem</t></is></c><c r="G268" s="2" t="inlineStr"><is><t>stosowanie leku u osób z 7-15 pkt wg skali Childa-Pugha</t></is></c><c r="H268" s="2" t="inlineStr" /><c r="I268" s="2" t="inlineStr" /><c r="J268" s="2" t="inlineStr" /><c r="K268" s="2" t="inlineStr"><is><t>wyłącznie dożylne podawanie leku</t></is></c><c r="L268" s="2" t="inlineStr"><is><t>redukcja dawki początkowej o ½ oszacowanej na podstawie m.c. i wyjściowej glikemii</t></is></c><c r="M268" s="2" t="inlineStr" /><c r="N268" s="2" t="inlineStr" /><c r="O268" s="2" t="inlineStr" /><c r="P268" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q268" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="269"><c r="A269" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B269" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C269" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D269" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E269" s="2" t="inlineStr"><is><t>Wartości ciśnienia tętniczego mogą się zwiększyć po włączeniu:</t></is></c><c r="F269" s="2" t="inlineStr"><is><t>metyloprednizolonu</t></is></c><c r="G269" s="2" t="inlineStr"><is><t>diklofenaku</t></is></c><c r="H269" s="2" t="inlineStr" /><c r="I269" s="2" t="inlineStr" /><c r="J269" s="2" t="inlineStr" /><c r="K269" s="2" t="inlineStr"><is><t>eplerenonu</t></is></c><c r="L269" s="2" t="inlineStr"><is><t>urapidylu</t></is></c><c r="M269" s="2" t="inlineStr" /><c r="N269" s="2" t="inlineStr" /><c r="O269" s="2" t="inlineStr" /><c r="P269" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q269" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="270"><c r="A270" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B270" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C270" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D270" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E270" s="2" t="inlineStr"><is><t>Farmakoterapię otyłości należy rozważyć, gdy:</t></is></c><c r="F270" s="2" t="inlineStr"><is><t>BMI&gt; 27 kg/m2 i glikemia na czczo &gt;100mg/dl</t></is></c><c r="G270" s="2" t="inlineStr"><is><t>BMI≥ 30 kg/m2 i stwierdzono ponowny wzrost masy ciała pomimo wdrożonych procedur niefarmakologicznych</t></is></c><c r="H270" s="2" t="inlineStr"><is><t>BMI&gt; 27 kg/m2 i SBP ≥160 mmHg</t></is></c><c r="I270" s="2" t="inlineStr" /><c r="J270" s="2" t="inlineStr" /><c r="K270" s="2" t="inlineStr"><is><t>BMI≥ 30 kg/m2, a wcześniejsze procedury niefarmakologiczne spowodowały redukcję masy ciała w przedziale 7-10 kg</t></is></c><c r="L270" s="2" t="inlineStr" /><c r="M270" s="2" t="inlineStr" /><c r="N270" s="2" t="inlineStr" /><c r="O270" s="2" t="inlineStr" /><c r="P270" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q270" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="271"><c r="A271" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B271" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C271" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D271" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E271" s="2" t="inlineStr"><is><t>Wzrost masy ciała mogą spowodować:</t></is></c><c r="F271" s="2" t="inlineStr"><is><t>chlorpromazyna</t></is></c><c r="G271" s="2" t="inlineStr"><is><t>insulina</t></is></c><c r="H271" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="I271" s="2" t="inlineStr" /><c r="J271" s="2" t="inlineStr" /><c r="K271" s="2" t="inlineStr"><is><t>liraglutyd</t></is></c><c r="L271" s="2" t="inlineStr" /><c r="M271" s="2" t="inlineStr" /><c r="N271" s="2" t="inlineStr" /><c r="O271" s="2" t="inlineStr" /><c r="P271" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q271" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="272"><c r="A272" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B272" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C272" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D272" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E272" s="2" t="inlineStr"><is><t>Który z leków istotnie zwiększa ryzyko napadów drgawkowych:</t></is></c><c r="F272" s="2" t="inlineStr"><is><t>tramadol</t></is></c><c r="G272" s="2" t="inlineStr"><is><t>amitryptylina</t></is></c><c r="H272" s="2" t="inlineStr"><is><t>prometazyna</t></is></c><c r="I272" s="2" t="inlineStr" /><c r="J272" s="2" t="inlineStr" /><c r="K272" s="2" t="inlineStr"><is><t>klorazepan</t></is></c><c r="L272" s="2" t="inlineStr" /><c r="M272" s="2" t="inlineStr" /><c r="N272" s="2" t="inlineStr" /><c r="O272" s="2" t="inlineStr" /><c r="P272" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q272" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="273"><c r="A273" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B273" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C273" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D273" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E273" s="2" t="inlineStr"><is><t>Zgoda komisji bioetycznej jest niezbędna, gdy planowane jest przeprowadzenie:</t></is></c><c r="F273" s="2" t="inlineStr"><is><t>badania klinicznego fazy III</t></is></c><c r="G273" s="2" t="inlineStr"><is><t>eksperymentu leczniczego</t></is></c><c r="H273" s="2" t="inlineStr"><is><t>badania klinicznego niekomercyjnego</t></is></c><c r="I273" s="2" t="inlineStr" /><c r="J273" s="2" t="inlineStr" /><c r="K273" s="2" t="inlineStr"><is><t>zastosowania leku off-label, ale zgodnie z aktualną wiedzą medyczną</t></is></c><c r="L273" s="2" t="inlineStr" /><c r="M273" s="2" t="inlineStr" /><c r="N273" s="2" t="inlineStr" /><c r="O273" s="2" t="inlineStr" /><c r="P273" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q273" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="274"><c r="A274" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B274" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C274" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D274" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E274" s="2" t="inlineStr"><is><t>W procedurze centralnej rejestruje się leki stosowane w:</t></is></c><c r="F274" s="2" t="inlineStr"><is><t>chorobach rzadkich</t></is></c><c r="G274" s="2" t="inlineStr"><is><t>terapii HIV</t></is></c><c r="H274" s="2" t="inlineStr"><is><t>terapii genowej</t></is></c><c r="I274" s="2" t="inlineStr" /><c r="J274" s="2" t="inlineStr" /><c r="K274" s="2" t="inlineStr"><is><t>populacji geriatrycznej</t></is></c><c r="L274" s="2" t="inlineStr" /><c r="M274" s="2" t="inlineStr" /><c r="N274" s="2" t="inlineStr" /><c r="O274" s="2" t="inlineStr" /><c r="P274" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q274" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="275"><c r="A275" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B275" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C275" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D275" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E275" s="2" t="inlineStr"><is><t>Pierwotnym źródłem wiedzy o lekach są:</t></is></c><c r="F275" s="2" t="inlineStr"><is><t>publikacje wyników badań klinicznych</t></is></c><c r="G275" s="2" t="inlineStr" /><c r="H275" s="2" t="inlineStr" /><c r="I275" s="2" t="inlineStr" /><c r="J275" s="2" t="inlineStr" /><c r="K275" s="2" t="inlineStr"><is><t>wytyczne praktyki klinicznej</t></is></c><c r="L275" s="2" t="inlineStr"><is><t>charakterystyki produktów leczniczych</t></is></c><c r="M275" s="2" t="inlineStr"><is><t>podręczniki farmakologii i indeksy leków</t></is></c><c r="N275" s="2" t="inlineStr" /><c r="O275" s="2" t="inlineStr" /><c r="P275" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q275" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="276"><c r="A276" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B276" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C276" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D276" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E276" s="2" t="inlineStr"><is><t>Wskazaniem do stosowania retinolu jest:</t></is></c><c r="F276" s="2" t="inlineStr"><is><t>łuszczyca</t></is></c><c r="G276" s="2" t="inlineStr"><is><t>niedowidzenie o zmierzchu</t></is></c><c r="H276" s="2" t="inlineStr" /><c r="I276" s="2" t="inlineStr" /><c r="J276" s="2" t="inlineStr" /><c r="K276" s="2" t="inlineStr"><is><t>polineuropatia obwodowa</t></is></c><c r="L276" s="2" t="inlineStr"><is><t>osteomalacja</t></is></c><c r="M276" s="2" t="inlineStr" /><c r="N276" s="2" t="inlineStr" /><c r="O276" s="2" t="inlineStr" /><c r="P276" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q276" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="277"><c r="A277" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B277" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C277" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D277" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E277" s="2" t="inlineStr"><is><t>Feksofenadyna:</t></is></c><c r="F277" s="2" t="inlineStr"><is><t>jest podawana doustnie</t></is></c><c r="G277" s="2" t="inlineStr" /><c r="H277" s="2" t="inlineStr" /><c r="I277" s="2" t="inlineStr" /><c r="J277" s="2" t="inlineStr" /><c r="K277" s="2" t="inlineStr"><is><t>działa nieselektywnie na rec. H1</t></is></c><c r="L277" s="2" t="inlineStr"><is><t>przenika w znacznym stopniu przez barierę krew- mózg</t></is></c><c r="M277" s="2" t="inlineStr"><is><t>działa kardiotoksycznie i jest przeciwwskazana w chorobie niedokrwiennej serca</t></is></c><c r="N277" s="2" t="inlineStr" /><c r="O277" s="2" t="inlineStr" /><c r="P277" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q277" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="278"><c r="A278" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B278" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C278" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D278" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E278" s="2" t="inlineStr"><is><t>Wskaż wady dekstranów:</t></is></c><c r="F278" s="2" t="inlineStr"><is><t>utrudniają wiarygodne oznaczenie grupy krwi i próby krzyżowej</t></is></c><c r="G278" s="2" t="inlineStr"><is><t>są immunogenne</t></is></c><c r="H278" s="2" t="inlineStr" /><c r="I278" s="2" t="inlineStr" /><c r="J278" s="2" t="inlineStr" /><c r="K278" s="2" t="inlineStr"><is><t>powodują przyrost objętości wewnątrznaczyniowej przekraczający ich objętość</t></is></c><c r="L278" s="2" t="inlineStr"><is><t>działają prozakrzepowo</t></is></c><c r="M278" s="2" t="inlineStr" /><c r="N278" s="2" t="inlineStr" /><c r="O278" s="2" t="inlineStr" /><c r="P278" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q278" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="279"><c r="A279" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B279" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C279" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D279" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E279" s="2" t="inlineStr"><is><t>Podanie rywastygminy jest uzasadnione u pacjentów z:</t></is></c><c r="F279" s="2" t="inlineStr"><is><t>otępieniem w przebiegu choroby Parkinsona</t></is></c><c r="G279" s="2" t="inlineStr"><is><t>chorobą Alzheimera</t></is></c><c r="H279" s="2" t="inlineStr" /><c r="I279" s="2" t="inlineStr" /><c r="J279" s="2" t="inlineStr" /><c r="K279" s="2" t="inlineStr"><is><t>otępieniem naczyniopochodnym</t></is></c><c r="L279" s="2" t="inlineStr"><is><t>otępieniem czołowo-skroniowym</t></is></c><c r="M279" s="2" t="inlineStr" /><c r="N279" s="2" t="inlineStr" /><c r="O279" s="2" t="inlineStr" /><c r="P279" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q279" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="280"><c r="A280" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B280" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C280" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D280" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E280" s="2" t="inlineStr"><is><t>Podanie rywastygminy jest uzasadnione u pacjentów z:</t></is></c><c r="F280" s="2" t="inlineStr"><is><t>otępieniem w przebiegu choroby Parkinsona</t></is></c><c r="G280" s="2" t="inlineStr"><is><t>chorobą Alzheimera</t></is></c><c r="H280" s="2" t="inlineStr" /><c r="I280" s="2" t="inlineStr" /><c r="J280" s="2" t="inlineStr" /><c r="K280" s="2" t="inlineStr"><is><t>otępieniem naczyniopochodnym</t></is></c><c r="L280" s="2" t="inlineStr"><is><t>łagodnymi zaburzeniami poznawczymi</t></is></c><c r="M280" s="2" t="inlineStr" /><c r="N280" s="2" t="inlineStr" /><c r="O280" s="2" t="inlineStr" /><c r="P280" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q280" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="281"><c r="A281" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B281" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C281" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D281" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E281" s="2" t="inlineStr"><is><t>W alkoholowym zespole odstawiennym celowe może być zastosowanie:</t></is></c><c r="F281" s="2" t="inlineStr"><is><t>tiaminy</t></is></c><c r="G281" s="2" t="inlineStr"><is><t>diazepamu</t></is></c><c r="H281" s="2" t="inlineStr"><is><t>płynoterapia z suplementacją elektrolitów</t></is></c><c r="I281" s="2" t="inlineStr" /><c r="J281" s="2" t="inlineStr" /><c r="K281" s="2" t="inlineStr"><is><t>akamprozatu</t></is></c><c r="L281" s="2" t="inlineStr" /><c r="M281" s="2" t="inlineStr" /><c r="N281" s="2" t="inlineStr" /><c r="O281" s="2" t="inlineStr" /><c r="P281" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q281" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="282"><c r="A282" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B282" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C282" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D282" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E282" s="2" t="inlineStr"><is><t>Mykofenolan mofetylu:</t></is></c><c r="F282" s="2" t="inlineStr"><is><t>jest wskazany w profilaktyce ostrego odrzucania przeszczepu serca</t></is></c><c r="G282" s="2" t="inlineStr"><is><t>zwiększa ryzyko wystąpienia nowotworów</t></is></c><c r="H282" s="2" t="inlineStr" /><c r="I282" s="2" t="inlineStr" /><c r="J282" s="2" t="inlineStr" /><c r="K282" s="2" t="inlineStr"><is><t>należy do inhibitorów mTOR</t></is></c><c r="L282" s="2" t="inlineStr"><is><t>stosowany w czasie ciąży jest bezpieczny dla płodu</t></is></c><c r="M282" s="2" t="inlineStr" /><c r="N282" s="2" t="inlineStr" /><c r="O282" s="2" t="inlineStr" /><c r="P282" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q282" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="283"><c r="A283" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B283" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C283" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D283" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E283" s="2" t="inlineStr"><is><t>Iwabradyna:</t></is></c><c r="F283" s="2" t="inlineStr"><is><t>może powodować zaburzenia widzenia</t></is></c><c r="G283" s="2" t="inlineStr"><is><t>wybiórczo i swoiście wpływa na na prąd If rozrusznika serca</t></is></c><c r="H283" s="2" t="inlineStr" /><c r="I283" s="2" t="inlineStr" /><c r="J283" s="2" t="inlineStr" /><c r="K283" s="2" t="inlineStr"><is><t>obniża kurczliwość mięśnia sercowego</t></is></c><c r="L283" s="2" t="inlineStr"><is><t>wydłuża czas repolaryzacji komór</t></is></c><c r="M283" s="2" t="inlineStr" /><c r="N283" s="2" t="inlineStr" /><c r="O283" s="2" t="inlineStr" /><c r="P283" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q283" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="284"><c r="A284" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B284" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C284" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D284" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E284" s="2" t="inlineStr"><is><t>Monoazotan izosorbidu:</t></is></c><c r="F284" s="2" t="inlineStr"><is><t>jest skuteczny po podaniu doustnym</t></is></c><c r="G284" s="2" t="inlineStr"><is><t>poprawia ukrwienie obszarów podwsierdziowych serca</t></is></c><c r="H284" s="2" t="inlineStr" /><c r="I284" s="2" t="inlineStr" /><c r="J284" s="2" t="inlineStr" /><c r="K284" s="2" t="inlineStr"><is><t>podlega istotnemu efektowi pierwszego przejścia przez wątrobę</t></is></c><c r="L284" s="2" t="inlineStr"><is><t>jest przeciwwskazany w naczynioskurczowej postaci choroby wieńcowej</t></is></c><c r="M284" s="2" t="inlineStr" /><c r="N284" s="2" t="inlineStr" /><c r="O284" s="2" t="inlineStr" /><c r="P284" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q284" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="285"><c r="A285" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B285" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C285" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D285" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E285" s="2" t="inlineStr"><is><t>W leczeniu owrzodzeń żylnych, jako leczenie uzupełniające, skuteczne są:</t></is></c><c r="F285" s="2" t="inlineStr"><is><t>mikronizowana diosmina</t></is></c><c r="G285" s="2" t="inlineStr"><is><t>opatrunki ze srebrem</t></is></c><c r="H285" s="2" t="inlineStr"><is><t>pentoksyfilina</t></is></c><c r="I285" s="2" t="inlineStr"><is><t>filgrastym</t></is></c><c r="J285" s="2" t="inlineStr" /><c r="K285" s="2" t="inlineStr" /><c r="L285" s="2" t="inlineStr" /><c r="M285" s="2" t="inlineStr" /><c r="N285" s="2" t="inlineStr" /><c r="O285" s="2" t="inlineStr" /><c r="P285" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q285" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="286"><c r="A286" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B286" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C286" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D286" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E286" s="2" t="inlineStr"><is><t>Funkcje kognitywne u osób bez zaburzeń poznawczych poprawiają:</t></is></c><c r="F286" s="2" t="inlineStr"><is><t>piracetam</t></is></c><c r="G286" s="2" t="inlineStr"><is><t>winpocetyna</t></is></c><c r="H286" s="2" t="inlineStr"><is><t>nicergolina</t></is></c><c r="I286" s="2" t="inlineStr"><is><t>metylfenidat</t></is></c><c r="J286" s="2" t="inlineStr" /><c r="K286" s="2" t="inlineStr" /><c r="L286" s="2" t="inlineStr" /><c r="M286" s="2" t="inlineStr" /><c r="N286" s="2" t="inlineStr" /><c r="O286" s="2" t="inlineStr" /><c r="P286" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q286" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="287"><c r="A287" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B287" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C287" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D287" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E287" s="2" t="inlineStr"><is><t>Klozapina:</t></is></c><c r="F287" s="2" t="inlineStr"><is><t>może być skuteczna w lekoopornej schizofrenii</t></is></c><c r="G287" s="2" t="inlineStr"><is><t>wymaga monitorowania morfologii krwi</t></is></c><c r="H287" s="2" t="inlineStr"><is><t>nasila objawy zespołu metabolicznego</t></is></c><c r="I287" s="2" t="inlineStr" /><c r="J287" s="2" t="inlineStr" /><c r="K287" s="2" t="inlineStr"><is><t>w małych dawkach zalecana jest do leczenia bezsenności</t></is></c><c r="L287" s="2" t="inlineStr" /><c r="M287" s="2" t="inlineStr" /><c r="N287" s="2" t="inlineStr" /><c r="O287" s="2" t="inlineStr" /><c r="P287" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q287" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="288"><c r="A288" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B288" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C288" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D288" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E288" s="2" t="inlineStr"><is><t>W terapii substytucyjnej uzależnienia od opioidów celowe może być zastosowanie:</t></is></c><c r="F288" s="2" t="inlineStr"><is><t>buprenorfiny</t></is></c><c r="G288" s="2" t="inlineStr"><is><t>metadonu</t></is></c><c r="H288" s="2" t="inlineStr" /><c r="I288" s="2" t="inlineStr" /><c r="J288" s="2" t="inlineStr" /><c r="K288" s="2" t="inlineStr"><is><t>nalokson</t></is></c><c r="L288" s="2" t="inlineStr"><is><t>warenikliny</t></is></c><c r="M288" s="2" t="inlineStr" /><c r="N288" s="2" t="inlineStr" /><c r="O288" s="2" t="inlineStr" /><c r="P288" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q288" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="289"><c r="A289" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B289" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C289" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D289" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E289" s="2" t="inlineStr"><is><t>Silnie hepatotoksycznie działa:</t></is></c><c r="F289" s="2" t="inlineStr"><is><t>izoniazyd</t></is></c><c r="G289" s="2" t="inlineStr"><is><t>pirazynamid</t></is></c><c r="H289" s="2" t="inlineStr"><is><t>ryfampicyna</t></is></c><c r="I289" s="2" t="inlineStr" /><c r="J289" s="2" t="inlineStr" /><c r="K289" s="2" t="inlineStr"><is><t>streptomycyna</t></is></c><c r="L289" s="2" t="inlineStr" /><c r="M289" s="2" t="inlineStr" /><c r="N289" s="2" t="inlineStr" /><c r="O289" s="2" t="inlineStr" /><c r="P289" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q289" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="290"><c r="A290" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B290" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C290" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D290" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E290" s="2" t="inlineStr"><is><t>Etambutol:</t></is></c><c r="F290" s="2" t="inlineStr"><is><t>zapobiega powstawaniu lekooporności na inne leki przeciwprątkowe</t></is></c><c r="G290" s="2" t="inlineStr"><is><t>może spowodować zaburzenia widzenia barwnego</t></is></c><c r="H290" s="2" t="inlineStr" /><c r="I290" s="2" t="inlineStr" /><c r="J290" s="2" t="inlineStr" /><c r="K290" s="2" t="inlineStr"><is><t>nie powinien być stosowany przez kobiety w ciąży</t></is></c><c r="L290" s="2" t="inlineStr"><is><t>nie jest stosowany w leczeniu gruźlicy pozapłucnej</t></is></c><c r="M290" s="2" t="inlineStr" /><c r="N290" s="2" t="inlineStr" /><c r="O290" s="2" t="inlineStr" /><c r="P290" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q290" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="291"><c r="A291" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B291" s="2" t="inlineStr"><is><t>Struktura chemiczna</t></is></c><c r="C291" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D291" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E291" s="2" t="inlineStr"><is><t>Jeśli leczymy depresję, to:</t></is></c><c r="F291" s="2" t="inlineStr"><is><t>u pacjentów z niewydolnością nerek lekiem pierwszego wyboru może być sertralina</t></is></c><c r="G291" s="2" t="inlineStr"><is><t>istnieje zwiększone ryzyko zachowań samobójczych u pacjentów w wieku poniżej 25 lat w okresie rozpoczynania leczenia przeciwdepresyjnego</t></is></c><c r="H291" s="2" t="inlineStr" /><c r="I291" s="2" t="inlineStr" /><c r="J291" s="2" t="inlineStr" /><c r="K291" s="2" t="inlineStr"><is><t>u osób starszych preferujemy trójpierścieniowe laki przeciwdepresyjne</t></is></c><c r="L291" s="2" t="inlineStr"><is><t>brak poprawy po 4 tygodniach leczenia sugeruje rozpoznanie depresji lekoopornej</t></is></c><c r="M291" s="2" t="inlineStr" /><c r="N291" s="2" t="inlineStr" /><c r="O291" s="2" t="inlineStr" /><c r="P291" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q291" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="292"><c r="A292" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B292" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C292" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D292" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E292" s="2" t="inlineStr"><is><t>Działanie przeciwkaszlowe wykazuje:</t></is></c><c r="F292" s="2" t="inlineStr"><is><t>dekstrometorfan</t></is></c><c r="G292" s="2" t="inlineStr"><is><t>kodeina</t></is></c><c r="H292" s="2" t="inlineStr" /><c r="I292" s="2" t="inlineStr" /><c r="J292" s="2" t="inlineStr" /><c r="K292" s="2" t="inlineStr"><is><t>loperamid</t></is></c><c r="L292" s="2" t="inlineStr"><is><t>prometazyna</t></is></c><c r="M292" s="2" t="inlineStr" /><c r="N292" s="2" t="inlineStr" /><c r="O292" s="2" t="inlineStr" /><c r="P292" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q292" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="293"><c r="A293" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B293" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C293" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D293" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E293" s="2" t="inlineStr"><is><t>Atropina jest stosowana w przypadku zatrucia:</t></is></c><c r="F293" s="2" t="inlineStr"><is><t>grzybami strzępiakami i lejkówkami</t></is></c><c r="G293" s="2" t="inlineStr"><is><t>glikozydami naparstnicy</t></is></c><c r="H293" s="2" t="inlineStr"><is><t>związkami fosforoorganicznymi</t></is></c><c r="I293" s="2" t="inlineStr" /><c r="J293" s="2" t="inlineStr" /><c r="K293" s="2" t="inlineStr"><is><t>pokrzykiem wilczą jagodą</t></is></c><c r="L293" s="2" t="inlineStr" /><c r="M293" s="2" t="inlineStr" /><c r="N293" s="2" t="inlineStr" /><c r="O293" s="2" t="inlineStr" /><c r="P293" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q293" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="294"><c r="A294" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B294" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C294" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D294" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E294" s="2" t="inlineStr"><is><t>W porównaniu do osób dorosłych w populacji pediatrycznej:</t></is></c><c r="F294" s="2" t="inlineStr"><is><t>zmieniona reakcja na leki jest uwarunkowana przede wszystkim zmianami w farmakokinetyce leków</t></is></c><c r="G294" s="2" t="inlineStr"><is><t>do osiągnięcia stężenia terapeutycznego leku mogą wystarczyć w pierwszym kwartale życia (w przeliczeniu na masę ciała) mniejsze dawki leku</t></is></c><c r="H294" s="2" t="inlineStr"><is><t>w pierwszym półroczu życia leki wydalane przez nerki są eliminowane wolniej, a ich biologiczny okres półtrwania jest dłuższy</t></is></c><c r="I294" s="2" t="inlineStr"><is><t>w pierwszym roku życia frakcja wolna leku może być większa</t></is></c><c r="J294" s="2" t="inlineStr" /><c r="K294" s="2" t="inlineStr" /><c r="L294" s="2" t="inlineStr" /><c r="M294" s="2" t="inlineStr" /><c r="N294" s="2" t="inlineStr" /><c r="O294" s="2" t="inlineStr" /><c r="P294" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q294" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="295"><c r="A295" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B295" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C295" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D295" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E295" s="2" t="inlineStr"><is><t>Inhibitory fosfodiesterazy typu 5:</t></is></c><c r="F295" s="2" t="inlineStr"><is><t>są skuteczne w leczeniu zaburzeń erekcji</t></is></c><c r="G295" s="2" t="inlineStr"><is><t>nie mogą być przyjmowane jednocześnie z azotanami z uwagi na duże ryzyko wystąpienia ciężkiej, niekorygowalnej hipotonii</t></is></c><c r="H295" s="2" t="inlineStr" /><c r="I295" s="2" t="inlineStr" /><c r="J295" s="2" t="inlineStr" /><c r="K295" s="2" t="inlineStr"><is><t>wydłużają dystans marszu bez bólu u pacjentów z chromaniem przestankowym</t></is></c><c r="L295" s="2" t="inlineStr"><is><t>mają działanie inotropowe dodatnie</t></is></c><c r="M295" s="2" t="inlineStr" /><c r="N295" s="2" t="inlineStr" /><c r="O295" s="2" t="inlineStr" /><c r="P295" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q295" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="296"><c r="A296" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B296" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C296" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D296" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E296" s="2" t="inlineStr"><is><t>Wpływ rozkurczający na mięśniówkę przewodu pokarmowego ma:</t></is></c><c r="F296" s="2" t="inlineStr"><is><t>drotaweryna</t></is></c><c r="G296" s="2" t="inlineStr" /><c r="H296" s="2" t="inlineStr" /><c r="I296" s="2" t="inlineStr" /><c r="J296" s="2" t="inlineStr" /><c r="K296" s="2" t="inlineStr"><is><t>itopryd</t></is></c><c r="L296" s="2" t="inlineStr"><is><t>mesalazyna</t></is></c><c r="M296" s="2" t="inlineStr"><is><t>ryfaksymina</t></is></c><c r="N296" s="2" t="inlineStr" /><c r="O296" s="2" t="inlineStr" /><c r="P296" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q296" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="297"><c r="A297" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B297" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C297" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D297" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E297" s="2" t="inlineStr"><is><t>Lanzoprazol stosowany przewlekle powoduje:</t></is></c><c r="F297" s="2" t="inlineStr"><is><t>wzrost ryzyka zakażenia Clostridum difficile</t></is></c><c r="G297" s="2" t="inlineStr"><is><t>wzrost ryzyka infekcji dróg oddechowych</t></is></c><c r="H297" s="2" t="inlineStr"><is><t>zmniejszenie wchłaniania wapnia z przewodu pokarmowego</t></is></c><c r="I297" s="2" t="inlineStr"><is><t>zmniejszenie przekształcania klopidogrelu do aktywnych pochodnych</t></is></c><c r="J297" s="2" t="inlineStr" /><c r="K297" s="2" t="inlineStr" /><c r="L297" s="2" t="inlineStr" /><c r="M297" s="2" t="inlineStr" /><c r="N297" s="2" t="inlineStr" /><c r="O297" s="2" t="inlineStr" /><c r="P297" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q297" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="298"><c r="A298" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B298" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C298" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D298" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E298" s="2" t="inlineStr"><is><t>Sposób eradykacji Helicobacter pylori zalecany w Polsce to:</t></is></c><c r="F298" s="2" t="inlineStr"><is><t>podwójna dawka IPP, metronidazol, tetracyklina, cytrynian bizmutu przez 14 dni</t></is></c><c r="G298" s="2" t="inlineStr" /><c r="H298" s="2" t="inlineStr" /><c r="I298" s="2" t="inlineStr" /><c r="J298" s="2" t="inlineStr" /><c r="K298" s="2" t="inlineStr"><is><t>terapia sekwencyjna przez 10 dni - podwójna dawka IPP (inhibitora pompy protonowej) z amoksycyliną (dni 1-5), a następnie z klarytromycyną i metronidazolem (dni 6-10)</t></is></c><c r="L298" s="2" t="inlineStr"><is><t>podwójna dawka IPP, amoksycylina, klarytromycyna przez 10 dni</t></is></c><c r="M298" s="2" t="inlineStr"><is><t>podwójna dawka IPP, amoksycylina, klarytromycyna, metronidazol przez 14 dni</t></is></c><c r="N298" s="2" t="inlineStr" /><c r="O298" s="2" t="inlineStr" /><c r="P298" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q298" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="299"><c r="A299" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B299" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C299" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D299" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E299" s="2" t="inlineStr"><is><t>Udokumentowane działanie teratogenne wykazuje:</t></is></c><c r="F299" s="2" t="inlineStr"><is><t>trimetoprim-sulfametoksazol</t></is></c><c r="G299" s="2" t="inlineStr"><is><t>warfaryna</t></is></c><c r="H299" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="I299" s="2" t="inlineStr"><is><t>gentamycyna</t></is></c><c r="J299" s="2" t="inlineStr" /><c r="K299" s="2" t="inlineStr" /><c r="L299" s="2" t="inlineStr" /><c r="M299" s="2" t="inlineStr" /><c r="N299" s="2" t="inlineStr" /><c r="O299" s="2" t="inlineStr" /><c r="P299" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q299" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="300"><c r="A300" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B300" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C300" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D300" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E300" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – odtrutka:</t></is></c><c r="F300" s="2" t="inlineStr"><is><t>oksazepam - flumazenil</t></is></c><c r="G300" s="2" t="inlineStr"><is><t>trójpierścieniowe leki przeciwdepresyjne – wodorowęglan sodu</t></is></c><c r="H300" s="2" t="inlineStr"><is><t>żelazo - deferoksamina</t></is></c><c r="I300" s="2" t="inlineStr"><is><t>warfaryna - fitomenadion</t></is></c><c r="J300" s="2" t="inlineStr" /><c r="K300" s="2" t="inlineStr" /><c r="L300" s="2" t="inlineStr" /><c r="M300" s="2" t="inlineStr" /><c r="N300" s="2" t="inlineStr" /><c r="O300" s="2" t="inlineStr" /><c r="P300" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q300" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="301"><c r="A301" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B301" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C301" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D301" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E301" s="2" t="inlineStr"><is><t>Wazodylatacyjny mechanizm działania azotanów zależy od:</t></is></c><c r="F301" s="2" t="inlineStr"><is><t>wzrostu stężenia cGMP</t></is></c><c r="G301" s="2" t="inlineStr"><is><t>defosforylacji łańcuchów lekkich miozyny</t></is></c><c r="H301" s="2" t="inlineStr" /><c r="I301" s="2" t="inlineStr" /><c r="J301" s="2" t="inlineStr" /><c r="K301" s="2" t="inlineStr"><is><t>hamowania aktywności cyklazy guanylowej</t></is></c><c r="L301" s="2" t="inlineStr"><is><t>pobudzania kanałów potasowych</t></is></c><c r="M301" s="2" t="inlineStr" /><c r="N301" s="2" t="inlineStr" /><c r="O301" s="2" t="inlineStr" /><c r="P301" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q301" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="302"><c r="A302" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B302" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C302" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D302" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E302" s="2" t="inlineStr"><is><t>Bradykardia może wystąpić po zastosowaniu:</t></is></c><c r="F302" s="2" t="inlineStr"><is><t>werapamilu</t></is></c><c r="G302" s="2" t="inlineStr" /><c r="H302" s="2" t="inlineStr" /><c r="I302" s="2" t="inlineStr" /><c r="J302" s="2" t="inlineStr" /><c r="K302" s="2" t="inlineStr"><is><t>nifedypiny</t></is></c><c r="L302" s="2" t="inlineStr"><is><t>trimetazydyny</t></is></c><c r="M302" s="2" t="inlineStr"><is><t>spironolaktonu</t></is></c><c r="N302" s="2" t="inlineStr" /><c r="O302" s="2" t="inlineStr" /><c r="P302" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q302" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="303"><c r="A303" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B303" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C303" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D303" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E303" s="2" t="inlineStr"><is><t>Teoretyczną przesłanką stosowania beta-adrenolityków w chorobie wieńcowej serca jest:</t></is></c><c r="F303" s="2" t="inlineStr"><is><t>usprawnienie metabolizmu kardiomiocytów</t></is></c><c r="G303" s="2" t="inlineStr"><is><t>zapobieganie proarytmicznemu działaniu katecholamin</t></is></c><c r="H303" s="2" t="inlineStr"><is><t>poprawa perfuzji warstwy podwsierdziowej</t></is></c><c r="I303" s="2" t="inlineStr"><is><t>korzystny wpływ hemodynamiczny zmniejszający zapotrzebowanie mięśnia sercowego na tlen</t></is></c><c r="J303" s="2" t="inlineStr" /><c r="K303" s="2" t="inlineStr" /><c r="L303" s="2" t="inlineStr" /><c r="M303" s="2" t="inlineStr" /><c r="N303" s="2" t="inlineStr" /><c r="O303" s="2" t="inlineStr" /><c r="P303" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q303" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="304"><c r="A304" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B304" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C304" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D304" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E304" s="2" t="inlineStr"><is><t>Do leków stosowanych w leczeniu nadciśnienia tętniczego ze wskazań naglących (RR&gt;180/120 mmHg z powikłaniami narządowymi) należą:</t></is></c><c r="F304" s="2" t="inlineStr"><is><t>esmolol</t></is></c><c r="G304" s="2" t="inlineStr"><is><t>urapidyl</t></is></c><c r="H304" s="2" t="inlineStr" /><c r="I304" s="2" t="inlineStr" /><c r="J304" s="2" t="inlineStr" /><c r="K304" s="2" t="inlineStr"><is><t>doksazosyna</t></is></c><c r="L304" s="2" t="inlineStr"><is><t>kaptopryl</t></is></c><c r="M304" s="2" t="inlineStr" /><c r="N304" s="2" t="inlineStr" /><c r="O304" s="2" t="inlineStr" /><c r="P304" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q304" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="305"><c r="A305" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B305" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C305" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D305" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E305" s="2" t="inlineStr"><is><t>Do leków zmniejszających ryzyko zgonu sercowo-naczyniowego w przebiegu skurczowej niewydolności serca należy:</t></is></c><c r="F305" s="2" t="inlineStr"><is><t>bisoprolol</t></is></c><c r="G305" s="2" t="inlineStr"><is><t>eplerenon</t></is></c><c r="H305" s="2" t="inlineStr"><is><t>sakubitril w skojarzeniu z walsartanem</t></is></c><c r="I305" s="2" t="inlineStr" /><c r="J305" s="2" t="inlineStr" /><c r="K305" s="2" t="inlineStr"><is><t>digoksyna</t></is></c><c r="L305" s="2" t="inlineStr" /><c r="M305" s="2" t="inlineStr" /><c r="N305" s="2" t="inlineStr" /><c r="O305" s="2" t="inlineStr" /><c r="P305" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q305" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="306"><c r="A306" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B306" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C306" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D306" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E306" s="2" t="inlineStr"><is><t>U 67-letniej kobiety z dyskomfortem zamostkowym występującym przy wchodzeniu na 3 piętro i ustępującym w spoczynku, z blokiem przedsionkowo-komorowym II stopnia typu Mobitza w badaniu met. Holtera należy zastosować:</t></is></c><c r="F306" s="2" t="inlineStr"><is><t>rosuwastatynę</t></is></c><c r="G306" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="H306" s="2" t="inlineStr"><is><t>triazotan glicerolu w aerozolu</t></is></c><c r="I306" s="2" t="inlineStr" /><c r="J306" s="2" t="inlineStr" /><c r="K306" s="2" t="inlineStr"><is><t>nebiwolol</t></is></c><c r="L306" s="2" t="inlineStr" /><c r="M306" s="2" t="inlineStr" /><c r="N306" s="2" t="inlineStr" /><c r="O306" s="2" t="inlineStr" /><c r="P306" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q306" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="307"><c r="A307" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B307" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C307" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D307" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E307" s="2" t="inlineStr"><is><t>Wskaż prawidłowe zasady prowadzenia terapii monitorowanej stężeniami leku:</t></is></c><c r="F307" s="2" t="inlineStr"><is><t>oznaczenia należy wykonywać po osiągnięciu przez lek stanu stacjonarnego</t></is></c><c r="G307" s="2" t="inlineStr"><is><t>pomiary należy wykonywać w momencie Cmin, czyli tuż przed podaniem kolejnej, zwykle porannej dawki leku</t></is></c><c r="H307" s="2" t="inlineStr"><is><t>w większości przypadków wystarczy oznaczenie całkowitego stężenia leku</t></is></c><c r="I307" s="2" t="inlineStr"><is><t>w przypadku leków o kinetyce liniowej można wyliczyć modyfikację dawki na podstawie pomiarów aktualnych i znajomości docelowych stężeń leku we krwi</t></is></c><c r="J307" s="2" t="inlineStr" /><c r="K307" s="2" t="inlineStr" /><c r="L307" s="2" t="inlineStr" /><c r="M307" s="2" t="inlineStr" /><c r="N307" s="2" t="inlineStr" /><c r="O307" s="2" t="inlineStr" /><c r="P307" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q307" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="308"><c r="A308" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B308" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C308" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D308" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E308" s="2" t="inlineStr"><is><t>W celu oceny działań niepożądanych w trakcie leczenia atorwastatyną należy sprawdzić:</t></is></c><c r="F308" s="2" t="inlineStr"><is><t>aktywność kinazy fosfokreatynowej (CPK)</t></is></c><c r="G308" s="2" t="inlineStr"><is><t>aktywność enzymów wątrobowych (AST/ALT)</t></is></c><c r="H308" s="2" t="inlineStr" /><c r="I308" s="2" t="inlineStr" /><c r="J308" s="2" t="inlineStr" /><c r="K308" s="2" t="inlineStr"><is><t>stężenie glukozy</t></is></c><c r="L308" s="2" t="inlineStr"><is><t>stężenie peptydu natriuretycznego typu B (BNP)</t></is></c><c r="M308" s="2" t="inlineStr" /><c r="N308" s="2" t="inlineStr" /><c r="O308" s="2" t="inlineStr" /><c r="P308" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q308" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="309"><c r="A309" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B309" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C309" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D309" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E309" s="2" t="inlineStr"><is><t>W leczeniu zagrażającej życiu hiperkaliemii można zastosować:</t></is></c><c r="F309" s="2" t="inlineStr"><is><t>10 ml 10% chlorku lub glukonianu wapnia i.v. w 10 min bolusie</t></is></c><c r="G309" s="2" t="inlineStr"><is><t>500 ml 20% glukozy z 20 j.m. insuliny krótkodziałającej i.v. przez 1-2 godziny</t></is></c><c r="H309" s="2" t="inlineStr"><is><t>hemodializę</t></is></c><c r="I309" s="2" t="inlineStr" /><c r="J309" s="2" t="inlineStr" /><c r="K309" s="2" t="inlineStr"><is><t>diuretyki pętlowe i.v</t></is></c><c r="L309" s="2" t="inlineStr" /><c r="M309" s="2" t="inlineStr" /><c r="N309" s="2" t="inlineStr" /><c r="O309" s="2" t="inlineStr" /><c r="P309" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q309" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="310"><c r="A310" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B310" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C310" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D310" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E310" s="2" t="inlineStr"><is><t>Powinowactwo do receptorów alfa-1-adrenergicznych wykazuje:</t></is></c><c r="F310" s="2" t="inlineStr"><is><t>doksazosyna</t></is></c><c r="G310" s="2" t="inlineStr"><is><t>labetalol</t></is></c><c r="H310" s="2" t="inlineStr"><is><t>adrenalina</t></is></c><c r="I310" s="2" t="inlineStr"><is><t>karwedilol</t></is></c><c r="J310" s="2" t="inlineStr" /><c r="K310" s="2" t="inlineStr" /><c r="L310" s="2" t="inlineStr" /><c r="M310" s="2" t="inlineStr" /><c r="N310" s="2" t="inlineStr" /><c r="O310" s="2" t="inlineStr" /><c r="P310" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q310" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="311"><c r="A311" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B311" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C311" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D311" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E311" s="2" t="inlineStr"><is><t>Apiksaban jest substratem dla P-gp. Co to oznacza?</t></is></c><c r="F311" s="2" t="inlineStr"><is><t>silne induktory P-gp o działaniu ogólnoustrojowym zmniejszają skuteczność apiksabanu</t></is></c><c r="G311" s="2" t="inlineStr" /><c r="H311" s="2" t="inlineStr" /><c r="I311" s="2" t="inlineStr" /><c r="J311" s="2" t="inlineStr" /><c r="K311" s="2" t="inlineStr"><is><t>lek jest wchłaniany z p. pokarmowego z wykorzystaniem transportu ułatwionego</t></is></c><c r="L311" s="2" t="inlineStr"><is><t>jest metabolizowany w wątrobie i nie powinien być stosowany u osób z 10- 15 pkt wg skali Childa-Pugha</t></is></c><c r="M311" s="2" t="inlineStr"><is><t>jest prawdopodobne, że hemodializa byłaby skutecznym środkiem zaradczym podczas przedawkowania apiksabanu</t></is></c><c r="N311" s="2" t="inlineStr" /><c r="O311" s="2" t="inlineStr" /><c r="P311" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q311" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="312"><c r="A312" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B312" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C312" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D312" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E312" s="2" t="inlineStr"><is><t>Opis rzedowości procesu:</t></is></c><c r="F312" s="2" t="inlineStr"><is><t>Dotyczy wszystkich etapów farmakokinetycznych</t></is></c><c r="G312" s="2" t="inlineStr"><is><t>Definiuje dynamiki zmian w układzie stężenie-czas w zależności od budowy chemicznej leku</t></is></c><c r="H312" s="2" t="inlineStr"><is><t>Może się zmienić dla leku w trakcie pojedynczej ekspozycji</t></is></c><c r="I312" s="2" t="inlineStr"><is><t>Powstaje ostatecznie w badaniach w medelu zwierzęcym</t></is></c><c r="J312" s="2" t="inlineStr" /><c r="K312" s="2" t="inlineStr" /><c r="L312" s="2" t="inlineStr" /><c r="M312" s="2" t="inlineStr" /><c r="N312" s="2" t="inlineStr" /><c r="O312" s="2" t="inlineStr" /><c r="P312" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q312" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="313"><c r="A313" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B313" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C313" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D313" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E313" s="2" t="inlineStr"><is><t>Jeśli proces eliminacji leku przez nerki jest opisany kinetyką zerowego rzędu to:</t></is></c><c r="F313" s="2" t="inlineStr"><is><t>Procesy wchłaniania i dystrybucji również opisane są kinetyką zerowego rzędu</t></is></c><c r="G313" s="2" t="inlineStr"><is><t>Szybkość procesu eliminacji nerkowej jest stała</t></is></c><c r="H313" s="2" t="inlineStr" /><c r="I313" s="2" t="inlineStr" /><c r="J313" s="2" t="inlineStr" /><c r="K313" s="2" t="inlineStr"><is><t>Stężenie leku w moczu jest odwrotnie proporocjonalne do stężenia leku we krwi</t></is></c><c r="L313" s="2" t="inlineStr"><is><t>Klirens nerkowy leku jest wprost proporcjonalny do stężeniu leku</t></is></c><c r="M313" s="2" t="inlineStr" /><c r="N313" s="2" t="inlineStr" /><c r="O313" s="2" t="inlineStr" /><c r="P313" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q313" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="314"><c r="A314" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B314" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C314" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D314" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E314" s="2" t="inlineStr"><is><t>Wskaż właściwie zdefiniowane parametry farmakokinetyczne</t></is></c><c r="F314" s="2" t="inlineStr"><is><t>AUC – pole pod krzywą zmian stężenia leku we krwi w czasie</t></is></c><c r="G314" s="2" t="inlineStr" /><c r="H314" s="2" t="inlineStr" /><c r="I314" s="2" t="inlineStr" /><c r="J314" s="2" t="inlineStr" /><c r="K314" s="2" t="inlineStr"><is><t>T1/2 – czas po którym stężenie leku we krwi jest równe stężeniu leku gdyby biodostępność wynosiła 50%</t></is></c><c r="L314" s="2" t="inlineStr"><is><t>Tmax – maksymalny czas w którym stężeniu leku we krwi jest wykrywalne</t></is></c><c r="M314" s="2" t="inlineStr"><is><t>Cmax – stężenie leku we krwi osiągane po podaniu dożylnym</t></is></c><c r="N314" s="2" t="inlineStr" /><c r="O314" s="2" t="inlineStr" /><c r="P314" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q314" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="315"><c r="A315" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B315" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C315" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D315" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E315" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie antybiotyk – mechanizm działania</t></is></c><c r="F315" s="2" t="inlineStr"><is><t>Trimetoprim – zaburzenia kwasu foliowego</t></is></c><c r="G315" s="2" t="inlineStr"><is><t>Amikacyna – hamowanie syntezy białek</t></is></c><c r="H315" s="2" t="inlineStr"><is><t>Cyprofloksacyna – hamowanie replikacji DNA</t></is></c><c r="I315" s="2" t="inlineStr" /><c r="J315" s="2" t="inlineStr" /><c r="K315" s="2" t="inlineStr"><is><t>Klindamycyna – hamowanie transkrypcji genów translacji</t></is></c><c r="L315" s="2" t="inlineStr" /><c r="M315" s="2" t="inlineStr" /><c r="N315" s="2" t="inlineStr" /><c r="O315" s="2" t="inlineStr" /><c r="P315" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q315" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="316"><c r="A316" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B316" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C316" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D316" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E316" s="2" t="inlineStr"><is><t>Azytromycyna</t></is></c><c r="F316" s="2" t="inlineStr"><is><t>Kumuluje się w makrofagach</t></is></c><c r="G316" s="2" t="inlineStr"><is><t>Ma długi okres półtrwania</t></is></c><c r="H316" s="2" t="inlineStr" /><c r="I316" s="2" t="inlineStr" /><c r="J316" s="2" t="inlineStr" /><c r="K316" s="2" t="inlineStr"><is><t>Słabo wchłania się z PP</t></is></c><c r="L316" s="2" t="inlineStr"><is><t>Hamuje enzymy cytochromu P-450</t></is></c><c r="M316" s="2" t="inlineStr" /><c r="N316" s="2" t="inlineStr" /><c r="O316" s="2" t="inlineStr" /><c r="P316" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q316" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="317"><c r="A317" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B317" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C317" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D317" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E317" s="2" t="inlineStr"><is><t>Azytromycyna:</t></is></c><c r="F317" s="2" t="inlineStr"><is><t>jest stosowana w nierzeżączkowym zapaleniu cewki moczowej</t></is></c><c r="G317" s="2" t="inlineStr" /><c r="H317" s="2" t="inlineStr" /><c r="I317" s="2" t="inlineStr" /><c r="J317" s="2" t="inlineStr" /><c r="K317" s="2" t="inlineStr"><is><t>jest słabo wchłaniana z przewodu pokarmowego</t></is></c><c r="L317" s="2" t="inlineStr"><is><t>ma bardzo krótki okres półtrwania</t></is></c><c r="M317" s="2" t="inlineStr"><is><t>istotnie klinicznie hamuje aktywność izoenzymu CYP3A4</t></is></c><c r="N317" s="2" t="inlineStr" /><c r="O317" s="2" t="inlineStr" /><c r="P317" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q317" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="318"><c r="A318" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B318" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C318" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D318" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E318" s="2" t="inlineStr"><is><t>Działanie ototoksyczne wskazują</t></is></c><c r="F318" s="2" t="inlineStr"><is><t>Salicylany</t></is></c><c r="G318" s="2" t="inlineStr"><is><t>Aminoglikozydy</t></is></c><c r="H318" s="2" t="inlineStr" /><c r="I318" s="2" t="inlineStr" /><c r="J318" s="2" t="inlineStr" /><c r="K318" s="2" t="inlineStr"><is><t>Glitazony</t></is></c><c r="L318" s="2" t="inlineStr"><is><t>Penicyliny</t></is></c><c r="M318" s="2" t="inlineStr" /><c r="N318" s="2" t="inlineStr" /><c r="O318" s="2" t="inlineStr" /><c r="P318" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q318" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="319"><c r="A319" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B319" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C319" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D319" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E319" s="2" t="inlineStr"><is><t>W leczeniu boreliozy można użyć</t></is></c><c r="F319" s="2" t="inlineStr"><is><t>Amoksycyliny</t></is></c><c r="G319" s="2" t="inlineStr"><is><t>Cefuroksymu aksetylu</t></is></c><c r="H319" s="2" t="inlineStr"><is><t>Azytromycyny</t></is></c><c r="I319" s="2" t="inlineStr"><is><t>Doksycykliny</t></is></c><c r="J319" s="2" t="inlineStr" /><c r="K319" s="2" t="inlineStr" /><c r="L319" s="2" t="inlineStr" /><c r="M319" s="2" t="inlineStr" /><c r="N319" s="2" t="inlineStr" /><c r="O319" s="2" t="inlineStr" /><c r="P319" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q319" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="320"><c r="A320" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B320" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C320" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D320" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E320" s="2" t="inlineStr"><is><t>Syntezę ściany komórkowej hamuje</t></is></c><c r="F320" s="2" t="inlineStr"><is><t>Imipenem</t></is></c><c r="G320" s="2" t="inlineStr"><is><t>Wankomycyna</t></is></c><c r="H320" s="2" t="inlineStr" /><c r="I320" s="2" t="inlineStr" /><c r="J320" s="2" t="inlineStr" /><c r="K320" s="2" t="inlineStr"><is><t>Erytromycyna</t></is></c><c r="L320" s="2" t="inlineStr"><is><t>Mupirocyna</t></is></c><c r="M320" s="2" t="inlineStr" /><c r="N320" s="2" t="inlineStr" /><c r="O320" s="2" t="inlineStr" /><c r="P320" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q320" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="321"><c r="A321" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B321" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C321" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D321" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E321" s="2" t="inlineStr"><is><t>Syntezę ściany komórkowej hamuje:</t></is></c><c r="F321" s="2" t="inlineStr"><is><t>Kaspofungina</t></is></c><c r="G321" s="2" t="inlineStr"><is><t>Imipenem</t></is></c><c r="H321" s="2" t="inlineStr" /><c r="I321" s="2" t="inlineStr" /><c r="J321" s="2" t="inlineStr" /><c r="K321" s="2" t="inlineStr"><is><t>Nystatyna</t></is></c><c r="L321" s="2" t="inlineStr"><is><t>Tygecyklina</t></is></c><c r="M321" s="2" t="inlineStr" /><c r="N321" s="2" t="inlineStr" /><c r="O321" s="2" t="inlineStr" /><c r="P321" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q321" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="322"><c r="A322" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B322" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C322" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D322" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E322" s="2" t="inlineStr"><is><t>Syntezę ściany komórkowej hamuje:</t></is></c><c r="F322" s="2" t="inlineStr"><is><t>fosfomycyna</t></is></c><c r="G322" s="2" t="inlineStr"><is><t>mykafungina</t></is></c><c r="H322" s="2" t="inlineStr"><is><t>teikoplanina</t></is></c><c r="I322" s="2" t="inlineStr" /><c r="J322" s="2" t="inlineStr" /><c r="K322" s="2" t="inlineStr"><is><t>nystatyna</t></is></c><c r="L322" s="2" t="inlineStr" /><c r="M322" s="2" t="inlineStr" /><c r="N322" s="2" t="inlineStr" /><c r="O322" s="2" t="inlineStr" /><c r="P322" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q322" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="323"><c r="A323" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B323" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C323" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D323" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E323" s="2" t="inlineStr"><is><t>Reakcje disulfiramową może spowodować spożycie alkoholu podczas terapii</t></is></c><c r="F323" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="G323" s="2" t="inlineStr" /><c r="H323" s="2" t="inlineStr" /><c r="I323" s="2" t="inlineStr" /><c r="J323" s="2" t="inlineStr" /><c r="K323" s="2" t="inlineStr"><is><t>Klindamycyną</t></is></c><c r="L323" s="2" t="inlineStr"><is><t>Piperalicyna</t></is></c><c r="M323" s="2" t="inlineStr"><is><t>Cyprofloksacyna</t></is></c><c r="N323" s="2" t="inlineStr" /><c r="O323" s="2" t="inlineStr" /><c r="P323" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q323" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="324"><c r="A324" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B324" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C324" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D324" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E324" s="2" t="inlineStr"><is><t>W zakażeniach Mycoplasama pneumoniae można zastosować</t></is></c><c r="F324" s="2" t="inlineStr"><is><t>Doksycykline</t></is></c><c r="G324" s="2" t="inlineStr"><is><t>Klarytromycyne</t></is></c><c r="H324" s="2" t="inlineStr" /><c r="I324" s="2" t="inlineStr" /><c r="J324" s="2" t="inlineStr" /><c r="K324" s="2" t="inlineStr"><is><t>Amoksycyline</t></is></c><c r="L324" s="2" t="inlineStr"><is><t>Ceftriakson</t></is></c><c r="M324" s="2" t="inlineStr" /><c r="N324" s="2" t="inlineStr" /><c r="O324" s="2" t="inlineStr" /><c r="P324" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q324" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="325"><c r="A325" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B325" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C325" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D325" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E325" s="2" t="inlineStr"><is><t>Makrolidy mogą być skuteczne w zakażeniach</t></is></c><c r="F325" s="2" t="inlineStr"><is><t>H. influenza</t></is></c><c r="G325" s="2" t="inlineStr"><is><t>L. pneumophila</t></is></c><c r="H325" s="2" t="inlineStr"><is><t>H. pylori</t></is></c><c r="I325" s="2" t="inlineStr"><is><t>T. gondi</t></is></c><c r="J325" s="2" t="inlineStr" /><c r="K325" s="2" t="inlineStr" /><c r="L325" s="2" t="inlineStr" /><c r="M325" s="2" t="inlineStr" /><c r="N325" s="2" t="inlineStr" /><c r="O325" s="2" t="inlineStr" /><c r="P325" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q325" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="326"><c r="A326" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B326" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C326" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D326" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E326" s="2" t="inlineStr"><is><t>W zakazeniu Clostridium diff. skuteczne sa:</t></is></c><c r="F326" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="G326" s="2" t="inlineStr"><is><t>Wankomycyna</t></is></c><c r="H326" s="2" t="inlineStr" /><c r="I326" s="2" t="inlineStr" /><c r="J326" s="2" t="inlineStr" /><c r="K326" s="2" t="inlineStr"><is><t>Amoksycylina</t></is></c><c r="L326" s="2" t="inlineStr"><is><t>Klindamycyna</t></is></c><c r="M326" s="2" t="inlineStr" /><c r="N326" s="2" t="inlineStr" /><c r="O326" s="2" t="inlineStr" /><c r="P326" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q326" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="327"><c r="A327" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B327" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C327" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D327" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E327" s="2" t="inlineStr"><is><t>Na MRSA działa</t></is></c><c r="F327" s="2" t="inlineStr"><is><t>Wankomycyna</t></is></c><c r="G327" s="2" t="inlineStr"><is><t>Linezolid</t></is></c><c r="H327" s="2" t="inlineStr" /><c r="I327" s="2" t="inlineStr" /><c r="J327" s="2" t="inlineStr" /><c r="K327" s="2" t="inlineStr"><is><t>Cefazolina</t></is></c><c r="L327" s="2" t="inlineStr"><is><t>Meropenem</t></is></c><c r="M327" s="2" t="inlineStr" /><c r="N327" s="2" t="inlineStr" /><c r="O327" s="2" t="inlineStr" /><c r="P327" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q327" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="328"><c r="A328" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B328" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C328" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D328" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E328" s="2" t="inlineStr"><is><t>Zagrożenia dla płodu jest mało prawdopodobne po</t></is></c><c r="F328" s="2" t="inlineStr"><is><t>Amoksycyliny z kwasem klawulanowym</t></is></c><c r="G328" s="2" t="inlineStr"><is><t>Erytromycyny</t></is></c><c r="H328" s="2" t="inlineStr"><is><t>Cefuroksymu</t></is></c><c r="I328" s="2" t="inlineStr" /><c r="J328" s="2" t="inlineStr" /><c r="K328" s="2" t="inlineStr"><is><t>Amikacyny</t></is></c><c r="L328" s="2" t="inlineStr" /><c r="M328" s="2" t="inlineStr" /><c r="N328" s="2" t="inlineStr" /><c r="O328" s="2" t="inlineStr" /><c r="P328" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q328" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="329"><c r="A329" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B329" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C329" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D329" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E329" s="2" t="inlineStr"><is><t>Ketokonazol</t></is></c><c r="F329" s="2" t="inlineStr"><is><t>Jest dostępny w postaci szamponu</t></is></c><c r="G329" s="2" t="inlineStr"><is><t>Ma zostosowanie w zespole Cushinga</t></is></c><c r="H329" s="2" t="inlineStr"><is><t>Wykazuje działanie hepatotoksyczne</t></is></c><c r="I329" s="2" t="inlineStr" /><c r="J329" s="2" t="inlineStr" /><c r="K329" s="2" t="inlineStr"><is><t>Nie wchłania się po podaniu doustnym</t></is></c><c r="L329" s="2" t="inlineStr" /><c r="M329" s="2" t="inlineStr" /><c r="N329" s="2" t="inlineStr" /><c r="O329" s="2" t="inlineStr" /><c r="P329" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q329" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="330"><c r="A330" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B330" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C330" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D330" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E330" s="2" t="inlineStr"><is><t>Do leków i rzutu w gruźlicy należy</t></is></c><c r="F330" s="2" t="inlineStr"><is><t>Ryfampicyna</t></is></c><c r="G330" s="2" t="inlineStr"><is><t>Izoniazyd</t></is></c><c r="H330" s="2" t="inlineStr"><is><t>Pyryzynamid</t></is></c><c r="I330" s="2" t="inlineStr" /><c r="J330" s="2" t="inlineStr" /><c r="K330" s="2" t="inlineStr"><is><t>Kanamycna</t></is></c><c r="L330" s="2" t="inlineStr" /><c r="M330" s="2" t="inlineStr" /><c r="N330" s="2" t="inlineStr" /><c r="O330" s="2" t="inlineStr" /><c r="P330" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q330" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="331"><c r="A331" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B331" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C331" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D331" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E331" s="2" t="inlineStr"><is><t>W farmakoterapii silnego bólu przebijającego stosujemy</t></is></c><c r="F331" s="2" t="inlineStr"><is><t>Morfinę doustnie w dawkach ratunkowych</t></is></c><c r="G331" s="2" t="inlineStr"><is><t>Fentanyl w postaci dopoliczkowej</t></is></c><c r="H331" s="2" t="inlineStr"><is><t>Buprenorfinę podjęzykowo</t></is></c><c r="I331" s="2" t="inlineStr"><is><t>Fentanyl w postaci donosowej</t></is></c><c r="J331" s="2" t="inlineStr" /><c r="K331" s="2" t="inlineStr" /><c r="L331" s="2" t="inlineStr" /><c r="M331" s="2" t="inlineStr" /><c r="N331" s="2" t="inlineStr" /><c r="O331" s="2" t="inlineStr" /><c r="P331" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q331" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="332"><c r="A332" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B332" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C332" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D332" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E332" s="2" t="inlineStr"><is><t>Ośrodkowe działania opioidów obejmują</t></is></c><c r="F332" s="2" t="inlineStr"><is><t>Działanie przeciwkaszlowe</t></is></c><c r="G332" s="2" t="inlineStr"><is><t>Wymioty</t></is></c><c r="H332" s="2" t="inlineStr" /><c r="I332" s="2" t="inlineStr" /><c r="J332" s="2" t="inlineStr" /><c r="K332" s="2" t="inlineStr"><is><t>Zwiększenie ciśnienia w drogach żółciowych</t></is></c><c r="L332" s="2" t="inlineStr"><is><t>Zaparcia</t></is></c><c r="M332" s="2" t="inlineStr" /><c r="N332" s="2" t="inlineStr" /><c r="O332" s="2" t="inlineStr" /><c r="P332" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q332" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="333"><c r="A333" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B333" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C333" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D333" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E333" s="2" t="inlineStr"><is><t>Efekt pułapowy wykazuje</t></is></c><c r="F333" s="2" t="inlineStr"><is><t>Buprenorfina</t></is></c><c r="G333" s="2" t="inlineStr" /><c r="H333" s="2" t="inlineStr" /><c r="I333" s="2" t="inlineStr" /><c r="J333" s="2" t="inlineStr" /><c r="K333" s="2" t="inlineStr"><is><t>Morfina</t></is></c><c r="L333" s="2" t="inlineStr"><is><t>Kodeina</t></is></c><c r="M333" s="2" t="inlineStr"><is><t>Metadon</t></is></c><c r="N333" s="2" t="inlineStr" /><c r="O333" s="2" t="inlineStr" /><c r="P333" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q333" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="334"><c r="A334" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B334" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C334" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D334" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E334" s="2" t="inlineStr"><is><t>Metformina</t></is></c><c r="F334" s="2" t="inlineStr"><is><t>Zaburza wchłanianie witaminy B12</t></is></c><c r="G334" s="2" t="inlineStr"><is><t>Może powodować kwasicę metaboliczną</t></is></c><c r="H334" s="2" t="inlineStr" /><c r="I334" s="2" t="inlineStr" /><c r="J334" s="2" t="inlineStr" /><c r="K334" s="2" t="inlineStr"><is><t>Stymuluje wydzielanie insuliny</t></is></c><c r="L334" s="2" t="inlineStr"><is><t>Powoduje przyrost masy ciała</t></is></c><c r="M334" s="2" t="inlineStr" /><c r="N334" s="2" t="inlineStr" /><c r="O334" s="2" t="inlineStr" /><c r="P334" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q334" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="335"><c r="A335" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B335" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C335" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D335" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E335" s="2" t="inlineStr"><is><t>Metformina:</t></is></c><c r="F335" s="2" t="inlineStr"><is><t>jest wskazana w stanie przedcukrzycowym</t></is></c><c r="G335" s="2" t="inlineStr"><is><t>zmniejsza śmiertelność w cukrzycy typu 2</t></is></c><c r="H335" s="2" t="inlineStr" /><c r="I335" s="2" t="inlineStr" /><c r="J335" s="2" t="inlineStr" /><c r="K335" s="2" t="inlineStr"><is><t>hamuje kanały potasowe zależne od ATP w komórkach B trzustki</t></is></c><c r="L335" s="2" t="inlineStr"><is><t>nie może być stosowana w skojarzeniu z insuliną</t></is></c><c r="M335" s="2" t="inlineStr" /><c r="N335" s="2" t="inlineStr" /><c r="O335" s="2" t="inlineStr" /><c r="P335" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q335" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="336"><c r="A336" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B336" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C336" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D336" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E336" s="2" t="inlineStr"><is><t>Metformina:</t></is></c><c r="F336" s="2" t="inlineStr"><is><t>wpływa korzystnie na profil lipidowy</t></is></c><c r="G336" s="2" t="inlineStr" /><c r="H336" s="2" t="inlineStr" /><c r="I336" s="2" t="inlineStr" /><c r="J336" s="2" t="inlineStr" /><c r="K336" s="2" t="inlineStr"><is><t>powoduje przyrost masy ciała</t></is></c><c r="L336" s="2" t="inlineStr"><is><t>zwiększa ryzyko hipoglikemii</t></is></c><c r="M336" s="2" t="inlineStr"><is><t>może być przyczyną uporczywych zaparć</t></is></c><c r="N336" s="2" t="inlineStr" /><c r="O336" s="2" t="inlineStr" /><c r="P336" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q336" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="337"><c r="A337" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B337" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C337" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D337" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E337" s="2" t="inlineStr"><is><t>Metformina:</t></is></c><c r="F337" s="2" t="inlineStr"><is><t>ma klirens nerkowy i nie powinna być stosowana jeśli eGFR &lt; 30 ml/min</t></is></c><c r="G337" s="2" t="inlineStr"><is><t>aktywuje kinazę AMP, co powoduje zwiększenie beztlenowego metabolizm glukozy w komórkach</t></is></c><c r="H337" s="2" t="inlineStr" /><c r="I337" s="2" t="inlineStr" /><c r="J337" s="2" t="inlineStr" /><c r="K337" s="2" t="inlineStr"><is><t>nie powoduje hipoglikemii u chorych na cukrzycę, ale ma taki efekt u osób bez cukrzycy</t></is></c><c r="L337" s="2" t="inlineStr"><is><t>nie jest skuteczna w zapobieganiu progresji stanu przedcukrzycowego do cukrzycy typu 2</t></is></c><c r="M337" s="2" t="inlineStr" /><c r="N337" s="2" t="inlineStr" /><c r="O337" s="2" t="inlineStr" /><c r="P337" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q337" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="338"><c r="A338" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B338" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C338" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D338" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E338" s="2" t="inlineStr"><is><t>Szybkie analogi insuliny</t></is></c><c r="F338" s="2" t="inlineStr"><is><t>Lispro</t></is></c><c r="G338" s="2" t="inlineStr"><is><t>Aspart</t></is></c><c r="H338" s="2" t="inlineStr" /><c r="I338" s="2" t="inlineStr" /><c r="J338" s="2" t="inlineStr" /><c r="K338" s="2" t="inlineStr"><is><t>Glargina</t></is></c><c r="L338" s="2" t="inlineStr"><is><t>Detemir</t></is></c><c r="M338" s="2" t="inlineStr" /><c r="N338" s="2" t="inlineStr" /><c r="O338" s="2" t="inlineStr" /><c r="P338" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q338" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="339"><c r="A339" s="2" t="inlineStr"><is><t>ANTYKONCEPCJA</t></is></c><c r="B339" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C339" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D339" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E339" s="2" t="inlineStr"><is><t>Działania niepożądane hormonalnych środków antykoncepcyjnych z powodu obecności gestagenu</t></is></c><c r="F339" s="2" t="inlineStr"><is><t>Przyrost masy ciała</t></is></c><c r="G339" s="2" t="inlineStr"><is><t>Obniżenie libido</t></is></c><c r="H339" s="2" t="inlineStr"><is><t>Depresja</t></is></c><c r="I339" s="2" t="inlineStr"><is><t>Hirsutyzm</t></is></c><c r="J339" s="2" t="inlineStr" /><c r="K339" s="2" t="inlineStr" /><c r="L339" s="2" t="inlineStr" /><c r="M339" s="2" t="inlineStr" /><c r="N339" s="2" t="inlineStr" /><c r="O339" s="2" t="inlineStr" /><c r="P339" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q339" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="340"><c r="A340" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B340" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C340" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D340" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E340" s="2" t="inlineStr"><is><t>Hiperprolaktynemia</t></is></c><c r="F340" s="2" t="inlineStr"><is><t>Karbegolina</t></is></c><c r="G340" s="2" t="inlineStr"><is><t>Bromokryptyna</t></is></c><c r="H340" s="2" t="inlineStr" /><c r="I340" s="2" t="inlineStr" /><c r="J340" s="2" t="inlineStr" /><c r="K340" s="2" t="inlineStr"><is><t>Gorserelina</t></is></c><c r="L340" s="2" t="inlineStr"><is><t>Finasteryd</t></is></c><c r="M340" s="2" t="inlineStr" /><c r="N340" s="2" t="inlineStr" /><c r="O340" s="2" t="inlineStr" /><c r="P340" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q340" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="341"><c r="A341" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B341" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C341" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D341" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E341" s="2" t="inlineStr"><is><t>Terapia cukrzycy typu 2 podskórnie</t></is></c><c r="F341" s="2" t="inlineStr"><is><t>Detemir</t></is></c><c r="G341" s="2" t="inlineStr" /><c r="H341" s="2" t="inlineStr" /><c r="I341" s="2" t="inlineStr" /><c r="J341" s="2" t="inlineStr" /><c r="K341" s="2" t="inlineStr"><is><t>Glipizyd</t></is></c><c r="L341" s="2" t="inlineStr"><is><t>Liraglutyd</t></is></c><c r="M341" s="2" t="inlineStr"><is><t>Linagliptyna</t></is></c><c r="N341" s="2" t="inlineStr" /><c r="O341" s="2" t="inlineStr" /><c r="P341" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q341" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="342"><c r="A342" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B342" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C342" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D342" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E342" s="2" t="inlineStr"><is><t>Terapia nadczynności tarczycy</t></is></c><c r="F342" s="2" t="inlineStr"><is><t>Jod radioaktywny</t></is></c><c r="G342" s="2" t="inlineStr"><is><t>Bisoprolol</t></is></c><c r="H342" s="2" t="inlineStr"><is><t>Tiamazol</t></is></c><c r="I342" s="2" t="inlineStr"><is><t>Propylotiouracyl</t></is></c><c r="J342" s="2" t="inlineStr" /><c r="K342" s="2" t="inlineStr" /><c r="L342" s="2" t="inlineStr" /><c r="M342" s="2" t="inlineStr" /><c r="N342" s="2" t="inlineStr" /><c r="O342" s="2" t="inlineStr" /><c r="P342" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q342" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="343"><c r="A343" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B343" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C343" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D343" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E343" s="2" t="inlineStr"><is><t>Podczas terapii GKS może dojsć do pogorszenia przebiegu</t></is></c><c r="F343" s="2" t="inlineStr"><is><t>Cukrzycy</t></is></c><c r="G343" s="2" t="inlineStr"><is><t>Gruźlicy</t></is></c><c r="H343" s="2" t="inlineStr"><is><t>Osteoporozy</t></is></c><c r="I343" s="2" t="inlineStr" /><c r="J343" s="2" t="inlineStr" /><c r="K343" s="2" t="inlineStr"><is><t>Małopłytkowości idiopatycznej</t></is></c><c r="L343" s="2" t="inlineStr" /><c r="M343" s="2" t="inlineStr" /><c r="N343" s="2" t="inlineStr" /><c r="O343" s="2" t="inlineStr" /><c r="P343" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q343" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="344"><c r="A344" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B344" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C344" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D344" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E344" s="2" t="inlineStr"><is><t>Wzrostu ryzyka sercowo-naczyniowego NIE powoduje</t></is></c><c r="F344" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="G344" s="2" t="inlineStr" /><c r="H344" s="2" t="inlineStr" /><c r="I344" s="2" t="inlineStr" /><c r="J344" s="2" t="inlineStr" /><c r="K344" s="2" t="inlineStr"><is><t>Celekoksyb</t></is></c><c r="L344" s="2" t="inlineStr"><is><t>Indometacyna</t></is></c><c r="M344" s="2" t="inlineStr"><is><t>Ketoprofen</t></is></c><c r="N344" s="2" t="inlineStr" /><c r="O344" s="2" t="inlineStr" /><c r="P344" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q344" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="345"><c r="A345" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B345" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C345" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D345" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E345" s="2" t="inlineStr"><is><t>Zmniejszenie ryzyka gastrotoksyczności NLPZ – co możemy</t></is></c><c r="F345" s="2" t="inlineStr"><is><t>Analogi PGE1</t></is></c><c r="G345" s="2" t="inlineStr"><is><t>IPP</t></is></c><c r="H345" s="2" t="inlineStr" /><c r="I345" s="2" t="inlineStr" /><c r="J345" s="2" t="inlineStr" /><c r="K345" s="2" t="inlineStr"><is><t>GKS</t></is></c><c r="L345" s="2" t="inlineStr"><is><t>Preparaty o wybiórczym powinowactwie do COX1</t></is></c><c r="M345" s="2" t="inlineStr" /><c r="N345" s="2" t="inlineStr" /><c r="O345" s="2" t="inlineStr" /><c r="P345" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q345" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="346"><c r="A346" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B346" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C346" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D346" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E346" s="2" t="inlineStr"><is><t>Paracetamol</t></is></c><c r="F346" s="2" t="inlineStr"><is><t>Jest metabolizowany przez enzymy cytochromu P-450</t></is></c><c r="G346" s="2" t="inlineStr" /><c r="H346" s="2" t="inlineStr" /><c r="I346" s="2" t="inlineStr" /><c r="J346" s="2" t="inlineStr" /><c r="K346" s="2" t="inlineStr"><is><t>Działa silnie przeciwzapalnie</t></is></c><c r="L346" s="2" t="inlineStr"><is><t>Hamuje COX2 w OUN</t></is></c><c r="M346" s="2" t="inlineStr"><is><t>Wykazuje działanie gastrotoksyczne</t></is></c><c r="N346" s="2" t="inlineStr" /><c r="O346" s="2" t="inlineStr" /><c r="P346" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q346" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="347"><c r="A347" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B347" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C347" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D347" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E347" s="2" t="inlineStr"><is><t>Paracetamol:</t></is></c><c r="F347" s="2" t="inlineStr"><is><t>u chorych przewlekle niedożywionych może działać hepatotoksycznie</t></is></c><c r="G347" s="2" t="inlineStr" /><c r="H347" s="2" t="inlineStr" /><c r="I347" s="2" t="inlineStr" /><c r="J347" s="2" t="inlineStr" /><c r="K347" s="2" t="inlineStr"><is><t>działa przeciwbólowo i przeciwzapalnie</t></is></c><c r="L347" s="2" t="inlineStr"><is><t>zwiększa ryzyko sercowo-naczyniowe</t></is></c><c r="M347" s="2" t="inlineStr"><is><t>wykazuje działanie teratogenne</t></is></c><c r="N347" s="2" t="inlineStr" /><c r="O347" s="2" t="inlineStr" /><c r="P347" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q347" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="348"><c r="A348" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B348" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C348" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D348" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E348" s="2" t="inlineStr"><is><t>Paracetamol:</t></is></c><c r="F348" s="2" t="inlineStr"><is><t>jest prawdopodobnie słabym niewybiórczym inhibitorem cyklooksygenaz (COX), ale bez działania przeciwzapalnego</t></is></c><c r="G348" s="2" t="inlineStr"><is><t>via aktywny metabolit hamuje wychwyt zwrotny endokanabinoidów</t></is></c><c r="H348" s="2" t="inlineStr"><is><t>ma maksymalną dawkę dobową ustaloną na 4 g/d (a u osób z zespołem zależności alkoholowej na 2 g/d)</t></is></c><c r="I348" s="2" t="inlineStr" /><c r="J348" s="2" t="inlineStr" /><c r="K348" s="2" t="inlineStr"><is><t>po przedawkowaniu jest antagonizowany przez dożylne wlewy glutationu (GSH)</t></is></c><c r="L348" s="2" t="inlineStr" /><c r="M348" s="2" t="inlineStr" /><c r="N348" s="2" t="inlineStr" /><c r="O348" s="2" t="inlineStr" /><c r="P348" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q348" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="349"><c r="A349" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B349" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C349" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D349" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E349" s="2" t="inlineStr"><is><t>Leki immunosupresyjne</t></is></c><c r="F349" s="2" t="inlineStr"><is><t>Powodują upośledzenie odporności komórkowej</t></is></c><c r="G349" s="2" t="inlineStr"><is><t>Są lekami o wąskim wskaźniku terapeutycznym</t></is></c><c r="H349" s="2" t="inlineStr" /><c r="I349" s="2" t="inlineStr" /><c r="J349" s="2" t="inlineStr" /><c r="K349" s="2" t="inlineStr"><is><t>Zapobiegają rozwojowi nowotworów</t></is></c><c r="L349" s="2" t="inlineStr"><is><t>Znajdują zastosowanie w terapii chorób neurodegeneracyjnych</t></is></c><c r="M349" s="2" t="inlineStr" /><c r="N349" s="2" t="inlineStr" /><c r="O349" s="2" t="inlineStr" /><c r="P349" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q349" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="350"><c r="A350" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B350" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C350" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D350" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E350" s="2" t="inlineStr"><is><t>Wskaż prawidłowe pary lek – wskazanie</t></is></c><c r="F350" s="2" t="inlineStr"><is><t>Bromoheksyna – astma oskrzelowa</t></is></c><c r="G350" s="2" t="inlineStr" /><c r="H350" s="2" t="inlineStr" /><c r="I350" s="2" t="inlineStr" /><c r="J350" s="2" t="inlineStr" /><c r="K350" s="2" t="inlineStr"><is><t>Acetylocysteina – ostre zapalenie zatok obocznych nosa</t></is></c><c r="L350" s="2" t="inlineStr"><is><t>Dornaza alfa – sarkoidoza</t></is></c><c r="M350" s="2" t="inlineStr"><is><t>Ambroksol – infekcyjne zaostrzenie POChP</t></is></c><c r="N350" s="2" t="inlineStr" /><c r="O350" s="2" t="inlineStr" /><c r="P350" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q350" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="351"><c r="A351" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B351" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C351" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D351" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E351" s="2" t="inlineStr"><is><t>W celu przerwania ataku duszności Zależy jakiej dusznosći. Duszności przygodnej będą same SABA, jak mamy zaostrzenie astmy to GKS też</t></is></c><c r="F351" s="2" t="inlineStr"><is><t>Fenoterol</t></is></c><c r="G351" s="2" t="inlineStr"><is><t>Salbutamol</t></is></c><c r="H351" s="2" t="inlineStr" /><c r="I351" s="2" t="inlineStr" /><c r="J351" s="2" t="inlineStr" /><c r="K351" s="2" t="inlineStr"><is><t>Salmeterol</t></is></c><c r="L351" s="2" t="inlineStr"><is><t>Flutikazon</t></is></c><c r="M351" s="2" t="inlineStr" /><c r="N351" s="2" t="inlineStr" /><c r="O351" s="2" t="inlineStr" /><c r="P351" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q351" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="352"><c r="A352" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B352" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C352" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D352" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E352" s="2" t="inlineStr"><is><t>Omalizumab</t></is></c><c r="F352" s="2" t="inlineStr"><is><t>Blokuje łączenie IgE z komórkami tucznymi</t></is></c><c r="G352" s="2" t="inlineStr"><is><t>Zmniejsza liczbę zaostrzeń astmy</t></is></c><c r="H352" s="2" t="inlineStr" /><c r="I352" s="2" t="inlineStr" /><c r="J352" s="2" t="inlineStr" /><c r="K352" s="2" t="inlineStr"><is><t>Stosowany jest w astmie o umiarkowanej ciężkości</t></is></c><c r="L352" s="2" t="inlineStr"><is><t>Zwiększa zapotrzebowanie na GKS</t></is></c><c r="M352" s="2" t="inlineStr" /><c r="N352" s="2" t="inlineStr" /><c r="O352" s="2" t="inlineStr" /><c r="P352" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q352" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="353"><c r="A353" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B353" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C353" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D353" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E353" s="2" t="inlineStr"><is><t>Farmakoterapia POChP kategoria A i B</t></is></c><c r="F353" s="2" t="inlineStr"><is><t>Krótko i długo działające cholinolityki</t></is></c><c r="G353" s="2" t="inlineStr"><is><t>Krótko i długo działające beta2 adrenomimetyki</t></is></c><c r="H353" s="2" t="inlineStr" /><c r="I353" s="2" t="inlineStr" /><c r="J353" s="2" t="inlineStr" /><c r="K353" s="2" t="inlineStr"><is><t>GKS</t></is></c><c r="L353" s="2" t="inlineStr"><is><t>Inhibitory fosfodiesterazy 4</t></is></c><c r="M353" s="2" t="inlineStr" /><c r="N353" s="2" t="inlineStr" /><c r="O353" s="2" t="inlineStr" /><c r="P353" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q353" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="354"><c r="A354" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B354" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C354" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D354" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E354" s="2" t="inlineStr"><is><t>Omeprazol</t></is></c><c r="F354" s="2" t="inlineStr"><is><t>Powoduje nieodwracalne zablokowanie pompy protonowej</t></is></c><c r="G354" s="2" t="inlineStr"><is><t>Jest inhibitorem enzymów cytochromu P-450</t></is></c><c r="H354" s="2" t="inlineStr" /><c r="I354" s="2" t="inlineStr" /><c r="J354" s="2" t="inlineStr" /><c r="K354" s="2" t="inlineStr"><is><t>Hamuje wydzielanie kwasu solnego przez 6-12h</t></is></c><c r="L354" s="2" t="inlineStr"><is><t>Jest aktywowany przez pepsynę</t></is></c><c r="M354" s="2" t="inlineStr" /><c r="N354" s="2" t="inlineStr" /><c r="O354" s="2" t="inlineStr" /><c r="P354" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q354" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="355"><c r="A355" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B355" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C355" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D355" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E355" s="2" t="inlineStr"><is><t>Metoklopramid</t></is></c><c r="F355" s="2" t="inlineStr"><is><t>Jest agonistą receptorów dopaminowych</t></is></c><c r="G355" s="2" t="inlineStr"><is><t>Działa przeciwwymiotnie</t></is></c><c r="H355" s="2" t="inlineStr" /><c r="I355" s="2" t="inlineStr" /><c r="J355" s="2" t="inlineStr" /><c r="K355" s="2" t="inlineStr"><is><t>Zmniejsza objawy pozapiramidowe</t></is></c><c r="L355" s="2" t="inlineStr"><is><t>Zmniejsza stężenie prolaktyny</t></is></c><c r="M355" s="2" t="inlineStr" /><c r="N355" s="2" t="inlineStr" /><c r="O355" s="2" t="inlineStr" /><c r="P355" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q355" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="356"><c r="A356" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B356" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C356" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D356" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E356" s="2" t="inlineStr"><is><t>Metoklopramid:</t></is></c><c r="F356" s="2" t="inlineStr"><is><t>to lek przeciwwymiotny</t></is></c><c r="G356" s="2" t="inlineStr"><is><t>może spowodować hiperprolaktynemię</t></is></c><c r="H356" s="2" t="inlineStr"><is><t>to lek prokinetyczny</t></is></c><c r="I356" s="2" t="inlineStr"><is><t>może spowodować objawy pozapiramidowe</t></is></c><c r="J356" s="2" t="inlineStr" /><c r="K356" s="2" t="inlineStr" /><c r="L356" s="2" t="inlineStr" /><c r="M356" s="2" t="inlineStr" /><c r="N356" s="2" t="inlineStr" /><c r="O356" s="2" t="inlineStr" /><c r="P356" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q356" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="357"><c r="A357" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B357" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C357" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D357" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E357" s="2" t="inlineStr"><is><t>Przewlekłe zapalenie trzustki z alkoholu</t></is></c><c r="F357" s="2" t="inlineStr"><is><t>Preparaty enzymów trzustkowych</t></is></c><c r="G357" s="2" t="inlineStr"><is><t>Leki przeciwbólowe</t></is></c><c r="H357" s="2" t="inlineStr" /><c r="I357" s="2" t="inlineStr" /><c r="J357" s="2" t="inlineStr" /><c r="K357" s="2" t="inlineStr"><is><t>GKS</t></is></c><c r="L357" s="2" t="inlineStr"><is><t>Leki przeciwbakteryjne</t></is></c><c r="M357" s="2" t="inlineStr" /><c r="N357" s="2" t="inlineStr" /><c r="O357" s="2" t="inlineStr" /><c r="P357" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q357" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="358"><c r="A358" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B358" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C358" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D358" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E358" s="2" t="inlineStr"><is><t>Chory z encefalopatią wątrobową, możemy</t></is></c><c r="F358" s="2" t="inlineStr"><is><t>Asparaginian ornityny</t></is></c><c r="G358" s="2" t="inlineStr"><is><t>Laktuloza</t></is></c><c r="H358" s="2" t="inlineStr"><is><t>Ryfaksymina</t></is></c><c r="I358" s="2" t="inlineStr" /><c r="J358" s="2" t="inlineStr" /><c r="K358" s="2" t="inlineStr"><is><t>Piracetam</t></is></c><c r="L358" s="2" t="inlineStr" /><c r="M358" s="2" t="inlineStr" /><c r="N358" s="2" t="inlineStr" /><c r="O358" s="2" t="inlineStr" /><c r="P358" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q358" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="359"><c r="A359" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B359" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C359" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D359" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E359" s="2" t="inlineStr"><is><t>Schematy eradykacji H. Pylori (rekomendowane)</t></is></c><c r="F359" s="2" t="inlineStr"><is><t>Pantoprazol/cytrynian bizmutu/tetracyklina/metronidazol</t></is></c><c r="G359" s="2" t="inlineStr" /><c r="H359" s="2" t="inlineStr" /><c r="I359" s="2" t="inlineStr" /><c r="J359" s="2" t="inlineStr" /><c r="K359" s="2" t="inlineStr"><is><t>Cytrynian bizmutu/metronidazol</t></is></c><c r="L359" s="2" t="inlineStr"><is><t>Mizoprostol/metronidazol/klarytromycyna</t></is></c><c r="M359" s="2" t="inlineStr"><is><t>Ranitydyna/amoksycylina/metronidazol</t></is></c><c r="N359" s="2" t="inlineStr" /><c r="O359" s="2" t="inlineStr" /><c r="P359" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q359" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="360"><c r="A360" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B360" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C360" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D360" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E360" s="2" t="inlineStr"><is><t>Lek przeciwzakrzepowy – czas odstawienia (planowa, duże ryzyko krwawienia, nerki prawidłowe)</t></is></c><c r="F360" s="2" t="inlineStr"><is><t>Dabigatran – 1 dzień</t></is></c><c r="G360" s="2" t="inlineStr" /><c r="H360" s="2" t="inlineStr" /><c r="I360" s="2" t="inlineStr" /><c r="J360" s="2" t="inlineStr" /><c r="K360" s="2" t="inlineStr"><is><t>Warfaryna – 2 dni</t></is></c><c r="L360" s="2" t="inlineStr"><is><t>Acenokumarol – 10 dni</t></is></c><c r="M360" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy – 5 dni</t></is></c><c r="N360" s="2" t="inlineStr" /><c r="O360" s="2" t="inlineStr" /><c r="P360" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q360" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="361"><c r="A361" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B361" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C361" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D361" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E361" s="2" t="inlineStr"><is><t>Lek – monitorowanie</t></is></c><c r="F361" s="2" t="inlineStr"><is><t>Heparyna niefrakcjonowana – APTT</t></is></c><c r="G361" s="2" t="inlineStr" /><c r="H361" s="2" t="inlineStr" /><c r="I361" s="2" t="inlineStr" /><c r="J361" s="2" t="inlineStr" /><c r="K361" s="2" t="inlineStr"><is><t>Dabigatran – INR</t></is></c><c r="L361" s="2" t="inlineStr"><is><t>Acenokumarol – czas ekarynowy</t></is></c><c r="M361" s="2" t="inlineStr"><is><t>Rywaroksaban – czas trombinowy</t></is></c><c r="N361" s="2" t="inlineStr" /><c r="O361" s="2" t="inlineStr" /><c r="P361" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q361" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="362"><c r="A362" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B362" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C362" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D362" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E362" s="2" t="inlineStr"><is><t>Działanie antyagregacyjne</t></is></c><c r="F362" s="2" t="inlineStr"><is><t>Antagoniści receptorów P2Y12</t></is></c><c r="G362" s="2" t="inlineStr" /><c r="H362" s="2" t="inlineStr" /><c r="I362" s="2" t="inlineStr" /><c r="J362" s="2" t="inlineStr" /><c r="K362" s="2" t="inlineStr"><is><t>Agoniści receptorów GP IIb/IIIa</t></is></c><c r="L362" s="2" t="inlineStr"><is><t>Inhibitory COX2</t></is></c><c r="M362" s="2" t="inlineStr"><is><t>Agoniści receptorów TXA2</t></is></c><c r="N362" s="2" t="inlineStr" /><c r="O362" s="2" t="inlineStr" /><c r="P362" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q362" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="363"><c r="A363" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B363" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C363" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D363" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E363" s="2" t="inlineStr"><is><t>Zahamowanie agregacji płytek zależne od ADP po</t></is></c><c r="F363" s="2" t="inlineStr"><is><t>Klopidogrelu</t></is></c><c r="G363" s="2" t="inlineStr"><is><t>Tikagreloru</t></is></c><c r="H363" s="2" t="inlineStr" /><c r="I363" s="2" t="inlineStr" /><c r="J363" s="2" t="inlineStr" /><c r="K363" s="2" t="inlineStr"><is><t>Enoksaparyny</t></is></c><c r="L363" s="2" t="inlineStr"><is><t>Dipyridamolu</t></is></c><c r="M363" s="2" t="inlineStr" /><c r="N363" s="2" t="inlineStr" /><c r="O363" s="2" t="inlineStr" /><c r="P363" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q363" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="364"><c r="A364" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B364" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C364" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D364" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E364" s="2" t="inlineStr"><is><t>Statyny</t></is></c><c r="F364" s="2" t="inlineStr"><is><t>Zmniejszają stężenie cholesterolu LDL</t></is></c><c r="G364" s="2" t="inlineStr"><is><t>Zmniejszą stężenie triglicerydów</t></is></c><c r="H364" s="2" t="inlineStr" /><c r="I364" s="2" t="inlineStr" /><c r="J364" s="2" t="inlineStr" /><c r="K364" s="2" t="inlineStr"><is><t>Nie wpływają na stężenie cholesterolu wewnątrzkomórkowego</t></is></c><c r="L364" s="2" t="inlineStr"><is><t>Zmniejszają stężęnie cholesterolu HDL</t></is></c><c r="M364" s="2" t="inlineStr" /><c r="N364" s="2" t="inlineStr" /><c r="O364" s="2" t="inlineStr" /><c r="P364" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q364" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="365"><c r="A365" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B365" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C365" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D365" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E365" s="2" t="inlineStr"><is><t>Wielokierunkowe działanie statyn</t></is></c><c r="F365" s="2" t="inlineStr"><is><t>Poprawę funkcji śródbłonka</t></is></c><c r="G365" s="2" t="inlineStr"><is><t>Efekt przeciwzapalny</t></is></c><c r="H365" s="2" t="inlineStr"><is><t>Wpływ na fibrynolizę</t></is></c><c r="I365" s="2" t="inlineStr"><is><t>Stabilizację blaszki miażdżycowej</t></is></c><c r="J365" s="2" t="inlineStr" /><c r="K365" s="2" t="inlineStr" /><c r="L365" s="2" t="inlineStr" /><c r="M365" s="2" t="inlineStr" /><c r="N365" s="2" t="inlineStr" /><c r="O365" s="2" t="inlineStr" /><c r="P365" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q365" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="366"><c r="A366" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B366" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C366" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D366" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E366" s="2" t="inlineStr"><is><t>Farmakoterapia otyłości</t></is></c><c r="F366" s="2" t="inlineStr"><is><t>Liraglutyd</t></is></c><c r="G366" s="2" t="inlineStr"><is><t>Orlistat</t></is></c><c r="H366" s="2" t="inlineStr" /><c r="I366" s="2" t="inlineStr" /><c r="J366" s="2" t="inlineStr" /><c r="K366" s="2" t="inlineStr"><is><t>Paroksetyna</t></is></c><c r="L366" s="2" t="inlineStr"><is><t>Naltrekson</t></is></c><c r="M366" s="2" t="inlineStr" /><c r="N366" s="2" t="inlineStr" /><c r="O366" s="2" t="inlineStr" /><c r="P366" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q366" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="367"><c r="A367" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B367" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C367" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D367" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E367" s="2" t="inlineStr"><is><t>Do beta adrenolityków zmniejszających śmiertelność w skurczowej niewydolności serca</t></is></c><c r="F367" s="2" t="inlineStr"><is><t>Nebiwolol</t></is></c><c r="G367" s="2" t="inlineStr" /><c r="H367" s="2" t="inlineStr" /><c r="I367" s="2" t="inlineStr" /><c r="J367" s="2" t="inlineStr" /><c r="K367" s="2" t="inlineStr"><is><t>Atenolol</t></is></c><c r="L367" s="2" t="inlineStr"><is><t>Esmolol</t></is></c><c r="M367" s="2" t="inlineStr"><is><t>Acebutolol</t></is></c><c r="N367" s="2" t="inlineStr" /><c r="O367" s="2" t="inlineStr" /><c r="P367" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q367" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="368"><c r="A368" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B368" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C368" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D368" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E368" s="2" t="inlineStr"><is><t>Donory NO</t></is></c><c r="F368" s="2" t="inlineStr"><is><t>Nikorandil</t></is></c><c r="G368" s="2" t="inlineStr"><is><t>Molsidomina</t></is></c><c r="H368" s="2" t="inlineStr"><is><t>Diazontanizosorbitol</t></is></c><c r="I368" s="2" t="inlineStr" /><c r="J368" s="2" t="inlineStr" /><c r="K368" s="2" t="inlineStr"><is><t>Trimetazydyna</t></is></c><c r="L368" s="2" t="inlineStr" /><c r="M368" s="2" t="inlineStr" /><c r="N368" s="2" t="inlineStr" /><c r="O368" s="2" t="inlineStr" /><c r="P368" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q368" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="369"><c r="A369" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B369" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C369" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D369" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E369" s="2" t="inlineStr"><is><t>Leki I wyborou w monoterapii NT</t></is></c><c r="F369" s="2" t="inlineStr"><is><t>Antagoniści receptora angiotensynowego</t></is></c><c r="G369" s="2" t="inlineStr"><is><t>Antagoniści kanałów wapniowych</t></is></c><c r="H369" s="2" t="inlineStr" /><c r="I369" s="2" t="inlineStr" /><c r="J369" s="2" t="inlineStr" /><c r="K369" s="2" t="inlineStr"><is><t>Alfa1 adrenolityki</t></is></c><c r="L369" s="2" t="inlineStr"><is><t>Inhibitory reniny</t></is></c><c r="M369" s="2" t="inlineStr" /><c r="N369" s="2" t="inlineStr" /><c r="O369" s="2" t="inlineStr" /><c r="P369" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q369" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="370"><c r="A370" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B370" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C370" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D370" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E370" s="2" t="inlineStr"><is><t>Zmniejszenie śmiertnelności w skurczowej niewydolności serca</t></is></c><c r="F370" s="2" t="inlineStr"><is><t>Inhibitory konwertazy angiotensyny</t></is></c><c r="G370" s="2" t="inlineStr"><is><t>Antagoniści aldosteronu</t></is></c><c r="H370" s="2" t="inlineStr" /><c r="I370" s="2" t="inlineStr" /><c r="J370" s="2" t="inlineStr" /><c r="K370" s="2" t="inlineStr"><is><t>Waptany</t></is></c><c r="L370" s="2" t="inlineStr"><is><t>Diuretyki pętlowe</t></is></c><c r="M370" s="2" t="inlineStr" /><c r="N370" s="2" t="inlineStr" /><c r="O370" s="2" t="inlineStr" /><c r="P370" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q370" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="371"><c r="A371" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B371" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C371" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D371" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E371" s="2" t="inlineStr"><is><t>Przeciwskane jest jednoczesne stosowanie beta adrenolityków i</t></is></c><c r="F371" s="2" t="inlineStr"><is><t>Werapamilu</t></is></c><c r="G371" s="2" t="inlineStr" /><c r="H371" s="2" t="inlineStr" /><c r="I371" s="2" t="inlineStr" /><c r="J371" s="2" t="inlineStr" /><c r="K371" s="2" t="inlineStr"><is><t>Kaptoprylu</t></is></c><c r="L371" s="2" t="inlineStr"><is><t>Torasemidu</t></is></c><c r="M371" s="2" t="inlineStr"><is><t>Irbesartanu</t></is></c><c r="N371" s="2" t="inlineStr" /><c r="O371" s="2" t="inlineStr" /><c r="P371" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q371" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="372"><c r="A372" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B372" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C372" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D372" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E372" s="2" t="inlineStr"><is><t>Stan kliniczny – lek nadciśnieniowy</t></is></c><c r="F372" s="2" t="inlineStr"><is><t>Mikroalbuminuria – peryndopryl</t></is></c><c r="G372" s="2" t="inlineStr"><is><t>Tętniak aorty – bisoprolol</t></is></c><c r="H372" s="2" t="inlineStr"><is><t>Ciąża – metyldopa</t></is></c><c r="I372" s="2" t="inlineStr"><is><t>Chory po 80 rż. – indapamid</t></is></c><c r="J372" s="2" t="inlineStr" /><c r="K372" s="2" t="inlineStr" /><c r="L372" s="2" t="inlineStr" /><c r="M372" s="2" t="inlineStr" /><c r="N372" s="2" t="inlineStr" /><c r="O372" s="2" t="inlineStr" /><c r="P372" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q372" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="373"><c r="A373" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B373" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C373" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D373" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E373" s="2" t="inlineStr"><is><t>Inotropowe dodatnie</t></is></c><c r="F373" s="2" t="inlineStr"><is><t>Lewosymendan</t></is></c><c r="G373" s="2" t="inlineStr"><is><t>Milrinon</t></is></c><c r="H373" s="2" t="inlineStr" /><c r="I373" s="2" t="inlineStr" /><c r="J373" s="2" t="inlineStr" /><c r="K373" s="2" t="inlineStr"><is><t>Nesirytyd</t></is></c><c r="L373" s="2" t="inlineStr"><is><t>Sakubitryl</t></is></c><c r="M373" s="2" t="inlineStr" /><c r="N373" s="2" t="inlineStr" /><c r="O373" s="2" t="inlineStr" /><c r="P373" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q373" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="374"><c r="A374" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B374" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C374" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D374" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E374" s="2" t="inlineStr"><is><t>Skojarzenia leków w nadciśnieniu</t></is></c><c r="F374" s="2" t="inlineStr"><is><t>Inhibitor konwertazy angiotensyny + diuretyk tiazydowy</t></is></c><c r="G374" s="2" t="inlineStr"><is><t>Inhibitor konwertazy angiotensyny + antagonista wapnia</t></is></c><c r="H374" s="2" t="inlineStr"><is><t>Diuretyk tiazydowy + antagonista wapnia</t></is></c><c r="I374" s="2" t="inlineStr" /><c r="J374" s="2" t="inlineStr" /><c r="K374" s="2" t="inlineStr"><is><t>Sartan + inhibitor konwertazy angiotensyny</t></is></c><c r="L374" s="2" t="inlineStr" /><c r="M374" s="2" t="inlineStr" /><c r="N374" s="2" t="inlineStr" /><c r="O374" s="2" t="inlineStr" /><c r="P374" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q374" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="375"><c r="A375" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B375" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C375" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D375" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E375" s="2" t="inlineStr"><is><t>Amlodypina – działanie</t></is></c><c r="F375" s="2" t="inlineStr"><is><t>Zmniejszające opór obwodowy</t></is></c><c r="G375" s="2" t="inlineStr" /><c r="H375" s="2" t="inlineStr" /><c r="I375" s="2" t="inlineStr" /><c r="J375" s="2" t="inlineStr" /><c r="K375" s="2" t="inlineStr"><is><t>Chronotropowe dodatnie</t></is></c><c r="L375" s="2" t="inlineStr"><is><t>Inotropowe ujemne</t></is></c><c r="M375" s="2" t="inlineStr"><is><t>Dromotropowe ujemne</t></is></c><c r="N375" s="2" t="inlineStr" /><c r="O375" s="2" t="inlineStr" /><c r="P375" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q375" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="376"><c r="A376" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B376" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C376" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D376" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E376" s="2" t="inlineStr"><is><t>Dławica naczynioskurczowa (Prinzmetala)</t></is></c><c r="F376" s="2" t="inlineStr"><is><t>Diltiazem</t></is></c><c r="G376" s="2" t="inlineStr"><is><t>Werapamil</t></is></c><c r="H376" s="2" t="inlineStr" /><c r="I376" s="2" t="inlineStr" /><c r="J376" s="2" t="inlineStr" /><c r="K376" s="2" t="inlineStr"><is><t>Atenolol</t></is></c><c r="L376" s="2" t="inlineStr"><is><t>Prazosyna</t></is></c><c r="M376" s="2" t="inlineStr" /><c r="N376" s="2" t="inlineStr" /><c r="O376" s="2" t="inlineStr" /><c r="P376" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q376" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="377"><c r="A377" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B377" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C377" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D377" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E377" s="2" t="inlineStr"><is><t>Hiperkaliemia przy stosowaniu</t></is></c><c r="F377" s="2" t="inlineStr"><is><t>Kaptoprylu</t></is></c><c r="G377" s="2" t="inlineStr"><is><t>Amilorlydu</t></is></c><c r="H377" s="2" t="inlineStr" /><c r="I377" s="2" t="inlineStr" /><c r="J377" s="2" t="inlineStr" /><c r="K377" s="2" t="inlineStr"><is><t>Torasemidu</t></is></c><c r="L377" s="2" t="inlineStr"><is><t>Hydrochlortiazydu</t></is></c><c r="M377" s="2" t="inlineStr" /><c r="N377" s="2" t="inlineStr" /><c r="O377" s="2" t="inlineStr" /><c r="P377" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q377" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="378"><c r="A378" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B378" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C378" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D378" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E378" s="2" t="inlineStr"><is><t>OZW – postepowanie</t></is></c><c r="F378" s="2" t="inlineStr"><is><t>Furasemidu i.m</t></is></c><c r="G378" s="2" t="inlineStr"><is><t>Tikaglerolu p.o Klopidogrel bardziej, ale powiedzmy ze tak</t></is></c><c r="H378" s="2" t="inlineStr"><is><t>Morfiny s.c</t></is></c><c r="I378" s="2" t="inlineStr"><is><t>Kwasu acetylosalicylowego p.o</t></is></c><c r="J378" s="2" t="inlineStr" /><c r="K378" s="2" t="inlineStr" /><c r="L378" s="2" t="inlineStr" /><c r="M378" s="2" t="inlineStr" /><c r="N378" s="2" t="inlineStr" /><c r="O378" s="2" t="inlineStr" /><c r="P378" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q378" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="379"><c r="A379" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B379" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C379" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D379" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E379" s="2" t="inlineStr"><is><t>Amiodaron:</t></is></c><c r="F379" s="2" t="inlineStr"><is><t>obniża energię potrzebną do skutecznej defibrylacji elektrycznej</t></is></c><c r="G379" s="2" t="inlineStr"><is><t>może być rozpuszczany w 5% glukozie</t></is></c><c r="H379" s="2" t="inlineStr" /><c r="I379" s="2" t="inlineStr" /><c r="J379" s="2" t="inlineStr" /><c r="K379" s="2" t="inlineStr"><is><t>jest antagonistą sercowych kanałów potasowych z wyjątkiem ikr</t></is></c><c r="L379" s="2" t="inlineStr"><is><t>jest stosowany alternatywnie z lidokainą w resuscytacji krążeniowo-oddechowej</t></is></c><c r="M379" s="2" t="inlineStr" /><c r="N379" s="2" t="inlineStr" /><c r="O379" s="2" t="inlineStr" /><c r="P379" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q379" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="380"><c r="A380" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B380" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C380" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D380" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E380" s="2" t="inlineStr"><is><t>Amiodaron:</t></is></c><c r="F380" s="2" t="inlineStr"><is><t>ma niezgodność farmaceutyczną z 0,9% NaCl</t></is></c><c r="G380" s="2" t="inlineStr"><is><t>ma działanie chronotropowe ujemne i hipotensyjne</t></is></c><c r="H380" s="2" t="inlineStr" /><c r="I380" s="2" t="inlineStr" /><c r="J380" s="2" t="inlineStr" /><c r="K380" s="2" t="inlineStr"><is><t>to niewybiórczy antagonista kanałów potasowych wiążący się z nimi w okresie ich otwarcia</t></is></c><c r="L380" s="2" t="inlineStr"><is><t>zwiększa próg defibrylacji elektrycznej</t></is></c><c r="M380" s="2" t="inlineStr" /><c r="N380" s="2" t="inlineStr" /><c r="O380" s="2" t="inlineStr" /><c r="P380" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q380" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="381"><c r="A381" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B381" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C381" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D381" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E381" s="2" t="inlineStr"><is><t>Eplerenon</t></is></c><c r="F381" s="2" t="inlineStr"><is><t>Selektywnie wiąże się z receptorem dla mineralokortykoidów</t></is></c><c r="G381" s="2" t="inlineStr" /><c r="H381" s="2" t="inlineStr" /><c r="I381" s="2" t="inlineStr" /><c r="J381" s="2" t="inlineStr" /><c r="K381" s="2" t="inlineStr"><is><t>Nie powoduje hiperkaliemii</t></is></c><c r="L381" s="2" t="inlineStr"><is><t>Jest agonistą receptorów dla androgenów</t></is></c><c r="M381" s="2" t="inlineStr"><is><t>Powoduje hipernatremię</t></is></c><c r="N381" s="2" t="inlineStr" /><c r="O381" s="2" t="inlineStr" /><c r="P381" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q381" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="382"><c r="A382" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B382" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C382" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D382" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E382" s="2" t="inlineStr"><is><t>TLPD – działania niepożądane</t></is></c><c r="F382" s="2" t="inlineStr"><is><t>Zwiększenie masy ciała</t></is></c><c r="G382" s="2" t="inlineStr"><is><t>Obniżenie progu drgawkowego</t></is></c><c r="H382" s="2" t="inlineStr"><is><t>Suchowść w ustach</t></is></c><c r="I382" s="2" t="inlineStr"><is><t>Nad lub niedociśnienie tętnicze</t></is></c><c r="J382" s="2" t="inlineStr" /><c r="K382" s="2" t="inlineStr" /><c r="L382" s="2" t="inlineStr" /><c r="M382" s="2" t="inlineStr" /><c r="N382" s="2" t="inlineStr" /><c r="O382" s="2" t="inlineStr" /><c r="P382" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q382" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="383"><c r="A383" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B383" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C383" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D383" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E383" s="2" t="inlineStr"><is><t>Lek przeciwpadaczkowy – mechanizm</t></is></c><c r="F383" s="2" t="inlineStr"><is><t>Gabapentyna – nasilenie transmisji GABA</t></is></c><c r="G383" s="2" t="inlineStr"><is><t>Karbamazepina – blokokowanie kanałów sodowych</t></is></c><c r="H383" s="2" t="inlineStr"><is><t>Etosuksymid – blokowanie kanałów wapniowych</t></is></c><c r="I383" s="2" t="inlineStr" /><c r="J383" s="2" t="inlineStr" /><c r="K383" s="2" t="inlineStr"><is><t>Lamotrygina – pobudzenie synaptycznego uwalniania aminokwasów</t></is></c><c r="L383" s="2" t="inlineStr" /><c r="M383" s="2" t="inlineStr" /><c r="N383" s="2" t="inlineStr" /><c r="O383" s="2" t="inlineStr" /><c r="P383" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q383" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="384"><c r="A384" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B384" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C384" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D384" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E384" s="2" t="inlineStr"><is><t>Klozapina wymaga monitorowania Wszystkie wymagają LPP</t></is></c><c r="F384" s="2" t="inlineStr"><is><t>Morfologii</t></is></c><c r="G384" s="2" t="inlineStr"><is><t>Masy ciała</t></is></c><c r="H384" s="2" t="inlineStr"><is><t>Lipidogramu</t></is></c><c r="I384" s="2" t="inlineStr"><is><t>Glikemii</t></is></c><c r="J384" s="2" t="inlineStr" /><c r="K384" s="2" t="inlineStr" /><c r="L384" s="2" t="inlineStr" /><c r="M384" s="2" t="inlineStr" /><c r="N384" s="2" t="inlineStr" /><c r="O384" s="2" t="inlineStr" /><c r="P384" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q384" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="385"><c r="A385" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B385" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C385" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D385" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E385" s="2" t="inlineStr"><is><t>Fluoksetyna</t></is></c><c r="F385" s="2" t="inlineStr"><is><t>Hamuje wychwyt zwrotny serotoniny</t></is></c><c r="G385" s="2" t="inlineStr" /><c r="H385" s="2" t="inlineStr" /><c r="I385" s="2" t="inlineStr" /><c r="J385" s="2" t="inlineStr" /><c r="K385" s="2" t="inlineStr"><is><t>Ma istotny wpływ na układ krążenia</t></is></c><c r="L385" s="2" t="inlineStr"><is><t>Często powoduje zaparcia</t></is></c><c r="M385" s="2" t="inlineStr"><is><t>Nie działa na enzymy cytochromu P-450</t></is></c><c r="N385" s="2" t="inlineStr" /><c r="O385" s="2" t="inlineStr" /><c r="P385" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q385" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="386"><c r="A386" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B386" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C386" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D386" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E386" s="2" t="inlineStr"><is><t>Zespoł serotoninowy – fluoksetyna i… MAO A i = 5-HT, NA, A, DA, tyramina.... MAO B i = DA i 5-HT</t></is></c><c r="F386" s="2" t="inlineStr"><is><t>Klomipramina</t></is></c><c r="G386" s="2" t="inlineStr"><is><t>Linezolid</t></is></c><c r="H386" s="2" t="inlineStr"><is><t>Wenlafaksyna</t></is></c><c r="I386" s="2" t="inlineStr"><is><t>Moklobemid</t></is></c><c r="J386" s="2" t="inlineStr" /><c r="K386" s="2" t="inlineStr" /><c r="L386" s="2" t="inlineStr" /><c r="M386" s="2" t="inlineStr" /><c r="N386" s="2" t="inlineStr" /><c r="O386" s="2" t="inlineStr" /><c r="P386" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q386" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="387"><c r="A387" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B387" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C387" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D387" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E387" s="2" t="inlineStr"><is><t>Choroba Wilsona</t></is></c><c r="F387" s="2" t="inlineStr"><is><t>Siarczan cynku</t></is></c><c r="G387" s="2" t="inlineStr"><is><t>D-penicylamina</t></is></c><c r="H387" s="2" t="inlineStr" /><c r="I387" s="2" t="inlineStr" /><c r="J387" s="2" t="inlineStr" /><c r="K387" s="2" t="inlineStr"><is><t>Ropinirol</t></is></c><c r="L387" s="2" t="inlineStr"><is><t>Siarczan magnezu</t></is></c><c r="M387" s="2" t="inlineStr" /><c r="N387" s="2" t="inlineStr" /><c r="O387" s="2" t="inlineStr" /><c r="P387" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q387" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="388"><c r="A388" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B388" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C388" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D388" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E388" s="2" t="inlineStr"><is><t>Farmakoterapia bólu neuropatycznego jakiego? :D Tako to wszystkie LPD i przeciwpadaczkowe</t></is></c><c r="F388" s="2" t="inlineStr"><is><t>Gabapentyna</t></is></c><c r="G388" s="2" t="inlineStr"><is><t>Amitryptylina</t></is></c><c r="H388" s="2" t="inlineStr"><is><t>Duloksetyna</t></is></c><c r="I388" s="2" t="inlineStr" /><c r="J388" s="2" t="inlineStr" /><c r="K388" s="2" t="inlineStr"><is><t>Ibuprofen</t></is></c><c r="L388" s="2" t="inlineStr" /><c r="M388" s="2" t="inlineStr" /><c r="N388" s="2" t="inlineStr" /><c r="O388" s="2" t="inlineStr" /><c r="P388" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q388" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="389"><c r="A389" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B389" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C389" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D389" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E389" s="2" t="inlineStr"><is><t>Profilaktyka migreny</t></is></c><c r="F389" s="2" t="inlineStr"><is><t>Metoprolol</t></is></c><c r="G389" s="2" t="inlineStr"><is><t>Flunaryzyna</t></is></c><c r="H389" s="2" t="inlineStr" /><c r="I389" s="2" t="inlineStr" /><c r="J389" s="2" t="inlineStr" /><c r="K389" s="2" t="inlineStr"><is><t>Indometacyna to w hemikranii</t></is></c><c r="L389" s="2" t="inlineStr"><is><t>Toksyna botulinowa</t></is></c><c r="M389" s="2" t="inlineStr" /><c r="N389" s="2" t="inlineStr" /><c r="O389" s="2" t="inlineStr" /><c r="P389" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q389" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="390"><c r="A390" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B390" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C390" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D390" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E390" s="2" t="inlineStr"><is><t>Alteplaza</t></is></c><c r="F390" s="2" t="inlineStr"><is><t>W udarze niedokrwiennym mózgu</t></is></c><c r="G390" s="2" t="inlineStr" /><c r="H390" s="2" t="inlineStr" /><c r="I390" s="2" t="inlineStr" /><c r="J390" s="2" t="inlineStr" /><c r="K390" s="2" t="inlineStr"><is><t>Przed planowaną kardiowersją</t></is></c><c r="L390" s="2" t="inlineStr"><is><t>W zatorowości płucnej niewysokiego ryzyka</t></is></c><c r="M390" s="2" t="inlineStr"><is><t>W TIA</t></is></c><c r="N390" s="2" t="inlineStr" /><c r="O390" s="2" t="inlineStr" /><c r="P390" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q390" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="391"><c r="A391" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B391" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C391" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D391" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E391" s="2" t="inlineStr"><is><t>Profilaktyka wtórna udaru mózgu</t></is></c><c r="F391" s="2" t="inlineStr"><is><t>Dipirydamol</t></is></c><c r="G391" s="2" t="inlineStr"><is><t>Atorwastatyna</t></is></c><c r="H391" s="2" t="inlineStr"><is><t>Enoksapyrana</t></is></c><c r="I391" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="J391" s="2" t="inlineStr" /><c r="K391" s="2" t="inlineStr" /><c r="L391" s="2" t="inlineStr" /><c r="M391" s="2" t="inlineStr" /><c r="N391" s="2" t="inlineStr" /><c r="O391" s="2" t="inlineStr" /><c r="P391" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q391" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="392"><c r="A392" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B392" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C392" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D392" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E392" s="2" t="inlineStr"><is><t>Do działań niepożądanych doksycykliny zaliczamy:</t></is></c><c r="F392" s="2" t="inlineStr"><is><t>fotodermatozy</t></is></c><c r="G392" s="2" t="inlineStr"><is><t>zaburzenia czynności cewek nerkowych wywołane przez jej produkty rozpadu</t></is></c><c r="H392" s="2" t="inlineStr"><is><t>zapalenie wątroby</t></is></c><c r="I392" s="2" t="inlineStr"><is><t>zaburzenia rozwoju zębów i kości</t></is></c><c r="J392" s="2" t="inlineStr" /><c r="K392" s="2" t="inlineStr" /><c r="L392" s="2" t="inlineStr" /><c r="M392" s="2" t="inlineStr" /><c r="N392" s="2" t="inlineStr" /><c r="O392" s="2" t="inlineStr" /><c r="P392" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q392" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="393"><c r="A393" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B393" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C393" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D393" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E393" s="2" t="inlineStr"><is><t>Ceftriakson:</t></is></c><c r="F393" s="2" t="inlineStr"><is><t>należy do cefalosporyn III generacji</t></is></c><c r="G393" s="2" t="inlineStr"><is><t>może być podawany dożylnie</t></is></c><c r="H393" s="2" t="inlineStr" /><c r="I393" s="2" t="inlineStr" /><c r="J393" s="2" t="inlineStr" /><c r="K393" s="2" t="inlineStr"><is><t>wykazuje aktywność wobec MRSA</t></is></c><c r="L393" s="2" t="inlineStr"><is><t>nie wykazuje aktywności wobec Borrelia burgdorferi</t></is></c><c r="M393" s="2" t="inlineStr" /><c r="N393" s="2" t="inlineStr" /><c r="O393" s="2" t="inlineStr" /><c r="P393" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q393" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="394"><c r="A394" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B394" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C394" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D394" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E394" s="2" t="inlineStr"><is><t>Pseudomonas aeruginosa jest wrażliwy na działanie:</t></is></c><c r="F394" s="2" t="inlineStr"><is><t>kolistyny</t></is></c><c r="G394" s="2" t="inlineStr"><is><t>tobramycyn</t></is></c><c r="H394" s="2" t="inlineStr" /><c r="I394" s="2" t="inlineStr" /><c r="J394" s="2" t="inlineStr" /><c r="K394" s="2" t="inlineStr"><is><t>telawancyny</t></is></c><c r="L394" s="2" t="inlineStr"><is><t>cefazoliny</t></is></c><c r="M394" s="2" t="inlineStr" /><c r="N394" s="2" t="inlineStr" /><c r="O394" s="2" t="inlineStr" /><c r="P394" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q394" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="395"><c r="A395" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B395" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C395" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D395" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E395" s="2" t="inlineStr"><is><t>W terapii empirycznej bakteryjnego zapalenia opon mózgowo-rdzeniowych u osób dorosłych zalecane są:</t></is></c><c r="F395" s="2" t="inlineStr"><is><t>cefotaksym z wankomycyną</t></is></c><c r="G395" s="2" t="inlineStr"><is><t>ceftriakson z wankomycyną</t></is></c><c r="H395" s="2" t="inlineStr" /><c r="I395" s="2" t="inlineStr" /><c r="J395" s="2" t="inlineStr" /><c r="K395" s="2" t="inlineStr"><is><t>ampicylina z gentamycyną</t></is></c><c r="L395" s="2" t="inlineStr"><is><t>ampicylina z deksametazonem</t></is></c><c r="M395" s="2" t="inlineStr" /><c r="N395" s="2" t="inlineStr" /><c r="O395" s="2" t="inlineStr" /><c r="P395" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q395" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="396"><c r="A396" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B396" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C396" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D396" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E396" s="2" t="inlineStr"><is><t>Efekt bakteriobójczy zależny od czasu, w którym stężenie leku jest większe od MIC wykazują:</t></is></c><c r="F396" s="2" t="inlineStr"><is><t>amoksycylina z kwasem klawulanowym</t></is></c><c r="G396" s="2" t="inlineStr"><is><t>ceftriakson</t></is></c><c r="H396" s="2" t="inlineStr" /><c r="I396" s="2" t="inlineStr" /><c r="J396" s="2" t="inlineStr" /><c r="K396" s="2" t="inlineStr"><is><t>lewofloksacyna</t></is></c><c r="L396" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="M396" s="2" t="inlineStr" /><c r="N396" s="2" t="inlineStr" /><c r="O396" s="2" t="inlineStr" /><c r="P396" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q396" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="397"><c r="A397" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B397" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C397" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D397" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E397" s="2" t="inlineStr"><is><t>Leki przeciwdrobnoustrojowe, których mechanizm działania polega na hamowaniu biosyntezy ściany komórkowej bakterii to:</t></is></c><c r="F397" s="2" t="inlineStr"><is><t>cefadroksyl</t></is></c><c r="G397" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="H397" s="2" t="inlineStr"><is><t>bacytracyna</t></is></c><c r="I397" s="2" t="inlineStr" /><c r="J397" s="2" t="inlineStr" /><c r="K397" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="L397" s="2" t="inlineStr" /><c r="M397" s="2" t="inlineStr" /><c r="N397" s="2" t="inlineStr" /><c r="O397" s="2" t="inlineStr" /><c r="P397" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q397" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="398"><c r="A398" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B398" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C398" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D398" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E398" s="2" t="inlineStr"><is><t>Aktywność przeciwbakteryjną względem Legionella spp. ma:</t></is></c><c r="F398" s="2" t="inlineStr"><is><t>moksyfloksacyna</t></is></c><c r="G398" s="2" t="inlineStr"><is><t>azytromycyna</t></is></c><c r="H398" s="2" t="inlineStr"><is><t>tygecyklina</t></is></c><c r="I398" s="2" t="inlineStr" /><c r="J398" s="2" t="inlineStr" /><c r="K398" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="L398" s="2" t="inlineStr" /><c r="M398" s="2" t="inlineStr" /><c r="N398" s="2" t="inlineStr" /><c r="O398" s="2" t="inlineStr" /><c r="P398" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q398" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="399"><c r="A399" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B399" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C399" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D399" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E399" s="2" t="inlineStr"><is><t>Jodopowidon znalazł zastosowanie w:</t></is></c><c r="F399" s="2" t="inlineStr"><is><t>dezynfekcji skóry przed nakłuciem</t></is></c><c r="G399" s="2" t="inlineStr"><is><t>leczeniu zakażeń pochwy florą mieszaną</t></is></c><c r="H399" s="2" t="inlineStr"><is><t>profilaktyce zakażeń ran</t></is></c><c r="I399" s="2" t="inlineStr"><is><t>leczeniu zakażeń błony śluzowej jamy ustnej</t></is></c><c r="J399" s="2" t="inlineStr" /><c r="K399" s="2" t="inlineStr" /><c r="L399" s="2" t="inlineStr" /><c r="M399" s="2" t="inlineStr" /><c r="N399" s="2" t="inlineStr" /><c r="O399" s="2" t="inlineStr" /><c r="P399" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q399" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="400"><c r="A400" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B400" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C400" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D400" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E400" s="2" t="inlineStr"><is><t>Inhibitory neuraminidazy:</t></is></c><c r="F400" s="2" t="inlineStr"><is><t>hamują uwalnianie wirusów z zakażonych komórek</t></is></c><c r="G400" s="2" t="inlineStr"><is><t>można je stosować w leczeniu grypy typu A i B</t></is></c><c r="H400" s="2" t="inlineStr" /><c r="I400" s="2" t="inlineStr" /><c r="J400" s="2" t="inlineStr" /><c r="K400" s="2" t="inlineStr"><is><t>nie różnią się między sobą pod względem skuteczności i działań niepożądanych</t></is></c><c r="L400" s="2" t="inlineStr"><is><t>nie są skuteczne w profilaktyce grypy</t></is></c><c r="M400" s="2" t="inlineStr" /><c r="N400" s="2" t="inlineStr" /><c r="O400" s="2" t="inlineStr" /><c r="P400" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q400" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="401"><c r="A401" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B401" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C401" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D401" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E401" s="2" t="inlineStr"><is><t>Cyprofloksacyna:</t></is></c><c r="F401" s="2" t="inlineStr"><is><t>ma efekt działania zależny od skumulowanej ekspozycji</t></is></c><c r="G401" s="2" t="inlineStr"><is><t>jest stosowana w leczeniu empirycznym niepowikłanego ostrego odmiedniczkowego zapalenia nerek</t></is></c><c r="H401" s="2" t="inlineStr"><is><t>może być podawana dożylnie</t></is></c><c r="I401" s="2" t="inlineStr" /><c r="J401" s="2" t="inlineStr" /><c r="K401" s="2" t="inlineStr"><is><t>nie wydłuża odstępu QT</t></is></c><c r="L401" s="2" t="inlineStr" /><c r="M401" s="2" t="inlineStr" /><c r="N401" s="2" t="inlineStr" /><c r="O401" s="2" t="inlineStr" /><c r="P401" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q401" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="402"><c r="A402" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B402" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C402" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D402" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E402" s="2" t="inlineStr"><is><t>Leczenie przeciwbakteryjne powinno być zlecone, jeśli w badaniu mikrobiologicznym zostanie stwierdzone:</t></is></c><c r="F402" s="2" t="inlineStr"><is><t>obecność Escherichia coli w dwóch posiewach krwi obwodowej</t></is></c><c r="G402" s="2" t="inlineStr"><is><t>brak wzrostu bakterii we krwi u osoby z klinicznymi i radiologicznymi cechami zapalenia płuc</t></is></c><c r="H402" s="2" t="inlineStr" /><c r="I402" s="2" t="inlineStr" /><c r="J402" s="2" t="inlineStr" /><c r="K402" s="2" t="inlineStr"><is><t>nosicielstwo szczepu alarmowego w przewodzie pokarmowym</t></is></c><c r="L402" s="2" t="inlineStr"><is><t>trzy gatunki bakterii w posiewie moczu</t></is></c><c r="M402" s="2" t="inlineStr" /><c r="N402" s="2" t="inlineStr" /><c r="O402" s="2" t="inlineStr" /><c r="P402" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q402" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="403"><c r="A403" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B403" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C403" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D403" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E403" s="2" t="inlineStr"><is><t>Przeciwinfekcyjna farmakoprofilaktyka medyczna jest zalecana:</t></is></c><c r="F403" s="2" t="inlineStr"><is><t>w ciężkiej neutropenii trwającej &gt; 7 dni u osób z ostrymi białaczkami</t></is></c><c r="G403" s="2" t="inlineStr"><is><t>nieszczepionym osobom z grup ryzyka ciężkiego przebiegu choroby po kontakcie z chorym na grypę</t></is></c><c r="H403" s="2" t="inlineStr" /><c r="I403" s="2" t="inlineStr" /><c r="J403" s="2" t="inlineStr" /><c r="K403" s="2" t="inlineStr"><is><t>po implantacji stentów wieńcowych przez 12 miesięcy</t></is></c><c r="L403" s="2" t="inlineStr"><is><t>podczas przewlekłego cewnikowania pęcherza moczowego</t></is></c><c r="M403" s="2" t="inlineStr" /><c r="N403" s="2" t="inlineStr" /><c r="O403" s="2" t="inlineStr" /><c r="P403" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q403" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="404"><c r="A404" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B404" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C404" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D404" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E404" s="2" t="inlineStr"><is><t>W grzybiczym zakażeniu paznokci zastosowanie ma:</t></is></c><c r="F404" s="2" t="inlineStr"><is><t>itrakonazol</t></is></c><c r="G404" s="2" t="inlineStr"><is><t>terbinafina</t></is></c><c r="H404" s="2" t="inlineStr" /><c r="I404" s="2" t="inlineStr" /><c r="J404" s="2" t="inlineStr" /><c r="K404" s="2" t="inlineStr"><is><t>natamycyna</t></is></c><c r="L404" s="2" t="inlineStr"><is><t>kaspofungina</t></is></c><c r="M404" s="2" t="inlineStr" /><c r="N404" s="2" t="inlineStr" /><c r="O404" s="2" t="inlineStr" /><c r="P404" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q404" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="405"><c r="A405" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B405" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C405" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D405" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E405" s="2" t="inlineStr"><is><t>Po ugryzieniu przez kleszcza, gdy obserwujemy rumień wędrujący, racjonalne jest zastosowanie:</t></is></c><c r="F405" s="2" t="inlineStr"><is><t>amoksycyliny</t></is></c><c r="G405" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="H405" s="2" t="inlineStr"><is><t>cefuroksymu</t></is></c><c r="I405" s="2" t="inlineStr"><is><t>azytromycyny</t></is></c><c r="J405" s="2" t="inlineStr" /><c r="K405" s="2" t="inlineStr" /><c r="L405" s="2" t="inlineStr" /><c r="M405" s="2" t="inlineStr" /><c r="N405" s="2" t="inlineStr" /><c r="O405" s="2" t="inlineStr" /><c r="P405" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q405" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="406"><c r="A406" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B406" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C406" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D406" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E406" s="2" t="inlineStr"><is><t>W leczeniu zakażenia wirusem opryszczki (Herpes) stosuje się:</t></is></c><c r="F406" s="2" t="inlineStr"><is><t>foskarnet</t></is></c><c r="G406" s="2" t="inlineStr"><is><t>acyklowir</t></is></c><c r="H406" s="2" t="inlineStr" /><c r="I406" s="2" t="inlineStr" /><c r="J406" s="2" t="inlineStr" /><c r="K406" s="2" t="inlineStr"><is><t>rymantadynę</t></is></c><c r="L406" s="2" t="inlineStr"><is><t>lamiwudynę</t></is></c><c r="M406" s="2" t="inlineStr" /><c r="N406" s="2" t="inlineStr" /><c r="O406" s="2" t="inlineStr" /><c r="P406" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q406" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="407"><c r="A407" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B407" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C407" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D407" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E407" s="2" t="inlineStr"><is><t>W leczeniu hipoglikemii stosuje się:</t></is></c><c r="F407" s="2" t="inlineStr"><is><t>węglowodany proste doustnie</t></is></c><c r="G407" s="2" t="inlineStr"><is><t>glukozę dożylnie</t></is></c><c r="H407" s="2" t="inlineStr"><is><t>węglowodany złożone doustnie</t></is></c><c r="I407" s="2" t="inlineStr" /><c r="J407" s="2" t="inlineStr" /><c r="K407" s="2" t="inlineStr"><is><t>glukagon doustnie</t></is></c><c r="L407" s="2" t="inlineStr" /><c r="M407" s="2" t="inlineStr" /><c r="N407" s="2" t="inlineStr" /><c r="O407" s="2" t="inlineStr" /><c r="P407" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q407" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="408"><c r="A408" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B408" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C408" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D408" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E408" s="2" t="inlineStr"><is><t>Liotyronina:</t></is></c><c r="F408" s="2" t="inlineStr"><is><t>odpowiada ona naturalnemu hormonowi T3</t></is></c><c r="G408" s="2" t="inlineStr"><is><t>ma krótszy okres półtrwania niż lewotyroksyna</t></is></c><c r="H408" s="2" t="inlineStr" /><c r="I408" s="2" t="inlineStr" /><c r="J408" s="2" t="inlineStr" /><c r="K408" s="2" t="inlineStr"><is><t>jest lekiem z wyboru w niedoczynności tarczycy</t></is></c><c r="L408" s="2" t="inlineStr"><is><t>jest przeciwwskazana w leczeniu śpiączki hipometabolicznej</t></is></c><c r="M408" s="2" t="inlineStr" /><c r="N408" s="2" t="inlineStr" /><c r="O408" s="2" t="inlineStr" /><c r="P408" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q408" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="409"><c r="A409" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B409" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C409" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D409" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E409" s="2" t="inlineStr"><is><t>Wskazaniem do zastosowania jodku potasu może być:</t></is></c><c r="F409" s="2" t="inlineStr"><is><t>ochrona tarczycy przed jodem radioaktywnym</t></is></c><c r="G409" s="2" t="inlineStr"><is><t>przygotowanie do usunięcia tarczycy</t></is></c><c r="H409" s="2" t="inlineStr"><is><t>przełom tyreotoksyczny</t></is></c><c r="I409" s="2" t="inlineStr"><is><t>zapobieganie powstawaniu wola z niedoboru jodu</t></is></c><c r="J409" s="2" t="inlineStr" /><c r="K409" s="2" t="inlineStr" /><c r="L409" s="2" t="inlineStr" /><c r="M409" s="2" t="inlineStr" /><c r="N409" s="2" t="inlineStr" /><c r="O409" s="2" t="inlineStr" /><c r="P409" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q409" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="410"><c r="A410" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B410" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C410" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D410" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E410" s="2" t="inlineStr"><is><t>W leczeniu hiperprolaktynemii stosuje się:</t></is></c><c r="F410" s="2" t="inlineStr"><is><t>bromokryptynę</t></is></c><c r="G410" s="2" t="inlineStr"><is><t>karbegolinę</t></is></c><c r="H410" s="2" t="inlineStr" /><c r="I410" s="2" t="inlineStr" /><c r="J410" s="2" t="inlineStr" /><c r="K410" s="2" t="inlineStr"><is><t>somatostatynę</t></is></c><c r="L410" s="2" t="inlineStr"><is><t>terlipresynę</t></is></c><c r="M410" s="2" t="inlineStr" /><c r="N410" s="2" t="inlineStr" /><c r="O410" s="2" t="inlineStr" /><c r="P410" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q410" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="411"><c r="A411" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B411" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C411" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D411" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E411" s="2" t="inlineStr"><is><t>Działanie antyandrogenne wykazuje:</t></is></c><c r="F411" s="2" t="inlineStr"><is><t>octan cyproteronu</t></is></c><c r="G411" s="2" t="inlineStr"><is><t>ketokonazol</t></is></c><c r="H411" s="2" t="inlineStr"><is><t>finasteryd</t></is></c><c r="I411" s="2" t="inlineStr"><is><t>bikalutamid</t></is></c><c r="J411" s="2" t="inlineStr" /><c r="K411" s="2" t="inlineStr" /><c r="L411" s="2" t="inlineStr" /><c r="M411" s="2" t="inlineStr" /><c r="N411" s="2" t="inlineStr" /><c r="O411" s="2" t="inlineStr" /><c r="P411" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q411" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="412"><c r="A412" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B412" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C412" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D412" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E412" s="2" t="inlineStr"><is><t>Glikokortykosteroidy zwiększają:</t></is></c><c r="F412" s="2" t="inlineStr"><is><t>produkcję surfaktantu</t></is></c><c r="G412" s="2" t="inlineStr" /><c r="H412" s="2" t="inlineStr" /><c r="I412" s="2" t="inlineStr" /><c r="J412" s="2" t="inlineStr" /><c r="K412" s="2" t="inlineStr"><is><t>ekspresję genu osteokalcyny</t></is></c><c r="L412" s="2" t="inlineStr"><is><t>stężenie wapnia w surowicy krwi</t></is></c><c r="M412" s="2" t="inlineStr"><is><t>syntezę testosteronu</t></is></c><c r="N412" s="2" t="inlineStr" /><c r="O412" s="2" t="inlineStr" /><c r="P412" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q412" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="413"><c r="A413" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B413" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C413" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D413" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E413" s="2" t="inlineStr"><is><t>Efektem nadmiaru gestagenów może być:</t></is></c><c r="F413" s="2" t="inlineStr"><is><t>depresja</t></is></c><c r="G413" s="2" t="inlineStr"><is><t>łojotok skóry</t></is></c><c r="H413" s="2" t="inlineStr"><is><t>przyrost masy ciała</t></is></c><c r="I413" s="2" t="inlineStr"><is><t>hirsutyzm</t></is></c><c r="J413" s="2" t="inlineStr" /><c r="K413" s="2" t="inlineStr" /><c r="L413" s="2" t="inlineStr" /><c r="M413" s="2" t="inlineStr" /><c r="N413" s="2" t="inlineStr" /><c r="O413" s="2" t="inlineStr" /><c r="P413" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q413" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="414"><c r="A414" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B414" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C414" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D414" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E414" s="2" t="inlineStr"><is><t>W leczeniu wągrzycy (cysticerkozy) stosujemy:</t></is></c><c r="F414" s="2" t="inlineStr"><is><t>prazykwantel</t></is></c><c r="G414" s="2" t="inlineStr"><is><t>albendazol</t></is></c><c r="H414" s="2" t="inlineStr" /><c r="I414" s="2" t="inlineStr" /><c r="J414" s="2" t="inlineStr" /><c r="K414" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="L414" s="2" t="inlineStr"><is><t>iwermektynę bo</t></is></c><c r="M414" s="2" t="inlineStr" /><c r="N414" s="2" t="inlineStr" /><c r="O414" s="2" t="inlineStr" /><c r="P414" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q414" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="415"><c r="A415" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B415" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C415" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D415" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E415" s="2" t="inlineStr"><is><t>Stosowanie kwasu acetylosalicylowego może być przyczyną:</t></is></c><c r="F415" s="2" t="inlineStr"><is><t>zaostrzenia astmy</t></is></c><c r="G415" s="2" t="inlineStr"><is><t>retencji sodu i wody</t></is></c><c r="H415" s="2" t="inlineStr"><is><t>niedokrwistości</t></is></c><c r="I415" s="2" t="inlineStr" /><c r="J415" s="2" t="inlineStr" /><c r="K415" s="2" t="inlineStr"><is><t>zakrzepicy żył głębokich</t></is></c><c r="L415" s="2" t="inlineStr" /><c r="M415" s="2" t="inlineStr" /><c r="N415" s="2" t="inlineStr" /><c r="O415" s="2" t="inlineStr" /><c r="P415" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q415" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="416"><c r="A416" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B416" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C416" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D416" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E416" s="2" t="inlineStr"><is><t>Efekty gastrotoksyczne związane ze stosowaniem niesteroidowych leków przeciwzapalnych może nasilać:</t></is></c><c r="F416" s="2" t="inlineStr"><is><t>zolendronian</t></is></c><c r="G416" s="2" t="inlineStr"><is><t>fluoksetyna tak, SSRI też</t></is></c><c r="H416" s="2" t="inlineStr"><is><t>acenokumarol</t></is></c><c r="I416" s="2" t="inlineStr"><is><t>prednizon</t></is></c><c r="J416" s="2" t="inlineStr" /><c r="K416" s="2" t="inlineStr" /><c r="L416" s="2" t="inlineStr" /><c r="M416" s="2" t="inlineStr" /><c r="N416" s="2" t="inlineStr" /><c r="O416" s="2" t="inlineStr" /><c r="P416" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q416" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="417"><c r="A417" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B417" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C417" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D417" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E417" s="2" t="inlineStr"><is><t>Zastosowanie ibuprofenu w 3 trymestrze ciąży może spowodować:</t></is></c><c r="F417" s="2" t="inlineStr"><is><t>przedwczesne zamknięcie przewodu Botalla</t></is></c><c r="G417" s="2" t="inlineStr"><is><t>zwiększone ryzyko krwawienia u matki</t></is></c><c r="H417" s="2" t="inlineStr"><is><t>zwiększone ryzyko obrzęków u matki</t></is></c><c r="I417" s="2" t="inlineStr" /><c r="J417" s="2" t="inlineStr" /><c r="K417" s="2" t="inlineStr"><is><t>zwiększenie czynności skurczowej macicy</t></is></c><c r="L417" s="2" t="inlineStr" /><c r="M417" s="2" t="inlineStr" /><c r="N417" s="2" t="inlineStr" /><c r="O417" s="2" t="inlineStr" /><c r="P417" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q417" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="418"><c r="A418" s="2" t="inlineStr"><is><t>BÓLE GŁOWY</t></is></c><c r="B418" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C418" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D418" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E418" s="2" t="inlineStr"><is><t>Napad migreny przerywa:</t></is></c><c r="F418" s="2" t="inlineStr"><is><t>winian ergotaminy</t></is></c><c r="G418" s="2" t="inlineStr"><is><t>sumatryptan</t></is></c><c r="H418" s="2" t="inlineStr"><is><t>ibuprofen</t></is></c><c r="I418" s="2" t="inlineStr" /><c r="J418" s="2" t="inlineStr" /><c r="K418" s="2" t="inlineStr"><is><t>metoklopramid</t></is></c><c r="L418" s="2" t="inlineStr" /><c r="M418" s="2" t="inlineStr" /><c r="N418" s="2" t="inlineStr" /><c r="O418" s="2" t="inlineStr" /><c r="P418" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q418" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="419"><c r="A419" s="2" t="inlineStr"><is><t>ZNIECZULENIA MIEJSCOWE</t></is></c><c r="B419" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C419" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D419" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E419" s="2" t="inlineStr"><is><t>W leczeniu neuralgii popółpaśćcowej można zastosować:</t></is></c><c r="F419" s="2" t="inlineStr"><is><t>8% kapsaicynę w kremie</t></is></c><c r="G419" s="2" t="inlineStr"><is><t>5% lidokainę w plastrach</t></is></c><c r="H419" s="2" t="inlineStr"><is><t>amitryptylinę</t></is></c><c r="I419" s="2" t="inlineStr" /><c r="J419" s="2" t="inlineStr" /><c r="K419" s="2" t="inlineStr"><is><t>metamizol</t></is></c><c r="L419" s="2" t="inlineStr" /><c r="M419" s="2" t="inlineStr" /><c r="N419" s="2" t="inlineStr" /><c r="O419" s="2" t="inlineStr" /><c r="P419" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q419" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="420"><c r="A420" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B420" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C420" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D420" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E420" s="2" t="inlineStr"><is><t>Loperamid:</t></is></c><c r="F420" s="2" t="inlineStr"><is><t>w dawkach terapeutycznych nie działa ośrodkowo</t></is></c><c r="G420" s="2" t="inlineStr"><is><t>jest przeciwwskazany we wrzodziejącym zapaleniu jelita grubego</t></is></c><c r="H420" s="2" t="inlineStr" /><c r="I420" s="2" t="inlineStr" /><c r="J420" s="2" t="inlineStr" /><c r="K420" s="2" t="inlineStr"><is><t>jest agonistą receptorów serotoninowych w jelicie</t></is></c><c r="L420" s="2" t="inlineStr"><is><t>wykazuje działanie przeciwbólowe</t></is></c><c r="M420" s="2" t="inlineStr" /><c r="N420" s="2" t="inlineStr" /><c r="O420" s="2" t="inlineStr" /><c r="P420" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q420" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="421"><c r="A421" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B421" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C421" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D421" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E421" s="2" t="inlineStr"><is><t>Fentanyl:</t></is></c><c r="F421" s="2" t="inlineStr"><is><t>hamuje ośrodek oddechowy</t></is></c><c r="G421" s="2" t="inlineStr" /><c r="H421" s="2" t="inlineStr" /><c r="I421" s="2" t="inlineStr" /><c r="J421" s="2" t="inlineStr" /><c r="K421" s="2" t="inlineStr"><is><t>działa neurotoksycznie</t></is></c><c r="L421" s="2" t="inlineStr"><is><t>ma aktywne metabolity</t></is></c><c r="M421" s="2" t="inlineStr"><is><t>uwalnia histaminę</t></is></c><c r="N421" s="2" t="inlineStr" /><c r="O421" s="2" t="inlineStr" /><c r="P421" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q421" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="422"><c r="A422" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B422" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C422" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D422" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E422" s="2" t="inlineStr"><is><t>Nefopam</t></is></c><c r="F422" s="2" t="inlineStr"><is><t>jest inhibitorem wychwytu zwrotnego serotoniny i noradrenaliny</t></is></c><c r="G422" s="2" t="inlineStr"><is><t>u osób starszych może wywoływać omamy</t></is></c><c r="H422" s="2" t="inlineStr" /><c r="I422" s="2" t="inlineStr" /><c r="J422" s="2" t="inlineStr" /><c r="K422" s="2" t="inlineStr"><is><t>hamuje wybiórczo cyklooksygenazę typu 2</t></is></c><c r="L422" s="2" t="inlineStr"><is><t>u dzieci może być stosowany w profilaktyce drgawek gorączkowych</t></is></c><c r="M422" s="2" t="inlineStr" /><c r="N422" s="2" t="inlineStr" /><c r="O422" s="2" t="inlineStr" /><c r="P422" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q422" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="423"><c r="A423" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B423" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C423" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D423" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E423" s="2" t="inlineStr"><is><t>W zespole abstynencyjnym w uzależnieniu od opioidów występują:</t></is></c><c r="F423" s="2" t="inlineStr"><is><t>rozszerzenie źrenic</t></is></c><c r="G423" s="2" t="inlineStr"><is><t>wymioty i biegunka</t></is></c><c r="H423" s="2" t="inlineStr"><is><t>bezsenność</t></is></c><c r="I423" s="2" t="inlineStr"><is><t>łzawienie i wyciek z nosa</t></is></c><c r="J423" s="2" t="inlineStr" /><c r="K423" s="2" t="inlineStr" /><c r="L423" s="2" t="inlineStr" /><c r="M423" s="2" t="inlineStr" /><c r="N423" s="2" t="inlineStr" /><c r="O423" s="2" t="inlineStr" /><c r="P423" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q423" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="424"><c r="A424" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B424" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C424" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D424" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E424" s="2" t="inlineStr"><is><t>Redukcję masy ciała może powodować stosowanie:</t></is></c><c r="F424" s="2" t="inlineStr"><is><t>fluoksetyny</t></is></c><c r="G424" s="2" t="inlineStr"><is><t>metforminy</t></is></c><c r="H424" s="2" t="inlineStr"><is><t>liraglutydu</t></is></c><c r="I424" s="2" t="inlineStr" /><c r="J424" s="2" t="inlineStr" /><c r="K424" s="2" t="inlineStr"><is><t>insuliny</t></is></c><c r="L424" s="2" t="inlineStr" /><c r="M424" s="2" t="inlineStr" /><c r="N424" s="2" t="inlineStr" /><c r="O424" s="2" t="inlineStr" /><c r="P424" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q424" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="425"><c r="A425" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B425" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C425" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D425" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E425" s="2" t="inlineStr"><is><t>W udarze niedokrwiennym mózgu możesz zastosować tkankowy aktywator plazminogenu jeśli stwierdzisz, że pacjent:</t></is></c><c r="F425" s="2" t="inlineStr"><is><t>doustne leczenie przeciwkrzepliwe (INR=1.5)</t></is></c><c r="G425" s="2" t="inlineStr"><is><t>ma wartości ciśnienia tętniczego: SBP ≤ 185 mm Hg lub DBP ≤ 110 mm Hg</t></is></c><c r="H425" s="2" t="inlineStr"><is><t>ma czas od wystąpienia objawów udaru mózgu nie przekraczający 4.5h</t></is></c><c r="I425" s="2" t="inlineStr" /><c r="J425" s="2" t="inlineStr" /><c r="K425" s="2" t="inlineStr"><is><t>jest w podeszłym wieku (&gt; 80 lat)</t></is></c><c r="L425" s="2" t="inlineStr" /><c r="M425" s="2" t="inlineStr" /><c r="N425" s="2" t="inlineStr" /><c r="O425" s="2" t="inlineStr" /><c r="P425" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q425" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="426"><c r="A426" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B426" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C426" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D426" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E426" s="2" t="inlineStr"><is><t>U 76 letniej kobiety z napadowym migotaniem przedsionków, cukrzycą i nadciśnieniem tętniczym (Cha2DS2VASc = 5 pkt) i niskim ryzykiem krwawienia (HAS-BLED = 2 pkt) wskazane w przewlekłej profilaktyce są:</t></is></c><c r="F426" s="2" t="inlineStr"><is><t>warfaryna</t></is></c><c r="G426" s="2" t="inlineStr"><is><t>eteksylan dabigatranu</t></is></c><c r="H426" s="2" t="inlineStr" /><c r="I426" s="2" t="inlineStr" /><c r="J426" s="2" t="inlineStr" /><c r="K426" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="L426" s="2" t="inlineStr"><is><t>fondaparynuks</t></is></c><c r="M426" s="2" t="inlineStr" /><c r="N426" s="2" t="inlineStr" /><c r="O426" s="2" t="inlineStr" /><c r="P426" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q426" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="427"><c r="A427" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B427" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C427" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D427" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E427" s="2" t="inlineStr"><is><t>Rywaroksaban:</t></is></c><c r="F427" s="2" t="inlineStr"><is><t>wymaga redukcji dawki w niewydolności nerek</t></is></c><c r="G427" s="2" t="inlineStr" /><c r="H427" s="2" t="inlineStr" /><c r="I427" s="2" t="inlineStr" /><c r="J427" s="2" t="inlineStr" /><c r="K427" s="2" t="inlineStr"><is><t>odwracalnie blokuje receptor GP IIb/IIIa</t></is></c><c r="L427" s="2" t="inlineStr"><is><t>występuje w postaci proleku</t></is></c><c r="M427" s="2" t="inlineStr"><is><t>jest stosowany w profilaktyce choroby zakrzepowo-zatorowej w czasie ciąży</t></is></c><c r="N427" s="2" t="inlineStr" /><c r="O427" s="2" t="inlineStr" /><c r="P427" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q427" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="428"><c r="A428" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B428" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C428" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D428" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E428" s="2" t="inlineStr"><is><t>Do leków działających na receptor P2Y12 zaliczamy:</t></is></c><c r="F428" s="2" t="inlineStr"><is><t>prasugrel</t></is></c><c r="G428" s="2" t="inlineStr" /><c r="H428" s="2" t="inlineStr" /><c r="I428" s="2" t="inlineStr" /><c r="J428" s="2" t="inlineStr" /><c r="K428" s="2" t="inlineStr"><is><t>apiksaban</t></is></c><c r="L428" s="2" t="inlineStr"><is><t>worapaksar</t></is></c><c r="M428" s="2" t="inlineStr"><is><t>dypirydamol</t></is></c><c r="N428" s="2" t="inlineStr" /><c r="O428" s="2" t="inlineStr" /><c r="P428" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q428" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="429"><c r="A429" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B429" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C429" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D429" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E429" s="2" t="inlineStr"><is><t>Do częstych działań niepożądanych atorwastatyny należy:</t></is></c><c r="F429" s="2" t="inlineStr"><is><t>uszkodzenie wątroby</t></is></c><c r="G429" s="2" t="inlineStr" /><c r="H429" s="2" t="inlineStr" /><c r="I429" s="2" t="inlineStr" /><c r="J429" s="2" t="inlineStr" /><c r="K429" s="2" t="inlineStr"><is><t>rogowacenie ciemne</t></is></c><c r="L429" s="2" t="inlineStr"><is><t>miopatia</t></is></c><c r="M429" s="2" t="inlineStr"><is><t>uderzenia gorąca</t></is></c><c r="N429" s="2" t="inlineStr" /><c r="O429" s="2" t="inlineStr" /><c r="P429" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q429" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="430"><c r="A430" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B430" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C430" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D430" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E430" s="2" t="inlineStr"><is><t>Orlistat:</t></is></c><c r="F430" s="2" t="inlineStr"><is><t>może być przyczyną wystąpienia tłuszczowych stolców</t></is></c><c r="G430" s="2" t="inlineStr"><is><t>może być stosowany u osób z chorobami układu krążenia</t></is></c><c r="H430" s="2" t="inlineStr" /><c r="I430" s="2" t="inlineStr" /><c r="J430" s="2" t="inlineStr" /><c r="K430" s="2" t="inlineStr"><is><t>ma wysoką biodostępność po podaniu doustnym</t></is></c><c r="L430" s="2" t="inlineStr"><is><t>zwiększa wchłanianie witaminy D</t></is></c><c r="M430" s="2" t="inlineStr" /><c r="N430" s="2" t="inlineStr" /><c r="O430" s="2" t="inlineStr" /><c r="P430" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q430" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="431"><c r="A431" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B431" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C431" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D431" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E431" s="2" t="inlineStr"><is><t>Wybierz właściwe zestawienia lek prekursorowy – jego aktywny metabolit:</t></is></c><c r="F431" s="2" t="inlineStr"><is><t>cileksetyl kandesartanu → kandesartan</t></is></c><c r="G431" s="2" t="inlineStr" /><c r="H431" s="2" t="inlineStr" /><c r="I431" s="2" t="inlineStr" /><c r="J431" s="2" t="inlineStr" /><c r="K431" s="2" t="inlineStr"><is><t>eplerenon → kanrenon</t></is></c><c r="L431" s="2" t="inlineStr"><is><t>lizynopryl → lizynoprylat</t></is></c><c r="M431" s="2" t="inlineStr"><is><t>nebiwolol → tlenek azotu</t></is></c><c r="N431" s="2" t="inlineStr" /><c r="O431" s="2" t="inlineStr" /><c r="P431" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q431" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="432"><c r="A432" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B432" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C432" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D432" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E432" s="2" t="inlineStr"><is><t>Torasemid w przeciwieństwie do furosemidu nie powoduje:</t></is></c><c r="F432" s="2" t="inlineStr"><is><t>retencji sodu po efekcie natiuretycznym przy podaniu 1 x 24 h</t></is></c><c r="G432" s="2" t="inlineStr" /><c r="H432" s="2" t="inlineStr" /><c r="I432" s="2" t="inlineStr" /><c r="J432" s="2" t="inlineStr" /><c r="K432" s="2" t="inlineStr"><is><t>efektu natiuretycznego po podaniu doustnym</t></is></c><c r="L432" s="2" t="inlineStr"><is><t>reakcji alergicznych w nadwrażliwości na związki sulfonamidowe</t></is></c><c r="M432" s="2" t="inlineStr"><is><t>hiperkalcemii</t></is></c><c r="N432" s="2" t="inlineStr" /><c r="O432" s="2" t="inlineStr" /><c r="P432" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q432" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="433"><c r="A433" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B433" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C433" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D433" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E433" s="2" t="inlineStr"><is><t>Hiponatremię z dużym stężeniem Na+ w moczu (&gt; 20 mmol/l) może spowodować:</t></is></c><c r="F433" s="2" t="inlineStr"><is><t>karbamazepina</t></is></c><c r="G433" s="2" t="inlineStr"><is><t>fluoksetyna</t></is></c><c r="H433" s="2" t="inlineStr"><is><t>indapamid</t></is></c><c r="I433" s="2" t="inlineStr" /><c r="J433" s="2" t="inlineStr" /><c r="K433" s="2" t="inlineStr"><is><t>prednizon</t></is></c><c r="L433" s="2" t="inlineStr" /><c r="M433" s="2" t="inlineStr" /><c r="N433" s="2" t="inlineStr" /><c r="O433" s="2" t="inlineStr" /><c r="P433" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q433" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="434"><c r="A434" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B434" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C434" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D434" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E434" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek-wskazanie:</t></is></c><c r="F434" s="2" t="inlineStr"><is><t>omalizumab – astma</t></is></c><c r="G434" s="2" t="inlineStr"><is><t>denosumab – osteoporoza</t></is></c><c r="H434" s="2" t="inlineStr" /><c r="I434" s="2" t="inlineStr" /><c r="J434" s="2" t="inlineStr" /><c r="K434" s="2" t="inlineStr"><is><t>natalizumab – reumatoidalne zapalenie stawów</t></is></c><c r="L434" s="2" t="inlineStr"><is><t>infliksymab – stwardnienie rozsiane</t></is></c><c r="M434" s="2" t="inlineStr" /><c r="N434" s="2" t="inlineStr" /><c r="O434" s="2" t="inlineStr" /><c r="P434" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q434" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="435"><c r="A435" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B435" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C435" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D435" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E435" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek – wskazanie:</t></is></c><c r="F435" s="2" t="inlineStr"><is><t>drżenie samoistne – propranolol</t></is></c><c r="G435" s="2" t="inlineStr"><is><t>zespół niespokojnych nóg – pramipeksol</t></is></c><c r="H435" s="2" t="inlineStr"><is><t>padaczka z napadami uogólnionymi toniczno-klonicznymi – kwas walproinowy</t></is></c><c r="I435" s="2" t="inlineStr"><is><t>immunologiczny obrzęk mózgu – deksametazon</t></is></c><c r="J435" s="2" t="inlineStr" /><c r="K435" s="2" t="inlineStr" /><c r="L435" s="2" t="inlineStr" /><c r="M435" s="2" t="inlineStr" /><c r="N435" s="2" t="inlineStr" /><c r="O435" s="2" t="inlineStr" /><c r="P435" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q435" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="436"><c r="A436" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B436" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C436" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D436" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E436" s="2" t="inlineStr"><is><t>Jeśli wartość AUC leku oceniona w badaniach przedklinicznych jest większa po podaniu dożylnym niż po podaniu doustnym, to oznacza, że:</t></is></c><c r="F436" s="2" t="inlineStr"><is><t>brak jest wystarczających danych do określenia przyczyny mniejszej wartości AUC leku po podaniu p.o</t></is></c><c r="G436" s="2" t="inlineStr"><is><t>biodostępność leku po podaniu i.v. jest większa niż po podaniu p.o</t></is></c><c r="H436" s="2" t="inlineStr" /><c r="I436" s="2" t="inlineStr" /><c r="J436" s="2" t="inlineStr" /><c r="K436" s="2" t="inlineStr"><is><t>AUC leku ocenione w badaniach klinicznych będzie podobne</t></is></c><c r="L436" s="2" t="inlineStr"><is><t>lek powinien być stosowany na czczo</t></is></c><c r="M436" s="2" t="inlineStr" /><c r="N436" s="2" t="inlineStr" /><c r="O436" s="2" t="inlineStr" /><c r="P436" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q436" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="437"><c r="A437" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B437" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C437" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D437" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E437" s="2" t="inlineStr"><is><t>Daptomycyna ma dwukompartmentowy model rozmieszczenia w organizmie (t 1/2 α= 7 min i t 1/2β = 5 h). Na tej podstawie uzasadniony jest następujący wniosek:</t></is></c><c r="F437" s="2" t="inlineStr"><is><t>po szybkiej fazie dystrybucji następuje wolniejsza faza eliminacji</t></is></c><c r="G437" s="2" t="inlineStr"><is><t>występuje utrudnienie w redystrybucji leku z tkanek do krążenia ogólnego</t></is></c><c r="H437" s="2" t="inlineStr" /><c r="I437" s="2" t="inlineStr" /><c r="J437" s="2" t="inlineStr" /><c r="K437" s="2" t="inlineStr"><is><t>lek wchłania się na dużej długości przewodu pokarmowego</t></is></c><c r="L437" s="2" t="inlineStr"><is><t>lek rozmieszcza się głównie w obszarach hydrofilnych</t></is></c><c r="M437" s="2" t="inlineStr" /><c r="N437" s="2" t="inlineStr" /><c r="O437" s="2" t="inlineStr" /><c r="P437" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q437" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="438"><c r="A438" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B438" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C438" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D438" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E438" s="2" t="inlineStr"><is><t>W terapii POChP u osób o niewielkim ryzyku i nasilonych objawach (kategoria B) stosuje się:</t></is></c><c r="F438" s="2" t="inlineStr"><is><t>salmeterol</t></is></c><c r="G438" s="2" t="inlineStr"><is><t>bromek aklidynium</t></is></c><c r="H438" s="2" t="inlineStr" /><c r="I438" s="2" t="inlineStr" /><c r="J438" s="2" t="inlineStr" /><c r="K438" s="2" t="inlineStr"><is><t>wziewne glikokortykosteroidy</t></is></c><c r="L438" s="2" t="inlineStr"><is><t>roflumilast</t></is></c><c r="M438" s="2" t="inlineStr" /><c r="N438" s="2" t="inlineStr" /><c r="O438" s="2" t="inlineStr" /><c r="P438" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q438" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="439"><c r="A439" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B439" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C439" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D439" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E439" s="2" t="inlineStr"><is><t>Działanie wykrztuśne ma:</t></is></c><c r="F439" s="2" t="inlineStr"><is><t>wyciąg z prawoślazu lekarskiego</t></is></c><c r="G439" s="2" t="inlineStr"><is><t>gwajafenazyna</t></is></c><c r="H439" s="2" t="inlineStr" /><c r="I439" s="2" t="inlineStr" /><c r="J439" s="2" t="inlineStr" /><c r="K439" s="2" t="inlineStr"><is><t>oksykodon</t></is></c><c r="L439" s="2" t="inlineStr"><is><t>mesna</t></is></c><c r="M439" s="2" t="inlineStr" /><c r="N439" s="2" t="inlineStr" /><c r="O439" s="2" t="inlineStr" /><c r="P439" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q439" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="440"><c r="A440" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B440" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C440" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D440" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E440" s="2" t="inlineStr"><is><t>Indakaterol:</t></is></c><c r="F440" s="2" t="inlineStr"><is><t>zwiększa aktywność ruchową rzęsek</t></is></c><c r="G440" s="2" t="inlineStr"><is><t>wykazuje synergizm działania z glikokortykosteroidami</t></is></c><c r="H440" s="2" t="inlineStr" /><c r="I440" s="2" t="inlineStr" /><c r="J440" s="2" t="inlineStr" /><c r="K440" s="2" t="inlineStr"><is><t>jest beta-adrenomimetykiem wziewnym o krótkim czasie działania (SABA)</t></is></c><c r="L440" s="2" t="inlineStr"><is><t>rozszczepia wiązania disiarczkowe w glikoproteinach śluzu</t></is></c><c r="M440" s="2" t="inlineStr" /><c r="N440" s="2" t="inlineStr" /><c r="O440" s="2" t="inlineStr" /><c r="P440" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q440" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="441"><c r="A441" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B441" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C441" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D441" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E441" s="2" t="inlineStr"><is><t>Meta-analiza badań klinicznych:</t></is></c><c r="F441" s="2" t="inlineStr"><is><t>jest uzupełnieniem przeglądu systematycznego</t></is></c><c r="G441" s="2" t="inlineStr"><is><t>może przynieść zupełnie nowe - odmienne wyniki niż badania, na których jest oparta</t></is></c><c r="H441" s="2" t="inlineStr"><is><t>pozwala zwiększyć precyzję oszacowania efektu klinicznego</t></is></c><c r="I441" s="2" t="inlineStr"><is><t>charakteryzuje się heterogenicznością statystyczną, która istotnie wpływa na interpretację wyników</t></is></c><c r="J441" s="2" t="inlineStr" /><c r="K441" s="2" t="inlineStr" /><c r="L441" s="2" t="inlineStr" /><c r="M441" s="2" t="inlineStr" /><c r="N441" s="2" t="inlineStr" /><c r="O441" s="2" t="inlineStr" /><c r="P441" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q441" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="442"><c r="A442" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B442" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C442" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D442" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E442" s="2" t="inlineStr"><is><t>Mieloidalne czynniki wzrostu (G-CSF oraz GM-CSF) znalazły zastosowanie u pacjentów:</t></is></c><c r="F442" s="2" t="inlineStr"><is><t>z ciężką przewlekłą neutropenią</t></is></c><c r="G442" s="2" t="inlineStr"><is><t>po przeszczepieniu komórek macierzystych szpiku kostnego</t></is></c><c r="H442" s="2" t="inlineStr" /><c r="I442" s="2" t="inlineStr" /><c r="J442" s="2" t="inlineStr" /><c r="K442" s="2" t="inlineStr"><is><t>zakażonych wirusem HIV</t></is></c><c r="L442" s="2" t="inlineStr"><is><t>z idiopatyczną plamicą małopłytkową</t></is></c><c r="M442" s="2" t="inlineStr" /><c r="N442" s="2" t="inlineStr" /><c r="O442" s="2" t="inlineStr" /><c r="P442" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q442" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="443"><c r="A443" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B443" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C443" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D443" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E443" s="2" t="inlineStr"><is><t>Które stwierdzenie dotyczące profilaktyki malarii jest prawdziwe?</t></is></c><c r="F443" s="2" t="inlineStr"><is><t>dla większości leków standardowy czas rozpoczynania stosowania leku w profilaktyce wynosi tydzień przed planowaną podróżą</t></is></c><c r="G443" s="2" t="inlineStr"><is><t>nie dysponujemy uniwersalnym lekiem stosowanym w profilaktyce</t></is></c><c r="H443" s="2" t="inlineStr"><is><t>profilaktyka farmakologiczna stanowi uzupełnienie profilaktyki barierowej (odpowiednie ubrania, moskitiery i siatki nasączone DEET)</t></is></c><c r="I443" s="2" t="inlineStr" /><c r="J443" s="2" t="inlineStr" /><c r="K443" s="2" t="inlineStr"><is><t>leki stosuje się profilaktycznie tylko przez tydzień w czasie pobytu na terenie endemicznym</t></is></c><c r="L443" s="2" t="inlineStr" /><c r="M443" s="2" t="inlineStr" /><c r="N443" s="2" t="inlineStr" /><c r="O443" s="2" t="inlineStr" /><c r="P443" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q443" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="444"><c r="A444" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B444" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C444" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D444" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E444" s="2" t="inlineStr"><is><t>Przeprowadzenie eksperymentu leczniczego:</t></is></c><c r="F444" s="2" t="inlineStr"><is><t>jest możliwe, jeśli dostępne metody leczenia okazały się nieskuteczne</t></is></c><c r="G444" s="2" t="inlineStr"><is><t>wymaga świadomej zgody pacjenta</t></is></c><c r="H444" s="2" t="inlineStr" /><c r="I444" s="2" t="inlineStr" /><c r="J444" s="2" t="inlineStr" /><c r="K444" s="2" t="inlineStr"><is><t>ma na celu głównie poszerzenie wiedzy medycznej</t></is></c><c r="L444" s="2" t="inlineStr"><is><t>nie wymaga pozytywnej opinii Komisji Bioetycznej</t></is></c><c r="M444" s="2" t="inlineStr" /><c r="N444" s="2" t="inlineStr" /><c r="O444" s="2" t="inlineStr" /><c r="P444" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q444" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="445"><c r="A445" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B445" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C445" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D445" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E445" s="2" t="inlineStr"><is><t>W leczeniu niedokrwistości megaloblastycznej zastosowanie ma:</t></is></c><c r="F445" s="2" t="inlineStr"><is><t>cyjanokobalamina</t></is></c><c r="G445" s="2" t="inlineStr"><is><t>kwas foliowy</t></is></c><c r="H445" s="2" t="inlineStr" /><c r="I445" s="2" t="inlineStr" /><c r="J445" s="2" t="inlineStr" /><c r="K445" s="2" t="inlineStr"><is><t>siarczan żelaza</t></is></c><c r="L445" s="2" t="inlineStr"><is><t>erytropoetyna</t></is></c><c r="M445" s="2" t="inlineStr" /><c r="N445" s="2" t="inlineStr" /><c r="O445" s="2" t="inlineStr" /><c r="P445" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q445" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="446"><c r="A446" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B446" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C446" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D446" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E446" s="2" t="inlineStr"><is><t>Preparat złożony naltreksonu z bupropionem:</t></is></c><c r="F446" s="2" t="inlineStr"><is><t>istotnie obniża masę ciała w porównaniu z placebo</t></is></c><c r="G446" s="2" t="inlineStr"><is><t>jest zarejestrowany w Europie do leczenia otyłości</t></is></c><c r="H446" s="2" t="inlineStr"><is><t>sprzyja pojawianiu się myśli samobójczych</t></is></c><c r="I446" s="2" t="inlineStr"><is><t>działa antagonistycznie na receptory 5HT2c</t></is></c><c r="J446" s="2" t="inlineStr" /><c r="K446" s="2" t="inlineStr" /><c r="L446" s="2" t="inlineStr" /><c r="M446" s="2" t="inlineStr" /><c r="N446" s="2" t="inlineStr" /><c r="O446" s="2" t="inlineStr" /><c r="P446" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q446" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="447"><c r="A447" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B447" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C447" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D447" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E447" s="2" t="inlineStr"><is><t>W leczeniu uzależnienia od nikotyny wykazano skuteczność:</t></is></c><c r="F447" s="2" t="inlineStr"><is><t>warenikliny</t></is></c><c r="G447" s="2" t="inlineStr"><is><t>cytyzyny</t></is></c><c r="H447" s="2" t="inlineStr"><is><t>nikotynowej terapii zastępczej</t></is></c><c r="I447" s="2" t="inlineStr" /><c r="J447" s="2" t="inlineStr" /><c r="K447" s="2" t="inlineStr"><is><t>benzodiazepin</t></is></c><c r="L447" s="2" t="inlineStr" /><c r="M447" s="2" t="inlineStr" /><c r="N447" s="2" t="inlineStr" /><c r="O447" s="2" t="inlineStr" /><c r="P447" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q447" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="448"><c r="A448" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B448" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C448" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D448" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E448" s="2" t="inlineStr"><is><t>Elementami nadzoru nad bezpieczeństwem farmakoterapii jest:</t></is></c><c r="F448" s="2" t="inlineStr"><is><t>plan Zarządzania Ryzykiem</t></is></c><c r="G448" s="2" t="inlineStr"><is><t>strona internetowa Urzędu Rejestracji Produktów Leczniczych, Wyrobów Medycznych i Produktów Biobójczych</t></is></c><c r="H448" s="2" t="inlineStr"><is><t>raport PSUR</t></is></c><c r="I448" s="2" t="inlineStr"><is><t>baza zarejestrowanych produktów leczniczych prowadzona przez Europejską Agencję Leków</t></is></c><c r="J448" s="2" t="inlineStr" /><c r="K448" s="2" t="inlineStr" /><c r="L448" s="2" t="inlineStr" /><c r="M448" s="2" t="inlineStr" /><c r="N448" s="2" t="inlineStr" /><c r="O448" s="2" t="inlineStr" /><c r="P448" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q448" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="449"><c r="A449" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B449" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C449" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D449" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E449" s="2" t="inlineStr"><is><t>URPL - Urząd Rejestracji Produktów Leczniczych, Wyrobów Medycznych i Produktów Biobójczych ocenia działania niepożądane zarejestrowanych:</t></is></c><c r="F449" s="2" t="inlineStr"><is><t>leków homeopatycznych</t></is></c><c r="G449" s="2" t="inlineStr"><is><t>leków dostępnych bez recepty</t></is></c><c r="H449" s="2" t="inlineStr"><is><t>leków pochodzenia roślinnego</t></is></c><c r="I449" s="2" t="inlineStr" /><c r="J449" s="2" t="inlineStr" /><c r="K449" s="2" t="inlineStr"><is><t>suplementów diety</t></is></c><c r="L449" s="2" t="inlineStr" /><c r="M449" s="2" t="inlineStr" /><c r="N449" s="2" t="inlineStr" /><c r="O449" s="2" t="inlineStr" /><c r="P449" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q449" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="450"><c r="A450" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B450" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C450" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D450" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E450" s="2" t="inlineStr"><is><t>Teratogenem człowieka o udokumentowanym działaniu jest:</t></is></c><c r="F450" s="2" t="inlineStr"><is><t>metotreksat</t></is></c><c r="G450" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="H450" s="2" t="inlineStr"><is><t>lit</t></is></c><c r="I450" s="2" t="inlineStr" /><c r="J450" s="2" t="inlineStr" /><c r="K450" s="2" t="inlineStr"><is><t>tiamazol tiamazol ma kategorię D</t></is></c><c r="L450" s="2" t="inlineStr" /><c r="M450" s="2" t="inlineStr" /><c r="N450" s="2" t="inlineStr" /><c r="O450" s="2" t="inlineStr" /><c r="P450" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q450" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="451"><c r="A451" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B451" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C451" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D451" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E451" s="2" t="inlineStr"><is><t>Alfakalcydol:</t></is></c><c r="F451" s="2" t="inlineStr"><is><t>koryguje zaburzenia wapniowe w przewlekłej chorobie nerek</t></is></c><c r="G451" s="2" t="inlineStr"><is><t>koryguje zaburzenia wapniowe w niedoczynności przytarczyc</t></is></c><c r="H451" s="2" t="inlineStr"><is><t>zmniejsza ryzyko osteoporotycznych złamań kości</t></is></c><c r="I451" s="2" t="inlineStr" /><c r="J451" s="2" t="inlineStr" /><c r="K451" s="2" t="inlineStr"><is><t>chroni przed chorobami wirusowymi</t></is></c><c r="L451" s="2" t="inlineStr" /><c r="M451" s="2" t="inlineStr" /><c r="N451" s="2" t="inlineStr" /><c r="O451" s="2" t="inlineStr" /><c r="P451" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q451" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="452"><c r="A452" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B452" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C452" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D452" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E452" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie:</t></is></c><c r="F452" s="2" t="inlineStr"><is><t>5% roztwór glukozy jest izotoniczny in vitro i hipotoniczny in vivo</t></is></c><c r="G452" s="2" t="inlineStr"><is><t>15% roztwór mannitolu jest hipertonicznym płynem stosowanym do leczenia obrzęku mózgu</t></is></c><c r="H452" s="2" t="inlineStr" /><c r="I452" s="2" t="inlineStr" /><c r="J452" s="2" t="inlineStr" /><c r="K452" s="2" t="inlineStr"><is><t>stosowanie roztworów hipotonicznych grozi dehydratacją komórek i plazmolizą</t></is></c><c r="L452" s="2" t="inlineStr"><is><t>stosowanie roztworów hipertonicznych grozi obrzękiem komórek i ich lizą</t></is></c><c r="M452" s="2" t="inlineStr" /><c r="N452" s="2" t="inlineStr" /><c r="O452" s="2" t="inlineStr" /><c r="P452" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q452" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="453"><c r="A453" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B453" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C453" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D453" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E453" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie:</t></is></c><c r="F453" s="2" t="inlineStr"><is><t>gliklazyd może powodować przyrost masy ciała</t></is></c><c r="G453" s="2" t="inlineStr"><is><t>metformina może być przyczyną kwasicy mleczanowej</t></is></c><c r="H453" s="2" t="inlineStr"><is><t>empagliflozyna zwiększa ryzyko zakażeń w obrębie miednicy mniejszej</t></is></c><c r="I453" s="2" t="inlineStr" /><c r="J453" s="2" t="inlineStr" /><c r="K453" s="2" t="inlineStr"><is><t>liraglutyd wykazuje niekorzystny efekt sercowo-naczyniowy</t></is></c><c r="L453" s="2" t="inlineStr" /><c r="M453" s="2" t="inlineStr" /><c r="N453" s="2" t="inlineStr" /><c r="O453" s="2" t="inlineStr" /><c r="P453" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q453" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="454"><c r="A454" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B454" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C454" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D454" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E454" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie:</t></is></c><c r="F454" s="2" t="inlineStr"><is><t>bisfosfoniany hamują resorpcję kości przez nasilenie działania osteoprotegeryny na RANKL</t></is></c><c r="G454" s="2" t="inlineStr"><is><t>teryparatyd w małych przerywanych dawkach paradoksalnie zwiększa tworzenie kości</t></is></c><c r="H454" s="2" t="inlineStr"><is><t>ranelinian strontu przez podwójnie korzystne działanie (zwiększa tworzenie i hamuje resorpcję kości) jest lekiem pierwszego wyboru w leczeniu osteoporozy</t></is></c><c r="I454" s="2" t="inlineStr"><is><t>denosumab hamuje resorpcję kości przez zablokowanie interakcji</t></is></c><c r="J454" s="2" t="inlineStr" /><c r="K454" s="2" t="inlineStr" /><c r="L454" s="2" t="inlineStr" /><c r="M454" s="2" t="inlineStr" /><c r="N454" s="2" t="inlineStr" /><c r="O454" s="2" t="inlineStr" /><c r="P454" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q454" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="455"><c r="A455" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B455" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C455" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D455" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E455" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie:</t></is></c><c r="F455" s="2" t="inlineStr"><is><t>furosemid bezpośrednio rozkurcza naczynia krwionośne</t></is></c><c r="G455" s="2" t="inlineStr"><is><t>mannitol redukuje ciśnienie osmotyczne w rdzeniu nerki</t></is></c><c r="H455" s="2" t="inlineStr" /><c r="I455" s="2" t="inlineStr" /><c r="J455" s="2" t="inlineStr" /><c r="K455" s="2" t="inlineStr"><is><t>hydrochlorotiazyd działa natiuretycznie niezależnie od eGFR (wskaźnika filtracji kłębuszkowej)</t></is></c><c r="L455" s="2" t="inlineStr"><is><t>sporonolakton zwiększa objętość krwi krążącej</t></is></c><c r="M455" s="2" t="inlineStr" /><c r="N455" s="2" t="inlineStr" /><c r="O455" s="2" t="inlineStr" /><c r="P455" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q455" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="456"><c r="A456" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B456" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C456" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D456" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E456" s="2" t="inlineStr"><is><t>Klemastyna:</t></is></c><c r="F456" s="2" t="inlineStr"><is><t>dobrze przenika przez barierę krew- mózg</t></is></c><c r="G456" s="2" t="inlineStr"><is><t>może być stosowana od 2 r. ż</t></is></c><c r="H456" s="2" t="inlineStr" /><c r="I456" s="2" t="inlineStr" /><c r="J456" s="2" t="inlineStr" /><c r="K456" s="2" t="inlineStr"><is><t>selektywnie działa na rec. H1</t></is></c><c r="L456" s="2" t="inlineStr"><is><t>jest lekiem z wyboru w leczeniu przewlekłego alergicznego nieżytu nosa</t></is></c><c r="M456" s="2" t="inlineStr" /><c r="N456" s="2" t="inlineStr" /><c r="O456" s="2" t="inlineStr" /><c r="P456" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q456" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="457"><c r="A457" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B457" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C457" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D457" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E457" s="2" t="inlineStr"><is><t>Klemastyna:</t></is></c><c r="F457" s="2" t="inlineStr"><is><t>może być podawana dożylnie</t></is></c><c r="G457" s="2" t="inlineStr"><is><t>powoduje senność i zaburzenia koordynacji ruchów</t></is></c><c r="H457" s="2" t="inlineStr" /><c r="I457" s="2" t="inlineStr" /><c r="J457" s="2" t="inlineStr" /><c r="K457" s="2" t="inlineStr"><is><t>jest selektywnym długodziałającym antagonistą receptorów histaminowych H1</t></is></c><c r="L457" s="2" t="inlineStr"><is><t>jest stosowana doustnie jako lek z wyboru w leczeniu przewlekłym alergii sezonowych</t></is></c><c r="M457" s="2" t="inlineStr" /><c r="N457" s="2" t="inlineStr" /><c r="O457" s="2" t="inlineStr" /><c r="P457" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q457" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="458"><c r="A458" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B458" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C458" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D458" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E458" s="2" t="inlineStr"><is><t>W stanie padaczkowym zalecane jest zastosowanie:</t></is></c><c r="F458" s="2" t="inlineStr"><is><t>lorazepamu dożylnie</t></is></c><c r="G458" s="2" t="inlineStr"><is><t>fenytoiny we wlewie dożylnym</t></is></c><c r="H458" s="2" t="inlineStr" /><c r="I458" s="2" t="inlineStr" /><c r="J458" s="2" t="inlineStr" /><c r="K458" s="2" t="inlineStr"><is><t>diazepamu domięśniowo</t></is></c><c r="L458" s="2" t="inlineStr"><is><t>fenobarbitalu podskórnie</t></is></c><c r="M458" s="2" t="inlineStr" /><c r="N458" s="2" t="inlineStr" /><c r="O458" s="2" t="inlineStr" /><c r="P458" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q458" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="459"><c r="A459" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B459" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C459" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D459" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E459" s="2" t="inlineStr"><is><t>Inhibitorem kinazy tyrozynowej o działaniu przeciwnowotworowym jest:</t></is></c><c r="F459" s="2" t="inlineStr"><is><t>imatynib</t></is></c><c r="G459" s="2" t="inlineStr"><is><t>sunitynib</t></is></c><c r="H459" s="2" t="inlineStr" /><c r="I459" s="2" t="inlineStr" /><c r="J459" s="2" t="inlineStr" /><c r="K459" s="2" t="inlineStr"><is><t>ewerolimus</t></is></c><c r="L459" s="2" t="inlineStr"><is><t>bortezomib</t></is></c><c r="M459" s="2" t="inlineStr" /><c r="N459" s="2" t="inlineStr" /><c r="O459" s="2" t="inlineStr" /><c r="P459" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q459" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="460"><c r="A460" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B460" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C460" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D460" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E460" s="2" t="inlineStr"><is><t>Skuteczne leczenie w owrzodzeniach żylnych obejmuje:</t></is></c><c r="F460" s="2" t="inlineStr"><is><t>opatrunki hydrokoloidowe</t></is></c><c r="G460" s="2" t="inlineStr" /><c r="H460" s="2" t="inlineStr" /><c r="I460" s="2" t="inlineStr" /><c r="J460" s="2" t="inlineStr" /><c r="K460" s="2" t="inlineStr"><is><t>wyciągi zawierające glikozydy kasztanowca</t></is></c><c r="L460" s="2" t="inlineStr"><is><t>heparynoidy do stosowania miejscowego</t></is></c><c r="M460" s="2" t="inlineStr"><is><t>dobesylan wapnia</t></is></c><c r="N460" s="2" t="inlineStr" /><c r="O460" s="2" t="inlineStr" /><c r="P460" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q460" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="461"><c r="A461" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B461" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C461" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D461" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E461" s="2" t="inlineStr"><is><t>W leczeniu zaburzeń lękowych z napadami paniki można zastosować:</t></is></c><c r="F461" s="2" t="inlineStr"><is><t>doksepinę</t></is></c><c r="G461" s="2" t="inlineStr"><is><t>alprazolam</t></is></c><c r="H461" s="2" t="inlineStr" /><c r="I461" s="2" t="inlineStr" /><c r="J461" s="2" t="inlineStr" /><c r="K461" s="2" t="inlineStr"><is><t>rysperydon</t></is></c><c r="L461" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="M461" s="2" t="inlineStr" /><c r="N461" s="2" t="inlineStr" /><c r="O461" s="2" t="inlineStr" /><c r="P461" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q461" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="462"><c r="A462" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B462" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C462" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D462" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E462" s="2" t="inlineStr"><is><t>Działanie przeciwwymiotne ma:</t></is></c><c r="F462" s="2" t="inlineStr"><is><t>skopolamina</t></is></c><c r="G462" s="2" t="inlineStr"><is><t>dimenhydrinat</t></is></c><c r="H462" s="2" t="inlineStr" /><c r="I462" s="2" t="inlineStr" /><c r="J462" s="2" t="inlineStr" /><c r="K462" s="2" t="inlineStr"><is><t>lewetyracetam</t></is></c><c r="L462" s="2" t="inlineStr"><is><t>wortioksetyna</t></is></c><c r="M462" s="2" t="inlineStr" /><c r="N462" s="2" t="inlineStr" /><c r="O462" s="2" t="inlineStr" /><c r="P462" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q462" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="463"><c r="A463" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B463" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C463" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D463" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E463" s="2" t="inlineStr"><is><t>Działanie przeciwwymiotne ma:</t></is></c><c r="F463" s="2" t="inlineStr"><is><t>metoklopramid</t></is></c><c r="G463" s="2" t="inlineStr"><is><t>prometazyna</t></is></c><c r="H463" s="2" t="inlineStr"><is><t>tietylperazyna</t></is></c><c r="I463" s="2" t="inlineStr"><is><t>palonosetron</t></is></c><c r="J463" s="2" t="inlineStr" /><c r="K463" s="2" t="inlineStr" /><c r="L463" s="2" t="inlineStr" /><c r="M463" s="2" t="inlineStr" /><c r="N463" s="2" t="inlineStr" /><c r="O463" s="2" t="inlineStr" /><c r="P463" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q463" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="464"><c r="A464" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B464" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C464" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D464" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E464" s="2" t="inlineStr"><is><t>Amfetamina:</t></is></c><c r="F464" s="2" t="inlineStr"><is><t>może działać neurotoksycznie</t></is></c><c r="G464" s="2" t="inlineStr" /><c r="H464" s="2" t="inlineStr" /><c r="I464" s="2" t="inlineStr" /><c r="J464" s="2" t="inlineStr" /><c r="K464" s="2" t="inlineStr"><is><t>bezpośrednio pobudza receptory dopaminergiczne</t></is></c><c r="L464" s="2" t="inlineStr"><is><t>wzmaga apetyt</t></is></c><c r="M464" s="2" t="inlineStr"><is><t>obniża ciśnienie tętnicze krwi</t></is></c><c r="N464" s="2" t="inlineStr" /><c r="O464" s="2" t="inlineStr" /><c r="P464" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q464" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="465"><c r="A465" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B465" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C465" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D465" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E465" s="2" t="inlineStr"><is><t>Kwetiapina:</t></is></c><c r="F465" s="2" t="inlineStr"><is><t>zwiększa ryzyko wystąpienia zespołu metabolicznego</t></is></c><c r="G465" s="2" t="inlineStr"><is><t>może być stosowana jako lek normotymiczny</t></is></c><c r="H465" s="2" t="inlineStr" /><c r="I465" s="2" t="inlineStr" /><c r="J465" s="2" t="inlineStr" /><c r="K465" s="2" t="inlineStr"><is><t>nie powoduje złośliwego zespołu neuroleptycznego</t></is></c><c r="L465" s="2" t="inlineStr"><is><t>nie wykazuje aktywności cholinolitycznej</t></is></c><c r="M465" s="2" t="inlineStr" /><c r="N465" s="2" t="inlineStr" /><c r="O465" s="2" t="inlineStr" /><c r="P465" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q465" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="466"><c r="A466" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B466" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C466" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D466" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E466" s="2" t="inlineStr"><is><t>Kwetiapina:</t></is></c><c r="F466" s="2" t="inlineStr"><is><t>wpływa na przekaźnictwo serotoninergiczne</t></is></c><c r="G466" s="2" t="inlineStr"><is><t>może być przyczyną zwiększenia masy ciała</t></is></c><c r="H466" s="2" t="inlineStr"><is><t>jest preferowana u pacjentów z współistniejącą chorobą Parkinsona</t></is></c><c r="I466" s="2" t="inlineStr"><is><t>reprezentuje neuroleptyki atypowe</t></is></c><c r="J466" s="2" t="inlineStr" /><c r="K466" s="2" t="inlineStr" /><c r="L466" s="2" t="inlineStr" /><c r="M466" s="2" t="inlineStr" /><c r="N466" s="2" t="inlineStr" /><c r="O466" s="2" t="inlineStr" /><c r="P466" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q466" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="467"><c r="A467" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B467" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C467" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D467" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E467" s="2" t="inlineStr"><is><t>W chorobie Parkinsona lewodopę można podawać jednocześnie z:</t></is></c><c r="F467" s="2" t="inlineStr"><is><t>benserazydem</t></is></c><c r="G467" s="2" t="inlineStr"><is><t>bromokryptyną</t></is></c><c r="H467" s="2" t="inlineStr"><is><t>rotygotyną</t></is></c><c r="I467" s="2" t="inlineStr"><is><t>entekaponem</t></is></c><c r="J467" s="2" t="inlineStr" /><c r="K467" s="2" t="inlineStr" /><c r="L467" s="2" t="inlineStr" /><c r="M467" s="2" t="inlineStr" /><c r="N467" s="2" t="inlineStr" /><c r="O467" s="2" t="inlineStr" /><c r="P467" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q467" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="468"><c r="A468" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B468" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C468" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D468" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E468" s="2" t="inlineStr"><is><t>Wystąpienie objawów pozapiramidowych w przebiegu leczenia lekami przeciwpsychotycznymi:</t></is></c><c r="F468" s="2" t="inlineStr"><is><t>jest wskazaniem do modyfikacji dawki leku</t></is></c><c r="G468" s="2" t="inlineStr"><is><t>zależy od procentu zablokowania receptorów D2 w układzie nigrostriatalnym</t></is></c><c r="H468" s="2" t="inlineStr" /><c r="I468" s="2" t="inlineStr" /><c r="J468" s="2" t="inlineStr" /><c r="K468" s="2" t="inlineStr"><is><t>jest wskazaniem do natychmiastowej zmiany leku</t></is></c><c r="L468" s="2" t="inlineStr"><is><t>jest nieodłącznym elementem leczenia przeciwpsychotycznego, obserwowanym u wszystkich leczonych pacjentów</t></is></c><c r="M468" s="2" t="inlineStr" /><c r="N468" s="2" t="inlineStr" /><c r="O468" s="2" t="inlineStr" /><c r="P468" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q468" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="469"><c r="A469" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B469" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C469" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D469" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E469" s="2" t="inlineStr"><is><t>W leczeniu epizodu depresyjnego można zastosować w monoterapii:</t></is></c><c r="F469" s="2" t="inlineStr"><is><t>sertralinę</t></is></c><c r="G469" s="2" t="inlineStr"><is><t>mirtazapinę</t></is></c><c r="H469" s="2" t="inlineStr" /><c r="I469" s="2" t="inlineStr" /><c r="J469" s="2" t="inlineStr" /><c r="K469" s="2" t="inlineStr"><is><t>sulpiryd</t></is></c><c r="L469" s="2" t="inlineStr"><is><t>sertindol</t></is></c><c r="M469" s="2" t="inlineStr" /><c r="N469" s="2" t="inlineStr" /><c r="O469" s="2" t="inlineStr" /><c r="P469" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q469" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="470"><c r="A470" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B470" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C470" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D470" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E470" s="2" t="inlineStr"><is><t>U chorego leczonego escitalopramem ryzyko wystąpienia zespołu serotoninergicznego rośnie gdy dołączymy do terapii:</t></is></c><c r="F470" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="G470" s="2" t="inlineStr"><is><t>tramadol</t></is></c><c r="H470" s="2" t="inlineStr"><is><t>ziele dziurawca</t></is></c><c r="I470" s="2" t="inlineStr"><is><t>korzeń żeń-szenia</t></is></c><c r="J470" s="2" t="inlineStr" /><c r="K470" s="2" t="inlineStr" /><c r="L470" s="2" t="inlineStr" /><c r="M470" s="2" t="inlineStr" /><c r="N470" s="2" t="inlineStr" /><c r="O470" s="2" t="inlineStr" /><c r="P470" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q470" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="471"><c r="A471" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B471" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C471" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D471" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E471" s="2" t="inlineStr"><is><t>Podanie węgla aktywowanego nie przyniesie efektu w przypadku zatrucia:</t></is></c><c r="F471" s="2" t="inlineStr"><is><t>etanolem</t></is></c><c r="G471" s="2" t="inlineStr"><is><t>ołowiem</t></is></c><c r="H471" s="2" t="inlineStr"><is><t>benzyną</t></is></c><c r="I471" s="2" t="inlineStr" /><c r="J471" s="2" t="inlineStr" /><c r="K471" s="2" t="inlineStr"><is><t>benzodiazepinami</t></is></c><c r="L471" s="2" t="inlineStr" /><c r="M471" s="2" t="inlineStr" /><c r="N471" s="2" t="inlineStr" /><c r="O471" s="2" t="inlineStr" /><c r="P471" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q471" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="472"><c r="A472" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B472" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C472" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D472" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E472" s="2" t="inlineStr"><is><t>U osób w starszym wieku na zmiany farmakokinetyki leków mogą wpływać:</t></is></c><c r="F472" s="2" t="inlineStr"><is><t>hipoproteinemia</t></is></c><c r="G472" s="2" t="inlineStr"><is><t>spadek masy wątroby</t></is></c><c r="H472" s="2" t="inlineStr" /><c r="I472" s="2" t="inlineStr" /><c r="J472" s="2" t="inlineStr" /><c r="K472" s="2" t="inlineStr"><is><t>zanik kosmków jelitowych</t></is></c><c r="L472" s="2" t="inlineStr"><is><t>obniżenie stężenia kwaśnej alfa-1 glikoproteiny</t></is></c><c r="M472" s="2" t="inlineStr" /><c r="N472" s="2" t="inlineStr" /><c r="O472" s="2" t="inlineStr" /><c r="P472" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q472" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="473"><c r="A473" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B473" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C473" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D473" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E473" s="2" t="inlineStr"><is><t>Inhibitorem fosfodiesterazy typu 5 jest:</t></is></c><c r="F473" s="2" t="inlineStr"><is><t>tadalafil</t></is></c><c r="G473" s="2" t="inlineStr" /><c r="H473" s="2" t="inlineStr" /><c r="I473" s="2" t="inlineStr" /><c r="J473" s="2" t="inlineStr" /><c r="K473" s="2" t="inlineStr"><is><t>trospium</t></is></c><c r="L473" s="2" t="inlineStr"><is><t>alprostadyl</t></is></c><c r="M473" s="2" t="inlineStr"><is><t>solifenacyna</t></is></c><c r="N473" s="2" t="inlineStr" /><c r="O473" s="2" t="inlineStr" /><c r="P473" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q473" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="474"><c r="A474" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B474" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C474" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D474" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E474" s="2" t="inlineStr"><is><t>W zespole jelita drażliwego może być skuteczne zastosowanie:</t></is></c><c r="F474" s="2" t="inlineStr"><is><t>mebeweryny</t></is></c><c r="G474" s="2" t="inlineStr"><is><t>atropiny z difenoksylatem</t></is></c><c r="H474" s="2" t="inlineStr"><is><t>trimebutyny</t></is></c><c r="I474" s="2" t="inlineStr"><is><t>Bifidobacterium</t></is></c><c r="J474" s="2" t="inlineStr" /><c r="K474" s="2" t="inlineStr" /><c r="L474" s="2" t="inlineStr" /><c r="M474" s="2" t="inlineStr" /><c r="N474" s="2" t="inlineStr" /><c r="O474" s="2" t="inlineStr" /><c r="P474" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q474" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="475"><c r="A475" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B475" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C475" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D475" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E475" s="2" t="inlineStr"><is><t>Przewlekłe stosowanie pantoprazolu:</t></is></c><c r="F475" s="2" t="inlineStr"><is><t>zwiększa ryzyko zakażeń dróg oddechowych</t></is></c><c r="G475" s="2" t="inlineStr"><is><t>zaburza wchłanianie wapnia z przewodu pokarmowego</t></is></c><c r="H475" s="2" t="inlineStr"><is><t>zmniejsza działanie klopidogrelu</t></is></c><c r="I475" s="2" t="inlineStr" /><c r="J475" s="2" t="inlineStr" /><c r="K475" s="2" t="inlineStr"><is><t>zmniejsza ryzyko złamania szyjki kości udowej</t></is></c><c r="L475" s="2" t="inlineStr" /><c r="M475" s="2" t="inlineStr" /><c r="N475" s="2" t="inlineStr" /><c r="O475" s="2" t="inlineStr" /><c r="P475" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q475" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="476"><c r="A476" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B476" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C476" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D476" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E476" s="2" t="inlineStr"><is><t>Wskazaniem do eradykacji Helicobacter pylori może być:</t></is></c><c r="F476" s="2" t="inlineStr"><is><t>planowane leczenie niesteroidowymi lekami przeciwzapalnymi</t></is></c><c r="G476" s="2" t="inlineStr"><is><t>niedokrwistość syderopeniczna</t></is></c><c r="H476" s="2" t="inlineStr"><is><t>chłoniak żołądka typu MALT</t></is></c><c r="I476" s="2" t="inlineStr"><is><t>aktywna choroba wrzodowa żołądka/dwunastnicy</t></is></c><c r="J476" s="2" t="inlineStr" /><c r="K476" s="2" t="inlineStr" /><c r="L476" s="2" t="inlineStr" /><c r="M476" s="2" t="inlineStr" /><c r="N476" s="2" t="inlineStr" /><c r="O476" s="2" t="inlineStr" /><c r="P476" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q476" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="477"><c r="A477" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B477" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C477" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D477" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E477" s="2" t="inlineStr"><is><t>W profilaktyce krwawienia z żylaków przełyku w przebiegu nadciśnienia wrotnego stosuje się:</t></is></c><c r="F477" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="G477" s="2" t="inlineStr"><is><t>karwedilol</t></is></c><c r="H477" s="2" t="inlineStr" /><c r="I477" s="2" t="inlineStr" /><c r="J477" s="2" t="inlineStr" /><c r="K477" s="2" t="inlineStr"><is><t>doksazosynę</t></is></c><c r="L477" s="2" t="inlineStr"><is><t>klonidynę</t></is></c><c r="M477" s="2" t="inlineStr" /><c r="N477" s="2" t="inlineStr" /><c r="O477" s="2" t="inlineStr" /><c r="P477" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q477" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="478"><c r="A478" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B478" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C478" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D478" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E478" s="2" t="inlineStr"><is><t>Noradrenalinę (NA) podaje się w dawce 0,2-1 μg/kg/min rozpoczynając od najmniejszej dawki. Wskaż właściwą szybkość wlewu w początkowym leczeniu 50 kg kobiety z ciśnieniem skurczowym ok. 60 mmHg w przebiegu ostrej niewydolności serca:</t></is></c><c r="F478" s="2" t="inlineStr"><is><t>roztwór 4 mg NA/40 ml 0,9% NaCl – 6 ml/h</t></is></c><c r="G478" s="2" t="inlineStr"><is><t>roztwór 1 mg NA/50 ml 0,9% NaCl – 30 ml/h</t></is></c><c r="H478" s="2" t="inlineStr"><is><t>roztwór 5 mg NA/25 ml 0,9% NaCl - 3 ml/h</t></is></c><c r="I478" s="2" t="inlineStr"><is><t>roztwór 3 mg NA/30 ml 0,9 % NaCl – 6 ml/h</t></is></c><c r="J478" s="2" t="inlineStr" /><c r="K478" s="2" t="inlineStr" /><c r="L478" s="2" t="inlineStr" /><c r="M478" s="2" t="inlineStr" /><c r="N478" s="2" t="inlineStr" /><c r="O478" s="2" t="inlineStr" /><c r="P478" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q478" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="479"><c r="A479" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B479" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C479" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D479" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E479" s="2" t="inlineStr"><is><t>Działanie naczyniorozszerzające ma:</t></is></c><c r="F479" s="2" t="inlineStr"><is><t>terazosyna</t></is></c><c r="G479" s="2" t="inlineStr"><is><t>nebiwolol</t></is></c><c r="H479" s="2" t="inlineStr"><is><t>zofenopryl</t></is></c><c r="I479" s="2" t="inlineStr"><is><t>lerkanidypina</t></is></c><c r="J479" s="2" t="inlineStr" /><c r="K479" s="2" t="inlineStr" /><c r="L479" s="2" t="inlineStr" /><c r="M479" s="2" t="inlineStr" /><c r="N479" s="2" t="inlineStr" /><c r="O479" s="2" t="inlineStr" /><c r="P479" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q479" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="480"><c r="A480" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B480" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C480" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D480" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E480" s="2" t="inlineStr"><is><t>Podobny mechanizm działania na poziomie molekularnym mają:</t></is></c><c r="F480" s="2" t="inlineStr"><is><t>monoazotan izosorbidu</t></is></c><c r="G480" s="2" t="inlineStr"><is><t>nesirytyd</t></is></c><c r="H480" s="2" t="inlineStr"><is><t>riociguat</t></is></c><c r="I480" s="2" t="inlineStr"><is><t>wardenafil</t></is></c><c r="J480" s="2" t="inlineStr" /><c r="K480" s="2" t="inlineStr" /><c r="L480" s="2" t="inlineStr" /><c r="M480" s="2" t="inlineStr" /><c r="N480" s="2" t="inlineStr" /><c r="O480" s="2" t="inlineStr" /><c r="P480" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q480" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="481"><c r="A481" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B481" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C481" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D481" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E481" s="2" t="inlineStr"><is><t>Beta-adrenolityki w chorobie niedokrwiennej serca:</t></is></c><c r="F481" s="2" t="inlineStr"><is><t>zmniejszają agregację płytek krwi</t></is></c><c r="G481" s="2" t="inlineStr"><is><t>zwiększają przepływ wieńcowy</t></is></c><c r="H481" s="2" t="inlineStr"><is><t>zapobiegają proarytmicznemu działaniu katecholamin</t></is></c><c r="I481" s="2" t="inlineStr"><is><t>zmniejszają kurczliwość mięśnia sercowego</t></is></c><c r="J481" s="2" t="inlineStr" /><c r="K481" s="2" t="inlineStr" /><c r="L481" s="2" t="inlineStr" /><c r="M481" s="2" t="inlineStr" /><c r="N481" s="2" t="inlineStr" /><c r="O481" s="2" t="inlineStr" /><c r="P481" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q481" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="482"><c r="A482" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B482" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C482" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D482" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E482" s="2" t="inlineStr"><is><t>Ranolazyna ma działanie:</t></is></c><c r="F482" s="2" t="inlineStr"><is><t>antyarytmiczne</t></is></c><c r="G482" s="2" t="inlineStr"><is><t>korzystne metaboliczne w kardiomiocytach</t></is></c><c r="H482" s="2" t="inlineStr"><is><t>zmniejszające naprężenie ściany lewej komory</t></is></c><c r="I482" s="2" t="inlineStr" /><c r="J482" s="2" t="inlineStr" /><c r="K482" s="2" t="inlineStr"><is><t>inotropowe dodatnie</t></is></c><c r="L482" s="2" t="inlineStr" /><c r="M482" s="2" t="inlineStr" /><c r="N482" s="2" t="inlineStr" /><c r="O482" s="2" t="inlineStr" /><c r="P482" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q482" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="483"><c r="A483" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B483" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C483" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D483" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E483" s="2" t="inlineStr"><is><t>Jakie leki zlecisz 48-letniemu bezobjawowemu mężczyźnie z BMI = 24,1 kg/m2, palącemu 20 papierosów dziennie od ok. 30 lat, z ciśnieniem tętniczym 150-155 mmHg w powtarzanych pomiarach i ze stężeniem cholesterolu LDL w surowicy = 200 mg/dl:</t></is></c><c r="F483" s="2" t="inlineStr"><is><t>ramipryl</t></is></c><c r="G483" s="2" t="inlineStr"><is><t>nikotynę w inhalacjach pod warunkiem zaprzestania palenia papierosów</t></is></c><c r="H483" s="2" t="inlineStr"><is><t>rosuwastatynę</t></is></c><c r="I483" s="2" t="inlineStr" /><c r="J483" s="2" t="inlineStr" /><c r="K483" s="2" t="inlineStr"><is><t>klopidogrel</t></is></c><c r="L483" s="2" t="inlineStr" /><c r="M483" s="2" t="inlineStr" /><c r="N483" s="2" t="inlineStr" /><c r="O483" s="2" t="inlineStr" /><c r="P483" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q483" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="484"><c r="A484" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B484" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C484" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D484" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E484" s="2" t="inlineStr"><is><t>W niewydolności serca przeżycie chorych poprawia:</t></is></c><c r="F484" s="2" t="inlineStr"><is><t>eplerenon</t></is></c><c r="G484" s="2" t="inlineStr" /><c r="H484" s="2" t="inlineStr" /><c r="I484" s="2" t="inlineStr" /><c r="J484" s="2" t="inlineStr" /><c r="K484" s="2" t="inlineStr"><is><t>atenolol</t></is></c><c r="L484" s="2" t="inlineStr"><is><t>tolwaptan</t></is></c><c r="M484" s="2" t="inlineStr"><is><t>digoksyna</t></is></c><c r="N484" s="2" t="inlineStr" /><c r="O484" s="2" t="inlineStr" /><c r="P484" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q484" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="485"><c r="A485" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B485" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C485" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D485" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E485" s="2" t="inlineStr"><is><t>55-letni mężczyzna ma trwający od ok. 60-min ucisk za mostkiem, który wystąpił podczas ubierania się po wstaniu z łóżka, w EKG rozlane obniżenia ST w odprowadzeniach znad ściany przedniej. Jako lekarz pierwszego kontaktu medycznego zastosujesz:</t></is></c><c r="F485" s="2" t="inlineStr"><is><t>tikagrelor w dawce 180 mg p.o</t></is></c><c r="G485" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy w dawce 300 mg p.o</t></is></c><c r="H485" s="2" t="inlineStr" /><c r="I485" s="2" t="inlineStr" /><c r="J485" s="2" t="inlineStr" /><c r="K485" s="2" t="inlineStr"><is><t>morfinę w dawkach frakcjonowanych i.v</t></is></c><c r="L485" s="2" t="inlineStr"><is><t>enoksaparynę w dawce leczniczej s.c</t></is></c><c r="M485" s="2" t="inlineStr" /><c r="N485" s="2" t="inlineStr" /><c r="O485" s="2" t="inlineStr" /><c r="P485" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q485" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="486"><c r="A486" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B486" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C486" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D486" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E486" s="2" t="inlineStr"><is><t>Które stwierdzenie dotyczące redukcji ryzyka sercowo-naczyniowego jest prawdziwe:</t></is></c><c r="F486" s="2" t="inlineStr"><is><t>nikotynowa terapia zastępcza jest bezpieczna i powinna być rutynowo oferowana</t></is></c><c r="G486" s="2" t="inlineStr" /><c r="H486" s="2" t="inlineStr" /><c r="I486" s="2" t="inlineStr" /><c r="J486" s="2" t="inlineStr" /><c r="K486" s="2" t="inlineStr"><is><t>niezależnie od wieku należy dążyć do redukcji ciśnienia tętniczego do &lt; 140/90 mmHg</t></is></c><c r="L486" s="2" t="inlineStr"><is><t>obniżenie poziomu hemoglobiny glikowanej HgbA1c do ≤ 6% u osób z cukrzycą poprawia przeżycie w porównaniu z wyższymi wartościami HbA1c</t></is></c><c r="M486" s="2" t="inlineStr"><is><t>wysokie prawidłowe ciśnienie krwi powinno być leczone farmakologicznie</t></is></c><c r="N486" s="2" t="inlineStr" /><c r="O486" s="2" t="inlineStr" /><c r="P486" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q486" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="487"><c r="A487" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B487" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C487" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D487" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E487" s="2" t="inlineStr"><is><t>W leczeniu nadciśnienia tętniczego przeciwwskazane jest połączenie:</t></is></c><c r="F487" s="2" t="inlineStr"><is><t>ramipryl + telmisartan</t></is></c><c r="G487" s="2" t="inlineStr" /><c r="H487" s="2" t="inlineStr" /><c r="I487" s="2" t="inlineStr" /><c r="J487" s="2" t="inlineStr" /><c r="K487" s="2" t="inlineStr"><is><t>amlodypina + chlortalidon</t></is></c><c r="L487" s="2" t="inlineStr"><is><t>amlodypina + peryndopryl</t></is></c><c r="M487" s="2" t="inlineStr"><is><t>peryndopryl + indapamid</t></is></c><c r="N487" s="2" t="inlineStr" /><c r="O487" s="2" t="inlineStr" /><c r="P487" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q487" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="488"><c r="A488" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B488" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C488" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D488" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E488" s="2" t="inlineStr"><is><t>U pacjenta z dławicą piersiową i niskim ciśnieniem tętniczym krwi można zastosować:</t></is></c><c r="F488" s="2" t="inlineStr"><is><t>ranolazynę</t></is></c><c r="G488" s="2" t="inlineStr"><is><t>iwabradynę</t></is></c><c r="H488" s="2" t="inlineStr"><is><t>trimetazydynę</t></is></c><c r="I488" s="2" t="inlineStr" /><c r="J488" s="2" t="inlineStr" /><c r="K488" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="L488" s="2" t="inlineStr" /><c r="M488" s="2" t="inlineStr" /><c r="N488" s="2" t="inlineStr" /><c r="O488" s="2" t="inlineStr" /><c r="P488" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q488" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="489"><c r="A489" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B489" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C489" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D489" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E489" s="2" t="inlineStr"><is><t>Propafenon:</t></is></c><c r="F489" s="2" t="inlineStr"><is><t>jest antagonistą kanału sodowego</t></is></c><c r="G489" s="2" t="inlineStr"><is><t>ma działanie betaadrenolityczne</t></is></c><c r="H489" s="2" t="inlineStr" /><c r="I489" s="2" t="inlineStr" /><c r="J489" s="2" t="inlineStr" /><c r="K489" s="2" t="inlineStr"><is><t>rozszerza nasierdziowe tętnice wieńcowe</t></is></c><c r="L489" s="2" t="inlineStr"><is><t>jest przeciwwskazany w zespole preekscytacji (WPW)</t></is></c><c r="M489" s="2" t="inlineStr" /><c r="N489" s="2" t="inlineStr" /><c r="O489" s="2" t="inlineStr" /><c r="P489" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q489" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="490"><c r="A490" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B490" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C490" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D490" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E490" s="2" t="inlineStr"><is><t>Teoretyczną przesłanką stosowania inhibitorów konwertazy angiotensyny w przewlekłej skurczowej niewydolności serca jest:</t></is></c><c r="F490" s="2" t="inlineStr"><is><t>odwracanie włóknienia miokardium</t></is></c><c r="G490" s="2" t="inlineStr"><is><t>odwracanie przerostu kardiomiocytów</t></is></c><c r="H490" s="2" t="inlineStr"><is><t>korzystne bezpośrednie działanie hemodynamiczne</t></is></c><c r="I490" s="2" t="inlineStr" /><c r="J490" s="2" t="inlineStr" /><c r="K490" s="2" t="inlineStr"><is><t>zwiększenie naprężenia ściany lewej komory</t></is></c><c r="L490" s="2" t="inlineStr" /><c r="M490" s="2" t="inlineStr" /><c r="N490" s="2" t="inlineStr" /><c r="O490" s="2" t="inlineStr" /><c r="P490" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q490" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="491"><c r="A491" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B491" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C491" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D491" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E491" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie:</t></is></c><c r="F491" s="2" t="inlineStr"><is><t>Diklofenak działa hepatotoksycznie</t></is></c><c r="G491" s="2" t="inlineStr" /><c r="H491" s="2" t="inlineStr" /><c r="I491" s="2" t="inlineStr" /><c r="J491" s="2" t="inlineStr" /><c r="K491" s="2" t="inlineStr"><is><t>Paracetamol działa antyagregacyjnie</t></is></c><c r="L491" s="2" t="inlineStr"><is><t>Naproksen działa hipotensyjnie</t></is></c><c r="M491" s="2" t="inlineStr"><is><t>Metamizol działa prozakrzepowo</t></is></c><c r="N491" s="2" t="inlineStr" /><c r="O491" s="2" t="inlineStr" /><c r="P491" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q491" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="492"><c r="A492" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B492" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C492" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D492" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E492" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie:</t></is></c><c r="F492" s="2" t="inlineStr"><is><t>buprenorfina może być stosowana w leczeniu substytucyjnym zamiast metadonu</t></is></c><c r="G492" s="2" t="inlineStr"><is><t>petydyna nie powinna być stosowana w okołoporodowym postępowaniu</t></is></c><c r="H492" s="2" t="inlineStr" /><c r="I492" s="2" t="inlineStr" /><c r="J492" s="2" t="inlineStr" /><c r="K492" s="2" t="inlineStr"><is><t>nalokson jest podawany dożylnie, z oksykodonem, w celu zapobiegania występowaniu zaparć poopioidowych</t></is></c><c r="L492" s="2" t="inlineStr"><is><t>fentanyl w plastrach jest stosowany w terapii pooperacyjnego bólu ostrego</t></is></c><c r="M492" s="2" t="inlineStr" /><c r="N492" s="2" t="inlineStr" /><c r="O492" s="2" t="inlineStr" /><c r="P492" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q492" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="493"><c r="A493" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B493" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C493" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D493" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E493" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie:</t></is></c><c r="F493" s="2" t="inlineStr"><is><t>tramadol jest inhibitorem wychwytu zwrotnego serotoniny</t></is></c><c r="G493" s="2" t="inlineStr"><is><t>petydyna jest metabolizowana do neurotoksycznego metabolitu</t></is></c><c r="H493" s="2" t="inlineStr" /><c r="I493" s="2" t="inlineStr" /><c r="J493" s="2" t="inlineStr" /><c r="K493" s="2" t="inlineStr"><is><t>buprenorfinę charakteryzuje wysoki potencjał uzależniający</t></is></c><c r="L493" s="2" t="inlineStr"><is><t>fentanyl w plastrach jest stosowany w leczeniu pooperacyjnego bólu ostrego</t></is></c><c r="M493" s="2" t="inlineStr" /><c r="N493" s="2" t="inlineStr" /><c r="O493" s="2" t="inlineStr" /><c r="P493" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q493" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="494"><c r="A494" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B494" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C494" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D494" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E494" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie:</t></is></c><c r="F494" s="2" t="inlineStr"><is><t>amitryptylina znajduje zastosowanie w terapii bólu neuropatycznego</t></is></c><c r="G494" s="2" t="inlineStr"><is><t>escitalopram hamuje wychwyt zwrotny serotoniny</t></is></c><c r="H494" s="2" t="inlineStr"><is><t>moklobemid może być niebezpieczny u pacjentów spożywających sery dojrzewające</t></is></c><c r="I494" s="2" t="inlineStr"><is><t>mianseryna jest przeciwskazana u osób z padaczką</t></is></c><c r="J494" s="2" t="inlineStr" /><c r="K494" s="2" t="inlineStr" /><c r="L494" s="2" t="inlineStr" /><c r="M494" s="2" t="inlineStr" /><c r="N494" s="2" t="inlineStr" /><c r="O494" s="2" t="inlineStr" /><c r="P494" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q494" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="495"><c r="A495" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B495" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C495" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D495" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E495" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie:</t></is></c><c r="F495" s="2" t="inlineStr"><is><t>Replikacja wirusa może zostać wznowiona po odstawieniu leków, które hamują czynną replikację</t></is></c><c r="G495" s="2" t="inlineStr"><is><t>Obecnie stosowane leki wykazują aktywność wobec wirusów w fazie replikacji</t></is></c><c r="H495" s="2" t="inlineStr" /><c r="I495" s="2" t="inlineStr" /><c r="J495" s="2" t="inlineStr" /><c r="K495" s="2" t="inlineStr"><is><t>Niektóre leki działają na wirusy będące w fazie utajenia</t></is></c><c r="L495" s="2" t="inlineStr"><is><t>Większość wirusów opornych na lek pochodzi od pacjentów z prawidłową odpornością</t></is></c><c r="M495" s="2" t="inlineStr" /><c r="N495" s="2" t="inlineStr" /><c r="O495" s="2" t="inlineStr" /><c r="P495" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q495" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="496"><c r="A496" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B496" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C496" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D496" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E496" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie:</t></is></c><c r="F496" s="2" t="inlineStr"><is><t>Worykonazol wykazuje aktywność wobec Aspergillus spp</t></is></c><c r="G496" s="2" t="inlineStr" /><c r="H496" s="2" t="inlineStr" /><c r="I496" s="2" t="inlineStr" /><c r="J496" s="2" t="inlineStr" /><c r="K496" s="2" t="inlineStr"><is><t>Flukonazol nie wykazuje istotnych klinicznie interakcji na poziomie cytochromu P450</t></is></c><c r="L496" s="2" t="inlineStr"><is><t>Itrakonazol nie wchłania się po podaniu doustnym</t></is></c><c r="M496" s="2" t="inlineStr"><is><t>Posakonazol hamuje syntezę ściany komórkowej grzyba</t></is></c><c r="N496" s="2" t="inlineStr" /><c r="O496" s="2" t="inlineStr" /><c r="P496" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q496" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="497"><c r="A497" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B497" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C497" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D497" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E497" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie:</t></is></c><c r="F497" s="2" t="inlineStr"><is><t>worykonazol jest istotnym klinicznie inhibitorem CYP3A4</t></is></c><c r="G497" s="2" t="inlineStr"><is><t>posakonazol hamuje syntezę ergosterolu</t></is></c><c r="H497" s="2" t="inlineStr" /><c r="I497" s="2" t="inlineStr" /><c r="J497" s="2" t="inlineStr" /><c r="K497" s="2" t="inlineStr"><is><t>flukonazol wykazuje aktywność wobec Aspergillus spp</t></is></c><c r="L497" s="2" t="inlineStr"><is><t>itrakonazol bardzo dobrze wchłania się z przewodu pokarmowego</t></is></c><c r="M497" s="2" t="inlineStr" /><c r="N497" s="2" t="inlineStr" /><c r="O497" s="2" t="inlineStr" /><c r="P497" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q497" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="498"><c r="A498" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B498" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C498" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D498" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E498" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie:</t></is></c><c r="F498" s="2" t="inlineStr"><is><t>ofatumumab to ludzkie przeciwciało skierowane przeciw receptorowi CD20 limfocytów B</t></is></c><c r="G498" s="2" t="inlineStr"><is><t>bazyliksymab to chimeryczne przeciwciało skierowane przeciw receptorowi CD25 na powierzchni limfocytów T</t></is></c><c r="H498" s="2" t="inlineStr" /><c r="I498" s="2" t="inlineStr" /><c r="J498" s="2" t="inlineStr" /><c r="K498" s="2" t="inlineStr"><is><t>rituksymab to chimeryczne przeciwciało skierowane przeciw receptorowi CD52 limfocytów B</t></is></c><c r="L498" s="2" t="inlineStr"><is><t>natalizumab to humanizowane przeciwciało monoklonalne przeciw CD11a limfocytów B</t></is></c><c r="M498" s="2" t="inlineStr" /><c r="N498" s="2" t="inlineStr" /><c r="O498" s="2" t="inlineStr" /><c r="P498" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q498" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="499"><c r="A499" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B499" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C499" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D499" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E499" s="2" t="inlineStr"><is><t>Tramadol jest:</t></is></c><c r="F499" s="2" t="inlineStr"><is><t>Inhibitorem wychwytu zwrotnego serotoniny</t></is></c><c r="G499" s="2" t="inlineStr"><is><t>Agonistą receptorów opioidowych typu μ</t></is></c><c r="H499" s="2" t="inlineStr" /><c r="I499" s="2" t="inlineStr" /><c r="J499" s="2" t="inlineStr" /><c r="K499" s="2" t="inlineStr"><is><t>Inhibitorem wychwytu zwrotnego dopaminy</t></is></c><c r="L499" s="2" t="inlineStr"><is><t>Agonistą receptorów NMDA</t></is></c><c r="M499" s="2" t="inlineStr" /><c r="N499" s="2" t="inlineStr" /><c r="O499" s="2" t="inlineStr" /><c r="P499" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q499" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="500"><c r="A500" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B500" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C500" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D500" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E500" s="2" t="inlineStr"><is><t>Hamowanie enzymu stanowi zasadniczy mechanizm działania:</t></is></c><c r="F500" s="2" t="inlineStr"><is><t>cyklosporyny</t></is></c><c r="G500" s="2" t="inlineStr" /><c r="H500" s="2" t="inlineStr" /><c r="I500" s="2" t="inlineStr" /><c r="J500" s="2" t="inlineStr" /><c r="K500" s="2" t="inlineStr"><is><t>Liraglutydu</t></is></c><c r="L500" s="2" t="inlineStr"><is><t>Lorazepamu</t></is></c><c r="M500" s="2" t="inlineStr"><is><t>Buprenorfiny</t></is></c><c r="N500" s="2" t="inlineStr" /><c r="O500" s="2" t="inlineStr" /><c r="P500" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q500" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="501"><c r="A501" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B501" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C501" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D501" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E501" s="2" t="inlineStr"><is><t>Ryzyko wzrostu masy ciała jest związane z terapią:</t></is></c><c r="F501" s="2" t="inlineStr"><is><t>Olanzapiną</t></is></c><c r="G501" s="2" t="inlineStr"><is><t>Insuliną</t></is></c><c r="H501" s="2" t="inlineStr"><is><t>prednizonem</t></is></c><c r="I501" s="2" t="inlineStr" /><c r="J501" s="2" t="inlineStr" /><c r="K501" s="2" t="inlineStr"><is><t>Liraglutydem</t></is></c><c r="L501" s="2" t="inlineStr" /><c r="M501" s="2" t="inlineStr" /><c r="N501" s="2" t="inlineStr" /><c r="O501" s="2" t="inlineStr" /><c r="P501" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q501" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="502"><c r="A502" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B502" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C502" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D502" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E502" s="2" t="inlineStr"><is><t>Lek A jest stosowany doustnie. Ma właściwości przeciwbólowe, ale nie ma właściwości przeciwzapalnych. Nie powoduje istotnego wzrostu ryzyka powikłań sercowo – naczyniowych. Lekiem A może być:</t></is></c><c r="F502" s="2" t="inlineStr"><is><t>Tramadol</t></is></c><c r="G502" s="2" t="inlineStr"><is><t>Paracetamol</t></is></c><c r="H502" s="2" t="inlineStr" /><c r="I502" s="2" t="inlineStr" /><c r="J502" s="2" t="inlineStr" /><c r="K502" s="2" t="inlineStr"><is><t>Naproksen</t></is></c><c r="L502" s="2" t="inlineStr"><is><t>Celekoksyb</t></is></c><c r="M502" s="2" t="inlineStr" /><c r="N502" s="2" t="inlineStr" /><c r="O502" s="2" t="inlineStr" /><c r="P502" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q502" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="503"><c r="A503" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B503" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C503" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D503" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E503" s="2" t="inlineStr"><is><t>Bisfosfoniany są stosowane:</t></is></c><c r="F503" s="2" t="inlineStr"><is><t>w leczeniu osteoporozy posteroidowej</t></is></c><c r="G503" s="2" t="inlineStr"><is><t>w leczeniu ciężkiej hiperkalcemii</t></is></c><c r="H503" s="2" t="inlineStr" /><c r="I503" s="2" t="inlineStr" /><c r="J503" s="2" t="inlineStr" /><c r="K503" s="2" t="inlineStr"><is><t>w celu przyspieszania zrostu kości po złamaniach</t></is></c><c r="L503" s="2" t="inlineStr"><is><t>przeciwbólowo w chorobie zwyrodnieniowej stawów</t></is></c><c r="M503" s="2" t="inlineStr" /><c r="N503" s="2" t="inlineStr" /><c r="O503" s="2" t="inlineStr" /><c r="P503" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q503" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="504"><c r="A504" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B504" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C504" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D504" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E504" s="2" t="inlineStr"><is><t>20% roztwór albumin to:</t></is></c><c r="F504" s="2" t="inlineStr"><is><t>lek krwiopochodny</t></is></c><c r="G504" s="2" t="inlineStr"><is><t>koloid zatrzymujący płyny w przestrzeni wewnątrznaczyniowej</t></is></c><c r="H504" s="2" t="inlineStr" /><c r="I504" s="2" t="inlineStr" /><c r="J504" s="2" t="inlineStr" /><c r="K504" s="2" t="inlineStr"><is><t>substancja do żywienia pozajelitowego</t></is></c><c r="L504" s="2" t="inlineStr"><is><t>łatwo dostępny i tani płyn do nawadniania</t></is></c><c r="M504" s="2" t="inlineStr" /><c r="N504" s="2" t="inlineStr" /><c r="O504" s="2" t="inlineStr" /><c r="P504" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q504" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="505"><c r="A505" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B505" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C505" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D505" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E505" s="2" t="inlineStr"><is><t>W leczeniu wymiotów indukowanych chemioterapią znajduje zastosowanie:</t></is></c><c r="F505" s="2" t="inlineStr"><is><t>Deksametazon</t></is></c><c r="G505" s="2" t="inlineStr"><is><t>Palonosetron</t></is></c><c r="H505" s="2" t="inlineStr"><is><t>metoklopramid</t></is></c><c r="I505" s="2" t="inlineStr" /><c r="J505" s="2" t="inlineStr" /><c r="K505" s="2" t="inlineStr"><is><t>Dimenhydrynat</t></is></c><c r="L505" s="2" t="inlineStr" /><c r="M505" s="2" t="inlineStr" /><c r="N505" s="2" t="inlineStr" /><c r="O505" s="2" t="inlineStr" /><c r="P505" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q505" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="506"><c r="A506" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B506" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C506" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D506" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E506" s="2" t="inlineStr"><is><t>Klozapina może być przyczyną:</t></is></c><c r="F506" s="2" t="inlineStr"><is><t>obniżenia progu drgawkowego</t></is></c><c r="G506" s="2" t="inlineStr"><is><t>przyrostu masy ciała</t></is></c><c r="H506" s="2" t="inlineStr"><is><t>agranulocytozy</t></is></c><c r="I506" s="2" t="inlineStr" /><c r="J506" s="2" t="inlineStr" /><c r="K506" s="2" t="inlineStr"><is><t>Hiperprolaktynemii</t></is></c><c r="L506" s="2" t="inlineStr" /><c r="M506" s="2" t="inlineStr" /><c r="N506" s="2" t="inlineStr" /><c r="O506" s="2" t="inlineStr" /><c r="P506" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q506" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="507"><c r="A507" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B507" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C507" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D507" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E507" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – mechanizm działania:</t></is></c><c r="F507" s="2" t="inlineStr"><is><t>buspiron – agonista rec. 5HT1A</t></is></c><c r="G507" s="2" t="inlineStr"><is><t>diazepam – agonista rec. GABA-A</t></is></c><c r="H507" s="2" t="inlineStr" /><c r="I507" s="2" t="inlineStr" /><c r="J507" s="2" t="inlineStr" /><c r="K507" s="2" t="inlineStr"><is><t>zolpidem – agonista rec. H2</t></is></c><c r="L507" s="2" t="inlineStr"><is><t>mirtazapina – agonista rec. alfa2</t></is></c><c r="M507" s="2" t="inlineStr" /><c r="N507" s="2" t="inlineStr" /><c r="O507" s="2" t="inlineStr" /><c r="P507" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q507" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="508"><c r="A508" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B508" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C508" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D508" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E508" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – mechanizm działania:</t></is></c><c r="F508" s="2" t="inlineStr"><is><t>plazomycyna – hamuje syntezę białek</t></is></c><c r="G508" s="2" t="inlineStr" /><c r="H508" s="2" t="inlineStr" /><c r="I508" s="2" t="inlineStr" /><c r="J508" s="2" t="inlineStr" /><c r="K508" s="2" t="inlineStr"><is><t>dalbawancyna – hamuje syntezy DNA</t></is></c><c r="L508" s="2" t="inlineStr"><is><t>spiramycyna – hamuje syntezę RNA</t></is></c><c r="M508" s="2" t="inlineStr"><is><t>telitromycyna – hamuje syntezę ściany komórkowej</t></is></c><c r="N508" s="2" t="inlineStr" /><c r="O508" s="2" t="inlineStr" /><c r="P508" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q508" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="509"><c r="A509" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B509" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C509" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D509" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E509" s="2" t="inlineStr"><is><t>Benzodiazepiny są stosowane w:</t></is></c><c r="F509" s="2" t="inlineStr"><is><t>premedykacji</t></is></c><c r="G509" s="2" t="inlineStr"><is><t>terapii padaczki</t></is></c><c r="H509" s="2" t="inlineStr" /><c r="I509" s="2" t="inlineStr" /><c r="J509" s="2" t="inlineStr" /><c r="K509" s="2" t="inlineStr"><is><t>długotrwałej terapii bezsenności</t></is></c><c r="L509" s="2" t="inlineStr"><is><t>zespole abstynencyjnym u chorych uzależnionych od morfiny</t></is></c><c r="M509" s="2" t="inlineStr" /><c r="N509" s="2" t="inlineStr" /><c r="O509" s="2" t="inlineStr" /><c r="P509" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q509" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="510"><c r="A510" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B510" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C510" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D510" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E510" s="2" t="inlineStr"><is><t>Zespół serotoninowy może być wynikiem interakcji cytalopramu z:</t></is></c><c r="F510" s="2" t="inlineStr"><is><t>Tramadolem</t></is></c><c r="G510" s="2" t="inlineStr"><is><t>klomipraminą</t></is></c><c r="H510" s="2" t="inlineStr" /><c r="I510" s="2" t="inlineStr" /><c r="J510" s="2" t="inlineStr" /><c r="K510" s="2" t="inlineStr"><is><t>Oksazepamem</t></is></c><c r="L510" s="2" t="inlineStr"><is><t>Buprenorfiną</t></is></c><c r="M510" s="2" t="inlineStr" /><c r="N510" s="2" t="inlineStr" /><c r="O510" s="2" t="inlineStr" /><c r="P510" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q510" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="511"><c r="A511" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B511" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C511" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D511" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E511" s="2" t="inlineStr"><is><t>Charakterystyka Produktu Leczniczego zawiera informacje o:</t></is></c><c r="F511" s="2" t="inlineStr"><is><t>przeciwwskazaniach do stosowania</t></is></c><c r="G511" s="2" t="inlineStr"><is><t>właściwościach farmakokinetycznych</t></is></c><c r="H511" s="2" t="inlineStr"><is><t>okresie ważności</t></is></c><c r="I511" s="2" t="inlineStr" /><c r="J511" s="2" t="inlineStr" /><c r="K511" s="2" t="inlineStr"><is><t>zakresie refundacji</t></is></c><c r="L511" s="2" t="inlineStr" /><c r="M511" s="2" t="inlineStr" /><c r="N511" s="2" t="inlineStr" /><c r="O511" s="2" t="inlineStr" /><c r="P511" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q511" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="512"><c r="A512" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B512" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C512" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D512" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E512" s="2" t="inlineStr"><is><t>Charakterystyka Produktu Leczniczego zawiera informacje o:</t></is></c><c r="F512" s="2" t="inlineStr"><is><t>mechanizmie działania</t></is></c><c r="G512" s="2" t="inlineStr"><is><t>interakcjach</t></is></c><c r="H512" s="2" t="inlineStr"><is><t>substancjach pomocniczych</t></is></c><c r="I512" s="2" t="inlineStr"><is><t>działaniach niepożądanych</t></is></c><c r="J512" s="2" t="inlineStr" /><c r="K512" s="2" t="inlineStr" /><c r="L512" s="2" t="inlineStr" /><c r="M512" s="2" t="inlineStr" /><c r="N512" s="2" t="inlineStr" /><c r="O512" s="2" t="inlineStr" /><c r="P512" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q512" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="513"><c r="A513" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B513" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C513" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D513" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E513" s="2" t="inlineStr"><is><t>Przyczyną nieliniowego przebiegu procesów farmakokinetycznych może być:</t></is></c><c r="F513" s="2" t="inlineStr"><is><t>autoindukcja metabolizmu</t></is></c><c r="G513" s="2" t="inlineStr"><is><t>niedobór kosubstratów w procesie sprzęgania</t></is></c><c r="H513" s="2" t="inlineStr"><is><t>wysycenie transporterów</t></is></c><c r="I513" s="2" t="inlineStr" /><c r="J513" s="2" t="inlineStr" /><c r="K513" s="2" t="inlineStr"><is><t>wąski wskaźnik terapeutyczny leku</t></is></c><c r="L513" s="2" t="inlineStr" /><c r="M513" s="2" t="inlineStr" /><c r="N513" s="2" t="inlineStr" /><c r="O513" s="2" t="inlineStr" /><c r="P513" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q513" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="514"><c r="A514" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B514" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C514" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D514" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E514" s="2" t="inlineStr"><is><t>Insulina aspart:</t></is></c><c r="F514" s="2" t="inlineStr"><is><t>działa za pośrednictwem receptora błonowego</t></is></c><c r="G514" s="2" t="inlineStr"><is><t>może być podawana we wstrzyknięciu podskórnym</t></is></c><c r="H514" s="2" t="inlineStr" /><c r="I514" s="2" t="inlineStr" /><c r="J514" s="2" t="inlineStr" /><c r="K514" s="2" t="inlineStr"><is><t>jest stosowana wyłącznie w cukrzycy typu 1</t></is></c><c r="L514" s="2" t="inlineStr"><is><t>jest analogiem długodziałającym</t></is></c><c r="M514" s="2" t="inlineStr" /><c r="N514" s="2" t="inlineStr" /><c r="O514" s="2" t="inlineStr" /><c r="P514" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q514" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="515"><c r="A515" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B515" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C515" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D515" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E515" s="2" t="inlineStr"><is><t>Na proces dystrybucji leku może mieć wpływ:</t></is></c><c r="F515" s="2" t="inlineStr"><is><t>niewydolność krążenia</t></is></c><c r="G515" s="2" t="inlineStr"><is><t>Hipoalbuminemia</t></is></c><c r="H515" s="2" t="inlineStr" /><c r="I515" s="2" t="inlineStr" /><c r="J515" s="2" t="inlineStr" /><c r="K515" s="2" t="inlineStr"><is><t>obecność pokarmu w przypadku podania doustnego</t></is></c><c r="L515" s="2" t="inlineStr"><is><t>możliwość sprzęgania z kwasem glukuronowym</t></is></c><c r="M515" s="2" t="inlineStr" /><c r="N515" s="2" t="inlineStr" /><c r="O515" s="2" t="inlineStr" /><c r="P515" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q515" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="516"><c r="A516" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B516" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C516" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D516" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E516" s="2" t="inlineStr"><is><t>Agonistą receptorów jest:</t></is></c><c r="F516" s="2" t="inlineStr"><is><t>tapentadol</t></is></c><c r="G516" s="2" t="inlineStr" /><c r="H516" s="2" t="inlineStr" /><c r="I516" s="2" t="inlineStr" /><c r="J516" s="2" t="inlineStr" /><c r="K516" s="2" t="inlineStr"><is><t>Sertralina</t></is></c><c r="L516" s="2" t="inlineStr"><is><t>Eplerenon</t></is></c><c r="M516" s="2" t="inlineStr"><is><t>Fenytoina</t></is></c><c r="N516" s="2" t="inlineStr" /><c r="O516" s="2" t="inlineStr" /><c r="P516" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q516" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="517"><c r="A517" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B517" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C517" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D517" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E517" s="2" t="inlineStr"><is><t>W trakcie długotrwałej terapii glikokortykosteroidami, wskazane jest monitorowanie:</t></is></c><c r="F517" s="2" t="inlineStr"><is><t>stężenia potasu we krwi</t></is></c><c r="G517" s="2" t="inlineStr"><is><t>ciśnienia tętniczego krwi</t></is></c><c r="H517" s="2" t="inlineStr"><is><t>ciśnienia wewnątrzgałkowego</t></is></c><c r="I517" s="2" t="inlineStr"><is><t>glikemii</t></is></c><c r="J517" s="2" t="inlineStr" /><c r="K517" s="2" t="inlineStr" /><c r="L517" s="2" t="inlineStr" /><c r="M517" s="2" t="inlineStr" /><c r="N517" s="2" t="inlineStr" /><c r="O517" s="2" t="inlineStr" /><c r="P517" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q517" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="518"><c r="A518" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B518" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C518" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D518" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E518" s="2" t="inlineStr"><is><t>Inhibitory kotransportera sodowo-glukozowego 2 (SGLT-2, flozyny):</t></is></c><c r="F518" s="2" t="inlineStr"><is><t>Mogą być stosowane łącznie z metforminą</t></is></c><c r="G518" s="2" t="inlineStr"><is><t>Mogą zwiększać diurezę</t></is></c><c r="H518" s="2" t="inlineStr"><is><t>Mają udowodnione korzystne działanie w zakresie ryzyka sercowo-naczyniowego</t></is></c><c r="I518" s="2" t="inlineStr" /><c r="J518" s="2" t="inlineStr" /><c r="K518" s="2" t="inlineStr"><is><t>Charakteryzują się wysokim ryzykiem wystąpienia hipoglikemii</t></is></c><c r="L518" s="2" t="inlineStr" /><c r="M518" s="2" t="inlineStr" /><c r="N518" s="2" t="inlineStr" /><c r="O518" s="2" t="inlineStr" /><c r="P518" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q518" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="519"><c r="A519" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B519" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C519" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D519" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E519" s="2" t="inlineStr"><is><t>Przeciwciała monoklonalne znajdują zastosowanie w terapii:</t></is></c><c r="F519" s="2" t="inlineStr"><is><t>choroby Leśniowskiego i Crohna</t></is></c><c r="G519" s="2" t="inlineStr"><is><t>stwardnienia rozsianego</t></is></c><c r="H519" s="2" t="inlineStr"><is><t>reumatoidalnego zapalenia stawów</t></is></c><c r="I519" s="2" t="inlineStr" /><c r="J519" s="2" t="inlineStr" /><c r="K519" s="2" t="inlineStr"><is><t>mononukleozy</t></is></c><c r="L519" s="2" t="inlineStr" /><c r="M519" s="2" t="inlineStr" /><c r="N519" s="2" t="inlineStr" /><c r="O519" s="2" t="inlineStr" /><c r="P519" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q519" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="520"><c r="A520" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B520" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C520" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D520" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E520" s="2" t="inlineStr"><is><t>Zaburzenia rytmu serca mogą wystąpić w trakcie podawania:</t></is></c><c r="F520" s="2" t="inlineStr"><is><t>Amisulpirydu</t></is></c><c r="G520" s="2" t="inlineStr"><is><t>Ondansetronu</t></is></c><c r="H520" s="2" t="inlineStr"><is><t>Chlorpromazyny</t></is></c><c r="I520" s="2" t="inlineStr"><is><t>metadonu</t></is></c><c r="J520" s="2" t="inlineStr" /><c r="K520" s="2" t="inlineStr" /><c r="L520" s="2" t="inlineStr" /><c r="M520" s="2" t="inlineStr" /><c r="N520" s="2" t="inlineStr" /><c r="O520" s="2" t="inlineStr" /><c r="P520" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q520" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="521"><c r="A521" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B521" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C521" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D521" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E521" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące terapii niedokrwistości z niedoboru żelaza:</t></is></c><c r="F521" s="2" t="inlineStr"><is><t>preferowana jest doustna suplementacja żelaza</t></is></c><c r="G521" s="2" t="inlineStr" /><c r="H521" s="2" t="inlineStr" /><c r="I521" s="2" t="inlineStr" /><c r="J521" s="2" t="inlineStr" /><c r="K521" s="2" t="inlineStr"><is><t>terapia trwa 2 tygodnie</t></is></c><c r="L521" s="2" t="inlineStr"><is><t>preparaty dożylne żelaza są przeciwwskazane u chorych z przewlekłą niewydolnością nerek</t></is></c><c r="M521" s="2" t="inlineStr"><is><t>tabletki z żelazem należy popijać herbatą</t></is></c><c r="N521" s="2" t="inlineStr" /><c r="O521" s="2" t="inlineStr" /><c r="P521" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q521" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="522"><c r="A522" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B522" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C522" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D522" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E522" s="2" t="inlineStr"><is><t>Działanie normotymizujące wykazują:</t></is></c><c r="F522" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="G522" s="2" t="inlineStr"><is><t>Lamotrygina</t></is></c><c r="H522" s="2" t="inlineStr"><is><t>Olanzapina</t></is></c><c r="I522" s="2" t="inlineStr"><is><t>sole litu</t></is></c><c r="J522" s="2" t="inlineStr" /><c r="K522" s="2" t="inlineStr" /><c r="L522" s="2" t="inlineStr" /><c r="M522" s="2" t="inlineStr" /><c r="N522" s="2" t="inlineStr" /><c r="O522" s="2" t="inlineStr" /><c r="P522" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q522" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="523"><c r="A523" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B523" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C523" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D523" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E523" s="2" t="inlineStr"><is><t>Udowodnione działanie immunostymulujące wykazuje:</t></is></c><c r="F523" s="2" t="inlineStr"><is><t>filgrastym</t></is></c><c r="G523" s="2" t="inlineStr" /><c r="H523" s="2" t="inlineStr" /><c r="I523" s="2" t="inlineStr" /><c r="J523" s="2" t="inlineStr" /><c r="K523" s="2" t="inlineStr"><is><t>wyciąg z korzenia jeżówki purpurowej</t></is></c><c r="L523" s="2" t="inlineStr"><is><t>pranobeks inozyny</t></is></c><c r="M523" s="2" t="inlineStr"><is><t>alkoholowy wyciąg z dziurawca</t></is></c><c r="N523" s="2" t="inlineStr" /><c r="O523" s="2" t="inlineStr" /><c r="P523" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q523" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="524"><c r="A524" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B524" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C524" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D524" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E524" s="2" t="inlineStr"><is><t>Ryzyka rozwoju zależności można się spodziewać przy stosowaniu:</t></is></c><c r="F524" s="2" t="inlineStr"><is><t>Dihydrokodeiny</t></is></c><c r="G524" s="2" t="inlineStr"><is><t>Diazepamu</t></is></c><c r="H524" s="2" t="inlineStr" /><c r="I524" s="2" t="inlineStr" /><c r="J524" s="2" t="inlineStr" /><c r="K524" s="2" t="inlineStr"><is><t>Diklofenaku</t></is></c><c r="L524" s="2" t="inlineStr"><is><t>duloksetyny</t></is></c><c r="M524" s="2" t="inlineStr" /><c r="N524" s="2" t="inlineStr" /><c r="O524" s="2" t="inlineStr" /><c r="P524" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q524" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="525"><c r="A525" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B525" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C525" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D525" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E525" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek przeciwdepresyjny – mechanizm działania:</t></is></c><c r="F525" s="2" t="inlineStr"><is><t>reboksetyna – selektywny inhibitor wychwytu zwrotnego noradrenaliny</t></is></c><c r="G525" s="2" t="inlineStr"><is><t>bupropion – inhibitor wychwytu zwrotnego noradrenaliny i dopaminy</t></is></c><c r="H525" s="2" t="inlineStr"><is><t>fluoksetyna – selektywny inhibitor wychwytu zwrotnego serotoniny</t></is></c><c r="I525" s="2" t="inlineStr"><is><t>wenlafaksyna – inhibitor wychwytu zwrotnego serotoniny i noradrenaliny</t></is></c><c r="J525" s="2" t="inlineStr" /><c r="K525" s="2" t="inlineStr" /><c r="L525" s="2" t="inlineStr" /><c r="M525" s="2" t="inlineStr" /><c r="N525" s="2" t="inlineStr" /><c r="O525" s="2" t="inlineStr" /><c r="P525" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q525" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="526"><c r="A526" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B526" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C526" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D526" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E526" s="2" t="inlineStr"><is><t>Ryzyko gastrotoksycznego działania ketoprofenu może istotnie wzrosnąć przy jednoczesnym podawaniu:</t></is></c><c r="F526" s="2" t="inlineStr"><is><t>Spironolaktonu</t></is></c><c r="G526" s="2" t="inlineStr"><is><t>prednizonu</t></is></c><c r="H526" s="2" t="inlineStr" /><c r="I526" s="2" t="inlineStr" /><c r="J526" s="2" t="inlineStr" /><c r="K526" s="2" t="inlineStr"><is><t>Mizoprostolu</t></is></c><c r="L526" s="2" t="inlineStr"><is><t>Omeprazolu</t></is></c><c r="M526" s="2" t="inlineStr" /><c r="N526" s="2" t="inlineStr" /><c r="O526" s="2" t="inlineStr" /><c r="P526" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q526" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="527"><c r="A527" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B527" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C527" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D527" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E527" s="2" t="inlineStr"><is><t>Morfina może być przyczyną:</t></is></c><c r="F527" s="2" t="inlineStr"><is><t>obniżenia progu drgawkowego</t></is></c><c r="G527" s="2" t="inlineStr"><is><t>skurczu oskrzeli</t></is></c><c r="H527" s="2" t="inlineStr" /><c r="I527" s="2" t="inlineStr" /><c r="J527" s="2" t="inlineStr" /><c r="K527" s="2" t="inlineStr"><is><t>rozszerzenia źrenic</t></is></c><c r="L527" s="2" t="inlineStr"><is><t>działania moczopędnego</t></is></c><c r="M527" s="2" t="inlineStr" /><c r="N527" s="2" t="inlineStr" /><c r="O527" s="2" t="inlineStr" /><c r="P527" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 1 termin</t></is></c><c r="Q527" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="528"><c r="A528" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B528" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C528" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D528" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E528" s="2" t="inlineStr"><is><t>Wskaż fałszywe stwierdzenie:</t></is></c><c r="F528" s="2" t="inlineStr"><is><t>suplement diety to lek stosowany wspomagająco</t></is></c><c r="G528" s="2" t="inlineStr" /><c r="H528" s="2" t="inlineStr" /><c r="I528" s="2" t="inlineStr" /><c r="J528" s="2" t="inlineStr" /><c r="K528" s="2" t="inlineStr"><is><t>produkt leczniczy to substancja, której przypisuje się, między innymi, właściwości zapobiegania chorobom występującym u ludzi</t></is></c><c r="L528" s="2" t="inlineStr"><is><t>wyrób medyczny to przyrząd lub inny artykuł stosowany w celu diagnozowania, zapobiegania, monitorowania, leczenia lub łagodzenia przebiegu chorób</t></is></c><c r="M528" s="2" t="inlineStr"><is><t>roztwór albumin należy do kategorii produktów krwiopochodnych</t></is></c><c r="N528" s="2" t="inlineStr" /><c r="O528" s="2" t="inlineStr" /><c r="P528" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q528" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="529"><c r="A529" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B529" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C529" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D529" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E529" s="2" t="inlineStr"><is><t>Nalokson:</t></is></c><c r="F529" s="2" t="inlineStr"><is><t>słabo wchłania się z przewodu pokarmowego</t></is></c><c r="G529" s="2" t="inlineStr"><is><t>nie wywołuje uzależnienia</t></is></c><c r="H529" s="2" t="inlineStr" /><c r="I529" s="2" t="inlineStr" /><c r="J529" s="2" t="inlineStr" /><c r="K529" s="2" t="inlineStr"><is><t>jest agonistą receptorów opioidowych</t></is></c><c r="L529" s="2" t="inlineStr"><is><t>powoduje depresję ośrodka oddechowego</t></is></c><c r="M529" s="2" t="inlineStr" /><c r="N529" s="2" t="inlineStr" /><c r="O529" s="2" t="inlineStr" /><c r="P529" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q529" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="530"><c r="A530" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B530" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C530" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D530" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E530" s="2" t="inlineStr"><is><t>Antagonizm wobec receptora stanowi zasadniczy mechanizm działania:</t></is></c><c r="F530" s="2" t="inlineStr"><is><t>flumazenilu</t></is></c><c r="G530" s="2" t="inlineStr" /><c r="H530" s="2" t="inlineStr" /><c r="I530" s="2" t="inlineStr" /><c r="J530" s="2" t="inlineStr" /><c r="K530" s="2" t="inlineStr"><is><t>Cyklosporyny</t></is></c><c r="L530" s="2" t="inlineStr"><is><t>Lorazepamu</t></is></c><c r="M530" s="2" t="inlineStr"><is><t>Tapentadolu</t></is></c><c r="N530" s="2" t="inlineStr" /><c r="O530" s="2" t="inlineStr" /><c r="P530" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q530" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="531"><c r="A531" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B531" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C531" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D531" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E531" s="2" t="inlineStr"><is><t>Zmniejszenie masy ciała może wiązać się z terapią:</t></is></c><c r="F531" s="2" t="inlineStr"><is><t>Lewotyroksyną</t></is></c><c r="G531" s="2" t="inlineStr"><is><t>metforminą</t></is></c><c r="H531" s="2" t="inlineStr" /><c r="I531" s="2" t="inlineStr" /><c r="J531" s="2" t="inlineStr" /><c r="K531" s="2" t="inlineStr"><is><t>Olanzapiną</t></is></c><c r="L531" s="2" t="inlineStr"><is><t>Prednizonem</t></is></c><c r="M531" s="2" t="inlineStr" /><c r="N531" s="2" t="inlineStr" /><c r="O531" s="2" t="inlineStr" /><c r="P531" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q531" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="532"><c r="A532" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B532" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C532" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D532" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E532" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – działanie niepożądane:</t></is></c><c r="F532" s="2" t="inlineStr"><is><t>tietylperazyna - akatyzja</t></is></c><c r="G532" s="2" t="inlineStr"><is><t>metoklopramid – późne dyskinezy</t></is></c><c r="H532" s="2" t="inlineStr"><is><t>ondansetron – wydłużenie odstępu QT</t></is></c><c r="I532" s="2" t="inlineStr" /><c r="J532" s="2" t="inlineStr" /><c r="K532" s="2" t="inlineStr"><is><t>dimenhydrynat - wymioty</t></is></c><c r="L532" s="2" t="inlineStr" /><c r="M532" s="2" t="inlineStr" /><c r="N532" s="2" t="inlineStr" /><c r="O532" s="2" t="inlineStr" /><c r="P532" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q532" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="533"><c r="A533" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B533" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C533" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D533" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E533" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek - działanie niepożądane:</t></is></c><c r="F533" s="2" t="inlineStr"><is><t>Izoniazyd – toczen polekowy</t></is></c><c r="G533" s="2" t="inlineStr"><is><t>Ryfampicyna - śródmiąższowe zapalenie nerek</t></is></c><c r="H533" s="2" t="inlineStr"><is><t>Pirazynamid – hiperurykemia</t></is></c><c r="I533" s="2" t="inlineStr"><is><t>Etambutol - pozagałkowa zapalenie nerwu wzrokowego</t></is></c><c r="J533" s="2" t="inlineStr" /><c r="K533" s="2" t="inlineStr" /><c r="L533" s="2" t="inlineStr" /><c r="M533" s="2" t="inlineStr" /><c r="N533" s="2" t="inlineStr" /><c r="O533" s="2" t="inlineStr" /><c r="P533" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q533" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="534"><c r="A534" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B534" s="2" t="inlineStr"><is><t>Struktura chemiczna</t></is></c><c r="C534" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D534" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E534" s="2" t="inlineStr"><is><t>Trójpierścieniowe leki przeciwdepresyjne:</t></is></c><c r="F534" s="2" t="inlineStr"><is><t>blokują receptory histaminowe</t></is></c><c r="G534" s="2" t="inlineStr"><is><t>hamują wychwyt zwrotny dopaminy</t></is></c><c r="H534" s="2" t="inlineStr" /><c r="I534" s="2" t="inlineStr" /><c r="J534" s="2" t="inlineStr" /><c r="K534" s="2" t="inlineStr"><is><t>pobudzają receptory muskarynowe</t></is></c><c r="L534" s="2" t="inlineStr"><is><t>nie wpływają na przekaźnictwo serotoninergiczne</t></is></c><c r="M534" s="2" t="inlineStr" /><c r="N534" s="2" t="inlineStr" /><c r="O534" s="2" t="inlineStr" /><c r="P534" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q534" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="535"><c r="A535" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B535" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C535" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D535" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E535" s="2" t="inlineStr"><is><t>Na dostępność biologiczną leku może mieć wpływ:</t></is></c><c r="F535" s="2" t="inlineStr"><is><t>stopień uwalniania substancji czynnej</t></is></c><c r="G535" s="2" t="inlineStr"><is><t>efekt I przejścia</t></is></c><c r="H535" s="2" t="inlineStr"><is><t>szybkość transportu substancji czynnej przez błony biologiczne</t></is></c><c r="I535" s="2" t="inlineStr" /><c r="J535" s="2" t="inlineStr" /><c r="K535" s="2" t="inlineStr"><is><t>stopień wiązania z białkami krwi</t></is></c><c r="L535" s="2" t="inlineStr" /><c r="M535" s="2" t="inlineStr" /><c r="N535" s="2" t="inlineStr" /><c r="O535" s="2" t="inlineStr" /><c r="P535" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q535" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="536"><c r="A536" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B536" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C536" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D536" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E536" s="2" t="inlineStr"><is><t>Stan stacjonarny leku ustala się:</t></is></c><c r="F536" s="2" t="inlineStr"><is><t>po okresie równym około 4–5 T1/2</t></is></c><c r="G536" s="2" t="inlineStr" /><c r="H536" s="2" t="inlineStr" /><c r="I536" s="2" t="inlineStr" /><c r="J536" s="2" t="inlineStr" /><c r="K536" s="2" t="inlineStr"><is><t>w momencie, który zależy od dawki leku</t></is></c><c r="L536" s="2" t="inlineStr"><is><t>jedynie w wyniku wielokrotnego podania doustnego</t></is></c><c r="M536" s="2" t="inlineStr"><is><t>w czasie wprost proporcjonalnym do klirensu leku</t></is></c><c r="N536" s="2" t="inlineStr" /><c r="O536" s="2" t="inlineStr" /><c r="P536" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q536" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="537"><c r="A537" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B537" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C537" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D537" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E537" s="2" t="inlineStr"><is><t>Biologiczny okres półtrwania (T1/2):</t></is></c><c r="F537" s="2" t="inlineStr"><is><t>zależy od objętości dystrybucji</t></is></c><c r="G537" s="2" t="inlineStr"><is><t>jest odwrotnie proporcjonalny do klirensu całkowitego</t></is></c><c r="H537" s="2" t="inlineStr"><is><t>ma wpływ na moment osiągnięcia stanu stacjonarnego</t></is></c><c r="I537" s="2" t="inlineStr" /><c r="J537" s="2" t="inlineStr" /><c r="K537" s="2" t="inlineStr"><is><t>zależy od szybkości wchłaniania</t></is></c><c r="L537" s="2" t="inlineStr" /><c r="M537" s="2" t="inlineStr" /><c r="N537" s="2" t="inlineStr" /><c r="O537" s="2" t="inlineStr" /><c r="P537" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q537" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="538"><c r="A538" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B538" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C538" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D538" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E538" s="2" t="inlineStr"><is><t>Do typowych objawów zatrucia opioidami należą:</t></is></c><c r="F538" s="2" t="inlineStr"><is><t>Śpiączka</t></is></c><c r="G538" s="2" t="inlineStr"><is><t>Depresja oddechowa</t></is></c><c r="H538" s="2" t="inlineStr" /><c r="I538" s="2" t="inlineStr" /><c r="J538" s="2" t="inlineStr" /><c r="K538" s="2" t="inlineStr"><is><t>Wzrost ciśnienia tętniczego</t></is></c><c r="L538" s="2" t="inlineStr"><is><t>wzrost temperatury ciała</t></is></c><c r="M538" s="2" t="inlineStr" /><c r="N538" s="2" t="inlineStr" /><c r="O538" s="2" t="inlineStr" /><c r="P538" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q538" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="539"><c r="A539" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B539" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C539" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D539" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E539" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące glikokortykosteroidów:</t></is></c><c r="F539" s="2" t="inlineStr"><is><t>Działają za pośrednictwem receptorów wewnątrzkomórkowych</t></is></c><c r="G539" s="2" t="inlineStr"><is><t>mechanizm niegenomowy odpowiedzialny jest za ich działanie rozkurczające mięśniówkę dróg oddechowych</t></is></c><c r="H539" s="2" t="inlineStr"><is><t>Nagłe ich odstawienie po co najmniej tygodniowym zastosowaniu dawek farmakologicznych może być przyczyną ostrej niewydolności kory nadnerczy</t></is></c><c r="I539" s="2" t="inlineStr" /><c r="J539" s="2" t="inlineStr" /><c r="K539" s="2" t="inlineStr"><is><t>Powodują zmniejszenie zapotrzebowania na insulinę u chorych na cukrzycę</t></is></c><c r="L539" s="2" t="inlineStr" /><c r="M539" s="2" t="inlineStr" /><c r="N539" s="2" t="inlineStr" /><c r="O539" s="2" t="inlineStr" /><c r="P539" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q539" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="540"><c r="A540" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B540" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C540" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D540" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E540" s="2" t="inlineStr"><is><t>Insulina ludzka neutralna:</t></is></c><c r="F540" s="2" t="inlineStr"><is><t>działa za pośrednictwem receptora błonowego</t></is></c><c r="G540" s="2" t="inlineStr"><is><t>jest otrzymywana metodą rekombinacji DNA</t></is></c><c r="H540" s="2" t="inlineStr" /><c r="I540" s="2" t="inlineStr" /><c r="J540" s="2" t="inlineStr" /><c r="K540" s="2" t="inlineStr"><is><t>może być podawana doustnie</t></is></c><c r="L540" s="2" t="inlineStr"><is><t>jest analogiem długodziałającym</t></is></c><c r="M540" s="2" t="inlineStr" /><c r="N540" s="2" t="inlineStr" /><c r="O540" s="2" t="inlineStr" /><c r="P540" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q540" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="541"><c r="A541" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B541" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C541" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D541" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E541" s="2" t="inlineStr"><is><t>Stosowanie estrogenów może być przyczyną:</t></is></c><c r="F541" s="2" t="inlineStr"><is><t>wzrostu ciśnienia tętniczego krwi</t></is></c><c r="G541" s="2" t="inlineStr"><is><t>kamicy żółciowej</t></is></c><c r="H541" s="2" t="inlineStr"><is><t>wzrostu ryzyka wystąpienia raka piersi</t></is></c><c r="I541" s="2" t="inlineStr"><is><t>zatorowości płucnej</t></is></c><c r="J541" s="2" t="inlineStr" /><c r="K541" s="2" t="inlineStr" /><c r="L541" s="2" t="inlineStr" /><c r="M541" s="2" t="inlineStr" /><c r="N541" s="2" t="inlineStr" /><c r="O541" s="2" t="inlineStr" /><c r="P541" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q541" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="542"><c r="A542" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B542" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C542" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D542" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E542" s="2" t="inlineStr"><is><t>Metamizol:</t></is></c><c r="F542" s="2" t="inlineStr"><is><t>działa przeciwbólowo i przeciwgorączkowo</t></is></c><c r="G542" s="2" t="inlineStr"><is><t>działa spazmolitycznie</t></is></c><c r="H542" s="2" t="inlineStr"><is><t>może być przyczyną agranulocytozy</t></is></c><c r="I542" s="2" t="inlineStr" /><c r="J542" s="2" t="inlineStr" /><c r="K542" s="2" t="inlineStr"><is><t>może być bezpiecznie stosowany w ciąży</t></is></c><c r="L542" s="2" t="inlineStr" /><c r="M542" s="2" t="inlineStr" /><c r="N542" s="2" t="inlineStr" /><c r="O542" s="2" t="inlineStr" /><c r="P542" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q542" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="543"><c r="A543" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B543" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C543" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D543" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E543" s="2" t="inlineStr"><is><t>Do leków biotechnologicznych należą:</t></is></c><c r="F543" s="2" t="inlineStr"><is><t>szczepionki</t></is></c><c r="G543" s="2" t="inlineStr"><is><t>przeciwciała monoklonalne</t></is></c><c r="H543" s="2" t="inlineStr"><is><t>Hormony</t></is></c><c r="I543" s="2" t="inlineStr"><is><t>czynniki krzepnięcia</t></is></c><c r="J543" s="2" t="inlineStr" /><c r="K543" s="2" t="inlineStr" /><c r="L543" s="2" t="inlineStr" /><c r="M543" s="2" t="inlineStr" /><c r="N543" s="2" t="inlineStr" /><c r="O543" s="2" t="inlineStr" /><c r="P543" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q543" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="544"><c r="A544" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B544" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C544" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D544" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E544" s="2" t="inlineStr"><is><t>Doustne preparaty żelaza:</t></is></c><c r="F544" s="2" t="inlineStr"><is><t>najlepiej przyswajalne zawierają żelazo dwuwartościowe</t></is></c><c r="G544" s="2" t="inlineStr"><is><t>należy przyjmować przez okres 3 miesięcy po uzyskaniu normalizacji morfologii</t></is></c><c r="H544" s="2" t="inlineStr" /><c r="I544" s="2" t="inlineStr" /><c r="J544" s="2" t="inlineStr" /><c r="K544" s="2" t="inlineStr"><is><t>należy przyjmować z posiłkiem wysokotłuszczowym</t></is></c><c r="L544" s="2" t="inlineStr"><is><t>mogą być przyczyną jasno-żółtego zabarwienia stolca</t></is></c><c r="M544" s="2" t="inlineStr" /><c r="N544" s="2" t="inlineStr" /><c r="O544" s="2" t="inlineStr" /><c r="P544" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q544" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="545"><c r="A545" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B545" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C545" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D545" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E545" s="2" t="inlineStr"><is><t>Diazepam:</t></is></c><c r="F545" s="2" t="inlineStr"><is><t>działa sedatywnie</t></is></c><c r="G545" s="2" t="inlineStr"><is><t>działa powyżej 24 godzin</t></is></c><c r="H545" s="2" t="inlineStr" /><c r="I545" s="2" t="inlineStr" /><c r="J545" s="2" t="inlineStr" /><c r="K545" s="2" t="inlineStr"><is><t>obniża próg drgawkowy</t></is></c><c r="L545" s="2" t="inlineStr"><is><t>nie podlega metabolizmowi</t></is></c><c r="M545" s="2" t="inlineStr" /><c r="N545" s="2" t="inlineStr" /><c r="O545" s="2" t="inlineStr" /><c r="P545" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q545" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="546"><c r="A546" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B546" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C546" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D546" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E546" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek przeciwpadaczkowy – mechanizm działania: B</t></is></c><c r="F546" s="2" t="inlineStr"><is><t>fenytoina – hamowanie kanałów sodowych</t></is></c><c r="G546" s="2" t="inlineStr"><is><t>karbamazepina - hamowanie kanałów sodowych i kanałów wapniowych</t></is></c><c r="H546" s="2" t="inlineStr" /><c r="I546" s="2" t="inlineStr" /><c r="J546" s="2" t="inlineStr" /><c r="K546" s="2" t="inlineStr"><is><t>fenobarbital – hamowanie transmisji GABA-ergicznej</t></is></c><c r="L546" s="2" t="inlineStr"><is><t>kwas walproinowy – hamowanie kanałów sodowych i transmisji GABA-ergicznej</t></is></c><c r="M546" s="2" t="inlineStr" /><c r="N546" s="2" t="inlineStr" /><c r="O546" s="2" t="inlineStr" /><c r="P546" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q546" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="547"><c r="A547" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B547" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C547" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D547" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E547" s="2" t="inlineStr"><is><t>Selektywne inhibitory wychwytu zwrotnego serotoniny (SSRI) charakteryzuje:</t></is></c><c r="F547" s="2" t="inlineStr"><is><t>niewielki wpływ na układ krążenia</t></is></c><c r="G547" s="2" t="inlineStr"><is><t>małe ryzyko teratogenności</t></is></c><c r="H547" s="2" t="inlineStr" /><c r="I547" s="2" t="inlineStr" /><c r="J547" s="2" t="inlineStr" /><c r="K547" s="2" t="inlineStr"><is><t>obniżanie progu drgawkowego</t></is></c><c r="L547" s="2" t="inlineStr"><is><t>brak ryzyka wystąpienia istotnych interakcji z inhibitorami MAO</t></is></c><c r="M547" s="2" t="inlineStr" /><c r="N547" s="2" t="inlineStr" /><c r="O547" s="2" t="inlineStr" /><c r="P547" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q547" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="548"><c r="A548" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B548" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C548" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D548" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E548" s="2" t="inlineStr"><is><t>Potencjał uzależniający wykazują:</t></is></c><c r="F548" s="2" t="inlineStr"><is><t>Kanabinoidy</t></is></c><c r="G548" s="2" t="inlineStr"><is><t>dysocjacyjne środki znieczulające</t></is></c><c r="H548" s="2" t="inlineStr"><is><t>Benzodiazepiny</t></is></c><c r="I548" s="2" t="inlineStr"><is><t>opioidy</t></is></c><c r="J548" s="2" t="inlineStr" /><c r="K548" s="2" t="inlineStr" /><c r="L548" s="2" t="inlineStr" /><c r="M548" s="2" t="inlineStr" /><c r="N548" s="2" t="inlineStr" /><c r="O548" s="2" t="inlineStr" /><c r="P548" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q548" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="549"><c r="A549" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B549" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C549" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D549" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E549" s="2" t="inlineStr"><is><t>Działanie immunosupresyjne wykazują:</t></is></c><c r="F549" s="2" t="inlineStr"><is><t>inhibitory kalcyneuryny</t></is></c><c r="G549" s="2" t="inlineStr"><is><t>alkilujące inhibitory proliferacji</t></is></c><c r="H549" s="2" t="inlineStr" /><c r="I549" s="2" t="inlineStr" /><c r="J549" s="2" t="inlineStr" /><c r="K549" s="2" t="inlineStr"><is><t>czynniki stymulujące tworzenie kolonii granulocytów</t></is></c><c r="L549" s="2" t="inlineStr"><is><t>interferon beta</t></is></c><c r="M549" s="2" t="inlineStr" /><c r="N549" s="2" t="inlineStr" /><c r="O549" s="2" t="inlineStr" /><c r="P549" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q549" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="550"><c r="A550" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B550" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C550" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D550" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E550" s="2" t="inlineStr"><is><t>Hamowanie transmisji dopaminergicznej może być przyczyną wystąpienia:</t></is></c><c r="F550" s="2" t="inlineStr"><is><t>Dyskinez</t></is></c><c r="G550" s="2" t="inlineStr"><is><t>zwiększenia masy ciała</t></is></c><c r="H550" s="2" t="inlineStr"><is><t>działania przeciwwymiotnego</t></is></c><c r="I550" s="2" t="inlineStr" /><c r="J550" s="2" t="inlineStr" /><c r="K550" s="2" t="inlineStr"><is><t>hipoprolaktynemii</t></is></c><c r="L550" s="2" t="inlineStr" /><c r="M550" s="2" t="inlineStr" /><c r="N550" s="2" t="inlineStr" /><c r="O550" s="2" t="inlineStr" /><c r="P550" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q550" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="551"><c r="A551" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B551" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C551" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D551" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E551" s="2" t="inlineStr"><is><t>W przypadku rozpoznania anginy paciorkowcowej można zastosować:</t></is></c><c r="F551" s="2" t="inlineStr"><is><t>Klindamycynę</t></is></c><c r="G551" s="2" t="inlineStr"><is><t>Fenoksymetylopenicylinę</t></is></c><c r="H551" s="2" t="inlineStr" /><c r="I551" s="2" t="inlineStr" /><c r="J551" s="2" t="inlineStr" /><c r="K551" s="2" t="inlineStr"><is><t>Cyprofloksacynę</t></is></c><c r="L551" s="2" t="inlineStr"><is><t>Amikacynę</t></is></c><c r="M551" s="2" t="inlineStr" /><c r="N551" s="2" t="inlineStr" /><c r="O551" s="2" t="inlineStr" /><c r="P551" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q551" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="552"><c r="A552" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B552" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C552" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D552" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E552" s="2" t="inlineStr"><is><t>Chlorochina:</t></is></c><c r="F552" s="2" t="inlineStr"><is><t>Może być przyczyną wypadania włosów</t></is></c><c r="G552" s="2" t="inlineStr"><is><t>Niszczy formy wewnątrzkrwinkowe pierwotniaka</t></is></c><c r="H552" s="2" t="inlineStr" /><c r="I552" s="2" t="inlineStr" /><c r="J552" s="2" t="inlineStr" /><c r="K552" s="2" t="inlineStr"><is><t>Jest stosowana w każdym schemacie profilaktyki malarii</t></is></c><c r="L552" s="2" t="inlineStr"><is><t>Jest szczególnie skuteczna w leczeniu zakażenia Plasmodium falciparium</t></is></c><c r="M552" s="2" t="inlineStr" /><c r="N552" s="2" t="inlineStr" /><c r="O552" s="2" t="inlineStr" /><c r="P552" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q552" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="553"><c r="A553" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B553" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C553" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D553" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E553" s="2" t="inlineStr"><is><t>Lek bakteriobójczy, którego aktywność przeciwbakteryjną najlepiej charakteryzuje AUC24/MIC, działający na bakterie atypowe. Lek jest wydalany głównie z moczem i jego stosowanie związane jest z ryzykiem wydłużenia odstępu QT. Opis może dotyczyć:</t></is></c><c r="F553" s="2" t="inlineStr"><is><t>Lewofloksacyny</t></is></c><c r="G553" s="2" t="inlineStr" /><c r="H553" s="2" t="inlineStr" /><c r="I553" s="2" t="inlineStr" /><c r="J553" s="2" t="inlineStr" /><c r="K553" s="2" t="inlineStr"><is><t>Doksycyliny</t></is></c><c r="L553" s="2" t="inlineStr"><is><t>Klarytromycyny</t></is></c><c r="M553" s="2" t="inlineStr"><is><t>Linezolidu</t></is></c><c r="N553" s="2" t="inlineStr" /><c r="O553" s="2" t="inlineStr" /><c r="P553" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q553" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="554"><c r="A554" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B554" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C554" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D554" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E554" s="2" t="inlineStr"><is><t>Lek bakteriobójczy, którego aktywność przeciwbakteryjną najlepiej charakteryzuje AUC24/MIC, działający na bakterie G(+). Lek nie ma aktywnych metabolitów i działa nefrotoksycznie. Opis może dotyczyć:</t></is></c><c r="F554" s="2" t="inlineStr"><is><t>Wankomycyny</t></is></c><c r="G554" s="2" t="inlineStr" /><c r="H554" s="2" t="inlineStr" /><c r="I554" s="2" t="inlineStr" /><c r="J554" s="2" t="inlineStr" /><c r="K554" s="2" t="inlineStr"><is><t>Kolistyny</t></is></c><c r="L554" s="2" t="inlineStr"><is><t>Klindamycyny</t></is></c><c r="M554" s="2" t="inlineStr"><is><t>Gentamycyny</t></is></c><c r="N554" s="2" t="inlineStr" /><c r="O554" s="2" t="inlineStr" /><c r="P554" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q554" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="555"><c r="A555" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B555" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C555" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D555" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E555" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Pseudomonas aeruginosa uzasadnione może być podanie:</t></is></c><c r="F555" s="2" t="inlineStr"><is><t>Piperacykliny z tazobaktamem</t></is></c><c r="G555" s="2" t="inlineStr"><is><t>Gentamycyny</t></is></c><c r="H555" s="2" t="inlineStr"><is><t>Cyprofloksacyny</t></is></c><c r="I555" s="2" t="inlineStr"><is><t>Ceftazydymu</t></is></c><c r="J555" s="2" t="inlineStr" /><c r="K555" s="2" t="inlineStr" /><c r="L555" s="2" t="inlineStr" /><c r="M555" s="2" t="inlineStr" /><c r="N555" s="2" t="inlineStr" /><c r="O555" s="2" t="inlineStr" /><c r="P555" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q555" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="556"><c r="A556" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B556" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C556" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D556" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E556" s="2" t="inlineStr"><is><t>Po podaniu doustnym działa miejscowo:</t></is></c><c r="F556" s="2" t="inlineStr"><is><t>Ryfaksymina</t></is></c><c r="G556" s="2" t="inlineStr"><is><t>Fidaksomycyna</t></is></c><c r="H556" s="2" t="inlineStr" /><c r="I556" s="2" t="inlineStr" /><c r="J556" s="2" t="inlineStr" /><c r="K556" s="2" t="inlineStr"><is><t>Kwas fusydowy</t></is></c><c r="L556" s="2" t="inlineStr"><is><t>Norfloksacyna</t></is></c><c r="M556" s="2" t="inlineStr" /><c r="N556" s="2" t="inlineStr" /><c r="O556" s="2" t="inlineStr" /><c r="P556" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q556" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="557"><c r="A557" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B557" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C557" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D557" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E557" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – punkt uchwytu:</t></is></c><c r="F557" s="2" t="inlineStr"><is><t>Acyklowir – polimeraza DNA</t></is></c><c r="G557" s="2" t="inlineStr"><is><t>Oseltamiwir – neuraminidaza</t></is></c><c r="H557" s="2" t="inlineStr"><is><t>Lamiwudyna – odwrotna transkryptaza</t></is></c><c r="I557" s="2" t="inlineStr"><is><t>Raltegrawir – integraza</t></is></c><c r="J557" s="2" t="inlineStr" /><c r="K557" s="2" t="inlineStr" /><c r="L557" s="2" t="inlineStr" /><c r="M557" s="2" t="inlineStr" /><c r="N557" s="2" t="inlineStr" /><c r="O557" s="2" t="inlineStr" /><c r="P557" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q557" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="558"><c r="A558" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B558" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C558" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D558" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E558" s="2" t="inlineStr"><is><t>Wybierz właściwe skojarzenie wskazanie – lek, który można zastosować jako alternatywę dla antybiotków beta-laktamowych u pacjenta z nadwrażliwością na tę grupę leków przeciwbakteryjnych</t></is></c><c r="F558" s="2" t="inlineStr"><is><t>Borelioza – azytromycyna</t></is></c><c r="G558" s="2" t="inlineStr"><is><t>Zapalenie płuc o etiologii pneumokokowej – lewofloksacyna</t></is></c><c r="H558" s="2" t="inlineStr"><is><t>Profilaktyka okołozabiegowa - wankomycyna</t></is></c><c r="I558" s="2" t="inlineStr" /><c r="J558" s="2" t="inlineStr" /><c r="K558" s="2" t="inlineStr"><is><t>Urosepsa o etiologii Escherichia coli – linezolid</t></is></c><c r="L558" s="2" t="inlineStr" /><c r="M558" s="2" t="inlineStr" /><c r="N558" s="2" t="inlineStr" /><c r="O558" s="2" t="inlineStr" /><c r="P558" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q558" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="559"><c r="A559" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B559" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C559" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D559" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E559" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – wskazanie:</t></is></c><c r="F559" s="2" t="inlineStr"><is><t>Metronidazol – lamblioza</t></is></c><c r="G559" s="2" t="inlineStr"><is><t>Spiramycyna – toksoplazmoza</t></is></c><c r="H559" s="2" t="inlineStr" /><c r="I559" s="2" t="inlineStr" /><c r="J559" s="2" t="inlineStr" /><c r="K559" s="2" t="inlineStr"><is><t>Nifuroksazyd – biegunka poantybiotykowa</t></is></c><c r="L559" s="2" t="inlineStr"><is><t>Amikacyna – borelioza</t></is></c><c r="M559" s="2" t="inlineStr" /><c r="N559" s="2" t="inlineStr" /><c r="O559" s="2" t="inlineStr" /><c r="P559" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q559" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="560"><c r="A560" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B560" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C560" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D560" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E560" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – wskazanie:</t></is></c><c r="F560" s="2" t="inlineStr"><is><t>spiramycyna – toksoplazmoza</t></is></c><c r="G560" s="2" t="inlineStr"><is><t>fenoksymetylopenicylina – angina paciorkowcowa</t></is></c><c r="H560" s="2" t="inlineStr"><is><t>metronidazol - lamblioza</t></is></c><c r="I560" s="2" t="inlineStr" /><c r="J560" s="2" t="inlineStr" /><c r="K560" s="2" t="inlineStr"><is><t>neomycyna – biegunka poantybiotykowa</t></is></c><c r="L560" s="2" t="inlineStr" /><c r="M560" s="2" t="inlineStr" /><c r="N560" s="2" t="inlineStr" /><c r="O560" s="2" t="inlineStr" /><c r="P560" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q560" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="561"><c r="A561" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B561" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C561" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D561" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E561" s="2" t="inlineStr"><is><t>Wskazaniem do doustnej terapii przeciwgrzybiczej jest:</t></is></c><c r="F561" s="2" t="inlineStr"><is><t>Nieskuteczność leczenia miejscowego</t></is></c><c r="G561" s="2" t="inlineStr"><is><t>Grzybica inwazyjna</t></is></c><c r="H561" s="2" t="inlineStr"><is><t>Stwierdzenie rozległych zmian skórnych</t></is></c><c r="I561" s="2" t="inlineStr" /><c r="J561" s="2" t="inlineStr" /><c r="K561" s="2" t="inlineStr"><is><t>Grzybica paznokci dotycząca pojedynczych płytek paznokciowych</t></is></c><c r="L561" s="2" t="inlineStr" /><c r="M561" s="2" t="inlineStr" /><c r="N561" s="2" t="inlineStr" /><c r="O561" s="2" t="inlineStr" /><c r="P561" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q561" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="562"><c r="A562" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B562" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C562" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D562" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E562" s="2" t="inlineStr"><is><t>Działanie neurotoksyczne wykazuje:</t></is></c><c r="F562" s="2" t="inlineStr"><is><t>Linezolid</t></is></c><c r="G562" s="2" t="inlineStr"><is><t>Cyprofloksacyna</t></is></c><c r="H562" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="I562" s="2" t="inlineStr" /><c r="J562" s="2" t="inlineStr" /><c r="K562" s="2" t="inlineStr"><is><t>Klindamycyna</t></is></c><c r="L562" s="2" t="inlineStr" /><c r="M562" s="2" t="inlineStr" /><c r="N562" s="2" t="inlineStr" /><c r="O562" s="2" t="inlineStr" /><c r="P562" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q562" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="563"><c r="A563" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B563" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C563" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D563" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E563" s="2" t="inlineStr"><is><t>Działanie neurotoksyczne wykazuje:</t></is></c><c r="F563" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="G563" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="H563" s="2" t="inlineStr"><is><t>kolistyna</t></is></c><c r="I563" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="J563" s="2" t="inlineStr" /><c r="K563" s="2" t="inlineStr" /><c r="L563" s="2" t="inlineStr" /><c r="M563" s="2" t="inlineStr" /><c r="N563" s="2" t="inlineStr" /><c r="O563" s="2" t="inlineStr" /><c r="P563" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q563" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="564"><c r="A564" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B564" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C564" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D564" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E564" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – mechanizm działania (należy uwzględnić główny mechanizm działania):</t></is></c><c r="F564" s="2" t="inlineStr"><is><t>Azytromycyna – hamowanie syntezy białek</t></is></c><c r="G564" s="2" t="inlineStr"><is><t>Daptomycyna – uszkodzenie błony komórkowej</t></is></c><c r="H564" s="2" t="inlineStr" /><c r="I564" s="2" t="inlineStr" /><c r="J564" s="2" t="inlineStr" /><c r="K564" s="2" t="inlineStr"><is><t>Cyprofloksacyna – hamowanie biosyntezy ściany komórkowej</t></is></c><c r="L564" s="2" t="inlineStr"><is><t>Amoksycyina – hamowanie syntezy DNA</t></is></c><c r="M564" s="2" t="inlineStr" /><c r="N564" s="2" t="inlineStr" /><c r="O564" s="2" t="inlineStr" /><c r="P564" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q564" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="565"><c r="A565" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B565" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C565" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D565" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E565" s="2" t="inlineStr"><is><t>W schematach eradykacji Helicobacter pylori znajdują zastosowanie:</t></is></c><c r="F565" s="2" t="inlineStr"><is><t>Amoksycylina</t></is></c><c r="G565" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="H565" s="2" t="inlineStr" /><c r="I565" s="2" t="inlineStr" /><c r="J565" s="2" t="inlineStr" /><c r="K565" s="2" t="inlineStr"><is><t>Lewofloksacyna</t></is></c><c r="L565" s="2" t="inlineStr"><is><t>Tetracyklina</t></is></c><c r="M565" s="2" t="inlineStr" /><c r="N565" s="2" t="inlineStr" /><c r="O565" s="2" t="inlineStr" /><c r="P565" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q565" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="566"><c r="A566" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B566" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C566" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D566" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E566" s="2" t="inlineStr"><is><t>Linezolid może być skuteczny w zakażeniach szczepami:</t></is></c><c r="F566" s="2" t="inlineStr"><is><t>MRSA (methicyllin-resistant Staphylococcus aureus)</t></is></c><c r="G566" s="2" t="inlineStr"><is><t>MSSA (methicyllin-sensitive Staphylococcus aureus)</t></is></c><c r="H566" s="2" t="inlineStr"><is><t>VRE (Vancomycin-resistant Enterococcus)</t></is></c><c r="I566" s="2" t="inlineStr" /><c r="J566" s="2" t="inlineStr" /><c r="K566" s="2" t="inlineStr"><is><t>CPE (Carbapenemase-producing Enterobacteriaceae)</t></is></c><c r="L566" s="2" t="inlineStr" /><c r="M566" s="2" t="inlineStr" /><c r="N566" s="2" t="inlineStr" /><c r="O566" s="2" t="inlineStr" /><c r="P566" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q566" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="567"><c r="A567" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B567" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C567" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D567" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E567" s="2" t="inlineStr"><is><t>Profilaktyczne zastosowanie leków przeciwinfekcyjnych jest uzasadnione:</t></is></c><c r="F567" s="2" t="inlineStr"><is><t>W planowej operacji cięcia cesarskiego (pole czyste-skażone)</t></is></c><c r="G567" s="2" t="inlineStr"><is><t>W planowej implantacji endoprotezy stawu kolanowego (pole czyste)</t></is></c><c r="H567" s="2" t="inlineStr" /><c r="I567" s="2" t="inlineStr" /><c r="J567" s="2" t="inlineStr" /><c r="K567" s="2" t="inlineStr"><is><t>W planowanym usunięciu zmiany skórnej w obrębie dłoni (pole czyste)</t></is></c><c r="L567" s="2" t="inlineStr"><is><t>W planowym usunięciu tarczycy w wolu guzkowym nadczynnym (pole czyste)</t></is></c><c r="M567" s="2" t="inlineStr" /><c r="N567" s="2" t="inlineStr" /><c r="O567" s="2" t="inlineStr" /><c r="P567" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q567" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="568"><c r="A568" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B568" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C568" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D568" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E568" s="2" t="inlineStr"><is><t>Profilaktyczne zastosowanie leków przeciwinfekcyjnych jest uzasadnione:</t></is></c><c r="F568" s="2" t="inlineStr"><is><t>w planowej operacji zmniejszenia żołądka w leczeniu otyłości olbrzymiej(pole czyste-skażone)</t></is></c><c r="G568" s="2" t="inlineStr"><is><t>w planowej implantacji sztucznej protezy stawu biodrowego (pole czyste)</t></is></c><c r="H568" s="2" t="inlineStr" /><c r="I568" s="2" t="inlineStr" /><c r="J568" s="2" t="inlineStr" /><c r="K568" s="2" t="inlineStr"><is><t>w planowym usunięciu znamienia skórnego do diagnostyki histo-patologicznej (pole czyste)</t></is></c><c r="L568" s="2" t="inlineStr"><is><t>w planowym usunięciu tarczycy w wolu guzkowym nadczynnym (pole czyste)</t></is></c><c r="M568" s="2" t="inlineStr" /><c r="N568" s="2" t="inlineStr" /><c r="O568" s="2" t="inlineStr" /><c r="P568" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q568" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="569"><c r="A569" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B569" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C569" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D569" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E569" s="2" t="inlineStr"><is><t>Do bezpiecznych i skutecznych środków do dezynfekcji należą:</t></is></c><c r="F569" s="2" t="inlineStr"><is><t>Oktenidyna</t></is></c><c r="G569" s="2" t="inlineStr" /><c r="H569" s="2" t="inlineStr" /><c r="I569" s="2" t="inlineStr" /><c r="J569" s="2" t="inlineStr" /><c r="K569" s="2" t="inlineStr"><is><t>Spirytus salicylowy</t></is></c><c r="L569" s="2" t="inlineStr"><is><t>Woda utleniona</t></is></c><c r="M569" s="2" t="inlineStr"><is><t>Mleczan etakrydyny</t></is></c><c r="N569" s="2" t="inlineStr" /><c r="O569" s="2" t="inlineStr" /><c r="P569" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q569" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="570"><c r="A570" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B570" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C570" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D570" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E570" s="2" t="inlineStr"><is><t>Do bezpiecznych i skutecznych środków do dezynfekcji należą:</t></is></c><c r="F570" s="2" t="inlineStr"><is><t>oktenidyna</t></is></c><c r="G570" s="2" t="inlineStr" /><c r="H570" s="2" t="inlineStr" /><c r="I570" s="2" t="inlineStr" /><c r="J570" s="2" t="inlineStr" /><c r="K570" s="2" t="inlineStr"><is><t>woda utleniona</t></is></c><c r="L570" s="2" t="inlineStr"><is><t>spirytusowy roztwór fioletu gencjanowego</t></is></c><c r="M570" s="2" t="inlineStr"><is><t>mleczan etakrydyny</t></is></c><c r="N570" s="2" t="inlineStr" /><c r="O570" s="2" t="inlineStr" /><c r="P570" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q570" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="571"><c r="A571" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B571" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C571" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D571" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E571" s="2" t="inlineStr"><is><t>U kobiety w ciąży można bezpiecznie zastosować:</t></is></c><c r="F571" s="2" t="inlineStr"><is><t>Cefuroksym</t></is></c><c r="G571" s="2" t="inlineStr"><is><t>Fenoksymetylopenicylinę</t></is></c><c r="H571" s="2" t="inlineStr" /><c r="I571" s="2" t="inlineStr" /><c r="J571" s="2" t="inlineStr" /><c r="K571" s="2" t="inlineStr"><is><t>Amikacynę</t></is></c><c r="L571" s="2" t="inlineStr"><is><t>Moksyfloksacynę</t></is></c><c r="M571" s="2" t="inlineStr" /><c r="N571" s="2" t="inlineStr" /><c r="O571" s="2" t="inlineStr" /><c r="P571" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q571" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="572"><c r="A572" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B572" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C572" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D572" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E572" s="2" t="inlineStr"><is><t>Wskaż właściwe skojarzenie lek – potencjalne działanie nipożądane:</t></is></c><c r="F572" s="2" t="inlineStr"><is><t>Doksycyklina – fotodermatoza</t></is></c><c r="G572" s="2" t="inlineStr"><is><t>Linezolid - zespół serotoninowy</t></is></c><c r="H572" s="2" t="inlineStr" /><c r="I572" s="2" t="inlineStr" /><c r="J572" s="2" t="inlineStr" /><c r="K572" s="2" t="inlineStr"><is><t>Mupirocyna - zespół czerwonego dziecka</t></is></c><c r="L572" s="2" t="inlineStr"><is><t>Gentamycyna - żółtaczka cholestatyczna</t></is></c><c r="M572" s="2" t="inlineStr" /><c r="N572" s="2" t="inlineStr" /><c r="O572" s="2" t="inlineStr" /><c r="P572" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q572" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="573"><c r="A573" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B573" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C573" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D573" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E573" s="2" t="inlineStr"><is><t>Działanie nefrotoksyczne wykazuje:</t></is></c><c r="F573" s="2" t="inlineStr"><is><t>Gentamycyna</t></is></c><c r="G573" s="2" t="inlineStr"><is><t>Kolistyna</t></is></c><c r="H573" s="2" t="inlineStr"><is><t>Wankomycyna</t></is></c><c r="I573" s="2" t="inlineStr" /><c r="J573" s="2" t="inlineStr" /><c r="K573" s="2" t="inlineStr"><is><t>Klindamycyna</t></is></c><c r="L573" s="2" t="inlineStr" /><c r="M573" s="2" t="inlineStr" /><c r="N573" s="2" t="inlineStr" /><c r="O573" s="2" t="inlineStr" /><c r="P573" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q573" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="574"><c r="A574" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B574" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C574" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D574" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E574" s="2" t="inlineStr"><is><t>W biegunce o etiologii Clostridioides difficile uzasadnione może być podanie doustne:</t></is></c><c r="F574" s="2" t="inlineStr"><is><t>Fidaksomycyny</t></is></c><c r="G574" s="2" t="inlineStr"><is><t>Metronidazolu</t></is></c><c r="H574" s="2" t="inlineStr" /><c r="I574" s="2" t="inlineStr" /><c r="J574" s="2" t="inlineStr" /><c r="K574" s="2" t="inlineStr"><is><t>Neomycyny</t></is></c><c r="L574" s="2" t="inlineStr"><is><t>Nifuroksazydu</t></is></c><c r="M574" s="2" t="inlineStr" /><c r="N574" s="2" t="inlineStr" /><c r="O574" s="2" t="inlineStr" /><c r="P574" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q574" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="575"><c r="A575" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B575" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C575" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D575" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E575" s="2" t="inlineStr"><is><t>Wskaż stwierdzenie/a prawdziwe:</t></is></c><c r="F575" s="2" t="inlineStr"><is><t>Ketokonazol stosuje się wyłącznie miejscowo w leczeniu grzybic</t></is></c><c r="G575" s="2" t="inlineStr" /><c r="H575" s="2" t="inlineStr" /><c r="I575" s="2" t="inlineStr" /><c r="J575" s="2" t="inlineStr" /><c r="K575" s="2" t="inlineStr"><is><t>Terbinafina hamuje enzym związany z ukłądem CYP450</t></is></c><c r="L575" s="2" t="inlineStr"><is><t>Zastosowanie technologii liposomów pozwoliło na otrzymanie preparatów amfoterycyny B o istotnie zmniejszonej hepatotoksyczności</t></is></c><c r="M575" s="2" t="inlineStr"><is><t>Kaspofungina osiąga bardzo wysokie stężenia w OUN</t></is></c><c r="N575" s="2" t="inlineStr" /><c r="O575" s="2" t="inlineStr" /><c r="P575" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q575" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="576"><c r="A576" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B576" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C576" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D576" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E576" s="2" t="inlineStr"><is><t>Metronidazol:</t></is></c><c r="F576" s="2" t="inlineStr"><is><t>Dobrze penetruje do OUN</t></is></c><c r="G576" s="2" t="inlineStr"><is><t>Działa na Entamoeba histolytica</t></is></c><c r="H576" s="2" t="inlineStr" /><c r="I576" s="2" t="inlineStr" /><c r="J576" s="2" t="inlineStr" /><c r="K576" s="2" t="inlineStr"><is><t>Bardzo często jest przyczyną zapalenia ścięgna Achillesa</t></is></c><c r="L576" s="2" t="inlineStr"><is><t>Jest stosowany w wewnątrzbrzusznych zakażeniach szczepami wielolekoopornymi</t></is></c><c r="M576" s="2" t="inlineStr" /><c r="N576" s="2" t="inlineStr" /><c r="O576" s="2" t="inlineStr" /><c r="P576" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q576" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="577"><c r="A577" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B577" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C577" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D577" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E577" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie drobnoustrój - lek, który może być skuteczny w zakażeniu o takiej etiologii:</t></is></c><c r="F577" s="2" t="inlineStr"><is><t>Staphylococcus aureus (MSSA) - kloksacylina</t></is></c><c r="G577" s="2" t="inlineStr"><is><t>Clostridioides difficile – wankomycyna</t></is></c><c r="H577" s="2" t="inlineStr" /><c r="I577" s="2" t="inlineStr" /><c r="J577" s="2" t="inlineStr" /><c r="K577" s="2" t="inlineStr"><is><t>Staphylococcus aureus (MRSA) - meropenem</t></is></c><c r="L577" s="2" t="inlineStr"><is><t>Trichomonas vaginalis - ketokonazol</t></is></c><c r="M577" s="2" t="inlineStr" /><c r="N577" s="2" t="inlineStr" /><c r="O577" s="2" t="inlineStr" /><c r="P577" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q577" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="578"><c r="A578" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B578" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C578" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D578" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E578" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek – wskazanie do leczenia:</t></is></c><c r="F578" s="2" t="inlineStr"><is><t>Acyklowir - półpasiec</t></is></c><c r="G578" s="2" t="inlineStr"><is><t>Gancyklowir – cytomegalowirusowe zapalenie siatkówki</t></is></c><c r="H578" s="2" t="inlineStr"><is><t>Osetamiwir – grypa</t></is></c><c r="I578" s="2" t="inlineStr" /><c r="J578" s="2" t="inlineStr" /><c r="K578" s="2" t="inlineStr"><is><t>Amantadyna – mononukleoza</t></is></c><c r="L578" s="2" t="inlineStr" /><c r="M578" s="2" t="inlineStr" /><c r="N578" s="2" t="inlineStr" /><c r="O578" s="2" t="inlineStr" /><c r="P578" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q578" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="579"><c r="A579" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B579" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C579" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D579" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E579" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie drobnoustrój - lek, który może być skuteczny w zakażeniu o tej etiologii:</t></is></c><c r="F579" s="2" t="inlineStr"><is><t>Helicobacter pylori – tetracyklina</t></is></c><c r="G579" s="2" t="inlineStr"><is><t>Staphylococcus aureus (MSSA) - cefazolina</t></is></c><c r="H579" s="2" t="inlineStr" /><c r="I579" s="2" t="inlineStr" /><c r="J579" s="2" t="inlineStr" /><c r="K579" s="2" t="inlineStr"><is><t>Escherichia coli – klindamycyna</t></is></c><c r="L579" s="2" t="inlineStr"><is><t>Mycoplasma pneumoniae - teikoplanina</t></is></c><c r="M579" s="2" t="inlineStr" /><c r="N579" s="2" t="inlineStr" /><c r="O579" s="2" t="inlineStr" /><c r="P579" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2019/20 - 1 termin (online)</t></is></c><c r="Q579" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="580"><c r="A580" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B580" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C580" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D580" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E580" s="2" t="inlineStr"><is><t>Wytyczne PRISMA:</t></is></c><c r="F580" s="2" t="inlineStr"><is><t>dotyczą prowadzenia przeglądów systematycznych i metaanaliz</t></is></c><c r="G580" s="2" t="inlineStr" /><c r="H580" s="2" t="inlineStr" /><c r="I580" s="2" t="inlineStr" /><c r="J580" s="2" t="inlineStr" /><c r="K580" s="2" t="inlineStr"><is><t>dotyczą prowadzenia randomizowanych badań klinicznych</t></is></c><c r="L580" s="2" t="inlineStr"><is><t>dotyczą formułowania wytycznych klinicznych</t></is></c><c r="M580" s="2" t="inlineStr"><is><t>dotyczą prowadzenia badań obserwacyjnych</t></is></c><c r="N580" s="2" t="inlineStr" /><c r="O580" s="2" t="inlineStr" /><c r="P580" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q580" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="581"><c r="A581" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B581" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C581" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D581" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E581" s="2" t="inlineStr"><is><t>Lek ma Vd=6 l/kg m.c. i CL=10 ml/min/kg m.c. Na tej podstawie spodziewasz się, że lek będzie:</t></is></c><c r="F581" s="2" t="inlineStr"><is><t>wymagał dużej dawki nasycającej</t></is></c><c r="G581" s="2" t="inlineStr" /><c r="H581" s="2" t="inlineStr" /><c r="I581" s="2" t="inlineStr" /><c r="J581" s="2" t="inlineStr" /><c r="K581" s="2" t="inlineStr"><is><t>kumulował się w tkance tłuszczowej</t></is></c><c r="L581" s="2" t="inlineStr"><is><t>miał długi okres półtrwania</t></is></c><c r="M581" s="2" t="inlineStr"><is><t>wymagał korekty dawkowania w niewydolności nerek</t></is></c><c r="N581" s="2" t="inlineStr" /><c r="O581" s="2" t="inlineStr" /><c r="P581" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q581" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="582"><c r="A582" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B582" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C582" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D582" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E582" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenia dotyczące wiązania leków z białkami osocza:</t></is></c><c r="F582" s="2" t="inlineStr"><is><t>może być przyczyną istotnych klinicznie interakcji lekowych</t></is></c><c r="G582" s="2" t="inlineStr" /><c r="H582" s="2" t="inlineStr" /><c r="I582" s="2" t="inlineStr" /><c r="J582" s="2" t="inlineStr" /><c r="K582" s="2" t="inlineStr"><is><t>z powodu zmniejszenia stężenia albumin we krwi leki o dużym stopniu wiązaniu z albuminami mogą wykazywać niedostateczny efekt terapeutyczny</t></is></c><c r="L582" s="2" t="inlineStr"><is><t>jest istotne klinicznie wtedy, gdy frakcja wolna wynosi 80%</t></is></c><c r="M582" s="2" t="inlineStr"><is><t>przebiega w wątrobie, gdzie zachodzi sprzęganie leku z albuminami</t></is></c><c r="N582" s="2" t="inlineStr" /><c r="O582" s="2" t="inlineStr" /><c r="P582" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q582" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="583"><c r="A583" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B583" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C583" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D583" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E583" s="2" t="inlineStr"><is><t>Lek o kinetyce pierwszego rzędu po podaniu doustnym ma biodostępność ok. 100% i okres półtrwania =12 godzin. Pacjent A przyjmuje doustnie ten lek w dawce D co 12 godzin (o godz. 8:00 i 20:00). Pacjent B przyjmuje doustnie ten lek w dawce 2D co 24 godziny (o godz. 8:00). Pacjent C przyjmuje ten lek w ciągłym wlewie dożylnym w dawce odpowiadającej 2D/24h. Wszyscy pacjenci mają prawidłową czynność narządów uczestniczących w eliminacji. Wskaż prawdziwe stwierdzenie:</t></is></c><c r="F583" s="2" t="inlineStr"><is><t>czas eliminacji leku po zakończeniu podawania jest taki sam u wszystkich pacjentów</t></is></c><c r="G583" s="2" t="inlineStr" /><c r="H583" s="2" t="inlineStr" /><c r="I583" s="2" t="inlineStr" /><c r="J583" s="2" t="inlineStr" /><c r="K583" s="2" t="inlineStr"><is><t>w stanie stacjonarnym po pobraniu próbki krwi o godzinie 7:30 rano stężenie tego leku we krwi ma taką samą wartość u wszystkich pacjentów</t></is></c><c r="L583" s="2" t="inlineStr"><is><t>stan stacjonarny ustala się szybciej u pacjenta A niż u pacjenta B</t></is></c><c r="M583" s="2" t="inlineStr"><is><t>wiązanie leku z białkami jest największe u pacjenta C, a najmniejsze u pacjenta A</t></is></c><c r="N583" s="2" t="inlineStr" /><c r="O583" s="2" t="inlineStr" /><c r="P583" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q583" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="584"><c r="A584" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B584" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C584" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D584" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E584" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące warfaryny:</t></is></c><c r="F584" s="2" t="inlineStr"><is><t>blokuje aktywność reduktazy epoksydowej fitomenadionu</t></is></c><c r="G584" s="2" t="inlineStr"><is><t>aktywność warfaryny zależy od polimorfizmu genetycznego izoenzymu CYP2C9</t></is></c><c r="H584" s="2" t="inlineStr" /><c r="I584" s="2" t="inlineStr" /><c r="J584" s="2" t="inlineStr" /><c r="K584" s="2" t="inlineStr"><is><t>zwiększa aktywność białka C i jego kofaktora - białka S o działaniu przeciwzakrzepowym</t></is></c><c r="L584" s="2" t="inlineStr"><is><t>zmniejsza aktywność biologiczną czynników krzepnięcia zespołu protrombiny skutecznie zapobiegając zakrzepicy od 2. doby po włączeniuleczenia</t></is></c><c r="M584" s="2" t="inlineStr" /><c r="N584" s="2" t="inlineStr" /><c r="O584" s="2" t="inlineStr" /><c r="P584" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q584" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="585"><c r="A585" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B585" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C585" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D585" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E585" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące małopłytkowości indukowanej heparyną (HIT) typu II:</t></is></c><c r="F585" s="2" t="inlineStr"><is><t>jest związana z podawaniem heparyny niefrakcjonowanej oraz heparyn drobnocząsteczkowych, ale nie fondaparyny</t></is></c><c r="G585" s="2" t="inlineStr"><is><t>charakteryzuje się spadkiem liczby płytek krwi do 30-50 tys./μl najczęściej w 5-10 dniu od rozpoczęcia leczenia</t></is></c><c r="H585" s="2" t="inlineStr"><is><t>bezpośrednie inhibitory trombiny są lekami z wyboru w leczeniu HIT II</t></is></c><c r="I585" s="2" t="inlineStr" /><c r="J585" s="2" t="inlineStr" /><c r="K585" s="2" t="inlineStr"><is><t>w ocenie klinicznej istotne dla rozpoznania HIT II jest stwierdzenie krwawienia z przewodu pokarmowego</t></is></c><c r="L585" s="2" t="inlineStr" /><c r="M585" s="2" t="inlineStr" /><c r="N585" s="2" t="inlineStr" /><c r="O585" s="2" t="inlineStr" /><c r="P585" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q585" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="586"><c r="A586" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B586" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C586" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D586" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E586" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące małopłytkowości indukowanej heparyną (HIT) typu II:</t></is></c><c r="F586" s="2" t="inlineStr"><is><t>Występuje typowo między 5. a 10. dniem ekspozycji na heparyny ze znacznym nadmiarem liczby płytek (30 000-50 000/mikrolitr)</t></is></c><c r="G586" s="2" t="inlineStr"><is><t>Stwarza istotne ryzyko powikła zakrzepowo-zatorowych</t></is></c><c r="H586" s="2" t="inlineStr"><is><t>Jest potwierdzana identyfikacją przeciwciał przeciw kompleksom heparyna-PF4 w surowicy</t></is></c><c r="I586" s="2" t="inlineStr"><is><t>Jest bezterminowym przeciwwskazaniem do reekspozycji chorego na heparyny</t></is></c><c r="J586" s="2" t="inlineStr" /><c r="K586" s="2" t="inlineStr" /><c r="L586" s="2" t="inlineStr" /><c r="M586" s="2" t="inlineStr" /><c r="N586" s="2" t="inlineStr" /><c r="O586" s="2" t="inlineStr" /><c r="P586" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q586" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="587"><c r="A587" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B587" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C587" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D587" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E587" s="2" t="inlineStr"><is><t>Kwas traneksamowy:</t></is></c><c r="F587" s="2" t="inlineStr"><is><t>hamuje aktywatory plazminogenu</t></is></c><c r="G587" s="2" t="inlineStr"><is><t>powoduje zagrożenie powikłaniami zakrzepowo-zatorowymi</t></is></c><c r="H587" s="2" t="inlineStr"><is><t>jest antidotum w krwawieniach związanych ze stosowaniem leków fibrynolitycznych</t></is></c><c r="I587" s="2" t="inlineStr" /><c r="J587" s="2" t="inlineStr" /><c r="K587" s="2" t="inlineStr"><is><t>zwiększa śmiertelność w krwotokach operacyjnych i pourazowych</t></is></c><c r="L587" s="2" t="inlineStr" /><c r="M587" s="2" t="inlineStr" /><c r="N587" s="2" t="inlineStr" /><c r="O587" s="2" t="inlineStr" /><c r="P587" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q587" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="588"><c r="A588" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B588" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C588" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D588" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E588" s="2" t="inlineStr"><is><t>Efekt działania w czasie do 10 minut od podania występuje po podaniu:</t></is></c><c r="F588" s="2" t="inlineStr"><is><t>fentanylu donosowo</t></is></c><c r="G588" s="2" t="inlineStr"><is><t>naloksonu dożylnie</t></is></c><c r="H588" s="2" t="inlineStr"><is><t>glukagonu domięśniowo</t></is></c><c r="I588" s="2" t="inlineStr" /><c r="J588" s="2" t="inlineStr" /><c r="K588" s="2" t="inlineStr"><is><t>węgla medycznego (aktywowanego) w dawce 1 g przez zgłębnik nosowo￾żoładkowy</t></is></c><c r="L588" s="2" t="inlineStr" /><c r="M588" s="2" t="inlineStr" /><c r="N588" s="2" t="inlineStr" /><c r="O588" s="2" t="inlineStr" /><c r="P588" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q588" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="589"><c r="A589" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B589" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C589" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D589" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E589" s="2" t="inlineStr"><is><t>Wskaż zestaw, gdzie prawidłowo uszeregowano insuliny od najkrócej do najdłużej działającej:</t></is></c><c r="F589" s="2" t="inlineStr"><is><t>lispro–insulina ludzka–glargina</t></is></c><c r="G589" s="2" t="inlineStr"><is><t>glulizyna–insulina ludzka izofanowa–degludec</t></is></c><c r="H589" s="2" t="inlineStr" /><c r="I589" s="2" t="inlineStr" /><c r="J589" s="2" t="inlineStr" /><c r="K589" s="2" t="inlineStr"><is><t>aspart – degludec – detemir</t></is></c><c r="L589" s="2" t="inlineStr"><is><t>detemir–glulizyna–insulina protaminowo-cynkowa</t></is></c><c r="M589" s="2" t="inlineStr" /><c r="N589" s="2" t="inlineStr" /><c r="O589" s="2" t="inlineStr" /><c r="P589" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q589" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="590"><c r="A590" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B590" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C590" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D590" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E590" s="2" t="inlineStr"><is><t>Ostre zapalenie trzustki może być powikłaniem stosowania:</t></is></c><c r="F590" s="2" t="inlineStr"><is><t>inhibitorów dipeptydylopeptydazy 4 (DPP-4)</t></is></c><c r="G590" s="2" t="inlineStr"><is><t>inhibitory reduktazy HMG-Ca</t></is></c><c r="H590" s="2" t="inlineStr"><is><t>związków kwasu 5-aminosalicylowego</t></is></c><c r="I590" s="2" t="inlineStr"><is><t>doustnych środków antykoncepcyjnych</t></is></c><c r="J590" s="2" t="inlineStr" /><c r="K590" s="2" t="inlineStr" /><c r="L590" s="2" t="inlineStr" /><c r="M590" s="2" t="inlineStr" /><c r="N590" s="2" t="inlineStr" /><c r="O590" s="2" t="inlineStr" /><c r="P590" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q590" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="591"><c r="A591" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B591" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C591" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D591" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E591" s="2" t="inlineStr"><is><t>Pacjentka z obustronnym ostrym pozagałkowym zapaleniem nerwu wzrokowego, co zagraża ślepotą, wymaga leczenia metyloprednizolonem (brak alternatywy leczniczej). Zostałeś poproszona/-y o konsultację w celu oceny przeciwwskazań do steroidoterapii. Która z chorób współistniejących jest w tej sytuacji przeciwwskazaniem do zastosowania leku:</t></is></c><c r="F591" s="2" t="inlineStr"><is><t>ciężka sepsa o niejasnej etiologii</t></is></c><c r="G591" s="2" t="inlineStr" /><c r="H591" s="2" t="inlineStr" /><c r="I591" s="2" t="inlineStr" /><c r="J591" s="2" t="inlineStr" /><c r="K591" s="2" t="inlineStr"><is><t>cukrzyca typu 1</t></is></c><c r="L591" s="2" t="inlineStr"><is><t>nadciśnienie tętnicze</t></is></c><c r="M591" s="2" t="inlineStr"><is><t>zaburzenia psychotyczne pod postacią omamów i agresji</t></is></c><c r="N591" s="2" t="inlineStr" /><c r="O591" s="2" t="inlineStr" /><c r="P591" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q591" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="592"><c r="A592" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B592" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C592" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D592" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E592" s="2" t="inlineStr"><is><t>Które połączenie rozważysz w przypadku nie osiągnięcia zakładanej redukcji stężenia cholesterolu frakcji LDL podczas stosowania diety i atorwastatyny?</t></is></c><c r="F592" s="2" t="inlineStr"><is><t>atorwastatyna + anacetrapib</t></is></c><c r="G592" s="2" t="inlineStr"><is><t>atorwastatyna + ezetymib</t></is></c><c r="H592" s="2" t="inlineStr"><is><t>atorwastatyna + kwas eikozapentaenowy</t></is></c><c r="I592" s="2" t="inlineStr"><is><t>atorwastatyna + ewolokumab</t></is></c><c r="J592" s="2" t="inlineStr" /><c r="K592" s="2" t="inlineStr" /><c r="L592" s="2" t="inlineStr" /><c r="M592" s="2" t="inlineStr" /><c r="N592" s="2" t="inlineStr" /><c r="O592" s="2" t="inlineStr" /><c r="P592" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q592" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="593"><c r="A593" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B593" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C593" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D593" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E593" s="2" t="inlineStr"><is><t>Taki sam mechanizm działania mają:</t></is></c><c r="F593" s="2" t="inlineStr"><is><t>bazyliksymab i daklizumab</t></is></c><c r="G593" s="2" t="inlineStr"><is><t>rytuksymab i okrelizumab</t></is></c><c r="H593" s="2" t="inlineStr" /><c r="I593" s="2" t="inlineStr" /><c r="J593" s="2" t="inlineStr" /><c r="K593" s="2" t="inlineStr"><is><t>natalizumab i fingolimod</t></is></c><c r="L593" s="2" t="inlineStr"><is><t>filgrastym i romiplostym</t></is></c><c r="M593" s="2" t="inlineStr" /><c r="N593" s="2" t="inlineStr" /><c r="O593" s="2" t="inlineStr" /><c r="P593" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q593" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="594"><c r="A594" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B594" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C594" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D594" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E594" s="2" t="inlineStr"><is><t>Powikłaniem stosowania inhibitora H+ K+ –ATPazy komórek okładzinowych może być:</t></is></c><c r="F594" s="2" t="inlineStr"><is><t>niedokrwistość makrocytarna z powodu niedoboru witaminy B12</t></is></c><c r="G594" s="2" t="inlineStr"><is><t>osteoporoza z powodu zaburzeń wchłaniania wapnia</t></is></c><c r="H594" s="2" t="inlineStr"><is><t>bakteryjne zakażenia przewodu pokarmowego</t></is></c><c r="I594" s="2" t="inlineStr"><is><t>zmiany wchłaniania wielu leków z przewodu pokarmowego</t></is></c><c r="J594" s="2" t="inlineStr" /><c r="K594" s="2" t="inlineStr" /><c r="L594" s="2" t="inlineStr" /><c r="M594" s="2" t="inlineStr" /><c r="N594" s="2" t="inlineStr" /><c r="O594" s="2" t="inlineStr" /><c r="P594" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q594" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="595"><c r="A595" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B595" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C595" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D595" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E595" s="2" t="inlineStr"><is><t>Lekiem stosowanym w objawach ze strony przewodu pokarmowego o wpływie na układ opioidowy jest:</t></is></c><c r="F595" s="2" t="inlineStr"><is><t>trimebutyna</t></is></c><c r="G595" s="2" t="inlineStr"><is><t>racekadotryl</t></is></c><c r="H595" s="2" t="inlineStr"><is><t>metylnaltrekson</t></is></c><c r="I595" s="2" t="inlineStr" /><c r="J595" s="2" t="inlineStr" /><c r="K595" s="2" t="inlineStr"><is><t>dekstrometorfan</t></is></c><c r="L595" s="2" t="inlineStr" /><c r="M595" s="2" t="inlineStr" /><c r="N595" s="2" t="inlineStr" /><c r="O595" s="2" t="inlineStr" /><c r="P595" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q595" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="596"><c r="A596" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B596" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C596" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D596" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E596" s="2" t="inlineStr"><is><t>W niewydolności nerek należy zmodyfikować dawkowanie:</t></is></c><c r="F596" s="2" t="inlineStr"><is><t>eteksylanu dabigatranu</t></is></c><c r="G596" s="2" t="inlineStr" /><c r="H596" s="2" t="inlineStr" /><c r="I596" s="2" t="inlineStr" /><c r="J596" s="2" t="inlineStr" /><c r="K596" s="2" t="inlineStr"><is><t>atorwastatyny</t></is></c><c r="L596" s="2" t="inlineStr"><is><t>kwasu acetylosalicylowego</t></is></c><c r="M596" s="2" t="inlineStr"><is><t>lewotyroksyny</t></is></c><c r="N596" s="2" t="inlineStr" /><c r="O596" s="2" t="inlineStr" /><c r="P596" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q596" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="597"><c r="A597" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B597" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C597" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D597" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E597" s="2" t="inlineStr"><is><t>Tramadol:</t></is></c><c r="F597" s="2" t="inlineStr"><is><t>ma mechanizm działania podobny do tapentadolu</t></is></c><c r="G597" s="2" t="inlineStr"><is><t>może powodować drgawki</t></is></c><c r="H597" s="2" t="inlineStr" /><c r="I597" s="2" t="inlineStr" /><c r="J597" s="2" t="inlineStr" /><c r="K597" s="2" t="inlineStr"><is><t>może zwiększać ryzyko hiperglikemii i pogarszać kontrolę cukrzycy</t></is></c><c r="L597" s="2" t="inlineStr"><is><t>działa przeciwbólowo skuteczniej w połączeniu z lekami przeciwdepresyjnymi z powodu synergizmu działania</t></is></c><c r="M597" s="2" t="inlineStr" /><c r="N597" s="2" t="inlineStr" /><c r="O597" s="2" t="inlineStr" /><c r="P597" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q597" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="598"><c r="A598" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B598" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C598" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D598" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E598" s="2" t="inlineStr"><is><t>Rotacja opioidów:</t></is></c><c r="F598" s="2" t="inlineStr"><is><t>wymaga ustalenia ekwianelgetycznych dawek zamienianych opioidów, np. morfina : oksykodon p.o. odpowiednio 10 mg : 6,67 mg</t></is></c><c r="G598" s="2" t="inlineStr" /><c r="H598" s="2" t="inlineStr" /><c r="I598" s="2" t="inlineStr" /><c r="J598" s="2" t="inlineStr" /><c r="K598" s="2" t="inlineStr"><is><t>wymaga nie łączenia opioidów z innymi lekami przeciwbólowymi</t></is></c><c r="L598" s="2" t="inlineStr"><is><t>pomaga zapobiec immunosupresyjnemu działaniu opioidów</t></is></c><c r="M598" s="2" t="inlineStr"><is><t>powinna być oparta o tą samą drogę podania, to znaczy rotowane opioidy powinny mieć tę samą postać farmaceutyczną</t></is></c><c r="N598" s="2" t="inlineStr" /><c r="O598" s="2" t="inlineStr" /><c r="P598" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q598" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="599"><c r="A599" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B599" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C599" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D599" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E599" s="2" t="inlineStr"><is><t>Pasażerowie podróżujący wagonem metra, w którym odnaleziono porzucony bagaż, zostali przyjęci na oddział ratunkowy z powodu bolesnych skurczów jelit, wymiotów, duszności i osłabienia siły mięśniowej. W badaniu fizykalnym stwierdzono zwiększoną częstość oddechów, świsty oskrzelowe, bradykardię i zwężenie źrenic. Lek/leki z wyboru w powyższej sytuacji to:</t></is></c><c r="F599" s="2" t="inlineStr"><is><t>acetylocysteina</t></is></c><c r="G599" s="2" t="inlineStr"><is><t>pralidoksym</t></is></c><c r="H599" s="2" t="inlineStr"><is><t>pirydostygmina</t></is></c><c r="I599" s="2" t="inlineStr"><is><t>atropina</t></is></c><c r="J599" s="2" t="inlineStr" /><c r="K599" s="2" t="inlineStr" /><c r="L599" s="2" t="inlineStr" /><c r="M599" s="2" t="inlineStr" /><c r="N599" s="2" t="inlineStr" /><c r="O599" s="2" t="inlineStr" /><c r="P599" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q599" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="600"><c r="A600" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B600" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C600" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D600" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E600" s="2" t="inlineStr"><is><t>Inhibitory immunologicznych punktów kontrolnych:</t></is></c><c r="F600" s="2" t="inlineStr"><is><t>są przeciwciałami monoklonalnymi przeciw CLTA-4, PD-1 i PDL-1</t></is></c><c r="G600" s="2" t="inlineStr"><is><t>nawiązują koncepcyjnie do immunostymulującego działania szczepionki BCG w raku pęcherza moczowego</t></is></c><c r="H600" s="2" t="inlineStr"><is><t>są skuteczne w leczeniu różnych typów nowotworów</t></is></c><c r="I600" s="2" t="inlineStr"><is><t>indukują zjawiska autoimmunologiczne</t></is></c><c r="J600" s="2" t="inlineStr" /><c r="K600" s="2" t="inlineStr" /><c r="L600" s="2" t="inlineStr" /><c r="M600" s="2" t="inlineStr" /><c r="N600" s="2" t="inlineStr" /><c r="O600" s="2" t="inlineStr" /><c r="P600" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q600" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="601"><c r="A601" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B601" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C601" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D601" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E601" s="2" t="inlineStr"><is><t>Projektant mody Alexander McQeen (1969-2010) był uzależniony od wielu substancji psychoaktywnych. Które cechy opisu jego zachowania z filmu biograficznego „Wizjoner. Buntownik. Geniusz” wskazują na ekspozycję na kokainę?</t></is></c><c r="F601" s="2" t="inlineStr"><is><t>gadatliwy, w świetnym nastroju, pełen energii i bardzo ruchliwy mimo 16 h pracy przed pokazem, ale spocony i z nawracającymi krwawieniami z nosa</t></is></c><c r="G601" s="2" t="inlineStr" /><c r="H601" s="2" t="inlineStr" /><c r="I601" s="2" t="inlineStr" /><c r="J601" s="2" t="inlineStr" /><c r="K601" s="2" t="inlineStr"><is><t>brawurowy i agresywny, z zaburzeniami mowy i równowagi ruchowej</t></is></c><c r="L601" s="2" t="inlineStr"><is><t>błyskotliwy, dowcipny, szybko przyswajający duże ilości nowych informacji, ale ciągle głodny i z okresowymi napadami paniki</t></is></c><c r="M601" s="2" t="inlineStr"><is><t>w euforii, komplementujący współpracowników, okresowo z barwnymi wizjami, okresowo podsypiający, z przekrwionymi twardówkami</t></is></c><c r="N601" s="2" t="inlineStr" /><c r="O601" s="2" t="inlineStr" /><c r="P601" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q601" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="602"><c r="A602" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B602" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C602" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D602" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E602" s="2" t="inlineStr"><is><t>Działanie farmakologiczne inne niż suplementacja w stanach niedoboru ma:</t></is></c><c r="F602" s="2" t="inlineStr"><is><t>fitomenadion w niewydolności wątroby i przedawkowaniu warfaryny</t></is></c><c r="G602" s="2" t="inlineStr"><is><t>cholekalcyferol w profilaktyce i leczeniu osteoporozy</t></is></c><c r="H602" s="2" t="inlineStr" /><c r="I602" s="2" t="inlineStr" /><c r="J602" s="2" t="inlineStr" /><c r="K602" s="2" t="inlineStr"><is><t>nikotynamid w hiperurykemii i atakach dny moczanowej</t></is></c><c r="L602" s="2" t="inlineStr"><is><t>tokoferol w profilatyce raka płuc</t></is></c><c r="M602" s="2" t="inlineStr" /><c r="N602" s="2" t="inlineStr" /><c r="O602" s="2" t="inlineStr" /><c r="P602" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q602" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="603"><c r="A603" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B603" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C603" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D603" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E603" s="2" t="inlineStr"><is><t>Obniżenie stężenia potasu w surowicy może być spowodowane zastosowaniem:</t></is></c><c r="F603" s="2" t="inlineStr"><is><t>bisakodylu</t></is></c><c r="G603" s="2" t="inlineStr"><is><t>prednizonu</t></is></c><c r="H603" s="2" t="inlineStr"><is><t>glukozy z insuliną</t></is></c><c r="I603" s="2" t="inlineStr" /><c r="J603" s="2" t="inlineStr" /><c r="K603" s="2" t="inlineStr"><is><t>glukonianu wapnia</t></is></c><c r="L603" s="2" t="inlineStr" /><c r="M603" s="2" t="inlineStr" /><c r="N603" s="2" t="inlineStr" /><c r="O603" s="2" t="inlineStr" /><c r="P603" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q603" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="604"><c r="A604" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B604" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C604" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D604" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E604" s="2" t="inlineStr"><is><t>Zasadzką płynoterapii jest:</t></is></c><c r="F604" s="2" t="inlineStr"><is><t>obrzęk płuc po nawadnianiu płynem wieloelektrolitowym</t></is></c><c r="G604" s="2" t="inlineStr"><is><t>brak możliwości wiarygodnego oznaczenia grupy krwi i wykonania próby krzyżowej po padaniu dekstranu 70 000</t></is></c><c r="H604" s="2" t="inlineStr"><is><t>hiperonkotyczna niewydolność nerek po podaniu hydroksyetylowanej skrobi 130/0,4</t></is></c><c r="I604" s="2" t="inlineStr" /><c r="J604" s="2" t="inlineStr" /><c r="K604" s="2" t="inlineStr"><is><t>zakrzepica podczas stosowania 20% roztworu albumin</t></is></c><c r="L604" s="2" t="inlineStr" /><c r="M604" s="2" t="inlineStr" /><c r="N604" s="2" t="inlineStr" /><c r="O604" s="2" t="inlineStr" /><c r="P604" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q604" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="605"><c r="A605" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B605" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C605" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D605" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E605" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenia:</t></is></c><c r="F605" s="2" t="inlineStr"><is><t>w USA obowiązuje nazewnictwo leków w pewnym zakresie autonomiczne od tworzonej przez WHO listy nazw międzynarodowych, przykłady paracetamol i acetaminofen czy petydyna i meperydyna</t></is></c><c r="G605" s="2" t="inlineStr" /><c r="H605" s="2" t="inlineStr" /><c r="I605" s="2" t="inlineStr" /><c r="J605" s="2" t="inlineStr" /><c r="K605" s="2" t="inlineStr"><is><t>po wygaśnięciu ochrony patentowej enoksaparyny wprowadzono jej odtwórcze odpowiedniki tylko na podstawie wykazania ich biorównoważności</t></is></c><c r="L605" s="2" t="inlineStr"><is><t>antysensowne oligonukleotydy mają w nazwie końcówkę -stim</t></is></c><c r="M605" s="2" t="inlineStr"><is><t>przy konwersji między lekami biopodobnymi obowiązuje zasada zamiany automatycznej (substytucji)</t></is></c><c r="N605" s="2" t="inlineStr" /><c r="O605" s="2" t="inlineStr" /><c r="P605" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q605" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="606"><c r="A606" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B606" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C606" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D606" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E606" s="2" t="inlineStr"><is><t>Wskaż prawidłowe zestawienia lek-spektrum działania:</t></is></c><c r="F606" s="2" t="inlineStr"><is><t>cyprofloksacyna – Pseudomonas aeruginosa, Mycoplasma pneumoniae</t></is></c><c r="G606" s="2" t="inlineStr"><is><t>penicylina G – Fusobacterium spp., Streptococcus pyogenes</t></is></c><c r="H606" s="2" t="inlineStr"><is><t>rifaksymina – Escherichia coli, Campylobacter jejuni</t></is></c><c r="I606" s="2" t="inlineStr" /><c r="J606" s="2" t="inlineStr" /><c r="K606" s="2" t="inlineStr"><is><t>gentamycyna – Clostridium spp., Helicobacter pylori</t></is></c><c r="L606" s="2" t="inlineStr" /><c r="M606" s="2" t="inlineStr" /><c r="N606" s="2" t="inlineStr" /><c r="O606" s="2" t="inlineStr" /><c r="P606" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q606" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="607"><c r="A607" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B607" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C607" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D607" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E607" s="2" t="inlineStr"><is><t>Wskaż zdania prawdziwe:</t></is></c><c r="F607" s="2" t="inlineStr"><is><t>zastosowanie technologii liposomów pozwoliło na otrzymanie preparatów amfoterycyny B o zmniejszonej nefrotoksyczności</t></is></c><c r="G607" s="2" t="inlineStr" /><c r="H607" s="2" t="inlineStr" /><c r="I607" s="2" t="inlineStr" /><c r="J607" s="2" t="inlineStr" /><c r="K607" s="2" t="inlineStr"><is><t>w przeciwieństwie do terbinafiny, azole hamują enzym szlaku biosyntezy ergosterolu niezwiązany z układem CYP450</t></is></c><c r="L607" s="2" t="inlineStr"><is><t>kaspofungina może być skuteczna w leczeniu i profilaktyce zapalenia opon mózgowo-rdzeniowych o etiologii Cryptococcus neoformans</t></is></c><c r="M607" s="2" t="inlineStr"><is><t>dla uzyskania możliwie najlepszych efektów leczenia amfoterycyną B najistotniejsze z punktu widzenia PK/PD jest, aby stężenie leku pomiędzy kolejnymi podaniami utrzymywało się na poziomie 4 x MIC optymalnie przez 100% czasu</t></is></c><c r="N607" s="2" t="inlineStr" /><c r="O607" s="2" t="inlineStr" /><c r="P607" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q607" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="608"><c r="A608" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B608" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C608" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D608" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E608" s="2" t="inlineStr"><is><t>Modyfikacja dawki nie jest wymagana u pacjenta z eGFR wg wzoru Cockcrofta- Gaulta = 24 ml/min podczas stosowania:</t></is></c><c r="F608" s="2" t="inlineStr"><is><t>ceftriaksonu</t></is></c><c r="G608" s="2" t="inlineStr"><is><t>cefoperazonu</t></is></c><c r="H608" s="2" t="inlineStr" /><c r="I608" s="2" t="inlineStr" /><c r="J608" s="2" t="inlineStr" /><c r="K608" s="2" t="inlineStr"><is><t>ceftazydymu</t></is></c><c r="L608" s="2" t="inlineStr"><is><t>cefepimu</t></is></c><c r="M608" s="2" t="inlineStr" /><c r="N608" s="2" t="inlineStr" /><c r="O608" s="2" t="inlineStr" /><c r="P608" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q608" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="609"><c r="A609" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B609" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C609" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D609" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E609" s="2" t="inlineStr"><is><t>Jaki lek można opisać w następujący sposób: ma działanie bójcze, jego celem farmakodynamicznym jest jak największy stosunek AUC24:MIC i łatwa jest jego sekwencja do stosowania doustnego:</t></is></c><c r="F609" s="2" t="inlineStr"><is><t>Lewofloksacyna</t></is></c><c r="G609" s="2" t="inlineStr" /><c r="H609" s="2" t="inlineStr" /><c r="I609" s="2" t="inlineStr" /><c r="J609" s="2" t="inlineStr" /><c r="K609" s="2" t="inlineStr"><is><t>Neomycyna</t></is></c><c r="L609" s="2" t="inlineStr"><is><t>Wankomycyna</t></is></c><c r="M609" s="2" t="inlineStr"><is><t>Klarytromycyna</t></is></c><c r="N609" s="2" t="inlineStr" /><c r="O609" s="2" t="inlineStr" /><c r="P609" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q609" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="610"><c r="A610" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B610" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C610" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D610" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E610" s="2" t="inlineStr"><is><t>Które stwierdzenie jest prawdziwe w leczeniu zakażeń?</t></is></c><c r="F610" s="2" t="inlineStr"><is><t>leki przeciwinfekcyjne są jedynie uzupełnieniem leczenia zabiegowego w postaci aspiracji lub drenażu w przypadku ropni i ropniaków</t></is></c><c r="G610" s="2" t="inlineStr"><is><t>leczenie zakażenia w obrębie tylnej komory oka (szklistki) wymaga podania leków przeciwinfekcyjnych doszklistkowo</t></is></c><c r="H610" s="2" t="inlineStr"><is><t>nie jest możliwe wyleczenia „zakażenia” sztucznych materiałów: protez, cewników, sztucznych zastawek</t></is></c><c r="I610" s="2" t="inlineStr"><is><t>w przewlekłym zapaleniu zatok konieczne jest chirurgiczna korekta nieprawidłowości anatomicznych, tj. polip czy, skrzywienie przegrody nosa</t></is></c><c r="J610" s="2" t="inlineStr" /><c r="K610" s="2" t="inlineStr" /><c r="L610" s="2" t="inlineStr" /><c r="M610" s="2" t="inlineStr" /><c r="N610" s="2" t="inlineStr" /><c r="O610" s="2" t="inlineStr" /><c r="P610" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q610" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="611"><c r="A611" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B611" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C611" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D611" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E611" s="2" t="inlineStr"><is><t>U pacjenta z podejrzeniem atypowego zakażenia układu oddechowego, stosującego na co dzień leki z grupy inhibitorów reduktazy HMG-CoA (pacjent nie pamięta nazwy leku), planujesz włączyć antybiotyk makrolidowy. Za bezpieczną opcję terapeutyczną w tej sytuacji uznasz:</t></is></c><c r="F611" s="2" t="inlineStr"><is><t>azytromycynę</t></is></c><c r="G611" s="2" t="inlineStr" /><c r="H611" s="2" t="inlineStr" /><c r="I611" s="2" t="inlineStr" /><c r="J611" s="2" t="inlineStr" /><c r="K611" s="2" t="inlineStr"><is><t>klarytromycynę</t></is></c><c r="L611" s="2" t="inlineStr"><is><t>telitromycynę</t></is></c><c r="M611" s="2" t="inlineStr"><is><t>erytromycynę</t></is></c><c r="N611" s="2" t="inlineStr" /><c r="O611" s="2" t="inlineStr" /><c r="P611" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q611" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="612"><c r="A612" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B612" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C612" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D612" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E612" s="2" t="inlineStr"><is><t>Wskaż prawidłowe zestawienia lek-działanie niepożądane:</t></is></c><c r="F612" s="2" t="inlineStr"><is><t>izoniazyd – toczeń polekowy</t></is></c><c r="G612" s="2" t="inlineStr"><is><t>pirazynamid– hiperurikemia</t></is></c><c r="H612" s="2" t="inlineStr"><is><t>ryfampicyna – małopłytkowość</t></is></c><c r="I612" s="2" t="inlineStr"><is><t>etambutol – pozagałkowe zapalenie nerwu wzrokowego</t></is></c><c r="J612" s="2" t="inlineStr" /><c r="K612" s="2" t="inlineStr" /><c r="L612" s="2" t="inlineStr" /><c r="M612" s="2" t="inlineStr" /><c r="N612" s="2" t="inlineStr" /><c r="O612" s="2" t="inlineStr" /><c r="P612" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q612" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="613"><c r="A613" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B613" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C613" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D613" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E613" s="2" t="inlineStr"><is><t>Leki przeciwbakteryjne o wysokim potencjale do selekcji szczepów Clostridium difficile to:</t></is></c><c r="F613" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="G613" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="H613" s="2" t="inlineStr" /><c r="I613" s="2" t="inlineStr" /><c r="J613" s="2" t="inlineStr" /><c r="K613" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="L613" s="2" t="inlineStr"><is><t>fidaksomycyna</t></is></c><c r="M613" s="2" t="inlineStr" /><c r="N613" s="2" t="inlineStr" /><c r="O613" s="2" t="inlineStr" /><c r="P613" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q613" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="614"><c r="A614" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B614" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C614" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D614" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E614" s="2" t="inlineStr"><is><t>Pacjent leczony jest dożylnie lekiem, którego farmakokinetyka opisana jest następująco: słabo wchłania się z przewodu pokarmowego, podlega ograniczonej dystrybucji do tkanek, nie jest metabolizowany (bądź jest metabolizowany w minimalnym stopniu), wydalany jest głównie przez nerki. Lekiem tym może być:</t></is></c><c r="F614" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="G614" s="2" t="inlineStr"><is><t>kolistymetat sodu</t></is></c><c r="H614" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="I614" s="2" t="inlineStr" /><c r="J614" s="2" t="inlineStr" /><c r="K614" s="2" t="inlineStr"><is><t>erytromycyna</t></is></c><c r="L614" s="2" t="inlineStr" /><c r="M614" s="2" t="inlineStr" /><c r="N614" s="2" t="inlineStr" /><c r="O614" s="2" t="inlineStr" /><c r="P614" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q614" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="615"><c r="A615" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B615" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C615" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D615" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E615" s="2" t="inlineStr"><is><t>W leczeniu inwazyjnej aspergilozy znalazły zastosowanie:</t></is></c><c r="F615" s="2" t="inlineStr"><is><t>amfoterycyna B podawana dożylnie</t></is></c><c r="G615" s="2" t="inlineStr"><is><t>worykonazol podawany dożylnie</t></is></c><c r="H615" s="2" t="inlineStr" /><c r="I615" s="2" t="inlineStr" /><c r="J615" s="2" t="inlineStr" /><c r="K615" s="2" t="inlineStr"><is><t>kaspofungina podawana doustnie</t></is></c><c r="L615" s="2" t="inlineStr"><is><t>terbinafina podawana doustnie</t></is></c><c r="M615" s="2" t="inlineStr" /><c r="N615" s="2" t="inlineStr" /><c r="O615" s="2" t="inlineStr" /><c r="P615" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q615" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="616"><c r="A616" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B616" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C616" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D616" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E616" s="2" t="inlineStr"><is><t>Dobrą dystrybucją do ośrodkowego układu nerwowego charakteryzuje się:</t></is></c><c r="F616" s="2" t="inlineStr"><is><t>ceftriakson</t></is></c><c r="G616" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="H616" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="I616" s="2" t="inlineStr" /><c r="J616" s="2" t="inlineStr" /><c r="K616" s="2" t="inlineStr"><is><t>kaspofungina</t></is></c><c r="L616" s="2" t="inlineStr" /><c r="M616" s="2" t="inlineStr" /><c r="N616" s="2" t="inlineStr" /><c r="O616" s="2" t="inlineStr" /><c r="P616" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q616" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="617"><c r="A617" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B617" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C617" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D617" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E617" s="2" t="inlineStr"><is><t>W schematach eradykacji Helicobacter pylori są stosowane:</t></is></c><c r="F617" s="2" t="inlineStr"><is><t>klarytromycyna</t></is></c><c r="G617" s="2" t="inlineStr"><is><t>Amoksycylina</t></is></c><c r="H617" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="I617" s="2" t="inlineStr"><is><t>tetracyklina</t></is></c><c r="J617" s="2" t="inlineStr" /><c r="K617" s="2" t="inlineStr" /><c r="L617" s="2" t="inlineStr" /><c r="M617" s="2" t="inlineStr" /><c r="N617" s="2" t="inlineStr" /><c r="O617" s="2" t="inlineStr" /><c r="P617" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q617" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="618"><c r="A618" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B618" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C618" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D618" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E618" s="2" t="inlineStr"><is><t>U kobiety w ciąży z rumieniem wędrującym można zastosować:</t></is></c><c r="F618" s="2" t="inlineStr"><is><t>azytromycynę</t></is></c><c r="G618" s="2" t="inlineStr"><is><t>amoksycylinę</t></is></c><c r="H618" s="2" t="inlineStr" /><c r="I618" s="2" t="inlineStr" /><c r="J618" s="2" t="inlineStr" /><c r="K618" s="2" t="inlineStr"><is><t>doksycyklinę</t></is></c><c r="L618" s="2" t="inlineStr"><is><t>klindamycynę</t></is></c><c r="M618" s="2" t="inlineStr" /><c r="N618" s="2" t="inlineStr" /><c r="O618" s="2" t="inlineStr" /><c r="P618" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q618" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="619"><c r="A619" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B619" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C619" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D619" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E619" s="2" t="inlineStr"><is><t>W zakażeniu o etiologii MRSA(methicyllin-resistant Staphylococcus aureus) zasadne jest zastosowanie:</t></is></c><c r="F619" s="2" t="inlineStr"><is><t>ceftaroliny</t></is></c><c r="G619" s="2" t="inlineStr"><is><t>linezolidu</t></is></c><c r="H619" s="2" t="inlineStr" /><c r="I619" s="2" t="inlineStr" /><c r="J619" s="2" t="inlineStr" /><c r="K619" s="2" t="inlineStr"><is><t>kloksacyliny</t></is></c><c r="L619" s="2" t="inlineStr"><is><t>meropenemu</t></is></c><c r="M619" s="2" t="inlineStr" /><c r="N619" s="2" t="inlineStr" /><c r="O619" s="2" t="inlineStr" /><c r="P619" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q619" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="620"><c r="A620" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B620" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C620" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D620" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E620" s="2" t="inlineStr"><is><t>W biegunce o etiologii Clostridium difficile uzasadnione może być podanie doustne:</t></is></c><c r="F620" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="G620" s="2" t="inlineStr"><is><t>metronidazolu</t></is></c><c r="H620" s="2" t="inlineStr"><is><t>fidaksomycyny</t></is></c><c r="I620" s="2" t="inlineStr" /><c r="J620" s="2" t="inlineStr" /><c r="K620" s="2" t="inlineStr"><is><t>nifuroksazydu</t></is></c><c r="L620" s="2" t="inlineStr" /><c r="M620" s="2" t="inlineStr" /><c r="N620" s="2" t="inlineStr" /><c r="O620" s="2" t="inlineStr" /><c r="P620" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q620" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="621"><c r="A621" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B621" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C621" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D621" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E621" s="2" t="inlineStr"><is><t>Wskaż właściwe skojarzenie lek – potencjalne działanie niepożądane:</t></is></c><c r="F621" s="2" t="inlineStr"><is><t>chloramfenikol – zespół szarego dziecka</t></is></c><c r="G621" s="2" t="inlineStr"><is><t>doksycyklina - fotodermatoza</t></is></c><c r="H621" s="2" t="inlineStr" /><c r="I621" s="2" t="inlineStr" /><c r="J621" s="2" t="inlineStr" /><c r="K621" s="2" t="inlineStr"><is><t>gentamycyna - żółtaczka cholestatyczna</t></is></c><c r="L621" s="2" t="inlineStr"><is><t>klindamycyna – zespół serotoninowy</t></is></c><c r="M621" s="2" t="inlineStr" /><c r="N621" s="2" t="inlineStr" /><c r="O621" s="2" t="inlineStr" /><c r="P621" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q621" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="622"><c r="A622" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B622" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C622" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D622" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E622" s="2" t="inlineStr"><is><t>Zaburzenia rytmu serca mogą wystąpić w trakcie stosowania:</t></is></c><c r="F622" s="2" t="inlineStr"><is><t>moksyfloksacyny</t></is></c><c r="G622" s="2" t="inlineStr"><is><t>klarytromycyny</t></is></c><c r="H622" s="2" t="inlineStr" /><c r="I622" s="2" t="inlineStr" /><c r="J622" s="2" t="inlineStr" /><c r="K622" s="2" t="inlineStr"><is><t>fidaksomycyny</t></is></c><c r="L622" s="2" t="inlineStr"><is><t>Mupirocyny</t></is></c><c r="M622" s="2" t="inlineStr" /><c r="N622" s="2" t="inlineStr" /><c r="O622" s="2" t="inlineStr" /><c r="P622" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q622" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="623"><c r="A623" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B623" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C623" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D623" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E623" s="2" t="inlineStr"><is><t>Kolistymetat sodu:</t></is></c><c r="F623" s="2" t="inlineStr"><is><t>jest prolekiem</t></is></c><c r="G623" s="2" t="inlineStr"><is><t>jest zarezerwowany do leczenia zakażeń szczepami wielolekoopornymi G(-)</t></is></c><c r="H623" s="2" t="inlineStr" /><c r="I623" s="2" t="inlineStr" /><c r="J623" s="2" t="inlineStr" /><c r="K623" s="2" t="inlineStr"><is><t>działa na VRE (Vancomycin-Resistant Enterococcus)</t></is></c><c r="L623" s="2" t="inlineStr"><is><t>dobrze wchłania się z przewodu pokarmowego</t></is></c><c r="M623" s="2" t="inlineStr" /><c r="N623" s="2" t="inlineStr" /><c r="O623" s="2" t="inlineStr" /><c r="P623" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q623" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="624"><c r="A624" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B624" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C624" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D624" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E624" s="2" t="inlineStr"><is><t>Kolistymetat sodu:</t></is></c><c r="F624" s="2" t="inlineStr"><is><t>jest prolekiem, który po przekształceniu w aktywną postać powoduje lizę błony komórek bakteryjnych</t></is></c><c r="G624" s="2" t="inlineStr"><is><t>może spowodować zaburzenia ruchowe (ataksja) i zaburzenia czuciowe (parestezje)</t></is></c><c r="H624" s="2" t="inlineStr"><is><t>jest stosowany w zakażeniach pałeczkami Gram (-) przy ograniczonych opcjach terapeutycznych</t></is></c><c r="I624" s="2" t="inlineStr" /><c r="J624" s="2" t="inlineStr" /><c r="K624" s="2" t="inlineStr"><is><t>jest stosowany wyłącznie dożylnie</t></is></c><c r="L624" s="2" t="inlineStr" /><c r="M624" s="2" t="inlineStr" /><c r="N624" s="2" t="inlineStr" /><c r="O624" s="2" t="inlineStr" /><c r="P624" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q624" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="625"><c r="A625" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B625" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C625" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D625" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E625" s="2" t="inlineStr"><is><t>Tygecyklina:</t></is></c><c r="F625" s="2" t="inlineStr"><is><t>jest stosowana w wewnątrzbrzusznych zakażeniach szczepami wielolekoopornymi</t></is></c><c r="G625" s="2" t="inlineStr" /><c r="H625" s="2" t="inlineStr" /><c r="I625" s="2" t="inlineStr" /><c r="J625" s="2" t="inlineStr" /><c r="K625" s="2" t="inlineStr"><is><t>dobrze wchłania się z przewodu pokarmowego</t></is></c><c r="L625" s="2" t="inlineStr"><is><t>bardzo często jest przyczyną zapalenia ścięgna Achillesa</t></is></c><c r="M625" s="2" t="inlineStr"><is><t>działa na Pseudomonas aeruginosa</t></is></c><c r="N625" s="2" t="inlineStr" /><c r="O625" s="2" t="inlineStr" /><c r="P625" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q625" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="626"><c r="A626" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B626" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C626" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D626" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E626" s="2" t="inlineStr"><is><t>Daptomycyna może być skuteczna w zakażeniach szczepami:</t></is></c><c r="F626" s="2" t="inlineStr"><is><t>MRSA (methicyllin-resistant Staphylococcus aureus)</t></is></c><c r="G626" s="2" t="inlineStr"><is><t>MSSA (methicillin-sensitive Staphylococcus aureus)</t></is></c><c r="H626" s="2" t="inlineStr"><is><t>VRE (Vancomycin-Resistant Enterococcus)</t></is></c><c r="I626" s="2" t="inlineStr" /><c r="J626" s="2" t="inlineStr" /><c r="K626" s="2" t="inlineStr"><is><t>CPE (Carbapenemase-producing Enterobacteriaceae)</t></is></c><c r="L626" s="2" t="inlineStr" /><c r="M626" s="2" t="inlineStr" /><c r="N626" s="2" t="inlineStr" /><c r="O626" s="2" t="inlineStr" /><c r="P626" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q626" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="627"><c r="A627" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B627" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C627" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D627" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E627" s="2" t="inlineStr"><is><t>Lewofloksacyna:</t></is></c><c r="F627" s="2" t="inlineStr"><is><t>wykazuje aktywność wobec Streptococcus pneumoniae</t></is></c><c r="G627" s="2" t="inlineStr"><is><t>wykazuje aktywność wobec Legionella pneumophila</t></is></c><c r="H627" s="2" t="inlineStr" /><c r="I627" s="2" t="inlineStr" /><c r="J627" s="2" t="inlineStr" /><c r="K627" s="2" t="inlineStr"><is><t>ma taki sam zakres działania jak moksyfloksacyna</t></is></c><c r="L627" s="2" t="inlineStr"><is><t>nie działa na Pseudomonas aeruginosa</t></is></c><c r="M627" s="2" t="inlineStr" /><c r="N627" s="2" t="inlineStr" /><c r="O627" s="2" t="inlineStr" /><c r="P627" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q627" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="628"><c r="A628" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B628" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C628" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D628" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E628" s="2" t="inlineStr"><is><t>W przypadku rozpoznania anginy paciorkowcowej u osoby uczulonej na antybiotyki beta￾laktamowe, można zastosować:</t></is></c><c r="F628" s="2" t="inlineStr"><is><t>klindamycynę</t></is></c><c r="G628" s="2" t="inlineStr"><is><t>azytromycynę</t></is></c><c r="H628" s="2" t="inlineStr" /><c r="I628" s="2" t="inlineStr" /><c r="J628" s="2" t="inlineStr" /><c r="K628" s="2" t="inlineStr"><is><t>norfloksacynę</t></is></c><c r="L628" s="2" t="inlineStr"><is><t>kloksacylinę</t></is></c><c r="M628" s="2" t="inlineStr" /><c r="N628" s="2" t="inlineStr" /><c r="O628" s="2" t="inlineStr" /><c r="P628" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q628" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="629"><c r="A629" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B629" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C629" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D629" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E629" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie:</t></is></c><c r="F629" s="2" t="inlineStr"><is><t>owsica – pyrantel, WZW C (wirusowe zapalenie wątroby typu C) – daklataswir</t></is></c><c r="G629" s="2" t="inlineStr"><is><t>wszawica – permetryna, CMV – walgancyklowir</t></is></c><c r="H629" s="2" t="inlineStr" /><c r="I629" s="2" t="inlineStr" /><c r="J629" s="2" t="inlineStr" /><c r="K629" s="2" t="inlineStr"><is><t>CMV (cytomegalovirus) – acyklowir, owsica – pyrantel</t></is></c><c r="L629" s="2" t="inlineStr"><is><t>acyklowir – HSV-2 (herpes simplex 2), amantadyna – profilaktyka grypy typu B</t></is></c><c r="M629" s="2" t="inlineStr" /><c r="N629" s="2" t="inlineStr" /><c r="O629" s="2" t="inlineStr" /><c r="P629" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2018/19</t></is></c><c r="Q629" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="630"><c r="A630" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B630" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C630" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D630" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E630" s="2" t="inlineStr"><is><t>Które pary leków mających ten sam zasadniczy mechanizm działania różnią się istotnie profilem działań klinicznych?</t></is></c><c r="F630" s="2" t="inlineStr"><is><t>werapamil i nitrendypina</t></is></c><c r="G630" s="2" t="inlineStr"><is><t>doksazosyna i tamsulozyna</t></is></c><c r="H630" s="2" t="inlineStr"><is><t>spironolakton i eplerenon</t></is></c><c r="I630" s="2" t="inlineStr" /><c r="J630" s="2" t="inlineStr" /><c r="K630" s="2" t="inlineStr"><is><t>moksonidyna i rylmenidyna</t></is></c><c r="L630" s="2" t="inlineStr" /><c r="M630" s="2" t="inlineStr" /><c r="N630" s="2" t="inlineStr" /><c r="O630" s="2" t="inlineStr" /><c r="P630" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q630" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="631"><c r="A631" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B631" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C631" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D631" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E631" s="2" t="inlineStr"><is><t>Które pary leków mających ten sam zasadniczy mechanizm działania różnią się istotnie profilem działań klinicznych?</t></is></c><c r="F631" s="2" t="inlineStr"><is><t>werapamil i nitrendypina</t></is></c><c r="G631" s="2" t="inlineStr"><is><t>doksazosyna i tamsulozyna</t></is></c><c r="H631" s="2" t="inlineStr" /><c r="I631" s="2" t="inlineStr" /><c r="J631" s="2" t="inlineStr" /><c r="K631" s="2" t="inlineStr"><is><t>moksonidyna i rylmenidyna</t></is></c><c r="L631" s="2" t="inlineStr"><is><t>spironolakton i kanrenon</t></is></c><c r="M631" s="2" t="inlineStr" /><c r="N631" s="2" t="inlineStr" /><c r="O631" s="2" t="inlineStr" /><c r="P631" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q631" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="632"><c r="A632" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B632" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C632" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D632" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E632" s="2" t="inlineStr"><is><t>Do leków aktywujących pośrednio lub bezpośrednio cyklazę guanylową komórek mięśniówki gładkiej naczyń należy:</t></is></c><c r="F632" s="2" t="inlineStr"><is><t>nitroprusydek sodu</t></is></c><c r="G632" s="2" t="inlineStr"><is><t>riocyguat</t></is></c><c r="H632" s="2" t="inlineStr"><is><t>sakubitryl</t></is></c><c r="I632" s="2" t="inlineStr" /><c r="J632" s="2" t="inlineStr" /><c r="K632" s="2" t="inlineStr"><is><t>wardenafil</t></is></c><c r="L632" s="2" t="inlineStr" /><c r="M632" s="2" t="inlineStr" /><c r="N632" s="2" t="inlineStr" /><c r="O632" s="2" t="inlineStr" /><c r="P632" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q632" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="633"><c r="A633" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B633" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C633" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D633" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E633" s="2" t="inlineStr"><is><t>Czy zaproponowany wlew poszczególnych amin katecholowych jest adekwatny na początku leczenia (wybierz najmniejszą dawkę zalecaną) u pacjenta z przedstawionym rozpoznaniem?</t></is></c><c r="F633" s="2" t="inlineStr"><is><t>pacjent = 50 kg z ostrą niewydolnością serca i ciśnieniem skurczowym 85 mmHg – dopamina 200 mg/40 ml 0,9% NaCl → wlew = 3 ml/h</t></is></c><c r="G633" s="2" t="inlineStr"><is><t>pacjent = 100 kg we wstrząsie septycznym z ciśnieniem skurczowym 60 mmHg – noradrenalina 4 mg/40 ml 0,9% NaCl → wlew = 12 ml/h</t></is></c><c r="H633" s="2" t="inlineStr"><is><t>pacjent = 50 kg z zaostrzeniem przewlekłej niewydolności serca skurczowym 105 mmHg – dobutamina 250 mg/50 ml 0,9% NaCl → wlew =1,2 ml/h</t></is></c><c r="I633" s="2" t="inlineStr" /><c r="J633" s="2" t="inlineStr" /><c r="K633" s="2" t="inlineStr"><is><t>pacjent = 100 kg z ostrą niewydolnością serca i ciśnieniem skurczowym 80 mmHg – dobutamina 250 mg/50 ml 0,9% NaCl → wlew = 2,4 ml/h</t></is></c><c r="L633" s="2" t="inlineStr" /><c r="M633" s="2" t="inlineStr" /><c r="N633" s="2" t="inlineStr" /><c r="O633" s="2" t="inlineStr" /><c r="P633" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q633" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="634"><c r="A634" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B634" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C634" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D634" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E634" s="2" t="inlineStr"><is><t>Wskaż lek o bardzo krótkim okresie półtrwania (&lt;5 min), który z tego powodu wymaga stosowania we wlewie dożylnym lub jest wykorzystywany w celu osiągnięcia błyskawicznego krótkotrwałego efektu terapeutycznego:</t></is></c><c r="F634" s="2" t="inlineStr"><is><t>esmolol</t></is></c><c r="G634" s="2" t="inlineStr"><is><t>sukcynylocholina</t></is></c><c r="H634" s="2" t="inlineStr"><is><t>adenozyna</t></is></c><c r="I634" s="2" t="inlineStr" /><c r="J634" s="2" t="inlineStr" /><c r="K634" s="2" t="inlineStr"><is><t>diazepam</t></is></c><c r="L634" s="2" t="inlineStr" /><c r="M634" s="2" t="inlineStr" /><c r="N634" s="2" t="inlineStr" /><c r="O634" s="2" t="inlineStr" /><c r="P634" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q634" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="635"><c r="A635" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B635" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C635" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D635" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E635" s="2" t="inlineStr"><is><t>Wskaż poprawną kombinację terapeutyczną w leczeniu zapalnego kaszlu w infekcji oskrzeli:</t></is></c><c r="F635" s="2" t="inlineStr"><is><t>ambroksol w nebulizacji + acetylocysteina doustnie</t></is></c><c r="G635" s="2" t="inlineStr" /><c r="H635" s="2" t="inlineStr" /><c r="I635" s="2" t="inlineStr" /><c r="J635" s="2" t="inlineStr" /><c r="K635" s="2" t="inlineStr"><is><t>wazycyna doustnie + 10% NaCl w nebulizacji</t></is></c><c r="L635" s="2" t="inlineStr"><is><t>sulfagwajakol + kodeina w doustnym preparacie złożonym</t></is></c><c r="M635" s="2" t="inlineStr"><is><t>dornaza alfa w inhalacjach + erdosteina doustnie</t></is></c><c r="N635" s="2" t="inlineStr" /><c r="O635" s="2" t="inlineStr" /><c r="P635" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q635" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="636"><c r="A636" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B636" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C636" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D636" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E636" s="2" t="inlineStr"><is><t>W napadzie duszności u osoby z cechami skurczu oskrzeli (cichy szmer pęcherzykowy, głośne świsty, wydłużona faza wydechu) w celu przerwania napadu zasadne jest zastosowanie:</t></is></c><c r="F636" s="2" t="inlineStr"><is><t>salbutamolu wziewnie w nebulizacji</t></is></c><c r="G636" s="2" t="inlineStr"><is><t>bromku ipratropium wziewnie w nebulizacji</t></is></c><c r="H636" s="2" t="inlineStr" /><c r="I636" s="2" t="inlineStr" /><c r="J636" s="2" t="inlineStr" /><c r="K636" s="2" t="inlineStr"><is><t>triazotanu glicerolu w aerozolu na błonę śluzową jamy ustnej</t></is></c><c r="L636" s="2" t="inlineStr"><is><t>cyklezonidu wziewnie z inhalatora aerozolowego</t></is></c><c r="M636" s="2" t="inlineStr" /><c r="N636" s="2" t="inlineStr" /><c r="O636" s="2" t="inlineStr" /><c r="P636" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q636" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="637"><c r="A637" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B637" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C637" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D637" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E637" s="2" t="inlineStr"><is><t>Który lek ma w swojej grupie farmakologicznej nietypową, wyróżniającą go farmakokinetykę:</t></is></c><c r="F637" s="2" t="inlineStr"><is><t>cyklezonid</t></is></c><c r="G637" s="2" t="inlineStr"><is><t>amlodypina</t></is></c><c r="H637" s="2" t="inlineStr" /><c r="I637" s="2" t="inlineStr" /><c r="J637" s="2" t="inlineStr" /><c r="K637" s="2" t="inlineStr"><is><t>metoprolol</t></is></c><c r="L637" s="2" t="inlineStr"><is><t>iwabradyna</t></is></c><c r="M637" s="2" t="inlineStr" /><c r="N637" s="2" t="inlineStr" /><c r="O637" s="2" t="inlineStr" /><c r="P637" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q637" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="638"><c r="A638" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B638" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C638" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D638" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E638" s="2" t="inlineStr"><is><t>Lekiem stosowanym „ratunkowo” w poważnych powikłaniach polekowych jest:</t></is></c><c r="F638" s="2" t="inlineStr"><is><t>adrenalina</t></is></c><c r="G638" s="2" t="inlineStr"><is><t>półbursztynian hydrokortyzonu</t></is></c><c r="H638" s="2" t="inlineStr"><is><t>dantrolen</t></is></c><c r="I638" s="2" t="inlineStr"><is><t>acetylocysteina</t></is></c><c r="J638" s="2" t="inlineStr" /><c r="K638" s="2" t="inlineStr" /><c r="L638" s="2" t="inlineStr" /><c r="M638" s="2" t="inlineStr" /><c r="N638" s="2" t="inlineStr" /><c r="O638" s="2" t="inlineStr" /><c r="P638" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q638" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="639"><c r="A639" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B639" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C639" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D639" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E639" s="2" t="inlineStr"><is><t>Do leków zmniejszających obciążenie wstępne należy:</t></is></c><c r="F639" s="2" t="inlineStr"><is><t>diazotan izosorbidu</t></is></c><c r="G639" s="2" t="inlineStr"><is><t>furosemid</t></is></c><c r="H639" s="2" t="inlineStr" /><c r="I639" s="2" t="inlineStr" /><c r="J639" s="2" t="inlineStr" /><c r="K639" s="2" t="inlineStr"><is><t>diosmina</t></is></c><c r="L639" s="2" t="inlineStr"><is><t>pentoksyfilina</t></is></c><c r="M639" s="2" t="inlineStr" /><c r="N639" s="2" t="inlineStr" /><c r="O639" s="2" t="inlineStr" /><c r="P639" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q639" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="640"><c r="A640" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B640" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C640" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D640" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E640" s="2" t="inlineStr"><is><t>Pacjentka z zespołem depresyjnym stosująca tryptany ma zwiększone ryzyko zespołu serotoninowego po włączeniu:</t></is></c><c r="F640" s="2" t="inlineStr"><is><t>fluoksetyny</t></is></c><c r="G640" s="2" t="inlineStr"><is><t>wenlafaksyny</t></is></c><c r="H640" s="2" t="inlineStr"><is><t>klomipraminy</t></is></c><c r="I640" s="2" t="inlineStr"><is><t>duloksetyny</t></is></c><c r="J640" s="2" t="inlineStr" /><c r="K640" s="2" t="inlineStr" /><c r="L640" s="2" t="inlineStr" /><c r="M640" s="2" t="inlineStr" /><c r="N640" s="2" t="inlineStr" /><c r="O640" s="2" t="inlineStr" /><c r="P640" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q640" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="641"><c r="A641" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B641" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C641" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D641" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E641" s="2" t="inlineStr"><is><t>Jeśli splątany i agresywny pacjent odmawia przyjmowania leków doustnie to po zastosowaniu krótkotrwałego unieruchomienia kończyn można mu podać dożylnie lek uspokajający, którym jest:</t></is></c><c r="F641" s="2" t="inlineStr"><is><t>midazolam</t></is></c><c r="G641" s="2" t="inlineStr" /><c r="H641" s="2" t="inlineStr" /><c r="I641" s="2" t="inlineStr" /><c r="J641" s="2" t="inlineStr" /><c r="K641" s="2" t="inlineStr"><is><t>piracetam</t></is></c><c r="L641" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="M641" s="2" t="inlineStr"><is><t>rysperydon</t></is></c><c r="N641" s="2" t="inlineStr" /><c r="O641" s="2" t="inlineStr" /><c r="P641" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q641" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="642"><c r="A642" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B642" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C642" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D642" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E642" s="2" t="inlineStr"><is><t>Jako lek normotymiczny w chorobie afektywnej dwubiegunowej można zastosować:</t></is></c><c r="F642" s="2" t="inlineStr"><is><t>lamotryginę</t></is></c><c r="G642" s="2" t="inlineStr"><is><t>olanzapinę</t></is></c><c r="H642" s="2" t="inlineStr" /><c r="I642" s="2" t="inlineStr" /><c r="J642" s="2" t="inlineStr" /><c r="K642" s="2" t="inlineStr"><is><t>fluoksetynę</t></is></c><c r="L642" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="M642" s="2" t="inlineStr" /><c r="N642" s="2" t="inlineStr" /><c r="O642" s="2" t="inlineStr" /><c r="P642" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q642" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="643"><c r="A643" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B643" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C643" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D643" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E643" s="2" t="inlineStr"><is><t>Który lek jest stosowany jedynie we wskazaniu wymienionym przy tym leku?</t></is></c><c r="F643" s="2" t="inlineStr"><is><t>netupitant – terapia wspomagająca stosowanie wysoce emetogennej chemioterapii przeciwnowotworowej</t></is></c><c r="G643" s="2" t="inlineStr"><is><t>memantyna – choroba Alzheimera</t></is></c><c r="H643" s="2" t="inlineStr" /><c r="I643" s="2" t="inlineStr" /><c r="J643" s="2" t="inlineStr" /><c r="K643" s="2" t="inlineStr"><is><t>karbamazepina – padaczka</t></is></c><c r="L643" s="2" t="inlineStr"><is><t>pregabalina – polineuropatia cukrzycowa</t></is></c><c r="M643" s="2" t="inlineStr" /><c r="N643" s="2" t="inlineStr" /><c r="O643" s="2" t="inlineStr" /><c r="P643" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q643" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="644"><c r="A644" s="2" t="inlineStr"><is><t>ZNIECZULENIA OGÓLNE</t></is></c><c r="B644" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C644" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D644" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E644" s="2" t="inlineStr"><is><t>Idealny lek znieczulenia ogólnego:</t></is></c><c r="F644" s="2" t="inlineStr"><is><t>jest skuteczny we wszystkich grupach pacjentów</t></is></c><c r="G644" s="2" t="inlineStr"><is><t>działa przeciwbólowo</t></is></c><c r="H644" s="2" t="inlineStr"><is><t>jest bezpieczny dla wszystkich grup pacjentów</t></is></c><c r="I644" s="2" t="inlineStr"><is><t>jest tani</t></is></c><c r="J644" s="2" t="inlineStr" /><c r="K644" s="2" t="inlineStr" /><c r="L644" s="2" t="inlineStr" /><c r="M644" s="2" t="inlineStr" /><c r="N644" s="2" t="inlineStr" /><c r="O644" s="2" t="inlineStr" /><c r="P644" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q644" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="645"><c r="A645" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B645" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C645" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D645" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E645" s="2" t="inlineStr"><is><t>Cholinolityki:</t></is></c><c r="F645" s="2" t="inlineStr"><is><t>są lekami z wyboru w polekowym zespole parkinsonowskim</t></is></c><c r="G645" s="2" t="inlineStr"><is><t>zmniejszają drżenie w chorobie Parkinsona</t></is></c><c r="H645" s="2" t="inlineStr"><is><t>nie różnią się skutecznością w chorobie Parkinsona</t></is></c><c r="I645" s="2" t="inlineStr"><is><t>można podawać w połączeniu z lewodopą</t></is></c><c r="J645" s="2" t="inlineStr" /><c r="K645" s="2" t="inlineStr" /><c r="L645" s="2" t="inlineStr" /><c r="M645" s="2" t="inlineStr" /><c r="N645" s="2" t="inlineStr" /><c r="O645" s="2" t="inlineStr" /><c r="P645" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q645" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="646"><c r="A646" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B646" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C646" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D646" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E646" s="2" t="inlineStr"><is><t>Cholinolityki</t></is></c><c r="F646" s="2" t="inlineStr"><is><t>są lekami z wyboru w polekowym zespole parkinsonowskim</t></is></c><c r="G646" s="2" t="inlineStr"><is><t>nie ma istotnych różnic w skuteczności leków tej grupy stosowanych w chorobie Parkinsona</t></is></c><c r="H646" s="2" t="inlineStr"><is><t>zmniejszają drżenie w chorobie Parkinsona</t></is></c><c r="I646" s="2" t="inlineStr"><is><t>można podawać w połączeniu z lewodopą</t></is></c><c r="J646" s="2" t="inlineStr" /><c r="K646" s="2" t="inlineStr" /><c r="L646" s="2" t="inlineStr" /><c r="M646" s="2" t="inlineStr" /><c r="N646" s="2" t="inlineStr" /><c r="O646" s="2" t="inlineStr" /><c r="P646" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q646" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="647"><c r="A647" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B647" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C647" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D647" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E647" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie mykotoksyny z zagrożeniem poekspozycyjnym:</t></is></c><c r="F647" s="2" t="inlineStr"><is><t>zearaleon – działanie estrogenne i anaboliczne</t></is></c><c r="G647" s="2" t="inlineStr"><is><t>aflatoksyna – ryzyko nowotworów wątroby</t></is></c><c r="H647" s="2" t="inlineStr" /><c r="I647" s="2" t="inlineStr" /><c r="J647" s="2" t="inlineStr" /><c r="K647" s="2" t="inlineStr"><is><t>patulina – ryzyko nowotworów dróg moczowych</t></is></c><c r="L647" s="2" t="inlineStr"><is><t>ochratoksyna – silne działanie alergizujące</t></is></c><c r="M647" s="2" t="inlineStr" /><c r="N647" s="2" t="inlineStr" /><c r="O647" s="2" t="inlineStr" /><c r="P647" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q647" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="648"><c r="A648" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B648" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C648" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D648" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E648" s="2" t="inlineStr"><is><t>Leki przeciwhistaminowe drugiej generacji blokujące receptor H1 w odróżnieniu od leków pierwszej generacji:</t></is></c><c r="F648" s="2" t="inlineStr"><is><t>są w znaczącym stopniu pozbawione działania sedatywnego</t></is></c><c r="G648" s="2" t="inlineStr" /><c r="H648" s="2" t="inlineStr" /><c r="I648" s="2" t="inlineStr" /><c r="J648" s="2" t="inlineStr" /><c r="K648" s="2" t="inlineStr"><is><t>mają istotne działanie cholinolityczne</t></is></c><c r="L648" s="2" t="inlineStr"><is><t>mogą być stosowane w postaci wstrzyknięć</t></is></c><c r="M648" s="2" t="inlineStr"><is><t>są skuteczne w profilaktyce choroby lokomocyjnej</t></is></c><c r="N648" s="2" t="inlineStr" /><c r="O648" s="2" t="inlineStr" /><c r="P648" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q648" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="649"><c r="A649" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B649" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C649" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D649" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E649" s="2" t="inlineStr"><is><t>W leczeniu ostrego napadu dny moczanowej stosuje się:</t></is></c><c r="F649" s="2" t="inlineStr"><is><t>kolchicynę</t></is></c><c r="G649" s="2" t="inlineStr"><is><t>glikokortykosteroidy</t></is></c><c r="H649" s="2" t="inlineStr"><is><t>niesteroidowe leki przeciwzapalne</t></is></c><c r="I649" s="2" t="inlineStr" /><c r="J649" s="2" t="inlineStr" /><c r="K649" s="2" t="inlineStr"><is><t>allopurynol</t></is></c><c r="L649" s="2" t="inlineStr" /><c r="M649" s="2" t="inlineStr" /><c r="N649" s="2" t="inlineStr" /><c r="O649" s="2" t="inlineStr" /><c r="P649" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q649" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="650"><c r="A650" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B650" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C650" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D650" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E650" s="2" t="inlineStr"><is><t>Diuretyki pętlowe:</t></is></c><c r="F650" s="2" t="inlineStr"><is><t>zwiększają filtrację kłębuszkową też przez korzystny wpływ na syntezę prostaglandyn w nerkach</t></is></c><c r="G650" s="2" t="inlineStr"><is><t>ulegają wydzielaniu cewkowemu w kanalikach proksymalnych</t></is></c><c r="H650" s="2" t="inlineStr"><is><t>tworzą wysoki ładunek sodowy w kanaliku dalszym aktywując układ reninowo￾angiotensynowy</t></is></c><c r="I650" s="2" t="inlineStr"><is><t>zwiększają pojemność łożyska żylnego jeszcze przed wystąpieniem efektu diuretycznego</t></is></c><c r="J650" s="2" t="inlineStr" /><c r="K650" s="2" t="inlineStr" /><c r="L650" s="2" t="inlineStr" /><c r="M650" s="2" t="inlineStr" /><c r="N650" s="2" t="inlineStr" /><c r="O650" s="2" t="inlineStr" /><c r="P650" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q650" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="651"><c r="A651" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B651" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C651" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D651" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E651" s="2" t="inlineStr"><is><t>Który lek może być zastosowany u chorego z nadwrażliwością na sulfonamidy?</t></is></c><c r="F651" s="2" t="inlineStr"><is><t>torasemid</t></is></c><c r="G651" s="2" t="inlineStr"><is><t>eplerenon</t></is></c><c r="H651" s="2" t="inlineStr" /><c r="I651" s="2" t="inlineStr" /><c r="J651" s="2" t="inlineStr" /><c r="K651" s="2" t="inlineStr"><is><t>furosemid</t></is></c><c r="L651" s="2" t="inlineStr"><is><t>hydrochlorotiazyd</t></is></c><c r="M651" s="2" t="inlineStr" /><c r="N651" s="2" t="inlineStr" /><c r="O651" s="2" t="inlineStr" /><c r="P651" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q651" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="652"><c r="A652" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B652" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C652" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D652" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E652" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące metoprololu:</t></is></c><c r="F652" s="2" t="inlineStr"><is><t>ma działanie hipotensyjne związane ze zmniejszeniem aktywności reninowej osocza</t></is></c><c r="G652" s="2" t="inlineStr"><is><t>zmienia działanie układu współczulnego na poziomie ośrodkowego układu nerwowego</t></is></c><c r="H652" s="2" t="inlineStr"><is><t>jest niebezpieczny w naczynioskurczowych chorobach tętnic</t></is></c><c r="I652" s="2" t="inlineStr" /><c r="J652" s="2" t="inlineStr" /><c r="K652" s="2" t="inlineStr"><is><t>w terapii przewlekłej powoduje down-regulację receptorów beta-adrenergicznych</t></is></c><c r="L652" s="2" t="inlineStr" /><c r="M652" s="2" t="inlineStr" /><c r="N652" s="2" t="inlineStr" /><c r="O652" s="2" t="inlineStr" /><c r="P652" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q652" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="653"><c r="A653" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B653" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C653" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D653" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E653" s="2" t="inlineStr"><is><t>W filmie „Piękny umysł” Alicia, żona chorego na schizofrenię Johna Nasha, pyta go: „Czy to przez lek?”, a on odpowiada: „Tak”. O którym działaniu niepożądanym chloropromazyny mogli rozmawiać?</t></is></c><c r="F653" s="2" t="inlineStr"><is><t>zmniejszeniu libido</t></is></c><c r="G653" s="2" t="inlineStr" /><c r="H653" s="2" t="inlineStr" /><c r="I653" s="2" t="inlineStr" /><c r="J653" s="2" t="inlineStr" /><c r="K653" s="2" t="inlineStr"><is><t>nadciśnieniu tętniczym</t></is></c><c r="L653" s="2" t="inlineStr"><is><t>ślinotoku</t></is></c><c r="M653" s="2" t="inlineStr"><is><t>przymusie robienia notatek na ścianach</t></is></c><c r="N653" s="2" t="inlineStr" /><c r="O653" s="2" t="inlineStr" /><c r="P653" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q653" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="654"><c r="A654" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B654" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C654" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D654" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E654" s="2" t="inlineStr"><is><t>W arcydziele „Sto lat samotności” Gabriela Garcii Marqueza wioskę Macondo nawiedza zaraza bezsenności i zapomnienia. Wskaż uzasadnioną opcję terapeutyczną do zaproponowania w leczeniu krótkotrwałej bezsenności, gdyby wydarzenia opisane przez Marqueza działy się współcześnie:</t></is></c><c r="F654" s="2" t="inlineStr"><is><t>trazodon</t></is></c><c r="G654" s="2" t="inlineStr" /><c r="H654" s="2" t="inlineStr" /><c r="I654" s="2" t="inlineStr" /><c r="J654" s="2" t="inlineStr" /><c r="K654" s="2" t="inlineStr"><is><t>triazolam</t></is></c><c r="L654" s="2" t="inlineStr"><is><t>dezimipramina</t></is></c><c r="M654" s="2" t="inlineStr"><is><t>hydroksyzyna</t></is></c><c r="N654" s="2" t="inlineStr" /><c r="O654" s="2" t="inlineStr" /><c r="P654" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q654" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="655"><c r="A655" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B655" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C655" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D655" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E655" s="2" t="inlineStr"><is><t>Amitryptylina w przeciwieństwie do wenlafaksyny:</t></is></c><c r="F655" s="2" t="inlineStr"><is><t>działa antagonistycznie wobec receptora muskarynowego (M1)</t></is></c><c r="G655" s="2" t="inlineStr" /><c r="H655" s="2" t="inlineStr" /><c r="I655" s="2" t="inlineStr" /><c r="J655" s="2" t="inlineStr" /><c r="K655" s="2" t="inlineStr"><is><t>jest skuteczna w bólach neuropatycznych</t></is></c><c r="L655" s="2" t="inlineStr"><is><t>zmniejsza wychwyt zwrotny noradrenaliny i serotoniny</t></is></c><c r="M655" s="2" t="inlineStr"><is><t>jest agonistą receptora dopaminowego (D2)</t></is></c><c r="N655" s="2" t="inlineStr" /><c r="O655" s="2" t="inlineStr" /><c r="P655" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q655" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="656"><c r="A656" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B656" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C656" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D656" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E656" s="2" t="inlineStr"><is><t>Za reakcję paradoksalną uznasz:</t></is></c><c r="F656" s="2" t="inlineStr"><is><t>zwiększenie ciśnienia krwi po metoprololu</t></is></c><c r="G656" s="2" t="inlineStr"><is><t>pobudzenie i agresję po alprazolamie</t></is></c><c r="H656" s="2" t="inlineStr" /><c r="I656" s="2" t="inlineStr" /><c r="J656" s="2" t="inlineStr" /><c r="K656" s="2" t="inlineStr"><is><t>drgawki po amitryptylinie</t></is></c><c r="L656" s="2" t="inlineStr"><is><t>zaburzenia koordynacji ruchowej po zopiklonie</t></is></c><c r="M656" s="2" t="inlineStr" /><c r="N656" s="2" t="inlineStr" /><c r="O656" s="2" t="inlineStr" /><c r="P656" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q656" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="657"><c r="A657" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B657" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C657" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D657" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E657" s="2" t="inlineStr"><is><t>Za reakcję paradoksalną uznasz:</t></is></c><c r="F657" s="2" t="inlineStr"><is><t>agresję po lorazepamie</t></is></c><c r="G657" s="2" t="inlineStr" /><c r="H657" s="2" t="inlineStr" /><c r="I657" s="2" t="inlineStr" /><c r="J657" s="2" t="inlineStr" /><c r="K657" s="2" t="inlineStr"><is><t>drgawki po amitryptylinie</t></is></c><c r="L657" s="2" t="inlineStr"><is><t>niepamięć następczą po zopiklonie</t></is></c><c r="M657" s="2" t="inlineStr"><is><t>jadłowstręt po fluoksetynie</t></is></c><c r="N657" s="2" t="inlineStr" /><c r="O657" s="2" t="inlineStr" /><c r="P657" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q657" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="658"><c r="A658" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B658" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C658" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D658" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E658" s="2" t="inlineStr"><is><t>Który lek ma zastosowanie w wymiotach związanych z chemioterapią przeciwnowotworową?</t></is></c><c r="F658" s="2" t="inlineStr"><is><t>deksametazon</t></is></c><c r="G658" s="2" t="inlineStr"><is><t>palonosetron</t></is></c><c r="H658" s="2" t="inlineStr"><is><t>aprepitant</t></is></c><c r="I658" s="2" t="inlineStr"><is><t>metoklopramid</t></is></c><c r="J658" s="2" t="inlineStr" /><c r="K658" s="2" t="inlineStr" /><c r="L658" s="2" t="inlineStr" /><c r="M658" s="2" t="inlineStr" /><c r="N658" s="2" t="inlineStr" /><c r="O658" s="2" t="inlineStr" /><c r="P658" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q658" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="659"><c r="A659" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B659" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C659" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D659" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E659" s="2" t="inlineStr"><is><t>Pacjentka od wielu lat otrzymuje perazynę, mianserynę i lorazepam. Na tej podstawie można rozpoznać (możliwe jest więcej niż jedno rozpoznanie):</t></is></c><c r="F659" s="2" t="inlineStr"><is><t>zaburzenia depresyjno-urojeniowe</t></is></c><c r="G659" s="2" t="inlineStr"><is><t>uzależnienie lekowe</t></is></c><c r="H659" s="2" t="inlineStr" /><c r="I659" s="2" t="inlineStr" /><c r="J659" s="2" t="inlineStr" /><c r="K659" s="2" t="inlineStr"><is><t>dwubiegunową chorobę afektywną</t></is></c><c r="L659" s="2" t="inlineStr"><is><t>fobię społeczną</t></is></c><c r="M659" s="2" t="inlineStr" /><c r="N659" s="2" t="inlineStr" /><c r="O659" s="2" t="inlineStr" /><c r="P659" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q659" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="660"><c r="A660" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B660" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C660" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D660" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E660" s="2" t="inlineStr"><is><t>Podczas stosowania kwetiapiny, bardzo popularnej w psychotycznych zaburzeniach zachowania u pacjentów oddziałów somatycznych, trzeba pamiętać, że zwiększa się ryzyko:</t></is></c><c r="F660" s="2" t="inlineStr"><is><t>hipertriglicerydemii</t></is></c><c r="G660" s="2" t="inlineStr"><is><t>zespołu pozapiramidowego</t></is></c><c r="H660" s="2" t="inlineStr"><is><t>hiperglikemii</t></is></c><c r="I660" s="2" t="inlineStr"><is><t>zakrzepowego zapalenia żył</t></is></c><c r="J660" s="2" t="inlineStr" /><c r="K660" s="2" t="inlineStr" /><c r="L660" s="2" t="inlineStr" /><c r="M660" s="2" t="inlineStr" /><c r="N660" s="2" t="inlineStr" /><c r="O660" s="2" t="inlineStr" /><c r="P660" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2018/19</t></is></c><c r="Q660" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="661"><c r="A661" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B661" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C661" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D661" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E661" s="2" t="inlineStr"><is><t>Która z poniższych informacji znajduje się w charakterystyce produktu leczniczego:</t></is></c><c r="F661" s="2" t="inlineStr"><is><t>informacja o warunkach przechowywania produktu leczniczego</t></is></c><c r="G661" s="2" t="inlineStr"><is><t>data wydania pierwszego pozwolenia na dopuszczenie do obrotu produktu leczniczego</t></is></c><c r="H661" s="2" t="inlineStr" /><c r="I661" s="2" t="inlineStr" /><c r="J661" s="2" t="inlineStr" /><c r="K661" s="2" t="inlineStr"><is><t>cena produktu leczniczego</t></is></c><c r="L661" s="2" t="inlineStr"><is><t>informacja o okresowym wstrzymaniu produktu leczniczego w obrocie</t></is></c><c r="M661" s="2" t="inlineStr" /><c r="N661" s="2" t="inlineStr" /><c r="O661" s="2" t="inlineStr" /><c r="P661" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q661" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="662"><c r="A662" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B662" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C662" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D662" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E662" s="2" t="inlineStr"><is><t>Do określenia biodostępności leku po podaniu doustnym konieczna jest znajomość:</t></is></c><c r="F662" s="2" t="inlineStr"><is><t>AUC0→t po podaniu dożylnym</t></is></c><c r="G662" s="2" t="inlineStr"><is><t>AUC0→t po podaniu doustnym</t></is></c><c r="H662" s="2" t="inlineStr" /><c r="I662" s="2" t="inlineStr" /><c r="J662" s="2" t="inlineStr" /><c r="K662" s="2" t="inlineStr"><is><t>stopnia wchłaniania ksylozy z przewodu pokarmowego</t></is></c><c r="L662" s="2" t="inlineStr"><is><t>Cmax leku po podaniu dożylnym</t></is></c><c r="M662" s="2" t="inlineStr" /><c r="N662" s="2" t="inlineStr" /><c r="O662" s="2" t="inlineStr" /><c r="P662" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q662" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="663"><c r="A663" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B663" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C663" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D663" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E663" s="2" t="inlineStr"><is><t>W stanie stacjonarnym objętość dystrybucji leku A = 6 l, a leku B = 206 l. Na podstawie tych danych można stwierdzić, że w stanie stacjonarnym lek A:</t></is></c><c r="F663" s="2" t="inlineStr"><is><t>osiąga większe stężenie we krwi niż lek B po podaniu takiej samej dawki obu leków i.v</t></is></c><c r="G663" s="2" t="inlineStr"><is><t>jest rozmieszczony nierównomiernie w przestrzeniach płynowych organizmu</t></is></c><c r="H663" s="2" t="inlineStr" /><c r="I663" s="2" t="inlineStr" /><c r="J663" s="2" t="inlineStr" /><c r="K663" s="2" t="inlineStr"><is><t>działa w kompartmencie obwodowym</t></is></c><c r="L663" s="2" t="inlineStr"><is><t>jest eliminowany zgodnie z kinetyką 0 rzędu</t></is></c><c r="M663" s="2" t="inlineStr" /><c r="N663" s="2" t="inlineStr" /><c r="O663" s="2" t="inlineStr" /><c r="P663" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q663" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="664"><c r="A664" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B664" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C664" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D664" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E664" s="2" t="inlineStr"><is><t>Która z poniższych par lek-zagrażające życiu działanie niepożądane jest prawdziwa?</t></is></c><c r="F664" s="2" t="inlineStr"><is><t>glargina – hipoglikemia</t></is></c><c r="G664" s="2" t="inlineStr" /><c r="H664" s="2" t="inlineStr" /><c r="I664" s="2" t="inlineStr" /><c r="J664" s="2" t="inlineStr" /><c r="K664" s="2" t="inlineStr"><is><t>metformina - zapalenie trzustki</t></is></c><c r="L664" s="2" t="inlineStr"><is><t>liraglutyd – kwasica ketonowa</t></is></c><c r="M664" s="2" t="inlineStr"><is><t>empagliflozyna – niewydolność serca</t></is></c><c r="N664" s="2" t="inlineStr" /><c r="O664" s="2" t="inlineStr" /><c r="P664" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q664" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="665"><c r="A665" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B665" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C665" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D665" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E665" s="2" t="inlineStr"><is><t>W celu obniżenia glikemii przed posiłkiem można podać:</t></is></c><c r="F665" s="2" t="inlineStr"><is><t>glulizynę</t></is></c><c r="G665" s="2" t="inlineStr" /><c r="H665" s="2" t="inlineStr" /><c r="I665" s="2" t="inlineStr" /><c r="J665" s="2" t="inlineStr" /><c r="K665" s="2" t="inlineStr"><is><t>degludec</t></is></c><c r="L665" s="2" t="inlineStr"><is><t>detemir</t></is></c><c r="M665" s="2" t="inlineStr"><is><t>glarginę</t></is></c><c r="N665" s="2" t="inlineStr" /><c r="O665" s="2" t="inlineStr" /><c r="P665" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q665" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="666"><c r="A666" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B666" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C666" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D666" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E666" s="2" t="inlineStr"><is><t>W leczeniu hiperprolaktynemii (prolaktynoma to najczęstszy typ gruczolaka przysadki) uzasadnione jest zastosowanie:</t></is></c><c r="F666" s="2" t="inlineStr"><is><t>bromokryptyny</t></is></c><c r="G666" s="2" t="inlineStr" /><c r="H666" s="2" t="inlineStr" /><c r="I666" s="2" t="inlineStr" /><c r="J666" s="2" t="inlineStr" /><c r="K666" s="2" t="inlineStr"><is><t>ketokonazolu</t></is></c><c r="L666" s="2" t="inlineStr"><is><t>eplerenonu</t></is></c><c r="M666" s="2" t="inlineStr"><is><t>klomifenu</t></is></c><c r="N666" s="2" t="inlineStr" /><c r="O666" s="2" t="inlineStr" /><c r="P666" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q666" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="667"><c r="A667" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B667" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C667" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D667" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E667" s="2" t="inlineStr"><is><t>Odtwórczy (generyczny) produkt leczniczy to produkt leczniczy :</t></is></c><c r="F667" s="2" t="inlineStr"><is><t>zawierający tę samą substancję aktywną co produkt oryginalny (innowacyjny)</t></is></c><c r="G667" s="2" t="inlineStr"><is><t>biorównoważny z produktem oryginalnym (innowacyjnym)</t></is></c><c r="H667" s="2" t="inlineStr" /><c r="I667" s="2" t="inlineStr" /><c r="J667" s="2" t="inlineStr" /><c r="K667" s="2" t="inlineStr"><is><t>mający ten sam skład co produkt oryginalny (innowacyjny)</t></is></c><c r="L667" s="2" t="inlineStr"><is><t>zarejestrowany także w innych wskazaniach niż produkt oryginalny (innowacyjny)</t></is></c><c r="M667" s="2" t="inlineStr" /><c r="N667" s="2" t="inlineStr" /><c r="O667" s="2" t="inlineStr" /><c r="P667" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q667" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="668"><c r="A668" s="2" t="inlineStr"><is><t>ANTYKONCEPCJA</t></is></c><c r="B668" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C668" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D668" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E668" s="2" t="inlineStr"><is><t>„Lekiem” o nieudokumentowanej skuteczności (de facto bezwartościowym) jest:</t></is></c><c r="F668" s="2" t="inlineStr"><is><t>beta-glukan</t></is></c><c r="G668" s="2" t="inlineStr" /><c r="H668" s="2" t="inlineStr" /><c r="I668" s="2" t="inlineStr" /><c r="J668" s="2" t="inlineStr" /><c r="K668" s="2" t="inlineStr"><is><t>drospirenon</t></is></c><c r="L668" s="2" t="inlineStr"><is><t>metamizol</t></is></c><c r="M668" s="2" t="inlineStr"><is><t>aprotynina</t></is></c><c r="N668" s="2" t="inlineStr" /><c r="O668" s="2" t="inlineStr" /><c r="P668" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q668" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="669"><c r="A669" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B669" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C669" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D669" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E669" s="2" t="inlineStr"><is><t>U chorych obciążonych dodatnią historią krwawienia z wrzodów żołądka w przypadku planowanego przewlekłego leczenia NLPZ należy:</t></is></c><c r="F669" s="2" t="inlineStr"><is><t>przepisać dodatkowo pantoprazol</t></is></c><c r="G669" s="2" t="inlineStr"><is><t>wykonać test na nosicielstwo Helicobacter pylori w celu ewentualnej eradykacji</t></is></c><c r="H669" s="2" t="inlineStr"><is><t>przy braku innych przeciwwskazań wybrać lek z grupy koksybów</t></is></c><c r="I669" s="2" t="inlineStr" /><c r="J669" s="2" t="inlineStr" /><c r="K669" s="2" t="inlineStr"><is><t>bezwzględnie odstąpić od terapii klasycznymi (nieselektywnymi) NLPZ</t></is></c><c r="L669" s="2" t="inlineStr" /><c r="M669" s="2" t="inlineStr" /><c r="N669" s="2" t="inlineStr" /><c r="O669" s="2" t="inlineStr" /><c r="P669" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q669" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="670"><c r="A670" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B670" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C670" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D670" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E670" s="2" t="inlineStr"><is><t>Do leków zwiększających niekorzystny wpływ NLPZ na przewód pokarmowy zaliczysz:</t></is></c><c r="F670" s="2" t="inlineStr"><is><t>warfarynę</t></is></c><c r="G670" s="2" t="inlineStr"><is><t>prednizon</t></is></c><c r="H670" s="2" t="inlineStr" /><c r="I670" s="2" t="inlineStr" /><c r="J670" s="2" t="inlineStr" /><c r="K670" s="2" t="inlineStr"><is><t>etamsylat</t></is></c><c r="L670" s="2" t="inlineStr"><is><t>sukralfat</t></is></c><c r="M670" s="2" t="inlineStr" /><c r="N670" s="2" t="inlineStr" /><c r="O670" s="2" t="inlineStr" /><c r="P670" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q670" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="671"><c r="A671" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B671" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C671" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D671" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E671" s="2" t="inlineStr"><is><t>Czynniki stymulujące erytropoezę:</t></is></c><c r="F671" s="2" t="inlineStr"><is><t>powodują przemijające objawy grypopodobne</t></is></c><c r="G671" s="2" t="inlineStr"><is><t>zwiększają ciśnienie tętnicze krwi</t></is></c><c r="H671" s="2" t="inlineStr"><is><t>rzadko powodują wybiórczą aplazję czerwonokrwinkową</t></is></c><c r="I671" s="2" t="inlineStr"><is><t>predysponują do powikłań zakrzepowych</t></is></c><c r="J671" s="2" t="inlineStr" /><c r="K671" s="2" t="inlineStr" /><c r="L671" s="2" t="inlineStr" /><c r="M671" s="2" t="inlineStr" /><c r="N671" s="2" t="inlineStr" /><c r="O671" s="2" t="inlineStr" /><c r="P671" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q671" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="672"><c r="A672" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B672" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C672" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D672" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E672" s="2" t="inlineStr"><is><t>Którego/których leków może dotyczyć poniższy opis: pośrednio hamuje aktywność czynnika krzepnięcia Xa:</t></is></c><c r="F672" s="2" t="inlineStr"><is><t>enoksaparyna</t></is></c><c r="G672" s="2" t="inlineStr"><is><t>fondaparyna</t></is></c><c r="H672" s="2" t="inlineStr" /><c r="I672" s="2" t="inlineStr" /><c r="J672" s="2" t="inlineStr" /><c r="K672" s="2" t="inlineStr"><is><t>edoksaban</t></is></c><c r="L672" s="2" t="inlineStr"><is><t>biwalirudyna</t></is></c><c r="M672" s="2" t="inlineStr" /><c r="N672" s="2" t="inlineStr" /><c r="O672" s="2" t="inlineStr" /><c r="P672" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q672" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="673"><c r="A673" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B673" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C673" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D673" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E673" s="2" t="inlineStr"><is><t>Którego/których leków może dotyczyć poniższy opis: prolek, nieodwracalnie blokujący receptory P2Y12:</t></is></c><c r="F673" s="2" t="inlineStr"><is><t>prasugrel</t></is></c><c r="G673" s="2" t="inlineStr" /><c r="H673" s="2" t="inlineStr" /><c r="I673" s="2" t="inlineStr" /><c r="J673" s="2" t="inlineStr" /><c r="K673" s="2" t="inlineStr"><is><t>dipyrydamol</t></is></c><c r="L673" s="2" t="inlineStr"><is><t>tikagrelor</t></is></c><c r="M673" s="2" t="inlineStr"><is><t>cilostazol</t></is></c><c r="N673" s="2" t="inlineStr" /><c r="O673" s="2" t="inlineStr" /><c r="P673" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q673" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="674"><c r="A674" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B674" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C674" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D674" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E674" s="2" t="inlineStr"><is><t>Wadą heparyny niefrakcjonowanej w porównaniu z drobnocząsteczkowymi jest:</t></is></c><c r="F674" s="2" t="inlineStr"><is><t>wymaga monitorowania APTT</t></is></c><c r="G674" s="2" t="inlineStr"><is><t>silniej indukuje powstawanie przeciwciał p-kompleksowi PF4 z heparyną</t></is></c><c r="H674" s="2" t="inlineStr" /><c r="I674" s="2" t="inlineStr" /><c r="J674" s="2" t="inlineStr" /><c r="K674" s="2" t="inlineStr"><is><t>jest mniej bezpieczna w niewydolności nerek</t></is></c><c r="L674" s="2" t="inlineStr"><is><t>trudniej jest zneutralizować jej działanie siarczanem protaminy</t></is></c><c r="M674" s="2" t="inlineStr" /><c r="N674" s="2" t="inlineStr" /><c r="O674" s="2" t="inlineStr" /><c r="P674" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q674" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="675"><c r="A675" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B675" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C675" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D675" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E675" s="2" t="inlineStr"><is><t>Rosuwastatyna zmniejsza:</t></is></c><c r="F675" s="2" t="inlineStr"><is><t>syntezę cholesterolu w wątrobie poprzez konkurencyjne hamowanie aktywności reduktazy HMG-CoA</t></is></c><c r="G675" s="2" t="inlineStr"><is><t>stężenie cholesterolu LDL</t></is></c><c r="H675" s="2" t="inlineStr"><is><t>stężenie lipoprotein zawierających apoB, w tym cząsteczek o dużej zawartości triglicerydów</t></is></c><c r="I675" s="2" t="inlineStr" /><c r="J675" s="2" t="inlineStr" /><c r="K675" s="2" t="inlineStr"><is><t>ekspresję receptorów dla LDL na powierzchni hepatocytów</t></is></c><c r="L675" s="2" t="inlineStr" /><c r="M675" s="2" t="inlineStr" /><c r="N675" s="2" t="inlineStr" /><c r="O675" s="2" t="inlineStr" /><c r="P675" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q675" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="676"><c r="A676" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B676" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C676" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D676" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E676" s="2" t="inlineStr"><is><t>W prawidłowo prowadzonej profilaktyce sercowo-naczyniowej (czyli profilaktyce miażdżycy) należy osiągnąć następujące cele terapeutyczne:</t></is></c><c r="F676" s="2" t="inlineStr"><is><t>w grupie osób dużego ryzyka zmniejszenie stężenia cholesterolu LDL w surowicy poniżej 70 mg/dl</t></is></c><c r="G676" s="2" t="inlineStr" /><c r="H676" s="2" t="inlineStr" /><c r="I676" s="2" t="inlineStr" /><c r="J676" s="2" t="inlineStr" /><c r="K676" s="2" t="inlineStr"><is><t>obniżenie stężenia trójglicerydów w surowicy poniżej 115 mg/dl</t></is></c><c r="L676" s="2" t="inlineStr"><is><t>zmniejszenie masy ciała do wartości BMI poniżej 27 kg/m2</t></is></c><c r="M676" s="2" t="inlineStr"><is><t>podwyższenie stężenia cholesterolu HDL w surowicy u mężczyzn powyżej 30 mg/dl</t></is></c><c r="N676" s="2" t="inlineStr" /><c r="O676" s="2" t="inlineStr" /><c r="P676" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q676" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="677"><c r="A677" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B677" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C677" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D677" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E677" s="2" t="inlineStr"><is><t>W leczeniu immunosupresyjnym jest/są stosowana/-e:</t></is></c><c r="F677" s="2" t="inlineStr"><is><t>przeciwciała przeciwtymocytarne królicze</t></is></c><c r="G677" s="2" t="inlineStr" /><c r="H677" s="2" t="inlineStr" /><c r="I677" s="2" t="inlineStr" /><c r="J677" s="2" t="inlineStr" /><c r="K677" s="2" t="inlineStr"><is><t>cyklofilina</t></is></c><c r="L677" s="2" t="inlineStr"><is><t>inozyna</t></is></c><c r="M677" s="2" t="inlineStr"><is><t>kolchicyna</t></is></c><c r="N677" s="2" t="inlineStr" /><c r="O677" s="2" t="inlineStr" /><c r="P677" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q677" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="678"><c r="A678" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B678" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C678" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D678" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E678" s="2" t="inlineStr"><is><t>Lekiem terapii genowej jest:</t></is></c><c r="F678" s="2" t="inlineStr"><is><t>fomiwirsen</t></is></c><c r="G678" s="2" t="inlineStr"><is><t>mipomersen</t></is></c><c r="H678" s="2" t="inlineStr"><is><t>typarwowek alipogenu</t></is></c><c r="I678" s="2" t="inlineStr" /><c r="J678" s="2" t="inlineStr" /><c r="K678" s="2" t="inlineStr"><is><t>OKT3</t></is></c><c r="L678" s="2" t="inlineStr" /><c r="M678" s="2" t="inlineStr" /><c r="N678" s="2" t="inlineStr" /><c r="O678" s="2" t="inlineStr" /><c r="P678" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q678" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="679"><c r="A679" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B679" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C679" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D679" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E679" s="2" t="inlineStr"><is><t>Długotrwałe stosowanie pantoprazolu może być przyczyną:</t></is></c><c r="F679" s="2" t="inlineStr"><is><t>zakażeń dolnego odcinka układu oddechowego</t></is></c><c r="G679" s="2" t="inlineStr"><is><t>zwyrodnienia tylnosznurowego z powodu zmniejszonego wchłaniania witaminy B12</t></is></c><c r="H679" s="2" t="inlineStr"><is><t>osteoporozy</t></is></c><c r="I679" s="2" t="inlineStr"><is><t>zakażeń przewodu pokarmowego</t></is></c><c r="J679" s="2" t="inlineStr" /><c r="K679" s="2" t="inlineStr" /><c r="L679" s="2" t="inlineStr" /><c r="M679" s="2" t="inlineStr" /><c r="N679" s="2" t="inlineStr" /><c r="O679" s="2" t="inlineStr" /><c r="P679" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q679" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="680"><c r="A680" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B680" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C680" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D680" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E680" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące inhibitorów pompy protonowej (IPP):</t></is></c><c r="F680" s="2" t="inlineStr"><is><t>są lekami prekursorowymi</t></is></c><c r="G680" s="2" t="inlineStr"><is><t>aktywność osiągają w komórkach okładzinowych w fazie czynnej=wydzielniczej</t></is></c><c r="H680" s="2" t="inlineStr"><is><t>powodują nieodwracalne zablokowanie pompy protonowej</t></is></c><c r="I680" s="2" t="inlineStr"><is><t>w różnym stopniu hamują izoenzymy CYP (CYP2C19 i CYP3A4)</t></is></c><c r="J680" s="2" t="inlineStr" /><c r="K680" s="2" t="inlineStr" /><c r="L680" s="2" t="inlineStr" /><c r="M680" s="2" t="inlineStr" /><c r="N680" s="2" t="inlineStr" /><c r="O680" s="2" t="inlineStr" /><c r="P680" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q680" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="681"><c r="A681" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B681" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C681" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D681" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E681" s="2" t="inlineStr"><is><t>W leczeniu zaparć będących działaniem niepożądanym agonistów receptorów opioidowych zastosowanie ma:</t></is></c><c r="F681" s="2" t="inlineStr"><is><t>alwimopan</t></is></c><c r="G681" s="2" t="inlineStr"><is><t>metylnaltrekson</t></is></c><c r="H681" s="2" t="inlineStr" /><c r="I681" s="2" t="inlineStr" /><c r="J681" s="2" t="inlineStr" /><c r="K681" s="2" t="inlineStr"><is><t>papaweryna</t></is></c><c r="L681" s="2" t="inlineStr"><is><t>metadon</t></is></c><c r="M681" s="2" t="inlineStr" /><c r="N681" s="2" t="inlineStr" /><c r="O681" s="2" t="inlineStr" /><c r="P681" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q681" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="682"><c r="A682" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B682" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C682" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D682" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E682" s="2" t="inlineStr"><is><t>Wybierz stwierdzenie opisujące 20% roztwór albumin:</t></is></c><c r="F682" s="2" t="inlineStr"><is><t>powoduje ponad 100% przyrost objętości osocza</t></is></c><c r="G682" s="2" t="inlineStr"><is><t>działa objętościowo do 6 h</t></is></c><c r="H682" s="2" t="inlineStr" /><c r="I682" s="2" t="inlineStr" /><c r="J682" s="2" t="inlineStr" /><c r="K682" s="2" t="inlineStr"><is><t>może spowodować uszkodzenie nerek</t></is></c><c r="L682" s="2" t="inlineStr"><is><t>ma istotny wpływ na krzepnięcie krwi</t></is></c><c r="M682" s="2" t="inlineStr" /><c r="N682" s="2" t="inlineStr" /><c r="O682" s="2" t="inlineStr" /><c r="P682" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q682" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="683"><c r="A683" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B683" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C683" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D683" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E683" s="2" t="inlineStr"><is><t>Lekiem genotoksycznym jest:</t></is></c><c r="F683" s="2" t="inlineStr"><is><t>cyklofosfamid</t></is></c><c r="G683" s="2" t="inlineStr"><is><t>cisplatyna</t></is></c><c r="H683" s="2" t="inlineStr"><is><t>doksorubicyna</t></is></c><c r="I683" s="2" t="inlineStr"><is><t>irinotekan</t></is></c><c r="J683" s="2" t="inlineStr" /><c r="K683" s="2" t="inlineStr" /><c r="L683" s="2" t="inlineStr" /><c r="M683" s="2" t="inlineStr" /><c r="N683" s="2" t="inlineStr" /><c r="O683" s="2" t="inlineStr" /><c r="P683" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q683" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="684"><c r="A684" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B684" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C684" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D684" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E684" s="2" t="inlineStr"><is><t>Lekiem genotoksycznym jest:</t></is></c><c r="F684" s="2" t="inlineStr"><is><t>busulfan</t></is></c><c r="G684" s="2" t="inlineStr"><is><t>mitomycyna</t></is></c><c r="H684" s="2" t="inlineStr"><is><t>daktynomycyna</t></is></c><c r="I684" s="2" t="inlineStr"><is><t>etopozyd</t></is></c><c r="J684" s="2" t="inlineStr" /><c r="K684" s="2" t="inlineStr" /><c r="L684" s="2" t="inlineStr" /><c r="M684" s="2" t="inlineStr" /><c r="N684" s="2" t="inlineStr" /><c r="O684" s="2" t="inlineStr" /><c r="P684" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q684" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="685"><c r="A685" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B685" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C685" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D685" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E685" s="2" t="inlineStr"><is><t>Psychoaktywne substancje uzależniające aktywują:</t></is></c><c r="F685" s="2" t="inlineStr"><is><t>obszar brzuszny nakrywki</t></is></c><c r="G685" s="2" t="inlineStr"><is><t>jądro półleżące</t></is></c><c r="H685" s="2" t="inlineStr"><is><t>korę przedczołową</t></is></c><c r="I685" s="2" t="inlineStr"><is><t>mezolimbiczny układ dopaminowy</t></is></c><c r="J685" s="2" t="inlineStr" /><c r="K685" s="2" t="inlineStr" /><c r="L685" s="2" t="inlineStr" /><c r="M685" s="2" t="inlineStr" /><c r="N685" s="2" t="inlineStr" /><c r="O685" s="2" t="inlineStr" /><c r="P685" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q685" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="686"><c r="A686" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B686" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C686" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D686" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E686" s="2" t="inlineStr"><is><t>Patulina:</t></is></c><c r="F686" s="2" t="inlineStr"><is><t>ma działanie mutagenne</t></is></c><c r="G686" s="2" t="inlineStr"><is><t>w warunkach naturalnych znana jest jako substancja skażająca jabłka i powodująca brązową zgniliznę innych owoców</t></is></c><c r="H686" s="2" t="inlineStr" /><c r="I686" s="2" t="inlineStr" /><c r="J686" s="2" t="inlineStr" /><c r="K686" s="2" t="inlineStr"><is><t>powoduje endemiczną epidemię bałkańską</t></is></c><c r="L686" s="2" t="inlineStr"><is><t>jest związkiem, który zwiększa ryzyko nowotworu wątroby</t></is></c><c r="M686" s="2" t="inlineStr" /><c r="N686" s="2" t="inlineStr" /><c r="O686" s="2" t="inlineStr" /><c r="P686" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q686" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="687"><c r="A687" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B687" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C687" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D687" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E687" s="2" t="inlineStr"><is><t>Blaszki miażdżycowe w naczyniach wieńcowych stabilizuje:</t></is></c><c r="F687" s="2" t="inlineStr"><is><t>atorwastatyna</t></is></c><c r="G687" s="2" t="inlineStr" /><c r="H687" s="2" t="inlineStr" /><c r="I687" s="2" t="inlineStr" /><c r="J687" s="2" t="inlineStr" /><c r="K687" s="2" t="inlineStr"><is><t>fondaparyna</t></is></c><c r="L687" s="2" t="inlineStr"><is><t>gliklazyd</t></is></c><c r="M687" s="2" t="inlineStr"><is><t>kwasy omega 6</t></is></c><c r="N687" s="2" t="inlineStr" /><c r="O687" s="2" t="inlineStr" /><c r="P687" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 1 termin</t></is></c><c r="Q687" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="688"><c r="A688" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B688" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C688" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D688" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E688" s="2" t="inlineStr"><is><t>Wyrób medyczny to narzędzie, przyrząd, aparat, sprzęt, materiał lub inny artykuł, który może służyć do:</t></is></c><c r="F688" s="2" t="inlineStr"><is><t>regulacji poczęć</t></is></c><c r="G688" s="2" t="inlineStr"><is><t>diagnozowania chorób</t></is></c><c r="H688" s="2" t="inlineStr"><is><t>modyfikowania procesów fizjologicznych</t></is></c><c r="I688" s="2" t="inlineStr" /><c r="J688" s="2" t="inlineStr" /><c r="K688" s="2" t="inlineStr"><is><t>leczenia farmakologicznego</t></is></c><c r="L688" s="2" t="inlineStr" /><c r="M688" s="2" t="inlineStr" /><c r="N688" s="2" t="inlineStr" /><c r="O688" s="2" t="inlineStr" /><c r="P688" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q688" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="689"><c r="A689" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B689" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C689" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D689" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E689" s="2" t="inlineStr"><is><t>W stosowanej do korekty dawkowania leków skali Childa-Turcotte’a-Pugh należy uwzględnić m.in. następujący parametr:</t></is></c><c r="F689" s="2" t="inlineStr"><is><t>stężenie albumin w surowicy</t></is></c><c r="G689" s="2" t="inlineStr"><is><t>stężenie bilirubiny w surowicy</t></is></c><c r="H689" s="2" t="inlineStr"><is><t>ocenę neurologiczną (zmiany osobowości, zaburzenia nastroju, spowolnienie myślenia, zaburzenia koncentracji uwagi, drżenia grubofaliste kończyn, zaburzenia mowy)</t></is></c><c r="I689" s="2" t="inlineStr" /><c r="J689" s="2" t="inlineStr" /><c r="K689" s="2" t="inlineStr"><is><t>stężenie kreatyniny w surowicy</t></is></c><c r="L689" s="2" t="inlineStr" /><c r="M689" s="2" t="inlineStr" /><c r="N689" s="2" t="inlineStr" /><c r="O689" s="2" t="inlineStr" /><c r="P689" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q689" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="690"><c r="A690" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B690" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C690" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D690" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E690" s="2" t="inlineStr"><is><t>Lek L jest metabolizowany w wątrobie przy udziale enzymów CYP do nieaktywnych i nietoksycznych metabolitów, które następnie wydalane są przez nerki. Można się zatem spodziewać, że wystąpienie działań toksycznych tego leku jest:</t></is></c><c r="F690" s="2" t="inlineStr"><is><t>bardziej prawdopodobne u osób pijących regularnie soki owocowe, zwłaszcza grejfrutowy</t></is></c><c r="G690" s="2" t="inlineStr" /><c r="H690" s="2" t="inlineStr" /><c r="I690" s="2" t="inlineStr" /><c r="J690" s="2" t="inlineStr" /><c r="K690" s="2" t="inlineStr"><is><t>zależne głównie od stopnia wydolności nerek</t></is></c><c r="L690" s="2" t="inlineStr"><is><t>częstsze podczas stosowania induktorów enzymów CYP</t></is></c><c r="M690" s="2" t="inlineStr"><is><t>związane ze stosowaniem leków wiążących kwasy żółciowe w przewodzie pokarmowym</t></is></c><c r="N690" s="2" t="inlineStr" /><c r="O690" s="2" t="inlineStr" /><c r="P690" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q690" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="691"><c r="A691" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B691" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C691" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D691" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E691" s="2" t="inlineStr"><is><t>Glikokortykosteroidy są stosowane w:</t></is></c><c r="F691" s="2" t="inlineStr"><is><t>diagnostyce zespołu Cushinga</t></is></c><c r="G691" s="2" t="inlineStr"><is><t>leczeniu chorób alergicznych</t></is></c><c r="H691" s="2" t="inlineStr"><is><t>leczeniu ostrej niewydolności kory nadnerczy</t></is></c><c r="I691" s="2" t="inlineStr" /><c r="J691" s="2" t="inlineStr" /><c r="K691" s="2" t="inlineStr"><is><t>w kardiogennym obrzęku płuc</t></is></c><c r="L691" s="2" t="inlineStr" /><c r="M691" s="2" t="inlineStr" /><c r="N691" s="2" t="inlineStr" /><c r="O691" s="2" t="inlineStr" /><c r="P691" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q691" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="692"><c r="A692" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B692" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C692" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D692" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E692" s="2" t="inlineStr"><is><t>Przyrost masy ciała powoduje:</t></is></c><c r="F692" s="2" t="inlineStr"><is><t>gliklazyd</t></is></c><c r="G692" s="2" t="inlineStr"><is><t>insulina izofanowa</t></is></c><c r="H692" s="2" t="inlineStr" /><c r="I692" s="2" t="inlineStr" /><c r="J692" s="2" t="inlineStr" /><c r="K692" s="2" t="inlineStr"><is><t>liraglutyd</t></is></c><c r="L692" s="2" t="inlineStr"><is><t>metformina</t></is></c><c r="M692" s="2" t="inlineStr" /><c r="N692" s="2" t="inlineStr" /><c r="O692" s="2" t="inlineStr" /><c r="P692" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q692" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="693"><c r="A693" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B693" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C693" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D693" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E693" s="2" t="inlineStr"><is><t>Glikokortykosteroidy dzieli się na słabo i silnie działające na podstawie:</t></is></c><c r="F693" s="2" t="inlineStr"><is><t>testu wazokonstrykcji naczyń (zblednięcia skóry)</t></is></c><c r="G693" s="2" t="inlineStr"><is><t>działania przeciwzapalnego</t></is></c><c r="H693" s="2" t="inlineStr" /><c r="I693" s="2" t="inlineStr" /><c r="J693" s="2" t="inlineStr" /><c r="K693" s="2" t="inlineStr"><is><t>działania mineralokortykoidowego</t></is></c><c r="L693" s="2" t="inlineStr"><is><t>działania immunosupresyjnego</t></is></c><c r="M693" s="2" t="inlineStr" /><c r="N693" s="2" t="inlineStr" /><c r="O693" s="2" t="inlineStr" /><c r="P693" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q693" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="694"><c r="A694" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B694" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C694" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D694" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E694" s="2" t="inlineStr"><is><t>Za typowe polekowe działanie niepożądane podczas stosowania niesteroidowych leków przeciwzapalnych uznasz:</t></is></c><c r="F694" s="2" t="inlineStr"><is><t>krwawienie z wrzodu dwunastnicy</t></is></c><c r="G694" s="2" t="inlineStr"><is><t>skurcz oskrzeli u chorego z polipami nosa i przewlekłym zapaleniem zatok</t></is></c><c r="H694" s="2" t="inlineStr"><is><t>hipernatremię (zwiększenie stężenia sodu w surowicy)</t></is></c><c r="I694" s="2" t="inlineStr" /><c r="J694" s="2" t="inlineStr" /><c r="K694" s="2" t="inlineStr"><is><t>hipokaliemię (obniżenie stężenia potasu w surowicy)</t></is></c><c r="L694" s="2" t="inlineStr" /><c r="M694" s="2" t="inlineStr" /><c r="N694" s="2" t="inlineStr" /><c r="O694" s="2" t="inlineStr" /><c r="P694" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q694" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="695"><c r="A695" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B695" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C695" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D695" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E695" s="2" t="inlineStr"><is><t>Wskaż poprawną definicję:</t></is></c><c r="F695" s="2" t="inlineStr"><is><t>wpółczynnik (indeks) terapeutyczny leku – zakres między najmniejszą dawką skuteczną a maksymalną nie powodującą efektów toksycznych, im większy tym korzystniej</t></is></c><c r="G695" s="2" t="inlineStr"><is><t>placebo - interwencja pozbawiona bezpośredniego działania biologicznego, mająca stworzyć u pacjenta wrażenie, że otrzymuje on leczenie</t></is></c><c r="H695" s="2" t="inlineStr" /><c r="I695" s="2" t="inlineStr" /><c r="J695" s="2" t="inlineStr" /><c r="K695" s="2" t="inlineStr"><is><t>polekowe działanie niepożądane – każde niepożądane i niezamierzone zdarzenie podczas stosowania leku, bez konieczności ustalenia związku przyczynowo-skutkowego</t></is></c><c r="L695" s="2" t="inlineStr"><is><t>metaanaliza - badanie wieloośrodkowe, w którym grupa eksperymentalna porównywana jest do grupy kontrolne</t></is></c><c r="M695" s="2" t="inlineStr" /><c r="N695" s="2" t="inlineStr" /><c r="O695" s="2" t="inlineStr" /><c r="P695" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q695" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="696"><c r="A696" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B696" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C696" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D696" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E696" s="2" t="inlineStr"><is><t>Objawy przedawkowania oksykodonu to:</t></is></c><c r="F696" s="2" t="inlineStr"><is><t>zmniejszenie częstości oddechów</t></is></c><c r="G696" s="2" t="inlineStr" /><c r="H696" s="2" t="inlineStr" /><c r="I696" s="2" t="inlineStr" /><c r="J696" s="2" t="inlineStr" /><c r="K696" s="2" t="inlineStr"><is><t>rozszerzone źrenice</t></is></c><c r="L696" s="2" t="inlineStr"><is><t>pobudzenie psychoruchowe</t></is></c><c r="M696" s="2" t="inlineStr"><is><t>gorączka obwodowa</t></is></c><c r="N696" s="2" t="inlineStr" /><c r="O696" s="2" t="inlineStr" /><c r="P696" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q696" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="697"><c r="A697" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B697" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C697" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D697" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E697" s="2" t="inlineStr"><is><t>Szybki efekt przeciwbólowy można osiągnąć, stosując:</t></is></c><c r="F697" s="2" t="inlineStr"><is><t>fentanyl w postaci donosowej</t></is></c><c r="G697" s="2" t="inlineStr"><is><t>buprenorfinę w tabletkach podjęzykowych</t></is></c><c r="H697" s="2" t="inlineStr" /><c r="I697" s="2" t="inlineStr" /><c r="J697" s="2" t="inlineStr" /><c r="K697" s="2" t="inlineStr"><is><t>tramadol w systemie transdermalnym</t></is></c><c r="L697" s="2" t="inlineStr"><is><t>nalokson we wlewie dożylnym</t></is></c><c r="M697" s="2" t="inlineStr" /><c r="N697" s="2" t="inlineStr" /><c r="O697" s="2" t="inlineStr" /><c r="P697" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q697" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="698"><c r="A698" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B698" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C698" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D698" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E698" s="2" t="inlineStr"><is><t>Działanie przeciwgorączkowe ma:</t></is></c><c r="F698" s="2" t="inlineStr"><is><t>metamizol</t></is></c><c r="G698" s="2" t="inlineStr"><is><t>paracetamol</t></is></c><c r="H698" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="I698" s="2" t="inlineStr"><is><t>ibuprofen</t></is></c><c r="J698" s="2" t="inlineStr" /><c r="K698" s="2" t="inlineStr" /><c r="L698" s="2" t="inlineStr" /><c r="M698" s="2" t="inlineStr" /><c r="N698" s="2" t="inlineStr" /><c r="O698" s="2" t="inlineStr" /><c r="P698" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q698" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="699"><c r="A699" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B699" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C699" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D699" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E699" s="2" t="inlineStr"><is><t>Popularna aspiryna, czyli poprawnie kwas acetylosalicylowy:</t></is></c><c r="F699" s="2" t="inlineStr"><is><t>jest przeciwwskazana u dzieci do 12 r.ż</t></is></c><c r="G699" s="2" t="inlineStr"><is><t>konkuruje o miejsce wiązania z ibuprofenem</t></is></c><c r="H699" s="2" t="inlineStr" /><c r="I699" s="2" t="inlineStr" /><c r="J699" s="2" t="inlineStr" /><c r="K699" s="2" t="inlineStr"><is><t>działa odwracalnie antyagregacyjnie</t></is></c><c r="L699" s="2" t="inlineStr"><is><t>w małych dawkach preferencyjnie hamuje cyklooksygenazę 2</t></is></c><c r="M699" s="2" t="inlineStr" /><c r="N699" s="2" t="inlineStr" /><c r="O699" s="2" t="inlineStr" /><c r="P699" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q699" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="700"><c r="A700" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B700" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C700" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D700" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E700" s="2" t="inlineStr"><is><t>Wskaż prawidłowy zestaw lek – antidotum:</t></is></c><c r="F700" s="2" t="inlineStr"><is><t>heparyna – siarczan protaminy</t></is></c><c r="G700" s="2" t="inlineStr"><is><t>warfaryna - fitomenadion</t></is></c><c r="H700" s="2" t="inlineStr"><is><t>dabigatraban – idarucizumab</t></is></c><c r="I700" s="2" t="inlineStr"><is><t>acenokumarol – koncentrat zespołu czynników protrombiny</t></is></c><c r="J700" s="2" t="inlineStr" /><c r="K700" s="2" t="inlineStr" /><c r="L700" s="2" t="inlineStr" /><c r="M700" s="2" t="inlineStr" /><c r="N700" s="2" t="inlineStr" /><c r="O700" s="2" t="inlineStr" /><c r="P700" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q700" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="701"><c r="A701" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B701" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C701" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D701" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E701" s="2" t="inlineStr"><is><t>U pacjentów z mechaniczną zastawką serca potwierdzono skuteczność przeciwzakrzepową:</t></is></c><c r="F701" s="2" t="inlineStr"><is><t>warfaryny</t></is></c><c r="G701" s="2" t="inlineStr" /><c r="H701" s="2" t="inlineStr" /><c r="I701" s="2" t="inlineStr" /><c r="J701" s="2" t="inlineStr" /><c r="K701" s="2" t="inlineStr"><is><t>fondaparyny</t></is></c><c r="L701" s="2" t="inlineStr"><is><t>kwasu acetylosalicylowego + klopidogrelu</t></is></c><c r="M701" s="2" t="inlineStr"><is><t>dabigatranu</t></is></c><c r="N701" s="2" t="inlineStr" /><c r="O701" s="2" t="inlineStr" /><c r="P701" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q701" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="702"><c r="A702" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B702" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C702" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D702" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E702" s="2" t="inlineStr"><is><t>Hematopoetycznymi czynnikami wzrostu, które znalazły zastosowanie kliniczne są:</t></is></c><c r="F702" s="2" t="inlineStr"><is><t>darbepoetyna</t></is></c><c r="G702" s="2" t="inlineStr"><is><t>filgrastym</t></is></c><c r="H702" s="2" t="inlineStr"><is><t>lenograstym</t></is></c><c r="I702" s="2" t="inlineStr"><is><t>interleukina-11</t></is></c><c r="J702" s="2" t="inlineStr" /><c r="K702" s="2" t="inlineStr" /><c r="L702" s="2" t="inlineStr" /><c r="M702" s="2" t="inlineStr" /><c r="N702" s="2" t="inlineStr" /><c r="O702" s="2" t="inlineStr" /><c r="P702" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q702" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="703"><c r="A703" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B703" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C703" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D703" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E703" s="2" t="inlineStr"><is><t>Przeciwwskazaniem do stosowania kwasu acetylosalicylowego w dawce antyagregacyjnej jest:</t></is></c><c r="F703" s="2" t="inlineStr"><is><t>nadwrażliwość na NLPZ (niesteroidowe leki przeciwzapalne)</t></is></c><c r="G703" s="2" t="inlineStr" /><c r="H703" s="2" t="inlineStr" /><c r="I703" s="2" t="inlineStr" /><c r="J703" s="2" t="inlineStr" /><c r="K703" s="2" t="inlineStr"><is><t>choroba wrzodowa górnego odcinka przewodu pokarmowego w wywiadach</t></is></c><c r="L703" s="2" t="inlineStr"><is><t>zespół zależności alkoholowej</t></is></c><c r="M703" s="2" t="inlineStr"><is><t>niewydolność nerek</t></is></c><c r="N703" s="2" t="inlineStr" /><c r="O703" s="2" t="inlineStr" /><c r="P703" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q703" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="704"><c r="A704" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B704" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C704" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D704" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E704" s="2" t="inlineStr"><is><t>Istotnemu metabolizmowi wątrobowemu za pośrednictwem izoenzymów CYP podlega:</t></is></c><c r="F704" s="2" t="inlineStr"><is><t>atorwastatyna</t></is></c><c r="G704" s="2" t="inlineStr"><is><t>symwastatyna</t></is></c><c r="H704" s="2" t="inlineStr" /><c r="I704" s="2" t="inlineStr" /><c r="J704" s="2" t="inlineStr" /><c r="K704" s="2" t="inlineStr"><is><t>rosuwastatyna</t></is></c><c r="L704" s="2" t="inlineStr"><is><t>prawastayna</t></is></c><c r="M704" s="2" t="inlineStr" /><c r="N704" s="2" t="inlineStr" /><c r="O704" s="2" t="inlineStr" /><c r="P704" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q704" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="705"><c r="A705" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B705" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C705" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D705" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E705" s="2" t="inlineStr"><is><t>Inhibitory reduktazy HMG-CoA:</t></is></c><c r="F705" s="2" t="inlineStr"><is><t>w większym stopniu zmniejszają stężenie cholesterolu LDL w surowicy w porównaniu z fibratami</t></is></c><c r="G705" s="2" t="inlineStr" /><c r="H705" s="2" t="inlineStr" /><c r="I705" s="2" t="inlineStr" /><c r="J705" s="2" t="inlineStr" /><c r="K705" s="2" t="inlineStr"><is><t>w większym stopniu zmniejszają stężenie triglicerydów w surowicy w porównaniu z fibratami</t></is></c><c r="L705" s="2" t="inlineStr"><is><t>mają istotny wpływ na stężenie Lp(a) = lipoproteiny a</t></is></c><c r="M705" s="2" t="inlineStr"><is><t>nie powinny być łączone z inhibitorami PCSK9</t></is></c><c r="N705" s="2" t="inlineStr" /><c r="O705" s="2" t="inlineStr" /><c r="P705" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q705" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="706"><c r="A706" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B706" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C706" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D706" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E706" s="2" t="inlineStr"><is><t>Wskaż prawidłowy zestaw lek – akceptowany sposób monitorowania działania:</t></is></c><c r="F706" s="2" t="inlineStr"><is><t>rywaroksaban – aktywność czynnika anty - Xa</t></is></c><c r="G706" s="2" t="inlineStr"><is><t>dabigatran - APTT</t></is></c><c r="H706" s="2" t="inlineStr"><is><t>acenokumarol – INR</t></is></c><c r="I706" s="2" t="inlineStr" /><c r="J706" s="2" t="inlineStr" /><c r="K706" s="2" t="inlineStr"><is><t>heparyna niefrakcjonowana – czas protrombinowy</t></is></c><c r="L706" s="2" t="inlineStr" /><c r="M706" s="2" t="inlineStr" /><c r="N706" s="2" t="inlineStr" /><c r="O706" s="2" t="inlineStr" /><c r="P706" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q706" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="707"><c r="A707" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B707" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C707" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D707" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E707" s="2" t="inlineStr"><is><t>Wskaż zestaw zawierający inhibitory kalcyneuryny:</t></is></c><c r="F707" s="2" t="inlineStr"><is><t>pimekrolimus, takrolimus, cyklosporyna</t></is></c><c r="G707" s="2" t="inlineStr" /><c r="H707" s="2" t="inlineStr" /><c r="I707" s="2" t="inlineStr" /><c r="J707" s="2" t="inlineStr" /><c r="K707" s="2" t="inlineStr"><is><t>cyklosporyna, pimekrolimus, sirolimus</t></is></c><c r="L707" s="2" t="inlineStr"><is><t>ewerolimus, takrolimus, cyklosporyna</t></is></c><c r="M707" s="2" t="inlineStr"><is><t>takrolimus, azatiopryna, pimekrolimus</t></is></c><c r="N707" s="2" t="inlineStr" /><c r="O707" s="2" t="inlineStr" /><c r="P707" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q707" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="708"><c r="A708" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B708" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C708" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D708" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E708" s="2" t="inlineStr"><is><t>W Europie dopuszczono do obrotu biopodobne produkty zawierające infliksymab. Oznacza to, że:</t></is></c><c r="F708" s="2" t="inlineStr"><is><t>wykazano ich podobieństwo farmaceutyczne z produktem oryginalnym</t></is></c><c r="G708" s="2" t="inlineStr"><is><t>wykazano ich podobieństwo z produktem oryginalnym w modelach przedklinicznych</t></is></c><c r="H708" s="2" t="inlineStr"><is><t>wykazano jego podobieństwo z produktem oryginalnym w badaniach klinicznych</t></is></c><c r="I708" s="2" t="inlineStr"><is><t>wykazano ich podobną immunogenność z produktem oryginalnym w badaniach klinicznych</t></is></c><c r="J708" s="2" t="inlineStr" /><c r="K708" s="2" t="inlineStr" /><c r="L708" s="2" t="inlineStr" /><c r="M708" s="2" t="inlineStr" /><c r="N708" s="2" t="inlineStr" /><c r="O708" s="2" t="inlineStr" /><c r="P708" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q708" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="709"><c r="A709" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B709" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C709" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D709" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E709" s="2" t="inlineStr"><is><t>Rozkurczający wpływ na mięśniówkę przewodu pokarmowego wywiera:</t></is></c><c r="F709" s="2" t="inlineStr"><is><t>mebeweryna</t></is></c><c r="G709" s="2" t="inlineStr" /><c r="H709" s="2" t="inlineStr" /><c r="I709" s="2" t="inlineStr" /><c r="J709" s="2" t="inlineStr" /><c r="K709" s="2" t="inlineStr"><is><t>racekadotryl</t></is></c><c r="L709" s="2" t="inlineStr"><is><t>mesalazyna</t></is></c><c r="M709" s="2" t="inlineStr"><is><t>ryfaksymina</t></is></c><c r="N709" s="2" t="inlineStr" /><c r="O709" s="2" t="inlineStr" /><c r="P709" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q709" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="710"><c r="A710" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B710" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C710" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D710" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E710" s="2" t="inlineStr"><is><t>W skojarzonej terapii eradykacyjnej H. pylori zastosujesz zgodnie z aktualną wiedzą medyczną:</t></is></c><c r="F710" s="2" t="inlineStr"><is><t>omeprazol</t></is></c><c r="G710" s="2" t="inlineStr"><is><t>pantoprazol</t></is></c><c r="H710" s="2" t="inlineStr"><is><t>cytrynian bizmutu</t></is></c><c r="I710" s="2" t="inlineStr" /><c r="J710" s="2" t="inlineStr" /><c r="K710" s="2" t="inlineStr"><is><t>ranitydynę</t></is></c><c r="L710" s="2" t="inlineStr" /><c r="M710" s="2" t="inlineStr" /><c r="N710" s="2" t="inlineStr" /><c r="O710" s="2" t="inlineStr" /><c r="P710" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q710" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="711"><c r="A711" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B711" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C711" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D711" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E711" s="2" t="inlineStr"><is><t>Izotonicznym krystaloidem do uzupełnienie płynów jest:</t></is></c><c r="F711" s="2" t="inlineStr"><is><t>0,9% NaCl</t></is></c><c r="G711" s="2" t="inlineStr"><is><t>płyn wieloelektrolitowy</t></is></c><c r="H711" s="2" t="inlineStr"><is><t>płyn 2 : 1 (5% glukoza + 0,9% NaCl)</t></is></c><c r="I711" s="2" t="inlineStr" /><c r="J711" s="2" t="inlineStr" /><c r="K711" s="2" t="inlineStr"><is><t>4% roztw. żelatyny</t></is></c><c r="L711" s="2" t="inlineStr" /><c r="M711" s="2" t="inlineStr" /><c r="N711" s="2" t="inlineStr" /><c r="O711" s="2" t="inlineStr" /><c r="P711" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q711" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="712"><c r="A712" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B712" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C712" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D712" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E712" s="2" t="inlineStr"><is><t>Dysforia, nudności, wymioty, biegunka, bóle mięśni, łzawienie, wyciek z nosa, pocenie, rozszerzenie źrenic, piloerekcja, ziewanie i gorączka to cechy zespołu odstawiennego u uzależnionych od:</t></is></c><c r="F712" s="2" t="inlineStr"><is><t>heroiny</t></is></c><c r="G712" s="2" t="inlineStr" /><c r="H712" s="2" t="inlineStr" /><c r="I712" s="2" t="inlineStr" /><c r="J712" s="2" t="inlineStr" /><c r="K712" s="2" t="inlineStr"><is><t>etanolu</t></is></c><c r="L712" s="2" t="inlineStr"><is><t>nikotyny</t></is></c><c r="M712" s="2" t="inlineStr"><is><t>kokainy</t></is></c><c r="N712" s="2" t="inlineStr" /><c r="O712" s="2" t="inlineStr" /><c r="P712" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q712" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="713"><c r="A713" s="2" t="inlineStr"><is><t>LEKI TOKSYCZNE W CIĄŻY</t></is></c><c r="B713" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C713" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D713" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E713" s="2" t="inlineStr"><is><t>Mykotoksyny:</t></is></c><c r="F713" s="2" t="inlineStr"><is><t>to produkty wtórnego metabolizmu różnych rodzajów grzybów pleśniowych</t></is></c><c r="G713" s="2" t="inlineStr"><is><t>są wytwarzane jako produkt uboczny w procesach metabolicznych lub są produktem wytwarzanym w celach obronnych</t></is></c><c r="H713" s="2" t="inlineStr"><is><t>mogą mieć silne właściwości mutagenne lub teratogenne</t></is></c><c r="I713" s="2" t="inlineStr"><is><t>są potencjalnie toksyczne dla ludzi i zwierząt</t></is></c><c r="J713" s="2" t="inlineStr" /><c r="K713" s="2" t="inlineStr" /><c r="L713" s="2" t="inlineStr" /><c r="M713" s="2" t="inlineStr" /><c r="N713" s="2" t="inlineStr" /><c r="O713" s="2" t="inlineStr" /><c r="P713" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q713" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="714"><c r="A714" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B714" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C714" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D714" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E714" s="2" t="inlineStr"><is><t>Wskaż korzystne cechy leku:</t></is></c><c r="F714" s="2" t="inlineStr"><is><t>biodostępność po podaniu p.o. dorównująca biodostępności po podaniu i.v</t></is></c><c r="G714" s="2" t="inlineStr"><is><t>dostępne swoiste antidotum</t></is></c><c r="H714" s="2" t="inlineStr" /><c r="I714" s="2" t="inlineStr" /><c r="J714" s="2" t="inlineStr" /><c r="K714" s="2" t="inlineStr"><is><t>procesy kinetyczne zgodne z kinetyką 0 rzędu</t></is></c><c r="L714" s="2" t="inlineStr"><is><t>duża kumulacja w tkankach – wiązanie z biomolekułami</t></is></c><c r="M714" s="2" t="inlineStr" /><c r="N714" s="2" t="inlineStr" /><c r="O714" s="2" t="inlineStr" /><c r="P714" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2017/18 - 2 termin</t></is></c><c r="Q714" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="715"><c r="A715" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B715" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C715" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D715" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E715" s="2" t="inlineStr"><is><t>Jaki lek przeciwbakteryjny może odpowiadać poniższej charakterystyce? Ma dobrą biodostępność po podaniu doustnym i jest skuteczny w zakażeniach Streptococcus pneumoniae przy obecnym profilu oporności tego gatunku pod warunkiem właściwego schematu ekspozycji na lek:</t></is></c><c r="F715" s="2" t="inlineStr"><is><t>lewofloksacyna</t></is></c><c r="G715" s="2" t="inlineStr"><is><t>amoksycylina</t></is></c><c r="H715" s="2" t="inlineStr" /><c r="I715" s="2" t="inlineStr" /><c r="J715" s="2" t="inlineStr" /><c r="K715" s="2" t="inlineStr"><is><t>doksycyklina</t></is></c><c r="L715" s="2" t="inlineStr"><is><t>ceftriakson</t></is></c><c r="M715" s="2" t="inlineStr" /><c r="N715" s="2" t="inlineStr" /><c r="O715" s="2" t="inlineStr" /><c r="P715" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q715" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="716"><c r="A716" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B716" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C716" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D716" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E716" s="2" t="inlineStr"><is><t>Co jest zasadniczym warunkiem skuteczności cefadroksylu w leczeniu niepowikłanych zakażeń układu moczowego?</t></is></c><c r="F716" s="2" t="inlineStr"><is><t>przestrzeganie stałego interwału dawkowania zgodnie z parametrami farmakokinetycznymi leku</t></is></c><c r="G716" s="2" t="inlineStr"><is><t>fT%&gt;MIC ≥ 60%</t></is></c><c r="H716" s="2" t="inlineStr" /><c r="I716" s="2" t="inlineStr" /><c r="J716" s="2" t="inlineStr" /><c r="K716" s="2" t="inlineStr"><is><t>stały 10-dniowy cykl leczenia</t></is></c><c r="L716" s="2" t="inlineStr"><is><t>podanie jak największej bezpiecznej dawki jednorazowej, czyli uzyskanie maksymalnego bezpiecznego stężenia leku w surowicy</t></is></c><c r="M716" s="2" t="inlineStr" /><c r="N716" s="2" t="inlineStr" /><c r="O716" s="2" t="inlineStr" /><c r="P716" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q716" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="717"><c r="A717" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B717" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C717" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D717" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E717" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenia dotyczące kwasu klawulanowego:</t></is></c><c r="F717" s="2" t="inlineStr"><is><t>kwas klawulanowy powoduje niezależnie działania niepożądane, np. Polekowe zapalenie wątroby</t></is></c><c r="G717" s="2" t="inlineStr"><is><t>zmniejszona wrażliwość Streptococcus pneumoniae na beta-laktamy ma mechanizm nieenzymatyczny, zatem stosowanie połączeń z kwasem klawulanowym w zakażeniach o tej etiologii nie ma uzasadnienia</t></is></c><c r="H717" s="2" t="inlineStr"><is><t>amoksycylina + kwas klawulanowy powodują znaczną dysbakteriozę i skłonność do nadkażeń florą szpitalną</t></is></c><c r="I717" s="2" t="inlineStr" /><c r="J717" s="2" t="inlineStr" /><c r="K717" s="2" t="inlineStr"><is><t>kwas klawulanowy jest przeciwwskazany w ciąży</t></is></c><c r="L717" s="2" t="inlineStr" /><c r="M717" s="2" t="inlineStr" /><c r="N717" s="2" t="inlineStr" /><c r="O717" s="2" t="inlineStr" /><c r="P717" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q717" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="718"><c r="A718" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B718" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C718" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D718" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E718" s="2" t="inlineStr"><is><t>Podaj prawidłową interpretację sytuacji klinicznej:</t></is></c><c r="F718" s="2" t="inlineStr"><is><t>w 1 h po zakończeniu dożylnego podania piperacyliny + tazobaktamu (pip + taz) wystąpiła pokrzywka i duszność, ciśnienie skurczowe = 80 mmHg → nadwrażliwość typu natychmiastowego na penicyliny → zakaz leczenia wszystkimi penicylinami</t></is></c><c r="G718" s="2" t="inlineStr"><is><t>po 1 tygodniu leczenia ceftriaksonem + azytromycyną domowego zapalenia płuc w szpitalu wystąpiła małopłytkowość PLT = 60 G/l → nadwrażliwość typu cytotoksycznego najprawdopodobniej po ceftriaksonie → zakaz leczenia wszystkimi cefalosporynami</t></is></c><c r="H718" s="2" t="inlineStr"><is><t>po 5 dniach leczenia ceftriaksonem z metronidazolem w ramach leczenia powikłanego zapalenia wyrostka robaczkowego po operacji apendektomii wystąpił atak kolki żółciowej, w USG złogi w pęcherzyku żółciowym → prawdopodobnie wzrost gęstości żółci z powodu wydzielania ceftriaksonu → zakaz kontynuacji ceftriaksonu</t></is></c><c r="I718" s="2" t="inlineStr" /><c r="J718" s="2" t="inlineStr" /><c r="K718" s="2" t="inlineStr"><is><t>po 1 tygodniu leczenia pip + taz z powodu powikłanego zakażenia jamy brzusznej wystąpiły uogólnione obrzęki, w bad. laboratoryjnych hipernatremia = 153 mmol/l → bez związku z antybiotykoterapią, należy szukać innej przyczyny → kontynuacja leczenia pip + taz</t></is></c><c r="L718" s="2" t="inlineStr" /><c r="M718" s="2" t="inlineStr" /><c r="N718" s="2" t="inlineStr" /><c r="O718" s="2" t="inlineStr" /><c r="P718" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q718" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="719"><c r="A719" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B719" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C719" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D719" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E719" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii metycylinooporne Staphylococcus spp. uzasadnione może być zastosowanie:</t></is></c><c r="F719" s="2" t="inlineStr"><is><t>tigecyklina</t></is></c><c r="G719" s="2" t="inlineStr" /><c r="H719" s="2" t="inlineStr" /><c r="I719" s="2" t="inlineStr" /><c r="J719" s="2" t="inlineStr" /><c r="K719" s="2" t="inlineStr"><is><t>ceftolozanu + tazobaktamu</t></is></c><c r="L719" s="2" t="inlineStr"><is><t>meropenemu</t></is></c><c r="M719" s="2" t="inlineStr"><is><t>ceftazydymu + awibaktamu</t></is></c><c r="N719" s="2" t="inlineStr" /><c r="O719" s="2" t="inlineStr" /><c r="P719" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q719" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="720"><c r="A720" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B720" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C720" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D720" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E720" s="2" t="inlineStr"><is><t>Łatwo jest prowadzić leczenie sekwencyjne w przypadku:</t></is></c><c r="F720" s="2" t="inlineStr"><is><t>kloksacyliny</t></is></c><c r="G720" s="2" t="inlineStr"><is><t>amoksycyliny + kwasu klawulanowego</t></is></c><c r="H720" s="2" t="inlineStr"><is><t>cefuroksymu</t></is></c><c r="I720" s="2" t="inlineStr" /><c r="J720" s="2" t="inlineStr" /><c r="K720" s="2" t="inlineStr"><is><t>ceftazydymu</t></is></c><c r="L720" s="2" t="inlineStr" /><c r="M720" s="2" t="inlineStr" /><c r="N720" s="2" t="inlineStr" /><c r="O720" s="2" t="inlineStr" /><c r="P720" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q720" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="721"><c r="A721" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B721" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C721" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D721" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E721" s="2" t="inlineStr"><is><t>Prawdziwe jest stwierdzenie:</t></is></c><c r="F721" s="2" t="inlineStr"><is><t>cefazolina i cefuroksym i.v. są lekami z wyboru w p-infekcyjnej profilaktyce okołozabiegowej</t></is></c><c r="G721" s="2" t="inlineStr"><is><t>amoksycylina + kwas klawulanowy p.o. jest lekiem z wyboru w leczeniu z wyprzedzeniem po pogryzieniu przez psa</t></is></c><c r="H721" s="2" t="inlineStr" /><c r="I721" s="2" t="inlineStr" /><c r="J721" s="2" t="inlineStr" /><c r="K721" s="2" t="inlineStr"><is><t>ampicylina i.v. jest lekiem z wyboru w p-infekcyjnej profilaktyce rany skórnej spowodowanej ostrym przedmiotem</t></is></c><c r="L721" s="2" t="inlineStr"><is><t>aksetyl cefuroksymu jest lekiem z wyboru w leczeniu z wyprzedzeniem asymptomatycznej bakteriurii u 75-letniej kobiety z nietrzymaniem moczu</t></is></c><c r="M721" s="2" t="inlineStr" /><c r="N721" s="2" t="inlineStr" /><c r="O721" s="2" t="inlineStr" /><c r="P721" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q721" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="722"><c r="A722" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B722" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C722" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D722" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E722" s="2" t="inlineStr"><is><t>W którym przypadku decyzja dotycząca racjonalnego leczenia początkowego domowego zakażenia jest prawidłowa u pacjenta bez nadwrażliwości na leki w wywiadach?</t></is></c><c r="F722" s="2" t="inlineStr"><is><t>grypa u nieszczepionego 80-letniego mężczyzny z POChP – oseltamiwir</t></is></c><c r="G722" s="2" t="inlineStr"><is><t>zapalenie płuc u osoby bez chorób współtowarzyszących – amoksycylina w dawce 3-4 g/24 h</t></is></c><c r="H722" s="2" t="inlineStr" /><c r="I722" s="2" t="inlineStr" /><c r="J722" s="2" t="inlineStr" /><c r="K722" s="2" t="inlineStr"><is><t>angina paciorkowcowa – azytromycyna</t></is></c><c r="L722" s="2" t="inlineStr"><is><t>niezapalna ostra biegunka – cyprofloksacyna</t></is></c><c r="M722" s="2" t="inlineStr" /><c r="N722" s="2" t="inlineStr" /><c r="O722" s="2" t="inlineStr" /><c r="P722" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q722" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="723"><c r="A723" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B723" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C723" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D723" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E723" s="2" t="inlineStr"><is><t>Linezolid jest wskazany w terapii zakażeń o etiologii:</t></is></c><c r="F723" s="2" t="inlineStr"><is><t>wankomycynooporny Enterococcus faecium (WRE)</t></is></c><c r="G723" s="2" t="inlineStr"><is><t>Streptococcus pneumoniae opornej na penicylinę</t></is></c><c r="H723" s="2" t="inlineStr"><is><t>metycylinooporny gronkowiec złocisty (MRSA)</t></is></c><c r="I723" s="2" t="inlineStr" /><c r="J723" s="2" t="inlineStr" /><c r="K723" s="2" t="inlineStr"><is><t>Klebsiella pneumonae oporna na karbapenemy</t></is></c><c r="L723" s="2" t="inlineStr" /><c r="M723" s="2" t="inlineStr" /><c r="N723" s="2" t="inlineStr" /><c r="O723" s="2" t="inlineStr" /><c r="P723" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q723" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="724"><c r="A724" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B724" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C724" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D724" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E724" s="2" t="inlineStr"><is><t>Który zestaw przedstawia leki od najwęższego do najszerszego spektrum działania przeciwbakteryjnego:</t></is></c><c r="F724" s="2" t="inlineStr"><is><t>ampicylina – piperacylina – piperacylina + tazobaktam</t></is></c><c r="G724" s="2" t="inlineStr"><is><t>ertapenem – imipenem – meropenem + waborbaktam</t></is></c><c r="H724" s="2" t="inlineStr" /><c r="I724" s="2" t="inlineStr" /><c r="J724" s="2" t="inlineStr" /><c r="K724" s="2" t="inlineStr"><is><t>ceftazydym – cefotaksym – cefepim</t></is></c><c r="L724" s="2" t="inlineStr"><is><t>ampicylina – fenoksymetylopenicylina – kloksacylina</t></is></c><c r="M724" s="2" t="inlineStr" /><c r="N724" s="2" t="inlineStr" /><c r="O724" s="2" t="inlineStr" /><c r="P724" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q724" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="725"><c r="A725" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B725" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C725" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D725" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E725" s="2" t="inlineStr"><is><t>W leczeniu zakażenia bakteriami atypowymi u chorego z pierwotnym wydłużeniem QTc racjonalne jest zastosowanie:</t></is></c><c r="F725" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="G725" s="2" t="inlineStr" /><c r="H725" s="2" t="inlineStr" /><c r="I725" s="2" t="inlineStr" /><c r="J725" s="2" t="inlineStr" /><c r="K725" s="2" t="inlineStr"><is><t>moksyfloksacyny</t></is></c><c r="L725" s="2" t="inlineStr"><is><t>klarytromycyny</t></is></c><c r="M725" s="2" t="inlineStr"><is><t>klindamycyny</t></is></c><c r="N725" s="2" t="inlineStr" /><c r="O725" s="2" t="inlineStr" /><c r="P725" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q725" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="726"><c r="A726" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B726" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C726" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D726" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E726" s="2" t="inlineStr"><is><t>Wskazaniem do zastosowania metronidazolu jest:</t></is></c><c r="F726" s="2" t="inlineStr"><is><t>biegunka o etiologii Clostridium difficile o nieciężkim przebiegu</t></is></c><c r="G726" s="2" t="inlineStr"><is><t>lamblioza</t></is></c><c r="H726" s="2" t="inlineStr" /><c r="I726" s="2" t="inlineStr" /><c r="J726" s="2" t="inlineStr" /><c r="K726" s="2" t="inlineStr"><is><t>eradykacja nosicielstwa Bacteroides fragilis z przewodu pokarmowego przed wszystkimi operacjami w polu czystym-skażonym</t></is></c><c r="L726" s="2" t="inlineStr"><is><t>toksoplazmoza</t></is></c><c r="M726" s="2" t="inlineStr" /><c r="N726" s="2" t="inlineStr" /><c r="O726" s="2" t="inlineStr" /><c r="P726" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q726" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="727"><c r="A727" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B727" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C727" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D727" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E727" s="2" t="inlineStr"><is><t>Ze względu na podobieństwo w farmakologicznym mechanizmie działania nie należy łączyć:</t></is></c><c r="F727" s="2" t="inlineStr"><is><t>kotrymoksazolu i trimetoprimu</t></is></c><c r="G727" s="2" t="inlineStr"><is><t>erytromycyny i klindamycyny</t></is></c><c r="H727" s="2" t="inlineStr" /><c r="I727" s="2" t="inlineStr" /><c r="J727" s="2" t="inlineStr" /><c r="K727" s="2" t="inlineStr"><is><t>ampicyliny i gentamycyny</t></is></c><c r="L727" s="2" t="inlineStr"><is><t>wankomycyny i aztreonamu</t></is></c><c r="M727" s="2" t="inlineStr" /><c r="N727" s="2" t="inlineStr" /><c r="O727" s="2" t="inlineStr" /><c r="P727" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q727" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="728"><c r="A728" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B728" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C728" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D728" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E728" s="2" t="inlineStr"><is><t>Nadwrażliwość na promieniowanie ultrafioletowe (UV) może być związana ze stosowaniem:</t></is></c><c r="F728" s="2" t="inlineStr"><is><t>doksycykliny</t></is></c><c r="G728" s="2" t="inlineStr"><is><t>lewofloksacyny</t></is></c><c r="H728" s="2" t="inlineStr"><is><t>kotrymoksazolu</t></is></c><c r="I728" s="2" t="inlineStr" /><c r="J728" s="2" t="inlineStr" /><c r="K728" s="2" t="inlineStr"><is><t>amoksycyliny</t></is></c><c r="L728" s="2" t="inlineStr" /><c r="M728" s="2" t="inlineStr" /><c r="N728" s="2" t="inlineStr" /><c r="O728" s="2" t="inlineStr" /><c r="P728" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q728" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="729"><c r="A729" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B729" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C729" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D729" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E729" s="2" t="inlineStr"><is><t>Za uzasadnione uznasz dodanie metronidazolu do:</t></is></c><c r="F729" s="2" t="inlineStr"><is><t>cyprofloksacyny w leczeniu zakażenia mieszanego dróg żółciowych z udziałem beztlenowców</t></is></c><c r="G729" s="2" t="inlineStr" /><c r="H729" s="2" t="inlineStr" /><c r="I729" s="2" t="inlineStr" /><c r="J729" s="2" t="inlineStr" /><c r="K729" s="2" t="inlineStr"><is><t>amoksycyliny + kwasu klawulanowego w leczeniu zakażenia mieszanego zatok szczękowych z udziałem beztlenowców</t></is></c><c r="L729" s="2" t="inlineStr"><is><t>piperacyliny + tazobaktamu w leczeniu zachłystowego zapalenia płuc (zakażenie florą przewodu pokarmowego)</t></is></c><c r="M729" s="2" t="inlineStr"><is><t>imipenemu + cilastatyny w leczeniu kałowego zapalenia otrzewnej po perforacji jelita grubego (zakażenie florą przewodu pokarmowego)</t></is></c><c r="N729" s="2" t="inlineStr" /><c r="O729" s="2" t="inlineStr" /><c r="P729" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q729" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="730"><c r="A730" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B730" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C730" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D730" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E730" s="2" t="inlineStr"><is><t>Właściwy wybór leku w infestacji pasożytniczej to:</t></is></c><c r="F730" s="2" t="inlineStr"><is><t>wszawica - permetryna</t></is></c><c r="G730" s="2" t="inlineStr"><is><t>rzęsistkowica - metronidazol</t></is></c><c r="H730" s="2" t="inlineStr"><is><t>toksoplazmoza – kotrymoksazol</t></is></c><c r="I730" s="2" t="inlineStr"><is><t>infestacja owsikiem - pyrantel</t></is></c><c r="J730" s="2" t="inlineStr" /><c r="K730" s="2" t="inlineStr" /><c r="L730" s="2" t="inlineStr" /><c r="M730" s="2" t="inlineStr" /><c r="N730" s="2" t="inlineStr" /><c r="O730" s="2" t="inlineStr" /><c r="P730" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q730" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="731"><c r="A731" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B731" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C731" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D731" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E731" s="2" t="inlineStr"><is><t>Właściwy wybór leku przeciwwirusowego w zakażeniu wirusowym to:</t></is></c><c r="F731" s="2" t="inlineStr"><is><t>wirus półpaśca – acyklowir</t></is></c><c r="G731" s="2" t="inlineStr"><is><t>przewlekłe wirusowe zapalenie wątroby typu C - bezpośrednio działające ledipaswir + sofosbuwir</t></is></c><c r="H731" s="2" t="inlineStr" /><c r="I731" s="2" t="inlineStr" /><c r="J731" s="2" t="inlineStr" /><c r="K731" s="2" t="inlineStr"><is><t>rotawirus – loperamid</t></is></c><c r="L731" s="2" t="inlineStr"><is><t>kłykciny kończyste – pranobeks inozyny</t></is></c><c r="M731" s="2" t="inlineStr" /><c r="N731" s="2" t="inlineStr" /><c r="O731" s="2" t="inlineStr" /><c r="P731" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q731" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="732"><c r="A732" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B732" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C732" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D732" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E732" s="2" t="inlineStr"><is><t>W dermatofitozach skuteczne jest miejscowe użycie:</t></is></c><c r="F732" s="2" t="inlineStr"><is><t>naftyfiny</t></is></c><c r="G732" s="2" t="inlineStr"><is><t>klotrimazolu</t></is></c><c r="H732" s="2" t="inlineStr" /><c r="I732" s="2" t="inlineStr" /><c r="J732" s="2" t="inlineStr" /><c r="K732" s="2" t="inlineStr"><is><t>natamycyny</t></is></c><c r="L732" s="2" t="inlineStr"><is><t>imikwimodu</t></is></c><c r="M732" s="2" t="inlineStr" /><c r="N732" s="2" t="inlineStr" /><c r="O732" s="2" t="inlineStr" /><c r="P732" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q732" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="733"><c r="A733" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B733" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C733" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D733" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E733" s="2" t="inlineStr"><is><t>W przypadku biegunki o etiologii Clostridium difficile uzasadnione może być stosowanie:</t></is></c><c r="F733" s="2" t="inlineStr"><is><t>fidaksomycyny doustnie</t></is></c><c r="G733" s="2" t="inlineStr"><is><t>wankomycyny doustnie</t></is></c><c r="H733" s="2" t="inlineStr" /><c r="I733" s="2" t="inlineStr" /><c r="J733" s="2" t="inlineStr" /><c r="K733" s="2" t="inlineStr"><is><t>nifuroksazydu doustnie</t></is></c><c r="L733" s="2" t="inlineStr"><is><t>kotrymoksazolu doustnie</t></is></c><c r="M733" s="2" t="inlineStr" /><c r="N733" s="2" t="inlineStr" /><c r="O733" s="2" t="inlineStr" /><c r="P733" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q733" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="734"><c r="A734" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B734" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C734" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D734" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E734" s="2" t="inlineStr"><is><t>W leczeniu gruźlicy wielolekoopornej (MDR-TB) do leków podstawowych (grupa A, B i C wg wytycznych WHO) należy:</t></is></c><c r="F734" s="2" t="inlineStr"><is><t>moksyfloksacyna</t></is></c><c r="G734" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="H734" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="I734" s="2" t="inlineStr"><is><t>kapreomycyna</t></is></c><c r="J734" s="2" t="inlineStr" /><c r="K734" s="2" t="inlineStr" /><c r="L734" s="2" t="inlineStr" /><c r="M734" s="2" t="inlineStr" /><c r="N734" s="2" t="inlineStr" /><c r="O734" s="2" t="inlineStr" /><c r="P734" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q734" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="735"><c r="A735" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B735" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C735" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D735" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E735" s="2" t="inlineStr"><is><t>Opis farmakokinetyki leku A: lek A dobrze wchłania się z przewodu pokarmowego, dobrze przenika przez barierę krew – mózg, podlega metabolizmowi wątrobowemu. Lekiem A może być:</t></is></c><c r="F735" s="2" t="inlineStr"><is><t>worykonazol</t></is></c><c r="G735" s="2" t="inlineStr" /><c r="H735" s="2" t="inlineStr" /><c r="I735" s="2" t="inlineStr" /><c r="J735" s="2" t="inlineStr" /><c r="K735" s="2" t="inlineStr"><is><t>amoksycylina</t></is></c><c r="L735" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="M735" s="2" t="inlineStr"><is><t>wankomycyna</t></is></c><c r="N735" s="2" t="inlineStr" /><c r="O735" s="2" t="inlineStr" /><c r="P735" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q735" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="736"><c r="A736" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B736" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C736" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D736" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E736" s="2" t="inlineStr"><is><t>Zmiany na płytkach paznokciowych polegające na ich zgrubieniu, przebarwieniu, łamliwości, nadmiernym rogowaceniu i pobruzdowaniu można leczyć:</t></is></c><c r="F736" s="2" t="inlineStr"><is><t>amorolfiną miejscowo</t></is></c><c r="G736" s="2" t="inlineStr"><is><t>terbinafiną doustnie</t></is></c><c r="H736" s="2" t="inlineStr"><is><t>itrakonazolem doustnie</t></is></c><c r="I736" s="2" t="inlineStr"><is><t>cyklopiroksolaminą miejscowo</t></is></c><c r="J736" s="2" t="inlineStr" /><c r="K736" s="2" t="inlineStr" /><c r="L736" s="2" t="inlineStr" /><c r="M736" s="2" t="inlineStr" /><c r="N736" s="2" t="inlineStr" /><c r="O736" s="2" t="inlineStr" /><c r="P736" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q736" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="737"><c r="A737" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B737" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C737" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D737" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E737" s="2" t="inlineStr"><is><t>Aktualnie wg komunikatu WHO krytyczny problem wielolekooporności na większość leków p-bakteryjnych dotyczy:</t></is></c><c r="F737" s="2" t="inlineStr"><is><t>Acinetobacter baumani z opornością na karbapenemy</t></is></c><c r="G737" s="2" t="inlineStr"><is><t>Pseudomonas aeruginosa z opornością na karbapenemy</t></is></c><c r="H737" s="2" t="inlineStr"><is><t>Enterobacteriacae z opornością na karbapenemy</t></is></c><c r="I737" s="2" t="inlineStr" /><c r="J737" s="2" t="inlineStr" /><c r="K737" s="2" t="inlineStr"><is><t>Stenotrophomonas maltophilia z opornością na karbapenemy</t></is></c><c r="L737" s="2" t="inlineStr" /><c r="M737" s="2" t="inlineStr" /><c r="N737" s="2" t="inlineStr" /><c r="O737" s="2" t="inlineStr" /><c r="P737" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q737" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="738"><c r="A738" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B738" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C738" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D738" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E738" s="2" t="inlineStr"><is><t>Dla leków p-infekcyjnych dla których celem farmakodynamicznym jest wysoka wartość fAUC : MIC, np. fluorochinolonów zasadne jest:</t></is></c><c r="F738" s="2" t="inlineStr"><is><t>zwiększenie w bezpiecznych granicach skumulowanej dobowej dawki leku</t></is></c><c r="G738" s="2" t="inlineStr" /><c r="H738" s="2" t="inlineStr" /><c r="I738" s="2" t="inlineStr" /><c r="J738" s="2" t="inlineStr" /><c r="K738" s="2" t="inlineStr"><is><t>precyzyjne ustalenie jak najczęstszego dawkowania leku</t></is></c><c r="L738" s="2" t="inlineStr"><is><t>monitorowanie stężenia maksymalnego (peak) w celu modyfikacji dawki</t></is></c><c r="M738" s="2" t="inlineStr"><is><t>osiągnięcie zdefiniowanej wartości fCmin : MIC</t></is></c><c r="N738" s="2" t="inlineStr" /><c r="O738" s="2" t="inlineStr" /><c r="P738" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q738" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="739"><c r="A739" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B739" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C739" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D739" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E739" s="2" t="inlineStr"><is><t>U pacjenta z eGFR &lt; 30 ml/min (wyliczony z wzoru Cockcrofta-Gaulta) należy zmodyfikować dawkowanie:</t></is></c><c r="F739" s="2" t="inlineStr"><is><t>gentamycyny</t></is></c><c r="G739" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="H739" s="2" t="inlineStr"><is><t>imipenemu</t></is></c><c r="I739" s="2" t="inlineStr" /><c r="J739" s="2" t="inlineStr" /><c r="K739" s="2" t="inlineStr"><is><t>klindamycyny</t></is></c><c r="L739" s="2" t="inlineStr" /><c r="M739" s="2" t="inlineStr" /><c r="N739" s="2" t="inlineStr" /><c r="O739" s="2" t="inlineStr" /><c r="P739" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q739" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="740"><c r="A740" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B740" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C740" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D740" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E740" s="2" t="inlineStr"><is><t>U pacjenta z eGFR &lt; 30 ml/min (wyliczony z wzoru Cockcrofta-Gaulta) należy zmodyfikować dawkowanie:</t></is></c><c r="F740" s="2" t="inlineStr"><is><t>oseltamiwiru</t></is></c><c r="G740" s="2" t="inlineStr"><is><t>flukonazolu</t></is></c><c r="H740" s="2" t="inlineStr" /><c r="I740" s="2" t="inlineStr" /><c r="J740" s="2" t="inlineStr" /><c r="K740" s="2" t="inlineStr"><is><t>ryfampicyny</t></is></c><c r="L740" s="2" t="inlineStr"><is><t>kaspofunginy</t></is></c><c r="M740" s="2" t="inlineStr" /><c r="N740" s="2" t="inlineStr" /><c r="O740" s="2" t="inlineStr" /><c r="P740" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q740" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="741"><c r="A741" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B741" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C741" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D741" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E741" s="2" t="inlineStr"><is><t>Do długoterminowych działań niepożądanych terapii HAART należy:</t></is></c><c r="F741" s="2" t="inlineStr"><is><t>uszkodzenie wątroby</t></is></c><c r="G741" s="2" t="inlineStr"><is><t>zespół lipodystrofii</t></is></c><c r="H741" s="2" t="inlineStr"><is><t>kwasica mleczanowa</t></is></c><c r="I741" s="2" t="inlineStr"><is><t>insulinooporność</t></is></c><c r="J741" s="2" t="inlineStr" /><c r="K741" s="2" t="inlineStr" /><c r="L741" s="2" t="inlineStr" /><c r="M741" s="2" t="inlineStr" /><c r="N741" s="2" t="inlineStr" /><c r="O741" s="2" t="inlineStr" /><c r="P741" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q741" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="742"><c r="A742" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B742" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C742" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D742" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E742" s="2" t="inlineStr"><is><t>Do jakiego związku może się odnosić następujący opis: ma słabe działanie antyseptyczne, po wchłonięciu może powodować ciężkie powikłania tj. Uszkodzenia wątroby i nerek, niewydolność serca, splątanie, a nawet zgon:</t></is></c><c r="F742" s="2" t="inlineStr"><is><t>boran sodu</t></is></c><c r="G742" s="2" t="inlineStr" /><c r="H742" s="2" t="inlineStr" /><c r="I742" s="2" t="inlineStr" /><c r="J742" s="2" t="inlineStr" /><c r="K742" s="2" t="inlineStr"><is><t>oktenidyna</t></is></c><c r="L742" s="2" t="inlineStr"><is><t>woda utleniona</t></is></c><c r="M742" s="2" t="inlineStr"><is><t>jodopowidon</t></is></c><c r="N742" s="2" t="inlineStr" /><c r="O742" s="2" t="inlineStr" /><c r="P742" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q742" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="743"><c r="A743" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B743" s="2" t="inlineStr"><is><t>Dawkowanie</t></is></c><c r="C743" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D743" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E743" s="2" t="inlineStr"><is><t>U pacjenta leczonego antagonistą witaminy K (warfaryną, acenokumarolem) zmianę efektu przeciwzakrzepowego bez adekwatnej modyfikacji dawki tego leku może spowodować:</t></is></c><c r="F743" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="G743" s="2" t="inlineStr"><is><t>klarytromycyna</t></is></c><c r="H743" s="2" t="inlineStr"><is><t>ryfampicyna</t></is></c><c r="I743" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="J743" s="2" t="inlineStr" /><c r="K743" s="2" t="inlineStr" /><c r="L743" s="2" t="inlineStr" /><c r="M743" s="2" t="inlineStr" /><c r="N743" s="2" t="inlineStr" /><c r="O743" s="2" t="inlineStr" /><c r="P743" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q743" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="744"><c r="A744" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B744" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C744" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D744" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E744" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Streptococcus pneumoniae skuteczny/a może być:</t></is></c><c r="F744" s="2" t="inlineStr"><is><t>ceftriakson</t></is></c><c r="G744" s="2" t="inlineStr"><is><t>klarytromycyna</t></is></c><c r="H744" s="2" t="inlineStr"><is><t>amoksycylina</t></is></c><c r="I744" s="2" t="inlineStr"><is><t>lewofloksacyna</t></is></c><c r="J744" s="2" t="inlineStr" /><c r="K744" s="2" t="inlineStr" /><c r="L744" s="2" t="inlineStr" /><c r="M744" s="2" t="inlineStr" /><c r="N744" s="2" t="inlineStr" /><c r="O744" s="2" t="inlineStr" /><c r="P744" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q744" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="745"><c r="A745" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B745" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C745" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D745" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E745" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Escherichia coli skuteczny/a może być:</t></is></c><c r="F745" s="2" t="inlineStr"><is><t>cefuroksym</t></is></c><c r="G745" s="2" t="inlineStr"><is><t>kotrymoksazol</t></is></c><c r="H745" s="2" t="inlineStr"><is><t>fosfomycyna</t></is></c><c r="I745" s="2" t="inlineStr" /><c r="J745" s="2" t="inlineStr" /><c r="K745" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="L745" s="2" t="inlineStr" /><c r="M745" s="2" t="inlineStr" /><c r="N745" s="2" t="inlineStr" /><c r="O745" s="2" t="inlineStr" /><c r="P745" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q745" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="746"><c r="A746" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B746" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C746" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D746" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E746" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Staphylococcus aureus metycylinowrażliwy (MSSA) skuteczny/a może być:</t></is></c><c r="F746" s="2" t="inlineStr"><is><t>cefadroksyl</t></is></c><c r="G746" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="H746" s="2" t="inlineStr"><is><t>kloksacylina</t></is></c><c r="I746" s="2" t="inlineStr" /><c r="J746" s="2" t="inlineStr" /><c r="K746" s="2" t="inlineStr"><is><t>fenoksymetylopenicylina</t></is></c><c r="L746" s="2" t="inlineStr" /><c r="M746" s="2" t="inlineStr" /><c r="N746" s="2" t="inlineStr" /><c r="O746" s="2" t="inlineStr" /><c r="P746" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q746" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="747"><c r="A747" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B747" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C747" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D747" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E747" s="2" t="inlineStr"><is><t>W zakażeniu o etiologii Streptococcus pyogenes skuteczny/a może być:</t></is></c><c r="F747" s="2" t="inlineStr"><is><t>penicylina benzylowa</t></is></c><c r="G747" s="2" t="inlineStr"><is><t>erytromycyna</t></is></c><c r="H747" s="2" t="inlineStr"><is><t>fenoksymetylopenicylina</t></is></c><c r="I747" s="2" t="inlineStr" /><c r="J747" s="2" t="inlineStr" /><c r="K747" s="2" t="inlineStr"><is><t>aztreonam</t></is></c><c r="L747" s="2" t="inlineStr" /><c r="M747" s="2" t="inlineStr" /><c r="N747" s="2" t="inlineStr" /><c r="O747" s="2" t="inlineStr" /><c r="P747" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q747" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="748"><c r="A748" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B748" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C748" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D748" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E748" s="2" t="inlineStr"><is><t>W zakażeniu o etiologii Pseudomonas aeruginosa skuteczny/a może być:</t></is></c><c r="F748" s="2" t="inlineStr"><is><t>gentamycyna</t></is></c><c r="G748" s="2" t="inlineStr"><is><t>cefepim</t></is></c><c r="H748" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="I748" s="2" t="inlineStr"><is><t>piperacylina</t></is></c><c r="J748" s="2" t="inlineStr" /><c r="K748" s="2" t="inlineStr" /><c r="L748" s="2" t="inlineStr" /><c r="M748" s="2" t="inlineStr" /><c r="N748" s="2" t="inlineStr" /><c r="O748" s="2" t="inlineStr" /><c r="P748" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q748" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="749"><c r="A749" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B749" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C749" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D749" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E749" s="2" t="inlineStr"><is><t>W zakażeniach wywołanych przez beztlenowce (w tym Bacteroides fragilis) skuteczny/a może być:</t></is></c><c r="F749" s="2" t="inlineStr"><is><t>amoksycylina + kwas klawulanowy</t></is></c><c r="G749" s="2" t="inlineStr"><is><t>imipenem + cilastatyna</t></is></c><c r="H749" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="I749" s="2" t="inlineStr" /><c r="J749" s="2" t="inlineStr" /><c r="K749" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="L749" s="2" t="inlineStr" /><c r="M749" s="2" t="inlineStr" /><c r="N749" s="2" t="inlineStr" /><c r="O749" s="2" t="inlineStr" /><c r="P749" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q749" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="750"><c r="A750" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B750" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C750" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D750" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E750" s="2" t="inlineStr"><is><t>W zakażeniach o etiologii Mycoplasma pneumoniae skuteczny/a może być:</t></is></c><c r="F750" s="2" t="inlineStr"><is><t>azytromycyna</t></is></c><c r="G750" s="2" t="inlineStr"><is><t>doksycyklina</t></is></c><c r="H750" s="2" t="inlineStr"><is><t>moksyfloksacyna</t></is></c><c r="I750" s="2" t="inlineStr" /><c r="J750" s="2" t="inlineStr" /><c r="K750" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="L750" s="2" t="inlineStr" /><c r="M750" s="2" t="inlineStr" /><c r="N750" s="2" t="inlineStr" /><c r="O750" s="2" t="inlineStr" /><c r="P750" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q750" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="751"><c r="A751" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B751" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C751" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D751" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E751" s="2" t="inlineStr"><is><t>W eradykacji Helicobacter pylori można zastosować:</t></is></c><c r="F751" s="2" t="inlineStr"><is><t>tetracyklina</t></is></c><c r="G751" s="2" t="inlineStr"><is><t>amoksycylina</t></is></c><c r="H751" s="2" t="inlineStr"><is><t>cytrynian bizmutu</t></is></c><c r="I751" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="J751" s="2" t="inlineStr" /><c r="K751" s="2" t="inlineStr" /><c r="L751" s="2" t="inlineStr" /><c r="M751" s="2" t="inlineStr" /><c r="N751" s="2" t="inlineStr" /><c r="O751" s="2" t="inlineStr" /><c r="P751" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q751" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="752"><c r="A752" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B752" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C752" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D752" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E752" s="2" t="inlineStr"><is><t>Ciężarna kobieta leczona była z konieczności gentamycyną z powodu powikłanego zapalenia nerek. Na jakie ryzyka narażone zostało jej dziecko w czasie takiej terapii?</t></is></c><c r="F752" s="2" t="inlineStr"><is><t>głuchotę</t></is></c><c r="G752" s="2" t="inlineStr" /><c r="H752" s="2" t="inlineStr" /><c r="I752" s="2" t="inlineStr" /><c r="J752" s="2" t="inlineStr" /><c r="K752" s="2" t="inlineStr"><is><t>powstanie deformacji kostnych</t></is></c><c r="L752" s="2" t="inlineStr"><is><t>utratę wzroku</t></is></c><c r="M752" s="2" t="inlineStr"><is><t>zahamowanie rozwoju chrząstek</t></is></c><c r="N752" s="2" t="inlineStr" /><c r="O752" s="2" t="inlineStr" /><c r="P752" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q752" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="753"><c r="A753" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B753" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C753" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D753" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E753" s="2" t="inlineStr"><is><t>Wskaż prawidłowe skojarzenie lek przeciwbakteryjny – mechanizm działania</t></is></c><c r="F753" s="2" t="inlineStr"><is><t>kolistyna – uszkadza błonę komórkową</t></is></c><c r="G753" s="2" t="inlineStr" /><c r="H753" s="2" t="inlineStr" /><c r="I753" s="2" t="inlineStr" /><c r="J753" s="2" t="inlineStr" /><c r="K753" s="2" t="inlineStr"><is><t>cyprofloksacyna – działa cytotoksycznie uszkadzając DNA</t></is></c><c r="L753" s="2" t="inlineStr"><is><t>azytromycyna – hamuje syntezę ściany bakteryjnej</t></is></c><c r="M753" s="2" t="inlineStr"><is><t>metronidazol – hamuje syntezę DNA</t></is></c><c r="N753" s="2" t="inlineStr" /><c r="O753" s="2" t="inlineStr" /><c r="P753" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q753" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="754"><c r="A754" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B754" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C754" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D754" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E754" s="2" t="inlineStr"><is><t>Aby uzyskać działanie ogólnoustrojowe, doustnie można podać:</t></is></c><c r="F754" s="2" t="inlineStr"><is><t>lewofloksacynę</t></is></c><c r="G754" s="2" t="inlineStr" /><c r="H754" s="2" t="inlineStr" /><c r="I754" s="2" t="inlineStr" /><c r="J754" s="2" t="inlineStr" /><c r="K754" s="2" t="inlineStr"><is><t>wankomycynę</t></is></c><c r="L754" s="2" t="inlineStr"><is><t>fidaksomycynę</t></is></c><c r="M754" s="2" t="inlineStr"><is><t>ryfaksyminę</t></is></c><c r="N754" s="2" t="inlineStr" /><c r="O754" s="2" t="inlineStr" /><c r="P754" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q754" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="755"><c r="A755" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B755" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C755" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D755" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E755" s="2" t="inlineStr"><is><t>Do antybiotyków o szerokim zakresie działania przeciwbakteryjnego na bakterie Gram (+) i Gram (-) należy:</t></is></c><c r="F755" s="2" t="inlineStr"><is><t>tygecyklina</t></is></c><c r="G755" s="2" t="inlineStr"><is><t>piperacylina + tazobaktam</t></is></c><c r="H755" s="2" t="inlineStr" /><c r="I755" s="2" t="inlineStr" /><c r="J755" s="2" t="inlineStr" /><c r="K755" s="2" t="inlineStr"><is><t>kolistyna</t></is></c><c r="L755" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="M755" s="2" t="inlineStr" /><c r="N755" s="2" t="inlineStr" /><c r="O755" s="2" t="inlineStr" /><c r="P755" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q755" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="756"><c r="A756" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B756" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C756" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D756" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E756" s="2" t="inlineStr"><is><t>Do leków do stosowania wyłącznie miejscowego należy:</t></is></c><c r="F756" s="2" t="inlineStr"><is><t>bacytracyna</t></is></c><c r="G756" s="2" t="inlineStr"><is><t>mupirocyna</t></is></c><c r="H756" s="2" t="inlineStr"><is><t>nystatyna</t></is></c><c r="I756" s="2" t="inlineStr" /><c r="J756" s="2" t="inlineStr" /><c r="K756" s="2" t="inlineStr"><is><t>fosfomycyna</t></is></c><c r="L756" s="2" t="inlineStr" /><c r="M756" s="2" t="inlineStr" /><c r="N756" s="2" t="inlineStr" /><c r="O756" s="2" t="inlineStr" /><c r="P756" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q756" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="757"><c r="A757" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B757" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C757" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D757" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E757" s="2" t="inlineStr"><is><t>Leki przeciwbakteryjne o wysokim potencjale selekcji szczepów Clostridium difficile to:</t></is></c><c r="F757" s="2" t="inlineStr"><is><t>amoksycylina + kwas klawulanowy</t></is></c><c r="G757" s="2" t="inlineStr"><is><t>klindamycyna</t></is></c><c r="H757" s="2" t="inlineStr"><is><t>cyprofloksacyna</t></is></c><c r="I757" s="2" t="inlineStr" /><c r="J757" s="2" t="inlineStr" /><c r="K757" s="2" t="inlineStr"><is><t>teikoplanina</t></is></c><c r="L757" s="2" t="inlineStr" /><c r="M757" s="2" t="inlineStr" /><c r="N757" s="2" t="inlineStr" /><c r="O757" s="2" t="inlineStr" /><c r="P757" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q757" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="758"><c r="A758" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B758" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C758" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D758" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E758" s="2" t="inlineStr"><is><t>Wskaż właściwe połączenia: mechanizm oporności na lek przeciwbakteryjny – lek unieczynniany w tym mechanizmie:</t></is></c><c r="F758" s="2" t="inlineStr"><is><t>wytwarzanie β-laktamaz – amoksycylina</t></is></c><c r="G758" s="2" t="inlineStr" /><c r="H758" s="2" t="inlineStr" /><c r="I758" s="2" t="inlineStr" /><c r="J758" s="2" t="inlineStr" /><c r="K758" s="2" t="inlineStr"><is><t>wytwarzanie karbapenemaz – tazobaktam</t></is></c><c r="L758" s="2" t="inlineStr"><is><t>metylacja podjednostki 50S rybosomu - fosfomycyna</t></is></c><c r="M758" s="2" t="inlineStr"><is><t>modyfikacja/ochrona topoizomerazy II – metronidazol</t></is></c><c r="N758" s="2" t="inlineStr" /><c r="O758" s="2" t="inlineStr" /><c r="P758" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q758" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="759"><c r="A759" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B759" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C759" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D759" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E759" s="2" t="inlineStr"><is><t>Cel farmakodynamiczny, jakim jest zależność efektu od czasu w jakim stężenie leku przekracza MIC (fT&gt;MIC) należy osiągnąć w trakcie stosowania:</t></is></c><c r="F759" s="2" t="inlineStr"><is><t>linezolidu</t></is></c><c r="G759" s="2" t="inlineStr"><is><t>ceftriaksonu</t></is></c><c r="H759" s="2" t="inlineStr" /><c r="I759" s="2" t="inlineStr" /><c r="J759" s="2" t="inlineStr" /><c r="K759" s="2" t="inlineStr"><is><t>metronidazolu</t></is></c><c r="L759" s="2" t="inlineStr"><is><t>cyprofloksacyny</t></is></c><c r="M759" s="2" t="inlineStr" /><c r="N759" s="2" t="inlineStr" /><c r="O759" s="2" t="inlineStr" /><c r="P759" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q759" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="760"><c r="A760" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B760" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C760" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D760" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E760" s="2" t="inlineStr"><is><t>Który z poniższych leków hamuje podjędnostkę 30S rybosomów?</t></is></c><c r="F760" s="2" t="inlineStr"><is><t>tygecyklina</t></is></c><c r="G760" s="2" t="inlineStr"><is><t>streptomycyna</t></is></c><c r="H760" s="2" t="inlineStr" /><c r="I760" s="2" t="inlineStr" /><c r="J760" s="2" t="inlineStr" /><c r="K760" s="2" t="inlineStr"><is><t>chinuprystyna-dalfoprystyna</t></is></c><c r="L760" s="2" t="inlineStr"><is><t>linezolid</t></is></c><c r="M760" s="2" t="inlineStr" /><c r="N760" s="2" t="inlineStr" /><c r="O760" s="2" t="inlineStr" /><c r="P760" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q760" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="761"><c r="A761" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B761" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C761" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D761" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E761" s="2" t="inlineStr"><is><t>Antybiotyki beta-laktamowe:</t></is></c><c r="F761" s="2" t="inlineStr"><is><t>cechują się bardzo dobrym profilem bezpieczeństwa</t></is></c><c r="G761" s="2" t="inlineStr"><is><t>są praktycznie pozbawione istotnych interakcji lekowych</t></is></c><c r="H761" s="2" t="inlineStr" /><c r="I761" s="2" t="inlineStr" /><c r="J761" s="2" t="inlineStr" /><c r="K761" s="2" t="inlineStr"><is><t>bardzo dobrze dystrybuują do płynu mózgowo rdzeniowego</t></is></c><c r="L761" s="2" t="inlineStr"><is><t>są przeciwwskazane w umiarkowanej i ciężkiej niewydolności wątroby</t></is></c><c r="M761" s="2" t="inlineStr" /><c r="N761" s="2" t="inlineStr" /><c r="O761" s="2" t="inlineStr" /><c r="P761" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q761" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="762"><c r="A762" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B762" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C762" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D762" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E762" s="2" t="inlineStr"><is><t>Tetracykliny:</t></is></c><c r="F762" s="2" t="inlineStr"><is><t>są przeciwwskazane u dzieci</t></is></c><c r="G762" s="2" t="inlineStr"><is><t>działają także na bakterie atypowe</t></is></c><c r="H762" s="2" t="inlineStr"><is><t>mogą być przyczyną fotosensytyzacji</t></is></c><c r="I762" s="2" t="inlineStr" /><c r="J762" s="2" t="inlineStr" /><c r="K762" s="2" t="inlineStr"><is><t>mają nadal szeroki zakres działania przeciwbakteryjnego wobec bakterii tlenowych i mogą być stosowane w empirycznym leczeniu wielu zespołów klinicznych</t></is></c><c r="L762" s="2" t="inlineStr" /><c r="M762" s="2" t="inlineStr" /><c r="N762" s="2" t="inlineStr" /><c r="O762" s="2" t="inlineStr" /><c r="P762" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q762" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="763"><c r="A763" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B763" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C763" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D763" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E763" s="2" t="inlineStr"><is><t>Oseltamiwir należy stosować u nieszczepionych osób z grup ryzyka ciężkiego przebiegu grypy, do których należą:</t></is></c><c r="F763" s="2" t="inlineStr"><is><t>kobiety w ciąży i w 2 tyg. po porodzie</t></is></c><c r="G763" s="2" t="inlineStr"><is><t>dzieci do 2 roku życia</t></is></c><c r="H763" s="2" t="inlineStr"><is><t>osoby z wieku podeszłym &gt;= 65 lat</t></is></c><c r="I763" s="2" t="inlineStr" /><c r="J763" s="2" t="inlineStr" /><c r="K763" s="2" t="inlineStr"><is><t>kobiety karmiące piersią</t></is></c><c r="L763" s="2" t="inlineStr" /><c r="M763" s="2" t="inlineStr" /><c r="N763" s="2" t="inlineStr" /><c r="O763" s="2" t="inlineStr" /><c r="P763" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q763" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="764"><c r="A764" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B764" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C764" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D764" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E764" s="2" t="inlineStr"><is><t>Acyklowir służy do leczenia:</t></is></c><c r="F764" s="2" t="inlineStr"><is><t>opryszczki pospolitej (HSV)</t></is></c><c r="G764" s="2" t="inlineStr"><is><t>ospy wietrznej i półpaśca (VZV)</t></is></c><c r="H764" s="2" t="inlineStr" /><c r="I764" s="2" t="inlineStr" /><c r="J764" s="2" t="inlineStr" /><c r="K764" s="2" t="inlineStr"><is><t>mononukleozy zakaźnej (EBV)</t></is></c><c r="L764" s="2" t="inlineStr"><is><t>cytomegalii (CMV)</t></is></c><c r="M764" s="2" t="inlineStr" /><c r="N764" s="2" t="inlineStr" /><c r="O764" s="2" t="inlineStr" /><c r="P764" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q764" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="765"><c r="A765" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B765" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C765" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D765" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E765" s="2" t="inlineStr"><is><t>W bezinterferonowej terapii przewlekłego wirusowego zapalenia wątroby typu C zastosowanie mają leki przeciwwirusowe działające bezpośrednio (DAA) na wirusa typu C, do których należy:</t></is></c><c r="F765" s="2" t="inlineStr"><is><t>symeprewir</t></is></c><c r="G765" s="2" t="inlineStr"><is><t>ledipaswir</t></is></c><c r="H765" s="2" t="inlineStr" /><c r="I765" s="2" t="inlineStr" /><c r="J765" s="2" t="inlineStr" /><c r="K765" s="2" t="inlineStr"><is><t>zydowudyna</t></is></c><c r="L765" s="2" t="inlineStr"><is><t>lamiwudyna</t></is></c><c r="M765" s="2" t="inlineStr" /><c r="N765" s="2" t="inlineStr" /><c r="O765" s="2" t="inlineStr" /><c r="P765" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q765" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="766"><c r="A766" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B766" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C766" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D766" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E766" s="2" t="inlineStr"><is><t>Metronidazol służy do leczenia:</t></is></c><c r="F766" s="2" t="inlineStr"><is><t>rzęsistkowicy (Trichomonas vaginalis)</t></is></c><c r="G766" s="2" t="inlineStr"><is><t>lambliozy (Giargia lamblia)</t></is></c><c r="H766" s="2" t="inlineStr" /><c r="I766" s="2" t="inlineStr" /><c r="J766" s="2" t="inlineStr" /><c r="K766" s="2" t="inlineStr"><is><t>toksoplazmozy (Toxoplasma godi)</t></is></c><c r="L766" s="2" t="inlineStr"><is><t>pneumocystozy (Pneumocystis jirovecii)</t></is></c><c r="M766" s="2" t="inlineStr" /><c r="N766" s="2" t="inlineStr" /><c r="O766" s="2" t="inlineStr" /><c r="P766" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q766" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="767"><c r="A767" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B767" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C767" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D767" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E767" s="2" t="inlineStr"><is><t>Do leków 2 fazy (kontynuacji) w leczeniu gruźlicy należą:</t></is></c><c r="F767" s="2" t="inlineStr"><is><t>izoniazyd</t></is></c><c r="G767" s="2" t="inlineStr"><is><t>ryfampicyna</t></is></c><c r="H767" s="2" t="inlineStr" /><c r="I767" s="2" t="inlineStr" /><c r="J767" s="2" t="inlineStr" /><c r="K767" s="2" t="inlineStr"><is><t>etambutol</t></is></c><c r="L767" s="2" t="inlineStr"><is><t>pirazynamid</t></is></c><c r="M767" s="2" t="inlineStr" /><c r="N767" s="2" t="inlineStr" /><c r="O767" s="2" t="inlineStr" /><c r="P767" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q767" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="768"><c r="A768" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B768" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C768" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D768" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E768" s="2" t="inlineStr"><is><t>Aktywność wobec dermatofitów ma:</t></is></c><c r="F768" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="G768" s="2" t="inlineStr"><is><t>amorolfina</t></is></c><c r="H768" s="2" t="inlineStr"><is><t>klotrymazol</t></is></c><c r="I768" s="2" t="inlineStr"><is><t>terbinafina</t></is></c><c r="J768" s="2" t="inlineStr" /><c r="K768" s="2" t="inlineStr" /><c r="L768" s="2" t="inlineStr" /><c r="M768" s="2" t="inlineStr" /><c r="N768" s="2" t="inlineStr" /><c r="O768" s="2" t="inlineStr" /><c r="P768" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q768" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="769"><c r="A769" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B769" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C769" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D769" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E769" s="2" t="inlineStr"><is><t>Cechą charakterystyczną dla azoli jest:</t></is></c><c r="F769" s="2" t="inlineStr"><is><t>hamowanie syntezy ergosterolu</t></is></c><c r="G769" s="2" t="inlineStr"><is><t>hamowanie izoenzymów CYP</t></is></c><c r="H769" s="2" t="inlineStr" /><c r="I769" s="2" t="inlineStr" /><c r="J769" s="2" t="inlineStr" /><c r="K769" s="2" t="inlineStr"><is><t>duże podobieństwo parametrów farmakokinetycznych leków tej grupy</t></is></c><c r="L769" s="2" t="inlineStr"><is><t>zależność ekspozycja-efekt typu fT&gt;MIC</t></is></c><c r="M769" s="2" t="inlineStr" /><c r="N769" s="2" t="inlineStr" /><c r="O769" s="2" t="inlineStr" /><c r="P769" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q769" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="770"><c r="A770" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B770" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C770" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D770" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E770" s="2" t="inlineStr"><is><t>Dobrą biodostępność po podaniu doustnym ma:</t></is></c><c r="F770" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="G770" s="2" t="inlineStr"><is><t>worykonazol</t></is></c><c r="H770" s="2" t="inlineStr" /><c r="I770" s="2" t="inlineStr" /><c r="J770" s="2" t="inlineStr" /><c r="K770" s="2" t="inlineStr"><is><t>amfoterycyna B</t></is></c><c r="L770" s="2" t="inlineStr"><is><t>pozakonazol</t></is></c><c r="M770" s="2" t="inlineStr" /><c r="N770" s="2" t="inlineStr" /><c r="O770" s="2" t="inlineStr" /><c r="P770" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q770" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="771"><c r="A771" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B771" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C771" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D771" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E771" s="2" t="inlineStr"><is><t>W kandydozie jamy ustnej (pleśniawkach) zastosować można:</t></is></c><c r="F771" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="G771" s="2" t="inlineStr"><is><t>nystatynę</t></is></c><c r="H771" s="2" t="inlineStr" /><c r="I771" s="2" t="inlineStr" /><c r="J771" s="2" t="inlineStr" /><c r="K771" s="2" t="inlineStr"><is><t>kwas borowy z gliceryną</t></is></c><c r="L771" s="2" t="inlineStr"><is><t>kaspofunginę</t></is></c><c r="M771" s="2" t="inlineStr" /><c r="N771" s="2" t="inlineStr" /><c r="O771" s="2" t="inlineStr" /><c r="P771" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q771" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="772"><c r="A772" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B772" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C772" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D772" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E772" s="2" t="inlineStr"><is><t>Spośród wymienionych glikokortykosteroidów stosowanych wziewnie w leczeniu chorób układu oddechowego w formie proleku dostępny jest:</t></is></c><c r="F772" s="2" t="inlineStr"><is><t>dipropionian beklometazonu</t></is></c><c r="G772" s="2" t="inlineStr"><is><t>cyklezonid</t></is></c><c r="H772" s="2" t="inlineStr" /><c r="I772" s="2" t="inlineStr" /><c r="J772" s="2" t="inlineStr" /><c r="K772" s="2" t="inlineStr"><is><t>budezonid</t></is></c><c r="L772" s="2" t="inlineStr"><is><t>propionian flutykazonu</t></is></c><c r="M772" s="2" t="inlineStr" /><c r="N772" s="2" t="inlineStr" /><c r="O772" s="2" t="inlineStr" /><c r="P772" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q772" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="773"><c r="A773" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B773" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C773" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D773" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E773" s="2" t="inlineStr"><is><t>Długodziałającym lekiem o wpływie na receptory komórkowe jest:</t></is></c><c r="F773" s="2" t="inlineStr"><is><t>bromek umeklidynium</t></is></c><c r="G773" s="2" t="inlineStr" /><c r="H773" s="2" t="inlineStr" /><c r="I773" s="2" t="inlineStr" /><c r="J773" s="2" t="inlineStr" /><c r="K773" s="2" t="inlineStr"><is><t>dornaza alfa</t></is></c><c r="L773" s="2" t="inlineStr"><is><t>nedokromil</t></is></c><c r="M773" s="2" t="inlineStr"><is><t>roflumilast</t></is></c><c r="N773" s="2" t="inlineStr" /><c r="O773" s="2" t="inlineStr" /><c r="P773" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q773" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="774"><c r="A774" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B774" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C774" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D774" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E774" s="2" t="inlineStr"><is><t>Unikalny profil działania klinicznego w swojej grupie farmakologicznej ma:</t></is></c><c r="F774" s="2" t="inlineStr"><is><t>formoterol</t></is></c><c r="G774" s="2" t="inlineStr"><is><t>celiprolol</t></is></c><c r="H774" s="2" t="inlineStr"><is><t>dekstrometorfan</t></is></c><c r="I774" s="2" t="inlineStr" /><c r="J774" s="2" t="inlineStr" /><c r="K774" s="2" t="inlineStr"><is><t>poraktant alfa</t></is></c><c r="L774" s="2" t="inlineStr" /><c r="M774" s="2" t="inlineStr" /><c r="N774" s="2" t="inlineStr" /><c r="O774" s="2" t="inlineStr" /><c r="P774" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q774" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="775"><c r="A775" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B775" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C775" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D775" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E775" s="2" t="inlineStr"><is><t>Do groźnych powikłań po podaniu ramiprylu może dojść w przypadku zastosowania leku u:</t></is></c><c r="F775" s="2" t="inlineStr"><is><t>20-letniej kobiety w ciąży</t></is></c><c r="G775" s="2" t="inlineStr"><is><t>35-letniej kobiety z obustronnym istotnym zwężeniem tętnic nerkowych w przebiegu dysplazji włóknistej</t></is></c><c r="H775" s="2" t="inlineStr" /><c r="I775" s="2" t="inlineStr" /><c r="J775" s="2" t="inlineStr" /><c r="K775" s="2" t="inlineStr"><is><t>70-letniego mężczyzny z POChP</t></is></c><c r="L775" s="2" t="inlineStr"><is><t>50-letniego mężczyzny ze źle kontrolowanym zespołem metabolicznym (otyłość, cukrzyca, nadciśnienie tętnicze, dyslipidemia), aktywnego palacza nikotyny b</t></is></c><c r="M775" s="2" t="inlineStr" /><c r="N775" s="2" t="inlineStr" /><c r="O775" s="2" t="inlineStr" /><c r="P775" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q775" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="776"><c r="A776" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B776" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C776" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D776" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E776" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące współczynnika T/P (trough-to-peak ratio):</t></is></c><c r="F776" s="2" t="inlineStr"><is><t>im większa dawka leku, tym lepszy T/P</t></is></c><c r="G776" s="2" t="inlineStr"><is><t>im dłuższy czas leczenia, tym lepszy T/P</t></is></c><c r="H776" s="2" t="inlineStr"><is><t>pożądany T/P jest większy od 0,75, a optymalny =1,0</t></is></c><c r="I776" s="2" t="inlineStr" /><c r="J776" s="2" t="inlineStr" /><c r="K776" s="2" t="inlineStr"><is><t>jest taki sam dla rozkurczowego i skurczowego ciśnienia tętniczego krwi</t></is></c><c r="L776" s="2" t="inlineStr" /><c r="M776" s="2" t="inlineStr" /><c r="N776" s="2" t="inlineStr" /><c r="O776" s="2" t="inlineStr" /><c r="P776" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q776" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="777"><c r="A777" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B777" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C777" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D777" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E777" s="2" t="inlineStr"><is><t>β – adrenolityki:</t></is></c><c r="F777" s="2" t="inlineStr"><is><t>zwalniają częstość rytmu serca, a przez to zapotrzebowanie serca na tlen</t></is></c><c r="G777" s="2" t="inlineStr" /><c r="H777" s="2" t="inlineStr" /><c r="I777" s="2" t="inlineStr" /><c r="J777" s="2" t="inlineStr" /><c r="K777" s="2" t="inlineStr"><is><t>zmniejszają ciśnienie tętnicze i w efekcie powodują spadek przepływu wieńcowego</t></is></c><c r="L777" s="2" t="inlineStr"><is><t>powodują wzrost stężenia glukozy we krwi i dlatego maskują objawy hipoglikemii</t></is></c><c r="M777" s="2" t="inlineStr"><is><t>powodują skurcz oskrzeli i dlatego są bezwzględnie przeciwwskazane w POChP</t></is></c><c r="N777" s="2" t="inlineStr" /><c r="O777" s="2" t="inlineStr" /><c r="P777" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q777" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="778"><c r="A778" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B778" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C778" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D778" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E778" s="2" t="inlineStr"><is><t>Zaburzenia widzenia powoduje:</t></is></c><c r="F778" s="2" t="inlineStr"><is><t>digoksyna</t></is></c><c r="G778" s="2" t="inlineStr"><is><t>sildenafil</t></is></c><c r="H778" s="2" t="inlineStr"><is><t>iwabradyna</t></is></c><c r="I778" s="2" t="inlineStr" /><c r="J778" s="2" t="inlineStr" /><c r="K778" s="2" t="inlineStr"><is><t>piracetam</t></is></c><c r="L778" s="2" t="inlineStr" /><c r="M778" s="2" t="inlineStr" /><c r="N778" s="2" t="inlineStr" /><c r="O778" s="2" t="inlineStr" /><c r="P778" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q778" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="779"><c r="A779" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B779" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C779" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D779" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E779" s="2" t="inlineStr"><is><t>Do kardiowersji farmakologicznej w migotaniu przedsionków stosuje się:</t></is></c><c r="F779" s="2" t="inlineStr"><is><t>amiodaron</t></is></c><c r="G779" s="2" t="inlineStr"><is><t>propafenon</t></is></c><c r="H779" s="2" t="inlineStr" /><c r="I779" s="2" t="inlineStr" /><c r="J779" s="2" t="inlineStr" /><c r="K779" s="2" t="inlineStr"><is><t>adenozynę</t></is></c><c r="L779" s="2" t="inlineStr"><is><t>lidokainę</t></is></c><c r="M779" s="2" t="inlineStr" /><c r="N779" s="2" t="inlineStr" /><c r="O779" s="2" t="inlineStr" /><c r="P779" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q779" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="780"><c r="A780" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B780" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C780" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D780" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E780" s="2" t="inlineStr"><is><t>Poprzez aktywację białkowej kinazy G via cGMP działa:</t></is></c><c r="F780" s="2" t="inlineStr"><is><t>nitroprusydek sodu</t></is></c><c r="G780" s="2" t="inlineStr"><is><t>sakubitryl</t></is></c><c r="H780" s="2" t="inlineStr"><is><t>riocyguat</t></is></c><c r="I780" s="2" t="inlineStr"><is><t>nesirytyd</t></is></c><c r="J780" s="2" t="inlineStr" /><c r="K780" s="2" t="inlineStr" /><c r="L780" s="2" t="inlineStr" /><c r="M780" s="2" t="inlineStr" /><c r="N780" s="2" t="inlineStr" /><c r="O780" s="2" t="inlineStr" /><c r="P780" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q780" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="781"><c r="A781" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B781" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C781" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D781" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E781" s="2" t="inlineStr"><is><t>Wybierz prawidłowy zestaw lek – wskazanie do stosowania:</t></is></c><c r="F781" s="2" t="inlineStr"><is><t>bupropion – uzależnienie od nikotyny</t></is></c><c r="G781" s="2" t="inlineStr"><is><t>atomoksetyna – ADHD (zespół nadpobudliwości z deficytem uwagi)</t></is></c><c r="H781" s="2" t="inlineStr"><is><t>lamotrygina - profilaktyka zaburzeń afektywnych dwubiegunowych</t></is></c><c r="I781" s="2" t="inlineStr" /><c r="J781" s="2" t="inlineStr" /><c r="K781" s="2" t="inlineStr"><is><t>agomelatyna – bezsenność krótkotrwała</t></is></c><c r="L781" s="2" t="inlineStr" /><c r="M781" s="2" t="inlineStr" /><c r="N781" s="2" t="inlineStr" /><c r="O781" s="2" t="inlineStr" /><c r="P781" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q781" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="782"><c r="A782" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B782" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C782" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D782" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E782" s="2" t="inlineStr"><is><t>Meghan skarżącej się na bezsenność, która związana jest ze stresem wywołanym planowanym wydarzeniem z jej udziałem emitowanym we wszystkich telewizjach świata za 2 tygodnie, przepiszesz:</t></is></c><c r="F782" s="2" t="inlineStr"><is><t>zaleplon</t></is></c><c r="G782" s="2" t="inlineStr" /><c r="H782" s="2" t="inlineStr" /><c r="I782" s="2" t="inlineStr" /><c r="J782" s="2" t="inlineStr" /><c r="K782" s="2" t="inlineStr"><is><t>diazepam</t></is></c><c r="L782" s="2" t="inlineStr"><is><t>mirtazapinę</t></is></c><c r="M782" s="2" t="inlineStr"><is><t>hydroksyzynę</t></is></c><c r="N782" s="2" t="inlineStr" /><c r="O782" s="2" t="inlineStr" /><c r="P782" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q782" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="783"><c r="A783" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B783" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C783" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D783" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E783" s="2" t="inlineStr"><is><t>Pozapsychiatryczne zastosowania leków przeciwdepresyjnych obejmują:</t></is></c><c r="F783" s="2" t="inlineStr"><is><t>ból neuropatyczny</t></is></c><c r="G783" s="2" t="inlineStr"><is><t>bezsenność przewlekłą po niepowodzeniu wprowadzenia zasad higieny snu</t></is></c><c r="H783" s="2" t="inlineStr" /><c r="I783" s="2" t="inlineStr" /><c r="J783" s="2" t="inlineStr" /><c r="K783" s="2" t="inlineStr"><is><t>otępienie naczyniopochodne</t></is></c><c r="L783" s="2" t="inlineStr"><is><t>przerywanie napadów migren</t></is></c><c r="M783" s="2" t="inlineStr" /><c r="N783" s="2" t="inlineStr" /><c r="O783" s="2" t="inlineStr" /><c r="P783" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q783" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="784"><c r="A784" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B784" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C784" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D784" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E784" s="2" t="inlineStr"><is><t>W leczeniu lęku uogólnionego zastosowanie ma:</t></is></c><c r="F784" s="2" t="inlineStr"><is><t>sertralina</t></is></c><c r="G784" s="2" t="inlineStr"><is><t>pregabalina</t></is></c><c r="H784" s="2" t="inlineStr"><is><t>buspiron</t></is></c><c r="I784" s="2" t="inlineStr" /><c r="J784" s="2" t="inlineStr" /><c r="K784" s="2" t="inlineStr"><is><t>klorazepat</t></is></c><c r="L784" s="2" t="inlineStr" /><c r="M784" s="2" t="inlineStr" /><c r="N784" s="2" t="inlineStr" /><c r="O784" s="2" t="inlineStr" /><c r="P784" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q784" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="785"><c r="A785" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B785" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C785" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D785" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E785" s="2" t="inlineStr"><is><t>W początkowym okresie leczenia depresji selektywnymi inhibitorami wychwytu zwrotnego serotoniny:</t></is></c><c r="F785" s="2" t="inlineStr"><is><t>mogą nasilać lęk, choć są uważane za leki przeciwlękowe podczas długotrwałej terapii</t></is></c><c r="G785" s="2" t="inlineStr"><is><t>częściej niż w późniejszym okresie terapii dochodzi do myśli lub prób samobójczych</t></is></c><c r="H785" s="2" t="inlineStr" /><c r="I785" s="2" t="inlineStr" /><c r="J785" s="2" t="inlineStr" /><c r="K785" s="2" t="inlineStr"><is><t>występują fluktuacje nastroju polegające na szybkiej poprawie, ale z okresami gwałtownych pogorszeń</t></is></c><c r="L785" s="2" t="inlineStr"><is><t>stosuje się równocześnie karbamazepinę aby zapobiec przejściu depresji w manię</t></is></c><c r="M785" s="2" t="inlineStr" /><c r="N785" s="2" t="inlineStr" /><c r="O785" s="2" t="inlineStr" /><c r="P785" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q785" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="786"><c r="A786" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B786" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C786" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D786" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E786" s="2" t="inlineStr"><is><t>Pacjentka od wielu lat otrzymuje perazynę, mianseryną i lorazepam. Na tej podstawie można rozpoznać:</t></is></c><c r="F786" s="2" t="inlineStr"><is><t>zaburzenia depresyjno-urojeniowe</t></is></c><c r="G786" s="2" t="inlineStr"><is><t>uzależnienie lekowe</t></is></c><c r="H786" s="2" t="inlineStr" /><c r="I786" s="2" t="inlineStr" /><c r="J786" s="2" t="inlineStr" /><c r="K786" s="2" t="inlineStr"><is><t>dwubiegunową chorobę afektywną</t></is></c><c r="L786" s="2" t="inlineStr"><is><t>fobię społeczną</t></is></c><c r="M786" s="2" t="inlineStr" /><c r="N786" s="2" t="inlineStr" /><c r="O786" s="2" t="inlineStr" /><c r="P786" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q786" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="787"><c r="A787" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B787" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C787" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D787" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E787" s="2" t="inlineStr"><is><t>Układ dopaminowy OUN aktywuje bezpośrednio:</t></is></c><c r="F787" s="2" t="inlineStr"><is><t>ropinirol</t></is></c><c r="G787" s="2" t="inlineStr"><is><t>metylfenidat</t></is></c><c r="H787" s="2" t="inlineStr" /><c r="I787" s="2" t="inlineStr" /><c r="J787" s="2" t="inlineStr" /><c r="K787" s="2" t="inlineStr"><is><t>piracetam</t></is></c><c r="L787" s="2" t="inlineStr"><is><t>kofeina</t></is></c><c r="M787" s="2" t="inlineStr" /><c r="N787" s="2" t="inlineStr" /><c r="O787" s="2" t="inlineStr" /><c r="P787" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q787" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="788"><c r="A788" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B788" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C788" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D788" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E788" s="2" t="inlineStr"><is><t>Przy stosowaniu neuroleptyków największe ryzyko przyrostu masy ciała dotyczy:</t></is></c><c r="F788" s="2" t="inlineStr"><is><t>chlorpromazyny</t></is></c><c r="G788" s="2" t="inlineStr"><is><t>olanzapiny</t></is></c><c r="H788" s="2" t="inlineStr" /><c r="I788" s="2" t="inlineStr" /><c r="J788" s="2" t="inlineStr" /><c r="K788" s="2" t="inlineStr"><is><t>arypiprazolu</t></is></c><c r="L788" s="2" t="inlineStr"><is><t>haloperidolu</t></is></c><c r="M788" s="2" t="inlineStr" /><c r="N788" s="2" t="inlineStr" /><c r="O788" s="2" t="inlineStr" /><c r="P788" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q788" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="789"><c r="A789" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B789" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C789" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D789" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E789" s="2" t="inlineStr"><is><t>Na acetylocholinestarazę ma wpływ:</t></is></c><c r="F789" s="2" t="inlineStr"><is><t>neostygmina</t></is></c><c r="G789" s="2" t="inlineStr"><is><t>donepezil</t></is></c><c r="H789" s="2" t="inlineStr" /><c r="I789" s="2" t="inlineStr" /><c r="J789" s="2" t="inlineStr" /><c r="K789" s="2" t="inlineStr"><is><t>suksametonium</t></is></c><c r="L789" s="2" t="inlineStr"><is><t>tropikamid</t></is></c><c r="M789" s="2" t="inlineStr" /><c r="N789" s="2" t="inlineStr" /><c r="O789" s="2" t="inlineStr" /><c r="P789" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q789" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="790"><c r="A790" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B790" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C790" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D790" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E790" s="2" t="inlineStr"><is><t>Hiponatremia polekowa może być rozpoznana podczas stosowania:</t></is></c><c r="F790" s="2" t="inlineStr"><is><t>torasemidu</t></is></c><c r="G790" s="2" t="inlineStr"><is><t>indapamidu</t></is></c><c r="H790" s="2" t="inlineStr"><is><t>karbamazepiny</t></is></c><c r="I790" s="2" t="inlineStr" /><c r="J790" s="2" t="inlineStr" /><c r="K790" s="2" t="inlineStr"><is><t>tolwaptanu</t></is></c><c r="L790" s="2" t="inlineStr" /><c r="M790" s="2" t="inlineStr" /><c r="N790" s="2" t="inlineStr" /><c r="O790" s="2" t="inlineStr" /><c r="P790" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q790" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="791"><c r="A791" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B791" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C791" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D791" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E791" s="2" t="inlineStr"><is><t>Czy na podstawie informacji o stosowaniu leku można jednoznacznie postawić wymienione rozpoznanie?</t></is></c><c r="F791" s="2" t="inlineStr"><is><t>fingolimod – stwardnienie rozsiane</t></is></c><c r="G791" s="2" t="inlineStr"><is><t>memantyna – choroba Alzheimera</t></is></c><c r="H791" s="2" t="inlineStr" /><c r="I791" s="2" t="inlineStr" /><c r="J791" s="2" t="inlineStr" /><c r="K791" s="2" t="inlineStr"><is><t>kwas walproinowy – padaczka</t></is></c><c r="L791" s="2" t="inlineStr"><is><t>pregabalina – polineuropatia cukrzycowa</t></is></c><c r="M791" s="2" t="inlineStr" /><c r="N791" s="2" t="inlineStr" /><c r="O791" s="2" t="inlineStr" /><c r="P791" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q791" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="792"><c r="A792" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B792" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C792" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D792" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E792" s="2" t="inlineStr"><is><t>Które z powyższych stwierdzeń jest prawdziwe?</t></is></c><c r="F792" s="2" t="inlineStr"><is><t>podczas leczenia takalcytolem należy monitorować stężenie wapnia w moczu</t></is></c><c r="G792" s="2" t="inlineStr"><is><t>metoksalen powinno się podawać 1-2 h przed planowaną ekspozycją na promieniowanie UVA</t></is></c><c r="H792" s="2" t="inlineStr"><is><t>nadtlenek benzoilu ma zastosowanie w leczeniu trądziku</t></is></c><c r="I792" s="2" t="inlineStr" /><c r="J792" s="2" t="inlineStr" /><c r="K792" s="2" t="inlineStr"><is><t>podczas stosowania acytretyny skuteczną antykoncepcję należy stosować przez miesiąc po zakończeniu terapii</t></is></c><c r="L792" s="2" t="inlineStr" /><c r="M792" s="2" t="inlineStr" /><c r="N792" s="2" t="inlineStr" /><c r="O792" s="2" t="inlineStr" /><c r="P792" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q792" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="793"><c r="A793" s="2" t="inlineStr"><is><t>LEKI ROŚLINNE I SUPLEMENTY</t></is></c><c r="B793" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C793" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D793" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E793" s="2" t="inlineStr"><is><t>Doping genetyczny może dotyczyć genu kodującego:</t></is></c><c r="F793" s="2" t="inlineStr"><is><t>enzym konwertujący angiotensynę</t></is></c><c r="G793" s="2" t="inlineStr"><is><t>erytropoetynę</t></is></c><c r="H793" s="2" t="inlineStr"><is><t>kolagen</t></is></c><c r="I793" s="2" t="inlineStr"><is><t>hormon wzrostu</t></is></c><c r="J793" s="2" t="inlineStr" /><c r="K793" s="2" t="inlineStr" /><c r="L793" s="2" t="inlineStr" /><c r="M793" s="2" t="inlineStr" /><c r="N793" s="2" t="inlineStr" /><c r="O793" s="2" t="inlineStr" /><c r="P793" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q793" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="794"><c r="A794" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B794" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C794" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D794" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E794" s="2" t="inlineStr"><is><t>Terapia genowa w okulistyce ma zastosowanie w leczeniu:</t></is></c><c r="F794" s="2" t="inlineStr"><is><t>zwyrodnienia barwnikowego siatkówki (retinitis pigmentosa)</t></is></c><c r="G794" s="2" t="inlineStr" /><c r="H794" s="2" t="inlineStr" /><c r="I794" s="2" t="inlineStr" /><c r="J794" s="2" t="inlineStr" /><c r="K794" s="2" t="inlineStr"><is><t>jaskry</t></is></c><c r="L794" s="2" t="inlineStr"><is><t>zapalenia współczulnego oka</t></is></c><c r="M794" s="2" t="inlineStr"><is><t>choroby Besta</t></is></c><c r="N794" s="2" t="inlineStr" /><c r="O794" s="2" t="inlineStr" /><c r="P794" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q794" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="795"><c r="A795" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B795" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C795" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D795" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E795" s="2" t="inlineStr"><is><t>W leczeniu astmy używane są wziewne postaci:</t></is></c><c r="F795" s="2" t="inlineStr"><is><t>propionianu flutykazonu</t></is></c><c r="G795" s="2" t="inlineStr"><is><t>indakaterolu</t></is></c><c r="H795" s="2" t="inlineStr" /><c r="I795" s="2" t="inlineStr" /><c r="J795" s="2" t="inlineStr" /><c r="K795" s="2" t="inlineStr"><is><t>montelukastu</t></is></c><c r="L795" s="2" t="inlineStr"><is><t>acetylocysteiny</t></is></c><c r="M795" s="2" t="inlineStr" /><c r="N795" s="2" t="inlineStr" /><c r="O795" s="2" t="inlineStr" /><c r="P795" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q795" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="796"><c r="A796" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B796" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C796" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D796" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E796" s="2" t="inlineStr"><is><t>U małego dziecka wygodną formą podania leku wziewnego jest:</t></is></c><c r="F796" s="2" t="inlineStr"><is><t>pomocnicze użycie komory inhalacyjnej, tzw. spacera</t></is></c><c r="G796" s="2" t="inlineStr"><is><t>nebulizacja</t></is></c><c r="H796" s="2" t="inlineStr" /><c r="I796" s="2" t="inlineStr" /><c r="J796" s="2" t="inlineStr" /><c r="K796" s="2" t="inlineStr"><is><t>inhalacja z inhalatora suchego proszku</t></is></c><c r="L796" s="2" t="inlineStr"><is><t>inhalacja z dozownika ciśnieniowego</t></is></c><c r="M796" s="2" t="inlineStr" /><c r="N796" s="2" t="inlineStr" /><c r="O796" s="2" t="inlineStr" /><c r="P796" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q796" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="797"><c r="A797" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B797" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C797" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D797" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E797" s="2" t="inlineStr"><is><t>Chorzy na pierwotne nadciśnienie tętnicze z towarzyszącą cukrzycą największe korzyści osiągają z zastosowania:</t></is></c><c r="F797" s="2" t="inlineStr"><is><t>ramiprylu</t></is></c><c r="G797" s="2" t="inlineStr"><is><t>telmisartanu</t></is></c><c r="H797" s="2" t="inlineStr" /><c r="I797" s="2" t="inlineStr" /><c r="J797" s="2" t="inlineStr" /><c r="K797" s="2" t="inlineStr"><is><t>metoprololu</t></is></c><c r="L797" s="2" t="inlineStr"><is><t>hydrochlorotiazydu</t></is></c><c r="M797" s="2" t="inlineStr" /><c r="N797" s="2" t="inlineStr" /><c r="O797" s="2" t="inlineStr" /><c r="P797" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q797" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="798"><c r="A798" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B798" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C798" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D798" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E798" s="2" t="inlineStr"><is><t>Istotnym działaniem niepożądanym inhibitorów konwertazy angiotensyny jest:</t></is></c><c r="F798" s="2" t="inlineStr"><is><t>kaszel</t></is></c><c r="G798" s="2" t="inlineStr"><is><t>obrzęk naczynioruchowy</t></is></c><c r="H798" s="2" t="inlineStr" /><c r="I798" s="2" t="inlineStr" /><c r="J798" s="2" t="inlineStr" /><c r="K798" s="2" t="inlineStr"><is><t>hipokaliemia</t></is></c><c r="L798" s="2" t="inlineStr"><is><t>nasilenie białkomoczu</t></is></c><c r="M798" s="2" t="inlineStr" /><c r="N798" s="2" t="inlineStr" /><c r="O798" s="2" t="inlineStr" /><c r="P798" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q798" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="799"><c r="A799" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B799" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C799" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D799" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E799" s="2" t="inlineStr"><is><t>Wybierz prawidłowe pary lek – efekt działania:</t></is></c><c r="F799" s="2" t="inlineStr"><is><t>torasemid - hiperurykemia</t></is></c><c r="G799" s="2" t="inlineStr"><is><t>indapamid - hiponatremia</t></is></c><c r="H799" s="2" t="inlineStr" /><c r="I799" s="2" t="inlineStr" /><c r="J799" s="2" t="inlineStr" /><c r="K799" s="2" t="inlineStr"><is><t>mannitol – hiperglikemia</t></is></c><c r="L799" s="2" t="inlineStr"><is><t>eplerenon - hipokaliemia</t></is></c><c r="M799" s="2" t="inlineStr" /><c r="N799" s="2" t="inlineStr" /><c r="O799" s="2" t="inlineStr" /><c r="P799" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q799" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="800"><c r="A800" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B800" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C800" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D800" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E800" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące digoksyny:</t></is></c><c r="F800" s="2" t="inlineStr"><is><t>jest wskazana u pacjentów z niewydolnością serca i migotaniem przedsionków</t></is></c><c r="G800" s="2" t="inlineStr"><is><t>zmniejsza chorobowość pacjentów z niewydolnością serca</t></is></c><c r="H800" s="2" t="inlineStr" /><c r="I800" s="2" t="inlineStr" /><c r="J800" s="2" t="inlineStr" /><c r="K800" s="2" t="inlineStr"><is><t>poprawia przeżycie chorych z niewydolnością serca</t></is></c><c r="L800" s="2" t="inlineStr"><is><t>jest pozbawiona działania proarytmicznego</t></is></c><c r="M800" s="2" t="inlineStr" /><c r="N800" s="2" t="inlineStr" /><c r="O800" s="2" t="inlineStr" /><c r="P800" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q800" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="801"><c r="A801" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B801" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C801" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D801" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E801" s="2" t="inlineStr"><is><t>Wskaż prawdziwe zdanie dotyczące leczenia niewydolności serca:</t></is></c><c r="F801" s="2" t="inlineStr"><is><t>enalapryl przez zniesienie niekorzystnej adaptacji zmniejsza umieralność chorych ze skurczową niewydolnością serca</t></is></c><c r="G801" s="2" t="inlineStr"><is><t>karwedilol przez zniesienie niekorzystnej adaptacji zmniejsza umieralność chorych ze skurczową niewydolnością serca</t></is></c><c r="H801" s="2" t="inlineStr"><is><t>leki moczopędne są zalecane w celu zmniejszenia objawów i poprawy wydolności wysiłkowej u pacjentów z objawami zastoju</t></is></c><c r="I801" s="2" t="inlineStr" /><c r="J801" s="2" t="inlineStr" /><c r="K801" s="2" t="inlineStr"><is><t>statyny powinny być stosowane rutynowo u wszystkich chorych z niewydolnością mięśnia sercowego</t></is></c><c r="L801" s="2" t="inlineStr" /><c r="M801" s="2" t="inlineStr" /><c r="N801" s="2" t="inlineStr" /><c r="O801" s="2" t="inlineStr" /><c r="P801" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q801" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="802"><c r="A802" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B802" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C802" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D802" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E802" s="2" t="inlineStr"><is><t>Do leków przeciwskazanych u pacjentów z niewydolnością serca należy:</t></is></c><c r="F802" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="G802" s="2" t="inlineStr"><is><t>ketoprofen</t></is></c><c r="H802" s="2" t="inlineStr" /><c r="I802" s="2" t="inlineStr" /><c r="J802" s="2" t="inlineStr" /><c r="K802" s="2" t="inlineStr"><is><t>nebiwolol</t></is></c><c r="L802" s="2" t="inlineStr"><is><t>iwabradyna</t></is></c><c r="M802" s="2" t="inlineStr" /><c r="N802" s="2" t="inlineStr" /><c r="O802" s="2" t="inlineStr" /><c r="P802" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q802" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="803"><c r="A803" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B803" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C803" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D803" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E803" s="2" t="inlineStr"><is><t>W postaci naczynioskurczowej choroby niedokrwiennej serca przeciwwskazane jest stosowanie:</t></is></c><c r="F803" s="2" t="inlineStr"><is><t>metoprololu</t></is></c><c r="G803" s="2" t="inlineStr" /><c r="H803" s="2" t="inlineStr" /><c r="I803" s="2" t="inlineStr" /><c r="J803" s="2" t="inlineStr" /><c r="K803" s="2" t="inlineStr"><is><t>diltiazemu</t></is></c><c r="L803" s="2" t="inlineStr"><is><t>diazotanu izosorbidu</t></is></c><c r="M803" s="2" t="inlineStr"><is><t>werapamilu</t></is></c><c r="N803" s="2" t="inlineStr" /><c r="O803" s="2" t="inlineStr" /><c r="P803" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q803" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="804"><c r="A804" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B804" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C804" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D804" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E804" s="2" t="inlineStr"><is><t>Do działań niepożądanych amiodaronu należy:</t></is></c><c r="F804" s="2" t="inlineStr"><is><t>hipotonia</t></is></c><c r="G804" s="2" t="inlineStr"><is><t>fotosensytyzacja</t></is></c><c r="H804" s="2" t="inlineStr"><is><t>śródmiąższowe zapalenie płuc</t></is></c><c r="I804" s="2" t="inlineStr" /><c r="J804" s="2" t="inlineStr" /><c r="K804" s="2" t="inlineStr"><is><t>tachykardia</t></is></c><c r="L804" s="2" t="inlineStr" /><c r="M804" s="2" t="inlineStr" /><c r="N804" s="2" t="inlineStr" /><c r="O804" s="2" t="inlineStr" /><c r="P804" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q804" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="805"><c r="A805" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B805" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C805" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D805" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E805" s="2" t="inlineStr"><is><t>Lekiem rozkurczającym tętnice pozawieńcowe jest:</t></is></c><c r="F805" s="2" t="inlineStr"><is><t>nicergolina</t></is></c><c r="G805" s="2" t="inlineStr"><is><t>alprostadyl</t></is></c><c r="H805" s="2" t="inlineStr"><is><t>fentolamina</t></is></c><c r="I805" s="2" t="inlineStr"><is><t>cilostazol</t></is></c><c r="J805" s="2" t="inlineStr" /><c r="K805" s="2" t="inlineStr" /><c r="L805" s="2" t="inlineStr" /><c r="M805" s="2" t="inlineStr" /><c r="N805" s="2" t="inlineStr" /><c r="O805" s="2" t="inlineStr" /><c r="P805" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q805" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="806"><c r="A806" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B806" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C806" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D806" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E806" s="2" t="inlineStr"><is><t>Midazolam może być stosowany zgodnie z aktualną wiedzą:</t></is></c><c r="F806" s="2" t="inlineStr"><is><t>doustnie do sedacji w premedykacji przed zabiegami chirurgicznymi</t></is></c><c r="G806" s="2" t="inlineStr"><is><t>dożylnie w sedacji do nieprzyjemnych zabiegów diagnostycznych</t></is></c><c r="H806" s="2" t="inlineStr"><is><t>dożylnie w długotrwałej sedacji na oddziale intensywnej opieki medycznej</t></is></c><c r="I806" s="2" t="inlineStr" /><c r="J806" s="2" t="inlineStr" /><c r="K806" s="2" t="inlineStr"><is><t>doustnie w przewlekłym leczeniu bezsenności</t></is></c><c r="L806" s="2" t="inlineStr" /><c r="M806" s="2" t="inlineStr" /><c r="N806" s="2" t="inlineStr" /><c r="O806" s="2" t="inlineStr" /><c r="P806" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q806" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="807"><c r="A807" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B807" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C807" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D807" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E807" s="2" t="inlineStr"><is><t>W zaburzeniach lękowych można racjonalnie zastosować:</t></is></c><c r="F807" s="2" t="inlineStr"><is><t>escitalopram</t></is></c><c r="G807" s="2" t="inlineStr"><is><t>alprazolam</t></is></c><c r="H807" s="2" t="inlineStr" /><c r="I807" s="2" t="inlineStr" /><c r="J807" s="2" t="inlineStr" /><c r="K807" s="2" t="inlineStr"><is><t>baklofen</t></is></c><c r="L807" s="2" t="inlineStr"><is><t>moklobemid</t></is></c><c r="M807" s="2" t="inlineStr" /><c r="N807" s="2" t="inlineStr" /><c r="O807" s="2" t="inlineStr" /><c r="P807" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q807" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="808"><c r="A808" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B808" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C808" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D808" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E808" s="2" t="inlineStr"><is><t>Flumazenil to:</t></is></c><c r="F808" s="2" t="inlineStr"><is><t>antagonista receptora benzodiazepinowego</t></is></c><c r="G808" s="2" t="inlineStr"><is><t>antidotum w przedawkowaniu benzodiazepin</t></is></c><c r="H808" s="2" t="inlineStr" /><c r="I808" s="2" t="inlineStr" /><c r="J808" s="2" t="inlineStr" /><c r="K808" s="2" t="inlineStr"><is><t>odwrotny agonista receptora GABA-A</t></is></c><c r="L808" s="2" t="inlineStr"><is><t>antidotum w przedawkowaniu trójpierścieniowych leków przeciwdepresyjnych</t></is></c><c r="M808" s="2" t="inlineStr" /><c r="N808" s="2" t="inlineStr" /><c r="O808" s="2" t="inlineStr" /><c r="P808" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q808" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="809"><c r="A809" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B809" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C809" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D809" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E809" s="2" t="inlineStr"><is><t>Do krótkodziałających benzodiazepin należy:</t></is></c><c r="F809" s="2" t="inlineStr"><is><t>midazolam</t></is></c><c r="G809" s="2" t="inlineStr"><is><t>triazolam</t></is></c><c r="H809" s="2" t="inlineStr" /><c r="I809" s="2" t="inlineStr" /><c r="J809" s="2" t="inlineStr" /><c r="K809" s="2" t="inlineStr"><is><t>diazepam</t></is></c><c r="L809" s="2" t="inlineStr"><is><t>flunitrazepam</t></is></c><c r="M809" s="2" t="inlineStr" /><c r="N809" s="2" t="inlineStr" /><c r="O809" s="2" t="inlineStr" /><c r="P809" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q809" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="810"><c r="A810" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B810" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C810" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D810" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E810" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek-mechanizm działania:</t></is></c><c r="F810" s="2" t="inlineStr"><is><t>mirtazapina – antagonista receptorów adrenergicznych alfa2 i serotoninowych 5HT2a, 5HT2c, 5HT3</t></is></c><c r="G810" s="2" t="inlineStr" /><c r="H810" s="2" t="inlineStr" /><c r="I810" s="2" t="inlineStr" /><c r="J810" s="2" t="inlineStr" /><c r="K810" s="2" t="inlineStr"><is><t>reboksetyna – hamowanie wychwytu zwrotnego serotoniny i noradrenaliny</t></is></c><c r="L810" s="2" t="inlineStr"><is><t>tianeptyna – selektywne hamowanie wychwytu zwrotnego noradrenaliny</t></is></c><c r="M810" s="2" t="inlineStr"><is><t>wenlafaksyna – nasilanie presynaptycznego wychwytu zwrotnego serotoniny</t></is></c><c r="N810" s="2" t="inlineStr" /><c r="O810" s="2" t="inlineStr" /><c r="P810" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q810" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="811"><c r="A811" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B811" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C811" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D811" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E811" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek – mechanizm działania:</t></is></c><c r="F811" s="2" t="inlineStr"><is><t>Roflumilast – inhibitor fosfodiestrazy 4</t></is></c><c r="G811" s="2" t="inlineStr" /><c r="H811" s="2" t="inlineStr" /><c r="I811" s="2" t="inlineStr" /><c r="J811" s="2" t="inlineStr" /><c r="K811" s="2" t="inlineStr"><is><t>Indakaterol – nieselektywny agonista receptorów beta-adrenergicznych</t></is></c><c r="L811" s="2" t="inlineStr"><is><t>Tiotropium - długodziałający gonista receptorów M3</t></is></c><c r="M811" s="2" t="inlineStr"><is><t>Omalizumab - przeciwciało monoklonalne przeciw ludzkim przeciwciałom klasy IgA</t></is></c><c r="N811" s="2" t="inlineStr" /><c r="O811" s="2" t="inlineStr" /><c r="P811" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q811" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="812"><c r="A812" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B812" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C812" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D812" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E812" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie lek – mechanizm działania:</t></is></c><c r="F812" s="2" t="inlineStr"><is><t>Iwabradyna – zahamowanie prądu potasowego w węźle przedsionkowo￾komorowym</t></is></c><c r="G812" s="2" t="inlineStr"><is><t>Sakubitril – zahamowanie aktywności neprylizyny</t></is></c><c r="H812" s="2" t="inlineStr"><is><t>Riociguat – aktywacja cyklazy adenylowej</t></is></c><c r="I812" s="2" t="inlineStr"><is><t>Digoksyna – aktywacja wymiennika sodowo-wapniowego</t></is></c><c r="J812" s="2" t="inlineStr" /><c r="K812" s="2" t="inlineStr" /><c r="L812" s="2" t="inlineStr" /><c r="M812" s="2" t="inlineStr" /><c r="N812" s="2" t="inlineStr" /><c r="O812" s="2" t="inlineStr" /><c r="P812" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q812" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="813"><c r="A813" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B813" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C813" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D813" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E813" s="2" t="inlineStr"><is><t>Do działań niepożądanych neuroleptyków zalicza się:</t></is></c><c r="F813" s="2" t="inlineStr"><is><t>dyskinezy</t></is></c><c r="G813" s="2" t="inlineStr"><is><t>dysfunkcje seksualne</t></is></c><c r="H813" s="2" t="inlineStr" /><c r="I813" s="2" t="inlineStr" /><c r="J813" s="2" t="inlineStr" /><c r="K813" s="2" t="inlineStr"><is><t>skłonność do hazardu</t></is></c><c r="L813" s="2" t="inlineStr"><is><t>somnambulizm (sennowłóctwo)</t></is></c><c r="M813" s="2" t="inlineStr" /><c r="N813" s="2" t="inlineStr" /><c r="O813" s="2" t="inlineStr" /><c r="P813" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q813" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="814"><c r="A814" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B814" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C814" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D814" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E814" s="2" t="inlineStr"><is><t>Stężenie cholesterolu LDL w surowicy zwiększa:</t></is></c><c r="F814" s="2" t="inlineStr"><is><t>olanzapina</t></is></c><c r="G814" s="2" t="inlineStr"><is><t>rysperydon</t></is></c><c r="H814" s="2" t="inlineStr"><is><t>kwetiapina</t></is></c><c r="I814" s="2" t="inlineStr" /><c r="J814" s="2" t="inlineStr" /><c r="K814" s="2" t="inlineStr"><is><t>zyprazydon</t></is></c><c r="L814" s="2" t="inlineStr" /><c r="M814" s="2" t="inlineStr" /><c r="N814" s="2" t="inlineStr" /><c r="O814" s="2" t="inlineStr" /><c r="P814" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q814" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="815"><c r="A815" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B815" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C815" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D815" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E815" s="2" t="inlineStr"><is><t>Przez wpływ na prąd sodowy działa:</t></is></c><c r="F815" s="2" t="inlineStr"><is><t>okskarbazepina</t></is></c><c r="G815" s="2" t="inlineStr"><is><t>kwas walproinowy</t></is></c><c r="H815" s="2" t="inlineStr"><is><t>lamotrygina</t></is></c><c r="I815" s="2" t="inlineStr" /><c r="J815" s="2" t="inlineStr" /><c r="K815" s="2" t="inlineStr"><is><t>pregabalina</t></is></c><c r="L815" s="2" t="inlineStr" /><c r="M815" s="2" t="inlineStr" /><c r="N815" s="2" t="inlineStr" /><c r="O815" s="2" t="inlineStr" /><c r="P815" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q815" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="816"><c r="A816" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B816" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C816" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D816" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E816" s="2" t="inlineStr"><is><t>W profilaktyce migreny wykazano skuteczność:</t></is></c><c r="F816" s="2" t="inlineStr"><is><t>kwasu walproinowego</t></is></c><c r="G816" s="2" t="inlineStr"><is><t>toksyny botulinowej (w migrenie występującej co najmniej 14 dni w miesiącu)</t></is></c><c r="H816" s="2" t="inlineStr"><is><t>topiramatu</t></is></c><c r="I816" s="2" t="inlineStr"><is><t>propranololu</t></is></c><c r="J816" s="2" t="inlineStr" /><c r="K816" s="2" t="inlineStr" /><c r="L816" s="2" t="inlineStr" /><c r="M816" s="2" t="inlineStr" /><c r="N816" s="2" t="inlineStr" /><c r="O816" s="2" t="inlineStr" /><c r="P816" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q816" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="817"><c r="A817" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B817" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C817" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D817" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E817" s="2" t="inlineStr"><is><t>W leczeniu bólu neuropatycznego stosuje się:</t></is></c><c r="F817" s="2" t="inlineStr"><is><t>wenlafaksynę</t></is></c><c r="G817" s="2" t="inlineStr"><is><t>duloksetynę</t></is></c><c r="H817" s="2" t="inlineStr"><is><t>amitryptylinę</t></is></c><c r="I817" s="2" t="inlineStr" /><c r="J817" s="2" t="inlineStr" /><c r="K817" s="2" t="inlineStr"><is><t>tianeptynę</t></is></c><c r="L817" s="2" t="inlineStr" /><c r="M817" s="2" t="inlineStr" /><c r="N817" s="2" t="inlineStr" /><c r="O817" s="2" t="inlineStr" /><c r="P817" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q817" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="818"><c r="A818" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B818" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C818" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D818" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E818" s="2" t="inlineStr"><is><t>W leczeniu łuszczycy stosuje się:</t></is></c><c r="F818" s="2" t="inlineStr"><is><t>preparaty dziegciowe</t></is></c><c r="G818" s="2" t="inlineStr"><is><t>adapalen</t></is></c><c r="H818" s="2" t="inlineStr"><is><t>adalimumab</t></is></c><c r="I818" s="2" t="inlineStr" /><c r="J818" s="2" t="inlineStr" /><c r="K818" s="2" t="inlineStr"><is><t>kwas azelainowy</t></is></c><c r="L818" s="2" t="inlineStr" /><c r="M818" s="2" t="inlineStr" /><c r="N818" s="2" t="inlineStr" /><c r="O818" s="2" t="inlineStr" /><c r="P818" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q818" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="819"><c r="A819" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B819" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C819" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D819" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E819" s="2" t="inlineStr"><is><t>Działanie niepożądane sterydów anabolicznych to:</t></is></c><c r="F819" s="2" t="inlineStr"><is><t>uszkodzenie ścięgien</t></is></c><c r="G819" s="2" t="inlineStr"><is><t>wzrost hematokrytu</t></is></c><c r="H819" s="2" t="inlineStr"><is><t>łysienie</t></is></c><c r="I819" s="2" t="inlineStr"><is><t>ginekomastia</t></is></c><c r="J819" s="2" t="inlineStr" /><c r="K819" s="2" t="inlineStr" /><c r="L819" s="2" t="inlineStr" /><c r="M819" s="2" t="inlineStr" /><c r="N819" s="2" t="inlineStr" /><c r="O819" s="2" t="inlineStr" /><c r="P819" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q819" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="820"><c r="A820" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B820" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C820" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D820" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E820" s="2" t="inlineStr"><is><t>Kwas walproinowy:</t></is></c><c r="F820" s="2" t="inlineStr"><is><t>może powodować zwiększenie masy ciała</t></is></c><c r="G820" s="2" t="inlineStr"><is><t>nie powinien być stosowany u ciężarnych</t></is></c><c r="H820" s="2" t="inlineStr"><is><t>może być zastosowany w profilaktyce dwubiegunowej choroby afektywnej</t></is></c><c r="I820" s="2" t="inlineStr" /><c r="J820" s="2" t="inlineStr" /><c r="K820" s="2" t="inlineStr"><is><t>jest induktorem izoenzymów CYP</t></is></c><c r="L820" s="2" t="inlineStr" /><c r="M820" s="2" t="inlineStr" /><c r="N820" s="2" t="inlineStr" /><c r="O820" s="2" t="inlineStr" /><c r="P820" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q820" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="821"><c r="A821" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B821" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C821" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D821" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E821" s="2" t="inlineStr"><is><t>W terapii jaskry pierwotnej otwartego kąta można zastosować:</t></is></c><c r="F821" s="2" t="inlineStr"><is><t>timolol</t></is></c><c r="G821" s="2" t="inlineStr"><is><t>dorzolamid</t></is></c><c r="H821" s="2" t="inlineStr"><is><t>betaksolol</t></is></c><c r="I821" s="2" t="inlineStr"><is><t>latanoprost</t></is></c><c r="J821" s="2" t="inlineStr" /><c r="K821" s="2" t="inlineStr" /><c r="L821" s="2" t="inlineStr" /><c r="M821" s="2" t="inlineStr" /><c r="N821" s="2" t="inlineStr" /><c r="O821" s="2" t="inlineStr" /><c r="P821" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q821" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="822"><c r="A822" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B822" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C822" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D822" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E822" s="2" t="inlineStr"><is><t>Wskazaniem do stosowania bisfosfonianów jest:</t></is></c><c r="F822" s="2" t="inlineStr"><is><t>osteoporoza posteroidowa</t></is></c><c r="G822" s="2" t="inlineStr"><is><t>ból z powodu osteolitycznych przerzutów nowotworowych do kości</t></is></c><c r="H822" s="2" t="inlineStr" /><c r="I822" s="2" t="inlineStr" /><c r="J822" s="2" t="inlineStr" /><c r="K822" s="2" t="inlineStr"><is><t>ciężka hiperkaliemia</t></is></c><c r="L822" s="2" t="inlineStr"><is><t>ciężka hipokalcemia</t></is></c><c r="M822" s="2" t="inlineStr" /><c r="N822" s="2" t="inlineStr" /><c r="O822" s="2" t="inlineStr" /><c r="P822" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q822" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="823"><c r="A823" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B823" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C823" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D823" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E823" s="2" t="inlineStr"><is><t>Korzystne cechy leku przeciwhistaminowego stosowanego do leczenia przewlekłego alergicznego nieżytu nosa to:</t></is></c><c r="F823" s="2" t="inlineStr"><is><t>utrudnione przechodzenie do ośrodkowego układu nerwowego</t></is></c><c r="G823" s="2" t="inlineStr" /><c r="H823" s="2" t="inlineStr" /><c r="I823" s="2" t="inlineStr" /><c r="J823" s="2" t="inlineStr" /><c r="K823" s="2" t="inlineStr"><is><t>krótki czas działania 3-6 godzin</t></is></c><c r="L823" s="2" t="inlineStr"><is><t>działanie cholinolityczne</t></is></c><c r="M823" s="2" t="inlineStr"><is><t>zdolność do kumulacji w tkankach obwodowych</t></is></c><c r="N823" s="2" t="inlineStr" /><c r="O823" s="2" t="inlineStr" /><c r="P823" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q823" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="824"><c r="A824" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B824" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C824" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D824" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E824" s="2" t="inlineStr"><is><t>Wskaż prawidłowe ordynacje lekarskie:</t></is></c><c r="F824" s="2" t="inlineStr"><is><t>biegunka o etiologii Clostridium difficile o nieciężkim przebiegu – metronidazol przez 10 dni</t></is></c><c r="G824" s="2" t="inlineStr" /><c r="H824" s="2" t="inlineStr" /><c r="I824" s="2" t="inlineStr" /><c r="J824" s="2" t="inlineStr" /><c r="K824" s="2" t="inlineStr"><is><t>nosicielstwo Klebsiella pneumoniae ESBL (+) w przewodzie pokarmowym – meropenem przez 5 dni</t></is></c><c r="L824" s="2" t="inlineStr"><is><t>posiew krwi Streptococcus epidermidis oporny na metycylinę (MR) w butelce tlenowej i beztlenowej u pacjenta niegorączkującego, leukocyty = 8,9 G/l (N 4-10 G/L), CRP – 100 mg/l (N do 10 mg/l), prokalcytonina = 0,01 ng/ml (N do 0,5ng/ml) – wankomycyna przez 3 tygodnie</t></is></c><c r="M824" s="2" t="inlineStr"><is><t>posiew moczu Escherichia coli &gt; 10 5 jtk/ml (cfu/ml) u pacjentki z objawami dysurycznymi – imipenem + cilastatyna z powodu najniższej wartości MIC wg antybiogramu przez 3 dni</t></is></c><c r="N824" s="2" t="inlineStr" /><c r="O824" s="2" t="inlineStr" /><c r="P824" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q824" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="825"><c r="A825" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B825" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C825" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D825" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E825" s="2" t="inlineStr"><is><t>Kobieta z zakażeniem Enteroccocus faecium opornym na glikopeptydy (VRE) jest leczona lekiem przeciwbakteryjnym wiążącym się z jednostką 50S rybosomu bakteryjnego. Zaznacz prawdziwe informacje dotyczące tego leku:</t></is></c><c r="F825" s="2" t="inlineStr"><is><t>podczas jego stosowania &gt;10 dni może dojść do rozwoju trombocytopenii</t></is></c><c r="G825" s="2" t="inlineStr"><is><t>może być bezpiecznie stosowany u pacjentów leczonych lekami blokującymi CYP3A4, ponieważ nie wchodzi z nimi w interakcje</t></is></c><c r="H825" s="2" t="inlineStr" /><c r="I825" s="2" t="inlineStr" /><c r="J825" s="2" t="inlineStr" /><c r="K825" s="2" t="inlineStr"><is><t>jego działanie przeciwbakteryjne zależy od stężenia maksymalnego</t></is></c><c r="L825" s="2" t="inlineStr"><is><t>może być bezpiecznie zastosowany w trakcie leczenia inhibitorami wychwytu zwrotnego serotoniny, ponieważ nie wchodzi z nimi w interakcje</t></is></c><c r="M825" s="2" t="inlineStr" /><c r="N825" s="2" t="inlineStr" /><c r="O825" s="2" t="inlineStr" /><c r="P825" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q825" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="826"><c r="A826" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B826" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C826" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D826" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E826" s="2" t="inlineStr"><is><t>60-letnia kobieta z domowym zapaleniem płuc, w skali CURB-65 = 0 pkt jest leczona zgodnie ze standardem postępowania uwzględniającym dominującą etiologię tego zakażenia u osób dorosłych. Zaznacz prawdziwe informacje dotyczące tego leczenia:</t></is></c><c r="F826" s="2" t="inlineStr"><is><t>wymaga stałych optymalnych przedziałów dawkowania w ciągu całej doby</t></is></c><c r="G826" s="2" t="inlineStr"><is><t>w razie nadwrażliwości na leczenie początkowe w wywiadach wskazane jest zastosowanie lewofloksacyny lub moksyfloksacyny</t></is></c><c r="H826" s="2" t="inlineStr" /><c r="I826" s="2" t="inlineStr" /><c r="J826" s="2" t="inlineStr" /><c r="K826" s="2" t="inlineStr"><is><t>konieczne jest leczenie skojarzone 2 lekami przeciwbakteryjnymi o różnych mechanizmach działania</t></is></c><c r="L826" s="2" t="inlineStr"><is><t>powinno trwać co najmniej 21 dni</t></is></c><c r="M826" s="2" t="inlineStr" /><c r="N826" s="2" t="inlineStr" /><c r="O826" s="2" t="inlineStr" /><c r="P826" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q826" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="827"><c r="A827" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B827" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C827" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D827" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E827" s="2" t="inlineStr"><is><t>Amoksycylina z kwasem klawulanowym jest powszechnie stosowanym połączeniem antybiotykowym, które ma jednak ograniczenia. Wskaż istotne wady tego połączenia:</t></is></c><c r="F827" s="2" t="inlineStr"><is><t>aktywność wobec fizjologicznego mikrobiomu przewodu pokarmowego człowieka</t></is></c><c r="G827" s="2" t="inlineStr"><is><t>zależne od kwasu klawulanowego biegunka i uszkodzenie wątroby</t></is></c><c r="H827" s="2" t="inlineStr"><is><t>konieczność korekty dawki proporcjonalnie do eGFR (wskaźnika filtracji kłębuszkowej)</t></is></c><c r="I827" s="2" t="inlineStr" /><c r="J827" s="2" t="inlineStr" /><c r="K827" s="2" t="inlineStr"><is><t>ograniczona biodostępność po podaniu doustnym</t></is></c><c r="L827" s="2" t="inlineStr" /><c r="M827" s="2" t="inlineStr" /><c r="N827" s="2" t="inlineStr" /><c r="O827" s="2" t="inlineStr" /><c r="P827" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q827" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="828"><c r="A828" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B828" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C828" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D828" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E828" s="2" t="inlineStr"><is><t>W zakażeniach dermatofitami stosuje się:</t></is></c><c r="F828" s="2" t="inlineStr"><is><t>klotrimazol</t></is></c><c r="G828" s="2" t="inlineStr"><is><t>terbinafinę</t></is></c><c r="H828" s="2" t="inlineStr"><is><t>itrakonazol</t></is></c><c r="I828" s="2" t="inlineStr" /><c r="J828" s="2" t="inlineStr" /><c r="K828" s="2" t="inlineStr"><is><t>natamycynę</t></is></c><c r="L828" s="2" t="inlineStr" /><c r="M828" s="2" t="inlineStr" /><c r="N828" s="2" t="inlineStr" /><c r="O828" s="2" t="inlineStr" /><c r="P828" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q828" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="829"><c r="A829" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B829" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C829" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D829" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E829" s="2" t="inlineStr"><is><t>Anidulafungina w odróżnieniu od amfoterycyny B:</t></is></c><c r="F829" s="2" t="inlineStr"><is><t>ma wąskie spektrum działania przeciwgrzybiczego</t></is></c><c r="G829" s="2" t="inlineStr"><is><t>działa poprzez zahamowanie syntezy ściany komórkowej grzyba</t></is></c><c r="H829" s="2" t="inlineStr"><is><t>nie powoduje uszkodzenia nerek</t></is></c><c r="I829" s="2" t="inlineStr" /><c r="J829" s="2" t="inlineStr" /><c r="K829" s="2" t="inlineStr"><is><t>w leczeniu inwazyjnej kandydozy podawana jest drogą dożylną</t></is></c><c r="L829" s="2" t="inlineStr" /><c r="M829" s="2" t="inlineStr" /><c r="N829" s="2" t="inlineStr" /><c r="O829" s="2" t="inlineStr" /><c r="P829" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q829" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="830"><c r="A830" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B830" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C830" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D830" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E830" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenia dotyczące inhibitorów neuraminidazy:</t></is></c><c r="F830" s="2" t="inlineStr"><is><t>są skuteczne wobec wirusa grypy A i B</t></is></c><c r="G830" s="2" t="inlineStr"><is><t>leczenie lekami tej grupy powinno być wdrożone do 48 h od początku objawów u nieszczepionych osób z grup ryzyka ciężkiego przebiegu grypy</t></is></c><c r="H830" s="2" t="inlineStr" /><c r="I830" s="2" t="inlineStr" /><c r="J830" s="2" t="inlineStr" /><c r="K830" s="2" t="inlineStr"><is><t>oseltamiwir ma działanie tylko w drogach oddechowych, a zanamiwir ogólnoustrojowe, co wiąże się ze sposobem podania tych leków</t></is></c><c r="L830" s="2" t="inlineStr"><is><t>są nieskuteczne wobec wirusa świńskiej grypy H1N1</t></is></c><c r="M830" s="2" t="inlineStr" /><c r="N830" s="2" t="inlineStr" /><c r="O830" s="2" t="inlineStr" /><c r="P830" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q830" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="831"><c r="A831" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B831" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C831" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D831" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E831" s="2" t="inlineStr"><is><t>Flukonazol zgodnie z aktualną widzą medyczną można zastosować w profilaktyce medycznej u:</t></is></c><c r="F831" s="2" t="inlineStr"><is><t>pacjentów z agranulocytozą przez czas jej trwania</t></is></c><c r="G831" s="2" t="inlineStr"><is><t>biorców przeszczepów wątroby w okresie okołoprzeszczepiennym</t></is></c><c r="H831" s="2" t="inlineStr" /><c r="I831" s="2" t="inlineStr" /><c r="J831" s="2" t="inlineStr" /><c r="K831" s="2" t="inlineStr"><is><t>pacjentów leczonych szerokospektralnymi lekami przeciwbakteryjnymi przez czas takiej antybiotykoterapii</t></is></c><c r="L831" s="2" t="inlineStr"><is><t>wszystkich pacjentów oddziałów intensywnej terapii</t></is></c><c r="M831" s="2" t="inlineStr" /><c r="N831" s="2" t="inlineStr" /><c r="O831" s="2" t="inlineStr" /><c r="P831" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q831" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="832"><c r="A832" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B832" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C832" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D832" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E832" s="2" t="inlineStr"><is><t>Intrygujące konsekwencje stosowania leków to:</t></is></c><c r="F832" s="2" t="inlineStr"><is><t>pomarańczowe łzy i pot podczas stosowania ryfampicyny</t></is></c><c r="G832" s="2" t="inlineStr"><is><t>widzenie przedmiotów w żółtych obwódkach, tzw. „halo”, podczas stosowania digoksyny</t></is></c><c r="H832" s="2" t="inlineStr"><is><t>lepsze wyniki sportowe podczas stosowania meldonium u zawodowych sportowców</t></is></c><c r="I832" s="2" t="inlineStr" /><c r="J832" s="2" t="inlineStr" /><c r="K832" s="2" t="inlineStr"><is><t>poprawa IQ podczas stosowania piracetamu u licealistów i studentów</t></is></c><c r="L832" s="2" t="inlineStr" /><c r="M832" s="2" t="inlineStr" /><c r="N832" s="2" t="inlineStr" /><c r="O832" s="2" t="inlineStr" /><c r="P832" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q832" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="833"><c r="A833" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B833" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C833" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D833" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E833" s="2" t="inlineStr"><is><t>Do antyseptyki na ranę zastosujesz:</t></is></c><c r="F833" s="2" t="inlineStr"><is><t>jodopowidon</t></is></c><c r="G833" s="2" t="inlineStr"><is><t>oktenidynę</t></is></c><c r="H833" s="2" t="inlineStr" /><c r="I833" s="2" t="inlineStr" /><c r="J833" s="2" t="inlineStr" /><c r="K833" s="2" t="inlineStr"><is><t>wodę utlenioną</t></is></c><c r="L833" s="2" t="inlineStr"><is><t>0,9% roztwór NaCl</t></is></c><c r="M833" s="2" t="inlineStr" /><c r="N833" s="2" t="inlineStr" /><c r="O833" s="2" t="inlineStr" /><c r="P833" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q833" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="834"><c r="A834" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B834" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C834" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D834" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E834" s="2" t="inlineStr"><is><t>W leczeniu astmy są stosowane leki z grupy:</t></is></c><c r="F834" s="2" t="inlineStr"><is><t>agonistów receptora glikokortykosteroidowego</t></is></c><c r="G834" s="2" t="inlineStr"><is><t>antagonistów receptora M 3</t></is></c><c r="H834" s="2" t="inlineStr" /><c r="I834" s="2" t="inlineStr" /><c r="J834" s="2" t="inlineStr" /><c r="K834" s="2" t="inlineStr"><is><t>przeciwciał monoklonalnych przeciwko receptorowi dla interleukiny 1 (IL-1)</t></is></c><c r="L834" s="2" t="inlineStr"><is><t>agonistów recepta leukotrienowego CysLT 1 (B)</t></is></c><c r="M834" s="2" t="inlineStr" /><c r="N834" s="2" t="inlineStr" /><c r="O834" s="2" t="inlineStr" /><c r="P834" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q834" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="835"><c r="A835" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B835" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C835" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D835" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E835" s="2" t="inlineStr"><is><t>Wskaż zestaw leków o identycznym molekularnym mechanizmie działania:</t></is></c><c r="F835" s="2" t="inlineStr"><is><t>acetylocysteina, mesna, erdosteina</t></is></c><c r="G835" s="2" t="inlineStr"><is><t>indekaterol, wilanterol, salbutamol</t></is></c><c r="H835" s="2" t="inlineStr"><is><t>tiotropium, glikopironium, umeklidynium</t></is></c><c r="I835" s="2" t="inlineStr" /><c r="J835" s="2" t="inlineStr" /><c r="K835" s="2" t="inlineStr"><is><t>zileuton, zafirlukast, cyklezonid</t></is></c><c r="L835" s="2" t="inlineStr" /><c r="M835" s="2" t="inlineStr" /><c r="N835" s="2" t="inlineStr" /><c r="O835" s="2" t="inlineStr" /><c r="P835" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q835" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="836"><c r="A836" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B836" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C836" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D836" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E836" s="2" t="inlineStr"><is><t>Obciążenie wstępne serca zmniejsza:</t></is></c><c r="F836" s="2" t="inlineStr"><is><t>triazotan izosorbidu</t></is></c><c r="G836" s="2" t="inlineStr"><is><t>torasemid</t></is></c><c r="H836" s="2" t="inlineStr" /><c r="I836" s="2" t="inlineStr" /><c r="J836" s="2" t="inlineStr" /><c r="K836" s="2" t="inlineStr"><is><t>amlodypina</t></is></c><c r="L836" s="2" t="inlineStr"><is><t>bisoprolol</t></is></c><c r="M836" s="2" t="inlineStr" /><c r="N836" s="2" t="inlineStr" /><c r="O836" s="2" t="inlineStr" /><c r="P836" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q836" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="837"><c r="A837" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B837" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C837" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D837" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E837" s="2" t="inlineStr"><is><t>Wskaż prawidłowe pary lek - działanie niepożądane:</t></is></c><c r="F837" s="2" t="inlineStr"><is><t>propafenon - epizody nieutrwalonego częstoskurczu komorowego</t></is></c><c r="G837" s="2" t="inlineStr"><is><t>adenozyna - ból w klatce piersiowej</t></is></c><c r="H837" s="2" t="inlineStr" /><c r="I837" s="2" t="inlineStr" /><c r="J837" s="2" t="inlineStr" /><c r="K837" s="2" t="inlineStr"><is><t>wernakalant - migotanie przedsionków</t></is></c><c r="L837" s="2" t="inlineStr"><is><t>sotalol – zwiększenie progu defibrylacji</t></is></c><c r="M837" s="2" t="inlineStr" /><c r="N837" s="2" t="inlineStr" /><c r="O837" s="2" t="inlineStr" /><c r="P837" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q837" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="838"><c r="A838" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B838" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C838" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D838" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E838" s="2" t="inlineStr"><is><t>Działanie inotropowe dodatnie i rozkurczające naczynia ma:</t></is></c><c r="F838" s="2" t="inlineStr"><is><t>lewosimendan</t></is></c><c r="G838" s="2" t="inlineStr"><is><t>dobutamina</t></is></c><c r="H838" s="2" t="inlineStr" /><c r="I838" s="2" t="inlineStr" /><c r="J838" s="2" t="inlineStr" /><c r="K838" s="2" t="inlineStr"><is><t>nebiwolol</t></is></c><c r="L838" s="2" t="inlineStr"><is><t>efedryna</t></is></c><c r="M838" s="2" t="inlineStr" /><c r="N838" s="2" t="inlineStr" /><c r="O838" s="2" t="inlineStr" /><c r="P838" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q838" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="839"><c r="A839" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B839" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C839" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D839" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E839" s="2" t="inlineStr"><is><t>Wskaż minusy leczenia lipofilnym beta-adrenolitykiem:</t></is></c><c r="F839" s="2" t="inlineStr"><is><t>zaburzenia potencji</t></is></c><c r="G839" s="2" t="inlineStr"><is><t>ograniczenie wydolności fizycznej</t></is></c><c r="H839" s="2" t="inlineStr"><is><t>zaburzenia lipidowe</t></is></c><c r="I839" s="2" t="inlineStr" /><c r="J839" s="2" t="inlineStr" /><c r="K839" s="2" t="inlineStr"><is><t>działanie proarytmiczne, w tym obniżenie progu migotania komór</t></is></c><c r="L839" s="2" t="inlineStr" /><c r="M839" s="2" t="inlineStr" /><c r="N839" s="2" t="inlineStr" /><c r="O839" s="2" t="inlineStr" /><c r="P839" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q839" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="840"><c r="A840" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B840" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C840" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D840" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E840" s="2" t="inlineStr"><is><t>U 70-letniego mężczyzny z przewlekłą niewydolnością żylną wspomagająco do kompresjoterapii zastosujesz:</t></is></c><c r="F840" s="2" t="inlineStr"><is><t>mikronizowaną diosminę + hesperydynę</t></is></c><c r="G840" s="2" t="inlineStr" /><c r="H840" s="2" t="inlineStr" /><c r="I840" s="2" t="inlineStr" /><c r="J840" s="2" t="inlineStr" /><c r="K840" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy w dawce antyagregacyjnej</t></is></c><c r="L840" s="2" t="inlineStr"><is><t>enoksaparynę w dawce profilaktycznej</t></is></c><c r="M840" s="2" t="inlineStr"><is><t>furosemid w dawce leczniczej</t></is></c><c r="N840" s="2" t="inlineStr" /><c r="O840" s="2" t="inlineStr" /><c r="P840" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q840" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="841"><c r="A841" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B841" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C841" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D841" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E841" s="2" t="inlineStr"><is><t>80-letniemu mężczyźnie przesypiającemu w nocy 5 h, uskarżającemu na trudności z zasypianiem należy zalecić:</t></is></c><c r="F841" s="2" t="inlineStr"><is><t>zasady higieny snu</t></is></c><c r="G841" s="2" t="inlineStr" /><c r="H841" s="2" t="inlineStr" /><c r="I841" s="2" t="inlineStr" /><c r="J841" s="2" t="inlineStr" /><c r="K841" s="2" t="inlineStr"><is><t>alprazolam</t></is></c><c r="L841" s="2" t="inlineStr"><is><t>zolpidem</t></is></c><c r="M841" s="2" t="inlineStr"><is><t>hydroksyzynę</t></is></c><c r="N841" s="2" t="inlineStr" /><c r="O841" s="2" t="inlineStr" /><c r="P841" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q841" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="842"><c r="A842" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B842" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C842" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D842" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E842" s="2" t="inlineStr"><is><t>Zyprazydonu, leku istotnie wydłużającego odstęp QT nie należy stosować:</t></is></c><c r="F842" s="2" t="inlineStr"><is><t>w hipokaliemii</t></is></c><c r="G842" s="2" t="inlineStr"><is><t>łącznie z moksyfloksacyną</t></is></c><c r="H842" s="2" t="inlineStr"><is><t>w objawowej bradykardii</t></is></c><c r="I842" s="2" t="inlineStr"><is><t>łącznie z amiodaronem</t></is></c><c r="J842" s="2" t="inlineStr" /><c r="K842" s="2" t="inlineStr" /><c r="L842" s="2" t="inlineStr" /><c r="M842" s="2" t="inlineStr" /><c r="N842" s="2" t="inlineStr" /><c r="O842" s="2" t="inlineStr" /><c r="P842" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q842" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="843"><c r="A843" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B843" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C843" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D843" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E843" s="2" t="inlineStr"><is><t>Zaburzenia pozapiramidowe mogą wystąpić w przebiegu stosowania:</t></is></c><c r="F843" s="2" t="inlineStr"><is><t>flunaryzyny</t></is></c><c r="G843" s="2" t="inlineStr"><is><t>metoklopramidu</t></is></c><c r="H843" s="2" t="inlineStr" /><c r="I843" s="2" t="inlineStr" /><c r="J843" s="2" t="inlineStr" /><c r="K843" s="2" t="inlineStr"><is><t>betahistyny</t></is></c><c r="L843" s="2" t="inlineStr"><is><t>rywastygminy</t></is></c><c r="M843" s="2" t="inlineStr" /><c r="N843" s="2" t="inlineStr" /><c r="O843" s="2" t="inlineStr" /><c r="P843" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q843" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="844"><c r="A844" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B844" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C844" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D844" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E844" s="2" t="inlineStr"><is><t>Parkinsonizm polekowy w przebiegu leczenia lekami przeciwpsychotycznymi wynika z:</t></is></c><c r="F844" s="2" t="inlineStr"><is><t>zmniejszania działania dopaminy w układzie nigrostriatalnym</t></is></c><c r="G844" s="2" t="inlineStr" /><c r="H844" s="2" t="inlineStr" /><c r="I844" s="2" t="inlineStr" /><c r="J844" s="2" t="inlineStr" /><c r="K844" s="2" t="inlineStr"><is><t>patogenezy schizofrenii</t></is></c><c r="L844" s="2" t="inlineStr"><is><t>zmniejszania działania dopaminy w obszarze mezokortykalnym</t></is></c><c r="M844" s="2" t="inlineStr"><is><t>blokowania receptorów muskarynowych</t></is></c><c r="N844" s="2" t="inlineStr" /><c r="O844" s="2" t="inlineStr" /><c r="P844" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q844" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="845"><c r="A845" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B845" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C845" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D845" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E845" s="2" t="inlineStr"><is><t>Napływ sodu do komórki hamuje:</t></is></c><c r="F845" s="2" t="inlineStr"><is><t>ranolzyna</t></is></c><c r="G845" s="2" t="inlineStr"><is><t>iwabradyna</t></is></c><c r="H845" s="2" t="inlineStr"><is><t>okskarbamazepina</t></is></c><c r="I845" s="2" t="inlineStr" /><c r="J845" s="2" t="inlineStr" /><c r="K845" s="2" t="inlineStr"><is><t>gabapentyna</t></is></c><c r="L845" s="2" t="inlineStr" /><c r="M845" s="2" t="inlineStr" /><c r="N845" s="2" t="inlineStr" /><c r="O845" s="2" t="inlineStr" /><c r="P845" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q845" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="846"><c r="A846" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B846" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C846" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D846" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E846" s="2" t="inlineStr"><is><t>W ramach badania geriatrycznego u 80-letniej kobiety ze średnim wykształceniem wynik MMSE = 25 pkt. Za niezgodne z aktualną wiedzą medyczną uznasz zastosowanie u niej:</t></is></c><c r="F846" s="2" t="inlineStr"><is><t>piracetamu</t></is></c><c r="G846" s="2" t="inlineStr"><is><t>winpocetyny</t></is></c><c r="H846" s="2" t="inlineStr"><is><t>suplementacji cynku</t></is></c><c r="I846" s="2" t="inlineStr" /><c r="J846" s="2" t="inlineStr" /><c r="K846" s="2" t="inlineStr"><is><t>treningu mózgu (np. zgadnij co to za zawód: arlzek)</t></is></c><c r="L846" s="2" t="inlineStr" /><c r="M846" s="2" t="inlineStr" /><c r="N846" s="2" t="inlineStr" /><c r="O846" s="2" t="inlineStr" /><c r="P846" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q846" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="847"><c r="A847" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B847" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C847" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D847" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E847" s="2" t="inlineStr"><is><t>W zapobieganiu wymiotom w przebiegu chemioterapii należy zastosować:</t></is></c><c r="F847" s="2" t="inlineStr"><is><t>aprepitant</t></is></c><c r="G847" s="2" t="inlineStr"><is><t>ondansetron</t></is></c><c r="H847" s="2" t="inlineStr" /><c r="I847" s="2" t="inlineStr" /><c r="J847" s="2" t="inlineStr" /><c r="K847" s="2" t="inlineStr"><is><t>skopolaminę</t></is></c><c r="L847" s="2" t="inlineStr"><is><t>dimenhydrinat</t></is></c><c r="M847" s="2" t="inlineStr" /><c r="N847" s="2" t="inlineStr" /><c r="O847" s="2" t="inlineStr" /><c r="P847" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q847" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="848"><c r="A848" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B848" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C848" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D848" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E848" s="2" t="inlineStr"><is><t>Wg Światowej Agencji Antydopingowej (WADA) za doping uważa się:</t></is></c><c r="F848" s="2" t="inlineStr"><is><t>użycie przez sportowców czynników stymulujących erytropoezę</t></is></c><c r="G848" s="2" t="inlineStr"><is><t>podanie sportowcowi autopreparatu krwinek czerwonych</t></is></c><c r="H848" s="2" t="inlineStr"><is><t>obecność we krwi sportowca egzogennych substancji o działaniu agonistycznym w stosunku do receptorów androgenowych i dla IGF-1</t></is></c><c r="I848" s="2" t="inlineStr"><is><t>podanie sportowcowi polimerów kwasów nukleinowych lub analogów kwasu nukleinowego</t></is></c><c r="J848" s="2" t="inlineStr" /><c r="K848" s="2" t="inlineStr" /><c r="L848" s="2" t="inlineStr" /><c r="M848" s="2" t="inlineStr" /><c r="N848" s="2" t="inlineStr" /><c r="O848" s="2" t="inlineStr" /><c r="P848" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q848" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="849"><c r="A849" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B849" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C849" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D849" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E849" s="2" t="inlineStr"><is><t>U chorego z zaburzeniami świadomości, sennością, zaburzeniami równowagi, mowy, widzenia, omamy, pobudzeniem psychoruchowym, drgawkami, hipotonia z nieutrwalonymi częstoskurczami komorowymi będziesz podejrzewał zatrucie i podasz:</t></is></c><c r="F849" s="2" t="inlineStr"><is><t>imipraminą - fizostygminę</t></is></c><c r="G849" s="2" t="inlineStr" /><c r="H849" s="2" t="inlineStr" /><c r="I849" s="2" t="inlineStr" /><c r="J849" s="2" t="inlineStr" /><c r="K849" s="2" t="inlineStr"><is><t>paracetamolem- N-acetylocysteinę</t></is></c><c r="L849" s="2" t="inlineStr"><is><t>kodeiną - naltrekson</t></is></c><c r="M849" s="2" t="inlineStr"><is><t>litem - fizostygminę</t></is></c><c r="N849" s="2" t="inlineStr" /><c r="O849" s="2" t="inlineStr" /><c r="P849" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 1 termin</t></is></c><c r="Q849" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="850"><c r="A850" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B850" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C850" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D850" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E850" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące przedawkowania leków znieczulenia miejscowego:</t></is></c><c r="F850" s="2" t="inlineStr"><is><t>Powodują drgawki, bradykardię i hipotonię</t></is></c><c r="G850" s="2" t="inlineStr"><is><t>Parestezje (drętwienie) języka i ust są wczesnym charakterystycznym objawem zwiastunowym</t></is></c><c r="H850" s="2" t="inlineStr"><is><t>W resuscytacji krążeniowo oddechowej, oprócz typowego algorytmu, stosuje się wlew emulsji tłuszczowej</t></is></c><c r="I850" s="2" t="inlineStr"><is><t>Na wystąpienie objawów nie ma wpływu miejscu wstrzyknięcia leku, a jedynie jego dawka</t></is></c><c r="J850" s="2" t="inlineStr" /><c r="K850" s="2" t="inlineStr" /><c r="L850" s="2" t="inlineStr" /><c r="M850" s="2" t="inlineStr" /><c r="N850" s="2" t="inlineStr" /><c r="O850" s="2" t="inlineStr" /><c r="P850" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q850" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="851"><c r="A851" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B851" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C851" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D851" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E851" s="2" t="inlineStr"><is><t>Do leków przeciwhistaminowych stosowanych wyłącznie miejscowo na błony śluzowe należą:</t></is></c><c r="F851" s="2" t="inlineStr"><is><t>Emedastyna</t></is></c><c r="G851" s="2" t="inlineStr"><is><t>Azelastyna</t></is></c><c r="H851" s="2" t="inlineStr" /><c r="I851" s="2" t="inlineStr" /><c r="J851" s="2" t="inlineStr" /><c r="K851" s="2" t="inlineStr"><is><t>Desforatadyna</t></is></c><c r="L851" s="2" t="inlineStr"><is><t>Bilastyna</t></is></c><c r="M851" s="2" t="inlineStr" /><c r="N851" s="2" t="inlineStr" /><c r="O851" s="2" t="inlineStr" /><c r="P851" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q851" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="852"><c r="A852" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B852" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C852" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D852" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E852" s="2" t="inlineStr"><is><t>Dorosły pacjent trafił do szpitala 3 godziny po samobójczym przedawkowaniu fenobarbitalu (pochodna kwasu barbiturowego). Należy zastosować:</t></is></c><c r="F852" s="2" t="inlineStr"><is><t>Rozcienczenie trucizny przez podanie do wypicia dużej ilości wody pitnej</t></is></c><c r="G852" s="2" t="inlineStr"><is><t>Alkalizację moczu do pH co najmniej 7,5 przez dodanie wodorowęglanu sodu do dożylnych płynów infuzyjnych</t></is></c><c r="H852" s="2" t="inlineStr" /><c r="I852" s="2" t="inlineStr" /><c r="J852" s="2" t="inlineStr" /><c r="K852" s="2" t="inlineStr"><is><t>Płukanie żołądka z zastosowaniem wody pitnej przez sondę ustno-żołądkową w małych porcjach jedna po drugiej</t></is></c><c r="L852" s="2" t="inlineStr"><is><t>Irygację całego jelita przez doustne podanie płynów elektrolitowych z polietylenoglikolem (tzw. makrogolami)</t></is></c><c r="M852" s="2" t="inlineStr" /><c r="N852" s="2" t="inlineStr" /><c r="O852" s="2" t="inlineStr" /><c r="P852" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q852" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="853"><c r="A853" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B853" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C853" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D853" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E853" s="2" t="inlineStr"><is><t>Wskaż prawidłowe połączenie trucizna – antidotum – mechanizm działania antidotum:</t></is></c><c r="F853" s="2" t="inlineStr"><is><t>Paracetamol – acetylocysteina – neutralizacja metaboliczna</t></is></c><c r="G853" s="2" t="inlineStr"><is><t>Amitryptylina - fizostygmina - antagonizm fizjologiczny</t></is></c><c r="H853" s="2" t="inlineStr"><is><t>Dabigatran – idarucyzumab - neutralizujące przeciwciało</t></is></c><c r="I853" s="2" t="inlineStr"><is><t>Diazepam – flomazenil – antagonizm receptorowy</t></is></c><c r="J853" s="2" t="inlineStr" /><c r="K853" s="2" t="inlineStr" /><c r="L853" s="2" t="inlineStr" /><c r="M853" s="2" t="inlineStr" /><c r="N853" s="2" t="inlineStr" /><c r="O853" s="2" t="inlineStr" /><c r="P853" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q853" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="854"><c r="A854" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B854" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C854" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D854" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E854" s="2" t="inlineStr"><is><t>Który z leków działa przeciwdrgawkowo głównie poprzez nasilenie transmisji GABA￾ergicznej:</t></is></c><c r="F854" s="2" t="inlineStr"><is><t>Tiagabina</t></is></c><c r="G854" s="2" t="inlineStr" /><c r="H854" s="2" t="inlineStr" /><c r="I854" s="2" t="inlineStr" /><c r="J854" s="2" t="inlineStr" /><c r="K854" s="2" t="inlineStr"><is><t>Lamotrygina</t></is></c><c r="L854" s="2" t="inlineStr"><is><t>Lewetriacetam</t></is></c><c r="M854" s="2" t="inlineStr"><is><t>Zonisamid</t></is></c><c r="N854" s="2" t="inlineStr" /><c r="O854" s="2" t="inlineStr" /><c r="P854" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q854" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="855"><c r="A855" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B855" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C855" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D855" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E855" s="2" t="inlineStr"><is><t>Które leki mogą zaostrzyć objawy otępienia u osoby z chorobą Alzheimera?</t></is></c><c r="F855" s="2" t="inlineStr"><is><t>Olanzapina</t></is></c><c r="G855" s="2" t="inlineStr"><is><t>Memantyna</t></is></c><c r="H855" s="2" t="inlineStr"><is><t>Biperiden</t></is></c><c r="I855" s="2" t="inlineStr" /><c r="J855" s="2" t="inlineStr" /><c r="K855" s="2" t="inlineStr"><is><t>Piracetam</t></is></c><c r="L855" s="2" t="inlineStr" /><c r="M855" s="2" t="inlineStr" /><c r="N855" s="2" t="inlineStr" /><c r="O855" s="2" t="inlineStr" /><c r="P855" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q855" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="856"><c r="A856" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B856" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C856" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D856" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E856" s="2" t="inlineStr"><is><t>Skłonność do hazardu, kompulsywne objadanie i obsesje seksualne to działania niepożądane obserwowane w terapii:</t></is></c><c r="F856" s="2" t="inlineStr"><is><t>L-dopą</t></is></c><c r="G856" s="2" t="inlineStr"><is><t>Pramipeksolem</t></is></c><c r="H856" s="2" t="inlineStr" /><c r="I856" s="2" t="inlineStr" /><c r="J856" s="2" t="inlineStr" /><c r="K856" s="2" t="inlineStr"><is><t>Metylofenidatem</t></is></c><c r="L856" s="2" t="inlineStr"><is><t>Zolpidemem</t></is></c><c r="M856" s="2" t="inlineStr" /><c r="N856" s="2" t="inlineStr" /><c r="O856" s="2" t="inlineStr" /><c r="P856" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q856" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="857"><c r="A857" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B857" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C857" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D857" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E857" s="2" t="inlineStr"><is><t>Zolendronian:</t></is></c><c r="F857" s="2" t="inlineStr"><is><t>Z dużym powinowactwem wiąże się ze zmineralizowaną kością</t></is></c><c r="G857" s="2" t="inlineStr"><is><t>Hamuje resorbcję kości</t></is></c><c r="H857" s="2" t="inlineStr" /><c r="I857" s="2" t="inlineStr" /><c r="J857" s="2" t="inlineStr" /><c r="K857" s="2" t="inlineStr"><is><t>Koryguje hiperkalcemię w chorobach nowotworowych zwiększając jednoczeście kalcurię</t></is></c><c r="L857" s="2" t="inlineStr"><is><t>Może spowodować martwicę szczęki szczególnie w przypadku złego stanu uzębienia</t></is></c><c r="M857" s="2" t="inlineStr" /><c r="N857" s="2" t="inlineStr" /><c r="O857" s="2" t="inlineStr" /><c r="P857" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q857" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="858"><c r="A858" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B858" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C858" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D858" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E858" s="2" t="inlineStr"><is><t>Leki stosowane przewlekle w stwardnieniu rozsianym w celu modyfikacji przebiegu choroby to:</t></is></c><c r="F858" s="2" t="inlineStr"><is><t>PEG-interferon-beta</t></is></c><c r="G858" s="2" t="inlineStr"><is><t>Natalizumab</t></is></c><c r="H858" s="2" t="inlineStr"><is><t>Adalimumab</t></is></c><c r="I858" s="2" t="inlineStr" /><c r="J858" s="2" t="inlineStr" /><c r="K858" s="2" t="inlineStr"><is><t>Interferon-gamma</t></is></c><c r="L858" s="2" t="inlineStr" /><c r="M858" s="2" t="inlineStr" /><c r="N858" s="2" t="inlineStr" /><c r="O858" s="2" t="inlineStr" /><c r="P858" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q858" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="859"><c r="A859" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B859" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C859" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D859" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E859" s="2" t="inlineStr"><is><t>Który mechanizm opisuje działanie aprepitantu:</t></is></c><c r="F859" s="2" t="inlineStr"><is><t>Stymulowanie receptora neurokininy (NK1) w strefie chemoreceptorowej mózgu</t></is></c><c r="G859" s="2" t="inlineStr" /><c r="H859" s="2" t="inlineStr" /><c r="I859" s="2" t="inlineStr" /><c r="J859" s="2" t="inlineStr" /><c r="K859" s="2" t="inlineStr"><is><t>Stymulowanie receptora O2 w strefie chemoreceptorowej mózgu</t></is></c><c r="L859" s="2" t="inlineStr"><is><t>Stymulowanie receptora 5-HT3 na włóknach aferentnych nerwu błędnego</t></is></c><c r="M859" s="2" t="inlineStr"><is><t>Blokowanie receptora muskarynowego w ośrodku wymiotnym w rdzeniu przedłużonym</t></is></c><c r="N859" s="2" t="inlineStr" /><c r="O859" s="2" t="inlineStr" /><c r="P859" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q859" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="860"><c r="A860" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B860" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C860" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D860" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E860" s="2" t="inlineStr"><is><t>Amitryptylina ma zastosowanie w leczeniu:</t></is></c><c r="F860" s="2" t="inlineStr"><is><t>Bólu neuropatycznego</t></is></c><c r="G860" s="2" t="inlineStr"><is><t>Choroby afektywnej jednobiegunowej</t></is></c><c r="H860" s="2" t="inlineStr" /><c r="I860" s="2" t="inlineStr" /><c r="J860" s="2" t="inlineStr" /><c r="K860" s="2" t="inlineStr"><is><t>Bezsenności</t></is></c><c r="L860" s="2" t="inlineStr"><is><t>Padaczki</t></is></c><c r="M860" s="2" t="inlineStr" /><c r="N860" s="2" t="inlineStr" /><c r="O860" s="2" t="inlineStr" /><c r="P860" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q860" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="861"><c r="A861" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B861" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C861" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D861" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E861" s="2" t="inlineStr"><is><t>Zespół serotoninowy może być wynikiem podawania:</t></is></c><c r="F861" s="2" t="inlineStr"><is><t>Tramadolu</t></is></c><c r="G861" s="2" t="inlineStr"><is><t>Escitalopramu</t></is></c><c r="H861" s="2" t="inlineStr" /><c r="I861" s="2" t="inlineStr" /><c r="J861" s="2" t="inlineStr" /><c r="K861" s="2" t="inlineStr"><is><t>Litu</t></is></c><c r="L861" s="2" t="inlineStr"><is><t>Buspironu</t></is></c><c r="M861" s="2" t="inlineStr" /><c r="N861" s="2" t="inlineStr" /><c r="O861" s="2" t="inlineStr" /><c r="P861" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q861" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="862"><c r="A862" s="2" t="inlineStr"><is><t>LEKI PRZECIWLĘKOWE</t></is></c><c r="B862" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C862" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D862" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E862" s="2" t="inlineStr"><is><t>Benzodiazepiną nie mającą wątrobowego metabolizmu jest:</t></is></c><c r="F862" s="2" t="inlineStr"><is><t>Lorazepam</t></is></c><c r="G862" s="2" t="inlineStr"><is><t>Oksazepam</t></is></c><c r="H862" s="2" t="inlineStr" /><c r="I862" s="2" t="inlineStr" /><c r="J862" s="2" t="inlineStr" /><c r="K862" s="2" t="inlineStr"><is><t>Nitrazepam</t></is></c><c r="L862" s="2" t="inlineStr"><is><t>Diazepam</t></is></c><c r="M862" s="2" t="inlineStr" /><c r="N862" s="2" t="inlineStr" /><c r="O862" s="2" t="inlineStr" /><c r="P862" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q862" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="863"><c r="A863" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B863" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C863" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D863" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E863" s="2" t="inlineStr"><is><t>Acetylocysteina:</t></is></c><c r="F863" s="2" t="inlineStr"><is><t>Jest odtrutką w zatruciu paracetamolem ze względu na udział w detoksykacji toksycznego metabolitu N-acetylo-4-benzochinoiminy (NAPO)</t></is></c><c r="G863" s="2" t="inlineStr" /><c r="H863" s="2" t="inlineStr" /><c r="I863" s="2" t="inlineStr" /><c r="J863" s="2" t="inlineStr" /><c r="K863" s="2" t="inlineStr"><is><t>Może być stosowana doustnie, dożylnie i wziewnie</t></is></c><c r="L863" s="2" t="inlineStr"><is><t>W dużej dawce pobudza ruchomość rzęsek nabłonka oddechowego</t></is></c><c r="M863" s="2" t="inlineStr"><is><t>Rozrzedza śluz poprzez zmniejszenie oddziaływania ładunków elektrycznych występujących w sieci mucyn (działanie niedestrukcyjne)</t></is></c><c r="N863" s="2" t="inlineStr" /><c r="O863" s="2" t="inlineStr" /><c r="P863" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q863" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="864"><c r="A864" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B864" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C864" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D864" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E864" s="2" t="inlineStr"><is><t>Przewlekłe stosowanie pantoprazolu może prowadzić do:</t></is></c><c r="F864" s="2" t="inlineStr"><is><t>Zmniejszonego wchłaniania witaminy B12, Mg2+, Ca2+</t></is></c><c r="G864" s="2" t="inlineStr"><is><t>Zwiększonego ryzyka zakażenia przewodu pokarmowego, np. biegunka Clostridium difficile</t></is></c><c r="H864" s="2" t="inlineStr"><is><t>Zwiększonego ryzyka złamania kościu udowej</t></is></c><c r="I864" s="2" t="inlineStr" /><c r="J864" s="2" t="inlineStr" /><c r="K864" s="2" t="inlineStr"><is><t>Zwiększonego ryzyka zakażenia układu oddechowego</t></is></c><c r="L864" s="2" t="inlineStr" /><c r="M864" s="2" t="inlineStr" /><c r="N864" s="2" t="inlineStr" /><c r="O864" s="2" t="inlineStr" /><c r="P864" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q864" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="865"><c r="A865" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B865" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C865" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D865" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E865" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie - lek prokinetyczny / mechanizm działania:</t></is></c><c r="F865" s="2" t="inlineStr"><is><t>Erytromycyna - agonista rec. Motylinowego</t></is></c><c r="G865" s="2" t="inlineStr"><is><t>Cizapryd – agonista rec. 5-HT4</t></is></c><c r="H865" s="2" t="inlineStr" /><c r="I865" s="2" t="inlineStr" /><c r="J865" s="2" t="inlineStr" /><c r="K865" s="2" t="inlineStr"><is><t>Metoklopramid – agonista rec. 5-HT3 i rec. D2</t></is></c><c r="L865" s="2" t="inlineStr"><is><t>Itopryd – agonista rec. 5-HT4 i rec. D2</t></is></c><c r="M865" s="2" t="inlineStr" /><c r="N865" s="2" t="inlineStr" /><c r="O865" s="2" t="inlineStr" /><c r="P865" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q865" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="866"><c r="A866" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B866" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C866" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D866" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E866" s="2" t="inlineStr"><is><t>Kwerolimus jest stosowany w:</t></is></c><c r="F866" s="2" t="inlineStr"><is><t>Kardiologii (stenty wiecowe)</t></is></c><c r="G866" s="2" t="inlineStr"><is><t>Onkologii (wybrane zaawansowane nowotwory piersi i nerki)</t></is></c><c r="H866" s="2" t="inlineStr" /><c r="I866" s="2" t="inlineStr" /><c r="J866" s="2" t="inlineStr" /><c r="K866" s="2" t="inlineStr"><is><t>Neurologii (stwardnieni rozsiane)</t></is></c><c r="L866" s="2" t="inlineStr"><is><t>Dermatologii (łuszczyca)</t></is></c><c r="M866" s="2" t="inlineStr" /><c r="N866" s="2" t="inlineStr" /><c r="O866" s="2" t="inlineStr" /><c r="P866" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q866" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="867"><c r="A867" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B867" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C867" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D867" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E867" s="2" t="inlineStr"><is><t>Mykofenolan mofetylu (MMF):</t></is></c><c r="F867" s="2" t="inlineStr"><is><t>Jest odwracalnym inhibitorem dehydrogenazy inozynomonofosforanu hamującym syntezę de novo nukleotydów guaninowych</t></is></c><c r="G867" s="2" t="inlineStr"><is><t>Działa silniej na limfocyty niż na inne komórki</t></is></c><c r="H867" s="2" t="inlineStr" /><c r="I867" s="2" t="inlineStr" /><c r="J867" s="2" t="inlineStr" /><c r="K867" s="2" t="inlineStr"><is><t>Bezpośrednio hamuje wytwarzanie interleukiny 2 (IL-2)</t></is></c><c r="L867" s="2" t="inlineStr"><is><t>Jest inhibitorem sygnału po pobudzeniu receptorów dla IL-2</t></is></c><c r="M867" s="2" t="inlineStr" /><c r="N867" s="2" t="inlineStr" /><c r="O867" s="2" t="inlineStr" /><c r="P867" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q867" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="868"><c r="A868" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B868" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C868" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D868" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E868" s="2" t="inlineStr"><is><t>Adenozyna</t></is></c><c r="F868" s="2" t="inlineStr"><is><t>To nukleotyd purynowy występujący we wszystkich komórkach organizmu</t></is></c><c r="G868" s="2" t="inlineStr" /><c r="H868" s="2" t="inlineStr" /><c r="I868" s="2" t="inlineStr" /><c r="J868" s="2" t="inlineStr" /><c r="K868" s="2" t="inlineStr"><is><t>Aktywuje kanały potasowe i powoduje depolaryzację komórek</t></is></c><c r="L868" s="2" t="inlineStr"><is><t>Działa dromotropowo ujemnie w węźle przedsionkowo-komorowym</t></is></c><c r="M868" s="2" t="inlineStr"><is><t>Jest skuteczna kardiowersji farmakologicznej częstoskurczów komorowych</t></is></c><c r="N868" s="2" t="inlineStr" /><c r="O868" s="2" t="inlineStr" /><c r="P868" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q868" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="869"><c r="A869" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B869" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C869" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D869" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E869" s="2" t="inlineStr"><is><t>Ewolokumab:</t></is></c><c r="F869" s="2" t="inlineStr"><is><t>Jest ludzkim przeciwciałem poliklonalnym</t></is></c><c r="G869" s="2" t="inlineStr"><is><t>Hamuje aktywność konwertazy białkowej subtylizyna/keksyna typu 9 (PCSK9) - enzymu biorącego udział w degradacji receptorów dla LDL</t></is></c><c r="H869" s="2" t="inlineStr" /><c r="I869" s="2" t="inlineStr" /><c r="J869" s="2" t="inlineStr" /><c r="K869" s="2" t="inlineStr"><is><t>Jest stosowany dożylnie</t></is></c><c r="L869" s="2" t="inlineStr"><is><t>Zwiększa stęężenie cholesterolu HDL o ponad 100%</t></is></c><c r="M869" s="2" t="inlineStr" /><c r="N869" s="2" t="inlineStr" /><c r="O869" s="2" t="inlineStr" /><c r="P869" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q869" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="870"><c r="A870" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B870" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C870" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D870" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E870" s="2" t="inlineStr"><is><t>Przyczyną wzrostu masy ciała może być:</t></is></c><c r="F870" s="2" t="inlineStr"><is><t>Klemastyny</t></is></c><c r="G870" s="2" t="inlineStr"><is><t>Kwetiapiny</t></is></c><c r="H870" s="2" t="inlineStr"><is><t>Citalopramu</t></is></c><c r="I870" s="2" t="inlineStr" /><c r="J870" s="2" t="inlineStr" /><c r="K870" s="2" t="inlineStr"><is><t>Liraglutydu</t></is></c><c r="L870" s="2" t="inlineStr" /><c r="M870" s="2" t="inlineStr" /><c r="N870" s="2" t="inlineStr" /><c r="O870" s="2" t="inlineStr" /><c r="P870" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q870" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="871"><c r="A871" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B871" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C871" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D871" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E871" s="2" t="inlineStr"><is><t>Reguła Robertsa mówi o:</t></is></c><c r="F871" s="2" t="inlineStr"><is><t>Podwajaniu dawki statyny</t></is></c><c r="G871" s="2" t="inlineStr"><is><t>Obniżeniu stężenia cholesterolu LDL o dodatkowe 7% po odpowiednim zwiększeniu dawki statyny</t></is></c><c r="H871" s="2" t="inlineStr" /><c r="I871" s="2" t="inlineStr" /><c r="J871" s="2" t="inlineStr" /><c r="K871" s="2" t="inlineStr"><is><t>Obniżeniu stężenia cholesterolu LDL o dodatkowe 5% po odpowiednim zwiększeniu dawki statyny</t></is></c><c r="L871" s="2" t="inlineStr"><is><t>Potrajaniu dawki statyny</t></is></c><c r="M871" s="2" t="inlineStr" /><c r="N871" s="2" t="inlineStr" /><c r="O871" s="2" t="inlineStr" /><c r="P871" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q871" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="872"><c r="A872" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B872" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C872" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D872" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E872" s="2" t="inlineStr"><is><t>Do leków hamujących układ RAA należy:</t></is></c><c r="F872" s="2" t="inlineStr"><is><t>Zofenopryl</t></is></c><c r="G872" s="2" t="inlineStr"><is><t>Eplerenon</t></is></c><c r="H872" s="2" t="inlineStr" /><c r="I872" s="2" t="inlineStr" /><c r="J872" s="2" t="inlineStr" /><c r="K872" s="2" t="inlineStr"><is><t>Aliskiren</t></is></c><c r="L872" s="2" t="inlineStr"><is><t>Nebiwolol</t></is></c><c r="M872" s="2" t="inlineStr" /><c r="N872" s="2" t="inlineStr" /><c r="O872" s="2" t="inlineStr" /><c r="P872" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q872" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="873"><c r="A873" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B873" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C873" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D873" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E873" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące torasemidu:</t></is></c><c r="F873" s="2" t="inlineStr"><is><t>Hamuje symporter sodowo-potasowo-chlorkowy części grubościennej ramienia wstępującego pętli Henlego</t></is></c><c r="G873" s="2" t="inlineStr"><is><t>Zwiększa aktywność reninową osocza</t></is></c><c r="H873" s="2" t="inlineStr" /><c r="I873" s="2" t="inlineStr" /><c r="J873" s="2" t="inlineStr" /><c r="K873" s="2" t="inlineStr"><is><t>Powoduje słabszy efekt natiuretyczny niż furosemid</t></is></c><c r="L873" s="2" t="inlineStr"><is><t>Jest nieskuteczny jeśli eGFR (wskaźnik filtracji kłębuszkowej) &lt; 30 ml/min</t></is></c><c r="M873" s="2" t="inlineStr" /><c r="N873" s="2" t="inlineStr" /><c r="O873" s="2" t="inlineStr" /><c r="P873" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q873" s="2" t="inlineStr"><is><t>srednia</t></is></c></row></sheetData><autoFilter ref="A1:Q873" /><pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5" /></worksheet>
 </file>
</xml_diff>

<commit_message>
Usun 4 pytania o sprzecznych wariantach
Usuniete z ARCYBAZY pytania, ktorych warianty studenci zaznaczyli w roznych
latach sprzecznie i ktorych zrodlo nie pozwala rozstrzygnac:
Farmakoterapia POChP kategoria A i B, Farmakoterapia otylosci, Metoklopramid,
Lek - monitorowanie.

Wariant Metoklopramid zaznaczal agonizm D2, co jest bledne (to antagonista).
Dopasowanie po DOKLADNEJ tresci pytania - Metoklopramid: (z dwukropkiem) oraz
Dzialanie przeciwwymiotne metoklopramidu... to inne, poprawne pytania i zostaja.

ARCYBAZA 872 -> 868; razem 1239 -> 1235.
Kontrola: 0 wierszy wadliwych, 0 duplikatow, 0 trafien detektora zanieczyszczen,
importer 1080/1235. Brak znanych nierozstrzygnietych rozbieznosci.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sDWkA2eXfHxFn4vQGjL1J
</commit_message>
<xml_diff>
--- a/farmakologia_ARCYBAZA_OnlyPharms.xlsx
+++ b/farmakologia_ARCYBAZA_OnlyPharms.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Pytania" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pytania'!$A$1:$Q$873</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pytania'!$A$1:$Q$869</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,5 +424,5 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"><sheetPr><outlinePr summaryBelow="1" summaryRight="1" /><pageSetUpPr /></sheetPr><dimension ref="A1:Q873" /><sheetFormatPr baseColWidth="8" defaultRowHeight="15" /><cols><col width="30" customWidth="1" min="1" max="1" /><col width="21" customWidth="1" min="2" max="2" /><col width="9" customWidth="1" min="3" max="3" /><col width="9" customWidth="1" min="4" max="4" /><col width="60" customWidth="1" min="5" max="5" /><col width="32" customWidth="1" min="6" max="6" /><col width="32" customWidth="1" min="7" max="7" /><col width="32" customWidth="1" min="8" max="8" /><col width="32" customWidth="1" min="9" max="9" /><col width="32" customWidth="1" min="10" max="10" /><col width="32" customWidth="1" min="11" max="11" /><col width="32" customWidth="1" min="12" max="12" /><col width="32" customWidth="1" min="13" max="13" /><col width="32" customWidth="1" min="14" max="14" /><col width="32" customWidth="1" min="15" max="15" /><col width="26" customWidth="1" min="16" max="16" /><col width="10" customWidth="1" min="17" max="17" /></cols><sheetData><row r="1"><c r="A1" s="1" t="inlineStr"><is><t>Section</t></is></c><c r="B1" s="1" t="inlineStr"><is><t>Category</t></is></c><c r="C1" s="1" t="inlineStr"><is><t>Poziom</t></is></c><c r="D1" s="1" t="inlineStr"><is><t>Type</t></is></c><c r="E1" s="1" t="inlineStr"><is><t>Question</t></is></c><c r="F1" s="1" t="inlineStr"><is><t>True 1</t></is></c><c r="G1" s="1" t="inlineStr"><is><t>True 2</t></is></c><c r="H1" s="1" t="inlineStr"><is><t>True 3</t></is></c><c r="I1" s="1" t="inlineStr"><is><t>True 4</t></is></c><c r="J1" s="1" t="inlineStr"><is><t>True 5</t></is></c><c r="K1" s="1" t="inlineStr"><is><t>False 1</t></is></c><c r="L1" s="1" t="inlineStr"><is><t>False 2</t></is></c><c r="M1" s="1" t="inlineStr"><is><t>False 3</t></is></c><c r="N1" s="1" t="inlineStr"><is><t>False 4</t></is></c><c r="O1" s="1" t="inlineStr"><is><t>False 5</t></is></c><c r="P1" s="1" t="inlineStr"><is><t>Zrodlo</t></is></c><c r="Q1" s="1" t="inlineStr"><is><t>Pewnosc</t></is></c></row><row r="2"><c r="A2" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B2" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C2" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D2" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E2" s="2" t="inlineStr"><is><t>Czarne zabarwienie stolca powoduje podanie preparatów:</t></is></c><c r="F2" s="2" t="inlineStr"><is><t>Bizmutu</t></is></c><c r="G2" s="2" t="inlineStr"><is><t>Żelaza</t></is></c><c r="H2" s="2" t="inlineStr" /><c r="I2" s="2" t="inlineStr" /><c r="J2" s="2" t="inlineStr" /><c r="K2" s="2" t="inlineStr"><is><t>Wapnia</t></is></c><c r="L2" s="2" t="inlineStr"><is><t>Glinu</t></is></c><c r="M2" s="2" t="inlineStr" /><c r="N2" s="2" t="inlineStr" /><c r="O2" s="2" t="inlineStr" /><c r="P2" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q2" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="3"><c r="A3" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B3" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C3" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D3" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E3" s="2" t="inlineStr"><is><t>Uzasadnionym wskazaniem do przewlekłego stosowania inhibitorów pompy protonowej jest:</t></is></c><c r="F3" s="2" t="inlineStr"><is><t>Choroba refluksowa żołądka</t></is></c><c r="G3" s="2" t="inlineStr"><is><t>Profilaktyka gastropatii u osób leczonych niesteroidowymi lekami przeciwzapalnymi powyżej 65 r.ż</t></is></c><c r="H3" s="2" t="inlineStr"><is><t>Eradykacja Helicobacter Pylori</t></is></c><c r="I3" s="2" t="inlineStr" /><c r="J3" s="2" t="inlineStr" /><c r="K3" s="2" t="inlineStr"><is><t>Profilaktyka wrzodów stresowych</t></is></c><c r="L3" s="2" t="inlineStr" /><c r="M3" s="2" t="inlineStr" /><c r="N3" s="2" t="inlineStr" /><c r="O3" s="2" t="inlineStr" /><c r="P3" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q3" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="4"><c r="A4" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B4" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C4" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D4" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E4" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek – wskazanie</t></is></c><c r="F4" s="2" t="inlineStr"><is><t>Mesalazyna – choroba Leśniowskiego crohna</t></is></c><c r="G4" s="2" t="inlineStr"><is><t>Rifaksymina – biegunka podróżnych</t></is></c><c r="H4" s="2" t="inlineStr"><is><t>Metylonaltrekson – zaparcia w trakcie terapii opioidami</t></is></c><c r="I4" s="2" t="inlineStr" /><c r="J4" s="2" t="inlineStr" /><c r="K4" s="2" t="inlineStr"><is><t>Racekadotryl – śpiączka wątrobowa</t></is></c><c r="L4" s="2" t="inlineStr" /><c r="M4" s="2" t="inlineStr" /><c r="N4" s="2" t="inlineStr" /><c r="O4" s="2" t="inlineStr" /><c r="P4" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q4" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="5"><c r="A5" s="2" t="inlineStr"><is><t>ZNIECZULENIA OGÓLNE</t></is></c><c r="B5" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C5" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D5" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E5" s="2" t="inlineStr"><is><t>Do leków które wykazują miejscowe działanie przeciwbólowe po podaniu na skórę należy:</t></is></c><c r="F5" s="2" t="inlineStr"><is><t>Kapsaicyna</t></is></c><c r="G5" s="2" t="inlineStr"><is><t>Ketoprofen</t></is></c><c r="H5" s="2" t="inlineStr" /><c r="I5" s="2" t="inlineStr" /><c r="J5" s="2" t="inlineStr" /><c r="K5" s="2" t="inlineStr"><is><t>Propofol</t></is></c><c r="L5" s="2" t="inlineStr"><is><t>Tiopental</t></is></c><c r="M5" s="2" t="inlineStr" /><c r="N5" s="2" t="inlineStr" /><c r="O5" s="2" t="inlineStr" /><c r="P5" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q5" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="6"><c r="A6" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B6" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C6" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D6" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E6" s="2" t="inlineStr"><is><t>Ryzyko uszkodzenia wątroby przez paracetamol rośnie w przypadku:</t></is></c><c r="F6" s="2" t="inlineStr"><is><t>Zespołu zależności alkoholowej (ZAA)</t></is></c><c r="G6" s="2" t="inlineStr"><is><t>Wygłodzenia (kacheksji)</t></is></c><c r="H6" s="2" t="inlineStr"><is><t>Indukcji enzymów mikrosomalnych wątroby</t></is></c><c r="I6" s="2" t="inlineStr"><is><t>Przedawkowania</t></is></c><c r="J6" s="2" t="inlineStr" /><c r="K6" s="2" t="inlineStr" /><c r="L6" s="2" t="inlineStr" /><c r="M6" s="2" t="inlineStr" /><c r="N6" s="2" t="inlineStr" /><c r="O6" s="2" t="inlineStr" /><c r="P6" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q6" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="7"><c r="A7" s="2" t="inlineStr"><is><t>BÓLE GŁOWY</t></is></c><c r="B7" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C7" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D7" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E7" s="2" t="inlineStr"><is><t>W przerywaniu bólów migrenowych stosuje się:</t></is></c><c r="F7" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="G7" s="2" t="inlineStr"><is><t>Dihydroergotaminę</t></is></c><c r="H7" s="2" t="inlineStr"><is><t>Zolmitryptan</t></is></c><c r="I7" s="2" t="inlineStr" /><c r="J7" s="2" t="inlineStr" /><c r="K7" s="2" t="inlineStr"><is><t>Morfinę</t></is></c><c r="L7" s="2" t="inlineStr" /><c r="M7" s="2" t="inlineStr" /><c r="N7" s="2" t="inlineStr" /><c r="O7" s="2" t="inlineStr" /><c r="P7" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q7" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="8"><c r="A8" s="2" t="inlineStr"><is><t>JASKRA</t></is></c><c r="B8" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C8" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D8" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E8" s="2" t="inlineStr"><is><t>Analogi prostaglandyny E1 mogą powodować</t></is></c><c r="F8" s="2" t="inlineStr"><is><t>Hamowanie wydzielania soku żołądkowego</t></is></c><c r="G8" s="2" t="inlineStr" /><c r="H8" s="2" t="inlineStr" /><c r="I8" s="2" t="inlineStr" /><c r="J8" s="2" t="inlineStr" /><c r="K8" s="2" t="inlineStr"><is><t>Poprawę odpływu cieczy wodnistej z oka</t></is></c><c r="L8" s="2" t="inlineStr"><is><t>Rozszerzanie naczyń krwionośnych tętniczych</t></is></c><c r="M8" s="2" t="inlineStr"><is><t>Hamowanie agregacji płytek krwi</t></is></c><c r="N8" s="2" t="inlineStr" /><c r="O8" s="2" t="inlineStr" /><c r="P8" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q8" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="9"><c r="A9" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B9" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C9" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D9" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E9" s="2" t="inlineStr"><is><t>Substytucja enzymów trzustkowych jest wskazana:</t></is></c><c r="F9" s="2" t="inlineStr"><is><t>W mukowiscydozie</t></is></c><c r="G9" s="2" t="inlineStr"><is><t>Po resekcji trzustki</t></is></c><c r="H9" s="2" t="inlineStr" /><c r="I9" s="2" t="inlineStr" /><c r="J9" s="2" t="inlineStr" /><c r="K9" s="2" t="inlineStr"><is><t>W cukrzycy typu 1</t></is></c><c r="L9" s="2" t="inlineStr"><is><t>W anoreksji</t></is></c><c r="M9" s="2" t="inlineStr" /><c r="N9" s="2" t="inlineStr" /><c r="O9" s="2" t="inlineStr" /><c r="P9" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q9" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="10"><c r="A10" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B10" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C10" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D10" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E10" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek – wskazanie do podania:</t></is></c><c r="F10" s="2" t="inlineStr"><is><t>Haloperydol – agresja u pacjentów z ograniczonym uszkodzeniem mózgu</t></is></c><c r="G10" s="2" t="inlineStr"><is><t>Betahistyna – zawroty głowy w przebiegu choroby Meniere’a</t></is></c><c r="H10" s="2" t="inlineStr"><is><t>Topiramat – profilaktyka migreny</t></is></c><c r="I10" s="2" t="inlineStr"><is><t>Lamotrygina – profilaktyka choroby afektywnej dwubiegunowej</t></is></c><c r="J10" s="2" t="inlineStr" /><c r="K10" s="2" t="inlineStr" /><c r="L10" s="2" t="inlineStr" /><c r="M10" s="2" t="inlineStr" /><c r="N10" s="2" t="inlineStr" /><c r="O10" s="2" t="inlineStr" /><c r="P10" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q10" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="11"><c r="A11" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B11" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C11" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D11" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E11" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy:</t></is></c><c r="F11" s="2" t="inlineStr"><is><t>Ma eliminację metabolitów zgodnie z kinetyką I rzędu po podaniu małych dawek kardiologicznych</t></is></c><c r="G11" s="2" t="inlineStr"><is><t>Może być przyczyną zapalenia jelita cienkiego</t></is></c><c r="H11" s="2" t="inlineStr"><is><t>Po przedawkowaniu szybciej wydala się przez nerki po dożylnym podaniu wodorowęglanu sodu</t></is></c><c r="I11" s="2" t="inlineStr" /><c r="J11" s="2" t="inlineStr" /><c r="K11" s="2" t="inlineStr"><is><t>Słabiej zapobiega powstawaniu zakrzepu na blaszce miażdżycowej</t></is></c><c r="L11" s="2" t="inlineStr" /><c r="M11" s="2" t="inlineStr" /><c r="N11" s="2" t="inlineStr" /><c r="O11" s="2" t="inlineStr" /><c r="P11" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q11" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="12"><c r="A12" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B12" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C12" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D12" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E12" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy:</t></is></c><c r="F12" s="2" t="inlineStr"><is><t>może być przyczyną wystąpienia szczególnej postaci astmy</t></is></c><c r="G12" s="2" t="inlineStr"><is><t>nieodwracalnie hamuje COX</t></is></c><c r="H12" s="2" t="inlineStr" /><c r="I12" s="2" t="inlineStr" /><c r="J12" s="2" t="inlineStr" /><c r="K12" s="2" t="inlineStr"><is><t>zwiększa ryzyko sercowo-naczyniowe</t></is></c><c r="L12" s="2" t="inlineStr"><is><t>podawany łącznie z ibuprofenem wykazuje silniejszy efekt przeciwzapalny</t></is></c><c r="M12" s="2" t="inlineStr" /><c r="N12" s="2" t="inlineStr" /><c r="O12" s="2" t="inlineStr" /><c r="P12" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q12" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="13"><c r="A13" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B13" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C13" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D13" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E13" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące leczenia heparyną niefrakcjonowaną:</t></is></c><c r="F13" s="2" t="inlineStr"><is><t>Może być podawana podskórnie ale jej biodostępność jest wtedy mała i zmienna osobniczo</t></is></c><c r="G13" s="2" t="inlineStr"><is><t>Białka osoczowe mogą zmniejszać jej działanie przeciwkrzepliwe i być przyczyną oporności na leczenie</t></is></c><c r="H13" s="2" t="inlineStr"><is><t>Przedłużenie aPTT 1,5-2 razy w stosunku do wartości wyjściowej jest pożądanym efektem terapeutycznym</t></is></c><c r="I13" s="2" t="inlineStr"><is><t>Jej antidotum jest siarczan protaminy</t></is></c><c r="J13" s="2" t="inlineStr" /><c r="K13" s="2" t="inlineStr" /><c r="L13" s="2" t="inlineStr" /><c r="M13" s="2" t="inlineStr" /><c r="N13" s="2" t="inlineStr" /><c r="O13" s="2" t="inlineStr" /><c r="P13" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q13" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="14"><c r="A14" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B14" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C14" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D14" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E14" s="2" t="inlineStr"><is><t>Przeciwwskazaniem do podania cholinolityków jest:</t></is></c><c r="F14" s="2" t="inlineStr"><is><t>Rozrost gruczołu krokowego</t></is></c><c r="G14" s="2" t="inlineStr"><is><t>Jaskra</t></is></c><c r="H14" s="2" t="inlineStr" /><c r="I14" s="2" t="inlineStr" /><c r="J14" s="2" t="inlineStr" /><c r="K14" s="2" t="inlineStr"><is><t>Choroba wrzodowa żołądka i dwunastnicy</t></is></c><c r="L14" s="2" t="inlineStr"><is><t>Choroba lokomocyjna</t></is></c><c r="M14" s="2" t="inlineStr" /><c r="N14" s="2" t="inlineStr" /><c r="O14" s="2" t="inlineStr" /><c r="P14" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q14" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="15"><c r="A15" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B15" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C15" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D15" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E15" s="2" t="inlineStr"><is><t>Warfaryna:</t></is></c><c r="F15" s="2" t="inlineStr"><is><t>Jest sotosowana w profilaktyce i leczeniu żylnej choroby zakrzepowo-zatorowej</t></is></c><c r="G15" s="2" t="inlineStr"><is><t>Może być przyczyną zespołu purpurowego palucha</t></is></c><c r="H15" s="2" t="inlineStr" /><c r="I15" s="2" t="inlineStr" /><c r="J15" s="2" t="inlineStr" /><c r="K15" s="2" t="inlineStr"><is><t>Wymaga utrzymania INR&gt;4</t></is></c><c r="L15" s="2" t="inlineStr"><is><t>Jest eliminowana niezmieniona przez nerki</t></is></c><c r="M15" s="2" t="inlineStr" /><c r="N15" s="2" t="inlineStr" /><c r="O15" s="2" t="inlineStr" /><c r="P15" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q15" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="16"><c r="A16" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B16" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C16" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D16" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E16" s="2" t="inlineStr"><is><t>Fondaparynuks:</t></is></c><c r="F16" s="2" t="inlineStr"><is><t>Jest stosowana u osób z zawałem serca z przetrwałym uniesieniem odcinka ST (STEMI) oraz bez jego uniesienia (NSTEMI)</t></is></c><c r="G16" s="2" t="inlineStr" /><c r="H16" s="2" t="inlineStr" /><c r="I16" s="2" t="inlineStr" /><c r="J16" s="2" t="inlineStr" /><c r="K16" s="2" t="inlineStr"><is><t>Wybiórczo hamuje czynnik IIa</t></is></c><c r="L16" s="2" t="inlineStr"><is><t>W zalecanych dawkach hamuje istotnie wydłuża aPTT</t></is></c><c r="M16" s="2" t="inlineStr"><is><t>Nie jest wydalany przez nerki i może być stosowany u pacjentów z klirensem kreatyniny poniżej 30ml/min</t></is></c><c r="N16" s="2" t="inlineStr" /><c r="O16" s="2" t="inlineStr" /><c r="P16" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q16" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="17"><c r="A17" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B17" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C17" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D17" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E17" s="2" t="inlineStr"><is><t>Bezpośrednim inhibitorem trombiny podawanym dożylnie jest:</t></is></c><c r="F17" s="2" t="inlineStr"><is><t>Argatroban</t></is></c><c r="G17" s="2" t="inlineStr"><is><t>Biwalirudyna</t></is></c><c r="H17" s="2" t="inlineStr" /><c r="I17" s="2" t="inlineStr" /><c r="J17" s="2" t="inlineStr" /><c r="K17" s="2" t="inlineStr"><is><t>Dabigatran</t></is></c><c r="L17" s="2" t="inlineStr"><is><t>Dalteparyna</t></is></c><c r="M17" s="2" t="inlineStr" /><c r="N17" s="2" t="inlineStr" /><c r="O17" s="2" t="inlineStr" /><c r="P17" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q17" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="18"><c r="A18" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B18" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C18" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D18" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E18" s="2" t="inlineStr"><is><t>Odwracalne inhibitory acetylocholinesterazy są stosowane w leczeniu:</t></is></c><c r="F18" s="2" t="inlineStr"><is><t>Nużliwości mięśni</t></is></c><c r="G18" s="2" t="inlineStr"><is><t>Pooperacyjnej niedrożności jelit</t></is></c><c r="H18" s="2" t="inlineStr"><is><t>Choroby Alzheimera</t></is></c><c r="I18" s="2" t="inlineStr" /><c r="J18" s="2" t="inlineStr" /><c r="K18" s="2" t="inlineStr"><is><t>Zatruć związakmi fosfoorganicznymi</t></is></c><c r="L18" s="2" t="inlineStr" /><c r="M18" s="2" t="inlineStr" /><c r="N18" s="2" t="inlineStr" /><c r="O18" s="2" t="inlineStr" /><c r="P18" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q18" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="19"><c r="A19" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B19" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C19" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D19" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E19" s="2" t="inlineStr"><is><t>Zaznacza prawidłowe pary dotyczące leczenia uzależnień i wybranego leku:</t></is></c><c r="F19" s="2" t="inlineStr"><is><t>Uzależnienie od alkoholu – nalmefen</t></is></c><c r="G19" s="2" t="inlineStr"><is><t>Uzależnienie od heroiny – metadon</t></is></c><c r="H19" s="2" t="inlineStr" /><c r="I19" s="2" t="inlineStr" /><c r="J19" s="2" t="inlineStr" /><c r="K19" s="2" t="inlineStr"><is><t>Uzależnienie od nikotyny – klonidyna</t></is></c><c r="L19" s="2" t="inlineStr"><is><t>Uzależnienie od amfetaminy – wereniklina</t></is></c><c r="M19" s="2" t="inlineStr" /><c r="N19" s="2" t="inlineStr" /><c r="O19" s="2" t="inlineStr" /><c r="P19" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q19" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="20"><c r="A20" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B20" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C20" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D20" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E20" s="2" t="inlineStr"><is><t>Wskaż prawidłowe pary płyn infuzyjny – możliwe działania niepożądane:</t></is></c><c r="F20" s="2" t="inlineStr"><is><t>5% roztwór glukozy – hiponatremia</t></is></c><c r="G20" s="2" t="inlineStr"><is><t>HES (hydroksyetylowana skrobia) – ostre uszkodzenie nerek</t></is></c><c r="H20" s="2" t="inlineStr"><is><t>5% roztwór albuminy – anafilaksja</t></is></c><c r="I20" s="2" t="inlineStr"><is><t>Dekstran 70000 – działanie przeciwkrzepliwe</t></is></c><c r="J20" s="2" t="inlineStr" /><c r="K20" s="2" t="inlineStr" /><c r="L20" s="2" t="inlineStr" /><c r="M20" s="2" t="inlineStr" /><c r="N20" s="2" t="inlineStr" /><c r="O20" s="2" t="inlineStr" /><c r="P20" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q20" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="21"><c r="A21" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B21" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C21" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D21" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E21" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące leczenia hipotensyjnego:</t></is></c><c r="F21" s="2" t="inlineStr"><is><t>Tiazydy mogą bezpośrednio oddziaływać na ścianę naczyń i zmniejszać systemowy opór naczyniowy</t></is></c><c r="G21" s="2" t="inlineStr"><is><t>Pełny efekt hipotensyjny występuje po kilkunastu dniach leczenia</t></is></c><c r="H21" s="2" t="inlineStr"><is><t>Blokada kotransportera Na-Cl w kanaliku dystalnym prowadzi do zwiększeniu natriurezy</t></is></c><c r="I21" s="2" t="inlineStr" /><c r="J21" s="2" t="inlineStr" /><c r="K21" s="2" t="inlineStr"><is><t>Ich skuteczność w leczeniu przewlekłym wynika przede wszystkim ze zmniejszenia objętości osocza i rzutu serca</t></is></c><c r="L21" s="2" t="inlineStr" /><c r="M21" s="2" t="inlineStr" /><c r="N21" s="2" t="inlineStr" /><c r="O21" s="2" t="inlineStr" /><c r="P21" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q21" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="22"><c r="A22" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B22" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C22" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D22" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E22" s="2" t="inlineStr"><is><t>Suksametonium może być przyczyną:</t></is></c><c r="F22" s="2" t="inlineStr"><is><t>Drżenia włókienkowego mięśni szkieletowych</t></is></c><c r="G22" s="2" t="inlineStr"><is><t>Zaburzeń oddychania</t></is></c><c r="H22" s="2" t="inlineStr"><is><t>Zespołu hipertermii złośliwej</t></is></c><c r="I22" s="2" t="inlineStr"><is><t>Długotrwałego efektu zwiotczającego u osób z dysfunkcją acetylocholinesterazy</t></is></c><c r="J22" s="2" t="inlineStr" /><c r="K22" s="2" t="inlineStr" /><c r="L22" s="2" t="inlineStr" /><c r="M22" s="2" t="inlineStr" /><c r="N22" s="2" t="inlineStr" /><c r="O22" s="2" t="inlineStr" /><c r="P22" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q22" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="23"><c r="A23" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B23" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C23" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D23" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E23" s="2" t="inlineStr"><is><t>W celu łagodzenia suchego kaszlu można wybrać:</t></is></c><c r="F23" s="2" t="inlineStr"><is><t>Dekstrometorfan</t></is></c><c r="G23" s="2" t="inlineStr"><is><t>Kodeinę</t></is></c><c r="H23" s="2" t="inlineStr"><is><t>Butamirat</t></is></c><c r="I23" s="2" t="inlineStr" /><c r="J23" s="2" t="inlineStr" /><c r="K23" s="2" t="inlineStr"><is><t>Bromheksynę</t></is></c><c r="L23" s="2" t="inlineStr" /><c r="M23" s="2" t="inlineStr" /><c r="N23" s="2" t="inlineStr" /><c r="O23" s="2" t="inlineStr" /><c r="P23" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q23" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="24"><c r="A24" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B24" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C24" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D24" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E24" s="2" t="inlineStr"><is><t>Albendazol stosowany jest w jelitowej infestacji:</t></is></c><c r="F24" s="2" t="inlineStr"><is><t>Glistą ludzką</t></is></c><c r="G24" s="2" t="inlineStr"><is><t>Tasiemcem uzbrojonym</t></is></c><c r="H24" s="2" t="inlineStr"><is><t>Owsikami</t></is></c><c r="I24" s="2" t="inlineStr" /><c r="J24" s="2" t="inlineStr" /><c r="K24" s="2" t="inlineStr"><is><t>Lambliami</t></is></c><c r="L24" s="2" t="inlineStr" /><c r="M24" s="2" t="inlineStr" /><c r="N24" s="2" t="inlineStr" /><c r="O24" s="2" t="inlineStr" /><c r="P24" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q24" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="25"><c r="A25" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B25" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C25" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D25" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E25" s="2" t="inlineStr"><is><t>Napad paniki należy leczyć stosując doraźnie:</t></is></c><c r="F25" s="2" t="inlineStr"><is><t>Techniki relaksacyjne</t></is></c><c r="G25" s="2" t="inlineStr"><is><t>Alprazolam</t></is></c><c r="H25" s="2" t="inlineStr" /><c r="I25" s="2" t="inlineStr" /><c r="J25" s="2" t="inlineStr" /><c r="K25" s="2" t="inlineStr"><is><t>Pregabalinę</t></is></c><c r="L25" s="2" t="inlineStr"><is><t>Fluoksetynę</t></is></c><c r="M25" s="2" t="inlineStr" /><c r="N25" s="2" t="inlineStr" /><c r="O25" s="2" t="inlineStr" /><c r="P25" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q25" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="26"><c r="A26" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B26" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C26" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D26" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E26" s="2" t="inlineStr"><is><t>Fenoterol może być przyczyną:</t></is></c><c r="F26" s="2" t="inlineStr"><is><t>Tachykardii</t></is></c><c r="G26" s="2" t="inlineStr"><is><t>Drżenia mięśni</t></is></c><c r="H26" s="2" t="inlineStr"><is><t>Hiperglikemii</t></is></c><c r="I26" s="2" t="inlineStr"><is><t>Hamowania skurczów ciężarnej macicy</t></is></c><c r="J26" s="2" t="inlineStr" /><c r="K26" s="2" t="inlineStr" /><c r="L26" s="2" t="inlineStr" /><c r="M26" s="2" t="inlineStr" /><c r="N26" s="2" t="inlineStr" /><c r="O26" s="2" t="inlineStr" /><c r="P26" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q26" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="27"><c r="A27" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B27" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C27" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D27" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E27" s="2" t="inlineStr"><is><t>Długo działające beta2-mimetyki (LABA):</t></is></c><c r="F27" s="2" t="inlineStr"><is><t>Podawane przewlekle powodują down-regulację receptorów beta2-adrenergicznych w oskrzelach</t></is></c><c r="G27" s="2" t="inlineStr" /><c r="H27" s="2" t="inlineStr" /><c r="I27" s="2" t="inlineStr" /><c r="J27" s="2" t="inlineStr" /><c r="K27" s="2" t="inlineStr"><is><t>Nie powinny być podawane razem z glikokortykosteroidami które blokują wytwarzanie białek receptorów beta2-adrenergicznych</t></is></c><c r="L27" s="2" t="inlineStr"><is><t>Mogą być przyczyną istotnej klinicznie hieprkaliemi</t></is></c><c r="M27" s="2" t="inlineStr"><is><t>Wykazują działanie przeciwzapalne</t></is></c><c r="N27" s="2" t="inlineStr" /><c r="O27" s="2" t="inlineStr" /><c r="P27" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q27" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="28"><c r="A28" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B28" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C28" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D28" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E28" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenie dotyczące NLPZ:</t></is></c><c r="F28" s="2" t="inlineStr"><is><t>Ketoprofen powoduje większe ryzyko krwawienia z górnego odcinka przewodu pokarmowego niż ibuprofen</t></is></c><c r="G28" s="2" t="inlineStr" /><c r="H28" s="2" t="inlineStr" /><c r="I28" s="2" t="inlineStr" /><c r="J28" s="2" t="inlineStr" /><c r="K28" s="2" t="inlineStr"><is><t>Meloksykam jest preferencyjnym inhibitorem COX-1</t></is></c><c r="L28" s="2" t="inlineStr"><is><t>Zastąpienie drogi doustnej podania diklofenaku drogą doodbytniczą zmniejsza ryzyko wystąpienia działań niepożądanych</t></is></c><c r="M28" s="2" t="inlineStr"><is><t>Nimesulid należy do najmniej hepatotoksycznych NLPZ</t></is></c><c r="N28" s="2" t="inlineStr" /><c r="O28" s="2" t="inlineStr" /><c r="P28" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q28" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="29"><c r="A29" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B29" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C29" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D29" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E29" s="2" t="inlineStr"><is><t>Lekiem prkeursorowym jest:</t></is></c><c r="F29" s="2" t="inlineStr"><is><t>Enalapryl</t></is></c><c r="G29" s="2" t="inlineStr"><is><t>Cyklezonid</t></is></c><c r="H29" s="2" t="inlineStr"><is><t>Lewodopa</t></is></c><c r="I29" s="2" t="inlineStr" /><c r="J29" s="2" t="inlineStr" /><c r="K29" s="2" t="inlineStr"><is><t>Furosemid</t></is></c><c r="L29" s="2" t="inlineStr" /><c r="M29" s="2" t="inlineStr" /><c r="N29" s="2" t="inlineStr" /><c r="O29" s="2" t="inlineStr" /><c r="P29" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q29" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="30"><c r="A30" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B30" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C30" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D30" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E30" s="2" t="inlineStr"><is><t>Cyklosporyna:</t></is></c><c r="F30" s="2" t="inlineStr"><is><t>Jest stosowana w zapobieganiu odrzucania przeszczepu allogenicznego narządów unaczynionych</t></is></c><c r="G30" s="2" t="inlineStr"><is><t>Zwiększa ryzyko chorób rozrostowych układu chłonnego</t></is></c><c r="H30" s="2" t="inlineStr" /><c r="I30" s="2" t="inlineStr" /><c r="J30" s="2" t="inlineStr" /><c r="K30" s="2" t="inlineStr"><is><t>Jest rekombinowanym w pełni ludzkim przeciwciałem monoklonalnym</t></is></c><c r="L30" s="2" t="inlineStr"><is><t>Neutralizuje biologiczną aktywność TNF</t></is></c><c r="M30" s="2" t="inlineStr" /><c r="N30" s="2" t="inlineStr" /><c r="O30" s="2" t="inlineStr" /><c r="P30" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q30" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="31"><c r="A31" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B31" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C31" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D31" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E31" s="2" t="inlineStr"><is><t>Cyklosporyna</t></is></c><c r="F31" s="2" t="inlineStr"><is><t>Jest eliminowana przez wątrobę</t></is></c><c r="G31" s="2" t="inlineStr"><is><t>Jest stosowana w celu zapobiegania odrzucania przeszczepów</t></is></c><c r="H31" s="2" t="inlineStr" /><c r="I31" s="2" t="inlineStr" /><c r="J31" s="2" t="inlineStr" /><c r="K31" s="2" t="inlineStr"><is><t>Jest aktywatorem kalcyneuryny</t></is></c><c r="L31" s="2" t="inlineStr"><is><t>Może powodować atrofię dziąseł</t></is></c><c r="M31" s="2" t="inlineStr" /><c r="N31" s="2" t="inlineStr" /><c r="O31" s="2" t="inlineStr" /><c r="P31" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q31" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="32"><c r="A32" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B32" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C32" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D32" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E32" s="2" t="inlineStr"><is><t>Do leków o udowodnionym korzystnym działaniu w profilaktyce wtórnej niedokrwiennego udaru mózgu należy:</t></is></c><c r="F32" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy</t></is></c><c r="G32" s="2" t="inlineStr"><is><t>Atorwastatyna</t></is></c><c r="H32" s="2" t="inlineStr"><is><t>Klopidogrel</t></is></c><c r="I32" s="2" t="inlineStr" /><c r="J32" s="2" t="inlineStr" /><c r="K32" s="2" t="inlineStr"><is><t>Kwas traneksamowy</t></is></c><c r="L32" s="2" t="inlineStr" /><c r="M32" s="2" t="inlineStr" /><c r="N32" s="2" t="inlineStr" /><c r="O32" s="2" t="inlineStr" /><c r="P32" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q32" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="33"><c r="A33" s="2" t="inlineStr"><is><t>CHOROBA PARKINSONA</t></is></c><c r="B33" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C33" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D33" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E33" s="2" t="inlineStr"><is><t>Lewodopa:</t></is></c><c r="F33" s="2" t="inlineStr"><is><t>Jest jednym z najskuteczniejszych leków stosowanych w terapii choroby Parkinsona</t></is></c><c r="G33" s="2" t="inlineStr"><is><t>Ma krótki okres półtrwania i dlatego wymaga wielokrotnego podawania w ciągu doby</t></is></c><c r="H33" s="2" t="inlineStr"><is><t>Podczas długotrwałego leczenia może wywołać fluktuacje ruchowe i dyskinezy</t></is></c><c r="I33" s="2" t="inlineStr"><is><t>Może wywoływać działania niepożądane ze strony przewodu pokarmowego</t></is></c><c r="J33" s="2" t="inlineStr" /><c r="K33" s="2" t="inlineStr" /><c r="L33" s="2" t="inlineStr" /><c r="M33" s="2" t="inlineStr" /><c r="N33" s="2" t="inlineStr" /><c r="O33" s="2" t="inlineStr" /><c r="P33" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q33" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="34"><c r="A34" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B34" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C34" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D34" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E34" s="2" t="inlineStr"><is><t>Kokaina:</t></is></c><c r="F34" s="2" t="inlineStr"><is><t>Hamuje wychwyt zwrotny dopaminy w szczelinie synaptycznej</t></is></c><c r="G34" s="2" t="inlineStr"><is><t>Może powodować wystąpienie zawału mięśnia sercowego</t></is></c><c r="H34" s="2" t="inlineStr"><is><t>Może powodować krwawienia wewnątrzczaszkowe</t></is></c><c r="I34" s="2" t="inlineStr" /><c r="J34" s="2" t="inlineStr" /><c r="K34" s="2" t="inlineStr"><is><t>Hamuje aktywność receptora dla kwasu glutaminowego</t></is></c><c r="L34" s="2" t="inlineStr" /><c r="M34" s="2" t="inlineStr" /><c r="N34" s="2" t="inlineStr" /><c r="O34" s="2" t="inlineStr" /><c r="P34" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q34" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="35"><c r="A35" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B35" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C35" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D35" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E35" s="2" t="inlineStr"><is><t>W alergicznym zapaleniu spojówek może stosować dospojówkowo:</t></is></c><c r="F35" s="2" t="inlineStr"><is><t>Antazolinę</t></is></c><c r="G35" s="2" t="inlineStr"><is><t>Azelastynę</t></is></c><c r="H35" s="2" t="inlineStr"><is><t>Kromoglikan sodowy</t></is></c><c r="I35" s="2" t="inlineStr"><is><t>Olopatadynę</t></is></c><c r="J35" s="2" t="inlineStr" /><c r="K35" s="2" t="inlineStr" /><c r="L35" s="2" t="inlineStr" /><c r="M35" s="2" t="inlineStr" /><c r="N35" s="2" t="inlineStr" /><c r="O35" s="2" t="inlineStr" /><c r="P35" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q35" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="36"><c r="A36" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B36" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C36" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D36" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E36" s="2" t="inlineStr"><is><t>Stosowanie preparatu złożonego bupropionu z naltreksonem w leczeniu otyłości:</t></is></c><c r="F36" s="2" t="inlineStr"><is><t>Ma wpływ na ośrodkowy układ nagrody</t></is></c><c r="G36" s="2" t="inlineStr"><is><t>Zwiększa i wydłuża uczucie sytości</t></is></c><c r="H36" s="2" t="inlineStr"><is><t>Ma zwiększoną skuteczność kliniczną ze względu na efekt synergistyczny bupropionu i naltreksonu</t></is></c><c r="I36" s="2" t="inlineStr" /><c r="J36" s="2" t="inlineStr" /><c r="K36" s="2" t="inlineStr"><is><t>Jest wskazane dla wszystkich osób z wyjściową wartością BMI wynoszącą ≥27</t></is></c><c r="L36" s="2" t="inlineStr" /><c r="M36" s="2" t="inlineStr" /><c r="N36" s="2" t="inlineStr" /><c r="O36" s="2" t="inlineStr" /><c r="P36" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q36" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="37"><c r="A37" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B37" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C37" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D37" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E37" s="2" t="inlineStr"><is><t>Dodatek adrenaliny do lidokainy w lekach do znieczulania miejscowego może powodować:</t></is></c><c r="F37" s="2" t="inlineStr"><is><t>Zwiększone ryzyko martwicy tkanek po podaniach obwodowych</t></is></c><c r="G37" s="2" t="inlineStr"><is><t>Wydłużenie czasu działania lidokainy</t></is></c><c r="H37" s="2" t="inlineStr" /><c r="I37" s="2" t="inlineStr" /><c r="J37" s="2" t="inlineStr" /><c r="K37" s="2" t="inlineStr"><is><t>Zwiększone niebezpieczeństwo zatrzymania oddechu</t></is></c><c r="L37" s="2" t="inlineStr"><is><t>Zahamowanie metabolizmu lidokainy</t></is></c><c r="M37" s="2" t="inlineStr" /><c r="N37" s="2" t="inlineStr" /><c r="O37" s="2" t="inlineStr" /><c r="P37" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q37" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="38"><c r="A38" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B38" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C38" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D38" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E38" s="2" t="inlineStr"><is><t>Digoksyna</t></is></c><c r="F38" s="2" t="inlineStr"><is><t>Podtrzymuje aktywację baroreceptorów zatoki szyjnej przy obniżeniu ciśnienia krwi u osób z niewydolnością serca</t></is></c><c r="G38" s="2" t="inlineStr"><is><t>Podana doustnie może być nieskuteczna z powodu dezaktywacji przez bakterie jelitowe</t></is></c><c r="H38" s="2" t="inlineStr" /><c r="I38" s="2" t="inlineStr" /><c r="J38" s="2" t="inlineStr" /><c r="K38" s="2" t="inlineStr"><is><t>Powoduje kardiowersję migotania przedsionków do rytmu zatokowego</t></is></c><c r="L38" s="2" t="inlineStr"><is><t>Jest lekiem o korzystnym działaniu rokowniczym w skurczowej niewydolności serca</t></is></c><c r="M38" s="2" t="inlineStr" /><c r="N38" s="2" t="inlineStr" /><c r="O38" s="2" t="inlineStr" /><c r="P38" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q38" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="39"><c r="A39" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B39" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C39" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D39" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E39" s="2" t="inlineStr"><is><t>Digoksyna:</t></is></c><c r="F39" s="2" t="inlineStr"><is><t>aktywuje układ przywspółczulny</t></is></c><c r="G39" s="2" t="inlineStr"><is><t>wywiera arytmie i zaburzenia przewodzenia</t></is></c><c r="H39" s="2" t="inlineStr"><is><t>jest stosowana w celu kontroli częstotliwości rytmu komór u chorych z migotaniem przedsionków</t></is></c><c r="I39" s="2" t="inlineStr"><is><t>w zatruciu można zastosować fragmenty Fab przeciwciał wiążących</t></is></c><c r="J39" s="2" t="inlineStr" /><c r="K39" s="2" t="inlineStr" /><c r="L39" s="2" t="inlineStr" /><c r="M39" s="2" t="inlineStr" /><c r="N39" s="2" t="inlineStr" /><c r="O39" s="2" t="inlineStr" /><c r="P39" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q39" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="40"><c r="A40" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B40" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C40" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D40" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E40" s="2" t="inlineStr"><is><t>Digoksyna:</t></is></c><c r="F40" s="2" t="inlineStr"><is><t>zmniejsza aktywację układu współczulnego u osób z niewydolnością serca</t></is></c><c r="G40" s="2" t="inlineStr"><is><t>może sprzyjać wystąpieniu depresji</t></is></c><c r="H40" s="2" t="inlineStr"><is><t>jest stosowana w celu kontroli rytmu serca w utrwalonym migotaniu przedsionków</t></is></c><c r="I40" s="2" t="inlineStr"><is><t>może być nieskuteczna z powodu dezaktywacji przez bakterie jelitowe</t></is></c><c r="J40" s="2" t="inlineStr" /><c r="K40" s="2" t="inlineStr" /><c r="L40" s="2" t="inlineStr" /><c r="M40" s="2" t="inlineStr" /><c r="N40" s="2" t="inlineStr" /><c r="O40" s="2" t="inlineStr" /><c r="P40" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q40" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="41"><c r="A41" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B41" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C41" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D41" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E41" s="2" t="inlineStr"><is><t>Teoretyczną przesłanką stosowania beta-adrenolityków w przewlekłej skurczowej niewydolności serca jest:</t></is></c><c r="F41" s="2" t="inlineStr"><is><t>Odwracanie beta-down regulacji</t></is></c><c r="G41" s="2" t="inlineStr"><is><t>Zapobieganie proarytmicznemu działaniu katecholamin</t></is></c><c r="H41" s="2" t="inlineStr" /><c r="I41" s="2" t="inlineStr" /><c r="J41" s="2" t="inlineStr" /><c r="K41" s="2" t="inlineStr"><is><t>Korzystny bezpośredni wpływ hemodynamiczny</t></is></c><c r="L41" s="2" t="inlineStr"><is><t>Zwiększenie naprężenia ściany lewej komory</t></is></c><c r="M41" s="2" t="inlineStr" /><c r="N41" s="2" t="inlineStr" /><c r="O41" s="2" t="inlineStr" /><c r="P41" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q41" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="42"><c r="A42" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B42" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C42" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D42" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E42" s="2" t="inlineStr"><is><t>Rupatadyna:</t></is></c><c r="F42" s="2" t="inlineStr"><is><t>Ma minimalny potencjał sedatywny</t></is></c><c r="G42" s="2" t="inlineStr"><is><t>Oprócz antagonizmu wobec receptora H1 wykazuje przeciwzapalną aktywność pozareceptorową</t></is></c><c r="H42" s="2" t="inlineStr"><is><t>W znacznym stopniu ulega efektowi pierwszego przejścia z powstaniem aktywnych metabolitów</t></is></c><c r="I42" s="2" t="inlineStr"><is><t>W dawkach zalecanych nie wydłuża skorygowanego odstępu cQT</t></is></c><c r="J42" s="2" t="inlineStr" /><c r="K42" s="2" t="inlineStr" /><c r="L42" s="2" t="inlineStr" /><c r="M42" s="2" t="inlineStr" /><c r="N42" s="2" t="inlineStr" /><c r="O42" s="2" t="inlineStr" /><c r="P42" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q42" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="43"><c r="A43" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B43" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C43" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D43" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E43" s="2" t="inlineStr"><is><t>Rupatadyna:</t></is></c><c r="F43" s="2" t="inlineStr"><is><t>jest selektywnym niesedatywnym antagonistą receptorów H1</t></is></c><c r="G43" s="2" t="inlineStr"><is><t>hamuje degranulację komórek tucznych in vitro</t></is></c><c r="H43" s="2" t="inlineStr"><is><t>ma aktywny metabolit – desloratadynę zaliczaną do 3 generacji leków przeciwhistaminowych</t></is></c><c r="I43" s="2" t="inlineStr"><is><t>w dawkach zalecanych nie wydłuża odstępu QTc</t></is></c><c r="J43" s="2" t="inlineStr" /><c r="K43" s="2" t="inlineStr" /><c r="L43" s="2" t="inlineStr" /><c r="M43" s="2" t="inlineStr" /><c r="N43" s="2" t="inlineStr" /><c r="O43" s="2" t="inlineStr" /><c r="P43" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q43" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="44"><c r="A44" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B44" s="2" t="inlineStr"><is><t>Przeciwwskazania</t></is></c><c r="C44" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D44" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E44" s="2" t="inlineStr"><is><t>U pacjentów z eGFR&lt;30ml/min należy rezygnować ze stosowania:</t></is></c><c r="F44" s="2" t="inlineStr"><is><t>Metyforminy</t></is></c><c r="G44" s="2" t="inlineStr"><is><t>Hydrochlorotiazydu</t></is></c><c r="H44" s="2" t="inlineStr" /><c r="I44" s="2" t="inlineStr" /><c r="J44" s="2" t="inlineStr" /><c r="K44" s="2" t="inlineStr"><is><t>Metoprololu</t></is></c><c r="L44" s="2" t="inlineStr"><is><t>Amlodypiny</t></is></c><c r="M44" s="2" t="inlineStr" /><c r="N44" s="2" t="inlineStr" /><c r="O44" s="2" t="inlineStr" /><c r="P44" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q44" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="45"><c r="A45" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B45" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C45" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D45" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E45" s="2" t="inlineStr"><is><t>Wenlafaksyna:</t></is></c><c r="F45" s="2" t="inlineStr"><is><t>Może być podawana w uogólnionych zaburzeniach lękowych</t></is></c><c r="G45" s="2" t="inlineStr"><is><t>Stosowana razem z tryptanami może powodować wystąpienie zespołu serotoninowego</t></is></c><c r="H45" s="2" t="inlineStr" /><c r="I45" s="2" t="inlineStr" /><c r="J45" s="2" t="inlineStr" /><c r="K45" s="2" t="inlineStr"><is><t>Ma istotne działanie cholinolityczne</t></is></c><c r="L45" s="2" t="inlineStr"><is><t>Można ją bezpiecznie stosować w terapii skojarzonej z inhibitorami MAO</t></is></c><c r="M45" s="2" t="inlineStr" /><c r="N45" s="2" t="inlineStr" /><c r="O45" s="2" t="inlineStr" /><c r="P45" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q45" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="46"><c r="A46" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B46" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C46" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D46" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E46" s="2" t="inlineStr"><is><t>Czy słuszna jest przedstawiona interpretacja działania leku na podstawie nazwy międzynarodowej:</t></is></c><c r="F46" s="2" t="inlineStr"><is><t>Paliwizumab – humanizowane przeciwciało monoklonalne o działaniu p￾wirusowym</t></is></c><c r="G46" s="2" t="inlineStr"><is><t>Ekulizumab – humanizowane przeciwciało monoklonalne o wpływie na układ odpornościowy</t></is></c><c r="H46" s="2" t="inlineStr" /><c r="I46" s="2" t="inlineStr" /><c r="J46" s="2" t="inlineStr" /><c r="K46" s="2" t="inlineStr"><is><t>Ofatumumab – mysie przeciwciało monoklonalne o wpływie p-nowotworowym</t></is></c><c r="L46" s="2" t="inlineStr"><is><t>Pomalidomid – mysie przeciwciało monoklonalne o wpływie na układ odpornościowy</t></is></c><c r="M46" s="2" t="inlineStr" /><c r="N46" s="2" t="inlineStr" /><c r="O46" s="2" t="inlineStr" /><c r="P46" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q46" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="47"><c r="A47" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B47" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C47" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D47" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E47" s="2" t="inlineStr"><is><t>Do przeciwciał monoklonalnych anty-TNF należy:</t></is></c><c r="F47" s="2" t="inlineStr"><is><t>Adalimumab</t></is></c><c r="G47" s="2" t="inlineStr" /><c r="H47" s="2" t="inlineStr" /><c r="I47" s="2" t="inlineStr" /><c r="J47" s="2" t="inlineStr" /><c r="K47" s="2" t="inlineStr"><is><t>Omalizumab</t></is></c><c r="L47" s="2" t="inlineStr"><is><t>Trastuzumab</t></is></c><c r="M47" s="2" t="inlineStr"><is><t>Rytuksymab</t></is></c><c r="N47" s="2" t="inlineStr" /><c r="O47" s="2" t="inlineStr" /><c r="P47" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q47" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="48"><c r="A48" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B48" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C48" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D48" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E48" s="2" t="inlineStr"><is><t>Werapamil można stosować w:</t></is></c><c r="F48" s="2" t="inlineStr"><is><t>Postaci naczynioskurczowej choroby niedokrwiennej serca</t></is></c><c r="G48" s="2" t="inlineStr"><is><t>Napadowym częstoskurczu z łącza przedsionkowo-komorowego</t></is></c><c r="H48" s="2" t="inlineStr" /><c r="I48" s="2" t="inlineStr" /><c r="J48" s="2" t="inlineStr" /><c r="K48" s="2" t="inlineStr"><is><t>Bradykardii</t></is></c><c r="L48" s="2" t="inlineStr"><is><t>Migotaniu przedsionków u osób z zespołem preekscytacji</t></is></c><c r="M48" s="2" t="inlineStr" /><c r="N48" s="2" t="inlineStr" /><c r="O48" s="2" t="inlineStr" /><c r="P48" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q48" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="49"><c r="A49" s="2" t="inlineStr"><is><t>NIEWYDOLNOŚĆ SERCA</t></is></c><c r="B49" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C49" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D49" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E49" s="2" t="inlineStr"><is><t>Inhibitory neprylizyny:</t></is></c><c r="F49" s="2" t="inlineStr"><is><t>Zmniejszają przebudowę mięśnia sercowego</t></is></c><c r="G49" s="2" t="inlineStr"><is><t>Zwiększają stężenie angiotensyny II</t></is></c><c r="H49" s="2" t="inlineStr"><is><t>Są stosowane w przewlekłej niewydolności serca z upośledzoną frakcją wyrzutową</t></is></c><c r="I49" s="2" t="inlineStr" /><c r="J49" s="2" t="inlineStr" /><c r="K49" s="2" t="inlineStr"><is><t>Rozkładają peptydy natriuretyczne</t></is></c><c r="L49" s="2" t="inlineStr" /><c r="M49" s="2" t="inlineStr" /><c r="N49" s="2" t="inlineStr" /><c r="O49" s="2" t="inlineStr" /><c r="P49" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q49" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="50"><c r="A50" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B50" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C50" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D50" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E50" s="2" t="inlineStr"><is><t>Biodostępność leku A po jednorazowym podaniu doustnym wynosi 50%. Tmax wynosi 30min, Cmax 2µg/dl. Oznacza to, że:</t></is></c><c r="F50" s="2" t="inlineStr"><is><t>Lek A może podlegać nawet w 50% efektowi pierwszego przejścia</t></is></c><c r="G50" s="2" t="inlineStr" /><c r="H50" s="2" t="inlineStr" /><c r="I50" s="2" t="inlineStr" /><c r="J50" s="2" t="inlineStr" /><c r="K50" s="2" t="inlineStr"><is><t>Dawka wynosiła 4µg</t></is></c><c r="L50" s="2" t="inlineStr"><is><t>Lek A słabo się wiąże z białkami krwi</t></is></c><c r="M50" s="2" t="inlineStr"><is><t>Okres półtrwania leku A wynosi również około 30min</t></is></c><c r="N50" s="2" t="inlineStr" /><c r="O50" s="2" t="inlineStr" /><c r="P50" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q50" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="51"><c r="A51" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B51" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C51" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D51" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E51" s="2" t="inlineStr"><is><t>Podanie doodbytnicze leku:</t></is></c><c r="F51" s="2" t="inlineStr"><is><t>Może łatwo doprowadzić do miejscowego uszkodzenia błony śluzowej odbytnicy</t></is></c><c r="G51" s="2" t="inlineStr" /><c r="H51" s="2" t="inlineStr" /><c r="I51" s="2" t="inlineStr" /><c r="J51" s="2" t="inlineStr" /><c r="K51" s="2" t="inlineStr"><is><t>Zwiększa efekt pierwszego przejścia</t></is></c><c r="L51" s="2" t="inlineStr"><is><t>Jest metodą z wyboru u dzieci</t></is></c><c r="M51" s="2" t="inlineStr"><is><t>Wymaga podania większej dawki leku w porównaniu do podania doustnego</t></is></c><c r="N51" s="2" t="inlineStr" /><c r="O51" s="2" t="inlineStr" /><c r="P51" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q51" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="52"><c r="A52" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B52" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C52" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D52" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E52" s="2" t="inlineStr"><is><t>Zaburzenia erekcji mogą być spowodowane stosowaniem:</t></is></c><c r="F52" s="2" t="inlineStr"><is><t>Inhibitorów 5-alfa reduktazy</t></is></c><c r="G52" s="2" t="inlineStr"><is><t>Tiazydów moczopędnych</t></is></c><c r="H52" s="2" t="inlineStr"><is><t>Beta-adrenolityków niekardioselektywnych</t></is></c><c r="I52" s="2" t="inlineStr"><is><t>Inhibitorów wychwytu zwrotnego serotoniny</t></is></c><c r="J52" s="2" t="inlineStr" /><c r="K52" s="2" t="inlineStr" /><c r="L52" s="2" t="inlineStr" /><c r="M52" s="2" t="inlineStr" /><c r="N52" s="2" t="inlineStr" /><c r="O52" s="2" t="inlineStr" /><c r="P52" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q52" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="53"><c r="A53" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B53" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C53" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D53" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E53" s="2" t="inlineStr"><is><t>Doneuronalny wychwyt monoamin jest hamowany przez:</t></is></c><c r="F53" s="2" t="inlineStr"><is><t>Citalopram</t></is></c><c r="G53" s="2" t="inlineStr"><is><t>Reboksetynę</t></is></c><c r="H53" s="2" t="inlineStr" /><c r="I53" s="2" t="inlineStr" /><c r="J53" s="2" t="inlineStr" /><c r="K53" s="2" t="inlineStr"><is><t>Tianeptynę</t></is></c><c r="L53" s="2" t="inlineStr"><is><t>Mirtazapinę</t></is></c><c r="M53" s="2" t="inlineStr" /><c r="N53" s="2" t="inlineStr" /><c r="O53" s="2" t="inlineStr" /><c r="P53" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q53" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="54"><c r="A54" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B54" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C54" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D54" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E54" s="2" t="inlineStr"><is><t>W leczeniu gruźlicy płucnej lekowrażliwej:</t></is></c><c r="F54" s="2" t="inlineStr"><is><t>Leczenie wyjaławiające powinno trwać co najmniej 4 miesiące</t></is></c><c r="G54" s="2" t="inlineStr"><is><t>U kobiet ciężarnych podaje się leki według zwykłego schematu z wyłączeniem streptomycyny</t></is></c><c r="H54" s="2" t="inlineStr" /><c r="I54" s="2" t="inlineStr" /><c r="J54" s="2" t="inlineStr" /><c r="K54" s="2" t="inlineStr"><is><t>W intensywnej fazie leczenia przez 2 miesiące podaje się 2 leki – rifampicynę i izoniazyd</t></is></c><c r="L54" s="2" t="inlineStr"><is><t>W fazie kontynuacji każdy pacjent powinien otrzymać etambutol</t></is></c><c r="M54" s="2" t="inlineStr" /><c r="N54" s="2" t="inlineStr" /><c r="O54" s="2" t="inlineStr" /><c r="P54" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q54" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="55"><c r="A55" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B55" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C55" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D55" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E55" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-wskazanie:</t></is></c><c r="F55" s="2" t="inlineStr"><is><t>Sulpiryd – schizofrenia</t></is></c><c r="G55" s="2" t="inlineStr"><is><t>Metylofenidat – ADHD</t></is></c><c r="H55" s="2" t="inlineStr" /><c r="I55" s="2" t="inlineStr" /><c r="J55" s="2" t="inlineStr" /><c r="K55" s="2" t="inlineStr"><is><t>Moklobemid – bezsenność</t></is></c><c r="L55" s="2" t="inlineStr"><is><t>Sertindol – depresja</t></is></c><c r="M55" s="2" t="inlineStr" /><c r="N55" s="2" t="inlineStr" /><c r="O55" s="2" t="inlineStr" /><c r="P55" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q55" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="56"><c r="A56" s="2" t="inlineStr"><is><t>LEKI NASENNE</t></is></c><c r="B56" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C56" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D56" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E56" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – wskazanie:</t></is></c><c r="F56" s="2" t="inlineStr"><is><t>zolpidem - bezsenność</t></is></c><c r="G56" s="2" t="inlineStr"><is><t>rotygotyna – zespół niespokojnych nóg</t></is></c><c r="H56" s="2" t="inlineStr"><is><t>alprazolam - napady paniki</t></is></c><c r="I56" s="2" t="inlineStr"><is><t>fluoksetyna – zaburzenia kompulsywne</t></is></c><c r="J56" s="2" t="inlineStr" /><c r="K56" s="2" t="inlineStr" /><c r="L56" s="2" t="inlineStr" /><c r="M56" s="2" t="inlineStr" /><c r="N56" s="2" t="inlineStr" /><c r="O56" s="2" t="inlineStr" /><c r="P56" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q56" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="57"><c r="A57" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B57" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C57" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D57" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E57" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – wskazanie:</t></is></c><c r="F57" s="2" t="inlineStr"><is><t>ranolazyna - stabilna choroba niedokrwienna serca</t></is></c><c r="G57" s="2" t="inlineStr" /><c r="H57" s="2" t="inlineStr" /><c r="I57" s="2" t="inlineStr" /><c r="J57" s="2" t="inlineStr" /><c r="K57" s="2" t="inlineStr"><is><t>cilostazol - ostra niewydolność mięśnia sercowego</t></is></c><c r="L57" s="2" t="inlineStr"><is><t>milrynon - migotanie przedsionków</t></is></c><c r="M57" s="2" t="inlineStr"><is><t>riocyguat - nadciśnienie tętnicze</t></is></c><c r="N57" s="2" t="inlineStr" /><c r="O57" s="2" t="inlineStr" /><c r="P57" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q57" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="58"><c r="A58" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B58" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C58" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D58" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E58" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – wskazanie:</t></is></c><c r="F58" s="2" t="inlineStr"><is><t>zolpidem-bezsenność</t></is></c><c r="G58" s="2" t="inlineStr"><is><t>ondansetron – wymioty w przebiegu chemioterapii przeciwnowotworowej</t></is></c><c r="H58" s="2" t="inlineStr"><is><t>alprazolam-napady paniki</t></is></c><c r="I58" s="2" t="inlineStr"><is><t>fluoksetyna–epizody dużej depresji</t></is></c><c r="J58" s="2" t="inlineStr" /><c r="K58" s="2" t="inlineStr" /><c r="L58" s="2" t="inlineStr" /><c r="M58" s="2" t="inlineStr" /><c r="N58" s="2" t="inlineStr" /><c r="O58" s="2" t="inlineStr" /><c r="P58" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2019/20 - 2 termin</t></is></c><c r="Q58" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="59"><c r="A59" s="2" t="inlineStr"><is><t>LEKI PRZECIWPSYCHOTYCZNE</t></is></c><c r="B59" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C59" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D59" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E59" s="2" t="inlineStr"><is><t>Hiperprolaktynemia może wiązać się z leczeniem:</t></is></c><c r="F59" s="2" t="inlineStr"><is><t>Promazyną</t></is></c><c r="G59" s="2" t="inlineStr"><is><t>Rysperydonem</t></is></c><c r="H59" s="2" t="inlineStr"><is><t>Metoklopramidem</t></is></c><c r="I59" s="2" t="inlineStr" /><c r="J59" s="2" t="inlineStr" /><c r="K59" s="2" t="inlineStr"><is><t>Bromokryptyną</t></is></c><c r="L59" s="2" t="inlineStr" /><c r="M59" s="2" t="inlineStr" /><c r="N59" s="2" t="inlineStr" /><c r="O59" s="2" t="inlineStr" /><c r="P59" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q59" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="60"><c r="A60" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B60" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C60" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D60" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E60" s="2" t="inlineStr"><is><t>Ośrodkowy zespół cholinolityczny może wystąpić w wyniku ostrego przedawkowania:</t></is></c><c r="F60" s="2" t="inlineStr"><is><t>Doksepiny</t></is></c><c r="G60" s="2" t="inlineStr"><is><t>Olanzapiny</t></is></c><c r="H60" s="2" t="inlineStr"><is><t>Perfenazyny</t></is></c><c r="I60" s="2" t="inlineStr"><is><t>Klemastyny</t></is></c><c r="J60" s="2" t="inlineStr" /><c r="K60" s="2" t="inlineStr" /><c r="L60" s="2" t="inlineStr" /><c r="M60" s="2" t="inlineStr" /><c r="N60" s="2" t="inlineStr" /><c r="O60" s="2" t="inlineStr" /><c r="P60" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q60" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="61"><c r="A61" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B61" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C61" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D61" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E61" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące metamizolu:</t></is></c><c r="F61" s="2" t="inlineStr"><is><t>Podczas szybkiego wstrzykiwania dożylnego leku może dojść do gwałtownych spadków ciśnienia krwi</t></is></c><c r="G61" s="2" t="inlineStr"><is><t>Może powodować ciężkie uszkodzenia szpiku w mechanizmie nadwrażliwości</t></is></c><c r="H61" s="2" t="inlineStr"><is><t>Zwiększa częstość występowania guzów Wilmsa (nephroblastoma, nerczak zarodkowy)</t></is></c><c r="I61" s="2" t="inlineStr" /><c r="J61" s="2" t="inlineStr" /><c r="K61" s="2" t="inlineStr"><is><t>Ma silne działanie przeciwzapalne</t></is></c><c r="L61" s="2" t="inlineStr" /><c r="M61" s="2" t="inlineStr" /><c r="N61" s="2" t="inlineStr" /><c r="O61" s="2" t="inlineStr" /><c r="P61" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q61" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="62"><c r="A62" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B62" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C62" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D62" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E62" s="2" t="inlineStr"><is><t>Które połączenie lekowe jest bezwzględnie konieczne w wymienionej sytuacji klinicznej:</t></is></c><c r="F62" s="2" t="inlineStr"><is><t>Sartan + sakubitryl w skurczowej niewydolności serca</t></is></c><c r="G62" s="2" t="inlineStr"><is><t>Kwas acetylosalicylowy + antagonista receptorów P2Y12 po angioplastyce wieńcowej z implantacją stentu</t></is></c><c r="H62" s="2" t="inlineStr" /><c r="I62" s="2" t="inlineStr" /><c r="J62" s="2" t="inlineStr" /><c r="K62" s="2" t="inlineStr"><is><t>Heparyna drobnocząsteczkowa + ksaban w początkowym okresie leczenia żylnej choroby zakrzepowo zatorowej</t></is></c><c r="L62" s="2" t="inlineStr"><is><t>Adrenalina + atropina w resuscytacji krążeniowo-oddechowej w przebiegu NZK z asystolią</t></is></c><c r="M62" s="2" t="inlineStr" /><c r="N62" s="2" t="inlineStr" /><c r="O62" s="2" t="inlineStr" /><c r="P62" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q62" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="63"><c r="A63" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B63" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C63" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D63" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E63" s="2" t="inlineStr"><is><t>Efekt prokinetyczny można uzyskać:</t></is></c><c r="F63" s="2" t="inlineStr"><is><t>Pobudzając receptory 5-HT4</t></is></c><c r="G63" s="2" t="inlineStr"><is><t>Blokując receptory dopaminowe D2</t></is></c><c r="H63" s="2" t="inlineStr"><is><t>Hamując aktywność acetylocholinoesterazy</t></is></c><c r="I63" s="2" t="inlineStr"><is><t>Pobudzając receptory motylinowe</t></is></c><c r="J63" s="2" t="inlineStr" /><c r="K63" s="2" t="inlineStr" /><c r="L63" s="2" t="inlineStr" /><c r="M63" s="2" t="inlineStr" /><c r="N63" s="2" t="inlineStr" /><c r="O63" s="2" t="inlineStr" /><c r="P63" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q63" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="64"><c r="A64" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B64" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C64" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D64" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E64" s="2" t="inlineStr"><is><t>Glukagon:</t></is></c><c r="F64" s="2" t="inlineStr"><is><t>Stosowany jest w leczeniu ciężkiej hipoglikemii gdy nie można podać dożylnie glukozy</t></is></c><c r="G64" s="2" t="inlineStr"><is><t>Jest podawany parenteralnie</t></is></c><c r="H64" s="2" t="inlineStr"><is><t>Ma zastosowanie w zatruciach lekami beta-adrenolitycznymi</t></is></c><c r="I64" s="2" t="inlineStr"><is><t>Jest nieskuteczny w przypadku glikemii</t></is></c><c r="J64" s="2" t="inlineStr" /><c r="K64" s="2" t="inlineStr" /><c r="L64" s="2" t="inlineStr" /><c r="M64" s="2" t="inlineStr" /><c r="N64" s="2" t="inlineStr" /><c r="O64" s="2" t="inlineStr" /><c r="P64" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q64" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="65"><c r="A65" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B65" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C65" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D65" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E65" s="2" t="inlineStr"><is><t>Ryzyko encefalopatii w przebiegu marskości wątroby zmniejsza stosowanie:</t></is></c><c r="F65" s="2" t="inlineStr"><is><t>Ryfaksyminy</t></is></c><c r="G65" s="2" t="inlineStr"><is><t>Asparaginianu ornityny</t></is></c><c r="H65" s="2" t="inlineStr"><is><t>Laktulozy</t></is></c><c r="I65" s="2" t="inlineStr" /><c r="J65" s="2" t="inlineStr" /><c r="K65" s="2" t="inlineStr"><is><t>Benzodiazepin</t></is></c><c r="L65" s="2" t="inlineStr" /><c r="M65" s="2" t="inlineStr" /><c r="N65" s="2" t="inlineStr" /><c r="O65" s="2" t="inlineStr" /><c r="P65" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q65" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="66"><c r="A66" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B66" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C66" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D66" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E66" s="2" t="inlineStr"><is><t>W celu przerwania ataku duszności uzasadnione jest podanie wziewne:</t></is></c><c r="F66" s="2" t="inlineStr"><is><t>Bromku ipratriopium</t></is></c><c r="G66" s="2" t="inlineStr"><is><t>Salbutamolu</t></is></c><c r="H66" s="2" t="inlineStr" /><c r="I66" s="2" t="inlineStr" /><c r="J66" s="2" t="inlineStr" /><c r="K66" s="2" t="inlineStr"><is><t>Roflumilastu</t></is></c><c r="L66" s="2" t="inlineStr"><is><t>flutykazonu</t></is></c><c r="M66" s="2" t="inlineStr" /><c r="N66" s="2" t="inlineStr" /><c r="O66" s="2" t="inlineStr" /><c r="P66" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q66" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="67"><c r="A67" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B67" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C67" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D67" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E67" s="2" t="inlineStr"><is><t>W leczeniu małopłytkowości stosuje się:</t></is></c><c r="F67" s="2" t="inlineStr"><is><t>Preparaty immunoglobulin poliwalentnych</t></is></c><c r="G67" s="2" t="inlineStr"><is><t>Eltrombopag</t></is></c><c r="H67" s="2" t="inlineStr"><is><t>Romiplostym</t></is></c><c r="I67" s="2" t="inlineStr"><is><t>Prednizon</t></is></c><c r="J67" s="2" t="inlineStr" /><c r="K67" s="2" t="inlineStr" /><c r="L67" s="2" t="inlineStr" /><c r="M67" s="2" t="inlineStr" /><c r="N67" s="2" t="inlineStr" /><c r="O67" s="2" t="inlineStr" /><c r="P67" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q67" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="68"><c r="A68" s="2" t="inlineStr"><is><t>LEKI PRZECIWNOWOTWOROWE</t></is></c><c r="B68" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C68" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D68" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E68" s="2" t="inlineStr"><is><t>Ewerolimus jest stosowany w:</t></is></c><c r="F68" s="2" t="inlineStr"><is><t>Kardiologii (stenty wieńcowe)</t></is></c><c r="G68" s="2" t="inlineStr"><is><t>Onkologii (wybrane zaawansowane nowotwory piersi i nerki)</t></is></c><c r="H68" s="2" t="inlineStr" /><c r="I68" s="2" t="inlineStr" /><c r="J68" s="2" t="inlineStr" /><c r="K68" s="2" t="inlineStr"><is><t>Neurologii (stwardnienie rozsiane)</t></is></c><c r="L68" s="2" t="inlineStr"><is><t>Dermatologii (łuszczyca)</t></is></c><c r="M68" s="2" t="inlineStr" /><c r="N68" s="2" t="inlineStr" /><c r="O68" s="2" t="inlineStr" /><c r="P68" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q68" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="69"><c r="A69" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B69" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C69" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D69" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E69" s="2" t="inlineStr"><is><t>Wskaż prawdziwe zdanie:</t></is></c><c r="F69" s="2" t="inlineStr"><is><t>W chromaniu przestankowym znaczenie kliniczne ma leczenie przeciwpłytkowe i hipolipemizujące</t></is></c><c r="G69" s="2" t="inlineStr"><is><t>Zaleca się podawanie inhibitora P2Y12 przed przezskórną interwencją wieńcową u osoby z ostrym zespołem wieńcowym, a następnie kontynuację tego leczenia przez co najmniej 12 miesięcy</t></is></c><c r="H69" s="2" t="inlineStr"><is><t>Po rozpoczęciu leczenia inhibitorami konwertazy angiotensyny należy się spodziewać niewielkiego wzrostu stężenia kreatyniny we krwi</t></is></c><c r="I69" s="2" t="inlineStr" /><c r="J69" s="2" t="inlineStr" /><c r="K69" s="2" t="inlineStr"><is><t>Niedihydropirydynowi antagoniści wapnia są wskazani w leczeniu pacjentów z niewydolnością serca z obniżoną frakcją wyrzutową</t></is></c><c r="L69" s="2" t="inlineStr" /><c r="M69" s="2" t="inlineStr" /><c r="N69" s="2" t="inlineStr" /><c r="O69" s="2" t="inlineStr" /><c r="P69" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q69" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="70"><c r="A70" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B70" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C70" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D70" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E70" s="2" t="inlineStr"><is><t>U osób z pierwotnym wydłużenie QTc bezpieczne jest zastosowanie:</t></is></c><c r="F70" s="2" t="inlineStr"><is><t>Propranololu</t></is></c><c r="G70" s="2" t="inlineStr" /><c r="H70" s="2" t="inlineStr" /><c r="I70" s="2" t="inlineStr" /><c r="J70" s="2" t="inlineStr" /><c r="K70" s="2" t="inlineStr"><is><t>Digoksyny</t></is></c><c r="L70" s="2" t="inlineStr"><is><t>Sotalolu</t></is></c><c r="M70" s="2" t="inlineStr"><is><t>Amiodaronu</t></is></c><c r="N70" s="2" t="inlineStr" /><c r="O70" s="2" t="inlineStr" /><c r="P70" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q70" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="71"><c r="A71" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B71" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C71" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D71" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E71" s="2" t="inlineStr"><is><t>Beta-adrenolityki można zastosować w:</t></is></c><c r="F71" s="2" t="inlineStr"><is><t>Tachykardii zatokowej</t></is></c><c r="G71" s="2" t="inlineStr"><is><t>Niewydolności mięśnia serca z upośledzoną frakcją wyrzutową</t></is></c><c r="H71" s="2" t="inlineStr"><is><t>W kontroli rytmu komór w migotaniu przedsionków</t></is></c><c r="I71" s="2" t="inlineStr" /><c r="J71" s="2" t="inlineStr" /><c r="K71" s="2" t="inlineStr"><is><t>Naczynioskurczowym wariancie choroby niedokrwiennej serca</t></is></c><c r="L71" s="2" t="inlineStr" /><c r="M71" s="2" t="inlineStr" /><c r="N71" s="2" t="inlineStr" /><c r="O71" s="2" t="inlineStr" /><c r="P71" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q71" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="72"><c r="A72" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B72" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C72" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D72" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E72" s="2" t="inlineStr"><is><t>Lidokaina:</t></is></c><c r="F72" s="2" t="inlineStr"><is><t>Jest skuteczna w znieczulaniu nasiękowym</t></is></c><c r="G72" s="2" t="inlineStr"><is><t>Jest metabolizowana w wątrobie</t></is></c><c r="H72" s="2" t="inlineStr"><is><t>Może powodować drgawki</t></is></c><c r="I72" s="2" t="inlineStr" /><c r="J72" s="2" t="inlineStr" /><c r="K72" s="2" t="inlineStr"><is><t>Silnie blokuje kanały potasowe</t></is></c><c r="L72" s="2" t="inlineStr" /><c r="M72" s="2" t="inlineStr" /><c r="N72" s="2" t="inlineStr" /><c r="O72" s="2" t="inlineStr" /><c r="P72" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q72" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="73"><c r="A73" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B73" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C73" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D73" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E73" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-działanie niepożądane:</t></is></c><c r="F73" s="2" t="inlineStr"><is><t>Ramipryl-obrzęk naczynioruchowy</t></is></c><c r="G73" s="2" t="inlineStr"><is><t>Metoprolol-zasłabnięcie lub omdlenie</t></is></c><c r="H73" s="2" t="inlineStr" /><c r="I73" s="2" t="inlineStr" /><c r="J73" s="2" t="inlineStr" /><c r="K73" s="2" t="inlineStr"><is><t>Losartan-zwiększenie stężenia kwasu moczowego</t></is></c><c r="L73" s="2" t="inlineStr"><is><t>Simwastatyna-poprawa tolerancji glukozy</t></is></c><c r="M73" s="2" t="inlineStr" /><c r="N73" s="2" t="inlineStr" /><c r="O73" s="2" t="inlineStr" /><c r="P73" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q73" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="74"><c r="A74" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B74" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C74" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D74" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E74" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – działanie niepożądane:</t></is></c><c r="F74" s="2" t="inlineStr"><is><t>metoprolol – blok przedsionkowo-komorowy I stopnia</t></is></c><c r="G74" s="2" t="inlineStr"><is><t>sotalol - wydłużenie odstępu QT</t></is></c><c r="H74" s="2" t="inlineStr"><is><t>propafenon - zaburzenia hematopoezy</t></is></c><c r="I74" s="2" t="inlineStr"><is><t>adenozyna - ból w klatce piersiowej</t></is></c><c r="J74" s="2" t="inlineStr" /><c r="K74" s="2" t="inlineStr" /><c r="L74" s="2" t="inlineStr" /><c r="M74" s="2" t="inlineStr" /><c r="N74" s="2" t="inlineStr" /><c r="O74" s="2" t="inlineStr" /><c r="P74" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q74" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="75"><c r="A75" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B75" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C75" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D75" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E75" s="2" t="inlineStr"><is><t>Która ordynacja jest błędna i wymaga korekty?</t></is></c><c r="F75" s="2" t="inlineStr"><is><t>Furosemid p.o. 1xd w obrzękach pochodzenia sercowego</t></is></c><c r="G75" s="2" t="inlineStr"><is><t>Hydrochlorotiazyd p.o. 1xd w obrzękach kończyn dolnych w przebiegu zespołu pozakrzepowego podudzi</t></is></c><c r="H75" s="2" t="inlineStr" /><c r="I75" s="2" t="inlineStr" /><c r="J75" s="2" t="inlineStr" /><c r="K75" s="2" t="inlineStr"><is><t>Torasemid p.o. 1xd w obrzękach pochodzenia nerkowego</t></is></c><c r="L75" s="2" t="inlineStr"><is><t>Spironolakton p.o. 1xd w wodobrzuszu w przebiegu niewydolności wątroby</t></is></c><c r="M75" s="2" t="inlineStr" /><c r="N75" s="2" t="inlineStr" /><c r="O75" s="2" t="inlineStr" /><c r="P75" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q75" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="76"><c r="A76" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B76" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C76" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D76" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E76" s="2" t="inlineStr"><is><t>Koangiokardianem, czyli lekiem działającym bezpośrednio na serce i naczynia jest:</t></is></c><c r="F76" s="2" t="inlineStr"><is><t>Lewosymendan</t></is></c><c r="G76" s="2" t="inlineStr" /><c r="H76" s="2" t="inlineStr" /><c r="I76" s="2" t="inlineStr" /><c r="J76" s="2" t="inlineStr" /><c r="K76" s="2" t="inlineStr"><is><t>Midodryna</t></is></c><c r="L76" s="2" t="inlineStr"><is><t>Epoprostenol</t></is></c><c r="M76" s="2" t="inlineStr"><is><t>Riocyguat</t></is></c><c r="N76" s="2" t="inlineStr" /><c r="O76" s="2" t="inlineStr" /><c r="P76" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q76" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="77"><c r="A77" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B77" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C77" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D77" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E77" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące bisfosfonianów:</t></is></c><c r="F77" s="2" t="inlineStr"><is><t>Są lekami pierwszego rzutu w profilaktyce i leczeniu osteoporozy pomenopauzalnej u kobiet</t></is></c><c r="G77" s="2" t="inlineStr"><is><t>Mogą być stosowane w zapobieganiu i leczeniu osteoporozy posteroidowej</t></is></c><c r="H77" s="2" t="inlineStr"><is><t>U osób z przerzutami nowotworowymi do układu kostnego łagodzą bóle kostne</t></is></c><c r="I77" s="2" t="inlineStr"><is><t>Przeciwwskazaniem do ich podawania jest ciężka niewydolność nerek (GFR&lt;30)</t></is></c><c r="J77" s="2" t="inlineStr" /><c r="K77" s="2" t="inlineStr" /><c r="L77" s="2" t="inlineStr" /><c r="M77" s="2" t="inlineStr" /><c r="N77" s="2" t="inlineStr" /><c r="O77" s="2" t="inlineStr" /><c r="P77" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q77" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="78"><c r="A78" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B78" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C78" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D78" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E78" s="2" t="inlineStr"><is><t>Zmniejszenie hipertriglicerydemii można osiągnąć stosując:</t></is></c><c r="F78" s="2" t="inlineStr"><is><t>Atorwastatynę</t></is></c><c r="G78" s="2" t="inlineStr"><is><t>Fenofibrat</t></is></c><c r="H78" s="2" t="inlineStr"><is><t>PUFA-wielonienasycone kwasy tłuszczowe</t></is></c><c r="I78" s="2" t="inlineStr" /><c r="J78" s="2" t="inlineStr" /><c r="K78" s="2" t="inlineStr"><is><t>Koleswelam</t></is></c><c r="L78" s="2" t="inlineStr" /><c r="M78" s="2" t="inlineStr" /><c r="N78" s="2" t="inlineStr" /><c r="O78" s="2" t="inlineStr" /><c r="P78" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q78" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="79"><c r="A79" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B79" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C79" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D79" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E79" s="2" t="inlineStr"><is><t>Lekiem wydłużającym dystans chromania przestankowego jest:</t></is></c><c r="F79" s="2" t="inlineStr"><is><t>Natydrofuryl</t></is></c><c r="G79" s="2" t="inlineStr"><is><t>Cilostazol</t></is></c><c r="H79" s="2" t="inlineStr" /><c r="I79" s="2" t="inlineStr" /><c r="J79" s="2" t="inlineStr" /><c r="K79" s="2" t="inlineStr"><is><t>Pentoksyfilina</t></is></c><c r="L79" s="2" t="inlineStr"><is><t>Diosmina mikronizowana</t></is></c><c r="M79" s="2" t="inlineStr" /><c r="N79" s="2" t="inlineStr" /><c r="O79" s="2" t="inlineStr" /><c r="P79" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q79" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="80"><c r="A80" s="2" t="inlineStr"><is><t>LEKI HIPOLIPEMIZUJĄCE</t></is></c><c r="B80" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C80" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D80" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E80" s="2" t="inlineStr"><is><t>W prawidłowo przeprowadzonym leczeniu statynami należy:</t></is></c><c r="F80" s="2" t="inlineStr"><is><t>Oznaczyć aktywność ALAT i CK w surowicy przed rozpoczęciem leczenia</t></is></c><c r="G80" s="2" t="inlineStr"><is><t>Odstawić statynę jeśli aktywność ALAT przekroczy w surowicy 3-krotnie górną granicę wartości prawidłowych</t></is></c><c r="H80" s="2" t="inlineStr" /><c r="I80" s="2" t="inlineStr" /><c r="J80" s="2" t="inlineStr" /><c r="K80" s="2" t="inlineStr"><is><t>Ocenić skuteczność leczenia hipolipemizującego po 2 tygodniach od jego rozpoczęcia</t></is></c><c r="L80" s="2" t="inlineStr"><is><t>Mintorować aktywność CK u każdego pacjenta</t></is></c><c r="M80" s="2" t="inlineStr" /><c r="N80" s="2" t="inlineStr" /><c r="O80" s="2" t="inlineStr" /><c r="P80" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q80" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="81"><c r="A81" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B81" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C81" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D81" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E81" s="2" t="inlineStr"><is><t>Na kanały sodowe ma wpływ:</t></is></c><c r="F81" s="2" t="inlineStr"><is><t>Ranolazyna</t></is></c><c r="G81" s="2" t="inlineStr"><is><t>Iwabradyna</t></is></c><c r="H81" s="2" t="inlineStr" /><c r="I81" s="2" t="inlineStr" /><c r="J81" s="2" t="inlineStr" /><c r="K81" s="2" t="inlineStr"><is><t>Adenozyna</t></is></c><c r="L81" s="2" t="inlineStr"><is><t>Nitrendypina</t></is></c><c r="M81" s="2" t="inlineStr" /><c r="N81" s="2" t="inlineStr" /><c r="O81" s="2" t="inlineStr" /><c r="P81" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q81" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="82"><c r="A82" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B82" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C82" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D82" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E82" s="2" t="inlineStr"><is><t>Na kanały sodowe ma wpływ:</t></is></c><c r="F82" s="2" t="inlineStr"><is><t>propafenon</t></is></c><c r="G82" s="2" t="inlineStr"><is><t>ranolazyna</t></is></c><c r="H82" s="2" t="inlineStr"><is><t>bupiwakaina</t></is></c><c r="I82" s="2" t="inlineStr" /><c r="J82" s="2" t="inlineStr" /><c r="K82" s="2" t="inlineStr"><is><t>adenozyna</t></is></c><c r="L82" s="2" t="inlineStr" /><c r="M82" s="2" t="inlineStr" /><c r="N82" s="2" t="inlineStr" /><c r="O82" s="2" t="inlineStr" /><c r="P82" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 1 termin</t></is></c><c r="Q82" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="83"><c r="A83" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B83" s="2" t="inlineStr"><is><t>Interakcje</t></is></c><c r="C83" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D83" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E83" s="2" t="inlineStr"><is><t>Interakcją farmakokinetyczną jest:</t></is></c><c r="F83" s="2" t="inlineStr"><is><t>Hamowanie wchłaniania z przewodu pokarmowego leków podawanych jednocześnie</t></is></c><c r="G83" s="2" t="inlineStr"><is><t>Zwiększanie metabolizmu leków podawanych jednocześnie</t></is></c><c r="H83" s="2" t="inlineStr" /><c r="I83" s="2" t="inlineStr" /><c r="J83" s="2" t="inlineStr" /><c r="K83" s="2" t="inlineStr"><is><t>Wytrącanie się osadu po zmieszaniu dwóch leków w jednym roztworze do wstrzyknięcia</t></is></c><c r="L83" s="2" t="inlineStr"><is><t>Nasilenie sedacji po skojarzeniu opioidów z etanolem</t></is></c><c r="M83" s="2" t="inlineStr" /><c r="N83" s="2" t="inlineStr" /><c r="O83" s="2" t="inlineStr" /><c r="P83" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q83" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="84"><c r="A84" s="2" t="inlineStr"><is><t>NARKOTYCZNE LEKI PRZECIWBÓLOWE</t></is></c><c r="B84" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C84" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D84" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E84" s="2" t="inlineStr"><is><t>Właściwości farmakodynamiczne i parametry farmakokinetyczne leków mają wpływ na podejmowanie decyzji klinicznych. Czy słuszne jest wobec tego:</t></is></c><c r="F84" s="2" t="inlineStr"><is><t>Wielokrotne powtórzenie dawki naloksonu(t1/2=63min+/-12min) po przedawkowaniu metadonu</t></is></c><c r="G84" s="2" t="inlineStr" /><c r="H84" s="2" t="inlineStr" /><c r="I84" s="2" t="inlineStr" /><c r="J84" s="2" t="inlineStr" /><c r="K84" s="2" t="inlineStr"><is><t>Przetoczenie koncentratu płytek krwi 13h po podaniu tikagrelolu (tikagrelol ze swoim czynnym metabolitem mają łączny czas półtrwania eliminacji 12h)</t></is></c><c r="L84" s="2" t="inlineStr"><is><t>Odstawienie suplementacji potasu w hiperaldosteronizmie pierwotnym po 16-17h po włączeniu spironolaktonu (Cmax karnenonu=16,5h po podaniu spironolaktonu)</t></is></c><c r="M84" s="2" t="inlineStr"><is><t>Przeprowadzenie operacji neurochirurgicznej po 36h po odstawieniu klopidogrelu(t1/2=6h, jego aktywne mają pomijalnie krótki t1/2)</t></is></c><c r="N84" s="2" t="inlineStr" /><c r="O84" s="2" t="inlineStr" /><c r="P84" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q84" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="85"><c r="A85" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B85" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C85" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D85" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E85" s="2" t="inlineStr"><is><t>Kolistyna:</t></is></c><c r="F85" s="2" t="inlineStr"><is><t>Może być podawana wziewnie u osób z mukowiscydozą</t></is></c><c r="G85" s="2" t="inlineStr"><is><t>Może być stosowana w leczeniu ciężkich zakażeń uogólnionych wywołanych prze Klebsiella pneumoniae wytwarzającą karbapenemazy</t></is></c><c r="H85" s="2" t="inlineStr"><is><t>Wykazuje aktywność wobec Pseudomonas aeruginosa</t></is></c><c r="I85" s="2" t="inlineStr" /><c r="J85" s="2" t="inlineStr" /><c r="K85" s="2" t="inlineStr"><is><t>Jest skuteczna w neuroinfekcjach</t></is></c><c r="L85" s="2" t="inlineStr" /><c r="M85" s="2" t="inlineStr" /><c r="N85" s="2" t="inlineStr" /><c r="O85" s="2" t="inlineStr" /><c r="P85" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q85" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="86"><c r="A86" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B86" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C86" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D86" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E86" s="2" t="inlineStr"><is><t>Kolistyna</t></is></c><c r="F86" s="2" t="inlineStr"><is><t>Działa nefrotoksycznie</t></is></c><c r="G86" s="2" t="inlineStr" /><c r="H86" s="2" t="inlineStr" /><c r="I86" s="2" t="inlineStr" /><c r="J86" s="2" t="inlineStr" /><c r="K86" s="2" t="inlineStr"><is><t>Działa głównie na bakterie Gram+</t></is></c><c r="L86" s="2" t="inlineStr"><is><t>Dobrze wchłania się po podaniu PO</t></is></c><c r="M86" s="2" t="inlineStr"><is><t>Jest wydalana głównie z kałem</t></is></c><c r="N86" s="2" t="inlineStr" /><c r="O86" s="2" t="inlineStr" /><c r="P86" s="2" t="inlineStr"><is><t>EGZ 2017 II termin</t></is></c><c r="Q86" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="87"><c r="A87" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B87" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C87" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D87" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E87" s="2" t="inlineStr"><is><t>Doksycyklina</t></is></c><c r="F87" s="2" t="inlineStr"><is><t>Działa na bakterie atypowe</t></is></c><c r="G87" s="2" t="inlineStr" /><c r="H87" s="2" t="inlineStr" /><c r="I87" s="2" t="inlineStr" /><c r="J87" s="2" t="inlineStr" /><c r="K87" s="2" t="inlineStr"><is><t>Może być bezpiecznie stosowana u dzieci powyżej 2r.ż</t></is></c><c r="L87" s="2" t="inlineStr"><is><t>Jest anatgonistą receptorów GABA-A wywołujących efekt sedatywny</t></is></c><c r="M87" s="2" t="inlineStr"><is><t>Jest bezpieczna w terapii kobiet w ciąży</t></is></c><c r="N87" s="2" t="inlineStr" /><c r="O87" s="2" t="inlineStr" /><c r="P87" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q87" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="88"><c r="A88" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B88" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C88" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D88" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E88" s="2" t="inlineStr"><is><t>Doksycyklina:</t></is></c><c r="F88" s="2" t="inlineStr"><is><t>w niewielkim stopniu penetruje do ośrodkowego układu nerwowego</t></is></c><c r="G88" s="2" t="inlineStr"><is><t>tworzy chelaty z solami żelaza</t></is></c><c r="H88" s="2" t="inlineStr"><is><t>jest stosowana w leczeniu zakażeń układu moczowego o etiologii Chlamydia trachomatis</t></is></c><c r="I88" s="2" t="inlineStr"><is><t>nie wykazuje aktywności wobec Pseudomonas aeruginosa</t></is></c><c r="J88" s="2" t="inlineStr" /><c r="K88" s="2" t="inlineStr" /><c r="L88" s="2" t="inlineStr" /><c r="M88" s="2" t="inlineStr" /><c r="N88" s="2" t="inlineStr" /><c r="O88" s="2" t="inlineStr" /><c r="P88" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q88" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="89"><c r="A89" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B89" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C89" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D89" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E89" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-mechanizm działania:</t></is></c><c r="F89" s="2" t="inlineStr"><is><t>Fosfomycyna-blokowanie syntezy ściany komórkowej bakterii</t></is></c><c r="G89" s="2" t="inlineStr" /><c r="H89" s="2" t="inlineStr" /><c r="I89" s="2" t="inlineStr" /><c r="J89" s="2" t="inlineStr" /><c r="K89" s="2" t="inlineStr"><is><t>Cefepim-hamowanie topoizomerazy II</t></is></c><c r="L89" s="2" t="inlineStr"><is><t>Pefloksacyna-hamowanie biosyntezy białka w komórkach bakterii poprzez wiązanie się z podjednostką 50S rybosomu</t></is></c><c r="M89" s="2" t="inlineStr"><is><t>Trimetoprim-bezpośrednie uszkodzenie DNA</t></is></c><c r="N89" s="2" t="inlineStr" /><c r="O89" s="2" t="inlineStr" /><c r="P89" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q89" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="90"><c r="A90" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B90" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C90" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D90" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E90" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – mechanizm działania:</t></is></c><c r="F90" s="2" t="inlineStr"><is><t>linezolid- hamowanie biosyntezy białka w komórkach bakterii poprzez wiązanie się z podjednostką 50 S rybosomu</t></is></c><c r="G90" s="2" t="inlineStr" /><c r="H90" s="2" t="inlineStr" /><c r="I90" s="2" t="inlineStr" /><c r="J90" s="2" t="inlineStr" /><c r="K90" s="2" t="inlineStr"><is><t>cefuroksym – hamowanie topoizomerazy II</t></is></c><c r="L90" s="2" t="inlineStr"><is><t>moksyfloksacyna - blokowanie syntezy ściany komórkowej bakterii</t></is></c><c r="M90" s="2" t="inlineStr"><is><t>wankomycyna - uszkodzenie DNA</t></is></c><c r="N90" s="2" t="inlineStr" /><c r="O90" s="2" t="inlineStr" /><c r="P90" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q90" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="91"><c r="A91" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B91" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C91" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D91" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E91" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – mechanizm działania:</t></is></c><c r="F91" s="2" t="inlineStr"><is><t>tygecyklina - hamowanie biosyntezy białka w komórkach bakterii poprzez wiązanie się z podjednostką 30 S rybosomu</t></is></c><c r="G91" s="2" t="inlineStr"><is><t>trimetoprim - inhibicja reduktazy kwasu dihydrofoliowego (DHFR)</t></is></c><c r="H91" s="2" t="inlineStr" /><c r="I91" s="2" t="inlineStr" /><c r="J91" s="2" t="inlineStr" /><c r="K91" s="2" t="inlineStr"><is><t>metronidazol - blokowanie syntezy ściany komórkowej bakterii</t></is></c><c r="L91" s="2" t="inlineStr"><is><t>teikoplanina - uszkodzenie DNA</t></is></c><c r="M91" s="2" t="inlineStr" /><c r="N91" s="2" t="inlineStr" /><c r="O91" s="2" t="inlineStr" /><c r="P91" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q91" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="92"><c r="A92" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B92" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C92" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D92" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E92" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – mechanizm działania:</t></is></c><c r="F92" s="2" t="inlineStr"><is><t>linagliptyna – pośrednio aktywacja wydzielania insuliny przez pobudzenie receptora dla GLP-1 (peptydu glukagonopodobnego typu 1)</t></is></c><c r="G92" s="2" t="inlineStr"><is><t>empagliflozyna – indukcja stałej łagodnej hiperketonemii ze zwiększeniem stężenia kwasu beta-hydroksymasłowego w surowicy</t></is></c><c r="H92" s="2" t="inlineStr"><is><t>ezetymib – redukcja jelitowego wchłaniania cholesterolu i steroli roślinnych</t></is></c><c r="I92" s="2" t="inlineStr" /><c r="J92" s="2" t="inlineStr" /><c r="K92" s="2" t="inlineStr"><is><t>orlistat – aktywacja lipazy trzustkowej w świetle przewodu pokarmowego</t></is></c><c r="L92" s="2" t="inlineStr" /><c r="M92" s="2" t="inlineStr" /><c r="N92" s="2" t="inlineStr" /><c r="O92" s="2" t="inlineStr" /><c r="P92" s="2" t="inlineStr"><is><t>KOLOKWIUM 1 – 2018/19</t></is></c><c r="Q92" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="93"><c r="A93" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B93" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C93" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D93" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E93" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-działania niepożądane:</t></is></c><c r="F93" s="2" t="inlineStr"><is><t>Amoksycylina-leukopenia w mechanizmie nadwrażliwości immunologicznej</t></is></c><c r="G93" s="2" t="inlineStr"><is><t>Tynidazol-neuropatia obwodowa</t></is></c><c r="H93" s="2" t="inlineStr"><is><t>Amikacyna-zaburzenia słuchu i równowagi</t></is></c><c r="I93" s="2" t="inlineStr" /><c r="J93" s="2" t="inlineStr" /><c r="K93" s="2" t="inlineStr"><is><t>Roksytromycyna-uszkodzenie nerek</t></is></c><c r="L93" s="2" t="inlineStr" /><c r="M93" s="2" t="inlineStr" /><c r="N93" s="2" t="inlineStr" /><c r="O93" s="2" t="inlineStr" /><c r="P93" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q93" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="94"><c r="A94" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B94" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C94" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D94" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E94" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – działania niepożądane:</t></is></c><c r="F94" s="2" t="inlineStr"><is><t>tygecyklina - nadwrażliwość na światło</t></is></c><c r="G94" s="2" t="inlineStr"><is><t>metronidazol - neuropatia obwodowa</t></is></c><c r="H94" s="2" t="inlineStr"><is><t>wankomycyna – uwalnianie histaminy</t></is></c><c r="I94" s="2" t="inlineStr" /><c r="J94" s="2" t="inlineStr" /><c r="K94" s="2" t="inlineStr"><is><t>azytromycyna – blokowanie wątrobowych enzymów mikrosomalnych (CYP)</t></is></c><c r="L94" s="2" t="inlineStr" /><c r="M94" s="2" t="inlineStr" /><c r="N94" s="2" t="inlineStr" /><c r="O94" s="2" t="inlineStr" /><c r="P94" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q94" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="95"><c r="A95" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B95" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C95" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D95" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E95" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – działania niepożądane:</t></is></c><c r="F95" s="2" t="inlineStr"><is><t>lewofloksacyna - drgawki</t></is></c><c r="G95" s="2" t="inlineStr"><is><t>ceftriakson – zagęszczenie żółci</t></is></c><c r="H95" s="2" t="inlineStr"><is><t>wankomycyna – zespół czerwonego karku</t></is></c><c r="I95" s="2" t="inlineStr"><is><t>linezolid – trombocytopenia</t></is></c><c r="J95" s="2" t="inlineStr" /><c r="K95" s="2" t="inlineStr" /><c r="L95" s="2" t="inlineStr" /><c r="M95" s="2" t="inlineStr" /><c r="N95" s="2" t="inlineStr" /><c r="O95" s="2" t="inlineStr" /><c r="P95" s="2" t="inlineStr"><is><t>EGZ 2017 I termin</t></is></c><c r="Q95" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="96"><c r="A96" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B96" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C96" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D96" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E96" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – działania niepożądane:</t></is></c><c r="F96" s="2" t="inlineStr"><is><t>bromek glikopironium - tachykardia</t></is></c><c r="G96" s="2" t="inlineStr"><is><t>budezonid – kandydoza jamy ustnej</t></is></c><c r="H96" s="2" t="inlineStr"><is><t>teofilina – zaburzenia rytmu serca</t></is></c><c r="I96" s="2" t="inlineStr"><is><t>omalizumab – reakcje w miejscu podskórnego podania leku, takie jak ból, zaczerwienienie, świąd, obrzęk</t></is></c><c r="J96" s="2" t="inlineStr" /><c r="K96" s="2" t="inlineStr" /><c r="L96" s="2" t="inlineStr" /><c r="M96" s="2" t="inlineStr" /><c r="N96" s="2" t="inlineStr" /><c r="O96" s="2" t="inlineStr" /><c r="P96" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2017/18 - 2 termin</t></is></c><c r="Q96" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="97"><c r="A97" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B97" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C97" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D97" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E97" s="2" t="inlineStr"><is><t>Właściwy wybór leku przeciwwirusowego w zakażeniu to:</t></is></c><c r="F97" s="2" t="inlineStr"><is><t>Wirus HBV-lamiwudyna</t></is></c><c r="G97" s="2" t="inlineStr"><is><t>Cytomegalowirus-walgancyklowir</t></is></c><c r="H97" s="2" t="inlineStr" /><c r="I97" s="2" t="inlineStr" /><c r="J97" s="2" t="inlineStr" /><c r="K97" s="2" t="inlineStr"><is><t>Norowirus-sakwinawir</t></is></c><c r="L97" s="2" t="inlineStr"><is><t>Wirus opryszczki-rybawiryna</t></is></c><c r="M97" s="2" t="inlineStr" /><c r="N97" s="2" t="inlineStr" /><c r="O97" s="2" t="inlineStr" /><c r="P97" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q97" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="98"><c r="A98" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B98" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C98" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D98" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E98" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek-wrażliwy drobnoustrój:</t></is></c><c r="F98" s="2" t="inlineStr"><is><t>Lewofloksacyna-Streptococcus pneumoniae</t></is></c><c r="G98" s="2" t="inlineStr"><is><t>Aksetyl cefuroksymu-Hemophilus influenzae</t></is></c><c r="H98" s="2" t="inlineStr" /><c r="I98" s="2" t="inlineStr" /><c r="J98" s="2" t="inlineStr" /><c r="K98" s="2" t="inlineStr"><is><t>Fenoksymetylopenicylina-Staphylococcus aureus MSSA</t></is></c><c r="L98" s="2" t="inlineStr"><is><t>Fidaksomycyna-Bacteroides fragilis</t></is></c><c r="M98" s="2" t="inlineStr" /><c r="N98" s="2" t="inlineStr" /><c r="O98" s="2" t="inlineStr" /><c r="P98" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q98" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="99"><c r="A99" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B99" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C99" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D99" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E99" s="2" t="inlineStr"><is><t>Wskaż prawdziwe połączenie lek – wrażliwy drobnoustrój:</t></is></c><c r="F99" s="2" t="inlineStr"><is><t>kaspofungina _ Candida spp</t></is></c><c r="G99" s="2" t="inlineStr"><is><t>amfoterycyna B – Cryptococcus neoformans</t></is></c><c r="H99" s="2" t="inlineStr"><is><t>worykonazol - Candida crusei</t></is></c><c r="I99" s="2" t="inlineStr" /><c r="J99" s="2" t="inlineStr" /><c r="K99" s="2" t="inlineStr"><is><t>flukonazol – Aspergillus fumigatus</t></is></c><c r="L99" s="2" t="inlineStr" /><c r="M99" s="2" t="inlineStr" /><c r="N99" s="2" t="inlineStr" /><c r="O99" s="2" t="inlineStr" /><c r="P99" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 1 termin</t></is></c><c r="Q99" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="100"><c r="A100" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B100" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C100" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D100" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E100" s="2" t="inlineStr"><is><t>Flukonazol:</t></is></c><c r="F100" s="2" t="inlineStr"><is><t>W leczeniu kandydozy jamy ustnej nie jest skuteczny po podaniu dawki jednorazowej</t></is></c><c r="G100" s="2" t="inlineStr" /><c r="H100" s="2" t="inlineStr" /><c r="I100" s="2" t="inlineStr" /><c r="J100" s="2" t="inlineStr" /><c r="K100" s="2" t="inlineStr"><is><t>Ma małą biodostępność po podaniu doustnym</t></is></c><c r="L100" s="2" t="inlineStr"><is><t>Powinien być podawany profilaktycznie pacjentom leczonym szerokospektralnymi lekami przeciwbakteryjnymi z powodu zakażenia układu oddechowego</t></is></c><c r="M100" s="2" t="inlineStr"><is><t>Istotnie hamuje syntezę hormonów steroidowych</t></is></c><c r="N100" s="2" t="inlineStr" /><c r="O100" s="2" t="inlineStr" /><c r="P100" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q100" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="101"><c r="A101" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B101" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C101" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D101" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E101" s="2" t="inlineStr"><is><t>Wyłącznie na ustroje gram dodatnie działa:</t></is></c><c r="F101" s="2" t="inlineStr"><is><t>Mupriocyna</t></is></c><c r="G101" s="2" t="inlineStr" /><c r="H101" s="2" t="inlineStr" /><c r="I101" s="2" t="inlineStr" /><c r="J101" s="2" t="inlineStr" /><c r="K101" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="L101" s="2" t="inlineStr"><is><t>Fosfomycyna</t></is></c><c r="M101" s="2" t="inlineStr"><is><t>Gentamycyna</t></is></c><c r="N101" s="2" t="inlineStr" /><c r="O101" s="2" t="inlineStr" /><c r="P101" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q101" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="102"><c r="A102" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B102" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C102" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D102" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E102" s="2" t="inlineStr"><is><t>W leczeniu rzęsistkowicy (Trichomonas Vaginalis) wykorzystuje się:</t></is></c><c r="F102" s="2" t="inlineStr"><is><t>Tynidazol</t></is></c><c r="G102" s="2" t="inlineStr"><is><t>Metronidazol</t></is></c><c r="H102" s="2" t="inlineStr" /><c r="I102" s="2" t="inlineStr" /><c r="J102" s="2" t="inlineStr" /><c r="K102" s="2" t="inlineStr"><is><t>Sulfametoksazol+trymetoprym</t></is></c><c r="L102" s="2" t="inlineStr"><is><t>Spiramycynę</t></is></c><c r="M102" s="2" t="inlineStr" /><c r="N102" s="2" t="inlineStr" /><c r="O102" s="2" t="inlineStr" /><c r="P102" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q102" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="103"><c r="A103" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B103" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C103" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D103" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E103" s="2" t="inlineStr"><is><t>Do charakterystycznych działań niepożądanych inhibitorów proteazy HIV należy/należą:</t></is></c><c r="F103" s="2" t="inlineStr"><is><t>Liczne interakcje lekowe</t></is></c><c r="G103" s="2" t="inlineStr"><is><t>Cukrzyca</t></is></c><c r="H103" s="2" t="inlineStr"><is><t>Uszkodzenie wątroby</t></is></c><c r="I103" s="2" t="inlineStr"><is><t>Hipertriglicerydemia</t></is></c><c r="J103" s="2" t="inlineStr" /><c r="K103" s="2" t="inlineStr" /><c r="L103" s="2" t="inlineStr" /><c r="M103" s="2" t="inlineStr" /><c r="N103" s="2" t="inlineStr" /><c r="O103" s="2" t="inlineStr" /><c r="P103" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q103" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="104"><c r="A104" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B104" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C104" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D104" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E104" s="2" t="inlineStr"><is><t>W zakażeniu o etiologii Candida albicans można zastosować miejscowo:</t></is></c><c r="F104" s="2" t="inlineStr"><is><t>Natamycynę</t></is></c><c r="G104" s="2" t="inlineStr"><is><t>Mykonazol</t></is></c><c r="H104" s="2" t="inlineStr" /><c r="I104" s="2" t="inlineStr" /><c r="J104" s="2" t="inlineStr" /><c r="K104" s="2" t="inlineStr"><is><t>Mykafunginę</t></is></c><c r="L104" s="2" t="inlineStr"><is><t>Izawukonazol</t></is></c><c r="M104" s="2" t="inlineStr" /><c r="N104" s="2" t="inlineStr" /><c r="O104" s="2" t="inlineStr" /><c r="P104" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q104" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="105"><c r="A105" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B105" s="2" t="inlineStr"><is><t>Monitorowanie</t></is></c><c r="C105" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D105" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E105" s="2" t="inlineStr"><is><t>Jeśli celem farmakodynamicznym dla stosowanego antybiotyku jest wysoka wartość T&gt;MIC to powinno się:</t></is></c><c r="F105" s="2" t="inlineStr"><is><t>Monitorować stężenie leku we krwi w celu modyfikacji dawkowania</t></is></c><c r="G105" s="2" t="inlineStr"><is><t>Podawać lek w przedłużonym wlewie dożylnym</t></is></c><c r="H105" s="2" t="inlineStr"><is><t>Zwiększać częstość podawania leku w ciągu doby</t></is></c><c r="I105" s="2" t="inlineStr" /><c r="J105" s="2" t="inlineStr" /><c r="K105" s="2" t="inlineStr"><is><t>Podać lek w pojedynczej skumulowanej dawce dobowej</t></is></c><c r="L105" s="2" t="inlineStr" /><c r="M105" s="2" t="inlineStr" /><c r="N105" s="2" t="inlineStr" /><c r="O105" s="2" t="inlineStr" /><c r="P105" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q105" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="106"><c r="A106" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B106" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C106" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D106" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E106" s="2" t="inlineStr"><is><t>Do przestarzałych środków odkażających, które z powodu braku skuteczności lub istotnych działań niepożądanych nie powinny być obecnie stosowane należy:</t></is></c><c r="F106" s="2" t="inlineStr"><is><t>Nadmanganian potasu</t></is></c><c r="G106" s="2" t="inlineStr"><is><t>Tetraboran sodowy</t></is></c><c r="H106" s="2" t="inlineStr" /><c r="I106" s="2" t="inlineStr" /><c r="J106" s="2" t="inlineStr" /><c r="K106" s="2" t="inlineStr"><is><t>Oktenidyna</t></is></c><c r="L106" s="2" t="inlineStr"><is><t>Jodopowidon</t></is></c><c r="M106" s="2" t="inlineStr" /><c r="N106" s="2" t="inlineStr" /><c r="O106" s="2" t="inlineStr" /><c r="P106" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q106" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="107"><c r="A107" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B107" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C107" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D107" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E107" s="2" t="inlineStr"><is><t>Wskaż prawidłowe stwierdzenia dotyczące profilaktyki i leczenia malarii:</t></is></c><c r="F107" s="2" t="inlineStr"><is><t>Lumefantryna w połączeniu z artemeterem może być skuteczna w zakażeniu Plasmodium falciparum</t></is></c><c r="G107" s="2" t="inlineStr"><is><t>W przypadkach wymagających profilaktyki długoterminowej można zastosować chlorochinę</t></is></c><c r="H107" s="2" t="inlineStr" /><c r="I107" s="2" t="inlineStr" /><c r="J107" s="2" t="inlineStr" /><c r="K107" s="2" t="inlineStr"><is><t>Pochodne artemizyniny zalecane są tylko do profilaktyki malarii</t></is></c><c r="L107" s="2" t="inlineStr"><is><t>Atowakwon z proguanilem może być stosowany u osób z upośledzoną czynnością nerek (GFR&lt;30)</t></is></c><c r="M107" s="2" t="inlineStr" /><c r="N107" s="2" t="inlineStr" /><c r="O107" s="2" t="inlineStr" /><c r="P107" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q107" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="108"><c r="A108" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B108" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C108" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D108" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E108" s="2" t="inlineStr"><is><t>Do przyczyn jatrogennej nefropatii można zaliczyć stosowanie:</t></is></c><c r="F108" s="2" t="inlineStr"><is><t>Jodowych środków kontrastowych podczas koronarografii</t></is></c><c r="G108" s="2" t="inlineStr"><is><t>Ibuprofenu przewlekle w reumatoidalnym zapaleniu stawów</t></is></c><c r="H108" s="2" t="inlineStr"><is><t>Ramiprylu w niewydolności serca</t></is></c><c r="I108" s="2" t="inlineStr" /><c r="J108" s="2" t="inlineStr" /><c r="K108" s="2" t="inlineStr"><is><t>Loratadyny przewlekle w alergicznym zapaleniu błony śluzowej nosa</t></is></c><c r="L108" s="2" t="inlineStr" /><c r="M108" s="2" t="inlineStr" /><c r="N108" s="2" t="inlineStr" /><c r="O108" s="2" t="inlineStr" /><c r="P108" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q108" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="109"><c r="A109" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B109" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C109" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D109" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E109" s="2" t="inlineStr"><is><t>Wskaż prawdziwe zdania dotyczące leczenia morfiną:</t></is></c><c r="F109" s="2" t="inlineStr"><is><t>Metabolity morfiny wydalane są przez nerki</t></is></c><c r="G109" s="2" t="inlineStr"><is><t>Przy przewlekłym stosowaniu morfiny powstaje morfino-6-glukuronian – metabolit, którego siła działania analgetycznego przewyższa siłę działania związku macierzystego</t></is></c><c r="H109" s="2" t="inlineStr"><is><t>Morfina może być podawana zewnątrzoponowo</t></is></c><c r="I109" s="2" t="inlineStr" /><c r="J109" s="2" t="inlineStr" /><c r="K109" s="2" t="inlineStr"><is><t>Morfina ma dużą biodostępność po podaniu doustnym</t></is></c><c r="L109" s="2" t="inlineStr" /><c r="M109" s="2" t="inlineStr" /><c r="N109" s="2" t="inlineStr" /><c r="O109" s="2" t="inlineStr" /><c r="P109" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q109" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="110"><c r="A110" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B110" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C110" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D110" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E110" s="2" t="inlineStr"><is><t>Wskazanie do insulinoterapii jest:</t></is></c><c r="F110" s="2" t="inlineStr"><is><t>Cukrzyca typu LADA</t></is></c><c r="G110" s="2" t="inlineStr"><is><t>Ostry zespół wieńcowy u osoby z cukrzycą typu II</t></is></c><c r="H110" s="2" t="inlineStr"><is><t>Znaczna hiperglikemia (&gt;300) w przebiegu cukrzycy typu II</t></is></c><c r="I110" s="2" t="inlineStr"><is><t>Cukrzyca ciężarnych</t></is></c><c r="J110" s="2" t="inlineStr" /><c r="K110" s="2" t="inlineStr" /><c r="L110" s="2" t="inlineStr" /><c r="M110" s="2" t="inlineStr" /><c r="N110" s="2" t="inlineStr" /><c r="O110" s="2" t="inlineStr" /><c r="P110" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q110" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="111"><c r="A111" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B111" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C111" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D111" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E111" s="2" t="inlineStr"><is><t>Długodziałające analogii insuliny w porównaniu do insuliny protaminowo-cynkowej (NPH) charakteryzują się:</t></is></c><c r="F111" s="2" t="inlineStr"><is><t>Mniejszym ryzykiem hipoglikemii</t></is></c><c r="G111" s="2" t="inlineStr" /><c r="H111" s="2" t="inlineStr" /><c r="I111" s="2" t="inlineStr" /><c r="J111" s="2" t="inlineStr" /><c r="K111" s="2" t="inlineStr"><is><t>Mniejszym ryzykiem onkologicznym</t></is></c><c r="L111" s="2" t="inlineStr"><is><t>Większym ryzykiem zjawiska brzasku</t></is></c><c r="M111" s="2" t="inlineStr"><is><t>Działaniem anorektycznym</t></is></c><c r="N111" s="2" t="inlineStr" /><c r="O111" s="2" t="inlineStr" /><c r="P111" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q111" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="112"><c r="A112" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B112" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C112" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D112" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E112" s="2" t="inlineStr"><is><t>Zmniejszenie obwodowej konwersji tyroksyny do trójjodotyroniny jest efektem stosowania:</t></is></c><c r="F112" s="2" t="inlineStr"><is><t>Hydrokortyzonu</t></is></c><c r="G112" s="2" t="inlineStr"><is><t>Propylotiouracylu</t></is></c><c r="H112" s="2" t="inlineStr"><is><t>Propanololu</t></is></c><c r="I112" s="2" t="inlineStr" /><c r="J112" s="2" t="inlineStr" /><c r="K112" s="2" t="inlineStr"><is><t>Płynu Lugola</t></is></c><c r="L112" s="2" t="inlineStr" /><c r="M112" s="2" t="inlineStr" /><c r="N112" s="2" t="inlineStr" /><c r="O112" s="2" t="inlineStr" /><c r="P112" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q112" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="113"><c r="A113" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B113" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C113" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D113" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E113" s="2" t="inlineStr"><is><t>Wskazaniem do stosowania hormonalnej terapii zastępczej u kobiet po menopauzie jest:</t></is></c><c r="F113" s="2" t="inlineStr"><is><t>Obecność objawów wypadowych</t></is></c><c r="G113" s="2" t="inlineStr" /><c r="H113" s="2" t="inlineStr" /><c r="I113" s="2" t="inlineStr" /><c r="J113" s="2" t="inlineStr" /><c r="K113" s="2" t="inlineStr"><is><t>Wtórna profilaktyka chorób układu krążenia</t></is></c><c r="L113" s="2" t="inlineStr"><is><t>Profilaktyka osteoporozy</t></is></c><c r="M113" s="2" t="inlineStr"><is><t>Zapobieganie chorobie Alzheimera</t></is></c><c r="N113" s="2" t="inlineStr" /><c r="O113" s="2" t="inlineStr" /><c r="P113" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q113" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="114"><c r="A114" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B114" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C114" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D114" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E114" s="2" t="inlineStr"><is><t>Przeciwbólowy efekt pułapowy wykazuje:</t></is></c><c r="F114" s="2" t="inlineStr"><is><t>Naproksen</t></is></c><c r="G114" s="2" t="inlineStr"><is><t>Buprenorfina</t></is></c><c r="H114" s="2" t="inlineStr"><is><t>Ibuprofen</t></is></c><c r="I114" s="2" t="inlineStr" /><c r="J114" s="2" t="inlineStr" /><c r="K114" s="2" t="inlineStr"><is><t>Oksykodon</t></is></c><c r="L114" s="2" t="inlineStr" /><c r="M114" s="2" t="inlineStr" /><c r="N114" s="2" t="inlineStr" /><c r="O114" s="2" t="inlineStr" /><c r="P114" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q114" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="115"><c r="A115" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B115" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C115" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D115" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E115" s="2" t="inlineStr"><is><t>Teofilina:</t></is></c><c r="F115" s="2" t="inlineStr"><is><t>Jest anatgonistą receptora adenozynowego</t></is></c><c r="G115" s="2" t="inlineStr"><is><t>Hamuje aktywność fosfodiesteraz</t></is></c><c r="H115" s="2" t="inlineStr"><is><t>Zwiększa przepływ nerkowy</t></is></c><c r="I115" s="2" t="inlineStr"><is><t>Pobudza ośrodek oddechowy w rdzeniu przedłużonym</t></is></c><c r="J115" s="2" t="inlineStr" /><c r="K115" s="2" t="inlineStr" /><c r="L115" s="2" t="inlineStr" /><c r="M115" s="2" t="inlineStr" /><c r="N115" s="2" t="inlineStr" /><c r="O115" s="2" t="inlineStr" /><c r="P115" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q115" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="116"><c r="A116" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B116" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C116" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D116" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E116" s="2" t="inlineStr"><is><t>Idealny glikokortykosteroid wziewny:</t></is></c><c r="F116" s="2" t="inlineStr"><is><t>Połknięty charakteryzuje się niewielką biodostępnością</t></is></c><c r="G116" s="2" t="inlineStr" /><c r="H116" s="2" t="inlineStr" /><c r="I116" s="2" t="inlineStr" /><c r="J116" s="2" t="inlineStr" /><c r="K116" s="2" t="inlineStr"><is><t>Dobrze wchłania się z pęcherzyków płucnych</t></is></c><c r="L116" s="2" t="inlineStr"><is><t>Nie podlega efektowi pierwszego przejścia przez wątrobę</t></is></c><c r="M116" s="2" t="inlineStr"><is><t>Ma krótki okres półtrwania kompleksu glikokortkosteroidu z receptorem t1/2=2-3h</t></is></c><c r="N116" s="2" t="inlineStr" /><c r="O116" s="2" t="inlineStr" /><c r="P116" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q116" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="117"><c r="A117" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B117" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C117" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D117" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E117" s="2" t="inlineStr"><is><t>Działanie keratolityczne wykazuje:</t></is></c><c r="F117" s="2" t="inlineStr"><is><t>Mocznik</t></is></c><c r="G117" s="2" t="inlineStr"><is><t>Kwas salicylowy</t></is></c><c r="H117" s="2" t="inlineStr"><is><t>Nadtlenek benzoilu</t></is></c><c r="I117" s="2" t="inlineStr" /><c r="J117" s="2" t="inlineStr" /><c r="K117" s="2" t="inlineStr"><is><t>Metoksalen</t></is></c><c r="L117" s="2" t="inlineStr" /><c r="M117" s="2" t="inlineStr" /><c r="N117" s="2" t="inlineStr" /><c r="O117" s="2" t="inlineStr" /><c r="P117" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q117" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="118"><c r="A118" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B118" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C118" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D118" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E118" s="2" t="inlineStr"><is><t>W zatruciu solami litu:</t></is></c><c r="F118" s="2" t="inlineStr"><is><t>Należy natychmiast zakończyć podawanie litu</t></is></c><c r="G118" s="2" t="inlineStr"><is><t>W leczeniu ostrego zatrucia istotne znaczenie ma intensywne wyrównanie zaburzeń gospodarki wodno-elektrolitowej, zwłaszcza uzupełnianie niedoboru sodu poprzez przetaczanie roztworu 0,9% NaCl dożylnie</t></is></c><c r="H118" s="2" t="inlineStr"><is><t>Podstawową metodą eliminacji leku jest hemodializa</t></is></c><c r="I118" s="2" t="inlineStr" /><c r="J118" s="2" t="inlineStr" /><c r="K118" s="2" t="inlineStr"><is><t>Korzystne działanie ma stosowanie węgla aktywowanego</t></is></c><c r="L118" s="2" t="inlineStr" /><c r="M118" s="2" t="inlineStr" /><c r="N118" s="2" t="inlineStr" /><c r="O118" s="2" t="inlineStr" /><c r="P118" s="2" t="inlineStr"><is><t>EGZ 2019 I termin</t></is></c><c r="Q118" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="119"><c r="A119" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B119" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C119" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D119" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E119" s="2" t="inlineStr"><is><t>Fluorochinolony:</t></is></c><c r="F119" s="2" t="inlineStr"><is><t>mogą spowodować zapalenie ścięgien</t></is></c><c r="G119" s="2" t="inlineStr"><is><t>mogą być przyczyną zaburzeń rytmu serca</t></is></c><c r="H119" s="2" t="inlineStr" /><c r="I119" s="2" t="inlineStr" /><c r="J119" s="2" t="inlineStr" /><c r="K119" s="2" t="inlineStr"><is><t>wszystkie generacje mają zbliżoną skuteczność przeciwko Gram ujemnym pałeczkom niefermentującym</t></is></c><c r="L119" s="2" t="inlineStr"><is><t>są agonistami receptorów GABA-A wywołując efekt sedatywny</t></is></c><c r="M119" s="2" t="inlineStr" /><c r="N119" s="2" t="inlineStr" /><c r="O119" s="2" t="inlineStr" /><c r="P119" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q119" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="120"><c r="A120" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B120" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C120" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D120" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E120" s="2" t="inlineStr"><is><t>Fluorochinolony:</t></is></c><c r="F120" s="2" t="inlineStr"><is><t>mogą powodować zapalenie więzadeł</t></is></c><c r="G120" s="2" t="inlineStr" /><c r="H120" s="2" t="inlineStr" /><c r="I120" s="2" t="inlineStr" /><c r="J120" s="2" t="inlineStr" /><c r="K120" s="2" t="inlineStr"><is><t>słabo wchłaniają się z przewodu pokarmowego</t></is></c><c r="L120" s="2" t="inlineStr"><is><t>są grupą, na którą rzadko stwierdza się oporność bakteryjną</t></is></c><c r="M120" s="2" t="inlineStr"><is><t>niezależnie od generacji wykazują aktywność wyłącznie wobec bakterii tlenowych</t></is></c><c r="N120" s="2" t="inlineStr" /><c r="O120" s="2" t="inlineStr" /><c r="P120" s="2" t="inlineStr"><is><t>KOLOKWIUM 2 – 2017/18 - 2 termin</t></is></c><c r="Q120" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="121"><c r="A121" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B121" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C121" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D121" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E121" s="2" t="inlineStr"><is><t>Błędny schemat terapeutyczny to zastosowanie:</t></is></c><c r="F121" s="2" t="inlineStr"><is><t>loperamidu w zapalnej biegunce poantybiotykowej przez 10 dni</t></is></c><c r="G121" s="2" t="inlineStr" /><c r="H121" s="2" t="inlineStr" /><c r="I121" s="2" t="inlineStr" /><c r="J121" s="2" t="inlineStr" /><c r="K121" s="2" t="inlineStr"><is><t>azytromycyny w krztuścu przez 5 dni</t></is></c><c r="L121" s="2" t="inlineStr"><is><t>kotrymoksazolu w niepowikłanym zakażeniu układu moczowego przez 3 dni</t></is></c><c r="M121" s="2" t="inlineStr"><is><t>fenoksymetylpenicyliny w anginie paciorkowcowej przez 10 dni</t></is></c><c r="N121" s="2" t="inlineStr" /><c r="O121" s="2" t="inlineStr" /><c r="P121" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q121" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="122"><c r="A122" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B122" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C122" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D122" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E122" s="2" t="inlineStr"><is><t>W leczeniu 60-letniego pacjenta z pozaszpitalnym zapaleniem płuc (skala CURB-0pkt) uwzględniającym typową etiologię zakażenia u dorosłych należy:</t></is></c><c r="F122" s="2" t="inlineStr"><is><t>stosować stałe optymalne przedziały dawkowania w ciągu całej doby</t></is></c><c r="G122" s="2" t="inlineStr"><is><t>w razie nadwrażliwości na leczenie początkowe w wywiadach zastosować lewofloksacynę lub moksyfloksacynę</t></is></c><c r="H122" s="2" t="inlineStr" /><c r="I122" s="2" t="inlineStr" /><c r="J122" s="2" t="inlineStr" /><c r="K122" s="2" t="inlineStr"><is><t>leczyć 2 lekami przeciwbakteryjnymi o różnych mechanizmach działania</t></is></c><c r="L122" s="2" t="inlineStr"><is><t>prowadzić terapię co najmniej 21 dni</t></is></c><c r="M122" s="2" t="inlineStr" /><c r="N122" s="2" t="inlineStr" /><c r="O122" s="2" t="inlineStr" /><c r="P122" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q122" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="123"><c r="A123" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B123" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C123" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D123" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E123" s="2" t="inlineStr"><is><t>W leczeniu zapalenia opon mózgowo-rdzeniowych uzasadnione jest zastosowanie:</t></is></c><c r="F123" s="2" t="inlineStr"><is><t>ceftriaksonu</t></is></c><c r="G123" s="2" t="inlineStr"><is><t>acyklowiru</t></is></c><c r="H123" s="2" t="inlineStr"><is><t>meropenemu</t></is></c><c r="I123" s="2" t="inlineStr"><is><t>flukonazol</t></is></c><c r="J123" s="2" t="inlineStr" /><c r="K123" s="2" t="inlineStr" /><c r="L123" s="2" t="inlineStr" /><c r="M123" s="2" t="inlineStr" /><c r="N123" s="2" t="inlineStr" /><c r="O123" s="2" t="inlineStr" /><c r="P123" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q123" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="124"><c r="A124" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B124" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C124" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D124" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E124" s="2" t="inlineStr"><is><t>Wyłącznie na drobnoustroje Gram ujemne działa:</t></is></c><c r="F124" s="2" t="inlineStr"><is><t>aztreonam</t></is></c><c r="G124" s="2" t="inlineStr" /><c r="H124" s="2" t="inlineStr" /><c r="I124" s="2" t="inlineStr" /><c r="J124" s="2" t="inlineStr" /><c r="K124" s="2" t="inlineStr"><is><t>mupirocyna</t></is></c><c r="L124" s="2" t="inlineStr"><is><t>kwas fusydowy</t></is></c><c r="M124" s="2" t="inlineStr"><is><t>metronidazol</t></is></c><c r="N124" s="2" t="inlineStr" /><c r="O124" s="2" t="inlineStr" /><c r="P124" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q124" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="125"><c r="A125" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B125" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C125" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D125" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E125" s="2" t="inlineStr"><is><t>W leczeniu toksoplazmozy wykorzystuje się:</t></is></c><c r="F125" s="2" t="inlineStr"><is><t>pirymetaminę z sulfadiazyną</t></is></c><c r="G125" s="2" t="inlineStr"><is><t>spiramycynę</t></is></c><c r="H125" s="2" t="inlineStr" /><c r="I125" s="2" t="inlineStr" /><c r="J125" s="2" t="inlineStr" /><c r="K125" s="2" t="inlineStr"><is><t>dalfoprystynę/chinuprystynę</t></is></c><c r="L125" s="2" t="inlineStr"><is><t>oksytetracyklinę</t></is></c><c r="M125" s="2" t="inlineStr" /><c r="N125" s="2" t="inlineStr" /><c r="O125" s="2" t="inlineStr" /><c r="P125" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q125" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="126"><c r="A126" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B126" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C126" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D126" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E126" s="2" t="inlineStr"><is><t>Do odległych działań niepożądanych terapii HAART (Highly Active Antiretroviral Therapy) należy:</t></is></c><c r="F126" s="2" t="inlineStr"><is><t>uszkodzenie wątroby</t></is></c><c r="G126" s="2" t="inlineStr"><is><t>lipodystrofia</t></is></c><c r="H126" s="2" t="inlineStr"><is><t>kwasica mleczanowa</t></is></c><c r="I126" s="2" t="inlineStr"><is><t>insulinooporność</t></is></c><c r="J126" s="2" t="inlineStr" /><c r="K126" s="2" t="inlineStr" /><c r="L126" s="2" t="inlineStr" /><c r="M126" s="2" t="inlineStr" /><c r="N126" s="2" t="inlineStr" /><c r="O126" s="2" t="inlineStr" /><c r="P126" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q126" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="127"><c r="A127" s="2" t="inlineStr"><is><t>LEKI PRZECIWGRZYBICZE</t></is></c><c r="B127" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C127" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D127" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E127" s="2" t="inlineStr"><is><t>W grzybiczym zakażeniu paznokci można zastosować</t></is></c><c r="F127" s="2" t="inlineStr"><is><t>amorolfinę</t></is></c><c r="G127" s="2" t="inlineStr" /><c r="H127" s="2" t="inlineStr" /><c r="I127" s="2" t="inlineStr" /><c r="J127" s="2" t="inlineStr" /><c r="K127" s="2" t="inlineStr"><is><t>natamycynę</t></is></c><c r="L127" s="2" t="inlineStr"><is><t>klotrymazol</t></is></c><c r="M127" s="2" t="inlineStr"><is><t>kaspofunginę</t></is></c><c r="N127" s="2" t="inlineStr" /><c r="O127" s="2" t="inlineStr" /><c r="P127" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q127" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="128"><c r="A128" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B128" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C128" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D128" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E128" s="2" t="inlineStr"><is><t>Efekt bakteriobójczy zależny od skumulowanej ekspozycji (AUC24/MIC) wykazuje:</t></is></c><c r="F128" s="2" t="inlineStr"><is><t>lewofloksacyna</t></is></c><c r="G128" s="2" t="inlineStr"><is><t>azytromycyna</t></is></c><c r="H128" s="2" t="inlineStr" /><c r="I128" s="2" t="inlineStr" /><c r="J128" s="2" t="inlineStr" /><c r="K128" s="2" t="inlineStr"><is><t>amoksycylina z kwasem klawulanowym</t></is></c><c r="L128" s="2" t="inlineStr"><is><t>amikacyna</t></is></c><c r="M128" s="2" t="inlineStr" /><c r="N128" s="2" t="inlineStr" /><c r="O128" s="2" t="inlineStr" /><c r="P128" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q128" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="129"><c r="A129" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B129" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C129" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D129" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E129" s="2" t="inlineStr"><is><t>Do odkażania rany w obrębie skóry można zastosować:</t></is></c><c r="F129" s="2" t="inlineStr"><is><t>oktenidynę</t></is></c><c r="G129" s="2" t="inlineStr"><is><t>jodopowidon</t></is></c><c r="H129" s="2" t="inlineStr" /><c r="I129" s="2" t="inlineStr" /><c r="J129" s="2" t="inlineStr" /><c r="K129" s="2" t="inlineStr"><is><t>wodę do wstrzyknięć</t></is></c><c r="L129" s="2" t="inlineStr"><is><t>kwas borowy</t></is></c><c r="M129" s="2" t="inlineStr" /><c r="N129" s="2" t="inlineStr" /><c r="O129" s="2" t="inlineStr" /><c r="P129" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q129" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="130"><c r="A130" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B130" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C130" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D130" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E130" s="2" t="inlineStr"><is><t>Koszt dodatkowego roku życia skorygowanego o jakość (ang. QALY – quality adjusted life year):</t></is></c><c r="F130" s="2" t="inlineStr"><is><t>stanowi formalne kryterium refundacyjne zgodnie z obowiązującymi regulacjami prawnymi</t></is></c><c r="G130" s="2" t="inlineStr"><is><t>jest wynikiem analizy kosztów użyteczności</t></is></c><c r="H130" s="2" t="inlineStr"><is><t>jego wartość progowa, czyli maksymalna dla procedur uznanych za kosztowo efektywne, stanowi 3-krotność produktu krajowego brutto per capita zgodnie z obowiązującymi regulacjami prawnymi</t></is></c><c r="I130" s="2" t="inlineStr" /><c r="J130" s="2" t="inlineStr" /><c r="K130" s="2" t="inlineStr"><is><t>możliwy jest do oszacowania tylko w przypadku procedur zmniejszających umieralność całkowitą</t></is></c><c r="L130" s="2" t="inlineStr" /><c r="M130" s="2" t="inlineStr" /><c r="N130" s="2" t="inlineStr" /><c r="O130" s="2" t="inlineStr" /><c r="P130" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q130" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="131"><c r="A131" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B131" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C131" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D131" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E131" s="2" t="inlineStr"><is><t>U pacjenta z niewydolnością nerek należy dokonać modyfikacji dawek:</t></is></c><c r="F131" s="2" t="inlineStr"><is><t>wankomycyny</t></is></c><c r="G131" s="2" t="inlineStr"><is><t>cyprofloksacyny</t></is></c><c r="H131" s="2" t="inlineStr"><is><t>gentamycyny</t></is></c><c r="I131" s="2" t="inlineStr" /><c r="J131" s="2" t="inlineStr" /><c r="K131" s="2" t="inlineStr"><is><t>erytromycyny</t></is></c><c r="L131" s="2" t="inlineStr" /><c r="M131" s="2" t="inlineStr" /><c r="N131" s="2" t="inlineStr" /><c r="O131" s="2" t="inlineStr" /><c r="P131" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q131" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="132"><c r="A132" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B132" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C132" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D132" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E132" s="2" t="inlineStr"><is><t>Rotacja opioidów jest uzasadniona w przypadku:</t></is></c><c r="F132" s="2" t="inlineStr"><is><t>nudności</t></is></c><c r="G132" s="2" t="inlineStr"><is><t>zaburzeń świadomości</t></is></c><c r="H132" s="2" t="inlineStr"><is><t>długotrwałej (bezterminowej) terapii w celu ułatwienia jej prowadzenia</t></is></c><c r="I132" s="2" t="inlineStr" /><c r="J132" s="2" t="inlineStr" /><c r="K132" s="2" t="inlineStr"><is><t>zaparć</t></is></c><c r="L132" s="2" t="inlineStr" /><c r="M132" s="2" t="inlineStr" /><c r="N132" s="2" t="inlineStr" /><c r="O132" s="2" t="inlineStr" /><c r="P132" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q132" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="133"><c r="A133" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B133" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C133" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D133" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E133" s="2" t="inlineStr"><is><t>Dapagliflozyna:</t></is></c><c r="F133" s="2" t="inlineStr"><is><t>zwiększa ryzyko zakażeń układu moczowo-płciowego</t></is></c><c r="G133" s="2" t="inlineStr"><is><t>może spowodować kwasicę ketonową</t></is></c><c r="H133" s="2" t="inlineStr" /><c r="I133" s="2" t="inlineStr" /><c r="J133" s="2" t="inlineStr" /><c r="K133" s="2" t="inlineStr"><is><t>zmniejsza glukozurię</t></is></c><c r="L133" s="2" t="inlineStr"><is><t>nie może być stosowana łącznie z insuliną</t></is></c><c r="M133" s="2" t="inlineStr" /><c r="N133" s="2" t="inlineStr" /><c r="O133" s="2" t="inlineStr" /><c r="P133" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q133" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="134"><c r="A134" s="2" t="inlineStr"><is><t>CUKRZYCA</t></is></c><c r="B134" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C134" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D134" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E134" s="2" t="inlineStr"><is><t>Wskaż zdanie prawdziwe:</t></is></c><c r="F134" s="2" t="inlineStr"><is><t>zwiększenie stężenia glukozy w godzinach porannych poprzedzone hipoglikemią nocną może być wskazaniem do zmniejszenia dawki insuliny bazowej</t></is></c><c r="G134" s="2" t="inlineStr"><is><t>efekt brzasku może zmniejszyć zastosowanie długodziałających bezszczytowych analogów insuliny</t></is></c><c r="H134" s="2" t="inlineStr"><is><t>kardioprotekcyjne działanie empagliflozyny może mieć związek z usprawnieniem procesów energetycznych w komórkach mięśnia sercowego</t></is></c><c r="I134" s="2" t="inlineStr" /><c r="J134" s="2" t="inlineStr" /><c r="K134" s="2" t="inlineStr"><is><t>insulina izofanowa (NPH) jest przeznaczona do stosowana przed głównymi posiłkami</t></is></c><c r="L134" s="2" t="inlineStr" /><c r="M134" s="2" t="inlineStr" /><c r="N134" s="2" t="inlineStr" /><c r="O134" s="2" t="inlineStr" /><c r="P134" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q134" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="135"><c r="A135" s="2" t="inlineStr"><is><t>TARCZYCA</t></is></c><c r="B135" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C135" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D135" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E135" s="2" t="inlineStr"><is><t>W leczeniu nadczynności tarczycy można zastosować:</t></is></c><c r="F135" s="2" t="inlineStr"><is><t>jod promieniotwórczy 131 I</t></is></c><c r="G135" s="2" t="inlineStr"><is><t>płyn Lugola</t></is></c><c r="H135" s="2" t="inlineStr"><is><t>tiamazol</t></is></c><c r="I135" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="J135" s="2" t="inlineStr" /><c r="K135" s="2" t="inlineStr" /><c r="L135" s="2" t="inlineStr" /><c r="M135" s="2" t="inlineStr" /><c r="N135" s="2" t="inlineStr" /><c r="O135" s="2" t="inlineStr" /><c r="P135" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q135" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="136"><c r="A136" s="2" t="inlineStr"><is><t>HORMONY PŁCIOWE</t></is></c><c r="B136" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C136" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D136" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E136" s="2" t="inlineStr"><is><t>Do progestagenów należy:</t></is></c><c r="F136" s="2" t="inlineStr"><is><t>megestrol</t></is></c><c r="G136" s="2" t="inlineStr"><is><t>noretysteron</t></is></c><c r="H136" s="2" t="inlineStr" /><c r="I136" s="2" t="inlineStr" /><c r="J136" s="2" t="inlineStr" /><c r="K136" s="2" t="inlineStr"><is><t>dutasteryd</t></is></c><c r="L136" s="2" t="inlineStr"><is><t>anastrozol</t></is></c><c r="M136" s="2" t="inlineStr" /><c r="N136" s="2" t="inlineStr" /><c r="O136" s="2" t="inlineStr" /><c r="P136" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q136" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="137"><c r="A137" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B137" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C137" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D137" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E137" s="2" t="inlineStr"><is><t>Do leków antyagregacyjnych stosowanych w profilaktyce wtórnej udaru niedokrwiennego mózgu na podłożu miażdżycy naczyń do- i mózgowych należą:</t></is></c><c r="F137" s="2" t="inlineStr"><is><t>klopidogrel</t></is></c><c r="G137" s="2" t="inlineStr"><is><t>kwas acetylosalicylowy</t></is></c><c r="H137" s="2" t="inlineStr" /><c r="I137" s="2" t="inlineStr" /><c r="J137" s="2" t="inlineStr" /><c r="K137" s="2" t="inlineStr"><is><t>tikagrelor</t></is></c><c r="L137" s="2" t="inlineStr"><is><t>prasugrel</t></is></c><c r="M137" s="2" t="inlineStr" /><c r="N137" s="2" t="inlineStr" /><c r="O137" s="2" t="inlineStr" /><c r="P137" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q137" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="138"><c r="A138" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B138" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C138" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D138" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E138" s="2" t="inlineStr"><is><t>W ciężkiej hiperkalcemii (&gt;15mg/dl) można zastosować dożylnie:</t></is></c><c r="F138" s="2" t="inlineStr"><is><t>kalcytoninę</t></is></c><c r="G138" s="2" t="inlineStr"><is><t>pamidronian</t></is></c><c r="H138" s="2" t="inlineStr"><is><t>hydrokortyzon</t></is></c><c r="I138" s="2" t="inlineStr"><is><t>furosemid</t></is></c><c r="J138" s="2" t="inlineStr" /><c r="K138" s="2" t="inlineStr" /><c r="L138" s="2" t="inlineStr" /><c r="M138" s="2" t="inlineStr" /><c r="N138" s="2" t="inlineStr" /><c r="O138" s="2" t="inlineStr" /><c r="P138" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q138" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="139"><c r="A139" s="2" t="inlineStr"><is><t>GLIKOKORTYKOSTEROIDY</t></is></c><c r="B139" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C139" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D139" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E139" s="2" t="inlineStr"><is><t>Immunosupresyjne działanie glikokortykosteroidów jest spowodowane:</t></is></c><c r="F139" s="2" t="inlineStr"><is><t>redukcją liczby limfocytów T</t></is></c><c r="G139" s="2" t="inlineStr"><is><t>zahamowaniem funkcji makrofagów tkankowych</t></is></c><c r="H139" s="2" t="inlineStr" /><c r="I139" s="2" t="inlineStr" /><c r="J139" s="2" t="inlineStr" /><c r="K139" s="2" t="inlineStr"><is><t>zwiększeniem syntezy IL-2</t></is></c><c r="L139" s="2" t="inlineStr"><is><t>aktywacją fosfolipazy A2 i zmniejszeniem syntezy prostaglandyn</t></is></c><c r="M139" s="2" t="inlineStr" /><c r="N139" s="2" t="inlineStr" /><c r="O139" s="2" t="inlineStr" /><c r="P139" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q139" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="140"><c r="A140" s="2" t="inlineStr"><is><t>OSTEOPOROZA</t></is></c><c r="B140" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C140" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D140" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E140" s="2" t="inlineStr"><is><t>91-letni mężczyzna jest leczony od co najmniej 6 miesięcy tamsulozyną, finasterydem, diosminą, piracetamem, zolpidemem, witaminą D3 w dużej dawce i węglanem wapnia. Na tej podstawie można powiedzieć, że:</t></is></c><c r="F140" s="2" t="inlineStr"><is><t>choruje na rozrost gruczołu krokowego</t></is></c><c r="G140" s="2" t="inlineStr"><is><t>jest uzależniony od zolpidemu</t></is></c><c r="H140" s="2" t="inlineStr"><is><t>można bez konsekwencji odstawić piracetam</t></is></c><c r="I140" s="2" t="inlineStr"><is><t>terapia zmniejsza ryzyko osteoporotycznych złamań kości</t></is></c><c r="J140" s="2" t="inlineStr" /><c r="K140" s="2" t="inlineStr" /><c r="L140" s="2" t="inlineStr" /><c r="M140" s="2" t="inlineStr" /><c r="N140" s="2" t="inlineStr" /><c r="O140" s="2" t="inlineStr" /><c r="P140" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q140" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="141"><c r="A141" s="2" t="inlineStr"><is><t>STANY NAGŁE</t></is></c><c r="B141" s="2" t="inlineStr"><is><t>Antidotum</t></is></c><c r="C141" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D141" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E141" s="2" t="inlineStr"><is><t>Witamina K1 (fitomenadion):</t></is></c><c r="F141" s="2" t="inlineStr"><is><t>może być wskazana u osób ze spontanicznym zwiększeniem INR&gt;GGN (górnej granicy normy) spowodowanym antybiotykami niszczącymi fizjologiczną florę jelit</t></is></c><c r="G141" s="2" t="inlineStr"><is><t>nie antagonizuje działania heparyny</t></is></c><c r="H141" s="2" t="inlineStr"><is><t>może spowodować reakcję rzekomoanafilaktyczną</t></is></c><c r="I141" s="2" t="inlineStr"><is><t>jest antidotum w przedawkowaniu pochodnych hydroksykumaryny</t></is></c><c r="J141" s="2" t="inlineStr" /><c r="K141" s="2" t="inlineStr" /><c r="L141" s="2" t="inlineStr" /><c r="M141" s="2" t="inlineStr" /><c r="N141" s="2" t="inlineStr" /><c r="O141" s="2" t="inlineStr" /><c r="P141" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q141" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="142"><c r="A142" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B142" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C142" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D142" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E142" s="2" t="inlineStr"><is><t>Działanie zapierające wykazuje:</t></is></c><c r="F142" s="2" t="inlineStr"><is><t>oksykodon</t></is></c><c r="G142" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="H142" s="2" t="inlineStr"><is><t>oktreotyd</t></is></c><c r="I142" s="2" t="inlineStr" /><c r="J142" s="2" t="inlineStr" /><c r="K142" s="2" t="inlineStr"><is><t>fosforan sodu</t></is></c><c r="L142" s="2" t="inlineStr" /><c r="M142" s="2" t="inlineStr" /><c r="N142" s="2" t="inlineStr" /><c r="O142" s="2" t="inlineStr" /><c r="P142" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q142" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="143"><c r="A143" s="2" t="inlineStr"><is><t>LEKI PRZECIWBAKTERYJNE</t></is></c><c r="B143" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C143" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D143" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E143" s="2" t="inlineStr"><is><t>Działanie zapierające wykazuje:</t></is></c><c r="F143" s="2" t="inlineStr"><is><t>werapamil</t></is></c><c r="G143" s="2" t="inlineStr"><is><t>węglan wapnia</t></is></c><c r="H143" s="2" t="inlineStr"><is><t>odwar z suchych owoców borówki czernicy</t></is></c><c r="I143" s="2" t="inlineStr" /><c r="J143" s="2" t="inlineStr" /><c r="K143" s="2" t="inlineStr"><is><t>erytromycyna</t></is></c><c r="L143" s="2" t="inlineStr" /><c r="M143" s="2" t="inlineStr" /><c r="N143" s="2" t="inlineStr" /><c r="O143" s="2" t="inlineStr" /><c r="P143" s="2" t="inlineStr"><is><t>EGZ 2016 I termin</t></is></c><c r="Q143" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="144"><c r="A144" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B144" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C144" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D144" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E144" s="2" t="inlineStr"><is><t>W leczeniu ostrej biegunki u dzieci uzasadnione jest zastosowanie:</t></is></c><c r="F144" s="2" t="inlineStr"><is><t>probiotyku S. boulardi</t></is></c><c r="G144" s="2" t="inlineStr"><is><t>racekadotrylu</t></is></c><c r="H144" s="2" t="inlineStr"><is><t>doustnego płynu nawadniającego</t></is></c><c r="I144" s="2" t="inlineStr" /><c r="J144" s="2" t="inlineStr" /><c r="K144" s="2" t="inlineStr"><is><t>loperamidu</t></is></c><c r="L144" s="2" t="inlineStr" /><c r="M144" s="2" t="inlineStr" /><c r="N144" s="2" t="inlineStr" /><c r="O144" s="2" t="inlineStr" /><c r="P144" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q144" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="145"><c r="A145" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B145" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C145" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D145" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E145" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek - mechanizm działania:</t></is></c><c r="F145" s="2" t="inlineStr"><is><t>itopryd - antagonista receptora D2</t></is></c><c r="G145" s="2" t="inlineStr"><is><t>alwimopan - antagonista receptora μ</t></is></c><c r="H145" s="2" t="inlineStr" /><c r="I145" s="2" t="inlineStr" /><c r="J145" s="2" t="inlineStr" /><c r="K145" s="2" t="inlineStr"><is><t>alweryna - agonista receptora motylinowego</t></is></c><c r="L145" s="2" t="inlineStr"><is><t>simetykon - agonista receptora 5-HT4</t></is></c><c r="M145" s="2" t="inlineStr" /><c r="N145" s="2" t="inlineStr" /><c r="O145" s="2" t="inlineStr" /><c r="P145" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q145" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="146"><c r="A146" s="2" t="inlineStr"><is><t>UKŁAD POKARMOWY</t></is></c><c r="B146" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C146" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D146" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E146" s="2" t="inlineStr"><is><t>Wybierz prawidłowe połączenie lek - mechanizm działania:</t></is></c><c r="F146" s="2" t="inlineStr"><is><t>orlistat - blokowanie lipaz wytwarzanych w przewodzie pokarmowym</t></is></c><c r="G146" s="2" t="inlineStr"><is><t>tramadol – blokowanie zwrotnego wychwytu noradrenaliny i serotoniny w synapsach zstępującego układu analgetycznego</t></is></c><c r="H146" s="2" t="inlineStr"><is><t>ezetymib – hamowanie aktywności białka NPC1L1 w nabłonku błony śluzowej jelita</t></is></c><c r="I146" s="2" t="inlineStr"><is><t>celekoksyb -wybiórcze zablokowanie COX-2</t></is></c><c r="J146" s="2" t="inlineStr" /><c r="K146" s="2" t="inlineStr" /><c r="L146" s="2" t="inlineStr" /><c r="M146" s="2" t="inlineStr" /><c r="N146" s="2" t="inlineStr" /><c r="O146" s="2" t="inlineStr" /><c r="P146" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q146" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="147"><c r="A147" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B147" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C147" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D147" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E147" s="2" t="inlineStr"><is><t>W kolce wątrobowej uzasadnione jest podanie:</t></is></c><c r="F147" s="2" t="inlineStr"><is><t>ketoprofenu i.v</t></is></c><c r="G147" s="2" t="inlineStr"><is><t>papaweryny i.m</t></is></c><c r="H147" s="2" t="inlineStr"><is><t>butylobromku skopolaminy p.r</t></is></c><c r="I147" s="2" t="inlineStr"><is><t>buprenorfiny i.m</t></is></c><c r="J147" s="2" t="inlineStr" /><c r="K147" s="2" t="inlineStr" /><c r="L147" s="2" t="inlineStr" /><c r="M147" s="2" t="inlineStr" /><c r="N147" s="2" t="inlineStr" /><c r="O147" s="2" t="inlineStr" /><c r="P147" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q147" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="148"><c r="A148" s="2" t="inlineStr"><is><t>BÓLE GŁOWY</t></is></c><c r="B148" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C148" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D148" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E148" s="2" t="inlineStr"><is><t>Sumatryptan:</t></is></c><c r="F148" s="2" t="inlineStr"><is><t>pobudzając receptory 5-HT1D wywołuje wybiórczy skurcz naczyń i przerywa napad migreny</t></is></c><c r="G148" s="2" t="inlineStr"><is><t>jest niezalecany u pacjentów z chorobą niedokrwienną serca</t></is></c><c r="H148" s="2" t="inlineStr" /><c r="I148" s="2" t="inlineStr" /><c r="J148" s="2" t="inlineStr" /><c r="K148" s="2" t="inlineStr"><is><t>może być stosowany jedynie podskórnie</t></is></c><c r="L148" s="2" t="inlineStr"><is><t>może być podawany w czasie ciąży</t></is></c><c r="M148" s="2" t="inlineStr" /><c r="N148" s="2" t="inlineStr" /><c r="O148" s="2" t="inlineStr" /><c r="P148" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q148" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="149"><c r="A149" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B149" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C149" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D149" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E149" s="2" t="inlineStr"><is><t>W profilaktyce bólów migrenowych znalazł zastosowanie:</t></is></c><c r="F149" s="2" t="inlineStr"><is><t>topiramat</t></is></c><c r="G149" s="2" t="inlineStr"><is><t>erenumab</t></is></c><c r="H149" s="2" t="inlineStr"><is><t>propranolol</t></is></c><c r="I149" s="2" t="inlineStr"><is><t>toksyna botulinowa</t></is></c><c r="J149" s="2" t="inlineStr" /><c r="K149" s="2" t="inlineStr" /><c r="L149" s="2" t="inlineStr" /><c r="M149" s="2" t="inlineStr" /><c r="N149" s="2" t="inlineStr" /><c r="O149" s="2" t="inlineStr" /><c r="P149" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q149" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="150"><c r="A150" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B150" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C150" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D150" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E150" s="2" t="inlineStr"><is><t>Erytropoetyna może zwiększyć:</t></is></c><c r="F150" s="2" t="inlineStr"><is><t>wartości ciśnienia tętniczego</t></is></c><c r="G150" s="2" t="inlineStr"><is><t>krzepliwość krwi</t></is></c><c r="H150" s="2" t="inlineStr"><is><t>maksymalną wydolność wysiłkową</t></is></c><c r="I150" s="2" t="inlineStr" /><c r="J150" s="2" t="inlineStr" /><c r="K150" s="2" t="inlineStr"><is><t>aktywność amylazy w surowicy</t></is></c><c r="L150" s="2" t="inlineStr" /><c r="M150" s="2" t="inlineStr" /><c r="N150" s="2" t="inlineStr" /><c r="O150" s="2" t="inlineStr" /><c r="P150" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q150" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="151"><c r="A151" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B151" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C151" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D151" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E151" s="2" t="inlineStr"><is><t>W profilaktyce wymiotów w przebiegu kinetoz stosuje się:</t></is></c><c r="F151" s="2" t="inlineStr"><is><t>skopolaminę</t></is></c><c r="G151" s="2" t="inlineStr"><is><t>dimenhydrinat</t></is></c><c r="H151" s="2" t="inlineStr" /><c r="I151" s="2" t="inlineStr" /><c r="J151" s="2" t="inlineStr" /><c r="K151" s="2" t="inlineStr"><is><t>haloperydol</t></is></c><c r="L151" s="2" t="inlineStr"><is><t>betahistynę</t></is></c><c r="M151" s="2" t="inlineStr" /><c r="N151" s="2" t="inlineStr" /><c r="O151" s="2" t="inlineStr" /><c r="P151" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q151" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="152"><c r="A152" s="2" t="inlineStr"><is><t>UKŁAD WSPÓŁCZULNY</t></is></c><c r="B152" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C152" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D152" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E152" s="2" t="inlineStr"><is><t>Oksymetazolina:</t></is></c><c r="F152" s="2" t="inlineStr"><is><t>może doprowadzić do wystąpienia tzw. efektu „ z odbicia”</t></is></c><c r="G152" s="2" t="inlineStr" /><c r="H152" s="2" t="inlineStr" /><c r="I152" s="2" t="inlineStr" /><c r="J152" s="2" t="inlineStr" /><c r="K152" s="2" t="inlineStr"><is><t>jest antagonistą receptorów adrenergicznych alfa</t></is></c><c r="L152" s="2" t="inlineStr"><is><t>wykazuje skuteczność kliniczną po 5. dniach terapii</t></is></c><c r="M152" s="2" t="inlineStr"><is><t>jest podawana doustnie</t></is></c><c r="N152" s="2" t="inlineStr" /><c r="O152" s="2" t="inlineStr" /><c r="P152" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q152" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="153"><c r="A153" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B153" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C153" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D153" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E153" s="2" t="inlineStr"><is><t>Petydyna:</t></is></c><c r="F153" s="2" t="inlineStr"><is><t>ma działanie zapierające</t></is></c><c r="G153" s="2" t="inlineStr"><is><t>nietypowo dla swojej grupy farmakologicznej rozszerza źrenice</t></is></c><c r="H153" s="2" t="inlineStr"><is><t>hamuje ośrodek oddechowy</t></is></c><c r="I153" s="2" t="inlineStr"><is><t>stosowana długotrwale działa neurotoksycznie przez kumulujący się metabolit</t></is></c><c r="J153" s="2" t="inlineStr" /><c r="K153" s="2" t="inlineStr" /><c r="L153" s="2" t="inlineStr" /><c r="M153" s="2" t="inlineStr" /><c r="N153" s="2" t="inlineStr" /><c r="O153" s="2" t="inlineStr" /><c r="P153" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q153" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="154"><c r="A154" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B154" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C154" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D154" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E154" s="2" t="inlineStr"><is><t>Wskaż prawdziwe stwierdzenie dotyczące małopłytkowości typu II wywołanej heparyną:</t></is></c><c r="F154" s="2" t="inlineStr"><is><t>stwierdzenie małopłytkowości immunologicznej w przebiegu leczenia heparyną jest wskazaniem do jej natychmiastowego odstawienia</t></is></c><c r="G154" s="2" t="inlineStr"><is><t>HIT II wiąże się z 20–40-krotnym zwiększeniem ryzyka zakrzepicy żylnej</t></is></c><c r="H154" s="2" t="inlineStr" /><c r="I154" s="2" t="inlineStr" /><c r="J154" s="2" t="inlineStr" /><c r="K154" s="2" t="inlineStr"><is><t>HIT II występuje najczęściej po 3 tygodniach od rozpoczęcia terapii heparyną</t></is></c><c r="L154" s="2" t="inlineStr"><is><t>heparyny drobnocząsteczkowe nie stwarzają ryzyka wystąpienia trombocytopenii immunologicznej</t></is></c><c r="M154" s="2" t="inlineStr" /><c r="N154" s="2" t="inlineStr" /><c r="O154" s="2" t="inlineStr" /><c r="P154" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q154" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="155"><c r="A155" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B155" s="2" t="inlineStr"><is><t>Ciąża</t></is></c><c r="C155" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D155" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E155" s="2" t="inlineStr"><is><t>U kobiet w trzecim trymestrze ciąży przeciwwskazany/-a jest:</t></is></c><c r="F155" s="2" t="inlineStr"><is><t>ketoprofen</t></is></c><c r="G155" s="2" t="inlineStr"><is><t>walsartan</t></is></c><c r="H155" s="2" t="inlineStr"><is><t>acenokumarol</t></is></c><c r="I155" s="2" t="inlineStr" /><c r="J155" s="2" t="inlineStr" /><c r="K155" s="2" t="inlineStr"><is><t>enoksaparyna</t></is></c><c r="L155" s="2" t="inlineStr" /><c r="M155" s="2" t="inlineStr" /><c r="N155" s="2" t="inlineStr" /><c r="O155" s="2" t="inlineStr" /><c r="P155" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q155" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="156"><c r="A156" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B156" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C156" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D156" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E156" s="2" t="inlineStr"><is><t>U pacjenta leczonego przeciwzakrzepowo dabigatranem ze stwierdzonym umiarkowanym aktywnym krwawieniem należy:</t></is></c><c r="F156" s="2" t="inlineStr"><is><t>odroczyć podanie kolejnej dawki leku</t></is></c><c r="G156" s="2" t="inlineStr"><is><t>zapewnić podaż płynów</t></is></c><c r="H156" s="2" t="inlineStr"><is><t>rozważyć podanie węgla aktywowanego jeśli dabigatran był podany niedawno</t></is></c><c r="I156" s="2" t="inlineStr" /><c r="J156" s="2" t="inlineStr" /><c r="K156" s="2" t="inlineStr"><is><t>zastosować siarczan protaminy</t></is></c><c r="L156" s="2" t="inlineStr" /><c r="M156" s="2" t="inlineStr" /><c r="N156" s="2" t="inlineStr" /><c r="O156" s="2" t="inlineStr" /><c r="P156" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q156" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="157"><c r="A157" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B157" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C157" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D157" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E157" s="2" t="inlineStr"><is><t>Nadroparyna:</t></is></c><c r="F157" s="2" t="inlineStr"><is><t>może być podawana dożylnie</t></is></c><c r="G157" s="2" t="inlineStr"><is><t>jest skuteczna w leczeniu zakrzepicy żył głębokich</t></is></c><c r="H157" s="2" t="inlineStr" /><c r="I157" s="2" t="inlineStr" /><c r="J157" s="2" t="inlineStr" /><c r="K157" s="2" t="inlineStr"><is><t>jest antagonistą receptora PAR-1</t></is></c><c r="L157" s="2" t="inlineStr"><is><t>w profilaktyce zakrzepicy żylnej powinna być podana nie później niż 36 godzin przed zabiegiem chirurgicznym</t></is></c><c r="M157" s="2" t="inlineStr" /><c r="N157" s="2" t="inlineStr" /><c r="O157" s="2" t="inlineStr" /><c r="P157" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q157" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="158"><c r="A158" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B158" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C158" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D158" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E158" s="2" t="inlineStr"><is><t>Wskazaniem do podania tkankowego aktywatora plazminogenu (t-PA) może być:</t></is></c><c r="F158" s="2" t="inlineStr"><is><t>zatorowość płucna wysokiego ryzyka (czyli z niestabilnością hemodynamiczną)</t></is></c><c r="G158" s="2" t="inlineStr"><is><t>ostry zator tętnicy kończyny dolnej</t></is></c><c r="H158" s="2" t="inlineStr"><is><t>ostry udar niedokrwienny mózgu</t></is></c><c r="I158" s="2" t="inlineStr" /><c r="J158" s="2" t="inlineStr" /><c r="K158" s="2" t="inlineStr"><is><t>ostry zespół wieńcowy bez uniesienia odcinka ST</t></is></c><c r="L158" s="2" t="inlineStr" /><c r="M158" s="2" t="inlineStr" /><c r="N158" s="2" t="inlineStr" /><c r="O158" s="2" t="inlineStr" /><c r="P158" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q158" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="159"><c r="A159" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B159" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C159" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D159" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E159" s="2" t="inlineStr"><is><t>W udarze niedokrwiennym mózgu należy:</t></is></c><c r="F159" s="2" t="inlineStr"><is><t>obniżać ciśnienie tętnicze jeśli przekracza wartości 220/120 mmHg</t></is></c><c r="G159" s="2" t="inlineStr"><is><t>podać doustnie kwas acetylosalicylowy jeżeli nie można zastosować leczenia trombolitycznego</t></is></c><c r="H159" s="2" t="inlineStr" /><c r="I159" s="2" t="inlineStr" /><c r="J159" s="2" t="inlineStr" /><c r="K159" s="2" t="inlineStr"><is><t>stosować duże dawki heparyny niefrakcjonowanej</t></is></c><c r="L159" s="2" t="inlineStr"><is><t>profilaktycznie podawać antybiotyki β-laktamowe ze względu na bardzo częste występowanie infekcji dróg oddechowych</t></is></c><c r="M159" s="2" t="inlineStr" /><c r="N159" s="2" t="inlineStr" /><c r="O159" s="2" t="inlineStr" /><c r="P159" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q159" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="160"><c r="A160" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B160" s="2" t="inlineStr"><is><t>Mechanizm działania</t></is></c><c r="C160" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D160" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E160" s="2" t="inlineStr"><is><t>Inhibitory reduktazy HMG-CoA zwiększają produkcję:</t></is></c><c r="F160" s="2" t="inlineStr"><is><t>tkankowego aktywatora plazminogenu</t></is></c><c r="G160" s="2" t="inlineStr"><is><t>tlenku azotu</t></is></c><c r="H160" s="2" t="inlineStr" /><c r="I160" s="2" t="inlineStr" /><c r="J160" s="2" t="inlineStr" /><c r="K160" s="2" t="inlineStr"><is><t>metaloproteinaz</t></is></c><c r="L160" s="2" t="inlineStr"><is><t>tromboksanu A2</t></is></c><c r="M160" s="2" t="inlineStr" /><c r="N160" s="2" t="inlineStr" /><c r="O160" s="2" t="inlineStr" /><c r="P160" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q160" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="161"><c r="A161" s="2" t="inlineStr"><is><t>HEMOSTAZA</t></is></c><c r="B161" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C161" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D161" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E161" s="2" t="inlineStr"><is><t>20% roztwór albumin:</t></is></c><c r="F161" s="2" t="inlineStr"><is><t>powoduje ponad 100% przyrost objętości osocza</t></is></c><c r="G161" s="2" t="inlineStr"><is><t>działa objętościowo do 6 h</t></is></c><c r="H161" s="2" t="inlineStr" /><c r="I161" s="2" t="inlineStr" /><c r="J161" s="2" t="inlineStr" /><c r="K161" s="2" t="inlineStr"><is><t>może spowodować uszkodzenie nerek</t></is></c><c r="L161" s="2" t="inlineStr"><is><t>ma istotny wpływ na krzepnięcie krwi</t></is></c><c r="M161" s="2" t="inlineStr" /><c r="N161" s="2" t="inlineStr" /><c r="O161" s="2" t="inlineStr" /><c r="P161" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q161" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="162"><c r="A162" s="2" t="inlineStr"><is><t>UKŁAD PRZYWSPÓŁCZULNY</t></is></c><c r="B162" s="2" t="inlineStr"><is><t>Działania niepożądane</t></is></c><c r="C162" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D162" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E162" s="2" t="inlineStr"><is><t>Zastosowanie atrakurium może być przyczyną:</t></is></c><c r="F162" s="2" t="inlineStr"><is><t>długotrwałego efektu zwiotczającego</t></is></c><c r="G162" s="2" t="inlineStr" /><c r="H162" s="2" t="inlineStr" /><c r="I162" s="2" t="inlineStr" /><c r="J162" s="2" t="inlineStr" /><c r="K162" s="2" t="inlineStr"><is><t>drżenia włókienkowego mięśni szkieletowych</t></is></c><c r="L162" s="2" t="inlineStr"><is><t>anestezji</t></is></c><c r="M162" s="2" t="inlineStr"><is><t>hipertermii złośliwej</t></is></c><c r="N162" s="2" t="inlineStr" /><c r="O162" s="2" t="inlineStr" /><c r="P162" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q162" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="163"><c r="A163" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B163" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C163" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D163" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E163" s="2" t="inlineStr"><is><t>Torasemid:</t></is></c><c r="F163" s="2" t="inlineStr"><is><t>hamuje symporter sodowo-potasowo-chlorkowy części grubościennej ramienia wstępującego pętli Henlego</t></is></c><c r="G163" s="2" t="inlineStr"><is><t>zwiększa aktywność reninową osocza</t></is></c><c r="H163" s="2" t="inlineStr" /><c r="I163" s="2" t="inlineStr" /><c r="J163" s="2" t="inlineStr" /><c r="K163" s="2" t="inlineStr"><is><t>zmniejsza wydalanie wapnia z moczem</t></is></c><c r="L163" s="2" t="inlineStr"><is><t>jest nieskuteczny, jeśli eGFRr &lt; 30 ml/min</t></is></c><c r="M163" s="2" t="inlineStr" /><c r="N163" s="2" t="inlineStr" /><c r="O163" s="2" t="inlineStr" /><c r="P163" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q163" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="164"><c r="A164" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B164" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C164" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D164" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E164" s="2" t="inlineStr"><is><t>Formularz świadomej zgody uczestnika na udział w badaniu klinicznym powinien zostać podpisany:</t></is></c><c r="F164" s="2" t="inlineStr"><is><t>przez uczestnika badania</t></is></c><c r="G164" s="2" t="inlineStr"><is><t>przez badacza</t></is></c><c r="H164" s="2" t="inlineStr"><is><t>w dwóch egzemplarzach</t></is></c><c r="I164" s="2" t="inlineStr" /><c r="J164" s="2" t="inlineStr" /><c r="K164" s="2" t="inlineStr"><is><t>bezpośrednio po badaniach oceniających czy pacjent spełnia kryteria włączenia do badania</t></is></c><c r="L164" s="2" t="inlineStr" /><c r="M164" s="2" t="inlineStr" /><c r="N164" s="2" t="inlineStr" /><c r="O164" s="2" t="inlineStr" /><c r="P164" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q164" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="165"><c r="A165" s="2" t="inlineStr"><is><t>LEKI PRZECIWPASOŻYTNICZE</t></is></c><c r="B165" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C165" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D165" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E165" s="2" t="inlineStr"><is><t>W leczeniu zarażenia owsikiem skuteczny jest:</t></is></c><c r="F165" s="2" t="inlineStr"><is><t>mebendazol</t></is></c><c r="G165" s="2" t="inlineStr"><is><t>albendazol</t></is></c><c r="H165" s="2" t="inlineStr"><is><t>pyrantel</t></is></c><c r="I165" s="2" t="inlineStr" /><c r="J165" s="2" t="inlineStr" /><c r="K165" s="2" t="inlineStr"><is><t>tynidazol</t></is></c><c r="L165" s="2" t="inlineStr" /><c r="M165" s="2" t="inlineStr" /><c r="N165" s="2" t="inlineStr" /><c r="O165" s="2" t="inlineStr" /><c r="P165" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q165" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="166"><c r="A166" s="2" t="inlineStr"><is><t>LEKI PRZECIWWIRUSOWE</t></is></c><c r="B166" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C166" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D166" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E166" s="2" t="inlineStr"><is><t>Cytomegalię u osób z niedoborami odporności należy leczyć stosując:</t></is></c><c r="F166" s="2" t="inlineStr"><is><t>gancyklowir</t></is></c><c r="G166" s="2" t="inlineStr" /><c r="H166" s="2" t="inlineStr" /><c r="I166" s="2" t="inlineStr" /><c r="J166" s="2" t="inlineStr" /><c r="K166" s="2" t="inlineStr"><is><t>zanamiwir</t></is></c><c r="L166" s="2" t="inlineStr"><is><t>acyklowir</t></is></c><c r="M166" s="2" t="inlineStr"><is><t>oseltamiwir</t></is></c><c r="N166" s="2" t="inlineStr" /><c r="O166" s="2" t="inlineStr" /><c r="P166" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q166" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="167"><c r="A167" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B167" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C167" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D167" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E167" s="2" t="inlineStr"><is><t>W terapii POChP u osób o wysokim ryzyku zaostrzeń i dużym nasileniu objawów (grupa</t></is></c><c r="F167" s="2" t="inlineStr"><is><t>bromek tiotropium z formoterolem i cyklezonidem</t></is></c><c r="G167" s="2" t="inlineStr"><is><t>budezonid z formoterolem</t></is></c><c r="H167" s="2" t="inlineStr"><is><t>bromek aklidynium z salmeterolem i flutikazonem</t></is></c><c r="I167" s="2" t="inlineStr"><is><t>bromek glikopironium z roflumilastem</t></is></c><c r="J167" s="2" t="inlineStr" /><c r="K167" s="2" t="inlineStr"><is><t>można zastosować:</t></is></c><c r="L167" s="2" t="inlineStr" /><c r="M167" s="2" t="inlineStr" /><c r="N167" s="2" t="inlineStr" /><c r="O167" s="2" t="inlineStr" /><c r="P167" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q167" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="168"><c r="A168" s="2" t="inlineStr"><is><t>UKŁAD ODDECHOWY</t></is></c><c r="B168" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C168" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D168" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E168" s="2" t="inlineStr"><is><t>Wskaż prawidłowe twierdzenie dotyczące farmakoterapii astmy oskrzelowej :</t></is></c><c r="F168" s="2" t="inlineStr"><is><t>wziewne glikokortykosteroidy zmniejszają częstość/liczbę hospitalizacji i umieralność z powodu astmy</t></is></c><c r="G168" s="2" t="inlineStr"><is><t>długodziałające wziewne betaadrenomimetyki w monoterapii mogą zwiększać ryzyko zgonu z powodu astmy</t></is></c><c r="H168" s="2" t="inlineStr"><is><t>kromony mogą być skuteczne u chorych ze skurczem oskrzeli wywoływanym przez wysiłek fizyczny</t></is></c><c r="I168" s="2" t="inlineStr" /><c r="J168" s="2" t="inlineStr" /><c r="K168" s="2" t="inlineStr"><is><t>leki przeciwleukotrienowe w monoterapii są bardziej skuteczne od wziewnych glikokortykosteroidów w małych dawkach</t></is></c><c r="L168" s="2" t="inlineStr" /><c r="M168" s="2" t="inlineStr" /><c r="N168" s="2" t="inlineStr" /><c r="O168" s="2" t="inlineStr" /><c r="P168" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q168" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="169"><c r="A169" s="2" t="inlineStr"><is><t>NADCIŚNIENIE TĘTNICZE</t></is></c><c r="B169" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C169" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D169" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E169" s="2" t="inlineStr"><is><t>W leczeniu wodobrzusza w przebiegu marskości wątroby wskazane jest stosowanie:</t></is></c><c r="F169" s="2" t="inlineStr"><is><t>furosemidu</t></is></c><c r="G169" s="2" t="inlineStr"><is><t>spironolaktonu</t></is></c><c r="H169" s="2" t="inlineStr"><is><t>karwedilolu</t></is></c><c r="I169" s="2" t="inlineStr" /><c r="J169" s="2" t="inlineStr" /><c r="K169" s="2" t="inlineStr"><is><t>ramiprylu</t></is></c><c r="L169" s="2" t="inlineStr" /><c r="M169" s="2" t="inlineStr" /><c r="N169" s="2" t="inlineStr" /><c r="O169" s="2" t="inlineStr" /><c r="P169" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q169" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="170"><c r="A170" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B170" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C170" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D170" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E170" s="2" t="inlineStr"><is><t>W leczeniu dny moczanowej należy:</t></is></c><c r="F170" s="2" t="inlineStr"><is><t>stosować dietę z ograniczeniem podaży mięs, podrobów i fruktozy</t></is></c><c r="G170" s="2" t="inlineStr"><is><t>objawowo stosować leki z grupy NLPZ</t></is></c><c r="H170" s="2" t="inlineStr" /><c r="I170" s="2" t="inlineStr" /><c r="J170" s="2" t="inlineStr" /><c r="K170" s="2" t="inlineStr"><is><t>podać jak najszybciej allopurynol przy podejrzeniu ostrego napadu</t></is></c><c r="L170" s="2" t="inlineStr"><is><t>w każdym przypadku bezobjawowej hiperurykemii stosować kolchicynę</t></is></c><c r="M170" s="2" t="inlineStr" /><c r="N170" s="2" t="inlineStr" /><c r="O170" s="2" t="inlineStr" /><c r="P170" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q170" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="171"><c r="A171" s="2" t="inlineStr"><is><t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t></is></c><c r="B171" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C171" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D171" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E171" s="2" t="inlineStr"><is><t>Zotarolimus:</t></is></c><c r="F171" s="2" t="inlineStr"><is><t>jest stosowany w stentach wieńcowych uwalniających lek</t></is></c><c r="G171" s="2" t="inlineStr" /><c r="H171" s="2" t="inlineStr" /><c r="I171" s="2" t="inlineStr" /><c r="J171" s="2" t="inlineStr" /><c r="K171" s="2" t="inlineStr"><is><t>jest rekombinowanym w pełni ludzkim przeciwciałem monoklonalnym</t></is></c><c r="L171" s="2" t="inlineStr"><is><t>nie może być stosowany łącznie z kwasem acetylosalicylowym</t></is></c><c r="M171" s="2" t="inlineStr"><is><t>neutralizuje biologiczną aktywność TNF</t></is></c><c r="N171" s="2" t="inlineStr" /><c r="O171" s="2" t="inlineStr" /><c r="P171" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q171" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="172"><c r="A172" s="2" t="inlineStr"><is><t>OTĘPIENIE</t></is></c><c r="B172" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C172" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D172" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E172" s="2" t="inlineStr"><is><t>W leczeniu choroby Alzheimera:</t></is></c><c r="F172" s="2" t="inlineStr"><is><t>w zaawansowanych przypadkach wskazane jest włączenie do leczenia antagonisty receptorów NMDA</t></is></c><c r="G172" s="2" t="inlineStr"><is><t>donepezil korzystnie wpływa na globalne zdolności intelektualne w łagodnych stadiach choroby</t></is></c><c r="H172" s="2" t="inlineStr" /><c r="I172" s="2" t="inlineStr" /><c r="J172" s="2" t="inlineStr" /><c r="K172" s="2" t="inlineStr"><is><t>stosuje się leki cholinolityczne</t></is></c><c r="L172" s="2" t="inlineStr"><is><t>istotną rolę odgrywa zastosowanie piracetamu</t></is></c><c r="M172" s="2" t="inlineStr" /><c r="N172" s="2" t="inlineStr" /><c r="O172" s="2" t="inlineStr" /><c r="P172" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q172" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="173"><c r="A173" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B173" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C173" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D173" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E173" s="2" t="inlineStr"><is><t>Przewlekłe stosowanie lorazepamu może spowodować:</t></is></c><c r="F173" s="2" t="inlineStr"><is><t>otępienie</t></is></c><c r="G173" s="2" t="inlineStr"><is><t>tolerancję na jego działanie</t></is></c><c r="H173" s="2" t="inlineStr"><is><t>uzależnienie psychiczne i fizyczne</t></is></c><c r="I173" s="2" t="inlineStr" /><c r="J173" s="2" t="inlineStr" /><c r="K173" s="2" t="inlineStr"><is><t>stan padaczkowy</t></is></c><c r="L173" s="2" t="inlineStr" /><c r="M173" s="2" t="inlineStr" /><c r="N173" s="2" t="inlineStr" /><c r="O173" s="2" t="inlineStr" /><c r="P173" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q173" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="174"><c r="A174" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B174" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C174" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D174" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E174" s="2" t="inlineStr"><is><t>Do leczenia ostrego zamknięcia kąta przesączania (potocznie ataku jaskry) można zastosować:</t></is></c><c r="F174" s="2" t="inlineStr"><is><t>tymolol</t></is></c><c r="G174" s="2" t="inlineStr"><is><t>acetazolamid</t></is></c><c r="H174" s="2" t="inlineStr"><is><t>mannitol</t></is></c><c r="I174" s="2" t="inlineStr" /><c r="J174" s="2" t="inlineStr" /><c r="K174" s="2" t="inlineStr"><is><t>zydowudynę</t></is></c><c r="L174" s="2" t="inlineStr" /><c r="M174" s="2" t="inlineStr" /><c r="N174" s="2" t="inlineStr" /><c r="O174" s="2" t="inlineStr" /><c r="P174" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q174" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="175"><c r="A175" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B175" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C175" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D175" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E175" s="2" t="inlineStr"><is><t>Do leczenia ostrego zamknięcia kąta przesączania (potocznie ataku jaskry) można zastosować:</t></is></c><c r="F175" s="2" t="inlineStr"><is><t>Timolol</t></is></c><c r="G175" s="2" t="inlineStr"><is><t>Acetazolamid</t></is></c><c r="H175" s="2" t="inlineStr"><is><t>Mannitol</t></is></c><c r="I175" s="2" t="inlineStr" /><c r="J175" s="2" t="inlineStr" /><c r="K175" s="2" t="inlineStr"><is><t>Zydowudynę</t></is></c><c r="L175" s="2" t="inlineStr" /><c r="M175" s="2" t="inlineStr" /><c r="N175" s="2" t="inlineStr" /><c r="O175" s="2" t="inlineStr" /><c r="P175" s="2" t="inlineStr"><is><t>KOLOKWIUM 3 – 2016/17 - 2 termin</t></is></c><c r="Q175" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="176"><c r="A176" s="2" t="inlineStr"><is><t>PADACZKA</t></is></c><c r="B176" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C176" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D176" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E176" s="2" t="inlineStr"><is><t>W leczeniu stanu padaczkowego:</t></is></c><c r="F176" s="2" t="inlineStr"><is><t>lekiem pierwszego rzutu jest diazepam i.v</t></is></c><c r="G176" s="2" t="inlineStr"><is><t>w przypadku postaci opornej na leczenie można zastosować wlew dożylny midazolamu</t></is></c><c r="H176" s="2" t="inlineStr" /><c r="I176" s="2" t="inlineStr" /><c r="J176" s="2" t="inlineStr" /><c r="K176" s="2" t="inlineStr"><is><t>nie powinno się stosować fenytoiny we wlewie dożylnym</t></is></c><c r="L176" s="2" t="inlineStr"><is><t>należy stosować duże dawki steroidów i.v</t></is></c><c r="M176" s="2" t="inlineStr" /><c r="N176" s="2" t="inlineStr" /><c r="O176" s="2" t="inlineStr" /><c r="P176" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q176" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="177"><c r="A177" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B177" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C177" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D177" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E177" s="2" t="inlineStr"><is><t>Charakterystyka Produktu Leczniczego (ChPL) zawiera informacje o:</t></is></c><c r="F177" s="2" t="inlineStr"><is><t>specjalnych środkach ostrożności podczas przechowywania produktu leczniczego</t></is></c><c r="G177" s="2" t="inlineStr"><is><t>właściwościach farmakokinetycznych leku</t></is></c><c r="H177" s="2" t="inlineStr"><is><t>dacie wydania pierwszego pozwolenia na dopuszczenie do obrotu</t></is></c><c r="I177" s="2" t="inlineStr" /><c r="J177" s="2" t="inlineStr" /><c r="K177" s="2" t="inlineStr"><is><t>cenie produktu leczniczego</t></is></c><c r="L177" s="2" t="inlineStr" /><c r="M177" s="2" t="inlineStr" /><c r="N177" s="2" t="inlineStr" /><c r="O177" s="2" t="inlineStr" /><c r="P177" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q177" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="178"><c r="A178" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B178" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C178" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D178" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E178" s="2" t="inlineStr"><is><t>Agencja Oceny Technologii Medycznych i Taryfikacji:</t></is></c><c r="F178" s="2" t="inlineStr"><is><t>wycenia procedury medyczne</t></is></c><c r="G178" s="2" t="inlineStr"><is><t>zajmuje stanowisko w sprawie skuteczności i bezpieczeństwa leków</t></is></c><c r="H178" s="2" t="inlineStr"><is><t>rekomenduje leki do refundacji</t></is></c><c r="I178" s="2" t="inlineStr" /><c r="J178" s="2" t="inlineStr" /><c r="K178" s="2" t="inlineStr"><is><t>rejestruje leki</t></is></c><c r="L178" s="2" t="inlineStr" /><c r="M178" s="2" t="inlineStr" /><c r="N178" s="2" t="inlineStr" /><c r="O178" s="2" t="inlineStr" /><c r="P178" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q178" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="179"><c r="A179" s="2" t="inlineStr"><is><t>FARMAKOLOGIA OGÓLNA I EBM</t></is></c><c r="B179" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C179" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D179" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E179" s="2" t="inlineStr"><is><t>W hierarchii badań naukowych:</t></is></c><c r="F179" s="2" t="inlineStr"><is><t>badania kohortowe mają wyższą pozycję niż serie przypadków</t></is></c><c r="G179" s="2" t="inlineStr" /><c r="H179" s="2" t="inlineStr" /><c r="I179" s="2" t="inlineStr" /><c r="J179" s="2" t="inlineStr" /><c r="K179" s="2" t="inlineStr"><is><t>metaanalizy są na tym samym poziomie co randomizowane badania kontrolowane</t></is></c><c r="L179" s="2" t="inlineStr"><is><t>najwyższą pozycję mają randomizowane badania kontrolowane</t></is></c><c r="M179" s="2" t="inlineStr"><is><t>badania kohortowe są na tym samym poziomie co randomizowane badania kliniczne</t></is></c><c r="N179" s="2" t="inlineStr" /><c r="O179" s="2" t="inlineStr" /><c r="P179" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q179" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="180"><c r="A180" s="2" t="inlineStr"><is><t>LEKI PRZECIWHISTAMINOWE</t></is></c><c r="B180" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C180" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D180" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E180" s="2" t="inlineStr"><is><t>Desloratadyna:</t></is></c><c r="F180" s="2" t="inlineStr"><is><t>selektywnie blokuje receptory H1</t></is></c><c r="G180" s="2" t="inlineStr"><is><t>ma zastosowanie w leczeniu przewlekłego alergicznego nieżytu nosa</t></is></c><c r="H180" s="2" t="inlineStr" /><c r="I180" s="2" t="inlineStr" /><c r="J180" s="2" t="inlineStr" /><c r="K180" s="2" t="inlineStr"><is><t>dobrze przenika przez barierę krew- mózg</t></is></c><c r="L180" s="2" t="inlineStr"><is><t>ma znaczące działanie proarytmiczne</t></is></c><c r="M180" s="2" t="inlineStr" /><c r="N180" s="2" t="inlineStr" /><c r="O180" s="2" t="inlineStr" /><c r="P180" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q180" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="181"><c r="A181" s="2" t="inlineStr"><is><t>LEKI MOCZOPĘDNE</t></is></c><c r="B181" s="2" t="inlineStr"><is><t>Farmakokinetyka</t></is></c><c r="C181" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D181" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E181" s="2" t="inlineStr"><is><t>Mannitol podany iv. zmniejsza:</t></is></c><c r="F181" s="2" t="inlineStr"><is><t>ciśnienie wewnątrzczaszkowe</t></is></c><c r="G181" s="2" t="inlineStr" /><c r="H181" s="2" t="inlineStr" /><c r="I181" s="2" t="inlineStr" /><c r="J181" s="2" t="inlineStr" /><c r="K181" s="2" t="inlineStr"><is><t>ciśnienie osmotyczne płynu zewnątrzkomórkowego</t></is></c><c r="L181" s="2" t="inlineStr"><is><t>wydalanie sodu i chlorków</t></is></c><c r="M181" s="2" t="inlineStr"><is><t>filtrację nerkową</t></is></c><c r="N181" s="2" t="inlineStr" /><c r="O181" s="2" t="inlineStr" /><c r="P181" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q181" s="2" t="inlineStr"><is><t>niska</t></is></c></row><row r="182"><c r="A182" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B182" s="2" t="inlineStr"><is><t>Wskazania</t></is></c><c r="C182" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D182" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E182" s="2" t="inlineStr"><is><t>Podanie inhibitorów wychwytu zwrotnego serotoniny (SSRI) jest uzasadnione u pacjentów z:</t></is></c><c r="F182" s="2" t="inlineStr"><is><t>lękiem uogólnionym</t></is></c><c r="G182" s="2" t="inlineStr"><is><t>chorobą afektywną dwubiegunową</t></is></c><c r="H182" s="2" t="inlineStr"><is><t>nerwicą natręctw</t></is></c><c r="I182" s="2" t="inlineStr"><is><t>chorobą afektywną jednobiegunową</t></is></c><c r="J182" s="2" t="inlineStr" /><c r="K182" s="2" t="inlineStr" /><c r="L182" s="2" t="inlineStr" /><c r="M182" s="2" t="inlineStr" /><c r="N182" s="2" t="inlineStr" /><c r="O182" s="2" t="inlineStr" /><c r="P182" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q182" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="183"><c r="A183" s="2" t="inlineStr"><is><t>LEKI PRZECIWDEPRESYJNE</t></is></c><c r="B183" s="2" t="inlineStr"><is><t>Struktura chemiczna</t></is></c><c r="C183" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D183" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E183" s="2" t="inlineStr"><is><t>Do wspólnych cech wenlafaksyny i amitryptyliny należy:</t></is></c><c r="F183" s="2" t="inlineStr"><is><t>hamowanie wychwytu zwrotnego serotoniny i noradrenaliny</t></is></c><c r="G183" s="2" t="inlineStr" /><c r="H183" s="2" t="inlineStr" /><c r="I183" s="2" t="inlineStr" /><c r="J183" s="2" t="inlineStr" /><c r="K183" s="2" t="inlineStr"><is><t>trójpierścieniowa budowa chemiczna</t></is></c><c r="L183" s="2" t="inlineStr"><is><t>konieczność znacznych ograniczeń dietetycznych podczas ich stosowania ze względu na ryzyko wystąpienia tzw. zespołu serowego (cheese effect)</t></is></c><c r="M183" s="2" t="inlineStr"><is><t>antagonizm wobec receptorów muskarynowych M1</t></is></c><c r="N183" s="2" t="inlineStr" /><c r="O183" s="2" t="inlineStr" /><c r="P183" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q183" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="184"><c r="A184" s="2" t="inlineStr"><is><t>LEKI IMMUNOSUPRESYJNE</t></is></c><c r="B184" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C184" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D184" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E184" s="2" t="inlineStr"><is><t>Leki, które hamują kompleks kalcyneuryny to:</t></is></c><c r="F184" s="2" t="inlineStr"><is><t>cyklosporyna</t></is></c><c r="G184" s="2" t="inlineStr"><is><t>takrolimus</t></is></c><c r="H184" s="2" t="inlineStr" /><c r="I184" s="2" t="inlineStr" /><c r="J184" s="2" t="inlineStr" /><c r="K184" s="2" t="inlineStr"><is><t>talidomid</t></is></c><c r="L184" s="2" t="inlineStr"><is><t>mykofenolan mofetylu</t></is></c><c r="M184" s="2" t="inlineStr" /><c r="N184" s="2" t="inlineStr" /><c r="O184" s="2" t="inlineStr" /><c r="P184" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q184" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="185"><c r="A185" s="2" t="inlineStr"><is><t>ZABURZENIA RYTMU SERCA</t></is></c><c r="B185" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C185" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D185" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E185" s="2" t="inlineStr"><is><t>Lacydypina:</t></is></c><c r="F185" s="2" t="inlineStr"><is><t>zmniejsza obciążenie następcze serca</t></is></c><c r="G185" s="2" t="inlineStr" /><c r="H185" s="2" t="inlineStr" /><c r="I185" s="2" t="inlineStr" /><c r="J185" s="2" t="inlineStr" /><c r="K185" s="2" t="inlineStr"><is><t>ma silne działanie inotropowe ujemne</t></is></c><c r="L185" s="2" t="inlineStr"><is><t>ma działanie dromotropowe ujemne</t></is></c><c r="M185" s="2" t="inlineStr"><is><t>ma działanie chronotropowe dodatnie</t></is></c><c r="N185" s="2" t="inlineStr" /><c r="O185" s="2" t="inlineStr" /><c r="P185" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q185" s="2" t="inlineStr"><is><t>srednia</t></is></c></row><row r="186"><c r="A186" s="2" t="inlineStr"><is><t>CHOROBA NIEDOKRWIENNA SERCA</t></is></c><c r="B186" s="2" t="inlineStr"><is><t>Klasyfikacja</t></is></c><c r="C186" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D186" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E186" s="2" t="inlineStr"><is><t>Do donorów tlenku azotu należy:</t></is></c><c r="F186" s="2" t="inlineStr"><is><t>nikorandil</t></is></c><c r="G186" s="2" t="inlineStr"><is><t>molsidomina</t></is></c><c r="H186" s="2" t="inlineStr"><is><t>diazotan izosorbitolu</t></is></c><c r="I186" s="2" t="inlineStr" /><c r="J186" s="2" t="inlineStr" /><c r="K186" s="2" t="inlineStr"><is><t>trimetazydyna</t></is></c><c r="L186" s="2" t="inlineStr" /><c r="M186" s="2" t="inlineStr" /><c r="N186" s="2" t="inlineStr" /><c r="O186" s="2" t="inlineStr" /><c r="P186" s="2" t="inlineStr"><is><t>EGZ 2018 I termin</t></is></c><c r="Q186" s="2" t="inlineStr"><is><t>wysoka</t></is></c></row><row r="187"><c r="A187" s="2" t="inlineStr"><is><t>FARMAKOKINETYKA</t></is></c><c r="B187" s="2" t="inlineStr"><is><t>Sposób podania</t></is></c><c r="C187" s="2" t="inlineStr"><is><t>lekarski</t></is></c><c r="D187" s="2" t="inlineStr"><is><t>testowe</t></is></c><c r="E187" s="2" t="inlineStr"><is><t>Względna dostępność biologiczna leku (biorównoważność) może być określona przez porównanie AUC:</t></is></c><c r="F187" s="2" t="inlineStr"><is><t>leku wzorcowego podanego drogą pozanaczyniową i dożylnie</t></is></c><c r="G187" s="2" t="inlineStr"><is><t>leku wzorcowego i badanego podanych tą samą drogą</t></is></c><c r="H187" s="2" t="inlineStr" /><c r="I187" s="2" t="inlineStr" /><c r="J187" s="2" t="inlineStr" /><c r="K187" s="2" t="inlineStr"><is><t>tylko leków podawanych drogą dożylną</t></is></c><c r="L187" s="2" t="inlineStr"><is><t>leku badanego podanego drogą pozanaczyniową i wzorcowego podanego dożylnie</t></is></c><c r="M187" s="2" t="inlineStr" /><c r="N187" s="2" t="inlineStr" /><c r="O187" s="2" t="inlineStr" /><c r="P187" s="2" t="i